<commit_message>
daily-news auto update 2026-05-28 (2026-05-27 23:13)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -110,7 +110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -137,6 +137,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1655,7 +1658,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1743,6 +1746,663 @@
       <c r="B2" s="8" t="inlineStr">
         <is>
           <t>（例）任天堂、Switch 2の累計販売数を発表 — 初年度XX万台へ</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>『007 First Light』5月27日発売、Metacritic88点で14年ぶりのBondゲーム高評価</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>https://www.thefpsreview.com/2026/05/27/007-first-light-is-out-today-and-critics-love-it-io-interactives-best-work-since-hitman/</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
+        <is>
+          <t>Hitmanで知られるIO Interactiveが、Activision版（2010年作）以降14年途絶えていたJames Bondゲームの権利を獲得し、若き26歳のBondを描くオリジンストーリーとして開発。Patrick Gibsonが声と演技を担当。</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="inlineStr">
+        <is>
+          <t>PS5/Xbox Series X|S/PC向けに2026年5月27日発売。Metacritic88点（50レビュー）、OpenCritic89点・推奨率97%と高評価。Hitman譲りのシステミックなステルスとUncharted風のシネマティック演出を融合。Switch 2版は夏に延期。</t>
+        </is>
+      </c>
+      <c r="F3" s="13" t="inlineStr">
+        <is>
+          <t>Metacritic 88点（過去30年のBondゲーム最高評価）
+IOI独立スタジオによる初の大型IPライセンス成功例
+ステルス+映画的演出のハイブリッドが評価
+Switch 2版は2026年Q3に延期</t>
+        </is>
+      </c>
+      <c r="G3" s="13" t="inlineStr">
+        <is>
+          <t>IOIはHitmanの自社IPに加えBond・007という大型ライセンスを獲得し、シングルプレイヤー大作スタジオとしての地位を確立する見込み。続編・シリーズ化が見込まれる。</t>
+        </is>
+      </c>
+      <c r="H3" s="13" t="inlineStr">
+        <is>
+          <t>シングルプレイヤー大作の収益構造、IPライセンス戦略</t>
+        </is>
+      </c>
+      <c r="I3" s="13" t="inlineStr">
+        <is>
+          <t>IO Interactive, MGM, Amazon, Sony, Microsoft</t>
+        </is>
+      </c>
+      <c r="J3" s="13" t="inlineStr">
+        <is>
+          <t>007 First Light, James Bond, Hitman</t>
+        </is>
+      </c>
+      <c r="K3" s="13" t="inlineStr">
+        <is>
+          <t>新作,海外</t>
+        </is>
+      </c>
+      <c r="L3" s="13" t="inlineStr">
+        <is>
+          <t>Switch 2版は2026年Q3予定</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>スクエニ『DRAGON QUEST XII: Beyond Dreams』発表、ドラクエ40周年で開発体制を刷新リスタート</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>https://gameinformer.com/2026/05/27/dragon-quest-xiis-development-was-restarted-from-scratch-and-it-has-a-new-name-and</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>ドラゴンクエスト40周年（1986年5月27日初代発売）を記念して開催されたDragon Quest Dayで、長期沈黙状態だった『DQXII』の進捗を初公開。元タイトル『The Flames of Fate』から『Beyond Dreams』へ改題し、開発体制を一新して事実上ゼロから再始動した経緯を斎藤プロデューサーが説明。</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="inlineStr">
+        <is>
+          <t>「不思議な夢を体験する主人公の冒険」を新コンセプトに据え、故・鳥山明のキャラデザインと故・すぎやまこういちの楽曲を継承。プラットフォーム・発売時期は未発表で「もう少し待ってほしい」と要請。同時に『DQ XI S』のSwitch 2版、『DQモンスターズ4 枯れ木の国のビアンカ・フローラ』も発表。</t>
+        </is>
+      </c>
+      <c r="F4" s="13" t="inlineStr">
+        <is>
+          <t>シリーズ完全新作の開発リスタート（コンセプト・体制刷新）
+タイトル変更（Flames of Fate → Beyond Dreams）
+鳥山明・すぎやまこういち遺産の継承
+プラットフォーム・発売時期は未定
+DQM4、DQXI S（Switch 2版）も同時発表</t>
+        </is>
+      </c>
+      <c r="G4" s="13" t="inlineStr">
+        <is>
+          <t>本作リリースまで「もう少し」とする一方、開発の長期化リスクは残る。一方でDQM4・DQXI S（Switch 2版）など派生・移植で40周年商戦をつなぐ戦略が見込まれる。</t>
+        </is>
+      </c>
+      <c r="H4" s="13" t="inlineStr">
+        <is>
+          <t>大型IPの長期開発マネジメント、ナンバリングと派生の収益バランス</t>
+        </is>
+      </c>
+      <c r="I4" s="13" t="inlineStr">
+        <is>
+          <t>スクウェア・エニックス, ソニー, 任天堂</t>
+        </is>
+      </c>
+      <c r="J4" s="13" t="inlineStr">
+        <is>
+          <t>ドラゴンクエスト, DQXII Beyond Dreams, DQM4, DQXI S</t>
+        </is>
+      </c>
+      <c r="K4" s="13" t="inlineStr">
+        <is>
+          <t>新作,国内</t>
+        </is>
+      </c>
+      <c r="L4" s="13" t="inlineStr">
+        <is>
+          <t>Dragon Quest 40周年企画</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>任天堂、Switch 2の日本国内価格を5月25日付で¥49,980→¥59,980（+20%）に改定</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>https://www.nintendo.co.jp/corporate/release/en/2026/260508.html</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>AI需要によるメモリ価格高騰、米国の輸入電子機器に対する関税、為替変動を主因として、任天堂が日本市場のSwitch 2本体および周辺機器の希望小売価格を引き上げ。日本市場が世界に先駆けて値上げ実施。</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>5月25日から日本国内のSwitch 2本体MSRPが¥49,980から¥59,980（約+20%）に改定。米国・欧州での同種値上げは2026年9月1日を予定。日本ユーザーは世界で最も急激な値上げ幅を負担する形に。</t>
+        </is>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
+        <is>
+          <t>値上げ幅は日本+20%（世界最高）
+米国は$449.99→$499.99、9月1日施行
+要因はAI由来のメモリ高騰・関税・為替
+旧Switchの一部周辺機器も値上げ</t>
+        </is>
+      </c>
+      <c r="G5" s="13" t="inlineStr">
+        <is>
+          <t>短期は需要前倒しによる増収、中長期は普及ペース鈍化リスク。ソフト価格の据え置き／引上げ判断、Switch Online料金改定の余地、競合のクラウド／低価格戦略への影響に注目。</t>
+        </is>
+      </c>
+      <c r="H5" s="13" t="inlineStr">
+        <is>
+          <t>ハードウェア価格戦略、為替・関税が消費財に与える影響</t>
+        </is>
+      </c>
+      <c r="I5" s="13" t="inlineStr">
+        <is>
+          <t>任天堂, ソニー, マイクロソフト</t>
+        </is>
+      </c>
+      <c r="J5" s="13" t="inlineStr">
+        <is>
+          <t>Nintendo Switch 2</t>
+        </is>
+      </c>
+      <c r="K5" s="13" t="inlineStr">
+        <is>
+          <t>業績,国内,規制</t>
+        </is>
+      </c>
+      <c r="L5" s="13" t="inlineStr">
+        <is>
+          <t>米欧は2026年9月1日に値上げ予定</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>任天堂2026年3月期決算、Switch 2効果で売上+98.6%・営業利益+27.5%の増収増益</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>https://www.gamebusiness.jp/article/2026/04/30/26816.html</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>2025年6月発売のSwitch 2が通期業績に初めて寄与する決算。Switch 2のローンチ・タイトル群（マリオカート、ゼルダ等）と既存Switchの長期販売効果が重なる構造。5月8日に決算発表。</t>
+        </is>
+      </c>
+      <c r="E6" s="13" t="inlineStr">
+        <is>
+          <t>売上高2兆3130億円（前期比+98.6%）、営業利益3601億円（同+27.5%）、経常利益5421億円（+45.6%）、当期純利益4240億円（+52.1%）。Switch 2の貢献で過去最高水準の売上を更新する一方、ローンチコスト先行で利益率は売上ほど伸びず。</t>
+        </is>
+      </c>
+      <c r="F6" s="13" t="inlineStr">
+        <is>
+          <t>売上ほぼ倍増（+98.6%）の歴史的決算
+営業利益は+27.5%・利益率は減少
+Switch 2初年度販売寄与が主因
+5月25日の日本値上げで来期は単価UP想定</t>
+        </is>
+      </c>
+      <c r="G6" s="13" t="inlineStr">
+        <is>
+          <t>Switch 2の継続的ソフト供給と価格改定後の販売推移が来期業績の鍵。米欧値上げの9月施行を踏まえ、Q2以降のセルスルー数字とパーティ／ファースト勢のラインアップ動向に注目。</t>
+        </is>
+      </c>
+      <c r="H6" s="13" t="inlineStr">
+        <is>
+          <t>コンソールサイクルの収益貢献カーブ、円安・関税環境下の収益管理</t>
+        </is>
+      </c>
+      <c r="I6" s="13" t="inlineStr">
+        <is>
+          <t>任天堂, ソニー, バンダイナムコ</t>
+        </is>
+      </c>
+      <c r="J6" s="13" t="inlineStr">
+        <is>
+          <t>Nintendo Switch 2, マリオ, ゼルダ</t>
+        </is>
+      </c>
+      <c r="K6" s="13" t="inlineStr">
+        <is>
+          <t>業績,国内</t>
+        </is>
+      </c>
+      <c r="L6" s="13" t="inlineStr">
+        <is>
+          <t>2026年5月8日決算発表</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Q1 2026のゲーム業界M&amp;A総額77億ドル、SavvyのMoonton 60億ドル買収が牽引</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>https://respawn.outlookindia.com/gaming/gaming-news/games-ma-surges-to-77b-as-console-revenue-climbs</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>サウジSavvy Games Group（PIF傘下）がモバイル大手Moontonを60億ドルで買収する案件が、四半期総額を押し上げ。EAの550億ドルTOB（2025年9月発表）に続き、PIFを軸とした大型ゲーム投資が継続。</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>2026年Q1のゲームM&amp;Aは52件・総額77億ドル。ScopelyがLoom Gamesを10億ドル、NCSoftがJustPlayの70%を2.02億ドル、MattelがMattel163完全子会社化を1.59億ドルで実施。モバイル領域の再編が中心。</t>
+        </is>
+      </c>
+      <c r="F7" s="13" t="inlineStr">
+        <is>
+          <t>Q1総額77億ドル・52件
+Moonton（Savvy 60億ドル）が最大案件
+モバイル中心の再編が継続
+PIF/Savvyによる業界集約が加速
+EA非公開化との並行進行</t>
+        </is>
+      </c>
+      <c r="G7" s="13" t="inlineStr">
+        <is>
+          <t>PIF/Savvyを軸にしたグローバル大型再編が今後も継続する見込み。日本企業（バンナム/コナミ/セガ）のIP・スタジオが対象となる可能性、または逆に北米買収を行う動きにも注目。</t>
+        </is>
+      </c>
+      <c r="H7" s="13" t="inlineStr">
+        <is>
+          <t>メガディール時代のゲーム業界再編構造、PIF/SWFのゲーム投資戦略</t>
+        </is>
+      </c>
+      <c r="I7" s="13" t="inlineStr">
+        <is>
+          <t>Savvy Games Group, PIF, Moonton, Scopely, NCSoft, Mattel</t>
+        </is>
+      </c>
+      <c r="J7" s="13" t="inlineStr">
+        <is>
+          <t>Mobile Legends: Bang Bang</t>
+        </is>
+      </c>
+      <c r="K7" s="13" t="inlineStr">
+        <is>
+          <t>M&amp;A,海外</t>
+        </is>
+      </c>
+      <c r="L7" s="13" t="inlineStr">
+        <is>
+          <t>EA 550億ドル買収案件と並行</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>NetEase Q1 2026決算、売上RMB306億（+6.1%）・ゲーム部門RMB257億（+6.9%）で安定成長</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/0001110646/000110465926064764/tm2615053d1_ex99-1.htm</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>5月21日にNetEaseがQ1 2026決算を発表。Marvel Rivals等の新規IPの貢献に加え、既存タイトル（Identity V、Knives Out等）の安定収益が継続。中国本土の版号交付の正常化も追い風。</t>
+        </is>
+      </c>
+      <c r="E8" s="13" t="inlineStr">
+        <is>
+          <t>売上高306億元（約44億ドル、前期比+6.1%）、ゲーム・付随サービス収益257億元（約37億ドル、+6.9%）と二桁成長には届かないものの堅調。前四半期比でもプラス成長を維持し、グローバルゲーム企業として安定した実績を示した。</t>
+        </is>
+      </c>
+      <c r="F8" s="13" t="inlineStr">
+        <is>
+          <t>売上+6.1%・ゲーム部門+6.9%
+Marvel Rivalsの寄与が継続
+中国マクロ低迷でも安定収益
+版号交付正常化が支援要因
+グローバル展開の継続強化</t>
+        </is>
+      </c>
+      <c r="G8" s="13" t="inlineStr">
+        <is>
+          <t>MMORPGからモバイル・PC・コンソール横断のIP育成へシフト中。Marvel Rivalsを軸にした北米シェア拡大が継続する見込みで、Tencentとのグローバル競争が加速。</t>
+        </is>
+      </c>
+      <c r="H8" s="13" t="inlineStr">
+        <is>
+          <t>中国ゲーム大手のIP輸出戦略、版号制度下での投資判断</t>
+        </is>
+      </c>
+      <c r="I8" s="13" t="inlineStr">
+        <is>
+          <t>NetEase, Marvel, Disney, Tencent</t>
+        </is>
+      </c>
+      <c r="J8" s="13" t="inlineStr">
+        <is>
+          <t>Marvel Rivals, Identity V, Knives Out</t>
+        </is>
+      </c>
+      <c r="K8" s="13" t="inlineStr">
+        <is>
+          <t>業績,海外</t>
+        </is>
+      </c>
+      <c r="L8" s="13" t="inlineStr">
+        <is>
+          <t>5月21日発表</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>Take-Two CEO、『GTA6』を2026年11月19日発売と再確認 — 「これ以上の延期なし」</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>https://www.theshortcut.com/p/gta-6-release-date-delay-update</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>もともと2025年秋発売予定だったGTA6は、Rockstarが2026年5月26日に延期、その後さらに11月19日へと延期。当初計画から約18ヶ月遅延。Take-Twoは次期会計年度の売上82億ドルをGTA6launchで見込む。</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>5月のTake-Two決算発表後、CEO Strauss Zelnickが「GTA6は2026年11月19日に必ず発売、これ以上の延期はない」と明言。Rockstarが「最高品質のための限定的な追加時間」を必要としたと説明し、次トレーラー公開時期も示唆。</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>発売日2026年11月19日を再確認
+これ以上の延期はないと明言
+当初予定から約18ヶ月遅延
+T2の来期売上見通し82億ドル
+PS5/Xbox Series X|S対応（PCは後日）</t>
+        </is>
+      </c>
+      <c r="G9" s="13" t="inlineStr">
+        <is>
+          <t>11月発売を前提に北米・欧州のホリデー商戦が動く。前後の大型タイトル（Marvel's Wolverine、Forza Horizon 6等）の発売タイミング再調整、コンソール需要の集中、Switch 2版の有無に注目。</t>
+        </is>
+      </c>
+      <c r="H9" s="13" t="inlineStr">
+        <is>
+          <t>メガフランチャイズのローンチ経済、コンソール販売との相関</t>
+        </is>
+      </c>
+      <c r="I9" s="13" t="inlineStr">
+        <is>
+          <t>Take-Two Interactive, Rockstar Games, ソニー, マイクロソフト</t>
+        </is>
+      </c>
+      <c r="J9" s="13" t="inlineStr">
+        <is>
+          <t>Grand Theft Auto VI</t>
+        </is>
+      </c>
+      <c r="K9" s="13" t="inlineStr">
+        <is>
+          <t>新作,業績,海外</t>
+        </is>
+      </c>
+      <c r="L9" s="13" t="inlineStr">
+        <is>
+          <t>PCは後日対応想定</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>Behaviour、『Dead by Daylight』10周年でJason Voorhees正式参戦を発表（6月17日実装）</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>https://www.dreadcentral.com/gaming/573864/friday-the-13th-icon-jason-voorhees-officially-joins-dead-by-daylight-this-june/</t>
+        </is>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>DBD 10周年配信でJason Voorhees（『13日の金曜日』）のキラー参戦を正式発表。長年ファンが望んでいたコラボがついに実現。法廷係争で停滞していたFriday the 13th IPの利用問題が解決した可能性を示唆。</t>
+        </is>
+      </c>
+      <c r="E10" s="13" t="inlineStr">
+        <is>
+          <t>5月26日からPTB（Steam版公開テスト）を開始し、6月17日に新チャプター『Dead by Daylight: Jason』を正式リリース。Jasonには「Omnipresent Evil」（瞬間移動・奇襲）と「Improvised Carnage」（投擲攻撃）の2大能力を実装。コスチューム3種も配信。</t>
+        </is>
+      </c>
+      <c r="F10" s="13" t="inlineStr">
+        <is>
+          <t>10周年記念キラーとしてJason参戦
+PTB 5月26日 / 本実装6月17日
+Friday the 13th IPライセンスを取得
+Omnipresent Evilで瞬間移動・奇襲
+DLCコスチューム3種</t>
+        </is>
+      </c>
+      <c r="G10" s="13" t="inlineStr">
+        <is>
+          <t>ホラーIPコラボDLC路線を強化することでGaaSとしてのDBDの寿命を延伸。Friday the 13thゲームの再展開可能性、他IPのコラボ拡大が見込まれる。</t>
+        </is>
+      </c>
+      <c r="H10" s="13" t="inlineStr">
+        <is>
+          <t>GaaSとIPコラボの相乗効果、ホラーIPの法務クリアランス</t>
+        </is>
+      </c>
+      <c r="I10" s="13" t="inlineStr">
+        <is>
+          <t>Behaviour Interactive, Sumo Group, Paramount</t>
+        </is>
+      </c>
+      <c r="J10" s="13" t="inlineStr">
+        <is>
+          <t>Dead by Daylight, Friday the 13th, Jason Voorhees</t>
+        </is>
+      </c>
+      <c r="K10" s="13" t="inlineStr">
+        <is>
+          <t>新作,海外</t>
+        </is>
+      </c>
+      <c r="L10" s="13" t="inlineStr">
+        <is>
+          <t>10周年記念チャプター</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>EVO Japan 2026閉幕、『スト6』ヤマグチ・『鉄拳8』iKARiが新王者、『2XKO』も初開催</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>https://esports-world.jp/report/61158</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>国内最大級の格闘ゲーム大会EVO Japan 2026が5月1-3日に東京ビッグサイトで開催。Riot Gamesの新作『2XKO』が初の公式競技種目として登場し、北米Hikariが優勝。日本のFGCシーンの国際的注目度が継続。</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
+          <t>『ストリートファイター6』はヤマグチ、『鉄拳8』はiKARiがGFを制し新王者に。『北斗の拳』『2XKO』など多彩なタイトルでドラマが生まれ、国内外プレイヤー・ファンを動員。Riot Games『2XKO』のEVO Japanデビューが特に注目を集めた。</t>
+        </is>
+      </c>
+      <c r="F11" s="13" t="inlineStr">
+        <is>
+          <t>『スト6』ヤマグチ優勝、『鉄拳8』iKARi優勝
+『2XKO』初の公式競技種目化
+北米Hikariが2XKO優勝
+3日間で東京ビッグサイトに集客
+格闘ゲーム国際大会の継続</t>
+        </is>
+      </c>
+      <c r="G11" s="13" t="inlineStr">
+        <is>
+          <t>Riot『2XKO』の正式リリース時期・E-sports経済圏拡大、ストリーマー文化と既存FGCの融合、JeSU/CESAによる賞金規制議論の動向に注目。</t>
+        </is>
+      </c>
+      <c r="H11" s="13" t="inlineStr">
+        <is>
+          <t>格闘ゲームeスポーツの経済構造、Riotの新規参入インパクト</t>
+        </is>
+      </c>
+      <c r="I11" s="13" t="inlineStr">
+        <is>
+          <t>Capcom, Bandai Namco, Riot Games, セガ, KONAMI</t>
+        </is>
+      </c>
+      <c r="J11" s="13" t="inlineStr">
+        <is>
+          <t>Street Fighter 6, Tekken 8, 2XKO, 北斗の拳</t>
+        </is>
+      </c>
+      <c r="K11" s="13" t="inlineStr">
+        <is>
+          <t>eスポーツ,国内</t>
+        </is>
+      </c>
+      <c r="L11" s="13" t="inlineStr">
+        <is>
+          <t>5月1-3日、東京ビッグサイト</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Morgan Stanley：AI活用でゲーム業界は220億ドルの利益機会、開発期間短縮と費用削減を予測</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>https://www.morganstanley.com/insights/articles/ai-gaming-22-billion-industry-earning-potential-2026</t>
+        </is>
+      </c>
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>Morgan Stanley Researchが、生成AI・AIエージェントがゲーム制作に与える経済効果について新たなレポートを公表。AAA制作費の高騰と工期長期化（GTA6が約18ヶ月延期した事象に象徴される）を背景に、AIによる生産性向上が中核論点に。</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="inlineStr">
+        <is>
+          <t>AI活用により、業界全体で約220億ドルの追加利益機会が生まれると試算。スクリプトベースのパスファインディングから深層学習による動的・パーソナライズドな環境生成へ。GDC 2026でもAIエージェントによる「次世代エージェンティック・ゲーム」が大きなテーマに。</t>
+        </is>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
+        <is>
+          <t>AI効果220億ドルの利益機会試算
+開発工期と制作費の同時削減
+NPC・レベルデザインの自動生成
+AIエージェント主導ゲームの台頭
+GDC 2026の主要テーマに</t>
+        </is>
+      </c>
+      <c r="G12" s="13" t="inlineStr">
+        <is>
+          <t>ファースト・サードパーティ各社のAIパイプライン整備、AI生成コンテンツの著作権・労組対応、AIモデル提供者（NVIDIA、Google、Microsoft）とゲーム会社の連携深化に注目。</t>
+        </is>
+      </c>
+      <c r="H12" s="13" t="inlineStr">
+        <is>
+          <t>ゲーム開発におけるAI活用、生成AIと著作権・労務問題</t>
+        </is>
+      </c>
+      <c r="I12" s="13" t="inlineStr">
+        <is>
+          <t>Morgan Stanley, NVIDIA, Google, Microsoft, ソニー, Embracer, EA</t>
+        </is>
+      </c>
+      <c r="J12" s="13" t="inlineStr">
+        <is>
+          <t>（業界全般）</t>
+        </is>
+      </c>
+      <c r="K12" s="13" t="inlineStr">
+        <is>
+          <t>技術,海外</t>
+        </is>
+      </c>
+      <c r="L12" s="13" t="inlineStr">
+        <is>
+          <t>AAA制作費高騰への解</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
weekly-trends update (2026-05-27 23:25)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -836,7 +836,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -882,6 +882,191 @@
       <c r="G1" s="7" t="inlineStr">
         <is>
           <t>参考リンク</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ライブサービス大量終了：2026年上半期で52本シャットダウン</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Game RantとDualShockersの集計によれば、2026年は半期で52本のライブサービスゲームがサービス終了。Destiny 2は最終ライブパッチを受領、Amazon GamesのMMO『New World』は7月にIAP停止し2027年1月にサーバー閉鎖予定、VRソーシャル代表格『Rec Room』も6月1日終了。BungieやUbisoftが提唱したGaaS最大化路線が、プレイヤー時間の有限性とリテンション飽和に直面し、業界全体で同時多発的に撤退している。コンシューマー側も『プレイ済み大型タイトルから新規GaaSへの移籍コストが釣り合わない』として、ソロ＋簡易Co-op型に需要が回帰している。</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Bungie, Ubisoft, Amazon Games, Rec Room</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>GaaS隆盛の前提だった『LTVの右肩上がり』が崩れた背景には、(1)既存タイトルへの時間ロックイン、(2)Game Pass等サブスクの可処分時間奪取、(3)F2P＋FOMO設計疲労、(4)開発期間長期化による初動失敗の致命傷化、がある。残るのは『短時間集中型』と『コミュニティ駆動型』の2極化。</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>他業界SaaSの『リテンション幻想終焉』と同型構造。可処分時間市場として再定義するべき。</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>https://gamerant.com/games-shut-down-2026-list-highguard-anthem/, https://www.dualshockers.com/its-officially-the-end-of-an-era-for-live-service-games/</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ARC Raiders現象：PvE協力エクストラクションが新主流に</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Embark Studios開発／Nexon配信の『ARC Raiders』が2025年11月の発売後、Steamで481,966同接のエクストラクションシューター記録を樹立、2026年1月には全プラットフォーム同接96万、週間アクティブ600万を達成。Nexonの2026年Q1は売上1522億円・営業利益582億円で過去最高、ARC Raidersとメイプルストーリーが牽引。Helldivers 2がCo-op PvEで切り開いた市場をARC Raidersが拡大しており、Exoborne／Project Spectrum／Toxic Commandoなど後続が続く。</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Embark Studios, Nexon, Arrowhead (Helldivers 2)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>PvP型バトロワの飽和に対し、PvE協力＋エクストラクションは『学習可能なAI挙動』『3〜4人少人数』『ボイチャ前提のソーシャル接着』という設計で残存。タルコフ系の硬派さを薄めつつ、Co-op文化を組み込んだハイブリッド型がジャンルとして定着しつつある。</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>PvE再評価は『勝ち負けではなく物語化されるプレイ体験』へのシフト。配信文化との相性も高い。</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>https://www.pcgamer.com/games/third-person-shooter/arc-raiders-had-nearly-1-million-concurrent-players-in-january-and-around-6-million-weekly-active-users-claims-nexon-putting-the-extraction-shooter-on-par-with-some-of-the-biggest-mmos/, https://breach.gg/blog/helldivers-2-weekly-2026-04-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Switch 2サードパーティ売上+76%・ユニット-2.5%の歪み</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Ampere Analysisによれば、Switch1+2のサードパーティソフト売上はQ2-Q4 2025で23億ドル、前年比+76%。一方でユニット販売数は-2.5%、つまり平均販売単価が約81%上昇したことで売上が押し上げられた構図。Warner Bros.が最大のサードパーティパブリッシャー、続いてBandai Namco、EA。Nintendoは2026年4月以降にサードパーティ主導の大型ローンチを多数予定しており、Switch 2は2026年末で累計31百万台想定。</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Nintendo, Warner Bros., Bandai Namco, EA, Ampere Analysis</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>『AAA価格を呑むコアユーザー比率』が上がり、ライトユーザーは値ごろ感のあるバンドル/旧作リマスターへ。プラットフォーマーが価格弾力性をテストできるフェーズに入り、$70→$80標準化への試金石になっている。ユニット減でも収益増を成立させるのは、Steamのフロントカタログ高価格化と同様の現象。</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>ハード成功＝ソフトユニット増、という前提が崩れている。ARPU/ARPDAU指標へ評価軸が移行する兆候。</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>https://www.thegamebusiness.com/p/it-was-the-biggest-console-launch, https://wnhub.io/news/analytics/item-50489</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Tencent ASI World：AI生成オープンワールドの『見せ方』と現実</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>GDC 2026最大の話題はTencentが披露したASI World (Artificial Super Intelligence World)。1プロンプトからSRPGを一括生成する統合AIパイプラインで、地形・建築・植生・NPC・クエスト・経済までを自動生成するデモを実施。一方で第三者検証では、クエストは雛形フェッチ型、NPC挙動はアイドル+定型、経済は数値が回るのみで均衡なし、と『歩ける世界』にとどまる。生成には数時間規模のGPUクラスタを要し、コンシューマー実装は当面非現実的。GDC開発者調査では『AIが業界を害している』との回答が49%→52%に増加。</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Tencent, Microsoft, GDC, ID@Xbox</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>生成AIは『開発支援ツール』としての成熟（QA・ローカライズ・アセット下書き）と『コンテンツそのもの』への適用フェーズに分岐。後者はインフラ・著作権・面白さの3つで壁。Procedural Generation 2.0として位置付けるべきで、人手キュレーションの介在は前提。</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>AAAは『生成AIを内製パイプラインに静かに統合』、インディーは『生成AI=コア機構』で実験。両極が並走する。</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>https://www.strayspark.studio/blog/gdc-2026-ai-takeaways-indie-developers, https://developer.microsoft.com/en-us/games/articles/2026/03/gdc-2026-future-proof-your-game/</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>BitSummit PUNCH 2026『High Impact』と日本インディーの第2フェーズ</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>BitSummitが京都・みやこめっせで5/22-24開催、14回目。2025年は5万8千人超を動員し、テーマは『High Impact』＝少人数でも世界に影響を与えるクリエイティブ宣言。金曜はBusiness Day化されており、商談・パブリッシング契約の場として国際的にも定着。Game*Sparkの『Indie Hype Train』など継続的なインディー特集と相まって、日本産インディーは『TokyoIndieGamesSummit→BitSummit→TGSインディーコーナー』という年間導線が確立した。</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>BitSummit実行委員会, Game*Spark, TOKYO INDIE GAMES SUMMIT</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>日本インディーは初期の『同人/個人開発』から『海外パブリッシャー向けピッチ装置』へと第2フェーズに移行。Annapurna・Devolver・Kepler等のグローバル発掘市場と直接接続している。コンソールマーケットの高価格化が進む中、$15-25帯のインディーが価格弾力性の受け皿となる構造。</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>日本のクリエイティブ輸出経路として『IP→アニメ→ゲーム』に加え『インディー→海外パブ』が定着。</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>https://micetimes.jp/en/bitsummit-punch-2026-news-2/, https://gamemakers.jp/article/2026_03_12_133353/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
weekly-releases + indie update (2026-05-29 11:01)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -2602,7 +2602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2684,6 +2684,433 @@
       <c r="M1" s="7" t="inlineStr">
         <is>
           <t>URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>007 First Light（007 ファーストライト）</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>IO Interactive</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>IO Interactive</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>PS5/Xbox Series X|S/PC/Switch 2</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>アクション/ステルス</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>88</v>
+      </c>
+      <c r="H2" t="n">
+        <v>90</v>
+      </c>
+      <c r="K2" t="n">
+        <v>5</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>James Bond原典オリジン。Metacritic 88 / OpenCritic 90でIOI過去最高評価。GoldenEye以来の最高ボンドゲームとの評。GOTY候補として早くも名前が挙がる。</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>https://opencritic.com/game/19224/007-first-light</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Forza Horizon 6（フォルツァ ホライゾン 6）</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Playground Games</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Xbox Game Studios / Microsoft</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Xbox Series X|S/PC/Steam</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>オープンワールド・レース</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>92</v>
+      </c>
+      <c r="H3" t="n">
+        <v>91</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>302,645 (Steam, SteamDB)</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>4,900,000本(推定/Alinea Analytics)</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>5</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>日本舞台。Steam同接30万超でXbox Game Studios歴代最高。初週6,000万プレイヤー超(GamePass含む)、推定売上3.25億ドル。発売週起点では『先週』。</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>https://www.pcgamer.com/games/racing/forza-horizon-6-speeds-into-steams-top-5-most-played-games-with-over-300k-concurrent-players/</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Deep Rock Galactic: Rogue Core（ディープロック ギャラクティック：ローグコア）</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Ghost Ship Games</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Ghost Ship Publishing</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>PC/Steam (Early Access)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Co-op FPS/ローグライト</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>3</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>DRGスピンオフ。Steamレビューは『賛否両論』(肯定69%/5,299件)。タイマー・パーク抽選・本家らしさの喪失に不満の声。今後のEAアップデート次第。</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>https://store.steampowered.com/app/2605790/Deep_Rock_Galactic_Rogue_Core/</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Final Fantasy VII Rebirth（ファイナルファンタジーVII リバース）</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Square Enix CBU1</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Square Enix</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Switch 2/Xbox Series X|S/PC</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>RPG</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>5</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>PS5独占からSwitch2/Xbox/PC展開。CBU1の大型タイトルがマルチプラットフォーム化、6月RPG枠の本命。</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/schedule</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>eFootball Kick Off!</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Konami Digital Entertainment</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Konami</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Switch 2</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>サッカー</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>3</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Switch2向けスタンドアロン版eFootball。任天堂新ハード参入タイトル。</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>https://www.nintendolife.com/guides/upcoming-nintendo-switch-2-games-and-accessories-for-may-and-june-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>The 7th Guest Remake（第7のゲスト リメイク）</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Vertigo Games</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Vertigo Games</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>PC/PS5/Switch/Switch 2/Xbox</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>ホラー/パズル/アドベンチャー</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>3</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>1993年名作FMVのフルリメイク。レトロ層+ホラー需要を狙う。</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>https://www.gamespot.com/articles/2026-upcoming-games-release-schedule/1100-6534941/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Gothic 1 Remake（ゴシック1 リメイク）</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Alkimia Interactive</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>THQ Nordic</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>PC/PS5/Xbox Series X|S</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>オープンワールドRPG</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>4</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2001年の名作ドイツ製RPGの完全リメイク。Piranha Bytes創業者陣監修。欧州PC RPG層の本命。</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>https://box.co.uk/blog/june-game-releases-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>The Adventures of Elliot: The Millennium Tales（冒険家エリオットの千年物語）</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Octeto Studios</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Square Enix</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>PC/PS5/Xbox Series X|S/Switch 2</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>HD-2D RPG</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>4</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>HD-2Dエンジン採用の新IP。Square Enix外部パブとして注目。中世ファンタジー×リアルタイム戦闘。</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/article/202605/72904</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Hell Let Loose: Vietnam（ヘル・レット・ルース：ヴェトナム）</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Expression Games</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Team17</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>PC/PS5/Xbox Series X|S</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>ミリタリーFPS</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>3</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Hell Let Looseシリーズのベトナム戦争スタンドアロン。50vs50大規模戦。Tactical FPS層に注目。</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>https://www.mensjournal.com/entertainment/top-10-video-games-releasing-in-june-2026</t>
         </is>
       </c>
     </row>
@@ -5869,7 +6296,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5930,6 +6357,147 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Mina the Hollower（ミナ・ザ・ホロワー）</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Yacht Club Games (~30人)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-05-29 発売</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>PC(Steam/GOG)/PS5/Xbox Series/Switch/Switch 2</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>アクションアドベンチャー</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Shovel Knight開発元による新作。Game Boy Color風ピクセルアート。Metacritic 93 / OpenCritic 92で2026年最高評価。$19.99の低価格。</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Steam同接 8,017 (SteamDB) ※発売直後/Shovel Knight(2,875)の約3倍。Steamレビュー 87% Positive (228件時点)</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Kickstarter発、Yacht Club自社パブ。ニッチGBCオマージュが大型作と肩を並べる稀有な例。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Paralives（パラライブス）</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Paralives Studio (~10人, モントリオール)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-05-25 Early Access</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>PC/Steam</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>ライフシム</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>The Sims対抗の独立系ライフシム。7年開発。Early Access価格$35.99-$39.99。DLCなし・1.0までアップデート無料を明言。</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Steam同接 78,603 (SteamDB)。8時間で25万本(出典: notebookcheck/開発元)。Steamレビュー 86-89% Positive(3,200件時点)。</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Sims市場における初の本格的競合。バグ・パフォーマンス課題は残るが、コミュニティの反応は強い。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Dead as Disco（デッド・アズ・ディスコ）</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Brain Jar Games</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-05-05 Early Access</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>PC/Steam</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>リズム/ベルトアクション</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>音楽とビートに同期するベルトアクション。ネオン色彩のミュージックビデオ風演出。複数媒体が『Essential』『93/100』評価。</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Steamレビュー 非常に好評。配信・SNSで継続的に言及。</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>リズムゲー×ベルトアクションのジャンル交配。低予算ながら高評価のスリーパーヒット候補。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
daily-news + cross-questions update (2026-05-29 21:40)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -1783,7 +1783,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1832,6 +1832,80 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>ゲームハードのメモリ高騰起点の値上げは、AIサーバ・スマホ・自動車などメモリ需要の高い業界でも同様に起きるか？</t>
+        </is>
+      </c>
+      <c r="C2" s="13" t="inlineStr">
+        <is>
+          <t>Valve, Steam Deck OLED値上げ +46% / 任天堂Switch 2値上げ / Sony PS6時期未定</t>
+        </is>
+      </c>
+      <c r="D2" s="13" t="inlineStr">
+        <is>
+          <t>Valve, Nintendo, Sony, Samsung, Micron, SK Hynix</t>
+        </is>
+      </c>
+      <c r="E2" s="13" t="inlineStr">
+        <is>
+          <t>半導体, AIサーバ, スマホ, 自動車, 家電</t>
+        </is>
+      </c>
+      <c r="F2" s="13" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="G2" s="13" t="inlineStr">
+        <is>
+          <t>メモリは2024〜26年でAI需要が席巻し、コンシューマ向けの確保が劣後する構造。ゲーム機・PC・スマホ・車載ECUが同じ供給制約を受ける。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>ゲームIPがファッションECや百貨店と組む流れは、小売業界の“体験販売”戦略のどのフェーズに相当するか？</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>鳴潮 × ZOZOTOWN コラボ受注開始 / ガンダム50周年プロジェクト / ウマ娘海外展開</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
+        <is>
+          <t>Kuro Games, ZOZO, バンダイナムコ, サイバーエージェント</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="inlineStr">
+        <is>
+          <t>小売, アパレル, 百貨店, 広告, ライセンス</t>
+        </is>
+      </c>
+      <c r="F3" s="13" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="G3" s="13" t="inlineStr">
+        <is>
+          <t>ライブイベント中心の「コト消費」から、ゲームIP起点の「キャラ消費×日常衣料」への接続が進む。EC側はパーソナライズ送客の素材にできる。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1843,7 +1917,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2588,6 +2662,666 @@
       <c r="L12" s="13" t="inlineStr">
         <is>
           <t>AAA制作費高騰への解</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>Valve、Steam Deck OLED価格を$649→$949（+46%）に大幅引き上げ、メモリ高騰・物流逼迫が背景</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>https://www.gamedeveloper.com/business/valve-raises-steam-deck-oled-prices-by-over-200</t>
+        </is>
+      </c>
+      <c r="D13" s="13" t="inlineStr">
+        <is>
+          <t>メモリ・ストレージ価格の世界的高騰と、ホルムズ海峡情勢に絡む物流逼迫を背景に、Valveが携帯ゲーミングPC「Steam Deck OLED」の値上げを断行。任天堂Switch 2やソニーPS5/PS5 Proも直前に値上げに動いており、ゲームハード価格上昇の流れが鮮明化した。</t>
+        </is>
+      </c>
+      <c r="E13" s="13" t="inlineStr">
+        <is>
+          <t>Valveは5月28日、Steam Deck OLED 512GBを$549→$789、1TBを$649→$949へ改定。北米・カナダ・欧州・豪・英でも同時に引き上げ、再販開始直後に両モデルが即完売。「新型ではなく価格改定のみ」と明言。AAA向けPCゲーミング市場のエントリー価格に直接影響する。</t>
+        </is>
+      </c>
+      <c r="F13" s="13" t="inlineStr">
+        <is>
+          <t>OLED 512GB: $549→$789（+44%）
+OLED 1TB: $649→$949（+46%）
+メモリ・ストレージ価格高騰が直接要因
+物流逼迫（ホルムズ海峡情勢）にも言及
+再販直後に両モデル完売</t>
+        </is>
+      </c>
+      <c r="G13" s="13" t="inlineStr">
+        <is>
+          <t>Switch 2・PS5・Steam Deckいずれも値上げで、2026年は「ハード値上げ＝据置キャリア利益確保」のパターンが定着する可能性。任天堂のSwitch 2需要は値上げ前駆け込みで上振れ余地、ValveはSteam OSの他社採用拡大で“ハード値上げ＋ソフト売上拡大”モデルへ。</t>
+        </is>
+      </c>
+      <c r="H13" s="13" t="inlineStr">
+        <is>
+          <t>メモリ・半導体相場とゲームハード原価の関係</t>
+        </is>
+      </c>
+      <c r="I13" s="13" t="inlineStr">
+        <is>
+          <t>Valve, Nintendo, Sony, Samsung, Micron</t>
+        </is>
+      </c>
+      <c r="J13" s="13" t="inlineStr">
+        <is>
+          <t>Steam Deck, Steam Deck OLED</t>
+        </is>
+      </c>
+      <c r="K13" s="13" t="inlineStr">
+        <is>
+          <t>業績,技術,海外</t>
+        </is>
+      </c>
+      <c r="L13" s="13" t="inlineStr">
+        <is>
+          <t>5/28付値上げ</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Embracer、Fellowship Entertainmentをスピンオフ – LotR・Tomb Raider・Metro等を分離し2027年Nasdaq上場へ</t>
+        </is>
+      </c>
+      <c r="C14" s="13" t="inlineStr">
+        <is>
+          <t>https://variety.com/2026/biz/global/embracer-fellowship-entertainment-nasdaq-sweden-1236754638/</t>
+        </is>
+      </c>
+      <c r="D14" s="13" t="inlineStr">
+        <is>
+          <t>Embracer Groupは買収を繰り返したコングロマリット路線が業績悪化と評価ディスカウントを招き、2023年以降のリストラとAsmodee分社（Coffee Stain）に続く第3の構造改革として、IPホールディング機能を持つ新会社「Fellowship Entertainment」のスピンオフを発表した。</t>
+        </is>
+      </c>
+      <c r="E14" s="13" t="inlineStr">
+        <is>
+          <t>5月20日、取締役会がFellowship Entertainmentの分割を承認。Lord of the Rings、Tomb Raider、Dead Island、Metro、Kingdom Come Deliverance等のIPを集約し、4A Games、Crystal Dynamics、Eidos-Montréal、Warhorse、Middle-earth Enterprises等のスタジオを抱える「IP志向」企業として2027年にNasdaq Stockholm上場予定。CEOはPhil Rogers氏。</t>
+        </is>
+      </c>
+      <c r="F14" s="13" t="inlineStr">
+        <is>
+          <t>Lord of the Rings IPがFellowship側へ
+Tomb Raider・Metro等の主要IPも分離
+2027年Nasdaq Stockholm上場予定
+既存Embracerはモバイル・PC/家庭用・物販に集中
+現EmbracerのCEO Phil Rogersが新社CEOへ</t>
+        </is>
+      </c>
+      <c r="G14" s="13" t="inlineStr">
+        <is>
+          <t>EAの$55B買収やTake-Twoの拡大に対抗するため、Fellowship単体でLotR/Tomb Raider映像化・ライセンス収益を最大化する戦略が見える。一方で残るEmbracerは“縮小均衡型”の選択を強いられ、AAA中心の業界再編が加速する。</t>
+        </is>
+      </c>
+      <c r="H14" s="13" t="inlineStr">
+        <is>
+          <t>IPホールディング型ゲーム企業のバリュエーション</t>
+        </is>
+      </c>
+      <c r="I14" s="13" t="inlineStr">
+        <is>
+          <t>Embracer Group, Fellowship Entertainment, Crystal Dynamics, Eidos-Montréal, Warhorse Studios, 4A Games</t>
+        </is>
+      </c>
+      <c r="J14" s="13" t="inlineStr">
+        <is>
+          <t>Lord of the Rings, Tomb Raider, Dead Island, Metro, Kingdom Come Deliverance, Darksiders, Remnant</t>
+        </is>
+      </c>
+      <c r="K14" s="13" t="inlineStr">
+        <is>
+          <t>M&amp;A,海外</t>
+        </is>
+      </c>
+      <c r="L14" s="13" t="inlineStr">
+        <is>
+          <t>5/20発表</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>Bungie、『Destiny 2』のライブ運営を6/9『Monument of Triumph』で終了、9年に幕</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>https://www.bungie.net/7/en/News/Article/d2_may_21_2026</t>
+        </is>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>Sony傘下のBungieは長期運営型FPS『Destiny 2』のサービス縮小と新IP転換を進めており、5月にSonyがBungie関連で$5.65億の減損を計上した直後に、本タイトルの開発終了が公式アナウンスされた。GaaS（運営型ゲーム）の長期収益化の難しさを象徴する出来事。</t>
+        </is>
+      </c>
+      <c r="E15" s="13" t="inlineStr">
+        <is>
+          <t>5月21日、Bungieは『Destiny 2』のラストアップデート『Monument of Triumph』を6月9日にリリースし、新規シーズン・拡張の追加を終了すると発表。Directorインターフェース復活、Sparrow Racing League恒久化、Pantheon活動の常設化など、プレイヤー資産を“凍結保存”する設計に。サーバは継続稼働。</t>
+        </is>
+      </c>
+      <c r="F15" s="13" t="inlineStr">
+        <is>
+          <t>6/9『Monument of Triumph』が最後の大型更新
+Director UI復活・SRL/Pantheon恒久化
+新シーズン・拡張は今後追加されず
+サーバ稼働は継続（プレイ可能）
+Destiny 3はグリーンライト前で停滞</t>
+        </is>
+      </c>
+      <c r="G15" s="13" t="inlineStr">
+        <is>
+          <t>BungieはSony傘下で『Marathon』など新IPに資源集約。GaaSの“EOS（サービス終了）戦略”として、Destiny 2は今後の長期GaaS設計のベンチマークに。BungieのリストラとDestiny 3不確定はSonyのファーストパーティ戦略の見直しを迫る。</t>
+        </is>
+      </c>
+      <c r="H15" s="13" t="inlineStr">
+        <is>
+          <t>GaaSのライフサイクル設計とEOS戦略</t>
+        </is>
+      </c>
+      <c r="I15" s="13" t="inlineStr">
+        <is>
+          <t>Bungie, Sony Interactive Entertainment</t>
+        </is>
+      </c>
+      <c r="J15" s="13" t="inlineStr">
+        <is>
+          <t>Destiny 2, Destiny 3, Marathon</t>
+        </is>
+      </c>
+      <c r="K15" s="13" t="inlineStr">
+        <is>
+          <t>業績,海外</t>
+        </is>
+      </c>
+      <c r="L15" s="13" t="inlineStr">
+        <is>
+          <t>5/21発表、6/9実装</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>任天堂、マイニンテンドーストアのSwitch 2購入条件「50時間プレイ」を撤廃、5/25値上げと同時に</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="inlineStr">
+        <is>
+          <t>https://news.denfaminicogamer.jp/news/2605252p</t>
+        </is>
+      </c>
+      <c r="D16" s="13" t="inlineStr">
+        <is>
+          <t>任天堂は5月25日、Nintendo Switch 2を¥49,980→¥59,980に値上げした。これに合わせて、これまでマイニンテンドーストアでの直販購入に課していた「Switch本体での累計プレイ時間50時間以上」「Nintendo Switch Online加入」等の条件を撤廃。値上げによる需要鈍化を見越した販売条件緩和とみられる。</t>
+        </is>
+      </c>
+      <c r="E16" s="13" t="inlineStr">
+        <is>
+          <t>値上げ実施と同日の5月25日付で、マイニンテンドーストア直販の購入条件を見直し。これまで転売対策として課していたプレイ時間・サブスク条件を実質撤廃し、より広い層が直販で購入できる体制に転換。同社決算では2027年3月期Switch 2出荷を1,650万台と想定。</t>
+        </is>
+      </c>
+      <c r="F16" s="13" t="inlineStr">
+        <is>
+          <t>5/25付で購入条件を緩和
+「プレイ時間50時間以上」が条件から消える
+値上げに伴う初期需要鈍化への対応
+転売対策から販売拡大優先へシフト
+2027年3月期Switch 2出荷想定1,650万台</t>
+        </is>
+      </c>
+      <c r="G16" s="13" t="inlineStr">
+        <is>
+          <t>値上げによる短期需要減を、直販条件緩和でカバーする戦略。並行輸入や転売価格との競合再燃の可能性。任天堂直販シェア拡大は中古市場・量販店との関係見直しを誘発する可能性がある。</t>
+        </is>
+      </c>
+      <c r="H16" s="13" t="inlineStr">
+        <is>
+          <t>ハード値上げ局面での販売チャネル戦略</t>
+        </is>
+      </c>
+      <c r="I16" s="13" t="inlineStr">
+        <is>
+          <t>任天堂</t>
+        </is>
+      </c>
+      <c r="J16" s="13" t="inlineStr">
+        <is>
+          <t>Nintendo Switch 2</t>
+        </is>
+      </c>
+      <c r="K16" s="13" t="inlineStr">
+        <is>
+          <t>業績,国内</t>
+        </is>
+      </c>
+      <c r="L16" s="13" t="inlineStr">
+        <is>
+          <t>5/25付</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>Global Game Jam、Endless財団と最大$2,500のマイクログラント新制度を始動、インディー支援強化</t>
+        </is>
+      </c>
+      <c r="C17" s="13" t="inlineStr">
+        <is>
+          <t>https://www.gamedeveloper.com/business/global-game-jam-launches-micro-grant-program-to-support-indies-and-emerging-talent</t>
+        </is>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
+        <is>
+          <t>AAA市場の制作費高騰と各社のレイオフ加速で、インディー・新人クリエイターの参入機会が縮小傾向にある中、Global Game Jam（GGJ）がEndless財団と共同で支援プログラムを開始。「Small Projects, Big Impact」を掲げる。</t>
+        </is>
+      </c>
+      <c r="E17" s="13" t="inlineStr">
+        <is>
+          <t>「GGJ Micro-Missions」として、インディースタジオに最大$2,500のマイクログラントを提供し、18歳以上の新人クリエイターに有償のマイクロプロジェクトを発注する制度。アート（小規模アセット）、サウンド（SE/BGM）、QAテストの3カテゴリ。年間1,500〜2,000件のプロジェクトを目指す。</t>
+        </is>
+      </c>
+      <c r="F17" s="13" t="inlineStr">
+        <is>
+          <t>最大$2,500のマイクログラント
+アート・サウンド・QAの3カテゴリ
+初年度1,500〜2,000プロジェクトを想定
+25スタジオ・500名超の参加を見込む
+GGJ × Endless Foundationの新パイロット</t>
+        </is>
+      </c>
+      <c r="G17" s="13" t="inlineStr">
+        <is>
+          <t>AAAレイオフ流出人材のインディー受け皿としての機能、ポートフォリオ形成・小規模ジョブの市場化が進む可能性。同種のマイクロタスク発注プラットフォーム（Unity Asset Store、Itch.io等）との競合・補完関係に注目。</t>
+        </is>
+      </c>
+      <c r="H17" s="13" t="inlineStr">
+        <is>
+          <t>インディー資金調達とマイクロタスク経済</t>
+        </is>
+      </c>
+      <c r="I17" s="13" t="inlineStr">
+        <is>
+          <t>Global Game Jam, Endless Foundation</t>
+        </is>
+      </c>
+      <c r="J17" s="13" t="inlineStr">
+        <is>
+          <t>（業界全般）</t>
+        </is>
+      </c>
+      <c r="K17" s="13" t="inlineStr">
+        <is>
+          <t>インディー,海外</t>
+        </is>
+      </c>
+      <c r="L17" s="13" t="inlineStr">
+        <is>
+          <t>パイロット制度</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>ソニーG、2026年3月期にBungie関連で5.65億ドルの減損計上、2024年来の合計は7.65億ドル</t>
+        </is>
+      </c>
+      <c r="C18" s="13" t="inlineStr">
+        <is>
+          <t>https://www.gamespot.com/articles/sony-writes-off-another-565-million-impairment-loss-against-bungie/1100-6539855/</t>
+        </is>
+      </c>
+      <c r="D18" s="13" t="inlineStr">
+        <is>
+          <t>ソニーG（SIE）は2022年に約36億ドルでBungieを買収したが、買収後のレイオフ繰り返しと『Marathon』ローンチ遅延、『Destiny 2』運営縮小により、のれん・無形資産の評価減を再度迫られた。GaaSへのSIE投資の見直しが本格化。</t>
+        </is>
+      </c>
+      <c r="E18" s="13" t="inlineStr">
+        <is>
+          <t>ソニーは2026年3月期決算（5/8発表）で、Bungie関連資産について5.65億ドル（約840億円）の追加減損を計上。2025年11月の2.00億ドルと合わせ累計7.65億ドル。同時期にBungieは『Destiny 2』の継続的アップデート終了を発表しており、評価減と事業縮小がリンクした形。</t>
+        </is>
+      </c>
+      <c r="F18" s="13" t="inlineStr">
+        <is>
+          <t>5月決算でBungie関連 $5.65億の減損
+2024年来の累計減損は$7.65億
+Destiny 2運営終了との連動
+Marathon発売延期がさらに影響懸念
+SIEのGaaS投資見直しが鮮明化</t>
+        </is>
+      </c>
+      <c r="G18" s="13" t="inlineStr">
+        <is>
+          <t>SIEは『Marathon』成否がBungie存続の試金石に。ファーストパーティGaaSの「内製拡張」より「外部スタジオ連携」へシフトする可能性。任天堂・Microsoftとの差別化として、シングルプレイ大作回帰が再評価される展開も。</t>
+        </is>
+      </c>
+      <c r="H18" s="13" t="inlineStr">
+        <is>
+          <t>ゲーム会社買収後の減損リスクと統合論</t>
+        </is>
+      </c>
+      <c r="I18" s="13" t="inlineStr">
+        <is>
+          <t>Sony Group, Sony Interactive Entertainment, Bungie</t>
+        </is>
+      </c>
+      <c r="J18" s="13" t="inlineStr">
+        <is>
+          <t>Destiny 2, Marathon</t>
+        </is>
+      </c>
+      <c r="K18" s="13" t="inlineStr">
+        <is>
+          <t>業績,海外</t>
+        </is>
+      </c>
+      <c r="L18" s="13" t="inlineStr">
+        <is>
+          <t>Bungie資産</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>サイバーエージェント中間決算、ゲーム事業営業益+106% 『ウマ娘』英語版で海外売上3.6倍に</t>
+        </is>
+      </c>
+      <c r="C19" s="13" t="inlineStr">
+        <is>
+          <t>https://gamebiz.jp/news/425828</t>
+        </is>
+      </c>
+      <c r="D19" s="13" t="inlineStr">
+        <is>
+          <t>サイバーエージェント子会社Cygamesが2025年に米欧向け『Umamusume Pretty Derby』英語版をリリースし、グローバル展開が国内ブランドの新たな成長ドライバとなった。25/26年期はCyberAgentグループ全体の業績を押し上げる構図に。</t>
+        </is>
+      </c>
+      <c r="E19" s="13" t="inlineStr">
+        <is>
+          <t>5月発表の2026年9月期1H決算で、ゲーム事業売上高は前年同期比+47.4%の1,322億円、営業利益は+106.3%の386億円。『ウマ娘』英語版の大ヒットで海外売上が3.6倍の272億円に拡大。新作『Project Awakening（仮）』『グラブル新作』等にも期待。</t>
+        </is>
+      </c>
+      <c r="F19" s="13" t="inlineStr">
+        <is>
+          <t>ゲーム事業売上+47.4%、営業益+106.3%
+海外売上が前年同期比3.6倍に
+『ウマ娘』英語版がドライバ
+下期も新作投入で成長期待
+Cygamesからの配当400億円も予定</t>
+        </is>
+      </c>
+      <c r="G19" s="13" t="inlineStr">
+        <is>
+          <t>国内アイドル/競馬ゲームジャンルのグローバル化成功事例として、他社も追随。中国ByteDance（Hypergryph）、NetEaseのグローバル展開と競合が激化。Cygamesの利益体質強化はCAホールディングス全体の配当原資にも貢献。</t>
+        </is>
+      </c>
+      <c r="H19" s="13" t="inlineStr">
+        <is>
+          <t>ハイカジュアル⇔国内尖りIPのグローバル戦略</t>
+        </is>
+      </c>
+      <c r="I19" s="13" t="inlineStr">
+        <is>
+          <t>サイバーエージェント, Cygames, KLab</t>
+        </is>
+      </c>
+      <c r="J19" s="13" t="inlineStr">
+        <is>
+          <t>ウマ娘プリティーダービー, グランブルーファンタジー</t>
+        </is>
+      </c>
+      <c r="K19" s="13" t="inlineStr">
+        <is>
+          <t>業績,国内</t>
+        </is>
+      </c>
+      <c r="L19" s="13" t="inlineStr">
+        <is>
+          <t>1H決算</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>アクアプラス『うたわれるもの 白への道標』5/28発売、シリーズ完結作で20年プロジェクトに幕</t>
+        </is>
+      </c>
+      <c r="C20" s="13" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/article/202605/74473</t>
+        </is>
+      </c>
+      <c r="D20" s="13" t="inlineStr">
+        <is>
+          <t>アクアプラスの長寿RPGシリーズ『うたわれるもの』は2002年初代発売以来、PCゲーム→家庭用→アニメ・舞台と展開を続けた看板IP。シリーズ完結作と位置付けられる新作リリースで、20年余のIPライフサイクルに一区切り。</t>
+        </is>
+      </c>
+      <c r="E20" s="13" t="inlineStr">
+        <is>
+          <t>5月28日、PS5/PS4/Switch/PC向けに『うたわれるもの 白への道標』を発売。シリーズ完結編にして「プロジェクトの最終作」と位置付けられ、これまでの3部作の物語を結ぶ。SRPG＋アドベンチャー形式を踏襲。Steam同日配信。</t>
+        </is>
+      </c>
+      <c r="F20" s="13" t="inlineStr">
+        <is>
+          <t>シリーズ完結編にして最終作
+5/28、マルチプラットフォーム発売
+20年余のシリーズプロジェクトに区切り
+アニメ・舞台展開も総決算
+SRPG＋ADVのハイブリッド形式</t>
+        </is>
+      </c>
+      <c r="G20" s="13" t="inlineStr">
+        <is>
+          <t>アクアプラスは『うたわれるもの』後の次期看板IP育成が課題に。完結という形でIP価値を確定させ、リマスター・サブスク配信・キャラクターグッズ等の二次収益化に注力する可能性。</t>
+        </is>
+      </c>
+      <c r="H20" s="13" t="inlineStr">
+        <is>
+          <t>国内中堅メーカーの長期IP運用と完結戦略</t>
+        </is>
+      </c>
+      <c r="I20" s="13" t="inlineStr">
+        <is>
+          <t>アクアプラス, Aquaplus</t>
+        </is>
+      </c>
+      <c r="J20" s="13" t="inlineStr">
+        <is>
+          <t>うたわれるもの 白への道標, うたわれるもの</t>
+        </is>
+      </c>
+      <c r="K20" s="13" t="inlineStr">
+        <is>
+          <t>新作,国内</t>
+        </is>
+      </c>
+      <c r="L20" s="13" t="inlineStr">
+        <is>
+          <t>シリーズ完結作</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <t>バンダイナムコ、「ガンダム50周年プロジェクト」始動を発表、IP横断で大型企画を順次展開へ</t>
+        </is>
+      </c>
+      <c r="C21" s="13" t="inlineStr">
+        <is>
+          <t>https://www.bandainamco.co.jp/releases/index.html</t>
+        </is>
+      </c>
+      <c r="D21" s="13" t="inlineStr">
+        <is>
+          <t>2029年に放送開始50周年を迎える『機動戦士ガンダム』は、バンダイナムコグループのIP別売上トップ級。模型（ガンプラ）、家庭用ゲーム、モバイル、映像、アパレル等の多角展開を統合的に強化するため、節目イヤーへの長期マーケティング計画を明確化。</t>
+        </is>
+      </c>
+      <c r="E21" s="13" t="inlineStr">
+        <is>
+          <t>5月15日、バンダイナムコグループは「ガンダム50周年プロジェクト」始動を発表。2026年から2029年まで複数年にわたり、ゲーム新作・映像・イベント・ガンプラ等の記念企画を連続展開。グループの中期経営計画とも連動し、IP単独の売上1兆円突破を視野。</t>
+        </is>
+      </c>
+      <c r="F21" s="13" t="inlineStr">
+        <is>
+          <t>2029年50周年に向けた複数年プロジェクト
+2026年からゲーム・映像・イベントを順次
+ガンプラ・アパレル・コラボも含む多角展開
+IP単独で売上1兆円規模を視野
+グループ中期経営計画と連動</t>
+        </is>
+      </c>
+      <c r="G21" s="13" t="inlineStr">
+        <is>
+          <t>ガンダム単一IPでの売上構成比上昇はバンダイナムコの収益安定化に貢献する一方、他IPの育成停滞リスクも。海外Z世代へのリーチ拡大（HBO実写・新作モバイル等）が鍵。</t>
+        </is>
+      </c>
+      <c r="H21" s="13" t="inlineStr">
+        <is>
+          <t>IP単体のメガフランチャイズ化と長期IRストーリー</t>
+        </is>
+      </c>
+      <c r="I21" s="13" t="inlineStr">
+        <is>
+          <t>バンダイナムコホールディングス, BANDAI SPIRITS, サンライズ</t>
+        </is>
+      </c>
+      <c r="J21" s="13" t="inlineStr">
+        <is>
+          <t>機動戦士ガンダム, ガンプラ</t>
+        </is>
+      </c>
+      <c r="K21" s="13" t="inlineStr">
+        <is>
+          <t>新作,国内</t>
+        </is>
+      </c>
+      <c r="L21" s="13" t="inlineStr">
+        <is>
+          <t>2029年50周年起点</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t>Kuro Games『鳴潮』×ZOZOTOWN、コラボコレクション受注を5/29 12:00開始、ゲームIP×ファッションEC連携</t>
+        </is>
+      </c>
+      <c r="C22" s="13" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/634/G063420/20260526020/</t>
+        </is>
+      </c>
+      <c r="D22" s="13" t="inlineStr">
+        <is>
+          <t>中国Kuro Games運営のオープンワールドRPG『鳴潮（Wuthering Waves）』は日本国内で安定的にトップセラー層に位置するモバイル/PCタイトル。ファッションEC大手ZOZOTOWNと組み、ゲームファッション化の流れを国内で具体化する事例。</t>
+        </is>
+      </c>
+      <c r="E22" s="13" t="inlineStr">
+        <is>
+          <t>ZOZOTOWNは5月29日12時から、『鳴潮』とのコラボコレクション「鳴潮 × ZOZOTOWN」の受注販売を開始。キャラクターをモチーフにしたアパレル・グッズを展開し、ゲームファンとファッションユーザーの相互送客を狙う。海外運営タイトルがJP小売プラットフォームと組む構図に。</t>
+        </is>
+      </c>
+      <c r="F22" s="13" t="inlineStr">
+        <is>
+          <t>受注開始 5/29 12:00
+Kuro Games『鳴潮』とZOZOの初コラボ
+キャラモチーフのアパレル展開
+海外運営タイトル×日本EC大手の事例
+ゲームの“ライフスタイル化”の進展</t>
+        </is>
+      </c>
+      <c r="G22" s="13" t="inlineStr">
+        <is>
+          <t>ゲームIPのファッション化（Genshin・原神、ホヨバ、サイゲ各社）が国内大型EC・百貨店と本格接続するフェーズ。アパレル受注はMRR的な“追加収益化”の重要チャネルとなる可能性。</t>
+        </is>
+      </c>
+      <c r="H22" s="13" t="inlineStr">
+        <is>
+          <t>ゲームIPのファッション・小売リテール接続</t>
+        </is>
+      </c>
+      <c r="I22" s="13" t="inlineStr">
+        <is>
+          <t>Kuro Games, ZOZO, ZOZOTOWN</t>
+        </is>
+      </c>
+      <c r="J22" s="13" t="inlineStr">
+        <is>
+          <t>鳴潮 (Wuthering Waves)</t>
+        </is>
+      </c>
+      <c r="K22" s="13" t="inlineStr">
+        <is>
+          <t>新作,国内,海外</t>
+        </is>
+      </c>
+      <c r="L22" s="13" t="inlineStr">
+        <is>
+          <t>5/29 12:00受注開始</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
daily-news + cross-questions update (2026-05-30) (2026-05-29 22:12)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -1783,7 +1783,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1906,6 +1906,80 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>大型M&amp;Aの株主代表訴訟（買収価格妥当性）は、ゲーム以外の通信・製薬・自動車などのメガディール多発業界でも同様に長期負債化するか？</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>Microsoft、Activision Blizzard買収巡る株主訴訟で2.5億ドル和解（うち40%自社負担）</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>Microsoft, Activision Blizzard, Sjunde AP-Fonden</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="inlineStr">
+        <is>
+          <t>通信, 製薬, 自動車, 半導体, 金融</t>
+        </is>
+      </c>
+      <c r="F4" s="13" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="G4" s="13" t="inlineStr">
+        <is>
+          <t>メガM&amp;Aではクロージング後3〜5年の株主訴訟が定番化しつつあり、D&amp;O保険スキームの厚みが投資判断に影響。買収側のキャッシュ流出は会計上の特別損失で計上され、ガイダンス変動材料に。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>ミーム株企業（GameStop）による本業を超えた既存大手リテール買収提案は、小売・通信・百貨店などの他業界でも『ミーム化』を起点に発生し得るか？</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>eBay、GameStopによる560億ドル買収提案を全会一致で拒絶</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>GameStop, eBay, Ryan Cohen</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>小売, 通信, 百貨店, ECマーケットプレイス, 暗号資産関連</t>
+        </is>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="G5" s="13" t="inlineStr">
+        <is>
+          <t>ミーム株プレミアムを「買収通貨」に転用する試みは前代未聞。リテール業界では『株価=買収通貨』のパラダイムが時価総額逆転M&amp;Aを可能にし得る。BitcoinやMEME銘柄保有企業の動きと並走して注視。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1917,7 +1991,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3322,6 +3396,666 @@
       <c r="L22" s="13" t="inlineStr">
         <is>
           <t>5/29 12:00受注開始</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B23" s="13" t="inlineStr">
+        <is>
+          <t>Microsoft、Activision Blizzard買収巡る株主訴訟で2.5億ドルの和解 — 内40%を自社負担</t>
+        </is>
+      </c>
+      <c r="C23" s="13" t="inlineStr">
+        <is>
+          <t>https://www.manilatimes.net/2026/05/29/business/foreign-business/activision-shareholders-reach-250-million-settlement-over-microsoft-buyout/2353712</t>
+        </is>
+      </c>
+      <c r="D23" s="13" t="inlineStr">
+        <is>
+          <t>2023年クローズの690億ドルActivision買収を巡り、スウェーデン年金基金Sjunde AP-Fonden主導で旧Activision株主が当時CEOコティック氏らの善管注意義務違反を提訴。1株95ドルの取引価格が安すぎ、CEOが地位と4億ドルのChange of Control報酬を守るため取引を急いだと主張。</t>
+        </is>
+      </c>
+      <c r="E23" s="13" t="inlineStr">
+        <is>
+          <t>Microsoftは5月22日、Activision Blizzard旧株主との集団訴訟を2.5億ドルで和解。うち約40%をMicrosoft、残り60%を旧Activision役員賠償責任保険(D&amp;O)で負担。1株あたり約30セント。Delawareの判事の最終承認待ち。Microsoftは違法行為を認めず和解。</t>
+        </is>
+      </c>
+      <c r="F23" s="13" t="inlineStr">
+        <is>
+          <t>和解総額2.5億ドル
+Microsoft直接負担40%/D&amp;O保険60%
+1株あたり約30セント
+Delaware判事の承認待ち
+Microsoftは法的責任認めず</t>
+        </is>
+      </c>
+      <c r="G23" s="13" t="inlineStr">
+        <is>
+          <t>メガM&amp;Aに対する株主訴訟は今後も発生確率高。買収側はクロージング後数年にわたるD&amp;O・追加引当が必須に。Game Pass戦略再検討（CoD Day1除外）と相まって、Microsoftゲーム部門の収益化圧力は続く見通し。</t>
+        </is>
+      </c>
+      <c r="H23" s="13" t="inlineStr">
+        <is>
+          <t>大型M&amp;Aの株主訴訟リスクとD&amp;O保険スキーム</t>
+        </is>
+      </c>
+      <c r="I23" s="13" t="inlineStr">
+        <is>
+          <t>Microsoft, Activision Blizzard, Sjunde AP-Fonden</t>
+        </is>
+      </c>
+      <c r="J23" s="13" t="inlineStr">
+        <is>
+          <t>Call of Duty</t>
+        </is>
+      </c>
+      <c r="K23" s="13" t="inlineStr">
+        <is>
+          <t>M&amp;A,規制,海外</t>
+        </is>
+      </c>
+      <c r="L23" s="13" t="inlineStr">
+        <is>
+          <t>和解は2026/5/22署名・5/29再報道</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B24" s="13" t="inlineStr">
+        <is>
+          <t>eBay、GameStopの560億ドル買収提案を「信頼性も魅力もない」と拒絶、株価は乖離維持</t>
+        </is>
+      </c>
+      <c r="C24" s="13" t="inlineStr">
+        <is>
+          <t>https://www.cnbc.com/amp/2026/05/12/ebay-rejects-gamestops-takeover-bid.html</t>
+        </is>
+      </c>
+      <c r="D24" s="13" t="inlineStr">
+        <is>
+          <t>GameStopのRyan Cohen CEOは2026年5月、自社の約4倍の時価総額のeBayに1株125ドル・総額560億ドルの現金・株式半々の買収提案を提示。TD銀行から200億ドルのコミットメントレターも確保していた。ミーム株企業による既存大手リテール買収の前代未聞の試み。</t>
+        </is>
+      </c>
+      <c r="E24" s="13" t="inlineStr">
+        <is>
+          <t>eBay取締役会は5月12日、財務アドバイザーの精査を経てGameStopの提案を全会一致で拒絶。「信頼性も魅力もない」とし、資金調達の不確実性、統合後のレバレッジ・事業リスク・ガバナンスを理由に挙げた。eBay株価は提示額125ドルを大きく下回って推移し、市場の懐疑を反映。</t>
+        </is>
+      </c>
+      <c r="F24" s="13" t="inlineStr">
+        <is>
+          <t>提示価格 1株125ドル/総額560億ドル
+現金・株式半々の構成
+TD銀行から200億ドルコミット
+eBay取締役会が全会一致で拒絶
+株価は提示額を大きく下回り推移</t>
+        </is>
+      </c>
+      <c r="G24" s="13" t="inlineStr">
+        <is>
+          <t>GameStopが敵対的買収に踏み切るかは不透明だが、Cohen氏は再提案・株式上乗せの可能性も示唆。リテール×Cマースの統合は他社の参入余地も。eBayは独自AI/コレクタブル路線の強化で対抗する見込み。</t>
+        </is>
+      </c>
+      <c r="H24" s="13" t="inlineStr">
+        <is>
+          <t>ミーム株企業×大型リテールM&amp;Aの実現可能性</t>
+        </is>
+      </c>
+      <c r="I24" s="13" t="inlineStr">
+        <is>
+          <t>GameStop, eBay, TD Bank, Ryan Cohen</t>
+        </is>
+      </c>
+      <c r="J24" s="13" t="inlineStr">
+        <is>
+          <t>GameStop, eBay Marketplace</t>
+        </is>
+      </c>
+      <c r="K24" s="13" t="inlineStr">
+        <is>
+          <t>M&amp;A,海外,規制</t>
+        </is>
+      </c>
+      <c r="L24" s="13" t="inlineStr">
+        <is>
+          <t>5/12拒否、その後も交渉動向続報</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>Alpha Compute、ゲーミング報酬PF「GAMEE」の過半数買収を完了、AI新部門Alpha Gamesを設立</t>
+        </is>
+      </c>
+      <c r="C25" s="13" t="inlineStr">
+        <is>
+          <t>https://www.globenewswire.com/news-release/2026/05/27/3302098/0/en/ALPHA-COMPUTE-CORP-COMPLETES-MAJORITY-ACQUISITION-OF-GAMING-COMPANY-GAMEE.html</t>
+        </is>
+      </c>
+      <c r="D25" s="13" t="inlineStr">
+        <is>
+          <t>AIインフラ／コンピュート企業のAlpha Compute Corp（NASDAQ）は、Web3寄りのゲーミング報酬プラットフォーム「GAMEE」を運営するスロバキア発スタートアップの過半数株式取得を完了。GAMEEは累計1.2億人のゲーミングユーザーと2025年売上350万ドルを擁する。</t>
+        </is>
+      </c>
+      <c r="E25" s="13" t="inlineStr">
+        <is>
+          <t>Alpha Computeは5月27日、GAMEEの過半数買収を完了したと発表。AI×ゲーミングを軸とした新部門「Alpha Games」を設立し、GAMEE創業者Bozena Rezab氏がEVPとして指揮。コンピュート提供事業者がエンドユーザー保持基盤を獲得する垂直統合型ディール。</t>
+        </is>
+      </c>
+      <c r="F25" s="13" t="inlineStr">
+        <is>
+          <t>過半数株式取得を完了（5/27）
+GAMEE: 1.2億ユーザー / 2025年売上350万ドル
+AI新部門「Alpha Games」設立
+創業者Bozena Rezab氏がEVP就任
+コンピュート×ゲーミング垂直統合</t>
+        </is>
+      </c>
+      <c r="G25" s="13" t="inlineStr">
+        <is>
+          <t>AIインフラ企業によるゲーミング基盤買収はトレンド化の可能性。コンシューマーAI体験のラボとしてゲーム配信プラットフォームの位置付けが上昇。Web3寄り報酬PFの再評価にも繋がる。</t>
+        </is>
+      </c>
+      <c r="H25" s="13" t="inlineStr">
+        <is>
+          <t>AIインフラ×ゲーミング垂直統合M&amp;A</t>
+        </is>
+      </c>
+      <c r="I25" s="13" t="inlineStr">
+        <is>
+          <t>Alpha Compute Corp, GAMEE, Alpha Games</t>
+        </is>
+      </c>
+      <c r="J25" s="13" t="inlineStr">
+        <is>
+          <t>GAMEE platform</t>
+        </is>
+      </c>
+      <c r="K25" s="13" t="inlineStr">
+        <is>
+          <t>M&amp;A,技術,海外</t>
+        </is>
+      </c>
+      <c r="L25" s="13" t="inlineStr">
+        <is>
+          <t>AI×ゲーミング垂直統合</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B26" s="13" t="inlineStr">
+        <is>
+          <t>Balatroのパブリッシャー「Playstack」、Integrated Media Companyが約1.5億ドルで買収へ</t>
+        </is>
+      </c>
+      <c r="C26" s="13" t="inlineStr">
+        <is>
+          <t>https://kotaku.com/gamespot-fandom-parent-company-to-acquire-the-publisher-of-balatro-2000700544</t>
+        </is>
+      </c>
+      <c r="D26" s="13" t="inlineStr">
+        <is>
+          <t>GameSpot・Fandom・Giant Bombを束ねるInvestment Vehicle「Integrated Media Company（IMC）」が、インディーヒット『Balatro』を世界的成功に導いたパブリッシャーPlaystackの全株式取得を発表。買収対価は約1.124億ポンド（約1.51億ドル）。</t>
+        </is>
+      </c>
+      <c r="E26" s="13" t="inlineStr">
+        <is>
+          <t>メディアコングロマリットがインディーパブリッシャーを傘下に収める異例のディール。Playstack CEO Harvey Elliott氏は「チーム・戦略・プレミアムインディー特化は不変」と強調。株主承認待ちで、メディア×パブリッシングの統合シナジー検証フェーズに入る。</t>
+        </is>
+      </c>
+      <c r="F26" s="13" t="inlineStr">
+        <is>
+          <t>買収対価 約1.124億ポンド（約1.51億ドル）
+IMCはGameSpot/Fandom/Giant Bombの親会社
+PlaystackはBalatroで世界的成功
+株主承認待ち
+チーム/戦略は維持と明言</t>
+        </is>
+      </c>
+      <c r="G26" s="13" t="inlineStr">
+        <is>
+          <t>ゲームメディアとパブリッシャーの統合は編集独立性の課題を孕む一方、データ・SEO・コミュニティ資産の活用余地大。Balatro IP（モバイル・ボードゲーム化）の収益化も鍵。</t>
+        </is>
+      </c>
+      <c r="H26" s="13" t="inlineStr">
+        <is>
+          <t>ゲームメディア×インディーパブリッシャーの統合シナジー</t>
+        </is>
+      </c>
+      <c r="I26" s="13" t="inlineStr">
+        <is>
+          <t>Integrated Media Company, Playstack, GameSpot, Fandom</t>
+        </is>
+      </c>
+      <c r="J26" s="13" t="inlineStr">
+        <is>
+          <t>Balatro</t>
+        </is>
+      </c>
+      <c r="K26" s="13" t="inlineStr">
+        <is>
+          <t>M&amp;A,インディー,海外</t>
+        </is>
+      </c>
+      <c r="L26" s="13" t="inlineStr">
+        <is>
+          <t>メディア×パブの統合事例</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B27" s="13" t="inlineStr">
+        <is>
+          <t>『Call of Duty: Modern Warfare 4』10/23発売決定、初日Game Pass除外・PS4/Xbox One非対応</t>
+        </is>
+      </c>
+      <c r="C27" s="13" t="inlineStr">
+        <is>
+          <t>https://news.xbox.com/en-us/2026/05/28/call-of-duty-modern-warfare-4-first-details-campaign/</t>
+        </is>
+      </c>
+      <c r="D27" s="13" t="inlineStr">
+        <is>
+          <t>MicrosoftがGame Passの戦略を見直し、新CoDシリーズはDay1配信から除外する方針へ転換。新作はInfinity Wardが開発、舞台は朝鮮半島で、北朝鮮の侵攻に対峙する韓国軍の若手分隊とPriceの復讐譚を並行描写。</t>
+        </is>
+      </c>
+      <c r="E27" s="13" t="inlineStr">
+        <is>
+          <t>Activisionは5月28日、『Call of Duty: Modern Warfare 4』を10月23日にPS5/Xbox Series/PC/Switch 2向けに発売すると正式発表。PS4/Xbox Oneは非対応、Game Passは初日除外で約1年後に追加見込み。GTA6発売（11月予定）の約1か月前。</t>
+        </is>
+      </c>
+      <c r="F27" s="13" t="inlineStr">
+        <is>
+          <t>発売日 2026/10/23
+PS5/Xbox Series/PC/Switch 2
+PS4/Xbox One非対応
+Game Pass初日除外（約1年後追加）
+GTA6の約1か月前にリリース</t>
+        </is>
+      </c>
+      <c r="G27" s="13" t="inlineStr">
+        <is>
+          <t>CoDのDay1除外はGame Pass値下げの収益補填策。AAAパブの「サブスク疲れ」対応が顕在化。Switch 2版同時発売は任天堂ハードのサードパーティ拡大を示す象徴。GTA6との販売バッティングは限定的か。</t>
+        </is>
+      </c>
+      <c r="H27" s="13" t="inlineStr">
+        <is>
+          <t>AAA×サブスクの再交渉とプラットフォーム分散</t>
+        </is>
+      </c>
+      <c r="I27" s="13" t="inlineStr">
+        <is>
+          <t>Activision, Microsoft, Infinity Ward, Nintendo</t>
+        </is>
+      </c>
+      <c r="J27" s="13" t="inlineStr">
+        <is>
+          <t>Call of Duty Modern Warfare</t>
+        </is>
+      </c>
+      <c r="K27" s="13" t="inlineStr">
+        <is>
+          <t>新作,業績,海外</t>
+        </is>
+      </c>
+      <c r="L27" s="13" t="inlineStr">
+        <is>
+          <t>Day1 Game Pass除外がトピック</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B28" s="13" t="inlineStr">
+        <is>
+          <t>Frontier Developments、『Planet Zoo 2』を10/13に発売と発表、水族館・鳥類舎を新追加</t>
+        </is>
+      </c>
+      <c r="C28" s="13" t="inlineStr">
+        <is>
+          <t>https://www.frontier.co.uk/news/2026-05-28/build-wilder-world-october-planet-zoo-2</t>
+        </is>
+      </c>
+      <c r="D28" s="13" t="inlineStr">
+        <is>
+          <t>英Frontier Developmentsは『Planet Zoo』『Planet Coaster』『Jurassic World Evolution』等の経営シミュ専業。前作Planet Zoo（2019）は中長期セールスで成功した一方、株価は近年低迷していた。続編で水族館・鳥類舎・保全RP要素を新規追加。</t>
+        </is>
+      </c>
+      <c r="E28" s="13" t="inlineStr">
+        <is>
+          <t>Frontier Developmentsは5月28日、『Planet Zoo 2』を10月13日にPC/PS5/Xbox Series X|Sで発売すると発表。標準版49.99ドル、デラックス版64.99ドル。水生・飛行動物、ワイルドライフリザーブ（自然保護区）を新搭載。Summer Game Fest 2026にも参加。</t>
+        </is>
+      </c>
+      <c r="F28" s="13" t="inlineStr">
+        <is>
+          <t>発売日 2026/10/13
+PC/PS5/Xbox Series X|S
+標準版 49.99ドル/デラックス版 64.99ドル
+水族館・鳥類舎を新搭載
+保全エリア「Wildlife Reserves」</t>
+        </is>
+      </c>
+      <c r="G28" s="13" t="inlineStr">
+        <is>
+          <t>Frontierの経営シミュ路線の再起動。前作からのMOD/UGC継承度合いと、PC→コンソール拡大の同時ローンチが成否の鍵。経営シミュは長期セールスで稼ぐジャンルで、株価リカバリ材料となる可能性。</t>
+        </is>
+      </c>
+      <c r="H28" s="13" t="inlineStr">
+        <is>
+          <t>経営シミュ続編×コンソール同時展開</t>
+        </is>
+      </c>
+      <c r="I28" s="13" t="inlineStr">
+        <is>
+          <t>Frontier Developments</t>
+        </is>
+      </c>
+      <c r="J28" s="13" t="inlineStr">
+        <is>
+          <t>Planet Zoo</t>
+        </is>
+      </c>
+      <c r="K28" s="13" t="inlineStr">
+        <is>
+          <t>新作,海外</t>
+        </is>
+      </c>
+      <c r="L28" s="13" t="inlineStr">
+        <is>
+          <t>Summer Game Fest 2026参加予定</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B29" s="13" t="inlineStr">
+        <is>
+          <t>任天堂、Nintendo Switch 2を5/25より日本国内で1万円値上げ実施、PS5デジタル版を上回る価格に</t>
+        </is>
+      </c>
+      <c r="C29" s="13" t="inlineStr">
+        <is>
+          <t>https://game.watch.impress.co.jp/docs/news/2109655.html</t>
+        </is>
+      </c>
+      <c r="D29" s="13" t="inlineStr">
+        <is>
+          <t>任天堂は5月8日に値上げを予告、半導体メモリ高騰・円安・関税措置の3要因を背景に挙げていた。Switch 2はローンチ後約1年でハード値上げという異例の判断で、ローンチ前の予約者・初期購入者層との温度差も議論に。</t>
+        </is>
+      </c>
+      <c r="E29" s="13" t="inlineStr">
+        <is>
+          <t>Nintendo Switch 2（日本語・国内専用）は5月25日より49,980円→59,980円へ1万円値上げで販売開始。PS5デジタル・エディション（55,000円）を上回る価格に。Switch有機ELモデルも+10,000円、Liteも+8,002円改定。海外価格改定は9月1日予定。</t>
+        </is>
+      </c>
+      <c r="F29" s="13" t="inlineStr">
+        <is>
+          <t>Switch 2: 49,980円→59,980円（+1万円）
+5/25から販売開始
+PS5デジタル版（55,000円）を上回る
+有機ELモデル+1万円、Lite+8,002円
+海外は9/1から改定</t>
+        </is>
+      </c>
+      <c r="G29" s="13" t="inlineStr">
+        <is>
+          <t>値上げ前駆け込み需要が5月後半に集中（247,880台/週）、6月以降は一時的に販売鈍化見込み。FY27販売台数予想は1,650万台と前年からの減速を任天堂自身が織り込み済み。為替・関税が更に振れた場合は再度の改定リスクも。</t>
+        </is>
+      </c>
+      <c r="H29" s="13" t="inlineStr">
+        <is>
+          <t>コンシューマハードの値上げ耐性と価格弾力性</t>
+        </is>
+      </c>
+      <c r="I29" s="13" t="inlineStr">
+        <is>
+          <t>任天堂, ソニー</t>
+        </is>
+      </c>
+      <c r="J29" s="13" t="inlineStr">
+        <is>
+          <t>Nintendo Switch 2</t>
+        </is>
+      </c>
+      <c r="K29" s="13" t="inlineStr">
+        <is>
+          <t>業績,規制,国内</t>
+        </is>
+      </c>
+      <c r="L29" s="13" t="inlineStr">
+        <is>
+          <t>為替・関税・メモリ価格起点</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B30" s="13" t="inlineStr">
+        <is>
+          <t>Google Cloud、CapcomのエンタープライズAgentic AI導入事例を公開、内製パイプラインに統合</t>
+        </is>
+      </c>
+      <c r="C30" s="13" t="inlineStr">
+        <is>
+          <t>https://www.googlecloudpresscorner.com/2026-04-22-How-Capcom-Is-Leading-the-Way-for-Enterprise-Agentic-AI</t>
+        </is>
+      </c>
+      <c r="D30" s="13" t="inlineStr">
+        <is>
+          <t>GDC 2026でGoogle Cloudが発表したAIエージェントスイートに、Capcomが先行採用企業として登場。ゲーム開発コストは2017年比で約90%上昇しているとされ、各社が生成AIを内製パイプラインに静かに統合するフェーズに移行。</t>
+        </is>
+      </c>
+      <c r="E30" s="13" t="inlineStr">
+        <is>
+          <t>Google CloudはCapcomがAgentic AIをエンタープライズ業務（QA・ローカライズ・アセット下書き・社内検索等）に導入した事例を5月時点で公開。Googleは学習データ・生成結果の両面でIPインデムニティを提供し、AAAスタジオの著作権懸念を緩和する仕組みを訴求。</t>
+        </is>
+      </c>
+      <c r="F30" s="13" t="inlineStr">
+        <is>
+          <t>Capcomがエンタープライズ向けAgentic AIを採用
+QA/ローカライズ/アセット下書き等に活用
+GoogleがIPインデムニティを2層で提供
+ゲーム開発コストは2017年比+90%
+GDC 2026で全体方針を発表</t>
+        </is>
+      </c>
+      <c r="G30" s="13" t="inlineStr">
+        <is>
+          <t>AAA各社の「裏側AI活用」は加速、明示的にユーザー向けに見せるよりも内製工程の効率化に集中。Microsoft/Amazonのクラウド勢も同様の囲い込みを進める。日本のCapcom採用例は他和ゲー（バンダイナムコ・スクエニ）にも波及見込み。</t>
+        </is>
+      </c>
+      <c r="H30" s="13" t="inlineStr">
+        <is>
+          <t>AAA内製パイプラインのAgentic AI統合</t>
+        </is>
+      </c>
+      <c r="I30" s="13" t="inlineStr">
+        <is>
+          <t>Capcom, Google Cloud, Microsoft, Amazon</t>
+        </is>
+      </c>
+      <c r="J30" s="13" t="inlineStr">
+        <is>
+          <t>なし（社内パイプライン）</t>
+        </is>
+      </c>
+      <c r="K30" s="13" t="inlineStr">
+        <is>
+          <t>技術,海外,国内</t>
+        </is>
+      </c>
+      <c r="L30" s="13" t="inlineStr">
+        <is>
+          <t>GDC 2026関連の続報</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B31" s="13" t="inlineStr">
+        <is>
+          <t>『Path of Exile 2』、5/30からSteamフリーウィークエンド実施、早期アクセスパックも50%OFF</t>
+        </is>
+      </c>
+      <c r="C31" s="13" t="inlineStr">
+        <is>
+          <t>https://www.gamer.ne.jp/news/202605300001/</t>
+        </is>
+      </c>
+      <c r="D31" s="13" t="inlineStr">
+        <is>
+          <t>Grinding Gear Games運営のハクスラRPG『Path of Exile 2』は2024年12月にEarly Access開始。Diablo 4対抗の本命とされるが、Early Access期間が長期化し新規取り込みが課題となっていた。シーズン更新と並走でフリーウィークエンドを実施。</t>
+        </is>
+      </c>
+      <c r="E31" s="13" t="inlineStr">
+        <is>
+          <t>Steam上で5月30日からフリーウィークエンドを開始し、期間中は全コンテンツが無料プレイ可能。Early Accessパックも50%OFFセール。新規ユーザー獲得とコアプレイヤーの呼び戻しを同時に狙う、Live Service型ハクスラの典型的なグロース施策。</t>
+        </is>
+      </c>
+      <c r="F31" s="13" t="inlineStr">
+        <is>
+          <t>5/30フリーウィークエンド開始
+Early Accessパック50%OFF
+Diablo 4対抗の主要タイトル
+Early Access期間中の新規取り込み施策
+Steamのアクティブ拡張を狙う</t>
+        </is>
+      </c>
+      <c r="G31" s="13" t="inlineStr">
+        <is>
+          <t>フリーウィークエンド→Early Access販売の転換率がKPI。コアユーザー層への新シーズン投入とセットで、夏のSteam Summer Saleに繋ぐ流れ。1.0正式版リリース時期の見通しが次の注目点。</t>
+        </is>
+      </c>
+      <c r="H31" s="13" t="inlineStr">
+        <is>
+          <t>Live Service型ハクスラのフリーウィークエンド効果</t>
+        </is>
+      </c>
+      <c r="I31" s="13" t="inlineStr">
+        <is>
+          <t>Grinding Gear Games, Valve, Tencent</t>
+        </is>
+      </c>
+      <c r="J31" s="13" t="inlineStr">
+        <is>
+          <t>Path of Exile 2</t>
+        </is>
+      </c>
+      <c r="K31" s="13" t="inlineStr">
+        <is>
+          <t>eスポーツ,海外</t>
+        </is>
+      </c>
+      <c r="L31" s="13" t="inlineStr">
+        <is>
+          <t>Steam Summer Saleへの導線</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B32" s="13" t="inlineStr">
+        <is>
+          <t>Griffin Gaming Partners、インディー支援1億ドルの「Special Opportunities Fund」を始動</t>
+        </is>
+      </c>
+      <c r="C32" s="13" t="inlineStr">
+        <is>
+          <t>https://www.gamedeveloper.com/business/griffin-gaming-partners-launches-100m-fund-to-support-indie-devs</t>
+        </is>
+      </c>
+      <c r="D32" s="13" t="inlineStr">
+        <is>
+          <t>ゲーム特化VCのGriffin Gaming Partnersは累計運用約9億ドル規模。コンソール価格高騰とAAA開発費の高騰を受けて、インディー帯（$15-25）の重要性が再評価される中、レベニューシェア型の新ファンドを設立。</t>
+        </is>
+      </c>
+      <c r="E32" s="13" t="inlineStr">
+        <is>
+          <t>Griffin Gaming Partnersは「Special Opportunities Fund」（1億ドル）を始動。世界水準のインディータイトルへの資金提供と引き換えにレベニューシェアを取得。Hooded Horse CEO Tim Benderがマネージングディレクター就任。Darkwood 2, Hellforged, Vaunted, Menaceなど既に15タイトルへ投資済。</t>
+        </is>
+      </c>
+      <c r="F32" s="13" t="inlineStr">
+        <is>
+          <t>ファンド規模 1億ドル
+レベニューシェア型ファイナンス
+Hooded Horse CEO Tim Benderが運用責任者
+既に15タイトルに投資
+Darkwood 2/Hellforged/Vaunted/Menace等</t>
+        </is>
+      </c>
+      <c r="G32" s="13" t="inlineStr">
+        <is>
+          <t>ゲームVCはエクイティ投資からレベニューシェア型へのモデル移行が顕在化。インディーは「VC→パブリッシャー→Steam」の資金供給網が多層化し、AAA代替の収益源として機能。日本のインディー（BitSummit・TGSインディー）への海外マネー流入も加速見込み。</t>
+        </is>
+      </c>
+      <c r="H32" s="13" t="inlineStr">
+        <is>
+          <t>ゲーム特化VCのレベニューシェア型モデル</t>
+        </is>
+      </c>
+      <c r="I32" s="13" t="inlineStr">
+        <is>
+          <t>Griffin Gaming Partners, Hooded Horse</t>
+        </is>
+      </c>
+      <c r="J32" s="13" t="inlineStr">
+        <is>
+          <t>Darkwood 2, Hellforged, Vaunted, Menace</t>
+        </is>
+      </c>
+      <c r="K32" s="13" t="inlineStr">
+        <is>
+          <t>M&amp;A,インディー,海外</t>
+        </is>
+      </c>
+      <c r="L32" s="13" t="inlineStr">
+        <is>
+          <t>レベニューシェア型ゲームVC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
monthly matrix (2026-05) + future predictions (2026-05-30 02:21)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -776,7 +776,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -822,6 +822,191 @@
       <c r="G1" s="7" t="inlineStr">
         <is>
           <t>検証メモ</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>ハード値上げの連鎖が欧米へ本格波及し、9月のMSRP改定後に年末商戦の販売ペースが鈍化する</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>2026年9月〜年内</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>任天堂, Valve, ソニー / Switch 2, Steam Deck</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>任天堂Switch 2を日本で+20%値上げ（米欧は9/1予定）／Valve Steam Deck OLEDを+46%値上げ</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>9月の欧米MSRP改定実施と各社Q3セルスルー数値を確認</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Capcomに続き和ゲー大手（バンダイナムコ・スクエニ）が内製工程へのAgentic AI導入を公表する</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>3〜6ヶ月後</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Capcom, Google Cloud, バンダイナムコ, スクウェア・エニックス</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Google CloudがCapcomのエンタープライズAgentic AI導入事例を公開／Morgan StanleyがAIで220億ドルの利益機会と試算</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>他社のAI導入IR・カンファレンス発表、著作権/労務対応の有無を確認</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>PIF/Savvyや中国大手による新たな大型モバイルM&amp;A（10億ドル超）が発表され、日本IPも対象観測が出る</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>年内</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Savvy Games Group, PIF, NetEase, Tencent</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Q1ゲームM&amp;A総額77億ドル、SavvyのMoonton 60億ドル買収が牽引</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>次四半期のM&amp;Aレポート、日本企業の被買収・出資観測を確認</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>ソニーがGaaS投資を一段縮小し、シングルプレイ大作・外部スタジオ連携へ軸足を移す方針を示す</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>6〜12ヶ月後</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Sony, Bungie / Destiny 2, Marathon</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Bungieが『Destiny 2』運営を6/9終了／ソニーがBungie関連で5.65億ドル減損計上</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Marathonの発売・評価、SIEの投資方針コメントを確認</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>レベニューシェア型のインディー資金供給が他社にも拡大し、日本インディーへの海外マネー流入が増える</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>6〜12ヶ月後</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Griffin Gaming Partners, Hooded Horse, Global Game Jam</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Griffin Gamingがインディー向け1億ドルファンド始動／GGJがマイクログラント制度を始動</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>BitSummit/TGS出展作への海外資本参加、新ファンド組成の有無を確認</t>
         </is>
       </c>
     </row>
@@ -1643,15 +1828,66 @@
           <t>5月</t>
         </is>
       </c>
-      <c r="C30" s="9" t="inlineStr"/>
-      <c r="D30" s="9" t="inlineStr"/>
-      <c r="E30" s="9" t="inlineStr"/>
-      <c r="F30" s="9" t="inlineStr"/>
-      <c r="G30" s="9" t="inlineStr"/>
-      <c r="H30" s="9" t="inlineStr"/>
-      <c r="I30" s="9" t="inlineStr"/>
-      <c r="J30" s="9" t="inlineStr"/>
-      <c r="K30" s="9" t="inlineStr"/>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>・任天堂Switch 2を日本で¥49,980→¥59,980に値上げ（5/25、+20%）、購入「50時間」条件も撤廃
+・任天堂FY26決算 売上+98.6%／営業益+27.5%、FY27出荷想定1,650万台
+・GTA6を11/19、CoD:MW4を10/23、Planet Zoo 2を10/13に発売決定
+・『007 First Light』Metacritic88点、スクエニDQXII開発リスタート</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>・Valve、Steam Deck OLEDを512GB$549→$789／1TB$649→$949（+46%）に値上げ、再販即完売
+・『Path of Exile 2』5/30よりSteamフリーウィークエンド＋EA版50%OFF</t>
+        </is>
+      </c>
+      <c r="E30" s="9" t="inlineStr">
+        <is>
+          <t>・サイバーエージェント1H ゲーム営業益+106%、ウマ娘英語版で海外売上3.6倍（272億円）
+・Kuro Games『鳴潮』×ZOZOTOWNコラボ受注開始（5/29）、IPのアパレル化進む
+・NetEase Q1ゲーム部門+6.9%（257億元）</t>
+        </is>
+      </c>
+      <c r="F30" s="9" t="inlineStr">
+        <is>
+          <t>・Bungie『Destiny 2』ライブ運営を6/9で終了、9年に幕（新拡張・シーズン停止、サーバは継続）
+・CoD:MW4はGame Pass初日除外（約1年後追加）、MSのサブスク戦略見直しが鮮明</t>
+        </is>
+      </c>
+      <c r="G30" s="9" t="inlineStr">
+        <is>
+          <t>・EVO Japan 2026開催（5/1-3、東京ビッグサイト）、『スト6』ヤマグチ・『鉄拳8』iKARiが新王者
+・Riot新作『2XKO』が初の公式競技種目化、北米Hikari優勝</t>
+        </is>
+      </c>
+      <c r="H30" s="9" t="inlineStr">
+        <is>
+          <t>・Q1ゲームM&amp;Aは総額77億ドル・52件、Savvy(PIF)のMoonton 60億ドル買収が牽引
+・EmbracerがLotR/Tomb Raider等をFellowshipに分離、2027年Nasdaq上場へ
+・GameStopのeBay買収提案(560億ドル)は拒絶、IMCがPlaystack(Balatro)を約1.5億ドルで取得
+・Griffin Gamingがインディー向け1億ドルファンド始動</t>
+        </is>
+      </c>
+      <c r="I30" s="9" t="inlineStr">
+        <is>
+          <t>・Microsoft、Activision買収巡る株主訴訟を2.5億ドルで和解（自社負担40%）
+・Switch 2値上げの主因にAIメモリ高騰・米関税・為替、ハード価格上昇が業界全体へ波及</t>
+        </is>
+      </c>
+      <c r="J30" s="9" t="inlineStr">
+        <is>
+          <t>・Morgan Stanley、生成AIでゲーム業界に220億ドルの利益機会と試算（工期短縮・費用削減）
+・Google CloudがCapcomのエンタープライズAgentic AI導入事例を公開（QA/ローカライズ等）、GDC2026の主要テーマに</t>
+        </is>
+      </c>
+      <c r="K30" s="9" t="inlineStr">
+        <is>
+          <t>・NetEase Q1売上+6.1%（306億元）、Marvel Rivalsが寄与
+・ソニーがBungie関連で5.65億ドル減損（累計7.65億ドル）、Destiny 2運営終了と連動
+・Take-Two/RockstarやMicrosoftの大型タイトル・サブスク戦略が再編局面に</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="56" customHeight="1">
       <c r="A31" s="12" t="inlineStr"/>

</xml_diff>

<commit_message>
weekly-trends + tech update (data)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -1021,7 +1021,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1252,6 +1252,154 @@
       <c r="G6" t="inlineStr">
         <is>
           <t>https://micetimes.jp/en/bitsummit-punch-2026-news-2/, https://gamemakers.jp/article/2026_03_12_133353/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>EA売却(PIF主導コンソーシアム)と西側パブリッシャーの資本再編</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>EAがサウジ公共投資基金(PIF)主導のコンソーシアムへ売却される方向と報じられた。PIFは既にSavvy Games Groupを擁し、モバイルからコンソールまで版図を拡大中。Take-Twoと並ぶ西側最大級の独立系パブリッシャーが政府系ファンド傘下に入る構図で、大型新作カレンダーの薄さと株主圧力という業界全体の再編圧力が背景にある。買収価格の妥当性を巡る株主代表訴訟リスクも指摘され、単独での持続的成長が難しくなった巨大パブリッシャーの選択として注目される。</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>EA, Savvy Games Group, PIF(サウジ公共投資基金), Take-Two</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>ソブリンファンドによるゲーム資産取得は、IP・人材・配信網を一括で押さえる垂直統合戦略。新作不足と株主圧力で独立系の単独存続が難化し、資本の集中が加速。M&amp;A対価の妥当性審査が新たな摩擦点に。</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>コンテンツIPが地政学・国家資本の対象に。メディア/エンタメ全般のオーナーシップ集中と同型の動き。</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>https://www.gamesindustry.biz/ , https://luminatedata.com/blog/gaming-industry-off-to-a-shaky-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Steam生成AI開示ポリシーの二分化とLarian騒動</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>2026年1月、ValveはSteamの生成AI開示ルールを改定。コーディング補助など『開発効率化ツール』は開示不要とする一方、出荷されるゲームアセットを生成する用途は『事前生成』と『ライブ生成』に二分し開示義務を維持した。改定直前にはLarianが初期開発での生成AI利用で批判を浴び、CEOが利用を控える方針を表明。直近もCapcomがGoogle CloudのAgentic AIを内製工程へ導入する事例が公表され、透明性・倫理・制作パイプラインでのAIの役割を巡る論争が続いている。</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Valve(Steam), Larian Studios, Capcom, Google Cloud</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>プラットフォーマーが『制作ツールとしてのAI』と『出荷物としてのAI生成物』を制度的に分離した点が要諦。開示は信頼コストであり、表示設計がストア健全性とクリエイター保護を左右する。</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>生成AIの『ツール/成果物』二分は、あらゆる制作産業の表示・責任論の雛形になり得る。</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>https://opencritic.com/news/25847/ , https://gamerant.com/steam-changed-its-ai-disclosure-requirements-for-developers/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>ガチャ規制の各国格差と継続する締め付け圧力</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>中国NPPAはデイリーログイン報酬や初回購入ボーナス等の『課金誘因』を狙う規制を継続検討し、未成年のプレイ時間制限(週3時間)も維持。韓国は確率表示義務に続く第二弾のガチャ規制を推進。日本は2024年の電子商取引促進法改正で射幸性の高い課金システムへの監視を強化した。各国で賭博的設計への締め付けが進む一方、基準は不揃いで、グローバル運営の対応コストが増している。</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>NPPA(中国), 韓国規制当局, 消費者庁(日本), テンセント, ネットイース</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>ガチャは確率・上限・誘因設計の組合せで収益化される。規制は確率表示→誘因制限→支出上限へと段階的に進行し、各国の文化・法体系差が『規制裁定(regulatory arbitrage)』を生む。</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>国別格差はグローバル運営の設計分岐コストを増大。フィンテック等の射幸性商材にも波及し得る。</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mmorpg.com/news/china-proposes-mobile-game-regulations-banning-gacha-incentives-including-daily-logins-2000129890 , https://www.igamingtoday.com/korea-targets-gacha-mechanics-in-second-regulatory-push/</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>5月のAAA新作ラッシュとGTA6待ちの『枯れたカレンダー』</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>5月はForza Horizon 6(5/19・東京舞台/Steam同接30万超)、007 First Light(5/27・Metacritic88)、Directive 8020(5/12)、Subnautica 2(アーリーアクセス)など13本級の大型タイトルが集中する豊作月となった。一方で業界では『この5月以降、延期続くRockstarのGTA6(11/19予定)まで大型カレンダーが枯れる』との観測が広がる。リリースの山と谷が極端化し、話題と売上が一部時期に偏る構造が鮮明になった。</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Microsoft(Forza), IO Interactive, Supermassive Games, Unknown Worlds, Rockstar(GTA6)</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>開発の長期化と高コスト化で各社の投入時期が集中し、谷では話題と売上が枯渇。プラットフォームのMAU維持が少数の超大作待ちに依存する脆さが露呈。</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>ヒット集中型のリリース設計はリスク。映画の大作カレンダーと同型の需要平準化課題。</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>https://www.pcgamer.com/games/pc-game-release-dates-may-2026/ , https://gamerant.com/steam-new-games-coming-out-soon-may-2026/</t>
         </is>
       </c>
     </row>
@@ -7656,7 +7804,7 @@
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B2" s="9" t="inlineStr">
@@ -7671,14 +7819,34 @@
       </c>
       <c r="D2" s="9" t="inlineStr">
         <is>
-          <t>NPC会話・アセット生成・QA自動化での導入が進む。Square Enix、Konamiが言及</t>
-        </is>
-      </c>
-      <c r="E2" s="9" t="inlineStr"/>
-      <c r="F2" s="9" t="inlineStr"/>
-      <c r="G2" s="9" t="inlineStr"/>
-      <c r="H2" s="9" t="inlineStr"/>
-      <c r="I2" s="9" t="inlineStr"/>
+          <t>NPC会話・アセット生成・QA自動化に加え、内製工程へのAgentic AI導入とプラットフォーム開示制度の整備が同時進行。</t>
+        </is>
+      </c>
+      <c r="E2" s="9" t="inlineStr">
+        <is>
+          <t>2026年1月Steamが開示ルールを改定（効率化ツールは開示不要／出荷生成物は事前・ライブで開示義務）。Larianが初期利用で批判→自粛表明。CapcomがGoogle CloudのAgentic AIを内製導入と公表。Morgan Stanleyは業界で約220億ドルの利益機会と試算。</t>
+        </is>
+      </c>
+      <c r="F2" s="9" t="inlineStr">
+        <is>
+          <t>Valve, Larian Studios, Capcom, Google Cloud</t>
+        </is>
+      </c>
+      <c r="G2" s="9" t="inlineStr">
+        <is>
+          <t>『ツール利用』と『生成物出荷』の線引きが各ストア・各国で標準化。開示の粒度と内製効率化が競争・信頼の要因に。</t>
+        </is>
+      </c>
+      <c r="H2" s="9" t="inlineStr">
+        <is>
+          <t>論点が『使うか否か』から『何を出荷したか』『どう開示するか』へ移行している。</t>
+        </is>
+      </c>
+      <c r="I2" s="9" t="inlineStr">
+        <is>
+          <t>https://opencritic.com/news/25847/</t>
+        </is>
+      </c>
       <c r="J2" s="9" t="inlineStr"/>
     </row>
     <row r="3">
@@ -7852,7 +8020,7 @@
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B9" s="9" t="inlineStr">
@@ -7867,14 +8035,34 @@
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>国内消費者庁、海外規制動向</t>
-        </is>
-      </c>
-      <c r="E9" s="9" t="inlineStr"/>
-      <c r="F9" s="9" t="inlineStr"/>
-      <c r="G9" s="9" t="inlineStr"/>
-      <c r="H9" s="9" t="inlineStr"/>
-      <c r="I9" s="9" t="inlineStr"/>
+          <t>各国で段階的に規制が進むが基準は不揃いで、対応コストが増大。</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>中国NPPAがデイリーログイン・初回購入ボーナス等の課金誘因を狙う規制を継続検討。韓国は確率表示に続く第二弾規制を推進。日本は2024年電子商取引促進法改正で射幸性課金への監視を強化。</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>NPPA, 韓国規制当局, 消費者庁(日本), テンセント, ネットイース</t>
+        </is>
+      </c>
+      <c r="G9" s="9" t="inlineStr">
+        <is>
+          <t>確率表示→誘因制限→支出上限の順に各国が追随し、グローバル設計の分岐コストが増大。『規制裁定』が拠点・展開地域選定に影響。</t>
+        </is>
+      </c>
+      <c r="H9" s="9" t="inlineStr">
+        <is>
+          <t>規制の照準が『確率の透明化』から『行動誘因そのもの』へ移動している。</t>
+        </is>
+      </c>
+      <c r="I9" s="9" t="inlineStr">
+        <is>
+          <t>https://www.mmorpg.com/news/china-proposes-mobile-game-regulations-banning-gacha-incentives-including-daily-logins-2000129890</t>
+        </is>
+      </c>
       <c r="J9" s="9" t="inlineStr"/>
     </row>
     <row r="10">
@@ -7908,7 +8096,7 @@
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
@@ -7923,20 +8111,40 @@
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>Steam Deckの普及、PC比率上昇</t>
-        </is>
-      </c>
-      <c r="E11" s="9" t="inlineStr"/>
-      <c r="F11" s="9" t="inlineStr"/>
-      <c r="G11" s="9" t="inlineStr"/>
-      <c r="H11" s="9" t="inlineStr"/>
-      <c r="I11" s="9" t="inlineStr"/>
+          <t>大型新作とアーリーアクセスが牽引し、5月は13本級が集中する豊作月。</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>Forza Horizon 6がSteam同接30万超でXbox Game Studios歴代最高。007 First Light・Subnautica 2(EA)等が集中。Path of Exile 2が5/30よりフリーウィークエンド実施。</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>Valve, Microsoft, IO Interactive, Unknown Worlds, Grinding Gear Games</t>
+        </is>
+      </c>
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>PCが同時発売(デイワン)の主戦場として比重を拡大。アーリーアクセス＆フリーウィークエンドによる獲得施策が定着。</t>
+        </is>
+      </c>
+      <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t>5月の山の後、GTA6(11/19予定)まで谷が予想され、話題と売上が偏る。</t>
+        </is>
+      </c>
+      <c r="I11" s="9" t="inlineStr">
+        <is>
+          <t>https://www.pcgamer.com/games/pc-game-release-dates-may-2026/</t>
+        </is>
+      </c>
       <c r="J11" s="9" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B12" s="9" t="inlineStr">
@@ -7951,14 +8159,34 @@
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>ローンチタイトル、サードパーティ対応</t>
-        </is>
-      </c>
-      <c r="E12" s="9" t="inlineStr"/>
-      <c r="F12" s="9" t="inlineStr"/>
-      <c r="G12" s="9" t="inlineStr"/>
-      <c r="H12" s="9" t="inlineStr"/>
-      <c r="I12" s="9" t="inlineStr"/>
+          <t>発売1年未満で異例の価格改定が実施され、本体は品薄基調。</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>5/25より日本国内専用機が49,980→59,980円に改定（+1万円）。マイニンテンドーストアの購入条件『Switchプレイ時間50時間以上』が撤廃。2026はサードのデイワン投入拡大の見通し。</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>任天堂, サードパーティ各社</t>
+        </is>
+      </c>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>メモリ高騰起点の値上げが9月に欧米MSRPへ波及する可能性。需要が吸収すれば強気の供給戦略を継続。</t>
+        </is>
+      </c>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>ハード値上げを需要が吸収できるかが普及曲線の分岐点。値上げ連鎖は他ハードにも波及し得る。</t>
+        </is>
+      </c>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/article/202605/75886</t>
+        </is>
+      </c>
       <c r="J12" s="9" t="inlineStr"/>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
daily-news + cross-questions update (2026-05-31 01:46)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -2167,7 +2167,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2364,6 +2364,80 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>メガイベントの『地政学リスクによる開催地変更』は、国際スポーツ・MICE・展示会業界でも同様の意思決定を迫るか？</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>Esports World Cup 2026がイラン情勢を背景にサウジ・リヤドからパリへ移転、賞金75M史上最高</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>Esports World Cup財団, PIF</t>
+        </is>
+      </c>
+      <c r="E6" s="13" t="inlineStr">
+        <is>
+          <t>国際スポーツ興行, MICE/展示会, 観光・インバウンド, 保険(イベント中止保険)</t>
+        </is>
+      </c>
+      <c r="F6" s="13" t="inlineStr">
+        <is>
+          <t>新規</t>
+        </is>
+      </c>
+      <c r="G6" s="13" t="inlineStr">
+        <is>
+          <t>ソブリンファンド主導の超大型イベントほど政治リスクに脆弱。開催地分散・複数拠点化と中止保険の需要増がeスポーツ以外にも波及し得る。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>ゲーム業界の構造的レイオフと『AIによる開発効率化』の同時進行は、ITサービス・メディア・製造のホワイトカラー削減と同型か？</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>2026年5月もSurvios/Metacore/2K傘下でレイオフ継続、一方でMorgan StanleyはAIで220億ドルの利益機会と予測</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>Survios, Metacore, 2K, (AI効率化文脈)</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>ITサービス/SaaS, 広告・メディア制作, 製造業ホワイトカラー, コンサル</t>
+        </is>
+      </c>
+      <c r="F7" s="13" t="inlineStr">
+        <is>
+          <t>新規</t>
+        </is>
+      </c>
+      <c r="G7" s="13" t="inlineStr">
+        <is>
+          <t>『需要鈍化＋AI効率化』の二重要因による雇用減は他業界共通の構図。AIが補助か代替かで雇用インパクトが分岐する点が観察軸になる。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2375,7 +2449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L32"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4442,6 +4516,311 @@
           <t>レベニューシェア型ゲームVC</t>
         </is>
       </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B33" s="13" t="inlineStr">
+        <is>
+          <t>Esports World Cup 2026、賞金総額7500万ドルでパリ開催決定 — 中東情勢でリヤドから移転</t>
+        </is>
+      </c>
+      <c r="C33" s="13" t="inlineStr">
+        <is>
+          <t>https://esportsworldcup.com/en/news/ewc26-to-be-hosted-in-paris-france</t>
+        </is>
+      </c>
+      <c r="D33" s="13" t="inlineStr">
+        <is>
+          <t>EWCは前年までサウジアラビア・リヤドで開催され、PIFが主導する世界最大級のeスポーツ大会。2026年はイランを巡る中東情勢の緊迫を受け、サウジのインフラ攻撃リスクなどから開催地の安全確保が課題となっていた。</t>
+        </is>
+      </c>
+      <c r="E33" s="13" t="inlineStr">
+        <is>
+          <t>主催のEsports World Cup財団は、2026年大会をパリのExpo Porte de Versaillesで7/6〜8/23に開催すると発表。賞金総額は史上最高の7500万ドル（前年7150万ドルを更新）で、24eスポーツ・25種目を実施。クラブ選手権の優勝クラブには700万ドルが配分される。</t>
+        </is>
+      </c>
+      <c r="F33" s="13" t="inlineStr">
+        <is>
+          <t>賞金総額は史上最高の7500万ドル
+開催地をサウジ・リヤドからフランス・パリへ移転
+移転理由は中東情勢（イラン情勢）による安全確保
+会期は7/6〜8/23、24競技25種目
+チケット販売を開始</t>
+        </is>
+      </c>
+      <c r="G33" s="13" t="inlineStr">
+        <is>
+          <t>地政学リスクが大型eスポーツ興行の開催地選定を左右する先例となり、今後はサウジ依存からの分散や欧州・アジアでの複数拠点化が進む可能性。賞金インフレは継続するが、PIF資金の持続性と政治リスクが論点に。</t>
+        </is>
+      </c>
+      <c r="H33" s="13" t="inlineStr">
+        <is>
+          <t>eスポーツ興行の経済圏とソブリンファンド依存</t>
+        </is>
+      </c>
+      <c r="I33" s="13" t="inlineStr">
+        <is>
+          <t>Esports World Cup財団, PIF(サウジ公共投資ファンド)</t>
+        </is>
+      </c>
+      <c r="J33" s="13" t="inlineStr">
+        <is>
+          <t>Esports World Cup</t>
+        </is>
+      </c>
+      <c r="K33" s="13" t="inlineStr">
+        <is>
+          <t>eスポーツ,海外</t>
+        </is>
+      </c>
+      <c r="L33" s="13" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B34" s="13" t="inlineStr">
+        <is>
+          <t>欧州消費者機構BEUCが各国政府にルートボックス規制を要請、PEGIは6月から年齢制限引き上げ</t>
+        </is>
+      </c>
+      <c r="C34" s="13" t="inlineStr">
+        <is>
+          <t>https://www.jc-press.com/?p=8333</t>
+        </is>
+      </c>
+      <c r="D34" s="13" t="inlineStr">
+        <is>
+          <t>欧州ではベルギー・オランダがガチャ（ルートボックス）を実質禁止する一方、EU全体では統一規制がなく、未成年保護やダークパターンを巡る懸念が長年指摘されてきた。レーティング機関PEGIは2026年3月に運営型ゲームのルール強化を公表していた。</t>
+        </is>
+      </c>
+      <c r="E34" s="13" t="inlineStr">
+        <is>
+          <t>BEUCは加盟各国政府に対し、ダークパターンの禁止、ゲーム内通貨とリアルマネーの併記、未成年向けゲームでのルートボックス販売禁止、確率・アルゴリズムの透明化などを求めた。改善されない場合は有料ルートボックスの全面禁止も検討すべきと提言。PEGIは6月からガチャ要素を含むゲームを原則PEGI16以上に引き上げる。</t>
+        </is>
+      </c>
+      <c r="F34" s="13" t="inlineStr">
+        <is>
+          <t>BEUCが各国政府に包括的なガチャ規制を要請
+未成年向けゲームでのルートボックス販売禁止を要求
+ダークパターン禁止・確率/通貨表示の透明化を提言
+是正されなければ有料ルートボックス全面禁止も視野
+PEGIは6月施行で年齢制限を引き上げ</t>
+        </is>
+      </c>
+      <c r="G34" s="13" t="inlineStr">
+        <is>
+          <t>欧州での規制圧力が高まり、グローバル運営タイトルは地域別の課金設計・年齢制限対応を迫られる。日本の射幸性課金監視強化や韓国の確率表示義務と合わせ、対応コスト増と『規制の各国格差』が一段と顕在化する見込み。</t>
+        </is>
+      </c>
+      <c r="H34" s="13" t="inlineStr">
+        <is>
+          <t>ガチャ/ルートボックス規制の国際比較</t>
+        </is>
+      </c>
+      <c r="I34" s="13" t="inlineStr">
+        <is>
+          <t>BEUC(欧州消費者機構), NCC(ノルウェー消費者機構), PEGI</t>
+        </is>
+      </c>
+      <c r="J34" s="13" t="inlineStr"/>
+      <c r="K34" s="13" t="inlineStr">
+        <is>
+          <t>規制,海外</t>
+        </is>
+      </c>
+      <c r="L34" s="13" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>Wargaming『World of Tanks: HEAT』正式リリース、戦車“ヒーローシューター”へ転換しF2P/クロスプレイ対応</t>
+        </is>
+      </c>
+      <c r="C35" s="13" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/937/G093797/20260526034/</t>
+        </is>
+      </c>
+      <c r="D35" s="13" t="inlineStr">
+        <is>
+          <t>WargamingのWorld of Tanksは10年以上続く戦車戦MMOの代表格だが、新規プレイヤー獲得とF2Pシューター市場での競争が課題。クラス制を廃しエージェントロール（ディフェンダー/アタッカー/スナイパー）を導入した新作で、より高速・アクション寄りの体験へ刷新した。</t>
+        </is>
+      </c>
+      <c r="E35" s="13" t="inlineStr">
+        <is>
+          <t>Wargamingは5/26、戦車ヒーローシューター『World of Tanks: HEAT』をPC/PS5/Xbox Series X|S向けに基本プレイ無料で正式リリース。8エージェント・15車両・8マップ・4モードを備え、クロスプラットフォーム/クロスプログレッションに対応。無料ウィークリーバトルパスを含む『シーズン0』を開幕した。</t>
+        </is>
+      </c>
+      <c r="F35" s="13" t="inlineStr">
+        <is>
+          <t>戦車戦をヒーローシューター化した新作IP
+基本プレイ無料・クロスプレイ/クロスプログレッション対応
+エージェント制（ロール）導入でアクション性を強化
+Steam初動レビューは『やや不評』、クラッシュ多発の指摘
+開発元は不具合対応を表明</t>
+        </is>
+      </c>
+      <c r="G35" s="13" t="inlineStr">
+        <is>
+          <t>既存IPをジャンル転換して新規層を取り込む『ライブサービス再構築』の典型例。初動の技術的トラブルが定着率に響くリスクがあり、シーズン運営とアップデート速度が成否を分ける。ヒーローシューター飽和市場での差別化が問われる。</t>
+        </is>
+      </c>
+      <c r="H35" s="13" t="inlineStr">
+        <is>
+          <t>既存IPのジャンル転換とライブサービス設計</t>
+        </is>
+      </c>
+      <c r="I35" s="13" t="inlineStr">
+        <is>
+          <t>Wargaming</t>
+        </is>
+      </c>
+      <c r="J35" s="13" t="inlineStr">
+        <is>
+          <t>World of Tanks: HEAT, World of Tanks</t>
+        </is>
+      </c>
+      <c r="K35" s="13" t="inlineStr">
+        <is>
+          <t>新作,海外</t>
+        </is>
+      </c>
+      <c r="L35" s="13" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>ゲーム業界のレイオフ継続、5月もSurvios・Metacore・2K傘下31st Unionで人員削減</t>
+        </is>
+      </c>
+      <c r="C36" s="13" t="inlineStr">
+        <is>
+          <t>https://gamerant.com/every-video-game-layoff-and-studio-closure-in-2026-so-far/</t>
+        </is>
+      </c>
+      <c r="D36" s="13" t="inlineStr">
+        <is>
+          <t>2022年以降の金利上昇とコロナ特需の反動で、ゲーム業界は大規模な人員削減と統合が続く。AAA開発費の高騰、薄い新作カレンダー、生成AIによる効率化圧力が重なり、2026年も構造調整が止まらない状況にある。</t>
+        </is>
+      </c>
+      <c r="E36" s="13" t="inlineStr">
+        <is>
+          <t>2026年5月もレイオフが相次ぎ、VR大手Surviosが開発チームの大半を削減（5/1）、Metacoreが最大160人規模の再編（5/5）、2K傘下の31st Union（Project Ethos）でも削減（5/8）が報じられた。年初来の業界全体の削減ペースは前年より緩んだものの、大手の統合・事業転換による不確実性は続いている。</t>
+        </is>
+      </c>
+      <c r="F36" s="13" t="inlineStr">
+        <is>
+          <t>Surviosが開発チームの大半を削減（VR領域の縮小）
+Metacoreが最大160人規模の再編
+2K傘下31st Unionでも人員削減
+2026年も構造調整が継続
+AAA開発費高騰と薄い新作カレンダーが背景</t>
+        </is>
+      </c>
+      <c r="G36" s="13" t="inlineStr">
+        <is>
+          <t>GTA6発売までの『枯れたカレンダー』が続く中、コスト圧縮と選択と集中が継続。VRやライブサービス不振領域の撤退が進み、AIによる効率化が雇用減を加速させる一方、インディー帯やレベニューシェア型支援への資金シフトも併存する見込み。</t>
+        </is>
+      </c>
+      <c r="H36" s="13" t="inlineStr">
+        <is>
+          <t>ゲーム業界の人員削減と開発費構造</t>
+        </is>
+      </c>
+      <c r="I36" s="13" t="inlineStr">
+        <is>
+          <t>Survios, Metacore, 2K(Take-Two), 31st Union</t>
+        </is>
+      </c>
+      <c r="J36" s="13" t="inlineStr">
+        <is>
+          <t>Project Ethos</t>
+        </is>
+      </c>
+      <c r="K36" s="13" t="inlineStr">
+        <is>
+          <t>業績,海外</t>
+        </is>
+      </c>
+      <c r="L36" s="13" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B37" s="13" t="inlineStr">
+        <is>
+          <t>Steamforged、R6 Siegeボードゲームの製造写真がAI生成と発覚し批判、制作の透明性問題が再燃</t>
+        </is>
+      </c>
+      <c r="C37" s="13" t="inlineStr">
+        <is>
+          <t>https://www.goonhammer.com/games-industry-news-roundup-may-26th-2026</t>
+        </is>
+      </c>
+      <c r="D37" s="13" t="inlineStr">
+        <is>
+          <t>ゲーム/ボードゲーム業界では生成AIの利用と開示を巡る論争が続いており、ValveのSteam開示ポリシーやLarian騒動など、制作プロセスの透明性が継続的な争点になっている。</t>
+        </is>
+      </c>
+      <c r="E37" s="13" t="inlineStr">
+        <is>
+          <t>Steamforged Gamesは『Rainbow Six: Siege』ボードゲームの進捗報告として、印刷会社から送られた『製造完了を示す写真』を公開したが、ファンの検証によりこの写真がAI生成であることが判明し、説明の信頼性を巡って批判が広がった。実物の制作状況や情報開示のあり方が問われる事態となった。</t>
+        </is>
+      </c>
+      <c r="F37" s="13" t="inlineStr">
+        <is>
+          <t>製造完了を示すとされた写真がAI生成と判明
+ファンの検証で発覚し信頼性に疑問
+ボードゲーム/ゲーム制作の透明性問題が再燃
+生成AIの開示・倫理を巡る論争が継続</t>
+        </is>
+      </c>
+      <c r="G37" s="13" t="inlineStr">
+        <is>
+          <t>生成AIの安易な利用が広報・IR文脈での信頼毀損リスクになることを示す事例。今後は『AI利用の開示ルール』整備や、検証可能な一次情報（実写・工程記録）の重視が進む。透明性を欠く運用はコミュニティの反発を招きやすい。</t>
+        </is>
+      </c>
+      <c r="H37" s="13" t="inlineStr">
+        <is>
+          <t>生成AIの開示ルールと広報リスク</t>
+        </is>
+      </c>
+      <c r="I37" s="13" t="inlineStr">
+        <is>
+          <t>Steamforged Games</t>
+        </is>
+      </c>
+      <c r="J37" s="13" t="inlineStr">
+        <is>
+          <t>Rainbow Six: Siege</t>
+        </is>
+      </c>
+      <c r="K37" s="13" t="inlineStr">
+        <is>
+          <t>技術,海外</t>
+        </is>
+      </c>
+      <c r="L37" s="13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monthly matrix 2026-05 + future predictions (2026-06-01 00:27)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -776,7 +776,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1007,6 +1007,154 @@
       <c r="G6" s="3" t="inlineStr">
         <is>
           <t>BitSummit/TGS出展作への海外資本参加、新ファンド組成の有無を確認</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>ライブサービスの大量終了が下半期も続き、大手が新規GaaS投資を縮小、PvE協力・エクストラクション型（ARC Raiders系）が新たな主流テンプレートとして定着する</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>3〜6ヶ月後</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Bungie, Embark/Nexon, Amazon Games / Destiny 2, ARC Raiders</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Bungie『Destiny 2』ライブ運営を6/9で終了／2026上半期で52本のライブサービスが終了（掘り下げ）</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>下期のGaaS新規発表数とPvEエクストラクション系の後続タイトル数・同接を確認</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>EUでルートボックスの法規制化が前進し、PEGIの年齢制限強化に追随する国・ストアの開示義務が拡大する</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>6〜12ヶ月後</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>BEUC, NCC, PEGI / モバイル課金全般</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>欧州消費者機構BEUCが各国政府にルートボックス規制を要請、PEGIは6月から年齢制限引き上げ</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>EU加盟国の立法動向、各ストアの課金確率開示ルール改定を追跡</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>出荷物のAI生成発覚による炎上が常態化し、Steam等のAI開示ルールがさらに厳格化、開示の有無が信頼・売上の分岐点になる</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>年内</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Valve, Steamforged, Larian, Capcom / 業界全般</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Steamforged、R6 Siegeボードゲーム宣材のAI生成発覚で批判／Google CloudがCapcomのAgentic AI導入事例を公開</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>各ストアのAI開示ルール改定、炎上事例の発生頻度とユーザー反応を確認</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>GTA6（11/19）発売を避けて年末商戦の大型タイトルが発売時期を再調整し、2027年Q1へ延期・前倒しする動きが相次ぐ</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>2026年Q4〜2027年Q1</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Take-Two/Rockstar, Activision, Frontier / GTA6, CoD:MW4</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Take-Two『GTA6』を11/19と再確認「これ以上の延期なし」／CoD:MW4を10/23発売決定</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Q4発売予定タイトルの発売日変更アナウンス、2027年Q1の新作集中度を確認</t>
         </is>
       </c>
     </row>
@@ -1978,62 +2126,63 @@
       </c>
       <c r="C30" s="9" t="inlineStr">
         <is>
-          <t>・任天堂Switch 2を日本で¥49,980→¥59,980に値上げ（5/25、+20%）、購入「50時間」条件も撤廃
-・任天堂FY26決算 売上+98.6%／営業益+27.5%、FY27出荷想定1,650万台
-・GTA6を11/19、CoD:MW4を10/23、Planet Zoo 2を10/13に発売決定
-・『007 First Light』Metacritic88点、スクエニDQXII開発リスタート</t>
+          <t>・任天堂Switch 2を日本で¥49,980→¥59,980（+20%、5/25）に値上げ、購入「50時間」条件も撤廃
+・任天堂FY26決算 売上+98.6%／営業益+27.5%、Switch 2効果で大幅増益
+・GTA6を11/19、CoD:MW4を10/23と発売日確定し年末商戦に大型作集中
+・新作『007 First Light』Metacritic88点、スクエニDQXII開発リスタート発表</t>
         </is>
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>・Valve、Steam Deck OLEDを512GB$549→$789／1TB$649→$949（+46%）に値上げ、再販即完売
+          <t>・Valve、Steam Deck OLEDを$649→$949（+46%）に大幅値上げ、メモリ高騰・物流逼迫が背景
 ・『Path of Exile 2』5/30よりSteamフリーウィークエンド＋EA版50%OFF</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>・サイバーエージェント1H ゲーム営業益+106%、ウマ娘英語版で海外売上3.6倍（272億円）
-・Kuro Games『鳴潮』×ZOZOTOWNコラボ受注開始（5/29）、IPのアパレル化進む
-・NetEase Q1ゲーム部門+6.9%（257億元）</t>
+          <t>・サイバーエージェント中間決算 ゲーム営業益+106%、ウマ娘英語版で海外売上3.6倍
+・Kuro Games『鳴潮』×ZOZOTOWNコラボ受注開始、ゲームIPのアパレルEC連携進む
+・NetEase Q1ゲーム部門RMB257億（+6.9%）で安定成長</t>
         </is>
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
-          <t>・Bungie『Destiny 2』ライブ運営を6/9で終了、9年に幕（新拡張・シーズン停止、サーバは継続）
+          <t>・Bungie『Destiny 2』ライブ運営を6/9で終了、9年に幕（サーバは継続）
 ・CoD:MW4はGame Pass初日除外（約1年後追加）、MSのサブスク戦略見直しが鮮明</t>
         </is>
       </c>
       <c r="G30" s="9" t="inlineStr">
         <is>
-          <t>・EVO Japan 2026開催（5/1-3、東京ビッグサイト）、『スト6』ヤマグチ・『鉄拳8』iKARiが新王者
-・Riot新作『2XKO』が初の公式競技種目化、北米Hikari優勝</t>
+          <t>・EVO Japan 2026閉幕、『スト6』ヤマグチ・『鉄拳8』iKARiが新王者、Riot『2XKO』初開催
+・Esports World Cup 2026、賞金総額7500万ドルでパリ開催決定（中東情勢でリヤドから移転）</t>
         </is>
       </c>
       <c r="H30" s="9" t="inlineStr">
         <is>
-          <t>・Q1ゲームM&amp;Aは総額77億ドル・52件、Savvy(PIF)のMoonton 60億ドル買収が牽引
+          <t>・Q1ゲームM&amp;A総額77億ドル、Savvy(PIF)のMoonton 60億ドル買収が牽引
 ・EmbracerがLotR/Tomb Raider等をFellowshipに分離、2027年Nasdaq上場へ
-・GameStopのeBay買収提案(560億ドル)は拒絶、IMCがPlaystack(Balatro)を約1.5億ドルで取得
+・eBayのGameStop買収提案(560億ドル)拒絶、IMCがPlaystack(Balatro)を約1.5億ドルで取得
 ・Griffin Gamingがインディー向け1億ドルファンド始動</t>
         </is>
       </c>
       <c r="I30" s="9" t="inlineStr">
         <is>
           <t>・Microsoft、Activision買収巡る株主訴訟を2.5億ドルで和解（自社負担40%）
-・Switch 2値上げの主因にAIメモリ高騰・米関税・為替、ハード価格上昇が業界全体へ波及</t>
+・欧州BEUCが各国にルートボックス規制を要請、PEGIは6月から年齢制限引き上げ</t>
         </is>
       </c>
       <c r="J30" s="9" t="inlineStr">
         <is>
           <t>・Morgan Stanley、生成AIでゲーム業界に220億ドルの利益機会と試算（工期短縮・費用削減）
-・Google CloudがCapcomのエンタープライズAgentic AI導入事例を公開（QA/ローカライズ等）、GDC2026の主要テーマに</t>
+・Google CloudがCapcomのエンタープライズAgentic AI導入事例を公開（内製パイプライン統合）
+・Steamforged、R6ボードゲーム宣材のAI生成発覚で炎上、制作の透明性問題が再燃</t>
         </is>
       </c>
       <c r="K30" s="9" t="inlineStr">
         <is>
-          <t>・NetEase Q1売上+6.1%（306億元）、Marvel Rivalsが寄与
-・ソニーがBungie関連で5.65億ドル減損（累計7.65億ドル）、Destiny 2運営終了と連動
-・Take-Two/RockstarやMicrosoftの大型タイトル・サブスク戦略が再編局面に</t>
+          <t>・NetEase Q1売上RMB306億（+6.1%）、Marvel Rivalsが寄与
+・ソニーがBungie関連で5.65億ドル減損（累計7.65億ドル）
+・Take-Two、GTA6を11/19と再確認「これ以上の延期なし」</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
daily-news + cross-questions update (2026-06-01)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -29,7 +29,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -69,6 +69,9 @@
       <name val="Yu Gothic"/>
       <b val="1"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Yu Gothic"/>
     </font>
   </fonts>
   <fills count="3">
@@ -110,7 +113,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -140,6 +143,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2316,7 +2322,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2587,6 +2593,80 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>ゲーム企業のM&amp;A対価に暗号資産を用いる動きは、他業界のM&amp;A決済でも一般化するか？</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="inlineStr">
+        <is>
+          <t>Pearl AbyssによるCCP Games売却（対価に2,000万ドル相当の暗号資産トークンを含む）</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>Pearl Abyss, CCP Games(Fenris Creations), Eve Online</t>
+        </is>
+      </c>
+      <c r="E8" s="14" t="inlineStr">
+        <is>
+          <t>金融（決済・M&amp;Aアドバイザリー）、暗号資産取引所、会計・税務</t>
+        </is>
+      </c>
+      <c r="F8" s="14" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="G8" s="14" t="inlineStr">
+        <is>
+          <t>トークンを対価に含めると評価額の変動リスクと税務処理が新たな論点になる。金融・不動産など高額取引の決済手段多様化の先行例になりうる。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>ゲーム開発で進む自律型AIエージェントによる工程自動化は、広告・ソフトウェア・製造の制作現場でも同様に起きるか？</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="inlineStr">
+        <is>
+          <t>Google Cloudのゲーム開発向け自律型AIエージェント群投入、NVIDIA ACEの自律NPC</t>
+        </is>
+      </c>
+      <c r="D9" s="14" t="inlineStr">
+        <is>
+          <t>Google Cloud, NVIDIA, NVIDIA ACE</t>
+        </is>
+      </c>
+      <c r="E9" s="14" t="inlineStr">
+        <is>
+          <t>広告（クリエイティブ制作）、ソフトウェア開発、製造（設計・QA）</t>
+        </is>
+      </c>
+      <c r="F9" s="14" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="G9" s="14" t="inlineStr">
+        <is>
+          <t>反復作業の自動化と知財補償の枠組みは、他のデジタル制作産業の内製化・省力化のテンプレートになりうる。生成物の権利処理が共通課題。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2598,7 +2678,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L37"/>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4970,6 +5050,550 @@
         </is>
       </c>
       <c r="L37" s="13" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B38" s="14" t="inlineStr">
+        <is>
+          <t>Pearl AbyssがCCP Gamesを経営陣に売却、AI研究でDeepMindと提携</t>
+        </is>
+      </c>
+      <c r="C38" s="14" t="inlineStr">
+        <is>
+          <t>https://www.goonhammer.com/games-industry-news-roundup-may-12th-2026</t>
+        </is>
+      </c>
+      <c r="D38" s="14" t="inlineStr">
+        <is>
+          <t>韓国Pearl Abyssは2018年に約4.25億ドルでEve Online開発元のCCP Gamesを買収していたが、本業のクラウン関連タイトルに集中するため売却を模索していた。北欧のサンドボックスMMO運営の独立性回復が背景にある。</t>
+        </is>
+      </c>
+      <c r="E38" s="14" t="inlineStr">
+        <is>
+          <t>CCP GamesがCEOへ1億ドル＋2,000万ドル相当の暗号資産トークンで買い戻され、Pearl Abyss傘下を離脱。社名をFenris Creationsに変更し、Google DeepMindとAIの研究・テストで提携すると発表した。</t>
+        </is>
+      </c>
+      <c r="F38" s="14" t="inlineStr">
+        <is>
+          <t>・買収額は現金1億ドル＋暗号資産2,000万ドル相当
+・社名をFenris Creationsへ変更
+・Google DeepMindとAI協業
+・Eve Online運営は継続</t>
+        </is>
+      </c>
+      <c r="G38" s="14" t="inlineStr">
+        <is>
+          <t>独立後はEve OnlineのライブサービスにAIを組み込み、NPC高度化や運営自動化を進める可能性。暗号資産を対価に含めた点はゲーム業界M&amp;Aの決済手段多様化の例として注目され、他の中堅スタジオのMBO機運を刺激しうる。</t>
+        </is>
+      </c>
+      <c r="H38" s="14" t="inlineStr">
+        <is>
+          <t>ゲームスタジオのMBOと暗号資産による買収対価</t>
+        </is>
+      </c>
+      <c r="I38" s="14" t="inlineStr">
+        <is>
+          <t>Pearl Abyss, CCP Games, Fenris Creations, Google DeepMind</t>
+        </is>
+      </c>
+      <c r="J38" s="14" t="inlineStr">
+        <is>
+          <t>Eve Online</t>
+        </is>
+      </c>
+      <c r="K38" s="14" t="inlineStr">
+        <is>
+          <t>M&amp;A,技術,海外</t>
+        </is>
+      </c>
+      <c r="L38" s="14" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B39" s="14" t="inlineStr">
+        <is>
+          <t>ボードゲーム大手Asmodeeが定番タイトル「Time's Up!」を買収</t>
+        </is>
+      </c>
+      <c r="C39" s="14" t="inlineStr">
+        <is>
+          <t>https://www.goonhammer.com/games-industry-news-roundup-may-19th-2026</t>
+        </is>
+      </c>
+      <c r="D39" s="14" t="inlineStr">
+        <is>
+          <t>フランス拠点のボードゲーム大手Asmodeeは流通・出版網を生かしたIP集約を進めており、パーティーゲームの定番「Time's Up!」の権利取得により人気ブランドの自社管理を強める狙いがある。</t>
+        </is>
+      </c>
+      <c r="E39" s="14" t="inlineStr">
+        <is>
+          <t>Asmodeeが人気パーティーボードゲーム「Time's Up!」を買収し、ボードゲーム分野での拡大を継続。デジタル化やグローバル展開を見据えたIPポートフォリオ強化の一環とみられる。</t>
+        </is>
+      </c>
+      <c r="F39" s="14" t="inlineStr">
+        <is>
+          <t>・対象は定番パーティーゲーム「Time's Up!」
+・Asmodeeのボードゲーム拡大戦略
+・人気IPの自社管理を強化</t>
+        </is>
+      </c>
+      <c r="G39" s="14" t="inlineStr">
+        <is>
+          <t>アナログIPのデジタル移植やアプリ展開が進む可能性。ボードゲーム業界でも大手による人気IP囲い込みが続き、デジタルゲーム企業との協業余地が広がる。</t>
+        </is>
+      </c>
+      <c r="H39" s="14" t="inlineStr">
+        <is>
+          <t>アナログIPのデジタル展開戦略</t>
+        </is>
+      </c>
+      <c r="I39" s="14" t="inlineStr">
+        <is>
+          <t>Asmodee</t>
+        </is>
+      </c>
+      <c r="J39" s="14" t="inlineStr">
+        <is>
+          <t>Time's Up!</t>
+        </is>
+      </c>
+      <c r="K39" s="14" t="inlineStr">
+        <is>
+          <t>M&amp;A,海外</t>
+        </is>
+      </c>
+      <c r="L39" s="14" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B40" s="14" t="inlineStr">
+        <is>
+          <t>ソニー、PS5・PS5 Pro・Portalの追加値上げを世界的に発表</t>
+        </is>
+      </c>
+      <c r="C40" s="14" t="inlineStr">
+        <is>
+          <t>https://www.msn.com/en-us/technology/consumer-electronics/sony-officially-confirms-even-more-playstation-5-price-hikes-in-may-2026/ar-AA21Vc3I</t>
+        </is>
+      </c>
+      <c r="D40" s="14" t="inlineStr">
+        <is>
+          <t>為替変動やメモリ価格上昇、関税など世界的なコスト圧力が続くなか、ハードメーカー各社は値上げを余儀なくされている。ソニーは2026年4月末に世界的な価格改定を公表した。</t>
+        </is>
+      </c>
+      <c r="E40" s="14" t="inlineStr">
+        <is>
+          <t>ソニーがPS5、PS5 Pro、PlayStation Portalの価格を世界的に引き上げると正式に確認。世界経済の継続的な圧力を理由に挙げており、ハード収益性の確保を優先する姿勢を示した。</t>
+        </is>
+      </c>
+      <c r="F40" s="14" t="inlineStr">
+        <is>
+          <t>・対象はPS5/PS5 Pro/Portal
+・値上げは世界的に適用
+・要因は経済情勢・コスト上昇
+・任天堂はSwitch2を450ドルで据え置き</t>
+        </is>
+      </c>
+      <c r="G40" s="14" t="inlineStr">
+        <is>
+          <t>値上げはソフト・サブスク収益への依存をさらに高める。価格据え置きの任天堂Switch2との競争で普及台数に差が出る可能性があり、次世代機PS6の価格設定にも影響しうる。</t>
+        </is>
+      </c>
+      <c r="H40" s="14" t="inlineStr">
+        <is>
+          <t>ハード値上げとソフト・サービス収益シフト</t>
+        </is>
+      </c>
+      <c r="I40" s="14" t="inlineStr">
+        <is>
+          <t>ソニー, Sony Interactive Entertainment</t>
+        </is>
+      </c>
+      <c r="J40" s="14" t="inlineStr">
+        <is>
+          <t>PlayStation 5</t>
+        </is>
+      </c>
+      <c r="K40" s="14" t="inlineStr">
+        <is>
+          <t>業績,海外</t>
+        </is>
+      </c>
+      <c r="L40" s="14" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B41" s="14" t="inlineStr">
+        <is>
+          <t>任天堂、Switch2販売目標を1,900万台へ引き上げ通期上方修正</t>
+        </is>
+      </c>
+      <c r="C41" s="14" t="inlineStr">
+        <is>
+          <t>https://www.gamebusiness.jp/article/2026/04/30/26816.html#nintendo</t>
+        </is>
+      </c>
+      <c r="D41" s="14" t="inlineStr">
+        <is>
+          <t>2026年はSwitch2にとって最初の通期。立ち上がりが好調で、ハード普及がソフト販売とオンライン収益を押し上げる構図のなか、当初想定を上回るペースで推移していた。</t>
+        </is>
+      </c>
+      <c r="E41" s="14" t="inlineStr">
+        <is>
+          <t>任天堂がNintendo Switch2の通期販売目標を1,500万台から1,900万台へ引き上げ、通期業績予想を上方修正。新ハードの立ち上がりが想定を超える好調さを示した。</t>
+        </is>
+      </c>
+      <c r="F41" s="14" t="inlineStr">
+        <is>
+          <t>・Switch2目標1,500万→1,900万台
+・通期業績を上方修正
+・新ハード立ち上がりが好調
+・価格は450ドルで据え置き</t>
+        </is>
+      </c>
+      <c r="G41" s="14" t="inlineStr">
+        <is>
+          <t>普及拡大に伴い対応ソフトとオンライン課金の収益貢献が増す。値上げを進める競合に対し価格据え置きは普及面で優位に働く一方、部材コスト上昇下での採算維持が課題となる。</t>
+        </is>
+      </c>
+      <c r="H41" s="14" t="inlineStr">
+        <is>
+          <t>新ハード立ち上げ期の業績インパクト</t>
+        </is>
+      </c>
+      <c r="I41" s="14" t="inlineStr">
+        <is>
+          <t>任天堂</t>
+        </is>
+      </c>
+      <c r="J41" s="14" t="inlineStr">
+        <is>
+          <t>Nintendo Switch 2</t>
+        </is>
+      </c>
+      <c r="K41" s="14" t="inlineStr">
+        <is>
+          <t>業績,国内</t>
+        </is>
+      </c>
+      <c r="L41" s="14" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B42" s="14" t="inlineStr">
+        <is>
+          <t>IO Interactiveの新作『007 First Light』5月27日発売</t>
+        </is>
+      </c>
+      <c r="C42" s="14" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/article/202605/72904</t>
+        </is>
+      </c>
+      <c r="D42" s="14" t="inlineStr">
+        <is>
+          <t>『Hitman』シリーズで知られるIO Interactiveが、若き日のジェームズ・ボンドを描く完全新規のスパイアクションを開発。映画IPのAAAゲーム復権を狙う大型プロジェクトとして注目されてきた。</t>
+        </is>
+      </c>
+      <c r="E42" s="14" t="inlineStr">
+        <is>
+          <t>新作『007 First Light』が5月27日に発売。MI6入局直後の新人ボンドを主人公に、Hitmanの開発元が手掛けるステルス・アクションとして展開する。PS5など主要機種で登場した。</t>
+        </is>
+      </c>
+      <c r="F42" s="14" t="inlineStr">
+        <is>
+          <t>・開発はIO Interactive
+・若き日のボンドが主人公
+・5月27日発売
+・映画IPのAAA復権を狙う</t>
+        </is>
+      </c>
+      <c r="G42" s="14" t="inlineStr">
+        <is>
+          <t>評価次第でIO Interactiveのボンド3部作構想が前進し、映画IPのゲーム化トレンドを後押し。Hitmanで培ったステルス設計の評価がシリーズ継続の鍵となる。</t>
+        </is>
+      </c>
+      <c r="H42" s="14" t="inlineStr">
+        <is>
+          <t>映画IPのAAAゲーム化と評価リスク</t>
+        </is>
+      </c>
+      <c r="I42" s="14" t="inlineStr">
+        <is>
+          <t>IO Interactive</t>
+        </is>
+      </c>
+      <c r="J42" s="14" t="inlineStr">
+        <is>
+          <t>007 First Light</t>
+        </is>
+      </c>
+      <c r="K42" s="14" t="inlineStr">
+        <is>
+          <t>新作,海外</t>
+        </is>
+      </c>
+      <c r="L42" s="14" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B43" s="14" t="inlineStr">
+        <is>
+          <t>Google Cloud、ゲーム開発向け自律型AIエージェント群を投入</t>
+        </is>
+      </c>
+      <c r="C43" s="14" t="inlineStr">
+        <is>
+          <t>https://cloud.google.com/transform/a-new-era-of-gaming-how-the-next-generation-of-play-is-being-redefined-by-ai-agents</t>
+        </is>
+      </c>
+      <c r="D43" s="14" t="inlineStr">
+        <is>
+          <t>生成AIがテスト・コーディング・ローカライズなど開発工程に浸透し、Google Cloudの調査では開発者の約9割が日常業務でAIを利用。プラットフォーマー間でAI開発基盤の競争が激化している。</t>
+        </is>
+      </c>
+      <c r="E43" s="14" t="inlineStr">
+        <is>
+          <t>Google Cloudがクラウドベースのゲーム開発を効率化する自律型AIエージェント群を展開。反復作業の自動化や動的環境生成を支援し、学習データ・生成物の知財補償も提供する。NVIDIAのACEも自律キャラを高度化。</t>
+        </is>
+      </c>
+      <c r="F43" s="14" t="inlineStr">
+        <is>
+          <t>・自律型AIエージェント群を提供
+・テスト/コーディング自動化
+・学習データの知財補償
+・NVIDIA ACEで自律NPC高度化</t>
+        </is>
+      </c>
+      <c r="G43" s="14" t="inlineStr">
+        <is>
+          <t>開発の省力化と運営自動化が進み中小スタジオの参入障壁が下がる一方、AI生成物の権利処理や品質担保が論点に。クラウド各社のAI基盤囲い込み競争がさらに激化する。</t>
+        </is>
+      </c>
+      <c r="H43" s="14" t="inlineStr">
+        <is>
+          <t>ゲーム開発の生成AI活用と知財補償</t>
+        </is>
+      </c>
+      <c r="I43" s="14" t="inlineStr">
+        <is>
+          <t>Google Cloud, NVIDIA</t>
+        </is>
+      </c>
+      <c r="J43" s="14" t="inlineStr">
+        <is>
+          <t>Google Cloud AI, NVIDIA ACE</t>
+        </is>
+      </c>
+      <c r="K43" s="14" t="inlineStr">
+        <is>
+          <t>技術,海外</t>
+        </is>
+      </c>
+      <c r="L43" s="14" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B44" s="14" t="inlineStr">
+        <is>
+          <t>PEGI、有料ランダムアイテムを6月から16歳以上指定へ</t>
+        </is>
+      </c>
+      <c r="C44" s="14" t="inlineStr">
+        <is>
+          <t>https://www.esports.net/news/loot-boxes-rated-16-rule/</t>
+        </is>
+      </c>
+      <c r="D44" s="14" t="inlineStr">
+        <is>
+          <t>ルートボックスを賭博類似とみなす議論が欧州で高まり、各国の規制が分岐。PEGIは年齢レーティング枠組みの見直しを2026年3月に公表し、6月からの適用を予定していた。</t>
+        </is>
+      </c>
+      <c r="E44" s="14" t="inlineStr">
+        <is>
+          <t>欧州のPEGIが、有料のランダム要素を含むゲームを原則PEGI16（場合により18）に指定する新ルールを6月から適用。EUはQ4にルートボックス規制を含むデジタル公正法の提案を予定する。</t>
+        </is>
+      </c>
+      <c r="F44" s="14" t="inlineStr">
+        <is>
+          <t>・有料ランダム要素はPEGI16/18へ
+・6月から適用
+・EUデジタル公正法をQ4提案予定
+・ブラジルは未成年向け禁止へ</t>
+        </is>
+      </c>
+      <c r="G44" s="14" t="inlineStr">
+        <is>
+          <t>年齢指定の引き上げはガチャ・課金設計の見直しを各社に迫る。EUや各国規制が出そろえば、収益モデルの透明化やバトルパスへの移行が加速する可能性が高い。</t>
+        </is>
+      </c>
+      <c r="H44" s="14" t="inlineStr">
+        <is>
+          <t>ルートボックス規制と課金モデル転換</t>
+        </is>
+      </c>
+      <c r="I44" s="14" t="inlineStr">
+        <is>
+          <t>PEGI, 欧州連合(EU)</t>
+        </is>
+      </c>
+      <c r="J44" s="14" t="inlineStr"/>
+      <c r="K44" s="14" t="inlineStr">
+        <is>
+          <t>規制,海外</t>
+        </is>
+      </c>
+      <c r="L44" s="14" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B45" s="14" t="inlineStr">
+        <is>
+          <t>Xbox新CEO、ショーケースから他社ロゴ削除を示唆 6/7開催</t>
+        </is>
+      </c>
+      <c r="C45" s="14" t="inlineStr">
+        <is>
+          <t>https://khelnow.com/gaming/xbox-ceo-asha-sharma-hints-removing-playstation-nintendo-logos-from-future-showcases-202605</t>
+        </is>
+      </c>
+      <c r="D45" s="14" t="inlineStr">
+        <is>
+          <t>マルチプラットフォーム戦略でXboxは自社タイトルを他機種にも展開してきたが、新ハード投入を控えブランド強化と独占確保を巡る議論が社内で活発化している。</t>
+        </is>
+      </c>
+      <c r="E45" s="14" t="inlineStr">
+        <is>
+          <t>Xboxの新CEOアシャ・シャルマが、今後のショーケースからPlayStationやNintendoのロゴを外す可能性を示唆。6月7日に自身初のXbox Games Showcaseを控え、独占強化の議論も報じられた。</t>
+        </is>
+      </c>
+      <c r="F45" s="14" t="inlineStr">
+        <is>
+          <t>・他社ロゴ削除を示唆
+・6/7に新CEO初のショーケース
+・独占確保の議論を報道
+・マルチ展開戦略の調整局面</t>
+        </is>
+      </c>
+      <c r="G45" s="14" t="inlineStr">
+        <is>
+          <t>マルチ展開とブランド再強化のバランスが焦点。6/7のショーケース内容と独占方針が、次世代Xboxの立ち位置とサードパーティ戦略の方向性を占う試金石となる。</t>
+        </is>
+      </c>
+      <c r="H45" s="14" t="inlineStr">
+        <is>
+          <t>プラットフォーム独占とマルチ展開戦略</t>
+        </is>
+      </c>
+      <c r="I45" s="14" t="inlineStr">
+        <is>
+          <t>Microsoft, Xbox</t>
+        </is>
+      </c>
+      <c r="J45" s="14" t="inlineStr">
+        <is>
+          <t>Xbox Games Showcase</t>
+        </is>
+      </c>
+      <c r="K45" s="14" t="inlineStr">
+        <is>
+          <t>海外</t>
+        </is>
+      </c>
+      <c r="L45" s="14" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="B46" s="14" t="inlineStr">
+        <is>
+          <t>無料idle RPG『タスクバーヒーロー』同接14万人超の人気に</t>
+        </is>
+      </c>
+      <c r="C46" s="14" t="inlineStr">
+        <is>
+          <t>https://news.yahoo.co.jp/articles/32cdf41ea07ab3549d7ce56a57880b4f5952adae</t>
+        </is>
+      </c>
+      <c r="D46" s="14" t="inlineStr">
+        <is>
+          <t>放置・idle系ゲームは低コストで手軽に遊べる点から世界的に人気が拡大。Steamの基本無料タイトルがSNSや配信を通じて短期間で大量のユーザーを集める事例が増えている。</t>
+        </is>
+      </c>
+      <c r="E46" s="14" t="inlineStr">
+        <is>
+          <t>Steam向け基本無料のidle RPG『タスクバーヒーロー』が5月27日配信。5月31日夜時点で同時接続143,508人を記録する人気となった。一方で出品アイテムの一部削除アナウンスも報じられている。</t>
+        </is>
+      </c>
+      <c r="F46" s="14" t="inlineStr">
+        <is>
+          <t>・5/27配信の基本無料idle RPG
+・同接143,508人を記録
+・SNS/配信で急拡大
+・一部アイテム削除のアナウンス</t>
+        </is>
+      </c>
+      <c r="G46" s="14" t="inlineStr">
+        <is>
+          <t>基本無料idle系の急成長は継続課金とユーザー維持が課題。短期の話題性をどうマネタイズと長期運営につなげるかが、同種インディータイトルの成否を分ける。</t>
+        </is>
+      </c>
+      <c r="H46" s="14" t="inlineStr">
+        <is>
+          <t>基本無料idleゲームの拡散と収益化</t>
+        </is>
+      </c>
+      <c r="I46" s="14" t="inlineStr">
+        <is>
+          <t>インディー開発</t>
+        </is>
+      </c>
+      <c r="J46" s="14" t="inlineStr">
+        <is>
+          <t>タスクバーヒーロー</t>
+        </is>
+      </c>
+      <c r="K46" s="14" t="inlineStr">
+        <is>
+          <t>インディー,国内</t>
+        </is>
+      </c>
+      <c r="L46" s="14" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
daily-news + cross-questions update (2026-06-01 23:10)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -2322,7 +2322,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2667,6 +2667,43 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>ゲーミングGPUを核にAIエージェント対応PC（RTX Spark）が主流化する流れは、PC・半導体業界の主戦場を『描画/演算性能』から『オンデバイスAI』へ移すか？他業界の買い替え基準は何に置き換わるか？</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="inlineStr">
+        <is>
+          <t>NVIDIAがComputex 2026でRTX Spark（Grace+Blackwell SoC、128GB統合メモリ）を発表（6/1）</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>NVIDIA, Microsoft, Dell, HP, Lenovo, MediaTek</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="inlineStr">
+        <is>
+          <t>PC・半導体（チップ設計）、エンタープライズIT（業務PC更新）、家電（デバイス選定基準）</t>
+        </is>
+      </c>
+      <c r="F10" s="14" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="G10" s="14" t="inlineStr">
+        <is>
+          <t>ゲーミング由来の高性能GPUがAIエージェント基盤として汎用化すると、PC購買の評価軸が一般オフィス/家電市場にも波及。ゲーム業界が他デジタル産業のハードウェア標準を先導する構図。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2678,7 +2715,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L46"/>
+  <dimension ref="A1:L51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5594,6 +5631,314 @@
         </is>
       </c>
       <c r="L46" s="14" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B47" s="14" t="inlineStr">
+        <is>
+          <t>PlayStation「State of Play」6月2日配信、『Marvel's Wolverine』先頭に60分超</t>
+        </is>
+      </c>
+      <c r="C47" s="14" t="inlineStr">
+        <is>
+          <t>https://blog.playstation.com/2026/05/20/state-of-play-returns-tuesday-june-2/</t>
+        </is>
+      </c>
+      <c r="D47" s="14" t="inlineStr">
+        <is>
+          <t>ソニーはE3亡き後、自社配信「State of Play」を新作発表の主戦場としてきた。今回はXbox Games Showcase（6/7）の直前という日程で、両陣営のショーケースが約1週間内に並ぶ事実上のE3型対決の構図となった。</t>
+        </is>
+      </c>
+      <c r="E47" s="14" t="inlineStr">
+        <is>
+          <t>ソニーは6月2日（米国時間、日本時間6月3日午前6時）に60分超のState of Playを配信。Insomniac開発の『Marvel's Wolverine』（9/15発売）のゲームプレイを冒頭で公開し、世界中のスタジオからの発表・映像を予告した。</t>
+        </is>
+      </c>
+      <c r="F47" s="14" t="inlineStr">
+        <is>
+          <t>・6/2配信、60分超の大型ショーケース
+・冒頭は『Marvel's Wolverine』（PS5、9/15発売）
+・Xbox Games Showcase（6/7）と1週間内で接近
+・「世界中のトップスタジオ」からの新発表を予告</t>
+        </is>
+      </c>
+      <c r="G47" s="14" t="inlineStr">
+        <is>
+          <t>Insomniacのマーベル路線の拡大とPS5独占タイトルの年末商戦布陣が焦点。Xboxショーケースとの近接日程は、夏の新作発表競争を激化させ、両陣営の独占・マルチ戦略の差を鮮明にする可能性が高い。</t>
+        </is>
+      </c>
+      <c r="H47" s="14" t="inlineStr">
+        <is>
+          <t>据置機メーカーの自社配信ショーケース戦略とE3後の発表競争</t>
+        </is>
+      </c>
+      <c r="I47" s="14" t="inlineStr">
+        <is>
+          <t>ソニー・インタラクティブエンタテインメント, Insomniac Games, マイクロソフト</t>
+        </is>
+      </c>
+      <c r="J47" s="14" t="inlineStr">
+        <is>
+          <t>Marvel's Wolverine</t>
+        </is>
+      </c>
+      <c r="K47" s="14" t="inlineStr">
+        <is>
+          <t>新作,海外</t>
+        </is>
+      </c>
+      <c r="L47" s="14" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B48" s="14" t="inlineStr">
+        <is>
+          <t>NVIDIA、Computex 2026で「RTX Spark」発表 Grace Blackwell SoCでWindows PCのAI化へ</t>
+        </is>
+      </c>
+      <c r="C48" s="14" t="inlineStr">
+        <is>
+          <t>https://nvidianews.nvidia.com/news/nvidia-microsoft-windows-pcs-agents-rtx-spark</t>
+        </is>
+      </c>
+      <c r="D48" s="14" t="inlineStr">
+        <is>
+          <t>ゲーミングGPUで圧倒的シェアを持つNVIDIAが、ArmベースCPUとBlackwell GPUを統合したSoCでPC本体市場に本格参入。生成AIの実用フェーズ移行を背景に、オンデバイスでAIエージェントを動かす「個人AI」時代のPCを打ち出した。</t>
+        </is>
+      </c>
+      <c r="E48" s="14" t="inlineStr">
+        <is>
+          <t>Jensen Huang CEOが台北Computex 2026の基調講演（6/1）でRTX Sparkを発表。Blackwell RTX GPU（6,144 CUDAコア）と20コアGrace CPUをNVLink-C2Cで接続、128GB統合メモリを搭載。Microsoft Surface、Dell、HP、Lenovo、ASUS、MSIから今秋投入予定。</t>
+        </is>
+      </c>
+      <c r="F48" s="14" t="inlineStr">
+        <is>
+          <t>・Computex 2026 基調講演（6/1）で発表
+・Grace CPU＋Blackwell GPUの統合SoC、128GB統合メモリ
+・Microsoft/Dell/HP/Lenovo/ASUS/MSIが今秋投入
+・ゲーミング性能とオンデバイスAIエージェントを両立
+・3世代ロードマップ（Rubin、Rosa等）も提示</t>
+        </is>
+      </c>
+      <c r="G48" s="14" t="inlineStr">
+        <is>
+          <t>ゲーミングPCの主戦場が純粋な描画性能からオンデバイスAI性能へ移行する転換点になり得る。AI PCの普及はゲーム開発の制作環境（生成・QA）やクラウドゲーミングとの競合関係にも波及する見込み。</t>
+        </is>
+      </c>
+      <c r="H48" s="14" t="inlineStr">
+        <is>
+          <t>オンデバイスAIとゲーミングPCアーキテクチャの融合</t>
+        </is>
+      </c>
+      <c r="I48" s="14" t="inlineStr">
+        <is>
+          <t>NVIDIA, Microsoft, Dell, HP, Lenovo, ASUS, MSI, MediaTek</t>
+        </is>
+      </c>
+      <c r="J48" s="14" t="inlineStr">
+        <is>
+          <t>RTX Spark, GeForce RTX</t>
+        </is>
+      </c>
+      <c r="K48" s="14" t="inlineStr">
+        <is>
+          <t>技術,海外</t>
+        </is>
+      </c>
+      <c r="L48" s="14" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B49" s="14" t="inlineStr">
+        <is>
+          <t>Gravity、『RAGNAROK』25年で初の単独RPGをコンソール向けに発表 4機種・2027年上期</t>
+        </is>
+      </c>
+      <c r="C49" s="14" t="inlineStr">
+        <is>
+          <t>https://www.gematsu.com/2026/05/ragnarok-console-project-announced-for-ps5-xbox-series-switch-2-and-pc</t>
+        </is>
+      </c>
+      <c r="D49" s="14" t="inlineStr">
+        <is>
+          <t>世界1億人以上が遊んだMMORPG『ラグナロクオンライン』を擁するGravityが、長年のオンライン路線から転換。シングルプレイRPGとして据置・携帯機（Switch 2含む）に展開し、既存IPの新規層獲得を狙う。</t>
+        </is>
+      </c>
+      <c r="E49" s="14" t="inlineStr">
+        <is>
+          <t>GravityとDaweon Game Media Lab、開発Waycoderが「Ragnarok Console Project」をPS5/Xbox Series/Switch 2/PC（Steam）向けに発表。2027年上期発売予定。シリーズ初のシングルプレイRPGで「選択と責任」をテーマにした物語重視の作品となる。</t>
+        </is>
+      </c>
+      <c r="F49" s="14" t="inlineStr">
+        <is>
+          <t>・シリーズ25年で初の単独（シングルプレイ）RPG
+・PS5/Xbox Series/Switch 2/PCのマルチ展開
+・2027年上期発売予定
+・ナイト/メイジ/プリースト/ハンター等の仲間が登場
+・原作MMOは世界1億人以上が体験</t>
+        </is>
+      </c>
+      <c r="G49" s="14" t="inlineStr">
+        <is>
+          <t>長寿MMO IPのシングルプレイ・コンソール転生は、韓国系オンラインIPの収益多角化モデルの試金石。Switch 2を含むマルチ展開は、アジア発IPのグローバル据置機市場での存在感拡大につながる可能性。</t>
+        </is>
+      </c>
+      <c r="H49" s="14" t="inlineStr">
+        <is>
+          <t>長寿オンラインIPのシングルプレイ・コンソール展開戦略</t>
+        </is>
+      </c>
+      <c r="I49" s="14" t="inlineStr">
+        <is>
+          <t>Gravity, Daweon Game Media Lab, Waycoder</t>
+        </is>
+      </c>
+      <c r="J49" s="14" t="inlineStr">
+        <is>
+          <t>RAGNAROK（ラグナロク）</t>
+        </is>
+      </c>
+      <c r="K49" s="14" t="inlineStr">
+        <is>
+          <t>新作,海外</t>
+        </is>
+      </c>
+      <c r="L49" s="14" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B50" s="14" t="inlineStr">
+        <is>
+          <t>Xbox、『Fable』を2027年2月へ延期 6/7ショーケースで新映像 GTA6など年末混雑回避</t>
+        </is>
+      </c>
+      <c r="C50" s="14" t="inlineStr">
+        <is>
+          <t>https://gameinformer.com/2026/05/29/fable-delayed-to-february-2027</t>
+        </is>
+      </c>
+      <c r="D50" s="14" t="inlineStr">
+        <is>
+          <t>2026年末はHalo: Campaign Evolved、Gears of War: E-Day、CoD: MW4、GTA6など大型タイトルが集中。Xboxは看板RPG『Fable』を混雑したカレンダーから外し、発売の見通しを確保する判断を下した。</t>
+        </is>
+      </c>
+      <c r="E50" s="14" t="inlineStr">
+        <is>
+          <t>マイクロソフトは『Fable』を当初の2026年秋から2027年2月へ延期すると5/29に発表。混雑する年末商戦を避ける狙い。同作は6/7のXbox Games Showcase（米時間10時PT）で大型の新映像を披露する予定。</t>
+        </is>
+      </c>
+      <c r="F50" s="14" t="inlineStr">
+        <is>
+          <t>・『Fable』を2026年秋→2027年2月へ延期
+・GTA6など年末大型タイトル集中の回避が理由
+・6/7 Xbox Games Showcaseで新映像予告
+・年末布陣はHalo CE、Gears E-Day、CoD MW4等</t>
+        </is>
+      </c>
+      <c r="G50" s="14" t="inlineStr">
+        <is>
+          <t>GTA6（11/19予定）の重力圏を避けるリリース設計が各社で続く見込み。第1四半期（2027年初頭）に大型タイトルが後ろ倒しで集中し、いわゆる『枯れたカレンダー』と『谷』の構造が一段と鮮明になる。</t>
+        </is>
+      </c>
+      <c r="H50" s="14" t="inlineStr">
+        <is>
+          <t>大型タイトルのリリース時期設計とGTA6回避ムーブ</t>
+        </is>
+      </c>
+      <c r="I50" s="14" t="inlineStr">
+        <is>
+          <t>マイクロソフト, Xbox Game Studios, Playground Games, Take-Two/Rockstar</t>
+        </is>
+      </c>
+      <c r="J50" s="14" t="inlineStr">
+        <is>
+          <t>Fable, GTA6</t>
+        </is>
+      </c>
+      <c r="K50" s="14" t="inlineStr">
+        <is>
+          <t>新作,海外</t>
+        </is>
+      </c>
+      <c r="L50" s="14" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B51" s="14" t="inlineStr">
+        <is>
+          <t>Minecraft Live（5月）開催、新バイオーム「Dappled Forest」と『Dungeons II』公開</t>
+        </is>
+      </c>
+      <c r="C51" s="14" t="inlineStr">
+        <is>
+          <t>https://www.pcgamesn.com/minecraft/live-may-2026-dappled-forest-biome</t>
+        </is>
+      </c>
+      <c r="D51" s="14" t="inlineStr">
+        <is>
+          <t>世界最大級の販売本数を誇るMinecraftは、定期配信「Minecraft Live」で新要素を小出しにし、巨大コミュニティの継続的な関与を維持する運営モデルを取る。続編『Dungeons II』の存在も明らかになった。</t>
+        </is>
+      </c>
+      <c r="E51" s="14" t="inlineStr">
+        <is>
+          <t>Minecraft Live（5月版、6/1前後に国内報道）で、ポプラと赤い低木が紅葉色を作る新バイオーム「Dappled Forest」と廃キャンプ、ウールの階段/ハーフブロックを発表。マルチプラットフォーム展開の続編『Minecraft Dungeons II』も今年後半投入を告知した。</t>
+        </is>
+      </c>
+      <c r="F51" s="14" t="inlineStr">
+        <is>
+          <t>・新バイオーム「Dappled Forest」（紅葉系・廃キャンプ）
+・ウールの階段/ハーフブロック追加、夏にテスト開始
+・続編『Minecraft Dungeons II』を今年後半に投入
+・Dungeons IIは新敵Twisted Wardenやディープダーク要素
+・全主要プラットフォーム＋Game Pass対応</t>
+        </is>
+      </c>
+      <c r="G51" s="14" t="inlineStr">
+        <is>
+          <t>巨大既存IPの『継続的アップデート＋スピンオフ続編』モデルは、新作リスクを抑えつつエンゲージメントを保つ王道として他の長寿IPにも波及。Game Pass連動はサブスク基盤の維持戦略として重要度を増す。</t>
+        </is>
+      </c>
+      <c r="H51" s="14" t="inlineStr">
+        <is>
+          <t>長寿サンドボックスIPの継続運営とスピンオフ展開</t>
+        </is>
+      </c>
+      <c r="I51" s="14" t="inlineStr">
+        <is>
+          <t>Mojang Studios, Microsoft</t>
+        </is>
+      </c>
+      <c r="J51" s="14" t="inlineStr">
+        <is>
+          <t>Minecraft, Minecraft Dungeons II</t>
+        </is>
+      </c>
+      <c r="K51" s="14" t="inlineStr">
+        <is>
+          <t>新作,海外</t>
+        </is>
+      </c>
+      <c r="L51" s="14" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
daily-news + cross-questions update (2026-06-02 22:09)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -2322,7 +2322,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2704,6 +2704,80 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="inlineStr">
+        <is>
+          <t>サウジ等ソブリンファンドによるゲーム大型買収（Savvy×Moonton 60億ドル）の波は、スポーツ・メディア・不動産など他のエンタメ/実物資産業界へのソブリンマネー流入と同じ構造か？</t>
+        </is>
+      </c>
+      <c r="C11" s="14" t="inlineStr">
+        <is>
+          <t>ゲーム業界M&amp;Aが2026年Q1に77億ドル、SavvyがMoontonを60億ドルで買収（PocketGamer.biz）</t>
+        </is>
+      </c>
+      <c r="D11" s="14" t="inlineStr">
+        <is>
+          <t>Savvy Games Group, Moonton, PIF</t>
+        </is>
+      </c>
+      <c r="E11" s="14" t="inlineStr">
+        <is>
+          <t>スポーツ（クラブ/リーグ買収）、メディア・エンタメ、不動産・インフラ</t>
+        </is>
+      </c>
+      <c r="F11" s="14" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="G11" s="14" t="inlineStr">
+        <is>
+          <t>ゲームは若年層リーチと知財を伴うため、国家戦略的なソフトパワー投資の対象になりやすい。他エンタメ資産との取得競合・価格形成への影響を観察したい。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>eスポーツ視聴のモバイル/TikTok Liveシフト（月33億時間）は、スポーツ中継・音楽ライブ配信など他の観戦型コンテンツの収益化・放映権モデルにも波及するか？</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>世界eスポーツ視聴が月33億時間で記録更新、モバイルが牽引（Esports Charts）</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>Moonton, TikTok, Riot Games</t>
+        </is>
+      </c>
+      <c r="E12" s="14" t="inlineStr">
+        <is>
+          <t>スポーツ放映権、音楽ライブ配信、TV/メディア</t>
+        </is>
+      </c>
+      <c r="F12" s="14" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="G12" s="14" t="inlineStr">
+        <is>
+          <t>短尺・縦型・無料配信への観戦移行は、従来の有料放映権モデルを侵食しうる。スポンサー収益と配信プラットフォーム分散の関係を要観察。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2715,7 +2789,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L51"/>
+  <dimension ref="A1:L61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5939,6 +6013,626 @@
         </is>
       </c>
       <c r="L51" s="14" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B52" s="14" t="inlineStr">
+        <is>
+          <t>ゲーム業界M&amp;Aが2026年Q1に77億ドル到達、SavvyがMoontonを60億ドルで買収</t>
+        </is>
+      </c>
+      <c r="C52" s="14" t="inlineStr">
+        <is>
+          <t>https://www.pocketgamer.biz/games-industry-manda-hits-77bn-in-q1-2026-led-by-savvy-games-group/</t>
+        </is>
+      </c>
+      <c r="D52" s="14" t="inlineStr">
+        <is>
+          <t>パンデミック後の調整局面を経て、潤沢な資金を持つ大手やソブリンファンドが割安となったスタジオの取得を加速。特にモバイル分野での統合が顕著で、市場は再編フェーズに入っている。</t>
+        </is>
+      </c>
+      <c r="E52" s="14" t="inlineStr">
+        <is>
+          <t>2026年Q1のゲームM&amp;Aは52件・総額77億ドルとメガディール除く過去最高。Savvy Games GroupによるMoonton買収（60億ドル）が牽引し、Scopelyやネクソン等も大型買収を実施した。</t>
+        </is>
+      </c>
+      <c r="F52" s="14" t="inlineStr">
+        <is>
+          <t>・Q1のM&amp;Aは52件で総額77億ドル
+・SavvyがMoontonを60億ドルで取得
+・ScopelyがLoom Gamesを10億ドル
+・NCSoftがJustPlay株70%を2.02億ドル
+・IPO/私募投資は低調が継続</t>
+        </is>
+      </c>
+      <c r="G52" s="14" t="inlineStr">
+        <is>
+          <t>金利や景気の不透明感の下でも、ソブリンマネーと大手プラットフォーマーの資金力を背景に統合は継続。モバイル・ライブサービス領域での買収が引き続き中心になる見込み。</t>
+        </is>
+      </c>
+      <c r="H52" s="14" t="inlineStr">
+        <is>
+          <t>ゲーム業界の資本再編とソブリンファンドの戦略</t>
+        </is>
+      </c>
+      <c r="I52" s="14" t="inlineStr">
+        <is>
+          <t>Savvy Games Group, Moonton, Scopely, NCSoft, Mattel</t>
+        </is>
+      </c>
+      <c r="J52" s="14" t="inlineStr">
+        <is>
+          <t>Mobile Legends: Bang Bang</t>
+        </is>
+      </c>
+      <c r="K52" s="14" t="inlineStr">
+        <is>
+          <t>M&amp;A,海外,業績</t>
+        </is>
+      </c>
+      <c r="L52" s="14" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B53" s="14" t="inlineStr">
+        <is>
+          <t>任天堂2026年3月期、売上2.31兆円で倍増 Switch2が1986万台</t>
+        </is>
+      </c>
+      <c r="C53" s="14" t="inlineStr">
+        <is>
+          <t>https://www.nintendo.co.jp/ir/pdf/2026/260508_4.pdf</t>
+        </is>
+      </c>
+      <c r="D53" s="14" t="inlineStr">
+        <is>
+          <t>2025年に投入したNintendo Switch 2が初年度から好調に推移。新ハード立ち上げ年として、本体販売台数・ソフト本数ともに前モデルの初年実績を上回った。</t>
+        </is>
+      </c>
+      <c r="E53" s="14" t="inlineStr">
+        <is>
+          <t>任天堂の2026年3月期は売上高2兆3130億円（前期比98.6%増）、営業利益3601億円（同27.5%増）。Switch2本体は1986万台、ソフトは4871万本を販売し増収増益を達成した。</t>
+        </is>
+      </c>
+      <c r="F53" s="14" t="inlineStr">
+        <is>
+          <t>・売上高2兆3130億円（+98.6%）
+・営業利益3601億円（+27.5%）
+・純利益4240億円（+52.1%）
+・Switch2本体1986万台
+・ソフト4871万本</t>
+        </is>
+      </c>
+      <c r="G53" s="14" t="inlineStr">
+        <is>
+          <t>ハード普及に伴うソフト・サブスク収益の積み上げが焦点。欧米年末商戦の動向と、5月実施の国内専用機の価格改定が需要に与える影響が次期業績の鍵となる。</t>
+        </is>
+      </c>
+      <c r="H53" s="14" t="inlineStr">
+        <is>
+          <t>新ハード立ち上げ期のハード/ソフト比率と収益構造</t>
+        </is>
+      </c>
+      <c r="I53" s="14" t="inlineStr">
+        <is>
+          <t>任天堂</t>
+        </is>
+      </c>
+      <c r="J53" s="14" t="inlineStr">
+        <is>
+          <t>Nintendo Switch 2</t>
+        </is>
+      </c>
+      <c r="K53" s="14" t="inlineStr">
+        <is>
+          <t>業績,国内</t>
+        </is>
+      </c>
+      <c r="L53" s="14" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B54" s="14" t="inlineStr">
+        <is>
+          <t>ソニーG 2025年度決算、売上12.5兆円・営業益1.45兆円で過去最高</t>
+        </is>
+      </c>
+      <c r="C54" s="14" t="inlineStr">
+        <is>
+          <t>https://xtrend.nikkei.com/atcl/contents/18/01182/00076/</t>
+        </is>
+      </c>
+      <c r="D54" s="14" t="inlineStr">
+        <is>
+          <t>ゲーム&amp;ネットワークサービス（G&amp;NS）を含む各事業が堅調に推移。PS5世代の安定運営とIP・音楽事業の成長が全社業績を押し上げた。</t>
+        </is>
+      </c>
+      <c r="E54" s="14" t="inlineStr">
+        <is>
+          <t>ソニーグループの2025年度（2026年3月期）は売上高12兆4796億円（前期比3.7%増）、営業利益1兆4475億円（同13.4%増）と、いずれも過去最高を更新した。</t>
+        </is>
+      </c>
+      <c r="F54" s="14" t="inlineStr">
+        <is>
+          <t>・売上高12兆4796億円（+3.7%）
+・営業利益1兆4475億円（+13.4%）
+・売上・営業益とも過去最高
+・G&amp;NS含む各事業が貢献
+・PS5は追加値上げを実施</t>
+        </is>
+      </c>
+      <c r="G54" s="14" t="inlineStr">
+        <is>
+          <t>PS5後半サイクルでのソフト・サービス収益の最大化と、値上げによる需要影響の見極めが課題。映画・音楽との横断IP戦略が成長ドライバーとなる見込み。</t>
+        </is>
+      </c>
+      <c r="H54" s="14" t="inlineStr">
+        <is>
+          <t>総合エンタメ企業のIP横断戦略とゲーム事業の位置づけ</t>
+        </is>
+      </c>
+      <c r="I54" s="14" t="inlineStr">
+        <is>
+          <t>ソニーグループ, SIE</t>
+        </is>
+      </c>
+      <c r="J54" s="14" t="inlineStr">
+        <is>
+          <t>PlayStation 5</t>
+        </is>
+      </c>
+      <c r="K54" s="14" t="inlineStr">
+        <is>
+          <t>業績,国内</t>
+        </is>
+      </c>
+      <c r="L54" s="14" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B55" s="14" t="inlineStr">
+        <is>
+          <t>NVIDIA「DLSS 5」、生成AIでゲーム映像のフォトリアリズムを向上</t>
+        </is>
+      </c>
+      <c r="C55" s="14" t="inlineStr">
+        <is>
+          <t>https://techcrunch.com/2026/03/16/nvidias-dlss-5-uses-generative-ai-to-boost-photo-realism-in-video-games-with-ambitions-beyond-gaming/</t>
+        </is>
+      </c>
+      <c r="D55" s="14" t="inlineStr">
+        <is>
+          <t>アップスケーリング技術DLSSの次世代版。従来の解像度補完に加え、生成AIで映像のリアリズムそのものを高める方向に進化し、ゲーム以外への応用も視野に入れる。</t>
+        </is>
+      </c>
+      <c r="E55" s="14" t="inlineStr">
+        <is>
+          <t>NVIDIAは生成AIを用いてゲーム映像のフォトリアリズムを高める「DLSS 5」を発表。従来のフレーム生成・超解像を超え、AIが描画品質を底上げする新世代技術として位置づけられる。</t>
+        </is>
+      </c>
+      <c r="F55" s="14" t="inlineStr">
+        <is>
+          <t>・DLSS 5は生成AIでリアリズム向上
+・従来の超解像/フレーム生成を発展
+・ゲーム外への応用も標榜
+・GPU性能とAIの融合が加速
+・描画パイプラインの再定義</t>
+        </is>
+      </c>
+      <c r="G55" s="14" t="inlineStr">
+        <is>
+          <t>生成AIによるリアルタイム描画補強が標準化すれば、開発側の制作負荷とハード要件の双方に影響。AI描画を前提とした次世代エンジン設計が進む可能性がある。</t>
+        </is>
+      </c>
+      <c r="H55" s="14" t="inlineStr">
+        <is>
+          <t>生成AI×リアルタイムレンダリングの技術潮流</t>
+        </is>
+      </c>
+      <c r="I55" s="14" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="J55" s="14" t="inlineStr">
+        <is>
+          <t>DLSS, GeForce</t>
+        </is>
+      </c>
+      <c r="K55" s="14" t="inlineStr">
+        <is>
+          <t>技術,海外</t>
+        </is>
+      </c>
+      <c r="L55" s="14" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B56" s="14" t="inlineStr">
+        <is>
+          <t>開発者の52%が「生成AIはゲーム業界に悪影響」、懸念が前年から急増</t>
+        </is>
+      </c>
+      <c r="C56" s="14" t="inlineStr">
+        <is>
+          <t>https://theweek.com/culture-life/personal-technology/ai-warping-video-game-industry</t>
+        </is>
+      </c>
+      <c r="D56" s="14" t="inlineStr">
+        <is>
+          <t>生成AIは制作コスト削減への期待がある一方、アーティストや声優の仕事減少・低品質量産への懸念が強い。GDC関連の調査で否定的な見方が前年から大きく増加した。</t>
+        </is>
+      </c>
+      <c r="E56" s="14" t="inlineStr">
+        <is>
+          <t>開発者の52%が生成AIをゲーム業界にネガティブと評価し、前年の30%から急増。コスト削減で最大220億ドルの利益機会との試算もあるが、雇用・品質を巡る不安が拡大している。</t>
+        </is>
+      </c>
+      <c r="F56" s="14" t="inlineStr">
+        <is>
+          <t>・生成AI否定的評価が52%（前年30%）
+・最大220億ドルの利益機会試算（Morgan Stanley）
+・アーティスト/声優の雇用懸念
+・「AIスロップ」量産への不安
+・GDC2026でもAIが主要議題</t>
+        </is>
+      </c>
+      <c r="G56" s="14" t="inlineStr">
+        <is>
+          <t>コスト圧力でAI導入は進む一方、開示ルールや労使交渉、ユーザーの忌避反応が普及ペースを左右。AI活用の是非がブランド価値の論点になる。</t>
+        </is>
+      </c>
+      <c r="H56" s="14" t="inlineStr">
+        <is>
+          <t>生成AI導入の経済効果とクリエイター労働問題</t>
+        </is>
+      </c>
+      <c r="I56" s="14" t="inlineStr">
+        <is>
+          <t>Unity, Morgan Stanley</t>
+        </is>
+      </c>
+      <c r="J56" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K56" s="14" t="inlineStr">
+        <is>
+          <t>技術,海外</t>
+        </is>
+      </c>
+      <c r="L56" s="14" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B57" s="14" t="inlineStr">
+        <is>
+          <t>「スマホ新法」施行でアプリ課金方式が変化、ゲーム収益に影響</t>
+        </is>
+      </c>
+      <c r="C57" s="14" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/999/G999904/20251023051/</t>
+        </is>
+      </c>
+      <c r="D57" s="14" t="inlineStr">
+        <is>
+          <t>日本のスマホソフトウェア競争促進法（スマホ新法）が2025年12月以降に段階適用。アプリストアの課金・決済の在り方に外部決済の選択肢が持ち込まれ、ゲーム課金にも波及する。</t>
+        </is>
+      </c>
+      <c r="E57" s="14" t="inlineStr">
+        <is>
+          <t>スマホ新法により、AppleやGoogleのアプリストアでの課金・決済方式の変更が求められ、外部決済の利用などが可能に。手数料構造やガチャ課金を含むゲーム収益モデルに影響が及ぶ。</t>
+        </is>
+      </c>
+      <c r="F57" s="14" t="inlineStr">
+        <is>
+          <t>・スマホ新法が2025年12月以降適用
+・アプリストアの課金/決済方式が変化
+・外部決済の選択肢が拡大
+・プラットフォーム手数料に影響
+・ガチャ収益モデルにも波及</t>
+        </is>
+      </c>
+      <c r="G57" s="14" t="inlineStr">
+        <is>
+          <t>決済選択肢の拡大はパブリッシャーの取り分改善につながる一方、ストア側の対抗策や規約変更も予想され、当面は実務運用の整備が焦点となる。</t>
+        </is>
+      </c>
+      <c r="H57" s="14" t="inlineStr">
+        <is>
+          <t>スマホ新法とアプリ内課金の規制動向</t>
+        </is>
+      </c>
+      <c r="I57" s="14" t="inlineStr">
+        <is>
+          <t>Apple, Google, モバイルゲーム各社</t>
+        </is>
+      </c>
+      <c r="J57" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K57" s="14" t="inlineStr">
+        <is>
+          <t>規制,国内</t>
+        </is>
+      </c>
+      <c r="L57" s="14" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B58" s="14" t="inlineStr">
+        <is>
+          <t>世界eスポーツ視聴が月33億時間で記録更新、モバイルが牽引</t>
+        </is>
+      </c>
+      <c r="C58" s="14" t="inlineStr">
+        <is>
+          <t>https://escharts.com/news/how-esports-viewership-going-global-2026</t>
+        </is>
+      </c>
+      <c r="D58" s="14" t="inlineStr">
+        <is>
+          <t>スマホ普及とTikTok Live等の新たな配信経路により、従来の配信プラットフォームを超えた観戦層が拡大。アジア太平洋が視聴者の過半を占め、モバイルタイトルが成長を主導している。</t>
+        </is>
+      </c>
+      <c r="E58" s="14" t="inlineStr">
+        <is>
+          <t>2026年5月の世界eスポーツ視聴は33億時間と過去最高。Mobile Legendsのモバイル大会が568万同接の最高記録を出すなど、モバイルeスポーツが市場拡大を牽引している。</t>
+        </is>
+      </c>
+      <c r="F58" s="14" t="inlineStr">
+        <is>
+          <t>・2026年5月の視聴は33億時間で記録更新
+・世界視聴者は6.4億人規模
+・MLBB大会が568万同接の最高記録
+・モバイルが視聴の56%
+・アジア太平洋が視聴者の57%</t>
+        </is>
+      </c>
+      <c r="G58" s="14" t="inlineStr">
+        <is>
+          <t>モバイル・短尺配信中心の観戦行動が定着し、スポンサーや放映権の重心がモバイル大会・新興プラットフォームへ移行。市場規模は2026年に約51億ドルへ拡大の見込み。</t>
+        </is>
+      </c>
+      <c r="H58" s="14" t="inlineStr">
+        <is>
+          <t>モバイルeスポーツの視聴行動と収益化モデル</t>
+        </is>
+      </c>
+      <c r="I58" s="14" t="inlineStr">
+        <is>
+          <t>Moonton, Riot Games, TikTok</t>
+        </is>
+      </c>
+      <c r="J58" s="14" t="inlineStr">
+        <is>
+          <t>Mobile Legends: Bang Bang, League of Legends</t>
+        </is>
+      </c>
+      <c r="K58" s="14" t="inlineStr">
+        <is>
+          <t>eスポーツ,海外</t>
+        </is>
+      </c>
+      <c r="L58" s="14" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B59" s="14" t="inlineStr">
+        <is>
+          <t>Bungie、『Destiny 2』開発終了でレイオフ 6/9に最終アップデート</t>
+        </is>
+      </c>
+      <c r="C59" s="14" t="inlineStr">
+        <is>
+          <t>https://www.metaintro.com/blog/sony-bungie-layoffs-destiny-2-sunset-2026</t>
+        </is>
+      </c>
+      <c r="D59" s="14" t="inlineStr">
+        <is>
+          <t>ソニーが2022年に36億ドルで買収したBungieは、看板ライブサービス『Destiny 2』の継続開発を終了。人員を抽出シューター新作『Marathon』へ振り向ける構造転換の途上にある。</t>
+        </is>
+      </c>
+      <c r="E59" s="14" t="inlineStr">
+        <is>
+          <t>BungieはDestiny 2の開発を終了し6月9日に最終コンテンツ更新を配信、米ベルビュー拠点で大規模レイオフを計画。買収以降も人員削減が続き、残る人材は不振の新作Marathonへ集約される。</t>
+        </is>
+      </c>
+      <c r="F59" s="14" t="inlineStr">
+        <is>
+          <t>・Destiny 2は6/9に最終アップデート
+・ベルビュー拠点で大規模レイオフ計画
+・2022年にソニーが36億ドルで買収
+・人材をMarathonに集約
+・業界全体でレイオフが継続</t>
+        </is>
+      </c>
+      <c r="G59" s="14" t="inlineStr">
+        <is>
+          <t>長寿ライブサービスの収益逓減とAAA投資回収難の構図が鮮明化。Marathonの成否がBungie存続とソニーの自社スタジオ戦略を左右する。</t>
+        </is>
+      </c>
+      <c r="H59" s="14" t="inlineStr">
+        <is>
+          <t>ライブサービスゲームの寿命と大型買収後のスタジオ運営</t>
+        </is>
+      </c>
+      <c r="I59" s="14" t="inlineStr">
+        <is>
+          <t>Bungie, ソニー（SIE）</t>
+        </is>
+      </c>
+      <c r="J59" s="14" t="inlineStr">
+        <is>
+          <t>Destiny 2, Marathon</t>
+        </is>
+      </c>
+      <c r="K59" s="14" t="inlineStr">
+        <is>
+          <t>業績,海外</t>
+        </is>
+      </c>
+      <c r="L59" s="14" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B60" s="14" t="inlineStr">
+        <is>
+          <t>『イナズマイレブン クロス』6月9日配信、新機能「クロスラウンジ」公開</t>
+        </is>
+      </c>
+      <c r="C60" s="14" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/schedule/switch2</t>
+        </is>
+      </c>
+      <c r="D60" s="14" t="inlineStr">
+        <is>
+          <t>レベルファイブの人気サッカーRPGシリーズ最新作。長期の開発・延期を経て配信時期が確定し、オンライン機能やコミュニティ要素を拡充して展開する。</t>
+        </is>
+      </c>
+      <c r="E60" s="14" t="inlineStr">
+        <is>
+          <t>レベルファイブは『イナズマイレブン クロス』を6月9日に配信予定と発表。新機能「クロスラウンジ」など新情報を公開し、長年の主力IPの再起動を図る。</t>
+        </is>
+      </c>
+      <c r="F60" s="14" t="inlineStr">
+        <is>
+          <t>・6月9日配信予定
+・新機能「クロスラウンジ」
+・レベルファイブの主力IP
+・長期開発を経た投入
+・マルチプラットフォーム展開</t>
+        </is>
+      </c>
+      <c r="G60" s="14" t="inlineStr">
+        <is>
+          <t>国内人気IPの復活が成功すれば、関連メディア・グッズ展開や対戦コミュニティの形成につながる可能性。レベルファイブの業績寄与が注目される。</t>
+        </is>
+      </c>
+      <c r="H60" s="14" t="inlineStr">
+        <is>
+          <t>国内IPの再起動とコミュニティ運営</t>
+        </is>
+      </c>
+      <c r="I60" s="14" t="inlineStr">
+        <is>
+          <t>レベルファイブ</t>
+        </is>
+      </c>
+      <c r="J60" s="14" t="inlineStr">
+        <is>
+          <t>イナズマイレブン</t>
+        </is>
+      </c>
+      <c r="K60" s="14" t="inlineStr">
+        <is>
+          <t>新作,国内</t>
+        </is>
+      </c>
+      <c r="L60" s="14" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B61" s="14" t="inlineStr">
+        <is>
+          <t>2026年夏のSteam新作ラッシュ、『サブノーティカ2』『Gothic 1 Remake』など期待作</t>
+        </is>
+      </c>
+      <c r="C61" s="14" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/article/202605/73731</t>
+        </is>
+      </c>
+      <c r="D61" s="14" t="inlineStr">
+        <is>
+          <t>GTA6（11月予定）待ちでAAAの谷間となる夏に、Steamではインディー・中規模の話題作が集中。サバイバル続編やリメイク、アドベンチャーなど多様なジャンルが投入される。</t>
+        </is>
+      </c>
+      <c r="E61" s="14" t="inlineStr">
+        <is>
+          <t>2026年5〜9月にSteamで配信予定の注目新作として『サブノーティカ2』『コーヒートーク トーキョー』『Gothic 1 Remake』（6/5）などが紹介され、インディー・中規模タイトルが活況を呈している。</t>
+        </is>
+      </c>
+      <c r="F61" s="14" t="inlineStr">
+        <is>
+          <t>・夏のSteamは中規模/インディーが活況
+・『Gothic 1 Remake』は6/5発売
+・『サブノーティカ2』の続編
+・『コーヒートーク トーキョー』
+・AAAの谷間を埋める投入設計</t>
+        </is>
+      </c>
+      <c r="G61" s="14" t="inlineStr">
+        <is>
+          <t>AAAの大型空白期はインディー・中規模の露出機会。Steam同接やレビュー評価次第でスマッシュヒットが生まれやすく、配信時期の戦略的分散が進む。</t>
+        </is>
+      </c>
+      <c r="H61" s="14" t="inlineStr">
+        <is>
+          <t>AAA谷間期のインディー/中規模タイトル戦略</t>
+        </is>
+      </c>
+      <c r="I61" s="14" t="inlineStr">
+        <is>
+          <t>Valve, THQ Nordic</t>
+        </is>
+      </c>
+      <c r="J61" s="14" t="inlineStr">
+        <is>
+          <t>Subnautica, Gothic</t>
+        </is>
+      </c>
+      <c r="K61" s="14" t="inlineStr">
+        <is>
+          <t>新作,インディー,海外</t>
+        </is>
+      </c>
+      <c r="L61" s="14" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
weekly-trends + tech update (2026-06-03 03:09)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -1175,7 +1175,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1554,6 +1554,154 @@
       <c r="G10" s="3" t="inlineStr">
         <is>
           <t>https://www.pcgamer.com/games/pc-game-release-dates-may-2026/ , https://gamerant.com/steam-new-games-coming-out-soon-may-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>GDC 2026業界調査が示す構造的疲弊と外注化の常態化</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>GDC 2026のState of the Game Industry調査（2,300人超）が示したのは、過去2年で28%の開発者が職を失い、94%がバーンアウトを経験、良好なメンタルは20%という危機的数値だった。生成AIは52%が『業界に害』と回答し、ビジュアル/技術アート(64%)・デザイン/ナラティブ(63%)で反発が突出。外注（co-development）はGDC史上最高水準に達し、内製大規模チームから外部委託への構造シフトが鮮明になった。学生の74%が将来の就職を不安視。単発のレイオフ報道ではなく、雇用モデルそのものの組み替えが進む点が今週あらためて可視化された。</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>GDC, Informa, 大手パブリッシャー各社, 外注スタジオ</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>背景にはAAA開発費の高騰と金利上昇後の投資縮小がある。固定費の重い内製大規模チームを維持できず、可変費化できる外注・co-devへ移行。AIは人件費圧縮の手段として経営側が推進する一方、制作現場は職の希少化と品質低下を懸念し対立構造が固定化。雇用の不安定化が人材流出と技能断絶を招き、長期の開発力低下リスクを孕む。</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>『正社員を抱える製造業』から『プロジェクト単位の映画製作型』への移行。ギグ化・スタジオ制という他産業と同じ論点で、人材育成と知見蓄積の外部化との両立が次の課題。</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>https://gdconf.com/article/gdc-2026-state-of-the-game-industry-reveals-impact-of-layoffs-generative-ai-and-more/ , https://www.gamedeveloper.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Game Pass値下げとCoD day-one撤回が示すサブスク経済の再設計</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Microsoftは4月にGame Pass Ultimateを$29.99→$22.99、PC Game Passを$13.99へ値下げし、XboxのCEOは『値下げが新規登録と継続率を改善した』と明言した。同時にCall of Dutyの新作day-one提供を取りやめ約1年遅れで追加する方針へ転換。5月にはDiscord Nitro Rewardsに月10時間クラウド付きのGame Pass Starterを組み込むなど入口を多様化。値上げ一辺倒だった近年から一転、価格を下げて母数を取りに行く戦略へ。PC/モバイルとハンドヘルドを取り込み、2027年初頭までに5,000万契約を狙う。</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Microsoft, Xbox, Activision(Call of Duty), Discord</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>サブスクは『ARPU最大化』と『契約者数最大化』のトレードオフ。値上げで離脱が進んだ反省から、目玉IPを敢えてday-one提供せず本体販売とのカニバリを抑えつつ、低価格・他社バンドルで裾野を広げる設計に。クラウドを無料体験の撒き餌に使い、ハードに依存しない収益基盤を作る狙い。</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>動画・音楽サブスクが通った『値下げ＋バンドル＋広告階層』へゲームも合流。プラットフォーム横断のディストリビューション争いが本質。</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>https://respawn.outlookindia.com/gaming/gaming-news/xbox-ceo-says-game-pass-price-cuts-improve-sign-ups-and-retention , https://9to5google.com/2026/04/21/xbox-game-pass-ultimate-price-cut/</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Mixtape炎上とSlay the Spire IIレビュー爆撃：表現を巡る対立の再燃</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>5月、配信されたMixtapeに対し作品の『クィアフレンドリー』な要素を標的とした組織的反発が起き、AftermathのNathan GraysonらはGamergateとの類似を指摘した。同月、Slay the Spire IIはクレジットにAnita Sarkeesianがコンサルタントとして記載されていたことを理由にレビュー爆撃を受けた。いずれも作品の品質ではなく制作者の属性や政治的立場を起点に評価が動員される構図で、Steamのユーザーレビューが文化的紛争の場として機能する現実を改めて示した。一過性の炎上ではなく定期的に再発するパターンとして観測される。</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Mixtape(Beethoven &amp; Dinosaur), Slay the Spire II(Mega Crit), Valve(Steam)</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>レビュースコアが購買とアルゴリズム露出に直結するため、レビュー欄が安価で効果的な政治的圧力手段になっている。プラットフォームは表現の自由とレビュー操作対策の板挟みで、Valveのレビュー爆撃検知は属性起点の動員に十分機能しない。制作者の可視性が上がるほど標的化リスクも上がる非対称性。</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>UGC評価系を持つ全産業（食べログ、Amazon等）共通の『評価の武器化』問題。信頼スコアの設計とモデレーションが鍵に。</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>https://www.thegamer.com/may-biggest-gaming-surprises/ , https://en.wikipedia.org/wiki/Gamergate</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>無料インディーTBHがSteam首位：13万同接が示すディスカバリーの変質</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>6月初週、小規模インディー開発の無料ゲーム『TBH: Task Bar Hero』が13.3万同接を記録し、2位の『007 First Light』に10万近い差をつけてSteamのトレンド首位に立った。広告予算もパブリッシャーの後ろ盾もない無料タイトルが、配信・SNSのバイラルだけで大型AAAを上回る瞬間を作った。同時期にはコージーサバイバル『Solarpunk』が7万フォロワーを集めるなど、価格ゼロ＋話題性で一気に母数を取るパターンが目立つ。無料化はマネタイズ放棄ではなく、注目という最も希少な資源を獲得する入口戦略として機能している。</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>TBH: Task Bar Hero, 007 First Light, Solarpunk, Valve(Steam)</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Steamの発見はウィッシュリストやレビュー数より、同接ピークと配信クリップの瞬間最大風速に左右される構造へ。無料は摩擦ゼロでインストール母数を最大化し、配信映え（クリップ性）が口コミを増幅。後からスキン/DLC/続編で回収する設計。広告ROAS悪化環境で有料獲得よりバイラル設計が合理的に。</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>アプリ・動画と同じ『無料で母数→課金で回収』のアテンション経済。プロダクトの配信映え設計が獲得チャネルそのものになる。</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>https://screenrant.com/steam-june-2026-trending-free-game/ , https://www.gamegrin.com/news/top-19-new-steam-games-this-week-1st7th-of-june-2026</t>
         </is>
       </c>
     </row>
@@ -9995,7 +10143,7 @@
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B2" s="9" t="inlineStr">
@@ -10010,32 +10158,32 @@
       </c>
       <c r="D2" s="9" t="inlineStr">
         <is>
-          <t>NPC会話・アセット生成・QA自動化に加え、内製工程へのAgentic AI導入とプラットフォーム開示制度の整備が同時進行。</t>
+          <t>GDC 2026調査で開発者の52%が生成AIを『業界に害』と回答（ビジュアル/技術アート64%が否定的）。Steamは1月にAI開示を二層化＝プレイヤーが消費するコンテンツと裏方の効率化ツールを区別。</t>
         </is>
       </c>
       <c r="E2" s="9" t="inlineStr">
         <is>
-          <t>2026年1月Steamが開示ルールを改定（効率化ツールは開示不要／出荷生成物は事前・ライブで開示義務）。Larianが初期利用で批判→自粛表明。CapcomがGoogle CloudのAgentic AIを内製導入と公表。Morgan Stanleyは業界で約220億ドルの利益機会と試算。</t>
+          <t>Larianが反発を受けgenAI使用を『控える』と表明、Jurassic World Evolution 3はAI生成ポートレートを撤回。開示済みは7,300本超。</t>
         </is>
       </c>
       <c r="F2" s="9" t="inlineStr">
         <is>
-          <t>Valve, Larian Studios, Capcom, Google Cloud</t>
+          <t>Valve, Larian, Frontier, GDC, 各AAAパブリッシャー</t>
         </is>
       </c>
       <c r="G2" s="9" t="inlineStr">
         <is>
-          <t>『ツール利用』と『生成物出荷』の線引きが各ストア・各国で標準化。開示の粒度と内製効率化が競争・信頼の要因に。</t>
+          <t>ランタイム生成（動的NPC会話）への表示要求・規制が次の焦点。経営の推進と現場の反発の溝は当面埋まらず。</t>
         </is>
       </c>
       <c r="H2" s="9" t="inlineStr">
         <is>
-          <t>論点が『使うか否か』から『何を出荷したか』『どう開示するか』へ移行している。</t>
+          <t>AIは『裏方の効率化』と『プレイヤーが見る成果物』で社会的許容度が分岐。境界設計が論点。</t>
         </is>
       </c>
       <c r="I2" s="9" t="inlineStr">
         <is>
-          <t>https://opencritic.com/news/25847/</t>
+          <t>https://www.pcgamer.com/software/ai/steam-updates-ai-disclosure-form-to-specify-that-its-focused-on-ai-generated-content-that-is-consumed-by-players-not-efficiency-tools-used-behind-the-scenes/</t>
         </is>
       </c>
       <c r="J2" s="9" t="inlineStr"/>
@@ -10043,7 +10191,7 @@
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B3" s="9" t="inlineStr">
@@ -10058,20 +10206,40 @@
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
-          <t>GeForce NOW/xCloud。MS-ABK買収後の動向</t>
-        </is>
-      </c>
-      <c r="E3" s="9" t="inlineStr"/>
-      <c r="F3" s="9" t="inlineStr"/>
-      <c r="G3" s="9" t="inlineStr"/>
-      <c r="H3" s="9" t="inlineStr"/>
-      <c r="I3" s="9" t="inlineStr"/>
+          <t>MicrosoftがGame Pass Ultimate（クラウド込み）を$29.99→$22.99へ値下げ。Discord Nitroに月10時間クラウド付きStarterを同梱。市場は2026年に約283億ドル規模との予測。</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>クラウドを無料/低価格の入口（撒き餌）に位置づけ、ハード非依存の獲得チャネル化が進む。</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="inlineStr">
+        <is>
+          <t>Microsoft, Xbox, Discord</t>
+        </is>
+      </c>
+      <c r="G3" s="9" t="inlineStr">
+        <is>
+          <t>広告階層・他社バンドル経由のクラウド配布が拡大。ハンドヘルド連携が次の戦場。</t>
+        </is>
+      </c>
+      <c r="H3" s="9" t="inlineStr">
+        <is>
+          <t>クラウドは単独事業より『サブスク/バンドルの付加価値』として普及する経路が現実的。</t>
+        </is>
+      </c>
+      <c r="I3" s="9" t="inlineStr">
+        <is>
+          <t>https://9to5google.com/2026/04/21/xbox-game-pass-ultimate-price-cut/</t>
+        </is>
+      </c>
       <c r="J3" s="9" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B4" s="9" t="inlineStr">
@@ -10086,14 +10254,34 @@
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>Xbox Game Pass/PS+/Apple Arcade</t>
-        </is>
-      </c>
-      <c r="E4" s="9" t="inlineStr"/>
-      <c r="F4" s="9" t="inlineStr"/>
-      <c r="G4" s="9" t="inlineStr"/>
-      <c r="H4" s="9" t="inlineStr"/>
-      <c r="I4" s="9" t="inlineStr"/>
+          <t>Game Pass Ultimate $22.99/PC $13.99へ値下げ。CEOは登録・継続率の改善を明言。CoD新作のday-one提供を撤回し約1年遅れに。</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>Discord Nitro Rewardsへ50本超のStarter同梱。PC/Premium統合や広告階層を2027年視野で検討。目標5,000万契約。</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>Microsoft, Xbox, Activision, Discord</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>値下げ＋バンドル＋広告階層へ。目玉IPはday-one非提供で本体販売とのカニバリ回避。</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>ARPU最大化から契約者数最大化へ軸足。動画/音楽サブスクの定石に合流。</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>https://respawn.outlookindia.com/gaming/gaming-news/xbox-ceo-says-game-pass-price-cuts-improve-sign-ups-and-retention</t>
+        </is>
+      </c>
       <c r="J4" s="9" t="inlineStr"/>
     </row>
     <row r="5">
@@ -10287,7 +10475,7 @@
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
@@ -10302,32 +10490,32 @@
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>大型新作とアーリーアクセスが牽引し、5月は13本級が集中する豊作月。</t>
+          <t>無料インディー『TBH: Task Bar Hero』が13.3万同接でトレンド首位、AAAの007 First Lightを圧倒。AI開示済みは7,300本超。</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>Forza Horizon 6がSteam同接30万超でXbox Game Studios歴代最高。007 First Light・Subnautica 2(EA)等が集中。Path of Exile 2が5/30よりフリーウィークエンド実施。</t>
+          <t>広告/パブリッシャー無しの無料タイトルがバイラルのみで首位。Solarpunk等コージー作も高フォロワー、Gothic 1 Remakeが6月最多ウィッシュリスト。</t>
         </is>
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t>Valve, Microsoft, IO Interactive, Unknown Worlds, Grinding Gear Games</t>
+          <t>Valve, インディー各社</t>
         </is>
       </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
-          <t>PCが同時発売(デイワン)の主戦場として比重を拡大。アーリーアクセス＆フリーウィークエンドによる獲得施策が定着。</t>
+          <t>同接ピークと配信クリップ起点のディスカバリーが主流化。無料→DLC/続編回収の設計が増加。</t>
         </is>
       </c>
       <c r="H11" s="9" t="inlineStr">
         <is>
-          <t>5月の山の後、GTA6(11/19予定)まで谷が予想され、話題と売上が偏る。</t>
+          <t>PCの発見はウィッシュリストより『瞬間最大同接×配信映え』へ重心移動。</t>
         </is>
       </c>
       <c r="I11" s="9" t="inlineStr">
         <is>
-          <t>https://www.pcgamer.com/games/pc-game-release-dates-may-2026/</t>
+          <t>https://screenrant.com/steam-june-2026-trending-free-game/</t>
         </is>
       </c>
       <c r="J11" s="9" t="inlineStr"/>

</xml_diff>

<commit_message>
daily-news + cross-questions update (2026-06-04) (2026-06-03 23:20)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -29,7 +29,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -73,6 +73,10 @@
     <font>
       <name val="Yu Gothic"/>
     </font>
+    <font>
+      <name val="Yu Gothic"/>
+      <sz val="11"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -113,7 +117,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -145,6 +149,9 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2470,7 +2477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2926,6 +2933,80 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="inlineStr">
+        <is>
+          <t>ゲーム/ギャンブル業界で露呈したAI戦略と統治の27ポイント乖離は、金融・保険など他の規制業界でも同様に起きるか？</t>
+        </is>
+      </c>
+      <c r="C13" s="15" t="inlineStr">
+        <is>
+          <t>UNLV×KPMG『State of AI in Gaming 2026』(AI戦略とガバナンスに27pt乖離)</t>
+        </is>
+      </c>
+      <c r="D13" s="15" t="inlineStr">
+        <is>
+          <t>KPMG,UNLV</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>金融,保険,医療（AI導入が先行し統治・監督が後追いになる規制業界全般）</t>
+        </is>
+      </c>
+      <c r="F13" s="15" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="G13" s="15" t="inlineStr">
+        <is>
+          <t>『戦略は先行、ガバナンスは後追い』はAI導入業界の共通パターンの可能性。規制当局側の監督能力ギャップが共通ボトルネック。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B14" s="15" t="inlineStr">
+        <is>
+          <t>ゲーム/eスポーツ起点の未成年保護規制（16歳未満の利用制限・年齢確認義務）は、SNS・動画配信・広告業界の年齢ゲートにも波及するか？</t>
+        </is>
+      </c>
+      <c r="C14" s="15" t="inlineStr">
+        <is>
+          <t>インドネシアPP TUNAS規制でTikTokが16歳未満170万アカウント停止、モバイルeスポーツに影響</t>
+        </is>
+      </c>
+      <c r="D14" s="15" t="inlineStr">
+        <is>
+          <t>TikTok,Moonton,Garena</t>
+        </is>
+      </c>
+      <c r="E14" s="15" t="inlineStr">
+        <is>
+          <t>SNS,動画配信,広告,通信（年齢確認義務化と未成年課金規制）</t>
+        </is>
+      </c>
+      <c r="F14" s="15" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="G14" s="15" t="inlineStr">
+        <is>
+          <t>未成年保護は『ゲーム規制』として始まり、年齢確認インフラを通じてプラットフォーム横断の共通規制に発展しやすい。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2937,7 +3018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L61"/>
+  <dimension ref="A1:L71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6781,6 +6862,656 @@
         </is>
       </c>
       <c r="L61" s="14" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B62" s="15" t="inlineStr">
+        <is>
+          <t>State of Play June 2026、新生『ゴッド・オブ・ウォー』とウルヴァリンを一挙公開</t>
+        </is>
+      </c>
+      <c r="C62" s="15" t="inlineStr">
+        <is>
+          <t>https://blog.playstation.com/2026/06/02/state-of-play-june-2026-all-announcements-trailers/</t>
+        </is>
+      </c>
+      <c r="D62" s="15" t="inlineStr">
+        <is>
+          <t>SIEはSummer Game Fest直前の6月2日に約60分のState of Playを配信。サマーゲームショー商戦の口火を切り、PS5向けファースト/サードパーティ作品を集中投下した。</t>
+        </is>
+      </c>
+      <c r="E62" s="15" t="inlineStr">
+        <is>
+          <t>クレイトス不在でFaye（ロウフェイ）を主役に据えた新生『ゴッド・オブ・ウォー LAUFEY』を初公開。『Marvel's Wolverine』(9/15)、『鬼武者 Way of the Sword』(9/25)、Firesprite開発『Until Dawn 2』、『Control Resonant』(8/27)などを発表した。</t>
+        </is>
+      </c>
+      <c r="F62" s="15" t="inlineStr">
+        <is>
+          <t>新生GoWはKratos以外を主役にしたシリーズ初の方向転換
+Wolverineは9/15発売でより高速・暴力的な戦闘へ刷新
+Until Dawn 2は新キャストの独立作
+夏商戦の主導権をSGF前に確保する狙い</t>
+        </is>
+      </c>
+      <c r="G62" s="15" t="inlineStr">
+        <is>
+          <t>9月にWolverine・鬼武者・Onimushaなど大型ソフトが集中し、年末商戦前の山場となる見込み。SGFやXbox Showcaseと合わせPS5後期のラインナップ確度が一段と高まる。</t>
+        </is>
+      </c>
+      <c r="H62" s="15" t="inlineStr">
+        <is>
+          <t>プラットフォーマーのショーケース戦略とリリース集中の功罪</t>
+        </is>
+      </c>
+      <c r="I62" s="15" t="inlineStr">
+        <is>
+          <t>ソニー,SIE,Santa Monica Studio,Firesprite,Insomniac Games</t>
+        </is>
+      </c>
+      <c r="J62" s="15" t="inlineStr">
+        <is>
+          <t>God of War,Marvel's Wolverine,Until Dawn,Control</t>
+        </is>
+      </c>
+      <c r="K62" s="15" t="inlineStr">
+        <is>
+          <t>新作,海外</t>
+        </is>
+      </c>
+      <c r="L62" s="15" t="inlineStr">
+        <is>
+          <t>SGF直前の集中投下</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B63" s="15" t="inlineStr">
+        <is>
+          <t>カプコン『鬼武者 Way of the Sword』9/25発売決定、6/3に体験版配信開始</t>
+        </is>
+      </c>
+      <c r="C63" s="15" t="inlineStr">
+        <is>
+          <t>https://www.capcom.co.jp/ir/english/news/html/e260603.html</t>
+        </is>
+      </c>
+      <c r="D63" s="15" t="inlineStr">
+        <is>
+          <t>シリーズ最新作は約20年ぶりのナンバリング級新作。State of Playでの発表に合わせ、カプコンがIRリリースとして発売日と体験版を正式告知した。</t>
+        </is>
+      </c>
+      <c r="E63" s="15" t="inlineStr">
+        <is>
+          <t>宮本武蔵を主人公に江戸初期の京都を舞台にした和風ダークファンタジー『鬼武者 Way of the Sword』を2026年9月25日に発売すると発表。PS5/Xbox Series/PC（Steam・Epic）向けで、6月3日には体験版『Onimusha: Way of the Sword DEMO』を配信開始した。</t>
+        </is>
+      </c>
+      <c r="F63" s="15" t="inlineStr">
+        <is>
+          <t>約20年ぶりの本格新作で旧来IPの再起動
+主人公は宮本武蔵、舞台は呪われた江戸期の京
+マルチプラットフォーム同時展開
+体験版先行配信で発売前の話題を醸成</t>
+        </is>
+      </c>
+      <c r="G63" s="15" t="inlineStr">
+        <is>
+          <t>9月に複数大作が集中する中、カプコンは『モンハンワイルズ』に続く新規/復活IPの収益柱化を狙う。体験版のユーザー反応が初週本数と評価形成の試金石となる。</t>
+        </is>
+      </c>
+      <c r="H63" s="15" t="inlineStr">
+        <is>
+          <t>休眠IPの再起動戦略と体験版マーケティング</t>
+        </is>
+      </c>
+      <c r="I63" s="15" t="inlineStr">
+        <is>
+          <t>カプコン</t>
+        </is>
+      </c>
+      <c r="J63" s="15" t="inlineStr">
+        <is>
+          <t>鬼武者,Onimusha</t>
+        </is>
+      </c>
+      <c r="K63" s="15" t="inlineStr">
+        <is>
+          <t>新作,業績,国内</t>
+        </is>
+      </c>
+      <c r="L63" s="15" t="inlineStr">
+        <is>
+          <t>IRリリース／適時開示連動</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B64" s="15" t="inlineStr">
+        <is>
+          <t>スクエニ『FF7 リバース』Switch 2・Xbox版を6/3発売、早期購入20%オフ</t>
+        </is>
+      </c>
+      <c r="C64" s="15" t="inlineStr">
+        <is>
+          <t>https://press.na.square-enix.com/FINAL-FANTASY-VII-REBIRTH-AVAILABLE-NOW-ON-NINTENDO-SWITCH-2-AND-XBOX-</t>
+        </is>
+      </c>
+      <c r="D64" s="15" t="inlineStr">
+        <is>
+          <t>PS5独占だったリメイク3部作の第2作を、発売から約2年を経て他プラットフォームへ展開。Switch 2・Xbox陣営のソフト拡充の一環でもある。</t>
+        </is>
+      </c>
+      <c r="E64" s="15" t="inlineStr">
+        <is>
+          <t>スクウェア・エニックスは6月3日、『FINAL FANTASY VII REBIRTH』のNintendo Switch 2・Xbox Series X|S・Windows版を発売。6月10日まで20%の早期購入割引を実施。標準版は49.99ドル。Switch 2版のMetacriticは86（PS5版は92）。</t>
+        </is>
+      </c>
+      <c r="F64" s="15" t="inlineStr">
+        <is>
+          <t>PS5独占から約2年でマルチ展開へ
+Switch 2のローンチ期ソフト拡充に寄与
+早期購入20%オフで初動を後押し
+Switch 2版スコアはPS5版を下回る86</t>
+        </is>
+      </c>
+      <c r="G64" s="15" t="inlineStr">
+        <is>
+          <t>リメイク3部作完結編の制作と並行し、過去作のマルチ展開で投資回収を最大化する戦略が続く見込み。Switch 2が大型RPGの新たな販売チャネルになるか注目。</t>
+        </is>
+      </c>
+      <c r="H64" s="15" t="inlineStr">
+        <is>
+          <t>独占解除によるIP収益の長期最大化</t>
+        </is>
+      </c>
+      <c r="I64" s="15" t="inlineStr">
+        <is>
+          <t>スクウェア・エニックス,任天堂,マイクロソフト</t>
+        </is>
+      </c>
+      <c r="J64" s="15" t="inlineStr">
+        <is>
+          <t>ファイナルファンタジーVII,FF7 Rebirth</t>
+        </is>
+      </c>
+      <c r="K64" s="15" t="inlineStr">
+        <is>
+          <t>新作,国内</t>
+        </is>
+      </c>
+      <c r="L64" s="15" t="inlineStr">
+        <is>
+          <t>Switch 2/Xbox同時</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B65" s="15" t="inlineStr">
+        <is>
+          <t>ゲーム業界ビジネスイベント『GAME FUTURE SUMMIT 2026』6/3渋谷で開催</t>
+        </is>
+      </c>
+      <c r="C65" s="15" t="inlineStr">
+        <is>
+          <t>https://www.gamebusiness.jp/</t>
+        </is>
+      </c>
+      <c r="D65" s="15" t="inlineStr">
+        <is>
+          <t>ゲーム産業のB2Bカンファレンスとして3回目。開発・運営・投資・人材など産業横断のテーマを扱い、業界の事業課題を議論する場として定着しつつある。</t>
+        </is>
+      </c>
+      <c r="E65" s="15" t="inlineStr">
+        <is>
+          <t>ゲーム業界向けビジネスイベント『GAME FUTURE SUMMIT 2026』が6月3日にベルサール渋谷ガーデンで開催。スポンサーは前回の27社から42社へ拡大し、登壇者は70名超。AI・開発効率化・グローバル展開・人材確保などが主要テーマとなった。</t>
+        </is>
+      </c>
+      <c r="F65" s="15" t="inlineStr">
+        <is>
+          <t>スポンサー27→42社、登壇70名超と規模拡大
+開発効率化・AI活用が中心議題
+産業横断のB2B交流の場として定着
+人材・採用課題も主要テーマ</t>
+        </is>
+      </c>
+      <c r="G65" s="15" t="inlineStr">
+        <is>
+          <t>国内ゲーム産業のビジネスカンファレンスは規模を拡大し、海外GDC的な位置づけへ成長する可能性。AI導入と人材確保が今後の継続論点になる。</t>
+        </is>
+      </c>
+      <c r="H65" s="15" t="inlineStr">
+        <is>
+          <t>国内ゲーム産業のB2Bエコシステム形成</t>
+        </is>
+      </c>
+      <c r="I65" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J65" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K65" s="15" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="L65" s="15" t="inlineStr">
+        <is>
+          <t>業界カンファレンス</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B66" s="15" t="inlineStr">
+        <is>
+          <t>Xbox、6/7に『Games Showcase』と『Gears of War: E-Day Direct』を連続配信予告</t>
+        </is>
+      </c>
+      <c r="C66" s="15" t="inlineStr">
+        <is>
+          <t>https://news.xbox.com/en-us/2026/06/01/xbox-games-showcase-2026-gears-of-war-e-day-direct-how-to-watch/</t>
+        </is>
+      </c>
+      <c r="D66" s="15" t="inlineStr">
+        <is>
+          <t>Xbox 25周年の節目に行われる大型ショーケース。Summer Game Festウィークに合わせ、ファースト/サードのラインナップを世界40言語以上で配信する。</t>
+        </is>
+      </c>
+      <c r="E66" s="15" t="inlineStr">
+        <is>
+          <t>マイクロソフトは6月7日（米太平洋時間10時）にXbox Games Showcaseを配信し、続けてThe Coalition開発の前日譚『Gears of War: E-Day』のDirectを実施すると告知。世界初公開や新規ゲームプレイ、手話・音声解説対応など包括配信を予告した。</t>
+        </is>
+      </c>
+      <c r="F66" s="15" t="inlineStr">
+        <is>
+          <t>Xbox 25周年記念の大型ショーケース
+Gears of War: E-Dayの深掘りDirectを連続実施
+世界40言語以上＋アクセシビリティ対応
+SGFウィークの目玉の一つ</t>
+        </is>
+      </c>
+      <c r="G66" s="15" t="inlineStr">
+        <is>
+          <t>Gears新作の発売時期や規模感が明らかになれば、Xbox陣営のソフト供給不安に対する市場の見方が変わる可能性。マルチ展開方針の言及も注目点。</t>
+        </is>
+      </c>
+      <c r="H66" s="15" t="inlineStr">
+        <is>
+          <t>プラットフォーマーの周年マーケと旗艦IP戦略</t>
+        </is>
+      </c>
+      <c r="I66" s="15" t="inlineStr">
+        <is>
+          <t>マイクロソフト,The Coalition</t>
+        </is>
+      </c>
+      <c r="J66" s="15" t="inlineStr">
+        <is>
+          <t>Gears of War,Gears of War: E-Day</t>
+        </is>
+      </c>
+      <c r="K66" s="15" t="inlineStr">
+        <is>
+          <t>新作,海外</t>
+        </is>
+      </c>
+      <c r="L66" s="15" t="inlineStr">
+        <is>
+          <t>6/7配信予告</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B67" s="15" t="inlineStr">
+        <is>
+          <t>『Summer Game Fest 2026』6/5にロサンゼルスで開幕、インディー60本超も披露</t>
+        </is>
+      </c>
+      <c r="C67" s="15" t="inlineStr">
+        <is>
+          <t>https://www.summergamefest.com/</t>
+        </is>
+      </c>
+      <c r="D67" s="15" t="inlineStr">
+        <is>
+          <t>Geoff Keighley主宰の夏商戦の中核イベント。各社ショーケースのハブとして、世界同時に新作発表が集中する数日間となる。</t>
+        </is>
+      </c>
+      <c r="E67" s="15" t="inlineStr">
+        <is>
+          <t>Summer Game Fest 2026の本編が6月5日（米太平洋14時）にDolby Theatreで開催。Geoff KeighleyとLucy Jamesが司会し、約2時間でワールドプレミアやゲームプレイ公開を実施。60本超のインディータイトルのショーケースも併催される。</t>
+        </is>
+      </c>
+      <c r="F67" s="15" t="inlineStr">
+        <is>
+          <t>6/5本編は約2時間でワールドプレミア中心
+60本超のインディー作品も併催
+各社ショーケースのハブイベント
+6/5〜6/8の4日間にわたり展開</t>
+        </is>
+      </c>
+      <c r="G67" s="15" t="inlineStr">
+        <is>
+          <t>PS State of Play・Xbox Showcaseと合わせ、6月前半に年内〜来年の新作情報が集中。発表内容次第で各社の株価・話題度に短期的影響が出やすい。</t>
+        </is>
+      </c>
+      <c r="H67" s="15" t="inlineStr">
+        <is>
+          <t>サマー商戦のショーケース集積効果</t>
+        </is>
+      </c>
+      <c r="I67" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J67" s="15" t="inlineStr">
+        <is>
+          <t>Summer Game Fest</t>
+        </is>
+      </c>
+      <c r="K67" s="15" t="inlineStr">
+        <is>
+          <t>新作,インディー,海外</t>
+        </is>
+      </c>
+      <c r="L67" s="15" t="inlineStr">
+        <is>
+          <t>6/5開幕</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B68" s="15" t="inlineStr">
+        <is>
+          <t>中国NPPA、5月に国内外158本のゲームを承認、2026年は前年比19%増ペース</t>
+        </is>
+      </c>
+      <c r="C68" s="15" t="inlineStr">
+        <is>
+          <t>https://substack.nikopartners.com/p/chinas-nppa-approves-158-video-games</t>
+        </is>
+      </c>
+      <c r="D68" s="15" t="inlineStr">
+        <is>
+          <t>中国では版号（ISBN）取得がゲーム配信の前提。承認本数の推移は当局の規制スタンスと市場開放度を映す指標として注視される。</t>
+        </is>
+      </c>
+      <c r="E68" s="15" t="inlineStr">
+        <is>
+          <t>中国のNPPAは5月26日、国内154本・輸入4本の計158本に版号を発給。2026年通年では2,300本超の承認が見込まれ、前年比19%増のペース。Tencent・NetEase・37 Interactive・Lilith・ByteDance等の新作が含まれた。</t>
+        </is>
+      </c>
+      <c r="F68" s="15" t="inlineStr">
+        <is>
+          <t>国内154＋輸入4の計158本を承認
+2026年は前年比+19%の承認ペース
+Tencent・NetEaseの新作も含む
+モバイル中心（国内135本がモバイル）</t>
+        </is>
+      </c>
+      <c r="G68" s="15" t="inlineStr">
+        <is>
+          <t>承認ペース加速が続けば中国市場の供給と各社の中国収益見通しが改善。輸入枠の動向次第で海外大手の中国展開余地も広がる可能性。</t>
+        </is>
+      </c>
+      <c r="H68" s="15" t="inlineStr">
+        <is>
+          <t>中国版号制度と市場開放度の読み解き</t>
+        </is>
+      </c>
+      <c r="I68" s="15" t="inlineStr">
+        <is>
+          <t>Tencent,NetEase,37 Interactive,Lilith Games,ByteDance</t>
+        </is>
+      </c>
+      <c r="J68" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K68" s="15" t="inlineStr">
+        <is>
+          <t>規制,海外</t>
+        </is>
+      </c>
+      <c r="L68" s="15" t="inlineStr">
+        <is>
+          <t>5/26発給分</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B69" s="15" t="inlineStr">
+        <is>
+          <t>UNLV×KPMG『State of AI in Gaming 2026』、AI戦略とガバナンスに27ポイントの乖離</t>
+        </is>
+      </c>
+      <c r="C69" s="15" t="inlineStr">
+        <is>
+          <t>https://www.newswise.com/articles/inaugural-state-of-ai-in-gaming-report-establishes-benchmark-for-ai-practice-and-policy-across-the-global-gambling-industry</t>
+        </is>
+      </c>
+      <c r="D69" s="15" t="inlineStr">
+        <is>
+          <t>ゲーム/ギャンブル業界へのAI導入が加速する一方、安全性・統治の整備が追いついていないとの問題意識から、初のベンチマーク調査が実施された。</t>
+        </is>
+      </c>
+      <c r="E69" s="15" t="inlineStr">
+        <is>
+          <t>UNLV国際ゲーミング研究所とKPMGが初の『State of AI in Gaming 2026』を公表。83社・113規制当局を調査し、企業のAI戦略とガバナンスに27ポイントの乖離があると指摘。ディープフェイクを筆頭にAI関連インシデントが2023年以降急増、責任あるAI慣行を持つ企業は70%にとどまる。</t>
+        </is>
+      </c>
+      <c r="F69" s="15" t="inlineStr">
+        <is>
+          <t>AI戦略と統治に27ポイントのギャップ
+ディープフェイクが最多のインシデント類型
+責任あるAI慣行の整備は7割止まり
+規制当局はライセンシーのAI利用把握に不安</t>
+        </is>
+      </c>
+      <c r="G69" s="15" t="inlineStr">
+        <is>
+          <t>業界のAI導入が先行する一方でガバナンス整備が遅れ、規制当局による監督枠組みの整備圧力が強まる見込み。コンプライアンスコストが新たな競争要因になる。</t>
+        </is>
+      </c>
+      <c r="H69" s="15" t="inlineStr">
+        <is>
+          <t>AIガバナンスと規制当局の監督フレーム</t>
+        </is>
+      </c>
+      <c r="I69" s="15" t="inlineStr">
+        <is>
+          <t>KPMG,UNLV</t>
+        </is>
+      </c>
+      <c r="J69" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K69" s="15" t="inlineStr">
+        <is>
+          <t>技術,規制,海外</t>
+        </is>
+      </c>
+      <c r="L69" s="15" t="inlineStr">
+        <is>
+          <t>初のベンチマーク調査</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B70" s="15" t="inlineStr">
+        <is>
+          <t>Bragg Gaming、ゲーム技術企業Drayton International買収で拘束的合意</t>
+        </is>
+      </c>
+      <c r="C70" s="15" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/0001867834/000110465926066323/tm2614911d1_ex99-4.htm</t>
+        </is>
+      </c>
+      <c r="D70" s="15" t="inlineStr">
+        <is>
+          <t>ゲーム業界のM&amp;Aは買収倍率が10倍売上から1.5〜3倍へ低下する調整局面。その中でB2Bゲーミング技術領域では選別的な統合が続いている。</t>
+        </is>
+      </c>
+      <c r="E70" s="15" t="inlineStr">
+        <is>
+          <t>Bragg Gaming Groupは5月14日、多様なゲーミング技術・コンテンツ基盤を持つDrayton Internationalの買収で拘束的タームシートを締結したと開示。正式契約と公表は6月15日までを予定する。コンテンツ配信基盤の強化が狙い。</t>
+        </is>
+      </c>
+      <c r="F70" s="15" t="inlineStr">
+        <is>
+          <t>拘束的タームシートで買収条件に合意
+正式契約・公表は6/15までを予定
+対象はゲーミング技術/コンテンツ基盤
+業界の買収倍率低下局面での選別的M&amp;A</t>
+        </is>
+      </c>
+      <c r="G70" s="15" t="inlineStr">
+        <is>
+          <t>コンテンツ・配信プラットフォーム領域では引き続き再編が進む見込み。倍率低下で買い手有利の環境が続き、B2Bゲーミング技術の集約が加速する可能性。</t>
+        </is>
+      </c>
+      <c r="H70" s="15" t="inlineStr">
+        <is>
+          <t>B2Bゲーミング技術のM&amp;Aと評価倍率</t>
+        </is>
+      </c>
+      <c r="I70" s="15" t="inlineStr">
+        <is>
+          <t>Bragg Gaming Group,Drayton International</t>
+        </is>
+      </c>
+      <c r="J70" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K70" s="15" t="inlineStr">
+        <is>
+          <t>M&amp;A,海外</t>
+        </is>
+      </c>
+      <c r="L70" s="15" t="inlineStr">
+        <is>
+          <t>6/15に正式契約予定</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B71" s="15" t="inlineStr">
+        <is>
+          <t>インドネシアの未成年保護規制PP TUNASでMLBB視聴が最大14%減の試算、eスポーツに波及</t>
+        </is>
+      </c>
+      <c r="C71" s="15" t="inlineStr">
+        <is>
+          <t>https://escharts.com/news/indonesias-under-16-social-media-ban-could-cut-viewership-select-esports-titles-14</t>
+        </is>
+      </c>
+      <c r="D71" s="15" t="inlineStr">
+        <is>
+          <t>インドネシアは3月28日施行のPP TUNAS（児童保護のための電子システム規律）で16歳未満のSNS利用を制限。プラットフォーム各社が対応を迫られ、ゲーム/eスポーツ市場にも波及している。</t>
+        </is>
+      </c>
+      <c r="E71" s="15" t="inlineStr">
+        <is>
+          <t>PP TUNAS対応でTikTokは16歳未満の約170万アカウントを停止（4/10の78万から4/28に170万へ急増）。Esports ChartsはMLBBの視聴が最大14%減と試算し、Free FireやPUBG Mobileを含む主要モバイルタイトルのエンゲージメント低下を招いている。</t>
+        </is>
+      </c>
+      <c r="F71" s="15" t="inlineStr">
+        <is>
+          <t>16歳未満170万アカウントが停止対象
+MLBB視聴は最大14%減との試算
+Free Fire/PUBG Mobileにも影響
+東南アジア最大級市場での構造変化</t>
+        </is>
+      </c>
+      <c r="G71" s="15" t="inlineStr">
+        <is>
+          <t>未成年保護規制は他アジア諸国にも波及し得る。年齢確認・課金制限がモバイルゲーム/eスポーツ事業の前提条件となり、地域別の規制対応力が競争差につながる。</t>
+        </is>
+      </c>
+      <c r="H71" s="15" t="inlineStr">
+        <is>
+          <t>未成年保護規制とモバイルeスポーツ経済圏</t>
+        </is>
+      </c>
+      <c r="I71" s="15" t="inlineStr">
+        <is>
+          <t>TikTok,Moonton,Garena</t>
+        </is>
+      </c>
+      <c r="J71" s="15" t="inlineStr">
+        <is>
+          <t>Mobile Legends,Free Fire,PUBG Mobile</t>
+        </is>
+      </c>
+      <c r="K71" s="15" t="inlineStr">
+        <is>
+          <t>規制,eスポーツ,海外</t>
+        </is>
+      </c>
+      <c r="L71" s="15" t="inlineStr">
+        <is>
+          <t>PP TUNAS（3/28施行）</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
daily-news + cross-questions update (2026-06-04 22:10)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -2477,7 +2477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3007,6 +3007,43 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B15" s="15" t="inlineStr">
+        <is>
+          <t>「20人で10億ドルEXIT」に象徴される超少人数・高生産性モデルは、SaaS・AIスタートアップなど他業界の人員効率トレンドと同型か？</t>
+        </is>
+      </c>
+      <c r="C15" s="15" t="inlineStr">
+        <is>
+          <t>ScopelyによるLoom Games（約20人）の10億ドル超買収と、業界の『最高収益×最大レイオフ』パラドックス</t>
+        </is>
+      </c>
+      <c r="D15" s="15" t="inlineStr">
+        <is>
+          <t>Scopely,Loom Games</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>SaaS,AIスタートアップ,広告制作,メディア（AIで1人当たり付加価値が上昇し、雇用総量が伸びにくい産業全般）</t>
+        </is>
+      </c>
+      <c r="F15" s="15" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="G15" s="15" t="inlineStr">
+        <is>
+          <t>『規模＝価値』から『1人当たり生産性＝価値』への評価軸転換。AI普及で各業界が採用を絞り込み、雇用なき成長が常態化する可能性。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3018,7 +3055,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L71"/>
+  <dimension ref="A1:L76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7510,6 +7547,334 @@
       <c r="L71" s="15" t="inlineStr">
         <is>
           <t>PP TUNAS（3/28施行）</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B72" s="15" t="inlineStr">
+        <is>
+          <t>E3後継の祭典「Summer Game Fest 2026」開幕、6/5にOpening Night Liveを生配信</t>
+        </is>
+      </c>
+      <c r="C72" s="15" t="inlineStr">
+        <is>
+          <t>https://www.gamesradar.com/summer-game-fest-schedule-2026/</t>
+        </is>
+      </c>
+      <c r="D72" s="15" t="inlineStr">
+        <is>
+          <t>E3が2023年に終了して以降、Geoff Keighley主催のSummer Game Fest（SGF）がゲーム発表シーズンの中核イベントに定着。State of PlayやXbox Games Showcaseと連動し、6月初旬に各社の新情報が集中する「ショーケース週間」が業界の年間カレンダーに組み込まれている。</t>
+        </is>
+      </c>
+      <c r="E72" s="15" t="inlineStr">
+        <is>
+          <t>米時間6月5日午後2時（PT）、ロサンゼルスのDolby TheatreからメインショーのOpening Night Liveを生配信。Geoff KeighleyとLucy Jamesが司会を務め、全プラットフォーム横断の新作発表やサプライズゲストを予定。約2時間の本編後にDay of the Devsやインディー系配信が週末まで連続開催される。</t>
+        </is>
+      </c>
+      <c r="F72" s="15" t="inlineStr">
+        <is>
+          <t>6/5（米時間14時PT）にDolby Theatreから約2時間生配信
+YouTube・Twitch・各種コストリームで視聴可能
+E3終了後のゲーム発表シーズンの中核イベント
+State of Play・Xbox Games Showcase（6/7）と連動した「ショーケース週間」
+Day of the Devs等インディー系配信も併催</t>
+        </is>
+      </c>
+      <c r="G72" s="15" t="inlineStr">
+        <is>
+          <t>大手の単独配信（State of Play/Xbox）とSGFの役割分担が定着し、各社は発表をこの時期に集中させてウィッシュリスト獲得とSNS拡散を最大化する。E3不在を埋める「分散型ショーケース」モデルが今後も標準化し、配信クリップの瞬間風速が話題量を左右する構造が強まる見込み。</t>
+        </is>
+      </c>
+      <c r="H72" s="15" t="inlineStr">
+        <is>
+          <t>E3後の分散型ショーケース経済と発表タイミング戦略</t>
+        </is>
+      </c>
+      <c r="I72" s="15" t="inlineStr">
+        <is>
+          <t>Summer Game Fest,Sony,Microsoft,各パブリッシャー</t>
+        </is>
+      </c>
+      <c r="J72" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K72" s="15" t="inlineStr">
+        <is>
+          <t>新作,海外</t>
+        </is>
+      </c>
+      <c r="L72" s="15" t="inlineStr">
+        <is>
+          <t>6/5開催（米時間）</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B73" s="15" t="inlineStr">
+        <is>
+          <t>ポケモン対戦特化新作「Pokémon Champions」、スマホ版を6/17配信と発表</t>
+        </is>
+      </c>
+      <c r="C73" s="15" t="inlineStr">
+        <is>
+          <t>https://press.pokemon.com/en/releases/Pokemon-Champions-Launches-June-17-on-iOS-and-Android-Devices-The-Poke</t>
+        </is>
+      </c>
+      <c r="D73" s="15" t="inlineStr">
+        <is>
+          <t>「Pokémon Champions」は対戦に特化したシリーズ新作として2026年4月にNintendo Switch/Switch 2で先行ローンチ。今回、モバイル展開でユーザー母数の拡大を狙い、競技ポケモンの裾野拡大とクロスプラットフォーム戦略を加速させる。</t>
+        </is>
+      </c>
+      <c r="E73" s="15" t="inlineStr">
+        <is>
+          <t>ポケモン社は6月4日、iOS/Android版を6月17日に配信すると発表。同一Nintendoアカウント連携でSwitch版のセーブデータを引き継げる。配信記念として6/17〜9/1にライチュウとメガストーン（Raichunite X/Y）を配布。事前登録は両ストアで受付中。</t>
+        </is>
+      </c>
+      <c r="F73" s="15" t="inlineStr">
+        <is>
+          <t>スマホ版（iOS/Android）を6/17配信、事前登録受付中
+Switch/Switch 2と同一アカウントでセーブ連携
+配信記念でライチュウ＋メガストーンを期間配布
+対戦特化でクロスプラットフォーム競技基盤を構築</t>
+        </is>
+      </c>
+      <c r="G73" s="15" t="inlineStr">
+        <is>
+          <t>モバイル開放により競技人口が一段拡大し、ポケモンのeスポーツ・大会施策の基盤が強化される。基本無料系の対戦タイトルとして、継続的なシーズン運営とアイテム配布によるリテンション設計が収益・継続率の鍵となる。</t>
+        </is>
+      </c>
+      <c r="H73" s="15" t="inlineStr">
+        <is>
+          <t>対戦特化IPのクロスプラットフォーム運営とリテンション設計</t>
+        </is>
+      </c>
+      <c r="I73" s="15" t="inlineStr">
+        <is>
+          <t>The Pokémon Company,任天堂</t>
+        </is>
+      </c>
+      <c r="J73" s="15" t="inlineStr">
+        <is>
+          <t>Pokémon Champions,ポケットモンスター</t>
+        </is>
+      </c>
+      <c r="K73" s="15" t="inlineStr">
+        <is>
+          <t>新作,国内</t>
+        </is>
+      </c>
+      <c r="L73" s="15" t="inlineStr">
+        <is>
+          <t>6/4発表</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B74" s="15" t="inlineStr">
+        <is>
+          <t>ゲーム業界「最高収益×最大レイオフ」のパラドックス、2026年も人員削減が継続</t>
+        </is>
+      </c>
+      <c r="C74" s="15" t="inlineStr">
+        <is>
+          <t>https://respawn.outlookindia.com/gaming/gaming-news/record-profits-record-layoffs-inside-gamings-2026-paradox</t>
+        </is>
+      </c>
+      <c r="D74" s="15" t="inlineStr">
+        <is>
+          <t>2025年の世界ゲーム業界のコンテンツ収益は約1,956億ドルと過去最高を記録した一方、雇用環境は悪化が継続。私的投資（VC等）は2025年に55%減少し、AAA・中堅スタジオで構造的な人員整理が続いている。</t>
+        </is>
+      </c>
+      <c r="E74" s="15" t="inlineStr">
+        <is>
+          <t>業界は記録的な収益にもかかわらず雇用が縮小する逆説に直面。2025年は約9,200人が職を失い、過去4年累計は約44,000人。2026年は年初来で2,000〜3,000人規模の削減が続く。3月にはEpic Gamesが従業員の約23%（1,000人超）を削減、EAはBattlefield系4スタジオ、Ubisoftも組織再編で追加削減・スタジオ閉鎖を実施した。</t>
+        </is>
+      </c>
+      <c r="F74" s="15" t="inlineStr">
+        <is>
+          <t>2025年業界収益は過去最高の約1,956億ドル
+それでも2026年初来で2,000〜3,000人を削減
+過去4年累計のレイオフは約44,000人
+Epic（23%超）・EA・Ubisoftが大型削減/再編
+私的投資は2025年に55%減</t>
+        </is>
+      </c>
+      <c r="G74" s="15" t="inlineStr">
+        <is>
+          <t>収益と雇用の乖離は当面続く見込み。AIによる開発効率化と投資環境の冷え込みが重なり、各社は「少人数・高効率」体制へ移行。タイトル数の絞り込みとライブサービス偏重が進み、人材は独立スタジオやインディーへ流動する構造が強まる。</t>
+        </is>
+      </c>
+      <c r="H74" s="15" t="inlineStr">
+        <is>
+          <t>業界の収益・雇用乖離とAI効率化の人員影響</t>
+        </is>
+      </c>
+      <c r="I74" s="15" t="inlineStr">
+        <is>
+          <t>Epic Games,Electronic Arts,Ubisoft</t>
+        </is>
+      </c>
+      <c r="J74" s="15" t="inlineStr">
+        <is>
+          <t>Battlefield,Fortnite</t>
+        </is>
+      </c>
+      <c r="K74" s="15" t="inlineStr">
+        <is>
+          <t>業績,海外</t>
+        </is>
+      </c>
+      <c r="L74" s="15" t="inlineStr">
+        <is>
+          <t>2026年初来の動向</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B75" s="15" t="inlineStr">
+        <is>
+          <t>6月はeスポーツ大型大会ラッシュ、VALORANT/LoL/CS2のメジャーが集中開催</t>
+        </is>
+      </c>
+      <c r="C75" s="15" t="inlineStr">
+        <is>
+          <t>https://esportsinsider.com/2026/01/esports-events-calendar-2026-every-major-tournament</t>
+        </is>
+      </c>
+      <c r="D75" s="15" t="inlineStr">
+        <is>
+          <t>6月は国際大会の集中期。E3後継のゲーム発表シーズンと並行し、各タイトルのメジャー大会が世界各地で開催され、視聴者・スポンサーの注目が一気に高まる時期となっている。</t>
+        </is>
+      </c>
+      <c r="E75" s="15" t="inlineStr">
+        <is>
+          <t>VALORANTは英国初開催となるMasters Londonで欧州にVCTが帰還、League of LegendsはMSI 2026を開催。ESLがIEM CologneをCS2 Majorに格上げし、米国ではEvo（FGC最大規模）やCall of Duty Leagueの第4 Major、PUBG Nations Cupも実施。Esports Nations CupのVALORANT予選は6/26-28に行われる。</t>
+        </is>
+      </c>
+      <c r="F75" s="15" t="inlineStr">
+        <is>
+          <t>VALORANT Masters London（英国初の国際開催）
+League of Legends MSI 2026を6月開催
+CS2 Major（IEM Cologne格上げ）をESLが主催
+Evo・CoD League第4 Major・PUBG Nations Cupも集中
+Esports Nations Cup VALORANT予選は6/26-28</t>
+        </is>
+      </c>
+      <c r="G75" s="15" t="inlineStr">
+        <is>
+          <t>メジャー大会の集中は開催地誘致・観光・放映権の競争を加速させる。英国・欧州での国際開催拡大はリージョン分散の流れを示し、視聴のモバイル/ライブ配信シフトと相まって収益化モデル（放映権・スポンサー・チケット）の多角化が進む。</t>
+        </is>
+      </c>
+      <c r="H75" s="15" t="inlineStr">
+        <is>
+          <t>国際eスポーツ大会の開催地誘致と放映権ビジネス</t>
+        </is>
+      </c>
+      <c r="I75" s="15" t="inlineStr">
+        <is>
+          <t>Riot Games,ESL,Valve,Activision</t>
+        </is>
+      </c>
+      <c r="J75" s="15" t="inlineStr">
+        <is>
+          <t>VALORANT,League of Legends,Counter-Strike 2,Call of Duty</t>
+        </is>
+      </c>
+      <c r="K75" s="15" t="inlineStr">
+        <is>
+          <t>eスポーツ,海外</t>
+        </is>
+      </c>
+      <c r="L75" s="15" t="inlineStr">
+        <is>
+          <t>6月の大会カレンダー</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B76" s="15" t="inlineStr">
+        <is>
+          <t>Loom Games「20人で10億ドルEXIT」、超少人数・高評価額がスタジオ雇用に問い</t>
+        </is>
+      </c>
+      <c r="C76" s="15" t="inlineStr">
+        <is>
+          <t>https://www.pocketgamer.biz/what-loom-games-1bn-exit-with-20-people-tells-us-about-the-future-of-game-studio-hiring/</t>
+        </is>
+      </c>
+      <c r="D76" s="15" t="inlineStr">
+        <is>
+          <t>Scopelyが2026年2月にイスタンブール拠点のモバイル開発Loom Gamesを評価額10億ドル超で買収。従業員わずか約20人での大型EXITが、AI活用と効率化が進む時代のスタジオ採用・組織規模のあり方を問う事例として再注目されている。</t>
+        </is>
+      </c>
+      <c r="E76" s="15" t="inlineStr">
+        <is>
+          <t>Loom Gamesは約20人の少人数体制で10億ドル級の評価額に到達。少人数・高生産性のスタジオが巨額のM&amp;A対価を生む構図は、人員拡大による成長という従来モデルへの転換を示唆。AIツールの普及で1人あたり付加価値が高まる中、雇用の量より質・効率を重視する採用戦略が議論を呼んでいる。</t>
+        </is>
+      </c>
+      <c r="F76" s="15" t="inlineStr">
+        <is>
+          <t>約20人のスタジオが10億ドル超の評価額でEXIT
+少人数・高生産性モデルがM&amp;A対価を最大化
+AI活用で1人あたり付加価値が上昇
+大量採用による拡大成長モデルからの転換を示唆</t>
+        </is>
+      </c>
+      <c r="G76" s="15" t="inlineStr">
+        <is>
+          <t>「超少人数で高評価額」の事例が増えれば、スタジオは採用を絞り込みAIと外部委託で生産性を高める方向へ。投資家は組織規模より1人当たり収益・IPの強さを評価軸とし、業界全体で雇用総量が伸びにくい構造が定着する可能性がある。</t>
+        </is>
+      </c>
+      <c r="H76" s="15" t="inlineStr">
+        <is>
+          <t>少人数・高生産性スタジオの評価モデルと採用戦略</t>
+        </is>
+      </c>
+      <c r="I76" s="15" t="inlineStr">
+        <is>
+          <t>Scopely,Loom Games,Savvy Games Group</t>
+        </is>
+      </c>
+      <c r="J76" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K76" s="15" t="inlineStr">
+        <is>
+          <t>M&amp;A,海外</t>
+        </is>
+      </c>
+      <c r="L76" s="15" t="inlineStr">
+        <is>
+          <t>2/19買収・分析記事</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
weekly-releases + indie update (2026-06-05 09:11)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -7889,7 +7889,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8398,6 +8398,231 @@
       <c r="M10" t="inlineStr">
         <is>
           <t>https://www.mensjournal.com/entertainment/top-10-video-games-releasing-in-june-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>House Flipper Remastered Collection（ハウスフリッパー リマスター・コレクション）</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Frozen District</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Frozen Way (PlayWay)</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>PC/PS5/Xbox Series X|S</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>シミュレーション</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>2</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>基本ゲーム+全DLC（Garden/Luxury/Pets/Farm）を統合し、ビジュアル刷新・フルボイス・新ストーリー追加。$49.99。既存所有者向け割引あり。</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>https://www.gematsu.com/2026/04/house-flipper-remastered-collection-launches-june-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Solarpunk: 天空の島（Solarpunk／ソーラーパンク）</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Cyberwave</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Cyberwave</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>PC/PS5/Xbox Series X|S/Switch 2</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>コージー・サバイバルクラフト</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
+        <v>3</v>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>飛行船で浮遊島を冒険するコージー建築サバイバル。Steamで7万超フォロワーを集め、無料体験版が高評価。発売前から話題（来週分・評価系空欄）。</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>https://screenrant.com/steam-june-2026-trending-free-game/</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>リズム天国 ミラクルスターズ（Rhythm Heaven Miracle Stars）</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>任天堂/TNX</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>任天堂</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Nintendo Switch/Switch 2</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>リズムアクション</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
+        <v>4</v>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>『リズム天国』シリーズ11年ぶりの完全新作。来月発売予定（評価系空欄）。</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/article/202605/72453</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>カルドセプト ビギンズ（Culdcept Begins）</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>大宮ソフト</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>任天堂</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Nintendo Switch 2/Switch/Steam</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>ボード×カードゲーム</t>
+        </is>
+      </c>
+      <c r="K14" t="n">
+        <v>3</v>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>『カルドセプト』シリーズ10年ぶりの完全新作。来月発売予定（評価系空欄）。</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/schedule/switch</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-07 (日付未定)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Assassin's Creed Black Flag Resynced（アサシン クリード ブラックフラッグ リシンクド）</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Ubisoft</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Ubisoft</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>PC/PS5/Xbox Series X|S</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>オープンワールドACT</t>
+        </is>
+      </c>
+      <c r="K15" t="n">
+        <v>4</v>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>『AC4 ブラックフラッグ』の現世代リメイク。7月発売で確定と報道。海洋探索リメイクの本命。来月分（評価系空欄）。</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>https://www.gamesradar.com/video-game-release-dates/</t>
         </is>
       </c>
     </row>
@@ -11703,7 +11928,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11905,6 +12130,100 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>TBH: Task Bar Hero</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>個人/小規模インディー</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>配信中（基本無料）</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>PC/Steam</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>カジュアル/バイラル</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>広告予算もパブリッシャーの後ろ盾もない無料作が、配信・SNSのバイラルのみで6月初週のSteamトレンド首位に。2位の大型『007 First Light』に約10万差をつけた。</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Steam同接ピーク 13.3万（出典: ScreenRant / GameGrin 週間まとめ）</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>無料×配信映えで一気に母数を取る『アテンション経済』型ヒットの象徴。後からDLC/続編回収の設計が増加。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>電車アタック（Denshattack!）</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Undercoders（スペイン・小規模）</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026-06-18 発売予定</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Nintendo Switch 2/PS5/Xbox Series X|S/Steam</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>アクロバティック電車アクションレース</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Nintendo『インディーワールド』で紹介され話題化。ディストピア日本を電車で疾走し、フリップや空中スタントをキメるハイテンション3Dトリックアクション。</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>体験版を配信中（インディーワールド連動）。SNSで実況・クリップが拡散。</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>低予算ながら唯一無二のコンセプトで配信映え。発売前から国内外メディアが言及。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
daily-news + cross-questions update (2026-06-05 22:10)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -2477,7 +2477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3044,6 +3044,80 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B16" s="14" t="inlineStr">
+        <is>
+          <t>ゲームのAI生成物に対する『開示・ラベリング義務』圧力は、広告・映像・音楽・出版などコンテンツ制作業界の表示義務化で何に該当するか？</t>
+        </is>
+      </c>
+      <c r="C16" s="14" t="inlineStr">
+        <is>
+          <t>Summer Game Fest 2026でAI生成アセットの開示が続出し『Tomb Raider』等にファン反発。カプコンはAI生成物の本編実装を否定。</t>
+        </is>
+      </c>
+      <c r="D16" s="14" t="inlineStr">
+        <is>
+          <t>Capcom,Crystal Dynamics,Steam/Valve</t>
+        </is>
+      </c>
+      <c r="E16" s="14" t="inlineStr">
+        <is>
+          <t>広告制作,映像/VFX,音楽,出版,SNS/動画配信(AI表示義務)</t>
+        </is>
+      </c>
+      <c r="F16" s="14" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="G16" s="14" t="inlineStr">
+        <is>
+          <t>消費者向け『AI使用の見える化』は規制ではなくコミュニティ圧力から先行。各業界も最終成果物へのAI混入が信頼の分水嶺になりうる。</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>ソブリンファンド主導の巨額LBOに対するEU外国補助金規則(FSR)審査は、通信・インフラ・半導体など他の戦略産業のM&amp;Aでも同様の関門になるか？</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="inlineStr">
+        <is>
+          <t>EA買収550億ドルLBO連合(PIF/Silver Lake/Affinity)が夏前にEUへFSR申請の見込み。</t>
+        </is>
+      </c>
+      <c r="D17" s="14" t="inlineStr">
+        <is>
+          <t>Electronic Arts,PIF,Silver Lake,Affinity Partners</t>
+        </is>
+      </c>
+      <c r="E17" s="14" t="inlineStr">
+        <is>
+          <t>通信,エネルギー/インフラ,半導体,防衛関連の越境M&amp;A</t>
+        </is>
+      </c>
+      <c r="F17" s="14" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="G17" s="14" t="inlineStr">
+        <is>
+          <t>国家系資金の越境買収はFSR等の補助金審査が新たな関門に。ゲームに限らず戦略産業のディール設計・期間に影響しうる。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3055,7 +3129,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L76"/>
+  <dimension ref="A1:L86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7875,6 +7949,657 @@
       <c r="L76" s="15" t="inlineStr">
         <is>
           <t>2/19買収・分析記事</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B77" s="14" t="inlineStr">
+        <is>
+          <t>EA買収550億ドルLBO連合、夏前に欧州委へFSR申請の見込み</t>
+        </is>
+      </c>
+      <c r="C77" s="14" t="inlineStr">
+        <is>
+          <t>https://www.datasite.com/en/resources/insights/market-spotlight-will-the-ea-buyout-level-up-gaming-m-and-a</t>
+        </is>
+      </c>
+      <c r="D77" s="14" t="inlineStr">
+        <is>
+          <t>サウジ公的投資基金(PIF)・Silver Lake・Affinity Partnersの連合が、Electronic Artsを総額550億ドルで買収する案を進めている。ゲーム史上2番目に大きい買収で、スポンサー主導としては史上最大のLBO（レバレッジド・バイアウト）に当たる。</t>
+        </is>
+      </c>
+      <c r="E77" s="14" t="inlineStr">
+        <is>
+          <t>連合は2026年6月初旬、EUの外国補助金規則(FSR)に基づき欧州委員会へ買収案を夏前に申請する見込みと報じられた。株主には1株210ドル（25%プレミアム）が支払われ、成立すればPIFがEAの過半数を握る。巨額負債を伴う構造が注目される。</t>
+        </is>
+      </c>
+      <c r="F77" s="14" t="inlineStr">
+        <is>
+          <t>買収額550億ドル＝ゲーム史上2位・スポンサー主導LBO史上最大
+PIFが過半数株主、Silver Lakeが少数株主、Affinityが5%
+EU外国補助金規則(FSR)の審査が成立の関門
+株主は1株210ドル(25%プレミアム)を受領</t>
+        </is>
+      </c>
+      <c r="G77" s="14" t="inlineStr">
+        <is>
+          <t>FSR審査やレバレッジ負担が焦点。承認されればソブリンファンドのゲーム支配が一段と進み、他の大型ディールの呼び水になる一方、規制当局の警戒で審査長期化の可能性もある。</t>
+        </is>
+      </c>
+      <c r="H77" s="14" t="inlineStr">
+        <is>
+          <t>外国補助金規則(FSR)とゲームM&amp;Aの規制審査構造</t>
+        </is>
+      </c>
+      <c r="I77" s="14" t="inlineStr">
+        <is>
+          <t>Electronic Arts,PIF(サウジ),Silver Lake,Affinity Partners</t>
+        </is>
+      </c>
+      <c r="J77" s="14" t="inlineStr">
+        <is>
+          <t>EA,FIFA/EA SPORTS FC,Battlefield,The Sims</t>
+        </is>
+      </c>
+      <c r="K77" s="14" t="inlineStr">
+        <is>
+          <t>M&amp;A,海外,規制</t>
+        </is>
+      </c>
+      <c r="L77" s="14" t="inlineStr">
+        <is>
+          <t>6/4報道・分析</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B78" s="14" t="inlineStr">
+        <is>
+          <t>Alpha Compute、GAMEE買収を完了しAIゲーム部門「Alpha Games」設立</t>
+        </is>
+      </c>
+      <c r="C78" s="14" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/0001095435/000117184326003721/exh_994.htm</t>
+        </is>
+      </c>
+      <c r="D78" s="14" t="inlineStr">
+        <is>
+          <t>AIインフラ企業Alpha Compute(旧称含む)が、HTML5/カジュアルゲームのGAMEEの過半数取得を進めていた。GAMEEは約1.2億人のゲーム利用者基盤を持ち、2025年売上は350万ドル。AIとゲームの融合を狙う買収案件。</t>
+        </is>
+      </c>
+      <c r="E78" s="14" t="inlineStr">
+        <is>
+          <t>Alpha Computeは2026年5月27日にGAMEEの過半数取得を完了し、創業者Bozena Rezab氏が率いる新AIゲーム部門「Alpha Games」を設立したと開示。1.2億人のユーザー基盤をAI活用のゲーム体験に転用する構想を示した。</t>
+        </is>
+      </c>
+      <c r="F78" s="14" t="inlineStr">
+        <is>
+          <t>5/27に過半数取得を完了、6-K開示
+GAMEEは約1.2億ユーザー・2025年売上350万ドル
+新部門Alpha GamesをGAMEE創業者Rezab氏が指揮
+AIインフラ企業がゲーム配信網を取り込む構図</t>
+        </is>
+      </c>
+      <c r="G78" s="14" t="inlineStr">
+        <is>
+          <t>AI企業がユーザー基盤を求めてゲーム資産を買う動きが拡大する可能性。配信網×生成AIで体験を作る試みが増えれば、従来のパブリッシャーとは異なる競合軸が生まれる。</t>
+        </is>
+      </c>
+      <c r="H78" s="14" t="inlineStr">
+        <is>
+          <t>AIインフラ企業によるゲーム資産取得とユーザー基盤の価値</t>
+        </is>
+      </c>
+      <c r="I78" s="14" t="inlineStr">
+        <is>
+          <t>Alpha Compute,GAMEE</t>
+        </is>
+      </c>
+      <c r="J78" s="14" t="inlineStr">
+        <is>
+          <t>Alpha Games</t>
+        </is>
+      </c>
+      <c r="K78" s="14" t="inlineStr">
+        <is>
+          <t>M&amp;A,技術,海外</t>
+        </is>
+      </c>
+      <c r="L78" s="14" t="inlineStr">
+        <is>
+          <t>6-K(FY2026)開示</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B79" s="14" t="inlineStr">
+        <is>
+          <t>Summer Game Fest 2026本編、RE：ベロニカやTMNT新作など一挙公開</t>
+        </is>
+      </c>
+      <c r="C79" s="14" t="inlineStr">
+        <is>
+          <t>https://www.gamespot.com/articles/summer-game-fest-live-2026-all-the-biggest-announcements-and-games/</t>
+        </is>
+      </c>
+      <c r="D79" s="14" t="inlineStr">
+        <is>
+          <t>毎夏恒例のゲーム発表祭典Summer Game FestがGeoff Keighley司会で6月6日(米時間)にロサンゼルスのDolby Theatreから開催。E3亡き後、業界最大級の新作発表ハブとなっている。</t>
+        </is>
+      </c>
+      <c r="E79" s="14" t="inlineStr">
+        <is>
+          <t>本編では『Resident Evil Veronica』(Code:Veronicaリメイク)、Paramount×PlatinumGamesの『TMNT: The Last Ronin』、Bandai Namcoの新作ガンダム(2027年)、『Assassin's Creed』(Edward Kenway編、7/9発売)、『Mortal Shell 2』オープンβなどが公開された。</t>
+        </is>
+      </c>
+      <c r="F79" s="14" t="inlineStr">
+        <is>
+          <t>カプコン『RE：ベロニカ』(Code:Veronicaリメイク)初公開
+Paramount×PlatinumGames『TMNT: The Last Ronin』
+Bandai Namcoが2027年向け新作ガンダムを発表
+『AC』Edward Kenway編が7/9発売
+Dead by Daylight10周年の続報は6/14</t>
+        </is>
+      </c>
+      <c r="G79" s="14" t="inlineStr">
+        <is>
+          <t>夏商戦・年末に向けた大型タイトルの実機/発売日情報が出そろう。リメイクと既存IP活用が主流で、各社が新規IPより手堅い回収を優先する傾向が続くと見られる。</t>
+        </is>
+      </c>
+      <c r="H79" s="14" t="inlineStr">
+        <is>
+          <t>E3後の発表祭典エコシステムとIP活用戦略</t>
+        </is>
+      </c>
+      <c r="I79" s="14" t="inlineStr">
+        <is>
+          <t>Capcom,Paramount,PlatinumGames,Bandai Namco,Ubisoft</t>
+        </is>
+      </c>
+      <c r="J79" s="14" t="inlineStr">
+        <is>
+          <t>Resident Evil,TMNT,Gundam,Assassin's Creed,Mortal Shell</t>
+        </is>
+      </c>
+      <c r="K79" s="14" t="inlineStr">
+        <is>
+          <t>新作,海外</t>
+        </is>
+      </c>
+      <c r="L79" s="14" t="inlineStr">
+        <is>
+          <t>6/6本編の発表まとめ</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B80" s="14" t="inlineStr">
+        <is>
+          <t>Paramount Skydanceが新ゲームスタジオ設立、初のAAAをSGFで発表</t>
+        </is>
+      </c>
+      <c r="C80" s="14" t="inlineStr">
+        <is>
+          <t>https://variety.com/2026/gaming/news/paramount-skydance-video-game-studio-1236767557/</t>
+        </is>
+      </c>
+      <c r="D80" s="14" t="inlineStr">
+        <is>
+          <t>Paramount Skydanceは映像・配信に続く「コンテンツ戦略の中核」としてゲーム事業の強化を打ち出してきた。ハリウッド資本がゲームを内製化する流れの象徴的な動き。</t>
+        </is>
+      </c>
+      <c r="E80" s="14" t="inlineStr">
+        <is>
+          <t>Paramountは新組織Paramount Game Studiosを設立し、社長にTony Driscoll氏を起用。Summer Game Fest(6/6)で初のAAAタイトルとしてPlatinumGames共同開発の『TMNT: The Last Ronin』を発表した。</t>
+        </is>
+      </c>
+      <c r="F80" s="14" t="inlineStr">
+        <is>
+          <t>Paramount Game Studiosを新設、社長にTony Driscoll氏
+ゲームを映像/配信と並ぶ戦略の柱と位置づけ
+初AAAはPlatinumGames共同の『TMNT: The Last Ronin』
+ハリウッド資本のゲーム内製化が加速</t>
+        </is>
+      </c>
+      <c r="G80" s="14" t="inlineStr">
+        <is>
+          <t>映像IPホルダーが自社ゲーム開発に踏み込む例が増える可能性。IPの相互送客とメディアミックスを軸に、既存パブリッシャーとの提携・競合構図が変化しうる。</t>
+        </is>
+      </c>
+      <c r="H80" s="14" t="inlineStr">
+        <is>
+          <t>メディア企業のゲーム内製化とIPメディアミックス戦略</t>
+        </is>
+      </c>
+      <c r="I80" s="14" t="inlineStr">
+        <is>
+          <t>Paramount Skydance,PlatinumGames</t>
+        </is>
+      </c>
+      <c r="J80" s="14" t="inlineStr">
+        <is>
+          <t>TMNT: The Last Ronin</t>
+        </is>
+      </c>
+      <c r="K80" s="14" t="inlineStr">
+        <is>
+          <t>新作,海外,M&amp;A</t>
+        </is>
+      </c>
+      <c r="L80" s="14" t="inlineStr">
+        <is>
+          <t>Variety独占報道</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B81" s="14" t="inlineStr">
+        <is>
+          <t>FromSoftware『ELDEN RING Tarnished Edition』Switch2版を8/28発売</t>
+        </is>
+      </c>
+      <c r="C81" s="14" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/</t>
+        </is>
+      </c>
+      <c r="D81" s="14" t="inlineStr">
+        <is>
+          <t>FromSoftwareの『ELDEN RING』は世界的ヒットを記録。任天堂の新ハードSwitch 2の登場で、人気タイトルの新ハード対応が相次いでいる。</t>
+        </is>
+      </c>
+      <c r="E81" s="14" t="inlineStr">
+        <is>
+          <t>FromSoftwareは『ELDEN RING Tarnished Edition』のNintendo Switch 2版を8月28日に全世界同時発売すると発表。パッケージ版の予約は6月5日、ダウンロード版は6月11日に開始される。</t>
+        </is>
+      </c>
+      <c r="F81" s="14" t="inlineStr">
+        <is>
+          <t>Switch 2版『ELDEN RING Tarnished Edition』8/28世界同時発売
+パッケージ予約は6/5、DL版予約は6/11開始
+人気作のSwitch 2対応ラッシュの一環
+FromSoftが新ハードでの裾野拡大を狙う</t>
+        </is>
+      </c>
+      <c r="G81" s="14" t="inlineStr">
+        <is>
+          <t>Switch 2向けに大型既存タイトルの移植・最適化版が続く見込み。新ハード初期の弾としてサードの実績作が並び、ハード普及とソフト販売が相互に押し上げられる。</t>
+        </is>
+      </c>
+      <c r="H81" s="14" t="inlineStr">
+        <is>
+          <t>新ハード初期のサードパーティ移植戦略</t>
+        </is>
+      </c>
+      <c r="I81" s="14" t="inlineStr">
+        <is>
+          <t>FromSoftware,Bandai Namco,任天堂</t>
+        </is>
+      </c>
+      <c r="J81" s="14" t="inlineStr">
+        <is>
+          <t>ELDEN RING</t>
+        </is>
+      </c>
+      <c r="K81" s="14" t="inlineStr">
+        <is>
+          <t>新作,国内</t>
+        </is>
+      </c>
+      <c r="L81" s="14" t="inlineStr">
+        <is>
+          <t>6/5予約開始</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B82" s="14" t="inlineStr">
+        <is>
+          <t>Summer Game FestでAI生成アセットの開示相次ぐ、ファンの反発も</t>
+        </is>
+      </c>
+      <c r="C82" s="14" t="inlineStr">
+        <is>
+          <t>https://www.pcgamer.com/software/ai/summer-game-fest-is-here-so-get-ready-for-a-lot-of-ugh-that-game-with-the-cool-trailer-used-ai/</t>
+        </is>
+      </c>
+      <c r="D82" s="14" t="inlineStr">
+        <is>
+          <t>生成AIの開発活用を巡り、ゲーマーの間では「AI slop(粗製乱造)」への反発が強まり、過去には抗議でタイトルが中止に追い込まれた例もある。SteamはAI利用の開示を義務付けている。</t>
+        </is>
+      </c>
+      <c r="E82" s="14" t="inlineStr">
+        <is>
+          <t>今年のSGF週間では、トレーラー公開後にSteamのAI開示で生成AI利用が判明する事例が続出。『Tomb Raider』では落胆と容認が混在する反応が出た。カプコンは「AI生成アセットは実装しない」が「効率化目的のAI活用は進める」と表明した。</t>
+        </is>
+      </c>
+      <c r="F82" s="14" t="inlineStr">
+        <is>
+          <t>SGF発表作で生成AIアセットの開示が続出
+『Tomb Raider』はファン反応が賛否混在
+カプコンはAI生成物の本編実装を否定、効率化AIは推進
+プロトタイプ用途と最終製品搭載で評価が分かれる</t>
+        </is>
+      </c>
+      <c r="G82" s="14" t="inlineStr">
+        <is>
+          <t>開示義務の運用が広がり、各社はAI利用範囲の明確化を迫られる。最終アセットへの搭載可否がブランド信頼やコミュニティ反応を左右する争点になり続ける。</t>
+        </is>
+      </c>
+      <c r="H82" s="14" t="inlineStr">
+        <is>
+          <t>生成AIの開示義務とゲーマーコミュニティの受容</t>
+        </is>
+      </c>
+      <c r="I82" s="14" t="inlineStr">
+        <is>
+          <t>Capcom,Crystal Dynamics</t>
+        </is>
+      </c>
+      <c r="J82" s="14" t="inlineStr">
+        <is>
+          <t>Tomb Raider</t>
+        </is>
+      </c>
+      <c r="K82" s="14" t="inlineStr">
+        <is>
+          <t>技術,海外</t>
+        </is>
+      </c>
+      <c r="L82" s="14" t="inlineStr">
+        <is>
+          <t>6/5-6/6 SGF週間</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B83" s="14" t="inlineStr">
+        <is>
+          <t>GameSquare、2026年Q2売上を137%超増・1850万ドル超へ上方示唆</t>
+        </is>
+      </c>
+      <c r="C83" s="14" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/0001714562/000149315226027282/ex99-1.htm</t>
+        </is>
+      </c>
+      <c r="D83" s="14" t="inlineStr">
+        <is>
+          <t>GameSquare Holdingsはゲーム/eスポーツ領域のメディア・ブランド事業を展開。クリエイター主導の広告キャンペーンや買収による事業拡大を進めてきた米上場企業。</t>
+        </is>
+      </c>
+      <c r="E83" s="14" t="inlineStr">
+        <is>
+          <t>GameSquareは2026年第2四半期の売上が前年同期比137%超増の少なくとも1850万ドルになる見通しと開示。ブランドプログラム拡大、パブリッシャー需要、クリエイター施策、直近買収の貢献が成長を牽引するとした。</t>
+        </is>
+      </c>
+      <c r="F83" s="14" t="inlineStr">
+        <is>
+          <t>Q2売上を前年比+137%超・1850万ドル超と示唆(8-K)
+ブランドプログラム拡大とパブリッシャー需要が寄与
+クリエイター主導キャンペーンが増加
+直近買収の統合効果も反映</t>
+        </is>
+      </c>
+      <c r="G83" s="14" t="inlineStr">
+        <is>
+          <t>ゲームメディア/マーケ領域は広告とクリエイター経済の追い風で成長余地。一方で利益化と買収統合が課題で、トップライン成長の質が問われる局面に入る。</t>
+        </is>
+      </c>
+      <c r="H83" s="14" t="inlineStr">
+        <is>
+          <t>ゲーム×クリエイターマーケティングの収益モデル</t>
+        </is>
+      </c>
+      <c r="I83" s="14" t="inlineStr">
+        <is>
+          <t>GameSquare Holdings</t>
+        </is>
+      </c>
+      <c r="J83" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K83" s="14" t="inlineStr">
+        <is>
+          <t>業績,海外</t>
+        </is>
+      </c>
+      <c r="L83" s="14" t="inlineStr">
+        <is>
+          <t>8-K(FY2026)開示</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B84" s="14" t="inlineStr">
+        <is>
+          <t>CS2『IEM Cologne Major 2026』開幕、初日44.8万同接・賞金125万ドル</t>
+        </is>
+      </c>
+      <c r="C84" s="14" t="inlineStr">
+        <is>
+          <t>https://escharts.com/news/how-watch-iem-cologne-major-2026</t>
+        </is>
+      </c>
+      <c r="D84" s="14" t="inlineStr">
+        <is>
+          <t>Counter-Strike 2はeスポーツの中核タイトルで、Majorは年間最高峰の大会。ドイツ・ケルンは伝統的に大型大会の聖地として知られる。</t>
+        </is>
+      </c>
+      <c r="E84" s="14" t="inlineStr">
+        <is>
+          <t>『IEM Cologne Major 2026』が6月2日〜21日にドイツで開催。賞金総額は125万ドルで優勝賞金は50万ドル。6/2のStage1初日は世界で44.8万超のピーク同接を記録し、滑り出しは好調。</t>
+        </is>
+      </c>
+      <c r="F84" s="14" t="inlineStr">
+        <is>
+          <t>会期は6/2〜21、ドイツ・ケルン開催
+賞金総額125万ドル・優勝50万ドル
+初日ピーク同接44.8万超
+CS2 Majorとして年間最大級の注目度</t>
+        </is>
+      </c>
+      <c r="G84" s="14" t="inlineStr">
+        <is>
+          <t>Major期間中は視聴・チーム成績が大きく動く。CS2は安定した観戦需要を維持し、スポンサー・配信プラットフォームの競争も活発化する見込み。</t>
+        </is>
+      </c>
+      <c r="H84" s="14" t="inlineStr">
+        <is>
+          <t>eスポーツMajor大会の視聴指標とスポンサー経済</t>
+        </is>
+      </c>
+      <c r="I84" s="14" t="inlineStr">
+        <is>
+          <t>ESL/FACEIT,Valve</t>
+        </is>
+      </c>
+      <c r="J84" s="14" t="inlineStr">
+        <is>
+          <t>Counter-Strike 2</t>
+        </is>
+      </c>
+      <c r="K84" s="14" t="inlineStr">
+        <is>
+          <t>eスポーツ,海外</t>
+        </is>
+      </c>
+      <c r="L84" s="14" t="inlineStr">
+        <is>
+          <t>6/2-21開催中</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B85" s="14" t="inlineStr">
+        <is>
+          <t>ガチャ／ルートボックス規制、2026年が転換点：EUは硬法化・日本は自主規制</t>
+        </is>
+      </c>
+      <c r="C85" s="14" t="inlineStr">
+        <is>
+          <t>https://gametyrant.com/news/the-loot-box-loophole-is-closing-why-2026-is-the-year-your-in-game-currency-finally-becomes-real-money</t>
+        </is>
+      </c>
+      <c r="D85" s="14" t="inlineStr">
+        <is>
+          <t>ルートボックスやガチャは射幸性と未成年保護の観点で各国の規制対象に。日本は「コンプガチャ」騒動以降、業界の自主規制（確率開示・天井等）で対応してきた。</t>
+        </is>
+      </c>
+      <c r="E85" s="14" t="inlineStr">
+        <is>
+          <t>2026年は政府・裁判所・市場の動きが収束し、ゲーム内通貨を「実質的な現金」として扱う流れが強まる年と分析される。EUはダークパターン・消費者保護の枠組みで硬法化を志向、日本は確率開示等の自主規制を維持。各社は地域別の二重設計で対応する。</t>
+        </is>
+      </c>
+      <c r="F85" s="14" t="inlineStr">
+        <is>
+          <t>2026年はゲーム内通貨を実質現金とみなす規制が収束
+EUは消費者保護/ダークパターン規制で硬法化志向
+日本は確率開示・天井など自主規制を継続
+各社は地域別「二重設計」で確率・UI・上限を出し分け</t>
+        </is>
+      </c>
+      <c r="G85" s="14" t="inlineStr">
+        <is>
+          <t>確率開示や支出上限、未成年保護の規制が地域ごとに強化される見通し。グローバル運営では地域別設計コストが増し、収益モデルの再設計が迫られる。</t>
+        </is>
+      </c>
+      <c r="H85" s="14" t="inlineStr">
+        <is>
+          <t>ルートボックス/ガチャの各国規制と二重設計の運用</t>
+        </is>
+      </c>
+      <c r="I85" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J85" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K85" s="14" t="inlineStr">
+        <is>
+          <t>規制,海外,国内</t>
+        </is>
+      </c>
+      <c r="L85" s="14" t="inlineStr">
+        <is>
+          <t>2026規制動向の分析</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B86" s="14" t="inlineStr">
+        <is>
+          <t>スクウェア・エニックスFY2026通期、減収増益で営業益547億円(+34.9%)</t>
+        </is>
+      </c>
+      <c r="C86" s="14" t="inlineStr">
+        <is>
+          <t>https://www.resetera.com/threads/square-enix-lifts-full-year-profit-forecasts-on-strong-game-and-royalty-earnings-q3-fy2026-results.1426429/</t>
+        </is>
+      </c>
+      <c r="D86" s="14" t="inlineStr">
+        <is>
+          <t>スクウェア・エニックスはFY2024の減損後、低採算のモバイル・HD案件を絞り込み「少数精鋭・高採算」へ路線転換を進めてきた。バックカタログのロイヤリティ収益が下支え。</t>
+        </is>
+      </c>
+      <c r="E86" s="14" t="inlineStr">
+        <is>
+          <t>2026年3月期通期は営業利益547億円(前年比+34.9%)と増益の一方、純売上は8.3%減の2976億円。タイトル数を絞り高採算化を進め、追加コストの低い旧作販売が好調。営業利益率18.4%は10年超ぶりの高水準となった。</t>
+        </is>
+      </c>
+      <c r="F86" s="14" t="inlineStr">
+        <is>
+          <t>通期営業益547億円(+34.9%)・純売上2976億円(-8.3%)の減収増益
+低採算モバイル/HD案件の整理が奏功
+バックカタログのロイヤリティが利益を下支え
+営業利益率18.4%は10年超ぶりの高水準</t>
+        </is>
+      </c>
+      <c r="G86" s="14" t="inlineStr">
+        <is>
+          <t>「数を絞り採算重視」の方針が定着すれば安定益は見込めるが、ヒット依存と新規IP育成のバランスが課題。次の大型タイトルの成否が成長余地を左右する。</t>
+        </is>
+      </c>
+      <c r="H86" s="14" t="inlineStr">
+        <is>
+          <t>ゲームパブリッシャーの選択と集中・高採算化戦略</t>
+        </is>
+      </c>
+      <c r="I86" s="14" t="inlineStr">
+        <is>
+          <t>Square Enix</t>
+        </is>
+      </c>
+      <c r="J86" s="14" t="inlineStr">
+        <is>
+          <t>FINAL FANTASY,DRAGON QUEST</t>
+        </is>
+      </c>
+      <c r="K86" s="14" t="inlineStr">
+        <is>
+          <t>業績,国内</t>
+        </is>
+      </c>
+      <c r="L86" s="14" t="inlineStr">
+        <is>
+          <t>FY2026通期決算</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
daily-news + cross-questions update (2026-06-07) (2026-06-07 00:03)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -2477,7 +2477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3118,6 +3118,43 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B18" s="14" t="inlineStr">
+        <is>
+          <t>ゲーム大型発表会のPrime Video/Fire TVなどOTT配信網への拡大は、自動車・家電・テックの製品発表(キーノート)の配信流通でも同様に主流化するか？</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="inlineStr">
+        <is>
+          <t>Xbox Games Showcase 2026が米国で初めてAmazon Live/Prime Video(Fire TV)経由でも配信。</t>
+        </is>
+      </c>
+      <c r="D18" s="14" t="inlineStr">
+        <is>
+          <t>Microsoft,Xbox,Amazon</t>
+        </is>
+      </c>
+      <c r="E18" s="14" t="inlineStr">
+        <is>
+          <t>家電/自動車/テックのプロダクトローンチ,動画配信/放送,広告</t>
+        </is>
+      </c>
+      <c r="F18" s="14" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="G18" s="14" t="inlineStr">
+        <is>
+          <t>自社サイト・YouTube/Twitch中心だった企業発表会が、リビングのTV/OTTへ越境。発表会が『放送番組化』し、配信枠とスポンサー設計が他業界のローンチにも波及しうる。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3129,7 +3166,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L86"/>
+  <dimension ref="A1:L91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8600,6 +8637,336 @@
       <c r="L86" s="14" t="inlineStr">
         <is>
           <t>FY2026通期決算</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B87" s="14" t="inlineStr">
+        <is>
+          <t>『Gears of War: E-Day』Direct公開、エメージェンス・デイ前夜を描く原点・2026年内発売へ</t>
+        </is>
+      </c>
+      <c r="C87" s="14" t="inlineStr">
+        <is>
+          <t>https://www.gamesradar.com/gears-of-war-e-day-guide/</t>
+        </is>
+      </c>
+      <c r="D87" s="14" t="inlineStr">
+        <is>
+          <t>Gears of Warシリーズ25周年に合わせ、The CoalitionとPeople Can Flyが共同開発するシリーズ原点を描く新作。オリジナル『Gears』の14年前、人類とローカストの戦端が開かれる『エメージェンス・デイ』を題材とする。</t>
+        </is>
+      </c>
+      <c r="E87" s="14" t="inlineStr">
+        <is>
+          <t>Xbox Games Showcase直後のE-Day Directで、開発元The Coalitionが新ゲームプレイと開発の詳細を公開。Windows/Xbox Series X|S向けに2026年内発売予定で、WWE Triplemania(9月)スポンサードなどから9月発売が有力視される。</t>
+        </is>
+      </c>
+      <c r="F87" s="14" t="inlineStr">
+        <is>
+          <t>The Coalition×People Can Flyの共同開発
+シリーズ原点(本編14年前)を描くナンバリング第6作
+2026年内発売、9月有力
+Windows/Xbox Series X|S対応
+25周年の目玉タイトル</t>
+        </is>
+      </c>
+      <c r="G87" s="14" t="inlineStr">
+        <is>
+          <t>Xboxの年末商戦の核として期待。Game Pass Day1配信が見込まれ、ハード牽引よりサブスク会員維持・獲得の指標として注目される。</t>
+        </is>
+      </c>
+      <c r="H87" s="14" t="inlineStr">
+        <is>
+          <t>看板IPのリブートとサブスク同梱戦略</t>
+        </is>
+      </c>
+      <c r="I87" s="14" t="inlineStr">
+        <is>
+          <t>Microsoft,The Coalition,People Can Fly</t>
+        </is>
+      </c>
+      <c r="J87" s="14" t="inlineStr">
+        <is>
+          <t>Gears of War</t>
+        </is>
+      </c>
+      <c r="K87" s="14" t="inlineStr">
+        <is>
+          <t>新作,海外</t>
+        </is>
+      </c>
+      <c r="L87" s="14" t="inlineStr">
+        <is>
+          <t>E-Day Direct(6/7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B88" s="14" t="inlineStr">
+        <is>
+          <t>PC Gaming Show 2026開催、50本超・20本以上の世界初公開——Control続編やExodus新情報</t>
+        </is>
+      </c>
+      <c r="C88" s="14" t="inlineStr">
+        <is>
+          <t>https://www.pcgamer.com/gaming-industry/events-conferences/pc-gaming-show-2026-how-to-watch/</t>
+        </is>
+      </c>
+      <c r="D88" s="14" t="inlineStr">
+        <is>
+          <t>PCゲームに特化したショーケースとして定着したPC Gaming Showが、SGF期間中の6/7に開催。インディーから中堅まで幅広いPCタイトルの発表枠として機能している。</t>
+        </is>
+      </c>
+      <c r="E88" s="14" t="inlineStr">
+        <is>
+          <t>6/7午後にPC Gaming Show 2026を配信し、50本超のPCゲーム・20本以上の世界初公開を実施。Remedyの『Control Resonant』(9/24発売)、SF RPG『Exodus』の拡張ゲームプレイ、『Stronghold』新作、Game Freakの『Beast of Reincarnation』(8/4)などが並んだ。</t>
+        </is>
+      </c>
+      <c r="F88" s="14" t="inlineStr">
+        <is>
+          <t>PCタイトル50本超・世界初公開20本以上
+『Control Resonant』9/24発売
+『Exodus』拡張ゲームプレイ公開
+『Stronghold』新作を初披露
+Game Freak『Beast of Reincarnation』8/4</t>
+        </is>
+      </c>
+      <c r="G88" s="14" t="inlineStr">
+        <is>
+          <t>PC市場の新作供給は中堅・インディーが牽引。Steam同接とウィッシュリストの初動が今後の販売を占う指標になり、発表直後の体験版配信が定石化する。</t>
+        </is>
+      </c>
+      <c r="H88" s="14" t="inlineStr">
+        <is>
+          <t>PC特化ショーケースとインディー発見戦略</t>
+        </is>
+      </c>
+      <c r="I88" s="14" t="inlineStr">
+        <is>
+          <t>Remedy,Game Freak</t>
+        </is>
+      </c>
+      <c r="J88" s="14" t="inlineStr">
+        <is>
+          <t>Control,Exodus,Stronghold,Beast of Reincarnation</t>
+        </is>
+      </c>
+      <c r="K88" s="14" t="inlineStr">
+        <is>
+          <t>新作,海外,PC</t>
+        </is>
+      </c>
+      <c r="L88" s="14" t="inlineStr">
+        <is>
+          <t>6/7配信</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B89" s="14" t="inlineStr">
+        <is>
+          <t>6/7はインディー系ショーケースも集中、Future Games Show等で新作多数・日本語対応も発表</t>
+        </is>
+      </c>
+      <c r="C89" s="14" t="inlineStr">
+        <is>
+          <t>https://news.denfaminicogamer.jp/news/260606b</t>
+        </is>
+      </c>
+      <c r="D89" s="14" t="inlineStr">
+        <is>
+          <t>SGF期間はメジャー発表会だけでなく、テーマ特化型の小規模ショーケースが連続開催される。6/7はStory-Rich Showcase、Green Games Showcase、Future Games Showなどが集中した。</t>
+        </is>
+      </c>
+      <c r="E89" s="14" t="inlineStr">
+        <is>
+          <t>6/7に複数のインディー/特化型ショーケースが開催され、Future Games Showは40本・世界初公開10本を披露。猫風クラフト村づくり『Tinkernest』や農業シムRPG『Fields of Mistria』の日本語対応など、国内ユーザー向け情報も発表された。</t>
+        </is>
+      </c>
+      <c r="F89" s="14" t="inlineStr">
+        <is>
+          <t>Future Games Showで40本・世界初公開10本
+Story-Rich/Green Gamesなど特化型が並走
+『Tinkernest』など新作インディー公開
+『Fields of Mistria』日本語対応
+国内向けローカライズ情報も拡充</t>
+        </is>
+      </c>
+      <c r="G89" s="14" t="inlineStr">
+        <is>
+          <t>特化型ショーケースはニッチ層への到達効率が高く、ジャンル別の発見チャネルとして定着。日本語対応の同時告知が国内初動の底上げに寄与する。</t>
+        </is>
+      </c>
+      <c r="H89" s="14" t="inlineStr">
+        <is>
+          <t>テーマ特化ショーケースとローカライズ戦略</t>
+        </is>
+      </c>
+      <c r="I89" s="14" t="inlineStr">
+        <is>
+          <t>なし(複数インディー)</t>
+        </is>
+      </c>
+      <c r="J89" s="14" t="inlineStr">
+        <is>
+          <t>Tinkernest,Fields of Mistria</t>
+        </is>
+      </c>
+      <c r="K89" s="14" t="inlineStr">
+        <is>
+          <t>新作,インディー,海外</t>
+        </is>
+      </c>
+      <c r="L89" s="14" t="inlineStr">
+        <is>
+          <t>6/7複数配信</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B90" s="14" t="inlineStr">
+        <is>
+          <t>CS2『IEM Cologne Major 2026』Stage 2進行中、BIGがNRGに12:0からの大逆転で通過</t>
+        </is>
+      </c>
+      <c r="C90" s="14" t="inlineStr">
+        <is>
+          <t>https://escharts.com/news/iem-cologne-major-stage1-results</t>
+        </is>
+      </c>
+      <c r="D90" s="14" t="inlineStr">
+        <is>
+          <t>Counter-Strike 2の今季メジャー。賞金総額125万ドル、6/2〜6/21にドイツ・ケルンで開催され、Stage 1(6/2〜5)を勝ち上がった8チームが6/6〜9のStage 2へ進んだ。</t>
+        </is>
+      </c>
+      <c r="E90" s="14" t="inlineStr">
+        <is>
+          <t>Stage 1ではBetBoom・B8が3-0で突破、計8チーム(BetBoom/B8/GamerLegion/MIBR/M80/TYLOO/FlyQuest/BIG)がStage 2入り。BIGは決勝マップで12:0の劣勢から逆転しNRGを2-1で破り最後の枠を確保。LiquidやHEROICは敗退した。</t>
+        </is>
+      </c>
+      <c r="F90" s="14" t="inlineStr">
+        <is>
+          <t>賞金125万ドル・優勝50万ドル
+Stage 1突破8チームが確定
+BIGがNRG相手に12:0から大逆転
+Liquid/HEROICが敗退
+Stage 2は6/9まで継続</t>
+        </is>
+      </c>
+      <c r="G90" s="14" t="inlineStr">
+        <is>
+          <t>上位の地力差が明確化する一方、下位帯の番狂わせが視聴の起点に。スイス式の緊張感が同接を支え、メジャーの放映価値を底上げする。</t>
+        </is>
+      </c>
+      <c r="H90" s="14" t="inlineStr">
+        <is>
+          <t>eスポーツメジャーの大会フォーマットと視聴維持</t>
+        </is>
+      </c>
+      <c r="I90" s="14" t="inlineStr">
+        <is>
+          <t>ESL,Intel,BIG,NRG</t>
+        </is>
+      </c>
+      <c r="J90" s="14" t="inlineStr">
+        <is>
+          <t>Counter-Strike 2</t>
+        </is>
+      </c>
+      <c r="K90" s="14" t="inlineStr">
+        <is>
+          <t>eスポーツ,海外</t>
+        </is>
+      </c>
+      <c r="L90" s="14" t="inlineStr">
+        <is>
+          <t>Stage 2(6/6-9)</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B91" s="14" t="inlineStr">
+        <is>
+          <t>『VALORANT Masters London 2026』スイスステージ進行、賞金100万ドルの国際大会が佳境</t>
+        </is>
+      </c>
+      <c r="C91" s="14" t="inlineStr">
+        <is>
+          <t>https://www.vlr.gg/event/2765/valorant-masters-london-2026</t>
+        </is>
+      </c>
+      <c r="D91" s="14" t="inlineStr">
+        <is>
+          <t>VALORANT Champions Tour(VCT)2026 Stage 2の国際大会として、ロンドンで開催。賞金総額100万ドルで、各地域リーグ上位チームが集結する年間最重要級イベントの一つ。</t>
+        </is>
+      </c>
+      <c r="E91" s="14" t="inlineStr">
+        <is>
+          <t>6/6開幕のMasters Londonはスイスステージ(6/10まで)に突入し、6/7はFULL SENSE対FUT Esports、LEVIATÁN対Global EsportsなどRound 1のBo3が組まれた。CS2のIEM Cologneと並び、6月のeスポーツ大型大会ラッシュを象徴する。</t>
+        </is>
+      </c>
+      <c r="F91" s="14" t="inlineStr">
+        <is>
+          <t>VCT 2026 Stage 2のMastersをロンドン開催
+賞金総額100万ドル
+スイスステージは6/10まで
+6/7に複数のBo3を実施
+CS2メジャーと時期が重なり大会ラッシュ</t>
+        </is>
+      </c>
+      <c r="G91" s="14" t="inlineStr">
+        <is>
+          <t>複数タイトルのメジャーが同時期に集中し、視聴者の可処分時間を奪い合う構図。配信枠の取り合いとコ・ストリーミングの扱いが収益面の論点になる。</t>
+        </is>
+      </c>
+      <c r="H91" s="14" t="inlineStr">
+        <is>
+          <t>国際eスポーツ大会の同時多発と視聴争奪</t>
+        </is>
+      </c>
+      <c r="I91" s="14" t="inlineStr">
+        <is>
+          <t>Riot Games</t>
+        </is>
+      </c>
+      <c r="J91" s="14" t="inlineStr">
+        <is>
+          <t>VALORANT</t>
+        </is>
+      </c>
+      <c r="K91" s="14" t="inlineStr">
+        <is>
+          <t>eスポーツ,海外</t>
+        </is>
+      </c>
+      <c r="L91" s="14" t="inlineStr">
+        <is>
+          <t>スイスステージ(6/7)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
daily-news + cross-questions update (2026-06-07 22:50)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -2477,7 +2477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3155,6 +3155,80 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B19" s="14" t="inlineStr">
+        <is>
+          <t>プラットフォーマーが“独占”へ回帰する動き(Xboxのコンソール専売再強化)は、動画配信・通信の独占コンテンツ囲い込み戦略の何に対応するか？</t>
+        </is>
+      </c>
+      <c r="C19" s="14" t="inlineStr">
+        <is>
+          <t>Xbox Games Showcase 2026でGears E-Day/Clockwork Revolutionを時限ではないコンソール専売と明言</t>
+        </is>
+      </c>
+      <c r="D19" s="14" t="inlineStr">
+        <is>
+          <t>Microsoft, Xbox</t>
+        </is>
+      </c>
+      <c r="E19" s="14" t="inlineStr">
+        <is>
+          <t>動画配信(独占作品競争), 通信(端末/回線囲い込み), 音楽サブスク</t>
+        </is>
+      </c>
+      <c r="F19" s="14" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="G19" s="14" t="inlineStr">
+        <is>
+          <t>マルチ展開で裾野を広げた後に独占で“城”を築き直す揺り戻し。配信・通信の独占×開放の振り子と同じ構造かを検証したい。</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B20" s="14" t="inlineStr">
+        <is>
+          <t>周年記念の半透明・限定復刻ハード(Xbox 25周年 Series X25)による収集需要喚起は、自動車・家電・スニーカー等の限定復刻商法と同じ収益構造か？</t>
+        </is>
+      </c>
+      <c r="C20" s="14" t="inlineStr">
+        <is>
+          <t>Xbox 25周年で初代インスパイアの半透明Series X25 Limited Editionを発表</t>
+        </is>
+      </c>
+      <c r="D20" s="14" t="inlineStr">
+        <is>
+          <t>Microsoft, Xbox</t>
+        </is>
+      </c>
+      <c r="E20" s="14" t="inlineStr">
+        <is>
+          <t>自動車(記念限定車), 家電(復刻デザイン), アパレル/スニーカー(限定復刻)</t>
+        </is>
+      </c>
+      <c r="F20" s="14" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="G20" s="14" t="inlineStr">
+        <is>
+          <t>機能差が小さい成熟プロダクトで“ノスタルジア×希少性”を価格に転嫁する手法。耐久財/嗜好品の周年商法と接続できるか。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3166,7 +3240,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L91"/>
+  <dimension ref="A1:L99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8967,6 +9041,526 @@
       <c r="L91" s="14" t="inlineStr">
         <is>
           <t>スイスステージ(6/7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B92" s="14" t="inlineStr">
+        <is>
+          <t>Xbox Games Showcase 2026開催、ブランド25周年で“独占回帰”——Halo再始動・Gears E-Day・Fable・P4Rを一挙公開</t>
+        </is>
+      </c>
+      <c r="C92" s="14" t="inlineStr">
+        <is>
+          <t>https://news.xbox.com/en-us/2026/06/07/xbox-games-showcase-2026-recap-everything-announced/</t>
+        </is>
+      </c>
+      <c r="D92" s="14" t="inlineStr">
+        <is>
+          <t>近年マルチプラットフォーム戦略を強めていたXboxが、ブランド誕生25周年の節目に大型ショーケースを実施。ハード・サブスク・独占タイトルの方向性に市場の注目が集まっていた。</t>
+        </is>
+      </c>
+      <c r="E92" s="14" t="inlineStr">
+        <is>
+          <t>6/7(米時間)のXbox Games Showcase 2026で、Halo: Campaign Evolved(7/28)、Gears of War: E-Day(10/6・コンソール専売)、Fable(2027/2/27)、Persona 4 Revival(2027/2/18)などを発表。25周年記念に半透明筐体のSeries X25 Limited Editionも公開した。</t>
+        </is>
+      </c>
+      <c r="F92" s="14" t="inlineStr">
+        <is>
+          <t>Gears E-DayとClockwork Revolutionをコンソール“専売”(時限ではない)と明言
+Halo: Campaign Evolvedを7/28発売、7/23から最大5日早期アクセス
+25周年で初代インスパイアの半透明限定ハードを投入
+多数タイトルがGame Pass初日対応</t>
+        </is>
+      </c>
+      <c r="G92" s="14" t="inlineStr">
+        <is>
+          <t>マルチ展開とハード独占を併用する“ハイブリッド”戦略が鮮明に。Game Pass加入導線を独占新作で太らせつつ、周年限定ハードでコレクター需要も取りにいく。年末商戦に向けGears/Haloの実機評価が試金石。</t>
+        </is>
+      </c>
+      <c r="H92" s="14" t="inlineStr">
+        <is>
+          <t>プラットフォーム独占とサブスク経済の両立戦略</t>
+        </is>
+      </c>
+      <c r="I92" s="14" t="inlineStr">
+        <is>
+          <t>Microsoft, Xbox, Halo Studios, The Coalition, Atlus</t>
+        </is>
+      </c>
+      <c r="J92" s="14" t="inlineStr">
+        <is>
+          <t>Halo, Gears of War, Fable, Persona 4</t>
+        </is>
+      </c>
+      <c r="K92" s="14" t="inlineStr">
+        <is>
+          <t>新作,海外</t>
+        </is>
+      </c>
+      <c r="L92" s="14" t="inlineStr">
+        <is>
+          <t>25周年記念ショーケース</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B93" s="14" t="inlineStr">
+        <is>
+          <t>『ストリートファイター6』Year 4にFF7『ティファ』参戦——マテリア等“FF”由来システムも実装(SGF2026)</t>
+        </is>
+      </c>
+      <c r="C93" s="14" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/article/202606/77238</t>
+        </is>
+      </c>
+      <c r="D93" s="14" t="inlineStr">
+        <is>
+          <t>カプコンは対戦格闘『スト6』を長期運営タイトルとして拡張中。コラボキャラ投入でプレイヤー層拡大とeスポーツ盛り上げを図っている。</t>
+        </is>
+      </c>
+      <c r="E93" s="14" t="inlineStr">
+        <is>
+          <t>Summer Game Fest 2026で『スト6』Year 4の新キャラ4名を公開。『FF7』のティファが参戦し、マテリアや“FFを象徴するシステム”を再現する独自要素が実装される。</t>
+        </is>
+      </c>
+      <c r="F93" s="14" t="inlineStr">
+        <is>
+          <t>FF7ティファを格闘ゲームに落とし込みマテリア要素を導入
+Year 4で計4キャラを順次追加
+国内人気IPコラボでカジュアル層を取り込み
+eスポーツ競技シーンの話題性も底上げ</t>
+        </is>
+      </c>
+      <c r="G93" s="14" t="inlineStr">
+        <is>
+          <t>人気RPG IPを格闘ゲームへ移植する“クロスIP”施策が定着。長期運営型タイトルは新規キャラのコラボ性が課金とプレイ継続の鍵になり、スクエニ×カプコンの相互送客が進む可能性。</t>
+        </is>
+      </c>
+      <c r="H93" s="14" t="inlineStr">
+        <is>
+          <t>長期運営型タイトルのコラボ設計と相互送客</t>
+        </is>
+      </c>
+      <c r="I93" s="14" t="inlineStr">
+        <is>
+          <t>カプコン, スクウェア・エニックス</t>
+        </is>
+      </c>
+      <c r="J93" s="14" t="inlineStr">
+        <is>
+          <t>ストリートファイター6, ファイナルファンタジーVII</t>
+        </is>
+      </c>
+      <c r="K93" s="14" t="inlineStr">
+        <is>
+          <t>新作,国内</t>
+        </is>
+      </c>
+      <c r="L93" s="14" t="inlineStr">
+        <is>
+          <t>Year 4新キャラ発表</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B94" s="14" t="inlineStr">
+        <is>
+          <t>スクエニ、FF7リメイク三部作の完結編『FINAL FANTASY VII REVELATION』を発表(SGF2026)</t>
+        </is>
+      </c>
+      <c r="C94" s="14" t="inlineStr">
+        <is>
+          <t>https://www.tomsguide.com/news/live/summer-game-fest-2026-live-updates</t>
+        </is>
+      </c>
+      <c r="D94" s="14" t="inlineStr">
+        <is>
+          <t>FF7リメイクは『リメイク』『リバース』に続く三部作構想で進行。完結編の正式タイトルとお披露目が長く待たれていた。</t>
+        </is>
+      </c>
+      <c r="E94" s="14" t="inlineStr">
+        <is>
+          <t>Summer Game Fest 2026で、FF7リメイク三部作の最終作タイトルが『FINAL FANTASY VII REVELATION』として明らかになった。シリーズの集大成として世界的に注目を集めている。</t>
+        </is>
+      </c>
+      <c r="F94" s="14" t="inlineStr">
+        <is>
+          <t>三部作完結編の正式タイトルを初公開
+スクエニの旗艦RPGとして世界市場を狙う
+PS主導の展開とマルチ化動向に注目
+長期開発IPの収益回収フェーズ入り</t>
+        </is>
+      </c>
+      <c r="G94" s="14" t="inlineStr">
+        <is>
+          <t>スクエニにとってFF7三部作の完結はロイヤリティ・パッケージ収益の山場。発売プラットフォームと時期次第で同社の通期業績を左右し、関連グッズ・サントラ等の二次収益も拡大が見込まれる。</t>
+        </is>
+      </c>
+      <c r="H94" s="14" t="inlineStr">
+        <is>
+          <t>三部作IPの完結と収益回収サイクル</t>
+        </is>
+      </c>
+      <c r="I94" s="14" t="inlineStr">
+        <is>
+          <t>スクウェア・エニックス, ソニー</t>
+        </is>
+      </c>
+      <c r="J94" s="14" t="inlineStr">
+        <is>
+          <t>ファイナルファンタジーVII リメイク</t>
+        </is>
+      </c>
+      <c r="K94" s="14" t="inlineStr">
+        <is>
+          <t>新作,国内</t>
+        </is>
+      </c>
+      <c r="L94" s="14" t="inlineStr">
+        <is>
+          <t>三部作完結編</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B95" s="14" t="inlineStr">
+        <is>
+          <t>2K/Hangar 13、『Mafia: The Old Country』に拡張「Man of Honor」を発表(SGF2026)</t>
+        </is>
+      </c>
+      <c r="C95" s="14" t="inlineStr">
+        <is>
+          <t>https://theartsshelf.com/2026/06/07/mafia-the-old-country-man-of-honor-expansion-summer-game-fest-2026/</t>
+        </is>
+      </c>
+      <c r="D95" s="14" t="inlineStr">
+        <is>
+          <t>2KのマフィアシリーズはOld Countryで世界観をシチリア前日譚へ刷新。本編後の追加コンテンツ展開が焦点だった。</t>
+        </is>
+      </c>
+      <c r="E95" s="14" t="inlineStr">
+        <is>
+          <t>Summer Game Fest 2026で、2KとHangar 13が『Mafia: The Old Country』の拡張「Man of Honor」を正式発表。本編の世界観を補強するストーリー拡張となる。</t>
+        </is>
+      </c>
+      <c r="F95" s="14" t="inlineStr">
+        <is>
+          <t>シングルプレイ大作に物語拡張DLCを追加
+2K/Hangar 13がIPの長期運用を継続
+プレミアム拡張でLTV最大化を狙う
+コンソール/PCマルチで展開</t>
+        </is>
+      </c>
+      <c r="G95" s="14" t="inlineStr">
+        <is>
+          <t>買い切り大作でも拡張DLCで収益を伸ばす“ポストローンチ”運用が標準化。シングルプレイ重視タイトルでも継続課金導線を設けることで、サービス型ほど摩耗せず追加収益を確保する流れ。</t>
+        </is>
+      </c>
+      <c r="H95" s="14" t="inlineStr">
+        <is>
+          <t>買い切り大作のポストローンチ収益設計</t>
+        </is>
+      </c>
+      <c r="I95" s="14" t="inlineStr">
+        <is>
+          <t>Take-Two, 2K, Hangar 13</t>
+        </is>
+      </c>
+      <c r="J95" s="14" t="inlineStr">
+        <is>
+          <t>Mafia: The Old Country</t>
+        </is>
+      </c>
+      <c r="K95" s="14" t="inlineStr">
+        <is>
+          <t>新作,海外</t>
+        </is>
+      </c>
+      <c r="L95" s="14" t="inlineStr">
+        <is>
+          <t>ストーリー拡張DLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B96" s="14" t="inlineStr">
+        <is>
+          <t>シリーズ再始動『Tomb Raider: Legacy of Atlantis』、新ララ・クロフト声優を起用しSGF2026で前進</t>
+        </is>
+      </c>
+      <c r="C96" s="14" t="inlineStr">
+        <is>
+          <t>https://deadline.com/2026/06/tomb-raider-legacy-of-atlantis-alix-wilton-regan-interview-1236942875/</t>
+        </is>
+      </c>
+      <c r="D96" s="14" t="inlineStr">
+        <is>
+          <t>Crystal Dynamicsが再構築を進めるトゥームレイダー新作は、Amazon主導の映像化も絡む大型IP再起動として動向が注目されていた。</t>
+        </is>
+      </c>
+      <c r="E96" s="14" t="inlineStr">
+        <is>
+          <t>Summer Game Fest 2026で『Tomb Raider: Legacy of Atlantis』が披露され、新ララ・クロフト役のAlix Wilton Reganが“より大胆になった”シリーズ再始動を語った。パフォーマンスキャプチャを駆使する。</t>
+        </is>
+      </c>
+      <c r="F96" s="14" t="inlineStr">
+        <is>
+          <t>象徴的女性主人公IPをリブートし新声優を起用
+パフォーマンスキャプチャで表現を刷新
+映像化(Amazon系)とのメディアミックス
+往年IPの世代更新を狙う</t>
+        </is>
+      </c>
+      <c r="G96" s="14" t="inlineStr">
+        <is>
+          <t>老舗IPの“世代交代型リブート”が活発化。ゲーム・映像・配信を横断するトランスメディア前提のキャスティングと演出投資が進み、IP価値の再評価が収益機会につながる。</t>
+        </is>
+      </c>
+      <c r="H96" s="14" t="inlineStr">
+        <is>
+          <t>老舗IPのリブートとトランスメディア展開</t>
+        </is>
+      </c>
+      <c r="I96" s="14" t="inlineStr">
+        <is>
+          <t>Crystal Dynamics, Amazon</t>
+        </is>
+      </c>
+      <c r="J96" s="14" t="inlineStr">
+        <is>
+          <t>Tomb Raider</t>
+        </is>
+      </c>
+      <c r="K96" s="14" t="inlineStr">
+        <is>
+          <t>新作,海外</t>
+        </is>
+      </c>
+      <c r="L96" s="14" t="inlineStr">
+        <is>
+          <t>シリーズ再始動</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B97" s="14" t="inlineStr">
+        <is>
+          <t>EU AI Act、透明性ルールが2026年8月施行へ——“Digital Omnibus”で一部簡素化、AIゲームは多くが最小リスク扱い</t>
+        </is>
+      </c>
+      <c r="C97" s="14" t="inlineStr">
+        <is>
+          <t>https://www.lexology.com/library/detail.aspx?g=c35fb8c9-f3b3-45a6-a475-1f5c967fe3a9</t>
+        </is>
+      </c>
+      <c r="D97" s="14" t="inlineStr">
+        <is>
+          <t>生成AIの普及で規制整備が進む欧州。AI Actの段階適用がゲーム含むコンテンツ業界の開示・コンプラ負担に直結するため動向が注視されていた。</t>
+        </is>
+      </c>
+      <c r="E97" s="14" t="inlineStr">
+        <is>
+          <t>EU AI Actは透明性関連ルールが2026年8月に発効予定。5/7に欧州議会・理事会が改正案“Digital Omnibus”で暫定合意し、一部規律を簡素化。AI搭載ゲームの多くは“最小/無リスク”区分とされ追加規律の対象外となる見込み。</t>
+        </is>
+      </c>
+      <c r="F97" s="14" t="inlineStr">
+        <is>
+          <t>透明性ルールが2026年8月に発効
+“Digital Omnibus”暫定合意で運用を簡素化
+AIゲームの大半は最小リスク区分で規律外
+クラウド/AIは欧州デジタル主権の中核</t>
+        </is>
+      </c>
+      <c r="G97" s="14" t="inlineStr">
+        <is>
+          <t>規制は“全面強化”ではなく実装容易性を意識した調整局面へ。ゲームのAI利用は当面軽い扱いだが、生成物の表示義務など透明性要件は残るため、グローバル展開企業は開示体制の整備が必要に。</t>
+        </is>
+      </c>
+      <c r="H97" s="14" t="inlineStr">
+        <is>
+          <t>EU AI Actの段階適用と透明性義務</t>
+        </is>
+      </c>
+      <c r="I97" s="14" t="inlineStr">
+        <is>
+          <t>European Commission, European Parliament</t>
+        </is>
+      </c>
+      <c r="J97" s="14" t="inlineStr">
+        <is>
+          <t>EU AI Act</t>
+        </is>
+      </c>
+      <c r="K97" s="14" t="inlineStr">
+        <is>
+          <t>規制,海外</t>
+        </is>
+      </c>
+      <c r="L97" s="14" t="inlineStr">
+        <is>
+          <t>8月施行・改正合意</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B98" s="14" t="inlineStr">
+        <is>
+          <t>ByteDance、モバイル大手Moontonをサウジ系Savvyへ60〜70億ドルで売却交渉が進行中</t>
+        </is>
+      </c>
+      <c r="C98" s="14" t="inlineStr">
+        <is>
+          <t>https://investgame.net/news/digest/7-2026/</t>
+        </is>
+      </c>
+      <c r="D98" s="14" t="inlineStr">
+        <is>
+          <t>サウジPIF系のゲーム投資攻勢が継続。EA買収に続き、中国モバイル資産の大型移管が業界再編の焦点になっている。</t>
+        </is>
+      </c>
+      <c r="E98" s="14" t="inlineStr">
+        <is>
+          <t>ByteDanceが上海のモバイルゲーム開発Moonton Technology(『Mobile Legends』)を、サウジのSavvy Games Groupへ60〜70億ドルで売却する交渉が最終段階にあると報じられた。実現すれば大型クロスボーダー再編となる。</t>
+        </is>
+      </c>
+      <c r="F98" s="14" t="inlineStr">
+        <is>
+          <t>ByteDanceがMoontonを60〜70億ドルで売却交渉
+買い手はサウジ系Savvy Games Group
+Mobile Legends等の人気IPが対象
+EA買収に続くPIF系の攻勢が継続</t>
+        </is>
+      </c>
+      <c r="G98" s="14" t="inlineStr">
+        <is>
+          <t>ソブリンファンドによるモバイルIP集約が加速。地政学・規制審査の壁はあるが、サウジは世界的eスポーツ/モバイル基盤の獲得を狙う。中国テック発のIPが中東マネーへ移る流れが鮮明に。</t>
+        </is>
+      </c>
+      <c r="H98" s="14" t="inlineStr">
+        <is>
+          <t>ソブリンファンドのモバイルIP集約戦略</t>
+        </is>
+      </c>
+      <c r="I98" s="14" t="inlineStr">
+        <is>
+          <t>ByteDance, Savvy Games Group, PIF, Moonton</t>
+        </is>
+      </c>
+      <c r="J98" s="14" t="inlineStr">
+        <is>
+          <t>Mobile Legends: Bang Bang</t>
+        </is>
+      </c>
+      <c r="K98" s="14" t="inlineStr">
+        <is>
+          <t>M&amp;A,海外</t>
+        </is>
+      </c>
+      <c r="L98" s="14" t="inlineStr">
+        <is>
+          <t>売却交渉が最終段階</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B99" s="14" t="inlineStr">
+        <is>
+          <t>『Dead by Daylight』に“ジェイソン”参戦、新チャプターが6/17配信決定——大型ホラーIPコラボでユーザー回帰狙う</t>
+        </is>
+      </c>
+      <c r="C99" s="14" t="inlineStr">
+        <is>
+          <t>https://www.goonhammer.com/games-industry-news-roundup-june-2nd-2026</t>
+        </is>
+      </c>
+      <c r="D99" s="14" t="inlineStr">
+        <is>
+          <t>長期運営の非対称対戦『DbD』はホラーIPコラボで話題を維持。象徴的キャラ参戦の有無がコミュニティの最大関心だった。</t>
+        </is>
+      </c>
+      <c r="E99" s="14" t="inlineStr">
+        <is>
+          <t>非対称対戦ホラー『Dead by Daylight』に『13日の金曜日』の“ジェイソン”が参戦する新チャプターが、2026年6月17日にリリースされると発表された。大型ホラーIPコラボでアクティブユーザーの回帰を図る。</t>
+        </is>
+      </c>
+      <c r="F99" s="14" t="inlineStr">
+        <is>
+          <t>象徴的ホラーIP“ジェイソン”を新チャプターに追加
+6/17配信でユーザー回帰イベント化
+長期運営タイトルのIPコラボ戦略
+配信・クリップ拡散で話題を再点火</t>
+        </is>
+      </c>
+      <c r="G99" s="14" t="inlineStr">
+        <is>
+          <t>ライブサービス型はIPコラボの“瞬間最大風速”で同接とDAUを押し上げる運用が定番化。版権交渉力と話題化のタイミング設計が、運営タイトルの寿命とマネタイズを左右する。</t>
+        </is>
+      </c>
+      <c r="H99" s="14" t="inlineStr">
+        <is>
+          <t>ライブサービスのIPコラボ運用</t>
+        </is>
+      </c>
+      <c r="I99" s="14" t="inlineStr">
+        <is>
+          <t>Behaviour Interactive</t>
+        </is>
+      </c>
+      <c r="J99" s="14" t="inlineStr">
+        <is>
+          <t>Dead by Daylight, Friday the 13th</t>
+        </is>
+      </c>
+      <c r="K99" s="14" t="inlineStr">
+        <is>
+          <t>新作,海外,eスポーツ</t>
+        </is>
+      </c>
+      <c r="L99" s="14" t="inlineStr">
+        <is>
+          <t>6/17新チャプター</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
weekly-stocks + IP watch update (2026-06-08 00:14)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -10643,8 +10643,16 @@
           <t>日本</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr"/>
-      <c r="E11" s="9" t="inlineStr"/>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>SGF2026でモンハンWildsのSwitch 2版開発を確認。大型拡張『Wilds: Ascendance』を2027年世界配信と発表。</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>MH Wilds: Ascendance(2027)、MH Stories 3: Twisted Reflection(2026/3/13)</t>
+        </is>
+      </c>
       <c r="F11" s="9" t="inlineStr"/>
       <c r="G11" s="9" t="inlineStr">
         <is>
@@ -10652,7 +10660,11 @@
         </is>
       </c>
       <c r="H11" s="9" t="inlineStr"/>
-      <c r="I11" s="9" t="inlineStr"/>
+      <c r="I11" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
@@ -10670,8 +10682,16 @@
           <t>日本</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr"/>
-      <c r="E12" s="9" t="inlineStr"/>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>SGF2026でCapcomが関連新作『Resident Evil Veronica』を披露(SGF2026話題作)。</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>Resident Evil新作を継続展開</t>
+        </is>
+      </c>
       <c r="F12" s="9" t="inlineStr"/>
       <c r="G12" s="9" t="inlineStr">
         <is>
@@ -10679,7 +10699,11 @@
         </is>
       </c>
       <c r="H12" s="9" t="inlineStr"/>
-      <c r="I12" s="9" t="inlineStr"/>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
@@ -10697,8 +10721,16 @@
           <t>日本</t>
         </is>
       </c>
-      <c r="D13" s="9" t="inlineStr"/>
-      <c r="E13" s="9" t="inlineStr"/>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>『ストリートファイター6』Switch 2版を2026/6/5発売。Year4キャラ(Tifa, Yasmine, Arjun, Bosch)を展開中。</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>SF6 Year 4 追加キャラ・パス</t>
+        </is>
+      </c>
       <c r="F13" s="9" t="inlineStr"/>
       <c r="G13" s="9" t="inlineStr">
         <is>
@@ -10706,7 +10738,11 @@
         </is>
       </c>
       <c r="H13" s="9" t="inlineStr"/>
-      <c r="I13" s="9" t="inlineStr"/>
+      <c r="I13" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
@@ -10805,8 +10841,16 @@
           <t>日本</t>
         </is>
       </c>
-      <c r="D17" s="9" t="inlineStr"/>
-      <c r="E17" s="9" t="inlineStr"/>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>2026/6/8のXbox Games Showcaseで『ペルソナ6』を正式発表(PS5/Xbox/PC、Game Pass初日対応)。シリーズ30周年。</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>ペルソナ6(時期未定)、ペルソナ4 Revival</t>
+        </is>
+      </c>
       <c r="F17" s="9" t="inlineStr"/>
       <c r="G17" s="9" t="inlineStr">
         <is>
@@ -10814,7 +10858,11 @@
         </is>
       </c>
       <c r="H17" s="9" t="inlineStr"/>
-      <c r="I17" s="9" t="inlineStr"/>
+      <c r="I17" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
@@ -11129,8 +11177,16 @@
           <t>海外</t>
         </is>
       </c>
-      <c r="D29" s="9" t="inlineStr"/>
-      <c r="E29" s="9" t="inlineStr"/>
+      <c r="D29" s="9" t="inlineStr">
+        <is>
+          <t>GTA6の発売日が2026年11月19日に。Piperは初年度3,500万本超を予測、TTWOはFY27に過去最高業績を計画。</t>
+        </is>
+      </c>
+      <c r="E29" s="9" t="inlineStr">
+        <is>
+          <t>Grand Theft Auto VI(2026/11/19予定)</t>
+        </is>
+      </c>
       <c r="F29" s="9" t="inlineStr"/>
       <c r="G29" s="9" t="inlineStr">
         <is>
@@ -11138,7 +11194,11 @@
         </is>
       </c>
       <c r="H29" s="9" t="inlineStr"/>
-      <c r="I29" s="9" t="inlineStr"/>
+      <c r="I29" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
@@ -11453,8 +11513,16 @@
           <t>海外</t>
         </is>
       </c>
-      <c r="D41" s="9" t="inlineStr"/>
-      <c r="E41" s="9" t="inlineStr"/>
+      <c r="D41" s="9" t="inlineStr">
+        <is>
+          <t>Battlefield 6がEA過去最高の年・フランチャイズ各種記録を更新。EAは約$550億での非公開化が進行中。</t>
+        </is>
+      </c>
+      <c r="E41" s="9" t="inlineStr">
+        <is>
+          <t>Battlefield 6のライブ運営継続</t>
+        </is>
+      </c>
       <c r="F41" s="9" t="inlineStr"/>
       <c r="G41" s="9" t="inlineStr">
         <is>
@@ -11462,7 +11530,11 @@
         </is>
       </c>
       <c r="H41" s="9" t="inlineStr"/>
-      <c r="I41" s="9" t="inlineStr"/>
+      <c r="I41" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="9" t="inlineStr">
@@ -11507,8 +11579,16 @@
           <t>海外</t>
         </is>
       </c>
-      <c r="D43" s="9" t="inlineStr"/>
-      <c r="E43" s="9" t="inlineStr"/>
+      <c r="D43" s="9" t="inlineStr">
+        <is>
+          <t>FY26通期で二桁の回復を達成し、EAのNet Bookings過去最高に貢献。</t>
+        </is>
+      </c>
+      <c r="E43" s="9" t="inlineStr">
+        <is>
+          <t>シーズン運営継続</t>
+        </is>
+      </c>
       <c r="F43" s="9" t="inlineStr"/>
       <c r="G43" s="9" t="inlineStr">
         <is>
@@ -11516,7 +11596,11 @@
         </is>
       </c>
       <c r="H43" s="9" t="inlineStr"/>
-      <c r="I43" s="9" t="inlineStr"/>
+      <c r="I43" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="9" t="inlineStr">
@@ -11534,8 +11618,16 @@
           <t>海外</t>
         </is>
       </c>
-      <c r="D44" s="9" t="inlineStr"/>
-      <c r="E44" s="9" t="inlineStr"/>
+      <c r="D44" s="9" t="inlineStr">
+        <is>
+          <t>運営元が新子会社Vantage Studiosへ集約。Tencentが€11.6億を出資(持分26.32%)し開発体制を再編。</t>
+        </is>
+      </c>
+      <c r="E44" s="9" t="inlineStr">
+        <is>
+          <t>Vantage Studios体制で新作開発</t>
+        </is>
+      </c>
       <c r="F44" s="9" t="inlineStr"/>
       <c r="G44" s="9" t="inlineStr">
         <is>
@@ -11543,7 +11635,11 @@
         </is>
       </c>
       <c r="H44" s="9" t="inlineStr"/>
-      <c r="I44" s="9" t="inlineStr"/>
+      <c r="I44" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="9" t="inlineStr">
@@ -11561,8 +11657,16 @@
           <t>海外</t>
         </is>
       </c>
-      <c r="D45" s="9" t="inlineStr"/>
-      <c r="E45" s="9" t="inlineStr"/>
+      <c r="D45" s="9" t="inlineStr">
+        <is>
+          <t>Vantage Studios(Tencent出資26.32%)へ移管され新体制で開発。</t>
+        </is>
+      </c>
+      <c r="E45" s="9" t="inlineStr">
+        <is>
+          <t>Vantage Studios体制で新作開発</t>
+        </is>
+      </c>
       <c r="F45" s="9" t="inlineStr"/>
       <c r="G45" s="9" t="inlineStr">
         <is>
@@ -11570,7 +11674,11 @@
         </is>
       </c>
       <c r="H45" s="9" t="inlineStr"/>
-      <c r="I45" s="9" t="inlineStr"/>
+      <c r="I45" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="9" t="inlineStr">
@@ -11588,8 +11696,16 @@
           <t>海外</t>
         </is>
       </c>
-      <c r="D46" s="9" t="inlineStr"/>
-      <c r="E46" s="9" t="inlineStr"/>
+      <c r="D46" s="9" t="inlineStr">
+        <is>
+          <t>Rainbow Six等を含めVantage Studiosへ集約、Tencentが€11.6億出資。</t>
+        </is>
+      </c>
+      <c r="E46" s="9" t="inlineStr">
+        <is>
+          <t>Rainbow Six等の運営をVantageで継続</t>
+        </is>
+      </c>
       <c r="F46" s="9" t="inlineStr"/>
       <c r="G46" s="9" t="inlineStr">
         <is>
@@ -11597,7 +11713,11 @@
         </is>
       </c>
       <c r="H46" s="9" t="inlineStr"/>
-      <c r="I46" s="9" t="inlineStr"/>
+      <c r="I46" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="9" t="inlineStr">
@@ -11804,8 +11924,16 @@
           <t>海外</t>
         </is>
       </c>
-      <c r="D54" s="9" t="inlineStr"/>
-      <c r="E54" s="9" t="inlineStr"/>
+      <c r="D54" s="9" t="inlineStr">
+        <is>
+          <t>5〜8歳向け『Roblox Kids』・9〜15歳向け『Roblox Select』を6月初に展開。年齢確認強化で短期のユーザー成長に摩擦も、Q1売上は$1.4bn(+39%)。</t>
+        </is>
+      </c>
+      <c r="E54" s="9" t="inlineStr">
+        <is>
+          <t>年齢別アカウント・安全機能の拡充</t>
+        </is>
+      </c>
       <c r="F54" s="9" t="inlineStr"/>
       <c r="G54" s="9" t="inlineStr">
         <is>
@@ -11813,7 +11941,11 @@
         </is>
       </c>
       <c r="H54" s="9" t="inlineStr"/>
-      <c r="I54" s="9" t="inlineStr"/>
+      <c r="I54" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="9" t="inlineStr">
@@ -11885,8 +12017,16 @@
           <t>海外/韓国</t>
         </is>
       </c>
-      <c r="D57" s="9" t="inlineStr"/>
-      <c r="E57" s="9" t="inlineStr"/>
+      <c r="D57" s="9" t="inlineStr">
+        <is>
+          <t>フランチャイズの成長継続でNexonの直近四半期業績に貢献。</t>
+        </is>
+      </c>
+      <c r="E57" s="9" t="inlineStr">
+        <is>
+          <t>季節アップデート・地域展開継続</t>
+        </is>
+      </c>
       <c r="F57" s="9" t="inlineStr"/>
       <c r="G57" s="9" t="inlineStr">
         <is>
@@ -11894,7 +12034,11 @@
         </is>
       </c>
       <c r="H57" s="9" t="inlineStr"/>
-      <c r="I57" s="9" t="inlineStr"/>
+      <c r="I57" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="9" t="inlineStr">
@@ -12063,20 +12207,48 @@
       <c r="E2" s="9" t="inlineStr"/>
       <c r="F2" s="9" t="inlineStr"/>
       <c r="G2" s="9" t="inlineStr"/>
-      <c r="H2" s="9" t="inlineStr"/>
+      <c r="H2" s="9" t="inlineStr">
+        <is>
+          <t>27.9（予想）</t>
+        </is>
+      </c>
       <c r="I2" s="9" t="inlineStr"/>
       <c r="J2" s="9" t="inlineStr"/>
-      <c r="K2" s="9" t="inlineStr"/>
+      <c r="K2" s="9" t="inlineStr">
+        <is>
+          <t>2.15（予想）</t>
+        </is>
+      </c>
       <c r="L2" s="9" t="inlineStr">
         <is>
           <t>Switch/マリオ/ゼルダ/ポケモン</t>
         </is>
       </c>
-      <c r="M2" s="9" t="inlineStr"/>
-      <c r="N2" s="9" t="inlineStr"/>
-      <c r="O2" s="9" t="inlineStr"/>
-      <c r="P2" s="9" t="inlineStr"/>
-      <c r="Q2" s="9" t="inlineStr"/>
+      <c r="M2" s="9" t="inlineStr">
+        <is>
+          <t>Switch 2発売後初の通期。5/8にFY26/3決算発表。株価は決算を挟み上下し6月初は7,600円前後、6/5時点で予想PER27.9倍・予想配当利回り2.15%。Summer Game Fest 2026でモンハンWildsのSwitch 2版開発が確認され同社ソフト供給期待が高まる。</t>
+        </is>
+      </c>
+      <c r="N2" s="9" t="inlineStr">
+        <is>
+          <t>Switch 2立ち上がり期の強力IP群、ソフト牽引力</t>
+        </is>
+      </c>
+      <c r="O2" s="9" t="inlineStr">
+        <is>
+          <t>端末移行期の費用増・ハード普及ペース不透明</t>
+        </is>
+      </c>
+      <c r="P2" s="9" t="inlineStr">
+        <is>
+          <t>Switch 2普及とファーストパーティ大型タイトル供給</t>
+        </is>
+      </c>
+      <c r="Q2" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
@@ -12107,11 +12279,31 @@
           <t>PlayStation/PS+/Bungie</t>
         </is>
       </c>
-      <c r="M3" s="9" t="inlineStr"/>
-      <c r="N3" s="9" t="inlineStr"/>
-      <c r="O3" s="9" t="inlineStr"/>
-      <c r="P3" s="9" t="inlineStr"/>
-      <c r="Q3" s="9" t="inlineStr"/>
+      <c r="M3" s="9" t="inlineStr">
+        <is>
+          <t>6/1の株価は3,562円(+3.43%)。来期会社計画は売上12.3兆円・営業益1.6兆円と増益基調。半導体・金融含むグループ全体は堅調で、ゲーム(G&amp;NS)はPS5後半サイクルとネットワークサービスが軸。</t>
+        </is>
+      </c>
+      <c r="N3" s="9" t="inlineStr">
+        <is>
+          <t>PS5インストールベースとネットワーク課金、IP・映像横展開</t>
+        </is>
+      </c>
+      <c r="O3" s="9" t="inlineStr">
+        <is>
+          <t>ハード成熟でハード収益鈍化、大型新規IPの不在感</t>
+        </is>
+      </c>
+      <c r="P3" s="9" t="inlineStr">
+        <is>
+          <t>次世代機戦略・Bungie等スタジオの新作と live service立て直し</t>
+        </is>
+      </c>
+      <c r="Q3" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
@@ -12142,11 +12334,31 @@
           <t>モンハン/バイオ/ストリートファイター</t>
         </is>
       </c>
-      <c r="M4" s="9" t="inlineStr"/>
-      <c r="N4" s="9" t="inlineStr"/>
-      <c r="O4" s="9" t="inlineStr"/>
-      <c r="P4" s="9" t="inlineStr"/>
-      <c r="Q4" s="9" t="inlineStr"/>
+      <c r="M4" s="9" t="inlineStr">
+        <is>
+          <t>6/3株価2,945円(-2.45%)。5/13発表のFY26/3決算は経常益前期比+12%で10期連続最高益、1円増配。6/5にSwitch 2版『ストリートファイター6』『祇:Path of the Goddess』発売。SGF2026でモンハンWildsのSwitch 2版と大型拡張『Ascendance』(2027世界配信)を発表。</t>
+        </is>
+      </c>
+      <c r="N4" s="9" t="inlineStr">
+        <is>
+          <t>モンハン/バイオ/SF6の強力IPと10期連続最高益、Switch 2展開で裾野拡大</t>
+        </is>
+      </c>
+      <c r="O4" s="9" t="inlineStr">
+        <is>
+          <t>大型新作端境期の反動、為替感応度</t>
+        </is>
+      </c>
+      <c r="P4" s="9" t="inlineStr">
+        <is>
+          <t>MH Wilds拡張・新規プラットフォーム展開・カタログ販売</t>
+        </is>
+      </c>
+      <c r="Q4" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -12165,9 +12377,21 @@
         </is>
       </c>
       <c r="D5" s="9" t="inlineStr"/>
-      <c r="E5" s="9" t="inlineStr"/>
-      <c r="F5" s="9" t="inlineStr"/>
-      <c r="G5" s="9" t="inlineStr"/>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>2,976.61億（FY26/3）</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>547.36億（FY26/3）</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>296.16億（FY26/3）</t>
+        </is>
+      </c>
       <c r="H5" s="9" t="inlineStr"/>
       <c r="I5" s="9" t="inlineStr"/>
       <c r="J5" s="9" t="inlineStr"/>
@@ -12177,11 +12401,31 @@
           <t>FF/ドラクエ/キングダムハーツ</t>
         </is>
       </c>
-      <c r="M5" s="9" t="inlineStr"/>
-      <c r="N5" s="9" t="inlineStr"/>
-      <c r="O5" s="9" t="inlineStr"/>
-      <c r="P5" s="9" t="inlineStr"/>
-      <c r="Q5" s="9" t="inlineStr"/>
+      <c r="M5" s="9" t="inlineStr">
+        <is>
+          <t>6/5株価2,518.5円(+1.61%)。FY26/3は売上2,976.61億(前期比-8.3%)も営業益547.36億(+34.9%)・純益296.16億(+21.3%)と構造改革で増益。FY27/3は売上横ばい・営業益490億(-10.5%)の保守的計画。HDゲーム選別と開発効率化が継続テーマ。</t>
+        </is>
+      </c>
+      <c r="N5" s="9" t="inlineStr">
+        <is>
+          <t>不採算整理による収益性改善、FF/DQ等基幹IP</t>
+        </is>
+      </c>
+      <c r="O5" s="9" t="inlineStr">
+        <is>
+          <t>新作本数減で売上トップライン縮小、ヒット依存</t>
+        </is>
+      </c>
+      <c r="P5" s="9" t="inlineStr">
+        <is>
+          <t>マルチプラットフォーム戦略と次期大型タイトルの成否</t>
+        </is>
+      </c>
+      <c r="Q5" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
@@ -12200,9 +12444,21 @@
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr"/>
-      <c r="E6" s="9" t="inlineStr"/>
-      <c r="F6" s="9" t="inlineStr"/>
-      <c r="G6" s="9" t="inlineStr"/>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>4,936億（FY26/3）</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>1,358億（FY26/3）</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>1,000.1億（FY26/3）</t>
+        </is>
+      </c>
       <c r="H6" s="9" t="inlineStr"/>
       <c r="I6" s="9" t="inlineStr"/>
       <c r="J6" s="9" t="inlineStr"/>
@@ -12212,11 +12468,31 @@
           <t>eFootball/パワプロ/遊戯王</t>
         </is>
       </c>
-      <c r="M6" s="9" t="inlineStr"/>
-      <c r="N6" s="9" t="inlineStr"/>
-      <c r="O6" s="9" t="inlineStr"/>
-      <c r="P6" s="9" t="inlineStr"/>
-      <c r="Q6" s="9" t="inlineStr"/>
+      <c r="M6" s="9" t="inlineStr">
+        <is>
+          <t>FY26/3は売上4,936億(+17.1%)・営業益1,358億(+33.3%)・純益1,000億(+33.9%)で3期連続最高益。デジタルエンタメが+21.5%と牽引。年間配当221.5円(前期165.5円から増配)、次期224円予想。eFootball/遊戯王/パワプロが堅調。</t>
+        </is>
+      </c>
+      <c r="N6" s="9" t="inlineStr">
+        <is>
+          <t>デジタルエンタメ高成長と3期連続最高益、安定したIP課金</t>
+        </is>
+      </c>
+      <c r="O6" s="9" t="inlineStr">
+        <is>
+          <t>アミューズメント/遊技機の構造的逆風</t>
+        </is>
+      </c>
+      <c r="P6" s="9" t="inlineStr">
+        <is>
+          <t>遊戯王・eFootballのグローバル課金とスポーツ事業</t>
+        </is>
+      </c>
+      <c r="Q6" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
@@ -12235,9 +12511,21 @@
         </is>
       </c>
       <c r="D7" s="9" t="inlineStr"/>
-      <c r="E7" s="9" t="inlineStr"/>
-      <c r="F7" s="9" t="inlineStr"/>
-      <c r="G7" s="9" t="inlineStr"/>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>1兆3,482億（FY26/3）</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>1,895億（FY26/3）</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>1,406億（FY26/3）</t>
+        </is>
+      </c>
       <c r="H7" s="9" t="inlineStr"/>
       <c r="I7" s="9" t="inlineStr"/>
       <c r="J7" s="9" t="inlineStr"/>
@@ -12247,11 +12535,31 @@
           <t>アイマス/鉄拳/ガンダム/ドラゴンボール</t>
         </is>
       </c>
-      <c r="M7" s="9" t="inlineStr"/>
-      <c r="N7" s="9" t="inlineStr"/>
-      <c r="O7" s="9" t="inlineStr"/>
-      <c r="P7" s="9" t="inlineStr"/>
-      <c r="Q7" s="9" t="inlineStr"/>
+      <c r="M7" s="9" t="inlineStr">
+        <is>
+          <t>5/13発表のFY26/3は売上1兆3,482億(+8.6%)・営業益1,895億(+5.2%)・純益1,406億(+8.8%)で過去最高更新。トイホビー好調とアミューズ回復が寄与。6/3に日系中堅証券が中立据置・目標株価4,130円へ引き下げ。株価は6/3で3,722円。</t>
+        </is>
+      </c>
+      <c r="N7" s="9" t="inlineStr">
+        <is>
+          <t>IP軸トイホビー＋ゲームの複合収益、過去最高業績</t>
+        </is>
+      </c>
+      <c r="O7" s="9" t="inlineStr">
+        <is>
+          <t>目標株価引き下げ、ゲーム大型新作の端境期</t>
+        </is>
+      </c>
+      <c r="P7" s="9" t="inlineStr">
+        <is>
+          <t>ガンダム/アイマス等IPの世界展開と新作投入ペース</t>
+        </is>
+      </c>
+      <c r="Q7" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
@@ -12282,11 +12590,31 @@
           <t>ペルソナ/龍が如く/ソニック/アトラス</t>
         </is>
       </c>
-      <c r="M8" s="9" t="inlineStr"/>
-      <c r="N8" s="9" t="inlineStr"/>
-      <c r="O8" s="9" t="inlineStr"/>
-      <c r="P8" s="9" t="inlineStr"/>
-      <c r="Q8" s="9" t="inlineStr"/>
+      <c r="M8" s="9" t="inlineStr">
+        <is>
+          <t>6/4株価2,357.5円(-0.11%)。前期は増収(+13.6%)も営業益は2期連続減益傾向。FY27/3は増収減益計画で、遊技機は原価増、ゲーミングは先行投資で損失幅拡大見込み。エンタメは新作投入と販売体制強化で成長狙う。6/8にアトラスが『ペルソナ6』を正式発表。</t>
+        </is>
+      </c>
+      <c r="N8" s="9" t="inlineStr">
+        <is>
+          <t>ペルソナ/龍が如く/ソニック等グローバルIP、ペルソナ30周年</t>
+        </is>
+      </c>
+      <c r="O8" s="9" t="inlineStr">
+        <is>
+          <t>遊技機原価高・ゲーミング先行投資で減益計画</t>
+        </is>
+      </c>
+      <c r="P8" s="9" t="inlineStr">
+        <is>
+          <t>ペルソナ6を含む新作パイプラインと海外展開</t>
+        </is>
+      </c>
+      <c r="Q8" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
@@ -12305,23 +12633,55 @@
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr"/>
-      <c r="E9" s="9" t="inlineStr"/>
-      <c r="F9" s="9" t="inlineStr"/>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>883.93億（FY26/3）</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>371.68億（FY26/3）</t>
+        </is>
+      </c>
       <c r="G9" s="9" t="inlineStr"/>
       <c r="H9" s="9" t="inlineStr"/>
       <c r="I9" s="9" t="inlineStr"/>
       <c r="J9" s="9" t="inlineStr"/>
-      <c r="K9" s="9" t="inlineStr"/>
+      <c r="K9" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="L9" s="9" t="inlineStr">
         <is>
           <t>信長の野望/三國志/仁王</t>
         </is>
       </c>
-      <c r="M9" s="9" t="inlineStr"/>
-      <c r="N9" s="9" t="inlineStr"/>
-      <c r="O9" s="9" t="inlineStr"/>
-      <c r="P9" s="9" t="inlineStr"/>
-      <c r="Q9" s="9" t="inlineStr"/>
+      <c r="M9" s="9" t="inlineStr">
+        <is>
+          <t>FY26/3は売上883.93億(+6.3%)・営業益371.68億(+15.7%)で売上・経常・純益とも過去最高。大型新作含む新作が寄与。FY27/3は人的資本投資増で経常益420億(-26.3%)とアナリスト予想下回る減益計画。配当は当期66円・次期48円予想。</t>
+        </is>
+      </c>
+      <c r="N9" s="9" t="inlineStr">
+        <is>
+          <t>無双/三國志等IPと高い営業利益率、過去最高更新</t>
+        </is>
+      </c>
+      <c r="O9" s="9" t="inlineStr">
+        <is>
+          <t>次期は投資増で大幅減益計画、市場予想未達</t>
+        </is>
+      </c>
+      <c r="P9" s="9" t="inlineStr">
+        <is>
+          <t>新作投入サイクルと海外/IPコラボ展開</t>
+        </is>
+      </c>
+      <c r="Q9" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
@@ -12340,8 +12700,16 @@
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr"/>
-      <c r="E10" s="9" t="inlineStr"/>
-      <c r="F10" s="9" t="inlineStr"/>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>1,713.69億（FY26/3）</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>222.56億（FY26/3）</t>
+        </is>
+      </c>
       <c r="G10" s="9" t="inlineStr"/>
       <c r="H10" s="9" t="inlineStr"/>
       <c r="I10" s="9" t="inlineStr"/>
@@ -12352,11 +12720,31 @@
           <t>モンスト</t>
         </is>
       </c>
-      <c r="M10" s="9" t="inlineStr"/>
-      <c r="N10" s="9" t="inlineStr"/>
-      <c r="O10" s="9" t="inlineStr"/>
-      <c r="P10" s="9" t="inlineStr"/>
-      <c r="Q10" s="9" t="inlineStr"/>
+      <c r="M10" s="9" t="inlineStr">
+        <is>
+          <t>FY26/3は売上1,713.69億(+10.7%)も営業益222.56億(-16.3%)と減益。スポーツ事業が成長する一方、主力モンストの減収と費用増が重し。FY27/3は売上1,850億(+8.0%)・営業益195億(-12.4%)計画。PointsBet連結化でベッティング拡大。</t>
+        </is>
+      </c>
+      <c r="N10" s="9" t="inlineStr">
+        <is>
+          <t>スポーツ/ベッティング事業の成長、みてね等の多角化</t>
+        </is>
+      </c>
+      <c r="O10" s="9" t="inlineStr">
+        <is>
+          <t>モンストMAU減で中核ゲーム収益が縮小</t>
+        </is>
+      </c>
+      <c r="P10" s="9" t="inlineStr">
+        <is>
+          <t>スポーツ事業の収益化とモンスト再活性化</t>
+        </is>
+      </c>
+      <c r="Q10" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
@@ -12387,11 +12775,31 @@
           <t>釣りスタ/モバイルゲーム</t>
         </is>
       </c>
-      <c r="M11" s="9" t="inlineStr"/>
-      <c r="N11" s="9" t="inlineStr"/>
-      <c r="O11" s="9" t="inlineStr"/>
-      <c r="P11" s="9" t="inlineStr"/>
-      <c r="Q11" s="9" t="inlineStr"/>
+      <c r="M11" s="9" t="inlineStr">
+        <is>
+          <t>5/29株価418円。FY26/6 3Qは売上384.44億(-10.9%)・営業益24.2億(-34.7%)も、為替差益で経常益32.1億(+11.1%)・純益19.1億(+112.4%)と大幅増益。期末配当21.5円へ増配予定。ゲーム/VTuber/IP/DX/投資の5事業を展開。</t>
+        </is>
+      </c>
+      <c r="N11" s="9" t="inlineStr">
+        <is>
+          <t>為替効果で増益、VTuber/IP等多角化</t>
+        </is>
+      </c>
+      <c r="O11" s="9" t="inlineStr">
+        <is>
+          <t>中核ゲーム事業の減収トレンド</t>
+        </is>
+      </c>
+      <c r="P11" s="9" t="inlineStr">
+        <is>
+          <t>新規ゲーム/メタバース・Wright Flyer系の収益化</t>
+        </is>
+      </c>
+      <c r="Q11" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
@@ -12410,8 +12818,16 @@
         </is>
       </c>
       <c r="D12" s="9" t="inlineStr"/>
-      <c r="E12" s="9" t="inlineStr"/>
-      <c r="F12" s="9" t="inlineStr"/>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>1,477億（FY26/3 売上収益）</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>186.94億（FY26/3）</t>
+        </is>
+      </c>
       <c r="G12" s="9" t="inlineStr"/>
       <c r="H12" s="9" t="inlineStr"/>
       <c r="I12" s="9" t="inlineStr"/>
@@ -12422,11 +12838,31 @@
           <t>Pokémon Sleep/モバイル</t>
         </is>
       </c>
-      <c r="M12" s="9" t="inlineStr"/>
-      <c r="N12" s="9" t="inlineStr"/>
-      <c r="O12" s="9" t="inlineStr"/>
-      <c r="P12" s="9" t="inlineStr"/>
-      <c r="Q12" s="9" t="inlineStr"/>
+      <c r="M12" s="9" t="inlineStr">
+        <is>
+          <t>FY26/3は売上収益1,477億(-9.9%)・営業益186.94億(-35.5%)。『ポケポケ(Pokémon TCG Pocket)』初速の反動でゲーム事業が減収減益。ライブストリーミングは黒字転換。5/13株価2,559円(-3.83%)。FY27/3は売上1,540億(+4.3%)・営業益150億(-19.8%)計画。</t>
+        </is>
+      </c>
+      <c r="N12" s="9" t="inlineStr">
+        <is>
+          <t>ポケポケ等任天堂系IP、ライブ配信の黒字化、事業多角化</t>
+        </is>
+      </c>
+      <c r="O12" s="9" t="inlineStr">
+        <is>
+          <t>ポケポケ初速の反動減、ゲーム収益のヒット依存</t>
+        </is>
+      </c>
+      <c r="P12" s="9" t="inlineStr">
+        <is>
+          <t>新規タイトル投入とヘルスケア/スポーツ事業の収益化</t>
+        </is>
+      </c>
+      <c r="Q12" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
@@ -12457,11 +12893,31 @@
           <t>ウマ娘/グランブルー/シャドバ</t>
         </is>
       </c>
-      <c r="M13" s="9" t="inlineStr"/>
-      <c r="N13" s="9" t="inlineStr"/>
-      <c r="O13" s="9" t="inlineStr"/>
-      <c r="P13" s="9" t="inlineStr"/>
-      <c r="Q13" s="9" t="inlineStr"/>
+      <c r="M13" s="9" t="inlineStr">
+        <is>
+          <t>FY26/9 2Q累計は売上4,785億(+14%)・純益273億(+72%)。ゲーム事業営業益は約2倍の385億で『ウマ娘』英語版ヒットが寄与し海外売上は前年比3.5倍(131億)。6/4株価1,381円(3か月で+12.4%)。通期は売上+1%・純益250〜300億見込み。</t>
+        </is>
+      </c>
+      <c r="N13" s="9" t="inlineStr">
+        <is>
+          <t>ウマ娘英語版の海外ヒット、AI・広告事業の成長</t>
+        </is>
+      </c>
+      <c r="O13" s="9" t="inlineStr">
+        <is>
+          <t>通期は減益予想、ゲーム収益のタイトル偏重</t>
+        </is>
+      </c>
+      <c r="P13" s="9" t="inlineStr">
+        <is>
+          <t>ウマ娘グローバル展開と新作・AI事業の収益貢献</t>
+        </is>
+      </c>
+      <c r="Q13" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -12605,11 +13061,31 @@
           <t>Xbox/Game Pass/Activision/Bethesda</t>
         </is>
       </c>
-      <c r="L2" s="9" t="inlineStr"/>
-      <c r="M2" s="9" t="inlineStr"/>
-      <c r="N2" s="9" t="inlineStr"/>
-      <c r="O2" s="9" t="inlineStr"/>
-      <c r="P2" s="9" t="inlineStr"/>
+      <c r="L2" s="9" t="inlineStr">
+        <is>
+          <t>Xboxは6/30の会計年度末までに数年来最大級となる4度目のレイオフ実施見込み。Activision統合でゲーム売上は増えるが、ハード収益減・Game Pass伸び悩みで構造改革継続。中欧の流通体制も再編。会社全体はAI/クラウド優先。</t>
+        </is>
+      </c>
+      <c r="M2" s="9" t="inlineStr">
+        <is>
+          <t>Activision/Bethesda/CoD等の巨大IPとGame Pass、AI・クラウド基盤</t>
+        </is>
+      </c>
+      <c r="N2" s="9" t="inlineStr">
+        <is>
+          <t>Xbox事業の連続レイオフ・ハード弱含み</t>
+        </is>
+      </c>
+      <c r="O2" s="9" t="inlineStr">
+        <is>
+          <t>マルチプラットフォーム化とGame Passの収益最適化</t>
+        </is>
+      </c>
+      <c r="P2" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
@@ -12628,7 +13104,11 @@
         </is>
       </c>
       <c r="D3" s="9" t="inlineStr"/>
-      <c r="E3" s="9" t="inlineStr"/>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>$6.72bn（FY26 Net Bookings）</t>
+        </is>
+      </c>
       <c r="F3" s="9" t="inlineStr"/>
       <c r="G3" s="9" t="inlineStr"/>
       <c r="H3" s="9" t="inlineStr"/>
@@ -12639,11 +13119,31 @@
           <t>GTA/RDR/NBA 2K/Zynga</t>
         </is>
       </c>
-      <c r="L3" s="9" t="inlineStr"/>
-      <c r="M3" s="9" t="inlineStr"/>
-      <c r="N3" s="9" t="inlineStr"/>
-      <c r="O3" s="9" t="inlineStr"/>
-      <c r="P3" s="9" t="inlineStr"/>
+      <c r="L3" s="9" t="inlineStr">
+        <is>
+          <t>FY26 Net Bookingsは$6.72bn、FY27は$8.0〜8.2bnへ大幅増の初期ガイダンス。GTA6が11/19発売予定で初年度3,500万本超(Piper予測)。株価は直近5営業日+8.6%、3月安値から+28.8%。Piper Sandlerがオーバーウェイト・目標$280で新規カバー。</t>
+        </is>
+      </c>
+      <c r="M3" s="9" t="inlineStr">
+        <is>
+          <t>GTA6発売を控えた史上最大級の収益拡大期待</t>
+        </is>
+      </c>
+      <c r="N3" s="9" t="inlineStr">
+        <is>
+          <t>発売延期リスクと期待先行の高バリュエーション</t>
+        </is>
+      </c>
+      <c r="O3" s="9" t="inlineStr">
+        <is>
+          <t>GTA6の11/19発売実現と初年度販売</t>
+        </is>
+      </c>
+      <c r="P3" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
@@ -12662,7 +13162,11 @@
         </is>
       </c>
       <c r="D4" s="9" t="inlineStr"/>
-      <c r="E4" s="9" t="inlineStr"/>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>$8.03bn（FY26 Net Bookings）</t>
+        </is>
+      </c>
       <c r="F4" s="9" t="inlineStr"/>
       <c r="G4" s="9" t="inlineStr"/>
       <c r="H4" s="9" t="inlineStr"/>
@@ -12673,11 +13177,31 @@
           <t>EA FC/Madden/Apex/The Sims</t>
         </is>
       </c>
-      <c r="L4" s="9" t="inlineStr"/>
-      <c r="M4" s="9" t="inlineStr"/>
-      <c r="N4" s="9" t="inlineStr"/>
-      <c r="O4" s="9" t="inlineStr"/>
-      <c r="P4" s="9" t="inlineStr"/>
+      <c r="L4" s="9" t="inlineStr">
+        <is>
+          <t>PIF/Silver Lake/Affinity連合による$210/株・総額約$550億の非公開化が進行、6/30までの完了見込みでCFIUS審査が最終関門(史上最大のLBO)。FY26はNet Bookings $8,026M(+9%)で過去最高、Battlefield 6がフランチャイズ最高の年・Apexも二桁回復。</t>
+        </is>
+      </c>
+      <c r="M4" s="9" t="inlineStr">
+        <is>
+          <t>$550億buyout進行と過去最高業績、Battlefield/FCの強さ</t>
+        </is>
+      </c>
+      <c r="N4" s="9" t="inlineStr">
+        <is>
+          <t>CFIUS等規制承認リスク、上場廃止後の不透明感</t>
+        </is>
+      </c>
+      <c r="O4" s="9" t="inlineStr">
+        <is>
+          <t>買収完了の可否とBattlefield/EA FCの継続成長</t>
+        </is>
+      </c>
+      <c r="P4" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -12707,11 +13231,31 @@
           <t>Assassin's Creed/Far Cry/Tom Clancy</t>
         </is>
       </c>
-      <c r="L5" s="9" t="inlineStr"/>
-      <c r="M5" s="9" t="inlineStr"/>
-      <c r="N5" s="9" t="inlineStr"/>
-      <c r="O5" s="9" t="inlineStr"/>
-      <c r="P5" s="9" t="inlineStr"/>
+      <c r="L5" s="9" t="inlineStr">
+        <is>
+          <t>6/5株価$30.33。Q1'26売上$508.2M(+35%)・Grow部門+49%で予想超え。6/2にPiper Sandlerが目標$40へ引き上げ・オーバーウェイト、Edgewaterも格上げ。広告主導の収益化とAI活用が評価され90日で+51%(年初来は-32%)。Q4'26にGAAP黒字化を目標。</t>
+        </is>
+      </c>
+      <c r="M5" s="9" t="inlineStr">
+        <is>
+          <t>広告(Grow)事業の回復とAI活用、アナリスト格上げ相次ぐ</t>
+        </is>
+      </c>
+      <c r="N5" s="9" t="inlineStr">
+        <is>
+          <t>年初来は下落、インサイダー売却と黒字化前の不確実性</t>
+        </is>
+      </c>
+      <c r="O5" s="9" t="inlineStr">
+        <is>
+          <t>Q4のGAAP黒字化達成と広告プラットフォーム成長</t>
+        </is>
+      </c>
+      <c r="P5" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
@@ -12741,11 +13285,31 @@
           <t>Honor of Kings/Riot/Epic出資</t>
         </is>
       </c>
-      <c r="L6" s="9" t="inlineStr"/>
-      <c r="M6" s="9" t="inlineStr"/>
-      <c r="N6" s="9" t="inlineStr"/>
-      <c r="O6" s="9" t="inlineStr"/>
-      <c r="P6" s="9" t="inlineStr"/>
+      <c r="L6" s="9" t="inlineStr">
+        <is>
+          <t>6月初の株価はHK$453前後(-1.26%)。5/13発表のQ1はEPS HK$8.51で予想超え、FY25売上CN¥751.8bn(+14%)・純益CN¥224.8bn(+16%)。WeChat向けAIエージェントを内部テスト中。ゲームはGDC 2026で20超セッション出展。次回決算は8/19。</t>
+        </is>
+      </c>
+      <c r="M6" s="9" t="inlineStr">
+        <is>
+          <t>国内外ゲームの安定課金とAIによる広告・効率化、Riot/Epic等出資網</t>
+        </is>
+      </c>
+      <c r="N6" s="9" t="inlineStr">
+        <is>
+          <t>中国ゲーム規制と国内マクロ、海外大型ヒットの再現性</t>
+        </is>
+      </c>
+      <c r="O6" s="9" t="inlineStr">
+        <is>
+          <t>AIエージェント収益化と海外スタジオ(Vantage等)の成果</t>
+        </is>
+      </c>
+      <c r="P6" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
@@ -12775,11 +13339,31 @@
           <t>Identity V/荒野行動/Naraka</t>
         </is>
       </c>
-      <c r="L7" s="9" t="inlineStr"/>
-      <c r="M7" s="9" t="inlineStr"/>
-      <c r="N7" s="9" t="inlineStr"/>
-      <c r="O7" s="9" t="inlineStr"/>
-      <c r="P7" s="9" t="inlineStr"/>
+      <c r="L7" s="9" t="inlineStr">
+        <is>
+          <t>6/1株価$122.43。Q1'26は売上RMB30.59bn(+6%)でEPS RMB17.46と予想超えも、販管費増で一時下落。粗利率は69.4%へ改善。新作『Sea of Elements』『Ananta(都市型オープンワールド)』を2026年内投入予定。アナリストはStrong Buy・平均目標$162。</t>
+        </is>
+      </c>
+      <c r="M7" s="9" t="inlineStr">
+        <is>
+          <t>高粗利のゲーム課金と強力な新作パイプライン</t>
+        </is>
+      </c>
+      <c r="N7" s="9" t="inlineStr">
+        <is>
+          <t>マーケ費用増と一部既存タイトルの減速懸念</t>
+        </is>
+      </c>
+      <c r="O7" s="9" t="inlineStr">
+        <is>
+          <t>AnantaなどAAA級新作のグローバル成否</t>
+        </is>
+      </c>
+      <c r="P7" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
@@ -12809,11 +13393,31 @@
           <t>PUBG/Subnautica</t>
         </is>
       </c>
-      <c r="L8" s="9" t="inlineStr"/>
-      <c r="M8" s="9" t="inlineStr"/>
-      <c r="N8" s="9" t="inlineStr"/>
-      <c r="O8" s="9" t="inlineStr"/>
-      <c r="P8" s="9" t="inlineStr"/>
+      <c r="L8" s="9" t="inlineStr">
+        <is>
+          <t>6/5株価約$167.9・時価総額$7.57bn。『Subnautica 2』が5/14アーリーアクセスで1週間400万本・粗収益$120M。好調の一方、Unknown Worlds旧株主への最大$250Mのアーンアウト支払い義務が発生し、関連訴訟でも開発陣復職とボーナス支払いを命じる判決。</t>
+        </is>
+      </c>
+      <c r="M8" s="9" t="inlineStr">
+        <is>
+          <t>PUBG依存からの脱却、Subnautica 2の大ヒット</t>
+        </is>
+      </c>
+      <c r="N8" s="9" t="inlineStr">
+        <is>
+          <t>最大$250Mのアーンアウト負担と訴訟、前年営業益の約35%相当</t>
+        </is>
+      </c>
+      <c r="O8" s="9" t="inlineStr">
+        <is>
+          <t>Subnautica 2の本格展開と新規IPの多様化</t>
+        </is>
+      </c>
+      <c r="P8" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
@@ -12843,11 +13447,31 @@
           <t>MapleStory/Dungeon&amp;Fighter</t>
         </is>
       </c>
-      <c r="L9" s="9" t="inlineStr"/>
-      <c r="M9" s="9" t="inlineStr"/>
-      <c r="N9" s="9" t="inlineStr"/>
-      <c r="O9" s="9" t="inlineStr"/>
-      <c r="P9" s="9" t="inlineStr"/>
+      <c r="L9" s="9" t="inlineStr">
+        <is>
+          <t>株価約2,250円(+2.0%)。MapleStoryフランチャイズの成長と新作『ARC Raiders』(Embark)の貢献で直近四半期は好調。年間配当を1株60円(前期45円)へ増配。6月に株主総会。中国Dungeon&amp;Fighterモバイル等のライブ運営が収益の柱。</t>
+        </is>
+      </c>
+      <c r="M9" s="9" t="inlineStr">
+        <is>
+          <t>MapleStory/DNFの長寿ライブ運営とARC Raidersの新規寄与</t>
+        </is>
+      </c>
+      <c r="N9" s="9" t="inlineStr">
+        <is>
+          <t>中国市況依存と四半期業績のボラティリティ</t>
+        </is>
+      </c>
+      <c r="O9" s="9" t="inlineStr">
+        <is>
+          <t>ARC Raiders定着と新規IPのグローバル展開</t>
+        </is>
+      </c>
+      <c r="P9" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
@@ -12877,11 +13501,31 @@
           <t>Saber/Coffee Stain等100超スタジオ</t>
         </is>
       </c>
-      <c r="L10" s="9" t="inlineStr"/>
-      <c r="M10" s="9" t="inlineStr"/>
-      <c r="N10" s="9" t="inlineStr"/>
-      <c r="O10" s="9" t="inlineStr"/>
-      <c r="P10" s="9" t="inlineStr"/>
+      <c r="L10" s="9" t="inlineStr">
+        <is>
+          <t>FY26は売上kr16.6bn(-26%)・純損失kr6.89bnと低迷。Coffee Stainグループを12/11にスピンオフ、残存本体を『Fellowship Entertainment』へ改称し2026年4月に分離・別上場。新CEOを公募中で、モバイル/PC・console/フィジカル流通等に集中し利益重視へ。</t>
+        </is>
+      </c>
+      <c r="M10" s="9" t="inlineStr">
+        <is>
+          <t>事業分割で身軽化、Tomb Raider映像化等2027パイプライン</t>
+        </is>
+      </c>
+      <c r="N10" s="9" t="inlineStr">
+        <is>
+          <t>大幅減収と赤字、相次ぐ再編で信頼回復途上</t>
+        </is>
+      </c>
+      <c r="O10" s="9" t="inlineStr">
+        <is>
+          <t>分割後の収益性回復と新CEO選任・2027年の製品群</t>
+        </is>
+      </c>
+      <c r="P10" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
@@ -12911,11 +13555,31 @@
           <t>Robloxプラットフォーム</t>
         </is>
       </c>
-      <c r="L11" s="9" t="inlineStr"/>
-      <c r="M11" s="9" t="inlineStr"/>
-      <c r="N11" s="9" t="inlineStr"/>
-      <c r="O11" s="9" t="inlineStr"/>
-      <c r="P11" s="9" t="inlineStr"/>
+      <c r="L11" s="9" t="inlineStr">
+        <is>
+          <t>6/7株価$41.75・年初来-42%。年齢確認/児童安全機能の強化が短期のユーザー成長を圧迫するとして通期ブッキング見通しを下方修正。5〜8歳向け『Roblox Kids』・9〜15歳向け『Roblox Select』を6月初に展開。Q1売上は$1.4bn(+39%)。アナリスト平均目標$64.81。</t>
+        </is>
+      </c>
+      <c r="M11" s="9" t="inlineStr">
+        <is>
+          <t>高成長のプラットフォーム売上とクリエイター経済</t>
+        </is>
+      </c>
+      <c r="N11" s="9" t="inlineStr">
+        <is>
+          <t>安全機能対応によるユーザー成長の短期摩擦、収益化の遅れ</t>
+        </is>
+      </c>
+      <c r="O11" s="9" t="inlineStr">
+        <is>
+          <t>年齢別アカウント定着と通期ブッキング回復</t>
+        </is>
+      </c>
+      <c r="P11" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
@@ -12968,7 +13632,11 @@
         </is>
       </c>
       <c r="D13" s="9" t="inlineStr"/>
-      <c r="E13" s="9" t="inlineStr"/>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>$1.84bn（Q1'26）</t>
+        </is>
+      </c>
       <c r="F13" s="9" t="inlineStr"/>
       <c r="G13" s="9" t="inlineStr"/>
       <c r="H13" s="9" t="inlineStr"/>
@@ -12979,11 +13647,31 @@
           <t>モバイル広告/AI Axon</t>
         </is>
       </c>
-      <c r="L13" s="9" t="inlineStr"/>
-      <c r="M13" s="9" t="inlineStr"/>
-      <c r="N13" s="9" t="inlineStr"/>
-      <c r="O13" s="9" t="inlineStr"/>
-      <c r="P13" s="9" t="inlineStr"/>
+      <c r="L13" s="9" t="inlineStr">
+        <is>
+          <t>6/2にS&amp;P500入り。Q1'26売上$1.84bn(+59%)・調整後EPS $3.56で予想超え、調整後EBITDAマージン約85%。自社運用型AXON広告プラットフォームを6月に全世界の広告主へ開放(成否を分けるバイナリーイベントと見られる)。目標株価は$646へ引き上げ。</t>
+        </is>
+      </c>
+      <c r="M13" s="9" t="inlineStr">
+        <is>
+          <t>AI広告(AXON)の高収益・高成長、S&amp;P500入り</t>
+        </is>
+      </c>
+      <c r="N13" s="9" t="inlineStr">
+        <is>
+          <t>AXON全面開放の実行リスクと高バリュエーション</t>
+        </is>
+      </c>
+      <c r="O13" s="9" t="inlineStr">
+        <is>
+          <t>AXONグローバル開放の成果と広告外領域への拡張</t>
+        </is>
+      </c>
+      <c r="P13" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
daily-news + cross-questions update (2026-06-09 00:01)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -2477,7 +2477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3229,6 +3229,80 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B21" s="14" t="inlineStr">
+        <is>
+          <t>運営型ゲームのサービス終了時に返金/プレイ継続を義務付ける動きは、SaaS・サブスク家電・コネクテッドカーなど『売り切りでない製品』全般のサポート終了義務化に波及するか？</t>
+        </is>
+      </c>
+      <c r="C21" s="14" t="inlineStr">
+        <is>
+          <t>米加州「ゲーム保護法案」AB1921が州下院を通過(2026-06)</t>
+        </is>
+      </c>
+      <c r="D21" s="14" t="inlineStr">
+        <is>
+          <t>カリフォルニア州議会, Stop Killing Games, 運営型ゲーム各社</t>
+        </is>
+      </c>
+      <c r="E21" s="14" t="inlineStr">
+        <is>
+          <t>SaaS/サブスク, スマート家電, コネクテッドカー, IoT</t>
+        </is>
+      </c>
+      <c r="F21" s="14" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="G21" s="14" t="inlineStr">
+        <is>
+          <t>“所有しない製品”の出口保証は、デジタル/コネクテッド製品全般の共通論点になりつつある。</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B22" s="14" t="inlineStr">
+        <is>
+          <t>ライブサービス『Destiny 2』の運営終了は、動画配信・SaaSなど継続課金モデルの“撤退の作法(サンセット設計)”として何に相当するか？</t>
+        </is>
+      </c>
+      <c r="C22" s="14" t="inlineStr">
+        <is>
+          <t>Bungie「Destiny 2」が6/9最終アップデートで開発終了(2026-06)</t>
+        </is>
+      </c>
+      <c r="D22" s="14" t="inlineStr">
+        <is>
+          <t>Bungie, Sony, Destiny 2</t>
+        </is>
+      </c>
+      <c r="E22" s="14" t="inlineStr">
+        <is>
+          <t>動画配信(SVOD), SaaS, サブスク全般</t>
+        </is>
+      </c>
+      <c r="F22" s="14" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="G22" s="14" t="inlineStr">
+        <is>
+          <t>高コスト運営の逓減局面では、撤退手順(返金/データ/継続)の巧拙がブランド毀損を左右する。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3240,7 +3314,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L99"/>
+  <dimension ref="A1:L109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9563,6 +9637,616 @@
           <t>6/17新チャプター</t>
         </is>
       </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B100" s="14" t="inlineStr">
+        <is>
+          <t>「ペルソナ6」がXbox Games Showcase 2026で正式発表、緑基調の新作RPG</t>
+        </is>
+      </c>
+      <c r="C100" s="14" t="inlineStr">
+        <is>
+          <t>https://www.videogameschronicle.com/news/persona-6-announced-xbox-games-showcase-2026/</t>
+        </is>
+      </c>
+      <c r="D100" s="14" t="inlineStr">
+        <is>
+          <t>アトラスの看板RPG「ペルソナ」シリーズは「P5」が世界1000万本超の大ヒットとなり続編が待望されていた。リーク情報が先行する中、6月8日のXbox Games Showcase 2026でセガ/アトラスが正式に新作を披露した。</t>
+        </is>
+      </c>
+      <c r="E100" s="14" t="inlineStr">
+        <is>
+          <t>ティザー映像で墓地を背景にロゴが公開され「ペルソナ6」が正式発表。緑を基調にしたビジュアルと現代日本を舞台にした完全新規キャスト・ストーリーが特徴。対応はXbox Series X/S・Xbox PC・PS5・Steamで、発売初日からGame Pass入りする見込み。</t>
+        </is>
+      </c>
+      <c r="F100" s="14" t="inlineStr">
+        <is>
+          <t>緑基調の新ビジュアルと完全新規キャスト
+Xbox・PS5・PC・Steamのマルチ展開
+初日Game Pass対応
+発売時期は未公表でウィッシュリスト開始</t>
+        </is>
+      </c>
+      <c r="G100" s="14" t="inlineStr">
+        <is>
+          <t>マルチプラットフォーム+初日Game Pass戦略は、かつてのソニー先行から大きく転換。発売は2027年以降とみられ、P4リバイバル等の周辺タイトルで熱量を維持しつつ、グローバル同時展開で初動最大化を狙う公算。</t>
+        </is>
+      </c>
+      <c r="H100" s="14" t="inlineStr">
+        <is>
+          <t>人気JRPGのマルチ/サブスク同時投入戦略</t>
+        </is>
+      </c>
+      <c r="I100" s="14" t="inlineStr">
+        <is>
+          <t>セガ, アトラス, Microsoft</t>
+        </is>
+      </c>
+      <c r="J100" s="14" t="inlineStr">
+        <is>
+          <t>ペルソナ6, Xbox Game Pass</t>
+        </is>
+      </c>
+      <c r="K100" s="14" t="inlineStr">
+        <is>
+          <t>新作,海外</t>
+        </is>
+      </c>
+      <c r="L100" s="14" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B101" s="14" t="inlineStr">
+        <is>
+          <t>「ペルソナ4 リバイバル」2027年2月18日発売決定、P4Gをフルリメイク</t>
+        </is>
+      </c>
+      <c r="C101" s="14" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/999/G999903/20260608001/</t>
+        </is>
+      </c>
+      <c r="D101" s="14" t="inlineStr">
+        <is>
+          <t>2008年発売の「ペルソナ4」は派生作品やアニメで根強い人気を持つ。アトラスはシリーズ過去作のリメイク強化を進めており、6月8日のショーケースでフルリメイク版の具体的な発売日を公開した。</t>
+        </is>
+      </c>
+      <c r="E101" s="14" t="inlineStr">
+        <is>
+          <t>「P4G」をベースにしたフルリメイク「ペルソナ4 リバイバル」が2027年2月18日発売と発表。最新エンジンでビジュアルとシステムを刷新し現行機向けに再構築する。ペルソナ6発表と合わせ、シリーズ資産の総動員でブランド価値を高める狙い。</t>
+        </is>
+      </c>
+      <c r="F101" s="14" t="inlineStr">
+        <is>
+          <t>発売日2027年2月18日に確定
+P4Gベースのフルリメイク
+最新世代機向けに刷新
+P6発表と同時でシリーズ機運を醸成</t>
+        </is>
+      </c>
+      <c r="G101" s="14" t="inlineStr">
+        <is>
+          <t>リメイクと新作の二段構えで旧作ファン再獲得と新規層取り込みを同時に進める。P3リロード→P4リバイバル→P6の流れで毎年なんらかのペルソナ関連投入が常態化し、IPの年次収益化が進むとみられる。</t>
+        </is>
+      </c>
+      <c r="H101" s="14" t="inlineStr">
+        <is>
+          <t>旧作リメイクによるIP延命と年次収益化</t>
+        </is>
+      </c>
+      <c r="I101" s="14" t="inlineStr">
+        <is>
+          <t>アトラス, セガ</t>
+        </is>
+      </c>
+      <c r="J101" s="14" t="inlineStr">
+        <is>
+          <t>ペルソナ4 リバイバル</t>
+        </is>
+      </c>
+      <c r="K101" s="14" t="inlineStr">
+        <is>
+          <t>新作,国内</t>
+        </is>
+      </c>
+      <c r="L101" s="14" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B102" s="14" t="inlineStr">
+        <is>
+          <t>「Gears of War: E-Day」発売日が2026年10月6日に決定、原点の戦いを描く</t>
+        </is>
+      </c>
+      <c r="C102" s="14" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/968/G096869/20260608002/</t>
+        </is>
+      </c>
+      <c r="D102" s="14" t="inlineStr">
+        <is>
+          <t>「Gears of War」はXboxを代表するシリーズで、E-Dayは若き日のマーカスとドムを描く前日譚。Microsoftは年末商戦に向けた看板タイトルと位置づけ、6月8日のショーケースで発売日を確定させた。</t>
+        </is>
+      </c>
+      <c r="E102" s="14" t="inlineStr">
+        <is>
+          <t>前日譚「Gears of War: E-Day」が2026年10月6日発売と発表。シリーズの原点となる“エマージェンス・デイ”の戦いを描く。年末商戦直前のローンチで、Game Pass初日対応によりハード/サブスク両面でXbox陣営を牽引する狙い。</t>
+        </is>
+      </c>
+      <c r="F102" s="14" t="inlineStr">
+        <is>
+          <t>発売日2026年10月6日に確定
+若き日のマーカス&amp;ドムの前日譚
+年末商戦前の旗艦タイトル
+Game Pass戦略の中核</t>
+        </is>
+      </c>
+      <c r="G102" s="14" t="inlineStr">
+        <is>
+          <t>マルチ展開を進めるMicrosoftにとってE-Dayは数少ない大型“独占級”タイトル。10月投入で年末のGame Pass新規獲得を狙うが、他プラットフォーム展開の有無が今後の収益最大化の焦点になる。</t>
+        </is>
+      </c>
+      <c r="H102" s="14" t="inlineStr">
+        <is>
+          <t>年末商戦×サブスクの旗艦タイトル戦略</t>
+        </is>
+      </c>
+      <c r="I102" s="14" t="inlineStr">
+        <is>
+          <t>Microsoft, The Coalition</t>
+        </is>
+      </c>
+      <c r="J102" s="14" t="inlineStr">
+        <is>
+          <t>Gears of War: E-Day</t>
+        </is>
+      </c>
+      <c r="K102" s="14" t="inlineStr">
+        <is>
+          <t>新作,海外</t>
+        </is>
+      </c>
+      <c r="L102" s="14" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B103" s="14" t="inlineStr">
+        <is>
+          <t>Nintendo Switch 2が世界2000万台目前、9月に各地域で値上げへ</t>
+        </is>
+      </c>
+      <c r="C103" s="14" t="inlineStr">
+        <is>
+          <t>https://www.nintendolife.com/news/2026/05/switch-2-has-sold-just-shy-of-20-million-units-nintendo-lowers-fy27-forecast</t>
+        </is>
+      </c>
+      <c r="D103" s="14" t="inlineStr">
+        <is>
+          <t>2025年6月発売のSwitch 2は初代を上回るペースで普及が進み、英国では発売52週で100万台に到達。一方で部材コスト上昇などを背景に、任天堂は価格改定と販売見通しの調整を迫られている。</t>
+        </is>
+      </c>
+      <c r="E103" s="14" t="inlineStr">
+        <is>
+          <t>Switch 2は世界販売が2000万台目前に達し任天堂史上最速級の立ち上がり。ただし9月1日から米国で499.99ドル(+50ドル)、欧州で+30ユーロ等各地域で値上げ予定で、下期の販売減速を織り込みFY27見通しを下方修正した。</t>
+        </is>
+      </c>
+      <c r="F103" s="14" t="inlineStr">
+        <is>
+          <t>世界販売2000万台目前
+英国は52週で100万台、初代より約30週速い
+9月から米欧加で値上げ
+FY27販売見通しを下方修正</t>
+        </is>
+      </c>
+      <c r="G103" s="14" t="inlineStr">
+        <is>
+          <t>値上げは短期的に需要を抑えるが、ソフト牽引でインストールベース拡大は継続見込み。値上げ前の駆け込み需要と年末のソフトラインナップが下期の実販売を左右する。為替・部材費が価格政策の鍵。</t>
+        </is>
+      </c>
+      <c r="H103" s="14" t="inlineStr">
+        <is>
+          <t>ハード値上げと普及曲線・粗利の関係</t>
+        </is>
+      </c>
+      <c r="I103" s="14" t="inlineStr">
+        <is>
+          <t>任天堂</t>
+        </is>
+      </c>
+      <c r="J103" s="14" t="inlineStr">
+        <is>
+          <t>Nintendo Switch 2</t>
+        </is>
+      </c>
+      <c r="K103" s="14" t="inlineStr">
+        <is>
+          <t>業績,国内</t>
+        </is>
+      </c>
+      <c r="L103" s="14" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B104" s="14" t="inlineStr">
+        <is>
+          <t>EAの約550億ドル非公開化、2026年内クローズへ最終局面</t>
+        </is>
+      </c>
+      <c r="C104" s="14" t="inlineStr">
+        <is>
+          <t>https://www.financierworldwide.com/ea-agrees-55bn-consortium-buyout</t>
+        </is>
+      </c>
+      <c r="D104" s="14" t="inlineStr">
+        <is>
+          <t>EAは2025年9月、サウジPIF・Silver Lake・Affinity Partnersの連合による約550億ドルのレバレッジドバイアウトで非公開化に合意。史上最大級のLBOとして規制審査の動向が注目されてきた。</t>
+        </is>
+      </c>
+      <c r="E104" s="14" t="inlineStr">
+        <is>
+          <t>EAの約550億ドル非公開化は2月にHSR独禁審査の待機期間が満了し主要なハードルを通過。5月時点で残る一部審査の完了を待つ段階で、FY27第1四半期(〜6月末)のクローズが見込まれる。完了すれば上場企業のLBOとして史上最大規模となる。</t>
+        </is>
+      </c>
+      <c r="F104" s="14" t="inlineStr">
+        <is>
+          <t>連合(PIF/Silver Lake/Affinity)による約550億ドルLBO
+HSR独禁審査は通過済み
+残る一部の規制審査が焦点
+2026年6月末までのクローズ見込み</t>
+        </is>
+      </c>
+      <c r="G104" s="14" t="inlineStr">
+        <is>
+          <t>クローズ後はEAが多額の買収負債を抱え、ライブサービスやEA Sports等の安定収益で返済原資を確保する構図に。短期の収益最大化圧力が強まり、人員・スタジオ再編やIP集中が進む可能性が高い。</t>
+        </is>
+      </c>
+      <c r="H104" s="14" t="inlineStr">
+        <is>
+          <t>大型LBO後の負債と収益構造の変化</t>
+        </is>
+      </c>
+      <c r="I104" s="14" t="inlineStr">
+        <is>
+          <t>Electronic Arts, PIF, Silver Lake, Affinity Partners</t>
+        </is>
+      </c>
+      <c r="J104" s="14" t="inlineStr">
+        <is>
+          <t>EA Sports FC, Battlefield</t>
+        </is>
+      </c>
+      <c r="K104" s="14" t="inlineStr">
+        <is>
+          <t>M&amp;A,海外</t>
+        </is>
+      </c>
+      <c r="L104" s="14" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B105" s="14" t="inlineStr">
+        <is>
+          <t>ゲームの生成AI市場、2026年に約22億ドルへ拡大の見通し</t>
+        </is>
+      </c>
+      <c r="C105" s="14" t="inlineStr">
+        <is>
+          <t>https://www.gii.co.jp/report/tbrc1973552-generative-ai-gaming-global-market-report.html</t>
+        </is>
+      </c>
+      <c r="D105" s="14" t="inlineStr">
+        <is>
+          <t>ゲーム開発はNPC生成・動的コンテンツ・ローカライズ・QA等で生成AI活用が急速に進む。市場調査では、ゲームが生成AI全体の成長を牽引する分野の一つと位置づけられている。</t>
+        </is>
+      </c>
+      <c r="E105" s="14" t="inlineStr">
+        <is>
+          <t>調査によると、ゲーム分野の生成AI市場は2025年の約17.9億ドルから2026年に約22.1億ドル(CAGR23.1%)へ拡大し、2030年に約50.9億ドルに達する見通し。NPCの自律化、手続き型生成、リアルタイム翻訳など実装が広がり、エージェント型AIの普及が後押しする。</t>
+        </is>
+      </c>
+      <c r="F105" s="14" t="inlineStr">
+        <is>
+          <t>2026年市場規模 約22.1億ドル、CAGR23.1%
+2030年に約50.9億ドルへ
+NPC自律化・手続き型生成・リアルタイム翻訳が拡大
+エージェント型AIが普及を牽引</t>
+        </is>
+      </c>
+      <c r="G105" s="14" t="inlineStr">
+        <is>
+          <t>開発効率化の一方で、AI生成物の権利・開示義務やクオリティ管理が論点化。クラウドとローカルのハイブリッド処理や専門特化モデルの採用が進み、コスト構造と雇用に構造的影響を及ぼす。</t>
+        </is>
+      </c>
+      <c r="H105" s="14" t="inlineStr">
+        <is>
+          <t>ゲーム開発における生成AIの実装領域と権利課題</t>
+        </is>
+      </c>
+      <c r="I105" s="14" t="inlineStr">
+        <is>
+          <t>NVIDIA, Microsoft, Google Cloud</t>
+        </is>
+      </c>
+      <c r="J105" s="14" t="inlineStr">
+        <is>
+          <t>生成AI, エージェント型AI</t>
+        </is>
+      </c>
+      <c r="K105" s="14" t="inlineStr">
+        <is>
+          <t>技術,海外</t>
+        </is>
+      </c>
+      <c r="L105" s="14" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B106" s="14" t="inlineStr">
+        <is>
+          <t>米加州「ゲーム保護法案」AB1921が下院通過、終了時の返金等を義務化</t>
+        </is>
+      </c>
+      <c r="C106" s="14" t="inlineStr">
+        <is>
+          <t>https://automaton-media.com/articles/newsjp/20260529-445864/</t>
+        </is>
+      </c>
+      <c r="D106" s="14" t="inlineStr">
+        <is>
+          <t>運営型(ライブサービス)ゲームのサービス終了で遊べなくなる問題に対し「Stop Killing Games」運動が世界的に拡大。米カリフォルニア州で、終了後の扱いを事業者に義務付ける法案が審議されてきた。</t>
+        </is>
+      </c>
+      <c r="E106" s="14" t="inlineStr">
+        <is>
+          <t>運営型ゲームの“終わり方”を規定する「ゲーム保護法案(AB1921)」がカリフォルニア州下院本会議を通過。サービス終了後もプレイ継続できる独立環境の提供、または不可能な場合のユーザー返金を義務付ける内容で、上院審議へ進む。</t>
+        </is>
+      </c>
+      <c r="F106" s="14" t="inlineStr">
+        <is>
+          <t>AB1921が州下院本会議を通過
+終了後のプレイ継続環境の提供を要求
+不可能なら返金を義務化
+Stop Killing Games運動が後押し</t>
+        </is>
+      </c>
+      <c r="G106" s="14" t="inlineStr">
+        <is>
+          <t>成立すれば運営型タイトルの設計・契約・引当に影響が及び、グローバル運営にも波及しうる。EUの市民イニシアチブと連動し、サービス終了時の“出口設計”が業界標準として整備される方向に向かう可能性。</t>
+        </is>
+      </c>
+      <c r="H106" s="14" t="inlineStr">
+        <is>
+          <t>ライブサービス終了の法規制と出口設計</t>
+        </is>
+      </c>
+      <c r="I106" s="14" t="inlineStr">
+        <is>
+          <t>カリフォルニア州議会, 運営型ゲーム各社</t>
+        </is>
+      </c>
+      <c r="J106" s="14" t="inlineStr">
+        <is>
+          <t>Stop Killing Games, AB1921</t>
+        </is>
+      </c>
+      <c r="K106" s="14" t="inlineStr">
+        <is>
+          <t>規制,海外</t>
+        </is>
+      </c>
+      <c r="L106" s="14" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B107" s="14" t="inlineStr">
+        <is>
+          <t>CS2「IEM Cologne Major 2026」視聴が急伸、7日にピーク約70万人</t>
+        </is>
+      </c>
+      <c r="C107" s="14" t="inlineStr">
+        <is>
+          <t>https://escharts.com/news/iem-cologne-major-matches-score-schedule</t>
+        </is>
+      </c>
+      <c r="D107" s="14" t="inlineStr">
+        <is>
+          <t>Counter-Strike 2の最高峰大会「IEM Cologne Major 2026」が6月2〜21日にドイツで開催。賞金総額125万ドル(優勝50万ドル)で世界的な注目を集めている。</t>
+        </is>
+      </c>
+      <c r="E107" s="14" t="inlineStr">
+        <is>
+          <t>IEM Cologne Major 2026は初日に約44.8万人のピーク視聴を記録し、6月7日には約70万人へ急伸。プレーオフ進行に伴いさらなる上昇が見込まれ、ピーク180万〜200万人超の可能性も指摘される。eスポーツ視聴の地力の強さを示す。</t>
+        </is>
+      </c>
+      <c r="F107" s="14" t="inlineStr">
+        <is>
+          <t>賞金総額125万ドル(優勝50万ドル)
+初日ピーク約44.8万人→7日約70万人
+プレーオフで更なる上昇見込み
+ピーク200万人超も視野</t>
+        </is>
+      </c>
+      <c r="G107" s="14" t="inlineStr">
+        <is>
+          <t>CS2はメジャー単位で安定して高視聴を維持しスポンサー・配信権の価値を支える。視聴のモバイル/共同配信シフトが進む中、計測方法を巡る議論も活発化し、商業価値の評価軸が再整理される。</t>
+        </is>
+      </c>
+      <c r="H107" s="14" t="inlineStr">
+        <is>
+          <t>eスポーツ視聴計測と商業価値の評価軸</t>
+        </is>
+      </c>
+      <c r="I107" s="14" t="inlineStr">
+        <is>
+          <t>ESL, Valve</t>
+        </is>
+      </c>
+      <c r="J107" s="14" t="inlineStr">
+        <is>
+          <t>Counter-Strike 2, IEM Cologne</t>
+        </is>
+      </c>
+      <c r="K107" s="14" t="inlineStr">
+        <is>
+          <t>eスポーツ,海外</t>
+        </is>
+      </c>
+      <c r="L107" s="14" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B108" s="14" t="inlineStr">
+        <is>
+          <t>Bungie「Destiny 2」6月9日の最終アップデートで開発終了へ</t>
+        </is>
+      </c>
+      <c r="C108" s="14" t="inlineStr">
+        <is>
+          <t>https://www.gamedeveloper.com/business/destiny-2-s-active-development-will-end-in-june</t>
+        </is>
+      </c>
+      <c r="D108" s="14" t="inlineStr">
+        <is>
+          <t>2017年発売の「Destiny 2」は長期運営型FPSの代表格。Sonyによる36億ドルの買収後もBungieはMarathon等の新規IPに注力しており、運営型タイトルの整理が進んでいた。</t>
+        </is>
+      </c>
+      <c r="E108" s="14" t="inlineStr">
+        <is>
+          <t>Bungieは6月9日配信のアップデート「Monument of Triumph」をもって「Destiny 2」の能動的開発を終了。新ストーリー拡張やシーズン活動の追加を停止し、サーバーは維持しつつメンテナンスモードへ移行する。配信後に大規模な人員削減が見込まれる。</t>
+        </is>
+      </c>
+      <c r="F108" s="14" t="inlineStr">
+        <is>
+          <t>6/9「Monument of Triumph」で開発終了
+新拡張・新シーズンの追加停止、サーバーは維持
+Destiny 3は未承認
+配信後に大規模レイオフの見込み</t>
+        </is>
+      </c>
+      <c r="G108" s="14" t="inlineStr">
+        <is>
+          <t>運営型の収益逓減と高コスト体質が露呈し、Bungieは新規IP Marathonに資源を集約。ライブサービスの“撤退の作法”が業界の関心事となり、長期運営タイトルの店じまい設計が他社の判断にも影響する。</t>
+        </is>
+      </c>
+      <c r="H108" s="14" t="inlineStr">
+        <is>
+          <t>ライブサービスの収益逓減と撤退設計</t>
+        </is>
+      </c>
+      <c r="I108" s="14" t="inlineStr">
+        <is>
+          <t>Bungie, Sony Interactive Entertainment</t>
+        </is>
+      </c>
+      <c r="J108" s="14" t="inlineStr">
+        <is>
+          <t>Destiny 2, Marathon</t>
+        </is>
+      </c>
+      <c r="K108" s="14" t="inlineStr">
+        <is>
+          <t>業績,海外</t>
+        </is>
+      </c>
+      <c r="L108" s="14" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B109" s="14" t="inlineStr">
+        <is>
+          <t>Summer Game Fest 2026、PS5向け注目6作のハンズオン詳細を公開</t>
+        </is>
+      </c>
+      <c r="C109" s="14" t="inlineStr">
+        <is>
+          <t>https://blog.playstation.com/2026/06/08/summer-game-fest-2026-hands-on-and-more-details-on-6-upcoming-ps5-games/</t>
+        </is>
+      </c>
+      <c r="D109" s="14" t="inlineStr">
+        <is>
+          <t>E3亡き後の夏商戦の中心となったSummer Game Festが6月5日にロサンゼルスで開催。各社が新作を一挙公開し、PlayStationも周辺イベントで自社向けタイトルを訴求した。</t>
+        </is>
+      </c>
+      <c r="E109" s="14" t="inlineStr">
+        <is>
+          <t>SGF2026に合わせPlayStation.Blogが今後のPS5向け6作のハンズオン詳細を公開。SGF本編ではFF7リベレーション、バイオRE:CV(Code Veronica)リメイク、ステラーブレイド続編などが発表されており、夏の新作ラッシュをPS5陣営の体験情報で補強した。</t>
+        </is>
+      </c>
+      <c r="F109" s="14" t="inlineStr">
+        <is>
+          <t>PS5向け6作のハンズオン詳細を公開
+SGF本編でFF7リベレーション等が発表
+夏商戦の話題をPS5体験情報で補強
+E3後のSGFが新作発表の中心に定着</t>
+        </is>
+      </c>
+      <c r="G109" s="14" t="inlineStr">
+        <is>
+          <t>大型発表はSGF・各社ショーケースへ分散が進み、体験記事や配信での“熱量の維持”が重要に。PS5は独占・先行体験を軸に差別化を図り、年末に向けてソフト牽引での販売押し上げを狙う。</t>
+        </is>
+      </c>
+      <c r="H109" s="14" t="inlineStr">
+        <is>
+          <t>E3後の新作発表エコシステムとPR設計</t>
+        </is>
+      </c>
+      <c r="I109" s="14" t="inlineStr">
+        <is>
+          <t>Sony Interactive Entertainment, Square Enix, Capcom</t>
+        </is>
+      </c>
+      <c r="J109" s="14" t="inlineStr">
+        <is>
+          <t>Final Fantasy VII Revelation, Resident Evil Code Veronica</t>
+        </is>
+      </c>
+      <c r="K109" s="14" t="inlineStr">
+        <is>
+          <t>新作,海外</t>
+        </is>
+      </c>
+      <c r="L109" s="14" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
daily-news + cross-questions update (2026-06-10) (2026-06-09 22:10)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -2477,7 +2477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3303,6 +3303,80 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>28年前の名作IP（時のオカリナ）をリメイクして新ハード需要を喚起する任天堂の手法は、映画・音楽・出版など他エンタメ業界のカタログ資産再活用（リマスター/リブート）と同じ収益構造か？</t>
+        </is>
+      </c>
+      <c r="C23" s="14" t="inlineStr">
+        <is>
+          <t>『ゼルダの伝説 時のオカリナ』Switch 2フルリメイク発表（Nintendo Direct 2026.6.9）</t>
+        </is>
+      </c>
+      <c r="D23" s="14" t="inlineStr">
+        <is>
+          <t>任天堂/ゼルダの伝説, スクウェア・エニックス/FF10 HD</t>
+        </is>
+      </c>
+      <c r="E23" s="14" t="inlineStr">
+        <is>
+          <t>映画（リブート・4Kリマスター）, 音楽（旧譜再発）, 出版（復刊）, アニメ</t>
+        </is>
+      </c>
+      <c r="F23" s="14" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="G23" s="14" t="inlineStr">
+        <is>
+          <t>Switch 2移行期に旧IPのリメイク/移植が集中。低リスクで確実性の高い既存資産の再収益化という点で、他のカタログ型エンタメ事業と同型の可能性。</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B24" s="14" t="inlineStr">
+        <is>
+          <t>クラウドゲーミングがXRヘッドセットの演算性能を肩代わりする流れ（GeForce Now×Quest/Vision Pro）は、通信・自動車など他業界の『性能のクラウド/エッジ移管』とどこまで同型か？</t>
+        </is>
+      </c>
+      <c r="C24" s="14" t="inlineStr">
+        <is>
+          <t>NVIDIA「GeForce Now」がQuest 3/S・Vision Pro・Pico対応（6/4）</t>
+        </is>
+      </c>
+      <c r="D24" s="14" t="inlineStr">
+        <is>
+          <t>NVIDIA, Meta, Apple/GeForce Now</t>
+        </is>
+      </c>
+      <c r="E24" s="14" t="inlineStr">
+        <is>
+          <t>通信（5G/エッジ）, 自動車（コネクテッド/車載演算）, PC・スマホ（端末性能のクラウド代替）</t>
+        </is>
+      </c>
+      <c r="F24" s="14" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="G24" s="14" t="inlineStr">
+        <is>
+          <t>既存の『オンデバイスAI主流化』論点と対をなす。デバイスの価値が自前性能か接続品質のどちらに寄るかで業界の競争軸が変わる。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3314,7 +3388,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L109"/>
+  <dimension ref="A1:L117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10247,6 +10321,490 @@
         </is>
       </c>
       <c r="L109" s="14" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B110" s="14" t="inlineStr">
+        <is>
+          <t>『ゼルダの伝説 時のオカリナ』Switch 2でフルリメイク、約28年ぶりに名作復活</t>
+        </is>
+      </c>
+      <c r="C110" s="14" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/article/202606/77809</t>
+        </is>
+      </c>
+      <c r="D110" s="14" t="inlineStr">
+        <is>
+          <t>1998年にNINTENDO 64で発売された3Dアクションの金字塔『時のオカリナ』。任天堂は2025年発売のSwitch 2の性能を活かし、後半商戦の目玉として往年の名作IPをリメイクで再投入する戦略を継続している。</t>
+        </is>
+      </c>
+      <c r="E110" s="14" t="inlineStr">
+        <is>
+          <t>Nintendo Direct 2026.6.9で、Switch 2向け『時のオカリナ』リメイクが発表され2026年内発売予定。現代グラフィックで再構築され、幼少期リンクが横たわる初映像のみ公開、ゲーム詳細は今後の続報となる。</t>
+        </is>
+      </c>
+      <c r="F110" s="14" t="inlineStr">
+        <is>
+          <t>・N64の名作を約28年ぶりにフルリメイク
+・対応はSwitch 2、2026年内発売予定
+・初出は短い映像のみで詳細は続報待ち
+・Switch 2後半商戦の中核タイトル</t>
+        </is>
+      </c>
+      <c r="G110" s="14" t="inlineStr">
+        <is>
+          <t>既存IPのリメイクはローンチ後のハード牽引に有効で、Switch 2普及拡大の起爆剤となる可能性。続編『ムジュラの仮面』系の展開や関連グッズも見込まれ、ホリデー商戦での販売台数押し上げが期待される。</t>
+        </is>
+      </c>
+      <c r="H110" s="14" t="inlineStr">
+        <is>
+          <t>名作IPのリメイク経済学とハード牽引効果</t>
+        </is>
+      </c>
+      <c r="I110" s="14" t="inlineStr">
+        <is>
+          <t>任天堂</t>
+        </is>
+      </c>
+      <c r="J110" s="14" t="inlineStr">
+        <is>
+          <t>ゼルダの伝説 時のオカリナ</t>
+        </is>
+      </c>
+      <c r="K110" s="14" t="inlineStr">
+        <is>
+          <t>新作,国内</t>
+        </is>
+      </c>
+      <c r="L110" s="14" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B111" s="14" t="inlineStr">
+        <is>
+          <t>『キングダム ハーツIV』Switch 2で発売決定、過去シリーズもSwitch 2版で展開</t>
+        </is>
+      </c>
+      <c r="C111" s="14" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/article/202606/77846</t>
+        </is>
+      </c>
+      <c r="D111" s="14" t="inlineStr">
+        <is>
+          <t>スクウェア・エニックスとディズニーの共同IP「キングダム ハーツ」。これまでPS/Xbox中心だった最新作が任天堂の新ハードにも対応し、マルチプラットフォーム展開を一段と強化する動きとなる。</t>
+        </is>
+      </c>
+      <c r="E111" s="14" t="inlineStr">
+        <is>
+          <t>Nintendo Direct 2026.6.9で『KINGDOM HEARTS IV』のSwitch 2版が発表。あわせて『1.5+2.5』『2.8』『3+リマインド』のSwitch 2版が10月8日配信、3作セットのコレクションも同時発売される。</t>
+        </is>
+      </c>
+      <c r="F111" s="14" t="inlineStr">
+        <is>
+          <t>・最新作KH4がSwitch 2に対応
+・過去作Switch 2版は10/8配信
+・3作セットのコレクションを同時展開
+・SEのマルチプラットフォーム戦略を象徴</t>
+        </is>
+      </c>
+      <c r="G111" s="14" t="inlineStr">
+        <is>
+          <t>大型RPGをSwitch 2へ広げることで携帯モードを含む新規層の取り込みが進む。SEは旧作移植で長期収益化を図りつつ、KH4本編の発売時期次第でホリデー商戦の競争が激化する見通し。</t>
+        </is>
+      </c>
+      <c r="H111" s="14" t="inlineStr">
+        <is>
+          <t>マルチプラットフォーム化とIP長期収益化</t>
+        </is>
+      </c>
+      <c r="I111" s="14" t="inlineStr">
+        <is>
+          <t>スクウェア・エニックス, ディズニー, 任天堂</t>
+        </is>
+      </c>
+      <c r="J111" s="14" t="inlineStr">
+        <is>
+          <t>キングダム ハーツ</t>
+        </is>
+      </c>
+      <c r="K111" s="14" t="inlineStr">
+        <is>
+          <t>新作,国内,海外</t>
+        </is>
+      </c>
+      <c r="L111" s="14" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B112" s="14" t="inlineStr">
+        <is>
+          <t>『ゼノブレイド ジェネシス』発表、高橋哲哉総監督の新作RPGが2027年Switch 2で登場</t>
+        </is>
+      </c>
+      <c r="C112" s="14" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/article/202606/77842</t>
+        </is>
+      </c>
+      <c r="D112" s="14" t="inlineStr">
+        <is>
+          <t>モノリスソフトが手掛ける任天堂のRPG「ゼノブレイド」シリーズ。前作群の世界観を引き継ぎつつ、Switch 2世代の旗艦RPGとしてシリーズの新生を打ち出す位置づけとなる。</t>
+        </is>
+      </c>
+      <c r="E112" s="14" t="inlineStr">
+        <is>
+          <t>Nintendo Direct 2026.6.9で新作『ゼノブレイド ジェネシス』を発表、2027年Switch 2発売予定。総監督は高橋哲哉氏、音楽は光田康典氏ら。「アニマ」が万物を形作る世界「アンシャル」が舞台となる。</t>
+        </is>
+      </c>
+      <c r="F112" s="14" t="inlineStr">
+        <is>
+          <t>・シリーズ完全新作、2027年Switch 2発売
+・総監督は高橋哲哉氏が続投
+・音楽は光田康典氏らが担当
+・あわせて旧3部作のSwitch 2版も発表</t>
+        </is>
+      </c>
+      <c r="G112" s="14" t="inlineStr">
+        <is>
+          <t>2027年発売のため当面は情報を小出しにしファン期待を醸成。旧3部作のSwitch 2版を先行投入し新規層を取り込みつつ、Switch 2の長期ソフト供給の柱とする狙い。モノリスの開発体制拡大も注目される。</t>
+        </is>
+      </c>
+      <c r="H112" s="14" t="inlineStr">
+        <is>
+          <t>ファーストRPGの長期IP育成戦略</t>
+        </is>
+      </c>
+      <c r="I112" s="14" t="inlineStr">
+        <is>
+          <t>任天堂, モノリスソフト</t>
+        </is>
+      </c>
+      <c r="J112" s="14" t="inlineStr">
+        <is>
+          <t>ゼノブレイド</t>
+        </is>
+      </c>
+      <c r="K112" s="14" t="inlineStr">
+        <is>
+          <t>新作,国内</t>
+        </is>
+      </c>
+      <c r="L112" s="14" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B113" s="14" t="inlineStr">
+        <is>
+          <t>『ファイアーエムブレム 万紫千紅』9月17日発売決定、『風花雪月』と繋がる世界設定</t>
+        </is>
+      </c>
+      <c r="C113" s="14" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/article/202606/77806</t>
+        </is>
+      </c>
+      <c r="D113" s="14" t="inlineStr">
+        <is>
+          <t>任天堂・インテリジェントシステムズのSRPG「ファイアーエムブレム」シリーズ最新作。2025年に発表済みで、今回のダイレクトで発売日と具体的な世界観・価格が確定した。</t>
+        </is>
+      </c>
+      <c r="E113" s="14" t="inlineStr">
+        <is>
+          <t>Nintendo Direct 2026.6.9で『FE 万紫千紅』の発売日が9月17日に決定。Switch 2対応で4人の主人公や『風花雪月』と繋がる世界観を公開。価格はパッケージ14,980円、DL版13,980円となる。</t>
+        </is>
+      </c>
+      <c r="F113" s="14" t="inlineStr">
+        <is>
+          <t>・発売日は9月17日に確定
+・4人の主人公制を採用
+・『風花雪月』と繋がる世界設定
+・価格はパッケージ14,980円/DL13,980円</t>
+        </is>
+      </c>
+      <c r="G113" s="14" t="inlineStr">
+        <is>
+          <t>秋商戦の先陣を切るファーストRPG。過去作『風花雪月』との世界観連動でシリーズファンの購買を喚起。Switch 2専用としてハード牽引も担い、年末商戦に向けた話題形成の起点となる。</t>
+        </is>
+      </c>
+      <c r="H113" s="14" t="inlineStr">
+        <is>
+          <t>シリーズ世界観連動による需要喚起</t>
+        </is>
+      </c>
+      <c r="I113" s="14" t="inlineStr">
+        <is>
+          <t>任天堂, インテリジェントシステムズ</t>
+        </is>
+      </c>
+      <c r="J113" s="14" t="inlineStr">
+        <is>
+          <t>ファイアーエムブレム</t>
+        </is>
+      </c>
+      <c r="K113" s="14" t="inlineStr">
+        <is>
+          <t>新作,国内</t>
+        </is>
+      </c>
+      <c r="L113" s="14" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B114" s="14" t="inlineStr">
+        <is>
+          <t>『FF10/10-2 HDリマスター』Switch 2版が7月23日配信、25周年記念パッケージも</t>
+        </is>
+      </c>
+      <c r="C114" s="14" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/article/202606/77755</t>
+        </is>
+      </c>
+      <c r="D114" s="14" t="inlineStr">
+        <is>
+          <t>2001年発売『FFX』の25周年を控え、スクウェア・エニックスは旧作の新ハード移植を加速。Switch 2のローンチ期ソフト拡充の一環として位置づけられる。</t>
+        </is>
+      </c>
+      <c r="E114" s="14" t="inlineStr">
+        <is>
+          <t>Nintendo Direct 2026.6.9で『FF10/10-2 HDリマスター』Switch 2版を発表。DL版は7月23日、25周年記念ケース付きパッケージ版は8月27日発売。価格はDL6,688円、パッケージ7,480円となる。</t>
+        </is>
+      </c>
+      <c r="F114" s="14" t="inlineStr">
+        <is>
+          <t>・Switch 2版DLは7/23、パッケージは8/27
+・FFX 25周年記念スリーブケース付属
+・価格はDL6,688円/パッケージ7,480円
+・SEの旧作移植による収益化策</t>
+        </is>
+      </c>
+      <c r="G114" s="14" t="inlineStr">
+        <is>
+          <t>低コストの旧作リマスター移植は安定収益源。25周年記念で関連作の移植やグッズ展開が続く可能性。Switch 2のライブラリ拡充でハード初期需要を下支えし、長期のロングテール販売が見込まれる。</t>
+        </is>
+      </c>
+      <c r="H114" s="14" t="inlineStr">
+        <is>
+          <t>旧作リマスターのロングテール収益</t>
+        </is>
+      </c>
+      <c r="I114" s="14" t="inlineStr">
+        <is>
+          <t>スクウェア・エニックス</t>
+        </is>
+      </c>
+      <c r="J114" s="14" t="inlineStr">
+        <is>
+          <t>ファイナルファンタジーX</t>
+        </is>
+      </c>
+      <c r="K114" s="14" t="inlineStr">
+        <is>
+          <t>新作,国内</t>
+        </is>
+      </c>
+      <c r="L114" s="14" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B115" s="14" t="inlineStr">
+        <is>
+          <t>NVIDIA「GeForce Now」がQuest 3/S・Vision Pro・Picoに対応、XRでクラウドゲーミング</t>
+        </is>
+      </c>
+      <c r="C115" s="14" t="inlineStr">
+        <is>
+          <t>https://roadtovr.com/nvidia-cloud-gaming-quest-3-vision-pro-pico/</t>
+        </is>
+      </c>
+      <c r="D115" s="14" t="inlineStr">
+        <is>
+          <t>高性能GPUを自前で持たずに高画質ゲームを遊べるクラウドゲーミングが、ヘッドセットの処理能力・発熱という課題を補う手段として注目される。XRの普及拡大が業界の大きなテーマとなっている。</t>
+        </is>
+      </c>
+      <c r="E115" s="14" t="inlineStr">
+        <is>
+          <t>NVIDIAは6月4日、クラウドゲーミング「GeForce Now」をMeta Quest 3/3S、Apple Vision Pro、Picoの各ヘッドセットに対応させると発表。端末側の演算性能に依存せず大型PCゲームを大画面・低遅延で配信する。</t>
+        </is>
+      </c>
+      <c r="F115" s="14" t="inlineStr">
+        <is>
+          <t>・主要XRヘッドセットでGeForce Nowが利用可能に
+・端末性能に依存しないクラウド配信
+・スマートグラス時代を見据えた布石
+・Sony/MicrosoftよりNVIDIAが先行</t>
+        </is>
+      </c>
+      <c r="G115" s="14" t="inlineStr">
+        <is>
+          <t>オンデバイス性能の制約をクラウドが肩代わりする流れが加速。スマートグラスやライト級ヘッドセットでもAAA級体験が可能になり、通信品質（低遅延・5G/エッジ）が新たな競争軸として浮上する。</t>
+        </is>
+      </c>
+      <c r="H115" s="14" t="inlineStr">
+        <is>
+          <t>クラウドゲーミングとXR/エッジ通信の融合</t>
+        </is>
+      </c>
+      <c r="I115" s="14" t="inlineStr">
+        <is>
+          <t>NVIDIA, Meta, Apple, ByteDance(Pico)</t>
+        </is>
+      </c>
+      <c r="J115" s="14" t="inlineStr">
+        <is>
+          <t>GeForce Now</t>
+        </is>
+      </c>
+      <c r="K115" s="14" t="inlineStr">
+        <is>
+          <t>技術,海外</t>
+        </is>
+      </c>
+      <c r="L115" s="14" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B116" s="14" t="inlineStr">
+        <is>
+          <t>eスポーツ「REJECT」Apex部門が『Esports World Cup 2026』パリ大会出場権を獲得</t>
+        </is>
+      </c>
+      <c r="C116" s="14" t="inlineStr">
+        <is>
+          <t>https://prtimes.jp/main/html/rd/p/000000548.000050979.html</t>
+        </is>
+      </c>
+      <c r="D116" s="14" t="inlineStr">
+        <is>
+          <t>サウジ主導の世界最大級eスポーツ大会EWCは賞金規模が突出。各タイトルの地域予選を勝ち抜いた強豪が集結し、日本勢の国際大会での存在感が問われる場となっている。</t>
+        </is>
+      </c>
+      <c r="E116" s="14" t="inlineStr">
+        <is>
+          <t>日本のeスポーツチームREJECTのApex Legends部門が、APAC North（4/5〜6/7開催）で2位となりEsports World Cup 2026の出場権を獲得。EWCのApex部門は7月7〜11日にフランス・パリで開催される。</t>
+        </is>
+      </c>
+      <c r="F116" s="14" t="inlineStr">
+        <is>
+          <t>・REJECT Apex部門がEWC2026出場権獲得
+・APAC North予選で2位通過
+・EWC Apexは7/7〜11にパリ開催
+・日本勢の国際大会での競争力向上</t>
+        </is>
+      </c>
+      <c r="G116" s="14" t="inlineStr">
+        <is>
+          <t>EWCの賞金・露出規模の拡大で国内チームの国際志向が強まる。スポンサー（食品・通信等）との連携で選手育成・栄養面投資が進み、eスポーツの事業化・プロ化が加速。視聴のグローバル化も収益機会を広げる。</t>
+        </is>
+      </c>
+      <c r="H116" s="14" t="inlineStr">
+        <is>
+          <t>eスポーツの国際大会経済とスポンサー構造</t>
+        </is>
+      </c>
+      <c r="I116" s="14" t="inlineStr">
+        <is>
+          <t>REJECT, Esports World Cup Foundation, Electronic Arts</t>
+        </is>
+      </c>
+      <c r="J116" s="14" t="inlineStr">
+        <is>
+          <t>Apex Legends</t>
+        </is>
+      </c>
+      <c r="K116" s="14" t="inlineStr">
+        <is>
+          <t>eスポーツ,国内,海外</t>
+        </is>
+      </c>
+      <c r="L116" s="14" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B117" s="14" t="inlineStr">
+        <is>
+          <t>2026年上半期の米ゲーム市場は不安定な滑り出し、新作販売の伸び鈍化（Luminate）</t>
+        </is>
+      </c>
+      <c r="C117" s="14" t="inlineStr">
+        <is>
+          <t>https://luminatedata.com/blog/gaming-industry-off-to-a-shaky-2026/</t>
+        </is>
+      </c>
+      <c r="D117" s="14" t="inlineStr">
+        <is>
+          <t>2025年は大型新作が市場を牽引したが、2026年前半は新作の端境期とハード移行期が重なり販売の勢いに陰り。記録的な業界収益の裏で構造的なレイオフも継続している。</t>
+        </is>
+      </c>
+      <c r="E117" s="14" t="inlineStr">
+        <is>
+          <t>調査会社Luminateは、2026年前半の米ゲーム市場が新作販売の伸び悩みで不安定な立ち上がりとなったと分析。記録的収益の一方でAAA/中堅スタジオの人員削減が続き、収益と雇用の乖離が鮮明になっている。</t>
+        </is>
+      </c>
+      <c r="F117" s="14" t="inlineStr">
+        <is>
+          <t>・2026年前半の新作販売は勢い鈍化
+・ハード移行期と新作端境期が重なる
+・記録的収益でも構造的レイオフ継続
+・収益と雇用の乖離が顕著</t>
+        </is>
+      </c>
+      <c r="G117" s="14" t="inlineStr">
+        <is>
+          <t>下半期は大型タイトル投入で持ち直しを図るが、開発費高騰とAIによる効率化圧力で雇用環境は厳しいまま。少数精鋭・高生産性モデルへ移行し、確実性の高いIP・リマスターへ投資が集中する見通し。</t>
+        </is>
+      </c>
+      <c r="H117" s="14" t="inlineStr">
+        <is>
+          <t>ゲーム市場の収益と雇用の構造的乖離</t>
+        </is>
+      </c>
+      <c r="I117" s="14" t="inlineStr">
+        <is>
+          <t>Electronic Arts, Ubisoft, Epic Games</t>
+        </is>
+      </c>
+      <c r="J117" s="14" t="inlineStr"/>
+      <c r="K117" s="14" t="inlineStr">
+        <is>
+          <t>業績,海外</t>
+        </is>
+      </c>
+      <c r="L117" s="14" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
weekly-trends + tech update (2026-06-10 03:09)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -1182,7 +1182,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1709,6 +1709,117 @@
       <c r="G14" s="3" t="inlineStr">
         <is>
           <t>https://screenrant.com/steam-june-2026-trending-free-game/ , https://www.gamegrin.com/news/top-19-new-steam-games-this-week-1st7th-of-june-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>ニンダイ6.9が示すSwitch 2の非独占マルチ化とリメイク依存</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>6月9日配信の「Nintendo Direct 2026.6.9」(約50分)は2026年後半のSwitch 2/Switch向け新作を中心に紹介。看板は『ゼルダの伝説 時のオカリナ』の約28年越しリメイク、『キングダム ハーツ4』Switch 2版、『ゼノブレイド』3作のSwitch 2エディションと新作『ゼノブレイド ジェネシス』など、既存IPのリメイク/リマスター/移植が中心だった。サードはドラゴンクエストモンスターズ4、鬼武者 Way of the Sword、信長の野望・飛翔、朧村正などが多数並んだが、その大半はPS5等とのマルチ展開で、Switch 2独占は限定的。発売1年を経てサード参入は量的に拡大した一方、『独占の薄さ』と『任天堂自身のリメイク依存』が同じ回で同時に可視化された。</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>任天堂, スクウェア・エニックス, バンダイナムコ, カプコン, コーエーテクモ, ゼルダの伝説, キングダムハーツ, ゼノブレイド</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Switch 2は性能向上でPS5世代マルチの『最小公倍数』に乗りやすくなり、サードはデイワン/同発を増やせる半面、専用最適化や独占契約のコストは負いにくい。結果、サードにとってSwitch 2は『追加販路』化し、プラットフォーム差別化はファースト＋旧作IPのリメイクに依存しやすくなる。任天堂は新規IPリスクを抑え普及初期の弾を旧資産で確保する戦略だが、マルチ前提が進むほどハード独自価値の訴求は難しくなる。</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>独占ではなく『普及台数×旧IP在庫』で戦うモデルは、配信PFやストリーミングの旧作ライブラリ戦略と同型。差別化軸が体験から品揃え/移植速度へ移る兆し。</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/999/G999905/20260608100/ , https://www.famitsu.com/article/202606/77772</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>AI音声複製を巡る労使紛争：SAG-AFTRA対Epic（Fortnite）</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>SAG-AFTRAは、Epic Games子会社Llama Productionsが団体交渉や事前通知なくAIでダース・ベイダーの音声を複製したとして不当労働行為(ULP)を申し立てた。2024年7月開始のAI保護を巡るゲーム声優ストは2025年7月に新契約で妥結し、声優は自分の声のAI利用可否を強く管理できるようになったが、運用段階の摩擦は続く。並行して、人手によるキュレーションを欠いたAI量産タイトル『gameslop』がストアに氾濫し、2025〜26年はキーアートの無開示AIや使い回し台詞への反発が相次いだ。2026年は『アートが人間制作か、声がクレジット済み実演者か』をプレイヤーが知る権利＝開示が、業界の信頼維持の前提と位置づけられた。</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Epic Games, Llama Productions, SAG-AFTRA, Fortnite, Inworld AI, NVIDIA ACE</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>AIは『裏方の効率化』と『プレイヤーが触れる成果物(声・顔・台詞)』で社会的許容度が割れる。前者は静かに浸透するが、後者は実演者の同一性・労務契約・パブリシティ権に直結し、団体交渉の射程に入る。LLM駆動NPCの普及で『声・人格の継続利用』が常態化するほど、事前合意と開示の制度設計が競争条件になる。開示は規制ではなく信頼の通貨として機能し始めた。</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>生成物の『出自表示』が品質シグナル化する流れは、映像・音楽・出版のクレジット/電子透かし議論と接続。労務×IP×消費者保護が一点で交差する。</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Artificial_intelligence_in_video_games , https://beyondtmrw.org/article/generative-ai-in-game-development-npcs-assets-and-ip-risk</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>記録的売上×記録的レイオフ：Netflixのゲーム参入と資本集約</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>2025年の世界ゲーム市場は約1,956億ドルと過去最高を更新した一方、過去2年で世界の開発者の28%(米国は33%)が職を失う『増収×人員削減』のパラドックスが続く。2026年は4月中旬時点で推定3,300人のレイオフ、13スタジオ閉鎖。Ubisoftはパリ本社の人員削減を含む大規模再編とスタジオ閉鎖を発表し、Microsoftは会計年度末(6/30)までに数年来最大級のレイオフを見込む。資本面では、Netflixが映画・HBOを含むWarner Bros.全体を買収する案件が進行し、縮小したWBのゲーム部門も対象に。Sonyはライブサービス路線を縮小し、2022年買収のBungieはMarathon難航でチーム縮小。市場拡大の果実が一部の巨大資本に集約されつつある。</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Ubisoft, Microsoft/Xbox, Netflix, Warner Bros., Sony, Bungie, Marathon</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>売上拡大とレイオフが両立するのは、(1)ヒットの寡占化と長期化する開発費、(2)ライブサービス失敗の人件費直撃、(3)AI/外注による工程圧縮、(4)金利環境下での資本効率優先、が重なるため。結果、IP・配信網・資本を持つ少数のプラットフォーマー(Microsoft, Sony, Tencent, そしてNetflix)への集約が進み、中堅スタジオは買収か清算かの二択に追われる。『作る人』の余剰が恒常化する成熟産業の典型。</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>増収下の人員削減はストリーミング・SaaSと同型の『勝者総取り＋効率化』局面。Netflixのゲーム参入は配信×ゲームの統合競争の号砲になりうる。</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>https://respawn.outlookindia.com/gaming/gaming-news/record-profits-record-layoffs-inside-gamings-2026-paradox , https://gamerant.com/every-video-game-layoff-and-studio-closure-in-2026-so-far/</t>
         </is>
       </c>
     </row>
@@ -15080,7 +15191,7 @@
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B2" s="9" t="inlineStr">
@@ -15095,32 +15206,32 @@
       </c>
       <c r="D2" s="9" t="inlineStr">
         <is>
-          <t>GDC 2026調査で開発者の52%が生成AIを『業界に害』と回答（ビジュアル/技術アート64%が否定的）。Steamは1月にAI開示を二層化＝プレイヤーが消費するコンテンツと裏方の効率化ツールを区別。</t>
+          <t>AI保護を巡る2024-25年のゲーム声優ストは新契約で妥結も、運用段階の摩擦が継続。LLM駆動NPC(Inworld/NVIDIA ACE)の実装拡大で『声・人格の継続利用』が現実問題に。</t>
         </is>
       </c>
       <c r="E2" s="9" t="inlineStr">
         <is>
-          <t>Larianが反発を受けgenAI使用を『控える』と表明、Jurassic World Evolution 3はAI生成ポートレートを撤回。開示済みは7,300本超。</t>
+          <t>SAG-AFTRAがEpic子会社Llama Productionsを、団交・事前通知なくAIでダース・ベイダー音声を複製したとしてULP申立て。『gameslop』氾濫を背景に、人間制作/クレジット済み実演者の開示が信頼維持の前提に。</t>
         </is>
       </c>
       <c r="F2" s="9" t="inlineStr">
         <is>
-          <t>Valve, Larian, Frontier, GDC, 各AAAパブリッシャー</t>
+          <t>Epic Games, Llama Productions, SAG-AFTRA, Inworld AI, NVIDIA</t>
         </is>
       </c>
       <c r="G2" s="9" t="inlineStr">
         <is>
-          <t>ランタイム生成（動的NPC会話）への表示要求・規制が次の焦点。経営の推進と現場の反発の溝は当面埋まらず。</t>
+          <t>ランタイム生成(声・人格)の常態化で、事前合意と出自開示が競争条件化。労務×IP×消費者保護が交差点に。</t>
         </is>
       </c>
       <c r="H2" s="9" t="inlineStr">
         <is>
-          <t>AIは『裏方の効率化』と『プレイヤーが見る成果物』で社会的許容度が分岐。境界設計が論点。</t>
+          <t>開示は規制ではなく『信頼の通貨』として機能し始めた。裏方効率化と成果物で許容度が分岐。</t>
         </is>
       </c>
       <c r="I2" s="9" t="inlineStr">
         <is>
-          <t>https://www.pcgamer.com/software/ai/steam-updates-ai-disclosure-form-to-specify-that-its-focused-on-ai-generated-content-that-is-consumed-by-players-not-efficiency-tools-used-behind-the-scenes/</t>
+          <t>https://en.wikipedia.org/wiki/Artificial_intelligence_in_video_games</t>
         </is>
       </c>
       <c r="J2" s="9" t="inlineStr"/>
@@ -15308,7 +15419,7 @@
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
@@ -15323,14 +15434,34 @@
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>EU AI Act、米FTC、ガチャ規制</t>
-        </is>
-      </c>
-      <c r="E8" s="9" t="inlineStr"/>
-      <c r="F8" s="9" t="inlineStr"/>
-      <c r="G8" s="9" t="inlineStr"/>
-      <c r="H8" s="9" t="inlineStr"/>
-      <c r="I8" s="9" t="inlineStr"/>
+          <t>EUはルートボックス/ガチャを『ダークパターン×消費者保護(特に未成年)』として捉える方向。蘭・白は最も厳格でループボックスを賭博として規制。Digital Fairness Actの草案公表が射程に。</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>全面禁止は2026年内には見込み薄も、Digital Fairness Actで開示・支出上限・データ透明性の各国ルールが収斂へ。グローバル各社は地域別の『デュアルデザイン』出荷が常態化。</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>欧州委員会, EA, 各F2Pパブリッシャー</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>確率/UI/支出上限/データの地域差を前提とした設計が標準化。日本は自主規制継続で欧州の硬化と対照的。</t>
+        </is>
+      </c>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>規制は『禁止』より『開示と上限』へ。同一ゲームが地域別に別設計化する分断が進む。</t>
+        </is>
+      </c>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>https://medium.com/@minsu057/gacha-at-a-crossroads-how-europe-regulates-while-japan-self-regulates-e32dfc5a8623</t>
+        </is>
+      </c>
       <c r="J8" s="9" t="inlineStr"/>
     </row>
     <row r="9">
@@ -15460,7 +15591,7 @@
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="B12" s="9" t="inlineStr">
@@ -15475,32 +15606,32 @@
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>発売1年未満で異例の価格改定が実施され、本体は品薄基調。</t>
+          <t>6/9配信『Nintendo Direct 2026.6.9』(約50分)で2026年後半のSwitch 2/Switch新作を多数公開。看板は『ゼルダ 時のオカリナ』約28年越しリメイク、『KH4』Switch 2版、『ゼノブレイド』3作Switch 2版＋新作『ジェネシス』。</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>5/25より日本国内専用機が49,980→59,980円に改定（+1万円）。マイニンテンドーストアの購入条件『Switchプレイ時間50時間以上』が撤廃。2026はサードのデイワン投入拡大の見通し。</t>
+          <t>サードはドラクエモンスターズ4・鬼武者・信長の野望・朧村正など多数並ぶが大半が他機種とのマルチ。『独占の薄さ』と任天堂自身の旧作リメイク依存が同時に可視化された。</t>
         </is>
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>任天堂, サードパーティ各社</t>
+          <t>任天堂, スクウェア・エニックス, バンダイナムコ, カプコン, コーエーテクモ</t>
         </is>
       </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
-          <t>メモリ高騰起点の値上げが9月に欧米MSRPへ波及する可能性。需要が吸収すれば強気の供給戦略を継続。</t>
+          <t>サードはSwitch 2を『追加販路』としてデイワン/同発を拡大。差別化はファースト＋移植速度に依存し、独占獲得競争は限定的に推移。</t>
         </is>
       </c>
       <c r="H12" s="9" t="inlineStr">
         <is>
-          <t>ハード値上げを需要が吸収できるかが普及曲線の分岐点。値上げ連鎖は他ハードにも波及し得る。</t>
+          <t>普及2年目は『独占で勝つ』から『台数×旧IP在庫で回す』局面へ。配信PFの旧作ライブラリ戦略と同型。</t>
         </is>
       </c>
       <c r="I12" s="9" t="inlineStr">
         <is>
-          <t>https://www.famitsu.com/article/202605/75886</t>
+          <t>https://www.4gamer.net/games/999/G999905/20260608100/</t>
         </is>
       </c>
       <c r="J12" s="9" t="inlineStr"/>

</xml_diff>

<commit_message>
daily-news + cross-questions update (2026-06-11 01:11)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -2588,7 +2588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3488,6 +3488,80 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B25" s="14" t="inlineStr">
+        <is>
+          <t>巨額先行投資（5年200億ドル）の回収難による事業『リセット』と人員削減は、動画配信・クラウド・通信など他の固定費先行型プラットフォーム産業でも同様に起きるか？</t>
+        </is>
+      </c>
+      <c r="C25" s="14" t="inlineStr">
+        <is>
+          <t>Xbox大規模レイオフ計画報道（Bloomberg 6/10）</t>
+        </is>
+      </c>
+      <c r="D25" s="14" t="inlineStr">
+        <is>
+          <t>Microsoft/Xbox, Game Pass</t>
+        </is>
+      </c>
+      <c r="E25" s="14" t="inlineStr">
+        <is>
+          <t>動画配信（コンテンツ投資回収）, 通信（5G設備投資）, クラウド（DC投資）, 広告（プラットフォーム間競争）</t>
+        </is>
+      </c>
+      <c r="F25" s="14" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="G25" s="14" t="inlineStr">
+        <is>
+          <t>コンテンツ投資額と利益率の乖離が限界に達した時、サブスクは値上げ・規模縮小・マルチ展開のどれを選ぶか。NetflixやDisney+の先行事例との比較が有効。</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B26" s="14" t="inlineStr">
+        <is>
+          <t>国家の遮断措置に対しプラットフォームが規制要求を受け入れて市場復帰する『順守と引き換えの再参入』は、SNS・動画配信・ECなど他業界でも標準的な交渉モデルになるか？</t>
+        </is>
+      </c>
+      <c r="C26" s="14" t="inlineStr">
+        <is>
+          <t>ロシアのRoblox遮断解除（6/10）</t>
+        </is>
+      </c>
+      <c r="D26" s="14" t="inlineStr">
+        <is>
+          <t>Roblox, Roskomnadzor</t>
+        </is>
+      </c>
+      <c r="E26" s="14" t="inlineStr">
+        <is>
+          <t>SNS（各国の年齢認証規制）, 動画配信（コンテンツ検閲対応）, EC（データローカライゼーション）, 金融（ライセンス再取得）</t>
+        </is>
+      </c>
+      <c r="F26" s="14" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="G26" s="14" t="inlineStr">
+        <is>
+          <t>市場規模と規制コストの天秤で各社の判断が割れる。子ども・ユーザー世論が政府側を動かした点は、規制当局にとっても撤回コストの存在を示した。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3499,7 +3573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L117"/>
+  <dimension ref="A1:L123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10916,6 +10990,378 @@
         </is>
       </c>
       <c r="L117" s="14" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B118" s="14" t="inlineStr">
+        <is>
+          <t>フロム新作『ダスクブラッド』クローズドネットワークテストを2026年夏に実施へ</t>
+        </is>
+      </c>
+      <c r="C118" s="14" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/article/202606/77818</t>
+        </is>
+      </c>
+      <c r="D118" s="14" t="inlineStr">
+        <is>
+          <t>Nintendo Direct 2026.6.9でフロム・ソフトウェアのSwitch 2専用完全新作『The Duskbloods』の続報が公開。本作は最大8人によるPvPvEマルチプレイアクションで、2026年発売予定。新トレイラーで世界観も初披露された。</t>
+        </is>
+      </c>
+      <c r="E118" s="14" t="inlineStr">
+        <is>
+          <t>クローズドネットワークテストが2026年夏に開催決定。テスター応募の詳細は後日、公式サイトとフロム公式Xで告知予定。発売前に大規模マルチプレイの負荷・バランス検証を行う狙いで、発売時期確定に向けた重要な節目となる。</t>
+        </is>
+      </c>
+      <c r="F118" s="14" t="inlineStr">
+        <is>
+          <t>Switch 2専用の完全新作PvPvEアクション
+2026年夏にクローズドネットワークテスト実施
+最大8人マルチプレイの検証が主目的
+テスター募集詳細は後日発表
+2026年内発売予定を維持</t>
+        </is>
+      </c>
+      <c r="G118" s="14" t="inlineStr">
+        <is>
+          <t>CNTの結果次第で2026年内発売の現実味が判明する。フロム初の本格マルチ専用タイトルとして、エルデンリング級のヒットになるかが任天堂のSwitch 2サードパーティ戦略の試金石になる。</t>
+        </is>
+      </c>
+      <c r="H118" s="14" t="inlineStr">
+        <is>
+          <t>PvPvE・運営型マルチタイトルの収益設計</t>
+        </is>
+      </c>
+      <c r="I118" s="14" t="inlineStr">
+        <is>
+          <t>フロム・ソフトウェア, 任天堂, KADOKAWA</t>
+        </is>
+      </c>
+      <c r="J118" s="14" t="inlineStr">
+        <is>
+          <t>The Duskbloods, ELDEN RING</t>
+        </is>
+      </c>
+      <c r="K118" s="14" t="inlineStr">
+        <is>
+          <t>新作,国内</t>
+        </is>
+      </c>
+      <c r="L118" s="14" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B119" s="14" t="inlineStr">
+        <is>
+          <t>Microsoft、Xbox部門で大規模レイオフ計画と報道。新CEAsha Sharmaの下で事業「リセット」へ</t>
+        </is>
+      </c>
+      <c r="C119" s="14" t="inlineStr">
+        <is>
+          <t>https://www.bloomberg.com/news/articles/2026-06-10/xbox-plans-significant-layoffs-as-it-transforms-under-new-ceo-asha-sharma</t>
+        </is>
+      </c>
+      <c r="D119" s="14" t="inlineStr">
+        <is>
+          <t>Xbox部門は過去5年間でコンテンツ等に200億ドル超を投資した一方、年間売上は約5億ドル減少し利益率は3%まで低下。新CEOのAsha Sharmaは「事業は健全な状態にない」としてリセットを宣言していた。</t>
+        </is>
+      </c>
+      <c r="E119" s="14" t="inlineStr">
+        <is>
+          <t>Bloombergによると、Microsoftは6月30日の会計年度末直後にXbox部門で大規模な人員削減を計画。マーケティング等の予算も大幅削減の見通し。昨夏の約9,000人削減からちょうど1年での再リストラとなる。規模は未公表。</t>
+        </is>
+      </c>
+      <c r="F119" s="14" t="inlineStr">
+        <is>
+          <t>会計年度末（6/30）直後に大規模レイオフ実施見込み
+5年で200億ドル投資も利益率3%に低迷
+マーケティング等の予算も大幅削減へ
+昨夏9,000人削減に続く2年連続の大規模リストラ
+新CEO Sharma体制での事業再構築の一環</t>
+        </is>
+      </c>
+      <c r="G119" s="14" t="inlineStr">
+        <is>
+          <t>ハード依存からGame Pass・マルチプラットフォーム展開への移行が加速し、スタジオ閉鎖や タイトル中止が再び発生する可能性。7月の決算発表前後に正式発表が出る公算が大きい。</t>
+        </is>
+      </c>
+      <c r="H119" s="14" t="inlineStr">
+        <is>
+          <t>プラットフォーマーの投資回収モデルとサブスク経済</t>
+        </is>
+      </c>
+      <c r="I119" s="14" t="inlineStr">
+        <is>
+          <t>Microsoft, Xbox Game Studios, Activision Blizzard</t>
+        </is>
+      </c>
+      <c r="J119" s="14" t="inlineStr">
+        <is>
+          <t>Game Pass, Call of Duty, Halo</t>
+        </is>
+      </c>
+      <c r="K119" s="14" t="inlineStr">
+        <is>
+          <t>業績,海外</t>
+        </is>
+      </c>
+      <c r="L119" s="14" t="n"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B120" s="14" t="inlineStr">
+        <is>
+          <t>ロシア、Robloxの接続遮断を解除。年齢制限・モデレーション強化の受け入れと引き換えに</t>
+        </is>
+      </c>
+      <c r="C120" s="14" t="inlineStr">
+        <is>
+          <t>https://www.themoscowtimes.com/2026/06/10/russia-backs-down-on-roblox-ban-after-childrens-complaints-a92976</t>
+        </is>
+      </c>
+      <c r="D120" s="14" t="inlineStr">
+        <is>
+          <t>ロシアは2025年12月に「過激派コンテンツ等の拡散」を理由にRobloxを全面遮断していた。子どもたちからの不満が殺到する中、6月初旬にデジタル発展省がRoblox側と利用条件で合意したと発表していた。</t>
+        </is>
+      </c>
+      <c r="E120" s="14" t="inlineStr">
+        <is>
+          <t>ロシア当局は6月10日、Robloxが「ユーザー保護に関する法的要件を完全に順守した」として遮断を解除。年齢別アクセス制限の導入と、児童に有害なコンテンツへのモデレーション強化が解除の条件となった。</t>
+        </is>
+      </c>
+      <c r="F120" s="14" t="inlineStr">
+        <is>
+          <t>2025年12月の全面遮断から約半年で解除
+年齢別アクセス制限の導入が条件
+有害コンテンツのモデレーション強化を約束
+国家の規制要求にプラットフォームが応じた形
+児童ユーザーの世論が政策転換を後押し</t>
+        </is>
+      </c>
+      <c r="G120" s="14" t="inlineStr">
+        <is>
+          <t>「規制順守と引き換えの市場復帰」モデルが他の権威主義圏にも波及する可能性。Robloxの月間ユーザー回復が確認されれば、各国の年齢認証規制への先行対応事例として参照されそうだ。</t>
+        </is>
+      </c>
+      <c r="H120" s="14" t="inlineStr">
+        <is>
+          <t>プラットフォームの国別コンプライアンス戦略</t>
+        </is>
+      </c>
+      <c r="I120" s="14" t="inlineStr">
+        <is>
+          <t>Roblox, Roskomnadzor（ロシア通信監督庁）</t>
+        </is>
+      </c>
+      <c r="J120" s="14" t="inlineStr">
+        <is>
+          <t>Roblox</t>
+        </is>
+      </c>
+      <c r="K120" s="14" t="inlineStr">
+        <is>
+          <t>規制,海外</t>
+        </is>
+      </c>
+      <c r="L120" s="14" t="n"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B121" s="14" t="inlineStr">
+        <is>
+          <t>『パワフルプロ野球2026-2027』本日発売。サクセス30周年、WBCモード搭載</t>
+        </is>
+      </c>
+      <c r="C121" s="14" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/article/202606/77867</t>
+        </is>
+      </c>
+      <c r="D121" s="14" t="inlineStr">
+        <is>
+          <t>パワプロシリーズはサクセスモード初登場の『パワプロ3』（1996年）から30年。今作は2026年WBC開催イヤーに合わせ、大谷翔平選手を前作に続きアンバサダーに起用して開発された。</t>
+        </is>
+      </c>
+      <c r="E121" s="14" t="inlineStr">
+        <is>
+          <t>KONAMIは6月11日、Switch/PS4向けに『パワフルプロ野球2026-2027』を発売。WBCテーマの「サクセス」「対決！レジェンドバトル」や歴代キャラ集結シナリオを収録。通常版8,470円、パワフルエディション10,670円。</t>
+        </is>
+      </c>
+      <c r="F121" s="14" t="inlineStr">
+        <is>
+          <t>6月11日にSwitch/PS4で発売
+サクセス30周年記念作品
+WBCテーマのモードを搭載、実在選手も登場
+アンバサダーは大谷翔平選手
+プロ野球球団との発売記念コラボも実施</t>
+        </is>
+      </c>
+      <c r="G121" s="14" t="inlineStr">
+        <is>
+          <t>WBC本大会との相乗効果で販売が伸びる可能性が高い。スポーツ実名IPの年次タイトルとして、国内パッケージ市場の堅調さを測る指標になる。Switch 2対応版の有無も今後の注目点。</t>
+        </is>
+      </c>
+      <c r="H121" s="14" t="inlineStr">
+        <is>
+          <t>スポーツ実名IPのライセンスビジネス</t>
+        </is>
+      </c>
+      <c r="I121" s="14" t="inlineStr">
+        <is>
+          <t>KONAMI, NPB, MLB</t>
+        </is>
+      </c>
+      <c r="J121" s="14" t="inlineStr">
+        <is>
+          <t>パワフルプロ野球, eBASEBALL</t>
+        </is>
+      </c>
+      <c r="K121" s="14" t="inlineStr">
+        <is>
+          <t>新作,国内</t>
+        </is>
+      </c>
+      <c r="L121" s="14" t="n"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B122" s="14" t="inlineStr">
+        <is>
+          <t>『スプラトゥーン レイダース』7月23日発売、『DQモンスターズ4』12月3日発売が決定</t>
+        </is>
+      </c>
+      <c r="C122" s="14" t="inlineStr">
+        <is>
+          <t>https://game.watch.impress.co.jp/docs/news/2115639.html</t>
+        </is>
+      </c>
+      <c r="D122" s="14" t="inlineStr">
+        <is>
+          <t>6月9日配信の「ニンテンドーダイレクト 2026.6.9」では約50分にわたり2026年後半のSwitch/Switch 2タイトルが多数公開。前日までに既報の大型リメイク以外にも、シリーズ派生作や年末商戦タイトルの日程が確定した。</t>
+        </is>
+      </c>
+      <c r="E122" s="14" t="inlineStr">
+        <is>
+          <t>スピンオフ『スプラトゥーン レイダース』が7月23日発売、『ドラゴンクエストモンスターズ4』が12月3日発売に決定。『リズム天国 ミラクルスターズ』はオール新作80種超のリズムゲームを収録して発売予定。</t>
+        </is>
+      </c>
+      <c r="F122" s="14" t="inlineStr">
+        <is>
+          <t>スプラトゥーン初のスピンオフが7月23日発売
+DQモンスターズ4が12月3日発売で年末商戦の柱に
+リズム天国新作はオール新作80種以上収録
+マインクラフトやステラーブレイドのSwitch 2版も発表
+2026年後半のSwitch 2ラインナップが充実</t>
+        </is>
+      </c>
+      <c r="G122" s="14" t="inlineStr">
+        <is>
+          <t>夏〜年末までSwitch 2向け大型タイトルが途切れない布陣となり、ハード普及の第2波を狙う構え。サードパーティの移植加速で、Switch 2のマルチプラットフォーム標準化が進む。</t>
+        </is>
+      </c>
+      <c r="H122" s="14" t="inlineStr">
+        <is>
+          <t>任天堂IPのスピンオフ戦略と年末商戦設計</t>
+        </is>
+      </c>
+      <c r="I122" s="14" t="inlineStr">
+        <is>
+          <t>任天堂, スクウェア・エニックス</t>
+        </is>
+      </c>
+      <c r="J122" s="14" t="inlineStr">
+        <is>
+          <t>スプラトゥーン, ドラゴンクエストモンスターズ, リズム天国</t>
+        </is>
+      </c>
+      <c r="K122" s="14" t="inlineStr">
+        <is>
+          <t>新作,国内</t>
+        </is>
+      </c>
+      <c r="L122" s="14" t="n"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B123" s="14" t="inlineStr">
+        <is>
+          <t>『Destiny 2』最終大型アップデート「Monument of Triumph」配信、12年の物語に区切り</t>
+        </is>
+      </c>
+      <c r="C123" s="14" t="inlineStr">
+        <is>
+          <t>https://www.pcgamer.com/games/live/news/destiny-2s-final-update-live-coverage-of-the-end-of-an-era/</t>
+        </is>
+      </c>
+      <c r="D123" s="14" t="inlineStr">
+        <is>
+          <t>Bungieは5月に『Destiny 2』のアクティブ開発を6月9日の最終コンテンツ更新をもって終了すると発表済み。『Destiny 3』は承認されておらず、同社は新作『Marathon』を旗艦タイトルに据える方針。</t>
+        </is>
+      </c>
+      <c r="E123" s="14" t="inlineStr">
+        <is>
+          <t>最終アップデート「Monument of Triumph」が予定通り配信され、2014年の初代から続いたフランチャイズの活発な運営が事実上終了。サーバーは維持されゲームは引き続きプレイ可能だが、週次ブログ等の情報発信も順次終了する。</t>
+        </is>
+      </c>
+      <c r="F123" s="14" t="inlineStr">
+        <is>
+          <t>6月9日に最終コンテンツ更新を配信
+サーバー維持でプレイは継続可能
+Destiny 3は未承認、後継はMarathon
+週次の公式情報発信も終了へ
+12年続いたライブサービスの「サンセット」事例に</t>
+        </is>
+      </c>
+      <c r="G123" s="14" t="inlineStr">
+        <is>
+          <t>大型ライブサービスの「終わらせ方」の先行事例として業界の参照点になる。Marathonの成否がBungieとSIEの追加リストラ有無を左右し、ライブサービス偏重戦略の見直し論にも影響しそうだ。</t>
+        </is>
+      </c>
+      <c r="H123" s="14" t="inlineStr">
+        <is>
+          <t>ライブサービスゲームのサンセット設計</t>
+        </is>
+      </c>
+      <c r="I123" s="14" t="inlineStr">
+        <is>
+          <t>Bungie, Sony Interactive Entertainment</t>
+        </is>
+      </c>
+      <c r="J123" s="14" t="inlineStr">
+        <is>
+          <t>Destiny 2, Marathon</t>
+        </is>
+      </c>
+      <c r="K123" s="14" t="inlineStr">
+        <is>
+          <t>海外,業績</t>
+        </is>
+      </c>
+      <c r="L123" s="14" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
daily-news + cross-questions update (2026-06-11 23:14)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -2588,7 +2588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3562,6 +3562,80 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B27" s="14" t="inlineStr">
+        <is>
+          <t>プレイ実績（利用50時間以上）で購入資格を絞る任天堂の転売対策は、チケット・スニーカー・限定品ECの本人確認/実績連動販売にどこまで波及するか？</t>
+        </is>
+      </c>
+      <c r="C27" s="14" t="inlineStr">
+        <is>
+          <t>任天堂がSwitch 2多言語版に「プレイ時間50時間以上」購入条件を復活（6/11, AUTOMATON）</t>
+        </is>
+      </c>
+      <c r="D27" s="14" t="inlineStr">
+        <is>
+          <t>任天堂 / Nintendo Switch 2</t>
+        </is>
+      </c>
+      <c r="E27" s="14" t="inlineStr">
+        <is>
+          <t>チケット興行（転売規制）, アパレル/スニーカー（限定抽選）, EC（アカウント実績審査）, 金融（本人確認/KYC）</t>
+        </is>
+      </c>
+      <c r="F27" s="14" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="G27" s="14" t="inlineStr">
+        <is>
+          <t>「金を払えるか」ではなく「実際に使ってきたか」で顧客を選別する手法。ロイヤルティデータが購買資格そのものになる点が新しい。</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B28" s="14" t="inlineStr">
+        <is>
+          <t>課金設計そのものを年齢レーティングで縛るPEGI新基準は、アプリストア・動画配信・SNSの格付け制度における「機能ベース格付け」の先行例になるか？</t>
+        </is>
+      </c>
+      <c r="C28" s="14" t="inlineStr">
+        <is>
+          <t>PEGI「インタラクティブリスク」新基準が6月提出分から適用開始（ルートボックス=16+、NFT=18）</t>
+        </is>
+      </c>
+      <c r="D28" s="14" t="inlineStr">
+        <is>
+          <t>PEGI, EA, Epic Games / EA Sports FC</t>
+        </is>
+      </c>
+      <c r="E28" s="14" t="inlineStr">
+        <is>
+          <t>アプリストア（App Store/Google Playの年齢区分）, 動画配信（レコメンド/課金機能の格付け）, SNS（未成年向け機能制限）, 広告（ターゲティング規制）</t>
+        </is>
+      </c>
+      <c r="F28" s="14" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="G28" s="14" t="inlineStr">
+        <is>
+          <t>表現内容ではなく「収益メカニクス」を理由に年齢制限を課す初の大規模制度。法規制を待たず業界自主規制が実質的な課金規制として機能する構図。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3573,7 +3647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L123"/>
+  <dimension ref="A1:L133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11362,6 +11436,613 @@
         </is>
       </c>
       <c r="L123" s="14" t="n"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B124" s="14" t="inlineStr">
+        <is>
+          <t>Ubisoft、ウィニペグスタジオ閉鎖。R6モバイル含むレインボーシックス系を大幅縮小</t>
+        </is>
+      </c>
+      <c r="C124" s="14" t="inlineStr">
+        <is>
+          <t>https://www.techtimes.com/articles/318241/20260611/ubisoft-layoffs-2026-gut-rainbow-six-franchise-winnipeg-closed-380-jobs-risk.htm</t>
+        </is>
+      </c>
+      <c r="D124" s="14" t="inlineStr">
+        <is>
+          <t>UbisoftはTencent出資のVantage Studios設立など大規模再編の渦中にあり、固定費削減と主力IPへの集中を進めている。R6 Mobileはグローバル配信開始から数ヶ月だが、モバイル市場の獲得コスト高騰で収益化が難航していた。</t>
+        </is>
+      </c>
+      <c r="E124" s="14" t="inlineStr">
+        <is>
+          <t>Ubisoftが6月10日にウィニペグスタジオを閉鎖。同スタジオの約50人を含むR6 Mobile開発体制を縮小し、モントリオールのSiege本体チームからも約120人（チームの約12%）を他プロジェクトへ再配置。合計380人規模に影響が及ぶと報じられた。</t>
+        </is>
+      </c>
+      <c r="F124" s="14" t="inlineStr">
+        <is>
+          <t>・ウィニペグ閉鎖で65人超に影響、うち約50人がR6 Mobile担当
+・Siege本体からも120人を他プロジェクトへ異動（レイオフ扱いではない）
+・R6 Mobileは運営継続もリソースは大幅減
+・Vantage Studios体制下での選択と集中が加速</t>
+        </is>
+      </c>
+      <c r="G124" s="14" t="inlineStr">
+        <is>
+          <t>R6 Mobileは段階的な運営縮小からサービス終了検討に進む可能性がある。Ubisoft再編はTencentの影響力拡大と並行しており、不採算ライブサービスの整理が他IPにも波及。年内にさらなるスタジオ統廃合が出る公算が高い。</t>
+        </is>
+      </c>
+      <c r="H124" s="14" t="inlineStr">
+        <is>
+          <t>大手パブリッシャーの選択と集中とライブサービス整理</t>
+        </is>
+      </c>
+      <c r="I124" s="14" t="inlineStr">
+        <is>
+          <t>Ubisoft, Tencent, Vantage Studios</t>
+        </is>
+      </c>
+      <c r="J124" s="14" t="inlineStr">
+        <is>
+          <t>Rainbow Six Siege, Rainbow Six Mobile</t>
+        </is>
+      </c>
+      <c r="K124" s="14" t="inlineStr">
+        <is>
+          <t>業績,海外</t>
+        </is>
+      </c>
+      <c r="L124" s="14" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B125" s="14" t="inlineStr">
+        <is>
+          <t>任天堂株が一時7%安、ニンダイ6.9への失望売り。5ヶ月で3割下落と先行き不透明感</t>
+        </is>
+      </c>
+      <c r="C125" s="14" t="inlineStr">
+        <is>
+          <t>https://news.yahoo.co.jp/articles/f2e6b130a12727002e057e63232c70ce7d23ae77</t>
+        </is>
+      </c>
+      <c r="D125" s="14" t="inlineStr">
+        <is>
+          <t>任天堂株は2026年に入りメモリ価格高騰によるコスト懸念やSwitch 2の年末商戦の不透明感から軟調が続き、直近5ヶ月で30%超下落。6月9日のNintendo Directは時オカリメイクやKH4などを発表したが、市場が期待した完全新作の弾は限定的だった。</t>
+        </is>
+      </c>
+      <c r="E125" s="14" t="inlineStr">
+        <is>
+          <t>6月10日の東京市場で任天堂株が急落し、終値は前日比523円安の7,215円（-6.76%）。ニンダイ発表がリメイク・移植中心で投資家の期待に届かず失望売りが拡大。メモリ高騰や2026年後半のソフトラインナップへの不安も重なった。</t>
+        </is>
+      </c>
+      <c r="F125" s="14" t="inlineStr">
+        <is>
+          <t>・6/10終値7,215円、下落率6.76%
+・ニンダイ内容がリメイク/他機種移植中心と受け止められた
+・メモリ価格高騰がハード採算を圧迫する懸念
+・株価は直近5ヶ月で30%超下落</t>
+        </is>
+      </c>
+      <c r="G125" s="14" t="inlineStr">
+        <is>
+          <t>株価回復にはSwitch 2普及ペースの維持と完全新作の提示が必要。秋以降のポケモンや来期の大型タイトル発表が材料になる一方、メモリコストが続けば本体再値上げか利益率低下のどちらかを迫られ、決算ガイダンスへの警戒が続く。</t>
+        </is>
+      </c>
+      <c r="H125" s="14" t="inlineStr">
+        <is>
+          <t>ゲーム株のバリュエーションと発表イベントの株価感応度</t>
+        </is>
+      </c>
+      <c r="I125" s="14" t="inlineStr">
+        <is>
+          <t>任天堂</t>
+        </is>
+      </c>
+      <c r="J125" s="14" t="inlineStr">
+        <is>
+          <t>Nintendo Switch 2, ゼルダの伝説, キングダムハーツ</t>
+        </is>
+      </c>
+      <c r="K125" s="14" t="inlineStr">
+        <is>
+          <t>業績,国内</t>
+        </is>
+      </c>
+      <c r="L125" s="14" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B126" s="14" t="inlineStr">
+        <is>
+          <t>GameStopのコーエンCEO、eBay買収を断念せず。持分9%に引き上げ株主直接提案へ</t>
+        </is>
+      </c>
+      <c r="C126" s="14" t="inlineStr">
+        <is>
+          <t>https://finance.yahoo.com/markets/stocks/articles/gme-ryan-cohen-isn-t-181529258.html</t>
+        </is>
+      </c>
+      <c r="D126" s="14" t="inlineStr">
+        <is>
+          <t>GameStopは5月12日にeBay取締役会から1株125ドル・総額555億ドルの買収提案を「信頼性も魅力もない」と全会一致で拒絶された。コーエンCEOはミーム株で積み上げた94億ドルの手元資金と200億ドルの信用枠を背景に攻勢を続けている。</t>
+        </is>
+      </c>
+      <c r="E126" s="14" t="inlineStr">
+        <is>
+          <t>コーエンCEOがeBay買収を継続追求していると報道。6月5日にはeBayへの経済的持分を約9%まで引き上げ、取締役会を迂回して株主へ直接テンダーオファーを行う構えを示した。GameStopのQ1決算はeBay株含み益2.68億ドルを含み過去最高益となった。</t>
+        </is>
+      </c>
+      <c r="F126" s="14" t="inlineStr">
+        <is>
+          <t>・eBay持分を約9%へ引き上げ
+・1株125ドル提案を株主に直接提示する敵対的TOBを準備
+・資金は手元94億ドル＋200億ドル信用枠
+・GameStop Q1は含み益込みで過去最高益</t>
+        </is>
+      </c>
+      <c r="G126" s="14" t="inlineStr">
+        <is>
+          <t>eBay側はポイズンピル等の買収防衛策導入が濃厚で、委任状争奪戦に発展する可能性がある。成立すればゲーム小売とECマーケットプレイスの統合という異例の再編。不成立でも株価変動を通じてGameStopの投資会社化がさらに進む。</t>
+        </is>
+      </c>
+      <c r="H126" s="14" t="inlineStr">
+        <is>
+          <t>敵対的TOBと買収防衛策の攻防</t>
+        </is>
+      </c>
+      <c r="I126" s="14" t="inlineStr">
+        <is>
+          <t>GameStop, eBay</t>
+        </is>
+      </c>
+      <c r="J126" s="14" t="inlineStr"/>
+      <c r="K126" s="14" t="inlineStr">
+        <is>
+          <t>M&amp;A,海外</t>
+        </is>
+      </c>
+      <c r="L126" s="14" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B127" s="14" t="inlineStr">
+        <is>
+          <t>任天堂、Switch 2多言語版に「プレイ50時間以上」購入条件を復活。買い占め対策で</t>
+        </is>
+      </c>
+      <c r="C127" s="14" t="inlineStr">
+        <is>
+          <t>https://automaton-media.com/articles/newsjp/20260611-449235/</t>
+        </is>
+      </c>
+      <c r="D127" s="14" t="inlineStr">
+        <is>
+          <t>マイニンテンドーストア限定の多言語対応版Switch 2は国外転売の標的となりやすく、任天堂は発売以来、抽選販売やプレイ実績条件などの転売対策を講じてきた。直近で買い占めが疑われる注文の増加が確認され、一時販売を停止していた。</t>
+        </is>
+      </c>
+      <c r="E127" s="14" t="inlineStr">
+        <is>
+          <t>任天堂は6月11日、多言語対応版Switch 2の購入条件として「2026年5月31日時点でSwitchのプレイ時間50時間以上」を復活させた。買い占めの疑いがある注文が増えたことへの対応で、実際の利用実績に基づき購入資格を絞り込む。</t>
+        </is>
+      </c>
+      <c r="F127" s="14" t="inlineStr">
+        <is>
+          <t>・対象はマイニンテンドーストアの多言語対応版Switch 2
+・プレイ時間50時間以上の条件を復活
+・買い占め疑い注文の増加を受けた措置
+・国外転売対策の側面が強い</t>
+        </is>
+      </c>
+      <c r="G127" s="14" t="inlineStr">
+        <is>
+          <t>プレイ実績連動の購入資格は転売対策の標準手法として定着し、人気ハード・限定品で他社にも広がる可能性。一方で新規ユーザーの排除という副作用もあり、本人確認や購入履歴と組み合わせた多層的な対策へ進化していく。</t>
+        </is>
+      </c>
+      <c r="H127" s="14" t="inlineStr">
+        <is>
+          <t>行動データを使った転売対策と顧客選別</t>
+        </is>
+      </c>
+      <c r="I127" s="14" t="inlineStr">
+        <is>
+          <t>任天堂</t>
+        </is>
+      </c>
+      <c r="J127" s="14" t="inlineStr">
+        <is>
+          <t>Nintendo Switch 2</t>
+        </is>
+      </c>
+      <c r="K127" s="14" t="inlineStr">
+        <is>
+          <t>国内,ユーザー動向</t>
+        </is>
+      </c>
+      <c r="L127" s="14" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B128" s="14" t="inlineStr">
+        <is>
+          <t>PEGI新基準が6月提出分から適用開始。有料ルートボックスは最低16歳指定に</t>
+        </is>
+      </c>
+      <c r="C128" s="14" t="inlineStr">
+        <is>
+          <t>https://www.reedsmith.com/articles/pegi-launches-interactive-risk-categories-overhauls-age-ratings-for-loot-boxes-in-game-spending-and-communication-features/</t>
+        </is>
+      </c>
+      <c r="D128" s="14" t="inlineStr">
+        <is>
+          <t>欧州ではBEUC等の消費者団体がルートボックスを未成年保護の観点から問題視し、規制圧力が継続。PEGIは3月に「インタラクティブリスク」分類の導入を発表しており、法規制に先んじた業界自主規制の強化として2026年6月から運用を開始する。</t>
+        </is>
+      </c>
+      <c r="E128" s="14" t="inlineStr">
+        <is>
+          <t>PEGIの新レーティング基準が6月の審査提出分から適用開始。有料ランダムアイテム（ルートボックス）を含むゲームは最低PEGI 16、期間・数量限定オファーは最低PEGI 12、NFT/ブロックチェーン要素は自動的にPEGI 18となる。</t>
+        </is>
+      </c>
+      <c r="F128" s="14" t="inlineStr">
+        <is>
+          <t>・6月提出分から新基準を適用
+・有料ルートボックス＝最低PEGI 16
+・時限オファー等の課金誘因＝最低PEGI 12
+・NFT/ブロックチェーン＝PEGI 18
+・EA Sports FCのような低年齢向け人気作も対象になりうる</t>
+        </is>
+      </c>
+      <c r="G128" s="14" t="inlineStr">
+        <is>
+          <t>ガチャ収益に依存するスポーツ・モバイル系大作はレーティング上昇で販路や広告に制約を受け、課金設計の見直しが進む。年齢区分の引き上げが事実上の課金規制として機能し、ESRBや日本のCEROにも同様の見直し圧力が波及しうる。</t>
+        </is>
+      </c>
+      <c r="H128" s="14" t="inlineStr">
+        <is>
+          <t>レーティング制度による課金設計規制</t>
+        </is>
+      </c>
+      <c r="I128" s="14" t="inlineStr">
+        <is>
+          <t>PEGI, EA, Epic Games</t>
+        </is>
+      </c>
+      <c r="J128" s="14" t="inlineStr">
+        <is>
+          <t>EA Sports FC</t>
+        </is>
+      </c>
+      <c r="K128" s="14" t="inlineStr">
+        <is>
+          <t>規制,海外</t>
+        </is>
+      </c>
+      <c r="L128" s="14" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B129" s="14" t="inlineStr">
+        <is>
+          <t>Epic「State of Unreal 2026」6月17日配信。Unreal Fest Chicagoから開発者向け新情報</t>
+        </is>
+      </c>
+      <c r="C129" s="14" t="inlineStr">
+        <is>
+          <t>https://www.unrealengine.com/events/unreal-fest-chicago-2026-state-of-unreal</t>
+        </is>
+      </c>
+      <c r="D129" s="14" t="inlineStr">
+        <is>
+          <t>EpicはGDC 2026でUnreal Engine 6を発表しており、エンジン世代交代の渦中にある。例年単独イベントだったState of Unrealを初めてUnreal Fest（シカゴ、6/16-18）内で開催する形に変更し、大規模デモより開発者との対話を重視する方針を示している。</t>
+        </is>
+      </c>
+      <c r="E129" s="14" t="inlineStr">
+        <is>
+          <t>Epic Gamesが「State of Unreal 2026」を6月17日朝7時（太平洋時間）からUnreal Fest Chicagoより配信すると告知。CEOティム・スウィーニーらが登壇し、開発ツール・サービスの最新情報、コミュニティハイライト、今後のロードマップを紹介する。</t>
+        </is>
+      </c>
+      <c r="F129" s="14" t="inlineStr">
+        <is>
+          <t>・6月17日にライブ配信、初のUnreal Fest内開催
+・ティム・スウィーニーCEOら登壇
+・UE6ロードマップやFortniteエコシステムの続報に注目
+・大型ライブデモより「対話」重視へ転換</t>
+        </is>
+      </c>
+      <c r="G129" s="14" t="inlineStr">
+        <is>
+          <t>UE6の提供スケジュールやAI支援ワークフローの具体化が焦点。エンジンのライセンスモデルやUEFN/クリエイターエコノミーの拡張が発表されれば、Unityとの開発者獲得競争やゲーム外産業（映像・自動車）への展開が加速する。</t>
+        </is>
+      </c>
+      <c r="H129" s="14" t="inlineStr">
+        <is>
+          <t>ゲームエンジンの世代交代とエコシステム競争</t>
+        </is>
+      </c>
+      <c r="I129" s="14" t="inlineStr">
+        <is>
+          <t>Epic Games</t>
+        </is>
+      </c>
+      <c r="J129" s="14" t="inlineStr">
+        <is>
+          <t>Unreal Engine, Fortnite</t>
+        </is>
+      </c>
+      <c r="K129" s="14" t="inlineStr">
+        <is>
+          <t>技術,海外</t>
+        </is>
+      </c>
+      <c r="L129" s="14" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B130" s="14" t="inlineStr">
+        <is>
+          <t>LoL「Hall of Legends」にUzi氏が殿堂入り。記念映画をメルセデス提供で6/11公開</t>
+        </is>
+      </c>
+      <c r="C130" s="14" t="inlineStr">
+        <is>
+          <t>https://lolesports.com/en-US/news/</t>
+        </is>
+      </c>
+      <c r="D130" s="14" t="inlineStr">
+        <is>
+          <t>Hall of LegendsはRiot Gamesが2024年に創設したLoL eスポーツの殿堂で、Faker氏に続く表彰。Uzi氏は中国LPLを代表する元プロ選手で、世界的人気を誇る。eスポーツでは高級ブランドのスポンサー参入が拡大している。</t>
+        </is>
+      </c>
+      <c r="E130" s="14" t="inlineStr">
+        <is>
+          <t>LoL eスポーツはUzi氏のHall of Legends殿堂入りを発表し、記念ドキュメンタリー映画を6月11日にプレミア公開。映画はMercedes-Benzの提供で制作され、殿堂入りを記念したイベントやコンテンツが展開される。</t>
+        </is>
+      </c>
+      <c r="F130" s="14" t="inlineStr">
+        <is>
+          <t>・Uzi氏がFaker氏らに続く殿堂入り
+・記念映画を6/11公開、Mercedes-Benzがプレゼンティングスポンサー
+・中国市場でのLoL eスポーツ人気を再喚起する狙い
+・高級ブランドのeスポーツ投資が継続</t>
+        </is>
+      </c>
+      <c r="G130" s="14" t="inlineStr">
+        <is>
+          <t>殿堂入りを軸にしたレジェンドのIP化（記念スキン・映像・イベント）はeスポーツの新たな収益源として定着する。スポーツ界の「背番号永久欠番」型のマーケティングがゲームでも一般化し、選手のセカンドキャリアにも好影響を与える。</t>
+        </is>
+      </c>
+      <c r="H130" s="14" t="inlineStr">
+        <is>
+          <t>eスポーツ選手のレジェンドIP化と高級ブランド協賛</t>
+        </is>
+      </c>
+      <c r="I130" s="14" t="inlineStr">
+        <is>
+          <t>Riot Games, Tencent, Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="J130" s="14" t="inlineStr">
+        <is>
+          <t>League of Legends</t>
+        </is>
+      </c>
+      <c r="K130" s="14" t="inlineStr">
+        <is>
+          <t>eスポーツ,海外</t>
+        </is>
+      </c>
+      <c r="L130" s="14" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B131" s="14" t="inlineStr">
+        <is>
+          <t>ファミ通週販：トモコレ7週連続首位、Switch 2版FF7リバースが初登場トップ10入り</t>
+        </is>
+      </c>
+      <c r="C131" s="14" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/article/202606/78042</t>
+        </is>
+      </c>
+      <c r="D131" s="14" t="inlineStr">
+        <is>
+          <t>Switch 2の普及が進む中、国内パッケージ市場は任天堂タイトルが牽引。6月第1週はFF7リバースSwitch 2版、eFootball Kick-Off!、A列車で行こう9 Evolutionなど他機種からの移植・新作が相次いで投入された。</t>
+        </is>
+      </c>
+      <c r="E131" s="14" t="inlineStr">
+        <is>
+          <t>ファミ通調べの週間販売数（6/1〜6/7）で『トモダチコレクション わくわく生活』が7週連続首位。Switch 2版『FF7リバース』『eFootball Kick-Off!』『A列車で行こう9 Evolution』もトップ10入りし、Switch 2向けソフトの存在感が増している。</t>
+        </is>
+      </c>
+      <c r="F131" s="14" t="inlineStr">
+        <is>
+          <t>・トモコレが7週連続1位のロングセラー
+・Switch 2版FF7リバースが初登場でトップ10入り
+・コナミ・アートディンク等サード移植も上位に
+・国内パッケージ市場はSwitch 2世代への移行が進行</t>
+        </is>
+      </c>
+      <c r="G131" s="14" t="inlineStr">
+        <is>
+          <t>夏商戦に向けスプラトゥーン レイダースやドラクエ関連など任天堂・スクエニの弾が控え、Switch 2ソフト比率はさらに上昇する。PS5世代マルチの移植が定番化し、国内ではSwitch 2が事実上の標準プラットフォームになっていく。</t>
+        </is>
+      </c>
+      <c r="H131" s="14" t="inlineStr">
+        <is>
+          <t>国内パッケージ市場のSwitch 2移行</t>
+        </is>
+      </c>
+      <c r="I131" s="14" t="inlineStr">
+        <is>
+          <t>任天堂, スクウェア・エニックス, コナミ, アートディンク</t>
+        </is>
+      </c>
+      <c r="J131" s="14" t="inlineStr">
+        <is>
+          <t>トモダチコレクション, FF7リバース, eFootball, A列車で行こう</t>
+        </is>
+      </c>
+      <c r="K131" s="14" t="inlineStr">
+        <is>
+          <t>国内,ユーザー動向,新作</t>
+        </is>
+      </c>
+      <c r="L131" s="14" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B132" s="14" t="inlineStr">
+        <is>
+          <t>韓国大統領訪中に合わせKraftonとTencent首脳が会談。韓中ゲーム交流の活性化を協議</t>
+        </is>
+      </c>
+      <c r="C132" s="14" t="inlineStr">
+        <is>
+          <t>https://www.invenglobal.com/articles/20037/president-lees-china-visit-puts-spotlight-on-game-industry-krafton-and-tencent-hold-high-level-talks</t>
+        </is>
+      </c>
+      <c r="D132" s="14" t="inlineStr">
+        <is>
+          <t>中国はPUBG Mobile（和平精英）などを通じKraftonの最大級の収益源であり、TencentはKraftonの第2位株主。一方、韓国ゲームの中国版号（販売許可）発給は長く制限されてきた。李在明大統領の訪中で経済交流の再活性化が議題となった。</t>
+        </is>
+      </c>
+      <c r="E132" s="14" t="inlineStr">
+        <is>
+          <t>李在明大統領の中国訪問に合わせ、KraftonのCEOキム・チャンハン氏がTencent幹部と会談し、韓中ゲーム産業の交流活性化を協議したと報じられた。版号問題の改善や共同事業の拡大が期待される。</t>
+        </is>
+      </c>
+      <c r="F132" s="14" t="inlineStr">
+        <is>
+          <t>・Krafton CEOとTencent幹部が対面会談
+・李在明大統領訪中の経済使節の文脈
+・TencentはKraftonの第2位株主で長年の戦略パートナー
+・韓国ゲームの中国版号発給改善への期待</t>
+        </is>
+      </c>
+      <c r="G132" s="14" t="inlineStr">
+        <is>
+          <t>韓中関係の改善が進めば、韓国タイトルへの版号発給が増え、NCソフトやネクソンなど他の韓国勢にも中国再進出の機会が広がる。逆にTencentによる韓国スタジオへの出資・買収も活発化し、資本面の相互依存が深まる。</t>
+        </is>
+      </c>
+      <c r="H132" s="14" t="inlineStr">
+        <is>
+          <t>ゲーム産業と地政学（版号・国家間交渉）</t>
+        </is>
+      </c>
+      <c r="I132" s="14" t="inlineStr">
+        <is>
+          <t>Krafton, Tencent</t>
+        </is>
+      </c>
+      <c r="J132" s="14" t="inlineStr">
+        <is>
+          <t>PUBG, PUBG Mobile</t>
+        </is>
+      </c>
+      <c r="K132" s="14" t="inlineStr">
+        <is>
+          <t>海外,M&amp;A</t>
+        </is>
+      </c>
+      <c r="L132" s="14" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B133" s="14" t="inlineStr">
+        <is>
+          <t>『スト6』Year 4インタビュー：ティファは固有システム持ち、新規キャラ3名追加の背景</t>
+        </is>
+      </c>
+      <c r="C133" s="14" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/article/202606/77640</t>
+        </is>
+      </c>
+      <c r="D133" s="14" t="inlineStr">
+        <is>
+          <t>『ストリートファイター6』は6月5日にSwitch 2版が発売されYear 4シーズンに突入。FF7コラボのティファ参戦が話題を集める一方、格闘ゲームのユーザー層拡大と高齢化への対応が開発課題となっている。</t>
+        </is>
+      </c>
+      <c r="E133" s="14" t="inlineStr">
+        <is>
+          <t>ファミ通がスト6開発陣のYear 4インタビューを掲載。ティファはリリーの風溜めに似た固有システムを持つ独自設計で、完全新規キャラクター3名の追加はユーザー年齢層の変化（新規・若年層の取り込み）が理由のひとつと明かされた。</t>
+        </is>
+      </c>
+      <c r="F133" s="14" t="inlineStr">
+        <is>
+          <t>・ティファは固有ゲージ/システムを持つ独自設計
+・Year 4で完全新規キャラ3名を追加
+・新規キャラ投入の背景にユーザー年齢層の変化
+・FF7コラボでスクエニIPとのクロスオーバー深化</t>
+        </is>
+      </c>
+      <c r="G133" s="14" t="inlineStr">
+        <is>
+          <t>大型IPコラボキャラは新規ユーザー獲得の主力施策として定着し、他社格闘ゲームtoo同様の路線を強化する。カプコンとスクエニのIP相互活用は今後も拡大し、格闘ゲームの「プラットフォーム化」（ゲスト参戦ビジネス）が進む。</t>
+        </is>
+      </c>
+      <c r="H133" s="14" t="inlineStr">
+        <is>
+          <t>格闘ゲームのIPコラボとユーザー層拡大戦略</t>
+        </is>
+      </c>
+      <c r="I133" s="14" t="inlineStr">
+        <is>
+          <t>カプコン, スクウェア・エニックス</t>
+        </is>
+      </c>
+      <c r="J133" s="14" t="inlineStr">
+        <is>
+          <t>ストリートファイター6, FF7</t>
+        </is>
+      </c>
+      <c r="K133" s="14" t="inlineStr">
+        <is>
+          <t>新作,国内</t>
+        </is>
+      </c>
+      <c r="L133" s="14" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
weekly-releases + indie update (2026-06-12 17:30)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -12055,7 +12055,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M15"/>
+  <dimension ref="A1:M21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12789,6 +12789,276 @@
       <c r="M15" t="inlineStr">
         <is>
           <t>https://www.gamesradar.com/video-game-release-dates/</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>33 Immortals（サーティスリー・イモータルズ）</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Thunder Lotus Games</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Thunder Lotus Games</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>PC(Steam/Epic)/Xbox Series X|S</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>協力アクションローグライク（33人co-op）</t>
+        </is>
+      </c>
+      <c r="K16" t="n">
+        <v>3</v>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>15ヶ月の早期アクセスを経て1.0。最終レルム“Paradiso”と隠し最終ボス追加。Steamレビュー82% Positive(397件・Very Positive)。Spiritfarerのスタジオ。Game Pass対応。Metacritic/OpenCriticの1.0集計は未確認。</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>https://www.techpowerup.com/345436/33-immortals-comes-to-steam-with-1-0-launch-after-long-early-access</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>STARSEEKER: Astroneer Expeditions（スターシーカー：アストロニーア・エクスペディションズ）</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>System Era Softworks</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Devolver Digital</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>PS5/Xbox Series X|S/Switch 2/PC(Steam)</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>協力探索アドベンチャー（Astroneer世界観）</t>
+        </is>
+      </c>
+      <c r="K17" t="n">
+        <v>3</v>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>早期アクセス開始。クロスプレイ/クロスプログレッション対応、Game Pass Day1。Steamレビュー37% Positive(187件・Mostly Negative)と滑り出しは苦戦。</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>https://store.steampowered.com/app/1454370/STARSEEKER_Astroneer_Expeditions/</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>パワフルプロ野球2026-2027</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>コナミデジタルエンタテインメント</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>KONAMI</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>PS5/Nintendo Switch ほか（公式参照）</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>野球/育成シミュレーション</t>
+        </is>
+      </c>
+      <c r="K18" t="n">
+        <v>3</v>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>サクセス30周年。新サクセス“パラレルオールスターズ編”、栄冠ナイン3年モード搭載。週刊ファミ通No.1951で発売記念特集。国内向け定番タイトル。</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>https://www.konami.com/pawa/2026-2027/</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Star Fox（スターフォックス）</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>任天堂</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>任天堂</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Nintendo Switch 2</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>3Dシューティング</t>
+        </is>
+      </c>
+      <c r="K19" t="n">
+        <v>4</v>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>『スターフォックス64』ベースにグラフィック一新＋新要素の新生スターフォックス。6/9のNintendo Directで体験版配信開始。約30年ぶりの本格新作として注目。</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>https://www.nintendo.com/jp/games/switch2/abgwa/index.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Palworld（パルワールド）正式版1.0</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>ポケットペア</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>ポケットペア</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>PC(Steam)/Xbox Series X|S ほか</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>オープンワールド・サバイバルクラフト</t>
+        </is>
+      </c>
+      <c r="K20" t="n">
+        <v>4</v>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>早期アクセスから約2年半で1.0正式版。7月最注目タイトルとの報。EA期の最大同接210万超の実績を持つ。</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>https://gamegator.net/calendar/2026/july</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Halo: Campaign Evolved（ヘイロー：キャンペーン エボルブド）</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Halo Studios</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Xbox Game Studios</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Xbox Series X|S/PC/PS5</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>FPS（初代Haloキャンペーンリメイク）</t>
+        </is>
+      </c>
+      <c r="K21" t="n">
+        <v>4</v>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>初代Halo:CEキャンペーンのUE5フルリメイク。PS5にも展開。7/23から最大5日間の早期アクセス。</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>https://www.gamespot.com/articles/2026-upcoming-games-release-schedule/1100-6534941/</t>
         </is>
       </c>
     </row>
@@ -16802,7 +17072,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17098,6 +17368,53 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Lost Castle 2（ロストキャッスル2）</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Hunter Studio（中国・小規模）</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2026-06-10 1.0正式リリース（早期アクセス卒業）</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2D協力ベルトスクロール・ローグライト</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>早期アクセスで70万本販売済み。1.0で最終ストーリーエンディング・高難度Ethereal Nightmare 4/5追加。発売30%オフ。</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Steamレビュー Mostly Positive（全言語11,240件、英語はVery Positive）</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>中華圏中心に強い人気。co-opローグライトとして今週Steamで露出増。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
add 週間ランキング sheet + seed data (2026-06-12 17:59)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -20,6 +20,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="掘り下げ・分析" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="業界マトリクス" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="横断的問い" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="週間ランキング" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3641,6 +3642,897 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>集計週</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>区分</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>順位</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>タイトル</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>プラットフォーム</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>週販本数</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>累計本数</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Steam同接ピーク</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>出典</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>メモ</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-06-01〜06-07</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>トモダチコレクション わくわく生活</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Switch</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>50151</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1309182</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週販 https://www.famitsu.com/article/202606/78042</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>7週連続首位</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-06-01〜06-07</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>ファイナルファンタジーVII リバース</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Switch 2</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>30657</v>
+      </c>
+      <c r="G3" t="n">
+        <v>30657</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週販 https://www.famitsu.com/article/202606/78042</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>初登場</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-06-01〜06-07</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>eFootball Kick-Off!</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Switch 2</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>20047</v>
+      </c>
+      <c r="G4" t="n">
+        <v>20047</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週販 https://www.famitsu.com/article/202606/78042</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>初登場</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-06-01〜06-07</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>ぽこ あ ポケモン</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Switch 2</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>10794</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1049201</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週販 https://www.famitsu.com/article/202606/78042</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>累計104.9万本</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-06-01〜06-07</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>ヨッシーとフカシギの図鑑</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Switch 2</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>8191</v>
+      </c>
+      <c r="G6" t="n">
+        <v>60553</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週販 https://www.famitsu.com/article/202606/78042</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-06-01〜06-07</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>6</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>マリオカート ワールド</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Switch 2</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>7381</v>
+      </c>
+      <c r="G7" t="n">
+        <v>2965454</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週販 https://www.famitsu.com/article/202606/78042</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>累計296.5万本</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-06-01〜06-07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>7</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>007 First Light（007 ファースト・ライト）</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>PS5</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>4388</v>
+      </c>
+      <c r="G8" t="n">
+        <v>25078</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週販 https://www.famitsu.com/article/202606/78042</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-06-01〜06-07</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>8</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Minecraft（マインクラフト）</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Switch</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>4381</v>
+      </c>
+      <c r="G9" t="n">
+        <v>4218943</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週販 https://www.famitsu.com/article/202606/78042</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-06-01〜06-07</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>9</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>A列車で行こう9 Evolution</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Switch 2</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>3550</v>
+      </c>
+      <c r="G10" t="n">
+        <v>3550</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週販 https://www.famitsu.com/article/202606/78042</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>初登場</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-06-01〜06-07</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>10</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>アストロボット</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>PS5</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>3460</v>
+      </c>
+      <c r="G11" t="n">
+        <v>103717</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週販 https://www.famitsu.com/article/202606/78042</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-06-03〜06-09</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Forza Horizon 6（フォルツァ ホライゾン 6）</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Steam週間グローバルトップセラー(売上額順・F2P除く) https://www.vgchartz.com/article/468148/steam-weekly-week-24-2026/</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>首位返り咲き</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-06-03〜06-09</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Gothic 1 Remake（ゴシック1 リメイク）</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Steam週間グローバルトップセラー(売上額順・F2P除く) https://www.vgchartz.com/article/468148/steam-weekly-week-24-2026/</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>6/5発売の新作</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-06-03〜06-09</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>3</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Path of Exile 2（パス・オブ・エグザイル2）</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Steam週間グローバルトップセラー(売上額順・F2P除く) https://www.vgchartz.com/article/468148/steam-weekly-week-24-2026/</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-06-03〜06-09</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>007 First Light（007 ファースト・ライト）</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Steam週間グローバルトップセラー(売上額順・F2P除く) https://www.vgchartz.com/article/468148/steam-weekly-week-24-2026/</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-06-03〜06-09</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>5</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Steam Deck</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Steam週間グローバルトップセラー(売上額順・F2P除く) https://www.vgchartz.com/article/468148/steam-weekly-week-24-2026/</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>ハードウェア</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-06-03〜06-09</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>6</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Paralives（パラライブス）</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Steam週間グローバルトップセラー(売上額順・F2P除く) https://www.vgchartz.com/article/468148/steam-weekly-week-24-2026/</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>インディーライフシム、EAから好調継続</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-06-03〜06-09</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>7</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Subnautica 2（サブノーティカ2）</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Steam週間グローバルトップセラー(売上額順・F2P除く) https://www.vgchartz.com/article/468148/steam-weekly-week-24-2026/</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-06-03〜06-09</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>8</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Resident Evil 4（バイオハザード RE:4）</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Steam週間グローバルトップセラー(売上額順・F2P除く) https://www.vgchartz.com/article/468148/steam-weekly-week-24-2026/</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-06-03〜06-09</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>9</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Resident Evil Requiem（バイオハザード レクイエム）</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Steam週間グローバルトップセラー(売上額順・F2P除く) https://www.vgchartz.com/article/468148/steam-weekly-week-24-2026/</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-06-03〜06-09</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>10</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>EA Sports FC 26</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Steam週間グローバルトップセラー(売上額順・F2P除く) https://www.vgchartz.com/article/468148/steam-weekly-week-24-2026/</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-05 (月間)</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>PS DL</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>007 First Light（007 ファースト・ライト）</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>PS5</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>PS Blog 月間DLランキング https://blog.ja.playstation.com/2026/06/09/20260609-monthly-ps-store-ranking-s/</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>週間が無いため月間で代替</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-05 (月間)</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>PS DL</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>2</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>プラグマタ（PRAGMATA）</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>PS5</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>PS Blog 月間DLランキング https://blog.ja.playstation.com/2026/06/09/20260609-monthly-ps-store-ranking-s/</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>週間が無いため月間で代替</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-05 (月間)</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>PS DL</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>3</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>バイオハザード RE:4</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>PS5</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>PS Blog 月間DLランキング https://blog.ja.playstation.com/2026/06/09/20260609-monthly-ps-store-ranking-s/</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>週間が無いため月間で代替</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
daily-news + cross-questions update (2026-06-12 22:11)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -2589,7 +2589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3634,6 +3634,80 @@
       <c r="G28" s="14" t="inlineStr">
         <is>
           <t>表現内容ではなく「収益メカニクス」を理由に年齢制限を課す初の大規模制度。法規制を待たず業界自主規制が実質的な課金規制として機能する構図。</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>ゲーム企業によるクリエイター支援ツール買収（GameSquare×TubeBuddy）の垂直統合は、広告・メディア業界のMCN・制作ツール統合の何に該当するか？</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>GameSquareの8-K開示（上期売上+125%、TubeBuddy買収効果）</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>GameSquare, FaZe Clan, TubeBuddy</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>広告・メディア（MCN統合）、SaaS（クリエイターツール）、フィンテック（クリエイター決済）</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>コスト重のチーム運営から粗利の高いツール/インフラへの軸足移動は、eスポーツ業界全体の生存戦略になりつつある。</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>運営11年目タイトルのエンジン刷新（FGO→Unity 6）のような「走りながらの基盤更改」は、銀行勘定系・航空予約システムなど他業界のレガシー刷新の何に相当するか？</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>FGOのUnity 6移行アップデート発表（6月22日実施）</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>FGO PROJECT, アニプレックス, Unity Technologies</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>金融（勘定系更改）、航空（PSS刷新）、小売（POS基盤更改）</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>ダウンタイム最小化と互換性維持が共通課題。ゲームは失敗時のユーザー離脱が即時に可視化される点で他業界の先行事例になり得る。</t>
         </is>
       </c>
     </row>
@@ -3902,7 +3976,6 @@
           <t>ファミ通.com 週販 https://www.famitsu.com/article/202606/78042</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3980,7 +4053,6 @@
           <t>ファミ通.com 週販 https://www.famitsu.com/article/202606/78042</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4017,7 +4089,6 @@
           <t>ファミ通.com 週販 https://www.famitsu.com/article/202606/78042</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4095,7 +4166,6 @@
           <t>ファミ通.com 週販 https://www.famitsu.com/article/202606/78042</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4196,7 +4266,6 @@
           <t>Steam週間グローバルトップセラー(売上額順・F2P除く) https://www.vgchartz.com/article/468148/steam-weekly-week-24-2026/</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -4227,7 +4296,6 @@
           <t>Steam週間グローバルトップセラー(売上額順・F2P除く) https://www.vgchartz.com/article/468148/steam-weekly-week-24-2026/</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -4328,7 +4396,6 @@
           <t>Steam週間グローバルトップセラー(売上額順・F2P除く) https://www.vgchartz.com/article/468148/steam-weekly-week-24-2026/</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -4359,7 +4426,6 @@
           <t>Steam週間グローバルトップセラー(売上額順・F2P除く) https://www.vgchartz.com/article/468148/steam-weekly-week-24-2026/</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4390,7 +4456,6 @@
           <t>Steam週間グローバルトップセラー(売上額順・F2P除く) https://www.vgchartz.com/article/468148/steam-weekly-week-24-2026/</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4421,7 +4486,6 @@
           <t>Steam週間グローバルトップセラー(売上額順・F2P除く) https://www.vgchartz.com/article/468148/steam-weekly-week-24-2026/</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4539,7 +4603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L133"/>
+  <dimension ref="A1:L142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12935,6 +12999,547 @@
         </is>
       </c>
       <c r="L133" s="14" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B134" s="5" t="inlineStr">
+        <is>
+          <t>Xbox、会計年度明け7月に大規模人員削減か。スタジオ閉鎖の可能性も浮上</t>
+        </is>
+      </c>
+      <c r="C134" s="5" t="inlineStr">
+        <is>
+          <t>https://games.gg/news/xbox-studio-closure-layoffs-2026/</t>
+        </is>
+      </c>
+      <c r="D134" s="5" t="inlineStr">
+        <is>
+          <t>Microsoftは2023年のActivision Blizzard買収（687億ドル）以降、ゲーム部門の投資回収圧力が増大。新CEO Asha Sharma体制下で事業「リセット」が進む中、6月30日の会計年度末以降に人員削減を発表するのが同社の通例とされる。</t>
+        </is>
+      </c>
+      <c r="E134" s="5" t="inlineStr">
+        <is>
+          <t>6/11報道の続報。レイオフは7月以降に正式発表される見込みで、少なくとも1つの未公表スタジオの閉鎖に波及する可能性が報じられた。Game Pass戦略の見直しやマルチプラットフォーム化と並行する構造改革の一環とみられる。</t>
+        </is>
+      </c>
+      <c r="F134" s="5" t="inlineStr">
+        <is>
+          <t>削減発表は会計年度末（6/30）以降の見込み
+少なくとも1スタジオの閉鎖可能性が浮上
+Activision買収687億ドルの回収圧力が背景
+新CEO体制下の「リセット」路線の一環</t>
+        </is>
+      </c>
+      <c r="G134" s="5" t="inlineStr">
+        <is>
+          <t>7月の発表でポートフォリオ整理の全容が明確化する見込み。クラウド・AIへの投資再配分とサードパーティ展開の拡大が進み、他社の追随リストラを誘発する可能性もある。</t>
+        </is>
+      </c>
+      <c r="H134" s="5" t="inlineStr">
+        <is>
+          <t>プラットフォーマーの事業リセットと投資回収</t>
+        </is>
+      </c>
+      <c r="I134" s="5" t="inlineStr">
+        <is>
+          <t>Microsoft, Xbox, Activision Blizzard</t>
+        </is>
+      </c>
+      <c r="J134" s="5" t="inlineStr">
+        <is>
+          <t>Game Pass</t>
+        </is>
+      </c>
+      <c r="K134" s="5" t="inlineStr">
+        <is>
+          <t>業績,海外</t>
+        </is>
+      </c>
+      <c r="L134" s="5" t="n"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B135" s="5" t="inlineStr">
+        <is>
+          <t>EWC2026のVALORANT部門、出場16チーム確定。7月パリ開催・賞金200万ドル</t>
+        </is>
+      </c>
+      <c r="C135" s="5" t="inlineStr">
+        <is>
+          <t>https://insider-gaming.com/esports-world-cup-2026-valorant-teams/</t>
+        </is>
+      </c>
+      <c r="D135" s="5" t="inlineStr">
+        <is>
+          <t>Esports World Cup 2026は5月20日に開催地をリヤドからパリへ変更。VALORANT部門は7月2日〜12日に開催され、地域予選とVCT Stage 1の結果を受けて出場チームが出揃った。</t>
+        </is>
+      </c>
+      <c r="E135" s="5" t="inlineStr">
+        <is>
+          <t>前回王者Team Hereticsに加え、地域予選通過の11チームとVCT各地域上位のVitality、G2 Esports、Paper Rex、EDward Gamingなど計16チームが確定。賞金総額200万ドルのSティア国際大会として開催準備が最終段階に入った。</t>
+        </is>
+      </c>
+      <c r="F135" s="5" t="inlineStr">
+        <is>
+          <t>7月2日〜12日にパリで開催
+賞金総額200万ドル
+前回王者Team Hereticsら16チームが出場
+開催地はリヤドからパリへ変更済み</t>
+        </is>
+      </c>
+      <c r="G135" s="5" t="inlineStr">
+        <is>
+          <t>パリ開催により欧州スポンサーと現地観客動員の拡大が見込まれる。サウジ主導大会の地政学リスク管理が、今後の国際大会設計の重要論点として定着しそう。</t>
+        </is>
+      </c>
+      <c r="H135" s="5" t="inlineStr">
+        <is>
+          <t>eスポーツ国際大会の開催地戦略と地政学</t>
+        </is>
+      </c>
+      <c r="I135" s="5" t="inlineStr">
+        <is>
+          <t>Riot Games, Esports World Cup Foundation, Team Heretics</t>
+        </is>
+      </c>
+      <c r="J135" s="5" t="inlineStr">
+        <is>
+          <t>VALORANT</t>
+        </is>
+      </c>
+      <c r="K135" s="5" t="inlineStr">
+        <is>
+          <t>eスポーツ,海外</t>
+        </is>
+      </c>
+      <c r="L135" s="5" t="n"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B136" s="5" t="inlineStr">
+        <is>
+          <t>日本ゲーム大賞2026「年間作品部門」一般投票開始。受付は7月17日まで</t>
+        </is>
+      </c>
+      <c r="C136" s="5" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/991/G999104/20260611045/</t>
+        </is>
+      </c>
+      <c r="D136" s="5" t="inlineStr">
+        <is>
+          <t>CESA主催の日本ゲーム大賞は国内最大級のゲーム表彰制度。年間作品部門は一般投票で大賞が決まり、例年9月の東京ゲームショウで発表される。</t>
+        </is>
+      </c>
+      <c r="E136" s="5" t="inlineStr">
+        <is>
+          <t>6月12日に一般投票の受付が開始。投票期間は7月17日23時59分まで。投票者を対象にPS5 ProやSwitch 2、Xbox Series Xなどが当たるプレゼントキャンペーンも実施される。</t>
+        </is>
+      </c>
+      <c r="F136" s="5" t="inlineStr">
+        <is>
+          <t>投票期間は7月17日23:59まで
+投票者対象にPS5 Pro/Switch 2等が当たるキャンペーン
+発表は例年TGSで実施
+ファン参加型アワードによる業界活性化策</t>
+        </is>
+      </c>
+      <c r="G136" s="5" t="inlineStr">
+        <is>
+          <t>トモダチコレクションやSwitch 2対応大型タイトルなど2026年上期の話題作が有力候補に。TGS2026に向けて各社の受賞狙いのプロモーションが活発化する。</t>
+        </is>
+      </c>
+      <c r="H136" s="5" t="inlineStr">
+        <is>
+          <t>国内ゲームアワードとマーケティングの関係</t>
+        </is>
+      </c>
+      <c r="I136" s="5" t="inlineStr">
+        <is>
+          <t>CESA</t>
+        </is>
+      </c>
+      <c r="J136" s="5" t="inlineStr"/>
+      <c r="K136" s="5" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="L136" s="5" t="n"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B137" s="5" t="inlineStr">
+        <is>
+          <t>『FGO』6月22日にUnity 6へエンジン移行。約16GBの再ダウンロードが必要に</t>
+        </is>
+      </c>
+      <c r="C137" s="5" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/266/G026651/20260612008/</t>
+        </is>
+      </c>
+      <c r="D137" s="5" t="inlineStr">
+        <is>
+          <t>2015年配信開始の『Fate/Grand Order』は運営11年目に突入。旧世代エンジンの継続利用は新OS対応や開発効率の面でリスクとなっており、長期運営タイトルの基盤刷新が業界共通の課題となっている。</t>
+        </is>
+      </c>
+      <c r="E137" s="5" t="inlineStr">
+        <is>
+          <t>FGO PROJECTは6月11日、ゲームエンジンをUnity 6へ移行するアプリアップデートを6月22日に実施すると発表。アップデート後は必要容量が約2GB増加し、約16GBのデータ再ダウンロードが必要になる。</t>
+        </is>
+      </c>
+      <c r="F137" s="5" t="inlineStr">
+        <is>
+          <t>6月22日にUnity 6移行アップデートを実施
+約16GBの再ダウンロードが必要
+運営11年目の長寿タイトルによる基盤刷新
+新OS・新端末対応への布石</t>
+        </is>
+      </c>
+      <c r="G137" s="5" t="inlineStr">
+        <is>
+          <t>移行直後の不具合対応が短期の焦点。円滑に完了すれば、長期運営タイトルのエンジン刷新の参照事例となり、他の長寿モバイルタイトルの追随が進む可能性がある。</t>
+        </is>
+      </c>
+      <c r="H137" s="5" t="inlineStr">
+        <is>
+          <t>長期運営タイトルの技術的負債と基盤刷新</t>
+        </is>
+      </c>
+      <c r="I137" s="5" t="inlineStr">
+        <is>
+          <t>FGO PROJECT, アニプレックス, Unity Technologies</t>
+        </is>
+      </c>
+      <c r="J137" s="5" t="inlineStr">
+        <is>
+          <t>Fate/Grand Order</t>
+        </is>
+      </c>
+      <c r="K137" s="5" t="inlineStr">
+        <is>
+          <t>技術,国内</t>
+        </is>
+      </c>
+      <c r="L137" s="5" t="n"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B138" s="5" t="inlineStr">
+        <is>
+          <t>SIE「PlayStation Link USBアダプター」単体販売を8月6日開始、3,480円</t>
+        </is>
+      </c>
+      <c r="C138" s="5" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/999/G999902/20260612009/</t>
+        </is>
+      </c>
+      <c r="D138" s="5" t="inlineStr">
+        <is>
+          <t>低遅延ワイヤレス接続規格「PlayStation Link」は従来、対応ヘッドセット等の同梱品としてのみ提供されてきたが、対応周辺機器の拡大により単体アダプターの需要が高まっていた。</t>
+        </is>
+      </c>
+      <c r="E138" s="5" t="inlineStr">
+        <is>
+          <t>SIEは6月12日、PlayStation Link対応周辺機器をPS5・PC・Macで利用するための「PlayStation Link USBアダプター」を8月6日に発売すると発表。希望小売価格は3,480円。</t>
+        </is>
+      </c>
+      <c r="F138" s="5" t="inlineStr">
+        <is>
+          <t>8月6日発売、希望小売価格3,480円
+PS5・PC・Macに対応
+低遅延ワイヤレス規格の普及拡大策
+PSブランド周辺機器エコシステムの強化</t>
+        </is>
+      </c>
+      <c r="G138" s="5" t="inlineStr">
+        <is>
+          <t>PC・Mac対応を明示したことで、PSブランド周辺機器の市場がプラットフォーム外へ拡大。ハード本体以外の収益源（周辺機器・PC展開）を強化する流れが続く。</t>
+        </is>
+      </c>
+      <c r="H138" s="5" t="inlineStr">
+        <is>
+          <t>ハードメーカーの周辺機器エコシステム戦略</t>
+        </is>
+      </c>
+      <c r="I138" s="5" t="inlineStr">
+        <is>
+          <t>ソニー・インタラクティブエンタテインメント</t>
+        </is>
+      </c>
+      <c r="J138" s="5" t="inlineStr">
+        <is>
+          <t>PlayStation Link</t>
+        </is>
+      </c>
+      <c r="K138" s="5" t="inlineStr">
+        <is>
+          <t>技術,国内</t>
+        </is>
+      </c>
+      <c r="L138" s="5" t="n"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B139" s="5" t="inlineStr">
+        <is>
+          <t>元Forza Horizon開発陣の新作『Clutch』詳細公開。物語×オープンワールド走行</t>
+        </is>
+      </c>
+      <c r="C139" s="5" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/012/G101234/20260610082/</t>
+        </is>
+      </c>
+      <c r="D139" s="5" t="inlineStr">
+        <is>
+          <t>Maverick GamesはPlayground Games（Forza Horizonシリーズ）出身のベテランが設立した英国スタジオ。Summer Game Fest 2026 Play Daysで新作のプレゼンテーションを実施した。</t>
+        </is>
+      </c>
+      <c r="E139" s="5" t="inlineStr">
+        <is>
+          <t>シネマティックな物語性とオープンワールドドライビングを融合した新作『Clutch』の約45分のプレゼン内容が公開された。レースゲームにナラティブを本格導入する野心作として注目を集めている。</t>
+        </is>
+      </c>
+      <c r="F139" s="5" t="inlineStr">
+        <is>
+          <t>SGF Play Daysで約45分のプレゼンを実施
+シネマティック物語×オープンワールド走行の融合
+Playground Games出身のベテラン開発陣
+レースジャンルのナラティブ化という新潮流</t>
+        </is>
+      </c>
+      <c r="G139" s="5" t="inlineStr">
+        <is>
+          <t>レースジャンルへの物語性導入の試金石となる。発売時期とプラットフォームの正式発表が次の節目で、大手パブリッシャーとの提携動向にも注目が集まる。</t>
+        </is>
+      </c>
+      <c r="H139" s="5" t="inlineStr">
+        <is>
+          <t>ジャンル融合による新規IP立ち上げ</t>
+        </is>
+      </c>
+      <c r="I139" s="5" t="inlineStr">
+        <is>
+          <t>Maverick Games</t>
+        </is>
+      </c>
+      <c r="J139" s="5" t="inlineStr">
+        <is>
+          <t>Clutch, Forza Horizon</t>
+        </is>
+      </c>
+      <c r="K139" s="5" t="inlineStr">
+        <is>
+          <t>新作,海外</t>
+        </is>
+      </c>
+      <c r="L139" s="5" t="n"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B140" s="5" t="inlineStr">
+        <is>
+          <t>GameSquare、上期売上3,430万ドル超見込みと開示。TubeBuddy買収で前年比+125%</t>
+        </is>
+      </c>
+      <c r="C140" s="5" t="inlineStr">
+        <is>
+          <t>https://www.stocktitan.net/sec-filings/GAME/8-k-game-square-holdings-inc-reports-material-event-422d6ad6aa84.html</t>
+        </is>
+      </c>
+      <c r="D140" s="5" t="inlineStr">
+        <is>
+          <t>eスポーツ・クリエイターエコノミー企業のGameSquare（FaZe Clan親会社）は、YouTubeクリエイター支援ツールTubeBuddyを買収し、メディア事業とクリエイターツールの統合を推進している。</t>
+        </is>
+      </c>
+      <c r="E140" s="5" t="inlineStr">
+        <is>
+          <t>8-K開示で、2026年Q2売上は1,850万ドル以上、TubeBuddy買収込みの上期プロフォーマ売上は3,430万ドル超（前年比125%以上増）になる見込みと発表。通期ガイダンス8,500万〜9,000万ドルも再確認した。</t>
+        </is>
+      </c>
+      <c r="F140" s="5" t="inlineStr">
+        <is>
+          <t>Q2売上は1,850万ドル以上の見込み
+上期プロフォーマ売上3,430万ドル超（前年比+125%）
+通期ガイダンス8,500万〜9,000万ドルを維持
+TubeBuddy買収によるクリエイターツール統合が寄与</t>
+        </is>
+      </c>
+      <c r="G140" s="5" t="inlineStr">
+        <is>
+          <t>コスト負担の重いチーム運営から、粗利の高いクリエイター向けツール・インフラへ軸足を移すモデルが、eスポーツ企業の生存戦略として業界に広がるか注目される。</t>
+        </is>
+      </c>
+      <c r="H140" s="5" t="inlineStr">
+        <is>
+          <t>eスポーツ企業の収益多角化とクリエイターエコノミー</t>
+        </is>
+      </c>
+      <c r="I140" s="5" t="inlineStr">
+        <is>
+          <t>GameSquare, FaZe Clan, TubeBuddy</t>
+        </is>
+      </c>
+      <c r="J140" s="5" t="inlineStr"/>
+      <c r="K140" s="5" t="inlineStr">
+        <is>
+          <t>業績,M&amp;A,eスポーツ,海外</t>
+        </is>
+      </c>
+      <c r="L140" s="5" t="n"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B141" s="5" t="inlineStr">
+        <is>
+          <t>『DQモンスターズ4』新情報公開。ビアンカとフローラの物語、500種族以上が登場</t>
+        </is>
+      </c>
+      <c r="C141" s="5" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/010/G101055/20260610066/</t>
+        </is>
+      </c>
+      <c r="D141" s="5" t="inlineStr">
+        <is>
+          <t>12月3日発売が決定している『ドラゴンクエストモンスターズ4 哀しみの故郷とビアンカ・フローラ編』の追加情報。『ドラゴンクエストV』の人気キャラクターを軸にした派生新作として注目度が高い。</t>
+        </is>
+      </c>
+      <c r="E141" s="5" t="inlineStr">
+        <is>
+          <t>スクウェア・エニックスは6月12日、ストーリー概要と新システムの詳細を公開。ビアンカとフローラが冒険を繰り広げる物語の概要や「ザレキの洞窟」などのフィールド、500種族以上のモンスターの登場が明らかになった。</t>
+        </is>
+      </c>
+      <c r="F141" s="5" t="inlineStr">
+        <is>
+          <t>12月3日発売予定
+DQ5のビアンカ・フローラを軸にした物語
+500種族以上のモンスターが登場
+シリーズ派生IPによる年末商戦の有力タイトル</t>
+        </is>
+      </c>
+      <c r="G141" s="5" t="inlineStr">
+        <is>
+          <t>DQ5世代のノスタルジー需要を取り込み、年末商戦の国内有力タイトルとなる見込み。HD-2D版DQ展開と合わせ、シリーズ資産の多面的な再活用が加速する。</t>
+        </is>
+      </c>
+      <c r="H141" s="5" t="inlineStr">
+        <is>
+          <t>派生IPによるシリーズ資産の再活用</t>
+        </is>
+      </c>
+      <c r="I141" s="5" t="inlineStr">
+        <is>
+          <t>スクウェア・エニックス</t>
+        </is>
+      </c>
+      <c r="J141" s="5" t="inlineStr">
+        <is>
+          <t>ドラゴンクエストモンスターズ4, ドラゴンクエストV</t>
+        </is>
+      </c>
+      <c r="K141" s="5" t="inlineStr">
+        <is>
+          <t>新作,国内</t>
+        </is>
+      </c>
+      <c r="L141" s="5" t="n"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B142" s="5" t="inlineStr">
+        <is>
+          <t>KAMITSUBAKI新作探索ADV『プロトニオスペース』体験版がSteamで配信開始</t>
+        </is>
+      </c>
+      <c r="C142" s="5" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/928/G092866/20260612017/</t>
+        </is>
+      </c>
+      <c r="D142" s="5" t="inlineStr">
+        <is>
+          <t>KAMITSUBAKI STUDIOは音楽レーベル発のクリエイティブスタジオで、バーチャルアーティスト事業からゲーム領域への展開を進めている。Steam Next Fest開催時期に合わせた露出となる。</t>
+        </is>
+      </c>
+      <c r="E142" s="5" t="inlineStr">
+        <is>
+          <t>音楽×サイコポップが特徴のサイエンスファンタジー探索アドベンチャー『プロトニオスペース』の体験版がSteamで配信開始。奇妙な「ループ」からの脱出を目指し、失われた声の記憶を呼び覚ます物語が描かれる。</t>
+        </is>
+      </c>
+      <c r="F142" s="5" t="inlineStr">
+        <is>
+          <t>体験版がSteamで配信開始
+音楽レーベル発スタジオによるゲーム展開
+Steam Next Fest時期に合わせた露出戦略
+音楽×ゲームのメディアミックス型IP開発</t>
+        </is>
+      </c>
+      <c r="G142" s="5" t="inlineStr">
+        <is>
+          <t>音楽・VTuber系レーベルによるゲーム参入の流れが続く。体験版の反響が製品版の規模とレーベルの今後のゲーム投資を左右する試金石になる。</t>
+        </is>
+      </c>
+      <c r="H142" s="5" t="inlineStr">
+        <is>
+          <t>音楽レーベルのゲーム参入とIPミックス戦略</t>
+        </is>
+      </c>
+      <c r="I142" s="5" t="inlineStr">
+        <is>
+          <t>KAMITSUBAKI STUDIO</t>
+        </is>
+      </c>
+      <c r="J142" s="5" t="inlineStr">
+        <is>
+          <t>プロトニオスペース</t>
+        </is>
+      </c>
+      <c r="K142" s="5" t="inlineStr">
+        <is>
+          <t>インディー,国内</t>
+        </is>
+      </c>
+      <c r="L142" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
daily-news + cross-questions update (2026-06-13 22:12)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -2589,7 +2589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3708,6 +3708,43 @@
       <c r="G30" s="5" t="inlineStr">
         <is>
           <t>ダウンタイム最小化と互換性維持が共通課題。ゲームは失敗時のユーザー離脱が即時に可視化される点で他業界の先行事例になり得る。</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>メーカー公認クリエイター（配信者）を競技の主役に据えた公式eスポーツイベントは、自動車・化粧品・食品などのアンバサダー/インフルエンサー起用マーケティングの何に該当するか？他業界でも『公認クリエイターリーグ』が成立するか？</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>スト6公式「Capcom Creators JP杯 Round 2」開幕（公認クリエイター12名・ホロライブ白上フブキらゲスト）</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>カプコン, ストリートファイター6, ホロライブ</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>広告・マーケティング（インフルエンサー起用）、エンタメ（タレント/VTuber IP）、小売（アンバサダー販促）</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="G31" s="5" t="inlineStr">
+        <is>
+          <t>公認クリエイターを“選手”として競わせる設計は、ブランドが自前のタレントリーグを持つ動きと同型。視聴・販促・採用導線を一体化でき、観戦型コンテンツのマーケ転用余地が大きい。</t>
         </is>
       </c>
     </row>
@@ -4603,7 +4640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L142"/>
+  <dimension ref="A1:L145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13540,6 +13577,189 @@
         </is>
       </c>
       <c r="L142" s="5" t="n"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B143" s="5" t="inlineStr">
+        <is>
+          <t>Paradox Interactive、Nasdaq Stockholm本市場へ上場区分を変更（時価総額約138億SEK）</t>
+        </is>
+      </c>
+      <c r="C143" s="5" t="inlineStr">
+        <is>
+          <t>https://www.marketscreener.com/news/first-day-of-trading-in-paradox-interactive-s-shares-on-nasdaq-stockholm-ce7f5dd3df8df42c</t>
+        </is>
+      </c>
+      <c r="D143" s="5" t="inlineStr">
+        <is>
+          <t>Paradoxはストラテジー大手で、従来は新興企業向けのNasdaq First North Growth Marketに上場していた。事業規模の拡大と投資家層の拡充を背景に、本則市場（Nasdaq Stockholmメインマーケット）への上場区分変更を申請していた。</t>
+        </is>
+      </c>
+      <c r="E143" s="5" t="inlineStr">
+        <is>
+          <t>6月9日にNasdaq Stockholm本市場での取引を開始し、First North Growth Marketからは上場廃止。新株発行は伴わず、ティッカー（PDX）・ISINは据え置き。上場区分変更時の時価総額は約138億スウェーデンクローナ。</t>
+        </is>
+      </c>
+      <c r="F143" s="5" t="inlineStr">
+        <is>
+          <t>新興市場→本則市場へのステップアップ上場
+新株発行・資金調達は伴わない区分変更
+ティッカーPDX・ISINは据え置き
+時価総額は約138億SEK</t>
+        </is>
+      </c>
+      <c r="G143" s="5" t="inlineStr">
+        <is>
+          <t>本則上場で機関投資家による組み入れ余地が広がり、流動性と知名度の向上が見込まれる。欧州ゲーム企業の資本市場での再評価が進む契機となり、他の新興上場スタジオの追随も意識される。</t>
+        </is>
+      </c>
+      <c r="H143" s="5" t="inlineStr">
+        <is>
+          <t>上場区分変更（アップリスティング）と資本市場戦略</t>
+        </is>
+      </c>
+      <c r="I143" s="5" t="inlineStr">
+        <is>
+          <t>Paradox Interactive</t>
+        </is>
+      </c>
+      <c r="J143" s="5" t="inlineStr">
+        <is>
+          <t>Crusader Kings, Europa Universalis, Stellaris, Cities: Skylines</t>
+        </is>
+      </c>
+      <c r="K143" s="5" t="inlineStr">
+        <is>
+          <t>業績,海外</t>
+        </is>
+      </c>
+      <c r="L143" s="5" t="n"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B144" s="5" t="inlineStr">
+        <is>
+          <t>「スト6」公式イベント「Capcom Creators JP杯 Round 2」開幕、特別ルール“トラップカード”導入</t>
+        </is>
+      </c>
+      <c r="C144" s="5" t="inlineStr">
+        <is>
+          <t>https://prtimes.jp/main/html/rd/p/000005813.000013450.html</t>
+        </is>
+      </c>
+      <c r="D144" s="5" t="inlineStr">
+        <is>
+          <t>カプコンは公認クリエイター制度「Capcom Creators」を通じ、配信者・実況者を巻き込んだ『ストリートファイター6』のコミュニティ拡大を進めてきた。その公式競技企画の第2弾が本イベントで、5月の予選を勝ち上がったメンバーも参加する。</t>
+        </is>
+      </c>
+      <c r="E144" s="5" t="inlineStr">
+        <is>
+          <t>6月13日18時よりYouTubeのCAPCOMチャンネルで開幕。CCJPメンバー12名が4チームに分かれて対戦し、試合展開を変える特別ルール「トラップカード」を導入。ホロライブの白上フブキやSF6開発陣がゲスト出演した。</t>
+        </is>
+      </c>
+      <c r="F144" s="5" t="inlineStr">
+        <is>
+          <t>公認クリエイター12名による4チーム対抗戦
+特別ルール「トラップカード」で波乱を演出
+ホロライブ白上フブキらがゲスト出演
+YouTube公式チャンネルで無料配信</t>
+        </is>
+      </c>
+      <c r="G144" s="5" t="inlineStr">
+        <is>
+          <t>メーカー公認クリエイターを主役にした公式競技イベントは、競技性より“観て盛り上がる”エンタメ性を重視する潮流を強める。タイトルの長期エンゲージメント施策として定着が見込まれる。</t>
+        </is>
+      </c>
+      <c r="H144" s="5" t="inlineStr">
+        <is>
+          <t>公認クリエイターを核にしたコミュニティ運営</t>
+        </is>
+      </c>
+      <c r="I144" s="5" t="inlineStr">
+        <is>
+          <t>カプコン</t>
+        </is>
+      </c>
+      <c r="J144" s="5" t="inlineStr">
+        <is>
+          <t>ストリートファイター6, Capcom Creators, ホロライブ</t>
+        </is>
+      </c>
+      <c r="K144" s="5" t="inlineStr">
+        <is>
+          <t>eスポーツ,国内</t>
+        </is>
+      </c>
+      <c r="L144" s="5" t="n"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B145" s="5" t="inlineStr">
+        <is>
+          <t>個人開発の無料音ゲー『CoLane』、Steam正式版を年内リリースへ。楽曲40曲以上を収録</t>
+        </is>
+      </c>
+      <c r="C145" s="5" t="inlineStr">
+        <is>
+          <t>https://automaton-media.com/articles/newsjp/colane-20260613-449560/</t>
+        </is>
+      </c>
+      <c r="D145" s="5" t="inlineStr">
+        <is>
+          <t>個人ゲーム開発者のハヤブサ氏による音楽ゲーム『CoLane』は、1つのノーツを複数キーで取れる独自システムが特徴。これまで無料のテスト版をPC向けに公開し、収録楽曲の公募も実施していた。音楽ゲームは同氏初の挑戦。</t>
+        </is>
+      </c>
+      <c r="E145" s="5" t="inlineStr">
+        <is>
+          <t>6月13日、Steamストアページを公開し、正式版を2026年内に無料でリリースすると発表。テスト版の10曲に公募採用の30曲以上を加え、計40曲超を無料提供する。スポットライトの色によってレーンが動的に変化する。</t>
+        </is>
+      </c>
+      <c r="F145" s="5" t="inlineStr">
+        <is>
+          <t>正式版は2026年内に無料リリース
+楽曲公募採用を含め40曲以上を収録
+スポットライトの色でレーンが変化する独自システム
+個人開発者にとって初の音ゲー挑戦</t>
+        </is>
+      </c>
+      <c r="G145" s="5" t="inlineStr">
+        <is>
+          <t>無料＋楽曲公募のモデルはコミュニティ主導の音ゲー文化と親和的で、配信映えする独自機構が話題化の鍵となる。個人開発でも独創的なシステムが国内外メディアの注目を集める流れが続く。</t>
+        </is>
+      </c>
+      <c r="H145" s="5" t="inlineStr">
+        <is>
+          <t>個人開発×無料配信×楽曲公募のコミュニティ戦略</t>
+        </is>
+      </c>
+      <c r="I145" s="5" t="inlineStr">
+        <is>
+          <t>ハヤブサ（個人開発者）</t>
+        </is>
+      </c>
+      <c r="J145" s="5" t="inlineStr">
+        <is>
+          <t>CoLane</t>
+        </is>
+      </c>
+      <c r="K145" s="5" t="inlineStr">
+        <is>
+          <t>インディー,国内</t>
+        </is>
+      </c>
+      <c r="L145" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
daily-news + cross-questions update (2026-06-14 22:11)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -2589,7 +2589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3745,6 +3745,80 @@
       <c r="G31" s="5" t="inlineStr">
         <is>
           <t>公認クリエイターを“選手”として競わせる設計は、ブランドが自前のタレントリーグを持つ動きと同型。視聴・販促・採用導線を一体化でき、観戦型コンテンツのマーケ転用余地が大きい。</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>ハード欠陥（Joy-Conドリフト）への当局制裁と無償修理義務化は、自動車・家電・スマホなど耐久消費財のリコール／製造物責任のどの段階に該当するか？</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>任天堂が仏DGCCRFと約35M€の制裁金で合意（Joy-Conドリフト問題、6月9日）</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>任天堂 / Nintendo Switch, Joy-Con</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>自動車（リコール制度）、家電（PL法対応）、スマホ（バッテリー回収）、医療機器（不具合報告義務）</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>不具合の『把握時期と公表の遅れ』が制裁の焦点になる構図は耐久財全般に共通。設計段階からの開示・回収体制がブランド毀損の防波堤になる。</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>大幅値上げ→大量解約→値下げという価格の揺り戻しは、動画配信・音楽・SaaS・新聞などサブスク業界共通の『価格弾力性の限界』をどう示すか？</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>Xbox幹部がGame Pass値上げで数百万人の解約を認め、$22.99へ値下げ（2026年）</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>Microsoft, Xbox / Xbox Game Pass</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>動画配信（Netflix等の値上げ）、音楽サブスク、SaaS（席課金見直し）、新聞・メディアの購読</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="inlineStr">
+        <is>
+          <t>値上げ余地はライブラリ価値とスイッチングコストに規定される。撤回コストが大きいため、ティア細分化や広告付き廉価プランで弾力性を吸収する設計が共通解になりつつある。</t>
         </is>
       </c>
     </row>
@@ -4640,7 +4714,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L145"/>
+  <dimension ref="A1:L155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13760,6 +13834,608 @@
         </is>
       </c>
       <c r="L145" s="5" t="n"/>
+    </row>
+    <row r="146">
+      <c r="A146" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B146" s="5" t="inlineStr">
+        <is>
+          <t>任天堂、仏当局とJoy-Conドリフト問題で約35M€（約40M$）の制裁金支払いに合意</t>
+        </is>
+      </c>
+      <c r="C146" s="5" t="inlineStr">
+        <is>
+          <t>https://www.engadget.com/2189455/nintendo-will-pay-a-dollar40-million-fine-for-faulty-joy-cons/</t>
+        </is>
+      </c>
+      <c r="D146" s="5" t="inlineStr">
+        <is>
+          <t>Switch初代から続くJoy-Conのスティック誤作動（ドリフト）問題で、仏競争・消費・不正抑止総局(DGCCRF)が任天堂欧州法人に対し誤認を招く商慣行があったと認定。任天堂は2018年に不具合を把握しつつ公表が2020年、無償修理開始は2023年と対応の遅れが問われた。</t>
+        </is>
+      </c>
+      <c r="E146" s="5" t="inlineStr">
+        <is>
+          <t>6月9日、任天堂欧州法人は約3,500万ユーロの制裁金支払いに合意した。任天堂は『故意に消費者を誤導していない』とし合意は有罪を認めるものではないと説明。仏サイトでの決定公表と該当地域での無償修理継続が条件に含まれる。英消費者団体Whichは初代Joy-Conの4割超がドリフトの影響を受けたと推計。</t>
+        </is>
+      </c>
+      <c r="F146" s="5" t="inlineStr">
+        <is>
+          <t>DGCCRFが欧州法人に約35M€の制裁金
+不具合把握(2018)から公表(2020)・無償修理(2023)まで対応遅延を認定
+任天堂は有罪認否せず合意で決着
+仏サイトでの決定公表＋無償修理継続が条件</t>
+        </is>
+      </c>
+      <c r="G146" s="5" t="inlineStr">
+        <is>
+          <t>ハード欠陥への当局制裁が定着すれば、メーカーは設計段階からの開示・リコール対応を前倒しせざるを得ず、品質保証コストと情報開示の透明性が競争要因になる。Switch 2世代でのコントローラ耐久性も注視点。</t>
+        </is>
+      </c>
+      <c r="H146" s="5" t="inlineStr">
+        <is>
+          <t>製造物責任・消費者保護規制とハード品質保証</t>
+        </is>
+      </c>
+      <c r="I146" s="5" t="inlineStr">
+        <is>
+          <t>任天堂</t>
+        </is>
+      </c>
+      <c r="J146" s="5" t="inlineStr">
+        <is>
+          <t>Nintendo Switch, Joy-Con</t>
+        </is>
+      </c>
+      <c r="K146" s="5" t="inlineStr">
+        <is>
+          <t>規制,海外</t>
+        </is>
+      </c>
+      <c r="L146" s="5" t="n"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B147" s="5" t="inlineStr">
+        <is>
+          <t>Ubisoft、2026年6度目の再編で2スタジオ閉鎖・約380人削減</t>
+        </is>
+      </c>
+      <c r="C147" s="5" t="inlineStr">
+        <is>
+          <t>https://www.engadget.com/2191677/ubisoft-reportedly-shuts-down-more-studios-and-lays-off-staff-in-barcelona-and-san-francisco</t>
+        </is>
+      </c>
+      <c r="D147" s="5" t="inlineStr">
+        <is>
+          <t>Ubisoftはカナダ・ウィニペグとセルビア・ベオグラードのスタジオを閉鎖し、バルセロナやサンフランシスコでも人員削減を実施。2026年だけで6度目の再編で、5月期の約15億ユーロ損失と2028年までの5億ユーロ規模のコスト削減計画が背景にある。</t>
+        </is>
+      </c>
+      <c r="E147" s="5" t="inlineStr">
+        <is>
+          <t>報道によれば、Ubisoftは2スタジオを閉鎖し少なくとも5拠点で計約380人を削減する。記録的な赤字決算を受けた構造改革の一環で、増収局面でも続くゲーム業界の人員整理を象徴する動き。今回のレイオフは報道規制（エンバーゴ）下で進められたとの指摘もあり、情報開示の姿勢にも批判が出ている。</t>
+        </is>
+      </c>
+      <c r="F147" s="5" t="inlineStr">
+        <is>
+          <t>ウィニペグ・ベオグラードの2スタジオ閉鎖
+少なくとも5拠点で計約380人削減
+2026年だけで6度目の再編
+5月期約15億ユーロ赤字／2028年まで5億ユーロ削減計画</t>
+        </is>
+      </c>
+      <c r="G147" s="5" t="inlineStr">
+        <is>
+          <t>大規模IP依存と開発費高騰が続く限り、四半期ごとの再編は常態化する見込み。Assassin's Creedなど主力IPの収益化と、Tencent出資の子会社切り出しによる再建の成否が今後の鍵。</t>
+        </is>
+      </c>
+      <c r="H147" s="5" t="inlineStr">
+        <is>
+          <t>増収下リストラと開発費高騰の構造</t>
+        </is>
+      </c>
+      <c r="I147" s="5" t="inlineStr">
+        <is>
+          <t>Ubisoft, Tencent</t>
+        </is>
+      </c>
+      <c r="J147" s="5" t="inlineStr">
+        <is>
+          <t>Assassin's Creed</t>
+        </is>
+      </c>
+      <c r="K147" s="5" t="inlineStr">
+        <is>
+          <t>業績,海外</t>
+        </is>
+      </c>
+      <c r="L147" s="5" t="n"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B148" s="5" t="inlineStr">
+        <is>
+          <t>Xbox幹部、Game Pass値上げで『数百万人』解約と認める—$22.99へ値下げ</t>
+        </is>
+      </c>
+      <c r="C148" s="5" t="inlineStr">
+        <is>
+          <t>https://www.windowscentral.com/gaming/xbox/xbox-executive-game-pass-lost-millions-of-subscribers-impact-of-price-hikes</t>
+        </is>
+      </c>
+      <c r="D148" s="5" t="inlineStr">
+        <is>
+          <t>Microsoftは2025年10月にGame Pass Ultimateを月19.99→29.99ドルへ約50%値上げしたが、解約が相次ぎ2026年に22.99ドルへ引き下げ。新作CoDのDay1提供も見直すなど、サブスク価格戦略の試行錯誤が続いている。</t>
+        </is>
+      </c>
+      <c r="E148" s="5" t="inlineStr">
+        <is>
+          <t>Xbox幹部は値上げが『数百万人』の解約に直結したと公に認めた。価格を22.99ドルへ戻し一部特典を縮小した結果、契約者の再成長と継続率改善が報告されている。ゲームのサブスクが価格弾力性の限界に直面したことを示す事例で、収益最大化と会員規模のトレードオフが鮮明になった。</t>
+        </is>
+      </c>
+      <c r="F148" s="5" t="inlineStr">
+        <is>
+          <t>2025年10月の約50%値上げで数百万人が解約
+2026年に29.99→22.99ドルへ値下げ
+新作CoDのDay1提供を見直し
+値下げ後は会員再成長・継続率改善を報告</t>
+        </is>
+      </c>
+      <c r="G148" s="5" t="inlineStr">
+        <is>
+          <t>値上げ→解約→値下げの揺り戻しは、コンテンツ単価とライブラリ価値の再評価を促す。今後はティア細分化や広告付き廉価プラン、年間契約の比重拡大など、価格設計の多様化が進む可能性。</t>
+        </is>
+      </c>
+      <c r="H148" s="5" t="inlineStr">
+        <is>
+          <t>サブスク価格弾力性とLTV設計</t>
+        </is>
+      </c>
+      <c r="I148" s="5" t="inlineStr">
+        <is>
+          <t>Microsoft, Xbox, Activision Blizzard</t>
+        </is>
+      </c>
+      <c r="J148" s="5" t="inlineStr">
+        <is>
+          <t>Xbox Game Pass, Call of Duty</t>
+        </is>
+      </c>
+      <c r="K148" s="5" t="inlineStr">
+        <is>
+          <t>業績,海外</t>
+        </is>
+      </c>
+      <c r="L148" s="5" t="n"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B149" s="5" t="inlineStr">
+        <is>
+          <t>Summer Game Fest 2026、FF7リメイク三部作完結編をフル公開—大型リビール相次ぐ</t>
+        </is>
+      </c>
+      <c r="C149" s="5" t="inlineStr">
+        <is>
+          <t>https://kotaku.com/the-13-biggest-video-game-reveals-and-surprises-from-all-of-sgfs-showcases-2000704059</t>
+        </is>
+      </c>
+      <c r="D149" s="5" t="inlineStr">
+        <is>
+          <t>6月5日に約2時間開催されたSummer Game Fest 2026本編とその周辺ショーケースで、新旧の大型タイトルが多数発表。E3不在後の夏の発表会の中心イベントとして定着し、各社の独占・マルチ展開戦略が見える場になっている。</t>
+        </is>
+      </c>
+      <c r="E149" s="5" t="inlineStr">
+        <is>
+          <t>本編の目玉はFF7リメイク三部作の完結編フル公開。ほかにResident Evil Veronica、Alien Isolation 2、Guild Wars 3、Until Dawn 2、進撃の巨人3などが明らかになった。Sonic Racing: CrossWorldsはTMNTやゴジラ、エヴァンゲリオンとのクロスオーバーDLCを発表し、コラボ前提のIP拡張が鮮明に。</t>
+        </is>
+      </c>
+      <c r="F149" s="5" t="inlineStr">
+        <is>
+          <t>FF7リメイク三部作の完結編をフル公開
+バイオRE Veronica・Alien Isolation 2・Guild Wars 3など
+Until Dawn 2は原作元と別スタジオが開発
+Sonic Racingがゴジラ・エヴァ等とコラボDLC</t>
+        </is>
+      </c>
+      <c r="G149" s="5" t="inlineStr">
+        <is>
+          <t>既存IPのリメイク・続編とクロスオーバーDLCが発表の主軸に。新規IPより安全志向が強まる一方、配信映えする話題作りでローンチ前の関心を最大化する設計が標準化する。</t>
+        </is>
+      </c>
+      <c r="H149" s="5" t="inlineStr">
+        <is>
+          <t>夏商戦のショーケース戦略とIP再活用</t>
+        </is>
+      </c>
+      <c r="I149" s="5" t="inlineStr">
+        <is>
+          <t>Square Enix, Capcom, Sega, Sony</t>
+        </is>
+      </c>
+      <c r="J149" s="5" t="inlineStr">
+        <is>
+          <t>FINAL FANTASY VII, Resident Evil, Sonic Racing</t>
+        </is>
+      </c>
+      <c r="K149" s="5" t="inlineStr">
+        <is>
+          <t>新作,海外</t>
+        </is>
+      </c>
+      <c r="L149" s="5" t="n"/>
+    </row>
+    <row r="150">
+      <c r="A150" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B150" s="5" t="inlineStr">
+        <is>
+          <t>Google Cloud、ゲーム開発向け自律型AIエージェント群を本格投入</t>
+        </is>
+      </c>
+      <c r="C150" s="5" t="inlineStr">
+        <is>
+          <t>https://www.gamedeveloper.com/production/google-cloud-s-vision-for-ai-in-the-game-industry</t>
+        </is>
+      </c>
+      <c r="D150" s="5" t="inlineStr">
+        <is>
+          <t>Google CloudはGDC 2026で『Living Games』構想の次段階として、Gemini基盤の自律型AIエージェント群を発表。アセット制作・プレイテスト・ローカライズなどの工程自動化と、学習データ・生成物双方をカバーする知財補償を打ち出した。</t>
+        </is>
+      </c>
+      <c r="E150" s="5" t="inlineStr">
+        <is>
+          <t>Google Cloudはクラウド型ゲーム開発の重労働を肩代わりする自律エージェント群を展開。Gemini連携ツールで高騰する制作コストの圧縮を狙い、業界初をうたう二段構えの知財補償で訓練データと生成物の法的リスクに対応する。開発者の97%が既にAIをアセット制作やテストに活用しているとされ、AI前提の制作体制が広がる。</t>
+        </is>
+      </c>
+      <c r="F150" s="5" t="inlineStr">
+        <is>
+          <t>GeminiベースのAIエージェントで工程自動化
+アセット制作・テスト・ローカライズを効率化
+学習データと生成物の双方を知財補償
+開発者の97%が既にAIを制作に活用</t>
+        </is>
+      </c>
+      <c r="G150" s="5" t="inlineStr">
+        <is>
+          <t>AIの守備範囲が裏方効率化から制作中核へ広がるほど、生成物の出自表示や権利処理が品質・信頼のシグナルになる。プラットフォーマー間でAI開発基盤と補償条件の競争が激化する見込み。</t>
+        </is>
+      </c>
+      <c r="H150" s="5" t="inlineStr">
+        <is>
+          <t>生成AIの工程統合と知財補償モデル</t>
+        </is>
+      </c>
+      <c r="I150" s="5" t="inlineStr">
+        <is>
+          <t>Google, Alphabet</t>
+        </is>
+      </c>
+      <c r="J150" s="5" t="inlineStr">
+        <is>
+          <t>Gemini, Google Cloud</t>
+        </is>
+      </c>
+      <c r="K150" s="5" t="inlineStr">
+        <is>
+          <t>技術,海外</t>
+        </is>
+      </c>
+      <c r="L150" s="5" t="n"/>
+    </row>
+    <row r="151">
+      <c r="A151" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B151" s="5" t="inlineStr">
+        <is>
+          <t>コーエーテクモゲームス、子会社ガストを吸収合併し主力ブランドを集約</t>
+        </is>
+      </c>
+      <c r="C151" s="5" t="inlineStr">
+        <is>
+          <t>https://gamebiz.jp/news/132851</t>
+        </is>
+      </c>
+      <c r="D151" s="5" t="inlineStr">
+        <is>
+          <t>コーエーテクモゲームスは『アトリエ』シリーズなどで知られるガストを吸収合併すると発表。グループ内に分散していた開発機能とIPを集約し、ブランド価値の最大化と開発効率の向上を図る再編の一環。</t>
+        </is>
+      </c>
+      <c r="E151" s="5" t="inlineStr">
+        <is>
+          <t>ガストは合併後『ガスト長野開発部』として存続し、開発拠点とチームは維持される。コーエーテクモはIPと人材を本体に統合することで意思決定を迅速化し、『アトリエ』など主力ブランドの世界展開を強化する狙い。国内大手による子会社の組織再編・ブランド集約の典型例といえる。</t>
+        </is>
+      </c>
+      <c r="F151" s="5" t="inlineStr">
+        <is>
+          <t>ガストを吸収合併しIP・開発機能を集約
+合併後は『ガスト長野開発部』として存続
+ブランド価値最大化と開発効率向上が目的
+『アトリエ』など主力IPの世界展開を強化</t>
+        </is>
+      </c>
+      <c r="G151" s="5" t="inlineStr">
+        <is>
+          <t>グループ内再編によるブランド集約は、分散した中小スタジオを抱える大手で今後も進む見込み。IP一元管理とマルチプラットフォーム展開の加速が競争力を左右する。</t>
+        </is>
+      </c>
+      <c r="H151" s="5" t="inlineStr">
+        <is>
+          <t>グループ内組織再編とIP集約戦略</t>
+        </is>
+      </c>
+      <c r="I151" s="5" t="inlineStr">
+        <is>
+          <t>コーエーテクモゲームス, ガスト</t>
+        </is>
+      </c>
+      <c r="J151" s="5" t="inlineStr">
+        <is>
+          <t>アトリエシリーズ</t>
+        </is>
+      </c>
+      <c r="K151" s="5" t="inlineStr">
+        <is>
+          <t>M&amp;A,国内</t>
+        </is>
+      </c>
+      <c r="L151" s="5" t="n"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B152" s="5" t="inlineStr">
+        <is>
+          <t>Globant『Game On 2026』レポート、ゲームの未来を再定義する5つの力を提示</t>
+        </is>
+      </c>
+      <c r="C152" s="5" t="inlineStr">
+        <is>
+          <t>https://www.barchart.com/story/news/36185681/globant-s-game-on-report-reveals-five-forces-redefining-gaming-s-digital-future-in-2026</t>
+        </is>
+      </c>
+      <c r="D152" s="5" t="inlineStr">
+        <is>
+          <t>Globantが2026年のゲーム開発とプレイヤー嗜好の潮流をまとめた『Game On』レポートを公開。AI活用、ポータブル/クラウド端末の普及、プレイヤー体験のパーソナライズなど、業界の構造を変える複数の力を分析した。</t>
+        </is>
+      </c>
+      <c r="E152" s="5" t="inlineStr">
+        <is>
+          <t>レポートは2026年のゲーミングを再定義する5つの力を提示。開発者の97%がアセット制作・プレイテスト・ローカライズの高速化にAIを活用し、ポータブル機やクラウド基盤が『どこで・どう遊ぶか』を変えていると指摘する。技術導入の巧拙が開発コストとプレイヤー体験の質を左右する局面に入ったことを示す。</t>
+        </is>
+      </c>
+      <c r="F152" s="5" t="inlineStr">
+        <is>
+          <t>ゲームの未来を再定義する5つの力を提示
+開発者の97%がAIを制作工程に活用
+ポータブル/クラウド端末がプレイ環境を変革
+体験のパーソナライズが競争軸に</t>
+        </is>
+      </c>
+      <c r="G152" s="5" t="inlineStr">
+        <is>
+          <t>AIとクラウド/ポータブルの普及で、制作の効率化とプレイ環境の流動化が同時進行。スタジオは技術投資の優先順位付けと、AI生成物の品質・権利管理の体制づくりが急務になる。</t>
+        </is>
+      </c>
+      <c r="H152" s="5" t="inlineStr">
+        <is>
+          <t>ゲーム業界のAI・クラウド構造変化</t>
+        </is>
+      </c>
+      <c r="I152" s="5" t="inlineStr">
+        <is>
+          <t>Globant</t>
+        </is>
+      </c>
+      <c r="J152" s="5" t="n"/>
+      <c r="K152" s="5" t="inlineStr">
+        <is>
+          <t>技術,海外</t>
+        </is>
+      </c>
+      <c r="L152" s="5" t="n"/>
+    </row>
+    <row r="153">
+      <c r="A153" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B153" s="5" t="inlineStr">
+        <is>
+          <t>Nintendo Switch 2、累計1,700万台超で任天堂史上最速のベストセラー機に</t>
+        </is>
+      </c>
+      <c r="C153" s="5" t="inlineStr">
+        <is>
+          <t>https://variety.com/2026/gaming/news/nintendo-switch-2-sales-17-million-1236650699/</t>
+        </is>
+      </c>
+      <c r="D153" s="5" t="inlineStr">
+        <is>
+          <t>2025年6月に発売されたSwitch 2は発売1年で英国でも歴代6番目の速さで100万台に到達するなど好調。一方で日本では5月25日の値上げ後に週販が急減し、9月予定の世界的値上げを前にした駆け込み需要と西側市場での減速懸念が併存する。</t>
+        </is>
+      </c>
+      <c r="E153" s="5" t="inlineStr">
+        <is>
+          <t>Switch 2は累計販売が1,700万台を超え、任天堂史上最速ペースのベストセラーハードになったと報じられた。日本では値上げで週販が前週比約87%減となった一方、累計は586万台を維持。普及2年目はソフト供給とハード価格戦略のバランスが販売モメンタムを左右する局面に入った。</t>
+        </is>
+      </c>
+      <c r="F153" s="5" t="inlineStr">
+        <is>
+          <t>累計1,700万台超で任天堂史上最速のベストセラー機
+英国で歴代6番目の速さで100万台到達
+日本は値上げ後に週販約87%減、累計586万台
+9月の世界的値上げ前後で需要変動の見通し</t>
+        </is>
+      </c>
+      <c r="G153" s="5" t="inlineStr">
+        <is>
+          <t>値上げによる地域別の需要変動が顕在化。年末商戦に向けたファースト/サードの大型タイトル供給と、価格改定後の西側市場の反応がFY27の業績見通しを左右する。</t>
+        </is>
+      </c>
+      <c r="H153" s="5" t="inlineStr">
+        <is>
+          <t>ハード普及曲線と価格弾力性</t>
+        </is>
+      </c>
+      <c r="I153" s="5" t="inlineStr">
+        <is>
+          <t>任天堂</t>
+        </is>
+      </c>
+      <c r="J153" s="5" t="inlineStr">
+        <is>
+          <t>Nintendo Switch 2</t>
+        </is>
+      </c>
+      <c r="K153" s="5" t="inlineStr">
+        <is>
+          <t>業績,海外</t>
+        </is>
+      </c>
+      <c r="L153" s="5" t="n"/>
+    </row>
+    <row r="154">
+      <c r="A154" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B154" s="5" t="inlineStr">
+        <is>
+          <t>LoL『LCK 2026 Road to MSI』でT1が優勝、ピーク218万人で歴代3例目の200万超</t>
+        </is>
+      </c>
+      <c r="C154" s="5" t="inlineStr">
+        <is>
+          <t>https://escharts.com/news/lck-2026-road-msi-recap</t>
+        </is>
+      </c>
+      <c r="D154" s="5" t="inlineStr">
+        <is>
+          <t>韓国LoLリーグLCKのMSI出場をかけた『Road to MSI』で、T1が接戦を制し国際大会への切符を獲得。視聴がモバイル/ライブ配信へシフトするなか、地域リーグの注目試合が世界的な視聴規模を集める傾向が続いている。</t>
+        </is>
+      </c>
+      <c r="E154" s="5" t="inlineStr">
+        <is>
+          <t>決勝でT1が3-2で勝利し、ピーク同時視聴218万人を記録。これはLCK全大会で3例目となる200万視聴超えで、地域リーグでもトップ層の試合がグローバル規模の関心を集めることを示した。2026年の世界eスポーツ視聴人口は約6.4億人に達するとされ、人気タイトルの主要試合が視聴の牽引役になっている。</t>
+        </is>
+      </c>
+      <c r="F154" s="5" t="inlineStr">
+        <is>
+          <t>T1が3-2でMSI出場権を獲得
+ピーク同時視聴218万人を記録
+LCK全大会で3例目の200万超
+2026年の世界eスポーツ視聴人口は約6.4億人</t>
+        </is>
+      </c>
+      <c r="G154" s="5" t="inlineStr">
+        <is>
+          <t>地域リーグの注目カードが国際大会級の視聴を集める構図が定着。モバイル/ライブ配信視聴の比重が高まり、放映権・スポンサー価値の評価軸も同接ピークとリーチへ移っていく。</t>
+        </is>
+      </c>
+      <c r="H154" s="5" t="inlineStr">
+        <is>
+          <t>eスポーツ視聴指標とメディア価値</t>
+        </is>
+      </c>
+      <c r="I154" s="5" t="inlineStr">
+        <is>
+          <t>Riot Games, T1</t>
+        </is>
+      </c>
+      <c r="J154" s="5" t="inlineStr">
+        <is>
+          <t>League of Legends, LCK, MSI</t>
+        </is>
+      </c>
+      <c r="K154" s="5" t="inlineStr">
+        <is>
+          <t>eスポーツ,海外</t>
+        </is>
+      </c>
+      <c r="L154" s="5" t="n"/>
+    </row>
+    <row r="155">
+      <c r="A155" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B155" s="5" t="inlineStr">
+        <is>
+          <t>中国ゲーム大手テンセント・ネットイース、世界的評価額低迷下で海外買収を加速</t>
+        </is>
+      </c>
+      <c r="C155" s="5" t="inlineStr">
+        <is>
+          <t>https://36kr.jp/202621/</t>
+        </is>
+      </c>
+      <c r="D155" s="5" t="inlineStr">
+        <is>
+          <t>世界のゲーム企業の評価額が低水準にあるなか、テンセントやネットイースなど中国大手が割安となった海外スタジオやIPへの出資・買収を相次いで進めている。国内市場の成熟と規制を背景に、海外展開と知財獲得を成長戦略の柱に据える動き。</t>
+        </is>
+      </c>
+      <c r="E155" s="5" t="inlineStr">
+        <is>
+          <t>テンセント・ネットイースは評価額が下がった局面を好機と捉え、欧米・日本のスタジオやIPへの出資を積み増している。安値での持分取得により、開発力とグローバルIPポートフォリオを拡充する狙い。日系エンタメへの相次ぐ出資も含め、中国マネーがゲーム業界の資本構造に与える影響が拡大している。</t>
+        </is>
+      </c>
+      <c r="F155" s="5" t="inlineStr">
+        <is>
+          <t>中国大手が評価額低迷を好機に海外買収を加速
+テンセント・ネットイースが欧米・日本のスタジオ/IPに出資
+国内市場の成熟と規制が海外志向を後押し
+日系エンタメへの出資も拡大</t>
+        </is>
+      </c>
+      <c r="G155" s="5" t="inlineStr">
+        <is>
+          <t>評価額が低位で推移する間は、潤沢な資本を持つ中国大手による出資・買収が続く見込み。被買収側の独立性確保や各国の外資・安全保障審査が今後の取引のハードルになる。</t>
+        </is>
+      </c>
+      <c r="H155" s="5" t="inlineStr">
+        <is>
+          <t>クロスボーダーM&amp;Aと資本再編</t>
+        </is>
+      </c>
+      <c r="I155" s="5" t="inlineStr">
+        <is>
+          <t>Tencent, NetEase</t>
+        </is>
+      </c>
+      <c r="J155" s="5" t="n"/>
+      <c r="K155" s="5" t="inlineStr">
+        <is>
+          <t>M&amp;A,海外</t>
+        </is>
+      </c>
+      <c r="L155" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
weekly-stocks + IP watch update (2026-06-15 03:34)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -15570,8 +15570,16 @@
           <t>日本</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr"/>
-      <c r="E3" s="9" t="inlineStr"/>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>6/9のニンダイで『ゼルダの伝説 時のオカリナ』のSwitch 2向けリメイクを正式発表。名作3DタイトルのリメイクとしてSGF/ニンダイ最大級の話題に。</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>ゼルダの伝説 時のオカリナ リメイク（Switch 2、2026年後半予定）</t>
+        </is>
+      </c>
       <c r="F3" s="9" t="inlineStr"/>
       <c r="G3" s="9" t="inlineStr">
         <is>
@@ -15579,7 +15587,11 @@
         </is>
       </c>
       <c r="H3" s="9" t="inlineStr"/>
-      <c r="I3" s="9" t="inlineStr"/>
+      <c r="I3" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
@@ -15597,8 +15609,16 @@
           <t>日本</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr"/>
-      <c r="E4" s="9" t="inlineStr"/>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>6/9のニンダイで『スカーレット・バイオレット』向け有料追加コンテンツ（DLC）が告知され、既存タイトルの追加展開が継続。</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>ポケモンSV 有料DLC（2026予定）</t>
+        </is>
+      </c>
       <c r="F4" s="9" t="inlineStr"/>
       <c r="G4" s="9" t="inlineStr">
         <is>
@@ -15606,7 +15626,11 @@
         </is>
       </c>
       <c r="H4" s="9" t="inlineStr"/>
-      <c r="I4" s="9" t="inlineStr"/>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -15759,8 +15783,16 @@
           <t>日本</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr"/>
-      <c r="E10" s="9" t="inlineStr"/>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>6/9のニンダイで『キングダムハーツIV』の新規映像が公開され、開発進捗が示された。</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>キングダムハーツIV（Switch 2含むマルチ、発売時期未定）</t>
+        </is>
+      </c>
       <c r="F10" s="9" t="inlineStr"/>
       <c r="G10" s="9" t="inlineStr">
         <is>
@@ -15768,7 +15800,11 @@
         </is>
       </c>
       <c r="H10" s="9" t="inlineStr"/>
-      <c r="I10" s="9" t="inlineStr"/>
+      <c r="I10" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
@@ -16185,8 +16221,16 @@
           <t>日本</t>
         </is>
       </c>
-      <c r="D24" s="9" t="inlineStr"/>
-      <c r="E24" s="9" t="inlineStr"/>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>6/9のニンダイでシリーズ最新作『信長の野望・主世』を2026年冬発売と発表。看板シミュレーションの新作が確定。</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>信長の野望・主世（2026年冬予定）</t>
+        </is>
+      </c>
       <c r="F24" s="9" t="inlineStr"/>
       <c r="G24" s="9" t="inlineStr">
         <is>
@@ -16194,7 +16238,11 @@
         </is>
       </c>
       <c r="H24" s="9" t="inlineStr"/>
-      <c r="I24" s="9" t="inlineStr"/>
+      <c r="I24" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
@@ -17369,7 +17417,7 @@
       </c>
       <c r="M2" s="9" t="inlineStr">
         <is>
-          <t>Switch 2発売後初の通期。5/8にFY26/3決算発表。株価は決算を挟み上下し6月初は7,600円前後、6/5時点で予想PER27.9倍・予想配当利回り2.15%。Summer Game Fest 2026でモンハンWildsのSwitch 2版開発が確認され同社ソフト供給期待が高まる。</t>
+          <t>6/9に「Nintendo Direct 2026.6.9」を配信し、ゼルダ『時のオカリナ』Switch 2リメイク、ゼノブレイド新作、KH4新映像など2026年後半タイトルを公開。同日にフランス当局の制裁金約65億円報道も。株価は6/9の7,738円から普及ペース懸念で6/12は7,174円へ反落（6/10は-6.76%）、大手証券が6/12にレーティング中立据え置き・目標株価を8,300円へ引き下げ。Switch 2値上げ後の普及速度が引き続き焦点。</t>
         </is>
       </c>
       <c r="N2" s="9" t="inlineStr">
@@ -17389,7 +17437,7 @@
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -17424,7 +17472,7 @@
       </c>
       <c r="M3" s="9" t="inlineStr">
         <is>
-          <t>6/1の株価は3,562円(+3.43%)。来期会社計画は売上12.3兆円・営業益1.6兆円と増益基調。半導体・金融含むグループ全体は堅調で、ゲーム(G&amp;NS)はPS5後半サイクルとネットワークサービスが軸。</t>
+          <t>6/8の株価は3,508円前後。5月発表の最大5,000億円の自社株買いを継続し5月末までに約1,900万株を取得、株主還元姿勢が下支え。音楽事業は増収増益と好調でカタログ取得も加速。一方ゲームはPS5販売が前年同期比約15%減とサイクル後半入りが鮮明。アナリスト平均目標株価は約4,657円で、現値からの上値余地を見込む声が多い。</t>
         </is>
       </c>
       <c r="N3" s="9" t="inlineStr">
@@ -17444,7 +17492,7 @@
       </c>
       <c r="Q3" s="9" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -17479,7 +17527,7 @@
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>6/3株価2,945円(-2.45%)。5/13発表のFY26/3決算は経常益前期比+12%で10期連続最高益、1円増配。6/5にSwitch 2版『ストリートファイター6』『祇:Path of the Goddess』発売。SGF2026でモンハンWildsのSwitch 2版と大型拡張『Ascendance』(2027世界配信)を発表。</t>
+          <t>先週末発表の『バイオハザード RE:Veronica』『モンハンWilds:Ascendance』（ともに2027年）を好感し6/8は+5.06%の3,031円。6/9のニンダイで『鬼武者 Way of the Sword』を9/25発売と告知。ただ6/10は任天堂主導のゲームセクター調整で連れ安。10期連続最高益のIP基盤は不変で、Switch 2展開と2027年の大型パイプラインが評価軸。</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
@@ -17499,7 +17547,7 @@
       </c>
       <c r="Q4" s="9" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -17546,7 +17594,7 @@
       </c>
       <c r="M5" s="9" t="inlineStr">
         <is>
-          <t>6/5株価2,518.5円(+1.61%)。FY26/3は売上2,976.61億(前期比-8.3%)も営業益547.36億(+34.9%)・純益296.16億(+21.3%)と構造改革で増益。FY27/3は売上横ばい・営業益490億(-10.5%)の保守的計画。HDゲーム選別と開発効率化が継続テーマ。</t>
+          <t>FY26/3は売上2,976.61億（-8.3%）も営業益547.36億（+34.9%）・純益296.16億（+21.3%）と構造改革で増益。6/9のニンダイで『キングダムハーツIV』の新規映像が公開され話題化。FY27/3は売上横ばい・営業益490億（-10.5%）の保守的計画で、HDゲーム選別と開発効率化が継続テーマ。</t>
         </is>
       </c>
       <c r="N5" s="9" t="inlineStr">
@@ -17566,7 +17614,7 @@
       </c>
       <c r="Q5" s="9" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -17802,7 +17850,7 @@
       </c>
       <c r="M9" s="9" t="inlineStr">
         <is>
-          <t>FY26/3は売上883.93億(+6.3%)・営業益371.68億(+15.7%)で売上・経常・純益とも過去最高。大型新作含む新作が寄与。FY27/3は人的資本投資増で経常益420億(-26.3%)とアナリスト予想下回る減益計画。配当は当期66円・次期48円予想。</t>
+          <t>FY26/3は売上883.93億（+6.3%）・営業益371.68億（+15.7%）で過去最高。6/9のニンダイで看板SLG最新作『信長の野望・主世』を2026年冬発売と発表し、定番シリーズの新作投入が確認された。FY27/3は人的資本投資増で経常益420億（-26.3%）と減益計画。新作サイクルと海外/IPコラボ展開が鍵。</t>
         </is>
       </c>
       <c r="N9" s="9" t="inlineStr">
@@ -17822,7 +17870,7 @@
       </c>
       <c r="Q9" s="9" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -17865,7 +17913,7 @@
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>FY26/3は売上1,713.69億(+10.7%)も営業益222.56億(-16.3%)と減益。スポーツ事業が成長する一方、主力モンストの減収と費用増が重し。FY27/3は売上1,850億(+8.0%)・営業益195億(-12.4%)計画。PointsBet連結化でベッティング拡大。</t>
+          <t>FY26/3は売上1,713.69億（+10.7%）も営業益222.56億（-16.3%）と減益。6/11のゲーム株概況でミクシィは上昇し、目標株価2万円を見込むアナリストも登場するなど、スポーツ・ベッティング事業（PointsBet連結）の成長期待が再評価。一方で主力モンストの減収は継続課題。スポーツ収益化とモンスト再活性化が引き続き焦点。</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
@@ -17885,7 +17933,7 @@
       </c>
       <c r="Q10" s="9" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -17983,7 +18031,7 @@
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>FY26/3は売上収益1,477億(-9.9%)・営業益186.94億(-35.5%)。『ポケポケ(Pokémon TCG Pocket)』初速の反動でゲーム事業が減収減益。ライブストリーミングは黒字転換。5/13株価2,559円(-3.83%)。FY27/3は売上1,540億(+4.3%)・営業益150億(-19.8%)計画。</t>
+          <t>FY26/3は売上収益1,477億（-9.9%）・営業益186.94億（-35.5%）とポケポケ初速の反動で減益。6/11のゲーム株概況ではミクシィ上昇の一方でDeNAは下落。ライブストリーミングは黒字転換し、FY27/3は売上1,540億（+4.3%）・営業益150億（-19.8%）計画。新規タイトル投入とヘルスケア/スポーツ事業の収益化が課題。</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
@@ -18003,7 +18051,7 @@
       </c>
       <c r="Q12" s="9" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -18206,7 +18254,7 @@
       </c>
       <c r="L2" s="9" t="inlineStr">
         <is>
-          <t>Xboxは6/30の会計年度末までに数年来最大級となる4度目のレイオフ実施見込み。Activision統合でゲーム売上は増えるが、ハード収益減・Game Pass伸び悩みで構造改革継続。中欧の流通体制も再編。会社全体はAI/クラウド優先。</t>
+          <t>Bloomberg（6/10）などが、Xboxが6/30の年度末後に数千人規模の大型レイオフを準備と報道。新ゲーム部門CEOのAsha Sharma氏が『事業が拡大しすぎた、優先順位を再評価する』と社内に伝達し、Game Pass等の高粗利サービスと収益性重視へ転換。マーケや一部予算も削減見込み。Activision/Bethesda等の巨大IPは維持しつつ構造改革を継続。</t>
         </is>
       </c>
       <c r="M2" s="9" t="inlineStr">
@@ -18216,17 +18264,17 @@
       </c>
       <c r="N2" s="9" t="inlineStr">
         <is>
-          <t>Xbox事業の連続レイオフ・ハード弱含み</t>
+          <t>Xbox事業の連続レイオフ・組織再編、ハード弱含み</t>
         </is>
       </c>
       <c r="O2" s="9" t="inlineStr">
         <is>
-          <t>マルチプラットフォーム化とGame Passの収益最適化</t>
+          <t>新CEO Sharma体制での収益性改善とGame Pass最適化</t>
         </is>
       </c>
       <c r="P2" s="9" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -18264,7 +18312,7 @@
       </c>
       <c r="L3" s="9" t="inlineStr">
         <is>
-          <t>FY26 Net Bookingsは$6.72bn、FY27は$8.0〜8.2bnへ大幅増の初期ガイダンス。GTA6が11/19発売予定で初年度3,500万本超(Piper予測)。株価は直近5営業日+8.6%、3月安値から+28.8%。Piper Sandlerがオーバーウェイト・目標$280で新規カバー。</t>
+          <t>FY26 Net Bookingsは$6.72bn、FY27は$8.0〜8.2bnへ大幅増ガイダンス。CEOゼルニック氏はGTA6を11/19発売と再明言し『延期しない』と強調、本格マーケティングは6月下旬以降に始動予定。GTA6初年度は3,500万本超予測。発売実現と立ち上げがFY27最高業績の鍵で、期待先行の高バリュエーションはリスク。</t>
         </is>
       </c>
       <c r="M3" s="9" t="inlineStr">
@@ -18284,7 +18332,7 @@
       </c>
       <c r="P3" s="9" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -18322,7 +18370,7 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>PIF/Silver Lake/Affinity連合による$210/株・総額約$550億の非公開化が進行、6/30までの完了見込みでCFIUS審査が最終関門(史上最大のLBO)。FY26はNet Bookings $8,026M(+9%)で過去最高、Battlefield 6がフランチャイズ最高の年・Apexも二桁回復。</t>
+          <t>PIF/Silver Lake/Affinity連合による$210/株・総額約$550億の非公開化は6/30のロングストップに向け進行中で、CFIUS審査が最終関門（契約上の最終期限は9/28）。現時点で正式な反対報道はなし。四半期配当$0.19は6/17支払い。FY26はNet Bookings $8,026M（+9%）で過去最高、Battlefield 6がフランチャイズ最高の年。買収完了の可否が当面の最大焦点。</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
@@ -18342,7 +18390,7 @@
       </c>
       <c r="P4" s="9" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -18700,7 +18748,7 @@
       </c>
       <c r="L11" s="9" t="inlineStr">
         <is>
-          <t>6/7株価$41.75・年初来-42%。年齢確認/児童安全機能の強化が短期のユーザー成長を圧迫するとして通期ブッキング見通しを下方修正。5〜8歳向け『Roblox Kids』・9〜15歳向け『Roblox Select』を6月初に展開。Q1売上は$1.4bn(+39%)。アナリスト平均目標$64.81。</t>
+          <t>6/12終値$43.31、年初来約-47%と低迷も、6/9にロシア政府機関が同プラットフォームの利用制限解除を検討との報道で株価が反発。5〜15歳向けの年齢別アカウントや児童安全機能を6月に展開し、$30億の自社株買いも実施。Q1売上は約$1.4bn（+39%）だが、安全対応がユーザー成長の短期摩擦に。年齢別アカウント定着と通期ブッキング回復が鍵。</t>
         </is>
       </c>
       <c r="M11" s="9" t="inlineStr">
@@ -18720,7 +18768,7 @@
       </c>
       <c r="P11" s="9" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>
@@ -18752,11 +18800,31 @@
           <t>Unityエンジン/ironSource</t>
         </is>
       </c>
-      <c r="L12" s="9" t="inlineStr"/>
-      <c r="M12" s="9" t="inlineStr"/>
-      <c r="N12" s="9" t="inlineStr"/>
-      <c r="O12" s="9" t="inlineStr"/>
-      <c r="P12" s="9" t="inlineStr"/>
+      <c r="L12" s="9" t="inlineStr">
+        <is>
+          <t>6/5にEdgewater ResearchがモバイルメディアのUnity・AppLovinをともにOutperformへ格上げし、広告課金型への業界シフトを評価。これを受けUnity株は約+5%。5月に開発ワークフローへ統合する『Unity AI』が公開ベータ入りし、コーディングやアセット生成の自動化で生産性向上を訴求。広告事業の回復とAI機能の収益化が当面の焦点。</t>
+        </is>
+      </c>
+      <c r="M12" s="9" t="inlineStr">
+        <is>
+          <t>広告事業の底打ちとUnity AIによる生産性向上、アナリスト格上げ</t>
+        </is>
+      </c>
+      <c r="N12" s="9" t="inlineStr">
+        <is>
+          <t>エンジン課金モデルの信頼回復途上、広告は競合と価格競争</t>
+        </is>
+      </c>
+      <c r="O12" s="9" t="inlineStr">
+        <is>
+          <t>Unity AIの収益貢献と広告プラットフォームのシェア回復</t>
+        </is>
+      </c>
+      <c r="P12" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
@@ -18792,7 +18860,7 @@
       </c>
       <c r="L13" s="9" t="inlineStr">
         <is>
-          <t>6/2にS&amp;P500入り。Q1'26売上$1.84bn(+59%)・調整後EPS $3.56で予想超え、調整後EBITDAマージン約85%。自社運用型AXON広告プラットフォームを6月に全世界の広告主へ開放(成否を分けるバイナリーイベントと見られる)。目標株価は$646へ引き上げ。</t>
+          <t>自社運用型AI広告基盤『AXON』を6月に全世界の広告主へ開放し、14年続いたクローズド運用に区切り。6/5のEdgewater格上げで株価は約+3%。Q1'26は売上$1.84bn（+59%）・調整後EPS$3.56で予想超え、EBITDAマージン約85%。6/2にS&amp;P500入り。AXON全面開放はバイナリーイベントと目され、広告外領域への拡張も成長余地。目標株価$646。</t>
         </is>
       </c>
       <c r="M13" s="9" t="inlineStr">
@@ -18812,7 +18880,7 @@
       </c>
       <c r="P13" s="9" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-15</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
daily-news + cross-questions update (2026-06-15 22:12)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -2589,7 +2589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3819,6 +3819,80 @@
       <c r="G33" s="5" t="inlineStr">
         <is>
           <t>値上げ余地はライブラリ価値とスイッチングコストに規定される。撤回コストが大きいため、ティア細分化や広告付き廉価プランで弾力性を吸収する設計が共通解になりつつある。</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>ゲームのNPC等に実装される『人格を持つ対話型AI』への規制は、カスタマーサポート・教育・ヘルスケアなど対話AIを実装する他業界にも同じ安全・開示義務を広げるか？</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>中国が対話型（人格型）AIサービスの暫定規則を7/15施行へ、EU AI Actも8/2本格適用</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>（規制）中国国家網信弁公室, EU / 生成AI・AI NPC</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>カスタマーサポート（対話ボット）、教育（AIチューター）、ヘルスケア（メンタル系AI）、金融（対話型アドバイザー）</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>ゲームの娯楽用AIが最も先行して『人格型AI』規制の試金石になり得る。安全・自傷防止・開示の要件は対人影響の大きい業界へ横展開されやすく、最も厳しい基準に合わせた設計が事実上の標準になる。</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>プラットフォームが年複数回の『デモ一斉解禁』イベント（Steam Next Fest）で需要を集中喚起する手法は、SaaS・出版・音楽・動画など無料トライアル設計を持つ他業界の購買導線と何が違い、何を学べるか？</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>Steam Next Fest 2026年6月版が約5,000本の無料デモで開幕（6/15〜22）、直後にサマーセール</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>Valve（Steam） / Steam Next Fest</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>SaaS（無料トライアル/フリーミアム）、出版（試し読み）、音楽・動画配信（無料体験）、EC（サンプリング）</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="G35" s="5" t="inlineStr">
+        <is>
+          <t>『期間限定の集中解禁→直後セール』はトライアルの常時提供と異なり、希少性と話題化でコンバージョンを底上げする。発見性が飽和する市場では、トライアルの質と直後の購買導線の連結が成否を分ける共通課題。</t>
         </is>
       </c>
     </row>
@@ -4714,7 +4788,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L155"/>
+  <dimension ref="A1:L160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14436,6 +14510,311 @@
         </is>
       </c>
       <c r="L155" s="5" t="n"/>
+    </row>
+    <row r="156">
+      <c r="A156" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B156" s="5" t="inlineStr">
+        <is>
+          <t>任天堂、Nintendo Directで『時のオカリナ』リメイクやKINGDOM HEARTS IV、Xenoblade Genesisを発表</t>
+        </is>
+      </c>
+      <c r="C156" s="5" t="inlineStr">
+        <is>
+          <t>https://www.nintendo.com/us/whatsnew/nintendo-direct-unveils-new-games-and-updates-for-nintendo-switch-2-and-nintendo-switch-including-the-legend-of-zelda-ocarina-of-time-kingdom-hearts-iv-xenoblade-genesis-and-more/</t>
+        </is>
+      </c>
+      <c r="D156" s="5" t="inlineStr">
+        <is>
+          <t>Summer Game Fest 2026期間中の6月9日に約50分のNintendo Directを実施。Switch 2の本格展開期に合わせ、自社IPの看板タイトルと大型サードパーティ作品を一気に投入し、ハードの牽引役となるソフトラインアップを提示した。</t>
+        </is>
+      </c>
+      <c r="E156" s="5" t="inlineStr">
+        <is>
+          <t>Directでは『ゼルダの伝説 時のオカリナ』のフルリメイク、スクウェア・エニックスの『KINGDOM HEARTS IV』、モノリスソフトの完全新作『Xenoblade Genesis』など多数を発表。時のオカリナは2026年内、Xenoblade Genesisは2027年予定。Switch/Switch 2双方向けに第一party・third partyを幅広く揃え、年末商戦に向けた布陣を固めた。</t>
+        </is>
+      </c>
+      <c r="F156" s="5" t="inlineStr">
+        <is>
+          <t>『時のオカリナ』フルリメイクを正式発表（2026年内）
+KINGDOM HEARTS IVがSwitch 2にday-and-dateで対応
+Xenoblade完全新作Genesisは2027年予定
+約50分でファースト/サードを横断する大型ラインアップ</t>
+        </is>
+      </c>
+      <c r="G156" s="5" t="inlineStr">
+        <is>
+          <t>看板IPのリメイクと完全新作でSwitch 2の購入動機を継続的に喚起する戦略が鮮明。時のオカリナの完成度とKHIVのマルチ展開が短期の販売を、Xenoblade Genesisが2027年の中期需要を支える構図。サードの初日対応拡大が普及を後押しする。</t>
+        </is>
+      </c>
+      <c r="H156" s="5" t="inlineStr">
+        <is>
+          <t>ファーストパーティIPのリメイク戦略とハード普及</t>
+        </is>
+      </c>
+      <c r="I156" s="5" t="inlineStr">
+        <is>
+          <t>任天堂, スクウェア・エニックス, モノリスソフト</t>
+        </is>
+      </c>
+      <c r="J156" s="5" t="inlineStr">
+        <is>
+          <t>ゼルダの伝説 時のオカリナ, KINGDOM HEARTS IV, Xenoblade Genesis</t>
+        </is>
+      </c>
+      <c r="K156" s="5" t="inlineStr">
+        <is>
+          <t>新作,国内,海外</t>
+        </is>
+      </c>
+      <c r="L156" s="5" t="n"/>
+    </row>
+    <row r="157">
+      <c r="A157" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B157" s="5" t="inlineStr">
+        <is>
+          <t>『ACE COMBAT 8: WINGS OF THEVE』発売日が2026年10月2日に決定、早期購入特典に『ACE ZERO』移植版</t>
+        </is>
+      </c>
+      <c r="C157" s="5" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/969/G096901/20260603010/</t>
+        </is>
+      </c>
+      <c r="D157" s="5" t="inlineStr">
+        <is>
+          <t>バンダイナムコのフライトアクション、エースコンバットシリーズのナンバリング最新作。State of Playで発売日が公開され、シリーズ累計2100万本超の人気IPの完全新作として、PC/PS5/Xbox Series X|Sでマルチ展開する。</t>
+        </is>
+      </c>
+      <c r="E157" s="5" t="inlineStr">
+        <is>
+          <t>『ACE COMBAT 8: WINGS OF THEVE』の発売日が2026年10月2日に決定。前作から10年後を舞台に、新たな空の表現やカスタマイズ、プレイアブル機体が紹介された。早期購入・プレオーダー特典として名作『エースコンバット・ゼロ ザ・ベルカン・ウォー』の移植版が付属する。開発はシリーズを手掛けるPROJECT ACES。</t>
+        </is>
+      </c>
+      <c r="F157" s="5" t="inlineStr">
+        <is>
+          <t>発売日は2026年10月2日（早期アクセス9月29日）に決定
+PC/PS5/Xbox Series X|Sでマルチ展開
+早期購入特典に『ACE ZERO』移植版を付属
+前作から10年後を舞台にした完全新作</t>
+        </is>
+      </c>
+      <c r="G157" s="5" t="inlineStr">
+        <is>
+          <t>10月発売は年末商戦の前哨として国内外のフライトファン需要を取り込む狙い。『ACE ZERO』移植の同梱は新規・復帰層の取り込みに有効。GTA6（11/19）など大型作と発売時期が近接するため、9〜10月の他作とのカニバリ回避が課題になる。</t>
+        </is>
+      </c>
+      <c r="H157" s="5" t="inlineStr">
+        <is>
+          <t>国産AAA IPのマルチ展開と発売時期戦略</t>
+        </is>
+      </c>
+      <c r="I157" s="5" t="inlineStr">
+        <is>
+          <t>バンダイナムコエンターテインメント</t>
+        </is>
+      </c>
+      <c r="J157" s="5" t="inlineStr">
+        <is>
+          <t>ACE COMBAT 8: WINGS OF THEVE</t>
+        </is>
+      </c>
+      <c r="K157" s="5" t="inlineStr">
+        <is>
+          <t>新作,国内</t>
+        </is>
+      </c>
+      <c r="L157" s="5" t="n"/>
+    </row>
+    <row r="158">
+      <c r="A158" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B158" s="5" t="inlineStr">
+        <is>
+          <t>Steam Next Fest（2026年6月）開幕、約5,000本の無料デモが公開（6/15〜22）</t>
+        </is>
+      </c>
+      <c r="C158" s="5" t="inlineStr">
+        <is>
+          <t>https://www.techtimes.com/articles/318387/20260615/steam-next-fest-june-2026-opens-today-nearly-5000-free-demos-are-now-live.htm</t>
+        </is>
+      </c>
+      <c r="D158" s="5" t="inlineStr">
+        <is>
+          <t>Valveが年に複数回開催する体験版集中イベント。発売前タイトルの無料デモをまとめて公開し、ウィッシュリスト獲得とユーザー認知の起点となる。インディーや中小開発にとって最大級の露出機会で、直後のサマーセールへの導線にもなる。</t>
+        </is>
+      </c>
+      <c r="E158" s="5" t="inlineStr">
+        <is>
+          <t>Steam Next Festの2026年6月版が6月15日（PDT）に開幕し、約5,000本の無料PCデモが一斉に公開された。期間は6月22日まで。過去最大級の規模で、ユーザーは多数の未発売作を試遊でき、開発側はフェス期間の遊びやすさとウィッシュリストの伸びを狙う。フェス終了後にはSteamサマーセールが控える。</t>
+        </is>
+      </c>
+      <c r="F158" s="5" t="inlineStr">
+        <is>
+          <t>6/15〜22に約5,000本の無料デモを集中公開
+過去最大級の規模、直後にサマーセールが控える
+ウィッシュリスト獲得とインディー露出の最重要機会
+PC市場の発見性（discoverability）を左右するイベント</t>
+        </is>
+      </c>
+      <c r="G158" s="5" t="inlineStr">
+        <is>
+          <t>デモ公開直後のウィッシュリスト増減が発売後の初動を強く規定する。供給過多のなか上位露出の獲得競争が激化し、デモの完成度とコンバージョン設計の巧拙が中小開発の明暗を分ける。フェス→セール連動の購買喚起モデルが定着する。</t>
+        </is>
+      </c>
+      <c r="H158" s="5" t="inlineStr">
+        <is>
+          <t>プラットフォームの発見性とデモ・マーケティング</t>
+        </is>
+      </c>
+      <c r="I158" s="5" t="inlineStr">
+        <is>
+          <t>Valve（Steam）</t>
+        </is>
+      </c>
+      <c r="J158" s="5" t="inlineStr">
+        <is>
+          <t>Steam Next Fest</t>
+        </is>
+      </c>
+      <c r="K158" s="5" t="inlineStr">
+        <is>
+          <t>インディー,海外,国内</t>
+        </is>
+      </c>
+      <c r="L158" s="5" t="n"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B159" s="5" t="inlineStr">
+        <is>
+          <t>CS2「IEM Cologne Major 2026」プレイオフ進出が確定、6/18〜21に決勝ステージへ（賞金総額125万ドル）</t>
+        </is>
+      </c>
+      <c r="C159" s="5" t="inlineStr">
+        <is>
+          <t>https://esports.gg/news/counter-strike-2/cologne-major-2026-stage-3-results-overview/</t>
+        </is>
+      </c>
+      <c r="D159" s="5" t="inlineStr">
+        <is>
+          <t>Counter-Strike 2の今期最大級の大会の一つで、ドイツ・ケルンで6月2〜21日に開催。賞金総額125万ドル（優勝50万ドル）、4月のVRSランキングを基に32チームが出場。Stage 3を経てプレイオフ進出チームが順次確定している。</t>
+        </is>
+      </c>
+      <c r="E159" s="5" t="inlineStr">
+        <is>
+          <t>IEM Cologne Major 2026はStage 3が6月11〜15日に行われ、9z、Aurora Gaming、Falconsらがプレイオフ進出を決めた。The MongolZやG2は敗退圏を勝ち抜き生き残り、FalconsはNAVIをAnubisの逆転で下した。プレイオフ（決勝ステージ）は6月18〜21日に実施され、優勝の行方が決まる。</t>
+        </is>
+      </c>
+      <c r="F159" s="5" t="inlineStr">
+        <is>
+          <t>賞金総額125万ドル（優勝50万ドル）の大型Major
+Stage 3を経てプレイオフ16チームが確定
+9z・Aurora・Falconsらが進出、NAVIは敗退
+決勝ステージは6/18〜21に開催</t>
+        </is>
+      </c>
+      <c r="G159" s="5" t="inlineStr">
+        <is>
+          <t>プレイオフでの強豪激突は視聴数のピークを生み、CS2競技シーンの勢力図と次期VRSランキングに影響。ホスト国ドイツでの大規模オフライン開催は観客動員とスポンサー露出を最大化し、Major優勝の実績が各チームの市場価値を押し上げる。</t>
+        </is>
+      </c>
+      <c r="H159" s="5" t="inlineStr">
+        <is>
+          <t>eスポーツMajorのVRS制度と興行モデル</t>
+        </is>
+      </c>
+      <c r="I159" s="5" t="inlineStr">
+        <is>
+          <t>ESL/Intel, NAVI, G2 Esports, Falcons, The MongolZ</t>
+        </is>
+      </c>
+      <c r="J159" s="5" t="inlineStr">
+        <is>
+          <t>Counter-Strike 2, IEM Cologne Major 2026</t>
+        </is>
+      </c>
+      <c r="K159" s="5" t="inlineStr">
+        <is>
+          <t>eスポーツ,海外</t>
+        </is>
+      </c>
+      <c r="L159" s="5" t="n"/>
+    </row>
+    <row r="160">
+      <c r="A160" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B160" s="5" t="inlineStr">
+        <is>
+          <t>中国、人格を持つ対話型AIサービスの暫定規則を7/15施行へ／EUのAI Actも8/2に本格適用</t>
+        </is>
+      </c>
+      <c r="C160" s="5" t="inlineStr">
+        <is>
+          <t>https://www.jetro.go.jp/biznews/2021/09/a66cee87da19a2cb.html</t>
+        </is>
+      </c>
+      <c r="D160" s="5" t="inlineStr">
+        <is>
+          <t>生成AIの実装がゲームのNPCや会話システムに広がるなか、各国の規制が具体化している。中国は対話型AIに関する暫定措置を、EUはAI Actの段階適用を進めており、ゲームを含むAI活用領域に表示義務や安全要件が及ぶ可能性が高い。</t>
+        </is>
+      </c>
+      <c r="E160" s="5" t="inlineStr">
+        <is>
+          <t>報道・各種解説によれば、中国は人格を持つように振る舞う対話型AIサービスに関する暫定措置を公表し、2026年7月15日からの施行を予定。安全保障を害する内容や自傷・精神的健康を害する言動などを禁止する。EUではAI Act全体の本格適用が2026年8月2日から始まり、汎用AIや高リスクAIへの規定が段階的に効力を持つ。ゲームのAI NPCや生成要素も射程に入る。</t>
+        </is>
+      </c>
+      <c r="F160" s="5" t="inlineStr">
+        <is>
+          <t>中国が対話型（人格型）AIの暫定規則を7/15施行予定
+EU AI Actは8/2に本格適用、汎用/高リスクAIを規律
+ゲームのAI NPCや生成コンテンツが規制対象になり得る
+安全・健康・開示に関する要件が強化される方向</t>
+        </is>
+      </c>
+      <c r="G160" s="5" t="inlineStr">
+        <is>
+          <t>AI NPCや生成ボイス・シナリオを実装する開発は、地域別の表示・安全要件への対応コストが増す。グローバル配信タイトルは最も厳しい基準に合わせた設計が現実解となり、AIラベリングやモデレーションの標準化が進む。規制適合がパブリッシャーの競争条件に組み込まれる。</t>
+        </is>
+      </c>
+      <c r="H160" s="5" t="inlineStr">
+        <is>
+          <t>ゲームAIへの各国規制とコンプライアンス設計</t>
+        </is>
+      </c>
+      <c r="I160" s="5" t="inlineStr">
+        <is>
+          <t>（規制当局）中国国家網信弁公室, 欧州連合</t>
+        </is>
+      </c>
+      <c r="J160" s="5" t="inlineStr">
+        <is>
+          <t>生成AI, AI NPC</t>
+        </is>
+      </c>
+      <c r="K160" s="5" t="inlineStr">
+        <is>
+          <t>規制,技術,海外</t>
+        </is>
+      </c>
+      <c r="L160" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
daily-news + cross-questions update (2026-06-16 22:11)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -2589,7 +2589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3893,6 +3893,80 @@
       <c r="G35" s="5" t="inlineStr">
         <is>
           <t>『期間限定の集中解禁→直後セール』はトライアルの常時提供と異なり、希少性と話題化でコンバージョンを底上げする。発見性が飽和する市場では、トライアルの質と直後の購買導線の連結が成否を分ける共通課題。</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>親会社が不採算子会社を『閉鎖』ではなく『独立化（MBO・スピンオフ）』で残す動きは、製造業・メディア・製薬のポートフォリオ再編でも同じ形で起きるか？</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>Xbox、Ninja Theory閉鎖の一方でDouble Fine・Compulsionは独立化（買い戻し）を交渉と報道（2026-06-16）</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Microsoft/Xbox Game Studios, Double Fine, Compulsion Games, Ninja Theory</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>製造業（事業カーブアウト）、メディア（番組・レーベルのスピンアウト）、製薬（パイプライン売却）、PE（カーブアウト投資）</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>『閉鎖か独立か』の選別は、IP/ブランド価値が人材と不可分なクリエイティブ事業に特有。のれん減損回避と人材流出防止の綱引きが他業界のカーブアウトと共通する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>ゲームNPCで進む『大規模モデルを軽量モデルに蒸留して端末上で動かす』オンデバイスAIの流れは、スマホ・自動車・家電など他業界のAI実装でも主流になるか？</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>NVIDIA、オンデバイスAI NPC向けACE Game Agent SDKベータとUE5プラグインを公開（Unreal Fest 2026, 2026-06-17）</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>NVIDIA ACE, Unreal Engine 5, PUBG: BATTLEGROUNDS</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>スマホ（端末AI）、自動車（車載音声・ADAS）、家電・ロボット（エッジAI）、コールセンター（低遅延対話）</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>遅延・コスト・データ保護の三点制約はゲーム外でも同じ。クラウドAPI課金型とオンデバイス型の主導権争いが、半導体・OS各社の戦略を左右する。</t>
         </is>
       </c>
     </row>
@@ -4788,7 +4862,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L160"/>
+  <dimension ref="A1:L164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14815,6 +14889,250 @@
         </is>
       </c>
       <c r="L160" s="5" t="n"/>
+    </row>
+    <row r="161">
+      <c r="A161" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B161" s="5" t="inlineStr">
+        <is>
+          <t>Xbox、Ninja Theory閉鎖を通告。Double Fine・Compulsionは独立化（買い戻し）を交渉と報道</t>
+        </is>
+      </c>
+      <c r="C161" s="5" t="inlineStr">
+        <is>
+          <t>https://www.techtimes.com/articles/318465/20260616/xbox-studio-closures-confirmed-ninja-theory-shut-down-nine-days-after-showcase.htm</t>
+        </is>
+      </c>
+      <c r="D161" s="5" t="inlineStr">
+        <is>
+          <t>Microsoftは6月末の会計年度末を前にXbox部門の大規模再編を進めており、6月7日のショーケース直後から複数スタジオの去就が取り沙汰されていた。Senua新作を発表したばかりのNinja Theoryを含む傘下スタジオが対象となり、買収・統合で抱えた制作体制の重さが収益圧力下で見直されている。</t>
+        </is>
+      </c>
+      <c r="E161" s="5" t="inlineStr">
+        <is>
+          <t>6月16日、Ninja Theoryの従業員に閉鎖が通告された一方、Double FineとCompulsion GamesはMicrosoftからの独立（自社買い戻し＝スピンオフ）を交渉中と複数メディアが報道。Ninja Theoryは存続に向け買い手を模索中とされ、他の複数チームも将来を協議しているという。買い戻しが成立しても相当数の人員削減は避けられない見込み。</t>
+        </is>
+      </c>
+      <c r="F161" s="5" t="inlineStr">
+        <is>
+          <t>Ninja Theoryは閉鎖通告、ただし買い手を探し存続を模索
+Double Fine・CompulsionはMBO型の独立化を交渉中
+ショーケースでSenua新作を発表した9日後の閉鎖通告
+他の複数Xboxスタジオも去就を協議との報道
+会計年度末（6/30）前後の大規模再編の一環</t>
+        </is>
+      </c>
+      <c r="G161" s="5" t="inlineStr">
+        <is>
+          <t>7月1日前後にXbox全体の人員削減・スタジオ整理が正式発表される可能性が高い。独立化が成立すればMicrosoftはIPライセンスや出版で関与を残す形が想定され、カーブアウト後の資金調達先（PE・他パブリッシャー）が次の焦点。Senua等の進行中タイトルの権利と継続可否が注目される。</t>
+        </is>
+      </c>
+      <c r="H161" s="5" t="inlineStr">
+        <is>
+          <t>大手による買収スタジオのカーブアウト・MBOの仕組み</t>
+        </is>
+      </c>
+      <c r="I161" s="5" t="inlineStr">
+        <is>
+          <t>Microsoft, Xbox Game Studios, Ninja Theory, Double Fine, Compulsion Games</t>
+        </is>
+      </c>
+      <c r="J161" s="5" t="inlineStr">
+        <is>
+          <t>Senua's Saga: Hellblade, Psychonauts</t>
+        </is>
+      </c>
+      <c r="K161" s="5" t="inlineStr">
+        <is>
+          <t>M&amp;A,業績,海外</t>
+        </is>
+      </c>
+      <c r="L161" s="5" t="n"/>
+    </row>
+    <row r="162">
+      <c r="A162" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B162" s="5" t="inlineStr">
+        <is>
+          <t>『Dead by Daylight』10周年、ジェイソン参戦の新章「Chapter 40」を全機種で解禁</t>
+        </is>
+      </c>
+      <c r="C162" s="5" t="inlineStr">
+        <is>
+          <t>https://www.techtimes.com/articles/318508/20260616/jason-voorhees-arrives-dead-daylight-today-decade-long-wait-ends.htm</t>
+        </is>
+      </c>
+      <c r="D162" s="5" t="inlineStr">
+        <is>
+          <t>非対称対戦ホラー『Dead by Daylight』はライセンスIPコラボでユーザー基盤を拡大してきた看板タイトル。10年来ファンが待ち望んだ『13日の金曜日』ジェイソン・ボーヒーズの版権問題が解け、サービス10周年のタイミングで実装に至った。</t>
+        </is>
+      </c>
+      <c r="E162" s="5" t="inlineStr">
+        <is>
+          <t>Behaviour Interactiveは6月16日（米東部11時）、サービス開始ちょうど10周年に合わせ「Chapter 40: Jason」を全プラットフォームへ実装。ジェイソンをプレイアブルキラーとして追加し、瞬間移動や投擲物を用いた固有能力、3種のスキンを用意。豪州など一部地域は時差で6月17日解禁。記念週として大型施策を展開する。</t>
+        </is>
+      </c>
+      <c r="F162" s="5" t="inlineStr">
+        <is>
+          <t>サービス開始10周年の節目にChapter 40を実装
+版権難航していた『13日の金曜日』ジェイソンが初参戦
+固有能力「Omnipresent Evil」「Improvised Carnage」
+地域時差により豪州等は6/17解禁
+記念週として過去最大級のキャンペーンを実施</t>
+        </is>
+      </c>
+      <c r="G162" s="5" t="inlineStr">
+        <is>
+          <t>看板ライセンスIPの追加で同接・課金が一時的に大きく伸び、10周年商戦の主力となる見込み。映画ホラーIPコラボの成功例として、他社の非対称・ライブサービス型タイトルでも著名IP獲得競争が加速する可能性。版権処理の長期化はライセンス調達リスクとして引き続き課題。</t>
+        </is>
+      </c>
+      <c r="H162" s="5" t="inlineStr">
+        <is>
+          <t>ライブサービスの著名IPコラボと版権調達の収益効果</t>
+        </is>
+      </c>
+      <c r="I162" s="5" t="inlineStr">
+        <is>
+          <t>Behaviour Interactive</t>
+        </is>
+      </c>
+      <c r="J162" s="5" t="inlineStr">
+        <is>
+          <t>Dead by Daylight, Friday the 13th, Jason Voorhees</t>
+        </is>
+      </c>
+      <c r="K162" s="5" t="inlineStr">
+        <is>
+          <t>新作,海外</t>
+        </is>
+      </c>
+      <c r="L162" s="5" t="n"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B163" s="5" t="inlineStr">
+        <is>
+          <t>NVIDIA、オンデバイスAI NPC向け「ACE Game Agent SDK」ベータとUE5プラグインを公開（Unreal Fest 2026）</t>
+        </is>
+      </c>
+      <c r="C163" s="5" t="inlineStr">
+        <is>
+          <t>https://developer.nvidia.com/blog/build-on-device-ai-companions-with-the-nvidia-ace-game-agent-sdk-and-unreal-engine-5-plugins/</t>
+        </is>
+      </c>
+      <c r="D163" s="5" t="inlineStr">
+        <is>
+          <t>生成AIによる動的NPCは各社が競う領域だが、クラウド往復による遅延・コスト・IP保護が実装の壁だった。NVIDIAはローカル（オンデバイス）実行で低遅延の対話NPCを実現する基盤整備を進めており、開発者会議Unreal Fest 2026に合わせ拡充を発表した。</t>
+        </is>
+      </c>
+      <c r="E163" s="5" t="inlineStr">
+        <is>
+          <t>NVIDIAはUnreal Fest 2026に合わせ、軽量C/C++フレームワーク「ACE Game Agent SDK」のベータと、音声認識・小規模言語モデル・音声合成のUE5プラグイン群を公開。RTX上でローカル実行する自律NPCを構築でき、PUBGやTotal War: PHARAOHでの実装例を提示。大規模教師モデルの挙動をLoRAで蒸留し端末上で動かすワークフローを6/17セッションで解説する。</t>
+        </is>
+      </c>
+      <c r="F163" s="5" t="inlineStr">
+        <is>
+          <t>ACE Game Agent SDKをベータ提供、UE5向けプラグインを追加
+ASR（Riva Parakeet）／TTS（Chatterbox）でオンデバイス対話
+クラウド往復を排し低遅延・IP保護を両立
+大規模モデルをLoRAで蒸留しRTX端末でローカル実行
+PUBG・Total War PHARAOH等で実装デモ</t>
+        </is>
+      </c>
+      <c r="G163" s="5" t="inlineStr">
+        <is>
+          <t>オンデバイス推論の前提が整い、対話型NPCの実装が一部AAAから量産フェーズへ進む可能性。Google Cloud等のクラウド型AI基盤と、NVIDIA/オンデバイス型が併存・競合する構図が強まる。RTX等の特定ハード依存と非対応環境での体験差、各国のAI規制対応が普及の鍵となる。</t>
+        </is>
+      </c>
+      <c r="H163" s="5" t="inlineStr">
+        <is>
+          <t>オンデバイスAI推論とモデル蒸留（LoRA）のゲーム実装</t>
+        </is>
+      </c>
+      <c r="I163" s="5" t="inlineStr">
+        <is>
+          <t>NVIDIA, Epic Games, Krafton, Creative Assembly</t>
+        </is>
+      </c>
+      <c r="J163" s="5" t="inlineStr">
+        <is>
+          <t>NVIDIA ACE, Unreal Engine 5, PUBG: BATTLEGROUNDS, Total War: PHARAOH</t>
+        </is>
+      </c>
+      <c r="K163" s="5" t="inlineStr">
+        <is>
+          <t>技術,海外</t>
+        </is>
+      </c>
+      <c r="L163" s="5" t="n"/>
+    </row>
+    <row r="164">
+      <c r="A164" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B164" s="5" t="inlineStr">
+        <is>
+          <t>ゲーム業界のレイオフがXboxを越え波及か。7月にSony・EA系スタジオへとの警告報道</t>
+        </is>
+      </c>
+      <c r="C164" s="5" t="inlineStr">
+        <is>
+          <t>https://www.techtimes.com/articles/318519/20260616/gaming-industry-layoffs-spread-beyond-xbox-july-purge-threatens-sony-ea-studios.htm</t>
+        </is>
+      </c>
+      <c r="D164" s="5" t="inlineStr">
+        <is>
+          <t>2025年の世界ゲーム市場は約1,956億ドルと過去最高ながら、ここ2年で開発者の約3割が職を失う『記録的売上×記録的レイオフ』が続く。MicrosoftのXbox再編を起点に、業界全体で会計年度末（6/30）後の追加削減が警戒されている。</t>
+        </is>
+      </c>
+      <c r="E164" s="5" t="inlineStr">
+        <is>
+          <t>6月16日、ジャーナリストのSylvain Trinel氏らの見解として、7月1日前後にXboxにとどまらずSony・EA・BioWareなどでもスタジオ閉鎖や削減が広がるとの警告が報じられた。Ninja Theoryの閉鎖は確定とされ、Arkane Lyonが次の対象になり得るとの指摘も。ヒットの寡占化と長期運営型タイトルへの集中が背景にあるとされる。</t>
+        </is>
+      </c>
+      <c r="F164" s="5" t="inlineStr">
+        <is>
+          <t>7/1前後に複数大手で人員削減・スタジオ整理の波及を警告
+Ninja Theory閉鎖は確定、Arkane Lyonが次の懸念
+対象にSony・EA・BioWareの名が挙がる（未確定の見通し含む）
+過去2年で開発者の約3割が失職との業界データ
+増収下の削減＝『勝者総取り』型構造の表れ</t>
+        </is>
+      </c>
+      <c r="G164" s="5" t="inlineStr">
+        <is>
+          <t>7月の各社決算・期初に合わせ、追加のリストラ発表が相次ぐ可能性。配信・SaaSと同型の収益集中が進み、中堅スタジオの独立化・身売り・解散が増える見通し。人材は独立スタジオ設立やパブリッシャー横断で再配置され、AI活用による省人化の是非が論点化する。</t>
+        </is>
+      </c>
+      <c r="H164" s="5" t="inlineStr">
+        <is>
+          <t>増収下のレイオフ構造（勝者総取り・長期運営集中）</t>
+        </is>
+      </c>
+      <c r="I164" s="5" t="inlineStr">
+        <is>
+          <t>Microsoft, Sony Interactive Entertainment, Electronic Arts, BioWare, Arkane Lyon</t>
+        </is>
+      </c>
+      <c r="J164" s="5" t="inlineStr"/>
+      <c r="K164" s="5" t="inlineStr">
+        <is>
+          <t>業績,海外</t>
+        </is>
+      </c>
+      <c r="L164" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
weekly-trends + tech update (2026-06-17 03:10)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -1183,7 +1183,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1821,6 +1821,154 @@
       <c r="G17" s="3" t="inlineStr">
         <is>
           <t>https://respawn.outlookindia.com/gaming/gaming-news/record-profits-record-layoffs-inside-gamings-2026-paradox , https://gamerant.com/every-video-game-layoff-and-studio-closure-in-2026-so-far/</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>007 First Light初週270万本——シングルAAA新規IPの『ライブ運営化』</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>IO Interactiveの新作スパイACT『007 First Light』が5/27発売後の初週で270万本超を販売し、6/5にはYear-1の無料アップデート計画（新ストーリーミッション、再訪ロケーション、定例の戦術シミュレーション配信）を公表した。買い切りのシングルプレイヤーAAA新規IPでありながら、発売直後から12カ月のライブサービス型ロードマップを敷くのが特徴。エンディングのティザーが続編期待をSNSで喚起し、Hitman運営で培ったポストローンチ運用をBondへ移植している。Amazon傘下入り後初の大型自社IPとしても注目される。</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>IO Interactive, 007/James Bond, Amazon, Hitman</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>シングルプレイヤーAAAは『売り切り→次回作』の不連続モデルだったが、開発費高騰でリリース間隔が長期化し、その谷を埋めるため『無料DLC＋定例コンテンツ』でエンゲージとウィッシュリスト在庫を維持する運用が広がる。ガチャ課金ではなく『話題の持続＝続編・関連商品の販売装置』としてのライブ運営であり、収益化と運営の目的が分離している点が新しい。</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>映画・ドラマの『フランチャイズ常時接続』と同型。買い切りでも『運営』が前提化すれば制作会社は配信スタジオ化する。IPの常時接続は出版・音楽にも波及する。</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>https://variety.com/2026/gaming/news/007-first-light-updates-bond-sequel-developer-io-amazon-1236768332/ , https://www.thejamesbonddossier.com/news/io-interactive-sets-out-first-year-of-007-first-light-updates.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Witcher 3新拡張『Songs of the Past』——11年選手IPの恒久カタログ化</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>CD Projekt Redが2015年発売『The Witcher 3: Wild Hunt』向けの新拡張『Songs of the Past』を発表した。The Witcher 3開発に携わった業界ベテランで構成されるFool's Theoryと共同開発する。発売から11年を経た旧作に新規の大型DLCを追加する異例の動きで、次世代版対応やMOD公式化に続くカタログ延命策の一環。新作（Witcher 4/Polaris）開発中に旧作の話題と販売を再点火し、シリーズ全体の生涯価値を最大化する狙いがうかがえる。外部ベテランスタジオへ委託し内製リソースを新作に集中させる体制も特徴。</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>CD Projekt Red, Fool's Theory, The Witcher</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>AAAのIPは『新作で売る』フロー型から、旧作を恒久商品として運用するストック型へ移行しつつある。リマスター・次世代対応・MOD公式化・新DLCはいずれもカタログの賞味期限を延ばす施策で、Steam等の長期セール環境と相性が良い。外注ベテランスタジオ活用は固定費を抑えつつIP資産を回す『製作委員会／映画的』分業の定着を示す。</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>旧IPの恒久収益化はディズニーのライブラリ運用と同型。コンテンツ企業の価値はフローよりストックで測られる時代へ向かう。</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>https://www.goonhammer.com/games-industry-news-roundup-june-9th-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>ゲーム・関連メディアの労組化加速——Dark Horse労組を経営陣が承認</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>米コミック大手Dark Horse Comicsの経営陣が、5/27にスタッフの過半数賛成で結成されたDark Horse Workers Unionを自主承認した。ゲーム関連メディアでは相次ぐレイオフと不安定な経済環境を背景に労働組合化が継続的な大テーマとなっており、開発・出版・関連メディアにわたり組織化の波が広がっている。記録的売上の一方で人員削減が続く業界構造への労働者側の対抗運動として、声優のSAG-AFTRAに続く動きと位置づけられる。</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Dark Horse Comics, Dark Horse Workers Union, SAG-AFTRA</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>ゲーム産業は増収下のレイオフ＝『勝者総取り＋効率化』局面にあり、プロジェクト単位の雇用・外注化（ギグ化）が進む。これに対し声優・QA・開発・出版の各層で組合化が進行。AI導入による職務代替の懸念が組織化の触媒となり、団体交渉の論点が賃金から『AI利用と同意・クレジット』へ拡張している。</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>労使の焦点がAI時代の『成果物の出自と同意』へ移るのは映像・音楽・出版共通。クリエイティブ全産業の労働契約の雛形になり得る。</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>https://www.goonhammer.com/games-industry-news-roundup-june-9th-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Dead by Daylight×ジェイソン——ライセンスIPで長寿ライブゲーム再点火</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Behaviour Interactiveの非対称ホラー『Dead by Daylight』に、6/16『13日の金曜日』のジェイソン・ボーヒーズがプレイアブルキラーとして参戦し、Steam同接が7万人超へ急回復した。長年運営のライブサービスが、ホラー映画の象徴的ライセンスIPコラボを起点に休眠プレイヤーを呼び戻す典型例。長く権利が宙に浮いていたジェイソンの実装は、権利調整を乗り越えたこと自体が話題化し、配信クリップを通じてバイラルに拡散した。</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Behaviour Interactive, Dead by Daylight, Friday the 13th/Jason Voorhees</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>長寿ライブサービスは新規獲得より『離脱者の再活性化』が収益の鍵で、月3で約6割が離脱するchurn構造（GDC/Ampere調査）を定例の大型コラボで打ち返す設計が標準化している。ホラー・格闘などキャラ依存ジャンルでは、外部ライセンスIPが『新キャラ＝新規SKU』として機能し、権利処理コストを超える集客・課金リフトを生む。</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>ライセンスの『重ね合わせ』でアテンションを買う構造は、音楽コラボやアパレルのIPコラボと同型。版権の流動化が再点火の燃料になる。</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>https://www.thegamer.com/steam-games-must-play-best-player-count-right-now/</t>
         </is>
       </c>
     </row>
@@ -19842,7 +19990,7 @@
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B4" s="9" t="inlineStr">
@@ -19857,32 +20005,32 @@
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>Game Pass Ultimate $22.99/PC $13.99へ値下げ。CEOは登録・継続率の改善を明言。CoD新作のday-one提供を撤回し約1年遅れに。</t>
+          <t>Game Pass Ultimate値下げ後の再編が継続。6月末でGame Passから8タイトルが離脱予定。</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
         <is>
-          <t>Discord Nitro Rewardsへ50本超のStarter同梱。PC/Premium統合や広告階層を2027年視野で検討。目標5,000万契約。</t>
+          <t>Ubisoft+ ClassicsがPC Game Pass提供から外れる一方、Xbox Game Pass UltimateはEA Play/Ubisoft+ Classicsを内包。UbisoftはR6 SiegeでXbox Game Pass公式パートナー契約を更新し6月から特典付与。Ubisoft+はPremium/Classicsの2階層へ。</t>
         </is>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
-          <t>Microsoft, Xbox, Activision, Discord</t>
+          <t>Microsoft/Xbox, Ubisoft, Sony(PS Plus), EA</t>
         </is>
       </c>
       <c r="G4" s="9" t="inlineStr">
         <is>
-          <t>値下げ＋バンドル＋広告階層へ。目玉IPはday-one非提供で本体販売とのカニバリ回避。</t>
+          <t>バンドルの再編成（どのカタログがどのサブスクに入るか）が競争軸に。目玉IPの出し入れとクロスバンドルが常態化。</t>
         </is>
       </c>
       <c r="H4" s="9" t="inlineStr">
         <is>
-          <t>ARPU最大化から契約者数最大化へ軸足。動画/音楽サブスクの定石に合流。</t>
+          <t>サブスクの価値は『独占タイトル』から『どれだけ他社カタログを束ねるか』のアグリゲーション競争へ。</t>
         </is>
       </c>
       <c r="I4" s="9" t="inlineStr">
         <is>
-          <t>https://respawn.outlookindia.com/gaming/gaming-news/xbox-ceo-says-game-pass-price-cuts-improve-sign-ups-and-retention</t>
+          <t>https://gg.deals/subscription-news/game-pass-is-losing-eight-games-at-the-end-of-june-2026 , https://www.thurrott.com/games/296198/</t>
         </is>
       </c>
       <c r="J4" s="9" t="inlineStr"/>
@@ -20098,7 +20246,7 @@
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
@@ -20113,32 +20261,32 @@
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>無料インディー『TBH: Task Bar Hero』が13.3万同接でトレンド首位、AAAの007 First Lightを圧倒。AI開示済みは7,300本超。</t>
+          <t>6/8-14だけで300本超が新規リリースし供給過多が加速。無料『TBH: Task Bar Hero』が13万同接で首位を継続。</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>広告/パブリッシャー無しの無料タイトルがバイラルのみで首位。Solarpunk等コージー作も高フォロワー、Gothic 1 Remakeが6月最多ウィッシュリスト。</t>
+          <t>Steam Next Fest出展約8,700本のうち約1,704本（約20%）が生成AI利用を開示。DbD×ジェイソン参戦で同接7万超などコラボ起点のスパイクも顕著。</t>
         </is>
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t>Valve, インディー各社</t>
+          <t>Valve, Behaviour Interactive, インディー各社</t>
         </is>
       </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
-          <t>同接ピークと配信クリップ起点のディスカバリーが主流化。無料→DLC/続編回収の設計が増加。</t>
+          <t>供給爆発で『発見』の希少性が増し、同接ピーク×配信映え×AI開示の有無が選別シグナル化。キュレーション/イベント依存が強まる。</t>
         </is>
       </c>
       <c r="H11" s="9" t="inlineStr">
         <is>
-          <t>PCの発見はウィッシュリストより『瞬間最大同接×配信映え』へ重心移動。</t>
+          <t>ディスカバリーの摩擦が最大のボトルネック。AI製の量産タイトル流入が『質の選別』を一段と重要にしている。</t>
         </is>
       </c>
       <c r="I11" s="9" t="inlineStr">
         <is>
-          <t>https://screenrant.com/steam-june-2026-trending-free-game/</t>
+          <t>https://www.gamegrin.com/news/weekly-top-trending-games-on-steam-8th14th-of-june-2026/ , https://www.engadget.com/2195840/around-a-fifth-of-steam-next-fest-demos-have-a-generative-ai-disclosure/</t>
         </is>
       </c>
       <c r="J11" s="9" t="inlineStr"/>

</xml_diff>

<commit_message>
daily-news + cross-questions + events update (2026-06-19 00:38)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -2747,7 +2747,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4125,6 +4125,80 @@
       <c r="G37" s="5" t="inlineStr">
         <is>
           <t>遅延・コスト・データ保護の三点制約はゲーム外でも同じ。クラウドAPI課金型とオンデバイス型の主導権争いが、半導体・OS各社の戦略を左右する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>戦略株主（Tencent）が独立スタジオへの短期追加出資を見送り資金枯渇に追い込まれる構図は、SaaS・バイオベンチャー・ディープテックなど外部資本依存業界でも同様に起きるか？</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>Don't NodがTencentの追加出資見送りで2026年11月にも資金枯渇の恐れ（2026-06）</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Don't Nod, Tencent / Life is Strange</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>SaaS, バイオベンチャー, ディープテック, スタートアップ全般（VC/CVC資本政策）</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t>「長期株主には留まるが短期増資はしない」というCVCの姿勢は各業界の出資先で同様のリスク。キャッシュランウェイと資本政策の脆弱性は業界横断のテーマ。</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>生成AIの氾濫に対しユーザーが「人間の手仕事」を選好する“オーセンティシティ（真正性）市場”の形成は、食品・アパレル・工芸・メディアなど他業界でも起きるか？</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>ポケットペアが生成AI不使用を再表明、「真正性市場」へのシフトを予測（2026-06）</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Pocketpair / Palworld</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>食品（クラフト/手作り）, アパレル, 工芸, メディア・出版, 音楽</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="G39" s="5" t="inlineStr">
+        <is>
+          <t>「ハンドメイド/オーガニック」プレミアムの構図がデジタル制作物にも波及する可能性。AI開示・ラベリングと表裏一体で“人手”が付加価値ラベルになるか。</t>
         </is>
       </c>
     </row>
@@ -5654,7 +5728,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L164"/>
+  <dimension ref="A1:L171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15925,6 +15999,433 @@
         </is>
       </c>
       <c r="L164" s="5" t="n"/>
+    </row>
+    <row r="165">
+      <c r="A165" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B165" s="5" t="inlineStr">
+        <is>
+          <t>「ライフ イズ ストレンジ」開発Don't Nod、Tencentが短期追加出資を見送り資金繰り難に</t>
+        </is>
+      </c>
+      <c r="C165" s="5" t="inlineStr">
+        <is>
+          <t>https://www.gamedeveloper.com/business/don-t-nod-pursuing-several-levers-to-secure-financial-future-after-tencent-decides-against-short-term-investment</t>
+        </is>
+      </c>
+      <c r="D165" s="5" t="inlineStr">
+        <is>
+          <t>仏Don't Nodは2024年以降のレイオフ後も赤字が続く。約42%を保有する筆頭株主Tencentが新規プロジェクトへの追加出資を見送ると通告。監査人は6月に「特別警告報告」を出し、2026年4月時点の現金は880万ユーロで11月にも資金枯渇の恐れと指摘した。</t>
+        </is>
+      </c>
+      <c r="E165" s="5" t="inlineStr">
+        <is>
+          <t>Don't Nodは「キャッシュランウェイ延長と財務基盤強化に向け複数のレバーを検討中」と表明。Tencentは長期株主に留まるものの短期の増資・新作出資を拒否し、独立スタジオは身売り・資産売却・新たな出資者探しを迫られている。</t>
+        </is>
+      </c>
+      <c r="F165" s="5" t="inlineStr">
+        <is>
+          <t>・Tencentは筆頭株主(約42%)だが短期の追加出資・新作出資を見送り
+・監査人が6月に「特別警告報告」、2026年4月時点の現金は880万ユーロ
+・このままなら2026年11月に資金枯渇の恐れ
+・身売り・資産売却を含む複数の財務施策を並行検討</t>
+        </is>
+      </c>
+      <c r="G165" s="5" t="inlineStr">
+        <is>
+          <t>11月の資金枯渇期限が迫る中、M&amp;Aや新たな出資者確保、IP売却、追加リストラのいずれかが現実味を帯びる。プラットフォーマーや他パブリッシャーによる救済買収、または開発規模の大幅縮小に向かう可能性が高い。</t>
+        </is>
+      </c>
+      <c r="H165" s="5" t="inlineStr">
+        <is>
+          <t>戦略株主の出資判断と独立スタジオの資本政策・キャッシュランウェイ</t>
+        </is>
+      </c>
+      <c r="I165" s="5" t="inlineStr">
+        <is>
+          <t>Don't Nod, Tencent</t>
+        </is>
+      </c>
+      <c r="J165" s="5" t="inlineStr">
+        <is>
+          <t>Life is Strange, Vampyr</t>
+        </is>
+      </c>
+      <c r="K165" s="5" t="inlineStr">
+        <is>
+          <t>M&amp;A,業績,海外</t>
+        </is>
+      </c>
+      <c r="L165" s="5" t="inlineStr"/>
+    </row>
+    <row r="166">
+      <c r="A166" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B166" s="5" t="inlineStr">
+        <is>
+          <t>SHIFT UP、三上真司氏の新スタジオUNBOUNDと提携。新作を自社パブリッシングで展開へ</t>
+        </is>
+      </c>
+      <c r="C166" s="5" t="inlineStr">
+        <is>
+          <t>https://www.gamerbraves.com/shift-up-confirms-new-stellar-blade-details-and-project-spirits-reveal-coming-in-2026/</t>
+        </is>
+      </c>
+      <c r="D166" s="5" t="inlineStr">
+        <is>
+          <t>韓国SHIFT UP（『勝利の女神：NIKKE』『ステラーブレイド』）は自社パブリッシング体制を強化中。『バイオハザード』生みの親・三上真司氏が率いる新スタジオUNBOUNDと、両社の創作・戦略方針の一致から提携を結んだ。</t>
+        </is>
+      </c>
+      <c r="E166" s="5" t="inlineStr">
+        <is>
+          <t>SHIFT UPはUNBOUNDの将来作を自社の第一者パブリッシング戦略の下で展開すると確認。あわせて『ステラーブレイド』新情報や新規IP「Project Spirits」公開を2026年中に予定していると明かした。</t>
+        </is>
+      </c>
+      <c r="F166" s="5" t="inlineStr">
+        <is>
+          <t>・三上真司氏のUNBOUNDと提携、SHIFT UPが自社パブリッシング
+・SHIFT UPの第一者パブ戦略の拡大策
+・『ステラーブレイド』新情報を2026年中に予定
+・新規IP「Project Spirits」も披露予定</t>
+        </is>
+      </c>
+      <c r="G166" s="5" t="inlineStr">
+        <is>
+          <t>開発スタジオが有力クリエイターを取り込みつつ自社流通網を拡張する垂直統合が加速。SHIFT UPはNIKKEの収益を背景にIPポートフォリオと開発体制を多角化し、コンソール・グローバル市場での存在感を一段と高めると見られる。</t>
+        </is>
+      </c>
+      <c r="H166" s="5" t="inlineStr">
+        <is>
+          <t>開発スタジオの自社パブリッシング化と有力クリエイター囲い込み戦略</t>
+        </is>
+      </c>
+      <c r="I166" s="5" t="inlineStr">
+        <is>
+          <t>SHIFT UP, UNBOUND</t>
+        </is>
+      </c>
+      <c r="J166" s="5" t="inlineStr">
+        <is>
+          <t>ステラーブレイド, 勝利の女神：NIKKE, Project Spirits</t>
+        </is>
+      </c>
+      <c r="K166" s="5" t="inlineStr">
+        <is>
+          <t>M&amp;A,新作,海外</t>
+        </is>
+      </c>
+      <c r="L166" s="5" t="inlineStr"/>
+    </row>
+    <row r="167">
+      <c r="A167" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B167" s="5" t="inlineStr">
+        <is>
+          <t>6/18の新作ラッシュ：『R-Type Tactics I・II Cosmos』『Hell Let Loose: Vietnam』など発売</t>
+        </is>
+      </c>
+      <c r="C167" s="5" t="inlineStr">
+        <is>
+          <t>https://www.dlcompare.com/gaming-news/this-week-s-video-game-releases-june-2026-week-25</t>
+        </is>
+      </c>
+      <c r="D167" s="5" t="inlineStr">
+        <is>
+          <t>夏商戦前のリリースが集中する第25週、6月18日に複数ジャンルの新作が一斉に発売された。シリーズ復活やスピンオフ、大規模マルチプレイの新展開などが並んだ。</t>
+        </is>
+      </c>
+      <c r="E167" s="5" t="inlineStr">
+        <is>
+          <t>6/18には、名作STGをターン制戦術に落とし込んだ『R-Type Tactics I・II Cosmos』、大規模戦闘FPS『Hell Let Loose』のベトナム戦版『Hell Let Loose: Vietnam』、ファンタジー冒険『The Adventures of Elliot』などが発売された。</t>
+        </is>
+      </c>
+      <c r="F167" s="5" t="inlineStr">
+        <is>
+          <t>・『R-Type Tactics I・II Cosmos』：名作STGのターン制戦術リバイバル
+・『Hell Let Loose: Vietnam』：WW2からベトナム戦へ舞台拡張
+・『The Adventures of Elliot: The Millennium Tales』も同日発売
+・夏商戦前の第25週にジャンル横断で新作集中</t>
+        </is>
+      </c>
+      <c r="G167" s="5" t="inlineStr">
+        <is>
+          <t>6/25開始のSteamサマーセール直前は、セール値引き前に定価で買う層を取り込む発売タイミングとして重視される。旧作IPの再解釈・スピンオフは低リスクで需要を喚起でき、今後もシリーズ資産の多角展開が続くとみられる。</t>
+        </is>
+      </c>
+      <c r="H167" s="5" t="inlineStr">
+        <is>
+          <t>季節セール直前のリリース戦略と旧作IPの再解釈・スピンオフ手法</t>
+        </is>
+      </c>
+      <c r="I167" s="5" t="inlineStr">
+        <is>
+          <t>Granzella, Team17</t>
+        </is>
+      </c>
+      <c r="J167" s="5" t="inlineStr">
+        <is>
+          <t>R-Type, Hell Let Loose</t>
+        </is>
+      </c>
+      <c r="K167" s="5" t="inlineStr">
+        <is>
+          <t>新作,海外</t>
+        </is>
+      </c>
+      <c r="L167" s="5" t="inlineStr"/>
+    </row>
+    <row r="168">
+      <c r="A168" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B168" s="5" t="inlineStr">
+        <is>
+          <t>ソニー、PS6の発売時期・価格は「現時点で未定」。メモリ価格高騰が次世代機の鍵に</t>
+        </is>
+      </c>
+      <c r="C168" s="5" t="inlineStr">
+        <is>
+          <t>https://news.yahoo.co.jp/articles/f3c0a4108e4c62d832c56623737e45976b40b0df</t>
+        </is>
+      </c>
+      <c r="D168" s="5" t="inlineStr">
+        <is>
+          <t>ソニーは2026年5月の決算説明会で次世代機PS6の時期・価格を未定とした。AIデータセンター需要でDRAM/NANDなどメモリ価格が高騰しており、ハードの部品コスト（BOM）上昇が次世代機の投入時期・価格設計の制約になっている。</t>
+        </is>
+      </c>
+      <c r="E168" s="5" t="inlineStr">
+        <is>
+          <t>最新リークではPS6は2027年登場の可能性が高まり、次世代Xboxも同時期とされる。ソニーはメモリ高騰への対応を価格・時期決定の鍵と位置づけ、慎重姿勢を崩していない。</t>
+        </is>
+      </c>
+      <c r="F168" s="5" t="inlineStr">
+        <is>
+          <t>・PS6の発売時期・価格は現時点で未定とソニーが明言
+・最有力リークは2027年登場、次世代Xboxも同時期
+・AIサーバ需要によるメモリ高騰がBOMを押し上げ
+・ハード価格設定の制約要因として顕在化</t>
+        </is>
+      </c>
+      <c r="G168" s="5" t="inlineStr">
+        <is>
+          <t>メモリ調達コストが据え置けない水準まで上がれば、次世代機は高価格スタートか投入後の値上げが避けられない。Switch 2の値上げと同様、ハードの逆ザヤ回避志向が強まり、サブスク・クラウド比重を高める戦略と並走するとみられる。</t>
+        </is>
+      </c>
+      <c r="H168" s="5" t="inlineStr">
+        <is>
+          <t>メモリ価格高騰がコンソールBOM・価格戦略に与える影響</t>
+        </is>
+      </c>
+      <c r="I168" s="5" t="inlineStr">
+        <is>
+          <t>ソニーグループ, Microsoft</t>
+        </is>
+      </c>
+      <c r="J168" s="5" t="inlineStr">
+        <is>
+          <t>PlayStation 6, Xbox</t>
+        </is>
+      </c>
+      <c r="K168" s="5" t="inlineStr">
+        <is>
+          <t>業績,技術,海外</t>
+        </is>
+      </c>
+      <c r="L168" s="5" t="inlineStr"/>
+    </row>
+    <row r="169">
+      <c r="A169" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B169" s="5" t="inlineStr">
+        <is>
+          <t>「Esports World Cup: Level Up」シーズン2、6/26にPrime Videoで全5話一挙配信</t>
+        </is>
+      </c>
+      <c r="C169" s="5" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/esports-world-cup-level-up-returns-to-prime-video-june-26-with-season-two-302804305.html</t>
+        </is>
+      </c>
+      <c r="D169" s="5" t="inlineStr">
+        <is>
+          <t>7/6パリ開幕のEsports World Cup 2026（賞金総額7,500万ドル）に向け、運営財団は競技の裏側を描くドキュメンタリーをOTTで展開。エミー賞受賞のR.J.カトラー監督が選手・クラブ・家族を追う。</t>
+        </is>
+      </c>
+      <c r="E169" s="5" t="inlineStr">
+        <is>
+          <t>ドキュメンタリー「Level Up」シーズン2が6月26日、全5話を一挙にPrime Video独占配信。2025年大会の選手の重圧と野心を描き、7月のEWC本戦への注目を高めるプロモーションとして機能する。</t>
+        </is>
+      </c>
+      <c r="F169" s="5" t="inlineStr">
+        <is>
+          <t>・6/26にPrime Videoで全5話一挙独占配信
+・R.J.カトラー監督（エミー賞）が制作
+・7/6パリ開幕のEWC 2026本戦への前哨プロモーション
+・eスポーツのストーリーテリングをOTTで拡張</t>
+        </is>
+      </c>
+      <c r="G169" s="5" t="inlineStr">
+        <is>
+          <t>大型eスポーツが競技配信に加え「ドキュメンタリー×OTT」で非ファン層に裾野を広げる手法が定着しつつある。スポーツのドキュメンタリー商法（F1等）に倣い、選手の物語性を軸にスポンサー・視聴者の獲得競争が激化するとみられる。</t>
+        </is>
+      </c>
+      <c r="H169" s="5" t="inlineStr">
+        <is>
+          <t>eスポーツのOTTドキュメンタリー展開と非ファン層への拡張戦略</t>
+        </is>
+      </c>
+      <c r="I169" s="5" t="inlineStr">
+        <is>
+          <t>Esports World Cup Foundation, Amazon</t>
+        </is>
+      </c>
+      <c r="J169" s="5" t="inlineStr">
+        <is>
+          <t>Esports World Cup</t>
+        </is>
+      </c>
+      <c r="K169" s="5" t="inlineStr">
+        <is>
+          <t>eスポーツ,海外</t>
+        </is>
+      </c>
+      <c r="L169" s="5" t="inlineStr"/>
+    </row>
+    <row r="170">
+      <c r="A170" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B170" s="5" t="inlineStr">
+        <is>
+          <t>任天堂、Switch/Switch 2本体更新22.5.0を配信。eショップ刷新と読み上げ多言語対応</t>
+        </is>
+      </c>
+      <c r="C170" s="5" t="inlineStr">
+        <is>
+          <t>https://game.watch.impress.co.jp/docs/news/2117416.html</t>
+        </is>
+      </c>
+      <c r="D170" s="5" t="inlineStr">
+        <is>
+          <t>任天堂は6月、Switch 2およびSwitch向けのシステムバージョン22.5.0を配信。ニンテンドーeショップのデザイン刷新や動作安定性向上に加え、Switch 2ではアクセシビリティの音声読み上げにオランダ語・ロシア語を追加した。</t>
+        </is>
+      </c>
+      <c r="E170" s="5" t="inlineStr">
+        <is>
+          <t>本体更新22.5.0でeショップのUIが刷新され、テーマカラー「ベーシックブラック」がeショップにも反映。読み上げ機能の対応言語拡充など、購入体験とアクセシビリティの改善が図られた。</t>
+        </is>
+      </c>
+      <c r="F170" s="5" t="inlineStr">
+        <is>
+          <t>・システムVer22.5.0をSwitch 2/Switch両機種に配信
+・ニンテンドーeショップのデザイン刷新・安定性向上
+・Switch 2の音声読み上げにオランダ語・ロシア語追加
+・テーマカラーがeショップにも反映</t>
+        </is>
+      </c>
+      <c r="G170" s="5" t="inlineStr">
+        <is>
+          <t>値上げ後の購買体験を磨くことで客単価維持と離反防止を狙う。OS・ストアのUX改善とアクセシビリティ拡充は、ハード普及期の継続的なエンゲージメント施策として今後も小刻みに続くとみられる。</t>
+        </is>
+      </c>
+      <c r="H170" s="5" t="inlineStr">
+        <is>
+          <t>プラットフォームのストアUX・アクセシビリティ改善とエンゲージメント維持</t>
+        </is>
+      </c>
+      <c r="I170" s="5" t="inlineStr">
+        <is>
+          <t>任天堂</t>
+        </is>
+      </c>
+      <c r="J170" s="5" t="inlineStr">
+        <is>
+          <t>Nintendo Switch 2, ニンテンドーeショップ</t>
+        </is>
+      </c>
+      <c r="K170" s="5" t="inlineStr">
+        <is>
+          <t>技術,国内</t>
+        </is>
+      </c>
+      <c r="L170" s="5" t="inlineStr"/>
+    </row>
+    <row r="171">
+      <c r="A171" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B171" s="5" t="inlineStr">
+        <is>
+          <t>『パルワールド』ポケットペア、生成AIを使わない方針を再表明「ゲーマーが望んでいない」</t>
+        </is>
+      </c>
+      <c r="C171" s="5" t="inlineStr">
+        <is>
+          <t>https://www.gamesradar.com/games/survival/gamers-dont-want-it-palworld-lead-says-pocketpair-doesnt-touch-ai-because-players-hate-it-and-artists-like-doing-stuff-themselves/</t>
+        </is>
+      </c>
+      <c r="D171" s="5" t="inlineStr">
+        <is>
+          <t>業界で生成AI活用が広がる中、Summer Game Fest 2026では『クレイジータクシー』新作などがAI利用を巡り釈明に追われた。こうした逆風下、ポケットペアのパブリッシング/広報責任者が改めて自社の不使用方針を語った。</t>
+        </is>
+      </c>
+      <c r="E171" s="5" t="inlineStr">
+        <is>
+          <t>ポケットペアは生成AIを使わず今後も採用予定はないと明言。「ゲーマーが望んでいない」とし、低品質なAI製ゲームが氾濫する一方で、人間の手仕事を評価する「オーセンティシティ（真正性）市場」へ需要がシフトすると予測した。</t>
+        </is>
+      </c>
+      <c r="F171" s="5" t="inlineStr">
+        <is>
+          <t>・ポケットペアは生成AIを使用せず、今後も不使用方針
+・「ゲーマーが望んでいない」と理由を説明
+・自社パブリッシングでもAI製ゲームは扱わない方針
+・低品質AIゲーム氾濫と「真正性市場」形成を予測</t>
+        </is>
+      </c>
+      <c r="G171" s="5" t="inlineStr">
+        <is>
+          <t>生成AI採用の是非がブランド価値の分岐点になりつつある。AI開示・ラベリング規制の強化と相まって、「人手による制作」を訴求する差別化と、効率重視のAI活用の二極化が進むと見られる。消費者の選好が市場を分けるか注目。</t>
+        </is>
+      </c>
+      <c r="H171" s="5" t="inlineStr">
+        <is>
+          <t>生成AIに対するユーザー選好の二極化と「真正性」によるブランド差別化</t>
+        </is>
+      </c>
+      <c r="I171" s="5" t="inlineStr">
+        <is>
+          <t>Pocketpair</t>
+        </is>
+      </c>
+      <c r="J171" s="5" t="inlineStr">
+        <is>
+          <t>Palworld</t>
+        </is>
+      </c>
+      <c r="K171" s="5" t="inlineStr">
+        <is>
+          <t>技術,規制,国内</t>
+        </is>
+      </c>
+      <c r="L171" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
weekly-releases + indie + rankings update (2026-06-19 11:36)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -4213,7 +4213,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:J43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5080,6 +5080,717 @@
       <c r="J24" t="inlineStr">
         <is>
           <t>週間が無いため月間で代替</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-06-08〜06-14</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>パワフルプロ野球2026-2027</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Switch</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>100,976</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週間販売数 https://www.famitsu.com/article/202606/78731</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>パワプロ最新作が約10万本で首位スタート</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-06-08〜06-14</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>2</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>トモダチコレクション わくわく生活</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Switch</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>37,888</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週間販売数 https://www.famitsu.com/article/202606/78731</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>パワプロ最新作が約10万本で首位スタート</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-06-08〜06-14</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>3</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>eFootball Kick-Off!</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Switch 2</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>8,143</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週間販売数 https://www.famitsu.com/article/202606/78731</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>パワプロ最新作が約10万本で首位スタート</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-06-08〜06-14</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>4</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>ぽこ あ ポケモン</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Switch 2</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>7,781</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週間販売数 https://www.famitsu.com/article/202606/78731</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>パワプロ最新作が約10万本で首位スタート</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-06-08〜06-14</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>5</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>アストロボット</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>PS5</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>6,533</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週間販売数 https://www.famitsu.com/article/202606/78731</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>パワプロ最新作が約10万本で首位スタート</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-06-08〜06-14</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>6</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>マリオカート ワールド</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Switch 2</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>5,042</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週間販売数 https://www.famitsu.com/article/202606/78731</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>パワプロ最新作が約10万本で首位スタート</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-06-08〜06-14</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>7</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>ヨッシーとフカシギの図鑑</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Switch 2</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>4,249</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週間販売数 https://www.famitsu.com/article/202606/78731</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>パワプロ最新作が約10万本で首位スタート</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-06-08〜06-14</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>8</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>ファイナルファンタジーVII リバース</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Switch 2</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>4,169</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週間販売数 https://www.famitsu.com/article/202606/78731</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>パワプロ最新作が約10万本で首位スタート</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-06-08〜06-14</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>9</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>イナズマイレブン 英雄たちのヴィクトリーロード</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Switch 2</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>3,544</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週間販売数 https://www.famitsu.com/article/202606/78731</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>パワプロ最新作が約10万本で首位スタート</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-06-08〜06-14</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>10</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Minecraft（マインクラフト）</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Switch</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>3,379</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週間販売数 https://www.famitsu.com/article/202606/78731</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>パワプロ最新作が約10万本で首位スタート</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-06-10〜06-16</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>MECCHA CHAMELEON（めっちゃカメレオン）</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>VGChartz Steam週間トップセラー Week25 https://www.vgchartz.com/article/468225/steam-weekly-week-25-2026/</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>個人開発の日本産インディーが初登場1位</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-06-10〜06-16</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>2</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Forza Horizon 6（フォルツァ ホライゾン 6）</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>VGChartz Steam週間トップセラー Week25 https://www.vgchartz.com/article/468225/steam-weekly-week-25-2026/</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>前週首位から2位へ</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-06-10〜06-16</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>3</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Steam Deck</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>ハードウェア</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>VGChartz Steam週間トップセラー Week25 https://www.vgchartz.com/article/468225/steam-weekly-week-25-2026/</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>ハード（携帯PC）</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-06-10〜06-16</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>4</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Path of Exile 2（パス・オブ・エグザイル2）</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>VGChartz Steam週間トップセラー Week25 https://www.vgchartz.com/article/468225/steam-weekly-week-25-2026/</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-06-10〜06-16</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>5</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>EA Sports FC 26</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>VGChartz Steam週間トップセラー Week25 https://www.vgchartz.com/article/468225/steam-weekly-week-25-2026/</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>トップ10再浮上（5〜7位の順は概算）</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-06-10〜06-16</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>6</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Destiny 2: Renegades（デスティニー2：レネゲイズ）</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>VGChartz Steam週間トップセラー Week25 https://www.vgchartz.com/article/468225/steam-weekly-week-25-2026/</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>トップ10再浮上（5〜7位の順は概算）</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-06-10〜06-16</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>7</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Final Fantasy VII Remake Intergrade（FF7 リメイク インターグレード）</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>VGChartz Steam週間トップセラー Week25 https://www.vgchartz.com/article/468225/steam-weekly-week-25-2026/</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>トップ10再浮上（5〜7位の順は概算）</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-06-10〜06-16</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>8</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>007 First Light（007 ファースト・ライト）</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>VGChartz Steam週間トップセラー Week25 https://www.vgchartz.com/article/468225/steam-weekly-week-25-2026/</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>8位へ後退</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-06-10〜06-16</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>9</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Gothic 1 Remake（ゴシック1 リメイク）</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>VGChartz Steam週間トップセラー Week25 https://www.vgchartz.com/article/468225/steam-weekly-week-25-2026/</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>9位へ後退</t>
         </is>
       </c>
     </row>
@@ -16438,7 +17149,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M21"/>
+  <dimension ref="A1:M24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16891,12 +17602,18 @@
           <t>HD-2D RPG</t>
         </is>
       </c>
+      <c r="G9" t="n">
+        <v>82</v>
+      </c>
+      <c r="H9" t="n">
+        <v>82</v>
+      </c>
       <c r="K9" t="n">
         <v>4</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>HD-2Dエンジン採用の新IP。Square Enix外部パブとして注目。中世ファンタジー×リアルタイム戦闘。</t>
+          <t>【6/18発売・実績反映】海外メタスコア平均82/100、好評89%。『聖剣伝説』を原点に4時代を行き来する探索＆魔石ビルドが好評。レベル概念なしでも成長実感のあるアクションRPGとして高評価。一部ペース/反復に指摘。</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -17442,6 +18159,141 @@
       <c r="M21" t="inlineStr">
         <is>
           <t>https://www.gamespot.com/articles/2026-upcoming-games-release-schedule/1100-6534941/</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>EA SPORTS UFC 6</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>EA Vancouver</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Electronic Arts</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>PS5/Xbox Series X|S</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>スポーツ（総合格闘技）</t>
+        </is>
+      </c>
+      <c r="K22" t="n">
+        <v>3</v>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>6/19発売の総合格闘技シム最新作。フィジカルや個性表現を強化。発売直後のためスコア未確定。早期アクセスも実施済み。</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>https://www.ea.com/en/games/ufc/ufc-6</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>DEAD OR ALIVE 6 Last Round（デッド オア アライブ6 ラストラウンド）</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Team NINJA</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>コーエーテクモゲームス</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>PS5</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>3D対戦格闘</t>
+        </is>
+      </c>
+      <c r="K23" t="n">
+        <v>3</v>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>既存DLCキャラ収録＋新コス・新フォトモード追加の完全版。同日に基本無料版も配信。来週リリース予定。</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>https://www.gamecity.ne.jp/game/27417.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>プロ野球スピリッツ2026</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>コナミ</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>コナミデジタルエンタテインメント</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>PS5</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>スポーツ（野球）</t>
+        </is>
+      </c>
+      <c r="K24" t="n">
+        <v>4</v>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>プロスピ家庭用シリーズ最新作。7/16発売予定の来月大型タイトル。4/16から予約受付開始。</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>https://www.konami.com/games/corporate/ja/news/topics/20260416/</t>
         </is>
       </c>
     </row>
@@ -21523,7 +22375,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -21866,6 +22718,53 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>MECCHA CHAMELEON（めっちゃカメレオン）</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>lemorion_1224（日本・個人開発）</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2026-06-09 配信中</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>マルチプレイ・かくれんぼタクティカル</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>白いカメレオンに色を塗って背景へ擬態し、鬼から隠れる対戦かくれんぼ。発売2日で50万本、その後100万本突破。Steam週間トップセラー世界1位に浮上。$5前後の低価格×配信映えで爆発的バイラルヒット。</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Steamレビュー『非常に好評』80%（約8,300件）。Steam週間トップセラー1位（週末6/16）。</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>個人開発の日本産インディーが世界1位。低価格×シンプル×配信映えの『TBH』に続くアテンション経済型ヒットの好例。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
daily-news + cross-questions + events update (2026-06-19 22:12)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -2747,7 +2747,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4199,6 +4199,43 @@
       <c r="G39" s="5" t="inlineStr">
         <is>
           <t>「ハンドメイド/オーガニック」プレミアムの構図がデジタル制作物にも波及する可能性。AI開示・ラベリングと表裏一体で“人手”が付加価値ラベルになるか。</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B40" s="15" t="inlineStr">
+        <is>
+          <t>AIノーコードで誰でもゲームを制作できる基盤の台頭は、Web制作・動画編集・アプリ開発など他の『制作系』業界の参入障壁を同様に消すか？</t>
+        </is>
+      </c>
+      <c r="C40" s="15" t="inlineStr">
+        <is>
+          <t>GameByteがAIノーコードのモバイルゲーム作成基盤に$1Mプレシード調達（2026-06）</t>
+        </is>
+      </c>
+      <c r="D40" s="15" t="inlineStr">
+        <is>
+          <t>GameByte</t>
+        </is>
+      </c>
+      <c r="E40" s="15" t="inlineStr">
+        <is>
+          <t>Web制作, 動画編集, アプリ開発（ローコード）, DTP/デザイン, 教育</t>
+        </is>
+      </c>
+      <c r="F40" s="15" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="G40" s="15" t="inlineStr">
+        <is>
+          <t>『専門スキル不要化』はクリエイティブ職の価値再定義を各制作業界で同時に迫る可能性がある</t>
         </is>
       </c>
     </row>
@@ -5617,7 +5654,6 @@
           <t>VGChartz Steam週間トップセラー Week25 https://www.vgchartz.com/article/468225/steam-weekly-week-25-2026/</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -5805,7 +5841,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6428,6 +6464,110 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="C13" s="15" t="inlineStr">
+        <is>
+          <t>Steam Next Fest（6月版）</t>
+        </is>
+      </c>
+      <c r="D13" s="15" t="inlineStr">
+        <is>
+          <t>セール</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>オンライン(Steam)</t>
+        </is>
+      </c>
+      <c r="F13" s="15" t="inlineStr">
+        <is>
+          <t>体験版一斉解禁</t>
+        </is>
+      </c>
+      <c r="G13" s="15" t="inlineStr">
+        <is>
+          <t>発売前タイトルの体験版を一斉公開する大型需要喚起イベント。約4,931本のデモが配信。6/25開幕のサマーセール直前。</t>
+        </is>
+      </c>
+      <c r="H13" s="15" t="inlineStr">
+        <is>
+          <t>https://www.techtimes.com/articles/318387/20260615/steam-next-fest-june-2026-opens-today-nearly-5000-free-demos-are-now-live.htm</t>
+        </is>
+      </c>
+      <c r="I13" s="15" t="inlineStr">
+        <is>
+          <t>開催中</t>
+        </is>
+      </c>
+      <c r="J13" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B14" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="C14" s="15" t="inlineStr">
+        <is>
+          <t>VALORANT Masters London 2026</t>
+        </is>
+      </c>
+      <c r="D14" s="15" t="inlineStr">
+        <is>
+          <t>eスポーツ</t>
+        </is>
+      </c>
+      <c r="E14" s="15" t="inlineStr">
+        <is>
+          <t>英ロンドン</t>
+        </is>
+      </c>
+      <c r="F14" s="15" t="inlineStr">
+        <is>
+          <t>オフライン大会</t>
+        </is>
+      </c>
+      <c r="G14" s="15" t="inlineStr">
+        <is>
+          <t>VCT 2026 Stage 2の国際大会。プレイオフ佳境でPaper Rexが優勝候補筆頭。グランドファイナルは6/21。</t>
+        </is>
+      </c>
+      <c r="H14" s="15" t="inlineStr">
+        <is>
+          <t>https://www.vlr.gg/event/2765/valorant-masters-london-2026</t>
+        </is>
+      </c>
+      <c r="I14" s="15" t="inlineStr">
+        <is>
+          <t>開催中</t>
+        </is>
+      </c>
+      <c r="J14" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6439,7 +6579,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L171"/>
+  <dimension ref="A1:L177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17137,6 +17277,364 @@
         </is>
       </c>
       <c r="L171" s="5" t="inlineStr"/>
+    </row>
+    <row r="172">
+      <c r="A172" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B172" s="15" t="inlineStr">
+        <is>
+          <t>任天堂『スターフォックス』Switch 2専用で6月25日発売、無料体験版を配信開始</t>
+        </is>
+      </c>
+      <c r="C172" s="15" t="inlineStr">
+        <is>
+          <t>https://www.nintendo.com/my/news/article/XLNwUoKaa2CveWIwQjCvi</t>
+        </is>
+      </c>
+      <c r="D172" s="15" t="inlineStr">
+        <is>
+          <t>スターフォックスはシリーズとして2016年以来の本格新作。Switch 2のマウス操作対応Joy-Con 2やGameChat機能を活かす任天堂の専用タイトル戦略の一環で、ハード普及の後押しが期待される。</t>
+        </is>
+      </c>
+      <c r="E172" s="15" t="inlineStr">
+        <is>
+          <t>任天堂はSwitch 2専用『スターフォックス』を2026年6月25日に発売すると告知し、eShopで無料体験版とプレオーダーを開始した。スターフォックス64を下敷きにキャラクター刷新・フルボイス・オーケストラ音源を採用し、オンラインマルチも搭載する。</t>
+        </is>
+      </c>
+      <c r="F172" s="15" t="inlineStr">
+        <is>
+          <t>・Switch 2専用、2026年6月25日発売
+・無料体験版とプレオーダーをeShopで開始
+・Joy-Con 2のマウス操作・GameChatに対応
+・シリーズ約10年ぶりの本格新作</t>
+        </is>
+      </c>
+      <c r="G172" s="15" t="inlineStr">
+        <is>
+          <t>GTA6不在の年末前にSwitch 2の弱含む販売を下支えするファーストパーティ大作の一つ。体験版の先行配信は購入転換率を高める狙いで、夏商戦のハード牽引役になるか注目される。</t>
+        </is>
+      </c>
+      <c r="H172" s="15" t="inlineStr">
+        <is>
+          <t>ファーストパーティ専用タイトルとハード普及の相関</t>
+        </is>
+      </c>
+      <c r="I172" s="15" t="inlineStr">
+        <is>
+          <t>任天堂</t>
+        </is>
+      </c>
+      <c r="J172" s="15" t="inlineStr">
+        <is>
+          <t>スターフォックス, Nintendo Switch 2</t>
+        </is>
+      </c>
+      <c r="K172" s="15" t="inlineStr">
+        <is>
+          <t>新作,国内</t>
+        </is>
+      </c>
+      <c r="L172" s="15" t="n"/>
+    </row>
+    <row r="173">
+      <c r="A173" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B173" s="15" t="inlineStr">
+        <is>
+          <t>受託大手Virtuos、蘭スタジオAbstractionをMBOで分離。開発受託の再編が加速</t>
+        </is>
+      </c>
+      <c r="C173" s="15" t="inlineStr">
+        <is>
+          <t>https://gam3s.gg/news/key-studio-acquisitions-and-funding-news/</t>
+        </is>
+      </c>
+      <c r="D173" s="15" t="inlineStr">
+        <is>
+          <t>ゲーム開発受託・外注業界は大手の整理が続く。AbstractionはDune: AwakeningやBaldur's Gate 3に貢献した移植・支援スタジオ。受託モデルの収益圧力下で事業ポートフォリオ見直しが進む。</t>
+        </is>
+      </c>
+      <c r="E173" s="15" t="inlineStr">
+        <is>
+          <t>シンガポール拠点のVirtuosは、オランダのAbstractionをマネジメント・バイアウト(MBO)で分離すると発表。同時にWeb3系のBLIFEとPortalの統合など、ゲーム周辺の再編・統合案件が相次いでいる。</t>
+        </is>
+      </c>
+      <c r="F173" s="15" t="inlineStr">
+        <is>
+          <t>・VirtuosがAbstractionをMBOで切り離し
+・AbstractionはBG3・Dune等の移植/支援に貢献
+・受託開発業界で事業整理が継続
+・BLIFE×Portal統合などWeb3再編も並行</t>
+        </is>
+      </c>
+      <c r="G173" s="15" t="inlineStr">
+        <is>
+          <t>大手パブリッシャーの開発費抑制で受託需要が不安定化する中、独立化・専門特化で生き残りを図る動きが続く見込み。中小スタジオの再編・M&amp;Aは2026年後半も活発化しそう。</t>
+        </is>
+      </c>
+      <c r="H173" s="15" t="inlineStr">
+        <is>
+          <t>ゲーム受託開発業界の再編とMBOによる独立化</t>
+        </is>
+      </c>
+      <c r="I173" s="15" t="inlineStr">
+        <is>
+          <t>Virtuos, Abstraction, BLIFE, Portal</t>
+        </is>
+      </c>
+      <c r="J173" s="15" t="inlineStr">
+        <is>
+          <t>Baldur's Gate 3, Dune: Awakening</t>
+        </is>
+      </c>
+      <c r="K173" s="15" t="inlineStr">
+        <is>
+          <t>M&amp;A,海外</t>
+        </is>
+      </c>
+      <c r="L173" s="15" t="n"/>
+    </row>
+    <row r="174">
+      <c r="A174" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B174" s="15" t="inlineStr">
+        <is>
+          <t>AIノーコードのゲーム作成基盤GameByteが$1Mプレシード調達。SF系新興も$2M確保</t>
+        </is>
+      </c>
+      <c r="C174" s="15" t="inlineStr">
+        <is>
+          <t>https://games.gg/news/key-studio-acquisitions-and-funding-news/</t>
+        </is>
+      </c>
+      <c r="D174" s="15" t="inlineStr">
+        <is>
+          <t>生成AIの普及でゲーム制作の参入障壁が下がりつつある。早期段階のスタジオやツール企業への投資が活発で、AI×ノーコードを軸にした制作の民主化が投資テーマ化している。</t>
+        </is>
+      </c>
+      <c r="E174" s="15" t="inlineStr">
+        <is>
+          <t>英GameByteはAI搭載ノーコードのモバイルゲーム作成プラットフォーム開発に向け、評価額$10Mで$1Mのプレシードを調達。米Imaginary Hazard Studiosもsci-fiローグライク開発で$2Mを確保した。</t>
+        </is>
+      </c>
+      <c r="F174" s="15" t="inlineStr">
+        <is>
+          <t>・GameByteが$1Mプレシード（評価額$10M）
+・AI搭載ノーコードのゲーム作成基盤を開発
+・Imaginary Hazard Studiosが$2M調達
+・早期段階×AIへの投資テーマが継続</t>
+        </is>
+      </c>
+      <c r="G174" s="15" t="inlineStr">
+        <is>
+          <t>AI×ノーコードは個人・小規模開発の生産性を押し上げ、UGC的なゲーム量産につながる可能性。一方で品質・著作権・差別化の課題も顕在化し、ツール企業間の競争が激化しそう。</t>
+        </is>
+      </c>
+      <c r="H174" s="15" t="inlineStr">
+        <is>
+          <t>AI×ノーコードによるゲーム制作の民主化</t>
+        </is>
+      </c>
+      <c r="I174" s="15" t="inlineStr">
+        <is>
+          <t>GameByte, Imaginary Hazard Studios</t>
+        </is>
+      </c>
+      <c r="J174" s="15" t="inlineStr"/>
+      <c r="K174" s="15" t="inlineStr">
+        <is>
+          <t>技術,海外</t>
+        </is>
+      </c>
+      <c r="L174" s="15" t="n"/>
+    </row>
+    <row r="175">
+      <c r="A175" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B175" s="15" t="inlineStr">
+        <is>
+          <t>VALORANT Masters London 2026、Paper RexがVitality撃破で上位決勝へ。6/21決勝</t>
+        </is>
+      </c>
+      <c r="C175" s="15" t="inlineStr">
+        <is>
+          <t>https://egamersworld.com/valorant/news/35526/valorant-masters-london-2026-paper-rex-defeat-team-ZCVhcgmcG</t>
+        </is>
+      </c>
+      <c r="D175" s="15" t="inlineStr">
+        <is>
+          <t>VCT 2026 Stage 2の国際大会Masters Londonがプレイオフ佳境。世界トップチームが集い、7月開幕のEWCを控えた各地域の勢力図を占う重要な前哨戦となっている。</t>
+        </is>
+      </c>
+      <c r="E175" s="15" t="inlineStr">
+        <is>
+          <t>Masters London 2026のプレイオフで、Paper RexがTeam Vitalityを2-1で下しアッパーブラケット決勝へ進出。優勝候補の筆頭と目される。グランドファイナルは6月21日に予定されている。</t>
+        </is>
+      </c>
+      <c r="F175" s="15" t="inlineStr">
+        <is>
+          <t>・Paper RexがVitalityを2-1で撃破
+・アッパーブラケット決勝へ進出、優勝候補筆頭
+・グランドファイナルは2026-06-21
+・7月開幕のEWCに向けた前哨戦</t>
+        </is>
+      </c>
+      <c r="G175" s="15" t="inlineStr">
+        <is>
+          <t>優勝チームはEWCのValorant部門で有利な評価を得る見込み。アジア勢Paper Rexの優勝なら地域勢力図の変化を印象づけ、視聴・スポンサー面でも波及が期待される。</t>
+        </is>
+      </c>
+      <c r="H175" s="15" t="inlineStr">
+        <is>
+          <t>VCT国際大会と地域勢力図・EWCへの連動</t>
+        </is>
+      </c>
+      <c r="I175" s="15" t="inlineStr">
+        <is>
+          <t>Riot Games, Paper Rex, Team Vitality</t>
+        </is>
+      </c>
+      <c r="J175" s="15" t="inlineStr">
+        <is>
+          <t>VALORANT</t>
+        </is>
+      </c>
+      <c r="K175" s="15" t="inlineStr">
+        <is>
+          <t>eスポーツ,海外</t>
+        </is>
+      </c>
+      <c r="L175" s="15" t="n"/>
+    </row>
+    <row r="176">
+      <c r="A176" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B176" s="15" t="inlineStr">
+        <is>
+          <t>サウジNEOM Gaming Accelerator、過去最大サイクル始動。買収に加え育成へ投資拡大</t>
+        </is>
+      </c>
+      <c r="C176" s="15" t="inlineStr">
+        <is>
+          <t>https://www.neom.com/en-us/newsroom/NEOM-Gaming-Accelerator-Welcomes-Largest-Ever-Cycle-of-Startup-Studios</t>
+        </is>
+      </c>
+      <c r="D176" s="15" t="inlineStr">
+        <is>
+          <t>サウジはソブリンファンド主導の大型買収に加え、スタジオ育成・誘致でもゲーム産業のハブ化を狙う。NEOMの加速器は中東のゲーム開発エコシステム構築の中核施策と位置づけられる。</t>
+        </is>
+      </c>
+      <c r="E176" s="15" t="inlineStr">
+        <is>
+          <t>NEOM Gaming Acceleratorが過去最大規模のスタートアップスタジオ受け入れサイクルを開始したと発表。資金・メンタリング・現地拠点を提供し、サウジを起点としたグローバル展開を支援する。</t>
+        </is>
+      </c>
+      <c r="F176" s="15" t="inlineStr">
+        <is>
+          <t>・過去最大規模の受け入れサイクル
+・スタジオ育成・誘致でハブ化を推進
+・買収だけでなく育成にも投資領域を拡大
+・中東発エコシステム構築を加速</t>
+        </is>
+      </c>
+      <c r="G176" s="15" t="inlineStr">
+        <is>
+          <t>サウジの『買収+育成』両輪戦略は中東のゲーム開発拠点化を後押し。欧米・アジアからの人材・スタジオ誘致が進めば、開発拠点の地理的分散が一段と進む可能性がある。</t>
+        </is>
+      </c>
+      <c r="H176" s="15" t="inlineStr">
+        <is>
+          <t>ソブリン資本によるゲーム産業ハブ化戦略</t>
+        </is>
+      </c>
+      <c r="I176" s="15" t="inlineStr">
+        <is>
+          <t>NEOM, Savvy Games Group</t>
+        </is>
+      </c>
+      <c r="J176" s="15" t="inlineStr"/>
+      <c r="K176" s="15" t="inlineStr">
+        <is>
+          <t>海外,M&amp;A</t>
+        </is>
+      </c>
+      <c r="L176" s="15" t="n"/>
+    </row>
+    <row r="177">
+      <c r="A177" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B177" s="15" t="inlineStr">
+        <is>
+          <t>Netflix×Warner Bros.（ゲーム部門含む$82.7B買収）、Discovery分離が26年Q3完了見込みで進行</t>
+        </is>
+      </c>
+      <c r="C177" s="15" t="inlineStr">
+        <is>
+          <t>https://www.gamedeveloper.com/business/yes-netflix-is-acquiring-warner-bros-games</t>
+        </is>
+      </c>
+      <c r="D177" s="15" t="inlineStr">
+        <is>
+          <t>NetflixはParamount Skydance・Comcastとの争奪戦を制し、WB（映画・TV・ゲーム部門・HBO Max）を総額$82.7Bで買収する合意に至った。ゲーム部門も対象に含まれる。</t>
+        </is>
+      </c>
+      <c r="E177" s="15" t="inlineStr">
+        <is>
+          <t>買収はWBDのネットワーク部門Discovery Globalの分離完了が前提で、その完了時期が2026年Q3に見込まれている。承認後、有力IPと併せてWBのゲーム事業がNetflix傘下に入る見通し。</t>
+        </is>
+      </c>
+      <c r="F177" s="15" t="inlineStr">
+        <is>
+          <t>・総額$82.7B、ゲーム部門・HBO Maxを含む
+・Discovery Global分離完了が前提（26年Q3見込み）
+・規制当局・株主の承認が残る
+・有力IPのゲーム化加速の可能性</t>
+        </is>
+      </c>
+      <c r="G177" s="15" t="inlineStr">
+        <is>
+          <t>動画配信×ゲームの統合で、強力IPを横断展開する戦略が加速する見込み。NetflixのゲームサービスにWBタイトル/IPが流入すれば、配信発のゲーム事業が一段と存在感を増す。</t>
+        </is>
+      </c>
+      <c r="H177" s="15" t="inlineStr">
+        <is>
+          <t>動画配信×ゲームのIP統合とクロス展開</t>
+        </is>
+      </c>
+      <c r="I177" s="15" t="inlineStr">
+        <is>
+          <t>Netflix, Warner Bros. Games, HBO Max</t>
+        </is>
+      </c>
+      <c r="J177" s="15" t="inlineStr">
+        <is>
+          <t>Harry Potter, Game of Thrones</t>
+        </is>
+      </c>
+      <c r="K177" s="15" t="inlineStr">
+        <is>
+          <t>M&amp;A,海外</t>
+        </is>
+      </c>
+      <c r="L177" s="15" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
daily-news + cross-questions + events update (2026-06-20 22:12)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -2747,7 +2747,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4236,6 +4236,80 @@
       <c r="G40" s="15" t="inlineStr">
         <is>
           <t>『専門スキル不要化』はクリエイティブ職の価値再定義を各制作業界で同時に迫る可能性がある</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B41" s="15" t="inlineStr">
+        <is>
+          <t>ゲーム部門の利益を親会社がAI領域へ再配分し祖業を縮小する『資本シフト』は、通信・メディア・小売など他業界のコングロマリットでも同様に起きるか？</t>
+        </is>
+      </c>
+      <c r="C41" s="15" t="inlineStr">
+        <is>
+          <t>Microsoft、6/30会計年度末後にXbox大規模リストラ報道</t>
+        </is>
+      </c>
+      <c r="D41" s="15" t="inlineStr">
+        <is>
+          <t>Microsoft/Xbox</t>
+        </is>
+      </c>
+      <c r="E41" s="15" t="inlineStr">
+        <is>
+          <t>通信(キャリアの非中核事業整理)/メディア(配信投資シフト)/小売(EC・物流へのAI集中)</t>
+        </is>
+      </c>
+      <c r="F41" s="15" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="G41" s="15" t="inlineStr">
+        <is>
+          <t>『稼ぎ頭でも親会社の戦略優先順位が下がれば縮小対象になる』構図。事業の良し悪しより資本配分の論理が支配する点が示唆的。</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B42" s="15" t="inlineStr">
+        <is>
+          <t>ゲーム由来のリアルタイム3D・シミュレーション・AI技術が防衛/ロボティクス産業へ転用される流れは、自動車・製造・建設など他産業でも加速するか？</t>
+        </is>
+      </c>
+      <c r="C42" s="15" t="inlineStr">
+        <is>
+          <t>Krafton×Hanwha Aerospace 約10億ドルのAI・ロボティクス協業</t>
+        </is>
+      </c>
+      <c r="D42" s="15" t="inlineStr">
+        <is>
+          <t>Krafton/Hanwha Aerospace</t>
+        </is>
+      </c>
+      <c r="E42" s="15" t="inlineStr">
+        <is>
+          <t>自動車(自動運転シミュ)/製造(デジタルツイン)/建設(BIM・遠隔操作)/防衛</t>
+        </is>
+      </c>
+      <c r="F42" s="15" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="G42" s="15" t="inlineStr">
+        <is>
+          <t>ゲームエンジンは『現実の安価な実験場』。エンタメ技術が産業の基盤技術へ昇格する“両用化”の典型例として追う価値あり。</t>
         </is>
       </c>
     </row>
@@ -6579,7 +6653,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L177"/>
+  <dimension ref="A1:L183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17635,6 +17709,371 @@
         </is>
       </c>
       <c r="L177" s="15" t="n"/>
+    </row>
+    <row r="178">
+      <c r="A178" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B178" s="15" t="inlineStr">
+        <is>
+          <t>VALORANT Masters London 2026、本日グランドファイナル開催。Paper Rexがアジア勢初制覇に挑む</t>
+        </is>
+      </c>
+      <c r="C178" s="15" t="inlineStr">
+        <is>
+          <t>https://esports.gg/news/valorant/masters-london-2026/</t>
+        </is>
+      </c>
+      <c r="D178" s="15" t="inlineStr">
+        <is>
+          <t>VCT2026 Stage2の世界大会「Masters London」が6/12より開催。賞金総額100万ドル・優勝35万ドルとVCTポイント8を懸け世界トップ12チームが激突した。アッパーブラケット決勝ではPaper RexがEDward Gamingを2-1で退け、グランドファイナルへ進出していた。</t>
+        </is>
+      </c>
+      <c r="E178" s="15" t="inlineStr">
+        <is>
+          <t>6/21の決勝はPaper Rexとローワーを勝ち上がったチームが対戦。Paper RexはAPAC(アジア太平洋)勢として国際大会制覇を狙う。VALORANTのeスポーツは地域対抗色が強まり、視聴数とスポンサー誘致の両面で各リーグの実力差が可視化される節目の一戦となる。</t>
+        </is>
+      </c>
+      <c r="F178" s="15" t="inlineStr">
+        <is>
+          <t>・賞金総額100万ドル／優勝35万ドル＋VCTポイント8
+・Paper Rex(APAC)が決勝進出、地域の威信を懸ける
+・結果が秋のChampionsシード争いに直結</t>
+        </is>
+      </c>
+      <c r="G178" s="15" t="inlineStr">
+        <is>
+          <t>優勝チームは秋のVALORANT Champions 2026へ弾みをつける。Riotは地域フランチャイズの収益化を進めており、好成績地域はスポンサー流入と放映権価値が上がる一方、低調な地域との格差拡大が続く見込み。</t>
+        </is>
+      </c>
+      <c r="H178" s="15" t="inlineStr">
+        <is>
+          <t>VCTのフランチャイズ制と地域リーグの収益構造</t>
+        </is>
+      </c>
+      <c r="I178" s="15" t="inlineStr">
+        <is>
+          <t>Riot Games, Paper Rex, EDward Gaming</t>
+        </is>
+      </c>
+      <c r="J178" s="15" t="inlineStr">
+        <is>
+          <t>VALORANT</t>
+        </is>
+      </c>
+      <c r="K178" s="15" t="inlineStr">
+        <is>
+          <t>eスポーツ,海外</t>
+        </is>
+      </c>
+      <c r="L178" s="15" t="inlineStr"/>
+    </row>
+    <row r="179">
+      <c r="A179" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B179" s="15" t="inlineStr">
+        <is>
+          <t>Microsoft、6/30会計年度末後にXbox部門で大規模リストラへ。Asha Sharma新体制で初の再編</t>
+        </is>
+      </c>
+      <c r="C179" s="15" t="inlineStr">
+        <is>
+          <t>https://kotaku.com/xbox-reportedly-major-layoffs-next-month-2000705023</t>
+        </is>
+      </c>
+      <c r="D179" s="15" t="inlineStr">
+        <is>
+          <t>MicrosoftはActivision Blizzard買収(約690億ドル)以降ゲーム部門に巨額投資を続けたが、Game Pass収益やハード販売は伸び悩み、親会社はAIへ資本を集中させている。複数報道が、6/30の会計年度末を境に追加の人員削減とマーケ等の予算縮小を伝えている。</t>
+        </is>
+      </c>
+      <c r="E179" s="15" t="inlineStr">
+        <is>
+          <t>今年就任したゲーム責任者Asha Sharmaの下で初の大規模組織再編となる見込み。削減規模は未確定だが、コンテンツ・サブスク事業の採算改善が狙い。Game Pass価格改定やCoDのDay-one配信見直しなど、一連の収益化施策の延長線上にある動きとみられる。</t>
+        </is>
+      </c>
+      <c r="F179" s="15" t="inlineStr">
+        <is>
+          <t>・実施は6/30会計年度末後、7月の見込み
+・Asha Sharma体制下で初の大規模再編
+・背景にAB買収の採算圧力とAIへの資本シフト
+・Game Pass価格改定・CoDのDay-one見直しと連動</t>
+        </is>
+      </c>
+      <c r="G179" s="15" t="inlineStr">
+        <is>
+          <t>ハード一本足からマルチプラットフォーム/サブスク中心への構造転換が加速。第一者スタジオの統廃合やプロジェクト中止が続く可能性が高く、Xboxは『プラットフォーマー』から『パブリッシャー』色を強めると見られる。</t>
+        </is>
+      </c>
+      <c r="H179" s="15" t="inlineStr">
+        <is>
+          <t>プラットフォーマーのサブスク採算とAIへの資本再配分</t>
+        </is>
+      </c>
+      <c r="I179" s="15" t="inlineStr">
+        <is>
+          <t>Microsoft, Xbox, Activision Blizzard</t>
+        </is>
+      </c>
+      <c r="J179" s="15" t="inlineStr">
+        <is>
+          <t>Game Pass, Call of Duty</t>
+        </is>
+      </c>
+      <c r="K179" s="15" t="inlineStr">
+        <is>
+          <t>業績,技術,海外</t>
+        </is>
+      </c>
+      <c r="L179" s="15" t="inlineStr"/>
+    </row>
+    <row r="180">
+      <c r="A180" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B180" s="15" t="inlineStr">
+        <is>
+          <t>EA、約550億ドルでの非公開化がクロージング目前。サウジPIF・Silver Lake・Affinityが出資</t>
+        </is>
+      </c>
+      <c r="C180" s="15" t="inlineStr">
+        <is>
+          <t>https://www.esports.net/news/industry/what-does-ea-acquisition-mean-for-its-esports-titles-apex-legends-fc-26-madden-more/</t>
+        </is>
+      </c>
+      <c r="D180" s="15" t="inlineStr">
+        <is>
+          <t>Electronic Artsは2025年、Silver Lake・サウジPIF・Jared Kushner氏のAffinity Partnersが組む陣営による約550億ドルのLBO(レバレッジド・バイアウト)で非公開化に合意。ゲーム業界史上最大級のテイクプライベート案件で、6月のクロージングが見込まれていた。</t>
+        </is>
+      </c>
+      <c r="E180" s="15" t="inlineStr">
+        <is>
+          <t>非公開化により短期的な株主圧力からは解放される一方、巨額の買収負債の返済負担が経営の自由度を縛る。Apex Legends、EA SPORTS FC、Maddenなど主力ライブサービス/eスポーツIPの運営方針への影響が注目される。</t>
+        </is>
+      </c>
+      <c r="F180" s="15" t="inlineStr">
+        <is>
+          <t>・買収総額は約550億ドル、ゲーム史上最大級のLBO
+・出資はSilver Lake／サウジPIF／Affinity Partners
+・主力はFC・Madden・Apexのライブサービス/eスポーツ
+・PIF関与でサウジのゲーム覇権戦略がさらに前進</t>
+        </is>
+      </c>
+      <c r="G180" s="15" t="inlineStr">
+        <is>
+          <t>負債返済のため不採算事業の整理やコスト削減が加速する一方、ライブサービス/スポーツIPへ集中投資する公算。PIFの影響力拡大で、サウジ主導のeスポーツ・大会との連携が強まる可能性がある。</t>
+        </is>
+      </c>
+      <c r="H180" s="15" t="inlineStr">
+        <is>
+          <t>大型LBOとレバレッジが事業運営に与える制約</t>
+        </is>
+      </c>
+      <c r="I180" s="15" t="inlineStr">
+        <is>
+          <t>Electronic Arts, Silver Lake, サウジPIF, Affinity Partners</t>
+        </is>
+      </c>
+      <c r="J180" s="15" t="inlineStr">
+        <is>
+          <t>EA SPORTS FC, Madden, Apex Legends</t>
+        </is>
+      </c>
+      <c r="K180" s="15" t="inlineStr">
+        <is>
+          <t>M&amp;A,業績,海外</t>
+        </is>
+      </c>
+      <c r="L180" s="15" t="inlineStr"/>
+    </row>
+    <row r="181">
+      <c r="A181" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B181" s="15" t="inlineStr">
+        <is>
+          <t>Netflix×Warner Bros.、契約を全額現金取引に修正。WB Gamesも統合対象に</t>
+        </is>
+      </c>
+      <c r="C181" s="15" t="inlineStr">
+        <is>
+          <t>https://ir.netflix.net/investor-news-and-events/financial-releases/press-release-details/2026/Netflix-and-Warner-Bros--Discovery-Amend-Agreement-to-All-Cash-Transaction/default.aspx</t>
+        </is>
+      </c>
+      <c r="D181" s="15" t="inlineStr">
+        <is>
+          <t>Netflixは2025年末にWarner Bros.(企業価値約827億ドル)の買収で合意。Discovery Globalの分離(Q3 2026完了見込み)を前提とし、Paramount Skydance陣営との競合も取り沙汰されてきた。両社は取引条件を全額現金取引に修正したと発表した。</t>
+        </is>
+      </c>
+      <c r="E181" s="15" t="inlineStr">
+        <is>
+          <t>修正で買収成立の確度を高める狙い。WB Gamesも取引に含まれるが、Netflix側は『ゲーム事業に価値を割り当てていない』と発言しており、IPの扱いは不透明。配信大手によるスタジオ統合がゲーム業界の地図を塗り替える可能性がある。</t>
+        </is>
+      </c>
+      <c r="F181" s="15" t="inlineStr">
+        <is>
+          <t>・取引を全額現金(オールキャッシュ)に変更
+・企業価値は約827億ドル、Discovery分離が前提
+・WB Games(Mortal Kombat等)も対象
+・Netflixはゲーム資産を低評価、IPの行方が焦点</t>
+        </is>
+      </c>
+      <c r="G181" s="15" t="inlineStr">
+        <is>
+          <t>規制当局の審査と対抗提案が変数。成立すればNetflixは強力なIP群を取得し配信とゲームのクロスメディア展開を加速する一方、WB Gamesの独立性低下やスタジオ再編リスクもある。</t>
+        </is>
+      </c>
+      <c r="H181" s="15" t="inlineStr">
+        <is>
+          <t>配信大手のIP獲得とクロスメディア戦略</t>
+        </is>
+      </c>
+      <c r="I181" s="15" t="inlineStr">
+        <is>
+          <t>Netflix, Warner Bros. Discovery</t>
+        </is>
+      </c>
+      <c r="J181" s="15" t="inlineStr">
+        <is>
+          <t>Mortal Kombat, Harry Potter/Hogwarts Legacy</t>
+        </is>
+      </c>
+      <c r="K181" s="15" t="inlineStr">
+        <is>
+          <t>M&amp;A,海外</t>
+        </is>
+      </c>
+      <c r="L181" s="15" t="inlineStr"/>
+    </row>
+    <row r="182">
+      <c r="A182" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B182" s="15" t="inlineStr">
+        <is>
+          <t>Krafton、Hanwha Aerospaceと約10億ドル規模のAI・ロボティクス協業を発表</t>
+        </is>
+      </c>
+      <c r="C182" s="15" t="inlineStr">
+        <is>
+          <t>https://www.gamedeveloper.com/business/ioi-partners-disowns-mindseye-krafton-collabs-with-arms-dealer-and-more-cuts-at-ubisoft-patch-notes-44</t>
+        </is>
+      </c>
+      <c r="D182" s="15" t="inlineStr">
+        <is>
+          <t>PUBG等で知られる韓国KraftonはAI技術への投資を強化している。航空・防衛大手のHanwha Aerospaceと約10億ドル規模で、AI・ロボティクス分野の協業に踏み出した。ゲーム企業のシミュレーション/AI技術を現実産業へ転用する動きとして注目される。</t>
+        </is>
+      </c>
+      <c r="E182" s="15" t="inlineStr">
+        <is>
+          <t>ゲーム開発で培ったリアルタイム3D・物理シミュレーション・強化学習などの技術は、ロボティクスや自律システムと親和性が高い。Kraftonは新規事業の柱としてAIを位置づけ、エンタメ外の収益源を確保する狙い。一方で防衛分野との関与には倫理的議論も伴う。</t>
+        </is>
+      </c>
+      <c r="F182" s="15" t="inlineStr">
+        <is>
+          <t>・協業規模は約10億ドル、AI・ロボティクス領域
+・相手は航空・防衛大手Hanwha Aerospace
+・ゲーム由来のシミュレーション/AI技術の産業転用
+・ゲーム企業のエンタメ外収益多角化の象徴</t>
+        </is>
+      </c>
+      <c r="G182" s="15" t="inlineStr">
+        <is>
+          <t>ゲーム技術の『産業両用』転用が今後も拡大する見込み。シミュレーション、デジタルツイン、自律エージェント分野で、ゲームエンジン企業や大手パブリッシャーが他産業と組む事例が増えると予想される。</t>
+        </is>
+      </c>
+      <c r="H182" s="15" t="inlineStr">
+        <is>
+          <t>ゲーム技術の産業転用(シミュレーション/デジタルツイン)</t>
+        </is>
+      </c>
+      <c r="I182" s="15" t="inlineStr">
+        <is>
+          <t>Krafton, Hanwha Aerospace</t>
+        </is>
+      </c>
+      <c r="J182" s="15" t="inlineStr">
+        <is>
+          <t>PUBG</t>
+        </is>
+      </c>
+      <c r="K182" s="15" t="inlineStr">
+        <is>
+          <t>技術,M&amp;A,海外</t>
+        </is>
+      </c>
+      <c r="L182" s="15" t="inlineStr"/>
+    </row>
+    <row r="183">
+      <c r="A183" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B183" s="15" t="inlineStr">
+        <is>
+          <t>スマホ新法施行半年、iPhone外部アプリストアにゲーム主要30社の出店ゼロ</t>
+        </is>
+      </c>
+      <c r="C183" s="15" t="inlineStr">
+        <is>
+          <t>https://www.nikkei.com/article/DGXZQOUC170OZ0X10C26A6000000/</t>
+        </is>
+      </c>
+      <c r="D183" s="15" t="inlineStr">
+        <is>
+          <t>2025年12月18日、アプリ配信・決済の外部開放を義務付ける『スマホソフトウェア競争促進法(スマホ新法)』が全面施行された。Apple/Googleの寡占に風穴を開ける狙いだが、施行半年の時点でiPhoneの外部アプリストアにゲーム主要30社の出店はゼロにとどまる。</t>
+        </is>
+      </c>
+      <c r="E183" s="15" t="inlineStr">
+        <is>
+          <t>外部決済の手数料水準や審査・セキュリティ負担への不満が根強く、開発各社は様子見の構え。MCF等の業界団体は外部決済を巡る問題解消を求める緊急共同声明も発表した。制度は整っても商習慣・信頼面の移行が進まず、競争促進の効果は限定的なのが現状だ。</t>
+        </is>
+      </c>
+      <c r="F183" s="15" t="inlineStr">
+        <is>
+          <t>・施行半年で外部ストアへのゲーム主要30社の出店ゼロ
+・外部決済の手数料・審査負担に開発者の不満
+・MCF等が問題解消を求める共同声明を発表
+・制度整備とエコシステム移行の間に大きな溝</t>
+        </is>
+      </c>
+      <c r="G183" s="15" t="inlineStr">
+        <is>
+          <t>当面はApple/Google公式ストアの優位が続く見込み。手数料体系の見直しや大手1社の先行出店があれば流れが変わる可能性があり、規制当局の運用強化と各社の収益設計の動向が鍵となる。</t>
+        </is>
+      </c>
+      <c r="H183" s="15" t="inlineStr">
+        <is>
+          <t>スマホ新法とアプリ流通/決済の競争政策</t>
+        </is>
+      </c>
+      <c r="I183" s="15" t="inlineStr">
+        <is>
+          <t>Apple, Google, MCF(モバイル・コンテンツ・フォーラム)</t>
+        </is>
+      </c>
+      <c r="J183" s="15" t="inlineStr">
+        <is>
+          <t>(モバイルゲーム全般)</t>
+        </is>
+      </c>
+      <c r="K183" s="15" t="inlineStr">
+        <is>
+          <t>規制,国内</t>
+        </is>
+      </c>
+      <c r="L183" s="15" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
events: add dev/indie events (CEDEC, Tokyo Game Dungeon, DigiGame Expo, INDIE Live Expo) (2026-06-21 02:21)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -5915,7 +5915,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6639,6 +6639,246 @@
       <c r="J14" s="15" t="inlineStr">
         <is>
           <t>2026-06-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B15" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C15" s="15" t="inlineStr">
+        <is>
+          <t>CEDEC 2026</t>
+        </is>
+      </c>
+      <c r="D15" s="15" t="inlineStr">
+        <is>
+          <t>展示会</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>パシフィコ横浜ノース(横浜)/オンライン</t>
+        </is>
+      </c>
+      <c r="F15" s="15" t="inlineStr">
+        <is>
+          <t>ハイブリッド</t>
+        </is>
+      </c>
+      <c r="G15" s="15" t="inlineStr">
+        <is>
+          <t>国内最大級のゲーム開発者向けカンファレンス。プログラミング・AI・アート・サウンド・ビジネス等、技術と知見を共有する3日間。</t>
+        </is>
+      </c>
+      <c r="H15" s="15" t="inlineStr">
+        <is>
+          <t>https://cedec.cesa.or.jp/2026/</t>
+        </is>
+      </c>
+      <c r="I15" s="15" t="inlineStr">
+        <is>
+          <t>開催予定</t>
+        </is>
+      </c>
+      <c r="J15" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B16" s="15" t="n"/>
+      <c r="C16" s="15" t="inlineStr">
+        <is>
+          <t>東京ゲームダンジョン13</t>
+        </is>
+      </c>
+      <c r="D16" s="15" t="inlineStr">
+        <is>
+          <t>展示会</t>
+        </is>
+      </c>
+      <c r="E16" s="15" t="inlineStr">
+        <is>
+          <t>東京・浜松町(都立産業貿易センター)</t>
+        </is>
+      </c>
+      <c r="F16" s="15" t="inlineStr">
+        <is>
+          <t>オフライン</t>
+        </is>
+      </c>
+      <c r="G16" s="15" t="inlineStr">
+        <is>
+          <t>個人・インディー開発者中心の同人/インディーゲーム展示会。先着順出展で個人開発に寄り添う運営方針。</t>
+        </is>
+      </c>
+      <c r="H16" s="15" t="inlineStr">
+        <is>
+          <t>https://tokyogamedungeon.com/</t>
+        </is>
+      </c>
+      <c r="I16" s="15" t="inlineStr">
+        <is>
+          <t>開催予定</t>
+        </is>
+      </c>
+      <c r="J16" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B17" s="15" t="n"/>
+      <c r="C17" s="15" t="inlineStr">
+        <is>
+          <t>東京ゲームダンジョン14</t>
+        </is>
+      </c>
+      <c r="D17" s="15" t="inlineStr">
+        <is>
+          <t>展示会</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>東京・浜松町</t>
+        </is>
+      </c>
+      <c r="F17" s="15" t="inlineStr">
+        <is>
+          <t>オフライン</t>
+        </is>
+      </c>
+      <c r="G17" s="15" t="inlineStr">
+        <is>
+          <t>東京ゲームダンジョンの2026年秋回。インディー/個人開発の新作プレイアブル展示が中心。</t>
+        </is>
+      </c>
+      <c r="H17" s="15" t="inlineStr">
+        <is>
+          <t>https://tokyogamedungeon.com/</t>
+        </is>
+      </c>
+      <c r="I17" s="15" t="inlineStr">
+        <is>
+          <t>開催予定</t>
+        </is>
+      </c>
+      <c r="J17" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="15" t="inlineStr">
+        <is>
+          <t>2026-11-08</t>
+        </is>
+      </c>
+      <c r="B18" s="15" t="n"/>
+      <c r="C18" s="15" t="inlineStr">
+        <is>
+          <t>デジゲー博2026</t>
+        </is>
+      </c>
+      <c r="D18" s="15" t="inlineStr">
+        <is>
+          <t>展示会</t>
+        </is>
+      </c>
+      <c r="E18" s="15" t="inlineStr">
+        <is>
+          <t>秋葉原UDX(東京)</t>
+        </is>
+      </c>
+      <c r="F18" s="15" t="inlineStr">
+        <is>
+          <t>オフライン</t>
+        </is>
+      </c>
+      <c r="G18" s="15" t="inlineStr">
+        <is>
+          <t>同人・インディーゲームオンリーの展示・即売会。14回目。サークル参加受付は7/22開始。実験的な個人開発作が多数。</t>
+        </is>
+      </c>
+      <c r="H18" s="15" t="inlineStr">
+        <is>
+          <t>https://digigame-expo.org/</t>
+        </is>
+      </c>
+      <c r="I18" s="15" t="inlineStr">
+        <is>
+          <t>開催予定</t>
+        </is>
+      </c>
+      <c r="J18" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="15" t="n"/>
+      <c r="B19" s="15" t="n"/>
+      <c r="C19" s="15" t="inlineStr">
+        <is>
+          <t>INDIE Live Expo 2026(冬)</t>
+        </is>
+      </c>
+      <c r="D19" s="15" t="inlineStr">
+        <is>
+          <t>ショーケース</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="inlineStr">
+        <is>
+          <t>オンライン配信</t>
+        </is>
+      </c>
+      <c r="F19" s="15" t="inlineStr">
+        <is>
+          <t>オンライン</t>
+        </is>
+      </c>
+      <c r="G19" s="15" t="inlineStr">
+        <is>
+          <t>アジア最大級のインディーゲーム情報番組。世界初公開タイトルや発売日発表が多数。次回は2026年冬開催予定(日程未定)。</t>
+        </is>
+      </c>
+      <c r="H19" s="15" t="inlineStr">
+        <is>
+          <t>https://indie.live-expo.games/</t>
+        </is>
+      </c>
+      <c r="I19" s="15" t="inlineStr">
+        <is>
+          <t>日程未確定</t>
+        </is>
+      </c>
+      <c r="J19" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
daily-news + cross-questions + events update (2026-06-21 22:13)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -6633,12 +6633,12 @@
       </c>
       <c r="I14" s="15" t="inlineStr">
         <is>
-          <t>開催中</t>
+          <t>終了</t>
         </is>
       </c>
       <c r="J14" s="15" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -6893,7 +6893,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L183"/>
+  <dimension ref="A1:L189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18314,6 +18314,376 @@
         </is>
       </c>
       <c r="L183" s="15" t="inlineStr"/>
+    </row>
+    <row r="184">
+      <c r="A184" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B184" s="5" t="inlineStr">
+        <is>
+          <t>スクエニ『ドラクエX オンライン』V8「時空の迷い子たち」6/25発売へ最新情報</t>
+        </is>
+      </c>
+      <c r="C184" s="5" t="inlineStr">
+        <is>
+          <t>https://hiroba.dqx.jp/sc/topics/detail/608b30e45f4b60adb254a8127a6da8ef/</t>
+        </is>
+      </c>
+      <c r="D184" s="5" t="inlineStr">
+        <is>
+          <t>『ドラゴンクエストXオンライン』はサービス開始から十数年続く長寿MMORPG。スクウェア・エニックスは年次の有料追加パッケージで物語と課金を継続しており、最新作バージョン8の発売を6/25に控え、6月中旬以降に大型アップデート情報を順次公開している。</t>
+        </is>
+      </c>
+      <c r="E184" s="5" t="inlineStr">
+        <is>
+          <t>バージョン8「時空の迷い子たち」が2026/6/25発売。新ストーリーや新システムに加え、バージョン1〜8を収録したDL専用『オールインワンパッケージ version 1-8』、堀井雄二氏の手紙付きグッズボックスも同日リリース。標準版は4950円(税込)。</t>
+        </is>
+      </c>
+      <c r="F184" s="5" t="inlineStr">
+        <is>
+          <t>・発売日2026/6/25、標準版4950円(税込)
+・新規/復帰両取りの『オールインワンパッケージ version 1-8』を同時投入
+・バージョン8.0の大型アップデート情報を6月中旬以降に順次公開
+・長寿MMOの『年次有料拡張』モデルを堅持</t>
+        </is>
+      </c>
+      <c r="G184" s="5" t="inlineStr">
+        <is>
+          <t>Switch 2世代でも旧IPの長寿運営タイトルは『新規＋復帰』導線を強化し、まとめ売りパッケージで休眠層の再課金を狙う流れが続く。終わりの見えない長寿MMOは各社の安定収益源として下支えになる。</t>
+        </is>
+      </c>
+      <c r="H184" s="5" t="inlineStr">
+        <is>
+          <t>長寿MMORPGの継続課金設計と復帰導線</t>
+        </is>
+      </c>
+      <c r="I184" s="5" t="inlineStr">
+        <is>
+          <t>スクウェア・エニックス</t>
+        </is>
+      </c>
+      <c r="J184" s="5" t="inlineStr">
+        <is>
+          <t>ドラゴンクエストX オンライン</t>
+        </is>
+      </c>
+      <c r="K184" s="5" t="inlineStr">
+        <is>
+          <t>新作,国内</t>
+        </is>
+      </c>
+      <c r="L184" s="5" t="n"/>
+    </row>
+    <row r="185">
+      <c r="A185" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B185" s="5" t="inlineStr">
+        <is>
+          <t>Cygames『シャドバWB』1周年＆シリーズ10周年、新パック6/29追加</t>
+        </is>
+      </c>
+      <c r="C185" s="5" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/760/G076035/20260620004/</t>
+        </is>
+      </c>
+      <c r="D185" s="5" t="inlineStr">
+        <is>
+          <t>Cygamesのデジタルカードゲーム『Shadowverse: Worlds Beyond』は2025年6月にサービス開始し、2026/6/20で1周年。シリーズ本体『Shadowverse』は10周年を迎え、両記念を絡めた大型施策を展開している。</t>
+        </is>
+      </c>
+      <c r="E185" s="5" t="inlineStr">
+        <is>
+          <t>1周年＆シリーズ10周年を記念し、前作の人気キャラ(バハムート、リュミオール等)が集結する新カードパック「クロニクル・オブ・デスティニー」を6/29に追加。最大120パック配布や総額1億円分が当たる記念キャンペーン、新メインストーリーも実装する。</t>
+        </is>
+      </c>
+      <c r="F185" s="5" t="inlineStr">
+        <is>
+          <t>・WB 1周年(6/20)＋『Shadowverse』10周年の二重記念
+・新パック「クロニクル・オブ・デスティニー」6/29追加
+・最大120パック配布・総額1億円分のキャンペーン
+・前作IP資産を新作へ流し込む『オールスター』設計</t>
+        </is>
+      </c>
+      <c r="G185" s="5" t="inlineStr">
+        <is>
+          <t>周年商戦では大型の無料配布と既存IPキャラの再登板で休眠層の復帰とアクティブ維持を図る手法が定着。デジタルCCGは『周年×オールスター』を年次の山場として運用していく。</t>
+        </is>
+      </c>
+      <c r="H185" s="5" t="inlineStr">
+        <is>
+          <t>デジタルCCGの周年運用とIP資産の再活用</t>
+        </is>
+      </c>
+      <c r="I185" s="5" t="inlineStr">
+        <is>
+          <t>Cygames</t>
+        </is>
+      </c>
+      <c r="J185" s="5" t="inlineStr">
+        <is>
+          <t>Shadowverse: Worlds Beyond, Shadowverse</t>
+        </is>
+      </c>
+      <c r="K185" s="5" t="inlineStr">
+        <is>
+          <t>新作,国内</t>
+        </is>
+      </c>
+      <c r="L185" s="5" t="n"/>
+    </row>
+    <row r="186">
+      <c r="A186" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B186" s="5" t="inlineStr">
+        <is>
+          <t>EU AI法、8/2全面適用迫る——AI生成透明性Code of Practice最終化へ</t>
+        </is>
+      </c>
+      <c r="C186" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pwc.com/jp/ja/knowledge/column/awareness-cyber-security/generative-ai-regulation10.html</t>
+        </is>
+      </c>
+      <c r="D186" s="5" t="inlineStr">
+        <is>
+          <t>EU AI法(AI Act)は段階適用が進み、2026/8/2に大半の条項が全面適用となる。AI生成コンテンツの透明性に関する行動規範(Code of Practice)は2025年末に初稿が公表され、2026年5〜6月頃に最終版が出る見込みで、生成AIを使うゲーム開発にも影響が及ぶ。</t>
+        </is>
+      </c>
+      <c r="E186" s="5" t="inlineStr">
+        <is>
+          <t>AI生成コンテンツの開示・ラベリングを求める透明性ルールが最終段階に入り、ゲームのAI実装(動的生成シーンやNPC対話)にも年齢区分やコンテンツ開示の義務が及び得る。日本企業にも域外適用があり、8/2の全面適用が当面の基準日となる。</t>
+        </is>
+      </c>
+      <c r="F186" s="5" t="inlineStr">
+        <is>
+          <t>・EU AI法は2026/8/2に大半の条項が全面適用
+・AI生成透明性のCode of Practice最終版が6月頃公表見込み
+・動的生成・対話型AIは年齢区分/開示義務の対象になり得る
+・域外適用で日本のゲーム企業も対応が必要</t>
+        </is>
+      </c>
+      <c r="G186" s="5" t="inlineStr">
+        <is>
+          <t>AI生成物の『開示・ラベリング』義務がゲームから広告・映像・出版へ横展開し、生成AIを使う制作現場全般でコンテンツの出自表示と年齢ゲートの実装が標準化していく。</t>
+        </is>
+      </c>
+      <c r="H186" s="5" t="inlineStr">
+        <is>
+          <t>EU AI法とAI生成コンテンツの開示義務</t>
+        </is>
+      </c>
+      <c r="I186" s="5" t="inlineStr">
+        <is>
+          <t>European Commission</t>
+        </is>
+      </c>
+      <c r="J186" s="5" t="inlineStr">
+        <is>
+          <t>(生成AI/ゲーム全般)</t>
+        </is>
+      </c>
+      <c r="K186" s="5" t="inlineStr">
+        <is>
+          <t>規制,技術,海外</t>
+        </is>
+      </c>
+      <c r="L186" s="5" t="n"/>
+    </row>
+    <row r="187">
+      <c r="A187" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B187" s="5" t="inlineStr">
+        <is>
+          <t>2K『シヴィライゼーションVII』追加アップデートを6/22週に配信</t>
+        </is>
+      </c>
+      <c r="C187" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pcgamer.com/games/strategy/civilization-7s-imminent-update-will-add-one-of-historys-most-famous-conquerors-for-free-in-firaxis-latest-bid-to-coax-you-back-to-its-controversial-sequel/</t>
+        </is>
+      </c>
+      <c r="D187" s="5" t="inlineStr">
+        <is>
+          <t>『シドマイヤーズ シヴィライゼーションVII』は発売後に賛否が割れ、Firaxis/2Kは5/19の大型アップデート「Test of Time」で勝利条件や時代システムを刷新。離反したプレイヤーの呼び戻しを狙い、無料コンテンツの追加投入を続けている。</t>
+        </is>
+      </c>
+      <c r="E187" s="5" t="inlineStr">
+        <is>
+          <t>「Test of Time」に続く追加アップデートを6/22の週に配信予定。歴史上著名な指導者を無料で追加するなど、無料コンテンツで休眠・離脱層の再活性化を図る、賛否が割れたタイトルのテコ入れ継続策。</t>
+        </is>
+      </c>
+      <c r="F187" s="5" t="inlineStr">
+        <is>
+          <t>・5/19「Test of Time」後の継続アップデートを6/22週配信
+・無料の新指導者追加で離脱層の再獲得を狙う
+・勝利条件・時代システム刷新後の調整フェーズ
+・『出してから直す』長期運営型の単品買い切りタイトル</t>
+        </is>
+      </c>
+      <c r="G187" s="5" t="inlineStr">
+        <is>
+          <t>賛否の割れたAAA単品タイトルは、発売後の大型無料アップデートで評価を立て直す『ライブサービス型の運営』が常態化。初動失敗からの長期回復を前提とした運営設計が広がる。</t>
+        </is>
+      </c>
+      <c r="H187" s="5" t="inlineStr">
+        <is>
+          <t>買い切りAAAの発売後リカバリー運営</t>
+        </is>
+      </c>
+      <c r="I187" s="5" t="inlineStr">
+        <is>
+          <t>2K, Firaxis Games</t>
+        </is>
+      </c>
+      <c r="J187" s="5" t="inlineStr">
+        <is>
+          <t>シドマイヤーズ シヴィライゼーションVII</t>
+        </is>
+      </c>
+      <c r="K187" s="5" t="inlineStr">
+        <is>
+          <t>新作,海外</t>
+        </is>
+      </c>
+      <c r="L187" s="5" t="n"/>
+    </row>
+    <row r="188">
+      <c r="A188" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B188" s="5" t="inlineStr">
+        <is>
+          <t>ネコノメ、オンライン将棋「棋桜」Google Play版を6/22配信</t>
+        </is>
+      </c>
+      <c r="C188" s="5" t="inlineStr">
+        <is>
+          <t>https://gamebiz.jp/news/427451</t>
+        </is>
+      </c>
+      <c r="D188" s="5" t="inlineStr">
+        <is>
+          <t>国内ゲームスタートアップのネコノメは2026/6にシリーズAの第三者割当増資で1.1億円(累計2億円)を調達。EXイノベーションファンドや三菱UFJキャピタル、SMBCベンチャーキャピタル等が出資し、新作開発・既存タイトルの海外展開・採用に充てる。</t>
+        </is>
+      </c>
+      <c r="E188" s="5" t="inlineStr">
+        <is>
+          <t>調達資金で開発を進めるオンライン将棋ゲーム「棋桜(KIOU)」のGoogle Play版を6/22に配信。小規模スタートアップが伝統ゲーム×オンライン対戦で参入し、VCマネーを背景にグローバル展開と人材採用を強化する国内の事例。</t>
+        </is>
+      </c>
+      <c r="F188" s="5" t="inlineStr">
+        <is>
+          <t>・シリーズAで1.1億円調達、累計2億円
+・出資はEXイノベ/三菱UFJキャピタル/SMBC VC等
+・「棋桜(KIOU)」Google Play版を6/22配信
+・資金用途は新作開発・海外展開・採用</t>
+        </is>
+      </c>
+      <c r="G188" s="5" t="inlineStr">
+        <is>
+          <t>大手のレイオフが続く一方、少人数×VC資金の国内ゲームスタートアップが伝統・ニッチ領域で立ち上がる二極化が進む。オンライン対戦×伝統ゲームはアジア圏での横展開余地が大きい。</t>
+        </is>
+      </c>
+      <c r="H188" s="5" t="inlineStr">
+        <is>
+          <t>国内ゲームスタートアップの資金調達動向</t>
+        </is>
+      </c>
+      <c r="I188" s="5" t="inlineStr">
+        <is>
+          <t>ネコノメ, 三菱UFJキャピタル, SMBCベンチャーキャピタル</t>
+        </is>
+      </c>
+      <c r="J188" s="5" t="inlineStr">
+        <is>
+          <t>棋桜(KIOU)</t>
+        </is>
+      </c>
+      <c r="K188" s="5" t="inlineStr">
+        <is>
+          <t>M&amp;A,インディー,国内</t>
+        </is>
+      </c>
+      <c r="L188" s="5" t="n"/>
+    </row>
+    <row r="189">
+      <c r="A189" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B189" s="5" t="inlineStr">
+        <is>
+          <t>Valve、Steamサマーセール2026トレーラー公開——6/25開幕(〜7/9)</t>
+        </is>
+      </c>
+      <c r="C189" s="5" t="inlineStr">
+        <is>
+          <t>https://steamcommunity.com/groups/steamworks/announcements/detail/493837645658461608</t>
+        </is>
+      </c>
+      <c r="D189" s="5" t="inlineStr">
+        <is>
+          <t>Valveは年複数回の大型セールで需要を集中喚起する。6/15-22のSteam Next Fest(体験版祭り)でウィッシュリストを積ませ、その直後にサマーセールを当てる『デモ→割引』の購買導線を例年構築している。</t>
+        </is>
+      </c>
+      <c r="E189" s="5" t="inlineStr">
+        <is>
+          <t>サマーセール2026は6/25開幕、7/9まで14日間。Valveは開幕に先立ちトレーラーと一部参加タイトルを公開。Next Fest終了(6/22)の数日後にセールを当て、ウィッシュリスト登録者の購入転換を狙う設計。</t>
+        </is>
+      </c>
+      <c r="F189" s="5" t="inlineStr">
+        <is>
+          <t>・Steamサマーセール2026は6/25〜7/9の14日間
+・割引は太平洋時間10時に一斉開始
+・Next Fest(6/15-22)直後に配置し購買転換を最大化
+・Valveがトレーラー＋参加タイトルを先行公開</t>
+        </is>
+      </c>
+      <c r="G189" s="5" t="inlineStr">
+        <is>
+          <t>PCゲーム需要はSteamの年次セール暦に強く同期し、Next Fest→セールの連続設計が業界標準の購買導線として定着。中小・インディーは露出ピークをこの暦に合わせ発売・値引きを最適化する。</t>
+        </is>
+      </c>
+      <c r="H189" s="5" t="inlineStr">
+        <is>
+          <t>Steamセール暦と購買導線の設計</t>
+        </is>
+      </c>
+      <c r="I189" s="5" t="inlineStr">
+        <is>
+          <t>Valve</t>
+        </is>
+      </c>
+      <c r="J189" s="5" t="inlineStr">
+        <is>
+          <t>Steam</t>
+        </is>
+      </c>
+      <c r="K189" s="5" t="inlineStr">
+        <is>
+          <t>海外</t>
+        </is>
+      </c>
+      <c r="L189" s="5" t="inlineStr">
+        <is>
+          <t>開催日程は太平洋時間基準(JSTでは前後する)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
weekly-stocks + IP watch update (2026-06-22 14:21)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -20145,8 +20145,16 @@
           <t>日本</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr"/>
-      <c r="E9" s="9" t="inlineStr"/>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>『ドラクエ12』の最新情報を6月に公開も発売時期は未定で続報待ち。『ドラゴンクエストX オンライン』Ver8『時空の迷い子たち』を6/25実装予定。</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>DQ12(時期未定)、DQXオンライン Ver8(2026/6/25)</t>
+        </is>
+      </c>
       <c r="F9" s="9" t="inlineStr"/>
       <c r="G9" s="9" t="inlineStr">
         <is>
@@ -20154,7 +20162,11 @@
         </is>
       </c>
       <c r="H9" s="9" t="inlineStr"/>
-      <c r="I9" s="9" t="inlineStr"/>
+      <c r="I9" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
@@ -20730,7 +20742,11 @@
           <t>日本</t>
         </is>
       </c>
-      <c r="D28" s="9" t="inlineStr"/>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>英語版が海外売上を前年同期比3.5倍に拡大しCygamesゲーム事業を牽引(FY2Q ゲーム売上+31.2%)。グローバル展開とコラボ施策を継続。</t>
+        </is>
+      </c>
       <c r="E28" s="9" t="inlineStr"/>
       <c r="F28" s="9" t="inlineStr"/>
       <c r="G28" s="9" t="inlineStr">
@@ -20739,7 +20755,11 @@
         </is>
       </c>
       <c r="H28" s="9" t="inlineStr"/>
-      <c r="I28" s="9" t="inlineStr"/>
+      <c r="I28" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="9" t="inlineStr">
@@ -20759,12 +20779,12 @@
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>GTA6の発売日が2026年11月19日に。Piperは初年度3,500万本超を予測、TTWOはFY27に過去最高業績を計画。</t>
+          <t>Take-Two CEOがGTA6の11/19発売を再明言、本格マーケティングは6月下旬から始動。初年度3,500万本超の販売予測。</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>Grand Theft Auto VI(2026/11/19予定)</t>
+          <t>Grand Theft Auto VI(2026/11/19)</t>
         </is>
       </c>
       <c r="F29" s="9" t="inlineStr"/>
@@ -20776,7 +20796,7 @@
       <c r="H29" s="9" t="inlineStr"/>
       <c r="I29" s="9" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -20850,8 +20870,16 @@
           <t>海外</t>
         </is>
       </c>
-      <c r="D32" s="9" t="inlineStr"/>
-      <c r="E32" s="9" t="inlineStr"/>
+      <c r="D32" s="9" t="inlineStr">
+        <is>
+          <t>Xbox Games Showcase(6/7)で『Modern Warfare 4』を披露、抽出型モード『DMZ』復活を発表。7月にプレイテスト実施予定。</t>
+        </is>
+      </c>
+      <c r="E32" s="9" t="inlineStr">
+        <is>
+          <t>Call of Duty: Modern Warfare 4(2026/10/23)</t>
+        </is>
+      </c>
       <c r="F32" s="9" t="inlineStr"/>
       <c r="G32" s="9" t="inlineStr">
         <is>
@@ -20859,7 +20887,11 @@
         </is>
       </c>
       <c r="H32" s="9" t="inlineStr"/>
-      <c r="I32" s="9" t="inlineStr"/>
+      <c r="I32" s="9" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="9" t="inlineStr">
@@ -21095,7 +21127,7 @@
       </c>
       <c r="D41" s="9" t="inlineStr">
         <is>
-          <t>Battlefield 6がEA過去最高の年・フランチャイズ各種記録を更新。EAは約$550億での非公開化が進行中。</t>
+          <t>『Battlefield 6』がシリーズ最高の年となりEAのFY26 Net Bookings過去最高($8,026m,+9%)を牽引。ライブサービス運営を強化。</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
@@ -21112,7 +21144,7 @@
       <c r="H41" s="9" t="inlineStr"/>
       <c r="I41" s="9" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -21161,7 +21193,7 @@
       </c>
       <c r="D43" s="9" t="inlineStr">
         <is>
-          <t>FY26通期で二桁の回復を達成し、EAのNet Bookings過去最高に貢献。</t>
+          <t>通年で二桁の回復を達成しEA FY26業績に寄与。シーズン運営とマネタイズ立て直しが進む。</t>
         </is>
       </c>
       <c r="E43" s="9" t="inlineStr">
@@ -21178,7 +21210,7 @@
       <c r="H43" s="9" t="inlineStr"/>
       <c r="I43" s="9" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -21200,7 +21232,7 @@
       </c>
       <c r="D44" s="9" t="inlineStr">
         <is>
-          <t>運営元が新子会社Vantage Studiosへ集約。Tencentが€11.6億を出資(持分26.32%)し開発体制を再編。</t>
+          <t>6/16に『AC Shadows』タイトルアップデート1.1.11を配信。Ubisoftは組織再編下でシリーズの運営を継続。</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
@@ -21217,7 +21249,7 @@
       <c r="H44" s="9" t="inlineStr"/>
       <c r="I44" s="9" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -21506,7 +21538,7 @@
       </c>
       <c r="D54" s="9" t="inlineStr">
         <is>
-          <t>5〜8歳向け『Roblox Kids』・9〜15歳向け『Roblox Select』を6月初に展開。年齢確認強化で短期のユーザー成長に摩擦も、Q1売上は$1.4bn(+39%)。</t>
+          <t>6/18時点でエンゲージメントが3週連続改善。『Roblox Kids』『Roblox Select』アカウントを世界展開し年齢別の安全設計を強化。</t>
         </is>
       </c>
       <c r="E54" s="9" t="inlineStr">
@@ -21523,7 +21555,7 @@
       <c r="H54" s="9" t="inlineStr"/>
       <c r="I54" s="9" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -21783,7 +21815,9 @@
           <t>コンソール/IP</t>
         </is>
       </c>
-      <c r="D2" s="9" t="inlineStr"/>
+      <c r="D2" s="9" t="n">
+        <v>9.1</v>
+      </c>
       <c r="E2" s="9" t="inlineStr"/>
       <c r="F2" s="9" t="inlineStr"/>
       <c r="G2" s="9" t="inlineStr"/>
@@ -21792,8 +21826,12 @@
           <t>27.9（予想）</t>
         </is>
       </c>
-      <c r="I2" s="9" t="inlineStr"/>
-      <c r="J2" s="9" t="inlineStr"/>
+      <c r="I2" s="9" t="n">
+        <v>2.76</v>
+      </c>
+      <c r="J2" s="9" t="n">
+        <v>10.5</v>
+      </c>
       <c r="K2" s="9" t="inlineStr">
         <is>
           <t>2.15（予想）</t>
@@ -21806,7 +21844,7 @@
       </c>
       <c r="M2" s="9" t="inlineStr">
         <is>
-          <t>6/9に「Nintendo Direct 2026.6.9」を配信し、ゼルダ『時のオカリナ』Switch 2リメイク、ゼノブレイド新作、KH4新映像など2026年後半タイトルを公開。同日にフランス当局の制裁金約65億円報道も。株価は6/9の7,738円から普及ペース懸念で6/12は7,174円へ反落（6/10は-6.76%）、大手証券が6/12にレーティング中立据え置き・目標株価を8,300円へ引き下げ。Switch 2値上げ後の普及速度が引き続き焦点。</t>
+          <t>6/26に第86期定時株主総会を控え、株価は材料待ちで軟調（6/16→6/19は7,218→7,076円へ軟化、年初来安値6,849円圏）。Switch 2の普及ペースと欧米年末商戦の不振懸念が引き続き重し。時価総額約9.1兆円・PBR2.76倍・予想ROE10.5%。大型ファーストパーティの供給と普及加速が次の株価材料。</t>
         </is>
       </c>
       <c r="N2" s="9" t="inlineStr">
@@ -21826,7 +21864,7 @@
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -21861,7 +21899,7 @@
       </c>
       <c r="M3" s="9" t="inlineStr">
         <is>
-          <t>6/8の株価は3,508円前後。5月発表の最大5,000億円の自社株買いを継続し5月末までに約1,900万株を取得、株主還元姿勢が下支え。音楽事業は増収増益と好調でカタログ取得も加速。一方ゲームはPS5販売が前年同期比約15%減とサイクル後半入りが鮮明。アナリスト平均目標株価は約4,657円で、現値からの上値余地を見込む声が多い。</t>
+          <t>6/19終値3,140円（前日比-3.38%）。PS5は後半サイクルで販売鈍化も、25年度はゲーム以外（音楽・センサー）が牽引し営業利益1.45兆円（+13.4%）。PS6が2027年以降発売との報道が出始め、26年はPS5ソフトで稼ぐ最終局面との見方。アナリストは強気継続で平均目標株価4,674円。</t>
         </is>
       </c>
       <c r="N3" s="9" t="inlineStr">
@@ -21881,7 +21919,7 @@
       </c>
       <c r="Q3" s="9" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -21916,7 +21954,7 @@
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>先週末発表の『バイオハザード RE:Veronica』『モンハンWilds:Ascendance』（ともに2027年）を好感し6/8は+5.06%の3,031円。6/9のニンダイで『鬼武者 Way of the Sword』を9/25発売と告知。ただ6/10は任天堂主導のゲームセクター調整で連れ安。10期連続最高益のIP基盤は不変で、Switch 2展開と2027年の大型パイプラインが評価軸。</t>
+          <t>6/9ニンダイ告知の『鬼武者 Way of the Sword』(9/25)の体験版が好評。先週発表のモンハン/バイオ新作(2027)期待は継続も、今週は新規材料に乏しく任天堂主導のゲームセクター調整に連れ安。10期連続最高益のIP基盤は不変で、2027年の大型パイプラインとSwitch 2展開が評価軸。</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
@@ -21936,7 +21974,7 @@
       </c>
       <c r="Q4" s="9" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -21983,7 +22021,7 @@
       </c>
       <c r="M5" s="9" t="inlineStr">
         <is>
-          <t>FY26/3は売上2,976.61億（-8.3%）も営業益547.36億（+34.9%）・純益296.16億（+21.3%）と構造改革で増益。6/9のニンダイで『キングダムハーツIV』の新規映像が公開され話題化。FY27/3は売上横ばい・営業益490億（-10.5%）の保守的計画で、HDゲーム選別と開発効率化が継続テーマ。</t>
+          <t>『ドラクエ12』の最新情報を公開も発売時期が未定だったため失望売りで株価下落。一方『ドラゴンクエストX オンライン』Ver8『時空の迷い子たち』を6/25実装予定。HD-2D系やFF7リメイク三部作の進捗、コンテンツの集中投下と海外展開が引き続き焦点。</t>
         </is>
       </c>
       <c r="N5" s="9" t="inlineStr">
@@ -22003,7 +22041,7 @@
       </c>
       <c r="Q5" s="9" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -22050,7 +22088,7 @@
       </c>
       <c r="M6" s="9" t="inlineStr">
         <is>
-          <t>FY26/3は売上4,936億(+17.1%)・営業益1,358億(+33.3%)・純益1,000億(+33.9%)で3期連続最高益。デジタルエンタメが+21.5%と牽引。年間配当221.5円(前期165.5円から増配)、次期224円予想。eFootball/遊戯王/パワプロが堅調。</t>
+          <t>FY26通期は純利益予想を750→860億円、営業利益を1,230億円(+20.7%)へ上方修正。eFootballやIP連動イベントが堅調。MGS/パワプロのIP活用と、アミューズメント・スポーツ・ジムの複合成長が継続テーマ。</t>
         </is>
       </c>
       <c r="N6" s="9" t="inlineStr">
@@ -22070,7 +22108,7 @@
       </c>
       <c r="Q6" s="9" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -22117,7 +22155,7 @@
       </c>
       <c r="M7" s="9" t="inlineStr">
         <is>
-          <t>5/13発表のFY26/3は売上1兆3,482億(+8.6%)・営業益1,895億(+5.2%)・純益1,406億(+8.8%)で過去最高更新。トイホビー好調とアミューズ回復が寄与。6/3に日系中堅証券が中立据置・目標株価4,130円へ引き下げ。株価は6/3で3,722円。</t>
+          <t>FY26は売上・利益が過去最高を更新、ガンダムIP売上が約7割増と牽引。State of Playで新作『ACE COMBAT 8』を10/2 PS5発売と告知。ガンダム/エルデンリング/アイマス等のIP軸を多面展開する戦略が強み。</t>
         </is>
       </c>
       <c r="N7" s="9" t="inlineStr">
@@ -22137,7 +22175,7 @@
       </c>
       <c r="Q7" s="9" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -22172,7 +22210,7 @@
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>6/4株価2,357.5円(-0.11%)。前期は増収(+13.6%)も営業益は2期連続減益傾向。FY27/3は増収減益計画で、遊技機は原価増、ゲーミングは先行投資で損失幅拡大見込み。エンタメは新作投入と販売体制強化で成長狙う。6/8にアトラスが『ペルソナ6』を正式発表。</t>
+          <t>FY26は最終赤字57億円。買収したRovio(313億)・Stakelogic(187億)の減損が直撃し、大型グローバル『Super Game』構想を中止。売上は4,875億円(+14%)も営業利益471億円(-2%)。『龍が如く』『ソニック』等のIP収益化と海外子会社の立て直しが課題。</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
@@ -22192,7 +22230,7 @@
       </c>
       <c r="Q8" s="9" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -22239,7 +22277,7 @@
       </c>
       <c r="M9" s="9" t="inlineStr">
         <is>
-          <t>FY26/3は売上883.93億（+6.3%）・営業益371.68億（+15.7%）で過去最高。6/9のニンダイで看板SLG最新作『信長の野望・主世』を2026年冬発売と発表し、定番シリーズの新作投入が確認された。FY27/3は人的資本投資増で経常益420億（-26.3%）と減益計画。新作サイクルと海外/IPコラボ展開が鍵。</t>
+          <t>FY26は『仁王3』『ゼルダ無双 封印戦記』等が寄与し売上825.4億円(+5.7%)・営業利益366.4億円(+16.4%)と増益。高い営業利益率と財テク収益が特徴。『信長の野望』『三國志』の周年施策や協業タイトルが継続テーマ。</t>
         </is>
       </c>
       <c r="N9" s="9" t="inlineStr">
@@ -22259,7 +22297,7 @@
       </c>
       <c r="Q9" s="9" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -22302,7 +22340,7 @@
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>FY26/3は売上1,713.69億（+10.7%）も営業益222.56億（-16.3%）と減益。6/11のゲーム株概況でミクシィは上昇し、目標株価2万円を見込むアナリストも登場するなど、スポーツ・ベッティング事業（PointsBet連結）の成長期待が再評価。一方で主力モンストの減収は継続課題。スポーツ収益化とモンスト再活性化が引き続き焦点。</t>
+          <t>FY26は売上1,713.7億円(+10.7%)も営業利益222.6億円(-16.3%)と減益。スポーツ事業(公営競技等)が成長する一方、主力モンストのデジタルエンタメ減収と費用増が利益を圧迫。新規事業の収益化とモンスト次施策が焦点。</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
@@ -22322,7 +22360,7 @@
       </c>
       <c r="Q10" s="9" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -22357,7 +22395,7 @@
       </c>
       <c r="M11" s="9" t="inlineStr">
         <is>
-          <t>5/29株価418円。FY26/6 3Qは売上384.44億(-10.9%)・営業益24.2億(-34.7%)も、為替差益で経常益32.1億(+11.1%)・純益19.1億(+112.4%)と大幅増益。期末配当21.5円へ増配予定。ゲーム/VTuber/IP/DX/投資の5事業を展開。</t>
+          <t>今週の適時開示は乏しい。メタバース『REALITY』、投資育成事業、コンシューマ向け新規IPの育成が継続テーマ。ソーシャルゲーム成熟下での新規収益柱の確立が課題。</t>
         </is>
       </c>
       <c r="N11" s="9" t="inlineStr">
@@ -22377,7 +22415,7 @@
       </c>
       <c r="Q11" s="9" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -22420,7 +22458,7 @@
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>FY26/3は売上収益1,477億（-9.9%）・営業益186.94億（-35.5%）とポケポケ初速の反動で減益。6/11のゲーム株概況ではミクシィ上昇の一方でDeNAは下落。ライブストリーミングは黒字転換し、FY27/3は売上1,540億（+4.3%）・営業益150億（-19.8%）計画。新規タイトル投入とヘルスケア/スポーツ事業の収益化が課題。</t>
+          <t>今週の新規開示は限定的。Pokémon系協業や横浜DeNAベイスターズ、ライブ配信『Pococha』、ヘルスケア/AI領域が事業の軸。ゲーム新作パイプラインと非ゲーム事業の収益化が引き続き注目。</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
@@ -22440,7 +22478,7 @@
       </c>
       <c r="Q12" s="9" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -22475,7 +22513,7 @@
       </c>
       <c r="M13" s="9" t="inlineStr">
         <is>
-          <t>FY26/9 2Q累計は売上4,785億(+14%)・純益273億(+72%)。ゲーム事業営業益は約2倍の385億で『ウマ娘』英語版ヒットが寄与し海外売上は前年比3.5倍(131億)。6/4株価1,381円(3か月で+12.4%)。通期は売上+1%・純益250〜300億見込み。</t>
+          <t>子会社CygamesのFY26 2Q(1-3月)はゲーム事業が売上675億円(+31.2%)・営業利益209億円(+36.3%)と急伸、『ウマ娘』英語版が海外売上3.5倍と牽引。下期に『ホロライブ』ゲーム化を控える。6/22に『Cygames クリエイティブコンテスト2026』開催を告知。AI・広告と新作ゲームの両輪が成長ドライバー。</t>
         </is>
       </c>
       <c r="N13" s="9" t="inlineStr">
@@ -22495,7 +22533,7 @@
       </c>
       <c r="Q13" s="9" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -22643,7 +22681,7 @@
       </c>
       <c r="L2" s="9" t="inlineStr">
         <is>
-          <t>Bloomberg（6/10）などが、Xboxが6/30の年度末後に数千人規模の大型レイオフを準備と報道。新ゲーム部門CEOのAsha Sharma氏が『事業が拡大しすぎた、優先順位を再評価する』と社内に伝達し、Game Pass等の高粗利サービスと収益性重視へ転換。マーケや一部予算も削減見込み。Activision/Bethesda等の巨大IPは維持しつつ構造改革を継続。</t>
+          <t>6/7のXbox Games Showcaseで『Gears of War: E-Day』『Clockwork Revolution』をコンソール独占と発表、Xbox 25周年記念ハードも公開。『Call of Duty: Modern Warfare 4』(10/23)はDMZ復活を披露し7月にプレイテスト。6/16にGame Pass第2弾を追加。AB統合後のソフト供給とGame Pass拡大が軸。</t>
         </is>
       </c>
       <c r="M2" s="9" t="inlineStr">
@@ -22663,7 +22701,7 @@
       </c>
       <c r="P2" s="9" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -22701,7 +22739,7 @@
       </c>
       <c r="L3" s="9" t="inlineStr">
         <is>
-          <t>FY26 Net Bookingsは$6.72bn、FY27は$8.0〜8.2bnへ大幅増ガイダンス。CEOゼルニック氏はGTA6を11/19発売と再明言し『延期しない』と強調、本格マーケティングは6月下旬以降に始動予定。GTA6初年度は3,500万本超予測。発売実現と立ち上げがFY27最高業績の鍵で、期待先行の高バリュエーションはリスク。</t>
+          <t>6/17 BNN Bloombergの『Hot Picks』でTTWOが推奨され株価は約$230へ+6%。CEOがGTA6の11/19発売を再明言し本格マーケは6月下旬始動。FY27 Net Bookingsガイダンスは$8.0〜8.2bn、GTA6初年度3,500万本超予測。発売実現が史上最高業績の鍵。</t>
         </is>
       </c>
       <c r="M3" s="9" t="inlineStr">
@@ -22721,7 +22759,7 @@
       </c>
       <c r="P3" s="9" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -22759,27 +22797,27 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>PIF/Silver Lake/Affinity連合による$210/株・総額約$550億の非公開化は6/30のロングストップに向け進行中で、CFIUS審査が最終関門（契約上の最終期限は9/28）。現時点で正式な反対報道はなし。四半期配当$0.19は6/17支払い。FY26はNet Bookings $8,026M（+9%）で過去最高、Battlefield 6がフランチャイズ最高の年。買収完了の可否が当面の最大焦点。</t>
+          <t>PIF・Silver Lake・Affinity主導の$55bn(=1株$210)take-private(史上最大級のLBO)が6/30のlong-stop dateに向け最終盤。残る関門はCFIUS審査で、株価は$210を約$9下回りディールスプレッドが残存。FY26はBattlefield 6が牽引しNet Bookings $8,026m(+9%)と過去最高。</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>$550億buyout進行と過去最高業績、Battlefield/FCの強さ</t>
+          <t>Battlefield 6の回復とNet Bookings過去最高、$210での非公開化(LBO)プレミアム</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>CFIUS等規制承認リスク、上場廃止後の不透明感</t>
+          <t>CFIUS審査・クロージング不確実性とディール破談リスク</t>
         </is>
       </c>
       <c r="O4" s="9" t="inlineStr">
         <is>
-          <t>買収完了の可否とBattlefield/EA FCの継続成長</t>
+          <t>$55bn take-privateの6/30までの完了可否(CFIUS)</t>
         </is>
       </c>
       <c r="P4" s="9" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -22813,7 +22851,7 @@
       </c>
       <c r="L5" s="9" t="inlineStr">
         <is>
-          <t>6/5株価$30.33。Q1'26売上$508.2M(+35%)・Grow部門+49%で予想超え。6/2にPiper Sandlerが目標$40へ引き上げ・オーバーウェイト、Edgewaterも格上げ。広告主導の収益化とAI活用が評価され90日で+51%(年初来は-32%)。Q4'26にGAAP黒字化を目標。</t>
+          <t>組織再編を継続し、未発表案件と『プリンス・オブ・ペルシャ 時の砂』リメイクを含む計6本を中止、パリ本社で追加人員削減を提案。一方6/16に『AC Shadows』アップデート1.1.11を配信し、State of Playで新作『Rayman』を発表。Tencent出資の専門子会社(Vantage)による主要IP切り出しが進行。</t>
         </is>
       </c>
       <c r="M5" s="9" t="inlineStr">
@@ -22833,7 +22871,7 @@
       </c>
       <c r="P5" s="9" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -22867,7 +22905,7 @@
       </c>
       <c r="L6" s="9" t="inlineStr">
         <is>
-          <t>6月初の株価はHK$453前後(-1.26%)。5/13発表のQ1はEPS HK$8.51で予想超え、FY25売上CN¥751.8bn(+14%)・純益CN¥224.8bn(+16%)。WeChat向けAIエージェントを内部テスト中。ゲームはGDC 2026で20超セッション出展。次回決算は8/19。</t>
+          <t>6/16に総額$2.45bn＋人民元150億の社債発行を完了。ゲームとAI需要が業績を押し上げとの観測。NexonをめぐりNexon Games株が買収観測で急騰したが、Tencentは買収報道を改めて否定。Honor of Kings/PUBG Mobile等の海外展開とAI投資が継続テーマ。</t>
         </is>
       </c>
       <c r="M6" s="9" t="inlineStr">
@@ -22887,7 +22925,7 @@
       </c>
       <c r="P6" s="9" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -22921,7 +22959,7 @@
       </c>
       <c r="L7" s="9" t="inlineStr">
         <is>
-          <t>6/1株価$122.43。Q1'26は売上RMB30.59bn(+6%)でEPS RMB17.46と予想超えも、販管費増で一時下落。粗利率は69.4%へ改善。新作『Sea of Elements』『Ananta(都市型オープンワールド)』を2026年内投入予定。アナリストはStrong Buy・平均目標$162。</t>
+          <t>『Marvel Rivals』が6/18にVer.20260618(シーズン8.5)を配信、新ソーシャルマップ『Hellfire Bay Beach』や夏イベントを追加。同IPはeスポーツ(MRC S8)も本格化。AI部門縮小報道は『事実無根』と否定。Marvel Rivals/Identity V等のグローバルIP運営が成長軸。</t>
         </is>
       </c>
       <c r="M7" s="9" t="inlineStr">
@@ -22941,7 +22979,7 @@
       </c>
       <c r="P7" s="9" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -22975,7 +23013,7 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>6/5株価約$167.9・時価総額$7.57bn。『Subnautica 2』が5/14アーリーアクセスで1週間400万本・粗収益$120M。好調の一方、Unknown Worlds旧株主への最大$250Mのアーンアウト支払い義務が発生し、関連訴訟でも開発陣復職とボーナス支払いを命じる判決。</t>
+          <t>『AIファースト』への転換を鮮明にし、Subnautica 2やPalworld Mobileを含む26プロジェクト/2年で12本のパイプラインを提示。主要証券は概ね買い継続で平均目標株価は約₩388,731(上値余地6割超との見方)。PUBGの収益基盤と新規IP/AI活用が評価軸。</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
@@ -22995,7 +23033,7 @@
       </c>
       <c r="P8" s="9" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -23029,7 +23067,7 @@
       </c>
       <c r="L9" s="9" t="inlineStr">
         <is>
-          <t>株価約2,250円(+2.0%)。MapleStoryフランチャイズの成長と新作『ARC Raiders』(Embark)の貢献で直近四半期は好調。年間配当を1株60円(前期45円)へ増配。6月に株主総会。中国Dungeon&amp;Fighterモバイル等のライブ運営が収益の柱。</t>
+          <t>TencentによるNexon買収観測(評価額約$15b)が報じられNexon Games株が急騰したが、Tencentは買収を否定。『メイプルストーリー』『DNF(地下城与勇士)』等の中韓モバイル収益が堅調。Tencent動向と既存IPのライブ運営・新作が注目。</t>
         </is>
       </c>
       <c r="M9" s="9" t="inlineStr">
@@ -23049,7 +23087,7 @@
       </c>
       <c r="P9" s="9" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -23083,7 +23121,7 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>FY26は売上kr16.6bn(-26%)・純損失kr6.89bnと低迷。Coffee Stainグループを12/11にスピンオフ、残存本体を『Fellowship Entertainment』へ改称し2026年4月に分離・別上場。新CEOを公募中で、モバイル/PC・console/フィジカル流通等に集中し利益重視へ。</t>
+          <t>二次パブリッシングレーベル『Fellowship Entertainment』設立を発表、LotR/Tomb Raider等の主要IPを束ね2027年にスピンオフ予定。Ubisoftの『Vantage』分社に続く動きで『IP主導のエンタメ企業』への転換を志向。グループ再編とIP価値最大化が継続テーマ。</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
@@ -23103,7 +23141,7 @@
       </c>
       <c r="P10" s="9" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -23137,7 +23175,7 @@
       </c>
       <c r="L11" s="9" t="inlineStr">
         <is>
-          <t>6/12終値$43.31、年初来約-47%と低迷も、6/9にロシア政府機関が同プラットフォームの利用制限解除を検討との報道で株価が反発。5〜15歳向けの年齢別アカウントや児童安全機能を6月に展開し、$30億の自社株買いも実施。Q1売上は約$1.4bn（+39%）だが、安全対応がユーザー成長の短期摩擦に。年齢別アカウント定着と通期ブッキング回復が鍵。</t>
+          <t>6/18時点でエンゲージメントが3週連続で改善。『Roblox Kids』『Roblox Select』アカウントを世界展開し、年齢別の安全設計と保護者向け機能を強化。広告・クリエイター経済の拡大とAppLovin/Unityとの競合が注目点。</t>
         </is>
       </c>
       <c r="M11" s="9" t="inlineStr">
@@ -23157,7 +23195,7 @@
       </c>
       <c r="P11" s="9" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -23191,7 +23229,7 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>6/5にEdgewater ResearchがモバイルメディアのUnity・AppLovinをともにOutperformへ格上げし、広告課金型への業界シフトを評価。これを受けUnity株は約+5%。5月に開発ワークフローへ統合する『Unity AI』が公開ベータ入りし、コーディングやアセット生成の自動化で生産性向上を訴求。広告事業の回復とAI機能の収益化が当面の焦点。</t>
+          <t>ゲーム/広告/AIクリエイターツールの融合領域でAppLovin・Roblox・Adobeに対する競争ポジションを強化。広告事業(Unity Vector/Grow)の改善とエンジン課金モデルの安定化が株価回復の鍵。</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
@@ -23211,7 +23249,7 @@
       </c>
       <c r="P12" s="9" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>
@@ -23249,7 +23287,7 @@
       </c>
       <c r="L13" s="9" t="inlineStr">
         <is>
-          <t>自社運用型AI広告基盤『AXON』を6月に全世界の広告主へ開放し、14年続いたクローズド運用に区切り。6/5のEdgewater格上げで株価は約+3%。Q1'26は売上$1.84bn（+59%）・調整後EPS$3.56で予想超え、EBITDAマージン約85%。6/2にS&amp;P500入り。AXON全面開放はバイナリーイベントと目され、広告外領域への拡張も成長余地。目標株価$646。</t>
+          <t>AXON広告プラットフォームを6月に世界の広告主へ開放。株価は$468前後(6/21)で4月高値$745から約3割安だが、広告売上は2026年に$3bnへ倍増見込み、EBITDAマージン80%超・FCFガイダンス$12.5bn。eコマース広告の立ち上がりとマージン維持が焦点。</t>
         </is>
       </c>
       <c r="M13" s="9" t="inlineStr">
@@ -23269,7 +23307,7 @@
       </c>
       <c r="P13" s="9" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
daily-news + cross-questions + events update (2026-06-23)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -2747,7 +2747,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:G43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4310,6 +4310,43 @@
       <c r="G42" s="15" t="inlineStr">
         <is>
           <t>ゲームエンジンは『現実の安価な実験場』。エンタメ技術が産業の基盤技術へ昇格する“両用化”の典型例として追う価値あり。</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B43" s="15" t="inlineStr">
+        <is>
+          <t>ゲーム/SNSで義務化が進む『年齢確認（age assurance）』の技術・コスト負担は、動画配信・成人向けEC・酒類/ギャンブル・金融などのオンラインサービスでも共通インフラ化するか？</t>
+        </is>
+      </c>
+      <c r="C43" s="15" t="inlineStr">
+        <is>
+          <t>英政府が16歳未満のオンライン利用制限措置を公表（英・豪、JETRO 2026/6）</t>
+        </is>
+      </c>
+      <c r="D43" s="15" t="inlineStr">
+        <is>
+          <t>Microsoft/Xbox, Discord</t>
+        </is>
+      </c>
+      <c r="E43" s="15" t="inlineStr">
+        <is>
+          <t>動画配信(年齢確認)/EC(酒類・成人向け)/金融(KYC・本人確認)/ギャンブル</t>
+        </is>
+      </c>
+      <c r="F43" s="15" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="G43" s="15" t="inlineStr">
+        <is>
+          <t>規制対応の『年齢確認』が、各社個別実装から業界横断の共通APIレイヤー（金融のKYCに類似）として産業化する可能性。コスト負担とプライバシーの両立が論点。</t>
         </is>
       </c>
     </row>
@@ -6581,12 +6618,12 @@
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
-          <t>開催中</t>
+          <t>終了</t>
         </is>
       </c>
       <c r="J13" s="15" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-23</t>
         </is>
       </c>
     </row>
@@ -6893,7 +6930,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L189"/>
+  <dimension ref="A1:L194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18682,6 +18719,311 @@
       <c r="L189" s="5" t="inlineStr">
         <is>
           <t>開催日程は太平洋時間基準(JSTでは前後する)</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B190" s="5" t="inlineStr">
+        <is>
+          <t>Ubisoft、米サンフランシスコ拠点で93人を削減——WARN通知で確定、北米再編が継続</t>
+        </is>
+      </c>
+      <c r="C190" s="5" t="inlineStr">
+        <is>
+          <t>https://www.gamedeveloper.com/business/ubisoft-eliminates-93-roles-in-san-francisco</t>
+        </is>
+      </c>
+      <c r="D190" s="5" t="inlineStr">
+        <is>
+          <t>Ubisoftは大型タイトルの不振と財務悪化を受け、Tencent出資の新子会社設立など構造改革を進行中。北米のパブリッシング/サポート機能を縮小し、開発資源を主力フランチャイズへ集約する動きが続いている。</t>
+        </is>
+      </c>
+      <c r="E190" s="5" t="inlineStr">
+        <is>
+          <t>Ubisoftが米サンフランシスコ事業所で93人を削減することがWARN通知で判明。同社は6月初旬から50〜100人規模の削減を示唆しており、今回その規模が公式に確定した。北米のコスト構造見直しの一環。</t>
+        </is>
+      </c>
+      <c r="F190" s="5" t="inlineStr">
+        <is>
+          <t>・WARN通知で93人削減が確定
+・6月から予告されていた削減の具体化
+・北米パブリッシング機能の縮小傾向
+・Tencent出資の新体制下でのコスト最適化</t>
+        </is>
+      </c>
+      <c r="G190" s="5" t="inlineStr">
+        <is>
+          <t>増収局面でも赤字体質の是正を優先する欧米大手のレイオフは当面続く見込み。Ubisoftは黒字化に向け人員・スタジオの整理を進め、開発リソースを少数の主力IPへ集中させる可能性が高い。</t>
+        </is>
+      </c>
+      <c r="H190" s="5" t="inlineStr">
+        <is>
+          <t>欧米パブリッシャーの構造改革とコスト最適化</t>
+        </is>
+      </c>
+      <c r="I190" s="5" t="inlineStr">
+        <is>
+          <t>Ubisoft, Tencent</t>
+        </is>
+      </c>
+      <c r="J190" s="5" t="inlineStr">
+        <is>
+          <t>Assassin's Creed, Far Cry</t>
+        </is>
+      </c>
+      <c r="K190" s="5" t="inlineStr">
+        <is>
+          <t>業績,海外</t>
+        </is>
+      </c>
+      <c r="L190" s="5" t="n"/>
+    </row>
+    <row r="191">
+      <c r="A191" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B191" s="5" t="inlineStr">
+        <is>
+          <t>CEDEC2026基調講演に吉田修平氏・登大遊氏が登壇決定——テーマは『Co-Create（共創）』</t>
+        </is>
+      </c>
+      <c r="C191" s="5" t="inlineStr">
+        <is>
+          <t>https://news.denfaminicogamer.jp/news/260622n</t>
+        </is>
+      </c>
+      <c r="D191" s="5" t="inlineStr">
+        <is>
+          <t>CEDECはCESA主催の国内最大級のゲーム開発者会議。AIによる開発変革や人材流動が進む中、業界横断・産学官の連携を促す『共創』が今年のキーワードに据えられた。</t>
+        </is>
+      </c>
+      <c r="E191" s="5" t="inlineStr">
+        <is>
+          <t>7/22〜24開催のCEDEC2026の基調講演者が発表され、元SIEの吉田修平氏（7/22）とIPAの登大遊氏（7/24）が登壇。今年のテーマキーワードは『Co-Create』で、産学官の技術連携や共創の在り方が中心テーマとなる。</t>
+        </is>
+      </c>
+      <c r="F191" s="5" t="inlineStr">
+        <is>
+          <t>・基調講演に吉田修平氏・登大遊氏
+・テーマキーワードは『Co-Create（共創）』
+・会場はパシフィコ横浜ノース＋オンラインのハイブリッド
+・7/22〜24の3日間開催</t>
+        </is>
+      </c>
+      <c r="G191" s="5" t="inlineStr">
+        <is>
+          <t>AI活用や開発効率化が論点の中心になる見込みで、生成AIの実務適用や産学官連携の事例共有が注目される。国内開発者の関心テーマ（AI・人材・共創）を映す内容になりそう。</t>
+        </is>
+      </c>
+      <c r="H191" s="5" t="inlineStr">
+        <is>
+          <t>ゲーム開発の産学官連携と『共創』モデル</t>
+        </is>
+      </c>
+      <c r="I191" s="5" t="inlineStr">
+        <is>
+          <t>CESA, yosp, 情報処理推進機構(IPA)</t>
+        </is>
+      </c>
+      <c r="J191" s="5" t="inlineStr">
+        <is>
+          <t>CEDEC2026</t>
+        </is>
+      </c>
+      <c r="K191" s="5" t="inlineStr">
+        <is>
+          <t>技術,国内</t>
+        </is>
+      </c>
+      <c r="L191" s="5" t="n"/>
+    </row>
+    <row r="192">
+      <c r="A192" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B192" s="5" t="inlineStr">
+        <is>
+          <t>コーエーテクモ『BLUE REFLECTION Quartet』デジタル版プレオーダー開始、7/30発売</t>
+        </is>
+      </c>
+      <c r="C192" s="5" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/990/G099078/20260622033/</t>
+        </is>
+      </c>
+      <c r="D192" s="5" t="inlineStr">
+        <is>
+          <t>『ブルリフ』はガストの美少女RPGシリーズ。コンソール作・アニメ・モバイル/PC作の4作品を1本に集約する集大成タイトルとして、シリーズ資産の再パッケージ販売を狙う。</t>
+        </is>
+      </c>
+      <c r="E192" s="5" t="inlineStr">
+        <is>
+          <t>コーエーテクモが『BLUE REFLECTION Quartet: 少女たちのキセキ』のデジタル版プレオーダーを6/22開始し、PV第2弾も公開。7/30発売で、PC/PS5/Switch/Switch2に対応し、シリーズ4作品を1本に収録する。</t>
+        </is>
+      </c>
+      <c r="F192" s="5" t="inlineStr">
+        <is>
+          <t>・デジタル版プレオーダー6/22開始＋PV第2弾公開
+・7/30発売、4プラットフォーム対応
+・シリーズ4作品を1本に集約
+・通常版7,480円〜特別版24,200円</t>
+        </is>
+      </c>
+      <c r="G192" s="5" t="inlineStr">
+        <is>
+          <t>新規IPが当たりにくい環境下、既存IPの再編集・集約パッケージは堅実な収益策として広がる見込み。Switch2対応で携帯需要も取り込み、シリーズファン中心に底堅い販売が想定される。</t>
+        </is>
+      </c>
+      <c r="H192" s="5" t="inlineStr">
+        <is>
+          <t>既存IPの集約・再パッケージ戦略</t>
+        </is>
+      </c>
+      <c r="I192" s="5" t="inlineStr">
+        <is>
+          <t>コーエーテクモゲームス, ガスト</t>
+        </is>
+      </c>
+      <c r="J192" s="5" t="inlineStr">
+        <is>
+          <t>BLUE REFLECTION（ブルーリフレクション）</t>
+        </is>
+      </c>
+      <c r="K192" s="5" t="inlineStr">
+        <is>
+          <t>新作,国内</t>
+        </is>
+      </c>
+      <c r="L192" s="5" t="n"/>
+    </row>
+    <row r="193">
+      <c r="A193" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B193" s="5" t="inlineStr">
+        <is>
+          <t>英政府、16歳未満のオンライン利用制限措置を公表——豪のSNS禁止法に続く年齢規制の波</t>
+        </is>
+      </c>
+      <c r="C193" s="5" t="inlineStr">
+        <is>
+          <t>https://www.jetro.go.jp/biznews/2026/06/d5c80f9d0d7e87d8.html</t>
+        </is>
+      </c>
+      <c r="D193" s="5" t="inlineStr">
+        <is>
+          <t>英国はオンライン安全法(OSA)の実施を進め、豪は2025年末に16歳未満のSNS禁止法を施行済み。未成年保護を名目に、ゲームを含むオンラインサービスへ年齢確認義務が拡大している。</t>
+        </is>
+      </c>
+      <c r="E193" s="5" t="inlineStr">
+        <is>
+          <t>英政府が16歳未満ユーザーについて、ゲームサイト等を含むオンラインサービスでのライブ配信や身元不明者からの連絡機能の利用を制限する措置を公表。先行する豪のSNS禁止法と合わせ、年齢確認の実装圧力が強まる。</t>
+        </is>
+      </c>
+      <c r="F193" s="5" t="inlineStr">
+        <is>
+          <t>・英政府が16歳未満の利用制限措置を公表
+・対象にゲームサイト等のオンラインサービスを含む
+・豪は16歳未満SNS禁止法を施行済み（約470万アカウント削除）
+・OSA違反は最大で全世界売上10％の罰金</t>
+        </is>
+      </c>
+      <c r="G193" s="5" t="inlineStr">
+        <is>
+          <t>年齢確認（age assurance）の実装が事実上の必須要件となり、対応コストや本人確認基盤の整備が各社に求められる。プラットフォーム横断の年齢確認インフラ整備が加速する見込み。</t>
+        </is>
+      </c>
+      <c r="H193" s="5" t="inlineStr">
+        <is>
+          <t>オンライン安全規制と年齢確認(age assurance)の実装</t>
+        </is>
+      </c>
+      <c r="I193" s="5" t="inlineStr">
+        <is>
+          <t>Microsoft/Xbox, Discord</t>
+        </is>
+      </c>
+      <c r="J193" s="5" t="n"/>
+      <c r="K193" s="5" t="inlineStr">
+        <is>
+          <t>規制,海外</t>
+        </is>
+      </c>
+      <c r="L193" s="5" t="n"/>
+    </row>
+    <row r="194">
+      <c r="A194" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B194" s="5" t="inlineStr">
+        <is>
+          <t>今週の主要リリース——『Frostpunk 2』拡張やDMC5 Switch2版など週末に集中</t>
+        </is>
+      </c>
+      <c r="C194" s="5" t="inlineStr">
+        <is>
+          <t>https://www.dlcompare.com/gaming-news/this-week-s-video-game-releases-june-2026-week-26</t>
+        </is>
+      </c>
+      <c r="D194" s="5" t="inlineStr">
+        <is>
+          <t>Steamサマーセール(6/25開幕)前の週は、セール需要と新作の話題が重なるタイミング。各社は週末リリースを集中させ、夏商戦の立ち上がりを狙う。</t>
+        </is>
+      </c>
+      <c r="E194" s="5" t="inlineStr">
+        <is>
+          <t>6/23週はリリースが集中。23日に『Frostpunk 2: Breach of Trust』拡張や『Devil May Cry 5』Switch2版、24日に『DEAD OR ALIVE 6 Last Round』、25日に『スターフォックス』新作が控える。</t>
+        </is>
+      </c>
+      <c r="F194" s="5" t="inlineStr">
+        <is>
+          <t>・6/23『Frostpunk 2』新拡張、DMC5 Switch2版
+・6/24『DEAD OR ALIVE 6 Last Round』
+・6/25 スターフォックス新作
+・Steamサマーセール6/25開幕と重なる週</t>
+        </is>
+      </c>
+      <c r="G194" s="5" t="inlineStr">
+        <is>
+          <t>サマーセール開幕と新作集中が重なり、PCを中心に消費が活性化する見込み。Switch2版の旧作移植が継続的な販路として機能し、旧IPの再収益化が進む。</t>
+        </is>
+      </c>
+      <c r="H194" s="5" t="inlineStr">
+        <is>
+          <t>夏商戦のリリース集中とセール暦の関係</t>
+        </is>
+      </c>
+      <c r="I194" s="5" t="inlineStr">
+        <is>
+          <t>カプコン, コーエーテクモ, 任天堂, 11 bit studios</t>
+        </is>
+      </c>
+      <c r="J194" s="5" t="inlineStr">
+        <is>
+          <t>Devil May Cry, DEAD OR ALIVE, Star Fox, Frostpunk</t>
+        </is>
+      </c>
+      <c r="K194" s="5" t="inlineStr">
+        <is>
+          <t>新作,海外,国内</t>
+        </is>
+      </c>
+      <c r="L194" s="5" t="inlineStr">
+        <is>
+          <t>発売日は地域により前後する場合あり</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
daily-news + cross-questions + events update (2026-06-23 22:10)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -2747,7 +2747,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4347,6 +4347,80 @@
       <c r="G43" s="15" t="inlineStr">
         <is>
           <t>規制対応の『年齢確認』が、各社個別実装から業界横断の共通APIレイヤー（金融のKYCに類似）として産業化する可能性。コスト負担とプライバシーの両立が論点。</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B44" s="14" t="inlineStr">
+        <is>
+          <t>巨額M&amp;A（Activision Blizzard買収）後にシナジーが出ず、祖業の大規模リストラ・事業縮小へ転じる『高すぎた買収の後始末』は、ロールアップ型M&amp;Aを進める他業界（メディア・製薬・半導体）でも同様に起きるか？</t>
+        </is>
+      </c>
+      <c r="C44" s="14" t="inlineStr">
+        <is>
+          <t>Xbox『リセット』と7月の大規模レイオフ計画報道</t>
+        </is>
+      </c>
+      <c r="D44" s="14" t="inlineStr">
+        <is>
+          <t>Microsoft/Xbox, Activision Blizzard</t>
+        </is>
+      </c>
+      <c r="E44" s="14" t="inlineStr">
+        <is>
+          <t>メディア（大型統合後のリストラ）, 製薬（買収パイプラインの減損）, 半導体（統合シナジー未達）</t>
+        </is>
+      </c>
+      <c r="F44" s="14" t="inlineStr">
+        <is>
+          <t>オープン</t>
+        </is>
+      </c>
+      <c r="G44" s="14" t="inlineStr">
+        <is>
+          <t>巨額買収→数年後に減損・人員削減という流れはゲーム特有ではなく、買収プレミアムの回収難という普遍的論点。買収後3-5年の統合KPIに着目すると他業界の予兆も読める。</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B45" s="14" t="inlineStr">
+        <is>
+          <t>ソフト流通プラットフォーマー（Valve）が自社ハードへ垂直統合し『箱』を握り直す動きは、動画配信・EC・決済など他のプラットフォーム業界の囲い込み戦略の何に該当するか？</t>
+        </is>
+      </c>
+      <c r="C45" s="14" t="inlineStr">
+        <is>
+          <t>Steam Machine 日本・台湾・香港で発売開始</t>
+        </is>
+      </c>
+      <c r="D45" s="14" t="inlineStr">
+        <is>
+          <t>Valve, KOMODO</t>
+        </is>
+      </c>
+      <c r="E45" s="14" t="inlineStr">
+        <is>
+          <t>動画配信（Apple TV/Amazon Fire等の自社デバイス）, EC（Amazonの物流・端末統合）, 決済（クローズドループ経済圏）</t>
+        </is>
+      </c>
+      <c r="F45" s="14" t="inlineStr">
+        <is>
+          <t>オープン</t>
+        </is>
+      </c>
+      <c r="G45" s="14" t="inlineStr">
+        <is>
+          <t>流通を握る側がハード（顧客接点）まで垂直統合する点は、配信・ECの自社デバイス戦略と相似。OS・ストア・決済を自社で閉じる経済圏設計が共通テーマ。</t>
         </is>
       </c>
     </row>
@@ -6930,7 +7004,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L194"/>
+  <dimension ref="A1:L201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19026,6 +19100,424 @@
           <t>発売日は地域により前後する場合あり</t>
         </is>
       </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B195" s="14" t="inlineStr">
+        <is>
+          <t>Valve「Steam Machine」日本・台湾・香港で販売開始——512GB18万9980円</t>
+        </is>
+      </c>
+      <c r="C195" s="14" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/999/G999902/20260622053/</t>
+        </is>
+      </c>
+      <c r="D195" s="14" t="inlineStr">
+        <is>
+          <t>ValveはPCゲームプラットフォームSteamを核に、携帯機Steam Deckで据置PC市場の一角を築いてきた。今回はリビング設置を想定した小型据置機「Steam Machine」を投入。日本では代理店KOMODOのKOMODO STATION経由で6月23日に発売され、SteamOSを採用したコンソール的な体験を打ち出す。</t>
+        </is>
+      </c>
+      <c r="E195" s="14" t="inlineStr">
+        <is>
+          <t>6月23日、SteamOS搭載の小型ゲーミングPC「Steam Machine」が日本・台湾・香港で販売開始。512GBモデルが18万9980円、2TBモデルが24万9980円で、専用Steam Controllerとのセットは1.5万円増し。発売直後からアクセスが集中し順番待ちとなった。Steam Deckの6倍超の性能をうたう。</t>
+        </is>
+      </c>
+      <c r="F195" s="14" t="inlineStr">
+        <is>
+          <t>SteamOS搭載の据置型小型PCで、テレビ・大型モニター接続を前提
+日本価格は512GB18万9980円／2TB24万9980円、Controllerセットは+1.5万円
+日本・台湾・香港は代理店KOMODO経由の小売販売、韓国は対象外
+Forza Horizon 6でレイトレを動かせるなどSteam Deck比6倍超の性能訴求
+発売直後に注文殺到で順番待ち状態</t>
+        </is>
+      </c>
+      <c r="G195" s="14" t="inlineStr">
+        <is>
+          <t>PlayStation/Xboxが据置の世代交代と値上げに直面する中、Valveは『箱』を握り直しSteamエコシステムの垂直統合を強める。SteamOSの最適化とサードのSteam移行が進めば、リビング市場でのPC陣営の存在感が増す。価格は高めで普及ペースは限定的だが、Steam Deckに続く第二の自社ハードとして長期的な布石となる。</t>
+        </is>
+      </c>
+      <c r="H195" s="14" t="inlineStr">
+        <is>
+          <t>プラットフォーマーの垂直統合とSteamOSエコシステム戦略</t>
+        </is>
+      </c>
+      <c r="I195" s="14" t="inlineStr">
+        <is>
+          <t>Valve, KOMODO</t>
+        </is>
+      </c>
+      <c r="J195" s="14" t="inlineStr">
+        <is>
+          <t>Steam Machine, SteamOS, Steam Deck, Forza Horizon 6</t>
+        </is>
+      </c>
+      <c r="K195" s="14" t="inlineStr">
+        <is>
+          <t>技術,新作,海外</t>
+        </is>
+      </c>
+      <c r="L195" s="14" t="inlineStr"/>
+    </row>
+    <row r="196">
+      <c r="A196" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B196" s="14" t="inlineStr">
+        <is>
+          <t>バンダイナムコ『ドラゴンボール ゼノバース3』第1弾PV公開——2027年発売、新システム“ソウルチェンジ”</t>
+        </is>
+      </c>
+      <c r="C196" s="14" t="inlineStr">
+        <is>
+          <t>https://news.denfaminicogamer.jp/news/260624b</t>
+        </is>
+      </c>
+      <c r="D196" s="14" t="inlineStr">
+        <is>
+          <t>『ドラゴンボール ゼノバース』はオンライン要素を備えたアクションRPGシリーズで、累計実績を持つバンナムの主力IP。2026年4月に『3』が2027年発売（PS5/Xbox Series/Steam）と発表されていた。今回ゲームプレイを初解禁する第1弾PVが公開され、開発の方向性が具体的に見えてきた。</t>
+        </is>
+      </c>
+      <c r="E196" s="14" t="inlineStr">
+        <is>
+          <t>バンダイナムコは『ドラゴンボール ゼノバース3』のゲームプレイ初解禁となる第1弾PVを公開。主人公が所属する『GS戦隊（グレートサイヤ戦隊）』や、舞台となる未来の“西の都”の大学で出会う仲間、歴戦の戦士の力を宿して戦う新バトル『ソウルチェンジ』のシーンを披露した。発売は2027年予定。</t>
+        </is>
+      </c>
+      <c r="F196" s="14" t="inlineStr">
+        <is>
+          <t>シリーズ最新作『ゼノバース3』の実機映像を初公開
+新バトルアクション『ソウルチェンジ』を搭載
+舞台は鳥山明氏が描く未来の“西の都”、新組織『GS戦隊』が登場
+プラットフォームはPS5/Xbox Series X|S/Steam、2027年発売予定
+海外イベント試遊ROMの先行プレイレポートも公開</t>
+        </is>
+      </c>
+      <c r="G196" s="14" t="inlineStr">
+        <is>
+          <t>発売は2027年と先だが、大型IPの早期PV解禁はTGS2026や年末商戦に向けた長期プロモーションの起点。オンライン対戦とキャラクリエイトを核とする本シリーズはライブサービス的な長期運用が見込まれ、バンナムのIP横展開（アニメ・カードと連動）と合わせ、安定収益源としての位置づけが強まる。</t>
+        </is>
+      </c>
+      <c r="H196" s="14" t="inlineStr">
+        <is>
+          <t>大型IPの長期プロモーション設計とライブサービス運用</t>
+        </is>
+      </c>
+      <c r="I196" s="14" t="inlineStr">
+        <is>
+          <t>バンダイナムコエンターテインメント</t>
+        </is>
+      </c>
+      <c r="J196" s="14" t="inlineStr">
+        <is>
+          <t>ドラゴンボール ゼノバース3</t>
+        </is>
+      </c>
+      <c r="K196" s="14" t="inlineStr">
+        <is>
+          <t>新作,国内</t>
+        </is>
+      </c>
+      <c r="L196" s="14" t="inlineStr"/>
+    </row>
+    <row r="197">
+      <c r="A197" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B197" s="14" t="inlineStr">
+        <is>
+          <t>『SAW: Genesis』ゲームプレイトレーラー公開——3対1非対称ホラー、7月上旬アルファ</t>
+        </is>
+      </c>
+      <c r="C197" s="14" t="inlineStr">
+        <is>
+          <t>https://news.denfaminicogamer.jp/news/260623x</t>
+        </is>
+      </c>
+      <c r="D197" s="14" t="inlineStr">
+        <is>
+          <t>映画『ソウ』を題材にした3対1の非対称対戦ホラー『SAW: Genesis』は、6月のSummer Game Fest 2026で発表。開発はBroken Mirror GamesとAnshar Studios、販売をBloober Teamが担当する。ジグソウ登場の100年前を舞台に、『殺人鬼が負けうる』設計を掲げる意欲作で、今回ゲームプレイ映像が公開された。</t>
+        </is>
+      </c>
+      <c r="E197" s="14" t="inlineStr">
+        <is>
+          <t>Bloober Teamは非対称対戦ホラー『SAW: Genesis』のゲームプレイトレーラーを公開。3人の『被告人』がトラップだらけのマップから脱出を図り、1人の『ジャッジ』が管理者として妨害する3v1構造を紹介。舞台は第一次大戦後の1920年代ロンドン。7月上旬にアルファテストを予定し、年内Q4にSteamアーリーアクセスを目指す。</t>
+        </is>
+      </c>
+      <c r="F197" s="14" t="inlineStr">
+        <is>
+          <t>映画『ソウ』原作の3対1非対称マルチプレイホラー
+『殺人鬼（ジャッジ）が負けうる』非対称設計が特徴
+7月上旬にアルファテストを実施予定
+Steamで買い切り型アーリーアクセス（2026年Q4目標）
+Bloober Teamが販売、開発はBroken Mirror／Anshar</t>
+        </is>
+      </c>
+      <c r="G197" s="14" t="inlineStr">
+        <is>
+          <t>Dead by Daylight以降定着した非対称対戦ジャンルに、強IPと『鬼側も負ける』バランス設計で挑む。ライセンスホラーの対戦化は配信映えと相性が良く、アルファの反応次第でローンチ規模が決まる。Bloober Teamにとっては自社ホラー（サイレントヒル等）に続く販売事業の多角化テストケースとなる。</t>
+        </is>
+      </c>
+      <c r="H197" s="14" t="inlineStr">
+        <is>
+          <t>非対称対戦ホラー市場とライセンスIPの対戦ゲーム化</t>
+        </is>
+      </c>
+      <c r="I197" s="14" t="inlineStr">
+        <is>
+          <t>Bloober Team, Broken Mirror Games, Anshar Studios, Lionsgate</t>
+        </is>
+      </c>
+      <c r="J197" s="14" t="inlineStr">
+        <is>
+          <t>SAW: Genesis</t>
+        </is>
+      </c>
+      <c r="K197" s="14" t="inlineStr">
+        <is>
+          <t>新作,海外</t>
+        </is>
+      </c>
+      <c r="L197" s="14" t="inlineStr"/>
+    </row>
+    <row r="198">
+      <c r="A198" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B198" s="14" t="inlineStr">
+        <is>
+          <t>Xbox、新CEOサルマ氏の下で“リセット”——7月に大規模レイオフ計画と報道</t>
+        </is>
+      </c>
+      <c r="C198" s="14" t="inlineStr">
+        <is>
+          <t>https://www.videogameschronicle.com/news/xbox-is-reportedly-planning-major-layoffs-as-sharma-tells-staff-we-need-to-reassess-our-priorities/</t>
+        </is>
+      </c>
+      <c r="D198" s="14" t="inlineStr">
+        <is>
+          <t>MicrosoftはActivision Blizzardを687億ドルで買収しゲーム事業を拡大したが、コンテンツ・ハード補助に巨額を投じる一方で収益が伸び悩む。新CEOアシャ・サルマ氏は『この状況は続けられない』として100日間の戦略見直し『Xbox Reset』を表明。会計年度末（6月30日）後にレイオフが見込まれる。</t>
+        </is>
+      </c>
+      <c r="E198" s="14" t="inlineStr">
+        <is>
+          <t>Bloomberg等によると、Microsoftは6月30日の会計年度末直後、Xbox部門で7月に大規模なレイオフを計画。新CEOサルマ氏は優先順位の再評価を社員に通達し、マーケティング・運営の予算削減も伴うとされる。規模は約1000人との数字が一部で流れるが未確認。687億ドルのActivision買収後も売上は減少傾向にある。</t>
+        </is>
+      </c>
+      <c r="F198" s="14" t="inlineStr">
+        <is>
+          <t>新CEOアシャ・サルマ氏が100日の戦略見直し『Xbox Reset』を主導
+7月（会計年度末6/30直後）に大規模レイオフを計画と報道
+マーケ・運営の予算削減も並行、規模は約1000人との未確認情報
+687億ドルのActivision Blizzard買収後も収益は伸び悩み
+低価格コンソール層の検討など事業モデル再設計の動き</t>
+        </is>
+      </c>
+      <c r="G198" s="14" t="inlineStr">
+        <is>
+          <t>巨額買収後の統合シナジー不全とプラットフォーム戦略の転換</t>
+        </is>
+      </c>
+      <c r="H198" s="14" t="inlineStr">
+        <is>
+          <t>Microsoft, Xbox, Activision Blizzard</t>
+        </is>
+      </c>
+      <c r="I198" s="14" t="inlineStr">
+        <is>
+          <t>Xbox, Activision Blizzard</t>
+        </is>
+      </c>
+      <c r="J198" s="14" t="inlineStr">
+        <is>
+          <t>業績,海外,M&amp;A</t>
+        </is>
+      </c>
+      <c r="K198" s="14" t="inlineStr"/>
+      <c r="L198" s="14" t="n"/>
+    </row>
+    <row r="199">
+      <c r="A199" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B199" s="14" t="inlineStr">
+        <is>
+          <t>Nexon、投資子会社『Nexon Partners』設立——元Tencent幹部を起用し早期投資強化</t>
+        </is>
+      </c>
+      <c r="C199" s="14" t="inlineStr">
+        <is>
+          <t>https://en.sedaily.com/technology/2026/05/29/nexon-launches-investment-arm-hires-former-tencent-executive</t>
+        </is>
+      </c>
+      <c r="D199" s="14" t="inlineStr">
+        <is>
+          <t>日本上場・韓国発のNexonはDungeon&amp;Fighter等を持つ大手で、近年はTencentとの中国向けパブリッシング提携を10年延長するなど資本・事業連携を深める。ゲームスタジオへの早期投資を組織化するため、専門の投資子会社を新設し、元Tencent幹部を経営陣に迎えた。</t>
+        </is>
+      </c>
+      <c r="E199" s="14" t="inlineStr">
+        <is>
+          <t>Nexonは5月末、ゲームスタートアップ発掘を担う投資子会社『Nexon Partners』を設立。元Tencentの幹部を起用し、韓国を中心とするアーリーステージ投資を活性化する狙い。Tencentとの『Dungeon&amp;Fighter PC』中国パブリッシング提携10年延長と並び、外部スタジオとの資本連携を強める動きが続く。</t>
+        </is>
+      </c>
+      <c r="F199" s="14" t="inlineStr">
+        <is>
+          <t>ゲームスタートアップ投資の専門子会社『Nexon Partners』を新設
+元Tencent幹部を経営陣に起用
+韓国中心にアーリーステージ投資を活性化
+TencentとのDungeon&amp;Fighter PC中国提携を10年延長
+大手による外部スタジオ囲い込み・CVC化の流れ</t>
+        </is>
+      </c>
+      <c r="G199" s="14" t="inlineStr">
+        <is>
+          <t>大手ゲーム企業のCVC（コーポレートベンチャーキャピタル）戦略</t>
+        </is>
+      </c>
+      <c r="H199" s="14" t="inlineStr">
+        <is>
+          <t>Nexon, Tencent, Nexon Partners</t>
+        </is>
+      </c>
+      <c r="I199" s="14" t="inlineStr">
+        <is>
+          <t>Dungeon &amp; Fighter</t>
+        </is>
+      </c>
+      <c r="J199" s="14" t="inlineStr">
+        <is>
+          <t>M&amp;A,海外</t>
+        </is>
+      </c>
+      <c r="K199" s="14" t="inlineStr"/>
+      <c r="L199" s="14" t="n"/>
+    </row>
+    <row r="200">
+      <c r="A200" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B200" s="14" t="inlineStr">
+        <is>
+          <t>VALORANT Masters London 2026、Leviatánが初優勝——Paper Rexを3-2で撃破</t>
+        </is>
+      </c>
+      <c r="C200" s="14" t="inlineStr">
+        <is>
+          <t>https://www.gamereactor.eu/esports/1738043/VCT+Masters+London+2026+Leviathan+crowned+champion+after+overcoming+Paper+Rex/</t>
+        </is>
+      </c>
+      <c r="D200" s="14" t="inlineStr">
+        <is>
+          <t>VALORANT Masters LondonはVCT2026 Stage2の国際大会（6/12-21、ロンドン）。Pacific地域のPaper Rexが優勝候補筆頭とされる中、Americas地域のLeviatánが敗者復活から勝ち上がり、グランドファイナルで激突した。</t>
+        </is>
+      </c>
+      <c r="E200" s="14" t="inlineStr">
+        <is>
+          <t>VCT Masters London 2026のグランドファイナルで、Leviatánが Paper Rex をフルマップ（3-2）の末に下し組織初の国際タイトルを獲得。敗者復活から勝ち上がる快挙で、Americas勢として4度目のMasters制覇、Pacificの4大会連続優勝を止めた。MVPはNeon選手、優勝賞金は35万ドル。</t>
+        </is>
+      </c>
+      <c r="F200" s="14" t="inlineStr">
+        <is>
+          <t>LeviatánがPaper Rexを3-2で破り組織初の国際優勝
+敗者復活ブラケットからの逆転制覇
+Americas勢4度目のMasters、Pacific連覇を阻止
+優勝賞金35万ドル、準優勝20万ドル
+MVPはBruno『Neon』Rodríguez選手</t>
+        </is>
+      </c>
+      <c r="G200" s="14" t="inlineStr">
+        <is>
+          <t>地域リーグ制eスポーツの勢力図とフランチャイズ収益</t>
+        </is>
+      </c>
+      <c r="H200" s="14" t="inlineStr">
+        <is>
+          <t>Leviatán, Paper Rex, Riot Games</t>
+        </is>
+      </c>
+      <c r="I200" s="14" t="inlineStr">
+        <is>
+          <t>VALORANT, VCT Masters London 2026</t>
+        </is>
+      </c>
+      <c r="J200" s="14" t="inlineStr">
+        <is>
+          <t>eスポーツ,海外</t>
+        </is>
+      </c>
+      <c r="K200" s="14" t="inlineStr"/>
+      <c r="L200" s="14" t="n"/>
+    </row>
+    <row r="201">
+      <c r="A201" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B201" s="14" t="inlineStr">
+        <is>
+          <t>Steam Next Fest 6月版が過去最大規模で閉幕——5000本弱のデモ、6/25サマーセール開幕へ</t>
+        </is>
+      </c>
+      <c r="C201" s="14" t="inlineStr">
+        <is>
+          <t>https://www.techtimes.com/articles/318748/20260620/steam-next-fest-last-call-4931-free-demos-disappear-monday-before-summer-sale.htm</t>
+        </is>
+      </c>
+      <c r="D201" s="14" t="inlineStr">
+        <is>
+          <t>Steam Next Festは発売前タイトルの体験版を一斉公開しウィッシュリストを喚起する需要創出イベント。6月版（6/15-22）は過去最大規模で、直後の6月25日にはSteamサマーセール2026（〜7/9）が控える。デモからの送客が初週販売に効く構造が定着している。</t>
+        </is>
+      </c>
+      <c r="E201" s="14" t="inlineStr">
+        <is>
+          <t>Steam Next Fest（6月版、6/15-22）は約4931本のデモを集め、2020年の開始以来最大規模で閉幕。プレイ可能な体験版でウィッシュリスト追加を促し、6月25日10時(PT)開幕のサマーセール2026（〜7/9）へ送客する流れができている。インディー含む新作の発見と初週購入への転換が狙い。</t>
+        </is>
+      </c>
+      <c r="F201" s="14" t="inlineStr">
+        <is>
+          <t>6月版Next Festは約4931本のデモで過去最大規模
+体験版→ウィッシュリスト→初週購入の送客導線が定着
+Steamサマーセール2026は6/25 10時(PT)開幕、7/9まで
+インディー新作の発見機会として影響力増大
+Valveのストア主導型マーケティングの強化</t>
+        </is>
+      </c>
+      <c r="G201" s="14" t="inlineStr">
+        <is>
+          <t>デモ施策とウィッシュリストが初動販売に与える影響</t>
+        </is>
+      </c>
+      <c r="H201" s="14" t="inlineStr">
+        <is>
+          <t>Valve</t>
+        </is>
+      </c>
+      <c r="I201" s="14" t="inlineStr">
+        <is>
+          <t>Steam Next Fest, Steam Summer Sale 2026</t>
+        </is>
+      </c>
+      <c r="J201" s="14" t="inlineStr">
+        <is>
+          <t>海外</t>
+        </is>
+      </c>
+      <c r="K201" s="14" t="inlineStr"/>
+      <c r="L201" s="14" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
weekly-trends + tech update (2026-06-24 03:12)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -1193,7 +1193,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1979,6 +1979,154 @@
       <c r="G21" s="3" t="inlineStr">
         <is>
           <t>https://www.thegamer.com/steam-games-must-play-best-player-count-right-now/</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Krafton×Hanwha提携が示すゲーム技術の防衛・産業転用</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>6月21日、PUBG運営のKraftonが韓国の防衛・航空大手Hanwha Aerospaceと提携。ゲームで培ったリアルタイム3Dレンダリング、物理シミュレーション、強化学習エージェント、合成データ生成といった技術を、防衛訓練シミュレータや産業用デジタルツインへ応用する狙い。前後してGoogle Cloudが自律型AI開発エージェントを、NVIDIAがオンデバイスのAI NPC「ACE」を相次ぎ発表し、ゲームエンジン由来の技術が「遊び」の外側へ滲み出す流れが鮮明化した。Krafton側はゲーム収益で得たキャッシュと人材を、単価が高く成長余地の大きいB2B・国家インフラ領域へ再配分する成長戦略の一環と位置づける。</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Krafton, Hanwha Aerospace, NVIDIA, Google Cloud, Unreal Engine</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>ゲームエンジンは本来『リアルタイムで世界をシミュレートする汎用基盤』であり、自動運転・建築・防衛・映像制作と地続き。エンタメ産業で磨かれた技術がより単価の高いB2B/官公需要へ横展開する『デュアルユース（軍民両用）』は、半導体やドローンと同型の構造。ゲーム企業がIPホルダーから『シミュレーション技術企業』へと自己定義を広げる転換点にある。</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>エンタメ発の技術が防衛・産業へ流れる構図は、ゲーム＝周辺ではなく基盤技術であることを示す。映像・教育・都市計画など他業界も同じエンジンを採用する余地が大きい。</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>https://www.gamedeveloper.com/ (Krafton×Hanwha提携)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>開発者の生成AI利用率低下と『非AI』を売りにする差別化</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>GDC 2026のState of the Game Industry調査で、生成AIを『業界に悪影響』と答えた開発者が52%（前年30%・一昨年18%）に上昇し、実際の利用率は前年36%から29%へ低下した。6月19日にはパルワールドのポケットペアが『プレイヤーが望まない』として生成AIを使わない方針を改めて表明。過去にLarianやCrystal Dynamics、SegaがAIアセット利用で炎上した反動もあり、『AIを使わないこと』自体をブランド価値・真正性（オーセンティシティ）の証として打ち出す動きが広がる。一方でNVIDIAのオンデバイスNPCやGameByteのAIノーコード基盤など技術提供側は推進を続けており、制作現場と基盤層の温度差が拡大している。</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>ポケットペア(パルワールド), Larian, Crystal Dynamics, Sega, NVIDIA, GameByte</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>生成AIは『コスト削減ツール』として導入が想定されたが、ゲームでは購買者がアウトプットの真正性を重視するため、供給側の効率化動機と需要側の選好がねじれる。手仕事・人間性が希少価値となり『非AI』がプレミアム化する逆説が生じる。技術の有無ではなく『誰がどんな意図で作ったか』が価値の源泉になる、ラグジュアリーやクラフト食品と同型の市場構造。</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>効率化技術が必ずしも採用されない『真正性が効率に勝つ』市場の存在は、出版・音楽・工芸など創作産業全般に通じる。AI時代の差別化軸は『人間が作った証明』になりうる。</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>https://www.gianty.com/ (GDC2026調査), https://www.gamesradar.com/ (パルワールド)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Xboxの『リセット』：記録収益下の構造縮小とAIへの資本再配分</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>6月24日、Microsoftは新Xbox CEOサルマ体制の下で事業を『リセット』する方針を表明。6月11日のBloomberg報道では7月の会計年度明けにXbox部門で大規模レイオフが計画され、Ninja Theory閉鎖も通告された。背景にはActivision Blizzard買収（約7.5兆円）後の重い投資回収負担と、親会社MicrosoftがAI・データセンターへ資本を集中させる優先順位の変化がある。ゲーム部門は史上最高水準の収益を上げながら人員と独立スタジオを削減する『記録的売上×記録的レイオフ』の典型例。ショーケースから他社ロゴを外し独占回帰も示唆するなど、戦略の振り子が大きく揺れている。</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Microsoft, Xbox, Activision Blizzard, Ninja Theory, Halo Studios</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>巨大テック傘下のゲーム事業は、単体採算より『グループ全体の資本配分』で命運が決まる。AIという桁違いの投資対象が出現したことで、ゲームのキャッシュフローは祖業の再投資ではなくAI設備へ吸い上げられる。コングロマリット内の事業間資本移動（インターナル・キャピタル・マーケット）が、好調な事業すら縮小させる構造が露わになった。</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>親会社の戦略次第で黒字事業が縮む構図は、AIブーム下の全産業に共通。映像・広告・SaaSなど他のテック子事業も同じ資本再配分の圧力に晒される。</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>https://www.bloomberg.com/ (Xboxレイオフ), https://www.videogameschronicle.com/ (Xboxリセット)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>スマホ新法とage assurance波がモバイル課金経済を再編</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>日本の『スマホ新法（スマホソフトウェア競争促進法）』施行から半年が経ち、6月21日時点でiPhoneの外部アプリストア・外部課金が現実に稼働し始めた。Appleの約30%手数料を回避できる経路が開くことで、ガチャ・サブスク中心のモバイルゲーム収益構造に変化圧力がかかる。同時に英政府が16歳未満のオンライン利用制限を公表（6/23）、EU AI法の透明性ルールが8月2日に全面適用、PEGIが有料ランダムアイテムを年齢レーティングへ反映する新基準を運用開始するなど、流通・年齢確認・課金設計を同時に縛る規制が世界で多発。プラットフォーム手数料と未成年保護の両面からモバイル経済が組み替えられつつある。</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Apple, Google, 任天堂, PEGI, EU, 英政府</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>モバイルゲーム経済はこれまで『プラットフォーム手数料30%＋ガチャ課金＋ターゲティング広告』を前提に最適化されてきた。DMA型のストア開放はこの土台の手数料を、age assuranceは課金・広告のターゲット母数を、それぞれ削る。複数レイヤーの規制が同時進行することで、単一の対策では吸収しきれない複合的な構造転換が起きる。</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>手数料・年齢確認・データ利用の同時規制は、アプリ経済全般（音楽・動画・EC）に波及する論点。プラットフォーム依存度の高い事業ほど再設計を迫られる。</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>https://www.nikkei.com/ (スマホ新法半年), https://www.jetro.go.jp/ (英年齢制限)</t>
         </is>
       </c>
     </row>
@@ -24246,7 +24394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -24310,7 +24458,7 @@
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B2" s="9" t="inlineStr">
@@ -24325,32 +24473,32 @@
       </c>
       <c r="D2" s="9" t="inlineStr">
         <is>
-          <t>AI保護を巡る2024-25年のゲーム声優ストは新契約で妥結も、運用段階の摩擦が継続。LLM駆動NPC(Inworld/NVIDIA ACE)の実装拡大で『声・人格の継続利用』が現実問題に。</t>
+          <t>開発現場の利用率は前年36%→29%へ低下、52%が『悪影響』と回答。基盤層（NVIDIA・Google Cloud）は推進継続で温度差が拡大。</t>
         </is>
       </c>
       <c r="E2" s="9" t="inlineStr">
         <is>
-          <t>SAG-AFTRAがEpic子会社Llama Productionsを、団交・事前通知なくAIでダース・ベイダー音声を複製したとしてULP申立て。『gameslop』氾濫を背景に、人間制作/クレジット済み実演者の開示が信頼維持の前提に。</t>
+          <t>パルワールドが生成AI不使用を再表明／GameByteがAIノーコード基盤で資金調達／NVIDIAがオンデバイスNPC『ACE』発表／DLSS 5が生成AIで映像補完。</t>
         </is>
       </c>
       <c r="F2" s="9" t="inlineStr">
         <is>
-          <t>Epic Games, Llama Productions, SAG-AFTRA, Inworld AI, NVIDIA</t>
+          <t>ポケットペア, NVIDIA, Google Cloud, GameByte, Larian</t>
         </is>
       </c>
       <c r="G2" s="9" t="inlineStr">
         <is>
-          <t>ランタイム生成(声・人格)の常態化で、事前合意と出自開示が競争条件化。労務×IP×消費者保護が交差点に。</t>
+          <t>『非AI』を真正性として打ち出す差別化が定着。基盤技術は推進されるが、エンドコンテンツへの直接適用は炎上回避で慎重姿勢が続く。</t>
         </is>
       </c>
       <c r="H2" s="9" t="inlineStr">
         <is>
-          <t>開示は規制ではなく『信頼の通貨』として機能し始めた。裏方効率化と成果物で許容度が分岐。</t>
+          <t>効率化技術が需要側選好で抑制される逆説。AIの主戦場は『見えない裏方（最適化・QA・運用）』へ移る。</t>
         </is>
       </c>
       <c r="I2" s="9" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Artificial_intelligence_in_video_games</t>
+          <t>https://www.gianty.com/ GDC2026 / https://www.gamesradar.com/ パルワールド</t>
         </is>
       </c>
       <c r="J2" s="9" t="inlineStr"/>
@@ -24406,7 +24554,7 @@
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B4" s="9" t="inlineStr">
@@ -24421,32 +24569,32 @@
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>Game Pass Ultimate値下げ後の再編が継続。6月末でGame Passから8タイトルが離脱予定。</t>
+          <t>Game Pass値上げで『数百万人解約』をXbox幹部が示唆。価格の揺り戻し局面に入った。</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
         <is>
-          <t>Ubisoft+ ClassicsがPC Game Pass提供から外れる一方、Xbox Game Pass UltimateはEA Play/Ubisoft+ Classicsを内包。UbisoftはR6 SiegeでXbox Game Pass公式パートナー契約を更新し6月から特典付与。Ubisoft+はPremium/Classicsの2階層へ。</t>
+          <t>Game Pass Ultimate値上げ＋CoD day-one提供の見直し報道／Xbox『リセット』で事業全体を再設計。</t>
         </is>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
-          <t>Microsoft/Xbox, Ubisoft, Sony(PS Plus), EA</t>
+          <t>Microsoft, Xbox</t>
         </is>
       </c>
       <c r="G4" s="9" t="inlineStr">
         <is>
-          <t>バンドルの再編成（どのカタログがどのサブスクに入るか）が競争軸に。目玉IPの出し入れとクロスバンドルが常態化。</t>
+          <t>大幅値上げ→解約増→調整の循環。サブスクは『無制限提供』から『選別された価値提供』へモデル再考。</t>
         </is>
       </c>
       <c r="H4" s="9" t="inlineStr">
         <is>
-          <t>サブスクの価値は『独占タイトル』から『どれだけ他社カタログを束ねるか』のアグリゲーション競争へ。</t>
+          <t>コンテンツ詰め放題モデルの限界。価格弾力性が顕在化し、day-one投入の採算が問われる。</t>
         </is>
       </c>
       <c r="I4" s="9" t="inlineStr">
         <is>
-          <t>https://gg.deals/subscription-news/game-pass-is-losing-eight-games-at-the-end-of-june-2026 , https://www.thurrott.com/games/296198/</t>
+          <t>https://www.windowscentral.com/ Game Pass値上げ</t>
         </is>
       </c>
       <c r="J4" s="9" t="inlineStr"/>
@@ -24482,7 +24630,7 @@
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B6" s="9" t="inlineStr">
@@ -24497,14 +24645,34 @@
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>LoL/Valorant/Mobile Legends/eFootball</t>
-        </is>
-      </c>
-      <c r="E6" s="9" t="inlineStr"/>
-      <c r="F6" s="9" t="inlineStr"/>
-      <c r="G6" s="9" t="inlineStr"/>
-      <c r="H6" s="9" t="inlineStr"/>
-      <c r="I6" s="9" t="inlineStr"/>
+          <t>VALORANT Masters London 2026が6/21閉幕。7/6開幕のEsports World Cupへ移行期。</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>VALORANT Masters London閉幕／EWC2026は賞金総額が過去最大規模／視聴はモバイル・TikTok Liveシフトで月33億時間と記録更新。</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>Riot Games, ESL FACEIT(サウジ), REJECT</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>サウジ資本主導の大型大会が年間カレンダーの中心に。視聴のモバイル・短尺シフトが収益構造を変える。</t>
+        </is>
+      </c>
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>競技シーンの重心がサウジ・モバイル視聴へ移動。地政学と視聴行動の両面で構造変化。</t>
+        </is>
+      </c>
+      <c r="I6" s="9" t="inlineStr">
+        <is>
+          <t>https://escharts.com/ 視聴記録 / https://egamersworld.com/ Masters</t>
+        </is>
+      </c>
       <c r="J6" s="9" t="inlineStr"/>
     </row>
     <row r="7">
@@ -24538,7 +24706,7 @@
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
@@ -24553,32 +24721,32 @@
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>EUはルートボックス/ガチャを『ダークパターン×消費者保護(特に未成年)』として捉える方向。蘭・白は最も厳格でループボックスを賭博として規制。Digital Fairness Actの草案公表が射程に。</t>
+          <t>EU AI法の透明性ルールが8/2全面適用へ。米加州AB1921（運営終了時のユーザー保護）が州下院を通過。</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
-          <t>全面禁止は2026年内には見込み薄も、Digital Fairness Actで開示・支出上限・データ透明性の各国ルールが収斂へ。グローバル各社は地域別の『デュアルデザイン』出荷が常態化。</t>
+          <t>英政府が16歳未満のオンライン利用制限を公表／PEGIが有料ランダムアイテムを年齢レーティングへ反映する新基準を運用開始／EU AI法のAI生成表示義務が迫る。</t>
         </is>
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>欧州委員会, EA, 各F2Pパブリッシャー</t>
+          <t>EU, 英政府, PEGI, Apple, Google</t>
         </is>
       </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t>確率/UI/支出上限/データの地域差を前提とした設計が標準化。日本は自主規制継続で欧州の硬化と対照的。</t>
+          <t>流通（ストア開放）・年齢確認・課金設計・AI表示の4軸で規制が同時進行。グローバル運営は地域別の複層対応が標準になる。</t>
         </is>
       </c>
       <c r="H8" s="9" t="inlineStr">
         <is>
-          <t>規制は『禁止』より『開示と上限』へ。同一ゲームが地域別に別設計化する分断が進む。</t>
+          <t>単一論点でなく『複数レイヤー同時規制』が新常態。コンプラ投資が中堅以下の参入障壁を押し上げる。</t>
         </is>
       </c>
       <c r="I8" s="9" t="inlineStr">
         <is>
-          <t>https://medium.com/@minsu057/gacha-at-a-crossroads-how-europe-regulates-while-japan-self-regulates-e32dfc5a8623</t>
+          <t>https://www.pwc.com/jp/ EU AI法 / https://www.jetro.go.jp/ 英年齢制限</t>
         </is>
       </c>
       <c r="J8" s="9" t="inlineStr"/>
@@ -24662,7 +24830,7 @@
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
@@ -24677,32 +24845,32 @@
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>6/8-14だけで300本超が新規リリースし供給過多が加速。無料『TBH: Task Bar Hero』が13万同接で首位を継続。</t>
+          <t>Steam Next Fest 6月版が過去最大規模。サマーセールが6/25開幕。無料・少人数インディーが上位を席巻。</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>Steam Next Fest出展約8,700本のうち約1,704本（約20%）が生成AI利用を開示。DbD×ジェイソン参戦で同接7万超などコラボ起点のスパイクも顕著。</t>
+          <t>ValveがSteam Machineを日本・台湾・香港で発売（自社ハードでリビングへ進出）／Gothic 1 RemakeがVery Positiveでヒット／TBH等の無料ゲームが同接トップ。</t>
         </is>
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t>Valve, Behaviour Interactive, インディー各社</t>
+          <t>Valve, THQ Nordic, インディー各社</t>
         </is>
       </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
-          <t>供給爆発で『発見』の希少性が増し、同接ピーク×配信映え×AI開示の有無が選別シグナル化。キュレーション/イベント依存が強まる。</t>
+          <t>Valveがストア＋ハードの垂直統合を強化。PCの『コンソール化』とインディー発見性向上が並走する。</t>
         </is>
       </c>
       <c r="H11" s="9" t="inlineStr">
         <is>
-          <t>ディスカバリーの摩擦が最大のボトルネック。AI製の量産タイトル流入が『質の選別』を一段と重要にしている。</t>
+          <t>流通プラットフォーマーが自社ハードでエコシステムを囲い込む、Apple型の垂直統合がPCにも到来。</t>
         </is>
       </c>
       <c r="I11" s="9" t="inlineStr">
         <is>
-          <t>https://www.gamegrin.com/news/weekly-top-trending-games-on-steam-8th14th-of-june-2026/ , https://www.engadget.com/2195840/around-a-fifth-of-steam-next-fest-demos-have-a-generative-ai-disclosure/</t>
+          <t>https://www.4gamer.net/ Steam Machine / https://www.techtimes.com/ Next Fest</t>
         </is>
       </c>
       <c r="J11" s="9" t="inlineStr"/>
@@ -24710,7 +24878,7 @@
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B12" s="9" t="inlineStr">
@@ -24725,32 +24893,32 @@
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>6/9配信『Nintendo Direct 2026.6.9』(約50分)で2026年後半のSwitch 2/Switch新作を多数公開。看板は『ゼルダ 時のオカリナ』約28年越しリメイク、『KH4』Switch 2版、『ゼノブレイド』3作Switch 2版＋新作『ジェネシス』。</t>
+          <t>累計約2,000万台でPS5を約100万台上回る。サードパーティ売上+76%、tie-ratioは4.0超へ。</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>サードはドラクエモンスターズ4・鬼武者・信長の野望・朧村正など多数並ぶが大半が他機種とのマルチ。『独占の薄さ』と任天堂自身の旧作リメイク依存が同時に可視化された。</t>
+          <t>Star FoxがSwitch 2専用で6/25発売／FF7リバース・FF10 HD・KH4・ゼノブレイド等の移植・新作が集中／ニンダイ6.9は非独占マルチ中心で株価一時7%安。一方ソニーはPS6時期『未定』。</t>
         </is>
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>任天堂, スクウェア・エニックス, バンダイナムコ, カプコン, コーエーテクモ</t>
+          <t>任天堂, スクウェア・エニックス, カプコン, ソニー</t>
         </is>
       </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
-          <t>サードはSwitch 2を『追加販路』としてデイワン/同発を拡大。差別化はファースト＋移植速度に依存し、独占獲得競争は限定的に推移。</t>
+          <t>サードパーティ day-one供給が常態化しAAAライブラリが拡充。据置世代交代は任天堂先行・ソニー様子見の非対称が続く。</t>
         </is>
       </c>
       <c r="H12" s="9" t="inlineStr">
         <is>
-          <t>普及2年目は『独占で勝つ』から『台数×旧IP在庫で回す』局面へ。配信PFの旧作ライブラリ戦略と同型。</t>
+          <t>『独占』より『全機種同発』が標準化。ハード優位はソフト供給の引力で自己強化される。</t>
         </is>
       </c>
       <c r="I12" s="9" t="inlineStr">
         <is>
-          <t>https://www.4gamer.net/games/999/G999905/20260608100/</t>
+          <t>https://www.nintendolife.com/ 2000万台 / https://www.videogameschronicle.com/</t>
         </is>
       </c>
       <c r="J12" s="9" t="inlineStr"/>
@@ -24782,6 +24950,53 @@
       <c r="H13" s="9" t="inlineStr"/>
       <c r="I13" s="9" t="inlineStr"/>
       <c r="J13" s="9" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ゲーム技術のデュアルユース（防衛・産業転用）</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>技術/B2B</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>ゲームエンジン由来のリアルタイム3D・物理シミュレーション・AIが防衛・産業領域へ横展開し始めた。</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>KraftonがHanwha Aerospaceと提携し技術を防衛・産業へ応用／NVIDIA・Google Cloudが自律型AIエージェントや軽量NPCを開発者へ提供。</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Krafton, Hanwha Aerospace, NVIDIA, Google Cloud</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>ゲーム企業が『シミュレーション技術企業』へ自己定義を拡張。B2B・官公需要が新たな収益源に。</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>エンタメで磨いた技術が単価の高い防衛・産業へ流出する軍民両用構造。ゲーム＝基盤技術。</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>https://www.gamedeveloper.com/ Krafton×Hanwha</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
add forward-looking predictions (今後起きそうなこと) (2026-06-24 11:37)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -800,7 +800,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1179,6 +1179,117 @@
       <c r="G10" s="3" t="inlineStr">
         <is>
           <t>Q4発売予定タイトルの発売日変更アナウンス、2027年Q1の新作集中度を確認</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="inlineStr">
+        <is>
+          <t>Xboxの7月レイオフ後、Microsoftがスタジオ統廃合と一部ファーストパーティIPのマルチプラットフォーム展開（PS5/Switch2/クラウド）をさらに加速する</t>
+        </is>
+      </c>
+      <c r="C11" s="14" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="D11" s="14" t="inlineStr">
+        <is>
+          <t>2026年7月〜年内</t>
+        </is>
+      </c>
+      <c r="E11" s="14" t="inlineStr">
+        <is>
+          <t>Microsoft/Xbox, Activision Blizzard</t>
+        </is>
+      </c>
+      <c r="F11" s="14" t="inlineStr">
+        <is>
+          <t>Xbox『リセット』と7月の大規模レイオフ計画報道（VGC/Bloomberg, 6/24集約）</t>
+        </is>
+      </c>
+      <c r="G11" s="14" t="inlineStr">
+        <is>
+          <t>7/30前後のMS第4四半期決算と人員削減の具体規模、ファーストパーティ新作のマルチ化発表を確認。約1000人規模の数字が裏取りされるか要追跡。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>Valve『Steam Machine』投入を機に、SteamOS対応の据置/リビング向けサードパーティ製ハードが追随し、PC陣営のリビング市場攻勢が強まる</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>6〜12ヶ月後</t>
+        </is>
+      </c>
+      <c r="E12" s="14" t="inlineStr">
+        <is>
+          <t>Valve, KOMODO, AMD</t>
+        </is>
+      </c>
+      <c r="F12" s="14" t="inlineStr">
+        <is>
+          <t>Steam Machine 日本・台湾・香港で発売開始（4Gamer, 6/24集約）</t>
+        </is>
+      </c>
+      <c r="G12" s="14" t="inlineStr">
+        <is>
+          <t>SteamOSのサード機ライセンス動向、初期出荷の売れ行きと在庫消化ペース、Forza等大型タイトルのSteam対応拡大を確認。高価格帯ゆえ普及速度は限定的か。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B13" s="14" t="inlineStr">
+        <is>
+          <t>大手のCVC化（Nexon Partners等）が広がり、アジア発の選別的アーリーステージ投資が増える一方、巨額フルM&amp;Aは減速する</t>
+        </is>
+      </c>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>年内〜12ヶ月後</t>
+        </is>
+      </c>
+      <c r="E13" s="14" t="inlineStr">
+        <is>
+          <t>Nexon, Tencent, Microsoft</t>
+        </is>
+      </c>
+      <c r="F13" s="14" t="inlineStr">
+        <is>
+          <t>Nexon投資子会社『Nexon Partners』設立（Seoul Economic Daily）＋Xbox巨額買収後リストラ（6/24集約）</t>
+        </is>
+      </c>
+      <c r="G13" s="14" t="inlineStr">
+        <is>
+          <t>韓国・日本大手のCVC設立・出資発表の件数、10億ドル超フルM&amp;Aの有無を四半期で比較。買収プレミアム回収難が選別投資シフトを後押しするか検証。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
daily-news + cross-questions + events + predictions update (2026-06-24 22:11)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -800,7 +800,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1290,6 +1290,43 @@
       <c r="G13" s="14" t="inlineStr">
         <is>
           <t>韓国・日本大手のCVC設立・出資発表の件数、10億ドル超フルM&amp;Aの有無を四半期で比較。買収プレミアム回収難が選別投資シフトを後押しするか検証。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B14" s="15" t="inlineStr">
+        <is>
+          <t>GTA6の価格(通常$79.99/9,800円・アルティメット$99.99/12,280円)が新たなフルプライス基準となり、他社AAAが2027年にかけて値上げ・上位版商法で追随する</t>
+        </is>
+      </c>
+      <c r="C14" s="15" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="D14" s="15" t="inlineStr">
+        <is>
+          <t>年内〜2027年</t>
+        </is>
+      </c>
+      <c r="E14" s="15" t="inlineStr">
+        <is>
+          <t>Rockstar Games, Take-Two, 各AAAパブリッシャー</t>
+        </is>
+      </c>
+      <c r="F14" s="15" t="inlineStr">
+        <is>
+          <t>『GTA6』価格・予約特典公開(ファミ通, 6/25)</t>
+        </is>
+      </c>
+      <c r="G14" s="15" t="inlineStr">
+        <is>
+          <t>主要パブリッシャーの新作AAA定価($79.99→の改定有無)とデラックス/アルティメット版の比率・初動売上を観測すれば当否が分かる。</t>
         </is>
       </c>
     </row>
@@ -3006,7 +3043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4680,6 +4717,43 @@
       <c r="G45" s="14" t="inlineStr">
         <is>
           <t>流通を握る側がハード（顧客接点）まで垂直統合する点は、配信・ECの自社デバイス戦略と相似。OS・ストア・決済を自社で閉じる経済圏設計が共通テーマ。</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B46" s="15" t="inlineStr">
+        <is>
+          <t>超大型タイトル(GTA6)の『通常版＋アルティメット版＋予約特典』による価格分割・早期予約囲い込みは、映画・音楽・出版の“デラックス商法”や自動車・家電の上位グレード戦略のどれに該当するか？</t>
+        </is>
+      </c>
+      <c r="C46" s="15" t="inlineStr">
+        <is>
+          <t>『GTA6』価格・予約特典公開、通常9,800円/アルティメット12,280円・6/25予約開始(ファミ通)</t>
+        </is>
+      </c>
+      <c r="D46" s="15" t="inlineStr">
+        <is>
+          <t>Rockstar Games, Take-Two Interactive / GTA6</t>
+        </is>
+      </c>
+      <c r="E46" s="15" t="inlineStr">
+        <is>
+          <t>映像・音楽(デラックス/限定版商法), 出版(特装版), 自動車・家電(上位グレード), 小売(予約特典販売)</t>
+        </is>
+      </c>
+      <c r="F46" s="15" t="inlineStr">
+        <is>
+          <t>オープン</t>
+        </is>
+      </c>
+      <c r="G46" s="15" t="inlineStr">
+        <is>
+          <t>“1本を版違い＋予約特典で多段階価格化”する手法はエンタメ横断で一般化しており、ゲームの価格上限引き上げが他コンテンツの値付けにも波及しうる。</t>
         </is>
       </c>
     </row>
@@ -6393,14 +6467,14 @@
           <t>https://www.pcgamer.com/steam-sale-dates/</t>
         </is>
       </c>
-      <c r="I2" s="5" t="inlineStr">
-        <is>
-          <t>開催予定</t>
-        </is>
-      </c>
-      <c r="J2" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-17</t>
+      <c r="I2" s="15" t="inlineStr">
+        <is>
+          <t>開催中</t>
+        </is>
+      </c>
+      <c r="J2" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
         </is>
       </c>
     </row>
@@ -7263,7 +7337,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L201"/>
+  <dimension ref="A1:L205"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19777,6 +19851,245 @@
       </c>
       <c r="K201" s="14" t="inlineStr"/>
       <c r="L201" s="14" t="n"/>
+    </row>
+    <row r="202">
+      <c r="A202" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B202" s="15" t="inlineStr">
+        <is>
+          <t>『GTA6』価格・予約特典が公開、6/25予約開始——通常9,800円/アルティメット12,280円、11/19発売</t>
+        </is>
+      </c>
+      <c r="C202" s="15" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/article/202606/79372</t>
+        </is>
+      </c>
+      <c r="D202" s="15" t="inlineStr">
+        <is>
+          <t>Rockstar Gamesの超大型新作『グランド・セフト・オートVI』はゲーム史上最大級の話題作。発売日は2026年11月19日でPS5/Xbox Series X|S向け。年末商戦の最重要タイトルとされ、他社が発売時期を避ける動きも出ている。</t>
+        </is>
+      </c>
+      <c r="E202" s="15" t="inlineStr">
+        <is>
+          <t>6月24日(現地)に価格と予約特典が判明し、日本では6/25深夜より予約開始。通常版9,800円、アルティメット・エディション12,280円(米$79.99/$99.99)。予約特典「ヴィンテージ・バイスシティパック」に車両・武器スキン・衣装等が付属する。</t>
+        </is>
+      </c>
+      <c r="F202" s="15" t="inlineStr">
+        <is>
+          <t>通常版9,800円・アルティメット12,280円(米$79.99/$99.99)の高価格設定
+予約は6/25深夜開始、発売は11/19(PS5/Xbox Series X|S)
+予約特典「ヴィンテージ・バイスシティパック」で車両・衣装・武器スキン提供
+フルプライスAAAの新たな価格基準として業界が注目</t>
+        </is>
+      </c>
+      <c r="G202" s="15" t="inlineStr">
+        <is>
+          <t>$79.99/9,800円が新たなAAA定価基準となり、他社が上位版商法・値上げで追随する可能性。11/19前後は他大型作が発売を回避し、年末〜2027年Q1へ発売時期の再調整が続く見込み。</t>
+        </is>
+      </c>
+      <c r="H202" s="15" t="inlineStr">
+        <is>
+          <t>AAAタイトルの価格戦略と上位版(アルティメット)商法</t>
+        </is>
+      </c>
+      <c r="I202" s="15" t="inlineStr">
+        <is>
+          <t>Rockstar Games, Take-Two Interactive</t>
+        </is>
+      </c>
+      <c r="J202" s="15" t="inlineStr">
+        <is>
+          <t>Grand Theft Auto VI</t>
+        </is>
+      </c>
+      <c r="K202" s="15" t="inlineStr">
+        <is>
+          <t>新作,海外</t>
+        </is>
+      </c>
+      <c r="L202" s="15" t="n"/>
+    </row>
+    <row r="203">
+      <c r="A203" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B203" s="15" t="inlineStr">
+        <is>
+          <t>コロプラ、金子一馬氏『KAZUMA KANEKO'S ツクヨミ』Steam版を発表——7/24配信、3,960円から</t>
+        </is>
+      </c>
+      <c r="C203" s="15" t="inlineStr">
+        <is>
+          <t>https://colopl.co.jp/news/pressrelease/2026062401.php</t>
+        </is>
+      </c>
+      <c r="D203" s="15" t="inlineStr">
+        <is>
+          <t>『真・女神転生』『ペルソナ』のキャラデザで知られる金子一馬氏の最新作。コロプラ初の本格コンシューマ向けタイトルとして2026年4月にSwitch版が発売済みで、塔を登り「神魔」に挑むデッキ構築型ローグライク。</t>
+        </is>
+      </c>
+      <c r="E203" s="15" t="inlineStr">
+        <is>
+          <t>6/24、コロプラはデッキ構築型ローグライク『KAZUMA KANEKO'S ツクヨミ』Steam版を発表し7/24配信開始と告知。通常版3,960円、追加DLCを同梱したデラックス版5,960円。同日にDLC第2弾もSwitch/Steam向けに配信される。</t>
+        </is>
+      </c>
+      <c r="F203" s="15" t="inlineStr">
+        <is>
+          <t>金子一馬氏の最新作Steam版を7/24配信(通常3,960円/デラックス5,960円)
+神話モチーフのデッキ構築型ローグライク戦略カードバトル
+Switch版に続くマルチ展開で海外PCユーザー取り込みを狙う
+同日にDLC第2弾も配信</t>
+        </is>
+      </c>
+      <c r="G203" s="15" t="inlineStr">
+        <is>
+          <t>Switch先行→Steam展開でグローバルのローグライク/カードゲーム層へ拡大。金子氏ブランドと低価格でインディー的訴求が見込まれ、コロプラのコンシューマ/PC路線強化の試金石となる。</t>
+        </is>
+      </c>
+      <c r="H203" s="15" t="inlineStr">
+        <is>
+          <t>モバイル企業のコンシューマ/Steam展開戦略</t>
+        </is>
+      </c>
+      <c r="I203" s="15" t="inlineStr">
+        <is>
+          <t>コロプラ</t>
+        </is>
+      </c>
+      <c r="J203" s="15" t="inlineStr">
+        <is>
+          <t>KAZUMA KANEKO'S ツクヨミ</t>
+        </is>
+      </c>
+      <c r="K203" s="15" t="inlineStr">
+        <is>
+          <t>新作,国内,インディー</t>
+        </is>
+      </c>
+      <c r="L203" s="15" t="n"/>
+    </row>
+    <row r="204">
+      <c r="A204" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B204" s="15" t="inlineStr">
+        <is>
+          <t>マウスコンピューター、事業説明会で今後のゲーマー向け新製品を公開——G TUNE/NEXTGEAR/iiyama</t>
+        </is>
+      </c>
+      <c r="C204" s="15" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/026/G002654/20260624016/</t>
+        </is>
+      </c>
+      <c r="D204" s="15" t="inlineStr">
+        <is>
+          <t>マウスコンピューターは国内BTO PC大手で、ゲーミングブランド「G TUNE」「NEXTGEAR」とディスプレイ「iiyama」を展開。Switch 2やSteam Machineなど新ハード登場でPCゲーミング市場の競争が激化している。</t>
+        </is>
+      </c>
+      <c r="E204" s="15" t="inlineStr">
+        <is>
+          <t>6/24、マウスコンピューターは東京で事業説明会を開き、今後発表予定のゲーマー向け製品を公開。有機ELディスプレイやエントリー向けノートPCなど、G TUNE/NEXTGEAR/iiyamaブランドの新ラインを示した。</t>
+        </is>
+      </c>
+      <c r="F204" s="15" t="inlineStr">
+        <is>
+          <t>ゲーミングブランドG TUNE/NEXTGEAR/iiyamaの新製品を予告
+有機ELディスプレイやエントリー向けゲーミングノートPCを準備
+国内BTO大手としてPCゲーミング需要拡大に対応</t>
+        </is>
+      </c>
+      <c r="G204" s="15" t="inlineStr">
+        <is>
+          <t>Steam Machine等の据置型PCやSwitch 2と競合/補完しつつ、国内BTO各社はエントリー〜ハイエンドの製品拡充を継続。有機EL等の高付加価値ディスプレイ投入で単価向上を図る見込み。</t>
+        </is>
+      </c>
+      <c r="H204" s="15" t="inlineStr">
+        <is>
+          <t>国内BTO/ゲーミングPC市場の競争動向</t>
+        </is>
+      </c>
+      <c r="I204" s="15" t="inlineStr">
+        <is>
+          <t>マウスコンピューター</t>
+        </is>
+      </c>
+      <c r="J204" s="15" t="inlineStr">
+        <is>
+          <t>G TUNE, NEXTGEAR, iiyama</t>
+        </is>
+      </c>
+      <c r="K204" s="15" t="inlineStr">
+        <is>
+          <t>技術,国内</t>
+        </is>
+      </c>
+      <c r="L204" s="15" t="n"/>
+    </row>
+    <row r="205">
+      <c r="A205" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B205" s="15" t="inlineStr">
+        <is>
+          <t>“次世代タイタンフォール”6v6ムーブメントシューター『EMPULSE』、本日6/25早期アクセス開始(PC/Xbox)</t>
+        </is>
+      </c>
+      <c r="C205" s="15" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/article/202606/79341</t>
+        </is>
+      </c>
+      <c r="D205" s="15" t="inlineStr">
+        <is>
+          <t>『EMPULSE』はメカ搭乗とウォールラン・グラップル等の高機動アクションが特徴の6対6対戦FPS。『タイタンフォール』後継との呼び声が高く、6/15からSteamでデモ版を配信し注目を集めていた。</t>
+        </is>
+      </c>
+      <c r="E205" s="15" t="inlineStr">
+        <is>
+          <t>6/25、6v6ムーブメントシューター『EMPULSE』がPC(Steam)/Xbox Series X|Sで早期アクセス開始。壁走り・空中ジャンプ・グラップルに加え、マップ中央で奪い合う搭乗可能なメカが特徴。PS5版はプラットフォーム審査の都合で延期。</t>
+        </is>
+      </c>
+      <c r="F205" s="15" t="inlineStr">
+        <is>
+          <t>本日6/25早期アクセス開始(PC/Xbox、PS5版は延期)
+ウォールラン・グラップル・空中ジャンプの立体的高速戦闘
+搭乗可能メカを中央objで奪い合う6対6設計
+『タイタンフォール』後継として競技シーンの期待大</t>
+        </is>
+      </c>
+      <c r="G205" s="15" t="inlineStr">
+        <is>
+          <t>アリーナ/ムーブメント系FPSの新規参入として、早期アクセスでの初動同接とコミュニティ定着が試金石。ヒーローシューター飽和市場で差別化できれば小規模eスポーツ化の可能性もある。</t>
+        </is>
+      </c>
+      <c r="H205" s="15" t="inlineStr">
+        <is>
+          <t>ムーブメント系対戦FPSのライブ運営と早期アクセス戦略</t>
+        </is>
+      </c>
+      <c r="I205" s="15" t="n"/>
+      <c r="J205" s="15" t="inlineStr">
+        <is>
+          <t>EMPULSE</t>
+        </is>
+      </c>
+      <c r="K205" s="15" t="inlineStr">
+        <is>
+          <t>新作,海外</t>
+        </is>
+      </c>
+      <c r="L205" s="15" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
daily-news + cross-questions + events + predictions update (2026-06-25 22:34)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -31,7 +31,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -85,6 +85,10 @@
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -125,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -163,6 +167,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -800,7 +807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1327,6 +1334,43 @@
       <c r="G14" s="15" t="inlineStr">
         <is>
           <t>主要パブリッシャーの新作AAA定価($79.99→の改定有無)とデラックス/アルティメット版の比率・初動売上を観測すれば当否が分かる。</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="17" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>EAのPIF主導LBO完了(6/30前後)後、非公開化を背景にコスト削減・人員整理とEA Sports FC等の課金/サブスク強化が進む</t>
+        </is>
+      </c>
+      <c r="C15" s="17" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="D15" s="17" t="inlineStr">
+        <is>
+          <t>数ヶ月後(年内)</t>
+        </is>
+      </c>
+      <c r="E15" s="17" t="inlineStr">
+        <is>
+          <t>Electronic Arts, サウジPIF</t>
+        </is>
+      </c>
+      <c r="F15" s="17" t="inlineStr">
+        <is>
+          <t>EA、サウジPIF主導の550億ドルLBO非公開化が6/30の最終期限へ(EA IR)</t>
+        </is>
+      </c>
+      <c r="G15" s="17" t="inlineStr">
+        <is>
+          <t>クロージング発表(6/30前後)の有無、その後の組織再編/人員削減リリース、EA Sports FCの課金・サブスク施策の変化を観測</t>
         </is>
       </c>
     </row>
@@ -3043,7 +3087,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G46"/>
+  <dimension ref="A1:G48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4754,6 +4798,80 @@
       <c r="G46" s="15" t="inlineStr">
         <is>
           <t>“1本を版違い＋予約特典で多段階価格化”する手法はエンタメ横断で一般化しており、ゲームの価格上限引き上げが他コンテンツの値付けにも波及しうる。</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>ソブリン・ウェルス・ファンド(PIF)が基幹エンタメ企業を巨額LBOで非公開化する動きは、スポーツ・音楽・映画など他のIP産業でも同様に起きるか？</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>EAの550億ドルPIF主導LBOが6/30の最終期限へ</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>Electronic Arts, サウジPIF, Silver Lake</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>スポーツ(クラブ・リーグ買収), 音楽(カタログ買収), 映画/映像スタジオ, 出版</t>
+        </is>
+      </c>
+      <c r="F47" s="5" t="inlineStr">
+        <is>
+          <t>オープン</t>
+        </is>
+      </c>
+      <c r="G47" s="5" t="inlineStr">
+        <is>
+          <t>国家系ファンドが『キャッシュフローの読めるIP資産』を負債込みで囲い込む構図。エンタメ全般で同型の非公開化が連鎖しうる</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>新ハード立ち上げによる『物理パッケージ需要の一時的回復』は、小売・流通の在庫/店頭戦略にどう作用し、他の耐久財(家電・自動車)の買い替えサイクルと類似するか？</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>Circana：Switch 2でUS物理ソフト販売が前年比+26%(一時的)</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>任天堂, Circana</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>小売/流通(在庫・店頭), 家電(買い替えサイクル), 出版(物理メディア)</t>
+        </is>
+      </c>
+      <c r="F48" s="5" t="inlineStr">
+        <is>
+          <t>オープン</t>
+        </is>
+      </c>
+      <c r="G48" s="5" t="inlineStr">
+        <is>
+          <t>デジタル化が進む市場でも『新世代ハード』が物理需要を一時的に押し上げる。耐久財の世代交代と在庫戦略の相似形として観察できる</t>
         </is>
       </c>
     </row>
@@ -6359,7 +6477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:J20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6521,12 +6639,12 @@
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>開催予定</t>
+          <t>開催中</t>
         </is>
       </c>
       <c r="J3" s="5" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-26</t>
         </is>
       </c>
     </row>
@@ -7323,6 +7441,58 @@
       <c r="J19" s="15" t="inlineStr">
         <is>
           <t>2026-06-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>VALORANT Esports Nations Cup 2026 予選</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>eスポーツ</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>オンライン</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>オンライン</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>国別対抗大会の地域予選。8地域から本戦(リヤド)進出枠を選出。VALORANT部門。</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>https://esportsnationscup.com/en/competitions/2026/valorant</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>開催中</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
         </is>
       </c>
     </row>
@@ -7337,7 +7507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L205"/>
+  <dimension ref="A1:L211"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -20090,6 +20260,368 @@
         </is>
       </c>
       <c r="L205" s="15" t="n"/>
+    </row>
+    <row r="206">
+      <c r="A206" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B206" s="5" t="inlineStr">
+        <is>
+          <t>EA、サウジPIF主導の550億ドルLBO非公開化が6/30の最終期限へ——史上最大の現金買収が大詰め</t>
+        </is>
+      </c>
+      <c r="C206" s="5" t="inlineStr">
+        <is>
+          <t>https://ir.ea.com/press-releases/press-release-details/2025/EA-Announces-Agreement-to-be-Acquired-by-PIF-Silver-Lake-and-Affinity-Partners-for-55-Billion/default.aspx</t>
+        </is>
+      </c>
+      <c r="D206" s="5" t="inlineStr">
+        <is>
+          <t>2025年9月、EAはサウジ公的投資基金(PIF)・Silver Lake・Affinity Partnersの連合に1株210ドル・総額約550億ドルで買収されることで合意。株主は2025年12月に承認済みで、規制当局の承認を残すのみ。完了の最終期限(long-stop date)は2026年6月30日に設定されている。</t>
+        </is>
+      </c>
+      <c r="E206" s="5" t="inlineStr">
+        <is>
+          <t>現金対価550億ドル(うち200億ドルは負債)で、企業の現金買収LBOとしては史上最大。クロージングが6/30の期限に向け最終局面に入り、完了後EAは非公開化される。EA Sports FCやApex、The Simsなど主要IPがソブリン・ウェルス・ファンド傘下に入る。</t>
+        </is>
+      </c>
+      <c r="F206" s="5" t="inlineStr">
+        <is>
+          <t>・最終期限は2026/6/30、現金対価1株210ドル(25%プレミアム)
+・PIF/Silver Lake/Affinityの連合、負債200億ドルを調達
+・史上最大の現金LBO、EAは上場廃止へ
+・主要スポーツ/ライブサービスIPがSWF傘下に</t>
+        </is>
+      </c>
+      <c r="G206" s="5" t="inlineStr">
+        <is>
+          <t>完了後は負債200億ドルの返済圧力から、コスト削減・人員整理とEA Sports FC等の課金/サブスク強化が進む可能性。非公開化で四半期開示が消え、長期投資と短期収益化のバランスが焦点に。</t>
+        </is>
+      </c>
+      <c r="H206" s="5" t="inlineStr">
+        <is>
+          <t>ソブリン・ウェルス・ファンドのゲーム/エンタメ投資とLBOの財務構造</t>
+        </is>
+      </c>
+      <c r="I206" s="5" t="inlineStr">
+        <is>
+          <t>Electronic Arts, サウジPIF, Silver Lake, Affinity Partners</t>
+        </is>
+      </c>
+      <c r="J206" s="5" t="inlineStr">
+        <is>
+          <t>EA Sports FC, Apex Legends, The Sims, Battlefield</t>
+        </is>
+      </c>
+      <c r="K206" s="5" t="inlineStr">
+        <is>
+          <t>M&amp;A,業績,海外</t>
+        </is>
+      </c>
+      <c r="L206" s="5" t="n"/>
+    </row>
+    <row r="207">
+      <c r="A207" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B207" s="5" t="inlineStr">
+        <is>
+          <t>MicrosoftのXbox、FY末(6/30)直前にスタジオ人員削減が開始——Compulsion Gamesで離職確認</t>
+        </is>
+      </c>
+      <c r="C207" s="5" t="inlineStr">
+        <is>
+          <t>https://www.techtimes.com/articles/319072/20260625/xbox-studio-layoffs-begin-compulsion-games-game-pass-accounting-punished-its-own-hits.htm</t>
+        </is>
+      </c>
+      <c r="D207" s="5" t="inlineStr">
+        <is>
+          <t>新Microsoft Gaming CEOアシャ・シャルマ氏の下、Xbox部門は収益減を背景にハード・スタジオ・マーケ・独占戦略の『リセット』を進行中。6/16にはNinja Theory(Hellbladeのスタジオ)が閉鎖確認されていた。</t>
+        </is>
+      </c>
+      <c r="E207" s="5" t="inlineStr">
+        <is>
+          <t>6/25、『We Happy Few』のCompulsion Gamesで人員削減が始まったとLinkedInで複数の離職が確認された。Microsoftの会計年度末(6/30)直前で、7月にかけて本格的な再編・人員整理が見込まれる。</t>
+        </is>
+      </c>
+      <c r="F207" s="5" t="inlineStr">
+        <is>
+          <t>・Compulsion Gamesで6/25にレイオフ開始
+・6/16にNinja Theory閉鎖が確認済み
+・FY末6/30直前、7月に本格再編の見通し
+・Game Passの会計処理がヒット作の評価を抑制との指摘</t>
+        </is>
+      </c>
+      <c r="G207" s="5" t="inlineStr">
+        <is>
+          <t>7月のFY切替後に統廃合と一部ファーストパーティIPの整理が進む可能性。親会社のAI再配分が続く中、Xboxは『黒字でも縮小』の構図が鮮明化。</t>
+        </is>
+      </c>
+      <c r="H207" s="5" t="inlineStr">
+        <is>
+          <t>プラットフォーマーのスタジオポートフォリオ管理とGame Pass会計</t>
+        </is>
+      </c>
+      <c r="I207" s="5" t="inlineStr">
+        <is>
+          <t>Microsoft, Xbox, Compulsion Games, Ninja Theory</t>
+        </is>
+      </c>
+      <c r="J207" s="5" t="inlineStr">
+        <is>
+          <t>We Happy Few, Hellblade</t>
+        </is>
+      </c>
+      <c r="K207" s="5" t="inlineStr">
+        <is>
+          <t>業績,海外</t>
+        </is>
+      </c>
+      <c r="L207" s="5" t="n"/>
+    </row>
+    <row r="208">
+      <c r="A208" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B208" s="5" t="inlineStr">
+        <is>
+          <t>Steamサマーセール2026が開幕(6/25〜7/9)——数千タイトルが大幅値引き、収集カードも配布</t>
+        </is>
+      </c>
+      <c r="C208" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pcgamer.com/games/steam-summer-sale-2026-live/</t>
+        </is>
+      </c>
+      <c r="D208" s="5" t="inlineStr">
+        <is>
+          <t>Steamの夏の大型セールは年間最大級の販促イベントで、PCゲーム市場の需要を牽引する。6/22には予告トレーラーが公開されていた。</t>
+        </is>
+      </c>
+      <c r="E208" s="5" t="inlineStr">
+        <is>
+          <t>6/25午前10時(PT)、Steamサマーセール2026が正式に開幕。7/9まで開催され、数千タイトルが最大90%超の割引に。期間中は収集カードのドロップも実施され、ウィッシュリスト消化と新規購入を促す。</t>
+        </is>
+      </c>
+      <c r="F208" s="5" t="inlineStr">
+        <is>
+          <t>・会期2026/6/25〜7/9、最大90%超の割引
+・数千タイトルが対象、収集カード配布
+・年末商戦前のPC需要を牽引
+・GeForce NOW等クラウド勢も連動</t>
+        </is>
+      </c>
+      <c r="G208" s="5" t="inlineStr">
+        <is>
+          <t>夏セールの規模はSteamの年間GMVに直結。GTA6など年末の大型新作を控え、既存タイトルのロングテール収益が積み上がる。インディーは露出機会として重要。</t>
+        </is>
+      </c>
+      <c r="H208" s="5" t="inlineStr">
+        <is>
+          <t>PCストアのセール設計とロングテール収益</t>
+        </is>
+      </c>
+      <c r="I208" s="5" t="inlineStr">
+        <is>
+          <t>Valve</t>
+        </is>
+      </c>
+      <c r="J208" s="5" t="inlineStr">
+        <is>
+          <t>Steam</t>
+        </is>
+      </c>
+      <c r="K208" s="5" t="inlineStr">
+        <is>
+          <t>セール,海外,国内</t>
+        </is>
+      </c>
+      <c r="L208" s="5" t="n"/>
+    </row>
+    <row r="209">
+      <c r="A209" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B209" s="5" t="inlineStr">
+        <is>
+          <t>Circana：Switch 2立ち上げで米国の物理ソフト販売が前年比+26%——ただし一時的との見方</t>
+        </is>
+      </c>
+      <c r="C209" s="5" t="inlineStr">
+        <is>
+          <t>https://mynintendonews.com/2026/06/25/us-nintendo-switch-2-launch-saw-a-big-bump-in-physical-video-games-sold/</t>
+        </is>
+      </c>
+      <c r="D209" s="5" t="inlineStr">
+        <is>
+          <t>デジタル販売が主流化する中、物理パッケージは縮小トレンドが続いていた。Switch 2は累計約1,986万台で任天堂史上最速級の立ち上がり。</t>
+        </is>
+      </c>
+      <c r="E209" s="5" t="inlineStr">
+        <is>
+          <t>6/25、CircanaのMat Piscatella氏は、Switch 2の発売により任天堂プラットフォームの物理ソフト販売が前年比で約26%増加したと報告。ただし新ハード立ち上げに伴う一時的な『blip(山)』である可能性が高いとした。</t>
+        </is>
+      </c>
+      <c r="F209" s="5" t="inlineStr">
+        <is>
+          <t>・任天堂プラットフォームの物理販売が前年比+26%(Circana)
+・Switch 2立ち上げによる一時的効果との分析
+・累計約1,986万台、PS5を四半期で上回る
+・デジタル化トレンドの中での反転</t>
+        </is>
+      </c>
+      <c r="G209" s="5" t="inlineStr">
+        <is>
+          <t>立ち上げ効果が一巡する後半は物理需要が再び鈍化する公算。小売・流通はローンチ商戦の在庫戦略の最適化が課題に。</t>
+        </is>
+      </c>
+      <c r="H209" s="5" t="inlineStr">
+        <is>
+          <t>物理パッケージ需要とハードサイクルの相関</t>
+        </is>
+      </c>
+      <c r="I209" s="5" t="inlineStr">
+        <is>
+          <t>任天堂, Circana</t>
+        </is>
+      </c>
+      <c r="J209" s="5" t="inlineStr">
+        <is>
+          <t>Nintendo Switch 2</t>
+        </is>
+      </c>
+      <c r="K209" s="5" t="inlineStr">
+        <is>
+          <t>業績,国内</t>
+        </is>
+      </c>
+      <c r="L209" s="5" t="n"/>
+    </row>
+    <row r="210">
+      <c r="A210" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B210" s="5" t="inlineStr">
+        <is>
+          <t>TCIC、コンテンツ系アクセラレータ『Pitch Campus 2026』採択7組を決定——AI・ゲーム・XR・IP領域を支援</t>
+        </is>
+      </c>
+      <c r="C210" s="5" t="inlineStr">
+        <is>
+          <t>https://www.gamebusiness.jp/article/2026/06/24/27314.html</t>
+        </is>
+      </c>
+      <c r="D210" s="5" t="inlineStr">
+        <is>
+          <t>東京コンテンツインキュベーションセンター(TCIC)は、アニメ・ゲーム・映像・XR・AI・IPビジネス等のスタートアップを対象にアクセラレーションプログラムを運営。資金調達や事業提携の場を提供する。</t>
+        </is>
+      </c>
+      <c r="E210" s="5" t="inlineStr">
+        <is>
+          <t>6/24、TCICは『TCIC Pitch Campus 2026 -Contents Business Acceleration-』の採択7組を発表。会期は6/15〜7/30で、最終回のDemo DayでVC・金融機関・コンテンツ事業会社へピッチし、資金調達・提携につなげる。</t>
+        </is>
+      </c>
+      <c r="F210" s="5" t="inlineStr">
+        <is>
+          <t>・採択7組、会期2026/6/15〜7/30
+・対象はゲーム/AI/XR/映像/IP領域
+・Demo DayでVC・事業会社へピッチ
+・国内コンテンツ系スタートアップの育成基盤</t>
+        </is>
+      </c>
+      <c r="G210" s="5" t="inlineStr">
+        <is>
+          <t>国内のコンテンツ系スタートアップへの資金供給が活性化。AI×ゲーム/XR領域での新規プレイヤー登場と、大手のCVC/出資との接続が進む可能性。</t>
+        </is>
+      </c>
+      <c r="H210" s="5" t="inlineStr">
+        <is>
+          <t>国内コンテンツ系スタートアップの資金調達エコシステム</t>
+        </is>
+      </c>
+      <c r="I210" s="5" t="inlineStr">
+        <is>
+          <t>TCIC(東京コンテンツインキュベーションセンター)</t>
+        </is>
+      </c>
+      <c r="J210" s="5" t="n"/>
+      <c r="K210" s="5" t="inlineStr">
+        <is>
+          <t>技術,国内,インディー</t>
+        </is>
+      </c>
+      <c r="L210" s="5" t="n"/>
+    </row>
+    <row r="211">
+      <c r="A211" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B211" s="5" t="inlineStr">
+        <is>
+          <t>VALORANT『Esports Nations Cup 2026』地域予選が6/26開幕——8地域から本戦進出枠を争う</t>
+        </is>
+      </c>
+      <c r="C211" s="5" t="inlineStr">
+        <is>
+          <t>https://esportsnationscup.com/en/competitions/2026/valorant</t>
+        </is>
+      </c>
+      <c r="D211" s="5" t="inlineStr">
+        <is>
+          <t>Esports Nations Cupは国・地域代表が複数タイトルで競う大会。VALORANT部門はオンライン地域予選を経て本戦(リヤド)へ進む構成。</t>
+        </is>
+      </c>
+      <c r="E211" s="5" t="inlineStr">
+        <is>
+          <t>6/26〜28、VALORANTのEsports Nations Cup 2026オンライン地域予選が開幕。北米・南米・西欧・東欧・アジア・東南アジア/オセアニアの上位2チームに、MENA・サブサハラの勝者を加えて本戦進出枠を争う。</t>
+        </is>
+      </c>
+      <c r="F211" s="5" t="inlineStr">
+        <is>
+          <t>・地域予選は2026/6/26〜28、オンライン開催
+・8地域から本戦進出枠を選出
+・国別対抗フォーマットで地域代表を編成
+・本戦は中東(リヤド)規模の大型賞金</t>
+        </is>
+      </c>
+      <c r="G211" s="5" t="inlineStr">
+        <is>
+          <t>国別対抗のeスポーツが大型賞金とともに定着。中東マネーを背景にした大会運営と地域代表編成は、各地域のプロシーン強化につながる。</t>
+        </is>
+      </c>
+      <c r="H211" s="5" t="inlineStr">
+        <is>
+          <t>国別対抗eスポーツの大会フォーマットと資金源</t>
+        </is>
+      </c>
+      <c r="I211" s="5" t="inlineStr">
+        <is>
+          <t>Riot Games, Esports Nations Cup</t>
+        </is>
+      </c>
+      <c r="J211" s="5" t="inlineStr">
+        <is>
+          <t>VALORANT</t>
+        </is>
+      </c>
+      <c r="K211" s="5" t="inlineStr">
+        <is>
+          <t>eスポーツ,海外</t>
+        </is>
+      </c>
+      <c r="L211" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
weekly-releases + indie + rankings update (2026-06-26 12:36)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -4886,7 +4886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J43"/>
+  <dimension ref="A1:J62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6463,6 +6463,669 @@
       <c r="J43" t="inlineStr">
         <is>
           <t>9位へ後退</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-06-15〜06-21</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>トモダチコレクション わくわく生活</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Switch</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
+        <v>34957</v>
+      </c>
+      <c r="G44" t="n">
+        <v>1382027</v>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週間販売数 https://www.famitsu.com/article/202606/79458</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>首位返り咲き</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-06-15〜06-21</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>2</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>パワフルプロ野球2026-2027</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Switch</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>28409</v>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週間販売数 https://www.famitsu.com/article/202606/79458</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>前週首位から2位へ</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-06-15〜06-21</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>3</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>冒険家エリオットの千年物語</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Switch 2</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>23674</v>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週間販売数 https://www.famitsu.com/article/202606/79458</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Switch2版が初週3位（2機種合算38,517本）</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-06-15〜06-21</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>4</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>冒険家エリオットの千年物語</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>PS5</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>14843</v>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週間販売数 https://www.famitsu.com/article/202606/79458</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>PS5版が初週4位</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-06-15〜06-21</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>5</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>ぽこ あ ポケモン</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Switch 2</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週間販売数 https://www.famitsu.com/article/202606/79458</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>5〜9位の順位・本数は速報の概算</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-06-15〜06-21</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>6</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>eFootball Kick-Off!</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Switch 2</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週間販売数 https://www.famitsu.com/article/202606/79458</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>5〜9位の順位・本数は速報の概算</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-06-15〜06-21</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>7</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>マリオカート ワールド</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Switch 2</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週間販売数 https://www.famitsu.com/article/202606/79458</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>5〜9位の順位・本数は速報の概算</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-06-15〜06-21</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>9</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>ヨッシーとフカシギの図鑑</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Switch 2</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週間販売数 https://www.famitsu.com/article/202606/79458</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>5〜9位の順位・本数は速報の概算</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-06-15〜06-21</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>10</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>カービィのエアライダー</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Switch 2</t>
+        </is>
+      </c>
+      <c r="F52" t="n">
+        <v>3332</v>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週間販売数 https://www.famitsu.com/article/202606/79458</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>18位→10位へ急浮上</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-06-17〜06-23</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>1</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>MECCHA CHAMELEON（めっちゃカメレオン）</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>VGChartz Steam週間トップセラー Week26 https://www.vgchartz.com/article/468281/</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>2週連続トップ級。サマーセール直前の好調継続</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-06-17〜06-23</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>2</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Cyberpunk 2077（サイバーパンク2077）</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>VGChartz Steam週間トップセラー Week26 https://www.vgchartz.com/article/468281/</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>拡張Phantom Liberty含むセール需要で2位</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-06-17〜06-23</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>3</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Dead by Daylight（デッドバイデイライト）</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>VGChartz Steam週間トップセラー Week26 https://www.vgchartz.com/article/468281/</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-06-17〜06-23</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>4</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Steam Deck</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>ハードウェア</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>VGChartz Steam週間トップセラー Week26 https://www.vgchartz.com/article/468281/</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>ハード（携帯PC）</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-06-17〜06-23</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>5</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Path of Exile 2（パス・オブ・エグザイル2）</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>VGChartz Steam週間トップセラー Week26 https://www.vgchartz.com/article/468281/</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-06-17〜06-23</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>6</v>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Forza Horizon 6（フォルツァ ホライゾン 6）</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>VGChartz Steam週間トップセラー Week26 https://www.vgchartz.com/article/468281/</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>累計約490万本(推定/Alinea Analytics)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-06-17〜06-23</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>7</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Cyberpunk 2077: Phantom Liberty</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>VGChartz Steam週間トップセラー Week26 https://www.vgchartz.com/article/468281/</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>拡張単体でランクイン</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-06-17〜06-23</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>8</v>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>雀魂 -じゃんたま-（MahjongSoul）</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>VGChartz Steam週間トップセラー Week26 https://www.vgchartz.com/article/468281/</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-06-17〜06-23</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>9</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Dave the Diver（デイヴ・ザ・ダイバー）</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>VGChartz Steam週間トップセラー Week26 https://www.vgchartz.com/article/468281/</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-06-17〜06-23</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>10</v>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Stellaris（ステラリス）</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>VGChartz Steam週間トップセラー Week26 https://www.vgchartz.com/article/468281/</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>6/25開始のサマーセール影響で順位は概算</t>
         </is>
       </c>
     </row>
@@ -20634,7 +21297,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M24"/>
+  <dimension ref="A1:M28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -21543,12 +22206,18 @@
           <t>3Dシューティング</t>
         </is>
       </c>
+      <c r="G19" t="n">
+        <v>82</v>
+      </c>
+      <c r="H19" t="n">
+        <v>84</v>
+      </c>
       <c r="K19" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>『スターフォックス64』ベースにグラフィック一新＋新要素の新生スターフォックス。6/9のNintendo Directで体験版配信開始。約30年ぶりの本格新作として注目。</t>
+          <t>【6/25発売・実績反映】海外メタスコア82/OpenCritic84でシリーズ史上2番目の高評価。『スターフォックス64』の丁寧なフルリメイクで、よりドラマティックに。レビュー76件・好評86%。IGNはチャレンジモードを高評価。約30年ぶりの本格新作としてSwitch2の看板に。</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -21779,6 +22448,186 @@
       <c r="M24" t="inlineStr">
         <is>
           <t>https://www.konami.com/games/corporate/ja/news/topics/20260416/</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Frostpunk 2: Breach of Trust（フロストパンク2：ブリーチ・オブ・トラスト）</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>11 bit studios</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>11 bit studios</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>PC/PS5/Xbox Series X|S</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>都市建設サバイバルSLG（拡張）</t>
+        </is>
+      </c>
+      <c r="K25" t="n">
+        <v>3</v>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>【今週・拡張DLC】『Frostpunk 2』の大型拡張。新たな政治的緊張と難しい指導者の決断を追加。本編のシビアな雪原世界を拡張。スコアは集計待ち。</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>https://www.dlcompare.com/gaming-news/this-week-s-video-game-releases-june-2026-week-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>GRANBLUE FANTASY: Relink – Endless Ragnarök（グランブルーファンタジー リリンク エンドレスラグナロク）</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Cygames</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Cygames</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Switch 2/PS5/PC</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>アクションRPG</t>
+        </is>
+      </c>
+      <c r="K26" t="n">
+        <v>4</v>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>来月予定（評価系空欄）。Switch2版はオンライン/ローカル/クロスプレイ対応。Relinkの大型拡張展開。</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/schedule</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>デジモンストーリー タイムストレンジャー（Digimon Story: Time Stranger）</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Media.Vision</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>バンダイナムコエンターテインメント</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Switch 2/PS5/PC/Xbox Series X|S</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>RPG</t>
+        </is>
+      </c>
+      <c r="K27" t="n">
+        <v>4</v>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>来月予定（評価系空欄）。Switch2版はクオリティ/パフォーマンスのモード選択を追加。デジモンRPGの最新作。</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/schedule</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-07 (日付未定)</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>流星のロックマン パーフェクトコレクション</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>カプコン</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>カプコン</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Switch/Switch 2/PS5/PC</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>アクション（コレクション）</t>
+        </is>
+      </c>
+      <c r="K28" t="n">
+        <v>3</v>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>来月予定（評価系空欄）。DSの『流星のロックマン』シリーズをまとめたコレクション。</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/schedule</t>
         </is>
       </c>
     </row>
@@ -25965,7 +26814,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -26355,6 +27204,53 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>IRON NEST（アイアン・ネスト）</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>小規模インディー（独立系）</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>体験版配信（Steam Nextフェス2026年6月）</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>戦術砲撃シミュレーション</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>6/15〜6/22のSteam Nextフェスで『よくプレイされたデモ』として名前が挙がった戦術砲撃シム。配信・ウィッシュリストで露出増。</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Nextフェス期間にデモ体験者・配信が増加（順位・本数の公式値は未取得）</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Nextフェス注目デモ。製品版未発売のため実績は限定的・要追跡。SAO新作『Echoes of Aincrad』やロボFPS『EMPULSE』も同フェスで話題。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
daily-news + cross-questions + events + predictions update (2026-06-26 22:12)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -807,7 +807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1371,6 +1371,80 @@
       <c r="G15" s="17" t="inlineStr">
         <is>
           <t>クロージング発表(6/30前後)の有無、その後の組織再編/人員削減リリース、EA Sports FCの課金・サブスク施策の変化を観測</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B16" s="14" t="inlineStr">
+        <is>
+          <t>メモリ／ストレージ高騰を理由に、SonyがPS5の価格改定（値上げ）を2026年内に実施しMicrosoftの値上げに追随する</t>
+        </is>
+      </c>
+      <c r="C16" s="14" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="D16" s="14" t="inlineStr">
+        <is>
+          <t>年内（2026 H2）</t>
+        </is>
+      </c>
+      <c r="E16" s="14" t="inlineStr">
+        <is>
+          <t>Sony, Microsoft</t>
+        </is>
+      </c>
+      <c r="F16" s="14" t="inlineStr">
+        <is>
+          <t>Microsoft、Xboxを8/1に最大150ドル値上げ（要因はメモリ高騰）（news.xbox, 6/25）</t>
+        </is>
+      </c>
+      <c r="G16" s="14" t="inlineStr">
+        <is>
+          <t>SIEの価格改定リリースの有無、四半期決算でのハード粗利・原価コメント、北米／日本／欧州での改定タイミングを観測する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>Bungieの抽出シューター『Marathon』が、開発体制縮小を受けて発売延期もしくは規模縮小の正式アナウンスに至る</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="D17" s="14" t="inlineStr">
+        <is>
+          <t>数ヶ月後</t>
+        </is>
+      </c>
+      <c r="E17" s="14" t="inlineStr">
+        <is>
+          <t>Sony Interactive Entertainment, Bungie</t>
+        </is>
+      </c>
+      <c r="F17" s="14" t="inlineStr">
+        <is>
+          <t>ソニー、Bungieで292名超レイオフ―Destinyチーム大半とMarathon一部が対象（Game Developer, 6/25）</t>
+        </is>
+      </c>
+      <c r="G17" s="14" t="inlineStr">
+        <is>
+          <t>Bungie／SIEからのMarathon発売日・スコープに関する公式告知、ベータ／テスト日程の変更、開発リーダーの異動を確認する。</t>
         </is>
       </c>
     </row>
@@ -3087,7 +3161,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G48"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4872,6 +4946,43 @@
       <c r="G48" s="5" t="inlineStr">
         <is>
           <t>デジタル化が進む市場でも『新世代ハード』が物理需要を一時的に押し上げる。耐久財の世代交代と在庫戦略の相似形として観察できる</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B49" s="14" t="inlineStr">
+        <is>
+          <t>AIデータセンター起因のメモリ／ストレージ高騰がゲーム機の原価・小売価格を押し上げる構図は、PC・スマホ・自動車・家電など他の電子機器産業の価格にも同時波及するか？</t>
+        </is>
+      </c>
+      <c r="C49" s="14" t="inlineStr">
+        <is>
+          <t>MicrosoftがXboxを8/1に最大150ドル値上げ、要因はAIデータセンター需要によるメモリ2.5倍超の高騰（news.xbox）</t>
+        </is>
+      </c>
+      <c r="D49" s="14" t="inlineStr">
+        <is>
+          <t>Microsoft, Xbox, Sony, Samsung, SK Hynix</t>
+        </is>
+      </c>
+      <c r="E49" s="14" t="inlineStr">
+        <is>
+          <t>PC／スマホ（部材コスト）, 自動車（車載半導体・メモリ）, 家電, データストレージ／クラウド</t>
+        </is>
+      </c>
+      <c r="F49" s="14" t="inlineStr">
+        <is>
+          <t>オープン</t>
+        </is>
+      </c>
+      <c r="G49" s="14" t="inlineStr">
+        <is>
+          <t>AIインフラ投資が川下の民生エレクトロニクス全般の原価を押し上げるクラウドアウト（締め出し）。ゲーム機はその影響が最初に可視化される消費財で、他の耐久財の価格・買い替えサイクルの先行指標になり得る。</t>
         </is>
       </c>
     </row>
@@ -7140,7 +7251,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8159,6 +8270,54 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B21" s="14" t="n"/>
+      <c r="C21" s="14" t="inlineStr">
+        <is>
+          <t>カプコンスポットライト 2026.6</t>
+        </is>
+      </c>
+      <c r="D21" s="14" t="inlineStr">
+        <is>
+          <t>ショーケース</t>
+        </is>
+      </c>
+      <c r="E21" s="14" t="inlineStr">
+        <is>
+          <t>オンライン配信</t>
+        </is>
+      </c>
+      <c r="F21" s="14" t="inlineStr">
+        <is>
+          <t>オンライン</t>
+        </is>
+      </c>
+      <c r="G21" s="14" t="inlineStr">
+        <is>
+          <t>カプコンの主力IPを約30分で紹介するデジタルイベント。『鬼武者 Way of the Sword』（9/25発売）新映像、『DD2 ダークアリズン』（10/9）、『MHStories3』ルディ編DLC（秋）などを発表。</t>
+        </is>
+      </c>
+      <c r="H21" s="14" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/article/202606/79524</t>
+        </is>
+      </c>
+      <c r="I21" s="14" t="inlineStr">
+        <is>
+          <t>終了</t>
+        </is>
+      </c>
+      <c r="J21" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8170,7 +8329,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L211"/>
+  <dimension ref="A1:L219"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -21285,6 +21444,490 @@
         </is>
       </c>
       <c r="L211" s="5" t="n"/>
+    </row>
+    <row r="212">
+      <c r="A212" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B212" s="14" t="inlineStr">
+        <is>
+          <t>ソニー、Bungieで292名以上をレイオフ―『Destiny』チーム大半が対象、スタジオ代表も退任</t>
+        </is>
+      </c>
+      <c r="C212" s="14" t="inlineStr">
+        <is>
+          <t>https://www.gamedeveloper.com/business/sony-is-laying-off-most-of-the-destiny-team-and-some-marathon-devs</t>
+        </is>
+      </c>
+      <c r="D212" s="14" t="inlineStr">
+        <is>
+          <t>Bungieは2022年にSonyが約36億ドルで買収。『Destiny 2』は今月のライブサービス最終大型アップデートで開発が一区切りとなり、次の柱は抽出シューター『Marathon』に移る局面にあった。2026年の業界は世界で3,700人超のレイオフが続いている。</t>
+        </is>
+      </c>
+      <c r="E212" s="14" t="inlineStr">
+        <is>
+          <t>6/25、SIEのHermen Hulstがレイオフを発表。ワシントン州WARN通知では少なくとも292名（ベルビュー拠点分）が対象で、Destinyチームの大半、Marathon開発の一部、SIE横断の支援職に及ぶ。離職は7/9発効。スタジオ代表Justin Trumanも退任し、11年在籍のPoria Torkanが後任に。</t>
+        </is>
+      </c>
+      <c r="F212" s="14" t="inlineStr">
+        <is>
+          <t>・Sony買収後3回目の大型レイオフ（292名超、WARNは拠点分のみ）
+・Destinyライブ運営を大幅縮小、Marathon開発にも一部影響
+・スタジオ代表交代（Justin Truman→Poria Torkan）
+・2026年の業界レイオフ累計は世界で3,700人超</t>
+        </is>
+      </c>
+      <c r="G212" s="14" t="inlineStr">
+        <is>
+          <t>ライブサービス偏重のリスクが顕在化。SIEはMarathonの規模・スケジュール見直しと固定費の再設計を迫られる。買収スタジオの統廃合と、自社IPのライブ運営体制の選別がさらに進む可能性が高い。</t>
+        </is>
+      </c>
+      <c r="H212" s="14" t="inlineStr">
+        <is>
+          <t>プラットフォーマー傘下スタジオのライブサービス採算と統廃合</t>
+        </is>
+      </c>
+      <c r="I212" s="14" t="inlineStr">
+        <is>
+          <t>Sony Interactive Entertainment, Bungie</t>
+        </is>
+      </c>
+      <c r="J212" s="14" t="inlineStr">
+        <is>
+          <t>Destiny 2, Marathon</t>
+        </is>
+      </c>
+      <c r="K212" s="14" t="inlineStr">
+        <is>
+          <t>業績,海外</t>
+        </is>
+      </c>
+      <c r="L212" s="14" t="n"/>
+    </row>
+    <row r="213">
+      <c r="A213" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B213" s="14" t="inlineStr">
+        <is>
+          <t>Microsoft、Xboxを8/1に最大150ドル値上げ―Series Xは799.99ドルへ、AI起因のメモリ高騰が要因</t>
+        </is>
+      </c>
+      <c r="C213" s="14" t="inlineStr">
+        <is>
+          <t>https://news.xbox.com/en-us/2026/06/25/xbox-console-price-update/</t>
+        </is>
+      </c>
+      <c r="D213" s="14" t="inlineStr">
+        <is>
+          <t>ストレージ／メモリ価格がAIデータセンター需要を背景に2.5倍超へ高騰し、2027年秋までにさらに倍増の見通し。Xboxは2026年に入り複数回の値上げを実施しており、今回は年内3回目に当たる。</t>
+        </is>
+      </c>
+      <c r="E213" s="14" t="inlineStr">
+        <is>
+          <t>6/25、Microsoftは8/1から512GBモデルを100ドル、1TBモデルを150ドル値上げすると発表。Series Xは649.99→799.99ドル、Series S 512GBは499.99ドルに。2TBモデルは終売で、Series X本体の生産縮小も報じられた。緩和策として分割払い（BNPL）や認定中古を導入。</t>
+        </is>
+      </c>
+      <c r="F213" s="14" t="inlineStr">
+        <is>
+          <t>・Series X 799.99ドル、Series S 512GB 499.99ドルへ
+・値上げ要因はAIデータセンター起因のメモリ／ストレージ高騰（2.5倍超）
+・2TBモデル終売、Series X生産縮小報道
+・分割払い・認定中古で負担緩和</t>
+        </is>
+      </c>
+      <c r="G213" s="14" t="inlineStr">
+        <is>
+          <t>メモリ高騰はSony等にも波及し、年内のハード価格上昇圧力が継続。PC版Game Passやクラウドへの誘導が強まり、専用機の価値提案と買い替えサイクルが問い直される。</t>
+        </is>
+      </c>
+      <c r="H213" s="14" t="inlineStr">
+        <is>
+          <t>半導体メモリ需給とゲーム機原価・価格戦略</t>
+        </is>
+      </c>
+      <c r="I213" s="14" t="inlineStr">
+        <is>
+          <t>Microsoft, Xbox</t>
+        </is>
+      </c>
+      <c r="J213" s="14" t="inlineStr">
+        <is>
+          <t>Xbox Series X|S</t>
+        </is>
+      </c>
+      <c r="K213" s="14" t="inlineStr">
+        <is>
+          <t>業績,技術,海外</t>
+        </is>
+      </c>
+      <c r="L213" s="14" t="n"/>
+    </row>
+    <row r="214">
+      <c r="A214" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B214" s="14" t="inlineStr">
+        <is>
+          <t>カプコン、カプコンスポットライトで『鬼武者 Way of the Sword』新映像―9/25発売、DD2 DLCも10/9</t>
+        </is>
+      </c>
+      <c r="C214" s="14" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/article/202606/79524</t>
+        </is>
+      </c>
+      <c r="D214" s="14" t="inlineStr">
+        <is>
+          <t>カプコンは自社の最新情報を約30分にまとめたデジタルイベント「カプコンスポットライト」を6/26朝6時に配信（ナレーション：子安武人）。複数の主力IPの発売日・追加コンテンツを一挙に公開した。</t>
+        </is>
+      </c>
+      <c r="E214" s="14" t="inlineStr">
+        <is>
+          <t>番組では『鬼武者 Way of the Sword』の曲者幻魔「怒伐天」との新規バトル映像を公開し、発売日を2026/9/25（通常版8,990円）と告知。あわせて『ドラゴンズドグマ2 ダークアリズン』10/9発売、『モンスターハンターストーリーズ3』ルディ編DLCの秋配信などを発表した。</t>
+        </is>
+      </c>
+      <c r="F214" s="14" t="inlineStr">
+        <is>
+          <t>・『鬼武者 Way of the Sword』2026/9/25発売（通常8,990円）
+・『DD2 ダークアリズン』10/9発売
+・『MHStories3』ルディ編DLC秋配信
+・約30分のショーケースで主力IPの日程を集中告知</t>
+        </is>
+      </c>
+      <c r="G214" s="14" t="inlineStr">
+        <is>
+          <t>カプコンは秋商戦に向け既存IPの新作・追加販売を厚く積む布陣。年末のGTA6・大型タイトルと時期が重なるため、9〜10月への発売集約でカレンダー競合を避ける戦略が鮮明になる。</t>
+        </is>
+      </c>
+      <c r="H214" s="14" t="inlineStr">
+        <is>
+          <t>パブリッシャーのショーケース戦略と発売カレンダー設計</t>
+        </is>
+      </c>
+      <c r="I214" s="14" t="inlineStr">
+        <is>
+          <t>カプコン</t>
+        </is>
+      </c>
+      <c r="J214" s="14" t="inlineStr">
+        <is>
+          <t>鬼武者 Way of the Sword, ドラゴンズドグマ2, モンスターハンターストーリーズ3</t>
+        </is>
+      </c>
+      <c r="K214" s="14" t="inlineStr">
+        <is>
+          <t>新作,国内</t>
+        </is>
+      </c>
+      <c r="L214" s="14" t="n"/>
+    </row>
+    <row r="215">
+      <c r="A215" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B215" s="14" t="inlineStr">
+        <is>
+          <t>『GTA6』予約受付開始―通常79.99ドル／アルティメット99.99ドル、Take-TwoはFY27純予約80億ドル超を予想</t>
+        </is>
+      </c>
+      <c r="C215" s="14" t="inlineStr">
+        <is>
+          <t>https://tech-insider.org/gta-6-pre-orders-june-25-2026/</t>
+        </is>
+      </c>
+      <c r="D215" s="14" t="inlineStr">
+        <is>
+          <t>『GTA6』は2026/11/19にPS5／Xbox Series X|Sで発売予定。AAAの新基準となる79.99ドルの定価が消費者に受容されるかが業界の注目点で、Take-Twoの通期業績は同作が最大のドライバーとなる。</t>
+        </is>
+      </c>
+      <c r="E215" s="14" t="inlineStr">
+        <is>
+          <t>6/25、予約受付が通常版79.99ドル・アルティメット版99.99ドルで開始。Take-TwoはFY2027の純予約（net bookings）ガイダンスを80〜82億ドルとし、GTA6を主因に挙げた。アナリスト予想は初年度35百万本（Piper Sandler）〜85百万本（Konvoy）と大きく割れる。</t>
+        </is>
+      </c>
+      <c r="F215" s="14" t="inlineStr">
+        <is>
+          <t>・予約価格 通常79.99ドル／アルティメット99.99ドル
+・発売は2026/11/19（PS5／Xbox）
+・Take-Two FY27純予約ガイダンス80〜82億ドル
+・初年度販売予想は35M〜85M本と大きく分散</t>
+        </is>
+      </c>
+      <c r="G215" s="14" t="inlineStr">
+        <is>
+          <t>79.99ドル定価の受容度が世代規模で試される。アルティメット版・予約特典による価格分割が定着すれば、他のAAAパブリッシャーも同価格帯へ追随し、フルプライスの基準が一段切り上がる。</t>
+        </is>
+      </c>
+      <c r="H215" s="14" t="inlineStr">
+        <is>
+          <t>AAA定価のアップシフトと予約・特典による価格分割</t>
+        </is>
+      </c>
+      <c r="I215" s="14" t="inlineStr">
+        <is>
+          <t>Take-Two Interactive, Rockstar Games</t>
+        </is>
+      </c>
+      <c r="J215" s="14" t="inlineStr">
+        <is>
+          <t>Grand Theft Auto VI</t>
+        </is>
+      </c>
+      <c r="K215" s="14" t="inlineStr">
+        <is>
+          <t>新作,業績,海外</t>
+        </is>
+      </c>
+      <c r="L215" s="14" t="n"/>
+    </row>
+    <row r="216">
+      <c r="A216" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B216" s="14" t="inlineStr">
+        <is>
+          <t>Circana報告：年末GTA6商戦でPS5／Xboxの品薄懸念―PS5の米5月販売は前年比大幅減</t>
+        </is>
+      </c>
+      <c r="C216" s="14" t="inlineStr">
+        <is>
+          <t>https://gamebastion.com/n/new-report-suggests-retailers-may-run-out-of/515501</t>
+        </is>
+      </c>
+      <c r="D216" s="14" t="inlineStr">
+        <is>
+          <t>市場調査会社Circanaは、GTA6発売を控えた年末にかけて据置ハードの需要が供給を上回る可能性を指摘。米国のPS5販売は2026年5月に前年比で大きく落ち込み、新世代への端境期と価格上昇が重なる局面にある。</t>
+        </is>
+      </c>
+      <c r="E216" s="14" t="inlineStr">
+        <is>
+          <t>Circanaは「GTA6発売前後で小売がPS5／Xboxの在庫を切らす恐れがあり、年末は需要が供給を上回りやすい」と分析。一方でPS5の米5月ユニット販売は前年同月比で大幅減（同社調べ）となり、ハードの世代後半の鈍化とメモリ高騰による値上げ環境が重なる。</t>
+        </is>
+      </c>
+      <c r="F216" s="14" t="inlineStr">
+        <is>
+          <t>・GTA6商戦でPS5／Xbox品薄の可能性
+・PS5の米5月販売は前年比大幅減（Circana）
+・据置ハードは世代後半の鈍化局面
+・メモリ高騰起因の値上げが需要をさらに圧迫</t>
+        </is>
+      </c>
+      <c r="G216" s="14" t="inlineStr">
+        <is>
+          <t>年末はGTA6需要でハード本体が一時的に逼迫する一方、価格上昇が普及の足かせに。メーカーは増産と価格・バンドル戦略の最適化を迫られ、流通は在庫配分の難度が上がる。</t>
+        </is>
+      </c>
+      <c r="H216" s="14" t="inlineStr">
+        <is>
+          <t>ハードのライフサイクル後半の需給と年末商戦の在庫戦略</t>
+        </is>
+      </c>
+      <c r="I216" s="14" t="inlineStr">
+        <is>
+          <t>Sony, Microsoft, Circana, Take-Two</t>
+        </is>
+      </c>
+      <c r="J216" s="14" t="inlineStr">
+        <is>
+          <t>PlayStation 5, Grand Theft Auto VI</t>
+        </is>
+      </c>
+      <c r="K216" s="14" t="inlineStr">
+        <is>
+          <t>業績,海外</t>
+        </is>
+      </c>
+      <c r="L216" s="14" t="n"/>
+    </row>
+    <row r="217">
+      <c r="A217" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B217" s="14" t="inlineStr">
+        <is>
+          <t>格ゲー世界大会EVO 2026がラスベガスで開幕―12タイトル、SF6は4年連続最多2,414名</t>
+        </is>
+      </c>
+      <c r="C217" s="14" t="inlineStr">
+        <is>
+          <t>https://www.techtimes.com/articles/318993/20260624/evo-2026-opens-friday-2xko-makes-arena-debut-capcom-saves-street-fighter-news-sunday.htm</t>
+        </is>
+      </c>
+      <c r="D217" s="14" t="inlineStr">
+        <is>
+          <t>EVO（Evolution Championship Series）は世界最大級の格闘ゲーム大会。タイトル採用や参加者数は各社のeスポーツ投資と新作プロモーションの指標となる。今年はラスベガス会場で6/26〜28に開催。</t>
+        </is>
+      </c>
+      <c r="E217" s="14" t="inlineStr">
+        <is>
+          <t>本戦は12タイトルで実施。Street Fighter 6が4年連続最多の2,414名、TEKKEN 8が1,354名、Riot Games『2XKO』が公式デビューながら1,080名でArena Finals枠を確保した。土日に分けてArena・Showcaseの両ステージで決勝を進行する。</t>
+        </is>
+      </c>
+      <c r="F217" s="14" t="inlineStr">
+        <is>
+          <t>・会場開催（ラスベガス）、本戦12タイトル
+・SF6が4年連続最多エントリー（2,414名）
+・新作『2XKO』『Invincible VS』が初参戦
+・決勝はArena/Showcaseの2ステージ制</t>
+        </is>
+      </c>
+      <c r="G217" s="14" t="inlineStr">
+        <is>
+          <t>新作格ゲー（2XKO等）のEVO初参戦は競技シーン立ち上げの試金石。各社はEVO期間に合わせた新情報投下を強め、大会を新作マーケティングのハブとして活用する流れが続く。</t>
+        </is>
+      </c>
+      <c r="H217" s="14" t="inlineStr">
+        <is>
+          <t>eスポーツ大会のタイトル採用と新作プロモーションの連動</t>
+        </is>
+      </c>
+      <c r="I217" s="14" t="inlineStr">
+        <is>
+          <t>EVO, Riot Games, カプコン, バンダイナムコ</t>
+        </is>
+      </c>
+      <c r="J217" s="14" t="inlineStr">
+        <is>
+          <t>Street Fighter 6, TEKKEN 8, 2XKO</t>
+        </is>
+      </c>
+      <c r="K217" s="14" t="inlineStr">
+        <is>
+          <t>eスポーツ,海外</t>
+        </is>
+      </c>
+      <c r="L217" s="14" t="n"/>
+    </row>
+    <row r="218">
+      <c r="A218" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B218" s="14" t="inlineStr">
+        <is>
+          <t>EAのPIF主導550億ドルLBO、EUの審査が大詰め―外国補助金は7/30、反トラストは7/22が期限</t>
+        </is>
+      </c>
+      <c r="C218" s="14" t="inlineStr">
+        <is>
+          <t>https://www.finance-monthly.com/saudi-pif-ea-buyout-eu-subsidy-clearance/</t>
+        </is>
+      </c>
+      <c r="D218" s="14" t="inlineStr">
+        <is>
+          <t>EAはサウジPIF・Silver Lake・Affinity Partnersによる総額550億ドル（1株210ドル）の非公開化に合意し、株主は2025/12に承認済み。クロージング期限（ロングストップ）は6/30で、残るは各国規制当局の承認。</t>
+        </is>
+      </c>
+      <c r="E218" s="14" t="inlineStr">
+        <is>
+          <t>PIF主導の買収陣営はEUの外国補助金規則（FSR）に基づく承認を申請し、欧州委員会は7/30を判断期限に設定。別途7/22に反トラストの判断期限が置かれた。期限が6/30の最終クロージングを越える形となり、完了時期がずれ込む可能性が出ている。</t>
+        </is>
+      </c>
+      <c r="F218" s="14" t="inlineStr">
+        <is>
+          <t>・取引総額550億ドル（1株210ドル）、史上最大級のLBO
+・EUのFSR審査期限7/30、反トラスト判断7/22
+・規制審査がロングストップ（6/30）を越える可能性
+・買収陣営にサウジPIFが参画</t>
+        </is>
+      </c>
+      <c r="G218" s="14" t="inlineStr">
+        <is>
+          <t>規制クリア後は非公開化を背景にコスト削減・人員整理が進む公算。国家系ファンドによる基幹IP資産の囲い込みが進み、欧州当局の外国補助金審査が今後の大型ディールの分水嶺となる。</t>
+        </is>
+      </c>
+      <c r="H218" s="14" t="inlineStr">
+        <is>
+          <t>外国補助金規則（FSR）と国家系ファンドによるエンタメM&amp;A審査</t>
+        </is>
+      </c>
+      <c r="I218" s="14" t="inlineStr">
+        <is>
+          <t>Electronic Arts, サウジPIF, Silver Lake, Affinity Partners</t>
+        </is>
+      </c>
+      <c r="J218" s="14" t="inlineStr">
+        <is>
+          <t>EA Sports FC, Battlefield</t>
+        </is>
+      </c>
+      <c r="K218" s="14" t="inlineStr">
+        <is>
+          <t>M&amp;A,規制,海外</t>
+        </is>
+      </c>
+      <c r="L218" s="14" t="n"/>
+    </row>
+    <row r="219">
+      <c r="A219" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B219" s="14" t="inlineStr">
+        <is>
+          <t>カプコン、生成AI素材はゲーム本編に実装しない方針を表明―開発の効率化には積極活用</t>
+        </is>
+      </c>
+      <c r="C219" s="14" t="inlineStr">
+        <is>
+          <t>https://news.yahoo.co.jp/articles/1fd3eed6a32319018bf92c575abe07d3ed4546d7</t>
+        </is>
+      </c>
+      <c r="D219" s="14" t="inlineStr">
+        <is>
+          <t>ゲーム業界では大手が二次創作ガイドラインにAI生成物の収益化制限を追記するなど、生成AIの線引きが進む。GDC2026調査では回答者の52%が「AIは業界に悪影響」と回答し、経営と現場の認識差も指摘されている。</t>
+        </is>
+      </c>
+      <c r="E219" s="14" t="inlineStr">
+        <is>
+          <t>カプコンは投資家との質疑応答で、生成AIで作った素材をゲームコンテンツに実装しない方針を明らかにした。一方、開発プロセスの効率化・生産性向上に資する技術としては積極活用する構えで、グラフィック・サウンド・プログラム各職域での活用法を検証中とした。</t>
+        </is>
+      </c>
+      <c r="F219" s="14" t="inlineStr">
+        <is>
+          <t>・生成AI素材はゲーム本編に実装しない
+・開発効率化・生産性向上には積極活用
+・各職域（絵／音／プログラム）で活用法を検証
+・権利・品質リスクを避ける慎重スタンス</t>
+        </is>
+      </c>
+      <c r="G219" s="14" t="inlineStr">
+        <is>
+          <t>「制作の道具としてのAI」と「成果物としてのAI」を切り分ける企業が増える見込み。権利・開示・品質の観点から、AI活用範囲の明文化が国内大手の標準的なIR／ガバナンス論点になる。</t>
+        </is>
+      </c>
+      <c r="H219" s="14" t="inlineStr">
+        <is>
+          <t>生成AIの開発活用と権利・開示ガバナンスの線引き</t>
+        </is>
+      </c>
+      <c r="I219" s="14" t="inlineStr">
+        <is>
+          <t>カプコン</t>
+        </is>
+      </c>
+      <c r="J219" s="14" t="n"/>
+      <c r="K219" s="14" t="inlineStr">
+        <is>
+          <t>技術,規制,国内</t>
+        </is>
+      </c>
+      <c r="L219" s="14" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
refine predictions granularity (non-obvious second-order, narrowed) (2026-06-27 02:31)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -807,7 +807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1382,7 +1382,7 @@
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>メモリ／ストレージ高騰を理由に、SonyがPS5の価格改定（値上げ）を2026年内に実施しMicrosoftの値上げに追随する</t>
+          <t>Xboxの値上げと同時投入された「認定中古・分割払い(BNPL)」を起点に、据置機メーカーが中古/リファービッシュ/与信を公式プログラムとして常設化し、これまで小売・二次流通(GameStop等)が握っていた中古・金融マージンをメーカー側が取り込む垂直統合が進む</t>
         </is>
       </c>
       <c r="C16" s="14" t="inlineStr">
@@ -1392,59 +1392,22 @@
       </c>
       <c r="D16" s="14" t="inlineStr">
         <is>
-          <t>年内（2026 H2）</t>
+          <t>半年〜年内(2026 H2〜2027 H1)</t>
         </is>
       </c>
       <c r="E16" s="14" t="inlineStr">
         <is>
-          <t>Sony, Microsoft</t>
+          <t>Microsoft, Sony, 任天堂, GameStop</t>
         </is>
       </c>
       <c r="F16" s="14" t="inlineStr">
         <is>
-          <t>Microsoft、Xboxを8/1に最大150ドル値上げ（要因はメモリ高騰）（news.xbox, 6/25）</t>
+          <t>Microsoft、Xboxを8/1に最大150ドル値上げ＋認定中古・分割払いを導入(news.xbox / 本日の日次ニュース)</t>
         </is>
       </c>
       <c r="G16" s="14" t="inlineStr">
         <is>
-          <t>SIEの価格改定リリースの有無、四半期決算でのハード粗利・原価コメント、北米／日本／欧州での改定タイミングを観測する。</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="14" t="inlineStr">
-        <is>
-          <t>2026-06-27</t>
-        </is>
-      </c>
-      <c r="B17" s="14" t="inlineStr">
-        <is>
-          <t>Bungieの抽出シューター『Marathon』が、開発体制縮小を受けて発売延期もしくは規模縮小の正式アナウンスに至る</t>
-        </is>
-      </c>
-      <c r="C17" s="14" t="inlineStr">
-        <is>
-          <t>中</t>
-        </is>
-      </c>
-      <c r="D17" s="14" t="inlineStr">
-        <is>
-          <t>数ヶ月後</t>
-        </is>
-      </c>
-      <c r="E17" s="14" t="inlineStr">
-        <is>
-          <t>Sony Interactive Entertainment, Bungie</t>
-        </is>
-      </c>
-      <c r="F17" s="14" t="inlineStr">
-        <is>
-          <t>ソニー、Bungieで292名超レイオフ―Destinyチーム大半とMarathon一部が対象（Game Developer, 6/25）</t>
-        </is>
-      </c>
-      <c r="G17" s="14" t="inlineStr">
-        <is>
-          <t>Bungie／SIEからのMarathon発売日・スコープに関する公式告知、ベータ／テスト日程の変更、開発リーダーの異動を確認する。</t>
+          <t>Sony・任天堂が公式リファービッシュ/分割払いプログラムを拡充するか、メーカー直販の中古/下取りが拡大するか、GameStop等の中古取扱条件・粗利が圧迫されるかを観測する。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
daily-news + cross-questions + events update (2026-06-27 22:14)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -3124,7 +3124,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4946,6 +4946,80 @@
       <c r="G49" s="14" t="inlineStr">
         <is>
           <t>AIインフラ投資が川下の民生エレクトロニクス全般の原価を押し上げるクラウドアウト（締め出し）。ゲーム機はその影響が最初に可視化される消費財で、他の耐久財の価格・買い替えサイクルの先行指標になり得る。</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B50" s="14" t="inlineStr">
+        <is>
+          <t>決済大手(Visa)がeスポーツ/ゲームコミュニティと複数年で組み『越境決済＋コミュニティ投資』を担う動きは、スポーツ・音楽ライブ・小売など他のコミュニティ経済における『決済の埋め込み』の何に該当するか？</t>
+        </is>
+      </c>
+      <c r="C50" s="14" t="inlineStr">
+        <is>
+          <t>EvoがVisaと複数年パートナーシップを締結(Evo, 6/28)</t>
+        </is>
+      </c>
+      <c r="D50" s="14" t="inlineStr">
+        <is>
+          <t>Evo, Visa</t>
+        </is>
+      </c>
+      <c r="E50" s="14" t="inlineStr">
+        <is>
+          <t>金融/決済(エンベデッドファイナンス), スポーツ(リーグ協賛), 音楽ライブ, 小売/EC(越境決済)</t>
+        </is>
+      </c>
+      <c r="F50" s="14" t="inlineStr">
+        <is>
+          <t>オープン</t>
+        </is>
+      </c>
+      <c r="G50" s="14" t="inlineStr">
+        <is>
+          <t>決済ブランドが『場所の協賛』から『コミュニティの決済インフラ＋投資家』へ役割を深め、熱量の高い中規模コミュニティが文化マーケの主戦場になりうる</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B51" s="14" t="inlineStr">
+        <is>
+          <t>競技団体が公式生成AIを全参加者へ平等配布しつつ『使用範囲を試合前後に限定』する線引きは、教育・士業・医療など『AI支援の公平性』が問われる領域で、どんなルール設計の雛形になるか？</t>
+        </is>
+      </c>
+      <c r="C51" s="14" t="inlineStr">
+        <is>
+          <t>FIFAがW杯2026全48チームに生成AI『Football AI Pro』を提供、利用は試合前後に限定(FIFA/Lenovo, 6/28)</t>
+        </is>
+      </c>
+      <c r="D51" s="14" t="inlineStr">
+        <is>
+          <t>FIFA, Lenovo</t>
+        </is>
+      </c>
+      <c r="E51" s="14" t="inlineStr">
+        <is>
+          <t>教育(試験/学習), 士業・コンサル, 医療(診断支援), eスポーツ</t>
+        </is>
+      </c>
+      <c r="F51" s="14" t="inlineStr">
+        <is>
+          <t>オープン</t>
+        </is>
+      </c>
+      <c r="G51" s="14" t="inlineStr">
+        <is>
+          <t>論点が『AIを使うか否か』から『どこまで・誰に平等に許すか』へ移り、組織が公式AIを調達・認証する『公認AIベンダー』の発想が他領域にも広がりうる</t>
         </is>
       </c>
     </row>
@@ -7214,7 +7288,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8281,6 +8355,54 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B22" s="14" t="n"/>
+      <c r="C22" s="14" t="inlineStr">
+        <is>
+          <t>MSI 2026（LoL Mid-Season Invitational）ファイナル</t>
+        </is>
+      </c>
+      <c r="D22" s="14" t="inlineStr">
+        <is>
+          <t>eスポーツ</t>
+        </is>
+      </c>
+      <c r="E22" s="14" t="inlineStr">
+        <is>
+          <t>韓国・大田(Daejeon)</t>
+        </is>
+      </c>
+      <c r="F22" s="14" t="inlineStr">
+        <is>
+          <t>オフライン</t>
+        </is>
+      </c>
+      <c r="G22" s="14" t="inlineStr">
+        <is>
+          <t>『LoL』シーズン中盤の国際大会の決勝。会場で復刻モード『League of Legends Classic』の詳細発表が予定されている。</t>
+        </is>
+      </c>
+      <c r="H22" s="14" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/073/G007372/20260627007/</t>
+        </is>
+      </c>
+      <c r="I22" s="14" t="inlineStr">
+        <is>
+          <t>開催予定</t>
+        </is>
+      </c>
+      <c r="J22" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8292,7 +8414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L219"/>
+  <dimension ref="A1:L225"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -21891,6 +22013,364 @@
         </is>
       </c>
       <c r="L219" s="14" t="n"/>
+    </row>
+    <row r="220">
+      <c r="A220" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B220" s="14" t="inlineStr">
+        <is>
+          <t>Evo、Visaと複数年パートナーシップ締結—越境決済とコミュニティ投資で格ゲーシーンを強化</t>
+        </is>
+      </c>
+      <c r="C220" s="14" t="inlineStr">
+        <is>
+          <t>https://evo.gg/news/evo-and-visa-announce-multi-year-partnership-to-power-the-global-fighting-game-community/</t>
+        </is>
+      </c>
+      <c r="D220" s="14" t="inlineStr">
+        <is>
+          <t>世界最大の格闘ゲーム大会Evoは近年、競技シーンの収益基盤づくりと観客体験・グローバル展開（越境物販/決済）の強化が課題だった。決済大手Visaは文化・コミュニティ領域での露出と越境取引の拡大を狙い、両者の利害が一致した。</t>
+        </is>
+      </c>
+      <c r="E220" s="14" t="inlineStr">
+        <is>
+          <t>EvoはVisaと2028年初頭までの複数年契約を発表。6/26-28のラスベガス大会から始動し、Friday Night Showdownやフラッシュトーナメント、カード会員向け物販割引を提供。2027年からは草の根トーナメント支援など、コミュニティへ再投資する施策へ拡大する。</t>
+        </is>
+      </c>
+      <c r="F220" s="14" t="inlineStr">
+        <is>
+          <t>・2028年初頭までの複数年契約、越境決済と会場体験の強化が狙い
+・初動はEvo Vegas 2026（6/26-28）、Tyler1×Ludwigのエキシビションも実施
+・2027年から草の根大会・新興プレイヤー支援へ拡張</t>
+        </is>
+      </c>
+      <c r="G220" s="14" t="inlineStr">
+        <is>
+          <t>決済・金融ブランドのeスポーツ/ゲームコミュニティへの長期スポンサー参入が増え、単発の大会協賛から『越境決済＋コミュニティ投資』型の継続関与へシフトする可能性。熱量の高い中規模コミュニティがブランドの文化マーケ対象として再評価される。</t>
+        </is>
+      </c>
+      <c r="H220" s="14" t="inlineStr">
+        <is>
+          <t>決済ブランドのコミュニティ×越境EC型スポンサーシップ設計</t>
+        </is>
+      </c>
+      <c r="I220" s="14" t="inlineStr">
+        <is>
+          <t>Evo, Visa, ソニー・インタラクティブエンタテインメント</t>
+        </is>
+      </c>
+      <c r="J220" s="14" t="inlineStr">
+        <is>
+          <t>Street Fighter 6, TEKKEN 8, GUILTY GEAR STRIVE</t>
+        </is>
+      </c>
+      <c r="K220" s="14" t="inlineStr">
+        <is>
+          <t>M&amp;A,eスポーツ,海外</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B221" s="14" t="inlineStr">
+        <is>
+          <t>Krafton『PUBG』にAI僚機『Ella』—NVIDIA ACE活用の新モード『Ally Duo』ベータ開始</t>
+        </is>
+      </c>
+      <c r="C221" s="14" t="inlineStr">
+        <is>
+          <t>https://en.sedaily.com/technology/2026/06/17/krafton-unveils-ally-duo-mode-to-play-pubg-with-ai-teammate</t>
+        </is>
+      </c>
+      <c r="D221" s="14" t="inlineStr">
+        <is>
+          <t>ゲームAIは事前スクリプト型NPCから、文脈を理解し自然言語で対話する『協働可能なAI』へ進化している。KraftonはNVIDIAのACE技術を採用し音声で指示できるAI僚機をPUBGに実装。GPUベンダーはAI機能を新規ハード需要の喚起策と位置づける。</t>
+        </is>
+      </c>
+      <c r="E221" s="14" t="inlineStr">
+        <is>
+          <t>Kraftonは6/17、PUBGの新アーケードモード『Ally Duo』のグローバルベータを開始（〜7/1）。Sanhokマップで対話型AI僚機『Ella』と2人プレイする。NVIDIAの小型LLM(Mistral-Nemo-Minitron 2B)＋音声認識Parakeet＋自社TTS(韓中英対応)で状況と指示をリアルタイム解釈。動作にはRTX(VRAM8GB以上)が必要。</t>
+        </is>
+      </c>
+      <c r="F221" s="14" t="inlineStr">
+        <is>
+          <t>・対話型AI僚機Ella、音声で指示可能（韓・中・英対応）
+・NVIDIA ACE＋小型LLM＋音声認識/合成のオンデバイス構成
+・要GeForce RTX(VRAM8GB以上)、PC限定・Update42.1で実装
+・ベータ期間は6/17〜7/1の限定</t>
+        </is>
+      </c>
+      <c r="G221" s="14" t="inlineStr">
+        <is>
+          <t>オンデバイス対話AIが『ハード要件を満たすほど良い体験』としてGPU/PCの買い替え誘因に組み込まれていく。対話型AIコンパニオンは協力ゲーム以外（チュートリアル・接客的UX）にも波及し、会話品質がゲームの差別化要素になる。</t>
+        </is>
+      </c>
+      <c r="H221" s="14" t="inlineStr">
+        <is>
+          <t>オンデバイス小型LLM＋音声I/Oの対話型ゲームAI構成</t>
+        </is>
+      </c>
+      <c r="I221" s="14" t="inlineStr">
+        <is>
+          <t>Krafton, NVIDIA</t>
+        </is>
+      </c>
+      <c r="J221" s="14" t="inlineStr">
+        <is>
+          <t>PUBG: BATTLEGROUNDS</t>
+        </is>
+      </c>
+      <c r="K221" s="14" t="inlineStr">
+        <is>
+          <t>技術,海外</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B222" s="14" t="inlineStr">
+        <is>
+          <t>FIFA、W杯2026の全48チームに生成AI『Football AI Pro』提供—使用は試合前後に限定</t>
+        </is>
+      </c>
+      <c r="C222" s="14" t="inlineStr">
+        <is>
+          <t>https://cryptobriefing.com/fifa-ai-agent-world-cup-teams/</t>
+        </is>
+      </c>
+      <c r="D222" s="14" t="inlineStr">
+        <is>
+          <t>スポーツとゲーム/AI技術の融合が進み、試合分析に生成AIエージェントを使う動きが拡大している。FIFAはLenovoと共同開発したAIアシスタントを全代表チームに配布する一方、競技の公平性を守るため利用範囲を明確に線引きした。</t>
+        </is>
+      </c>
+      <c r="E222" s="14" t="inlineStr">
+        <is>
+          <t>FIFAは2026 W杯(米・加・墨)に出場する全48チームへ、Lenovoと共同開発の生成AIアシスタント『Football AI Pro』を提供。用途を試合前後の分析に限定し、試合中（ベンチ・ハーフタイム）の利用は禁止。準備の高度化と試合への介入を明確に区別した設計とした。</t>
+        </is>
+      </c>
+      <c r="F222" s="14" t="inlineStr">
+        <is>
+          <t>・全48代表チームに公式配布、Lenovoと共同開発
+・利用は試合前後のみ、試合中の使用は禁止
+・『準備の補助』と『試合への介入』を線引きする統治設計</t>
+        </is>
+      </c>
+      <c r="G222" s="14" t="inlineStr">
+        <is>
+          <t>競技団体が『公式AIツールを全参加者へ平等配布し使用範囲を規定する』モデルが他競技・eスポーツへ波及する可能性。AIの利用是非ではなく『どこまで許すか』のルール整備と、リーグ公認AIベンダーの選定・認証が新たな論点になる。</t>
+        </is>
+      </c>
+      <c r="H222" s="14" t="inlineStr">
+        <is>
+          <t>競技AI利用の公平性ルールと公認AI調達</t>
+        </is>
+      </c>
+      <c r="I222" s="14" t="inlineStr">
+        <is>
+          <t>FIFA, Lenovo</t>
+        </is>
+      </c>
+      <c r="J222" s="14" t="inlineStr">
+        <is>
+          <t>FIFA World Cup 2026</t>
+        </is>
+      </c>
+      <c r="K222" s="14" t="inlineStr">
+        <is>
+          <t>技術,規制,海外</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B223" s="14" t="inlineStr">
+        <is>
+          <t>Riot、『League of Legends Classic』を予告—初期版を再現する復刻モード、詳細は7月MSIで</t>
+        </is>
+      </c>
+      <c r="C223" s="14" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/073/G007372/20260627007/</t>
+        </is>
+      </c>
+      <c r="D223" s="14" t="inlineStr">
+        <is>
+          <t>長寿運営タイトルでは、過去のゲーム体験を懐古コンテンツとして再提供する『復刻』需要が高まっている。Riotは『LoL』の最初期体験（旧チャンピオン性能・旧ルーン/マスタリー・旧アイテム・旧マップ）を再現する新モードを予告した。</t>
+        </is>
+      </c>
+      <c r="E223" s="14" t="inlineStr">
+        <is>
+          <t>Riot Gamesは6/27、過去のLoL体験を再現する特別モード『League of Legends Classic』を発表。開発者動画『200 Years of Experience』で予告し、初期40体のチャンピオンや旧ルーン/マスタリー、レガシーアイテム、旧サモナーズリフトの見た目を復活させる。詳細は7/11のMSI 2026決勝で公開予定。</t>
+        </is>
+      </c>
+      <c r="F223" s="14" t="inlineStr">
+        <is>
+          <t>・初期版LoLを再現する復刻モード、独立サーバではなくゲーム内の特別モード
+・旧チャンピオン性能・旧ルーン/マスタリー・レガシーアイテムを復活
+・1→30の専用レベリング搭載、新アカウント不要
+・詳細は7/11 MSI 2026ファイナル（韓国・大田）で発表予定</t>
+        </is>
+      </c>
+      <c r="G223" s="14" t="inlineStr">
+        <is>
+          <t>長寿タイトルの『当時を遊べる復刻モード』が定番施策化し、新規獲得より既存・離脱ユーザーの呼び戻しとコミュニティ熱量の再点火を狙う運営が増える。eスポーツ大会と復刻発表を連動させ話題を集中させる手法も広がる。</t>
+        </is>
+      </c>
+      <c r="H223" s="14" t="inlineStr">
+        <is>
+          <t>長寿運営タイトルの『復刻モード』によるリテンション設計</t>
+        </is>
+      </c>
+      <c r="I223" s="14" t="inlineStr">
+        <is>
+          <t>Riot Games</t>
+        </is>
+      </c>
+      <c r="J223" s="14" t="inlineStr">
+        <is>
+          <t>League of Legends</t>
+        </is>
+      </c>
+      <c r="K223" s="14" t="inlineStr">
+        <is>
+          <t>新作,eスポーツ,海外</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B224" s="14" t="inlineStr">
+        <is>
+          <t>KURO GAMES『鳴潮』Ver3.5を7/10配信—新属性『電導』と新エリア『夢州・玄方地界』</t>
+        </is>
+      </c>
+      <c r="C224" s="14" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/634/G063420/20260627008/</t>
+        </is>
+      </c>
+      <c r="D224" s="14" t="inlineStr">
+        <is>
+          <t>中国産オープンワールドRPGはグローバル運営の大型アップデートを軸にユーザーを維持する。KURO GAMESの『鳴潮』はストーリー新展開・新エリア・新キャラ・新属性を投入し、リアルコンサート連動など多面的なエンゲージメント施策を展開する。</t>
+        </is>
+      </c>
+      <c r="E224" s="14" t="inlineStr">
+        <is>
+          <t>KURO GAMESは6/27、『鳴潮』アップデートVer.3.5「遺志を紡ぐは剣，夢に響くは歌」を7/10配信と発表。新エリア「夢州・玄方地界」、漂泊者の新属性「電導」、新共鳴者（秧秧・玄翎／穂穂）を実装。PC版は約20GBの容量削減も実施し、コンサートツアー連動パックも用意する。</t>
+        </is>
+      </c>
+      <c r="F224" s="14" t="inlineStr">
+        <is>
+          <t>・配信日は7/10、ストーリー新展開と新エリア追加
+・漂泊者に新属性「電導」、新キャラ2体を前後半で実装
+・PC版で約20GBの容量削減、モバイルもリソース整理を強化
+・リアルコンサートツアー「To the New World」連動パック</t>
+        </is>
+      </c>
+      <c r="G224" s="14" t="inlineStr">
+        <is>
+          <t>グローバル運営の中国産大型タイトルは、アップデートの新規性に加え『容量最適化』『リアルイベント連動』など運営品質・体験設計での差別化競争が進む。属性追加などキャラ拡張ロードマップがガチャ収益の継続性を左右する。</t>
+        </is>
+      </c>
+      <c r="H224" s="14" t="inlineStr">
+        <is>
+          <t>中国産GaaSの大型UPと容量最適化・IPイベント連動</t>
+        </is>
+      </c>
+      <c r="I224" s="14" t="inlineStr">
+        <is>
+          <t>KURO GAMES</t>
+        </is>
+      </c>
+      <c r="J224" s="14" t="inlineStr">
+        <is>
+          <t>鳴潮(Wuthering Waves)</t>
+        </is>
+      </c>
+      <c r="K224" s="14" t="inlineStr">
+        <is>
+          <t>新作,海外</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B225" s="14" t="inlineStr">
+        <is>
+          <t>Cygames『ウマ娘』新育成シナリオ『らっしゃい！トレセン軒！』を6/29追加—テーマは“ラーメン”</t>
+        </is>
+      </c>
+      <c r="C225" s="14" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/414/G041434/20260615028/</t>
+        </is>
+      </c>
+      <c r="D225" s="14" t="inlineStr">
+        <is>
+          <t>『ウマ娘』は育成シナリオの刷新で長期運営の鮮度を保ってきた。今回はラーメンをモチーフにした新シナリオを投入し、「ラーメンWalker」監修協力など実在コンテンツとのコラボで話題化を図る。国内モバイル収益の主力IPの継続強化策。</t>
+        </is>
+      </c>
+      <c r="E225" s="14" t="inlineStr">
+        <is>
+          <t>Cygamesは新育成シナリオ「らっしゃい！トレセン軒！ ～恩返し，始めました～」を6/29に追加。ラーメンをテーマに、地域選び→ラーメン作り学習→トレーニングでコツ習得→試食会で強化→年末「ラーメン・ジャンボリー」で恩返し、という流れ。特効友人サポにSSR駿川たづな、新衣装トプロも実装。</t>
+        </is>
+      </c>
+      <c r="F225" s="14" t="inlineStr">
+        <is>
+          <t>・6/29追加、テーマは“ラーメン”（ラーメンWalker監修協力）
+・地域選択→学習→トレーニング→試食会→RMJの育成サイクル
+・特効友人サポSSR「一杯のノスタルジア」駿川たづな
+・最大80連サポカガチャ無料や新衣装ナリタトップロードも</t>
+        </is>
+      </c>
+      <c r="G225" s="14" t="inlineStr">
+        <is>
+          <t>長期運営モバイルは育成/シナリオの世界観コラボ（食・地域・実在メディア）で鮮度と話題を作り続ける。海外版展開が進む中、国内向けの濃いネタ系シナリオと海外向けの普遍的訴求の二層運営が課題になる。</t>
+        </is>
+      </c>
+      <c r="H225" s="14" t="inlineStr">
+        <is>
+          <t>長寿モバイルの育成シナリオ刷新とコラボ話題設計</t>
+        </is>
+      </c>
+      <c r="I225" s="14" t="inlineStr">
+        <is>
+          <t>Cygames, サイバーエージェント</t>
+        </is>
+      </c>
+      <c r="J225" s="14" t="inlineStr">
+        <is>
+          <t>ウマ娘 プリティーダービー</t>
+        </is>
+      </c>
+      <c r="K225" s="14" t="inlineStr">
+        <is>
+          <t>新作,国内</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add ゲームデザイン・トレンド sheet (design trend tracking) + generator/nav support
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -22,6 +22,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="横断的問い" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="週間ランキング" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="イベントカレンダー" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ゲームデザイン・トレンド" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -31,7 +32,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -89,6 +90,11 @@
       <name val="Calibri"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Yu Gothic"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -129,7 +135,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -171,6 +177,9 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -8408,6 +8417,584 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="18" t="inlineStr">
+        <is>
+          <t>記録日</t>
+        </is>
+      </c>
+      <c r="B1" s="18" t="inlineStr">
+        <is>
+          <t>デザイン名/パターン</t>
+        </is>
+      </c>
+      <c r="C1" s="18" t="inlineStr">
+        <is>
+          <t>分類</t>
+        </is>
+      </c>
+      <c r="D1" s="18" t="inlineStr">
+        <is>
+          <t>ステータス</t>
+        </is>
+      </c>
+      <c r="E1" s="18" t="inlineStr">
+        <is>
+          <t>概要・特徴</t>
+        </is>
+      </c>
+      <c r="F1" s="18" t="inlineStr">
+        <is>
+          <t>代表タイトル</t>
+        </is>
+      </c>
+      <c r="G1" s="18" t="inlineStr">
+        <is>
+          <t>流行/変化の要因</t>
+        </is>
+      </c>
+      <c r="H1" s="18" t="inlineStr">
+        <is>
+          <t>今後の見立て</t>
+        </is>
+      </c>
+      <c r="I1" s="18" t="inlineStr">
+        <is>
+          <t>発火元ニュース</t>
+        </is>
+      </c>
+      <c r="J1" s="18" t="inlineStr">
+        <is>
+          <t>注目度(1-5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B2" s="14" t="inlineStr">
+        <is>
+          <t>対話型AI NPC／AIコンパニオン</t>
+        </is>
+      </c>
+      <c r="C2" s="14" t="inlineStr">
+        <is>
+          <t>技術/UX</t>
+        </is>
+      </c>
+      <c r="D2" s="14" t="inlineStr">
+        <is>
+          <t>台頭</t>
+        </is>
+      </c>
+      <c r="E2" s="14" t="inlineStr">
+        <is>
+          <t>LLM＋音声認識・合成をオンデバイスで動かし、文脈を理解して自然言語で協働するNPCや僚機。事前スクリプト型AIからの脱却。</t>
+        </is>
+      </c>
+      <c r="F2" s="14" t="inlineStr">
+        <is>
+          <t>PUBG「Ella」(Ally Duo)</t>
+        </is>
+      </c>
+      <c r="G2" s="14" t="inlineStr">
+        <is>
+          <t>小型LLMの軽量化とGPUのAI処理能力向上、NVIDIA ACE等のミドルウェア整備。各社が体験差別化策として実装。</t>
+        </is>
+      </c>
+      <c r="H2" s="14" t="inlineStr">
+        <is>
+          <t>会話品質が差別化要素に。高いハード要件が買い替え誘因化する一方、暴走・コスト・倫理面の運用設計が課題。</t>
+        </is>
+      </c>
+      <c r="I2" s="14" t="inlineStr">
+        <is>
+          <t>Krafton『PUBG』Ally Duo/Ella(6/28)</t>
+        </is>
+      </c>
+      <c r="J2" s="14" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B3" s="14" t="inlineStr">
+        <is>
+          <t>エクストラクションシューター</t>
+        </is>
+      </c>
+      <c r="C3" s="14" t="inlineStr">
+        <is>
+          <t>メカニクス/構造</t>
+        </is>
+      </c>
+      <c r="D3" s="14" t="inlineStr">
+        <is>
+          <t>過熱→再評価</t>
+        </is>
+      </c>
+      <c r="E3" s="14" t="inlineStr">
+        <is>
+          <t>高リスク高報酬で物資を「持ち帰る」PvPvE。一時は各社が参入したが、大型タイトルの不振で選別局面に。</t>
+        </is>
+      </c>
+      <c r="F3" s="14" t="inlineStr">
+        <is>
+          <t>Marathon(失速), Escape from Tarkov, ARC Raiders</t>
+        </is>
+      </c>
+      <c r="G3" s="14" t="inlineStr">
+        <is>
+          <t>差別化難・運営負荷・PvPの参入障壁。Sony/BungieのMarathon不振が過熱に冷や水。</t>
+        </is>
+      </c>
+      <c r="H3" s="14" t="inlineStr">
+        <is>
+          <t>ジャンル自体は残るが「大手の旗艦」より中規模・既存IP内モードへ。Bungie人材流出で競争構図が変化。</t>
+        </is>
+      </c>
+      <c r="I3" s="14" t="inlineStr">
+        <is>
+          <t>Sony、Bungieで大量解雇/Marathon減損(6/27)</t>
+        </is>
+      </c>
+      <c r="J3" s="14" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>復刻モード／レガシー再現</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>運営/ナラティブ</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>台頭</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>長寿運営タイトルが過去バージョンを公式に再現し、懐古と話題を喚起する常設/期間限定モード。</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>League of Legends Classic, WoW Classic</t>
+        </is>
+      </c>
+      <c r="G4" s="14" t="inlineStr">
+        <is>
+          <t>長期運営タイトルの新規獲得鈍化、既存・離脱層の呼び戻し需要、コミュニティの懐古熱。</t>
+        </is>
+      </c>
+      <c r="H4" s="14" t="inlineStr">
+        <is>
+          <t>定番施策化。eスポーツ大会との連動で話題集中。運営コストと「現行版の否定にしない」設計が鍵。</t>
+        </is>
+      </c>
+      <c r="I4" s="14" t="inlineStr">
+        <is>
+          <t>Riot『League of Legends Classic』予告(6/28)</t>
+        </is>
+      </c>
+      <c r="J4" s="14" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>ライブサービス／GaaS</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="inlineStr">
+        <is>
+          <t>マネタイズ/運営</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="inlineStr">
+        <is>
+          <t>成熟→選別(逆風)</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="inlineStr">
+        <is>
+          <t>継続課金・長期運営前提の大型タイトル。市場飽和とユーザー時間の奪い合いでサービス終了が相次ぐ。</t>
+        </is>
+      </c>
+      <c r="F5" s="14" t="inlineStr">
+        <is>
+          <t>Destiny 2(縮小), Fortnite, 各種運営型</t>
+        </is>
+      </c>
+      <c r="G5" s="14" t="inlineStr">
+        <is>
+          <t>供給過多・高い運営コスト・ヒット集中。大手が新規GaaS投資を抑制し選択と集中へ。</t>
+        </is>
+      </c>
+      <c r="H5" s="14" t="inlineStr">
+        <is>
+          <t>「広く薄く」から「絞って深く」へ。撤退の作法(返金/プレイ継続)も論点。PvE協力型へのシフト観測。</t>
+        </is>
+      </c>
+      <c r="I5" s="14" t="inlineStr">
+        <is>
+          <t>Bungie/Destiny縮小・大量解雇(6/27)</t>
+        </is>
+      </c>
+      <c r="J5" s="14" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>有料ランダム(ガチャ/ルートボックス)</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>マネタイズ</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>成熟→規制逆風</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>確率型アイテム販売。モバイル収益の柱だが、各国で年齢規制・確率開示義務が強化されている。</t>
+        </is>
+      </c>
+      <c r="F6" s="14" t="inlineStr">
+        <is>
+          <t>モバイルガチャ全般</t>
+        </is>
+      </c>
+      <c r="G6" s="14" t="inlineStr">
+        <is>
+          <t>PEGIが2026年6月以降の新規提出作で有料ランダム含有を最低PEGI16に。EU等で規制が前進。</t>
+        </is>
+      </c>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t>欧州で年齢ゲート化。確定入手(直接購入)・バトルパス比率の上昇など課金設計の見直し圧力。</t>
+        </is>
+      </c>
+      <c r="I6" s="14" t="inlineStr">
+        <is>
+          <t>PEGI新基準(2026年6月施行)</t>
+        </is>
+      </c>
+      <c r="J6" s="14" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>オーセンティシティ(「非AI・人の手」訴求)</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="inlineStr">
+        <is>
+          <t>ナラティブ/マーケ</t>
+        </is>
+      </c>
+      <c r="D7" s="14" t="inlineStr">
+        <is>
+          <t>台頭</t>
+        </is>
+      </c>
+      <c r="E7" s="14" t="inlineStr">
+        <is>
+          <t>生成AI氾濫への反動で「人間が作った」ことを差別化価値として掲げる動き。</t>
+        </is>
+      </c>
+      <c r="F7" s="14" t="inlineStr">
+        <is>
+          <t>一部インディー, Larian等の姿勢</t>
+        </is>
+      </c>
+      <c r="G7" s="14" t="inlineStr">
+        <is>
+          <t>生成AIコンテンツの氾濫とユーザーの真正性選好。プラットフォームのAI開示ルール強化。</t>
+        </is>
+      </c>
+      <c r="H7" s="14" t="inlineStr">
+        <is>
+          <t>「真正性が効率に勝つ」ニッチ市場が形成。AI活用と非AI訴求の二極化が進む。</t>
+        </is>
+      </c>
+      <c r="I7" s="14" t="inlineStr">
+        <is>
+          <t>GDC2026 開発者のAI利用率低下(6/24)</t>
+        </is>
+      </c>
+      <c r="J7" s="14" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>少人数・高生産性開発(AI支援)</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="inlineStr">
+        <is>
+          <t>構造/制作</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>台頭</t>
+        </is>
+      </c>
+      <c r="E8" s="14" t="inlineStr">
+        <is>
+          <t>AIツールで小規模チームが高収益を出すモデル。「少人数で巨額EXIT」が象徴。</t>
+        </is>
+      </c>
+      <c r="F8" s="14" t="inlineStr">
+        <is>
+          <t>小規模スタジオの成功例</t>
+        </is>
+      </c>
+      <c r="G8" s="14" t="inlineStr">
+        <is>
+          <t>生成AI・エンジンの生産性向上、レベニューシェア型の資金供給拡大。</t>
+        </is>
+      </c>
+      <c r="H8" s="14" t="inlineStr">
+        <is>
+          <t>中規模スタジオの新設・独立が増加。大量解雇で流出した熟練人材の受け皿になりうる。</t>
+        </is>
+      </c>
+      <c r="I8" s="14" t="inlineStr">
+        <is>
+          <t>インディー資金・少人数EXIT潮流(6月)</t>
+        </is>
+      </c>
+      <c r="J8" s="14" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>メタバース／Web3・NFTゲーム</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="inlineStr">
+        <is>
+          <t>技術/マネタイズ</t>
+        </is>
+      </c>
+      <c r="D9" s="14" t="inlineStr">
+        <is>
+          <t>衰退</t>
+        </is>
+      </c>
+      <c r="E9" s="14" t="inlineStr">
+        <is>
+          <t>ブロックチェーン資産・仮想空間を軸にしたゲーム。期待先行から縮小・撤退が続く。</t>
+        </is>
+      </c>
+      <c r="F9" s="14" t="inlineStr">
+        <is>
+          <t>各種Web3/NFTゲーム</t>
+        </is>
+      </c>
+      <c r="G9" s="14" t="inlineStr">
+        <is>
+          <t>投機性・規制(PEGIはNFT/ブロックチェーンをPEGI18)・体験価値の薄さ。</t>
+        </is>
+      </c>
+      <c r="H9" s="14" t="inlineStr">
+        <is>
+          <t>大半は淘汰。技術は「所有」より「相互運用・実用」文脈で部分的に残存。</t>
+        </is>
+      </c>
+      <c r="I9" s="14" t="inlineStr">
+        <is>
+          <t>PEGI新基準でNFT=PEGI18(2026年6月)</t>
+        </is>
+      </c>
+      <c r="J9" s="14" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>シングルプレイ大作(物語主導)</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="inlineStr">
+        <is>
+          <t>構造/ナラティブ</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>再評価/復権</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="inlineStr">
+        <is>
+          <t>GaaSの揺り戻しで、買い切り・物語体験の大作が再評価される流れ。</t>
+        </is>
+      </c>
+      <c r="F10" s="14" t="inlineStr">
+        <is>
+          <t>各社の大型シングル作</t>
+        </is>
+      </c>
+      <c r="G10" s="14" t="inlineStr">
+        <is>
+          <t>GaaSの飽和・失敗、確実な収益と評価。大手が外部スタジオ連携・シングル軸へ軌道修正。</t>
+        </is>
+      </c>
+      <c r="H10" s="14" t="inlineStr">
+        <is>
+          <t>「ライブサービス一辺倒」からの修正。超大型作回避の発売時期分散も顕在化。</t>
+        </is>
+      </c>
+      <c r="I10" s="14" t="inlineStr">
+        <is>
+          <t>GaaS縮小・大手戦略観測(6月)</t>
+        </is>
+      </c>
+      <c r="J10" s="14" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="inlineStr">
+        <is>
+          <t>ローグライト／ローグライク</t>
+        </is>
+      </c>
+      <c r="C11" s="14" t="inlineStr">
+        <is>
+          <t>メカニクス</t>
+        </is>
+      </c>
+      <c r="D11" s="14" t="inlineStr">
+        <is>
+          <t>成熟(定番化)</t>
+        </is>
+      </c>
+      <c r="E11" s="14" t="inlineStr">
+        <is>
+          <t>ランダム生成＋周回成長。インディーの定番ジャンルとして安定した人気。</t>
+        </is>
+      </c>
+      <c r="F11" s="14" t="inlineStr">
+        <is>
+          <t>Lost Castle 2, Hades系</t>
+        </is>
+      </c>
+      <c r="G11" s="14" t="inlineStr">
+        <is>
+          <t>リプレイ性・開発規模に対する手応えの良さ、配信映え。</t>
+        </is>
+      </c>
+      <c r="H11" s="14" t="inlineStr">
+        <is>
+          <t>飽和気味だが定番として安定。他ジャンルとの掛け合わせで差別化が進む。</t>
+        </is>
+      </c>
+      <c r="I11" s="14" t="inlineStr">
+        <is>
+          <t>インディー動向(Lost Castle 2等)</t>
+        </is>
+      </c>
+      <c r="J11" s="14" t="n">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
weekly-stocks + IP watch update (2026-06-29 00:29)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -24685,12 +24685,12 @@
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>SGF2026でモンハンWildsのSwitch 2版開発を確認。大型拡張『Wilds: Ascendance』を2027年世界配信と発表。</t>
+          <t>MHワイルズ大型拡張『Ascendance』と新作(2027)発表に続き、関連IP『鬼武者 Way of the Sword』(9/25)体験版が好評。シリーズのSwitch 2展開も進む。</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>MH Wilds: Ascendance(2027)、MH Stories 3: Twisted Reflection(2026/3/13)</t>
+          <t>Monster Hunter Wilds 拡張『Ascendance』展開中。次期ナンバリングは2027年想定。</t>
         </is>
       </c>
       <c r="F11" s="9" t="inlineStr"/>
@@ -24702,7 +24702,7 @@
       <c r="H11" s="9" t="inlineStr"/>
       <c r="I11" s="9" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>
@@ -25204,10 +25204,14 @@
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>英語版が海外売上を前年同期比3.5倍に拡大しCygamesゲーム事業を牽引(FY2Q ゲーム売上+31.2%)。グローバル展開とコラボ施策を継続。</t>
-        </is>
-      </c>
-      <c r="E28" s="9" t="inlineStr"/>
+          <t>6/21に『ウマ娘』韓国語版が配信開始しApp Storeセールス首位を獲得、CyberAgent株反発の材料に。英語版の海外ヒットに続きグローバル展開が加速。</t>
+        </is>
+      </c>
+      <c r="E28" s="9" t="inlineStr">
+        <is>
+          <t>韓国版6/21配信・セルラン1位。英語版好調に続く多言語グローバル展開を推進。</t>
+        </is>
+      </c>
       <c r="F28" s="9" t="inlineStr"/>
       <c r="G28" s="9" t="inlineStr">
         <is>
@@ -25217,7 +25221,7 @@
       <c r="H28" s="9" t="inlineStr"/>
       <c r="I28" s="9" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>
@@ -25239,12 +25243,12 @@
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>Take-Two CEOがGTA6の11/19発売を再明言、本格マーケティングは6月下旬から始動。初年度3,500万本超の販売予測。</t>
+          <t>6/25午前0時にGTA6予約開始、発売日11/19を確定。標準版$79.99・アルティメット版$99.99(限定車両/アパレル同梱)。価格巡り一部失望も予約は活況。</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>Grand Theft Auto VI(2026/11/19)</t>
+          <t>Grand Theft Auto VI: 2026/11/19発売(PS5/Xbox Series X|S)。初年度6,000〜7,000万本予測。</t>
         </is>
       </c>
       <c r="F29" s="9" t="inlineStr"/>
@@ -25256,7 +25260,7 @@
       <c r="H29" s="9" t="inlineStr"/>
       <c r="I29" s="9" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>
@@ -26304,7 +26308,7 @@
       </c>
       <c r="M2" s="9" t="inlineStr">
         <is>
-          <t>6/26に第86期定時株主総会を控え、株価は材料待ちで軟調（6/16→6/19は7,218→7,076円へ軟化、年初来安値6,849円圏）。Switch 2の普及ペースと欧米年末商戦の不振懸念が引き続き重し。時価総額約9.1兆円・PBR2.76倍・予想ROE10.5%。大型ファーストパーティの供給と普及加速が次の株価材料。</t>
+          <t>6/26に第86期定時株主総会を開催。株価は7,000円前後で軟調が続き、年初来安値6,849円圏に接近（6/28時点予想7,430円、当日レンジ約7,005〜7,359円）。過去1年では約-45%と大幅安。FY26はSwitch 2立ち上げで売上2.313兆円(+98.6%)・営業益3,601億円(+27.5%)規模と急回復も、年末商戦と端末普及ペースを見極める材料待ち局面。</t>
         </is>
       </c>
       <c r="N2" s="9" t="inlineStr">
@@ -26324,7 +26328,7 @@
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>
@@ -26359,7 +26363,7 @@
       </c>
       <c r="M3" s="9" t="inlineStr">
         <is>
-          <t>6/19終値3,140円（前日比-3.38%）。PS5は後半サイクルで販売鈍化も、25年度はゲーム以外（音楽・センサー）が牽引し営業利益1.45兆円（+13.4%）。PS6が2027年以降発売との報道が出始め、26年はPS5ソフトで稼ぐ最終局面との見方。アナリストは強気継続で平均目標株価4,674円。</t>
+          <t>PS5はサイクル後半で販売鈍化（直近四半期約800万台・前年比-15%）。メモリ価格高騰でハード採算悪化懸念が重しとなり株価は下落基調（ピークから2割超安）。一方ゲーム・音楽・映画のエンタメ基盤は底堅く本業は崩れていないとの見方。次世代機戦略とライブサービス立て直しが焦点。</t>
         </is>
       </c>
       <c r="N3" s="9" t="inlineStr">
@@ -26379,7 +26383,7 @@
       </c>
       <c r="Q3" s="9" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>
@@ -26414,7 +26418,7 @@
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>6/9ニンダイ告知の『鬼武者 Way of the Sword』(9/25)の体験版が好評。先週発表のモンハン/バイオ新作(2027)期待は継続も、今週は新規材料に乏しく任天堂主導のゲームセクター調整に連れ安。10期連続最高益のIP基盤は不変で、2027年の大型パイプラインとSwitch 2展開が評価軸。</t>
+          <t>『鬼武者 Way of the Sword』(9/25)体験版が好評。先週発表のMHワイルズ大型拡張『Ascendance』・バイオ新作(2027)期待を背景に、6月中旬に株価は一時+5%の3,031円。13期連続増収増益のIP基盤は不変で、2027年の大型パイプラインとSwitch 2展開が評価軸。今週は新規材料に乏しく高値圏もみ合い。</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
@@ -26434,7 +26438,7 @@
       </c>
       <c r="Q4" s="9" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>
@@ -26481,7 +26485,7 @@
       </c>
       <c r="M5" s="9" t="inlineStr">
         <is>
-          <t>『ドラクエ12』の最新情報を公開も発売時期が未定だったため失望売りで株価下落。一方『ドラゴンクエストX オンライン』Ver8『時空の迷い子たち』を6/25実装予定。HD-2D系やFF7リメイク三部作の進捗、コンテンツの集中投下と海外展開が引き続き焦点。</t>
+          <t>6/26終値約2,340円(-0.95%)。5/27公開の『ドラクエ12』が発売時期未定で失望売りした流れが尾を引く。『ドラゴンクエストX オンライン』Ver8を6/25実装。FY26は新作減で減収も不採算整理で営業益+34.9%と収益性改善。FF7リメイク三部作・HD-2D系の進捗と海外展開が引き続き焦点。</t>
         </is>
       </c>
       <c r="N5" s="9" t="inlineStr">
@@ -26501,7 +26505,7 @@
       </c>
       <c r="Q5" s="9" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>
@@ -26548,7 +26552,7 @@
       </c>
       <c r="M6" s="9" t="inlineStr">
         <is>
-          <t>FY26通期は純利益予想を750→860億円、営業利益を1,230億円(+20.7%)へ上方修正。eFootballやIP連動イベントが堅調。MGS/パワプロのIP活用と、アミューズメント・スポーツ・ジムの複合成長が継続テーマ。</t>
+          <t>FY26はデジタルエンタメ主導で2四半期連続最高益更新（Q3累計 売上3,530億・営業益1,017億, +17.4%）。eFootball・遊戯王のグローバル課金が牽引。株価は1.9万円台で堅調。MGS・パワプロ等IP活用とスポーツ・ジム事業の複合成長が継続テーマ。今週は新規開示乏しく高値圏を維持。</t>
         </is>
       </c>
       <c r="N6" s="9" t="inlineStr">
@@ -26568,7 +26572,7 @@
       </c>
       <c r="Q6" s="9" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>
@@ -26615,7 +26619,7 @@
       </c>
       <c r="M7" s="9" t="inlineStr">
         <is>
-          <t>FY26は売上・利益が過去最高を更新、ガンダムIP売上が約7割増と牽引。State of Playで新作『ACE COMBAT 8』を10/2 PS5発売と告知。ガンダム/エルデンリング/アイマス等のIP軸を多面展開する戦略が強み。</t>
+          <t>FY26は売上1兆3,482億・営業益1,895億と過去最高。ガンダムIP売上が約7割増と牽引。State of Playで『ACE COMBAT 8』を10/2 PS5発売と告知済み。6/22株価は約3,644円(+1.48%)。ガンダム/エルデンリング/アイマス等のIPを多面展開する戦略が強み。今週は新作投入ペースが評価軸。</t>
         </is>
       </c>
       <c r="N7" s="9" t="inlineStr">
@@ -26635,7 +26639,7 @@
       </c>
       <c r="Q7" s="9" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>
@@ -26670,7 +26674,7 @@
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>FY26は最終赤字57億円。買収したRovio(313億)・Stakelogic(187億)の減損が直撃し、大型グローバル『Super Game』構想を中止。売上は4,875億円(+14%)も営業利益471億円(-2%)。『龍が如く』『ソニック』等のIP収益化と海外子会社の立て直しが課題。</t>
+          <t>6/26株価約2,140円(-0.14%)。FY26はRovio等の減損で最終赤字も、売上4,875億(+13.7%)・営業益471億(-2.1%)。大型『Super Game』構想中止後はペルソナ/龍が如く/ソニック等の既存グローバルIP収益化と海外子会社立て直しが課題。ペルソナ6を含む新作パイプラインが鍵。</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
@@ -26690,7 +26694,7 @@
       </c>
       <c r="Q8" s="9" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>
@@ -26737,7 +26741,7 @@
       </c>
       <c r="M9" s="9" t="inlineStr">
         <is>
-          <t>FY26は『仁王3』『ゼルダ無双 封印戦記』等が寄与し売上825.4億円(+5.7%)・営業利益366.4億円(+16.4%)と増益。高い営業利益率と財テク収益が特徴。『信長の野望』『三國志』の周年施策や協業タイトルが継続テーマ。</t>
+          <t>FY26は『仁王3』『ゼルダ無双 封印戦記』等が寄与し売上825億(+5.7%)・営業益366億(+16.4%)と増益、高営業利益率と財テク収益が特徴。『信長の野望』『三國志』の周年・協業施策が継続テーマ。今週は新規開示乏しいが、次期は投資増で減益計画の点に留意。</t>
         </is>
       </c>
       <c r="N9" s="9" t="inlineStr">
@@ -26757,7 +26761,7 @@
       </c>
       <c r="Q9" s="9" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>
@@ -26800,7 +26804,7 @@
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>FY26は売上1,713.7億円(+10.7%)も営業利益222.6億円(-16.3%)と減益。スポーツ事業(公営競技等)が成長する一方、主力モンストのデジタルエンタメ減収と費用増が利益を圧迫。新規事業の収益化とモンスト次施策が焦点。</t>
+          <t>FY26は売上1,713.7億(+10.7%)も営業益222.6億(-16.3%)と減益。Q3累計では営業益-22.7%。公営競技等スポーツ事業が成長する一方、主力モンストのデジタルエンタメ減収と費用増が利益を圧迫。今週は新規開示乏しく、新規事業の収益化とモンスト次施策が焦点。</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
@@ -26820,7 +26824,7 @@
       </c>
       <c r="Q10" s="9" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>
@@ -26855,7 +26859,7 @@
       </c>
       <c r="M11" s="9" t="inlineStr">
         <is>
-          <t>今週の適時開示は乏しい。メタバース『REALITY』、投資育成事業、コンシューマ向け新規IPの育成が継続テーマ。ソーシャルゲーム成熟下での新規収益柱の確立が課題。</t>
+          <t>DeNAと共に株価が連騰し、一時2,800円台と2017年11月以来の水準を回復。『ポケポケ(Pokémon TCG Pocket)』のテーマ拡張等が材料視。釣りスタ・REALITY等の既存事業に加え、任天堂系協業IPと新規育成が継続テーマ。今週はゲーム外の多角化進捗が注目点。</t>
         </is>
       </c>
       <c r="N11" s="9" t="inlineStr">
@@ -26875,7 +26879,7 @@
       </c>
       <c r="Q11" s="9" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>
@@ -26918,7 +26922,7 @@
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>今週の新規開示は限定的。Pokémon系協業や横浜DeNAベイスターズ、ライブ配信『Pococha』、ヘルスケア/AI領域が事業の軸。ゲーム新作パイプラインと非ゲーム事業の収益化が引き続き注目。</t>
+          <t>株価は5日続伸し一時2,800円台と2017年11月以来の高値圏を回復。『ポケポケ』のテーマ拡張パック追加が好感された。横浜DeNAベイスターズ、ライブ配信Pococha、ヘルスケア/AI領域が事業の軸。ゲーム新作パイプラインと非ゲーム事業の収益化が引き続き注目。</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
@@ -26938,7 +26942,7 @@
       </c>
       <c r="Q12" s="9" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>
@@ -26973,7 +26977,7 @@
       </c>
       <c r="M13" s="9" t="inlineStr">
         <is>
-          <t>子会社CygamesのFY26 2Q(1-3月)はゲーム事業が売上675億円(+31.2%)・営業利益209億円(+36.3%)と急伸、『ウマ娘』英語版が海外売上3.5倍と牽引。下期に『ホロライブ』ゲーム化を控える。6/22に『Cygames クリエイティブコンテスト2026』開催を告知。AI・広告と新作ゲームの両輪が成長ドライバー。</t>
+          <t>6月下旬株価約1,329円(年初来安値1,204円圏から戻り)。6/21に子会社Cygamesの『ウマ娘』韓国語版が配信開始しApp Storeセールス首位を獲得、株価反発の材料に。FY26 2Qはゲーム事業 売上1,322億(+47.4%)・営業益386億(+106%)と急伸。AI・広告とウマ娘グローバル展開が成長ドライバー。</t>
         </is>
       </c>
       <c r="N13" s="9" t="inlineStr">
@@ -26993,7 +26997,7 @@
       </c>
       <c r="Q13" s="9" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>
@@ -27141,7 +27145,7 @@
       </c>
       <c r="L2" s="9" t="inlineStr">
         <is>
-          <t>6/7のXbox Games Showcaseで『Gears of War: E-Day』『Clockwork Revolution』をコンソール独占と発表、Xbox 25周年記念ハードも公開。『Call of Duty: Modern Warfare 4』(10/23)はDMZ復活を披露し7月にプレイテスト。6/16にGame Pass第2弾を追加。AB統合後のソフト供給とGame Pass拡大が軸。</t>
+          <t>8/1から全世界でXbox本体を値上げ（512GB +$100/1TB +$150）、2TBモデルは販売終了と発表。メモリ/ストレージ価格が2.5倍超に高騰したのが背景。Stifelの目標株価引き下げと値上げ嫌気で6/25に株価-3.8〜4.5%。Xboxはハード収益-33%でマージン圧迫、約1,000名の追加レイオフ計画。Game Pass最適化とCoD/Bethesda供給が軸。</t>
         </is>
       </c>
       <c r="M2" s="9" t="inlineStr">
@@ -27151,7 +27155,7 @@
       </c>
       <c r="N2" s="9" t="inlineStr">
         <is>
-          <t>Xbox事業の連続レイオフ・組織再編、ハード弱含み</t>
+          <t>Xboxハード収益-33%・連続レイオフ・本体値上げによる需要減リスク</t>
         </is>
       </c>
       <c r="O2" s="9" t="inlineStr">
@@ -27161,7 +27165,7 @@
       </c>
       <c r="P2" s="9" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>
@@ -27199,7 +27203,7 @@
       </c>
       <c r="L3" s="9" t="inlineStr">
         <is>
-          <t>6/17 BNN Bloombergの『Hot Picks』でTTWOが推奨され株価は約$230へ+6%。CEOがGTA6の11/19発売を再明言し本格マーケは6月下旬始動。FY27 Net Bookingsガイダンスは$8.0〜8.2bn、GTA6初年度3,500万本超予測。発売実現が史上最高業績の鍵。</t>
+          <t>GTA6予約が6/25午前0時に開始、発売日11/19を確定。標準版$79.99・アルティメット版$99.99。価格巡り一部失望売りも、6/28株価は約$239(レンジ$233〜242)。BofAは買い・目標$368、MorningstarはFY27販売6,000〜7,000万本予測。11/19発売実現が史上最高業績の最大の鍵。</t>
         </is>
       </c>
       <c r="M3" s="9" t="inlineStr">
@@ -27219,7 +27223,7 @@
       </c>
       <c r="P3" s="9" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>
@@ -27257,7 +27261,7 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>PIF・Silver Lake・Affinity主導の$55bn(=1株$210)take-private(史上最大級のLBO)が6/30のlong-stop dateに向け最終盤。残る関門はCFIUS審査で、株価は$210を約$9下回りディールスプレッドが残存。FY26はBattlefield 6が牽引しNet Bookings $8,026m(+9%)と過去最高。</t>
+          <t>PIF/Silver Lake/Affinity主導の$55bn($210/株)take-privateは6/30クローズ目標だが、CFIUS審査が長引きアウトサイドデートは9/28に。データガバナンス（サウジPIFの関与）が規制上の焦点で、6/30完了は不透明に。FY26はBattlefield 6が牽引しNet Bookings $8.03bn(+9%)と過去最高。</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
@@ -27267,17 +27271,17 @@
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>CFIUS審査・クロージング不確実性とディール破談リスク</t>
+          <t>CFIUS審査長期化で6/30完了が不透明、アウトサイドデート9/28</t>
         </is>
       </c>
       <c r="O4" s="9" t="inlineStr">
         <is>
-          <t>$55bn take-privateの6/30までの完了可否(CFIUS)</t>
+          <t>CFIUSクリアランス取得とディール完了時期</t>
         </is>
       </c>
       <c r="P4" s="9" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>
@@ -27311,7 +27315,7 @@
       </c>
       <c r="L5" s="9" t="inlineStr">
         <is>
-          <t>組織再編を継続し、未発表案件と『プリンス・オブ・ペルシャ 時の砂』リメイクを含む計6本を中止、パリ本社で追加人員削減を提案。一方6/16に『AC Shadows』アップデート1.1.11を配信し、State of Playで新作『Rayman』を発表。Tencent出資の専門子会社(Vantage)による主要IP切り出しが進行。</t>
+          <t>共同創業者Claude Guillemot氏が6/20に仏での航空機事故で死去と報道。FY26は営業損失€1.3bn・Net Bookings €1.5bn(-17.4%)。再編で7本中止・6本延期、2028/3までに€2億超のコスト削減を追加。Tencent出資の専門子会社(Vantage)による主要IP切り出しが進行。アナリスト平均は『中立』、目標€5.60。</t>
         </is>
       </c>
       <c r="M5" s="9" t="inlineStr">
@@ -27321,7 +27325,7 @@
       </c>
       <c r="N5" s="9" t="inlineStr">
         <is>
-          <t>年初来は下落、インサイダー売却と黒字化前の不確実性</t>
+          <t>共同創業者の急逝・大幅赤字・度重なる再編で先行き不透明</t>
         </is>
       </c>
       <c r="O5" s="9" t="inlineStr">
@@ -27331,7 +27335,7 @@
       </c>
       <c r="P5" s="9" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>
@@ -27365,7 +27369,7 @@
       </c>
       <c r="L6" s="9" t="inlineStr">
         <is>
-          <t>6/16に総額$2.45bn＋人民元150億の社債発行を完了。ゲームとAI需要が業績を押し上げとの観測。NexonをめぐりNexon Games株が買収観測で急騰したが、Tencentは買収報道を改めて否定。Honor of Kings/PUBG Mobile等の海外展開とAI投資が継続テーマ。</t>
+          <t>8月の取締役会で中間決算・配当を審議予定と発表。ゲームとAI需要が業績を押し上げとの観測。Honor of Kings/PUBG Mobile等の海外展開とRiot/Epic出資網が強み。Nexon買収観測は改めて否定。今週は大きな新規開示は限定的で、AIエージェント収益化と中間期業績が次の焦点。</t>
         </is>
       </c>
       <c r="M6" s="9" t="inlineStr">
@@ -27385,7 +27389,7 @@
       </c>
       <c r="P6" s="9" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>
@@ -27419,12 +27423,12 @@
       </c>
       <c r="L7" s="9" t="inlineStr">
         <is>
-          <t>『Marvel Rivals』が6/18にVer.20260618(シーズン8.5)を配信、新ソーシャルマップ『Hellfire Bay Beach』や夏イベントを追加。同IPはeスポーツ(MRC S8)も本格化。AI部門縮小報道は『事実無根』と否定。Marvel Rivals/Identity V等のグローバルIP運営が成長軸。</t>
+          <t>6/25に香港取引所への二次上場(dual primary listing)を6/30付で発表、アジア投資家層の拡大を狙う。『Marvel Rivals』はシーズン8.5を配信しeスポーツも本格化。高粗利のゲーム課金と強力な新作パイプラインが成長軸。AI部門縮小報道は否定。Ananta等AAA級新作のグローバル成否が鍵。</t>
         </is>
       </c>
       <c r="M7" s="9" t="inlineStr">
         <is>
-          <t>高粗利のゲーム課金と強力な新作パイプライン</t>
+          <t>高粗利ゲーム課金・Marvel Rivals好調・香港二次上場で投資家層拡大</t>
         </is>
       </c>
       <c r="N7" s="9" t="inlineStr">
@@ -27439,7 +27443,7 @@
       </c>
       <c r="P7" s="9" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>
@@ -27473,17 +27477,17 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>『AIファースト』への転換を鮮明にし、Subnautica 2やPalworld Mobileを含む26プロジェクト/2年で12本のパイプラインを提示。主要証券は概ね買い継続で平均目標株価は約₩388,731(上値余地6割超との見方)。PUBGの収益基盤と新規IP/AI活用が評価軸。</t>
+          <t>6/25株価約₩134,69x水準・時価総額約$6.07bn。早期アクセスの『Subnautica 2』は5日で400万本・売上$120M。好調ゆえ旧Unknown Worlds株主への最大$250Mアーンアウト支払い義務が発生（係争中）。Q1営業益約$373MでNexonを抜き韓国ゲーム首位を奪還。新規IPとAIファースト戦略が評価軸。</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>PUBG依存からの脱却、Subnautica 2の大ヒット</t>
+          <t>PUBG依存脱却・Subnautica 2大ヒット・Q1で韓国首位奪還</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>最大$250Mのアーンアウト負担と訴訟、前年営業益の約35%相当</t>
+          <t>最大$250Mアーンアウト負担と関連訴訟</t>
         </is>
       </c>
       <c r="O8" s="9" t="inlineStr">
@@ -27493,7 +27497,7 @@
       </c>
       <c r="P8" s="9" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>
@@ -27527,7 +27531,7 @@
       </c>
       <c r="L9" s="9" t="inlineStr">
         <is>
-          <t>TencentによるNexon買収観測(評価額約$15b)が報じられNexon Games株が急騰したが、Tencentは買収を否定。『メイプルストーリー』『DNF(地下城与勇士)』等の中韓モバイル収益が堅調。Tencent動向と既存IPのライブ運営・新作が注目。</t>
+          <t>KraftonがQ1営業益で韓国ゲーム首位を奪還し、Nexonは2位に。Tencentによる買収観測(評価額約$15b)は当事者が否定済み。『メイプルストーリー』『DNF』等の中韓モバイル収益とARC Raidersの新規寄与が業績を下支え。今週は新規開示乏しく、既存IPのライブ運営と新作展開が注目。</t>
         </is>
       </c>
       <c r="M9" s="9" t="inlineStr">
@@ -27547,7 +27551,7 @@
       </c>
       <c r="P9" s="9" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>
@@ -27581,7 +27585,7 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>二次パブリッシングレーベル『Fellowship Entertainment』設立を発表、LotR/Tomb Raider等の主要IPを束ね2027年にスピンオフ予定。Ubisoftの『Vantage』分社に続く動きで『IP主導のエンタメ企業』への転換を志向。グループ再編とIP価値最大化が継続テーマ。</t>
+          <t>二次パブリッシングレーベル『Fellowship Entertainment』を設立し、LotR/Tomb Raider等の主要IPを束ね2027年にスピンオフ予定。Ubisoftの『Vantage』分社に続く『IP主導エンタメ企業』への転換志向。今週は新規開示乏しいが、グループ再編とIP価値最大化が継続テーマ。</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
@@ -27601,7 +27605,7 @@
       </c>
       <c r="P10" s="9" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>
@@ -27635,7 +27639,7 @@
       </c>
       <c r="L11" s="9" t="inlineStr">
         <is>
-          <t>6/18時点でエンゲージメントが3週連続で改善。『Roblox Kids』『Roblox Select』アカウントを世界展開し、年齢別の安全設計と保護者向け機能を強化。広告・クリエイター経済の拡大とAppLovin/Unityとの競合が注目点。</t>
+          <t>6/28株価約$47.45(レンジ$44.7〜47.7)・時価総額約$297億。Citiのエンゲージメント鈍化指摘で週初に-8.3%急落。年齢確認導入を巡る証券訴訟も浮上。一方ARK(Cathie Wood)が下落局面で約49万株を買い増し、ロシアの利用禁止も解除。年齢別アカウント定着と通期ブッキング回復が鍵。年初来-42%。</t>
         </is>
       </c>
       <c r="M11" s="9" t="inlineStr">
@@ -27645,7 +27649,7 @@
       </c>
       <c r="N11" s="9" t="inlineStr">
         <is>
-          <t>安全機能対応によるユーザー成長の短期摩擦、収益化の遅れ</t>
+          <t>エンゲージメント鈍化懸念・年齢確認巡る証券訴訟・年初来-42%</t>
         </is>
       </c>
       <c r="O11" s="9" t="inlineStr">
@@ -27655,7 +27659,7 @@
       </c>
       <c r="P11" s="9" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>
@@ -27689,7 +27693,7 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>ゲーム/広告/AIクリエイターツールの融合領域でAppLovin・Roblox・Adobeに対する競争ポジションを強化。広告事業(Unity Vector/Grow)の改善とエンジン課金モデルの安定化が株価回復の鍵。</t>
+          <t>ゲーム/広告/AIクリエイターツールの融合領域でAppLovin・Roblox・Adobeに対する競争ポジションを強化。広告事業(Unity Vector/Grow)の改善とエンジン課金モデルの安定化が株価回復の鍵。今週は目立った新規開示は乏しく、Unity AIの収益貢献と広告シェア回復が引き続き焦点。</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
@@ -27709,7 +27713,7 @@
       </c>
       <c r="P12" s="9" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>
@@ -27747,7 +27751,7 @@
       </c>
       <c r="L13" s="9" t="inlineStr">
         <is>
-          <t>AXON広告プラットフォームを6月に世界の広告主へ開放。株価は$468前後(6/21)で4月高値$745から約3割安だが、広告売上は2026年に$3bnへ倍増見込み、EBITDAマージン80%超・FCFガイダンス$12.5bn。eコマース広告の立ち上がりとマージン維持が焦点。</t>
+          <t>AXON AI広告基盤を6月下旬に全世界の広告主へセルフサーブ開放。Q1はEPS・売上が予想を上回りQ2ガイダンスも上振れ、年率+30.4%成長・FCFマージン71.9%。一方CEO・取締役の大量株式売却(6月中旬)が嫌気され6/25に-3.6%。Citiは買い・目標$710。全面開放の実行リスクとマージン維持が焦点。</t>
         </is>
       </c>
       <c r="M13" s="9" t="inlineStr">
@@ -27757,17 +27761,17 @@
       </c>
       <c r="N13" s="9" t="inlineStr">
         <is>
-          <t>AXON全面開放の実行リスクと高バリュエーション</t>
+          <t>AXON全面開放の実行・希薄化リスクと幹部の大量株式売却</t>
         </is>
       </c>
       <c r="O13" s="9" t="inlineStr">
         <is>
-          <t>AXONグローバル開放の成果と広告外領域への拡張</t>
+          <t>AXONグローバル開放の成果とeコマース広告の立ち上がり</t>
         </is>
       </c>
       <c r="P13" s="9" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
daily-news + cross-questions + events + predictions + game-design update (2026-06-30)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -816,7 +816,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1417,6 +1417,43 @@
       <c r="G16" s="14" t="inlineStr">
         <is>
           <t>Sony・任天堂が公式リファービッシュ/分割払いプログラムを拡充するか、メーカー直販の中古/下取りが拡大するか、GameStop等の中古取扱条件・粗利が圧迫されるかを観測する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>PEGIの新区分で課金カードパックが最低PEGI 16となるのを避けるため、EA Sports FCやeFootball等のマス向けスポーツ系が『有料ランダム』を縮小し、確定報酬型（直接購入/バトルパス/段階開封）へ設計転換。Ultimate Team型ガチャを生んだ当ジャンルから、確定型マネタイズへの構造シフトが起きる</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="D17" s="14" t="inlineStr">
+        <is>
+          <t>次のスポーツ年次作サイクル（2026 H2〜2027）</t>
+        </is>
+      </c>
+      <c r="E17" s="14" t="inlineStr">
+        <is>
+          <t>Electronic Arts, Konami, PEGI</t>
+        </is>
+      </c>
+      <c r="F17" s="14" t="inlineStr">
+        <is>
+          <t>PEGI、新リスク区分を6月適用—課金ルートボックス含む新規申請は最低PEGI 16(VGC, 2026-06-30 日次)</t>
+        </is>
+      </c>
+      <c r="G17" s="14" t="inlineStr">
+        <is>
+          <t>EA Sports FC 27/eFootballの次年度版のPEGIレーティングと、パック（Ultimate Team）課金の仕様変更（確率配布→確定/選択購入）の有無を観測。低年齢レーティング維持の動きが出るか。</t>
         </is>
       </c>
     </row>
@@ -3133,7 +3170,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5029,6 +5066,43 @@
       <c r="G51" s="14" t="inlineStr">
         <is>
           <t>論点が『AIを使うか否か』から『どこまで・誰に平等に許すか』へ移り、組織が公式AIを調達・認証する『公認AIベンダー』の発想が他領域にも広がりうる</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B52" s="14" t="inlineStr">
+        <is>
+          <t>課金メカニクス（ルートボックス等）の有無を年齢レーティングに自動的に内包させるPEGIの『リスク区分』方式は、金融商品のリスク表示・食品の成分/警告表示・たばこの注意喚起など、他業界の『製品ラベルへのリスク内包』と同じ規制思想か？ゲームで先行した設計は他業界の表示規制をどう先取り/追随するか</t>
+        </is>
+      </c>
+      <c r="C52" s="14" t="inlineStr">
+        <is>
+          <t>PEGIが新リスク区分を6月適用、課金ルートボックス含む新規申請は最低PEGI 16(VGC, 2026-06)</t>
+        </is>
+      </c>
+      <c r="D52" s="14" t="inlineStr">
+        <is>
+          <t>PEGI, EA, Konami</t>
+        </is>
+      </c>
+      <c r="E52" s="14" t="inlineStr">
+        <is>
+          <t>金融(商品リスク表示), 食品(成分/警告表示), たばこ(注意喚起), 広告/消費者保護</t>
+        </is>
+      </c>
+      <c r="F52" s="14" t="inlineStr">
+        <is>
+          <t>オープン</t>
+        </is>
+      </c>
+      <c r="G52" s="14" t="inlineStr">
+        <is>
+          <t>規制の論点が『行為の禁止』から『リスクを製品ラベルに強制内包』へ移行。設計（マネタイズ）そのものが格付け対象になる点が金融商品の適合性原則に近い。</t>
         </is>
       </c>
     </row>
@@ -7459,12 +7533,12 @@
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>開催中</t>
+          <t>終了</t>
         </is>
       </c>
       <c r="J3" s="5" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
     </row>
@@ -8307,12 +8381,12 @@
       </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
-          <t>開催中</t>
+          <t>終了</t>
         </is>
       </c>
       <c r="J20" s="5" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-30</t>
         </is>
       </c>
     </row>
@@ -8693,7 +8767,7 @@
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
@@ -8708,7 +8782,7 @@
       </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
-          <t>成熟→規制逆風</t>
+          <t>成熟→規制逆風（区分強化で加速）</t>
         </is>
       </c>
       <c r="E6" s="14" t="inlineStr">
@@ -8728,12 +8802,12 @@
       </c>
       <c r="H6" s="14" t="inlineStr">
         <is>
-          <t>欧州で年齢ゲート化。確定入手(直接購入)・バトルパス比率の上昇など課金設計の見直し圧力。</t>
+          <t>PEGIの新リスク区分で課金ルートボックスは最低PEGI 16に。低年齢レーティング維持のため確定報酬型（直接購入/バトルパス）への置換が進む見込み。NFTはPEGI 18でWeb3型の逆風も継続。</t>
         </is>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
-          <t>PEGI新基準(2026年6月施行)</t>
+          <t>PEGI新リスク区分が6月適用、課金ルートボックス含む新規申請は最低PEGI 16(VGC, 2026-06-30)</t>
         </is>
       </c>
       <c r="J6" s="14" t="n">
@@ -9001,7 +9075,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L225"/>
+  <dimension ref="A1:L228"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -22956,6 +23030,187 @@
       <c r="K225" s="14" t="inlineStr">
         <is>
           <t>新作,国内</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B226" s="14" t="inlineStr">
+        <is>
+          <t>PEGI、新「インタラクティブ・リスク区分」を6月から適用開始—課金ルートボックス含む新規申請は最低PEGI 16</t>
+        </is>
+      </c>
+      <c r="C226" s="14" t="inlineStr">
+        <is>
+          <t>https://www.videogameschronicle.com/news/all-games-with-loot-boxes-in-them-will-be-rated-minimum-pegi-16-starting-this-summer/</t>
+        </is>
+      </c>
+      <c r="D226" s="14" t="inlineStr">
+        <is>
+          <t>欧州のレーティング機関PEGIは3月12日、10年超で最大規模の改革を発表。マネタイズ・コミュニケーション・エンゲージメント設計を年齢区分に統合する新枠組みを示し、その適用が6月から始まった。ルートボックス規制を巡る欧州各国の動きが背景。</t>
+        </is>
+      </c>
+      <c r="E226" s="14" t="inlineStr">
+        <is>
+          <t>PEGIは新規申請タイトルから新区分を適用。実装課金の『有料ランダムアイテム（ルートボックス）』を含むゲームは原則最低PEGI 16、期間/数量限定の購入訴求は最低PEGI 12、NFT/ブロックチェーン要素は自動でPEGI 18となる。既存タイトルは更新時を除き再判定なし。</t>
+        </is>
+      </c>
+      <c r="F226" s="14" t="inlineStr">
+        <is>
+          <t>・新区分の適用は2026年6月の新規申請から
+・ルートボックス→最低PEGI 16（スポーツ系の低年齢タイトルが直撃）
+・期間/数量限定オファー→最低PEGI 12
+・NFT/ブロックチェーン→自動PEGI 18
+・既存タイトルは原則再判定なし</t>
+        </is>
+      </c>
+      <c r="G226" s="14" t="inlineStr">
+        <is>
+          <t>課金設計そのものが年齢区分に直結するため、FIFA系(EA Sports FC)やeFootball等のマス向け課金カードパックを持つタイトルは、レーティング維持のため確定報酬型へ設計変更を迫られる可能性。欧州発の枠組みが他地域のレーティングにも波及しうる。</t>
+        </is>
+      </c>
+      <c r="H226" s="14" t="inlineStr">
+        <is>
+          <t>課金メカニクスと年齢レーティングの統合（リスクベース表示）</t>
+        </is>
+      </c>
+      <c r="I226" s="14" t="inlineStr">
+        <is>
+          <t>PEGI, Electronic Arts, Konami</t>
+        </is>
+      </c>
+      <c r="J226" s="14" t="inlineStr">
+        <is>
+          <t>EA Sports FC, eFootball</t>
+        </is>
+      </c>
+      <c r="K226" s="14" t="inlineStr">
+        <is>
+          <t>規制,海外</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B227" s="14" t="inlineStr">
+        <is>
+          <t>Roblox、UKで年齢別アカウント「Roblox Kids／Roblox Select」を6月導入—Ofcomの是正圧力下で顔推定の年齢確認を全面化</t>
+        </is>
+      </c>
+      <c r="C227" s="14" t="inlineStr">
+        <is>
+          <t>https://www.ofcom.org.uk/online-safety/protecting-children/keep-underage-children-off-your-platforms-ofcom-tells-tech-firms</t>
+        </is>
+      </c>
+      <c r="D227" s="14" t="inlineStr">
+        <is>
+          <t>英Ofcomはオンライン安全法に基づき、Roblox・Meta・TikTok等に未成年保護の強化（最低年齢の実効化・グルーミング対策・年齢確認）を要求。Robloxは1月にチャット利用で顔年齢推定を必須化しており、その延長線上の対応。</t>
+        </is>
+      </c>
+      <c r="E227" s="14" t="inlineStr">
+        <is>
+          <t>RobloxはUK向けに年齢帯別アカウント『Roblox Kids（5-8歳）』『Roblox Select（9-15歳）』を6月に導入。チェックボックスでの自己申告では不可となり、顔年齢推定など実効的な年齢確認に基づき保護機能を出し分ける。</t>
+        </is>
+      </c>
+      <c r="F227" s="14" t="inlineStr">
+        <is>
+          <t>・年齢帯別アカウント Kids(5-8)/Select(9-15) をUKで導入
+・自己申告のみでは非準拠、顔推定等で年齢を確認/推定
+・Ofcomが主要プラットフォームへ是正を要求
+・年齢に応じてチャット/コンテンツ保護を出し分け</t>
+        </is>
+      </c>
+      <c r="G227" s="14" t="inlineStr">
+        <is>
+          <t>年齢確認(age assurance)はUGCプラットフォームの標準要件化が進み、Roblox型の年齢帯別UXが他のUGC/ソーシャルゲームにも波及。確認コストとUX摩擦が新規ユーザー獲得の論点になる。</t>
+        </is>
+      </c>
+      <c r="H227" s="14" t="inlineStr">
+        <is>
+          <t>Age assurance（年齢確認）とUGCプラットフォーム規制</t>
+        </is>
+      </c>
+      <c r="I227" s="14" t="inlineStr">
+        <is>
+          <t>Roblox, Ofcom</t>
+        </is>
+      </c>
+      <c r="J227" s="14" t="inlineStr">
+        <is>
+          <t>Roblox</t>
+        </is>
+      </c>
+      <c r="K227" s="14" t="inlineStr">
+        <is>
+          <t>規制,海外</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B228" s="14" t="inlineStr">
+        <is>
+          <t>Valve『Steam Machine』予約抽選が締切—当選者への購入招待が6/29週から順次、72時間の購入枠</t>
+        </is>
+      </c>
+      <c r="C228" s="14" t="inlineStr">
+        <is>
+          <t>https://www.techtimes.com/articles/319082/20260625/steam-summer-sale-2026-live-90-deals-pc-games-machine-lottery-closes.htm</t>
+        </is>
+      </c>
+      <c r="D228" s="14" t="inlineStr">
+        <is>
+          <t>Valveは新型据置機『Steam Machine』を投入予定で、需要把握のため予約抽選方式を採用。サマーセール(6/25-7/9)と同時並行で抽選が締め切られた。SteamOS据置機の本格普及の試金石。</t>
+        </is>
+      </c>
+      <c r="E228" s="14" t="inlineStr">
+        <is>
+          <t>『Steam Machine』の予約抽選が締め切られ、当選者への購入招待が6/29の週から順次配信される。当選者は72時間以内に注文を確定する必要があり、抽選＋時間制限枠という需給管理型の販売手法が採られた。</t>
+        </is>
+      </c>
+      <c r="F228" s="14" t="inlineStr">
+        <is>
+          <t>・予約抽選が締切、招待は6/29週から順次配信
+・当選者は72時間以内に購入確定が必要
+・サマーセール(6/25-7/9)と同時並行
+・SteamOS据置機の普及に向けた需給管理型販売</t>
+        </is>
+      </c>
+      <c r="G228" s="14" t="inlineStr">
+        <is>
+          <t>抽選＋短時間購入枠は転売抑制と需要観測を兼ねる。SteamOS据置機が一定数普及すれば、SteamOS対応のサードパーティ製リビング向けハードや最適化対応が広がる契機になりうる。</t>
+        </is>
+      </c>
+      <c r="H228" s="14" t="inlineStr">
+        <is>
+          <t>SteamOS据置機の普及と需給管理型ハード販売</t>
+        </is>
+      </c>
+      <c r="I228" s="14" t="inlineStr">
+        <is>
+          <t>Valve</t>
+        </is>
+      </c>
+      <c r="J228" s="14" t="inlineStr">
+        <is>
+          <t>Steam Machine, SteamOS</t>
+        </is>
+      </c>
+      <c r="K228" s="14" t="inlineStr">
+        <is>
+          <t>技術,海外</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
daily-news + cross-questions + events + predictions + game-design update (2026-07-01)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -816,7 +816,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1454,6 +1454,43 @@
       <c r="G17" s="14" t="inlineStr">
         <is>
           <t>EA Sports FC 27/eFootballの次年度版のPEGIレーティングと、パック（Ultimate Team）課金の仕様変更（確率配布→確定/選択購入）の有無を観測。低年齢レーティング維持の動きが出るか。</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B18" s="14" t="inlineStr">
+        <is>
+          <t>ライセンスIP発タイトル(『Marvel’s Blade』)の開発中止・採算難を機に、IPホルダー(Disney/Marvel等)がゲーム化を『専属スタジオへの長期委託』から『プロジェクト単位の短期受託/レベニューシェア(映画の製作委員会型)』へ契約形態を切り替える動きが出る。</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="D18" s="14" t="inlineStr">
+        <is>
+          <t>12ヶ月以内(2026 H2〜2027 H1)</t>
+        </is>
+      </c>
+      <c r="E18" s="14" t="inlineStr">
+        <is>
+          <t>Microsoft, Arkane, Marvel, Disney</t>
+        </is>
+      </c>
+      <c r="F18" s="14" t="inlineStr">
+        <is>
+          <t>Microsoft、Arkane閉鎖と『Marvel’s Blade』中止を検討(Game Informer/The Verge, 7/1付日次)</t>
+        </is>
+      </c>
+      <c r="G18" s="14" t="inlineStr">
+        <is>
+          <t>Marvel/Disney発の新規ゲーム契約の形態(短期受託・RevShare・複数社分担)発表の有無、他ライセンスIPゲームの開発体制変更を観測する。</t>
         </is>
       </c>
     </row>
@@ -3170,7 +3207,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G52"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5103,6 +5140,80 @@
       <c r="G52" s="14" t="inlineStr">
         <is>
           <t>規制の論点が『行為の禁止』から『リスクを製品ラベルに強制内包』へ移行。設計（マネタイズ）そのものが格付け対象になる点が金融商品の適合性原則に近い。</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B53" s="14" t="inlineStr">
+        <is>
+          <t>IPを持つ制作スタジオを『閉鎖』せず『売却・スピンオフ』して二次流通させるプラットフォーマーの動きは、映画スタジオのライブラリ売買や音楽カタログ取引と同じ構造になるか？</t>
+        </is>
+      </c>
+      <c r="C53" s="14" t="inlineStr">
+        <is>
+          <t>Microsoftが Arkane等5スタジオの閉鎖でなく売却を模索(The Verge報道, 6/30)</t>
+        </is>
+      </c>
+      <c r="D53" s="14" t="inlineStr">
+        <is>
+          <t>Microsoft, Arkane, Marvel</t>
+        </is>
+      </c>
+      <c r="E53" s="14" t="inlineStr">
+        <is>
+          <t>映画(ライブラリ売買), 音楽(カタログ取引), PE/M&amp;A</t>
+        </is>
+      </c>
+      <c r="F53" s="14" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="G53" s="14" t="inlineStr">
+        <is>
+          <t>『IP＋制作チーム』が映画ライブラリのように資産取引される兆し。買い手がPEか中東SWFか事業会社かで業界の所有構造が変わる。</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B54" s="14" t="inlineStr">
+        <is>
+          <t>人気ゲームが著名アーティスト(YOASOBI)に作品世界連動の楽曲を『書き下ろし発注』しIPを拡張する動きは、広告・アニメ・ブランドのアーティストタイアップと何が同じで何が違うか？</t>
+        </is>
+      </c>
+      <c r="C54" s="14" t="inlineStr">
+        <is>
+          <t>『オーバーウォッチ』×YOASOBI、書き下ろし新曲『オリオン』を実装(4Gamer, 6/30)</t>
+        </is>
+      </c>
+      <c r="D54" s="14" t="inlineStr">
+        <is>
+          <t>Blizzard, YOASOBI, OW</t>
+        </is>
+      </c>
+      <c r="E54" s="14" t="inlineStr">
+        <is>
+          <t>音楽(タイアップ/原盤), 広告, アニメ</t>
+        </is>
+      </c>
+      <c r="F54" s="14" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="G54" s="14" t="inlineStr">
+        <is>
+          <t>ゲームが『発注主』として音楽制作を駆動する構図。IP相互送客の経済圏が広告タイアップより深い世界観統合に向かう可能性。</t>
         </is>
       </c>
     </row>
@@ -7371,7 +7482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8486,6 +8597,54 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="n"/>
+      <c r="C23" s="14" t="inlineStr">
+        <is>
+          <t>スプラトゥーン レイダース Direct 2026.6.30</t>
+        </is>
+      </c>
+      <c r="D23" s="14" t="inlineStr">
+        <is>
+          <t>ショーケース</t>
+        </is>
+      </c>
+      <c r="E23" s="14" t="inlineStr">
+        <is>
+          <t>オンライン</t>
+        </is>
+      </c>
+      <c r="F23" s="14" t="inlineStr">
+        <is>
+          <t>配信(約15分)</t>
+        </is>
+      </c>
+      <c r="G23" s="14" t="inlineStr">
+        <is>
+          <t>シリーズ初スピンオフ『スプラトゥーン レイダース』(Switch 2/7-23発売)の情報を公開。新主人公『メカニック』とすりみ連合の協力アクションADV。</t>
+        </is>
+      </c>
+      <c r="H23" s="14" t="inlineStr">
+        <is>
+          <t>https://www.nintendo.com/jp/nintendo-direct/20260630/index.html</t>
+        </is>
+      </c>
+      <c r="I23" s="14" t="inlineStr">
+        <is>
+          <t>終了</t>
+        </is>
+      </c>
+      <c r="J23" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8497,7 +8656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9064,6 +9223,56 @@
         <v>3</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>外部IP・アーティスト連携型コラボ・ライブオプス</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>運営/マネタイズ</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>流行中</t>
+        </is>
+      </c>
+      <c r="E12" s="14" t="inlineStr">
+        <is>
+          <t>ライブサービス/対戦タイトルが外部の文化IPや著名アーティストとコラボし、書き下ろし楽曲・ゲストキャラ・限定スキンを定期投入してリテンションと話題性を設計する運営の型。単発販促でなく作品世界に統合する点が特徴。</t>
+        </is>
+      </c>
+      <c r="F12" s="14" t="inlineStr">
+        <is>
+          <t>オーバーウォッチ(×YOASOBI), 餓狼伝説CotW(×北斗の拳), Fortnite</t>
+        </is>
+      </c>
+      <c r="G12" s="14" t="inlineStr">
+        <is>
+          <t>新規流入鈍化の中、既存IPの相互送客と話題波及でCACを抑えつつ稼働を維持する効率の良さ。音楽・アニメ側もファン拡張の場として歓迎。</t>
+        </is>
+      </c>
+      <c r="H12" s="14" t="inlineStr">
+        <is>
+          <t>ライブサービスの標準運営として定着。コラボ調達力・世界観統合の巧拙が差別化要因に。質より量の乱発はノイズ化リスク。</t>
+        </is>
+      </c>
+      <c r="I12" s="14" t="inlineStr">
+        <is>
+          <t>OW×YOASOBI(7/1開幕)/餓狼伝説CotW×北斗の拳ケンシロウ(6/29)</t>
+        </is>
+      </c>
+      <c r="J12" s="14" t="n">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9075,7 +9284,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L228"/>
+  <dimension ref="A1:L232"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -23211,6 +23420,266 @@
       <c r="K228" s="14" t="inlineStr">
         <is>
           <t>技術,海外</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B229" s="14" t="inlineStr">
+        <is>
+          <t>Microsoft、Arkane Studios閉鎖と『Marvel’s Blade』中止を検討―7/6開始の大規模リストラで5スタジオが対象に</t>
+        </is>
+      </c>
+      <c r="C229" s="14" t="inlineStr">
+        <is>
+          <t>https://gameinformer.com/2026/06/30/report-microsoft-is-considering-shutting-down-arkane-studios-and-canceling-marvels-blade</t>
+        </is>
+      </c>
+      <c r="D229" s="14" t="inlineStr">
+        <is>
+          <t>Xboxは新CEO体制下で記録的収益にもかかわらず採算改善とコスト削減を進める『リセット』方針を打ち出しており、Activision Blizzard買収後の組織肥大と低採算スタジオの整理が課題となっていた。</t>
+        </is>
+      </c>
+      <c r="E229" s="14" t="inlineStr">
+        <is>
+          <t>The Verge報道として、MicrosoftがArkane Studios閉鎖と開発中の『Marvel’s Blade』中止を検討中と6/30に伝わった。Bladeは予算超過で2026年内発売が困難。閉鎖検討対象はCompulsion、Double Fine、Ninja Theory、Undead Labsを含む最大5スタジオ規模で、リストラは7/6開始の見込み。</t>
+        </is>
+      </c>
+      <c r="F229" s="14" t="inlineStr">
+        <is>
+          <t>Arkaneは閉鎖でなく『売却』も模索中
+の対象は計5スタジオ・約500人＋他部門1,000人規模との観測
+『Marvel’s Blade』は2027年後半へ延期後に中止リスク
+7/6にレイオフ開始予定、Microsoftは未公表</t>
+        </is>
+      </c>
+      <c r="G229" s="14" t="inlineStr">
+        <is>
+          <t>ファーストパーティの選別が進み、IPを持つ中堅スタジオは閉鎖より売却・スピンオフへ向かう可能性。熟練人材の流出と独立スタジオ新設、ライセンスIP(Marvel)ゲームの座組み見直しが連鎖しうる。</t>
+        </is>
+      </c>
+      <c r="H229" s="14" t="inlineStr">
+        <is>
+          <t>プラットフォーマーのスタジオ再編とIP資産化</t>
+        </is>
+      </c>
+      <c r="I229" s="14" t="inlineStr">
+        <is>
+          <t>Microsoft, Xbox, Arkane Studios, Marvel, Disney</t>
+        </is>
+      </c>
+      <c r="J229" s="14" t="inlineStr">
+        <is>
+          <t>Marvel’s Blade, Dishonored, Prey, Deathloop</t>
+        </is>
+      </c>
+      <c r="K229" s="14" t="inlineStr">
+        <is>
+          <t>業績,海外</t>
+        </is>
+      </c>
+      <c r="L229" s="14" t="inlineStr">
+        <is>
+          <t>出典:Game Informer(The Verge報道)</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B230" s="14" t="inlineStr">
+        <is>
+          <t>任天堂、『スプラトゥーン レイダース』Direct配信―シリーズ初スピンオフを7/23発売、新主人公『メカニック』を公開</t>
+        </is>
+      </c>
+      <c r="C230" s="14" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/919/G091973/20260630014/</t>
+        </is>
+      </c>
+      <c r="D230" s="14" t="inlineStr">
+        <is>
+          <t>『スプラトゥーン』はSwitch世代で国内最大級のIPに成長。Switch 2の値上げ後のソフト牽引役が問われる中、シリーズ初のスピンオフ投入で裾野拡大を狙う。</t>
+        </is>
+      </c>
+      <c r="E230" s="14" t="inlineStr">
+        <is>
+          <t>任天堂は6/30 23時に約15分の『スプラトゥーン レイダース Direct』を配信。Switch 2向けのシリーズ初スピンオフで、新主人公『メカニック』が『すりみ連合』とウズシオ諸島でオタカラを求める協力アクションADV。発売は2026/7/23、パッケージ7,480円/DL6,480円(税込)。</t>
+        </is>
+      </c>
+      <c r="F230" s="14" t="inlineStr">
+        <is>
+          <t>シリーズ初のスピンオフ・協力アクションADV
+新主人公『メカニック』＋すりみ連合が主役
+Switch 2専用、2026/7/23発売
+価格はパッケージ7,480円/DL6,480円</t>
+        </is>
+      </c>
+      <c r="G230" s="14" t="inlineStr">
+        <is>
+          <t>Switch 2値上げ後の年末商戦に向けた主力IPの横展開。スピンオフ成否がシリーズのマルチタイトル化・年次運営化の試金石になる。</t>
+        </is>
+      </c>
+      <c r="H230" s="14" t="inlineStr">
+        <is>
+          <t>看板IPのスピンオフ展開とSwitch 2ソフト戦略</t>
+        </is>
+      </c>
+      <c r="I230" s="14" t="inlineStr">
+        <is>
+          <t>任天堂</t>
+        </is>
+      </c>
+      <c r="J230" s="14" t="inlineStr">
+        <is>
+          <t>スプラトゥーン, スプラトゥーン レイダース</t>
+        </is>
+      </c>
+      <c r="K230" s="14" t="inlineStr">
+        <is>
+          <t>新作,国内</t>
+        </is>
+      </c>
+      <c r="L230" s="14" t="inlineStr">
+        <is>
+          <t>出典:4Gamer</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B231" s="14" t="inlineStr">
+        <is>
+          <t>SNK『餓狼伝説 City of the Wolves』にアニメ『北斗の拳』ケンシロウ参戦―6/29配信開始、7月よりSeason3始動</t>
+        </is>
+      </c>
+      <c r="C231" s="14" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/649/G064915/20260629005/</t>
+        </is>
+      </c>
+      <c r="D231" s="14" t="inlineStr">
+        <is>
+          <t>格闘ゲーム市場は競技シーンとコラボ施策で熱量を維持。SNKは復活シリーズ『餓狼伝説CotW』のDLC・シーズン運営でユーザーを繋ぎ留めている。</t>
+        </is>
+      </c>
+      <c r="E231" s="14" t="inlineStr">
+        <is>
+          <t>SNKは6/29、『餓狼伝説 City of the Wolves』のコラボDLCキャラ『ケンシロウ』(アニメ『北斗の拳』)を配信開始。EVO 2026で先行試遊も実施。あわせて新シーズン『Season3』が7月に始動することを告知した。</t>
+        </is>
+      </c>
+      <c r="F231" s="14" t="inlineStr">
+        <is>
+          <t>コラボキャラ『ケンシロウ』を6/29配信
+『北斗神拳』の秘孔=状態変化を再現した設計
+EVO 2026で先行試遊を実施
+7月にSeason3開幕を告知</t>
+        </is>
+      </c>
+      <c r="G231" s="14" t="inlineStr">
+        <is>
+          <t>人気アニメIPのゲストキャラ参戦＋シーズン運営で長期エンゲージメントを設計する格ゲー運営が定着。コラボの話題性が競技シーンと相互送客する。</t>
+        </is>
+      </c>
+      <c r="H231" s="14" t="inlineStr">
+        <is>
+          <t>格ゲーのライブ運営とクロスIPコラボ設計</t>
+        </is>
+      </c>
+      <c r="I231" s="14" t="inlineStr">
+        <is>
+          <t>SNK</t>
+        </is>
+      </c>
+      <c r="J231" s="14" t="inlineStr">
+        <is>
+          <t>餓狼伝説 City of the Wolves, 北斗の拳</t>
+        </is>
+      </c>
+      <c r="K231" s="14" t="inlineStr">
+        <is>
+          <t>新作,国内,eスポーツ</t>
+        </is>
+      </c>
+      <c r="L231" s="14" t="inlineStr">
+        <is>
+          <t>出典:4Gamer(EVO2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B232" s="14" t="inlineStr">
+        <is>
+          <t>『オーバーウォッチ』×YOASOBIコラボが7/1開幕―書き下ろし新曲『オリオン』と6種コラボスキンを実装</t>
+        </is>
+      </c>
+      <c r="C232" s="14" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/484/G048450/20260630036/</t>
+        </is>
+      </c>
+      <c r="D232" s="14" t="inlineStr">
+        <is>
+          <t>ライブサービスのヒーローシューターは新規流入の鈍化が課題。Blizzardは大型音楽IPとのタイアップで話題性とリテンションの両立を図る。</t>
+        </is>
+      </c>
+      <c r="E232" s="14" t="inlineStr">
+        <is>
+          <t>Blizzardは『オーバーウォッチ』とYOASOBIのコラボを7/1開幕。6/30公開のトレーラーでは短編小説から着想した書き下ろし新曲『オリオン』が流れ、キリコ/ゲンジ/ハンゾー/ミズキ/ジュノ/アンランの6コラボスキンと各種報酬を実装する。</t>
+        </is>
+      </c>
+      <c r="F232" s="14" t="inlineStr">
+        <is>
+          <t>コラボ開始は7/1、トレーラーは6/30公開
+YOASOBIが書き下ろし新曲『オリオン』を制作
+6キャラのコラボスキンを実装
+ゲーム内ストーリー連動の楽曲タイアップ</t>
+        </is>
+      </c>
+      <c r="G232" s="14" t="inlineStr">
+        <is>
+          <t>人気アーティストへの書き下ろし発注でゲーム世界を拡張するコラボ・ライブオプスが定着。音楽IPとの相互送客がライブサービスの新規獲得の定石になる。</t>
+        </is>
+      </c>
+      <c r="H232" s="14" t="inlineStr">
+        <is>
+          <t>ライブサービスのアーティスト・タイアップ運営</t>
+        </is>
+      </c>
+      <c r="I232" s="14" t="inlineStr">
+        <is>
+          <t>Blizzard Entertainment, Microsoft</t>
+        </is>
+      </c>
+      <c r="J232" s="14" t="inlineStr">
+        <is>
+          <t>オーバーウォッチ, YOASOBI</t>
+        </is>
+      </c>
+      <c r="K232" s="14" t="inlineStr">
+        <is>
+          <t>国内,海外</t>
+        </is>
+      </c>
+      <c r="L232" s="14" t="inlineStr">
+        <is>
+          <t>出典:4Gamer</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
monthly matrix + future predictions (2026-07-01 00:06)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -816,7 +816,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1491,6 +1491,80 @@
       <c r="G18" s="14" t="inlineStr">
         <is>
           <t>Marvel/Disney発の新規ゲーム契約の形態(短期受託・RevShare・複数社分担)発表の有無、他ライセンスIPゲームの開発体制変更を観測する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>未成年保護を目的とする年齢確認(age assurance)義務化が英・EU・アジアで同時進行し、年齢推定・本人確認がプラットフォーム標準機能として据置/モバイル/UGC全般に組み込まれる。UGC・ソーシャル型(Roblox等)が最初の適用対象となる</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>6〜12ヶ月後</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Roblox, Ofcom(英), 欧州委, Garena/Moonton(インドネシア)</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>英政府が16歳未満のオンライン利用制限を公表(6/23)／Roblox UKで年齢別アカウント導入・顔推定の年齢確認を全面化(Ofcom圧力,6/30)／インドネシアPP TUNASの未成年保護規制がMLBB視聴に波及(6/4)</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>他国(豪・EU加盟国)の年齢確認義務化立法、主要プラットフォーム(Xbox/PSN/Steam/モバイルストア)の年齢推定・本人確認導入、UGC系の未成年アカウント分離の広がりを四半期で追跡。複数地域で同時進行しており方向性は明確。</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>AIデータセンター起因のDRAM/メモリ価格高騰が構造的コスト要因となり、現行機のさらなる値上げに加え次世代機(PS6)の投入時期・価格・粗利設計を規定する。ハード各社はBOM上昇分を値上げ・上位版・サブスクで回収する動きを強める</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>年内〜2027(次世代機発表サイクル)</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Microsoft/Xbox, Sony/PS6, 任天堂</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>MicrosoftがXboxを8/1に最大150ドル値上げ、AI起因のメモリ高騰を要因と明言(6/27)／ソニーがPS6の発売時期・価格を『未定』とし、メモリ価格高騰が次世代機の鍵と説明(6/19)</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>PS6の正式な発売時期・価格発表とメモリ調達コメント、任天堂/MSの追加値上げ、DRAMスポット価格の推移、上位版・サブスク値上げによる回収策の有無を確認。2社が独立にメモリ要因へ言及。</t>
         </is>
       </c>
     </row>
@@ -3084,15 +3158,77 @@
           <t>6月</t>
         </is>
       </c>
-      <c r="C31" s="9" t="inlineStr"/>
-      <c r="D31" s="9" t="inlineStr"/>
-      <c r="E31" s="9" t="inlineStr"/>
-      <c r="F31" s="9" t="inlineStr"/>
-      <c r="G31" s="9" t="inlineStr"/>
-      <c r="H31" s="9" t="inlineStr"/>
-      <c r="I31" s="9" t="inlineStr"/>
-      <c r="J31" s="9" t="inlineStr"/>
-      <c r="K31" s="9" t="inlineStr"/>
+      <c r="C31" s="9" t="inlineStr">
+        <is>
+          <t>・任天堂Switch 2が累計1,700万台超で自社最速ベストセラー、通期目標を1,900万台へ上方修正
+・ソニーがPS5/Pro/Portalを追加値上げ、PS6は時期・価格とも未定
+・MicrosoftがXboxを8/1に最大$150値上げ(Series X $799.99)、25周年で独占回帰
+・Valve『Steam Machine』日本上陸(189,980円)</t>
+        </is>
+      </c>
+      <c r="D31" s="9" t="inlineStr">
+        <is>
+          <t>・Steam Next Fest 6月版が過去最大の約5,000本デモで閉幕
+・Steamサマーセール2026が6/25開幕(〜7/9)
+・PC Gaming Show 2026でControl続編など50本超を公開
+・『Steam Machine』日本発売でPC陣営のリビング市場攻勢</t>
+        </is>
+      </c>
+      <c r="E31" s="9" t="inlineStr">
+        <is>
+          <t>・スマホ新法施行半年もiPhone外部アプリストアにゲーム主要30社の出店ゼロ
+・ポケモン対戦特化『Pokémon Champions』スマホ版を6/17配信
+・『FGO』がUnity 6へエンジン移行(約16GB再DL)
+・ByteDance系Moonton売却交渉(60〜70億ドル)</t>
+        </is>
+      </c>
+      <c r="F31" s="9" t="inlineStr">
+        <is>
+          <t>・NVIDIA『GeForce Now』がQuest 3/Vision Pro/Pico対応、XRでクラウドゲーミング拡大
+・Xbox幹部がGame Pass値上げで「数百万人」解約と認め、$22.99へ価格調整</t>
+        </is>
+      </c>
+      <c r="G31" s="9" t="inlineStr">
+        <is>
+          <t>・CS2『IEM Cologne Major 2026』がピーク約70万人・賞金125万ドル
+・VALORANT Masters London 2026でLeviatánが初優勝
+・LoL『LCK Road to MSI』でT1優勝、ピーク218万人
+・EVO 2026開幕、SF6が4年連続最多2,414名</t>
+        </is>
+      </c>
+      <c r="H31" s="9" t="inlineStr">
+        <is>
+          <t>・EA 550億ドルLBO非公開化が6/30最終局面、EU審査(7/22・7/30期限)
+・Netflix×Warner Bros.($82.7B)を全額現金取引に修正しWB Games統合
+・Nexonが投資子会社『Nexon Partners』設立
+・コーエーテクモがガストを吸収合併</t>
+        </is>
+      </c>
+      <c r="I31" s="9" t="inlineStr">
+        <is>
+          <t>・PEGI新リスク区分で課金ルートボックスは最低16歳指定を6月適用
+・EU AI法が8/2全面適用へ
+・米加州『ゲーム保護法案』AB1921が下院通過
+・任天堂が仏当局にJoy-Conドリフトで約35M€の制裁金
+・英が16歳未満のオンライン制限、Robloxは年齢確認を強化</t>
+        </is>
+      </c>
+      <c r="J31" s="9" t="inlineStr">
+        <is>
+          <t>・NVIDIAが『ACE Game Agent SDK』ベータ公開、KraftonがPUBGにAI僚機を実装
+・Google Cloudが自律型AIエージェント群を本格投入
+・ゲーム生成AI市場は2026年に約22億ドル見通し
+・一方カプコン・ポケットペアは生成AIの本編不使用を表明</t>
+        </is>
+      </c>
+      <c r="K31" s="9" t="inlineStr">
+        <is>
+          <t>・Microsoft/Xboxが7月に大規模レイオフ、Ninja Theory閉鎖、25周年で独占回帰
+・Take-Two『GTA6』予約開始($79.99/11-19)、FY27純予約80億ドル超予想
+・Ubisoftが年6度目の再編で複数スタジオ閉鎖・約380人削減
+・Tencent・NetEaseが海外買収を加速</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="56" customHeight="1">
       <c r="A32" s="12" t="inlineStr"/>

</xml_diff>

<commit_message>
weekly-trends + tech update (2026-07-01 03:09)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -1579,7 +1579,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2513,6 +2513,154 @@
       <c r="G25" t="inlineStr">
         <is>
           <t>https://www.nikkei.com/ (スマホ新法半年), https://www.jetro.go.jp/ (英年齢制限)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Unreal Engine 6の生成AI全面統合とBlueprints将来廃止への反発</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Epicは6/17、Unreal Engine 6を2027年末アーリーアクセスで投入すると発表。LLM・生成AIモデル（ClaudeやCodexを含む）が「コンテンツ制作を高速化する中心的役割」を担うと明言した。同時に、コードを書かずにゲームロジックを組めるノードベースのビジュアルスクリプティング「Blueprints」を初期版では維持しつつ将来的に非推奨（deprecated）とし、独自言語Verseへ移行する方針を示した。Blueprintsはインディーや小規模スタジオの生命線であり、開発者コミュニティは強く反発。Vampire SurvivorsのponcleはFortnite協業を「見直し中」と表明した。EpicのCEOがSteamの生成AI開示タグを「緋文字（scarlet letter）」と批判した経緯とも連動し、業界標準エンジンの設計思想そのものが争点化している。</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Epic Games, Unreal Engine, Fortnite, poncle(Vampire Survivors), Anthropic(Claude), Godot</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>争点は3層構造。(1)ツール層＝Blueprints→Verse＋生成AIへの移行で、ノーコード資産と学習投資が陳腐化するリスク。(2)政治層＝EpicはSteamのAI開示義務を「無責任」と攻撃し、開示なきAI活用を正当化。(3)エコシステム層＝業界標準エンジンの方針が全開発者の制作フローを規定するため、Epic単独の決定が事実上の業界標準となる。中立的代替としてGodotへの関心が再燃。</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>ツールベンダーの設計思想がクリエイターの主権を左右する構造は、生成AI時代の映像・音楽・コード等あらゆる制作産業で反復する。標準の集中は効率と引き換えにロックインを生む。</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>https://www.shacknews.com/article/149693/unreal-engine-6-generative-ai-models-claude-codex , https://www.creativebloq.com/3d/video-game-design/unreal-engines-ai-push-sparks-backlash-as-developers-fear-the-end-of-blueprints</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Steam Machine発売＝Valveの「赤字販売しない」リビングPC戦略</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Valveは6/23にSteam Machineの価格（512GB $1,049〜、2TB $1,349）を発表し、ランダム抽選予約を開始、6/30に出荷を始めた。Steam Deckの約6倍の性能を持つSteamOS搭載の小型リビングPCで、再設計版Steam ControllerとVRヘッドセットSteam Frameも同時展開する。最大の論点は価格思想で、ValveはSony/Microsoftと異なり「本体を赤字で売らない」と明言。従来コンソールの逆ザヤ（ハードで損してソフト/サブスクで回収）モデルを否定し、PCとしての原価積み上げ型価格を採った。$1,049は同性能ゲーミングPCと同等で、コンソールの「安さ」を捨てる代わりにSteamエコシステムの自由度で勝負する構図。MicrosoftがXbox本体を値上げ・2TBモデル販売終了へ動いた局面とも重なり、リビングルームの主導権争いが再点火した。</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Valve, SteamOS, Steam Deck, Steam Frame, Microsoft(Xbox), Sony(PlayStation)</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>コンソール経済は長らく「ハード逆ザヤ×ソフト/ライセンス回収」が前提だった。Valveはストア手数料（Steam 30%）で十分な収益基盤を持つため、ハードを利益商品化できる。半導体・メモリ高騰で逆ザヤの原価負担が増す中、MSはXbox本体を値上げ・2TB撤退へ動いた。Valveの選択は「ハードは薄利のPC、儲けはストア」という構造を鮮明にし、垂直統合コンソール勢との分岐を示す。</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>「入口を赤字にして囲い込む」プラットフォーム経済は原価高騰局面で持続困難になる。回収エンジンを別レイヤー（ストア/サブスク）に持つ者だけがハード価格を自由化できる。</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>https://www.geekwire.com/2026/surprise-valves-new-steam-machine-is-here-but-the-price-is-the-real-shocker/ , https://www.pcgamesn.com/steam-machine/launch</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>MOLE現象——マイクロスタジオ心理ホラーが口コミだけで急伸</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>6/15発売の心理ホラーシム『MOLE』（Off Black Creations開発／Oro Interactive販売）が、大型マーケティングなしにSteamトレンド上位に居座り続け、98%「圧倒的に好評」を獲得した。スラブ圏の戦後神話を土台にした独自世界観で、レビューでは『Iron Lung』『Mouthwashing』の系譜に位置づけられ、一部は「それらが約束した以上」と評す。ソロ〜極小チーム制作でありながら口コミ（word of mouth）だけで拡散した点が特徴。同時期に『Voidling Bound』も94%好評（1,617件）を記録し、6月は見過ごされがちな小規模作の高評価が相次いだ。潤沢な広告費を持たない作品が、明確な情緒的コアと短時間で語れる体験設計によってディスカバリーを突破する構図が続いている。</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Off Black Creations, Oro Interactive, MOLE, Voidling Bound, (系譜)Iron Lung/Mouthwashing</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>心理ホラーは(1)低予算でも情緒的インパクトを最大化しやすい、(2)配信・実況との相性が良く無償の拡散導線を持つ、(3)短尺で「語れる」ため口コミ単価が高い、という三点でマイクロスタジオの構造的勝ち筋になっている。Steamのディスカバリーはウィッシュリストとトレンド滞在で自己強化するため、初速の好評が指数的露出を生む。広告費ではなく「語りたくなる密度」が分配関数を握る。</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>注意経済では、広告投下量よりも「他者に語らせる情緒的フック」がディスカバリーを規定する。低予算×高密度体験の勝ち筋は動画・出版など他コンテンツ産業にも通じる。</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>https://bestof.games/en/articles/mole-steam-horror-hit-june-2026 , https://livecards.net/en/all-blogs/game-releases-you-probably-missed-june-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Switch 2発売1年、19.86M台でPS5超え——サードパーティ本格回帰</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Switch 2は発売1年で累計19.86M台に到達し、同期間のPS5を上回った。象徴的なのはサードパーティの本格回帰で、6月には『Final Fantasy VII Rebirth』が任天堂機に初上陸、Capcomも『Devil May Cry 5』を6/23に投入。旧Switchの非力さゆえに「移植の最後の砦（port of last resort）」扱いだった大型タイトルが、Switch 2のグラフィック性能向上で標準的な出荷先へ転じつつある。Not-E3 2026（6/1〜9）では13本前後のサード作が集中発表され、週約3本のペースで配信された。任天堂エコシステムのサード売上は前年比+76%（2024年13億ドル→2025年23億ドル）と伸長。急速な普及がSwitch 2を「無視できない必須プラットフォーム」へ押し上げ、マルチプラットフォーム前提の開発計画を後押ししている。</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>任天堂, Square Enix(FF7 Rebirth), Capcom(DMC5), Warner Bros., Switch 2</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>サードパーティの投資判断はインストールベースの規模と成長率で決まる。旧Switchは巨大な台数を持ちつつ性能制約で大型作を弾いたため「規模はあるが載らない」状態だった。Switch 2は台数の立ち上がりと性能向上を同時に満たしこの矛盾を解消。結果、最後の移植先から初期ラインアップに組み込む前提の必須機へ格上げされた。普及速度そのものが開発優先順位を書き換える。</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>プラットフォームの価値は「規模×能力」の積で決まり、片方だけでは開発者を動かせない。両輪が揃った瞬間にエコシステムの引力が非線形に強まる。</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>https://tech-insider.org/nintendo-switch-2-sales-19-million-2026/ , https://famiboards.com/threads/all-of-the-third-party-switch-2-games-dates-announced-during-not-e3-2026-june-1st-june-9th.17747/</t>
         </is>
       </c>
     </row>
@@ -28800,7 +28948,7 @@
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B2" s="9" t="inlineStr">
@@ -28815,32 +28963,32 @@
       </c>
       <c r="D2" s="9" t="inlineStr">
         <is>
-          <t>開発現場の利用率は前年36%→29%へ低下、52%が『悪影響』と回答。基盤層（NVIDIA・Google Cloud）は推進継続で温度差が拡大。</t>
+          <t>開発現場の生成AI利用率は前年比で低下傾向が続く一方、ツール層では標準エンジンへの生成AI組み込みが加速。制作フロー上流（エンジン・パイプライン）と現場適用の温度差が拡大。</t>
         </is>
       </c>
       <c r="E2" s="9" t="inlineStr">
         <is>
-          <t>パルワールドが生成AI不使用を再表明／GameByteがAIノーコード基盤で資金調達／NVIDIAがオンデバイスNPC『ACE』発表／DLSS 5が生成AIで映像補完。</t>
+          <t>Epicが6/17にUnreal Engine 6を発表、LLM・生成AI（Claude/Codex含む）を制作の中核に据え、Blueprintsを将来非推奨としVerseへ移行。開発者は反発、poncleがFortnite協業見直しを表明。EpicはSteamのAI開示タグを「緋文字」と批判。</t>
         </is>
       </c>
       <c r="F2" s="9" t="inlineStr">
         <is>
-          <t>ポケットペア, NVIDIA, Google Cloud, GameByte, Larian</t>
+          <t>Epic Games, Anthropic(Claude), poncle, Valve, Godot</t>
         </is>
       </c>
       <c r="G2" s="9" t="inlineStr">
         <is>
-          <t>『非AI』を真正性として打ち出す差別化が定着。基盤技術は推進されるが、エンドコンテンツへの直接適用は炎上回避で慎重姿勢が続く。</t>
+          <t>標準エンジンのAI組み込みは不可逆。ノーコード資産の陳腐化を嫌う層がGodot等中立ツールへ分散する二極化が進む。開示義務化の是非がプラットフォーム間対立の焦点に。</t>
         </is>
       </c>
       <c r="H2" s="9" t="inlineStr">
         <is>
-          <t>効率化技術が需要側選好で抑制される逆説。AIの主戦場は『見えない裏方（最適化・QA・運用）』へ移る。</t>
+          <t>AIの主戦場が「現場の生成」から「制作基盤の設計思想」へ移動。誰がツール標準を握るかがクリエイター主権を左右する。</t>
         </is>
       </c>
       <c r="I2" s="9" t="inlineStr">
         <is>
-          <t>https://www.gianty.com/ GDC2026 / https://www.gamesradar.com/ パルワールド</t>
+          <t>https://www.shacknews.com/article/149693/unreal-engine-6-generative-ai-models-claude-codex</t>
         </is>
       </c>
       <c r="J2" s="9" t="inlineStr"/>
@@ -29172,7 +29320,7 @@
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
@@ -29187,32 +29335,32 @@
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>Steam Next Fest 6月版が過去最大規模。サマーセールが6/25開幕。無料・少人数インディーが上位を席巻。</t>
+          <t>Steamはサマーセール開催中（6/25〜7/9）。Valveがハード領域へ本格進出し、PCゲーミングをリビングルームへ拡張する局面。</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>ValveがSteam Machineを日本・台湾・香港で発売（自社ハードでリビングへ進出）／Gothic 1 RemakeがVery Positiveでヒット／TBH等の無料ゲームが同接トップ。</t>
+          <t>Valveが6/23にSteam Machine（512GB $1,049〜）を発表し6/30出荷開始。Steam Deck比約6倍性能のSteamOS小型PC。再設計Steam Controller、VRのSteam Frameも同時展開。「本体を赤字で売らない」と明言し従来コンソールの逆ザヤモデルを否定。</t>
         </is>
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t>Valve, THQ Nordic, インディー各社</t>
+          <t>Valve, SteamOS, Steam Frame, Microsoft, Sony</t>
         </is>
       </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
-          <t>Valveがストア＋ハードの垂直統合を強化。PCの『コンソール化』とインディー発見性向上が並走する。</t>
+          <t>「薄利ハード×ストア回収」モデルが原価高騰下で優位に。垂直統合コンソール勢との価格思想の分岐が鮮明化。リビングルームPCがコンソールとPCの境界を溶かす。</t>
         </is>
       </c>
       <c r="H11" s="9" t="inlineStr">
         <is>
-          <t>流通プラットフォーマーが自社ハードでエコシステムを囲い込む、Apple型の垂直統合がPCにも到来。</t>
+          <t>回収レイヤー（ストア30%）を別に持つ者だけがハード価格を自由化できる。プラットフォーム経済の逆ザヤ前提が崩れつつある。</t>
         </is>
       </c>
       <c r="I11" s="9" t="inlineStr">
         <is>
-          <t>https://www.4gamer.net/ Steam Machine / https://www.techtimes.com/ Next Fest</t>
+          <t>https://www.geekwire.com/2026/surprise-valves-new-steam-machine-is-here-but-the-price-is-the-real-shocker/</t>
         </is>
       </c>
       <c r="J11" s="9" t="inlineStr"/>
@@ -29220,7 +29368,7 @@
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B12" s="9" t="inlineStr">
@@ -29235,32 +29383,32 @@
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>累計約2,000万台でPS5を約100万台上回る。サードパーティ売上+76%、tie-ratioは4.0超へ。</t>
+          <t>発売1年で累計19.86M台、同期間のPS5を上回る立ち上がり。サードパーティが本格回帰する局面。</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>Star FoxがSwitch 2専用で6/25発売／FF7リバース・FF10 HD・KH4・ゼノブレイド等の移植・新作が集中／ニンダイ6.9は非独占マルチ中心で株価一時7%安。一方ソニーはPS6時期『未定』。</t>
+          <t>6月に『FF7 Rebirth』が任天堂機初上陸、Capcom『DMC5』も6/23投入。Not-E3 2026で13本前後のサード作が集中発表（週約3本ペース）。任天堂エコシステムのサード売上は前年比+76%（13億→23億ドル）。</t>
         </is>
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>任天堂, スクウェア・エニックス, カプコン, ソニー</t>
+          <t>任天堂, Square Enix, Capcom, Warner Bros.</t>
         </is>
       </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
-          <t>サードパーティ day-one供給が常態化しAAAライブラリが拡充。据置世代交代は任天堂先行・ソニー様子見の非対称が続く。</t>
+          <t>「移植の最後の砦」から初期ラインアップ前提の必須機へ。年末商戦の端末普及ペースとファースト大型作の供給、値上げの需要影響が次の焦点。</t>
         </is>
       </c>
       <c r="H12" s="9" t="inlineStr">
         <is>
-          <t>『独占』より『全機種同発』が標準化。ハード優位はソフト供給の引力で自己強化される。</t>
+          <t>普及速度そのものが開発優先順位を書き換える。「規模×性能」が揃った瞬間にエコシステムの引力が非線形化。</t>
         </is>
       </c>
       <c r="I12" s="9" t="inlineStr">
         <is>
-          <t>https://www.nintendolife.com/ 2000万台 / https://www.videogameschronicle.com/</t>
+          <t>https://tech-insider.org/nintendo-switch-2-sales-19-million-2026/</t>
         </is>
       </c>
       <c r="J12" s="9" t="inlineStr"/>

</xml_diff>

<commit_message>
add title/hit news (MECCHA CHAMELEON 10M, Suikoden STAR LEAP) 2026-07-01
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -9568,7 +9568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L232"/>
+  <dimension ref="A1:L234"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -23964,6 +23964,136 @@
       <c r="L232" s="14" t="inlineStr">
         <is>
           <t>出典:4Gamer</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B233" s="14" t="inlineStr">
+        <is>
+          <t>インディー『めっちゃカメレオン』発売16日で1000万本突破―個人開発の“ぬり絵かくれんぼ”が国内外で大ヒット</t>
+        </is>
+      </c>
+      <c r="C233" s="14" t="inlineStr">
+        <is>
+          <t>https://news.denfaminicogamer.jp/interview/260630w</t>
+        </is>
+      </c>
+      <c r="D233" s="14" t="inlineStr">
+        <is>
+          <t>日本の個人開発者LEMORION(lemorion_1224)が2026/6/10にSteamで配信した低価格マルチプレイ作品。“オニ”と“隠れる側”に分かれ、白い体に塗って背景に擬態する『ぬり絵かくれんぼ』の独自性と実況・口コミで人気が急拡大した。</t>
+        </is>
+      </c>
+      <c r="E233" s="14" t="inlineStr">
+        <is>
+          <t>『めっちゃカメレオン』が発売16日(6/26)で販売本数1000万本を突破。100万本(発売1週間以内)→500万本(6/20)→700万本(6/22)→1000万本(6/26)と加速し、推定売上は約44〜55億円。6/30には達成記念の開発者インタビューも公開された。</t>
+        </is>
+      </c>
+      <c r="F233" s="14" t="inlineStr">
+        <is>
+          <t>個人開発の“ぬり絵かくれんぼ”マルチ
+発売16日で1000万本を突破
+2週連続でSteam買い切りゲー売上トップ
+6/25アプデで新キャラ『キューブ』追加</t>
+        </is>
+      </c>
+      <c r="G233" s="14" t="inlineStr">
+        <is>
+          <t>低価格×口コミ駆動のインディーが短期で桁違いの規模に到達しうる事例。少人数開発でもバイラル設計次第で大手級ヒットが生まれる潮流が強まる。</t>
+        </is>
+      </c>
+      <c r="H233" s="14" t="inlineStr">
+        <is>
+          <t>バイラル型インディーのグロースとマルチ設計</t>
+        </is>
+      </c>
+      <c r="I233" s="14" t="inlineStr">
+        <is>
+          <t>LEMORION(lemorion_1224)</t>
+        </is>
+      </c>
+      <c r="J233" s="14" t="inlineStr">
+        <is>
+          <t>めっちゃカメレオン(MECCHA CHAMELEON)</t>
+        </is>
+      </c>
+      <c r="K233" s="14" t="inlineStr">
+        <is>
+          <t>新作,インディー,国内</t>
+        </is>
+      </c>
+      <c r="L233" s="14" t="inlineStr">
+        <is>
+          <t>出典:電ファミニコゲーマー/Game*Spark</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B234" s="14" t="inlineStr">
+        <is>
+          <t>コナミ、シリーズ新作『幻想水滸伝 STAR LEAP』最新情報を7/1公式番組で公開へ―スマホ/PC向けRPG</t>
+        </is>
+      </c>
+      <c r="C234" s="14" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/article/202606/79566</t>
+        </is>
+      </c>
+      <c r="D234" s="14" t="inlineStr">
+        <is>
+          <t>名作JRPG『幻想水滸伝』の休眠IPを活かした新作。まず国内向けにiOS/Android版から配信し、海外展開・PC版は後日対応する方針が示されていた。</t>
+        </is>
+      </c>
+      <c r="E234" s="14" t="inlineStr">
+        <is>
+          <t>コナミは公式番組『幻想水滸伝Live vol.6』を7/1 20時に配信し、シリーズ新作『幻想水滸伝 STAR LEAP(スターリープ)』の最新情報を公開する。武術家三姉妹“乱凛天”役の佐々木未来・愛美・伊藤彩紗がゲスト出演。国内スマホ版先行で展開予定。</t>
+        </is>
+      </c>
+      <c r="F234" s="14" t="inlineStr">
+        <is>
+          <t>シリーズ新作RPG『STAR LEAP』の最新情報
+7/1 20時に公式番組で公開
+国内iOS/Android先行、PC・海外は後日
+声優ゲストが出演</t>
+        </is>
+      </c>
+      <c r="G234" s="14" t="inlineStr">
+        <is>
+          <t>休眠JRPG IPのスマホ起点での再始動。旧作ファンの掘り起こしとモバイル課金モデルの相性、初動のサービス品質が成否の鍵になる。</t>
+        </is>
+      </c>
+      <c r="H234" s="14" t="inlineStr">
+        <is>
+          <t>休眠IPのモバイル再launchとサービス設計</t>
+        </is>
+      </c>
+      <c r="I234" s="14" t="inlineStr">
+        <is>
+          <t>コナミデジタルエンタテインメント</t>
+        </is>
+      </c>
+      <c r="J234" s="14" t="inlineStr">
+        <is>
+          <t>幻想水滸伝, 幻想水滸伝 STAR LEAP</t>
+        </is>
+      </c>
+      <c r="K234" s="14" t="inlineStr">
+        <is>
+          <t>新作,国内</t>
+        </is>
+      </c>
+      <c r="L234" s="14" t="inlineStr">
+        <is>
+          <t>出典:ファミ通/4Gamer(7/1 20時配信)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
daily-news(7) + cross-question(1) + event(1) update 2026-07-02
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -3491,7 +3491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:G55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5498,6 +5498,43 @@
       <c r="G54" s="14" t="inlineStr">
         <is>
           <t>ゲームが『発注主』として音楽制作を駆動する構図。IP相互送客の経済圏が広告タイアップより深い世界観統合に向かう可能性。</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B55" s="14" t="inlineStr">
+        <is>
+          <t>ゲームメディア(IGN)が業界見本市の公式番組・プレビュー制作まで担う『メディアのイベント運営化』は、映画祭・音楽フェス・展示会など他のイベント産業でも、編集メディアが主催機能を取り込む形で起きるか？その時、広告とコンテンツの境界(編集/スポンサー枠)はどう再設計されるか。</t>
+        </is>
+      </c>
+      <c r="C55" s="14" t="inlineStr">
+        <is>
+          <t>gamescomがIGNと提携拡大、公式インディー番組の制作を初委託(GamesBeat/GamesIndustry.biz, 7/1)</t>
+        </is>
+      </c>
+      <c r="D55" s="14" t="inlineStr">
+        <is>
+          <t>IGN,Koelnmesse,gamescom</t>
+        </is>
+      </c>
+      <c r="E55" s="14" t="inlineStr">
+        <is>
+          <t>メディア/広告,イベント/興行,映画祭・音楽フェス</t>
+        </is>
+      </c>
+      <c r="F55" s="14" t="inlineStr">
+        <is>
+          <t>新規</t>
+        </is>
+      </c>
+      <c r="G55" s="14" t="inlineStr">
+        <is>
+          <t>露出枠の『編集×スポンサー』統合は、パブリッシャーのマーケ予算を純広告からイベント連動へ移す。他業界でも専門メディアが主催化する兆候を観測したい。</t>
         </is>
       </c>
     </row>
@@ -7766,7 +7803,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:J24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8926,6 +8963,58 @@
       <c r="J23" s="14" t="inlineStr">
         <is>
           <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B24" s="14" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="C24" s="14" t="inlineStr">
+        <is>
+          <t>MLBB Mid Season Cup 2026 (MSC)</t>
+        </is>
+      </c>
+      <c r="D24" s="14" t="inlineStr">
+        <is>
+          <t>eスポーツ</t>
+        </is>
+      </c>
+      <c r="E24" s="14" t="inlineStr">
+        <is>
+          <t>EWC 2026連動（会場詳細は要確認）</t>
+        </is>
+      </c>
+      <c r="F24" s="14" t="inlineStr">
+        <is>
+          <t>オフライン大会</t>
+        </is>
+      </c>
+      <c r="G24" s="14" t="inlineStr">
+        <is>
+          <t>MoontonのMLBB年央国際大会。賞金総額300万ドル。EWC 2026の枠組みと連動。ダブルイリミGS＋シングルイリミKOで8/1決勝。ワイルドカード7/1-4。</t>
+        </is>
+      </c>
+      <c r="H24" s="14" t="inlineStr">
+        <is>
+          <t>https://liquipedia.net/mobilelegends/MSC/2026</t>
+        </is>
+      </c>
+      <c r="I24" s="14" t="inlineStr">
+        <is>
+          <t>開催中</t>
+        </is>
+      </c>
+      <c r="J24" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
         </is>
       </c>
     </row>
@@ -9568,7 +9657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L234"/>
+  <dimension ref="A1:L241"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -24096,6 +24185,441 @@
           <t>出典:ファミ通/4Gamer(7/1 20時配信)</t>
         </is>
       </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B235" s="14" t="inlineStr">
+        <is>
+          <t>任天堂・古川社長、株主総会で生成AIへの見解を表明―「ゲーム開発とAIはもともと近い」一方で権利侵害リスクに慎重姿勢</t>
+        </is>
+      </c>
+      <c r="C235" s="14" t="inlineStr">
+        <is>
+          <t>https://www.itmedia.co.jp/aiplus/article/2607/01/2000000150/</t>
+        </is>
+      </c>
+      <c r="D235" s="14" t="inlineStr">
+        <is>
+          <t>セガ・コロプラ・カプコン・スクエニなど大手が生成AIの活用度合いを相次いで開示する中、任天堂の姿勢が注目されていた。第86期定時株主総会の質疑応答概要が7/1に公開された。</t>
+        </is>
+      </c>
+      <c r="E235" s="14" t="inlineStr">
+        <is>
+          <t>古川俊太郎社長は敵キャラの挙動制御など従来からAI的技術を活用してきたとしつつ、生成AIについては知的財産権の侵害リスクに留意し慎重に扱う考えを示した。効率化での活用と権利保護を両立させる構え。</t>
+        </is>
+      </c>
+      <c r="F235" s="14" t="inlineStr">
+        <is>
+          <t>大手各社がAI活用度を開示する潮流
+任天堂はIP侵害リスクを理由に慎重姿勢
+従来型AI（敵AI等）と生成AIを区別
+開示の有無がブランド価値の分岐点に</t>
+        </is>
+      </c>
+      <c r="G235" s="14" t="inlineStr">
+        <is>
+          <t>任天堂は生成AIの本編実装には慎重な一方、開発効率化では技術活用を否定せず。今後はIP保護を軸に「どこまで使い、どこを人手に残すか」の線引きが各社のブランド戦略として明確化する見込み。</t>
+        </is>
+      </c>
+      <c r="H235" s="14" t="inlineStr">
+        <is>
+          <t>生成AIの知財リスクとゲーム各社の開示・活用方針の違い</t>
+        </is>
+      </c>
+      <c r="I235" s="14" t="inlineStr">
+        <is>
+          <t>任天堂</t>
+        </is>
+      </c>
+      <c r="J235" s="14" t="inlineStr">
+        <is>
+          <t>―</t>
+        </is>
+      </c>
+      <c r="K235" s="14" t="inlineStr">
+        <is>
+          <t>技術,国内</t>
+        </is>
+      </c>
+      <c r="L235" s="14" t="inlineStr"/>
+    </row>
+    <row r="236">
+      <c r="A236" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B236" s="14" t="inlineStr">
+        <is>
+          <t>ポケットペア『パルワールド』、正式版1.0を7/10配信決定―約2年半の早期アクセスを終了、PC/PS5/Xbox/Game Passで同時展開</t>
+        </is>
+      </c>
+      <c r="C236" s="14" t="inlineStr">
+        <is>
+          <t>https://saiganak.com/news/palworld-ver1-announcement/</t>
+        </is>
+      </c>
+      <c r="D236" s="14" t="inlineStr">
+        <is>
+          <t>2024年1月の早期アクセス開始以来、初動で世界的ヒットとなった『パルワールド』。Summer Game Fest 2026で最新シネマティックとともに1.0の情報が公開された。</t>
+        </is>
+      </c>
+      <c r="E236" s="14" t="inlineStr">
+        <is>
+          <t>ポケットペアは『パルワールド』の正式版1.0を7/10に配信すると発表。ワールドツリー地域と新島の追加でマップ面積が約2倍に拡大し、繁殖システムやサーバークラスタリングを実装。Game Pass初日対応で幅広い層に届ける。</t>
+        </is>
+      </c>
+      <c r="F236" s="14" t="inlineStr">
+        <is>
+          <t>早期アクセスを約2.5年で終了し1.0へ
+マップ面積が初期比で約2倍に拡大
+PC/PS5/Xbox/Game Pass同時展開
+パッチノートは27ページに及ぶ大型更新</t>
+        </is>
+      </c>
+      <c r="G236" s="14" t="inlineStr">
+        <is>
+          <t>1.0を機に売上・同接の再ピークが見込まれ、Game Pass初日対応が新規流入を後押し。ポケットペアの次IP・訴訟（任天堂）動向とあわせ、インディー発大型IPの持続性を占う節目になる。</t>
+        </is>
+      </c>
+      <c r="H236" s="14" t="inlineStr">
+        <is>
+          <t>早期アクセス卒業タイミングの設計とサブスク初日対応の効果</t>
+        </is>
+      </c>
+      <c r="I236" s="14" t="inlineStr">
+        <is>
+          <t>ポケットペア</t>
+        </is>
+      </c>
+      <c r="J236" s="14" t="inlineStr">
+        <is>
+          <t>パルワールド</t>
+        </is>
+      </c>
+      <c r="K236" s="14" t="inlineStr">
+        <is>
+          <t>新作,海外,インディー</t>
+        </is>
+      </c>
+      <c r="L236" s="14" t="inlineStr">
+        <is>
+          <t>生成AI不使用方針は既報(6/19)</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B237" s="14" t="inlineStr">
+        <is>
+          <t>ベセスダ、『The Elder Scrolls IV: Oblivion Remastered』Switch 2版を8/12発売決定―全DLC収録・カートリッジに本編フル収録</t>
+        </is>
+      </c>
+      <c r="C237" s="14" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/981/G098137/20260701018/</t>
+        </is>
+      </c>
+      <c r="D237" s="14" t="inlineStr">
+        <is>
+          <t>2025年に発表・配信された『Oblivion Remastered』のSwitch 2版が7/1に発売日確定。Switch 2のサードパーティ大型移植の一例として注目される。</t>
+        </is>
+      </c>
+      <c r="E237" s="14" t="inlineStr">
+        <is>
+          <t>Switch 2版『Oblivion Remastered』は8/12発売、通常版6050円／デラックス版7260円。『Shivering Isles』『Knights of the Nine』等を含む全追加コンテンツを収録し、ゲームキーカードでなくカートリッジに本編を収める。</t>
+        </is>
+      </c>
+      <c r="F237" s="14" t="inlineStr">
+        <is>
+          <t>Switch 2版が8/12発売、価格6050円〜
+過去の全DLCを収録
+カートリッジに本編フル収録（キーカード非採用）
+Switch 2向け大型サード移植の実例</t>
+        </is>
+      </c>
+      <c r="G237" s="14" t="inlineStr">
+        <is>
+          <t>Switch 2の据置マルチ受け皿としての価値を示す事例。カートリッジ本編収録は物理派の支持を集めやすく、サード各社の移植戦略（キーカードvs本編収録）の判断材料になる。</t>
+        </is>
+      </c>
+      <c r="H237" s="14" t="inlineStr">
+        <is>
+          <t>Switch 2のサード移植戦略とゲームキーカード論争</t>
+        </is>
+      </c>
+      <c r="I237" s="14" t="inlineStr">
+        <is>
+          <t>ベセスダ・ソフトワークス,Microsoft</t>
+        </is>
+      </c>
+      <c r="J237" s="14" t="inlineStr">
+        <is>
+          <t>The Elder Scrolls IV: Oblivion</t>
+        </is>
+      </c>
+      <c r="K237" s="14" t="inlineStr">
+        <is>
+          <t>新作,海外,国内</t>
+        </is>
+      </c>
+      <c r="L237" s="14" t="inlineStr">
+        <is>
+          <t>Switch 2向け</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B238" s="14" t="inlineStr">
+        <is>
+          <t>gamescom、IGNとの提携を拡大―公式番組『gamescom awesome indies show』の制作を初めてIGNが担当、プレビュー企画を新導入</t>
+        </is>
+      </c>
+      <c r="C238" s="14" t="inlineStr">
+        <is>
+          <t>https://gamesbeat.com/ign-and-gamescom-team-up-on-indies-show/</t>
+        </is>
+      </c>
+      <c r="D238" s="14" t="inlineStr">
+        <is>
+          <t>IGNは従来からgamescom公式コンシューマー配信の制作パートナーを務めてきた。主催のKoelnmesseとgame（独ゲーム産業協会）が7/1に提携拡大を発表。</t>
+        </is>
+      </c>
+      <c r="E238" s="14" t="inlineStr">
+        <is>
+          <t>IGNが『gamescom awesome indies show』（8/27配信・60〜75分）の制作を初担当。トレーラーや開発者インタビューに加え、IGN定番のプレビュー企画を新導入する。編集/スポンサー枠の応募も受付、掲載要件は会場出展。</t>
+        </is>
+      </c>
+      <c r="F238" s="14" t="inlineStr">
+        <is>
+          <t>IGNがインディー公式番組の制作を初担当
+8/27に世界配信、プレビュー企画を新導入
+編集・スポンサー枠を出展社に開放
+応募締切8/2、素材提出7/19</t>
+        </is>
+      </c>
+      <c r="G238" s="14" t="inlineStr">
+        <is>
+          <t>メディア企業が業界見本市の公式番組・編集企画を統合的に握る動きが進む。インディーの露出設計が『広告』から『編集×イベント』へ寄り、パブリッシャーのマーケ予算配分に影響しうる。</t>
+        </is>
+      </c>
+      <c r="H238" s="14" t="inlineStr">
+        <is>
+          <t>ゲームメディアのイベント運営化と露出設計</t>
+        </is>
+      </c>
+      <c r="I238" s="14" t="inlineStr">
+        <is>
+          <t>IGN,Koelnmesse,game（独ゲーム産業協会）</t>
+        </is>
+      </c>
+      <c r="J238" s="14" t="inlineStr">
+        <is>
+          <t>gamescom</t>
+        </is>
+      </c>
+      <c r="K238" s="14" t="inlineStr">
+        <is>
+          <t>提携,海外,インディー</t>
+        </is>
+      </c>
+      <c r="L238" s="14" t="inlineStr"/>
+    </row>
+    <row r="239">
+      <c r="A239" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B239" s="14" t="inlineStr">
+        <is>
+          <t>『モバイルレジェンド』MLBB Mid Season Cup 2026が開幕―賞金総額300万ドル、EWC 2026連動でワイルドカード〜決勝を8/1まで実施</t>
+        </is>
+      </c>
+      <c r="C239" s="14" t="inlineStr">
+        <is>
+          <t>https://liquipedia.net/mobilelegends/MSC/2026</t>
+        </is>
+      </c>
+      <c r="D239" s="14" t="inlineStr">
+        <is>
+          <t>MSCはMoontonのMLBBにおける年央の国際大会。2026年はEsports World Cup 2026の枠組みと連動して実施される。ワイルドカードが7/1〜4に開幕。</t>
+        </is>
+      </c>
+      <c r="E239" s="14" t="inlineStr">
+        <is>
+          <t>MLBB MSC 2026が7/1開幕、賞金総額300万ドル。ダブルイリミのグループステージとシングルイリミのノックアウトを経て8/1に決勝。EWC 2026と連動し、モバイルeスポーツの旗艦大会として展開する。</t>
+        </is>
+      </c>
+      <c r="F239" s="14" t="inlineStr">
+        <is>
+          <t>賞金総額300万ドルで7/1開幕
+EWC 2026の枠組みと連動
+ワイルドカード7/1〜4、決勝8/1
+モバイルeスポーツ最大級の国際大会</t>
+        </is>
+      </c>
+      <c r="G239" s="14" t="inlineStr">
+        <is>
+          <t>モバイル発の大型大会がEWCの傘下で束ねられる構図が定着。東南アジア中心のMLBB経済圏がサウジ資本のeスポーツ統合戦略に組み込まれ、地域リーグの国際露出が加速する。</t>
+        </is>
+      </c>
+      <c r="H239" s="14" t="inlineStr">
+        <is>
+          <t>モバイルeスポーツとEWC統合による大会経済圏の再編</t>
+        </is>
+      </c>
+      <c r="I239" s="14" t="inlineStr">
+        <is>
+          <t>Moonton,Esports World Cup Foundation</t>
+        </is>
+      </c>
+      <c r="J239" s="14" t="inlineStr">
+        <is>
+          <t>Mobile Legends: Bang Bang</t>
+        </is>
+      </c>
+      <c r="K239" s="14" t="inlineStr">
+        <is>
+          <t>eスポーツ,海外</t>
+        </is>
+      </c>
+      <c r="L239" s="14" t="inlineStr"/>
+    </row>
+    <row r="240">
+      <c r="A240" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B240" s="14" t="inlineStr">
+        <is>
+          <t>NCSOFT、新作オープンワールドTPS『シンダーシティ(CINDER CITY)』のSteamページを公開―崩壊した近未来ソウル舞台の大規模マルチPvE</t>
+        </is>
+      </c>
+      <c r="C240" s="14" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/668/G066861/20260701015/</t>
+        </is>
+      </c>
+      <c r="D240" s="14" t="inlineStr">
+        <is>
+          <t>NCの開発スタジオBigFire Gamesが手掛ける新作。2025年に正式発表され、G-STAR 2025で試遊も公開。7/1にSteamページとゲームプレイをまとめたPVを公開した。</t>
+        </is>
+      </c>
+      <c r="E240" s="14" t="inlineStr">
+        <is>
+          <t>『シンダーシティ』はUE5製のシネマティックTPSで、荒廃した未来都市ソウルを舞台に大規模マルチプレイPvEを中核に据える。7/1にSteamストアページを開設しウィッシュリスト受付を開始、実プレイ映像も公開した。</t>
+        </is>
+      </c>
+      <c r="F240" s="14" t="inlineStr">
+        <is>
+          <t>NC子会社BigFire Gamesの新作TPS
+Steamページ公開・ウィッシュリスト開始
+崩壊した近未来ソウル舞台の大規模PvE
+ソロキャンペーンも用意される見込み</t>
+        </is>
+      </c>
+      <c r="G240" s="14" t="inlineStr">
+        <is>
+          <t>MMO依存からの脱却を図るNCが、買い切り／PvE志向のPCシューターで西欧・グローバル市場を狙う布石。抽出型・PvPの過熱が一巡する中、協力PvE路線の成否が韓国大手の多角化を占う。</t>
+        </is>
+      </c>
+      <c r="H240" s="14" t="inlineStr">
+        <is>
+          <t>韓国大手のMMO脱却とPC/コンソール向けPvEシューター戦略</t>
+        </is>
+      </c>
+      <c r="I240" s="14" t="inlineStr">
+        <is>
+          <t>NCSOFT,BigFire Games</t>
+        </is>
+      </c>
+      <c r="J240" s="14" t="inlineStr">
+        <is>
+          <t>シンダーシティ(CINDER CITY)</t>
+        </is>
+      </c>
+      <c r="K240" s="14" t="inlineStr">
+        <is>
+          <t>新作,海外</t>
+        </is>
+      </c>
+      <c r="L240" s="14" t="inlineStr"/>
+    </row>
+    <row r="241">
+      <c r="A241" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B241" s="14" t="inlineStr">
+        <is>
+          <t>CESA、『東京ゲームショウ2026』オフィシャルサポーターに宮田俊哉さん(Kis-My-Ft2)を起用―特別インタビュー動画も公開</t>
+        </is>
+      </c>
+      <c r="C241" s="14" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/991/G999110/20260630037/</t>
+        </is>
+      </c>
+      <c r="D241" s="14" t="inlineStr">
+        <is>
+          <t>TGS2026は30周年・史上初の5日間開催（9/17〜21、幕張メッセ）。開催に向けたプロモーションの一環として、7/1にオフィシャルサポーターが発表された。</t>
+        </is>
+      </c>
+      <c r="E241" s="14" t="inlineStr">
+        <is>
+          <t>コンピュータエンターテインメント協会は、TGS2026のオフィシャルサポーターに宮田俊哉さん(Kis-My-Ft2)を起用すると発表。ゲーム実況チャンネルも持つ同氏を起用し、就任記念の特別インタビュー動画を7/1から配信開始した。</t>
+        </is>
+      </c>
+      <c r="F241" s="14" t="inlineStr">
+        <is>
+          <t>TGS2026サポーターに宮田俊哉さん就任
+30周年・史上初の5日間開催をPR
+ゲーム実況の実績あるタレントを起用
+就任記念インタビュー動画を配信</t>
+        </is>
+      </c>
+      <c r="G241" s="14" t="inlineStr">
+        <is>
+          <t>タレント起用でコアゲーマー以外への訴求を強化する狙い。5日間拡大・30周年という節目に向け、来場30万人目標達成へ話題づくりが本格化する。</t>
+        </is>
+      </c>
+      <c r="H241" s="14" t="inlineStr">
+        <is>
+          <t>国内最大級見本市のプロモーション設計と来場者拡大策</t>
+        </is>
+      </c>
+      <c r="I241" s="14" t="inlineStr">
+        <is>
+          <t>CESA</t>
+        </is>
+      </c>
+      <c r="J241" s="14" t="inlineStr">
+        <is>
+          <t>東京ゲームショウ2026</t>
+        </is>
+      </c>
+      <c r="K241" s="14" t="inlineStr">
+        <is>
+          <t>国内</t>
+        </is>
+      </c>
+      <c r="L241" s="14" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
daily-news + cross-questions + events + predictions + game-design update (2026-07-03)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -816,7 +816,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1565,6 +1565,43 @@
       <c r="G20" t="inlineStr">
         <is>
           <t>PS6の正式な発売時期・価格発表とメモリ調達コメント、任天堂/MSの追加値上げ、DRAMスポット価格の推移、上位版・サブスク値上げによる回収策の有無を確認。2社が独立にメモリ要因へ言及。</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B21" s="15" t="inlineStr">
+        <is>
+          <t>テンセントが日本の少数出資を実際に売却し始めると、対象の中堅上場ゲーム会社（マーベラス等）で株主構成が流動化し、国内事業会社・PEファンドによる資本参加/TOB、あるいはサウジ系ファンド・国内商社が「中国マネーの受け皿」として登場する再編第2波が起きる</t>
+        </is>
+      </c>
+      <c r="C21" s="15" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="D21" s="15" t="inlineStr">
+        <is>
+          <t>年内〜2027年上期</t>
+        </is>
+      </c>
+      <c r="E21" s="15" t="inlineStr">
+        <is>
+          <t>テンセント,マーベラス,サウジPIF系,国内PE</t>
+        </is>
+      </c>
+      <c r="F21" s="15" t="inlineStr">
+        <is>
+          <t>「テンセント、マーベラスなど日本のゲーム会社株の売却を協議」（Bloomberg, 7/3日次ニュース）</t>
+        </is>
+      </c>
+      <c r="G21" s="15" t="inlineStr">
+        <is>
+          <t>マーベラス等対象銘柄の大量保有報告書・変更報告書、TOB公告、テンセントの持分変動開示を観測。売却先が経営陣(MBO型)か第三者かで再編の広がりが判別できる。</t>
         </is>
       </c>
     </row>
@@ -3491,7 +3528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G55"/>
+  <dimension ref="A1:G57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5535,6 +5572,80 @@
       <c r="G55" s="14" t="inlineStr">
         <is>
           <t>露出枠の『編集×スポンサー』統合は、パブリッシャーのマーケ予算を純広告からイベント連動へ移す。他業界でも専門メディアが主催化する兆候を観測したい。</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B56" s="15" t="inlineStr">
+        <is>
+          <t>開発拠点の大量解雇に対しストライキで「数年間の解雇禁止」を要求する動き（Ubisoftバルセロナ）は、日本のアニメ・映像・IT受託など他のクリエイティブ産業の労働慣行にも波及するか？</t>
+        </is>
+      </c>
+      <c r="C56" s="15" t="inlineStr">
+        <is>
+          <t>Ubisoftバルセロナがストライキ—レイオフに抗議し6/30から7/16まで断続的に実施（GameDeveloper, 7/3記録）</t>
+        </is>
+      </c>
+      <c r="D56" s="15" t="inlineStr">
+        <is>
+          <t>Ubisoft</t>
+        </is>
+      </c>
+      <c r="E56" s="15" t="inlineStr">
+        <is>
+          <t>労働市場・アニメ制作・IT受託・労働法制</t>
+        </is>
+      </c>
+      <c r="F56" s="15" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="G56" s="15" t="inlineStr">
+        <is>
+          <t>欧州の労働法制が強い地域から先例が生まれると、リモート越境雇用の多い業界全体の雇用設計（正社員比率・契約形態）に影響し得る。</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B57" s="15" t="inlineStr">
+        <is>
+          <t>戦略株主（テンセント）の撤退で浮動株化した中堅コンテンツ企業は、放送・出版業界で起きたアクティビスト標的化・再編と同じ道を辿るか？</t>
+        </is>
+      </c>
+      <c r="C57" s="15" t="inlineStr">
+        <is>
+          <t>テンセント、マーベラスなど日本のゲーム会社株の売却を協議（Bloomberg, 7/3記録）</t>
+        </is>
+      </c>
+      <c r="D57" s="15" t="inlineStr">
+        <is>
+          <t>テンセント,マーベラス</t>
+        </is>
+      </c>
+      <c r="E57" s="15" t="inlineStr">
+        <is>
+          <t>金融（アクティビスト）・放送・出版・商社</t>
+        </is>
+      </c>
+      <c r="F57" s="15" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="G57" s="15" t="inlineStr">
+        <is>
+          <t>中国資本の退潮はガバナンス・地政学起点であり、受け皿が国内か中東系かで業界の資本地図が変わる。大量保有報告書の動きが先行指標。</t>
         </is>
       </c>
     </row>
@@ -8005,9 +8116,9 @@
           <t>オフライン大会(7週間)</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
-        <is>
-          <t>賞金総額7,500万ドルで史上最大。25タイトル・200クラブ。開会式7/8(La Seine Musicale)。リヤドからパリへ会場変更。</t>
+      <c r="G4" s="15" t="inlineStr">
+        <is>
+          <t>リヤドから移転し史上初の国外(パリ)開催。7/8にラ・セーヌ・ミュジカルで開幕セレモニー、競技は7/9〜。賞金総額7,500万ドル・24競技25種目。ソニーが技術・放送パートナーシップを拡大(7/2発表)。</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
@@ -8020,9 +8131,9 @@
           <t>開催予定</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-17</t>
+      <c r="J4" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
         </is>
       </c>
     </row>
@@ -9597,9 +9708,9 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="14" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
+      <c r="A12" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
@@ -9632,14 +9743,14 @@
           <t>新規流入鈍化の中、既存IPの相互送客と話題波及でCACを抑えつつ稼働を維持する効率の良さ。音楽・アニメ側もファン拡張の場として歓迎。</t>
         </is>
       </c>
-      <c r="H12" s="14" t="inlineStr">
-        <is>
-          <t>ライブサービスの標準運営として定着。コラボ調達力・世界観統合の巧拙が差別化要因に。質より量の乱発はノイズ化リスク。</t>
-        </is>
-      </c>
-      <c r="I12" s="14" t="inlineStr">
-        <is>
-          <t>OW×YOASOBI(7/1開幕)/餓狼伝説CotW×北斗の拳ケンシロウ(6/29)</t>
+      <c r="H12" s="15" t="inlineStr">
+        <is>
+          <t>外部IP連携に加え「自社IP同士の社内クロスオーバー」（カプコン：バイオ×モンハン）へ拡張。許諾コストが低い自社IP回遊型は他社も追随しやすく、運営型の標準装備化が進む。</t>
+        </is>
+      </c>
+      <c r="I12" s="15" t="inlineStr">
+        <is>
+          <t>『BIOHAZARD Survival Unit』×『モンスターハンター』コラボ開始（4Gamer, 7/3日次）／『NIKKE』新章配信（4Gamer, 7/2）</t>
         </is>
       </c>
       <c r="J12" s="14" t="n">
@@ -9657,7 +9768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L241"/>
+  <dimension ref="A1:L251"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -24620,6 +24731,600 @@
         </is>
       </c>
       <c r="L241" s="14" t="inlineStr"/>
+    </row>
+    <row r="242">
+      <c r="A242" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B242" s="15" t="inlineStr">
+        <is>
+          <t>カプコン『鬼武者 Way of the Sword』発売日を9/25→9/4に3週間前倒し</t>
+        </is>
+      </c>
+      <c r="C242" s="15" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/865/G086595/20260702003/</t>
+        </is>
+      </c>
+      <c r="D242" s="15" t="inlineStr">
+        <is>
+          <t>カプコンの完全新作アクション『鬼武者 Way of the Sword』は6月のカプコンスポットライトで9/25発売と告知されたばかりだった。開発が予定より順調に進んだことを受け、発売日を3週間前倒しする異例の変更を7/2に発表した。</t>
+        </is>
+      </c>
+      <c r="E242" s="15" t="inlineStr">
+        <is>
+          <t>発売日は2026年9月4日に確定。延期が常態化する業界で「前倒し」は極めて珍しく、品質完成度への自信の表れと受け止められている。9月上旬は競合大作が比較的少ない時期で、販売面でも有利に働く可能性がある。</t>
+        </is>
+      </c>
+      <c r="F242" s="15" t="inlineStr">
+        <is>
+          <t>・延期ではなく前倒しという異例の日程変更
+・9/4は劇場アニメ『SEKIRO: NO DEFEAT』公開と同日で和風アクションが集中
+・6月配信済みの体験版で事前評価は良好
+・年末商戦前に販売の初速を確保する狙い</t>
+        </is>
+      </c>
+      <c r="G242" s="15" t="inlineStr">
+        <is>
+          <t>前倒しにより9月第1週の「和風アクション週間」が形成され、話題の相乗効果が見込まれる。初速が好調ならカプコンの2027年3月期第2四半期業績の上振れ要因となり、休眠IP復活路線がさらに加速しそうだ。</t>
+        </is>
+      </c>
+      <c r="H242" s="15" t="inlineStr">
+        <is>
+          <t>AAAタイトルの発売時期戦略と競合回避</t>
+        </is>
+      </c>
+      <c r="I242" s="15" t="inlineStr">
+        <is>
+          <t>カプコン</t>
+        </is>
+      </c>
+      <c r="J242" s="15" t="inlineStr">
+        <is>
+          <t>鬼武者 Way of the Sword</t>
+        </is>
+      </c>
+      <c r="K242" s="15" t="inlineStr">
+        <is>
+          <t>新作,国内</t>
+        </is>
+      </c>
+      <c r="L242" s="15" t="inlineStr"/>
+    </row>
+    <row r="243">
+      <c r="A243" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B243" s="15" t="inlineStr">
+        <is>
+          <t>任天堂『リズム天国 ミラクルスターズ』7/2発売—シリーズ11年ぶりの完全新作</t>
+        </is>
+      </c>
+      <c r="C243" s="15" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/895/G089553/20260629023/</t>
+        </is>
+      </c>
+      <c r="D243" s="15" t="inlineStr">
+        <is>
+          <t>『リズム天国』シリーズは2015年の『ザ・ベスト＋』を最後に新作が途絶えていた。つんく♂氏監修の音楽ゲームとして根強いファンを持ち、11年ぶりの完全新作がSwitch/Switch 2向けに7/2発売された。</t>
+        </is>
+      </c>
+      <c r="E243" s="15" t="inlineStr">
+        <is>
+          <t>シリーズ伝統の「ノリ」を重視した1ボタン主体のリズムアクションを継承しつつ、新規ミニゲームを多数収録。シリーズ未経験者でも遊びやすい設計で、発売日から国内で高い注目を集めている。</t>
+        </is>
+      </c>
+      <c r="F243" s="15" t="inlineStr">
+        <is>
+          <t>・11年ぶりのシリーズ完全新作
+・Switch 2普及期のファーストパーティ供給強化の一環
+・つんく♂氏関与の音楽主導設計が健在
+・休眠IP復活の任天堂側の代表例</t>
+        </is>
+      </c>
+      <c r="G243" s="15" t="inlineStr">
+        <is>
+          <t>Switch 2の普及局面で任天堂は休眠IPの復活を続ける見込み。中小規模タイトルでリリース間隔を埋める戦略は、大作偏重の他社に対する対照例として業界内で参照されそうだ。</t>
+        </is>
+      </c>
+      <c r="H243" s="15" t="inlineStr">
+        <is>
+          <t>休眠IPのリバイバル戦略</t>
+        </is>
+      </c>
+      <c r="I243" s="15" t="inlineStr">
+        <is>
+          <t>任天堂</t>
+        </is>
+      </c>
+      <c r="J243" s="15" t="inlineStr">
+        <is>
+          <t>リズム天国 ミラクルスターズ</t>
+        </is>
+      </c>
+      <c r="K243" s="15" t="inlineStr">
+        <is>
+          <t>新作,国内</t>
+        </is>
+      </c>
+      <c r="L243" s="15" t="inlineStr"/>
+    </row>
+    <row r="244">
+      <c r="A244" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B244" s="15" t="inlineStr">
+        <is>
+          <t>劇場アニメ『SEKIRO: NO DEFEAT』9/4公開へ—完成披露試写会の実施を発表</t>
+        </is>
+      </c>
+      <c r="C244" s="15" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/422/G042247/20260701025/</t>
+        </is>
+      </c>
+      <c r="D244" s="15" t="inlineStr">
+        <is>
+          <t>フロム・ソフトウェアの『SEKIRO: SHADOWS DIE TWICE』を原作とする劇場アニメ。gamescom 2025で発表され、9/4から3週間限定で上映される。公開に先立ち完成披露試写会の開催が発表された。</t>
+        </is>
+      </c>
+      <c r="E244" s="15" t="inlineStr">
+        <is>
+          <t>主要キャストによる舞台挨拶付きの完成披露試写会を実施予定。ゲームIPの劇場アニメ化は『ニーア』『ペルソナ』等に続く流れで、3週間限定上映＋前売り特典という興行設計も特徴的。</t>
+        </is>
+      </c>
+      <c r="F244" s="15" t="inlineStr">
+        <is>
+          <t>・9/4より3週間限定上映という短期集中型興行
+・原作ゲームの声優陣が続投しファン層を直撃
+・ゲームIPの映像化が国内で活発化
+・カプコン『鬼武者』発売と同日で和風IPが集中</t>
+        </is>
+      </c>
+      <c r="G244" s="15" t="inlineStr">
+        <is>
+          <t>ゲームIP映画・アニメ化の成功例が積み上がれば、パブリッシャーは映像部門への投資を拡大する。限定上映＋配信展開のハイブリッド型が国内ゲームIP映像化の標準モデルになる可能性がある。</t>
+        </is>
+      </c>
+      <c r="H244" s="15" t="inlineStr">
+        <is>
+          <t>ゲームIPのトランスメディア展開</t>
+        </is>
+      </c>
+      <c r="I244" s="15" t="inlineStr">
+        <is>
+          <t>フロム・ソフトウェア,アニプレックス</t>
+        </is>
+      </c>
+      <c r="J244" s="15" t="inlineStr">
+        <is>
+          <t>SEKIRO: SHADOWS DIE TWICE</t>
+        </is>
+      </c>
+      <c r="K244" s="15" t="inlineStr">
+        <is>
+          <t>国内,新作</t>
+        </is>
+      </c>
+      <c r="L244" s="15" t="inlineStr"/>
+    </row>
+    <row r="245">
+      <c r="A245" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B245" s="15" t="inlineStr">
+        <is>
+          <t>NCSOFT『AION2』グローバル版を9月開始へ—UE5製MMORPGのメディア体験会</t>
+        </is>
+      </c>
+      <c r="C245" s="15" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/440/G044032/20260615030/</t>
+        </is>
+      </c>
+      <c r="D245" s="15" t="inlineStr">
+        <is>
+          <t>韓国NCSOFTの主力IP『AION』の続編となるPC向けMMORPG。韓国・台湾では先行サービス中で、2026年9月にグローバル(日本含む)展開を予定。日本メディア向け体験会が開催され7/2にレポートが解禁された。</t>
+        </is>
+      </c>
+      <c r="E245" s="15" t="inlineStr">
+        <is>
+          <t>UE5による表現力と自由度の高いキャラクターメイク、ポテンシャル(成長)システムが特徴。MMORPGが縮小傾向の日本市場に大型タイトルが投入される数少ない機会となる。</t>
+        </is>
+      </c>
+      <c r="F245" s="15" t="inlineStr">
+        <is>
+          <t>・9月グローバルローンチで日本市場に再挑戦
+・UE5採用による次世代MMORPGの試金石
+・NCSOFTは『シンダーシティ』等新規IPも同時展開中
+・韓国大手の海外売上比率引き上げ戦略の中核</t>
+        </is>
+      </c>
+      <c r="G245" s="15" t="inlineStr">
+        <is>
+          <t>国内MMORPG市場は縮小が続くが、AION2の成否は韓国大手の日本再進出判断に影響する。失敗すればモバイル・サブカル系への戦略転換が加速し、成功すればPC大型オンラインの再評価につながる。</t>
+        </is>
+      </c>
+      <c r="H245" s="15" t="inlineStr">
+        <is>
+          <t>韓国ゲーム大手のグローバル展開戦略</t>
+        </is>
+      </c>
+      <c r="I245" s="15" t="inlineStr">
+        <is>
+          <t>NCSOFT</t>
+        </is>
+      </c>
+      <c r="J245" s="15" t="inlineStr">
+        <is>
+          <t>AION2</t>
+        </is>
+      </c>
+      <c r="K245" s="15" t="inlineStr">
+        <is>
+          <t>新作,海外</t>
+        </is>
+      </c>
+      <c r="L245" s="15" t="inlineStr"/>
+    </row>
+    <row r="246">
+      <c r="A246" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B246" s="15" t="inlineStr">
+        <is>
+          <t>Esports World Cup 2026、ソニーとのパートナーシップ拡大を発表—パリ大会は7/8開幕</t>
+        </is>
+      </c>
+      <c r="C246" s="15" t="inlineStr">
+        <is>
+          <t>https://www.sportsvideo.org/2026/07/02/esports-world-cup-2026-announces-expanded-sony-partnership-for-paris-event/</t>
+        </is>
+      </c>
+      <c r="D246" s="15" t="inlineStr">
+        <is>
+          <t>EWC 2026は中東情勢を受けリヤドからパリへ移転して開催される初の国外大会。開幕(7/8のオープニングセレモニー、競技は7/9〜)を前に、ソニーとの技術・放送分野でのパートナーシップ拡大が7/2に発表された。</t>
+        </is>
+      </c>
+      <c r="E246" s="15" t="inlineStr">
+        <is>
+          <t>賞金総額7,500万ドル・24競技25種目という過去最大規模を維持したままパリのラ・セーヌ・ミュジカルで開幕する。ソニーは映像・音響技術や中継制作面で関与を深め、エンタメ企業としての露出を拡大する。</t>
+        </is>
+      </c>
+      <c r="F246" s="15" t="inlineStr">
+        <is>
+          <t>・EWC史上初の国外(パリ)開催が目前
+・ソニーが技術・放送パートナーとして関与拡大
+・賞金総額7,500万ドルは前年から増額
+・DJ Snake等が出演する開幕セレモニーを7/8に単独開催</t>
+        </is>
+      </c>
+      <c r="G246" s="15" t="inlineStr">
+        <is>
+          <t>サウジ主導のeスポーツ興行に日米欧のエレクトロニクス・エンタメ大手が相乗りする構図が固まりつつある。ソニーはハード販売に加え中継技術・音楽で興行のインフラ側を押さえ、eスポーツの「放送産業化」が進みそうだ。</t>
+        </is>
+      </c>
+      <c r="H246" s="15" t="inlineStr">
+        <is>
+          <t>eスポーツ興行のスポンサー構造</t>
+        </is>
+      </c>
+      <c r="I246" s="15" t="inlineStr">
+        <is>
+          <t>ソニー,Esports World Cup Foundation</t>
+        </is>
+      </c>
+      <c r="J246" s="15" t="inlineStr"/>
+      <c r="K246" s="15" t="inlineStr">
+        <is>
+          <t>eスポーツ,海外</t>
+        </is>
+      </c>
+      <c r="L246" s="15" t="inlineStr"/>
+    </row>
+    <row r="247">
+      <c r="A247" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B247" s="15" t="inlineStr">
+        <is>
+          <t>Ubisoftバルセロナがストライキ—レイオフに抗議し6/30から7/16まで断続的に実施</t>
+        </is>
+      </c>
+      <c r="C247" s="15" t="inlineStr">
+        <is>
+          <t>https://www.gamedeveloper.com/business/ubisoft-barcelona-to-go-on-strike-over-proposed-layoffs</t>
+        </is>
+      </c>
+      <c r="D247" s="15" t="inlineStr">
+        <is>
+          <t>Ubisoftは6月の再編でバルセロナ拠点の51人(在籍の約28%)を削減対象とした。これに抗議し労働組合主導で6/30から7/16まで断続的なストライキが開始された。同社は2026年に入り6度の再編を実施している。</t>
+        </is>
+      </c>
+      <c r="E247" s="15" t="inlineStr">
+        <is>
+          <t>組合は5年間の集団解雇禁止と対象者の保護を要求。欧州のゲーム開発拠点で本格的なストライキに発展するのは異例で、業界の労働運動の転換点として注目される。</t>
+        </is>
+      </c>
+      <c r="F247" s="15" t="inlineStr">
+        <is>
+          <t>・欧州ゲーム開発拠点で異例の本格ストライキ
+・要求は「5年間の集団解雇禁止」と雇用保護
+・Ubisoftは2026年だけで6度目の再編・約380人削減
+・業界累計のレイオフは2022年以降4.5万人規模</t>
+        </is>
+      </c>
+      <c r="G247" s="15" t="inlineStr">
+        <is>
+          <t>要求が一部でも通れば欧州他拠点・他社の組合活動が一気に活性化する。スペイン・フランスの労働法制下では長期化リスクがあり、Ubisoftの開発パイプライン(進行中タイトル)への遅延波及が現実味を帯びる。</t>
+        </is>
+      </c>
+      <c r="H247" s="15" t="inlineStr">
+        <is>
+          <t>ゲーム産業の労働運動・組合化</t>
+        </is>
+      </c>
+      <c r="I247" s="15" t="inlineStr">
+        <is>
+          <t>Ubisoft</t>
+        </is>
+      </c>
+      <c r="J247" s="15" t="inlineStr"/>
+      <c r="K247" s="15" t="inlineStr">
+        <is>
+          <t>海外</t>
+        </is>
+      </c>
+      <c r="L247" s="15" t="inlineStr"/>
+    </row>
+    <row r="248">
+      <c r="A248" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B248" s="15" t="inlineStr">
+        <is>
+          <t>IVS2026パネル：AI時代のゲームマーケ「7割は自動化しても3割は人に残る」—Moloco/Braze登壇</t>
+        </is>
+      </c>
+      <c r="C248" s="15" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/991/G999110/20260617035/</t>
+        </is>
+      </c>
+      <c r="D248" s="15" t="inlineStr">
+        <is>
+          <t>京都で開催されたスタートアップカンファレンスIVS2026 KYOTOで、Moloco・Braze等のマーケティングテック企業がゲーム市場向けパネルを実施。AI活用でユーザー獲得(UA)がどう変わるかが議論された。</t>
+        </is>
+      </c>
+      <c r="E248" s="15" t="inlineStr">
+        <is>
+          <t>広告運用・クリエイティブ生成の約7割はAIで自動化が進む一方、ブランド判断・文化的文脈の理解など3割は人の仕事として残るとの見解が示された。LTV予測やパーソナライズ配信でのAI実装事例が共有された。</t>
+        </is>
+      </c>
+      <c r="F248" s="15" t="inlineStr">
+        <is>
+          <t>・UA運用の大半がAI自動化へ移行中
+・LTV予測・クリエイティブ生成が主戦場
+・MolocoやBraze等ツール企業が日本市場を重視
+・「人に残る3割」の定義が採用・組織設計の論点に</t>
+        </is>
+      </c>
+      <c r="G248" s="15" t="inlineStr">
+        <is>
+          <t>マーケ職の再定義が進み、ゲーム会社のUA部門は少人数化・ツール支出増へ。国内パブリッシャーもAIマーケSaaSへの依存を深め、広告代理店の中抜きが進む可能性が高い。</t>
+        </is>
+      </c>
+      <c r="H248" s="15" t="inlineStr">
+        <is>
+          <t>AIによるゲームマーケティング自動化</t>
+        </is>
+      </c>
+      <c r="I248" s="15" t="inlineStr">
+        <is>
+          <t>Moloco,Braze</t>
+        </is>
+      </c>
+      <c r="J248" s="15" t="inlineStr"/>
+      <c r="K248" s="15" t="inlineStr">
+        <is>
+          <t>技術,国内</t>
+        </is>
+      </c>
+      <c r="L248" s="15" t="inlineStr"/>
+    </row>
+    <row r="249">
+      <c r="A249" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B249" s="15" t="inlineStr">
+        <is>
+          <t>『BIOHAZARD Survival Unit』×『モンスターハンター』コラボ開始—カプコンIP同士の越境展開</t>
+        </is>
+      </c>
+      <c r="C249" s="15" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/926/G092667/20260702002/</t>
+        </is>
+      </c>
+      <c r="D249" s="15" t="inlineStr">
+        <is>
+          <t>カプコンとJOYCITYが共同展開するモバイル戦略ゲーム『BIOHAZARD Survival Unit』で、同じカプコンの『モンスターハンター』とのコラボが7/2に開始された。リオレウスやアイルーが登場する。</t>
+        </is>
+      </c>
+      <c r="E249" s="15" t="inlineStr">
+        <is>
+          <t>7/30までの期間限定でコラボイベントを実施。自社IP同士を外部開発の運営型タイトル内で掛け合わせる手法で、IPの相互送客とモバイル運営の活性化を狙う。</t>
+        </is>
+      </c>
+      <c r="F249" s="15" t="inlineStr">
+        <is>
+          <t>・カプコンIP同士の社内クロスオーバー
+・外部(韓国JOYCITY)開発の運営型タイトルが舞台
+・期間限定イベントで復帰・新規ユーザーを獲得
+・IPライセンスビジネスの多層化の例</t>
+        </is>
+      </c>
+      <c r="G249" s="15" t="inlineStr">
+        <is>
+          <t>自社IP間コラボは追加許諾コストが低く、他社も追随しやすい。運営型ゲームの「コラボ枠」が自社IPポートフォリオの回遊装置になり、IPホルダーの運営型参入がさらに進むと見られる。</t>
+        </is>
+      </c>
+      <c r="H249" s="15" t="inlineStr">
+        <is>
+          <t>IPクロスオーバーによる運営活性化</t>
+        </is>
+      </c>
+      <c r="I249" s="15" t="inlineStr">
+        <is>
+          <t>カプコン,JOYCITY</t>
+        </is>
+      </c>
+      <c r="J249" s="15" t="inlineStr">
+        <is>
+          <t>BIOHAZARD,モンスターハンター</t>
+        </is>
+      </c>
+      <c r="K249" s="15" t="inlineStr">
+        <is>
+          <t>国内,新作</t>
+        </is>
+      </c>
+      <c r="L249" s="15" t="inlineStr"/>
+    </row>
+    <row r="250">
+      <c r="A250" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B250" s="15" t="inlineStr">
+        <is>
+          <t>『Kingdom Come: Deliverance』公式ボードゲーム発表—Czech Games Editionがプレオーダー開始</t>
+        </is>
+      </c>
+      <c r="C250" s="15" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/022/G102212/20260702001/</t>
+        </is>
+      </c>
+      <c r="D250" s="15" t="inlineStr">
+        <is>
+          <t>Warhorse Studiosの中世RPG『Kingdom Come: Deliverance』を原作とするボードゲームが7/2に発表された。ボードゲーム大手Czech Games Editionが手がけ、プレオーダーが開始された。</t>
+        </is>
+      </c>
+      <c r="E250" s="15" t="inlineStr">
+        <is>
+          <t>デジタルゲームIPのアナログ(卓上)展開は『フロストパンク』『ダークソウル』等で定着しつつある流れ。原作の中世サバイバル要素を卓上で再現し、コアファン向け高単価商材として展開される。</t>
+        </is>
+      </c>
+      <c r="F250" s="15" t="inlineStr">
+        <is>
+          <t>・ゲームIPのボードゲーム化という定番化しつつある収益源
+・チェコの開発元と同国ボドゲ大手の地元連携
+・クラウドファンディング/プレオーダー型の販売手法
+・原作は続編ヒットでIP価値が上昇中</t>
+        </is>
+      </c>
+      <c r="G250" s="15" t="inlineStr">
+        <is>
+          <t>IPホルダーにとりボードゲーム化は低リスクのライセンス収益源として定着し、欧州スタジオ間の「地産地消」型IP連携が増える。国内IPでも同様の卓上展開が広がる余地がある。</t>
+        </is>
+      </c>
+      <c r="H250" s="15" t="inlineStr">
+        <is>
+          <t>ゲームIPのアナログ展開</t>
+        </is>
+      </c>
+      <c r="I250" s="15" t="inlineStr">
+        <is>
+          <t>Warhorse Studios,Czech Games Edition</t>
+        </is>
+      </c>
+      <c r="J250" s="15" t="inlineStr">
+        <is>
+          <t>Kingdom Come: Deliverance</t>
+        </is>
+      </c>
+      <c r="K250" s="15" t="inlineStr">
+        <is>
+          <t>新作,海外</t>
+        </is>
+      </c>
+      <c r="L250" s="15" t="inlineStr"/>
+    </row>
+    <row r="251">
+      <c r="A251" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B251" s="15" t="inlineStr">
+        <is>
+          <t>テンセント、マーベラスなど日本のゲーム会社株の売却を協議—投資先ポートフォリオを精査</t>
+        </is>
+      </c>
+      <c r="C251" s="15" t="inlineStr">
+        <is>
+          <t>https://www.bloomberg.com/jp/news/articles/2026-06-23/TH2I4XT9NJLS00</t>
+        </is>
+      </c>
+      <c r="D251" s="15" t="inlineStr">
+        <is>
+          <t>テンセントは世界的な投資先見直しの一環として、マーベラスを含む日本のゲーム会社への少数出資の売却を協議していると6月下旬にBloombergが報道。AI投資への資源再配分が背景にある。</t>
+        </is>
+      </c>
+      <c r="E251" s="15" t="inlineStr">
+        <is>
+          <t>損失覚悟で経営陣への売り戻しも検討対象とされる。一方フロム・ソフトウェア/KADOKAWA、プラチナゲームズへの出資は見直し対象外の見込み。日本の中堅ゲーム会社の株主構成に影響が及ぶ。</t>
+        </is>
+      </c>
+      <c r="F251" s="15" t="inlineStr">
+        <is>
+          <t>・テンセントが日本の投資先の選別を本格化
+・マーベラス等の少数出資が売却協議の対象
+・フロム/KADOKAWA等の戦略出資は維持見込み
+・背景はAIへの投資シフトと業界逆風</t>
+        </is>
+      </c>
+      <c r="G251" s="15" t="inlineStr">
+        <is>
+          <t>売却が実現すれば対象企業の株主構成が流動化し、国内事業会社・ファンドによる資本参加やTOB観測が浮上する。中国マネー退潮の受け皿として、サウジ系ファンドや国内商社の動きが焦点となる。</t>
+        </is>
+      </c>
+      <c r="H251" s="15" t="inlineStr">
+        <is>
+          <t>中国資本の日本ゲーム投資の転換点</t>
+        </is>
+      </c>
+      <c r="I251" s="15" t="inlineStr">
+        <is>
+          <t>テンセント,マーベラス</t>
+        </is>
+      </c>
+      <c r="J251" s="15" t="inlineStr"/>
+      <c r="K251" s="15" t="inlineStr">
+        <is>
+          <t>M&amp;A,海外,国内</t>
+        </is>
+      </c>
+      <c r="L251" s="15" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
daily-news(4) + cross-question + game-design update (2026-07-04)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -3528,7 +3528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G57"/>
+  <dimension ref="A1:G58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5646,6 +5646,43 @@
       <c r="G57" s="15" t="inlineStr">
         <is>
           <t>中国資本の退潮はガバナンス・地政学起点であり、受け皿が国内か中東系かで業界の資本地図が変わる。大量保有報告書の動きが先行指標。</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B58" s="14" t="inlineStr">
+        <is>
+          <t>VTuber/タレント事務所が自社IPで公式ゲームを内製・パブリッシングする垂直統合（カバー『hololive Dreams』）は、芸能事務所・アニメ製作委員会・スポーツクラブなど他のIP保有主体でも『許諾提供』から『自社パブリッシング』へ進むか？</t>
+        </is>
+      </c>
+      <c r="C58" s="14" t="inlineStr">
+        <is>
+          <t>カバー×QualiArts『hololive Dreams』7/23全世界同時リリース発表（7/4日次）</t>
+        </is>
+      </c>
+      <c r="D58" s="14" t="inlineStr">
+        <is>
+          <t>カバー, QualiArts, ホロライブ</t>
+        </is>
+      </c>
+      <c r="E58" s="14" t="inlineStr">
+        <is>
+          <t>芸能事務所, アニメ製作委員会, スポーツクラブ/リーグ, アイドル・音楽IP</t>
+        </is>
+      </c>
+      <c r="F58" s="14" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="G58" s="14" t="inlineStr">
+        <is>
+          <t>従来は外部にIPを許諾していた保有主体が、ファンダムの課金力を自ら取り込むため『発行主体』を自社へ寄せる動き。ライセンス料収入からレベニューシェア/自社売上への転換が論点。</t>
         </is>
       </c>
     </row>
@@ -9708,9 +9745,9 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="15" t="inlineStr">
-        <is>
-          <t>2026-07-03</t>
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
@@ -9748,9 +9785,9 @@
           <t>外部IP連携に加え「自社IP同士の社内クロスオーバー」（カプコン：バイオ×モンハン）へ拡張。許諾コストが低い自社IP回遊型は他社も追随しやすく、運営型の標準装備化が進む。</t>
         </is>
       </c>
-      <c r="I12" s="15" t="inlineStr">
-        <is>
-          <t>『BIOHAZARD Survival Unit』×『モンスターハンター』コラボ開始（4Gamer, 7/3日次）／『NIKKE』新章配信（4Gamer, 7/2）</t>
+      <c r="I12" s="14" t="inlineStr">
+        <is>
+          <t>『BIOHAZARD Survival Unit』×『モンスターハンター』コラボ開始（4Gamer, 7/3日次）／『NIKKE』新章配信（4Gamer, 7/2）／『荒野行動』×エヴァコラボ第8弾（4Gamer, 7/4）／崩壊：スターレイル×Fateコラボ第2弾（7/4日次）</t>
         </is>
       </c>
       <c r="J12" s="14" t="n">
@@ -9768,7 +9805,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L251"/>
+  <dimension ref="A1:L255"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -25325,6 +25362,266 @@
         </is>
       </c>
       <c r="L251" s="15" t="inlineStr"/>
+    </row>
+    <row r="252">
+      <c r="A252" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B252" s="14" t="inlineStr">
+        <is>
+          <t>HoYoverse『崩壊：スターレイル』Ver.4.4予告番組公開—7/15更新へ、星5「姫子・旅立ち」実装＆Fateコラボ第2弾</t>
+        </is>
+      </c>
+      <c r="C252" s="14" t="inlineStr">
+        <is>
+          <t>https://dengekionline.com/article/202607/80327</t>
+        </is>
+      </c>
+      <c r="D252" s="14" t="inlineStr">
+        <is>
+          <t>HoYoverseの主力RPG『崩壊：スターレイル』は2023年配信開始のライブサービス型。約6週間ごとの大型アップデートで新キャラ・ストーリー・イベントを供給し、ガチャ課金と話題性を回し続けるモデルを確立している。</t>
+        </is>
+      </c>
+      <c r="E252" s="14" t="inlineStr">
+        <is>
+          <t>7/3配信の予告番組でVer.4.4「汽笛は轟く、帰寂のさなかに」を7/15配信と告知。新星5「姫子・旅立ち」(炎・知恵)を実装し、7/24からはFate/stay night[UBW]コラボ第2弾で遠坂凛・ギルガメッシュが登場する。</t>
+        </is>
+      </c>
+      <c r="F252" s="14" t="inlineStr">
+        <is>
+          <t>・約6週間サイクルの定例大型アップデートを堅持
+・看板キャラの新バージョンで既存ユーザーの再課金を喚起
+・人気アニメIP(Fate)との反復コラボで新規流入と話題を設計
+・ガチャ復刻で過去キャラの取りこぼし需要も回収</t>
+        </is>
+      </c>
+      <c r="G252" s="14" t="inlineStr">
+        <is>
+          <t>定例アプデ＋外部IPコラボの反復という運営型の勝ちパターンは継続。話題の谷を作らぬため、成功IPを繰り返し起用する「IP再利用」が中国系ライブサービス全体で標準化していく。</t>
+        </is>
+      </c>
+      <c r="H252" s="14" t="inlineStr">
+        <is>
+          <t>ライブサービスの更新サイクル設計とコラボ運用</t>
+        </is>
+      </c>
+      <c r="I252" s="14" t="inlineStr">
+        <is>
+          <t>HoYoverse, Type-Moon/Aniplex</t>
+        </is>
+      </c>
+      <c r="J252" s="14" t="inlineStr">
+        <is>
+          <t>崩壊：スターレイル, Fate/stay night</t>
+        </is>
+      </c>
+      <c r="K252" s="14" t="inlineStr">
+        <is>
+          <t>新作,海外</t>
+        </is>
+      </c>
+      <c r="L252" s="14" t="inlineStr">
+        <is>
+          <t>予告番組7/3 20:30配信、更新7/15予定</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B253" s="14" t="inlineStr">
+        <is>
+          <t>カバー×QualiArts『hololive Dreams（ホロドリ）』7/23全世界同時リリース決定—Steam版も展開</t>
+        </is>
+      </c>
+      <c r="C253" s="14" t="inlineStr">
+        <is>
+          <t>https://news.denfaminicogamer.jp/news/2607033h</t>
+        </is>
+      </c>
+      <c r="D253" s="14" t="inlineStr">
+        <is>
+          <t>VTuber事務所ホロライブを運営するカバーは、タレントIPをグッズ・ライブ・ゲームへ多面展開してきた。ゲームは外部への許諾提供が中心だったが、公式スマホゲームとして自社IPを直接ゲーム化・パブリッシングする動きを本格化させている。</t>
+        </is>
+      </c>
+      <c r="E253" s="14" t="inlineStr">
+        <is>
+          <t>カバーとサイバーエージェント傘下QualiArtsが共同開発したホロライブ初の公式スマホゲーム『hololive Dreams』を7/23に全世界同時リリースと発表。テーマパークが舞台のリズム&amp;RPGで基本無料・一部課金。Steam版も予定しデータ同期に対応する。</t>
+        </is>
+      </c>
+      <c r="F253" s="14" t="inlineStr">
+        <is>
+          <t>・タレントIPホルダーが公式ゲームを内製・パブリッシング
+・スマホ＋Steamのマルチプラットフォーム同時展開
+・全世界同時配信でグローバルファンダムを取り込み
+・リズム＋RPGでライブ・音楽資産をゲーム内に転用</t>
+        </is>
+      </c>
+      <c r="G253" s="14" t="inlineStr">
+        <is>
+          <t>VTuber/タレント事務所が自社IPのゲームを外部許諾に頼らず内製・パブリッシングする垂直統合が拡大。ファンダムの熱量を課金に直結させやすく、他のライバー事務所やアイドル系IPも追随する可能性が高い。</t>
+        </is>
+      </c>
+      <c r="H253" s="14" t="inlineStr">
+        <is>
+          <t>IPホルダーによるゲーム内製・パブリッシング垂直統合</t>
+        </is>
+      </c>
+      <c r="I253" s="14" t="inlineStr">
+        <is>
+          <t>カバー, QualiArts(サイバーエージェント)</t>
+        </is>
+      </c>
+      <c r="J253" s="14" t="inlineStr">
+        <is>
+          <t>ホロライブ, hololive Dreams</t>
+        </is>
+      </c>
+      <c r="K253" s="14" t="inlineStr">
+        <is>
+          <t>新作,国内</t>
+        </is>
+      </c>
+      <c r="L253" s="14" t="inlineStr">
+        <is>
+          <t>リズム&amp;RPG。基本無料＋一部課金</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B254" s="14" t="inlineStr">
+        <is>
+          <t>NetEase『荒野行動』×『エヴァンゲリオン』コラボ第8弾を7/4開始—覚醒初号機モチーフの殿堂級アイテム</t>
+        </is>
+      </c>
+      <c r="C254" s="14" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/402/G040245/20260704001/</t>
+        </is>
+      </c>
+      <c r="D254" s="14" t="inlineStr">
+        <is>
+          <t>NetEaseのバトルロイヤル『荒野行動』は日本で長期運営される看板タイトル。人気アニメIPとの反復コラボを重ね、限定スキン販売でリテンションと課金を維持してきた。エヴァとのコラボはこれで8回目となる。</t>
+        </is>
+      </c>
+      <c r="E254" s="14" t="inlineStr">
+        <is>
+          <t>7/4より『エヴァンゲリオン』コラボ第8弾を開始。『ヱヴァンゲリヲン新劇場版：破』の覚醒初号機をモチーフにした「殿堂級」コラボアイテムが登場。人気IPの反復起用で長期運営タイトルの稼働を下支えする。</t>
+        </is>
+      </c>
+      <c r="F254" s="14" t="inlineStr">
+        <is>
+          <t>・同一IPとの8回目という反復コラボ
+・「殿堂級」上位レア枠で高単価課金を設計
+・長期運営BRのリテンション施策としてのIPコラボ
+・アニメIP側もファン接点として継続活用</t>
+        </is>
+      </c>
+      <c r="G254" s="14" t="inlineStr">
+        <is>
+          <t>長期運営タイトルは新規IP開拓より「実績あるIPの反復コラボ」に回帰。許諾関係が確立した相手との継続コラボはコスト・成果が読みやすく、運営型の定番装備として定着する。</t>
+        </is>
+      </c>
+      <c r="H254" s="14" t="inlineStr">
+        <is>
+          <t>長期運営タイトルの反復IPコラボ経済</t>
+        </is>
+      </c>
+      <c r="I254" s="14" t="inlineStr">
+        <is>
+          <t>NetEase Games, カラー(エヴァ)</t>
+        </is>
+      </c>
+      <c r="J254" s="14" t="inlineStr">
+        <is>
+          <t>荒野行動, エヴァンゲリオン</t>
+        </is>
+      </c>
+      <c r="K254" s="14" t="inlineStr">
+        <is>
+          <t>新作,海外</t>
+        </is>
+      </c>
+      <c r="L254" s="14" t="inlineStr">
+        <is>
+          <t>コラボ第8弾。4Gamer 7/4</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B255" s="14" t="inlineStr">
+        <is>
+          <t>Steamサマーセール最中に同時接続が過去最高を更新、『Cyberpunk 2077』が累計4,000万本突破</t>
+        </is>
+      </c>
+      <c r="C255" s="14" t="inlineStr">
+        <is>
+          <t>https://www.neowin.net/news/steam-just-hit-a-new-all-time-concurrent-player-record-in-the-middle-of-its-summer-sale/</t>
+        </is>
+      </c>
+      <c r="D255" s="14" t="inlineStr">
+        <is>
+          <t>Steamは季節セールで大量の値引きとウィッシュリスト消化を促し、同時接続数を押し上げてきた。2026年サマーセール(6/25-7/9)期間中にプラットフォーム全体の稼働が過去最高圏に達し、旧作の長期販売も伸びている。</t>
+        </is>
+      </c>
+      <c r="E255" s="14" t="inlineStr">
+        <is>
+          <t>サマーセール開催中にSteamの同時接続ユーザーが過去最高水準を更新。あわせてCD Projekt REDの『Cyberpunk 2077』が累計販売4,000万本を突破し、値引きと継続アップデートによる旧作ロングテール販売の強さを示した。</t>
+        </is>
+      </c>
+      <c r="F255" s="14" t="inlineStr">
+        <is>
+          <t>・季節セールがプラットフォーム全体の同接を記録圏へ押し上げ
+・『Cyberpunk 2077』累計4,000万本、発売後の巻き返し
+・値引き＋アプデによる旧作ロングテールの収益貢献
+・PCゲーム市場の地力の強さを示す指標</t>
+        </is>
+      </c>
+      <c r="G255" s="14" t="inlineStr">
+        <is>
+          <t>新作不足が続く中、大型旧作の値引き＋継続運営によるロングテール販売がパブリッシャー収益の柱として重みを増す。カタログ資産の再評価が進み、旧作リマスター/再販売への投資が加速する。</t>
+        </is>
+      </c>
+      <c r="H255" s="14" t="inlineStr">
+        <is>
+          <t>PC旧作のロングテール収益とセール設計</t>
+        </is>
+      </c>
+      <c r="I255" s="14" t="inlineStr">
+        <is>
+          <t>Valve, CD Projekt RED</t>
+        </is>
+      </c>
+      <c r="J255" s="14" t="inlineStr">
+        <is>
+          <t>Steam, Cyberpunk 2077</t>
+        </is>
+      </c>
+      <c r="K255" s="14" t="inlineStr">
+        <is>
+          <t>海外</t>
+        </is>
+      </c>
+      <c r="L255" s="14" t="inlineStr">
+        <is>
+          <t>サマーセール6/25-7/9。Cyberpunk累計4,000万本</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
daily-news(3) + cross-question(1) + prediction(1): Alim ブレフロ / エヌアイン全国大会 / Paramount×WBD
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -816,7 +816,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1602,6 +1602,43 @@
       <c r="G21" s="15" t="inlineStr">
         <is>
           <t>マーベラス等対象銘柄の大量保有報告書・変更報告書、TOB公告、テンセントの持分変動開示を観測。売却先が経営陣(MBO型)か第三者かで再編の広がりが判別できる。</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B22" s="15" t="inlineStr">
+        <is>
+          <t>パラマウント×WBD統合の承認後、映像・配信を主眼とする新オーナーがコア外と位置づけたWB Games(Rocksteady・NetherRealm・TT・Avalanche)を分離・売却、または一部IPのライセンス外出しに動き、買い手にPIF/サウジ系・中堅パブリッシャーが付く二次的な業界再編が起きる。</t>
+        </is>
+      </c>
+      <c r="C22" s="15" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="D22" s="15" t="inlineStr">
+        <is>
+          <t>承認後〜2027年上期(2026 Q4〜)</t>
+        </is>
+      </c>
+      <c r="E22" s="15" t="inlineStr">
+        <is>
+          <t>Paramount Skydance, WBD, WB Games, Rocksteady, PIF/Savvy</t>
+        </is>
+      </c>
+      <c r="F22" s="15" t="inlineStr">
+        <is>
+          <t>「パラマウント×WBD買収、EUに是正案提示し承認期限を7/22へ延期」(daily 2026-07-01, Wikipedia/報道)</t>
+        </is>
+      </c>
+      <c r="G22" s="15" t="inlineStr">
+        <is>
+          <t>承認完了後のWB Gamesに関する分社・売却・スタジオ帰属変更の適時開示/報道、DC・Harry Potter等IPの第三者ライセンス提供発表を観測する。</t>
         </is>
       </c>
     </row>
@@ -3528,7 +3565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G58"/>
+  <dimension ref="A1:G59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5683,6 +5720,43 @@
       <c r="G58" s="14" t="inlineStr">
         <is>
           <t>従来は外部にIPを許諾していた保有主体が、ファンダムの課金力を自ら取り込むため『発行主体』を自社へ寄せる動き。ライセンス料収入からレベニューシェア/自社売上への転換が論点。</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B59" s="14" t="inlineStr">
+        <is>
+          <t>巨大メディア統合(Paramount×WBD)でゲーム事業が“中核ではない付随資産”として売買・埋没する構図は、映画・音楽・出版・放送のM&amp;Aで周辺事業が受ける扱いと同じか？——ゲーム部門はどの業界の“非中核事業”に該当するか？</t>
+        </is>
+      </c>
+      <c r="C59" s="14" t="inlineStr">
+        <is>
+          <t>パラマウント×WBD買収、EUに是正案提示し承認期限を7/22へ延期(daily 2026-07-01)</t>
+        </is>
+      </c>
+      <c r="D59" s="14" t="inlineStr">
+        <is>
+          <t>Paramount Skydance, WBD, WB Games</t>
+        </is>
+      </c>
+      <c r="E59" s="14" t="inlineStr">
+        <is>
+          <t>映画・映像, 音楽レーベル, 出版, 放送, 総合メディアコングロマリット</t>
+        </is>
+      </c>
+      <c r="F59" s="14" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="G59" s="14" t="inlineStr">
+        <is>
+          <t>統合の主目的が配信・映像にあるほど、ゲームは“シナジーで語られるが実行では後回し”になりやすい。買収後にどのタイミングで分離・ライセンス化されるかが、非中核事業の運命を占う共通パターンになり得る。</t>
         </is>
       </c>
     </row>
@@ -9805,7 +9879,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L255"/>
+  <dimension ref="A1:L258"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -25620,6 +25694,201 @@
       <c r="L255" s="14" t="inlineStr">
         <is>
           <t>サマーセール6/25-7/9。Cyberpunk累計4,000万本</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B256" s="14" t="inlineStr">
+        <is>
+          <t>アリム『ブレイブ フロンティア オリジン』2027年に日本・北米配信を発表——“原点回帰”のドット絵RPG</t>
+        </is>
+      </c>
+      <c r="C256" s="14" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/022/G102259/20260703012/</t>
+        </is>
+      </c>
+      <c r="D256" s="14" t="inlineStr">
+        <is>
+          <t>アリムの『ブレイブ フロンティア』は2014年配信のドット絵RPGで海外含め一時代を築いたが、近年は新規流入が鈍化。スマホRPG市場は大型IP・高精細3Dが主流化する一方、開発費高騰と競争激化で中堅パブリッシャーは差別化に苦戦し、過去の成功IPを“原点回帰”で再起動する動きが出ている。</t>
+        </is>
+      </c>
+      <c r="E256" s="14" t="inlineStr">
+        <is>
+          <t>アリムは新作スマホRPG『ブレイブ フロンティア オリジン』を2027年に日本・北米で配信すると発表。ティザーサイトを公開し、ドット絵のスピリットやフリック操作のブレイブバースト攻撃など初代の要素を継承しつつ“原点回帰”をテーマに掲げる。既存ファンの呼び戻しと海外同時展開を狙う。</t>
+        </is>
+      </c>
+      <c r="F256" s="14" t="inlineStr">
+        <is>
+          <t>・2014年の看板IPを“原点回帰”で再起動
+・日本と北米で2027年配信を予告
+・ドット絵×フリック操作という初代の意匠を継承
+・大型3D全盛の市場で懐古・ニッチ需要を狙う</t>
+        </is>
+      </c>
+      <c r="G256" s="14" t="inlineStr">
+        <is>
+          <t>高精細3D・大型IPの物量競争が続くスマホRPG市場では、中堅は“懐古・低容量・唯一性”を武器にニッチを深掘りする方向へ二極化しやすい。ブレフロ オリジンの初速と海外反応が、旧IP再起動という選択肢の採算性を占う試金石になる。</t>
+        </is>
+      </c>
+      <c r="H256" s="14" t="inlineStr">
+        <is>
+          <t>旧IP“原点回帰”再起動の採算とレトロ表現のニッチ戦略</t>
+        </is>
+      </c>
+      <c r="I256" s="14" t="inlineStr">
+        <is>
+          <t>アリム(Alim)</t>
+        </is>
+      </c>
+      <c r="J256" s="14" t="inlineStr">
+        <is>
+          <t>ブレイブ フロンティア, ブレイブ フロンティア オリジン</t>
+        </is>
+      </c>
+      <c r="K256" s="14" t="inlineStr">
+        <is>
+          <t>新作,国内</t>
+        </is>
+      </c>
+      <c r="L256" s="14" t="inlineStr">
+        <is>
+          <t>4Gamer 7/3。2027年配信予告・ティザー公開</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B257" s="14" t="inlineStr">
+        <is>
+          <t>アーケード格闘『エヌアイン完全世界 Anastasis』公式全国大会“第十次電光大戦”、7/11に予選開始</t>
+        </is>
+      </c>
+      <c r="C257" s="14" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/618/G061891/20260703057/</t>
+        </is>
+      </c>
+      <c r="D257" s="14" t="inlineStr">
+        <is>
+          <t>SUBTLE STYLE開発のアーケード対戦格闘『エヌアイン完全世界 Anastasis』は、タイトーのNESiCAxLive2で稼働する根強い人気タイトル。アーケード格闘は家庭用・オンライン中心の潮流の中で店舗集客の核として草の根大会が重要な役割を担い、メーカー公認の全国大会がコミュニティ維持のエンジンになっている。</t>
+        </is>
+      </c>
+      <c r="E257" s="14" t="inlineStr">
+        <is>
+          <t>SUBTLE STYLEは公式全国大会「第十次電光大戦 -Das ist Meine Welt-」を発表。7/11から全国8店舗で1on1の店舗予選を順次実施し、8/29-30に大阪KO-HATSUで決勝を開催。参加者には描き下ろしポストカードを配布し、来店誘引と競技コミュニティの活性化を図る。</t>
+        </is>
+      </c>
+      <c r="F257" s="14" t="inlineStr">
+        <is>
+          <t>・メーカー公認の全国大会“第十次”を開催
+・7/11予選開始〜8/29-30に大阪で決勝
+・全国8店舗の店舗予選＋描き下ろし特典で集客
+・アーケード格闘の草の根eスポーツ運営の一例</t>
+        </is>
+      </c>
+      <c r="G257" s="14" t="inlineStr">
+        <is>
+          <t>家庭用・配信が主戦場となる中でも、アーケード格闘は“店舗回帰の体験価値”と公認大会を軸にコミュニティを維持する路線が続く。ロケーション運営と連動した特典が来店KPIにどう効くかが、同種タイトルの大会設計の参考になる。</t>
+        </is>
+      </c>
+      <c r="H257" s="14" t="inlineStr">
+        <is>
+          <t>アーケード格闘の公認大会と店舗集客の連動設計</t>
+        </is>
+      </c>
+      <c r="I257" s="14" t="inlineStr">
+        <is>
+          <t>SUBTLE STYLE, タイトー</t>
+        </is>
+      </c>
+      <c r="J257" s="14" t="inlineStr">
+        <is>
+          <t>エヌアイン完全世界 Anastasis</t>
+        </is>
+      </c>
+      <c r="K257" s="14" t="inlineStr">
+        <is>
+          <t>eスポーツ,国内</t>
+        </is>
+      </c>
+      <c r="L257" s="14" t="inlineStr">
+        <is>
+          <t>4Gamer 7/3。予選7/11〜、決勝8/29-30大阪KO-HATSU</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B258" s="14" t="inlineStr">
+        <is>
+          <t>パラマウント×WBD買収、EUに是正案提示し承認期限を7/22へ延期——WBゲーム部門の帰属も焦点</t>
+        </is>
+      </c>
+      <c r="C258" s="14" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Proposed_acquisition_of_Warner_Bros._Discovery_by_Paramount_Skydance</t>
+        </is>
+      </c>
+      <c r="D258" s="14" t="inlineStr">
+        <is>
+          <t>WBDを巡ってはNetflixの提案をParamount Skydance(Ellison陣営)が上回り、WBD取締役会が“優越提案”と評価。約1,100億ドル規模の統合には、Rocksteady・NetherRealm・TT Games・AvalancheなどWB Gamesの主要スタジオとDC/ハリー・ポッター等のIPが含まれ、映像・配信中心のディールにゲーム事業が付随する構図となっている。</t>
+        </is>
+      </c>
+      <c r="E258" s="14" t="inlineStr">
+        <is>
+          <t>Paramount SkydanceはWBD買収を巡りEU競争当局の懸念に対応する是正案(remedies)を提示し、承認判断の期限を7/7から7/22へ延期したと報じられた。巨大メディア統合は最終盤の規制審査に入り、WB Gamesの主要スタジオ・IPの帰属と新オーナー下での位置づけが業界の関心事となっている。</t>
+        </is>
+      </c>
+      <c r="F258" s="14" t="inlineStr">
+        <is>
+          <t>・NetflixではなくParamount Skydanceが優越提案で先行
+・EUへ是正案提示、承認期限を7/22へ延期
+・約1,100億ドル規模の映像・配信中心ディール
+・Rocksteady等WB Gamesの帰属が付随論点に</t>
+        </is>
+      </c>
+      <c r="G258" s="14" t="inlineStr">
+        <is>
+          <t>承認が下りれば、映像・配信を主眼とする新オーナーがコア外のゲーム事業をどう扱うかが次の焦点。人気IPを抱えるWB Gamesは統合維持よりもライセンス活用や一部スタジオの分離を選ぶ余地があり、中堅パブリッシャー再編の起点になり得る。</t>
+        </is>
+      </c>
+      <c r="H258" s="14" t="inlineStr">
+        <is>
+          <t>メディア統合下でゲーム事業が付随資産化する力学</t>
+        </is>
+      </c>
+      <c r="I258" s="14" t="inlineStr">
+        <is>
+          <t>Paramount Skydance, Warner Bros. Discovery, Netflix</t>
+        </is>
+      </c>
+      <c r="J258" s="14" t="inlineStr">
+        <is>
+          <t>WB Games, Rocksteady, NetherRealm, DC, Harry Potter</t>
+        </is>
+      </c>
+      <c r="K258" s="14" t="inlineStr">
+        <is>
+          <t>M&amp;A,規制,海外</t>
+        </is>
+      </c>
+      <c r="L258" s="14" t="inlineStr">
+        <is>
+          <t>承認期限7/7→7/22に延期(EU是正案)。7/1報道</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
daily-news + cross-questions + events + predictions + game-design update
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -816,7 +816,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1639,6 +1639,43 @@
       <c r="G22" s="15" t="inlineStr">
         <is>
           <t>承認完了後のWB Gamesに関する分社・売却・スタジオ帰属変更の適時開示/報道、DC・Harry Potter等IPの第三者ライセンス提供発表を観測する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>ソニーの新作物理ディスク全廃を機に、限定版・コレクター向け物理版の需要がLimited Run Games等の専門レーベルへ集約し、パブリッシャーが自社流通せず専門レーベルへ委託する『物理版の外部化・寡占化』が進む</t>
+        </is>
+      </c>
+      <c r="C23" s="14" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="D23" s="14" t="inlineStr">
+        <is>
+          <t>1〜2年</t>
+        </is>
+      </c>
+      <c r="E23" s="14" t="inlineStr">
+        <is>
+          <t>ソニー(SIE), Limited Run Games</t>
+        </is>
+      </c>
+      <c r="F23" s="14" t="inlineStr">
+        <is>
+          <t>ソニー、PS新作の物理ディスク製造を2028年1月終了(PlayStation.Blog, 本日日次)</t>
+        </is>
+      </c>
+      <c r="G23" s="14" t="inlineStr">
+        <is>
+          <t>専門物理版レーベルの新規タイトル契約・提携数の増加、ソニー系IPの物理版が専門レーベル経由へ移行するかを観測</t>
         </is>
       </c>
     </row>
@@ -3565,7 +3602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G59"/>
+  <dimension ref="A1:G61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5757,6 +5794,80 @@
       <c r="G59" s="14" t="inlineStr">
         <is>
           <t>統合の主目的が配信・映像にあるほど、ゲームは“シナジーで語られるが実行では後回し”になりやすい。買収後にどのタイミングで分離・ライセンス化されるかが、非中核事業の運命を占う共通パターンになり得る。</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B60" s="14" t="inlineStr">
+        <is>
+          <t>ソニーの物理ディスク全廃が示す『所有からアクセスへ』の完全移行は、音楽・映像・書籍で起きた所有権消滅と同じ論点をゲームで再燃させ、中古・レンタル・与信ビジネスの何を消し何を生むか？</t>
+        </is>
+      </c>
+      <c r="C60" s="14" t="inlineStr">
+        <is>
+          <t>ソニー、PS新作の物理ディスク製造を2028年1月終了(PlayStation.Blog)</t>
+        </is>
+      </c>
+      <c r="D60" s="14" t="inlineStr">
+        <is>
+          <t>ソニー(SIE), GameStop</t>
+        </is>
+      </c>
+      <c r="E60" s="14" t="inlineStr">
+        <is>
+          <t>小売(中古流通), 金融(与信・分割), 音楽・映像(所有権論争)</t>
+        </is>
+      </c>
+      <c r="F60" s="14" t="inlineStr">
+        <is>
+          <t>オープン</t>
+        </is>
+      </c>
+      <c r="G60" s="14" t="inlineStr">
+        <is>
+          <t>所有権消滅は他メディアで先行済み。ゲームは中古・貸与の商流が大きい分、影響が非対称に出る可能性</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B61" s="14" t="inlineStr">
+        <is>
+          <t>AIデータセンター向けHBMがコンシューマ向けメモリを締め出す『部材の奪い合い』は、ゲーム機だけでなくPC・スマホ・自動車(車載半導体)でも同時に起きる構造問題ではないか？</t>
+        </is>
+      </c>
+      <c r="C61" s="14" t="inlineStr">
+        <is>
+          <t>DRAM価格Q2に最大89%高騰、2028年まで改善見込みなし(PC Gamer)</t>
+        </is>
+      </c>
+      <c r="D61" s="14" t="inlineStr">
+        <is>
+          <t>Samsung, SK hynix, Micron, ソニー</t>
+        </is>
+      </c>
+      <c r="E61" s="14" t="inlineStr">
+        <is>
+          <t>自動車(車載半導体), 通信・スマホ, PC・家電</t>
+        </is>
+      </c>
+      <c r="F61" s="14" t="inlineStr">
+        <is>
+          <t>オープン</t>
+        </is>
+      </c>
+      <c r="G61" s="14" t="inlineStr">
+        <is>
+          <t>AI投資が川上の部材配分を歪め、川下の民生機器全般のコスト構造を横断的に押し上げる論点</t>
         </is>
       </c>
     </row>
@@ -8197,54 +8308,54 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="14" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="14" t="inlineStr">
         <is>
           <t>Esports World Cup 2026</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="14" t="inlineStr">
         <is>
           <t>eスポーツ</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="14" t="inlineStr">
         <is>
           <t>仏パリ(Paris Expo Porte de Versailles)</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="14" t="inlineStr">
         <is>
           <t>オフライン大会(7週間)</t>
         </is>
       </c>
-      <c r="G4" s="15" t="inlineStr">
+      <c r="G4" s="14" t="inlineStr">
         <is>
           <t>リヤドから移転し史上初の国外(パリ)開催。7/8にラ・セーヌ・ミュジカルで開幕セレモニー、競技は7/9〜。賞金総額7,500万ドル・24競技25種目。ソニーが技術・放送パートナーシップを拡大(7/2発表)。</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H4" s="14" t="inlineStr">
         <is>
           <t>https://en.wikipedia.org/wiki/2026_Esports_World_Cup</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
-        <is>
-          <t>開催予定</t>
-        </is>
-      </c>
-      <c r="J4" s="15" t="inlineStr">
-        <is>
-          <t>2026-07-03</t>
+      <c r="I4" s="14" t="inlineStr">
+        <is>
+          <t>開催中</t>
+        </is>
+      </c>
+      <c r="J4" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>
@@ -9821,7 +9932,7 @@
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
@@ -9854,14 +9965,14 @@
           <t>新規流入鈍化の中、既存IPの相互送客と話題波及でCACを抑えつつ稼働を維持する効率の良さ。音楽・アニメ側もファン拡張の場として歓迎。</t>
         </is>
       </c>
-      <c r="H12" s="15" t="inlineStr">
-        <is>
-          <t>外部IP連携に加え「自社IP同士の社内クロスオーバー」（カプコン：バイオ×モンハン）へ拡張。許諾コストが低い自社IP回遊型は他社も追随しやすく、運営型の標準装備化が進む。</t>
+      <c r="H12" s="14" t="inlineStr">
+        <is>
+          <t>外部IP連携に加え「自社IP同士の社内クロスオーバー」（カプコン：バイオ×モンハン）へ拡張。許諾コストが低い自社IP回遊型は他社も追随しやすく、運営型の標準装備化が進む。 格闘ゲームでも外部IPゲストキャラを継続運営フックにする商法が定着。</t>
         </is>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
-          <t>『BIOHAZARD Survival Unit』×『モンスターハンター』コラボ開始（4Gamer, 7/3日次）／『NIKKE』新章配信（4Gamer, 7/2）／『荒野行動』×エヴァコラボ第8弾（4Gamer, 7/4）／崩壊：スターレイル×Fateコラボ第2弾（7/4日次）</t>
+          <t>『BIOHAZARD Survival Unit』×『モンスターハンター』コラボ開始（4Gamer, 7/3日次）／『NIKKE』新章配信（4Gamer, 7/2）／『荒野行動』×エヴァコラボ第8弾（4Gamer, 7/4）／崩壊：スターレイル×Fateコラボ第2弾（7/4日次）／『GGST』SP5に新ゲストキャラ参戦発表(4Gamer, 7/5日次)</t>
         </is>
       </c>
       <c r="J12" s="14" t="n">
@@ -9879,7 +9990,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L258"/>
+  <dimension ref="A1:L266"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -25889,6 +26000,514 @@
       <c r="L258" s="14" t="inlineStr">
         <is>
           <t>承認期限7/7→7/22に延期(EU是正案)。7/1報道</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B259" s="14" t="inlineStr">
+        <is>
+          <t>ソニー、PS新作の物理ディスク製造を2028年1月に終了へ</t>
+        </is>
+      </c>
+      <c r="C259" s="14" t="inlineStr">
+        <is>
+          <t>https://blog.playstation.com/2026/07/01/physical-disc-production-ending-in-january-2028-for-new-games-releasing-on-playstation-consoles/</t>
+        </is>
+      </c>
+      <c r="D259" s="14" t="inlineStr">
+        <is>
+          <t>PS4/PS5のフルゲームDL販売比率が85%に達し物理は15%まで縮小。デジタル移行が消費者側で先行するなか、ソニーは製造コストと需要動向を踏まえ物理媒体の段階的縮小を判断した。</t>
+        </is>
+      </c>
+      <c r="E259" s="14" t="inlineStr">
+        <is>
+          <t>ソニーは2028年1月以降、新作PSタイトルの物理ディスク製造を終了し、PS Storeと小売店ともデジタル販売のみへ移行すると7/1に発表。ゲーム保存・所有権を巡りコミュニティから強い反発が出ている。</t>
+        </is>
+      </c>
+      <c r="F259" s="14" t="inlineStr">
+        <is>
+          <t>DL比率85%到達が判断根拠
+新作は2028年1月以降デジタルのみ
+ゲーム保存・所有権問題に懸念
+発表直後にソニーはSNS運用を一時停止</t>
+        </is>
+      </c>
+      <c r="G259" s="14" t="inlineStr">
+        <is>
+          <t>任天堂・Xboxの物理縮小観測が強まる一方、限定版・コレクター需要を担う専門物理版レーベルの存在感が高まる。中古・レンタル・与信系ビジネスの再編も論点化する。</t>
+        </is>
+      </c>
+      <c r="H259" s="14" t="inlineStr">
+        <is>
+          <t>所有権(ownership)からアクセス権への移行</t>
+        </is>
+      </c>
+      <c r="I259" s="14" t="inlineStr">
+        <is>
+          <t>ソニー(SIE), GameStop</t>
+        </is>
+      </c>
+      <c r="J259" s="14" t="inlineStr">
+        <is>
+          <t>PlayStation</t>
+        </is>
+      </c>
+      <c r="K259" s="14" t="inlineStr">
+        <is>
+          <t>技術,海外,国内</t>
+        </is>
+      </c>
+      <c r="L259" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-01発表</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B260" s="14" t="inlineStr">
+        <is>
+          <t>GameStop、FY2026見通し上方修正しeBay買収を継続表明</t>
+        </is>
+      </c>
+      <c r="C260" s="14" t="inlineStr">
+        <is>
+          <t>https://investor.gamestop.com/news-releases/news-details/2026/GameStop-Provides-Fiscal-Year-2026-Outlook/default.aspx</t>
+        </is>
+      </c>
+      <c r="D260" s="14" t="inlineStr">
+        <is>
+          <t>GameStopは5月にeBayへ1株125ドル(総額約555億ドル)の買収を提案しeBayは「信頼性も魅力もない」と拒絶。以降もCohen CEOは持分を積み増し、買収意欲を維持していた。</t>
+        </is>
+      </c>
+      <c r="E260" s="14" t="inlineStr">
+        <is>
+          <t>GameStopはFY2026(27年1月期)の調整後EBITDAを前期3.45億ドルから6億ドル超へと見込む上方見通しを提示。あわせてeBay買収の追求を改めて表明し、株価は小幅上昇した。</t>
+        </is>
+      </c>
+      <c r="F260" s="14" t="inlineStr">
+        <is>
+          <t>調整後EBITDA見通し6億ドル超へ
+eBay買収提案(約555億ドル)を継続追求
+eBay株を約7.8%まで積み増し
+eBay取締役会は提案を拒絶済み</t>
+        </is>
+      </c>
+      <c r="G260" s="14" t="inlineStr">
+        <is>
+          <t>eBayの拒絶が続くなか、委任状争奪や更なる持分積み増しで圧力を強める可能性。ゲーム小売から二次流通プラットフォームへの業態転換を狙う動きが鮮明化する。</t>
+        </is>
+      </c>
+      <c r="H260" s="14" t="inlineStr">
+        <is>
+          <t>ゲーム小売の中古流通プラットフォーム化</t>
+        </is>
+      </c>
+      <c r="I260" s="14" t="inlineStr">
+        <is>
+          <t>GameStop, eBay</t>
+        </is>
+      </c>
+      <c r="J260" s="14" t="inlineStr"/>
+      <c r="K260" s="14" t="inlineStr">
+        <is>
+          <t>M&amp;A,業績,海外</t>
+        </is>
+      </c>
+      <c r="L260" s="14" t="inlineStr">
+        <is>
+          <t>FY2026見通し6/26公表</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B261" s="14" t="inlineStr">
+        <is>
+          <t>『GUILTY GEAR -STRIVE-』SP5に新ゲストキャラ、26年冬参戦</t>
+        </is>
+      </c>
+      <c r="C261" s="14" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/527/G052700/20260705003/</t>
+        </is>
+      </c>
+      <c r="D261" s="14" t="inlineStr">
+        <is>
+          <t>『GGST』はシーズンパスで継続運営するライブサービス型格闘ゲーム。既にCyberpunk: Edgerunnersの『ルーシー』をゲスト参戦させた実績があり、外部IPコラボが集客フックとなっている。</t>
+        </is>
+      </c>
+      <c r="E261" s="14" t="inlineStr">
+        <is>
+          <t>アークシステムワークスは7/5、Anime Expoの開発者パネルで『GGST』シーズンパス5に新たなゲストキャラを参戦させると発表。参戦時期は2026年冬で、キャラの正体は未公開。宮内ケンP が明かした。</t>
+        </is>
+      </c>
+      <c r="F261" s="14" t="inlineStr">
+        <is>
+          <t>SP5に2人目のゲストキャラ参戦
+参戦時期は2026年冬
+Anime Expoの開発者パネルで発表
+キャラ正体は未公開(前例はEdgerunnersルーシー)</t>
+        </is>
+      </c>
+      <c r="G261" s="14" t="inlineStr">
+        <is>
+          <t>格闘ゲームでの外部IPゲストキャラ商法が継続運営の定番フックとして定着。話題性の高いIPコラボが、eスポーツ視聴と新規参入の両面で運営指標を左右する。</t>
+        </is>
+      </c>
+      <c r="H261" s="14" t="inlineStr">
+        <is>
+          <t>格闘ゲームのライブサービス化とゲストキャラ商法</t>
+        </is>
+      </c>
+      <c r="I261" s="14" t="inlineStr">
+        <is>
+          <t>アークシステムワークス</t>
+        </is>
+      </c>
+      <c r="J261" s="14" t="inlineStr">
+        <is>
+          <t>GUILTY GEAR -STRIVE-</t>
+        </is>
+      </c>
+      <c r="K261" s="14" t="inlineStr">
+        <is>
+          <t>新作,国内</t>
+        </is>
+      </c>
+      <c r="L261" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-05発表(Anime Expo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B262" s="14" t="inlineStr">
+        <is>
+          <t>KONAMI原作アニメ『幻想水滸伝』10月放送決定、全国32局で</t>
+        </is>
+      </c>
+      <c r="C262" s="14" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/659/G065911/20260703035/</t>
+        </is>
+      </c>
+      <c r="D262" s="14" t="inlineStr">
+        <is>
+          <t>KONAMIは休眠自社IPの再活性を推進中。『幻想水滸伝』は完全リメイク発表に続きアニメ化が進行し、旧作RPGファンと新規層双方に向けたメディアミックス展開を強めている。</t>
+        </is>
+      </c>
+      <c r="E262" s="14" t="inlineStr">
+        <is>
+          <t>KONAMI原作アニメ『幻想水滸伝』が10月よりTOKYO MX・関西テレビ・BS朝日ほか全国32局で順次放送決定。amazarashiのOP主題歌を使った第2弾PVと追加キャストも公開された。</t>
+        </is>
+      </c>
+      <c r="F262" s="14" t="inlineStr">
+        <is>
+          <t>10月放送・全国32局で展開
+第2弾PV公開(OPはamazarashi)
+追加キャスト発表
+初回は60分スペシャル</t>
+        </is>
+      </c>
+      <c r="G262" s="14" t="inlineStr">
+        <is>
+          <t>休眠IPをアニメ等で再点火しリメイク版ゲームの販売に接続する手法が国内パブリッシャーで拡大。KONAMIは複数の旧作IPで同様の展開を進める公算。</t>
+        </is>
+      </c>
+      <c r="H262" s="14" t="inlineStr">
+        <is>
+          <t>休眠IPのメディアミックス再活性戦略</t>
+        </is>
+      </c>
+      <c r="I262" s="14" t="inlineStr">
+        <is>
+          <t>KONAMI</t>
+        </is>
+      </c>
+      <c r="J262" s="14" t="inlineStr">
+        <is>
+          <t>幻想水滸伝(Suikoden)</t>
+        </is>
+      </c>
+      <c r="K262" s="14" t="inlineStr">
+        <is>
+          <t>新作,国内</t>
+        </is>
+      </c>
+      <c r="L262" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-03公開</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B263" s="14" t="inlineStr">
+        <is>
+          <t>テトリスがCGアニメ『Tetris: World Builders』でIP拡張</t>
+        </is>
+      </c>
+      <c r="C263" s="14" t="inlineStr">
+        <is>
+          <t>https://tetris.com/news/teamto-and-the-tetris-company-announce-animated-series-tetristm-world-builders</t>
+        </is>
+      </c>
+      <c r="D263" s="14" t="inlineStr">
+        <is>
+          <t>The Tetris Companyは実写映画などに続きIPの多面展開を推進。抽象パズルIPを物語性のある子ども向けフランチャイズへ広げ、ライセンス収益の裾野拡大を狙う。</t>
+        </is>
+      </c>
+      <c r="E263" s="14" t="inlineStr">
+        <is>
+          <t>The Tetris CompanyとTeamTOは6歳以上向けCGアニメ『Tetris: World Builders』(52×11分)を発表。ソニック映画化で知られるChuck WilliamsがEPを務めSTEAM教育要素を織り込む。アヌシー映画祭で披露、現在は初期開発段階。</t>
+        </is>
+      </c>
+      <c r="F263" s="14" t="inlineStr">
+        <is>
+          <t>52×11分のCGアニメシリーズ
+6歳以上向け・STEAM教育要素
+EPはChuck Williams(ソニック映画)
+アヌシー映画祭で発表・初期開発段階</t>
+        </is>
+      </c>
+      <c r="G263" s="14" t="inlineStr">
+        <is>
+          <t>抽象ゲームIPでも映像化・教育コンテンツ化で長期ライセンス収益を狙う流れが加速。ゲーム発IPのファミリー/子ども向けメディア展開が任天堂・セガに続き拡大する。</t>
+        </is>
+      </c>
+      <c r="H263" s="14" t="inlineStr">
+        <is>
+          <t>ゲームIPの映像化・ライセンス多角化</t>
+        </is>
+      </c>
+      <c r="I263" s="14" t="inlineStr">
+        <is>
+          <t>The Tetris Company, TeamTO</t>
+        </is>
+      </c>
+      <c r="J263" s="14" t="inlineStr">
+        <is>
+          <t>Tetris</t>
+        </is>
+      </c>
+      <c r="K263" s="14" t="inlineStr">
+        <is>
+          <t>新作,海外</t>
+        </is>
+      </c>
+      <c r="L263" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-23発表</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B264" s="14" t="inlineStr">
+        <is>
+          <t>Esports World Cup 2026、パリで7/6開幕。7週間24タイトル</t>
+        </is>
+      </c>
+      <c r="C264" s="14" t="inlineStr">
+        <is>
+          <t>https://esportsworldcup.com/en/news/ewc26-week-1-overview</t>
+        </is>
+      </c>
+      <c r="D264" s="14" t="inlineStr">
+        <is>
+          <t>サウジ資本が主導するEWCは賞金総額で世界最大級のeスポーツ大会。2026年は開催地をパリに移し、規模・注目度とも前年を上回る布陣で臨む。ソニーとのパートナーシップ拡大も発表済み。</t>
+        </is>
+      </c>
+      <c r="E264" s="14" t="inlineStr">
+        <is>
+          <t>Esports World Cup 2026が7/6にパリで開幕。8/23まで7週間にわたり24タイトル25大会を実施する。初週はVALORANT・Dota 2・Apex等が並び、開会式は7/8にラ・セーヌ・ミュジカルで開催予定。</t>
+        </is>
+      </c>
+      <c r="F264" s="14" t="inlineStr">
+        <is>
+          <t>7/6開幕〜8/23まで7週間
+24タイトル25大会・過去最大級賞金
+開催地はパリ
+開会式は7/8</t>
+        </is>
+      </c>
+      <c r="G264" s="14" t="inlineStr">
+        <is>
+          <t>サウジ主導の大型化でeスポーツの賞金・放映・スポンサー経済圏が一段と集約。国別・タイトル別のプロシーンが夏の集客ピークとしてEWCへの依存を深める。</t>
+        </is>
+      </c>
+      <c r="H264" s="14" t="inlineStr">
+        <is>
+          <t>国家資本主導のeスポーツ経済圏</t>
+        </is>
+      </c>
+      <c r="I264" s="14" t="inlineStr">
+        <is>
+          <t>Esports World Cup Foundation, ソニー</t>
+        </is>
+      </c>
+      <c r="J264" s="14" t="inlineStr">
+        <is>
+          <t>VALORANT, Dota 2, Apex Legends</t>
+        </is>
+      </c>
+      <c r="K264" s="14" t="inlineStr">
+        <is>
+          <t>eスポーツ,海外</t>
+        </is>
+      </c>
+      <c r="L264" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-06開幕</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B265" s="14" t="inlineStr">
+        <is>
+          <t>DRAM価格がQ2に最大89%高騰、2028年まで改善見込みなし</t>
+        </is>
+      </c>
+      <c r="C265" s="14" t="inlineStr">
+        <is>
+          <t>https://www.pcgamer.com/hardware/memory/memory-crisis-and-sky-high-dram-prices-could-run-past-2028-as-samsung-and-sk-hynix-opt-to-minimize-the-risk-of-oversupply/</t>
+        </is>
+      </c>
+      <c r="D265" s="14" t="inlineStr">
+        <is>
+          <t>AIデータセンター向けHBMの利益率がコンシューマ向けDDR5の約10倍に達し、Samsung・SK hynix・Micronが生産をHBMへ優先配分。コンシューマ向けメモリの供給が細り価格が急騰している。</t>
+        </is>
+      </c>
+      <c r="E265" s="14" t="inlineStr">
+        <is>
+          <t>2026年Q2にDRAM価格がLPDDR5Xで最大89%、DDR4で最大51%高騰。大手はHBM優先で供給を絞り、価格改善は早くて2027年末〜2028年との観測。Steam Machine等ゲーム機/PCの値上げ圧力が続く。</t>
+        </is>
+      </c>
+      <c r="F265" s="14" t="inlineStr">
+        <is>
+          <t>Q2にLPDDR5X +89%、DDR4 +51%
+要因はAI向けHBMへの生産優先
+価格正常化は2028年以降か
+ゲーム機/PCの値上げ・出荷減に直結</t>
+        </is>
+      </c>
+      <c r="G265" s="14" t="inlineStr">
+        <is>
+          <t>部材コスト高が次世代機の価格・投入時期を左右する構造要因として長期化。PS6等の価格設定や、メモリ搭載量を抑えた設計・クラウド寄せの回避策が検討される。</t>
+        </is>
+      </c>
+      <c r="H265" s="14" t="inlineStr">
+        <is>
+          <t>AI需要と半導体の生産配分競合</t>
+        </is>
+      </c>
+      <c r="I265" s="14" t="inlineStr">
+        <is>
+          <t>Samsung, SK hynix, Micron, ソニー, Valve</t>
+        </is>
+      </c>
+      <c r="J265" s="14" t="inlineStr"/>
+      <c r="K265" s="14" t="inlineStr">
+        <is>
+          <t>技術,海外</t>
+        </is>
+      </c>
+      <c r="L265" s="14" t="inlineStr">
+        <is>
+          <t>PC Gamer報道</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B266" s="14" t="inlineStr">
+        <is>
+          <t>PEGI新基準6月施行、ガチャ・課金要素が年齢区分に直接反映</t>
+        </is>
+      </c>
+      <c r="C266" s="14" t="inlineStr">
+        <is>
+          <t>https://biggo.jp/news/202603121826_PEGI_New_Age_Rating_Rules_Loot_Boxes_In_Game_Purchases</t>
+        </is>
+      </c>
+      <c r="D266" s="14" t="inlineStr">
+        <is>
+          <t>欧州の年齢レーティングPEGIは、ビジネスモデルやオンライン機能を直接レーティングに反映する『インタラクティブ・リスク区分』を導入。ルートボックスや常時課金設計への規制圧力が高まっている。</t>
+        </is>
+      </c>
+      <c r="E266" s="14" t="inlineStr">
+        <is>
+          <t>2026年6月施行のPEGI新基準では、有料ランダムアイテム(ルートボックス)・ゲーム内課金・ログイン強制型の設計・オンライン安全性が評価対象化。バトルパスやデイリー報酬の一部はPEGI 7〜12へ引き上げられる。</t>
+        </is>
+      </c>
+      <c r="F266" s="14" t="inlineStr">
+        <is>
+          <t>課金・ランダム要素が年齢区分に直接影響
+ログイン強制設計はレーティング上昇
+オランダはガチャ全面禁止方針
+消費者団体は有料ルートボックス禁止も要請</t>
+        </is>
+      </c>
+      <c r="G266" s="14" t="inlineStr">
+        <is>
+          <t>レーティング上昇を避けるため課金設計を見直す動きが欧州向けタイトルで加速。年齢確認義務化とあわせ、ライブサービスのマネタイズ設計が地域ごとに分岐する。</t>
+        </is>
+      </c>
+      <c r="H266" s="14" t="inlineStr">
+        <is>
+          <t>課金設計と年齢レーティング・規制の連動</t>
+        </is>
+      </c>
+      <c r="I266" s="14" t="inlineStr">
+        <is>
+          <t>PEGI, EA, Electronic Arts</t>
+        </is>
+      </c>
+      <c r="J266" s="14" t="inlineStr"/>
+      <c r="K266" s="14" t="inlineStr">
+        <is>
+          <t>規制,海外</t>
+        </is>
+      </c>
+      <c r="L266" s="14" t="inlineStr">
+        <is>
+          <t>2026-06施行</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
weekly-stocks + IP watch update (2026-07-06)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -28130,8 +28130,16 @@
           <t>日本</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr"/>
-      <c r="E8" s="9" t="inlineStr"/>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>『FFVIIリメイク』3部作が話題継続。3部作第2弾のマルチプラットフォーム対応拡大が意識される。</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>FFVIIリメイク3部作 第2弾をSwitch 2/Xbox Series X|S/Windowsにも対応拡大の見込み。</t>
+        </is>
+      </c>
       <c r="F8" s="9" t="inlineStr"/>
       <c r="G8" s="9" t="inlineStr">
         <is>
@@ -28139,7 +28147,11 @@
         </is>
       </c>
       <c r="H8" s="9" t="inlineStr"/>
-      <c r="I8" s="9" t="inlineStr"/>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
@@ -28159,12 +28171,12 @@
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>『ドラクエ12』の最新情報を6月に公開も発売時期は未定で続報待ち。『ドラゴンクエストX オンライン』Ver8『時空の迷い子たち』を6/25実装予定。</t>
+          <t>スクエニが2027年3月以降の大型タイトル定期発売方針を継続表明。</t>
         </is>
       </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>DQ12(時期未定)、DQXオンライン Ver8(2026/6/25)</t>
+          <t>『ドラゴンクエストXII』が2027年3月以降の大型タイトル群に含まれる可能性が取り沙汰される。</t>
         </is>
       </c>
       <c r="F9" s="9" t="inlineStr"/>
@@ -28176,7 +28188,7 @@
       <c r="H9" s="9" t="inlineStr"/>
       <c r="I9" s="9" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>
@@ -28379,8 +28391,16 @@
           <t>日本</t>
         </is>
       </c>
-      <c r="D15" s="9" t="inlineStr"/>
-      <c r="E15" s="9" t="inlineStr"/>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>KONAMIが新作ラインアップでMGSブランドの展開を強化。</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>8月に『METAL GEAR SOLID: MASTER COLLECTION Vol.2』をグローバル発売予定。</t>
+        </is>
+      </c>
       <c r="F15" s="9" t="inlineStr"/>
       <c r="G15" s="9" t="inlineStr">
         <is>
@@ -28388,7 +28408,11 @@
         </is>
       </c>
       <c r="H15" s="9" t="inlineStr"/>
-      <c r="I15" s="9" t="inlineStr"/>
+      <c r="I15" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
@@ -28406,8 +28430,16 @@
           <t>日本</t>
         </is>
       </c>
-      <c r="D16" s="9" t="inlineStr"/>
-      <c r="E16" s="9" t="inlineStr"/>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>『実況パワフルプロ野球2026-2027』を国内展開。Switch/PS4向け。</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>パワプロ2026-2027の継続アップデート、Switch 2向け展開も視野。</t>
+        </is>
+      </c>
       <c r="F16" s="9" t="inlineStr"/>
       <c r="G16" s="9" t="inlineStr">
         <is>
@@ -28415,7 +28447,11 @@
         </is>
       </c>
       <c r="H16" s="9" t="inlineStr"/>
-      <c r="I16" s="9" t="inlineStr"/>
+      <c r="I16" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
@@ -28435,12 +28471,12 @@
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>2026/6/8のXbox Games Showcaseで『ペルソナ6』を正式発表(PS5/Xbox/PC、Game Pass初日対応)。シリーズ30周年。</t>
+          <t>『ペルソナ5X』は今夏展開で概ね想定通りに推移。</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>ペルソナ6(時期未定)、ペルソナ4 Revival</t>
+          <t>『ペルソナ4 リバイバル』を2027年3月期に投入予定(PS5/Xbox/Win/Steam、Game Pass対応)。</t>
         </is>
       </c>
       <c r="F17" s="9" t="inlineStr"/>
@@ -28452,7 +28488,7 @@
       <c r="H17" s="9" t="inlineStr"/>
       <c r="I17" s="9" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>
@@ -28499,8 +28535,16 @@
           <t>日本</t>
         </is>
       </c>
-      <c r="D19" s="9" t="inlineStr"/>
-      <c r="E19" s="9" t="inlineStr"/>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>『龍が如く 極3』『龍が如く3外伝 Dark Ties』が2026/2/12発売済。</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>新作『STRANGER THAN HEAVEN』を2027年3月期に投入予定。</t>
+        </is>
+      </c>
       <c r="F19" s="9" t="inlineStr"/>
       <c r="G19" s="9" t="inlineStr">
         <is>
@@ -28508,7 +28552,11 @@
         </is>
       </c>
       <c r="H19" s="9" t="inlineStr"/>
-      <c r="I19" s="9" t="inlineStr"/>
+      <c r="I19" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
@@ -28526,8 +28574,16 @@
           <t>日本</t>
         </is>
       </c>
-      <c r="D20" s="9" t="inlineStr"/>
-      <c r="E20" s="9" t="inlineStr"/>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>『ソニックランブル』(2025/11グローバル配信)や映像展開でIP伸長。</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>ゲーム・映像のクロスメディア展開を継続。</t>
+        </is>
+      </c>
       <c r="F20" s="9" t="inlineStr"/>
       <c r="G20" s="9" t="inlineStr">
         <is>
@@ -28535,7 +28591,11 @@
         </is>
       </c>
       <c r="H20" s="9" t="inlineStr"/>
-      <c r="I20" s="9" t="inlineStr"/>
+      <c r="I20" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
@@ -28673,8 +28733,16 @@
           <t>日本</t>
         </is>
       </c>
-      <c r="D25" s="9" t="inlineStr"/>
-      <c r="E25" s="9" t="inlineStr"/>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>『仁王3』がシリーズ最速で全世界累計100万本達成、シリーズ累計1000万本突破。</t>
+        </is>
+      </c>
+      <c r="E25" s="9" t="inlineStr">
+        <is>
+          <t>『仁王3』の追加コンテンツ/継続販売に注力。</t>
+        </is>
+      </c>
       <c r="F25" s="9" t="inlineStr"/>
       <c r="G25" s="9" t="inlineStr">
         <is>
@@ -28682,7 +28750,11 @@
         </is>
       </c>
       <c r="H25" s="9" t="inlineStr"/>
-      <c r="I25" s="9" t="inlineStr"/>
+      <c r="I25" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
@@ -28727,8 +28799,16 @@
           <t>日本</t>
         </is>
       </c>
-      <c r="D27" s="9" t="inlineStr"/>
-      <c r="E27" s="9" t="inlineStr"/>
+      <c r="D27" s="9" t="inlineStr">
+        <is>
+          <t>『モンスト』はMAU減少が続き、mixiのデジタルエンタメ事業は減益要因に。</t>
+        </is>
+      </c>
+      <c r="E27" s="9" t="inlineStr">
+        <is>
+          <t>IPコラボ・周年施策でのMAU底打ちを模索。</t>
+        </is>
+      </c>
       <c r="F27" s="9" t="inlineStr"/>
       <c r="G27" s="9" t="inlineStr">
         <is>
@@ -28736,7 +28816,11 @@
         </is>
       </c>
       <c r="H27" s="9" t="inlineStr"/>
-      <c r="I27" s="9" t="inlineStr"/>
+      <c r="I27" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
@@ -28756,12 +28840,12 @@
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>6/21に『ウマ娘』韓国語版が配信開始しApp Storeセールス首位を獲得、CyberAgent株反発の材料に。英語版の海外ヒットに続きグローバル展開が加速。</t>
+          <t>英語版『ウマ娘』が海外でヒットし、サイバーエージェントの業績を牽引。</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>韓国版6/21配信・セルラン1位。英語版好調に続く多言語グローバル展開を推進。</t>
+          <t>海外展開の継続拡大とアップデート施策。</t>
         </is>
       </c>
       <c r="F28" s="9" t="inlineStr"/>
@@ -28773,7 +28857,7 @@
       <c r="H28" s="9" t="inlineStr"/>
       <c r="I28" s="9" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>
@@ -28795,12 +28879,12 @@
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>6/25午前0時にGTA6予約開始、発売日11/19を確定。標準版$79.99・アルティメット版$99.99(限定車両/アパレル同梱)。価格巡り一部失望も予約は活況。</t>
+          <t>最重要作として市場の注目を一身に集める。発売日は据え置きを維持。</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>Grand Theft Auto VI: 2026/11/19発売(PS5/Xbox Series X|S)。初年度6,000〜7,000万本予測。</t>
+          <t>『Grand Theft Auto VI』は2026年11月19日にPS5/Xbox Series X|Sで発売予定。</t>
         </is>
       </c>
       <c r="F29" s="9" t="inlineStr"/>
@@ -28812,7 +28896,7 @@
       <c r="H29" s="9" t="inlineStr"/>
       <c r="I29" s="9" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>
@@ -29143,12 +29227,12 @@
       </c>
       <c r="D41" s="9" t="inlineStr">
         <is>
-          <t>『Battlefield 6』がシリーズ最高の年となりEAのFY26 Net Bookings過去最高($8,026m,+9%)を牽引。ライブサービス運営を強化。</t>
+          <t>『Battlefield 6』が10月発売以降1,000万本超を販売、2025年ベストセラーに。</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
         <is>
-          <t>Battlefield 6のライブ運営継続</t>
+          <t>ライブサービスとしての継続コンテンツ供給を強化。</t>
         </is>
       </c>
       <c r="F41" s="9" t="inlineStr"/>
@@ -29160,7 +29244,7 @@
       <c r="H41" s="9" t="inlineStr"/>
       <c r="I41" s="9" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>
@@ -29444,8 +29528,16 @@
           <t>海外/韓国</t>
         </is>
       </c>
-      <c r="D50" s="9" t="inlineStr"/>
-      <c r="E50" s="9" t="inlineStr"/>
+      <c r="D50" s="9" t="inlineStr">
+        <is>
+          <t>KraftonがPUBG依存低減の『Franchise IP』戦略へ転換。PUBG Mobileは引き続き主力収益。</t>
+        </is>
+      </c>
+      <c r="E50" s="9" t="inlineStr">
+        <is>
+          <t>新規IP群(Subnautica 2等)投入でポートフォリオ多様化。</t>
+        </is>
+      </c>
       <c r="F50" s="9" t="inlineStr"/>
       <c r="G50" s="9" t="inlineStr">
         <is>
@@ -29453,7 +29545,11 @@
         </is>
       </c>
       <c r="H50" s="9" t="inlineStr"/>
-      <c r="I50" s="9" t="inlineStr"/>
+      <c r="I50" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="9" t="inlineStr">
@@ -29554,12 +29650,12 @@
       </c>
       <c r="D54" s="9" t="inlineStr">
         <is>
-          <t>6/18時点でエンゲージメントが3週連続改善。『Roblox Kids』『Roblox Select』アカウントを世界展開し年齢別の安全設計を強化。</t>
+          <t>Q1 2026は売上が予想未達、安全対策強化で通期ガイダンスを下方修正。株価は6か月で約-51%。</t>
         </is>
       </c>
       <c r="E54" s="9" t="inlineStr">
         <is>
-          <t>年齢別アカウント・安全機能の拡充</t>
+          <t>未成年保護機能の拡充と広告・課金の収益化施策を継続。</t>
         </is>
       </c>
       <c r="F54" s="9" t="inlineStr"/>
@@ -29571,7 +29667,7 @@
       <c r="H54" s="9" t="inlineStr"/>
       <c r="I54" s="9" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>
@@ -29860,7 +29956,7 @@
       </c>
       <c r="M2" s="9" t="inlineStr">
         <is>
-          <t>6/26に第86期定時株主総会を開催。株価は7,000円前後で軟調が続き、年初来安値6,849円圏に接近（6/28時点予想7,430円、当日レンジ約7,005〜7,359円）。過去1年では約-45%と大幅安。FY26はSwitch 2立ち上げで売上2.313兆円(+98.6%)・営業益3,601億円(+27.5%)規模と急回復も、年末商戦と端末普及ペースを見極める材料待ち局面。</t>
+          <t>7/3に年初来安値6,544円をつけ株価軟調が継続。メモリなど部材急騰観測と先行き不透明感で過去5か月で30%超下落。FY26はSwitch 2立ち上げで売上2.313兆円(+98.6%)・営業益3,601億円(+27.5%)と急回復済だが、年末商戦とハード普及ペース、部材コスト増を見極める材料待ちの調整局面。</t>
         </is>
       </c>
       <c r="N2" s="9" t="inlineStr">
@@ -29870,17 +29966,17 @@
       </c>
       <c r="O2" s="9" t="inlineStr">
         <is>
-          <t>端末移行期の費用増・ハード普及ペース不透明</t>
+          <t>メモリ等部材急騰によるコスト増懸念、ハード普及ペース不透明、株価の下値模索</t>
         </is>
       </c>
       <c r="P2" s="9" t="inlineStr">
         <is>
-          <t>Switch 2普及とファーストパーティ大型タイトル供給</t>
+          <t>Switch 2普及ペースとファーストパーティ大型タイトル供給、部材コスト管理</t>
         </is>
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>
@@ -29915,12 +30011,12 @@
       </c>
       <c r="M3" s="9" t="inlineStr">
         <is>
-          <t>PS5はサイクル後半で販売鈍化（直近四半期約800万台・前年比-15%）。メモリ価格高騰でハード採算悪化懸念が重しとなり株価は下落基調（ピークから2割超安）。一方ゲーム・音楽・映画のエンタメ基盤は底堅く本業は崩れていないとの見方。次世代機戦略とライブサービス立て直しが焦点。</t>
+          <t>7/2にG&amp;NS期待などから株価一時+4.6%高。PS新作の『ディスク版販売終了』報道が話題。GTAⅥ(11/19)がPS5/Xboxのみ対応となる見込みで、PS Plusなどネットワークサービス収入の増加期待が改めて意識される。FY25は全社売上・営業益とも過去最高を更新済み。</t>
         </is>
       </c>
       <c r="N3" s="9" t="inlineStr">
         <is>
-          <t>PS5インストールベースとネットワーク課金、IP・映像横展開</t>
+          <t>GTAⅥ効果でのPS5エンゲージメント/ネットワーク収入期待、全社最高業績</t>
         </is>
       </c>
       <c r="O3" s="9" t="inlineStr">
@@ -29930,12 +30026,12 @@
       </c>
       <c r="P3" s="9" t="inlineStr">
         <is>
-          <t>次世代機戦略・Bungie等スタジオの新作と live service立て直し</t>
+          <t>GTAⅥ商戦でのPS5牽引、ゲーム&amp;ネットワークサービスの収益拡大</t>
         </is>
       </c>
       <c r="Q3" s="9" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>
@@ -29970,12 +30066,12 @@
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>『鬼武者 Way of the Sword』(9/25)体験版が好評。先週発表のMHワイルズ大型拡張『Ascendance』・バイオ新作(2027)期待を背景に、6月中旬に株価は一時+5%の3,031円。13期連続増収増益のIP基盤は不変で、2027年の大型パイプラインとSwitch 2展開が評価軸。今週は新規材料に乏しく高値圏もみ合い。</t>
+          <t>7/2に適時開示、期待の新作『鬼武者 Way of the Sword』の発売日を9月4日へ前倒しと発表。FY26通期は13期連続営業増益・売上/営業益とも過去最高で好調継続。強力IPのリピート販売とデジタル比率上昇が寄与。</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>モンハン/バイオ/SF6の強力IPと10期連続最高益、Switch 2展開で裾野拡大</t>
+          <t>『鬼武者』新作前倒しで年内販売寄与、13期連続営業増益の収益体質</t>
         </is>
       </c>
       <c r="O4" s="9" t="inlineStr">
@@ -29985,12 +30081,12 @@
       </c>
       <c r="P4" s="9" t="inlineStr">
         <is>
-          <t>MH Wilds拡張・新規プラットフォーム展開・カタログ販売</t>
+          <t>『鬼武者 Way of the Sword』(9/4)の初動、主力IPの継続的なリピート販売</t>
         </is>
       </c>
       <c r="Q4" s="9" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>
@@ -30037,12 +30133,12 @@
       </c>
       <c r="M5" s="9" t="inlineStr">
         <is>
-          <t>6/26終値約2,340円(-0.95%)。5/27公開の『ドラクエ12』が発売時期未定で失望売りした流れが尾を引く。『ドラゴンクエストX オンライン』Ver8を6/25実装。FY26は新作減で減収も不採算整理で営業益+34.9%と収益性改善。FF7リメイク三部作・HD-2D系の進捗と海外展開が引き続き焦点。</t>
+          <t>『FFVIIリメイク』3部作第2弾がSwitch 2/Xbox Series X|S/Windowsにも対応拡大の見込み。2027年3月以降は大型タイトルを定期発売する方針を継続表明し、『ドラゴンクエストXII』が含まれる可能性も取り沙汰される。FY26は減収増益。</t>
         </is>
       </c>
       <c r="N5" s="9" t="inlineStr">
         <is>
-          <t>不採算整理による収益性改善、FF/DQ等基幹IP</t>
+          <t>マルチプラットフォーム展開の拡大、大型IPの定期供給方針</t>
         </is>
       </c>
       <c r="O5" s="9" t="inlineStr">
@@ -30052,12 +30148,12 @@
       </c>
       <c r="P5" s="9" t="inlineStr">
         <is>
-          <t>マルチプラットフォーム戦略と次期大型タイトルの成否</t>
+          <t>FFVIIリメイク第2弾のマルチ展開、DQ新作など大型タイトルの発売時期</t>
         </is>
       </c>
       <c r="Q5" s="9" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>
@@ -30104,12 +30200,12 @@
       </c>
       <c r="M6" s="9" t="inlineStr">
         <is>
-          <t>FY26はデジタルエンタメ主導で2四半期連続最高益更新（Q3累計 売上3,530億・営業益1,017億, +17.4%）。eFootball・遊戯王のグローバル課金が牽引。株価は1.9万円台で堅調。MGS・パワプロ等IP活用とスポーツ・ジム事業の複合成長が継続テーマ。今週は新規開示乏しく高値圏を維持。</t>
+          <t>新作ラインアップを公開し過去人気IP復活やスポーツタイトルでSwitch 2向けを積極化。『パワフルプロ野球2026-2027』を展開、8月には『METAL GEAR SOLID: MASTER COLLECTION Vol.2』をグローバル発売予定。デジタル・スポーツIPが業績を下支え。</t>
         </is>
       </c>
       <c r="N6" s="9" t="inlineStr">
         <is>
-          <t>デジタルエンタメ高成長と3期連続最高益、安定したIP課金</t>
+          <t>パワプロ/MGS等の強力IPパイプライン、Switch 2向け積極展開</t>
         </is>
       </c>
       <c r="O6" s="9" t="inlineStr">
@@ -30119,12 +30215,12 @@
       </c>
       <c r="P6" s="9" t="inlineStr">
         <is>
-          <t>遊戯王・eFootballのグローバル課金とスポーツ事業</t>
+          <t>MGS Master Collection Vol.2(8月)の反応、Switch 2向け新作の立ち上がり</t>
         </is>
       </c>
       <c r="Q6" s="9" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>
@@ -30171,12 +30267,12 @@
       </c>
       <c r="M7" s="9" t="inlineStr">
         <is>
-          <t>FY26は売上1兆3,482億・営業益1,895億と過去最高。ガンダムIP売上が約7割増と牽引。State of Playで『ACE COMBAT 8』を10/2 PS5発売と告知済み。6/22株価は約3,644円(+1.48%)。ガンダム/エルデンリング/アイマス等のIPを多面展開する戦略が強み。今週は新作投入ペースが評価軸。</t>
+          <t>FY26は『機動戦士ガンダム』シリーズ牽引で売上・全利益項目が過去最高を更新済み。IP軸(ガンダム/ドラゴンボール等)のグローバル展開とトイホビー好調が継続。大きな新規開示は乏しく、好業績の持続力を見極める局面。</t>
         </is>
       </c>
       <c r="N7" s="9" t="inlineStr">
         <is>
-          <t>IP軸トイホビー＋ゲームの複合収益、過去最高業績</t>
+          <t>ガンダム等主力IPの世界的伸長、全利益項目で過去最高更新</t>
         </is>
       </c>
       <c r="O7" s="9" t="inlineStr">
@@ -30186,12 +30282,12 @@
       </c>
       <c r="P7" s="9" t="inlineStr">
         <is>
-          <t>ガンダム/アイマス等IPの世界展開と新作投入ペース</t>
+          <t>IP軸戦略の持続力、家庭用新作とトイホビーの両輪</t>
         </is>
       </c>
       <c r="Q7" s="9" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>
@@ -30226,27 +30322,27 @@
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>6/26株価約2,140円(-0.14%)。FY26はRovio等の減損で最終赤字も、売上4,875億(+13.7%)・営業益471億(-2.1%)。大型『Super Game』構想中止後はペルソナ/龍が如く/ソニック等の既存グローバルIP収益化と海外子会社立て直しが課題。ペルソナ6を含む新作パイプラインが鍵。</t>
+          <t>2027年3月期に主力4本(『STRANGER THAN HEAVEN』『ペルソナ4 リバイバル』＋主要IP新作2本)を投入する計画。『ペルソナ5X』は今夏展開で概ね想定通り。FY26のセガ(エンタメ)営業益は新作の遅れ等で大幅減益だった反動から、次期の大型タイトル集中に期待。</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>ペルソナ/龍が如く/ソニック等グローバルIP、ペルソナ30周年</t>
+          <t>『ペルソナ』『龍が如く』等の強力IP、2027年3月期の大型新作4本計画</t>
         </is>
       </c>
       <c r="O8" s="9" t="inlineStr">
         <is>
-          <t>遊技機原価高・ゲーミング先行投資で減益計画</t>
+          <t>新作リリース遅延・一部タイトルの想定下振れ、エンタメ営業益の変動</t>
         </is>
       </c>
       <c r="P8" s="9" t="inlineStr">
         <is>
-          <t>ペルソナ6を含む新作パイプラインと海外展開</t>
+          <t>『STRANGER THAN HEAVEN』『ペルソナ4リバイバル』等の投入と初動</t>
         </is>
       </c>
       <c r="Q8" s="9" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>
@@ -30293,27 +30389,27 @@
       </c>
       <c r="M9" s="9" t="inlineStr">
         <is>
-          <t>FY26は『仁王3』『ゼルダ無双 封印戦記』等が寄与し売上825億(+5.7%)・営業益366億(+16.4%)と増益、高営業利益率と財テク収益が特徴。『信長の野望』『三國志』の周年・協業施策が継続テーマ。今週は新規開示乏しいが、次期は投資増で減益計画の点に留意。</t>
+          <t>『仁王3』がシリーズ最速で全世界累計100万本を達成し、シリーズ累計は1000万本を突破。コンソール新作は好調だがモバイル減速と先行投資で足元は減収減益。第4四半期に大型タイトルが集中し挽回を図る構図。</t>
         </is>
       </c>
       <c r="N9" s="9" t="inlineStr">
         <is>
-          <t>無双/三國志等IPと高い営業利益率、過去最高更新</t>
+          <t>『仁王3』ヒットとアクションIPの海外評価、コンソール新作好調</t>
         </is>
       </c>
       <c r="O9" s="9" t="inlineStr">
         <is>
-          <t>次期は投資増で大幅減益計画、市場予想未達</t>
+          <t>モバイル事業の減速、先行投資による利益圧迫</t>
         </is>
       </c>
       <c r="P9" s="9" t="inlineStr">
         <is>
-          <t>新作投入サイクルと海外/IPコラボ展開</t>
+          <t>『仁王3』の販売継続と大型コンソール新作の寄与</t>
         </is>
       </c>
       <c r="Q9" s="9" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>
@@ -30356,7 +30452,7 @@
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>FY26は売上1,713.7億(+10.7%)も営業益222.6億(-16.3%)と減益。Q3累計では営業益-22.7%。公営競技等スポーツ事業が成長する一方、主力モンストのデジタルエンタメ減収と費用増が利益を圧迫。今週は新規開示乏しく、新規事業の収益化とモンスト次施策が焦点。</t>
+          <t>FY26は売上1,713.69億円(+10.7%)も営業益222.56億円(-16.3%)と減益。主力『モンスターストライク』のMAU減少とアニメ等広告宣伝費が重し。スポーツ(千葉ジェッツ/TIPSTAR)は黒字化。PointsBet連結化で事業ポートフォリオ多角化を進める。株価は6/末2,685円前後。</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
@@ -30366,17 +30462,17 @@
       </c>
       <c r="O10" s="9" t="inlineStr">
         <is>
-          <t>モンストMAU減で中核ゲーム収益が縮小</t>
+          <t>『モンスト』MAU減少による中核収益の鈍化、広告宣伝費増</t>
         </is>
       </c>
       <c r="P10" s="9" t="inlineStr">
         <is>
-          <t>スポーツ事業の収益化とモンスト再活性化</t>
+          <t>『モンスト』の底打ち、スポーツ・投資事業の収益貢献拡大</t>
         </is>
       </c>
       <c r="Q10" s="9" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>
@@ -30411,7 +30507,7 @@
       </c>
       <c r="M11" s="9" t="inlineStr">
         <is>
-          <t>DeNAと共に株価が連騰し、一時2,800円台と2017年11月以来の水準を回復。『ポケポケ(Pokémon TCG Pocket)』のテーマ拡張等が材料視。釣りスタ・REALITY等の既存事業に加え、任天堂系協業IPと新規育成が継続テーマ。今週はゲーム外の多角化進捗が注目点。</t>
+          <t>大きな新規適時開示は限定的。既存タイトル運営とメタバース『REALITY』、投資事業を軸に事業構造転換を継続。ゲーム単体の新規モメンタムは乏しく、コスト管理と新規事業の育成が焦点。</t>
         </is>
       </c>
       <c r="N11" s="9" t="inlineStr">
@@ -30426,12 +30522,12 @@
       </c>
       <c r="P11" s="9" t="inlineStr">
         <is>
-          <t>新規ゲーム/メタバース・Wright Flyer系の収益化</t>
+          <t>新規タイトル/新規事業の育成、コスト構造の最適化</t>
         </is>
       </c>
       <c r="Q11" s="9" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>
@@ -30474,12 +30570,12 @@
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>株価は5日続伸し一時2,800円台と2017年11月以来の高値圏を回復。『ポケポケ』のテーマ拡張パック追加が好感された。横浜DeNAベイスターズ、ライブ配信Pococha、ヘルスケア/AI領域が事業の軸。ゲーム新作パイプラインと非ゲーム事業の収益化が引き続き注目。</t>
+          <t>『Pokémon Trading Card Game Pocket(ポケポケ)』の収益インパクトが引き続き注目。ゲーム事業に加えヘルスケア・スポーツ(横浜DeNAベイスターズ)を展開。大型の新規開示は乏しく、ポケポケの収益持続性が業績のカギ。</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>ポケポケ等任天堂系IP、ライブ配信の黒字化、事業多角化</t>
+          <t>『ポケポケ』の高収益、球団など多角的な事業ポートフォリオ</t>
         </is>
       </c>
       <c r="O12" s="9" t="inlineStr">
@@ -30489,12 +30585,12 @@
       </c>
       <c r="P12" s="9" t="inlineStr">
         <is>
-          <t>新規タイトル投入とヘルスケア/スポーツ事業の収益化</t>
+          <t>『ポケポケ』の収益持続、ライブサービス運営の安定化</t>
         </is>
       </c>
       <c r="Q12" s="9" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>
@@ -30529,12 +30625,12 @@
       </c>
       <c r="M13" s="9" t="inlineStr">
         <is>
-          <t>6月下旬株価約1,329円(年初来安値1,204円圏から戻り)。6/21に子会社Cygamesの『ウマ娘』韓国語版が配信開始しApp Storeセールス首位を獲得、株価反発の材料に。FY26 2Qはゲーム事業 売上1,322億(+47.4%)・営業益386億(+106%)と急伸。AI・広告とウマ娘グローバル展開が成長ドライバー。</t>
+          <t>英語版『ウマ娘』のヒットで海外展開が加速し、10〜3月は純利益72%増、ゲーム事業は増収増益。7/9に自社IP『グランブルーファンタジー リリンク：エンドレスラグナロク』の発売を控える。ゲーム/メディア/AI・広告の各事業が業績を牽引。</t>
         </is>
       </c>
       <c r="N13" s="9" t="inlineStr">
         <is>
-          <t>ウマ娘英語版の海外ヒット、AI・広告事業の成長</t>
+          <t>英語版『ウマ娘』の海外ヒット、グラブル新作など自社IP強化</t>
         </is>
       </c>
       <c r="O13" s="9" t="inlineStr">
@@ -30544,12 +30640,12 @@
       </c>
       <c r="P13" s="9" t="inlineStr">
         <is>
-          <t>ウマ娘グローバル展開と新作・AI事業の収益貢献</t>
+          <t>『ウマ娘』海外定着とグラブル リリンク新作、AI広告事業の成長</t>
         </is>
       </c>
       <c r="Q13" s="9" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>
@@ -30697,7 +30793,7 @@
       </c>
       <c r="L2" s="9" t="inlineStr">
         <is>
-          <t>8/1から全世界でXbox本体を値上げ（512GB +$100/1TB +$150）、2TBモデルは販売終了と発表。メモリ/ストレージ価格が2.5倍超に高騰したのが背景。Stifelの目標株価引き下げと値上げ嫌気で6/25に株価-3.8〜4.5%。Xboxはハード収益-33%でマージン圧迫、約1,000名の追加レイオフ計画。Game Pass最適化とCoD/Bethesda供給が軸。</t>
+          <t>Xbox部門が新CEO Asha Sharma体制で大規模『reset』に着手。6/30の会計年度末後(7月)に大規模レイオフ(業界推計~1,000人規模)を実施見込みで、Double Fine/Undead Labs/Compulsion/Ninja Theory等のスタジオ再編・閉鎖の可能性も。Activision除くと5年で年間約$500M収益減が背景。</t>
         </is>
       </c>
       <c r="M2" s="9" t="inlineStr">
@@ -30707,17 +30803,17 @@
       </c>
       <c r="N2" s="9" t="inlineStr">
         <is>
-          <t>Xboxハード収益-33%・連続レイオフ・本体値上げによる需要減リスク</t>
+          <t>Xbox大規模レイオフ・スタジオ再編、ハード事業の収益悪化</t>
         </is>
       </c>
       <c r="O2" s="9" t="inlineStr">
         <is>
-          <t>新CEO Sharma体制での収益性改善とGame Pass最適化</t>
+          <t>『reset』後のファーストパーティ体制、GTAⅥ商戦・Game Passの立て直し</t>
         </is>
       </c>
       <c r="P2" s="9" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>
@@ -30755,12 +30851,12 @@
       </c>
       <c r="L3" s="9" t="inlineStr">
         <is>
-          <t>GTA6予約が6/25午前0時に開始、発売日11/19を確定。標準版$79.99・アルティメット版$99.99。価格巡り一部失望売りも、6/28株価は約$239(レンジ$233〜242)。BofAは買い・目標$368、MorningstarはFY27販売6,000〜7,000万本予測。11/19発売実現が史上最高業績の最大の鍵。</t>
+          <t>最重要作『Grand Theft Auto VI』は2026年11月19日(PS5/Xbox)発売の据え置きを維持。延期後もライブサービス依存が薄い株として相対評価は良好。GTAⅥ発売を控え、期待先行の株価と発売遅延リスクが綱引き。</t>
         </is>
       </c>
       <c r="M3" s="9" t="inlineStr">
         <is>
-          <t>GTA6発売を控えた史上最大級の収益拡大期待</t>
+          <t>GTAⅥ発売期待、Rockstar/2K/NBA 2Kの強力IP群</t>
         </is>
       </c>
       <c r="N3" s="9" t="inlineStr">
@@ -30770,12 +30866,12 @@
       </c>
       <c r="O3" s="9" t="inlineStr">
         <is>
-          <t>GTA6の11/19発売実現と初年度販売</t>
+          <t>GTAⅥ(11/19)の発売実現と初動規模、遅延リスクの解消</t>
         </is>
       </c>
       <c r="P3" s="9" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>
@@ -30813,12 +30909,12 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>PIF/Silver Lake/Affinity主導の$55bn($210/株)take-privateは6/30クローズ目標だが、CFIUS審査が長引きアウトサイドデートは9/28に。データガバナンス（サウジPIFの関与）が規制上の焦点で、6/30完了は不透明に。FY26はBattlefield 6が牽引しNet Bookings $8.03bn(+9%)と過去最高。</t>
+          <t>『Battlefield 6』が10月発売以降1,000万本超を販売し2025年ベストセラーに。GTAⅥ延期の間隙を突いた戦略が奏功。EA SPORTS FC等ライブサービスと合わせ収益基盤は堅調で、フランチャイズ再興が評価される局面。</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>Battlefield 6の回復とNet Bookings過去最高、$210での非公開化(LBO)プレミアム</t>
+          <t>『Battlefield 6』1,000万本超の大ヒット、EA SPORTS FC等の安定収益</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
@@ -30828,12 +30924,12 @@
       </c>
       <c r="O4" s="9" t="inlineStr">
         <is>
-          <t>CFIUSクリアランス取得とディール完了時期</t>
+          <t>Battlefieldライブサービス化の定着、次期スポーツタイトルの更新需要</t>
         </is>
       </c>
       <c r="P4" s="9" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>
@@ -30867,7 +30963,7 @@
       </c>
       <c r="L5" s="9" t="inlineStr">
         <is>
-          <t>共同創業者Claude Guillemot氏が6/20に仏での航空機事故で死去と報道。FY26は営業損失€1.3bn・Net Bookings €1.5bn(-17.4%)。再編で7本中止・6本延期、2028/3までに€2億超のコスト削減を追加。Tencent出資の専門子会社(Vantage)による主要IP切り出しが進行。アナリスト平均は『中立』、目標€5.60。</t>
+          <t>直近開示で純損失€1,475.2m/売上€1,395.7mと依然赤字、資金は外部借入依存で株価は仏エンタメ指数に劣後。Tencent出資の新子会社への主力IP切り出しなど再建策の進捗が焦点。</t>
         </is>
       </c>
       <c r="M5" s="9" t="inlineStr">
@@ -30877,17 +30973,17 @@
       </c>
       <c r="N5" s="9" t="inlineStr">
         <is>
-          <t>共同創業者の急逝・大幅赤字・度重なる再編で先行き不透明</t>
+          <t>継続赤字と借入依存、株価の低迷、主力IPパイプラインの遅延</t>
         </is>
       </c>
       <c r="O5" s="9" t="inlineStr">
         <is>
-          <t>Q4のGAAP黒字化達成と広告プラットフォーム成長</t>
+          <t>Assassin's Creed等主力IPの立て直し、新子会社を通じた再建策の実行</t>
         </is>
       </c>
       <c r="P5" s="9" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>
@@ -30921,12 +31017,12 @@
       </c>
       <c r="L6" s="9" t="inlineStr">
         <is>
-          <t>8月の取締役会で中間決算・配当を審議予定と発表。ゲームとAI需要が業績を押し上げとの観測。Honor of Kings/PUBG Mobile等の海外展開とRiot/Epic出資網が強み。Nexon買収観測は改めて否定。今週は大きな新規開示は限定的で、AIエージェント収益化と中間期業績が次の焦点。</t>
+          <t>世界最大のゲーム企業として、ゲーム部門へのAI統合と海外展開が投資家の焦点。一部日本スタジオ保有株を損失覚悟でも売却する方向で交渉との報道。PUBG MobileやHonor of Kings等が引き続き稼ぎ頭。2026年は新作ローンチが堅調と目される。</t>
         </is>
       </c>
       <c r="M6" s="9" t="inlineStr">
         <is>
-          <t>国内外ゲームの安定課金とAIによる広告・効率化、Riot/Epic等出資網</t>
+          <t>AI×ゲーム統合、Honor of Kings/PUBG Mobile等の巨大収益基盤</t>
         </is>
       </c>
       <c r="N6" s="9" t="inlineStr">
@@ -30936,12 +31032,12 @@
       </c>
       <c r="O6" s="9" t="inlineStr">
         <is>
-          <t>AIエージェント収益化と海外スタジオ(Vantage等)の成果</t>
+          <t>国内外の新作パイプライン、投資ポートフォリオ再編とAI収益化</t>
         </is>
       </c>
       <c r="P6" s="9" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>
@@ -30975,12 +31071,12 @@
       </c>
       <c r="L7" s="9" t="inlineStr">
         <is>
-          <t>6/25に香港取引所への二次上場(dual primary listing)を6/30付で発表、アジア投資家層の拡大を狙う。『Marvel Rivals』はシーズン8.5を配信しeスポーツも本格化。高粗利のゲーム課金と強力な新作パイプラインが成長軸。AI部門縮小報道は否定。Ananta等AAA級新作のグローバル成否が鍵。</t>
+          <t>2026年はTencentと並び新作ローンチが堅調と市場は評価。Identity V/荒野行動などライブサービスとグローバル向け新規IP投入が成長ドライバー。大きな新規開示は限定的で、次の四半期決算と新作の立ち上がり待ち。</t>
         </is>
       </c>
       <c r="M7" s="9" t="inlineStr">
         <is>
-          <t>高粗利ゲーム課金・Marvel Rivals好調・香港二次上場で投資家層拡大</t>
+          <t>多数の自社開発IPとグローバル展開、堅調な新作パイプライン</t>
         </is>
       </c>
       <c r="N7" s="9" t="inlineStr">
@@ -30990,12 +31086,12 @@
       </c>
       <c r="O7" s="9" t="inlineStr">
         <is>
-          <t>AnantaなどAAA級新作のグローバル成否</t>
+          <t>新規IPの海外定着、モバイル/PCマルチ展開の収益化</t>
         </is>
       </c>
       <c r="P7" s="9" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>
@@ -31029,12 +31125,12 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>6/25株価約₩134,69x水準・時価総額約$6.07bn。早期アクセスの『Subnautica 2』は5日で400万本・売上$120M。好調ゆえ旧Unknown Worlds株主への最大$250Mアーンアウト支払い義務が発生（係争中）。Q1営業益約$373MでNexonを抜き韓国ゲーム首位を奪還。新規IPとAIファースト戦略が評価軸。</t>
+          <t>単一タイトル依存を減らす『Franchise IP』戦略に転換。CEO CH Kimが2年内リリースの26プロジェクト(『Subnautica 2』『Palworld Mobile』など12作)を提示。Hanwha AerospaceとフィジカルAI開発で提携するなど事業領域を拡張。</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>PUBG依存脱却・Subnautica 2大ヒット・Q1で韓国首位奪還</t>
+          <t>PUBG基盤＋『Franchise IP』戦略による新規IP拡充、豊富なパイプライン</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
@@ -31044,12 +31140,12 @@
       </c>
       <c r="O8" s="9" t="inlineStr">
         <is>
-          <t>Subnautica 2の本格展開と新規IPの多様化</t>
+          <t>Subnautica 2等新規IPの成功、PUBG以外の収益源多様化</t>
         </is>
       </c>
       <c r="P8" s="9" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>
@@ -31083,12 +31179,12 @@
       </c>
       <c r="L9" s="9" t="inlineStr">
         <is>
-          <t>KraftonがQ1営業益で韓国ゲーム首位を奪還し、Nexonは2位に。Tencentによる買収観測(評価額約$15b)は当事者が否定済み。『メイプルストーリー』『DNF』等の中韓モバイル収益とARC Raidersの新規寄与が業績を下支え。今週は新規開示乏しく、既存IPのライブ運営と新作展開が注目。</t>
+          <t>7/3時点で株価$14.18・時価総額約$11.2B、TTM売上$3.17B。『メイプルストーリー』『Dungeon&amp;Fighter』等ロングラン運営が収益基盤。大型の新規開示は乏しく、中国DnF/モバイルの課金動向が業績を左右する構図。</t>
         </is>
       </c>
       <c r="M9" s="9" t="inlineStr">
         <is>
-          <t>MapleStory/DNFの長寿ライブ運営とARC Raidersの新規寄与</t>
+          <t>MapleStory/DnF等ロングランIPの安定収益、堅実な運営力</t>
         </is>
       </c>
       <c r="N9" s="9" t="inlineStr">
@@ -31098,12 +31194,12 @@
       </c>
       <c r="O9" s="9" t="inlineStr">
         <is>
-          <t>ARC Raiders定着と新規IPのグローバル展開</t>
+          <t>中国DnFモバイルの課金動向、新規タイトルの寄与</t>
         </is>
       </c>
       <c r="P9" s="9" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>
@@ -31137,7 +31233,7 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>二次パブリッシングレーベル『Fellowship Entertainment』を設立し、LotR/Tomb Raider等の主要IPを束ね2027年にスピンオフ予定。Ubisoftの『Vantage』分社に続く『IP主導エンタメ企業』への転換志向。今週は新規開示乏しいが、グループ再編とIP価値最大化が継続テーマ。</t>
+          <t>分社化・事業再編を継続中で、直近の大きな新規開示は限定的。負債圧縮とポートフォリオ整理の進捗、分割後の各社の独立採算化が引き続き市場の関心事。</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
@@ -31147,17 +31243,17 @@
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>大幅減収と赤字、相次ぐ再編で信頼回復途上</t>
+          <t>再編途上の不確実性、負債圧縮の必要性</t>
         </is>
       </c>
       <c r="O10" s="9" t="inlineStr">
         <is>
-          <t>分割後の収益性回復と新CEO選任・2027年の製品群</t>
+          <t>分社化後の各社の独立採算化と収益改善</t>
         </is>
       </c>
       <c r="P10" s="9" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>
@@ -31191,7 +31287,7 @@
       </c>
       <c r="L11" s="9" t="inlineStr">
         <is>
-          <t>6/28株価約$47.45(レンジ$44.7〜47.7)・時価総額約$297億。Citiのエンゲージメント鈍化指摘で週初に-8.3%急落。年齢確認導入を巡る証券訴訟も浮上。一方ARK(Cathie Wood)が下落局面で約49万株を買い増し、ロシアの利用禁止も解除。年齢別アカウント定着と通期ブッキング回復が鍵。年初来-42%。</t>
+          <t>Q1 2026はEPS -$0.35(予想-$0.41を上回る)も売上$1.4Bは予想$1.74Bに未達。安全対策強化を背景に通期ガイダンスを下方修正(売上成長20-25%、ブッキング成長8-12%)。株価は約$56で6か月で-51%と低迷。次回決算は7/30頃の見込み。</t>
         </is>
       </c>
       <c r="M11" s="9" t="inlineStr">
@@ -31201,17 +31297,17 @@
       </c>
       <c r="N11" s="9" t="inlineStr">
         <is>
-          <t>エンゲージメント鈍化懸念・年齢確認巡る証券訴訟・年初来-42%</t>
+          <t>未成年安全対策コスト・規制圧力、ブッキング成長鈍化、株価大幅安</t>
         </is>
       </c>
       <c r="O11" s="9" t="inlineStr">
         <is>
-          <t>年齢別アカウント定着と通期ブッキング回復</t>
+          <t>安全対策と成長の両立、ブッキング再加速と広告収益の伸長</t>
         </is>
       </c>
       <c r="P11" s="9" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>
@@ -31245,12 +31341,12 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>ゲーム/広告/AIクリエイターツールの融合領域でAppLovin・Roblox・Adobeに対する競争ポジションを強化。広告事業(Unity Vector/Grow)の改善とエンジン課金モデルの安定化が株価回復の鍵。今週は目立った新規開示は乏しく、Unity AIの収益貢献と広告シェア回復が引き続き焦点。</t>
+          <t>Q1 2026予備売上$505-508Mでガイダンス($480-490M)を上回る。中国事業を$10億超で売却、ironSource Ads Networkを終了し広告を『Unity Vector』AIプラットフォームへ集約。中国売却観測で株価が一時+10%。AI広告のGrow売上は前年比+48%見込み。</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>広告事業の底打ちとUnity AIによる生産性向上、アナリスト格上げ</t>
+          <t>『Unity Vector』AI広告の急成長、中国事業売却でのバランスシート改善</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
@@ -31260,12 +31356,12 @@
       </c>
       <c r="O12" s="9" t="inlineStr">
         <is>
-          <t>Unity AIの収益貢献と広告プラットフォームのシェア回復</t>
+          <t>Vector広告の収益化加速、エンジン課金モデルの安定化</t>
         </is>
       </c>
       <c r="P12" s="9" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>
@@ -31303,27 +31399,27 @@
       </c>
       <c r="L13" s="9" t="inlineStr">
         <is>
-          <t>AXON AI広告基盤を6月下旬に全世界の広告主へセルフサーブ開放。Q1はEPS・売上が予想を上回りQ2ガイダンスも上振れ、年率+30.4%成長・FCFマージン71.9%。一方CEO・取締役の大量株式売却(6月中旬)が嫌気され6/25に-3.6%。Citiは買い・目標$710。全面開放の実行リスクとマージン維持が焦点。</t>
+          <t>株価は約$390でYTD -42%と、2026年のad-tech全般への逆風で調整。ただしAXON広告エンジンで依然として業界の支配的プレーヤーの地位を維持し高EBITDAマージンを確保。広告需要環境と規制動向が株価の変動要因。</t>
         </is>
       </c>
       <c r="M13" s="9" t="inlineStr">
         <is>
-          <t>AI広告(AXON)の高収益・高成長、S&amp;P500入り</t>
+          <t>AXON広告エンジンの高収益・高マージン、ad-tech内での支配的地位</t>
         </is>
       </c>
       <c r="N13" s="9" t="inlineStr">
         <is>
-          <t>AXON全面開放の実行・希薄化リスクと幹部の大量株式売却</t>
+          <t>ad-techセクター全体への逆風、株価のボラティリティ拡大</t>
         </is>
       </c>
       <c r="O13" s="9" t="inlineStr">
         <is>
-          <t>AXONグローバル開放の成果とeコマース広告の立ち上がり</t>
+          <t>広告需要の回復、eコマース等新領域への広告拡張</t>
         </is>
       </c>
       <c r="P13" s="9" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
daily-news + cross-questions + predictions update (2026-07-07)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -816,7 +816,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1676,6 +1676,43 @@
       <c r="G23" s="14" t="inlineStr">
         <is>
           <t>専門物理版レーベルの新規タイトル契約・提携数の増加、ソニー系IPの物理版が専門レーベル経由へ移行するかを観測</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B24" s="14" t="inlineStr">
+        <is>
+          <t>Xboxが手放したスタジオ（Ninja Theory等）やその熟練人材を、Tencent/NetEase等の中国系やSavvy(サウジ)など非欧米資本が出資・買収で受け皿化し、欧米AAA系スタジオ/IP周辺の権益が非欧米資本へ静かに移動する。</t>
+        </is>
+      </c>
+      <c r="C24" s="14" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="D24" s="14" t="inlineStr">
+        <is>
+          <t>6〜18ヶ月</t>
+        </is>
+      </c>
+      <c r="E24" s="14" t="inlineStr">
+        <is>
+          <t>Ninja Theory, Undead Labs, Tencent, NetEase, Savvy Games</t>
+        </is>
+      </c>
+      <c r="F24" s="14" t="inlineStr">
+        <is>
+          <t>Xbox、3,200人超削減し4スタジオを分離・売却（Game Informer, 2026-07-06）</t>
+        </is>
+      </c>
+      <c r="G24" s="14" t="inlineStr">
+        <is>
+          <t>分離/売却スタジオの新オーナー発表、元Xbox人材が設立/参画する新スタジオの出資元を観測。非欧米資本が絡めば的中。</t>
         </is>
       </c>
     </row>
@@ -3602,7 +3639,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G61"/>
+  <dimension ref="A1:G62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5868,6 +5905,43 @@
       <c r="G61" s="14" t="inlineStr">
         <is>
           <t>AI投資が川上の部材配分を歪め、川下の民生機器全般のコスト構造を横断的に押し上げる論点</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B62" s="14" t="inlineStr">
+        <is>
+          <t>プラットフォーマーが買収したスタジオを再び分離・独立させる『垂直統合の巻き戻し』は、メディア・小売・製造で起きた買収→不採算部門スピンオフの周期と同じか？</t>
+        </is>
+      </c>
+      <c r="C62" s="14" t="inlineStr">
+        <is>
+          <t>Xboxが3,200人超削減と4スタジオ分離/売却を発表（Game Informer, 2026-07-06）</t>
+        </is>
+      </c>
+      <c r="D62" s="14" t="inlineStr">
+        <is>
+          <t>Microsoft/Xbox, Compulsion, Double Fine, Ninja Theory, Undead Labs</t>
+        </is>
+      </c>
+      <c r="E62" s="14" t="inlineStr">
+        <is>
+          <t>メディア・コングロマリット, 小売(PB/事業売却), 製造(非中核事業スピンオフ), PE/再編ファンド</t>
+        </is>
+      </c>
+      <c r="F62" s="14" t="inlineStr">
+        <is>
+          <t>オープン</t>
+        </is>
+      </c>
+      <c r="G62" s="14" t="inlineStr">
+        <is>
+          <t>買収による内製化は景気・戦略局面で反転し、コア回帰＋スピンオフに転じる。ゲームも他産業の事業ポートフォリオ管理と同じ周期に入った可能性。</t>
         </is>
       </c>
     </row>
@@ -9990,7 +10064,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L266"/>
+  <dimension ref="A1:L271"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -26508,6 +26582,329 @@
       <c r="L266" s="14" t="inlineStr">
         <is>
           <t>2026-06施行</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B267" s="14" t="inlineStr">
+        <is>
+          <t>Xbox、3,200人超を削減し4スタジオを分離・売却——Compulsion・Double Fineは独立へ</t>
+        </is>
+      </c>
+      <c r="C267" s="14" t="inlineStr">
+        <is>
+          <t>https://gameinformer.com/2026/07/06/xbox-parts-ways-with-four-studios-over-3000-layoffs-announced</t>
+        </is>
+      </c>
+      <c r="D267" s="14" t="inlineStr">
+        <is>
+          <t>MicrosoftのゲームCEOアーシャ・シャルマが7月6日、大規模な組織再編を発表。2018年以降の買収拡大でXboxは30近いスタジオを抱えたが、収益性重視への転換で買収済みスタジオの整理に踏み切った。</t>
+        </is>
+      </c>
+      <c r="E267" s="14" t="inlineStr">
+        <is>
+          <t>Xboxは3,200人超の人員削減とともに、Compulsion GamesとDouble Fineを独立スタジオとして分離（IPは各社が保持）、Ninja TheoryとUndead Labsは資金付きで新オーナーへ売却交渉中と発表。既発表タイトルは中止しないとした。</t>
+        </is>
+      </c>
+      <c r="F267" s="14" t="inlineStr">
+        <is>
+          <t>3,200人超を数か月かけて削減
+買収スタジオ4社を分離・売却、IPは各社保持
+Compulsion/Double Fineは再びインディーへ
+Ninja Theory/Undead Labsは資金付きで新オーナー交渉
+既発表プロジェクトは中止せず</t>
+        </is>
+      </c>
+      <c r="G267" s="14" t="inlineStr">
+        <is>
+          <t>2010年代後半の買収競争で膨張したファーストパーティ体制の巻き戻しが進む。放出スタジオの新たな出資者・パブリッシャー探しが活発化し、業界の人材・IPの再配置が加速する見込み。</t>
+        </is>
+      </c>
+      <c r="H267" s="14" t="inlineStr">
+        <is>
+          <t>プラットフォーマーの垂直統合と『買収→分離』サイクル</t>
+        </is>
+      </c>
+      <c r="I267" s="14" t="inlineStr">
+        <is>
+          <t>Microsoft, Xbox, Compulsion Games, Double Fine, Ninja Theory, Undead Labs</t>
+        </is>
+      </c>
+      <c r="J267" s="14" t="inlineStr">
+        <is>
+          <t>South of Midnight, Psychonauts, Hellblade, State of Decay</t>
+        </is>
+      </c>
+      <c r="K267" s="14" t="inlineStr">
+        <is>
+          <t>M&amp;A,業績,海外</t>
+        </is>
+      </c>
+      <c r="L267" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-06発表</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B268" s="14" t="inlineStr">
+        <is>
+          <t>ZeniMax Online（Elder Scrolls Online）でも大規模解雇、スタッフ最大半減の報道</t>
+        </is>
+      </c>
+      <c r="C268" s="14" t="inlineStr">
+        <is>
+          <t>https://www.pcgamer.com/gaming-industry/bethesda-game-studios-and-zenimax-hit-hard-by-xbox-layoffs-says-union/</t>
+        </is>
+      </c>
+      <c r="D268" s="14" t="inlineStr">
+        <is>
+          <t>7月6日のXbox再編に伴い、Bethesda/ZeniMax傘下も影響。労働組合はBethesda Game StudiosやZeniMaxが特に強く打撃を受けたと表明した。</t>
+        </is>
+      </c>
+      <c r="E268" s="14" t="inlineStr">
+        <is>
+          <t>『The Elder Scrolls Online』を運営するZeniMax Online Studiosで大規模な人員削減が報じられ、一部報道はスタッフの最大半数が対象になり得るとする。ZeniMaxは主要IP中心に再編・リアラインされる。</t>
+        </is>
+      </c>
+      <c r="F268" s="14" t="inlineStr">
+        <is>
+          <t>ESO運営のZeniMax Onlineが人員削減対象
+最大でスタッフ半減の可能性との報道
+労組がBethesda/ZeniMaxの打撃を指摘
+主要IPに絞った再編・リアライン</t>
+        </is>
+      </c>
+      <c r="G268" s="14" t="inlineStr">
+        <is>
+          <t>運営型MMOの体制縮小で長期運営タイトルの更新頻度・新規投資に影響が及ぶ可能性。熟練運営人材の流出が他社のライブサービス立ち上げに波及しうる。</t>
+        </is>
+      </c>
+      <c r="H268" s="14" t="inlineStr">
+        <is>
+          <t>長期運営MMOの体制縮小と運営人材の流動</t>
+        </is>
+      </c>
+      <c r="I268" s="14" t="inlineStr">
+        <is>
+          <t>Microsoft, ZeniMax Online, Bethesda</t>
+        </is>
+      </c>
+      <c r="J268" s="14" t="inlineStr">
+        <is>
+          <t>The Elder Scrolls Online</t>
+        </is>
+      </c>
+      <c r="K268" s="14" t="inlineStr">
+        <is>
+          <t>業績,海外</t>
+        </is>
+      </c>
+      <c r="L268" s="14" t="inlineStr">
+        <is>
+          <t>労組コメント/2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B269" s="14" t="inlineStr">
+        <is>
+          <t>生成AIゲーム市場、2026年に22.1億ドルへ拡大（年23.1%成長）との市場レポート公開</t>
+        </is>
+      </c>
+      <c r="C269" s="14" t="inlineStr">
+        <is>
+          <t>https://www.globenewswire.com/news-release/2026/07/03/3321771/0/en/generative-ai-in-gaming-market-report-2026.html</t>
+        </is>
+      </c>
+      <c r="D269" s="14" t="inlineStr">
+        <is>
+          <t>生成AIのゲーム開発・運用への浸透が進むなか、7月3日に市場調査レポートが公開。3D/没入型ゲームや手続き型生成、マルチプレイの拡大が需要を押し上げているとする。</t>
+        </is>
+      </c>
+      <c r="E269" s="14" t="inlineStr">
+        <is>
+          <t>レポートは生成AIゲーム市場が2025年17.9億ドルから2026年22.1億ドル（CAGR23.1%）へ拡大し、2030年に50.9億ドルへ達すると予測。手続き型生成・適応型ゲームプレイ・AIテストが主要トレンドで、アジア太平洋が最大市場とした。</t>
+        </is>
+      </c>
+      <c r="F269" s="14" t="inlineStr">
+        <is>
+          <t>2026年市場規模22.1億ドル、CAGR23.1%
+2030年に50.9億ドル予測
+手続き型生成・適応型メカ・AIテストが牽引
+アジア太平洋が最大地域
+主要各社（MS,EA,Ubisoft,SE等）が投資</t>
+        </is>
+      </c>
+      <c r="G269" s="14" t="inlineStr">
+        <is>
+          <t>AIによる開発コスト圧縮と少人数開発の加速が続き、コンテンツ生成の内製化が進む。一方で品質・著作権・雇用面の論点が並行して顕在化する。</t>
+        </is>
+      </c>
+      <c r="H269" s="14" t="inlineStr">
+        <is>
+          <t>生成AIの開発・運用適用と市場規模トレンド</t>
+        </is>
+      </c>
+      <c r="I269" s="14" t="inlineStr">
+        <is>
+          <t>Microsoft, Electronic Arts, Ubisoft, Square Enix</t>
+        </is>
+      </c>
+      <c r="J269" s="14" t="inlineStr"/>
+      <c r="K269" s="14" t="inlineStr">
+        <is>
+          <t>技術,海外</t>
+        </is>
+      </c>
+      <c r="L269" s="14" t="inlineStr">
+        <is>
+          <t>市場調査レポート(2026-07-03)</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B270" s="14" t="inlineStr">
+        <is>
+          <t>Valve、Steam Machineの2026年内投入に慎重姿勢——メモリ・ストレージ不足が影響</t>
+        </is>
+      </c>
+      <c r="C270" s="14" t="inlineStr">
+        <is>
+          <t>https://gamerant.com/valve-steam-machine-summer-release-news-update-2026/</t>
+        </is>
+      </c>
+      <c r="D270" s="14" t="inlineStr">
+        <is>
+          <t>AIデータセンター需要でメモリ・ストレージ価格が高騰するなか、Valveは新ハード「Steam Machine」について7月に慎重な進捗アップデートを出した。</t>
+        </is>
+      </c>
+      <c r="E270" s="14" t="inlineStr">
+        <is>
+          <t>Valveはメモリ・ストレージの供給不足を継続課題として挙げ、ハイブリッド機Steam Machineが2026年の投入目標を超える可能性に言及。部材制約がコンシューマ機のコスト・供給に波及している。</t>
+        </is>
+      </c>
+      <c r="F270" s="14" t="inlineStr">
+        <is>
+          <t>Steam Machineの2026年内発売に黄信号
+メモリ・ストレージ不足が主因
+部材高騰がハード計画を圧迫
+DRAM高騰(既報)と同根の供給問題</t>
+        </is>
+      </c>
+      <c r="G270" s="14" t="inlineStr">
+        <is>
+          <t>部材高騰が続けば新ハードの価格上昇・発売延期が常態化。据置/携帯機のBOMコスト上昇がプラットフォーム各社の値付けに波及する。</t>
+        </is>
+      </c>
+      <c r="H270" s="14" t="inlineStr">
+        <is>
+          <t>半導体・メモリ供給制約とゲームハード計画</t>
+        </is>
+      </c>
+      <c r="I270" s="14" t="inlineStr">
+        <is>
+          <t>Valve</t>
+        </is>
+      </c>
+      <c r="J270" s="14" t="inlineStr">
+        <is>
+          <t>Steam Machine, Steam Deck</t>
+        </is>
+      </c>
+      <c r="K270" s="14" t="inlineStr">
+        <is>
+          <t>技術,海外</t>
+        </is>
+      </c>
+      <c r="L270" s="14" t="inlineStr">
+        <is>
+          <t>2026-07 Valve更新</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B271" s="14" t="inlineStr">
+        <is>
+          <t>コーエーテクモ『進撃の巨人3』、最新情報の公式番組を7/2配信——実機プレイ初公開</t>
+        </is>
+      </c>
+      <c r="C271" s="14" t="inlineStr">
+        <is>
+          <t>https://gamebiz.jp/news/428758</t>
+        </is>
+      </c>
+      <c r="D271" s="14" t="inlineStr">
+        <is>
+          <t>コーエーテクモ（ω-Force開発）は6月のSummer Game Festで『進撃の巨人3』を発表。原作を最初から最後まで描く集大成として、7月2日に続報の公式番組を配信した。</t>
+        </is>
+      </c>
+      <c r="E271" s="14" t="inlineStr">
+        <is>
+          <t>『進撃の巨人3』はPS5/Switch 2/Xbox/Steam向けのタクティカルハンティングアクション。7月2日の公式番組で世界初のゲーム実機プレイを公開し、立体機動アクションなどを披露した。</t>
+        </is>
+      </c>
+      <c r="F271" s="14" t="inlineStr">
+        <is>
+          <t>7/2に公式番組で続報公開
+世界初のゲーム実機プレイを披露
+ω-Force開発、原作を完結まで描く集大成
+マルチ展開（PS5/Switch2/Xbox/Steam）</t>
+        </is>
+      </c>
+      <c r="G271" s="14" t="inlineStr">
+        <is>
+          <t>人気アニメIPの完結編需要を取り込み、国内外での販売が期待される。Switch 2の普及拡大がマルチ展開の追い風。</t>
+        </is>
+      </c>
+      <c r="H271" s="14" t="inlineStr">
+        <is>
+          <t>人気アニメIPのゲーム化と完結編需要</t>
+        </is>
+      </c>
+      <c r="I271" s="14" t="inlineStr">
+        <is>
+          <t>コーエーテクモゲームス, ω-Force</t>
+        </is>
+      </c>
+      <c r="J271" s="14" t="inlineStr">
+        <is>
+          <t>進撃の巨人</t>
+        </is>
+      </c>
+      <c r="K271" s="14" t="inlineStr">
+        <is>
+          <t>新作,国内</t>
+        </is>
+      </c>
+      <c r="L271" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-02配信</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
daily-news + cross-questions + events + predictions + game-design update (2026-07-08)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -816,7 +816,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1713,6 +1713,43 @@
       <c r="G24" s="14" t="inlineStr">
         <is>
           <t>分離/売却スタジオの新オーナー発表、元Xbox人材が設立/参画する新スタジオの出資元を観測。非欧米資本が絡めば的中。</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B25" s="14" t="inlineStr">
+        <is>
+          <t>Switch 2本体の499.99ドルへの値上げとメモリ高騰で、任天堂がファーストパーティを高価格帯に固定すると、サードパーティは価格追随できず“Switch 2向けは廉価・小規模タイトルに寄せ、AAAはクラウド/ストリーミング版で逃がす”二極化が進む（＝値上げ追随ではなく、サードのラインナップ設計とデリバリー形態の分岐）。</t>
+        </is>
+      </c>
+      <c r="C25" s="14" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="D25" s="14" t="inlineStr">
+        <is>
+          <t>年内〜2027年</t>
+        </is>
+      </c>
+      <c r="E25" s="14" t="inlineStr">
+        <is>
+          <t>任天堂, サードパーティ各社</t>
+        </is>
+      </c>
+      <c r="F25" s="14" t="inlineStr">
+        <is>
+          <t>任天堂、米Switch 2を9/1に499.99ドルへ値上げ（Nintendo Everything）</t>
+        </is>
+      </c>
+      <c r="G25" s="14" t="inlineStr">
+        <is>
+          <t>観測対象：今後発表されるSwitch 2向けサードAAAの提供形態（パッケージ/ダウンロード vs クラウド版）と価格帯、初週販売。クラウド版比率が上がれば当たり。</t>
         </is>
       </c>
     </row>
@@ -3639,7 +3676,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G62"/>
+  <dimension ref="A1:G63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5942,6 +5979,43 @@
       <c r="G62" s="14" t="inlineStr">
         <is>
           <t>買収による内製化は景気・戦略局面で反転し、コア回帰＋スピンオフに転じる。ゲームも他産業の事業ポートフォリオ管理と同じ周期に入った可能性。</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B63" s="14" t="inlineStr">
+        <is>
+          <t>EUのDFAに見る『確率型・ダークパターン規制』の潮流は、ゲームだけでなく金融（仕組み債・射幸性商品）や広告（ダークパターン規制）でも同じ“射幸性×消費者保護”の論点として同時進行するか？ゲームの有料ランダムは金融の何に該当するか。</t>
+        </is>
+      </c>
+      <c r="C63" s="14" t="inlineStr">
+        <is>
+          <t>EUデジタル公正法(DFA)、ルートボックス規制方向（Freshfields/2026）</t>
+        </is>
+      </c>
+      <c r="D63" s="14" t="inlineStr">
+        <is>
+          <t>Electronic Arts, Epic Games, Roblox</t>
+        </is>
+      </c>
+      <c r="E63" s="14" t="inlineStr">
+        <is>
+          <t>金融（射幸性商品・仕組み債の適合性規制）, 広告（ダークパターン/DFA）, 決済</t>
+        </is>
+      </c>
+      <c r="F63" s="14" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="G63" s="14" t="inlineStr">
+        <is>
+          <t>ガチャ規制は“ギャンブル論”から“消費者保護・ダークパターン論”へ軸が移りつつある。金融の適合性原則と接続すると論点が整理できる。</t>
         </is>
       </c>
     </row>
@@ -8278,54 +8352,54 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B2" s="14" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C2" s="14" t="inlineStr">
         <is>
           <t>Steam サマーセール 2026</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="D2" s="14" t="inlineStr">
         <is>
           <t>セール</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="E2" s="14" t="inlineStr">
         <is>
           <t>オンライン(Steam)</t>
         </is>
       </c>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="F2" s="14" t="inlineStr">
         <is>
           <t>ストアセール</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="G2" s="14" t="inlineStr">
         <is>
           <t>Steam最大級の季節セール。値引き合戦と販売ブースト。次回Next Festに向けたウィッシュリスト施策も活発化。</t>
         </is>
       </c>
-      <c r="H2" s="5" t="inlineStr">
+      <c r="H2" s="14" t="inlineStr">
         <is>
           <t>https://www.pcgamer.com/steam-sale-dates/</t>
         </is>
       </c>
-      <c r="I2" s="15" t="inlineStr">
+      <c r="I2" s="14" t="inlineStr">
         <is>
           <t>開催中</t>
         </is>
       </c>
-      <c r="J2" s="15" t="inlineStr">
-        <is>
-          <t>2026-06-25</t>
+      <c r="J2" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
         </is>
       </c>
     </row>
@@ -9706,7 +9780,7 @@
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
@@ -9721,7 +9795,7 @@
       </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
-          <t>成熟→規制逆風（区分強化で加速）</t>
+          <t>成熟→規制逆風（DFAで欧州規制が具体化）</t>
         </is>
       </c>
       <c r="E6" s="14" t="inlineStr">
@@ -9741,12 +9815,12 @@
       </c>
       <c r="H6" s="14" t="inlineStr">
         <is>
-          <t>PEGIの新リスク区分で課金ルートボックスは最低PEGI 16に。低年齢レーティング維持のため確定報酬型（直接購入/バトルパス）への置換が進む見込み。NFTはPEGI 18でWeb3型の逆風も継続。</t>
+          <t>EUのDFAで全面禁止/保護者同意・ニアミス演出禁止・実額表示が現実味。ブラジル未成年禁止・豪15+と合わせ地域規制がモザイク化し、確定報酬型（直接購入/バトルパス/段階開封）への移行圧力が強まる。</t>
         </is>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
-          <t>PEGI新リスク区分が6月適用、課金ルートボックス含む新規申請は最低PEGI 16(VGC, 2026-06-30)</t>
+          <t>EUデジタル公正法(DFA)ルートボックス規制方向（Freshfields/2026-07）</t>
         </is>
       </c>
       <c r="J6" s="14" t="n">
@@ -10064,7 +10138,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L271"/>
+  <dimension ref="A1:L275"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -26907,6 +26981,243 @@
           <t>2026-07-02配信</t>
         </is>
       </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B272" s="14" t="inlineStr">
+        <is>
+          <t>オープンワールドRPG『NTE: Neverness to Everness』Steam/Epic版が7/8ローンチ、V1.2から開始</t>
+        </is>
+      </c>
+      <c r="C272" s="14" t="inlineStr">
+        <is>
+          <t>https://store.steampowered.com/news/app/4508340/view/684131849711125585</t>
+        </is>
+      </c>
+      <c r="D272" s="14" t="inlineStr">
+        <is>
+          <t>Hotta Studio（テンセント系）開発の都市系オープンワールドRPG。モバイル/PCで先行運営していたタイトルをSteam・Epic Games Storeへ拡大投入し、既存プラットフォームとクロスプログレッションで接続する。</t>
+        </is>
+      </c>
+      <c r="E272" s="14" t="inlineStr">
+        <is>
+          <t>7/8にSteam版とEpic版を同時ローンチ。アジア/米州/欧州/SEAサーバーでクロスセーブに対応し、いきなり最新のVersion 1.2コンテンツから遊べる。中国系スタジオのグローバルPC展開の一例。</t>
+        </is>
+      </c>
+      <c r="F272" s="14" t="inlineStr">
+        <is>
+          <t>Steam/Epic同時ローンチ
+モバイル・PC・PCストア間でクロスプログレッション対応
+Version 1.2コンテンツから開始
+Hotta Studio（『幻塔』開発元、テンセント系）</t>
+        </is>
+      </c>
+      <c r="G272" s="14" t="inlineStr">
+        <is>
+          <t>中国系運営型オープンワールドのPC/グローバル展開が加速。Steamでの同接・課金の立ち上がりが、後続の中国発GaaSのPC戦略を左右する。</t>
+        </is>
+      </c>
+      <c r="H272" s="14" t="inlineStr">
+        <is>
+          <t>運営型OWのクロスプラットフォーム設計とグローバル同時運営</t>
+        </is>
+      </c>
+      <c r="I272" s="14" t="inlineStr">
+        <is>
+          <t>テンセント, Hotta Studio, Valve, Epic Games</t>
+        </is>
+      </c>
+      <c r="J272" s="14" t="inlineStr">
+        <is>
+          <t>NTE, 幻塔</t>
+        </is>
+      </c>
+      <c r="K272" s="14" t="inlineStr">
+        <is>
+          <t>新作,海外</t>
+        </is>
+      </c>
+      <c r="L272" s="14" t="inlineStr"/>
+    </row>
+    <row r="273">
+      <c r="A273" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B273" s="14" t="inlineStr">
+        <is>
+          <t>任天堂、米Switch 2を9/1に449.99→499.99ドルへ値上げ——直前サマーセールで駆け込み需要を喚起</t>
+        </is>
+      </c>
+      <c r="C273" s="14" t="inlineStr">
+        <is>
+          <t>https://nintendoeverything.com/nintendo-announces-2026-summer-sale-for-switch-2-and-switch-heres-the-full-list-of-deals/</t>
+        </is>
+      </c>
+      <c r="D273" s="14" t="inlineStr">
+        <is>
+          <t>DRAM等のメモリ価格高騰が続くなか、任天堂は米国のSwitch 2本体価格を9/1に449.99ドルから499.99ドルへ引き上げると案内。発売2年目に入り、値上げ直前のこの時期にSwitch 2/Switch向けの2026サマーセールを実施している。</t>
+        </is>
+      </c>
+      <c r="E273" s="14" t="inlineStr">
+        <is>
+          <t>米国Switch 2は9/1から実質50ドル高い499.99ドルへ。値上げ前の販促としてeShopでサマーセールを展開し、ソフト・旧世代を含めた駆け込み需要を取りにいく。ハード原価上昇を価格転嫁する動きが鮮明。</t>
+        </is>
+      </c>
+      <c r="F273" s="14" t="inlineStr">
+        <is>
+          <t>米Switch 2本体を9/1に449.99→499.99ドルへ値上げ
+値上げ直前にサマーセールを実施
+Switch 2は初年度で世界1,986万台出荷（3月末時点）
+背景にDRAM/メモリ価格高騰</t>
+        </is>
+      </c>
+      <c r="G273" s="14" t="inlineStr">
+        <is>
+          <t>本体値上げがソフト価格帯（ファーストパーティ高価格化）や販売数量に波及。年末商戦での値上げ後の失速有無が焦点。</t>
+        </is>
+      </c>
+      <c r="H273" s="14" t="inlineStr">
+        <is>
+          <t>コンソール原価（BOM）と価格転嫁・数量弾力性</t>
+        </is>
+      </c>
+      <c r="I273" s="14" t="inlineStr">
+        <is>
+          <t>任天堂</t>
+        </is>
+      </c>
+      <c r="J273" s="14" t="inlineStr">
+        <is>
+          <t>Nintendo Switch 2</t>
+        </is>
+      </c>
+      <c r="K273" s="14" t="inlineStr">
+        <is>
+          <t>業績,国内</t>
+        </is>
+      </c>
+      <c r="L273" s="14" t="inlineStr"/>
+    </row>
+    <row r="274">
+      <c r="A274" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B274" s="14" t="inlineStr">
+        <is>
+          <t>韓国ゲーム大手Nexon・Netmarble・Krafton、公取委の大企業集団で資産増——アジア資本の地位固め</t>
+        </is>
+      </c>
+      <c r="C274" s="14" t="inlineStr">
+        <is>
+          <t>https://www.koreaherald.com/article/10489159</t>
+        </is>
+      </c>
+      <c r="D274" s="14" t="inlineStr">
+        <is>
+          <t>韓国公正取引委員会が公表した2026年の大企業集団リストで、Nexon・Netmarble・Kraftonがそろって指定を維持。欧米の大量解雇・再編とは対照的に、韓国大手は資産・売上を伸ばして存在感を高めている。</t>
+        </is>
+      </c>
+      <c r="E274" s="14" t="inlineStr">
+        <is>
+          <t>Nexonは公正資産15.1兆ウォン（前年比+7.3%）で業界首位、全体順位も41→40位に上昇。Netmarbleは13兆ウォン（+10.5%）、Kraftonは9.2兆ウォン（+8.8%）と最大の伸び。好調な決算を背景に規模を拡大。</t>
+        </is>
+      </c>
+      <c r="F274" s="14" t="inlineStr">
+        <is>
+          <t>Nexon 15.1兆ウォン（首位、+7.3%）
+Netmarble 13兆ウォン（+10.5%）
+Krafton 9.2兆ウォン（+8.8%、伸び最大）
+欧米の縮小局面と対照的にアジア勢が拡大</t>
+        </is>
+      </c>
+      <c r="G274" s="14" t="inlineStr">
+        <is>
+          <t>潤沢な資産を背景に韓国大手が欧米のリストラ放出スタジオ/IPの受け皿となる可能性。中東資本と並ぶ買い手として存在感が増す。</t>
+        </is>
+      </c>
+      <c r="H274" s="14" t="inlineStr">
+        <is>
+          <t>韓国ゲーム大手の資本力とグローバルM&amp;A余力</t>
+        </is>
+      </c>
+      <c r="I274" s="14" t="inlineStr">
+        <is>
+          <t>Nexon, Netmarble, Krafton</t>
+        </is>
+      </c>
+      <c r="J274" s="14" t="inlineStr"/>
+      <c r="K274" s="14" t="inlineStr">
+        <is>
+          <t>業績,海外</t>
+        </is>
+      </c>
+      <c r="L274" s="14" t="inlineStr"/>
+    </row>
+    <row r="275">
+      <c r="A275" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B275" s="14" t="inlineStr">
+        <is>
+          <t>EUデジタル公正法(DFA)、ルートボックス規制へ——メーカーに「略奪的でない」立証やニアミス演出禁止を要求する方向</t>
+        </is>
+      </c>
+      <c r="C275" s="14" t="inlineStr">
+        <is>
+          <t>https://technologyquotient.freshfields.com/post/102ltio/the-eus-proposed-digital-fairness-act-a-game-developers-guide-to-potential-imp</t>
+        </is>
+      </c>
+      <c r="D275" s="14" t="inlineStr">
+        <is>
+          <t>EUは消費者保護をデジタル時代に合わせて更新するデジタル公正法(DFA)を2026年作業計画のQ4に位置づけ。ルートボックス等のランダム課金に対し、EU横断での規制枠組みを準備している。</t>
+        </is>
+      </c>
+      <c r="E275" s="14" t="inlineStr">
+        <is>
+          <t>DFAはルートボックスの全面禁止か、未成年の有料購入に保護者同意を求める案を含む。メーカーに仕組みが『略奪的でない』ことの立証を課し、『ニアミス』演出の全面禁止やゲーム内通貨の実額表示も検討。適用は2029年以降の見込み。</t>
+        </is>
+      </c>
+      <c r="F275" s="14" t="inlineStr">
+        <is>
+          <t>Q4 2026に提案予定
+ルートボックス全面禁止または未成年に保護者同意
+『略奪的でない』立証責任をメーカーに
+ニアミス演出禁止・実額表示
+適用は2029年以降の見込み</t>
+        </is>
+      </c>
+      <c r="G275" s="14" t="inlineStr">
+        <is>
+          <t>確率型課金の設計自由度がEUで制約され、確定報酬型（直接購入/バトルパス/段階開封）への転換圧力が強まる。ブラジル未成年禁止・豪15+と合わせ地域規制がモザイク化。</t>
+        </is>
+      </c>
+      <c r="H275" s="14" t="inlineStr">
+        <is>
+          <t>ランダム課金規制（DFA/各国法）とマネタイズ設計の適法化</t>
+        </is>
+      </c>
+      <c r="I275" s="14" t="inlineStr">
+        <is>
+          <t>Electronic Arts, Epic Games, Roblox</t>
+        </is>
+      </c>
+      <c r="J275" s="14" t="inlineStr"/>
+      <c r="K275" s="14" t="inlineStr">
+        <is>
+          <t>規制,海外</t>
+        </is>
+      </c>
+      <c r="L275" s="14" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
weekly-trends + tech update (2026-07-08 14:28)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -1764,7 +1764,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2846,6 +2846,117 @@
       <c r="G29" t="inlineStr">
         <is>
           <t>https://tech-insider.org/nintendo-switch-2-sales-19-million-2026/ , https://famiboards.com/threads/all-of-the-third-party-switch-2-games-dates-announced-during-not-e3-2026-june-1st-june-9th.17747/</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>韓国ゲーム大手のオーナー株売却連鎖と海外資本流入</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Wemade創業者パク・グァンホ会長が6/30、保有株の全てを香港の投資プラットフォーム「NeoPulse」へ約9200億ウォン(約960億円)で売却すると発表。4Gamerは7/7の記事で、韓国大手に相次ぐ大型M&amp;Aを「業界の危機なのか、グローバル飛躍への再編なのか」と両論で分析した。MMO/リネージュ型のヘビー課金モデルが成熟し、国内市場の飽和と中国市場の閉塞で成長が鈍化する中、創業者世代が資本を回収(exit)する一方、香港・中国系マネーが経営権を取りに来る構図が同時進行している。単発の提携(先週のKrafton×Hanwha)ではなく、オーナー交代を伴う支配権移動である点が今回の特徴で、経営方針やIP戦略の転換リスクを孕む。</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Wemade, NeoPulse(香港), Krafton, Netmarble, Nexon, NCSoft</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>韓国産業は輸出主導かつ少数大手寡占。成長エンジンだったPC-MMOとモバイルガチャが頭打ちとなり、株式市場評価も低迷。創業者の高齢化と後継不在が重なり、事業承継の出口として外部・海外資本への売却が現実解に。支配権が海外に移ると開発拠点・IP・人材が越境再配置される。</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>日本大手も創業者高齢化・承継局面に入りつつあり、優良IP/スタジオが海外資本の買収標的になる構図は対岸の火事ではない。</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/991/G999101/20260707014/</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>「コージーホラー」の本格ジャンル化とマイクロスタジオ上位進出</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>The Rat Zone開発『Creature Kitchen』(2/6発売)が、レビュー5689件で99%好評を獲得しSteam2026年最高評価タイトルに。直近30日でも99%を維持。約6〜8ドルの低価格・3〜6時間の短尺ながら、森の家の不気味なオーブンでラクーンやUMAに餌を与えるという「癒し×不穏」の設計が刺さった。Cult of the LambやGrave Seasonsが先行した「Stardew Valley meets horror」がサブジャンルとして定着しつつあり、PC Gamer・Kotaku・IGN系も相次いで特集。同週のSteamトレンドでは早期アクセスの『Far Far West』も97%(17,366件)と、大手ではなくマイクロ/インディーが評価上位を占める傾向が続く。</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>The Rat Zone(Creature Kitchen), Massive Monster(Cult of the Lamb), Valve/Steam</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>「コージー」の低リスク・探索・情緒という体験要件を満たしたまま、意図的に不穏さ(subversion)を混ぜることで既存の飽和ジャンルを差別化。低予算・短尺・口コミ駆動というコスト構造が、レビュースコアとキュレーション経由でマイクロスタジオを可視化するSteamのディスカバリーと噛み合う。</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>ジャンルの掛け合わせによる差別化はレッドオーシャン回避の定石。安心×不穏のミックスは映像・出版など他エンタメにも移植可能。</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>https://kotaku.com/creature-kitchen-cozy-game-horror-cooking-steam-overwhelmingly-positive-2000687920</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>PEGI「有料ランダムアイテム」強制16+レーティング開始</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>PEGIが「インタラクティブ・リスク・カテゴリ」を新設し、2026年6月以降の新規申請から、ルートボックス・ガチャ・カードパック・アイテム解錠キーなど「有料ランダムアイテム」を販売するタイトルは原則PEGI 16(場合により18)を付与する運用を開始。デイリークエスト等の再訪誘導設計や、ブロック/通報手段のないコミュニケーション機能も新たに分類対象となった。並行して蘭では裁判所がEAへの1000万ユーロ制裁金を撤回し(ゲームプレイ統合型ガチャは独立した賭博商品ではないと判断)、直接的な賭博規制は足踏み。一方でEU全体はDigital Fairness Actで未成年向けルートボックス規制へ動く可能性があり、「直接規制」と「レーティング/開示」の二方面から課金設計に圧力がかかる。</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>PEGI, Electronic Arts(EA Sports FC), Netherlands当局, EU</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>禁止ではなく年齢レーティングの引き上げという「情報開示型」の介入。16+化は最も課金効率の高い若年層への訴求を削ぎ、F2P/ガチャの収益基盤を間接的に侵食する。国別の賭博規制(蘭・白)と汎欧州レーティング統一が並存し、パブリッシャーは設計変更かレーティング上昇かの二択を迫られる。</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>「禁止」でなく「可視化・格付け」で行動変容を促す規制は、食品表示や金融商品規制と同型。日本のガチャ確率表示自主規制の次段階を占う。</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>https://www.reedsmith.com/articles/pegi-launches-interactive-risk-categories-overhauls-age-ratings-for-loot-boxes-in-game-spending-and-communication-features/</t>
         </is>
       </c>
     </row>
@@ -32232,7 +32343,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -32544,7 +32655,7 @@
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
@@ -32559,32 +32670,32 @@
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>EU AI法の透明性ルールが8/2全面適用へ。米加州AB1921（運営終了時のユーザー保護）が州下院を通過。</t>
+          <t>EUはレーティング統一とDigital Fairness Actで課金・ダークパターン規制を前進。</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
-          <t>英政府が16歳未満のオンライン利用制限を公表／PEGIが有料ランダムアイテムを年齢レーティングへ反映する新基準を運用開始／EU AI法のAI生成表示義務が迫る。</t>
+          <t>PEGIが「インタラクティブ・リスク・カテゴリ」を導入し、課金・再訪誘導・コミュニケーション機能を分類対象化(6月〜新規申請)。</t>
         </is>
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>EU, 英政府, PEGI, Apple, Google</t>
+          <t>PEGI, EU, EA</t>
         </is>
       </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t>流通（ストア開放）・年齢確認・課金設計・AI表示の4軸で規制が同時進行。グローバル運営は地域別の複層対応が標準になる。</t>
+          <t>汎欧州でのレーティング厳格化が事実上のデファクト基準となり、グローバル配信の設計に波及。</t>
         </is>
       </c>
       <c r="H8" s="9" t="inlineStr">
         <is>
-          <t>単一論点でなく『複数レイヤー同時規制』が新常態。コンプラ投資が中堅以下の参入障壁を押し上げる。</t>
+          <t>レーティング団体が実質的なルールメーカー化している。</t>
         </is>
       </c>
       <c r="I8" s="9" t="inlineStr">
         <is>
-          <t>https://www.pwc.com/jp/ EU AI法 / https://www.jetro.go.jp/ 英年齢制限</t>
+          <t>https://www.reedsmith.com/articles/pegi-launches-interactive-risk-categories-overhauls-age-ratings-for-loot-boxes-in-game-spending-and-communication-features/</t>
         </is>
       </c>
       <c r="J8" s="9" t="inlineStr"/>
@@ -32592,7 +32703,7 @@
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B9" s="9" t="inlineStr">
@@ -32607,32 +32718,32 @@
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>各国で段階的に規制が進むが基準は不揃いで、対応コストが増大。</t>
+          <t>レーティングによる間接規制フェーズへ。直接的賭博規制は国ごとに温度差。</t>
         </is>
       </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>中国NPPAがデイリーログイン・初回購入ボーナス等の課金誘因を狙う規制を継続検討。韓国は確率表示に続く第二弾規制を推進。日本は2024年電子商取引促進法改正で射幸性課金への監視を強化。</t>
+          <t>PEGIが6月以降、有料ランダムアイテム(ルートボックス/ガチャ/カードパック/キー)含有タイトルを原則16+に。蘭裁判所はEAへの1000万ユーロ制裁を撤回。</t>
         </is>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t>NPPA, 韓国規制当局, 消費者庁(日本), テンセント, ネットイース</t>
+          <t>PEGI, EA, Netherlands当局</t>
         </is>
       </c>
       <c r="G9" s="9" t="inlineStr">
         <is>
-          <t>確率表示→誘因制限→支出上限の順に各国が追随し、グローバル設計の分岐コストが増大。『規制裁定』が拠点・展開地域選定に影響。</t>
+          <t>16+化で若年層訴求が制約され、課金設計の見直し圧力が強まる。EU Digital Fairness Actが未成年向け規制を上乗せする可能性。</t>
         </is>
       </c>
       <c r="H9" s="9" t="inlineStr">
         <is>
-          <t>規制の照準が『確率の透明化』から『行動誘因そのもの』へ移動している。</t>
+          <t>「禁止」から「格付け・開示」への規制シフトが鮮明。</t>
         </is>
       </c>
       <c r="I9" s="9" t="inlineStr">
         <is>
-          <t>https://www.mmorpg.com/news/china-proposes-mobile-game-regulations-banning-gacha-incentives-including-daily-logins-2000129890</t>
+          <t>https://www.nintendolife.com/news/2026/03/pegi-targets-loot-boxes-with-its-new-overhauled-ratings-system</t>
         </is>
       </c>
       <c r="J9" s="9" t="inlineStr"/>
@@ -32668,7 +32779,7 @@
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
@@ -32683,32 +32794,32 @@
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>Steamはサマーセール開催中（6/25〜7/9）。Valveがハード領域へ本格進出し、PCゲーミングをリビングルームへ拡張する局面。</t>
+          <t>マイクロ/インディーが評価上位を独占するディスカバリー構造が継続。</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>Valveが6/23にSteam Machine（512GB $1,049〜）を発表し6/30出荷開始。Steam Deck比約6倍性能のSteamOS小型PC。再設計Steam Controller、VRのSteam Frameも同時展開。「本体を赤字で売らない」と明言し従来コンソールの逆ザヤモデルを否定。</t>
+          <t>コージーホラー『Creature Kitchen』が99%(5689件)で2026年Steam最高評価に。早期アクセス『Far Far West』も97%。低価格・短尺・口コミ駆動が上位進出。</t>
         </is>
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t>Valve, SteamOS, Steam Frame, Microsoft, Sony</t>
+          <t>The Rat Zone, Valve/Steam</t>
         </is>
       </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
-          <t>「薄利ハード×ストア回収」モデルが原価高騰下で優位に。垂直統合コンソール勢との価格思想の分岐が鮮明化。リビングルームPCがコンソールとPCの境界を溶かす。</t>
+          <t>ジャンル掛け合わせ(cozy×horror)と低予算短尺の組合せが、レビュースコア駆動のキュレーションで再現的にヒット化。</t>
         </is>
       </c>
       <c r="H11" s="9" t="inlineStr">
         <is>
-          <t>回収レイヤー（ストア30%）を別に持つ者だけがハード価格を自由化できる。プラットフォーム経済の逆ザヤ前提が崩れつつある。</t>
+          <t>資本規模でなくレビュー品質がSteam露出の主変数。</t>
         </is>
       </c>
       <c r="I11" s="9" t="inlineStr">
         <is>
-          <t>https://www.geekwire.com/2026/surprise-valves-new-steam-machine-is-here-but-the-price-is-the-real-shocker/</t>
+          <t>https://intoindiegames.com/features/news/creature-kitchen-is-steams-highest-rated-game-of-2026-so-far/</t>
         </is>
       </c>
       <c r="J11" s="9" t="inlineStr"/>
@@ -32833,6 +32944,53 @@
       <c r="I14" t="inlineStr">
         <is>
           <t>https://www.gamedeveloper.com/ Krafton×Hanwha</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>アジア・ゲーム資本再編</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>M&amp;A/資本</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>韓国大手でオーナー株売却・海外資本流入による支配権移動が連続。</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Wemade創業者が保有株全てを香港NeoPulseへ約9200億ウォンで売却(6/30)。4Gamerが業界再編として分析(7/7)。</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Wemade, NeoPulse(香港), Krafton, Netmarble</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>MMO/ガチャ成熟と国内飽和で、創業者exitと海外資本の取得が同時進行。IP・拠点の越境再配置が進む。</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>単発提携でなくオーナー交代型M&amp;Aが増加。</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/991/G999101/20260707014/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
daily-news(+4) + cross-questions(+2) + predictions(+1) + game-design(+1) update 2026-07-10
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -816,7 +816,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1787,6 +1787,43 @@
       <c r="G26" s="14" t="inlineStr">
         <is>
           <t>他社の買い切りアクション/RPGが同様に『大型有料拡張＋アップグレードキット』方式を採用するか、およびリリンク拡張の販売本数・同接推移を観測。採用が広がれば的中。</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B27" s="14" t="inlineStr">
+        <is>
+          <t>スタジオ買収契約で『創業者・キーメンバーの残留と報酬を守るエスクロー/リテンション条項』が標準化し、買収額の一部を後払い留保する設計が広がる(アーンアウト紛争の反動)。</t>
+        </is>
+      </c>
+      <c r="C27" s="14" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="D27" s="14" t="inlineStr">
+        <is>
+          <t>6〜12ヶ月</t>
+        </is>
+      </c>
+      <c r="E27" s="14" t="inlineStr">
+        <is>
+          <t>Krafton,Unknown Worlds 他</t>
+        </is>
+      </c>
+      <c r="F27" s="14" t="inlineStr">
+        <is>
+          <t>Krafton『Subnautica 2』開発元にボーナス支払いで和解・復職CEO辞任(Bloomberg,7/1)</t>
+        </is>
+      </c>
+      <c r="G27" s="14" t="inlineStr">
+        <is>
+          <t>今後発表されるゲームスタジオ買収案件で、アーンアウト/報酬エスクロー/キーマン残留条項の開示有無を観測する。</t>
         </is>
       </c>
     </row>
@@ -3824,7 +3861,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G64"/>
+  <dimension ref="A1:G66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6201,6 +6238,80 @@
       <c r="G64" s="14" t="inlineStr">
         <is>
           <t>配信全盛でもリアル見本市が拡大する点は、EC全盛でも旗艦店・体験型店舗が再評価される小売の構図と相似。露出とBtoB商談の集約装置としてのイベント価値。</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B65" s="14" t="inlineStr">
+        <is>
+          <t>クラウドソーシング/業務委託を悪用した『架空発注×稟議書偽装』型の内部横領は、外注を多用する広告・建設・IT受託など他業界でも同じ構造で起きるか？</t>
+        </is>
+      </c>
+      <c r="C65" s="14" t="inlineStr">
+        <is>
+          <t>ガンホー元システム本部長を背任容疑で逮捕・架空発注で約4,000万円(ITmedia/警視庁,7/8)</t>
+        </is>
+      </c>
+      <c r="D65" s="14" t="inlineStr">
+        <is>
+          <t>ガンホー</t>
+        </is>
+      </c>
+      <c r="E65" s="14" t="inlineStr">
+        <is>
+          <t>広告(外注制作),建設(下請発注),IT受託,BPO</t>
+        </is>
+      </c>
+      <c r="F65" s="14" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="G65" s="14" t="inlineStr">
+        <is>
+          <t>承認プロセスがある大企業ほど『稟議書という正規手続きの偽装』で不正が通る逆説。外注が多い業種ほど発注統制が弱点になる。</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B66" s="14" t="inlineStr">
+        <is>
+          <t>買収後のアーンアウト(業績連動報酬)不払いを狙った経営者解任は、テック・製薬などスタートアップM&amp;A全般でも起きる普遍的な紛争か？</t>
+        </is>
+      </c>
+      <c r="C66" s="14" t="inlineStr">
+        <is>
+          <t>Krafton『Subnautica 2』開発元にボーナス支払いで和解・復職CEO辞任(Bloomberg,7/1)</t>
+        </is>
+      </c>
+      <c r="D66" s="14" t="inlineStr">
+        <is>
+          <t>Krafton,Unknown Worlds</t>
+        </is>
+      </c>
+      <c r="E66" s="14" t="inlineStr">
+        <is>
+          <t>テックスタートアップ買収,製薬・バイオM&amp;A,PE/VC</t>
+        </is>
+      </c>
+      <c r="F66" s="14" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="G66" s="14" t="inlineStr">
+        <is>
+          <t>買収は『クロージング』より『アーンアウト期間中の統治』が火種。創業者の報酬保護は業界横断の設計課題。</t>
         </is>
       </c>
     </row>
@@ -9695,7 +9806,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10362,6 +10473,56 @@
         <v>4</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B14" s="14" t="inlineStr">
+        <is>
+          <t>サバイバルクラフト×クリーチャー収集(モンスター牧場×建築×マルチ)</t>
+        </is>
+      </c>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>メカニクス/構造</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>流行中(成熟)</t>
+        </is>
+      </c>
+      <c r="E14" s="14" t="inlineStr">
+        <is>
+          <t>モンスター収集・育成をオープンワールドのサバイバルクラフト＆自動化生産に接続し、協力/対戦マルチで長期運営する複合ジャンル。収集の中毒性とクラフト・拠点構築のやり込みを掛け合わせる。</t>
+        </is>
+      </c>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>Palworld/パルワールド</t>
+        </is>
+      </c>
+      <c r="G14" s="14" t="inlineStr">
+        <is>
+          <t>Palworldが早期アクセスで大量プレイヤーを獲得し2026/7/10に1.0化。収集×サバイバルの融合が一つの完成型として定着。</t>
+        </is>
+      </c>
+      <c r="H14" s="14" t="inlineStr">
+        <is>
+          <t>追随タイトルが増える一方、収集デザインの意匠・特許リスク(任天堂/ポケモン訴訟)が参入時の設計制約に。無料大型アップデート運営が標準化。</t>
+        </is>
+      </c>
+      <c r="I14" s="14" t="inlineStr">
+        <is>
+          <t>Palworld 1.0正式リリース(Gematsu,2026-07-10)</t>
+        </is>
+      </c>
+      <c r="J14" s="14" t="n">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10373,7 +10534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L282"/>
+  <dimension ref="A1:L286"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -27873,6 +28034,246 @@
         </is>
       </c>
       <c r="L282" s="14" t="inlineStr"/>
+    </row>
+    <row r="283">
+      <c r="A283" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B283" s="14" t="inlineStr">
+        <is>
+          <t>Palworld 1.0が正式リリース、累計4,000万人突破・価格$29.99据え置きでGame Pass初日対応</t>
+        </is>
+      </c>
+      <c r="C283" s="14" t="inlineStr">
+        <is>
+          <t>https://www.gematsu.com/2026/07/palworld-early-access-tops-40-million-players</t>
+        </is>
+      </c>
+      <c r="D283" s="14" t="inlineStr">
+        <is>
+          <t>ポケットペア(日本)の『Palworld』は2024年1月に早期アクセス開始後、モンスター収集とサバイバルクラフトを融合した設計で大ヒット。任天堂・ポケモンとの特許訴訟を抱えたまま、約2年半の早期アクセスを経て2026年7月10日に正式版1.0へ移行した。</t>
+        </is>
+      </c>
+      <c r="E283" s="14" t="inlineStr">
+        <is>
+          <t>1.0は無料大型アップデートとして全プラットフォーム同時配信。ワールドツリー実装やWing Pack追加など大規模改修を行いつつ価格は$29.99に据え置き。累計プレイヤーは早期アクセス中に4,000万人を突破し、Game Pass(PC/コンソール)にも初日対応した。</t>
+        </is>
+      </c>
+      <c r="F283" s="14" t="inlineStr">
+        <is>
+          <t>累計4,000万人突破
+1.0は無料アップデートで価格$29.99据え置き
+全プラットフォーム同時＋Game Pass初日対応
+任天堂/ポケモン特許訴訟は継続(想定賠償は最大計約6.2万ドル)</t>
+        </is>
+      </c>
+      <c r="G283" s="14" t="inlineStr">
+        <is>
+          <t>買い切り＋長期早期アクセス＋無料大型化という運営型が中堅スタジオの成長モデルとして参照される。訴訟の帰趨が収集系デザインの意匠・特許リスク評価に影響する。</t>
+        </is>
+      </c>
+      <c r="H283" s="14" t="inlineStr">
+        <is>
+          <t>早期アクセス長期運営とジャンル融合(サバイバル×収集)の収益設計</t>
+        </is>
+      </c>
+      <c r="I283" s="14" t="inlineStr">
+        <is>
+          <t>ポケットペア,Microsoft,任天堂,ポケモン</t>
+        </is>
+      </c>
+      <c r="J283" s="14" t="inlineStr">
+        <is>
+          <t>Palworld/パルワールド</t>
+        </is>
+      </c>
+      <c r="K283" s="14" t="inlineStr">
+        <is>
+          <t>新作,インディー,国内,海外</t>
+        </is>
+      </c>
+      <c r="L283" s="14" t="n"/>
+    </row>
+    <row r="284">
+      <c r="A284" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B284" s="14" t="inlineStr">
+        <is>
+          <t>Obsidianの『Avowed』続編が中止、Josh Sawyer主導の新作『Fallout』開発へ軸足</t>
+        </is>
+      </c>
+      <c r="C284" s="14" t="inlineStr">
+        <is>
+          <t>https://www.pcgamer.com/games/fallout/obsidian-is-reportedly-making-a-new-fallout-game-headed-by-josh-sawyer-after-microsoft-pulled-the-plug-on-an-avowed-sequel/</t>
+        </is>
+      </c>
+      <c r="D284" s="14" t="inlineStr">
+        <is>
+          <t>MicrosoftはXbox部門で3,200人規模のレイオフと複数スタジオ再編を進行中。その一環でObsidian Entertainmentでも約52名(全体の約1/4)が解雇され、複数プロジェクトが中止された。</t>
+        </is>
+      </c>
+      <c r="E284" s="14" t="inlineStr">
+        <is>
+          <t>Bloomberg報道によれば、社内で順調に進み2027年公開予定だった『Avowed』続編が中止に。ObsidianはJosh Sawyer(Fallout: New Vegas監督)が率いる新作『Fallout』開発へ注力する。MicrosoftはElder Scrolls/Doom/Fallout等の実績IPにスタジオを集中させる方針。</t>
+        </is>
+      </c>
+      <c r="F284" s="14" t="inlineStr">
+        <is>
+          <t>Avowed続編を中止(2027公開予定だった)
+Obsidianで約52名(約1/4)を解雇
+Josh Sawyer主導で新作Fallout開発
+実績IPへの選択と集中</t>
+        </is>
+      </c>
+      <c r="G284" s="14" t="inlineStr">
+        <is>
+          <t>新規IP(Avowed)より確立ブランド(Fallout)を優先する戦略が鮮明化。ファーストパーティは当たるIPに資源集中し、中規模の新規IP育成はサードや独立スタジオへ移る。</t>
+        </is>
+      </c>
+      <c r="H284" s="14" t="inlineStr">
+        <is>
+          <t>プラットフォーマーのIPポートフォリオ選択と集中戦略</t>
+        </is>
+      </c>
+      <c r="I284" s="14" t="inlineStr">
+        <is>
+          <t>Microsoft,Xbox,Obsidian Entertainment,Bethesda</t>
+        </is>
+      </c>
+      <c r="J284" s="14" t="inlineStr">
+        <is>
+          <t>Avowed,Fallout</t>
+        </is>
+      </c>
+      <c r="K284" s="14" t="inlineStr">
+        <is>
+          <t>新作,M&amp;A,海外</t>
+        </is>
+      </c>
+      <c r="L284" s="14" t="n"/>
+    </row>
+    <row r="285">
+      <c r="A285" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B285" s="14" t="inlineStr">
+        <is>
+          <t>ガンホー元システム本部長を背任容疑で逮捕、架空発注で約4,000万円・被害総額は約2.46億円</t>
+        </is>
+      </c>
+      <c r="C285" s="14" t="inlineStr">
+        <is>
+          <t>https://www.itmedia.co.jp/news/articles/2607/08/news098.html</t>
+        </is>
+      </c>
+      <c r="D285" s="14" t="inlineStr">
+        <is>
+          <t>スマホゲーム大手ガンホーは社内調査で経理不正を発見し、元システム本部長の菊池貴則容疑者(48)を2025年7月に懲戒解雇、同10月に告訴。クラウドソーシングを悪用し部下に稟議書を作らせる架空発注の手口が問題視されていた。</t>
+        </is>
+      </c>
+      <c r="E285" s="14" t="inlineStr">
+        <is>
+          <t>警視庁は2026年7月8日、菊池容疑者を背任容疑で逮捕。2022年1〜12月に架空の業務発注で計12回・約4,000万円を自身名義の口座に入金させた疑い。社内では2017〜25年の被害総額が約2.46億円に上るとみられる。</t>
+        </is>
+      </c>
+      <c r="F285" s="14" t="inlineStr">
+        <is>
+          <t>背任容疑で7/8逮捕
+架空発注で約4,000万円を着服
+被害総額は2017〜25年で約2.46億円
+クラウドソーシング悪用・稟議書偽装の手口</t>
+        </is>
+      </c>
+      <c r="G285" s="14" t="inlineStr">
+        <is>
+          <t>外注・業務委託を多用する開発現場での稟議・発注統制の見直しが進む。上場ゲーム各社で経理承認フローの厳格化や内部統制強化が求められる。</t>
+        </is>
+      </c>
+      <c r="H285" s="14" t="inlineStr">
+        <is>
+          <t>ゲーム開発企業の内部統制と外注発注ガバナンス</t>
+        </is>
+      </c>
+      <c r="I285" s="14" t="inlineStr">
+        <is>
+          <t>ガンホー・オンライン・エンターテイメント</t>
+        </is>
+      </c>
+      <c r="J285" s="14" t="n"/>
+      <c r="K285" s="14" t="inlineStr">
+        <is>
+          <t>国内,規制</t>
+        </is>
+      </c>
+      <c r="L285" s="14" t="n"/>
+    </row>
+    <row r="286">
+      <c r="A286" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B286" s="14" t="inlineStr">
+        <is>
+          <t>Krafton、『Subnautica 2』開発元にボーナス支払いで和解——復職したCEOが再び辞任</t>
+        </is>
+      </c>
+      <c r="C286" s="14" t="inlineStr">
+        <is>
+          <t>https://www.bloomberg.com/news/articles/2026-07-01/krafton-agrees-to-pay-subnautica-2-bonuses-as-developer-s-ceo-resigns</t>
+        </is>
+      </c>
+      <c r="D286" s="14" t="inlineStr">
+        <is>
+          <t>2025年、KraftonはUnknown Worldsのテッド・ギルCEOら創業者を解任し『Subnautica 2』を延期。創業者側はボーナス支払い回避が目的の解任だとして提訴し、3月に裁判所がギル氏の復職を命じていた。</t>
+        </is>
+      </c>
+      <c r="E286" s="14" t="inlineStr">
+        <is>
+          <t>Kraftonは子会社Unknown Worlds全社員へのボーナス支払いで和解。復職していたギルCEOは円満合意の上で自ら辞任した。ボーナスは新規入社者も含む全社員へ3回に分けて支払われ、当初条件より増額される。</t>
+        </is>
+      </c>
+      <c r="F286" s="14" t="inlineStr">
+        <is>
+          <t>全社員へのボーナス支払いで和解
+復職CEOテッド・ギル氏が再び辞任
+当初条件より増額・3年分割で支給
+買収先とのアーンアウト/報酬紛争が決着</t>
+        </is>
+      </c>
+      <c r="G286" s="14" t="inlineStr">
+        <is>
+          <t>買収後のアーンアウト(業績連動報酬)や創業者処遇を巡る紛争が可視化され、今後のスタジオ買収契約でクリエイター残留・報酬保護条項の設計が重視される。</t>
+        </is>
+      </c>
+      <c r="H286" s="14" t="inlineStr">
+        <is>
+          <t>スタジオM&amp;Aのアーンアウト条項と創業者リテンション設計</t>
+        </is>
+      </c>
+      <c r="I286" s="14" t="inlineStr">
+        <is>
+          <t>Krafton,Unknown Worlds</t>
+        </is>
+      </c>
+      <c r="J286" s="14" t="inlineStr">
+        <is>
+          <t>Subnautica 2</t>
+        </is>
+      </c>
+      <c r="K286" s="14" t="inlineStr">
+        <is>
+          <t>M&amp;A,海外</t>
+        </is>
+      </c>
+      <c r="L286" s="14" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
weekly-releases + indie + rankings update (2026-07-10 18:13)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -6326,7 +6326,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J62"/>
+  <dimension ref="A1:J82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8566,6 +8566,711 @@
       <c r="J62" t="inlineStr">
         <is>
           <t>6/25開始のサマーセール影響で順位は概算</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-06-29〜07-05</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>1</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>リズム天国 ミラクルスターズ</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Switch</t>
+        </is>
+      </c>
+      <c r="F63" t="n">
+        <v>393378</v>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週間販売数 https://www.famitsu.com/article/202607/80856</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>初登場首位</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-06-29〜07-05</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>2</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>がんばれゴエモン大集合！</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Switch</t>
+        </is>
+      </c>
+      <c r="F64" t="n">
+        <v>60428</v>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週間販売数 https://www.famitsu.com/article/202607/80856</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>初登場</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-06-29〜07-05</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>3</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>トモダチコレクション わくわく生活</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Switch</t>
+        </is>
+      </c>
+      <c r="F65" t="n">
+        <v>26552</v>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週間販売数 https://www.famitsu.com/article/202607/80856</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>前回2位</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-06-29〜07-05</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>4</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>パワフルプロ野球2026-2027</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Switch</t>
+        </is>
+      </c>
+      <c r="F66" t="n">
+        <v>13261</v>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週間販売数 https://www.famitsu.com/article/202607/80856</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>前回3位</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-06-29〜07-05</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>5</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Star Fox（スターフォックス）</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Switch 2</t>
+        </is>
+      </c>
+      <c r="F67" t="n">
+        <v>10388</v>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週間販売数 https://www.famitsu.com/article/202607/80856</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>前回1位</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-06-29〜07-05</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>6</v>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>がんばれゴエモン大集合！</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>PS5</t>
+        </is>
+      </c>
+      <c r="F68" t="n">
+        <v>8773</v>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週間販売数 https://www.famitsu.com/article/202607/80856</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>初登場</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-06-29〜07-05</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>7</v>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>ぽこ あ ポケモン</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Switch 2</t>
+        </is>
+      </c>
+      <c r="F69" t="n">
+        <v>6724</v>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週間販売数 https://www.famitsu.com/article/202607/80856</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>前回5位</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-06-29〜07-05</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>8</v>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>マリオカート ワールド</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Switch 2</t>
+        </is>
+      </c>
+      <c r="F70" t="n">
+        <v>5976</v>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週間販売数 https://www.famitsu.com/article/202607/80856</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>前回6位</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-06-29〜07-05</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>9</v>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>eFootball Kick-Off！</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Switch 2</t>
+        </is>
+      </c>
+      <c r="F71" t="n">
+        <v>5946</v>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週間販売数 https://www.famitsu.com/article/202607/80856</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>前回4位</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-06-29〜07-05</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>10</v>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Minecraft（マインクラフト）</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Switch</t>
+        </is>
+      </c>
+      <c r="F72" t="n">
+        <v>4027</v>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週間販売数 https://www.famitsu.com/article/202607/80856</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>前回10位</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-06-29〜07-05</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>1</v>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>MECCHA CHAMELEON（めっちゃカメレオン）</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>GameGrin/SteamDB Steam週間トップセラー Week28(〜7/5) https://www.gamegrin.com/news/weekly-top-selling-games-on-steam-29th-of-june-to-5th-of-july-2026</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>日本産インディーが継続首位</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-06-29〜07-05</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>2</v>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Cyberpunk 2077（サイバーパンク2077）</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>GameGrin/SteamDB Steam週間トップセラー Week28(〜7/5) https://www.gamegrin.com/news/weekly-top-selling-games-on-steam-29th-of-june-to-5th-of-july-2026</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>累計4,000万本突破と大型セールで再燃</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-06-29〜07-05</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>3</v>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Dead by Daylight（デッドバイデイライト）</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>GameGrin/SteamDB Steam週間トップセラー Week28(〜7/5) https://www.gamegrin.com/news/weekly-top-selling-games-on-steam-29th-of-june-to-5th-of-july-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-06-29〜07-05</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>4</v>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Assassin's Creed Black Flag Resynced（アサシン クリード ブラックフラッグ リシンク）</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>99,451（発売直後ピーク・SteamDB）</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>GameGrin/SteamDB Steam週間トップセラー Week28(〜7/5) https://www.gamegrin.com/news/weekly-top-selling-games-on-steam-29th-of-june-to-5th-of-july-2026</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>予約分含む。発売後は同接99,451</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-06-29〜07-05</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>5</v>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Steam Deck（ハードウェア）</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>ハードウェア</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>GameGrin/SteamDB Steam週間トップセラー Week28(〜7/5) https://www.gamegrin.com/news/weekly-top-selling-games-on-steam-29th-of-june-to-5th-of-july-2026</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>収益ベースのためハード含む</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-06-29〜07-05</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>6</v>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>EA Sports FC 26</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>GameGrin/SteamDB Steam週間トップセラー Week28(〜7/5) https://www.gamegrin.com/news/weekly-top-selling-games-on-steam-29th-of-june-to-5th-of-july-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-06-29〜07-05</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>7</v>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>ARK: Survival Ascended（アーク：サバイバル アセンデッド）</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>GameGrin/SteamDB Steam週間トップセラー Week28(〜7/5) https://www.gamegrin.com/news/weekly-top-selling-games-on-steam-29th-of-june-to-5th-of-july-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-06-29〜07-05</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>8</v>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Grand Theft Auto V Enhanced（GTA5 エンハンスド）</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>GameGrin/SteamDB Steam週間トップセラー Week28(〜7/5) https://www.gamegrin.com/news/weekly-top-selling-games-on-steam-29th-of-june-to-5th-of-july-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-06-29〜07-05</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>9</v>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>The Binding of Isaac: Rebirth</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>GameGrin/SteamDB Steam週間トップセラー Week28(〜7/5) https://www.gamegrin.com/news/weekly-top-selling-games-on-steam-29th-of-june-to-5th-of-july-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-06-29〜07-05</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>10</v>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Red Dead Redemption 2（レッド・デッド・リデンプション2）</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>GameGrin/SteamDB Steam週間トップセラー Week28(〜7/5) https://www.gamegrin.com/news/weekly-top-selling-games-on-steam-29th-of-june-to-5th-of-july-2026</t>
         </is>
       </c>
     </row>
@@ -28286,7 +28991,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M28"/>
+  <dimension ref="A1:M32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -28987,7 +29692,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-07 (日付未定)</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -29015,12 +29720,20 @@
           <t>オープンワールドACT</t>
         </is>
       </c>
+      <c r="G15" t="n">
+        <v>84</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>99,451（GamingBolt/SteamDB, 発売直後ピーク）</t>
+        </is>
+      </c>
       <c r="K15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>『AC4 ブラックフラッグ』の現世代リメイク。7月発売で確定と報道。海洋探索リメイクの本命。来月分（評価系空欄）。</t>
+          <t>発売済。批評は好評(MC84・シリーズ2013年以来の高評価)だが、Steamユーザーは『賛否両論〜やや不評』(約41.5%好評/5.6万件)。カットシーン30fps・マイクロトランザクション・ストーリーカットへの不満が噴出。同接は発売直後に99,451(AC Shadowsの生涯ピーク64,825超)。</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -29516,12 +30229,15 @@
           <t>アクションRPG</t>
         </is>
       </c>
+      <c r="H26" t="n">
+        <v>81</v>
+      </c>
       <c r="K26" t="n">
         <v>4</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>来月予定（評価系空欄）。Switch2版はオンライン/ローカル/クロスプレイ対応。Relinkの大型拡張展開。</t>
+          <t>発売済。OpenCritic『Strong』81(28レビュー)。Steam直近30日で87%好評『非常に好評』。エンドゲームを深化させる大型有料拡張で、ハードコア層に好評だがストーリー面の新規性は限定的との評。買い切り作の“エバーグリーン化”の代表例。</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -29617,6 +30333,186 @@
       <c r="M28" t="inlineStr">
         <is>
           <t>https://www.famitsu.com/schedule</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Outward 2（アウトワード2）</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Nine Dots Studio</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Nine Dots Studio</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>PC(Steam/EGS/GOG)</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>サバイバルアクションRPG</t>
+        </is>
+      </c>
+      <c r="K29" t="n">
+        <v>3</v>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>早期アクセス開始。前作Outwardは高評価(PC Gamer 89%)。あえて“反パワーファンタジー”の硬派サバイバル設計。EA中のため批評スコアは未確定。</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>https://store.steampowered.com/app/2849490/Outward_2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>EA Sports College Football 27</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>EA Sports</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Electronic Arts</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>PS5/Xbox Series X|S</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>スポーツ(アメフト)</t>
+        </is>
+      </c>
+      <c r="K30" t="n">
+        <v>3</v>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>北米カレッジフットボールの年次最新作。国内での話題は限定的だが米市場では定番の大型スポーツタイトル。</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>https://www.metacritic.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>スプラトゥーン レイダース（Splatoon Raiders）</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>任天堂</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>任天堂</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Switch 2</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>三人称アクションADV</t>
+        </is>
+      </c>
+      <c r="K31" t="n">
+        <v>4</v>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>来週〜今月後半予定（評価系空欄）。シリーズ初スピンオフでSwitch 2専用。単独プレイ＋最大4人協力。すりみ連合(シヴァ/フウカ/マンタロー)と遺物探索。</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>https://www.nintendo.com/us/store/products/splatoon-raiders-switch-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>METAL GEAR SOLID: MASTER COLLECTION Vol.2</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>KONAMI</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>KONAMI</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>PS5/Switch 2/Xbox/PC</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>アクション（コレクション）</t>
+        </is>
+      </c>
+      <c r="K32" t="n">
+        <v>3</v>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>来月予定（評価系空欄）。MGSシリーズをまとめたマスターコレクション第2弾のボーナスコンテンツ含む展開。</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/schedule/all-platforms/202608</t>
         </is>
       </c>
     </row>
@@ -33950,7 +34846,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -34434,6 +35330,100 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>にゃんこ郵便局（Nyanko Post Office）</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>小規模インディー（日本）</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2026-07-10 配信</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>癒し系仕分けシミュレーション</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>静かな島の郵便局で船で届く荷物を仕分けて経営を立て直す。制限時間・ペナルティなしで自分のペースで遊べる“癒し系”。低価格×まったり設計でSNS・実況で言及増。</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>配信初日で注目インディーとして各メディアが紹介(公式値は追跡中)。</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Indie Freaks 7月注目インディー10本で紹介。コージー/クリッカー的な短尺癒し系の系譜。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Tears of Metal（ティアーズ・オブ・メタル）</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>小規模インディー（独立系）</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2026-07-23 早期アクセス開始予定</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>協力型ローグライク・ハック&amp;スラッシュ</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>中世を舞台にした最大協力プレイのハクスラ・ローグライク。多人数で敵の大群を薙ぎ倒す設計が配信向き。EA開始前からウィッシュリスト増。</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>早期アクセス前のため実績値は限定的・要追跡。</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>協力ハクスラ×ローグライクの掛け合わせ。7月注目インディーとして複数メディアで言及。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
daily-news + cross-questions + events + predictions + game-design update (2026-07-11)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -816,7 +816,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1824,6 +1824,43 @@
       <c r="G27" s="14" t="inlineStr">
         <is>
           <t>今後発表されるゲームスタジオ買収案件で、アーンアウト/報酬エスクロー/キーマン残留条項の開示有無を観測する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B28" s="14" t="inlineStr">
+        <is>
+          <t>コカ・コーラ×ポケモンGOを皮切りに、位置情報ゲームが『スポンサードPoI(有料スポット)』を商品化し、コンビニ・外食・鉄道など他チェーンが追随。ナイアンティック等の収益がアプリ内課金から『O2O送客広告』へ多角化する。</t>
+        </is>
+      </c>
+      <c r="C28" s="14" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="D28" s="14" t="inlineStr">
+        <is>
+          <t>6〜12ヶ月</t>
+        </is>
+      </c>
+      <c r="E28" s="14" t="inlineStr">
+        <is>
+          <t>ナイアンティック,ポケモン,日本コカ・コーラ</t>
+        </is>
+      </c>
+      <c r="F28" s="14" t="inlineStr">
+        <is>
+          <t>日本コカ・コーラ、『ポケモンGO』と提携・約3万台の自販機がポケストップ化(4Gamer,2026-07-10)</t>
+        </is>
+      </c>
+      <c r="G28" s="14" t="inlineStr">
+        <is>
+          <t>別の小売/外食/交通チェーンとの同種スポンサード提携が追加発表されるか、ナイアンティック/Scopelyが位置情報スポンサー収益を開示・強調するかを観測。</t>
         </is>
       </c>
     </row>
@@ -3861,7 +3898,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G66"/>
+  <dimension ref="A1:G67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6312,6 +6349,43 @@
       <c r="G66" s="14" t="inlineStr">
         <is>
           <t>買収は『クロージング』より『アーンアウト期間中の統治』が火種。創業者の報酬保護は業界横断の設計課題。</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B67" s="14" t="inlineStr">
+        <is>
+          <t>位置情報ゲームのMAUを『実店舗・自販機への送客インフラ(O2O)』として外部業界が組み込む動きは、飲料・小売・不動産の集客/広告投資の受け皿になるか？</t>
+        </is>
+      </c>
+      <c r="C67" s="14" t="inlineStr">
+        <is>
+          <t>日本コカ・コーラ×『ポケモンGO』提携(約3万台の自販機をポケストップ/ジム化)</t>
+        </is>
+      </c>
+      <c r="D67" s="14" t="inlineStr">
+        <is>
+          <t>ナイアンティック,ポケモン,日本コカ・コーラ</t>
+        </is>
+      </c>
+      <c r="E67" s="14" t="inlineStr">
+        <is>
+          <t>飲料・小売・自販機/OOH・屋外広告/商業不動産・店舗集客/観光・地域送客</t>
+        </is>
+      </c>
+      <c r="F67" s="14" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="G67" s="14" t="inlineStr">
+        <is>
+          <t>『広告枠』ではなく『来店導線(足を運ばせる力)』そのものを売る。ゲームのMAUが位置情報×購買データを介して集客インフラ化する。</t>
         </is>
       </c>
     </row>
@@ -10391,12 +10465,12 @@
       </c>
       <c r="I22" s="14" t="inlineStr">
         <is>
-          <t>開催予定</t>
+          <t>開催中</t>
         </is>
       </c>
       <c r="J22" s="14" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-07-11</t>
         </is>
       </c>
     </row>
@@ -11081,7 +11155,7 @@
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
@@ -11116,12 +11190,12 @@
       </c>
       <c r="H12" s="14" t="inlineStr">
         <is>
-          <t>外部IP連携に加え「自社IP同士の社内クロスオーバー」（カプコン：バイオ×モンハン）へ拡張。許諾コストが低い自社IP回遊型は他社も追随しやすく、運営型の標準装備化が進む。 格闘ゲームでも外部IPゲストキャラを継続運営フックにする商法が定着。</t>
+          <t>ジャンル・地域を越えた他社IPコラボが集客の標準手段として定着。単発の話題づくりから、IP同士の相互送客・ファン交換を狙う設計へ高度化が進む。過熱による飽和・費用対効果の見極めが次の論点。</t>
         </is>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
-          <t>『BIOHAZARD Survival Unit』×『モンスターハンター』コラボ開始（4Gamer, 7/3日次）／『NIKKE』新章配信（4Gamer, 7/2）／『荒野行動』×エヴァコラボ第8弾（4Gamer, 7/4）／崩壊：スターレイル×Fateコラボ第2弾（7/4日次）／『GGST』SP5に新ゲストキャラ参戦発表(4Gamer, 7/5日次)</t>
+          <t>『リバース：1999』×Atomic Heart(7/23)、『アークナイツ：エンドフィールド』×フォートナイト/GiGO(4Gamer,2026-07-10/11)</t>
         </is>
       </c>
       <c r="J12" s="14" t="n">
@@ -11239,7 +11313,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L286"/>
+  <dimension ref="A1:L291"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -28979,6 +29053,316 @@
         </is>
       </c>
       <c r="L286" s="14" t="n"/>
+    </row>
+    <row r="287">
+      <c r="A287" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B287" s="14" t="inlineStr">
+        <is>
+          <t>JOGA市場レポート2026、25年国内オンラインゲーム市場9899億円・開発現場の生成AI活用率100%</t>
+        </is>
+      </c>
+      <c r="C287" s="14" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/article/202607/80926</t>
+        </is>
+      </c>
+      <c r="D287" s="14" t="inlineStr">
+        <is>
+          <t>日本オンラインゲーム協会(JOGA)が毎年発行する市場調査レポートの2026年版が7/10発売。国内オンラインゲーム市場規模や開発現場の実態、生成AI導入状況、ユーザー意識をまとめた業界の定点観測資料。</t>
+        </is>
+      </c>
+      <c r="E287" s="14" t="inlineStr">
+        <is>
+          <t>2025年の国内オンラインゲーム市場は9899億円。開発・運営現場での生成AIツール活用率は100%に達し、ツール別ではGemini94%・Claude84%・GitHub Copilot76%。1タイトル平均運営スタッフ数は10年前の4.6倍の37人に増加した。</t>
+        </is>
+      </c>
+      <c r="F287" s="14" t="inlineStr">
+        <is>
+          <t>生成AI活用率が現場で100%到達
+ツール別トップはGemini、次いでClaude・Copilot
+委ねたい業務は嗜好性分析・行動予測が最多
+ユーザー側は著作権侵害・同質化を懸念
+運営人員は10年で4.6倍に肥大</t>
+        </is>
+      </c>
+      <c r="G287" s="14" t="inlineStr">
+        <is>
+          <t>生成AIは既に前提技術化し、今後は『どの業務をどのAIに任せるか』の設計・運用ノウハウが競争軸に。一方でユーザーの著作権・同質化懸念に応える開示や差別化が運営の必須要件になる。</t>
+        </is>
+      </c>
+      <c r="H287" s="14" t="inlineStr">
+        <is>
+          <t>生成AIの運用設計とゲーム運営コスト構造</t>
+        </is>
+      </c>
+      <c r="I287" s="14" t="inlineStr">
+        <is>
+          <t>日本オンラインゲーム協会(JOGA),Google,Anthropic,GitHub</t>
+        </is>
+      </c>
+      <c r="J287" s="14" t="inlineStr">
+        <is>
+          <t>オンラインゲーム市場全般</t>
+        </is>
+      </c>
+      <c r="K287" s="14" t="inlineStr">
+        <is>
+          <t>業績,技術,国内</t>
+        </is>
+      </c>
+      <c r="L287" s="14" t="inlineStr"/>
+    </row>
+    <row r="288">
+      <c r="A288" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B288" s="14" t="inlineStr">
+        <is>
+          <t>日本コカ・コーラ、『ポケモンGO』と提携——全国約3万台の自販機がポケストップ/ジム化</t>
+        </is>
+      </c>
+      <c r="C288" s="14" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/316/G031663/20260710050/</t>
+        </is>
+      </c>
+      <c r="D288" s="14" t="inlineStr">
+        <is>
+          <t>位置情報ゲーム『ポケモンGO』(ナイアンティック/ポケモン)と日本コカ・コーラが7/10にパートナーシップを締結。ともに10周年を迎えるアプリ『Coke ON』とGOを連動させ、飲料の購買行動とゲーム内行動を接続する。</t>
+        </is>
+      </c>
+      <c r="E288" s="14" t="inlineStr">
+        <is>
+          <t>日本全国約3万台のコカ・コーラ自販機が順次GO内の『ポケストップ』として登場し、一部は『ジム』にもなる。9月にはCoke ONでの製品購入者にGOオリジナルスタンプを配布する記念キャンペーンを実施予定。</t>
+        </is>
+      </c>
+      <c r="F288" s="14" t="inlineStr">
+        <is>
+          <t>約3万台の自販機をゲーム内スポット化
+一部自販機はバトル拠点『ジム』に
+Coke ON購買とゲーム内特典を連動
+両サービス10周年の共同企画
+半年ぶりに自販機ポケストップが復活</t>
+        </is>
+      </c>
+      <c r="G288" s="14" t="inlineStr">
+        <is>
+          <t>ゲームのMAUを『実店舗・自販機への送客インフラ』として使う動きが強まる。飲料・小売・OOH各社がスポンサードPoI(スポット)枠を求め、位置情報ゲームの収益が課金からO2O集客・広告へ多角化する可能性。</t>
+        </is>
+      </c>
+      <c r="H288" s="14" t="inlineStr">
+        <is>
+          <t>位置情報ゲームのO2O送客とスポンサードPoI</t>
+        </is>
+      </c>
+      <c r="I288" s="14" t="inlineStr">
+        <is>
+          <t>日本コカ・コーラ,ナイアンティック,ポケモン</t>
+        </is>
+      </c>
+      <c r="J288" s="14" t="inlineStr">
+        <is>
+          <t>Pokémon GO,Coke ON</t>
+        </is>
+      </c>
+      <c r="K288" s="14" t="inlineStr">
+        <is>
+          <t>提携,国内</t>
+        </is>
+      </c>
+      <c r="L288" s="14" t="inlineStr"/>
+    </row>
+    <row r="289">
+      <c r="A289" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B289" s="14" t="inlineStr">
+        <is>
+          <t>NetEaseのサバイバルMMO『Once Human』、8/25にPS5/Xbox版配信——一人称視点追加・フルクロスプレイ対応</t>
+        </is>
+      </c>
+      <c r="C289" s="14" t="inlineStr">
+        <is>
+          <t>https://www.neteasegames.com/news/20260710/37000_1307198.html</t>
+        </is>
+      </c>
+      <c r="D289" s="14" t="inlineStr">
+        <is>
+          <t>NetEase傘下Starry Studioの基本無料サバイバルMMO『Once Human』は24年のPC版から拡大を続けており、7/10にコンソール展開の詳細を発表。PC/コンソール間のクロスプレイ・クロスプログレッションを実現する。</t>
+        </is>
+      </c>
+      <c r="E289" s="14" t="inlineStr">
+        <is>
+          <t>PS5とXbox Series X|S版を8/25に配信。従来の三人称に加え一人称視点を実装し、画質モードは4K/60fps、パフォーマンスモードは最大120fps。6シナリオ＋PvPスピンオフを同梱し300時間超のコンテンツを用意する。</t>
+        </is>
+      </c>
+      <c r="F289" s="14" t="inlineStr">
+        <is>
+          <t>PS5/Xbox版を8/25グローバル配信
+PC/コンソール完全クロスプレイ・進行共有
+新規に一人称視点を追加
+最大120fpsのパフォーマンスモード
+300時間超・基本無料で参入障壁を低減</t>
+        </is>
+      </c>
+      <c r="G289" s="14" t="inlineStr">
+        <is>
+          <t>基本無料サバイバルMMOのマルチプラットフォーム・クロスプレイ化がさらに進み、コンソール勢を取り込む競争が激化。ライブサービス型サバイバルの新規流入をどうLTVに変えるかが各社の焦点になる。</t>
+        </is>
+      </c>
+      <c r="H289" s="14" t="inlineStr">
+        <is>
+          <t>クロスプレイ設計とF2Pサバイバルの収益化</t>
+        </is>
+      </c>
+      <c r="I289" s="14" t="inlineStr">
+        <is>
+          <t>NetEase,Starry Studio</t>
+        </is>
+      </c>
+      <c r="J289" s="14" t="inlineStr">
+        <is>
+          <t>Once Human</t>
+        </is>
+      </c>
+      <c r="K289" s="14" t="inlineStr">
+        <is>
+          <t>新作,海外</t>
+        </is>
+      </c>
+      <c r="L289" s="14" t="inlineStr"/>
+    </row>
+    <row r="290">
+      <c r="A290" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B290" s="14" t="inlineStr">
+        <is>
+          <t>『リバース：1999』×『Atomic Heart』コラボを7/23実装——中国発RPGが海外PC/コンソールIPと相互送客</t>
+        </is>
+      </c>
+      <c r="C290" s="14" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/724/G072407/20260711001/</t>
+        </is>
+      </c>
+      <c r="D290" s="14" t="inlineStr">
+        <is>
+          <t>BLUEPOCHのタイムリバースRPG『リバース：1999』が、Mundfishのシューター『Atomic Heart』とのコラボを7/11告知。異なるジャンル・地域のIP同士を掛け合わせたライブサービス運営の一環。</t>
+        </is>
+      </c>
+      <c r="E290" s="14" t="inlineStr">
+        <is>
+          <t>7/23にコラボバージョンを実装し、新キャラクター『双子』『ノラ』が登場。月間パス『咆哮の祝祭』やログインイベント等を展開する。基本無料スマホRPGが海外の買い切り系IPを取り込む形。</t>
+        </is>
+      </c>
+      <c r="F290" s="14" t="inlineStr">
+        <is>
+          <t>7/23にコラボ版を実装
+新キャラ2体を追加
+月パス・ログインイベントで回遊促進
+スマホRPG×海外シューターIPの越境コラボ
+Mundfishブランドの認知を相互活用</t>
+        </is>
+      </c>
+      <c r="G290" s="14" t="inlineStr">
+        <is>
+          <t>ジャンル・地域をまたぐ他社IPコラボがライブサービスの標準的な集客手段として定着。単発の話題づくりから、IP同士の相互送客・ファン交換を狙う設計へと運営が高度化する。</t>
+        </is>
+      </c>
+      <c r="H290" s="14" t="inlineStr">
+        <is>
+          <t>越境IPコラボによるライブオプス設計</t>
+        </is>
+      </c>
+      <c r="I290" s="14" t="inlineStr">
+        <is>
+          <t>BLUEPOCH,Mundfish</t>
+        </is>
+      </c>
+      <c r="J290" s="14" t="inlineStr">
+        <is>
+          <t>リバース：1999,Atomic Heart</t>
+        </is>
+      </c>
+      <c r="K290" s="14" t="inlineStr">
+        <is>
+          <t>新作,国内,海外</t>
+        </is>
+      </c>
+      <c r="L290" s="14" t="inlineStr"/>
+    </row>
+    <row r="291">
+      <c r="A291" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B291" s="14" t="inlineStr">
+        <is>
+          <t>『アークナイツ：エンドフィールド』7/16に武陵決戦篇『向淵行』配信——GiGO・フォートナイトコラボも決定</t>
+        </is>
+      </c>
+      <c r="C291" s="14" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/622/G062211/20260710052/</t>
+        </is>
+      </c>
+      <c r="D291" s="14" t="inlineStr">
+        <is>
+          <t>GRYPHLINEの3DリアルタイムストラテジーアクションRPG『アークナイツ：エンドフィールド』が7/10、ハーフアニバーサリーに向けた大型アップデートを予告。人気IP『アークナイツ』の3D新作として展開中。</t>
+        </is>
+      </c>
+      <c r="E291" s="14" t="inlineStr">
+        <is>
+          <t>7/16に武陵決戦篇コアバージョン『向淵行』を配信。過去最大の新マップ『応龍関』等を追加し新オペレーター『オクギ』『リーノ』を実装、メイン任務先行解放で復帰・入門障壁を緩和。GiGO・フォートナイトとのコラボも決定した。</t>
+        </is>
+      </c>
+      <c r="F291" s="14" t="inlineStr">
+        <is>
+          <t>7/16に大型バージョン『向淵行』配信
+過去最大規模の新マップを追加
+新オペレーター2体を実装
+メイン任務先行解放で入門障壁を緩和
+GiGO・フォートナイトコラボを予告</t>
+        </is>
+      </c>
+      <c r="G291" s="14" t="inlineStr">
+        <is>
+          <t>人気2D IPの3D展開作がハーフアニバーサリーで入門障壁緩和とコラボを同時投入。既存ファン維持と新規/復帰獲得を両立させる運営設計が、中国発大型タイトルの定石として続く。</t>
+        </is>
+      </c>
+      <c r="H291" s="14" t="inlineStr">
+        <is>
+          <t>IP横展開(2D→3D)とライブ運営の新規獲得設計</t>
+        </is>
+      </c>
+      <c r="I291" s="14" t="inlineStr">
+        <is>
+          <t>GRYPHLINE,Epic Games,GiGO</t>
+        </is>
+      </c>
+      <c r="J291" s="14" t="inlineStr">
+        <is>
+          <t>アークナイツ：エンドフィールド</t>
+        </is>
+      </c>
+      <c r="K291" s="14" t="inlineStr">
+        <is>
+          <t>新作,海外</t>
+        </is>
+      </c>
+      <c r="L291" s="14" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
design-map: representative titles on nodes + unified lineage genealogy (Section C); rebuilt on latest xlsx (incl. 2026-07-11 news)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -23,6 +23,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="週間ランキング" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="イベントカレンダー" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ゲームデザイン・トレンド" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="デザイン派生系統" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -11307,6 +11308,1271 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G40"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>系統名</t>
+        </is>
+      </c>
+      <c r="B1" s="14" t="inlineStr">
+        <is>
+          <t>年</t>
+        </is>
+      </c>
+      <c r="C1" s="14" t="inlineStr">
+        <is>
+          <t>ノード(タイトル/技術)</t>
+        </is>
+      </c>
+      <c r="D1" s="14" t="inlineStr">
+        <is>
+          <t>種別</t>
+        </is>
+      </c>
+      <c r="E1" s="14" t="inlineStr">
+        <is>
+          <t>派生元</t>
+        </is>
+      </c>
+      <c r="F1" s="14" t="inlineStr">
+        <is>
+          <t>現行型</t>
+        </is>
+      </c>
+      <c r="G1" s="14" t="inlineStr">
+        <is>
+          <t>メモ</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="14" t="inlineStr">
+        <is>
+          <t>対話型AI系</t>
+        </is>
+      </c>
+      <c r="B2" s="14" t="n">
+        <v>2000</v>
+      </c>
+      <c r="C2" s="14" t="inlineStr">
+        <is>
+          <t>The Sims</t>
+        </is>
+      </c>
+      <c r="D2" s="14" t="inlineStr">
+        <is>
+          <t>祖先</t>
+        </is>
+      </c>
+      <c r="E2" s="14" t="inlineStr"/>
+      <c r="F2" s="14" t="inlineStr"/>
+      <c r="G2" s="14" t="inlineStr">
+        <is>
+          <t>シムの疑似感情・自律行動NPC。エージェント的NPCの原型</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="14" t="inlineStr">
+        <is>
+          <t>対話型AI系</t>
+        </is>
+      </c>
+      <c r="B3" s="14" t="n">
+        <v>2005</v>
+      </c>
+      <c r="C3" s="14" t="inlineStr">
+        <is>
+          <t>Façade</t>
+        </is>
+      </c>
+      <c r="D3" s="14" t="inlineStr">
+        <is>
+          <t>発展</t>
+        </is>
+      </c>
+      <c r="E3" s="14" t="inlineStr">
+        <is>
+          <t>The Sims</t>
+        </is>
+      </c>
+      <c r="F3" s="14" t="inlineStr"/>
+      <c r="G3" s="14" t="inlineStr">
+        <is>
+          <t>自然言語入力の対話型インタラクティブドラマ</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>対話型AI系</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>AI Dungeon</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>発展</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>Façade</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="inlineStr"/>
+      <c r="G4" s="14" t="inlineStr">
+        <is>
+          <t>LLM(GPT)による無限生成テキストアドベンチャー</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>対話型AI系</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C5" s="14" t="inlineStr">
+        <is>
+          <t>Suck Up!</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="inlineStr">
+        <is>
+          <t>確立</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="inlineStr">
+        <is>
+          <t>AI Dungeon</t>
+        </is>
+      </c>
+      <c r="F5" s="14" t="inlineStr"/>
+      <c r="G5" s="14" t="inlineStr">
+        <is>
+          <t>LLM NPCを言葉で説得する対話ゲーム。実用化の先行例</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>対話型AI系</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>NVIDIA ACE</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>確立</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>AI Dungeon</t>
+        </is>
+      </c>
+      <c r="F6" s="14" t="inlineStr"/>
+      <c r="G6" s="14" t="inlineStr">
+        <is>
+          <t>オンデバイス音声AI NPC基盤。PUBG/Total War等で実装</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>対話型AI系</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C7" s="14" t="inlineStr">
+        <is>
+          <t>対話型AI NPC（各社実装）</t>
+        </is>
+      </c>
+      <c r="D7" s="14" t="inlineStr">
+        <is>
+          <t>現在(型)</t>
+        </is>
+      </c>
+      <c r="E7" s="14" t="inlineStr">
+        <is>
+          <t>Suck Up!,NVIDIA ACE</t>
+        </is>
+      </c>
+      <c r="F7" s="14" t="inlineStr">
+        <is>
+          <t>対話型AI NPC／AIコンパニオン</t>
+        </is>
+      </c>
+      <c r="G7" s="14" t="inlineStr">
+        <is>
+          <t>LLM＋音声でNPCが記憶・即応。台頭フェーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>ローグ系</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="n">
+        <v>1980</v>
+      </c>
+      <c r="C8" s="14" t="inlineStr">
+        <is>
+          <t>Rogue</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>祖先</t>
+        </is>
+      </c>
+      <c r="E8" s="14" t="inlineStr"/>
+      <c r="F8" s="14" t="inlineStr"/>
+      <c r="G8" s="14" t="inlineStr">
+        <is>
+          <t>パーマデス＋自動生成ダンジョンの始祖</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>ローグ系</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="n">
+        <v>2008</v>
+      </c>
+      <c r="C9" s="14" t="inlineStr">
+        <is>
+          <t>Spelunky</t>
+        </is>
+      </c>
+      <c r="D9" s="14" t="inlineStr">
+        <is>
+          <t>発展</t>
+        </is>
+      </c>
+      <c r="E9" s="14" t="inlineStr">
+        <is>
+          <t>Rogue</t>
+        </is>
+      </c>
+      <c r="F9" s="14" t="inlineStr"/>
+      <c r="G9" s="14" t="inlineStr">
+        <is>
+          <t>自動生成アクションでローグライトを大衆化</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>ローグ系</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="n">
+        <v>2011</v>
+      </c>
+      <c r="C10" s="14" t="inlineStr">
+        <is>
+          <t>The Binding of Isaac</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>発展</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="inlineStr">
+        <is>
+          <t>Spelunky</t>
+        </is>
+      </c>
+      <c r="F10" s="14" t="inlineStr"/>
+      <c r="G10" s="14" t="inlineStr">
+        <is>
+          <t>ビルド構築×反復プレイでインディー定番化</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>ローグ系</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="n">
+        <v>2017</v>
+      </c>
+      <c r="C11" s="14" t="inlineStr">
+        <is>
+          <t>Dead Cells</t>
+        </is>
+      </c>
+      <c r="D11" s="14" t="inlineStr">
+        <is>
+          <t>確立</t>
+        </is>
+      </c>
+      <c r="E11" s="14" t="inlineStr">
+        <is>
+          <t>Spelunky</t>
+        </is>
+      </c>
+      <c r="F11" s="14" t="inlineStr"/>
+      <c r="G11" s="14" t="inlineStr">
+        <is>
+          <t>メトロヴァニア×ローグライトの完成度</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>ローグ系</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>Hades</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>確立</t>
+        </is>
+      </c>
+      <c r="E12" s="14" t="inlineStr">
+        <is>
+          <t>The Binding of Isaac</t>
+        </is>
+      </c>
+      <c r="F12" s="14" t="inlineStr"/>
+      <c r="G12" s="14" t="inlineStr">
+        <is>
+          <t>物語統合で賞を席巻、ジャンルを主流化</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="14" t="inlineStr">
+        <is>
+          <t>ローグ系</t>
+        </is>
+      </c>
+      <c r="B13" s="14" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>Balatro</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>現在(型)</t>
+        </is>
+      </c>
+      <c r="E13" s="14" t="inlineStr">
+        <is>
+          <t>Hades,Dead Cells</t>
+        </is>
+      </c>
+      <c r="F13" s="14" t="inlineStr">
+        <is>
+          <t>ローグライト／ローグライク</t>
+        </is>
+      </c>
+      <c r="G13" s="14" t="inlineStr">
+        <is>
+          <t>カード×ローグライトの大ヒット。掛け合わせで再活性</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="inlineStr">
+        <is>
+          <t>抽出/PvPvE系</t>
+        </is>
+      </c>
+      <c r="B14" s="14" t="n">
+        <v>2012</v>
+      </c>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>DayZ (Mod)</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>祖先</t>
+        </is>
+      </c>
+      <c r="E14" s="14" t="inlineStr"/>
+      <c r="F14" s="14" t="inlineStr"/>
+      <c r="G14" s="14" t="inlineStr">
+        <is>
+          <t>オープンワールド・サバイバルPvPの原型</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="14" t="inlineStr">
+        <is>
+          <t>抽出/PvPvE系</t>
+        </is>
+      </c>
+      <c r="B15" s="14" t="n">
+        <v>2017</v>
+      </c>
+      <c r="C15" s="14" t="inlineStr">
+        <is>
+          <t>Escape from Tarkov</t>
+        </is>
+      </c>
+      <c r="D15" s="14" t="inlineStr">
+        <is>
+          <t>確立</t>
+        </is>
+      </c>
+      <c r="E15" s="14" t="inlineStr">
+        <is>
+          <t>DayZ,Rogue</t>
+        </is>
+      </c>
+      <c r="F15" s="14" t="inlineStr"/>
+      <c r="G15" s="14" t="inlineStr">
+        <is>
+          <t>高リスクの抽出(持ち出し)戦を確立。パーマデス的緊張</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>抽出/PvPvE系</t>
+        </is>
+      </c>
+      <c r="B16" s="14" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C16" s="14" t="inlineStr">
+        <is>
+          <t>Hunt: Showdown</t>
+        </is>
+      </c>
+      <c r="D16" s="14" t="inlineStr">
+        <is>
+          <t>発展</t>
+        </is>
+      </c>
+      <c r="E16" s="14" t="inlineStr">
+        <is>
+          <t>DayZ</t>
+        </is>
+      </c>
+      <c r="F16" s="14" t="inlineStr"/>
+      <c r="G16" s="14" t="inlineStr">
+        <is>
+          <t>抽出シューターをコンソールへ拡張</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>抽出/PvPvE系</t>
+        </is>
+      </c>
+      <c r="B17" s="14" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C17" s="14" t="inlineStr">
+        <is>
+          <t>抽出シューター各作（過熱）</t>
+        </is>
+      </c>
+      <c r="D17" s="14" t="inlineStr">
+        <is>
+          <t>現在(型)</t>
+        </is>
+      </c>
+      <c r="E17" s="14" t="inlineStr">
+        <is>
+          <t>Escape from Tarkov</t>
+        </is>
+      </c>
+      <c r="F17" s="14" t="inlineStr">
+        <is>
+          <t>エクストラクションシューター</t>
+        </is>
+      </c>
+      <c r="G17" s="14" t="inlineStr">
+        <is>
+          <t>参入過多で過熱→再評価フェーズへ</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>MMO→GaaS系</t>
+        </is>
+      </c>
+      <c r="B18" s="14" t="n">
+        <v>1997</v>
+      </c>
+      <c r="C18" s="14" t="inlineStr">
+        <is>
+          <t>Ultima Online</t>
+        </is>
+      </c>
+      <c r="D18" s="14" t="inlineStr">
+        <is>
+          <t>祖先</t>
+        </is>
+      </c>
+      <c r="E18" s="14" t="inlineStr"/>
+      <c r="F18" s="14" t="inlineStr"/>
+      <c r="G18" s="14" t="inlineStr">
+        <is>
+          <t>課金制MMOの商業的成立</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="14" t="inlineStr">
+        <is>
+          <t>MMO→GaaS系</t>
+        </is>
+      </c>
+      <c r="B19" s="14" t="n">
+        <v>2004</v>
+      </c>
+      <c r="C19" s="14" t="inlineStr">
+        <is>
+          <t>World of Warcraft</t>
+        </is>
+      </c>
+      <c r="D19" s="14" t="inlineStr">
+        <is>
+          <t>発展</t>
+        </is>
+      </c>
+      <c r="E19" s="14" t="inlineStr">
+        <is>
+          <t>Ultima Online</t>
+        </is>
+      </c>
+      <c r="F19" s="14" t="inlineStr"/>
+      <c r="G19" s="14" t="inlineStr">
+        <is>
+          <t>サブスクMMOの黄金期を築く</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>MMO→GaaS系</t>
+        </is>
+      </c>
+      <c r="B20" s="14" t="n">
+        <v>2009</v>
+      </c>
+      <c r="C20" s="14" t="inlineStr">
+        <is>
+          <t>League of Legends</t>
+        </is>
+      </c>
+      <c r="D20" s="14" t="inlineStr">
+        <is>
+          <t>確立</t>
+        </is>
+      </c>
+      <c r="E20" s="14" t="inlineStr">
+        <is>
+          <t>World of Warcraft</t>
+        </is>
+      </c>
+      <c r="F20" s="14" t="inlineStr"/>
+      <c r="G20" s="14" t="inlineStr">
+        <is>
+          <t>F2P＋継続運営(ライブサービス)の型</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t>MMO→GaaS系</t>
+        </is>
+      </c>
+      <c r="B21" s="14" t="n">
+        <v>2017</v>
+      </c>
+      <c r="C21" s="14" t="inlineStr">
+        <is>
+          <t>Fortnite</t>
+        </is>
+      </c>
+      <c r="D21" s="14" t="inlineStr">
+        <is>
+          <t>確立</t>
+        </is>
+      </c>
+      <c r="E21" s="14" t="inlineStr">
+        <is>
+          <t>League of Legends</t>
+        </is>
+      </c>
+      <c r="F21" s="14" t="inlineStr"/>
+      <c r="G21" s="14" t="inlineStr">
+        <is>
+          <t>バトルパス×シーズン運営でGaaSを標準化</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="14" t="inlineStr">
+        <is>
+          <t>MMO→GaaS系</t>
+        </is>
+      </c>
+      <c r="B22" s="14" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C22" s="14" t="inlineStr">
+        <is>
+          <t>Genshin Impact</t>
+        </is>
+      </c>
+      <c r="D22" s="14" t="inlineStr">
+        <is>
+          <t>確立</t>
+        </is>
+      </c>
+      <c r="E22" s="14" t="inlineStr">
+        <is>
+          <t>Fortnite</t>
+        </is>
+      </c>
+      <c r="F22" s="14" t="inlineStr"/>
+      <c r="G22" s="14" t="inlineStr">
+        <is>
+          <t>ガチャ×オープンワールドのGaaSを世界規模に</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="14" t="inlineStr">
+        <is>
+          <t>MMO→GaaS系</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C23" s="14" t="inlineStr">
+        <is>
+          <t>ライブサービス／GaaS（選別・逆風）</t>
+        </is>
+      </c>
+      <c r="D23" s="14" t="inlineStr">
+        <is>
+          <t>現在(型)</t>
+        </is>
+      </c>
+      <c r="E23" s="14" t="inlineStr">
+        <is>
+          <t>Fortnite,Genshin Impact</t>
+        </is>
+      </c>
+      <c r="F23" s="14" t="inlineStr">
+        <is>
+          <t>ライブサービス／GaaS</t>
+        </is>
+      </c>
+      <c r="G23" s="14" t="inlineStr">
+        <is>
+          <t>大量終了・投資縮小で成熟→選別フェーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="14" t="inlineStr">
+        <is>
+          <t>買い切りエバーグリーン系</t>
+        </is>
+      </c>
+      <c r="B24" s="14" t="n">
+        <v>2016</v>
+      </c>
+      <c r="C24" s="14" t="inlineStr">
+        <is>
+          <t>The Witcher 3: Blood and Wine</t>
+        </is>
+      </c>
+      <c r="D24" s="14" t="inlineStr">
+        <is>
+          <t>祖先</t>
+        </is>
+      </c>
+      <c r="E24" s="14" t="inlineStr"/>
+      <c r="F24" s="14" t="inlineStr"/>
+      <c r="G24" s="14" t="inlineStr">
+        <is>
+          <t>大型有料拡張で買い切りを長寿命化した先例</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="14" t="inlineStr">
+        <is>
+          <t>買い切りエバーグリーン系</t>
+        </is>
+      </c>
+      <c r="B25" s="14" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C25" s="14" t="inlineStr">
+        <is>
+          <t>Elden Ring</t>
+        </is>
+      </c>
+      <c r="D25" s="14" t="inlineStr">
+        <is>
+          <t>発展</t>
+        </is>
+      </c>
+      <c r="E25" s="14" t="inlineStr">
+        <is>
+          <t>The Witcher 3: Blood and Wine</t>
+        </is>
+      </c>
+      <c r="F25" s="14" t="inlineStr"/>
+      <c r="G25" s="14" t="inlineStr">
+        <is>
+          <t>買い切り大作の世界的大ヒット</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="14" t="inlineStr">
+        <is>
+          <t>買い切りエバーグリーン系</t>
+        </is>
+      </c>
+      <c r="B26" s="14" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C26" s="14" t="inlineStr">
+        <is>
+          <t>Cyberpunk 2077: Phantom Liberty</t>
+        </is>
+      </c>
+      <c r="D26" s="14" t="inlineStr">
+        <is>
+          <t>確立</t>
+        </is>
+      </c>
+      <c r="E26" s="14" t="inlineStr">
+        <is>
+          <t>The Witcher 3: Blood and Wine</t>
+        </is>
+      </c>
+      <c r="F26" s="14" t="inlineStr"/>
+      <c r="G26" s="14" t="inlineStr">
+        <is>
+          <t>無料大型UP＋有料拡張で準ライブ運営化・復活</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="14" t="inlineStr">
+        <is>
+          <t>買い切りエバーグリーン系</t>
+        </is>
+      </c>
+      <c r="B27" s="14" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C27" s="14" t="inlineStr">
+        <is>
+          <t>Elden Ring: Shadow of the Erdtree</t>
+        </is>
+      </c>
+      <c r="D27" s="14" t="inlineStr">
+        <is>
+          <t>確立</t>
+        </is>
+      </c>
+      <c r="E27" s="14" t="inlineStr">
+        <is>
+          <t>Elden Ring</t>
+        </is>
+      </c>
+      <c r="F27" s="14" t="inlineStr"/>
+      <c r="G27" s="14" t="inlineStr">
+        <is>
+          <t>単体拡張で大規模セールス。エバーグリーン化の象徴</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="14" t="inlineStr">
+        <is>
+          <t>買い切りエバーグリーン系</t>
+        </is>
+      </c>
+      <c r="B28" s="14" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C28" s="14" t="inlineStr">
+        <is>
+          <t>買い切り大作のエバーグリーン化</t>
+        </is>
+      </c>
+      <c r="D28" s="14" t="inlineStr">
+        <is>
+          <t>現在(型)</t>
+        </is>
+      </c>
+      <c r="E28" s="14" t="inlineStr">
+        <is>
+          <t>Cyberpunk 2077: Phantom Liberty,Shadow of the Erdtree,ライブサービス／GaaS（選別・逆風）</t>
+        </is>
+      </c>
+      <c r="F28" s="14" t="inlineStr">
+        <is>
+          <t>買い切り大作のエバーグリーン化(有料大型拡張・準ライブ運営)</t>
+        </is>
+      </c>
+      <c r="G28" s="14" t="inlineStr">
+        <is>
+          <t>GaaS逆風の受け皿として台頭。第三の道</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="14" t="inlineStr">
+        <is>
+          <t>サバイバル×収集系</t>
+        </is>
+      </c>
+      <c r="B29" s="14" t="n">
+        <v>1996</v>
+      </c>
+      <c r="C29" s="14" t="inlineStr">
+        <is>
+          <t>Pokémon 赤・緑</t>
+        </is>
+      </c>
+      <c r="D29" s="14" t="inlineStr">
+        <is>
+          <t>祖先</t>
+        </is>
+      </c>
+      <c r="E29" s="14" t="inlineStr"/>
+      <c r="F29" s="14" t="inlineStr"/>
+      <c r="G29" s="14" t="inlineStr">
+        <is>
+          <t>モンスター収集・育成・対戦の原型</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="14" t="inlineStr">
+        <is>
+          <t>サバイバル×収集系</t>
+        </is>
+      </c>
+      <c r="B30" s="14" t="n">
+        <v>2011</v>
+      </c>
+      <c r="C30" s="14" t="inlineStr">
+        <is>
+          <t>Minecraft</t>
+        </is>
+      </c>
+      <c r="D30" s="14" t="inlineStr">
+        <is>
+          <t>祖先</t>
+        </is>
+      </c>
+      <c r="E30" s="14" t="inlineStr"/>
+      <c r="F30" s="14" t="inlineStr"/>
+      <c r="G30" s="14" t="inlineStr">
+        <is>
+          <t>サンドボックス・クラフト/建築の大衆化</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="14" t="inlineStr">
+        <is>
+          <t>サバイバル×収集系</t>
+        </is>
+      </c>
+      <c r="B31" s="14" t="n">
+        <v>2015</v>
+      </c>
+      <c r="C31" s="14" t="inlineStr">
+        <is>
+          <t>ARK: Survival Evolved</t>
+        </is>
+      </c>
+      <c r="D31" s="14" t="inlineStr">
+        <is>
+          <t>発展</t>
+        </is>
+      </c>
+      <c r="E31" s="14" t="inlineStr">
+        <is>
+          <t>Minecraft</t>
+        </is>
+      </c>
+      <c r="F31" s="14" t="inlineStr"/>
+      <c r="G31" s="14" t="inlineStr">
+        <is>
+          <t>生物のテイム×サバイバルクラフトを融合</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="14" t="inlineStr">
+        <is>
+          <t>サバイバル×収集系</t>
+        </is>
+      </c>
+      <c r="B32" s="14" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C32" s="14" t="inlineStr">
+        <is>
+          <t>Valheim</t>
+        </is>
+      </c>
+      <c r="D32" s="14" t="inlineStr">
+        <is>
+          <t>発展</t>
+        </is>
+      </c>
+      <c r="E32" s="14" t="inlineStr">
+        <is>
+          <t>Minecraft</t>
+        </is>
+      </c>
+      <c r="F32" s="14" t="inlineStr"/>
+      <c r="G32" s="14" t="inlineStr">
+        <is>
+          <t>協力サバイバルクラフトの大ヒット</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="14" t="inlineStr">
+        <is>
+          <t>サバイバル×収集系</t>
+        </is>
+      </c>
+      <c r="B33" s="14" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C33" s="14" t="inlineStr">
+        <is>
+          <t>Palworld（早期アクセス）</t>
+        </is>
+      </c>
+      <c r="D33" s="14" t="inlineStr">
+        <is>
+          <t>確立</t>
+        </is>
+      </c>
+      <c r="E33" s="14" t="inlineStr">
+        <is>
+          <t>Pokémon 赤・緑,ARK: Survival Evolved</t>
+        </is>
+      </c>
+      <c r="F33" s="14" t="inlineStr"/>
+      <c r="G33" s="14" t="inlineStr">
+        <is>
+          <t>収集×サバイバルクラフトを結合、爆発的普及</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="14" t="inlineStr">
+        <is>
+          <t>サバイバル×収集系</t>
+        </is>
+      </c>
+      <c r="B34" s="14" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C34" s="14" t="inlineStr">
+        <is>
+          <t>サバイバルクラフト×クリーチャー収集</t>
+        </is>
+      </c>
+      <c r="D34" s="14" t="inlineStr">
+        <is>
+          <t>現在(型)</t>
+        </is>
+      </c>
+      <c r="E34" s="14" t="inlineStr">
+        <is>
+          <t>Palworld（早期アクセス）</t>
+        </is>
+      </c>
+      <c r="F34" s="14" t="inlineStr">
+        <is>
+          <t>サバイバルクラフト×クリーチャー収集(モンスター牧場×建築×マルチ)</t>
+        </is>
+      </c>
+      <c r="G34" s="14" t="inlineStr">
+        <is>
+          <t>1.0化。融合ジャンルが一つの完成型に</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="14" t="inlineStr">
+        <is>
+          <t>シネマティック物語系</t>
+        </is>
+      </c>
+      <c r="B35" s="14" t="n">
+        <v>1998</v>
+      </c>
+      <c r="C35" s="14" t="inlineStr">
+        <is>
+          <t>Half-Life</t>
+        </is>
+      </c>
+      <c r="D35" s="14" t="inlineStr">
+        <is>
+          <t>祖先</t>
+        </is>
+      </c>
+      <c r="E35" s="14" t="inlineStr"/>
+      <c r="F35" s="14" t="inlineStr"/>
+      <c r="G35" s="14" t="inlineStr">
+        <is>
+          <t>シームレスな環境ナラティブの原型</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="14" t="inlineStr">
+        <is>
+          <t>シネマティック物語系</t>
+        </is>
+      </c>
+      <c r="B36" s="14" t="n">
+        <v>2007</v>
+      </c>
+      <c r="C36" s="14" t="inlineStr">
+        <is>
+          <t>Uncharted</t>
+        </is>
+      </c>
+      <c r="D36" s="14" t="inlineStr">
+        <is>
+          <t>発展</t>
+        </is>
+      </c>
+      <c r="E36" s="14" t="inlineStr">
+        <is>
+          <t>Half-Life</t>
+        </is>
+      </c>
+      <c r="F36" s="14" t="inlineStr"/>
+      <c r="G36" s="14" t="inlineStr">
+        <is>
+          <t>映画的演出×アクションの確立</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="14" t="inlineStr">
+        <is>
+          <t>シネマティック物語系</t>
+        </is>
+      </c>
+      <c r="B37" s="14" t="n">
+        <v>2013</v>
+      </c>
+      <c r="C37" s="14" t="inlineStr">
+        <is>
+          <t>The Last of Us</t>
+        </is>
+      </c>
+      <c r="D37" s="14" t="inlineStr">
+        <is>
+          <t>確立</t>
+        </is>
+      </c>
+      <c r="E37" s="14" t="inlineStr">
+        <is>
+          <t>Uncharted</t>
+        </is>
+      </c>
+      <c r="F37" s="14" t="inlineStr"/>
+      <c r="G37" s="14" t="inlineStr">
+        <is>
+          <t>物語主導AAAの到達点</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="14" t="inlineStr">
+        <is>
+          <t>シネマティック物語系</t>
+        </is>
+      </c>
+      <c r="B38" s="14" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C38" s="14" t="inlineStr">
+        <is>
+          <t>God of War</t>
+        </is>
+      </c>
+      <c r="D38" s="14" t="inlineStr">
+        <is>
+          <t>確立</t>
+        </is>
+      </c>
+      <c r="E38" s="14" t="inlineStr">
+        <is>
+          <t>The Last of Us</t>
+        </is>
+      </c>
+      <c r="F38" s="14" t="inlineStr"/>
+      <c r="G38" s="14" t="inlineStr">
+        <is>
+          <t>ワンショット演出で物語体験を刷新</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="14" t="inlineStr">
+        <is>
+          <t>シネマティック物語系</t>
+        </is>
+      </c>
+      <c r="B39" s="14" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C39" s="14" t="inlineStr">
+        <is>
+          <t>Baldur's Gate 3</t>
+        </is>
+      </c>
+      <c r="D39" s="14" t="inlineStr">
+        <is>
+          <t>確立</t>
+        </is>
+      </c>
+      <c r="E39" s="14" t="inlineStr">
+        <is>
+          <t>The Last of Us</t>
+        </is>
+      </c>
+      <c r="F39" s="14" t="inlineStr"/>
+      <c r="G39" s="14" t="inlineStr">
+        <is>
+          <t>選択分岐×物語密度でGOTY。買い切り物語の強さ</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="14" t="inlineStr">
+        <is>
+          <t>シネマティック物語系</t>
+        </is>
+      </c>
+      <c r="B40" s="14" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C40" s="14" t="inlineStr">
+        <is>
+          <t>シングルプレイ大作（物語主導）</t>
+        </is>
+      </c>
+      <c r="D40" s="14" t="inlineStr">
+        <is>
+          <t>現在(型)</t>
+        </is>
+      </c>
+      <c r="E40" s="14" t="inlineStr">
+        <is>
+          <t>God of War,Baldur's Gate 3,ライブサービス／GaaS（選別・逆風）</t>
+        </is>
+      </c>
+      <c r="F40" s="14" t="inlineStr">
+        <is>
+          <t>シングルプレイ大作(物語主導)</t>
+        </is>
+      </c>
+      <c r="G40" s="14" t="inlineStr">
+        <is>
+          <t>GaaS逆風の反動で再評価/復権</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
daily-news + cross-questions + events + predictions + game-design update (2026-07-12)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -817,7 +817,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1862,6 +1862,43 @@
       <c r="G28" s="14" t="inlineStr">
         <is>
           <t>別の小売/外食/交通チェーンとの同種スポンサード提携が追加発表されるか、ナイアンティック/Scopelyが位置情報スポンサー収益を開示・強調するかを観測。</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B29" s="14" t="inlineStr">
+        <is>
+          <t>AI生成アセットの開示義務化（EU AI Act）を逆手に、『人の手/非AI保証』が差別化ラベルとして商品価値化。Steam等で制作にAI不使用のストア表記やフィルタ需要が生まれ、インディーのマーケ訴求軸として定着する。</t>
+        </is>
+      </c>
+      <c r="C29" s="14" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="D29" s="14" t="inlineStr">
+        <is>
+          <t>半年〜年内</t>
+        </is>
+      </c>
+      <c r="E29" s="14" t="inlineStr">
+        <is>
+          <t>Valve, インディー各社</t>
+        </is>
+      </c>
+      <c r="F29" s="14" t="inlineStr">
+        <is>
+          <t>EU AI Actの透明性義務8/2適用開始（本日追記の日次ニュース・EU公式）</t>
+        </is>
+      </c>
+      <c r="G29" s="14" t="inlineStr">
+        <is>
+          <t>Steamのストアページで『No Gen-AI』表記や絞り込み/バッジが増えるか、インディーが非AIを訴求軸に据える事例が増えるかを観測。</t>
         </is>
       </c>
     </row>
@@ -3899,7 +3936,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G67"/>
+  <dimension ref="A1:G69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6387,6 +6424,80 @@
       <c r="G67" s="14" t="inlineStr">
         <is>
           <t>『広告枠』ではなく『来店導線(足を運ばせる力)』そのものを売る。ゲームのMAUが位置情報×購買データを介して集客インフラ化する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B68" s="14" t="inlineStr">
+        <is>
+          <t>AI生成コンテンツのラベリング義務化（EU AI Act 8月施行）は、ゲームだけでなく広告・報道・EC商品画像など『AI生成物の開示』を他業界にどこまで波及させるか？</t>
+        </is>
+      </c>
+      <c r="C68" s="14" t="inlineStr">
+        <is>
+          <t>EU AI Actの透明性義務が8/2適用開始（EU公式）</t>
+        </is>
+      </c>
+      <c r="D68" s="14" t="inlineStr">
+        <is>
+          <t>European Commission, Valve</t>
+        </is>
+      </c>
+      <c r="E68" s="14" t="inlineStr">
+        <is>
+          <t>広告（AIクリエイティブ表示）/ EC（AI商品画像の開示）/ 報道（AI生成記事の明示）</t>
+        </is>
+      </c>
+      <c r="F68" s="14" t="inlineStr">
+        <is>
+          <t>オープン</t>
+        </is>
+      </c>
+      <c r="G68" s="14" t="inlineStr">
+        <is>
+          <t>表示義務は横断的規制になりやすく、ゲームは先行実装される表示UXの実験場になりうる。</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B69" s="14" t="inlineStr">
+        <is>
+          <t>ゲームメディアのアフィリエイト/コマース（購入導線）依存モデルの解体（GameSpot）は、家電・金融・旅行など比較サイトを持つ他業界メディアでも同じ収益崩壊を招くか？</t>
+        </is>
+      </c>
+      <c r="C69" s="14" t="inlineStr">
+        <is>
+          <t>GameSpotで再度のレイオフ、Fandomがコマースチームを整理（Aftermath）</t>
+        </is>
+      </c>
+      <c r="D69" s="14" t="inlineStr">
+        <is>
+          <t>Fandom, GameSpot</t>
+        </is>
+      </c>
+      <c r="E69" s="14" t="inlineStr">
+        <is>
+          <t>メディア全般（家電・金融・旅行の比較/レビュー）/ EC（送客マージン）/ アフィリエイト</t>
+        </is>
+      </c>
+      <c r="F69" s="14" t="inlineStr">
+        <is>
+          <t>オープン</t>
+        </is>
+      </c>
+      <c r="G69" s="14" t="inlineStr">
+        <is>
+          <t>プラットフォームが購入導線を内製化する構図はゲーム外でも進行中で、第三者メディアの中抜き余地が縮む共通課題。</t>
         </is>
       </c>
     </row>
@@ -9360,7 +9471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10572,6 +10683,110 @@
       <c r="J24" s="14" t="inlineStr">
         <is>
           <t>2026-07-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B25" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="C25" s="14" t="inlineStr">
+        <is>
+          <t>bilibili World 2026</t>
+        </is>
+      </c>
+      <c r="D25" s="14" t="inlineStr">
+        <is>
+          <t>展示会</t>
+        </is>
+      </c>
+      <c r="E25" s="14" t="inlineStr">
+        <is>
+          <t>上海（国家会展中心）</t>
+        </is>
+      </c>
+      <c r="F25" s="14" t="inlineStr">
+        <is>
+          <t>オフライン</t>
+        </is>
+      </c>
+      <c r="G25" s="14" t="inlineStr">
+        <is>
+          <t>中国最大級のサブカル/ゲーム展。世界130社が出展、Black Myth陣営やTotal War新作、Kevin Feige登壇。</t>
+        </is>
+      </c>
+      <c r="H25" s="14" t="inlineStr">
+        <is>
+          <t>https://www.invenglobal.com/articles/23379/bilibili-world-2026-a-subculture-hub-featuring-kevin-feige</t>
+        </is>
+      </c>
+      <c r="I25" s="14" t="inlineStr">
+        <is>
+          <t>開催中</t>
+        </is>
+      </c>
+      <c r="J25" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B26" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="C26" s="14" t="inlineStr">
+        <is>
+          <t>Taipei Game Developers Forum 2026 (TGDF)</t>
+        </is>
+      </c>
+      <c r="D26" s="14" t="inlineStr">
+        <is>
+          <t>展示会</t>
+        </is>
+      </c>
+      <c r="E26" s="14" t="inlineStr">
+        <is>
+          <t>台北（Taipei New Horizon）</t>
+        </is>
+      </c>
+      <c r="F26" s="14" t="inlineStr">
+        <is>
+          <t>オフライン</t>
+        </is>
+      </c>
+      <c r="G26" s="14" t="inlineStr">
+        <is>
+          <t>台湾最大級のゲーム開発者カンファレンス。アジア各国の開発者が集う。東映ゲームズ等日本勢も登壇。</t>
+        </is>
+      </c>
+      <c r="H26" s="14" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/991/G999104/20260708042/</t>
+        </is>
+      </c>
+      <c r="I26" s="14" t="inlineStr">
+        <is>
+          <t>開催予定</t>
+        </is>
+      </c>
+      <c r="J26" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
         </is>
       </c>
     </row>
@@ -10906,7 +11121,7 @@
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
@@ -10936,17 +11151,17 @@
       </c>
       <c r="G7" s="14" t="inlineStr">
         <is>
-          <t>生成AIコンテンツの氾濫とユーザーの真正性選好。プラットフォームのAI開示ルール強化。</t>
+          <t>生成AIコンテンツの氾濫とユーザーの真正性選好。プラットフォームのAI開示ルール強化に加え、EU AI Actの透明性義務(8/2適用)でAI生成表示が制度化。</t>
         </is>
       </c>
       <c r="H7" s="14" t="inlineStr">
         <is>
-          <t>「真正性が効率に勝つ」ニッチ市場が形成。AI活用と非AI訴求の二極化が進む。</t>
+          <t>真正性が効率に勝つニッチが拡大。表示義務化で非AIがラベル/フィルタとして商品価値化し、AI活用と非AI訴求の二極化が加速。</t>
         </is>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
-          <t>GDC2026 開発者のAI利用率低下(6/24)</t>
+          <t>EU AI Act透明性義務が8/2適用開始(本日追記の日次ニュース)</t>
         </is>
       </c>
       <c r="J7" s="14" t="n">
@@ -12579,7 +12794,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L291"/>
+  <dimension ref="A1:L296"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -30629,6 +30844,300 @@
         </is>
       </c>
       <c r="L291" s="14" t="inlineStr"/>
+    </row>
+    <row r="292">
+      <c r="A292" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B292" s="14" t="inlineStr">
+        <is>
+          <t>中国最大級のサブカル展「bilibili World 2026」が上海で開幕（7/10〜12）——Black Myth陣営やTotal War新作が出展</t>
+        </is>
+      </c>
+      <c r="C292" s="14" t="inlineStr">
+        <is>
+          <t>https://www.invenglobal.com/articles/23379/bilibili-world-2026-a-subculture-hub-featuring-kevin-feige</t>
+        </is>
+      </c>
+      <c r="D292" s="14" t="inlineStr">
+        <is>
+          <t>E3消滅後、アジアではbilibili WorldがサブカルとゲームのハブとしてTGS・gamescomに並ぶ規模に成長。中国のゲーム消費と海外パブリッシャーの中国市場攻略の重要接点になっている。</t>
+        </is>
+      </c>
+      <c r="E292" s="14" t="inlineStr">
+        <is>
+          <t>上海の国家会展中心で7/10〜12開催。170超の出展者・700超のブースに世界130社のゲーム開発者が集結。原神・ブルアカ・鳴潮・アークナイツ：エンドフィールド等が出展し、Game Science（黒神話）やCreative AssemblyのTotal War新作もアピールした。</t>
+        </is>
+      </c>
+      <c r="F292" s="14" t="inlineStr">
+        <is>
+          <t>・7/10〜12・上海、世界130社が参加する中国最大級のサブカル/ゲーム展
+・Game Science（黒神話：鍾馗の続報に注目）が『Black Myth』名義で出展
+・Creative Assembly『Total War: WARHAMMER 40,000』が新エンジンWarCoreで初のオフライン出展
+・マーベル・スタジオのKevin Feige氏が登壇
+・『Love and Deepspace』は炎上を受け出展を辞退</t>
+        </is>
+      </c>
+      <c r="G292" s="14" t="inlineStr">
+        <is>
+          <t>中国国内の版号回復と大型IPの海外展開を背景に、bilibili Worldは中国市場攻略の実質的な商談・PRの場として比重が高まる。海外AAAの中国オフライン出展が定着すれば、gamescom/TGSと並ぶ第3極の見本市化が進む。</t>
+        </is>
+      </c>
+      <c r="H292" s="14" t="inlineStr">
+        <is>
+          <t>中国ゲーム市場と見本市エコシステム</t>
+        </is>
+      </c>
+      <c r="I292" s="14" t="inlineStr">
+        <is>
+          <t>bilibili, Game Science, Creative Assembly, SEGA</t>
+        </is>
+      </c>
+      <c r="J292" s="14" t="inlineStr">
+        <is>
+          <t>黒神話, Total War, 原神, ブルーアーカイブ</t>
+        </is>
+      </c>
+      <c r="K292" s="14" t="inlineStr">
+        <is>
+          <t>海外,新作,eスポーツ</t>
+        </is>
+      </c>
+      <c r="L292" s="14" t="inlineStr"/>
+    </row>
+    <row r="293">
+      <c r="A293" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B293" s="14" t="inlineStr">
+        <is>
+          <t>eスポーツ・ワールドカップ2026、VALORANT部門が7/12にグランドファイナル——賞金総額200万ドル、パリで開催</t>
+        </is>
+      </c>
+      <c r="C293" s="14" t="inlineStr">
+        <is>
+          <t>https://dotesports.com/valorant/guides/ewc-2026-valorant</t>
+        </is>
+      </c>
+      <c r="D293" s="14" t="inlineStr">
+        <is>
+          <t>EWCは中東（リヤド）で2回開催後、2026年は情勢を受けパリに会場を移転。7/6〜8/23の長期会期で24競技25大会を実施する世界最大級のeスポーツ祭典で、クラブの複数タイトル横断ポイント制が特徴。</t>
+        </is>
+      </c>
+      <c r="E293" s="14" t="inlineStr">
+        <is>
+          <t>パリのParis Expo Porte de Versaillesで開催中のEWC2026で、VALORANT部門（16チーム・賞金200万ドル）が7/2〜12の日程を終え、7/12に3位決定戦とグランドファイナルを実施。EWC全体は8/23まで継続する。</t>
+        </is>
+      </c>
+      <c r="F293" s="14" t="inlineStr">
+        <is>
+          <t>・EWC2026はパリ開催、会期7/6〜8/23の過去最大規模
+・VALORANT部門の決勝が7/12、賞金プールは200万ドル
+・今年はTrackmaniaが新規参入、Fortniteがリロードモードで復帰
+・クラブ横断のポイントで年間王者を決定</t>
+        </is>
+      </c>
+      <c r="G293" s="14" t="inlineStr">
+        <is>
+          <t>パリ移転で欧州の観客動員と放映がどこまで伸びるかが今後の開催地戦略を左右する。会期の長期化・多タイトル化により、単発大会からクラブ経営（横断ポイント×スポンサー）モデルへの移行がさらに進む。</t>
+        </is>
+      </c>
+      <c r="H293" s="14" t="inlineStr">
+        <is>
+          <t>eスポーツの興行・クラブ経営モデル</t>
+        </is>
+      </c>
+      <c r="I293" s="14" t="inlineStr">
+        <is>
+          <t>Esports World Cup Foundation, Riot Games</t>
+        </is>
+      </c>
+      <c r="J293" s="14" t="inlineStr">
+        <is>
+          <t>VALORANT, Trackmania, Fortnite</t>
+        </is>
+      </c>
+      <c r="K293" s="14" t="inlineStr">
+        <is>
+          <t>eスポーツ,海外</t>
+        </is>
+      </c>
+      <c r="L293" s="14" t="inlineStr"/>
+    </row>
+    <row r="294">
+      <c r="A294" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B294" s="14" t="inlineStr">
+        <is>
+          <t>GameSpotで再びレイオフ——親会社FandomがコマースチームとゲームVPを整理、購入ガイド部門が消滅</t>
+        </is>
+      </c>
+      <c r="C294" s="14" t="inlineStr">
+        <is>
+          <t>https://aftermath.site/gamespot-layoffs-july-2026/</t>
+        </is>
+      </c>
+      <c r="D294" s="14" t="inlineStr">
+        <is>
+          <t>2023年にFandom傘下入りしたGameSpotは断続的な人員削減が続く。ゲームメディアはレビュー広告からアフィリエイト/コマース（セール・予約ガイド）収益へ依存を強めてきたが、その中核部門にメスが入った。</t>
+        </is>
+      </c>
+      <c r="E294" s="14" t="inlineStr">
+        <is>
+          <t>Fandomが木曜にGameSpotのコマースチーム（正社員4名＋フリー5名）とゲーム・エンタメ担当VPのChris Grant氏を整理。セール記事や予約・購入ガイドを担っていた部門が実質消滅した。2026年に入って2度目の削減となる。</t>
+        </is>
+      </c>
+      <c r="F294" s="14" t="inlineStr">
+        <is>
+          <t>・Fandomがコマースチーム全体とゲーム担当VPを削減
+・対象は購入/予約ガイド・セール記事の中核部門
+・2026年に入り2度目、Fandom買収後は繰り返しの削減
+・ゲームメディアの購入導線マネタイズモデルへの逆風を象徴</t>
+        </is>
+      </c>
+      <c r="G294" s="14" t="inlineStr">
+        <is>
+          <t>プラットフォーム（Steam/ストア）が購入導線とキュレーションを内製化するなか、第三者メディアの送客マージンは縮小。メディアはB2B（データ・コンサル）や直接課金（会員制）への再編を迫られる。</t>
+        </is>
+      </c>
+      <c r="H294" s="14" t="inlineStr">
+        <is>
+          <t>ゲームメディアの収益構造とアフィリエイト依存</t>
+        </is>
+      </c>
+      <c r="I294" s="14" t="inlineStr">
+        <is>
+          <t>Fandom, GameSpot</t>
+        </is>
+      </c>
+      <c r="J294" s="14" t="inlineStr"/>
+      <c r="K294" s="14" t="inlineStr">
+        <is>
+          <t>海外</t>
+        </is>
+      </c>
+      <c r="L294" s="14" t="inlineStr"/>
+    </row>
+    <row r="295">
+      <c r="A295" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B295" s="14" t="inlineStr">
+        <is>
+          <t>EU AI Actの透明性義務が8/2適用開始へ——AI生成コンテンツの識別・表示がゲーム開発にも波及</t>
+        </is>
+      </c>
+      <c r="C295" s="14" t="inlineStr">
+        <is>
+          <t>https://digital-strategy.ec.europa.eu/en/policies/regulatory-framework-ai</t>
+        </is>
+      </c>
+      <c r="D295" s="14" t="inlineStr">
+        <is>
+          <t>EU AI Actは段階施行中で、生成AIの透明性ルールが2026年8月に本格適用。ディープフェイクやAI生成物の識別可能性・表示を求める。ゲームは最小リスク区分だが、Steam/Apple/GoogleがAI利用開示ポリシーを整備しつつある。</t>
+        </is>
+      </c>
+      <c r="E295" s="14" t="inlineStr">
+        <is>
+          <t>EU AI Actの透明性条項が2026年8月2日から適用開始。AI生成コンテンツは機械可読な識別を付し、ディープフェイク等は明示的にラベリングする必要がある。ストアプラットフォーム側のAIアセット開示要求とも連動し、開発工程の記録・表示対応が求められる。</t>
+        </is>
+      </c>
+      <c r="F295" s="14" t="inlineStr">
+        <is>
+          <t>・生成AIの透明性ルールが8/2から適用開始
+・AI生成物の識別可能性とディープフェイクの明示ラベルが必要
+・ゲーム自体は最小リスク区分だが表示・開示の実務対応は発生
+・Steam/Apple/GoogleもAIアセット開示ポリシーを整備中</t>
+        </is>
+      </c>
+      <c r="G295" s="14" t="inlineStr">
+        <is>
+          <t>EUでの表示義務が事実上のグローバル標準化圧力となり、ストアページでのAI利用開示が一般化。開発側は生成物のトレーサビリティ管理が新たな運用コストになる一方、非AI訴求の差別化余地も広がる。</t>
+        </is>
+      </c>
+      <c r="H295" s="14" t="inlineStr">
+        <is>
+          <t>AI規制（EU AI Act）とAI生成物の開示実務</t>
+        </is>
+      </c>
+      <c r="I295" s="14" t="inlineStr">
+        <is>
+          <t>European Commission, Valve, Apple, Google</t>
+        </is>
+      </c>
+      <c r="J295" s="14" t="inlineStr"/>
+      <c r="K295" s="14" t="inlineStr">
+        <is>
+          <t>規制,技術,海外</t>
+        </is>
+      </c>
+      <c r="L295" s="14" t="inlineStr"/>
+    </row>
+    <row r="296">
+      <c r="A296" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B296" s="14" t="inlineStr">
+        <is>
+          <t>東映ゲームズ、台湾最大級の開発者会議「TGDF 2026」（7/15〜16）に登壇——日台のゲーム市場連携を議論</t>
+        </is>
+      </c>
+      <c r="C296" s="14" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/991/G999104/20260708042/</t>
+        </is>
+      </c>
+      <c r="D296" s="14" t="inlineStr">
+        <is>
+          <t>東映は映像資産を核にゲーム事業を強化中で、アジア市場、とりわけ成長する台湾のインディー/開発者コミュニティとの連携を模索。TGDFは台湾最大級の開発者カンファレンスで、アジア各国の開発者が集う。</t>
+        </is>
+      </c>
+      <c r="E296" s="14" t="inlineStr">
+        <is>
+          <t>東映ゲームズが7/15〜16に台北で開かれる「Taipei Game Developers Forum 2026」に登壇。7/16に新規事業開発マネージャーの長島寛晃氏が事業戦略セッションを行い、日本と台湾のゲーム市場の関係や協業の展望を語る。</t>
+        </is>
+      </c>
+      <c r="F296" s="14" t="inlineStr">
+        <is>
+          <t>・東映ゲームズがTGDF 2026（7/15〜16・台北）に登壇
+・7/16に事業戦略セッション（日本語・中文字幕）
+・テーマは日台ゲーム市場の連携と東映の事業戦略
+・映像IPを持つ東映のゲーム分野アジア展開の一環</t>
+        </is>
+      </c>
+      <c r="G296" s="14" t="inlineStr">
+        <is>
+          <t>日本の映像・IPホルダーが台湾/東南アジアの開発力と組む座組が増え、受託・共同開発やIPライセンスの日台クロスボーダー案件が拡大する可能性。</t>
+        </is>
+      </c>
+      <c r="H296" s="14" t="inlineStr">
+        <is>
+          <t>日台クロスボーダーのゲーム協業とIP活用</t>
+        </is>
+      </c>
+      <c r="I296" s="14" t="inlineStr">
+        <is>
+          <t>東映, 東映ゲームズ</t>
+        </is>
+      </c>
+      <c r="J296" s="14" t="inlineStr"/>
+      <c r="K296" s="14" t="inlineStr">
+        <is>
+          <t>国内,海外</t>
+        </is>
+      </c>
+      <c r="L296" s="14" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
weekly-stocks + IP watch update (2026-07-13 21:23)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -32831,7 +32831,7 @@
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>6/9のニンダイで『スカーレット・バイオレット』向け有料追加コンテンツ（DLC）が告知され、既存タイトルの追加展開が継続。</t>
+          <t>DeNAの『ポケポケ(Pokémon TCG Pocket)』が初のテーマ拡張パック『幻のいる島』を追加し好調継続、DeNAの収益ドライバーに。本編・カード・アプリ横断で高い集客力を維持。</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
@@ -32848,7 +32848,7 @@
       <c r="H4" s="9" t="inlineStr"/>
       <c r="I4" s="9" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
@@ -33212,7 +33212,7 @@
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>KONAMIが新作ラインアップでMGSブランドの展開を強化。</t>
+          <t>Steamサマーセール(6/26〜7/10)で『MGSΔ SNAKE EATER』が40%オフとなり話題化。オンラインモード『Fox Hunt』搭載済。</t>
         </is>
       </c>
       <c r="E15" s="9" t="inlineStr">
@@ -33229,7 +33229,7 @@
       <c r="H15" s="9" t="inlineStr"/>
       <c r="I15" s="9" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
@@ -33290,12 +33290,12 @@
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>『ペルソナ5X』は今夏展開で概ね想定通りに推移。</t>
+          <t>『ペルソナ5X』は今夏展開で概ね想定通り。セガサミーは2027年3月期の大型4本計画の中核にペルソナ系を位置付け。</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>『ペルソナ4 リバイバル』を2027年3月期に投入予定(PS5/Xbox/Win/Steam、Game Pass対応)。</t>
+          <t>『ペルソナ4 リバイバル』2027/2/18発売決定(PC/PS5/Xbox、Game Pass初日対応)。『ペルソナ6』はストアページ公開済。</t>
         </is>
       </c>
       <c r="F17" s="9" t="inlineStr"/>
@@ -33307,7 +33307,7 @@
       <c r="H17" s="9" t="inlineStr"/>
       <c r="I17" s="9" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
@@ -33698,12 +33698,12 @@
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>最重要作として市場の注目を一身に集める。発売日は据え置きを維持。</t>
+          <t>予約が本格化。仏Cdiscountでの予約は通常大型作の約6倍。Take-Two株は52週高値圏($260台)で発売期待が先行。</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>『Grand Theft Auto VI』は2026年11月19日にPS5/Xbox Series X|Sで発売予定。</t>
+          <t>『GTAⅥ』2026/11/19発売(PS5/Xbox Series X|S)。標準版$79.99/アルティメット版$99.99を確定。</t>
         </is>
       </c>
       <c r="F29" s="9" t="inlineStr"/>
@@ -33715,7 +33715,7 @@
       <c r="H29" s="9" t="inlineStr"/>
       <c r="I29" s="9" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
@@ -34151,12 +34151,12 @@
       </c>
       <c r="D44" s="9" t="inlineStr">
         <is>
-          <t>6/16に『AC Shadows』タイトルアップデート1.1.11を配信。Ubisoftは組織再編下でシリーズの運営を継続。</t>
+          <t>『AC Mirage』が無料拡張Valley of Memory(舞台:AlUla)投入で1,000万プレイヤー到達。7/9に『AC ブラックフラッグ リシンクド』を発売。</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
         <is>
-          <t>Vantage Studios体制で新作開発</t>
+          <t>AC/Far Cry/Rainbow SixはTencent出資の新子会社Vantage Studios(評価額約€3.8〜4bn)に集約し開発体制を再編。</t>
         </is>
       </c>
       <c r="F44" s="9" t="inlineStr"/>
@@ -34168,7 +34168,7 @@
       <c r="H44" s="9" t="inlineStr"/>
       <c r="I44" s="9" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
@@ -34775,7 +34775,7 @@
       </c>
       <c r="M2" s="9" t="inlineStr">
         <is>
-          <t>7/3に年初来安値6,544円をつけ株価軟調が継続。メモリなど部材急騰観測と先行き不透明感で過去5か月で30%超下落。FY26はSwitch 2立ち上げで売上2.313兆円(+98.6%)・営業益3,601億円(+27.5%)と急回復済だが、年末商戦とハード普及ペース、部材コスト増を見極める材料待ちの調整局面。</t>
+          <t>株価は6/26の6,589円を安値に7/2に7,137円へ反発、その後7,120円前後で横ばい推移し材料出尽くし後の水準確認局面。Switch 2値上げ(国内5.998万円)による普及ペース鈍化懸念は根強いが、FY26は売上2.31兆円(+98.6%)営業益3,601億円(+27.5%)と急回復済。次期は減収減益予想で新作ソフト継続投入が焦点。</t>
         </is>
       </c>
       <c r="N2" s="9" t="inlineStr">
@@ -34785,17 +34785,17 @@
       </c>
       <c r="O2" s="9" t="inlineStr">
         <is>
-          <t>メモリ等部材急騰によるコスト増懸念、ハード普及ペース不透明、株価の下値模索</t>
+          <t>Switch 2値上げによる普及ペース鈍化懸念、部材コスト増、次期減収減益予想</t>
         </is>
       </c>
       <c r="P2" s="9" t="inlineStr">
         <is>
-          <t>Switch 2普及ペースとファーストパーティ大型タイトル供給、部材コスト管理</t>
+          <t>Switch 2普及ペースと年末商戦、ファーストパーティ大型タイトル供給、部材コスト管理</t>
         </is>
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
@@ -34830,7 +34830,7 @@
       </c>
       <c r="M3" s="9" t="inlineStr">
         <is>
-          <t>7/2にG&amp;NS期待などから株価一時+4.6%高。PS新作の『ディスク版販売終了』報道が話題。GTAⅥ(11/19)がPS5/Xboxのみ対応となる見込みで、PS Plusなどネットワークサービス収入の増加期待が改めて意識される。FY25は全社売上・営業益とも過去最高を更新済み。</t>
+          <t>『GTAⅥ』が11/19にPS5/Xbox向けで発売(標準$79.99/アルティメット$99.99)と価格が確定し、PS5エンゲージメント/ネットワーク収入拡大への期待が改めて意識される。FY25は全社売上・営業益とも過去最高を更新済で、大型新規開示は乏しく好業績持続力を見極める局面。</t>
         </is>
       </c>
       <c r="N3" s="9" t="inlineStr">
@@ -34850,7 +34850,7 @@
       </c>
       <c r="Q3" s="9" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
@@ -34885,7 +34885,7 @@
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>7/2に適時開示、期待の新作『鬼武者 Way of the Sword』の発売日を9月4日へ前倒しと発表。FY26通期は13期連続営業増益・売上/営業益とも過去最高で好調継続。強力IPのリピート販売とデジタル比率上昇が寄与。</t>
+          <t>『鬼武者 Way of the Sword』発売日9/4前倒し発表(7/2)を受け株価は一時+8.4%高の3,272円まで上昇。13期連続営業増益・売上/営業益とも過去最高で好調継続。強力IPのリピート販売とデジタル比率上昇が寄与し、年内の新作寄与への期待が高まる。</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
@@ -34900,12 +34900,12 @@
       </c>
       <c r="P4" s="9" t="inlineStr">
         <is>
-          <t>『鬼武者 Way of the Sword』(9/4)の初動、主力IPの継続的なリピート販売</t>
+          <t>『鬼武者 Way of the Sword』(9/4)の初動、主力IPの継続的なリピート販売とデジタル化進展</t>
         </is>
       </c>
       <c r="Q4" s="9" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
@@ -34952,7 +34952,7 @@
       </c>
       <c r="M5" s="9" t="inlineStr">
         <is>
-          <t>『FFVIIリメイク』3部作第2弾がSwitch 2/Xbox Series X|S/Windowsにも対応拡大の見込み。2027年3月以降は大型タイトルを定期発売する方針を継続表明し、『ドラゴンクエストXII』が含まれる可能性も取り沙汰される。FY26は減収増益。</t>
+          <t>株価は2,601円(7/7 +1.8%)で推移。FY26は減収増益(売上-8.3%、営業益+34.9%)を達成しデジタル/ライツ事業が収益性改善に寄与。次回決算は8/10予定。『FFVIIリメイク』第2弾のマルチ展開拡大と2027年3月以降の大型タイトル定期供給方針を継続表明。</t>
         </is>
       </c>
       <c r="N5" s="9" t="inlineStr">
@@ -34972,7 +34972,7 @@
       </c>
       <c r="Q5" s="9" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
@@ -35019,7 +35019,7 @@
       </c>
       <c r="M6" s="9" t="inlineStr">
         <is>
-          <t>新作ラインアップを公開し過去人気IP復活やスポーツタイトルでSwitch 2向けを積極化。『パワフルプロ野球2026-2027』を展開、8月には『METAL GEAR SOLID: MASTER COLLECTION Vol.2』をグローバル発売予定。デジタル・スポーツIPが業績を下支え。</t>
+          <t>Steamサマーセール(6/26〜7/10)で『MGSΔ SNAKE EATER』を40%オフ販売し話題化。8月に『METAL GEAR SOLID: MASTER COLLECTION Vol.2』のグローバル発売を予定。過去人気IP復活とSwitch 2向け展開を積極化し、デジタル・スポーツIPが業績を下支え。</t>
         </is>
       </c>
       <c r="N6" s="9" t="inlineStr">
@@ -35039,7 +35039,7 @@
       </c>
       <c r="Q6" s="9" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
@@ -35086,7 +35086,7 @@
       </c>
       <c r="M7" s="9" t="inlineStr">
         <is>
-          <t>FY26は『機動戦士ガンダム』シリーズ牽引で売上・全利益項目が過去最高を更新済み。IP軸(ガンダム/ドラゴンボール等)のグローバル展開とトイホビー好調が継続。大きな新規開示は乏しく、好業績の持続力を見極める局面。</t>
+          <t>株価は4,074円前後(7/7)で推移、アナリスト平均目標株価は4,817円。FY26はガンダム牽引で売上1.348兆円(+8.6%)営業益1,895億円(+5.2%)と過去最高を更新済。IP軸のグローバル展開とトイホビー好調が継続し、大きな新規開示は乏しく好業績の持続力を見極める局面。</t>
         </is>
       </c>
       <c r="N7" s="9" t="inlineStr">
@@ -35106,7 +35106,7 @@
       </c>
       <c r="Q7" s="9" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
@@ -35141,27 +35141,27 @@
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>2027年3月期に主力4本(『STRANGER THAN HEAVEN』『ペルソナ4 リバイバル』＋主要IP新作2本)を投入する計画。『ペルソナ5X』は今夏展開で概ね想定通り。FY26のセガ(エンタメ)営業益は新作の遅れ等で大幅減益だった反動から、次期の大型タイトル集中に期待。</t>
+          <t>FY26は売上4,875.42億円(+13.7%)も営業益471.28億円(-2.1%)、Rovio等の減損で純損失を計上。遊技機は好調もエンタメコンテンツが低調。次回決算8/7予定。『ペルソナ5X』は今夏展開、『ペルソナ4 リバイバル』は2027/2/18発売決定と、2027年3月期の大型新作4本計画に期待。</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>『ペルソナ』『龍が如く』等の強力IP、2027年3月期の大型新作4本計画</t>
+          <t>『ペルソナ』『龍が如く』等の強力IP、2027年3月期の大型新作4本計画、遊技機好調</t>
         </is>
       </c>
       <c r="O8" s="9" t="inlineStr">
         <is>
-          <t>新作リリース遅延・一部タイトルの想定下振れ、エンタメ営業益の変動</t>
+          <t>Rovio等の減損による純損失、エンタメコンテンツ事業の低調、新作リリース遅延リスク</t>
         </is>
       </c>
       <c r="P8" s="9" t="inlineStr">
         <is>
-          <t>『STRANGER THAN HEAVEN』『ペルソナ4リバイバル』等の投入と初動</t>
+          <t>『STRANGER THAN HEAVEN』『ペルソナ4リバイバル』(2027/2/18)等の投入と初動</t>
         </is>
       </c>
       <c r="Q8" s="9" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
@@ -35208,7 +35208,7 @@
       </c>
       <c r="M9" s="9" t="inlineStr">
         <is>
-          <t>『仁王3』がシリーズ最速で全世界累計100万本を達成し、シリーズ累計は1000万本を突破。コンソール新作は好調だがモバイル減速と先行投資で足元は減収減益。第4四半期に大型タイトルが集中し挽回を図る構図。</t>
+          <t>株価は1,593.5円(7/10)で推移、次回決算は7/27予定。鯉沼社長が『2035年までに営業利益で世界トップ10』を掲げ開発ライン増設・5,000人規模組織を目指す長期戦略を表明。『仁王3』はシリーズ最速で全世界100万本突破。足元はモバイル減速と先行投資で減収減益。</t>
         </is>
       </c>
       <c r="N9" s="9" t="inlineStr">
@@ -35223,12 +35223,12 @@
       </c>
       <c r="P9" s="9" t="inlineStr">
         <is>
-          <t>『仁王3』の販売継続と大型コンソール新作の寄与</t>
+          <t>『仁王3』の販売継続と大型コンソール新作、開発ライン増設に伴う中長期の成長投資</t>
         </is>
       </c>
       <c r="Q9" s="9" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
@@ -35271,7 +35271,7 @@
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>FY26は売上1,713.69億円(+10.7%)も営業益222.56億円(-16.3%)と減益。主力『モンスターストライク』のMAU減少とアニメ等広告宣伝費が重し。スポーツ(千葉ジェッツ/TIPSTAR)は黒字化。PointsBet連結化で事業ポートフォリオ多角化を進める。株価は6/末2,685円前後。</t>
+          <t>米Runwayと提携し動画AIで『モンスト』広告制作時間を半減(6/30発表)。FY26Q3は売上1,164.25億円(+5.5%)も営業益131.68億円(-22.7%)と増収減益で、主力デジタルエンタメの減収が重し。スポーツ事業は伸長。『モンスト』MAU底打ちと多角化事業の収益貢献が焦点。</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
@@ -35291,7 +35291,7 @@
       </c>
       <c r="Q10" s="9" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
@@ -35326,7 +35326,7 @@
       </c>
       <c r="M11" s="9" t="inlineStr">
         <is>
-          <t>大きな新規適時開示は限定的。既存タイトル運営とメタバース『REALITY』、投資事業を軸に事業構造転換を継続。ゲーム単体の新規モメンタムは乏しく、コスト管理と新規事業の育成が焦点。</t>
+          <t>FY26Q3(5/13発表)は売上384.44億円(-10.9%)営業益24.2億円(-34.7%)と減収減益も、為替差益で純利益は+112.4%と大幅増益。次回決算は8月上旬予定。既存タイトル運営とメタバース『REALITY』、投資事業を軸に事業構造転換を継続。</t>
         </is>
       </c>
       <c r="N11" s="9" t="inlineStr">
@@ -35346,7 +35346,7 @@
       </c>
       <c r="Q11" s="9" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
@@ -35389,7 +35389,7 @@
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>『Pokémon Trading Card Game Pocket(ポケポケ)』の収益インパクトが引き続き注目。ゲーム事業に加えヘルスケア・スポーツ(横浜DeNAベイスターズ)を展開。大型の新規開示は乏しく、ポケポケの収益持続性が業績のカギ。</t>
+          <t>『ポケポケ(Pokémon TCG Pocket)』で初のテーマ拡張パック『幻のいる島』を追加し好材料視。ゲーム事業に加えヘルスケア・スポーツ(横浜DeNAベイスターズ)を展開。大型の新規開示は乏しく、ポケポケの収益持続性が業績のカギ。</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
@@ -35409,7 +35409,7 @@
       </c>
       <c r="Q12" s="9" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
@@ -35444,12 +35444,12 @@
       </c>
       <c r="M13" s="9" t="inlineStr">
         <is>
-          <t>英語版『ウマ娘』のヒットで海外展開が加速し、10〜3月は純利益72%増、ゲーム事業は増収増益。7/9に自社IP『グランブルーファンタジー リリンク：エンドレスラグナロク』の発売を控える。ゲーム/メディア/AI・広告の各事業が業績を牽引。</t>
+          <t>7/7に9日続伸で年初来高値を更新。FY9/26上期は売上4,785.84億円(+13.6%)営業益524.59億円(+79.8%)、ゲーム事業は売上1,322.27億円(+47.4%)営業益385.96億円(+106.3%)と急伸。7/9に『グラブル リリンク：エンドレスラグナロク』を発売、『ホロドリ』事前登録150万人突破。</t>
         </is>
       </c>
       <c r="N13" s="9" t="inlineStr">
         <is>
-          <t>英語版『ウマ娘』の海外ヒット、グラブル新作など自社IP強化</t>
+          <t>英語版『ウマ娘』の海外ヒットとゲーム事業の急伸、グラブル新作など自社IP強化、AI広告成長</t>
         </is>
       </c>
       <c r="O13" s="9" t="inlineStr">
@@ -35459,12 +35459,12 @@
       </c>
       <c r="P13" s="9" t="inlineStr">
         <is>
-          <t>『ウマ娘』海外定着とグラブル リリンク新作、AI広告事業の成長</t>
+          <t>『ウマ娘』海外定着とグラブル リリンク新作の初動、AI広告事業の成長</t>
         </is>
       </c>
       <c r="Q13" s="9" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
@@ -35612,7 +35612,7 @@
       </c>
       <c r="L2" s="9" t="inlineStr">
         <is>
-          <t>Xbox部門が新CEO Asha Sharma体制で大規模『reset』に着手。6/30の会計年度末後(7月)に大規模レイオフ(業界推計~1,000人規模)を実施見込みで、Double Fine/Undead Labs/Compulsion/Ninja Theory等のスタジオ再編・閉鎖の可能性も。Activision除くと5年で年間約$500M収益減が背景。</t>
+          <t>7/6にXbox部門で約3,200人(部門の約20%)の人員削減を発表、全社では約4,800人規模。Double Fine/Compulsion(IP保持し独立)・Ninja Theory/Undead Labs(新オーナーの下でSenua/State of Decay 3継続)の4スタジオを分離、Arkaneも仏労使審査次第。Asha Sharma新CEOは『マージンが同業の3〜10分の1』と説明。</t>
         </is>
       </c>
       <c r="M2" s="9" t="inlineStr">
@@ -35622,17 +35622,17 @@
       </c>
       <c r="N2" s="9" t="inlineStr">
         <is>
-          <t>Xbox大規模レイオフ・スタジオ再編、ハード事業の収益悪化</t>
+          <t>Xbox大規模レイオフ・スタジオ分離、ハード事業の低マージン、ファーストパーティ体制の再編途上</t>
         </is>
       </c>
       <c r="O2" s="9" t="inlineStr">
         <is>
-          <t>『reset』後のファーストパーティ体制、GTAⅥ商戦・Game Passの立て直し</t>
+          <t>『reset』後のファーストパーティ体制、GTAⅥ商戦・Game Passの立て直し、AI/クラウド基盤との統合</t>
         </is>
       </c>
       <c r="P2" s="9" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
@@ -35670,7 +35670,7 @@
       </c>
       <c r="L3" s="9" t="inlineStr">
         <is>
-          <t>最重要作『Grand Theft Auto VI』は2026年11月19日(PS5/Xbox)発売の据え置きを維持。延期後もライブサービス依存が薄い株として相対評価は良好。GTAⅥ発売を控え、期待先行の株価と発売遅延リスクが綱引き。</t>
+          <t>株価は$260.63と52週高値$264.79に接近(7/7)。BenchmarkはBuy/目標$300、BofAは$368へ引上げ。『GTAⅥ』は11/19発売・標準$79.99/アルティメット$99.99が確定し、仏Cdiscountの予約は通常大型作の6倍。FY27ネットブッキングは$8〜8.2bn(FY26約$6.7bn)を見込む。</t>
         </is>
       </c>
       <c r="M3" s="9" t="inlineStr">
@@ -35685,12 +35685,12 @@
       </c>
       <c r="O3" s="9" t="inlineStr">
         <is>
-          <t>GTAⅥ(11/19)の発売実現と初動規模、遅延リスクの解消</t>
+          <t>GTAⅥ(11/19)の発売実現と初動規模、FY27ネットブッキング$8bn超への牽引、遅延リスクの解消</t>
         </is>
       </c>
       <c r="P3" s="9" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
@@ -35728,7 +35728,7 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>『Battlefield 6』が10月発売以降1,000万本超を販売し2025年ベストセラーに。GTAⅥ延期の間隙を突いた戦略が奏功。EA SPORTS FC等ライブサービスと合わせ収益基盤は堅調で、フランチャイズ再興が評価される局面。</t>
+          <t>サウジPIF主導(Silver Lake/Affinity)の$55bn(1株$210)買収が進行、株価は過去最高$205.96(7/2)。欧州委員会は7/22までに承認可否を判断予定で、成立すれば史上最大のLBO・非公開化。『Battlefield 6』は1,000万本超の大ヒットでフランチャイズ戦略が奏功。</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
@@ -35738,17 +35738,17 @@
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>CFIUS審査長期化で6/30完了が不透明、アウトサイドデート9/28</t>
+          <t>欧州委の審査(7/22期限)など買収完了の不確実性、非公開化に伴う戦略変化、期待先行の株価</t>
         </is>
       </c>
       <c r="O4" s="9" t="inlineStr">
         <is>
-          <t>Battlefieldライブサービス化の定着、次期スポーツタイトルの更新需要</t>
+          <t>$55bn買収(7/22 EU判断)の成否、Battlefieldライブサービス化の定着、次期スポーツ更新需要</t>
         </is>
       </c>
       <c r="P4" s="9" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
@@ -35782,12 +35782,12 @@
       </c>
       <c r="L5" s="9" t="inlineStr">
         <is>
-          <t>直近開示で純損失€1,475.2m/売上€1,395.7mと依然赤字、資金は外部借入依存で株価は仏エンタメ指数に劣後。Tencent出資の新子会社への主力IP切り出しなど再建策の進捗が焦点。</t>
+          <t>7/9に『アサシン クリード ブラックフラッグ リシンクド』を発売。Tencentが新子会社Vantage Studios(AC/Far Cry/Rainbow Six保有)に€1.16bn出資し26.32%取得(評価額約€3.8〜4bn)、時価総額約$647Mの親会社を上回る。『AC Mirage』は無料拡張Valley of Memoryで1,000万プレイヤー到達。継続赤字と借入依存が重し。</t>
         </is>
       </c>
       <c r="M5" s="9" t="inlineStr">
         <is>
-          <t>広告(Grow)事業の回復とAI活用、アナリスト格上げ相次ぐ</t>
+          <t>Vantage Studiosへの巨額Tencent出資と主力IP集約、AC Mirage 1,000万PL到達、広告(Grow)回復</t>
         </is>
       </c>
       <c r="N5" s="9" t="inlineStr">
@@ -35797,12 +35797,12 @@
       </c>
       <c r="O5" s="9" t="inlineStr">
         <is>
-          <t>Assassin's Creed等主力IPの立て直し、新子会社を通じた再建策の実行</t>
+          <t>Assassin's Creed等主力IPの立て直し、Vantage Studiosを通じた再建策の実行、赤字縮小</t>
         </is>
       </c>
       <c r="P5" s="9" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
@@ -35836,7 +35836,7 @@
       </c>
       <c r="L6" s="9" t="inlineStr">
         <is>
-          <t>世界最大のゲーム企業として、ゲーム部門へのAI統合と海外展開が投資家の焦点。一部日本スタジオ保有株を損失覚悟でも売却する方向で交渉との報道。PUBG MobileやHonor of Kings等が引き続き稼ぎ頭。2026年は新作ローンチが堅調と目される。</t>
+          <t>7/5に香港のモバイルゲーム株が急伸しTencent(TCEHY)は$55.35で堅調。中国当局が2026年Q2に483本(前年比+13%)のゲーム版号を承認し規制緩和の転機と評価される。Honor of Kings/PUBG Mobile等が稼ぎ頭で、2026年は射撃・アクション中心にモバイル/PC/コンソールで新作投入を計画。</t>
         </is>
       </c>
       <c r="M6" s="9" t="inlineStr">
@@ -35851,12 +35851,12 @@
       </c>
       <c r="O6" s="9" t="inlineStr">
         <is>
-          <t>国内外の新作パイプライン、投資ポートフォリオ再編とAI収益化</t>
+          <t>版号増加を追い風にした新作パイプライン、AI×ゲーム統合と海外展開、投資ポートフォリオ再編</t>
         </is>
       </c>
       <c r="P6" s="9" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
@@ -35890,7 +35890,7 @@
       </c>
       <c r="L7" s="9" t="inlineStr">
         <is>
-          <t>2026年はTencentと並び新作ローンチが堅調と市場は評価。Identity V/荒野行動などライブサービスとグローバル向け新規IP投入が成長ドライバー。大きな新規開示は限定的で、次の四半期決算と新作の立ち上がり待ち。</t>
+          <t>新作PC『Sea of Ruin(逆水寒系)』の国内ローンチを7月に予定。『Justice: New World(燕雲十六聲)』は6/26配信後に売上ランキング5〜10位・プレイヤー数が2年ぶり高水準。二次上場完了を受け9月までにStock Connect組入れ見込み。堅調な新作パイプラインが成長ドライバー。</t>
         </is>
       </c>
       <c r="M7" s="9" t="inlineStr">
@@ -35905,12 +35905,12 @@
       </c>
       <c r="O7" s="9" t="inlineStr">
         <is>
-          <t>新規IPの海外定着、モバイル/PCマルチ展開の収益化</t>
+          <t>新規IPの海外定着とStock Connect組入れ、モバイル/PCマルチ展開の収益化</t>
         </is>
       </c>
       <c r="P7" s="9" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
@@ -35944,27 +35944,27 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>単一タイトル依存を減らす『Franchise IP』戦略に転換。CEO CH Kimが2年内リリースの26プロジェクト(『Subnautica 2』『Palworld Mobile』など12作)を提示。Hanwha AerospaceとフィジカルAI開発で提携するなど事業領域を拡張。</t>
+          <t>『Subnautica 2』が発売1時間で100万本・12時間で200万本・初週400万本の大ヒット。一方で開発元Unknown Worldsの全従業員へ$250M超のボーナス支払いで和解、CEO Ted Gillは辞任(7/1)。単一タイトル依存を減らす『Franchise IP』戦略の成果が問われる局面。</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>PUBG基盤＋『Franchise IP』戦略による新規IP拡充、豊富なパイプライン</t>
+          <t>『Subnautica 2』の大ヒット(初週400万本)、PUBG基盤＋Franchise IP戦略による新規IP拡充</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>最大$250Mアーンアウト負担と関連訴訟</t>
+          <t>$250M超のボーナス/アーンアウト負担と関連訴訟、経営陣交代、PUBG依存脱却の途上</t>
         </is>
       </c>
       <c r="O8" s="9" t="inlineStr">
         <is>
-          <t>Subnautica 2等新規IPの成功、PUBG以外の収益源多様化</t>
+          <t>Subnautica 2の販売継続と収益貢献、PUBG以外の新規IP多様化</t>
         </is>
       </c>
       <c r="P8" s="9" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
@@ -35998,7 +35998,7 @@
       </c>
       <c r="L9" s="9" t="inlineStr">
         <is>
-          <t>7/3時点で株価$14.18・時価総額約$11.2B、TTM売上$3.17B。『メイプルストーリー』『Dungeon&amp;Fighter』等ロングラン運営が収益基盤。大型の新規開示は乏しく、中国DnF/モバイルの課金動向が業績を左右する構図。</t>
+          <t>大型の新規開示は乏しく、『メイプルストーリー』『Dungeon&amp;Fighter』等ロングラン運営が収益基盤。中国DnF/モバイルの課金動向が業績を左右する構図が継続。Embark StudiosのシューターARC Raidersの販売動向も注目材料。</t>
         </is>
       </c>
       <c r="M9" s="9" t="inlineStr">
@@ -36018,7 +36018,7 @@
       </c>
       <c r="P9" s="9" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
@@ -36052,12 +36052,12 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>分社化・事業再編を継続中で、直近の大きな新規開示は限定的。負債圧縮とポートフォリオ整理の進捗、分割後の各社の独立採算化が引き続き市場の関心事。</t>
+          <t>2社への分割方針を推進。Tomb Raider/Lord of the Rings等のIPとCrystal Dynamicsを『Fellowship Entertainment』に集約し2027年にNasdaq Stockholm上場予定。Coffee Stain/Asmodeeは既に分離上場済。直近四半期は純売上SEK 5.2bn・調整後EBIT SEK 528mと改善。</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>事業分割で身軽化、Tomb Raider映像化等2027パイプライン</t>
+          <t>IP集約と事業分割で身軽化、Fellowship Entertainment上場計画、直近四半期の収益改善</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
@@ -36067,12 +36067,12 @@
       </c>
       <c r="O10" s="9" t="inlineStr">
         <is>
-          <t>分社化後の各社の独立採算化と収益改善</t>
+          <t>分社化後の各社の独立採算化、Fellowship(Tomb Raider/LotR)の2027上場、負債圧縮</t>
         </is>
       </c>
       <c r="P10" s="9" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
@@ -36106,7 +36106,7 @@
       </c>
       <c r="L11" s="9" t="inlineStr">
         <is>
-          <t>Q1 2026はEPS -$0.35(予想-$0.41を上回る)も売上$1.4Bは予想$1.74Bに未達。安全対策強化を背景に通期ガイダンスを下方修正(売上成長20-25%、ブッキング成長8-12%)。株価は約$56で6か月で-51%と低迷。次回決算は7/30頃の見込み。</t>
+          <t>Q2 2026決算を7/30に発表予定(EPS予想-$0.34、売上予想$1.59B/+10.7%)。未成年の年齢確認規制強化を背景に通期ブッキング成長見通しを8-12%へ下方修正済。株価は約$54.6でテクニカルは弱含み、決算前で様子見。アナリスト平均レーティングはBuy。</t>
         </is>
       </c>
       <c r="M11" s="9" t="inlineStr">
@@ -36126,7 +36126,7 @@
       </c>
       <c r="P11" s="9" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
@@ -36160,7 +36160,7 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Q1 2026予備売上$505-508Mでガイダンス($480-490M)を上回る。中国事業を$10億超で売却、ironSource Ads Networkを終了し広告を『Unity Vector』AIプラットフォームへ集約。中国売却観測で株価が一時+10%。AI広告のGrow売上は前年比+48%見込み。</t>
+          <t>株価は約$29.3で20/50/100日移動平均を上回り上向き。Q1売上$508M(+35% YoY)、Q4 2026にGAAP黒字化を見込む。『Unity Vector』AI広告が成長を牽引。Russell成長指数からの除外で機関投資家の可視性低下も、アナリスト平均目標$35.73でBuy優勢。</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
@@ -36175,12 +36175,12 @@
       </c>
       <c r="O12" s="9" t="inlineStr">
         <is>
-          <t>Vector広告の収益化加速、エンジン課金モデルの安定化</t>
+          <t>Vector AI広告の収益化加速、Q4 2026 GAAP黒字化、エンジン課金モデルの安定化</t>
         </is>
       </c>
       <c r="P12" s="9" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
@@ -36218,7 +36218,7 @@
       </c>
       <c r="L13" s="9" t="inlineStr">
         <is>
-          <t>株価は約$390でYTD -42%と、2026年のad-tech全般への逆風で調整。ただしAXON広告エンジンで依然として業界の支配的プレーヤーの地位を維持し高EBITDAマージンを確保。広告需要環境と規制動向が株価の変動要因。</t>
+          <t>株価は$543.79(7/7 +3.2%)。eコマース広告で広告主予算シェアを11.1%(+169bp)へ拡大。Q2売上は$1.815〜1.945Bの見通しでアナリストは強気(平均目標$658.71)。粗利益率約88%・EBITマージン80%超とAXON広告エンジンの高収益性が際立つ。</t>
         </is>
       </c>
       <c r="M13" s="9" t="inlineStr">
@@ -36233,12 +36233,12 @@
       </c>
       <c r="O13" s="9" t="inlineStr">
         <is>
-          <t>広告需要の回復、eコマース等新領域への広告拡張</t>
+          <t>AXON広告エンジンの拡張、eコマース等新領域への広告拡大、Q2決算での成長持続</t>
         </is>
       </c>
       <c r="P13" s="9" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
daily-news + cross-questions + events + predictions + game-design update (2026-07-13)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -817,7 +817,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1899,6 +1899,43 @@
       <c r="G29" s="14" t="inlineStr">
         <is>
           <t>Steamのストアページで『No Gen-AI』表記や絞り込み/バッジが増えるか、インディーが非AIを訴求軸に据える事例が増えるかを観測。</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B30" s="14" t="inlineStr">
+        <is>
+          <t>モバイルF2P専業各社が『枯れかけた主力IPの延命チャネル』として買い切りコンソール移植/新作を常設化し、Switch2向けミドル市場に移植専門ラインを新設する動きが広がる</t>
+        </is>
+      </c>
+      <c r="C30" s="14" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="D30" s="14" t="inlineStr">
+        <is>
+          <t>6〜12ヶ月</t>
+        </is>
+      </c>
+      <c r="E30" s="14" t="inlineStr">
+        <is>
+          <t>コロプラ,ミクシィ,gumi,任天堂</t>
+        </is>
+      </c>
+      <c r="F30" s="14" t="inlineStr">
+        <is>
+          <t>コロプラ『白猫プロジェクト INFINITY』Switch/Switch2で2027年発売発表（4Gamer, 2026-07-12）</t>
+        </is>
+      </c>
+      <c r="G30" s="14" t="inlineStr">
+        <is>
+          <t>他モバイル専業が既存IPのコンシューマ移植/新作を発表するか、各社IRで『コンシューマ事業』への言及・専門組織の新設が増えるかを観測。Switch2向け中規模タイトル本数の推移も指標。</t>
         </is>
       </c>
     </row>
@@ -3936,7 +3973,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G69"/>
+  <dimension ref="A1:G71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6498,6 +6535,80 @@
       <c r="G69" s="14" t="inlineStr">
         <is>
           <t>プラットフォームが購入導線を内製化する構図はゲーム外でも進行中で、第三者メディアの中抜き余地が縮む共通課題。</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B70" s="14" t="inlineStr">
+        <is>
+          <t>ゲーム/マンガ制作ツールのサブスク化×AI追い風による最高益は、映像・音楽・設計(CAD)など他クリエイティブツール業界でも同時に起きるか？</t>
+        </is>
+      </c>
+      <c r="C70" s="14" t="inlineStr">
+        <is>
+          <t>セルシス上期42%上方修正・過去最高益（株探）</t>
+        </is>
+      </c>
+      <c r="D70" s="14" t="inlineStr">
+        <is>
+          <t>セルシス,CLIP STUDIO PAINT</t>
+        </is>
+      </c>
+      <c r="E70" s="14" t="inlineStr">
+        <is>
+          <t>SaaS/クリエイティブツール（Adobe等）、映像・音楽制作、CAD/設計ソフト</t>
+        </is>
+      </c>
+      <c r="F70" s="14" t="inlineStr">
+        <is>
+          <t>オープン</t>
+        </is>
+      </c>
+      <c r="G70" s="14" t="inlineStr">
+        <is>
+          <t>生成AIは制作ツールの脅威と語られがちだが、プロ現場ツールは逆に追い風で最高益。『AIが代替する層』と『AIで底上げされる専門ツール層』の二極化を他業界にも当てはめて観測したい。</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B71" s="14" t="inlineStr">
+        <is>
+          <t>アミューズメント運営の増益が本業でなく為替差益ドリブンである構造は、他の内需×海外展開企業(小売・外食)の決算の質をどう見分けるべきか？</t>
+        </is>
+      </c>
+      <c r="C71" s="14" t="inlineStr">
+        <is>
+          <t>イオンファンタジー1Q 純利益577%増（TDnet）</t>
+        </is>
+      </c>
+      <c r="D71" s="14" t="inlineStr">
+        <is>
+          <t>イオンファンタジー,イオン</t>
+        </is>
+      </c>
+      <c r="E71" s="14" t="inlineStr">
+        <is>
+          <t>小売・外食のグローバル展開、インバウンド関連、商社</t>
+        </is>
+      </c>
+      <c r="F71" s="14" t="inlineStr">
+        <is>
+          <t>オープン</t>
+        </is>
+      </c>
+      <c r="G71" s="14" t="inlineStr">
+        <is>
+          <t>純利益の急伸見出しに対し、営業利益ベースでは+9%。海外比率の高い内需企業は円安局面で純利益が膨らみやすく、決算の『実力』を営業利益で見る目線が他業界の海外展開企業にも共通で必要。</t>
         </is>
       </c>
     </row>
@@ -10729,12 +10840,12 @@
       </c>
       <c r="I25" s="14" t="inlineStr">
         <is>
-          <t>開催中</t>
+          <t>終了</t>
         </is>
       </c>
       <c r="J25" s="14" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
@@ -10801,7 +10912,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11516,6 +11627,56 @@
       </c>
       <c r="J14" s="14" t="n">
         <v>4</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B15" s="14" t="inlineStr">
+        <is>
+          <t>モバイルF2P-IPの買い切りコンソール化（脱ガチャ移植）</t>
+        </is>
+      </c>
+      <c r="C15" s="14" t="inlineStr">
+        <is>
+          <t>マネタイズ/構造</t>
+        </is>
+      </c>
+      <c r="D15" s="14" t="inlineStr">
+        <is>
+          <t>台頭</t>
+        </is>
+      </c>
+      <c r="E15" s="14" t="inlineStr">
+        <is>
+          <t>モバイルでガチャ運営してきた主力IPを、コンシューマ向けの買い切り/オリジナル新作として再構築する型。運営疲弊・モバイル新規頭打ちの受け皿として、IP資産をコンソールの一括販売モデルに載せ替える。</t>
+        </is>
+      </c>
+      <c r="F15" s="14" t="inlineStr">
+        <is>
+          <t>白猫プロジェクト INFINITY(コロプラ)</t>
+        </is>
+      </c>
+      <c r="G15" s="14" t="inlineStr">
+        <is>
+          <t>モバイル新作の低調・ユーザー獲得コスト高騰と、Switch2という新ハードのインストールベース拡大。既存モバイルIPの認知を活かしつつ課金モデルを買い切りに転換する動機。</t>
+        </is>
+      </c>
+      <c r="H15" s="14" t="inlineStr">
+        <is>
+          <t>モバイル専業のコンソール移植が定着すれば、ガチャ運営IPの『第二の人生』としてコンソール買い切り版が標準オプション化する可能性。成否は移植版の売上とIP再燃効果に依存。</t>
+        </is>
+      </c>
+      <c r="I15" s="14" t="inlineStr">
+        <is>
+          <t>『白猫プロジェクト INFINITY』2027年発売発表（4Gamer, 2026-07-12）</t>
+        </is>
+      </c>
+      <c r="J15" s="14" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -12794,7 +12955,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L296"/>
+  <dimension ref="A1:L302"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -31138,6 +31299,374 @@
         </is>
       </c>
       <c r="L296" s="14" t="inlineStr"/>
+    </row>
+    <row r="297">
+      <c r="A297" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B297" s="14" t="inlineStr">
+        <is>
+          <t>コロプラ、Switch/Switch2向け新作『白猫プロジェクト INFINITY』を2027年発売と発表</t>
+        </is>
+      </c>
+      <c r="C297" s="14" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/024/G102434/20260712005/</t>
+        </is>
+      </c>
+      <c r="D297" s="14" t="inlineStr">
+        <is>
+          <t>スマホ向けアクションRPG『白猫プロジェクト』は12周年を迎える長寿F2Pタイトル。コロプラはモバイル新作低調が続くなか、PC/コンシューマ10本規模の開発パイプラインを公言しており、主力IPの据置機展開はその中核施策。12周年記念ステージで発表された。</t>
+        </is>
+      </c>
+      <c r="E297" s="14" t="inlineStr">
+        <is>
+          <t>コロプラが『白猫プロジェクト INFINITY』をNintendo Switch/Switch 2向けに2027年発売予定と発表。移植ではなくオリジナルのアクション作で、シリーズキャラ50人以上が登場、「キャラリンクが爆増する爽快アクション」をコンセプトに据える。モバイル専業がコンシューマ買い切りへ本格進出する象徴例。</t>
+        </is>
+      </c>
+      <c r="F297" s="14" t="inlineStr">
+        <is>
+          <t>モバイル専業コロプラが主力IPを据置機の新作として展開
+Switch/Switch2両対応、2027年発売予定
+移植でなくオリジナルのアクションゲーム
+登場キャラ50人以上・オリジナルキャラも
+12周年イベントで発表、コンシューマ事業強化の一環</t>
+        </is>
+      </c>
+      <c r="G297" s="14" t="inlineStr">
+        <is>
+          <t>モバイルF2Pで成熟したIPを買い切りコンソールで延命・再評価する流れが強まる見込み。ミクシィ・gumi等の他モバイル専業も、既存IPのコンシューマ移植・新作部隊を新設して追随する可能性がある。Switch2の中規模市場が受け皿になるか注目。</t>
+        </is>
+      </c>
+      <c r="H297" s="14" t="inlineStr">
+        <is>
+          <t>モバイルIPのマルチプラットフォーム/コンシューマ移行戦略</t>
+        </is>
+      </c>
+      <c r="I297" s="14" t="inlineStr">
+        <is>
+          <t>コロプラ,任天堂</t>
+        </is>
+      </c>
+      <c r="J297" s="14" t="inlineStr">
+        <is>
+          <t>白猫プロジェクト,白猫プロジェクト INFINITY,Nintendo Switch 2</t>
+        </is>
+      </c>
+      <c r="K297" s="14" t="inlineStr">
+        <is>
+          <t>新作,国内</t>
+        </is>
+      </c>
+      <c r="L297" s="14" t="n"/>
+    </row>
+    <row r="298">
+      <c r="A298" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B298" s="14" t="inlineStr">
+        <is>
+          <t>セルシス、上期経常を42%上方修正——『CLIP STUDIO PAINT』好調で過去最高益予想に上乗せ</t>
+        </is>
+      </c>
+      <c r="C298" s="14" t="inlineStr">
+        <is>
+          <t>https://s.kabutan.jp/news/k202607100002/</t>
+        </is>
+      </c>
+      <c r="D298" s="14" t="inlineStr">
+        <is>
+          <t>セルシスはマンガ・イラスト・アニメ制作ソフト『CLIP STUDIO PAINT』を主力とする上場企業（3663）。2026年3月にver.5.0メジャーアップデートを投入し、買い切り・サブスク双方が計画を上回って推移していた。35周年で記念増配も実施済み。</t>
+        </is>
+      </c>
+      <c r="E298" s="14" t="inlineStr">
+        <is>
+          <t>セルシスが2026年12月期上期の経常利益予想を15.7億円→22.4億円へ41.9%上方修正し、過去最高益予想を上乗せ。ver.5.0好評とプロモ奏功で買い切り・サブスク双方が計画超過、コスト抑制も寄与。クリエイター向けツールの生成AI時代における底堅さを示す決算。</t>
+        </is>
+      </c>
+      <c r="F298" s="14" t="inlineStr">
+        <is>
+          <t>上期経常を42%上方修正、過去最高益予想に
+CLIP STUDIO PAINT ver.5.0が牽引
+買い切り・サブスク双方が計画超過
+広告費・原価のコスト抑制も利益に寄与
+35周年記念で増配（年40円→50円）</t>
+        </is>
+      </c>
+      <c r="G298" s="14" t="inlineStr">
+        <is>
+          <t>生成AIによる画像生成が普及するなかでも、プロ制作の現場ツールとしてのクリスタ需要は堅調に推移する見込み。制作管理システム連携などプロ現場への浸透が続けば、サブスク比率上昇でストック収益がさらに厚くなる可能性が高い。</t>
+        </is>
+      </c>
+      <c r="H298" s="14" t="inlineStr">
+        <is>
+          <t>クリエイティブSaaSのサブスク化とAI時代の競争優位</t>
+        </is>
+      </c>
+      <c r="I298" s="14" t="inlineStr">
+        <is>
+          <t>セルシス</t>
+        </is>
+      </c>
+      <c r="J298" s="14" t="inlineStr">
+        <is>
+          <t>CLIP STUDIO PAINT</t>
+        </is>
+      </c>
+      <c r="K298" s="14" t="inlineStr">
+        <is>
+          <t>業績,国内</t>
+        </is>
+      </c>
+      <c r="L298" s="14" t="n"/>
+    </row>
+    <row r="299">
+      <c r="A299" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B299" s="14" t="inlineStr">
+        <is>
+          <t>イオンファンタジー1Q、純利益577%増——増収増益で売上・営業益とも過去最高</t>
+        </is>
+      </c>
+      <c r="C299" s="14" t="inlineStr">
+        <is>
+          <t>https://www.release.tdnet.info/inbs/140120260710591450.pdf</t>
+        </is>
+      </c>
+      <c r="D299" s="14" t="inlineStr">
+        <is>
+          <t>イオンファンタジー（4343）はイオンモール等で屋内遊園地・アミューズメント施設を国内外展開する上場企業。国内は堅調、海外（中国・ASEAN）比率が高く為替感応度が大きい。2027年2月期第1四半期（3〜5月）決算を7/10開示した。</t>
+        </is>
+      </c>
+      <c r="E299" s="14" t="inlineStr">
+        <is>
+          <t>イオンファンタジーの1Q連結は売上高245.75億円（前年比+12.2%）、営業利益13.36億円（+9.3%）で共に過去最高。円安による為替差益5.47億円を計上し、純利益は9.86億円（+577.1%）と急伸。ただし純利益急増の主因は本業でなく為替差益である点に留意。</t>
+        </is>
+      </c>
+      <c r="F299" s="14" t="inlineStr">
+        <is>
+          <t>売上・営業益とも過去最高（4期・2期連続）
+純利益は前年比577.1%増の9.86億円
+急増の主因は為替差益5.47億円（前年は差損）
+海外アミューズメント比率の高さが為替感応度に直結
+インバウンド/国内も堅調</t>
+        </is>
+      </c>
+      <c r="G299" s="14" t="inlineStr">
+        <is>
+          <t>本業（施設運営）の増益基調は続くが、純利益は為替次第で振れが大きい。円高転換局面では逆に差損計上で純利益が急減するリスクがあり、営業利益ベースでの実力評価が重要になる。海外出店ペースが今後の成長ドライバー。</t>
+        </is>
+      </c>
+      <c r="H299" s="14" t="inlineStr">
+        <is>
+          <t>決算の質（本業利益vs為替/一時要因）の見分け方</t>
+        </is>
+      </c>
+      <c r="I299" s="14" t="inlineStr">
+        <is>
+          <t>イオンファンタジー,イオン</t>
+        </is>
+      </c>
+      <c r="J299" s="14" t="inlineStr"/>
+      <c r="K299" s="14" t="inlineStr">
+        <is>
+          <t>業績,国内</t>
+        </is>
+      </c>
+      <c r="L299" s="14" t="n"/>
+    </row>
+    <row r="300">
+      <c r="A300" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B300" s="14" t="inlineStr">
+        <is>
+          <t>eスポーツW杯2026 VALORANT部門、100 ThievesがNRGを3-1で下し優勝</t>
+        </is>
+      </c>
+      <c r="C300" s="14" t="inlineStr">
+        <is>
+          <t>https://www.vlr.gg/event/2952/esports-world-cup-2026</t>
+        </is>
+      </c>
+      <c r="D300" s="14" t="inlineStr">
+        <is>
+          <t>サウジ主導のEsports World Cup 2026（7/6〜8/23、賞金総額最大規模）は複数タイトルを横断する大型eスポーツ大会。VALORANT部門は7/2〜7/12にパリで開催、16チームが賞金200万ドルを争った。決勝は北米勢同士の対戦に。</t>
+        </is>
+      </c>
+      <c r="E300" s="14" t="inlineStr">
+        <is>
+          <t>EWC2026 VALORANT部門のグランドファイナルで、100 ThievesがNRGを3-1で破り優勝。北米勢同士の頂上決戦を制した。EWCはクラブ横断のポイント争いも兼ねており、各運営組織の年間表彰・スポンサー価値に直結する。VALORANT eスポーツの北米地域の強さを示す結果。</t>
+        </is>
+      </c>
+      <c r="F300" s="14" t="inlineStr">
+        <is>
+          <t>100 ThievesがNRGを3-1で下し優勝
+北米勢同士のグランドファイナル
+賞金プール200万ドル、16チーム参加
+EWCクラブ選手権のポイントにも加算
+VALORANT部門はパリで7/2〜7/12開催</t>
+        </is>
+      </c>
+      <c r="G300" s="14" t="inlineStr">
+        <is>
+          <t>EWCの高額賞金・クラブポイント制は、運営組織の収益源をスポンサー依存から大会賞金・順位報酬へ多様化させる。サウジ資本主導の賞金インフレが続けば、他地域リーグの選手年俸・移籍市場にも波及する可能性がある。</t>
+        </is>
+      </c>
+      <c r="H300" s="14" t="inlineStr">
+        <is>
+          <t>eスポーツの賞金設計とクラブ経営の収益多様化</t>
+        </is>
+      </c>
+      <c r="I300" s="14" t="inlineStr">
+        <is>
+          <t>Riot Games,100 Thieves,NRG</t>
+        </is>
+      </c>
+      <c r="J300" s="14" t="inlineStr">
+        <is>
+          <t>VALORANT,Esports World Cup 2026</t>
+        </is>
+      </c>
+      <c r="K300" s="14" t="inlineStr">
+        <is>
+          <t>eスポーツ,海外</t>
+        </is>
+      </c>
+      <c r="L300" s="14" t="n"/>
+    </row>
+    <row r="301">
+      <c r="A301" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B301" s="14" t="inlineStr">
+        <is>
+          <t>サイバーエージェント上期、営業利益524億円超——ゲーム『学マス』とネット広告好調で通期レンジ下限超過</t>
+        </is>
+      </c>
+      <c r="C301" s="14" t="inlineStr">
+        <is>
+          <t>https://news.livedoor.com/topics/detail/31769508/</t>
+        </is>
+      </c>
+      <c r="D301" s="14" t="inlineStr">
+        <is>
+          <t>サイバーエージェント（4751）はゲーム（『学園アイドルマスター』等）・ネット広告・メディア（ABEMA）を展開。ゲーム事業と広告事業がともに堅調で、上期段階から通期会社計画に対する進捗が良好だった。</t>
+        </is>
+      </c>
+      <c r="E301" s="14" t="inlineStr">
+        <is>
+          <t>サイバーエージェントの上期業績が、ゲーム・ネット広告事業の好調で上期営業利益524億円超と、通期予想レンジの下限値を上期時点で既に超過。『学園アイドルマスター』の貢献と広告の回復が寄与。ゲームIPと広告の両輪が業績を押し上げる構図が続く。</t>
+        </is>
+      </c>
+      <c r="F301" s="14" t="inlineStr">
+        <is>
+          <t>上期営業利益524億円超で通期レンジ下限を超過
+ゲーム『学マス』が業績に大きく貢献
+ネット広告事業も回復・好調
+ゲームと広告の両輪で収益ドライブ
+通期上振れ期待が高まる決算</t>
+        </is>
+      </c>
+      <c r="G301" s="14" t="inlineStr">
+        <is>
+          <t>単一ヒットIP（学マス）への依存度が高い分、次の柱育成とライブオプス継続が課題。広告の回復基調が続けば全社利益の下支えになるが、ゲーム収益の逓減リスクに対する新作パイプラインの厚みが今後の鍵。</t>
+        </is>
+      </c>
+      <c r="H301" s="14" t="inlineStr">
+        <is>
+          <t>ゲームIPポートフォリオと広告事業のシナジー</t>
+        </is>
+      </c>
+      <c r="I301" s="14" t="inlineStr">
+        <is>
+          <t>サイバーエージェント,QualiArts</t>
+        </is>
+      </c>
+      <c r="J301" s="14" t="inlineStr">
+        <is>
+          <t>学園アイドルマスター</t>
+        </is>
+      </c>
+      <c r="K301" s="14" t="inlineStr">
+        <is>
+          <t>業績,国内</t>
+        </is>
+      </c>
+      <c r="L301" s="14" t="n"/>
+    </row>
+    <row r="302">
+      <c r="A302" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B302" s="14" t="inlineStr">
+        <is>
+          <t>Amazonプライムデー2026（〜7/13）、ゲーム関連セール・IPコラボ商品が集中</t>
+        </is>
+      </c>
+      <c r="C302" s="14" t="inlineStr">
+        <is>
+          <t>https://www.nbcnews.com/select/shopping/prime-day-gaming-deals-nintendo-playstation-xbox-2026-rcna351952</t>
+        </is>
+      </c>
+      <c r="D302" s="14" t="inlineStr">
+        <is>
+          <t>Amazonのプライム会員向け大型セール「プライムデー2026」が7/13まで開催。ゲームソフト・ハード周辺機器が最大7割超引きとなり、国内でも『崩壊：スターレイル』コラボ充電器など人気IPを絡めた限定商品が投入された。Steam/eShopの各サマーセールと時期が重なる。</t>
+        </is>
+      </c>
+      <c r="E302" s="14" t="inlineStr">
+        <is>
+          <t>プライムデー2026でPS5/Switch向けAAA（『ペルソナ3 リロード』73%オフ等）やハード周辺機器が大幅値引き。国内ではゲームIPコラボのガジェット限定モデルも展開。プラットフォーム横断でセールが集中し、夏商戦の需要が特定ウィンドウに前倒しで集中する構図が強まる。</t>
+        </is>
+      </c>
+      <c r="F302" s="14" t="inlineStr">
+        <is>
+          <t>プライム会員限定でゲーム関連が最大7割超引き
+PS5/Switch向けAAAタイトルが対象
+ゲームIPコラボの周辺機器・ガジェット限定モデルも
+Steam/eShopサマーセールと時期が重複
+7/13まで開催</t>
+        </is>
+      </c>
+      <c r="G302" s="14" t="inlineStr">
+        <is>
+          <t>小売プラットフォーム主導のセール集中は、パブリッシャーの値引き原資と発売タイミング戦略に影響。夏商戦がプライムデー/Steamセールの短期ウィンドウに集約されるほど、その期間外の新作は埋没しやすく、発売日設計がセール暦に従属していく可能性。</t>
+        </is>
+      </c>
+      <c r="H302" s="14" t="inlineStr">
+        <is>
+          <t>小売プラットフォームのセール暦とゲーム販売設計</t>
+        </is>
+      </c>
+      <c r="I302" s="14" t="inlineStr">
+        <is>
+          <t>Amazon,ソニー,任天堂</t>
+        </is>
+      </c>
+      <c r="J302" s="14" t="inlineStr">
+        <is>
+          <t>ペルソナ3 リロード,崩壊：スターレイル</t>
+        </is>
+      </c>
+      <c r="K302" s="14" t="inlineStr">
+        <is>
+          <t>eスポーツ,国内,海外</t>
+        </is>
+      </c>
+      <c r="L302" s="14" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
daily-news + cross-questions + events + predictions + game-design update (2026-07-14)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -817,7 +817,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1936,6 +1936,43 @@
       <c r="G30" s="14" t="inlineStr">
         <is>
           <t>他モバイル専業が既存IPのコンシューマ移植/新作を発表するか、各社IRで『コンシューマ事業』への言及・専門組織の新設が増えるかを観測。Switch2向け中規模タイトル本数の推移も指標。</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B31" s="14" t="inlineStr">
+        <is>
+          <t>中国の版号承認回復(+13%)で国内リリース枠は開くが、供給過多で中堅スタジオの採算が悪化し、Tencent/NetEase等の大手による“救済的な被買収/海外パブリッシング委託”に回る中堅が増える(下流の垂直吸収)</t>
+        </is>
+      </c>
+      <c r="C31" s="14" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="D31" s="14" t="inlineStr">
+        <is>
+          <t>6〜12ヶ月</t>
+        </is>
+      </c>
+      <c r="E31" s="14" t="inlineStr">
+        <is>
+          <t>Tencent, NetEase, 中国中堅スタジオ</t>
+        </is>
+      </c>
+      <c r="F31" s="14" t="inlineStr">
+        <is>
+          <t>①中国NPPA Q2 483版号+13%→モバイル株上昇(GuruFocus) ②2026年Q2ゲームM&amp;A 23億ドルで最高(Outlook Respawn)</t>
+        </is>
+      </c>
+      <c r="G31" s="14" t="inlineStr">
+        <is>
+          <t>InvestGame等の四半期M&amp;Aレポートで中国発ディール(被買収・出資)件数の増減を観測。大手の海外パブリッシング契約数の推移も指標。</t>
         </is>
       </c>
     </row>
@@ -3973,7 +4010,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G71"/>
+  <dimension ref="A1:G73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6609,6 +6646,80 @@
       <c r="G71" s="14" t="inlineStr">
         <is>
           <t>純利益の急伸見出しに対し、営業利益ベースでは+9%。海外比率の高い内需企業は円安局面で純利益が膨らみやすく、決算の『実力』を営業利益で見る目線が他業界の海外展開企業にも共通で必要。</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B72" s="14" t="inlineStr">
+        <is>
+          <t>プラットフォーマー/巨大資本が『非支配的な少数出資の束』で業界横断の影響力を確立する構造(Tencentの韓国勢筆頭級株主化)は、日本の商社の政策保有株やメディアの資本業務提携ネットワークと同じ現象か？</t>
+        </is>
+      </c>
+      <c r="C72" s="14" t="inlineStr">
+        <is>
+          <t>Tencentが韓国ゲーム勢(Shift Up/Krafton/Netmarble)で筆頭級株主に(Korea Herald)</t>
+        </is>
+      </c>
+      <c r="D72" s="14" t="inlineStr">
+        <is>
+          <t>Tencent, Shift Up, Krafton, Netmarble</t>
+        </is>
+      </c>
+      <c r="E72" s="14" t="inlineStr">
+        <is>
+          <t>総合商社(政策保有), メディア(資本業務提携/持ち合い), 金融(GP-LP・アンカー出資)</t>
+        </is>
+      </c>
+      <c r="F72" s="14" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="G72" s="14" t="inlineStr">
+        <is>
+          <t>『支配なき影響力』は議決権比率では測れない。配信網・IPアクセスの依存度が実効的な支配になる点が共通軸。</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B73" s="14" t="inlineStr">
+        <is>
+          <t>規制当局の『発行枠(ライセンス数)』が実質的に業界の供給量と株価を統制する構造(中国の版号交付ペース→モバイル株上昇)は、ゲーム版号だけでなく医薬品承認・カジノ免許・放送/通信免許でも同型か？</t>
+        </is>
+      </c>
+      <c r="C73" s="14" t="inlineStr">
+        <is>
+          <t>中国NPPAがQ2に483版号交付(+13%)、香港モバイルゲーム株が上昇(GuruFocus)</t>
+        </is>
+      </c>
+      <c r="D73" s="14" t="inlineStr">
+        <is>
+          <t>Tencent, NetEase, Bilibili, IGG</t>
+        </is>
+      </c>
+      <c r="E73" s="14" t="inlineStr">
+        <is>
+          <t>医薬(承認件数と株価), カジノ/公営競技(免許数), 放送・通信(免許/周波数割当)</t>
+        </is>
+      </c>
+      <c r="F73" s="14" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="G73" s="14" t="inlineStr">
+        <is>
+          <t>供給を数量で絞る規制は、モノの良し悪しより『枠の開閉』が業績・株価を動かす。政策変数の可視化が投資判断の鍵。</t>
         </is>
       </c>
     </row>
@@ -11232,7 +11343,7 @@
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
@@ -11247,7 +11358,7 @@
       </c>
       <c r="D7" s="14" t="inlineStr">
         <is>
-          <t>台頭</t>
+          <t>台頭(加速)</t>
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr">
@@ -11267,12 +11378,12 @@
       </c>
       <c r="H7" s="14" t="inlineStr">
         <is>
-          <t>真正性が効率に勝つニッチが拡大。表示義務化で非AIがラベル/フィルタとして商品価値化し、AI活用と非AI訴求の二極化が加速。</t>
+          <t>生成AI逆風(開発者52%が悪影響)とgameslop氾濫を追い風に、『非AI・人の手』保証が購買シグナルとして定着へ</t>
         </is>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
-          <t>EU AI Act透明性義務が8/2適用開始(本日追記の日次ニュース)</t>
+          <t>EU AI Act透明性義務が8/2適用開始(本日追記の日次ニュース) / 生成AI逆風・開発者52%が悪影響/gameslop(GameDeveloper/2026-07-14)</t>
         </is>
       </c>
       <c r="J7" s="14" t="n">
@@ -11582,7 +11693,7 @@
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B14" s="14" t="inlineStr">
@@ -11612,21 +11723,21 @@
       </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
-          <t>Palworldが早期アクセスで大量プレイヤーを獲得し2026/7/10に1.0化。収集×サバイバルの融合が一つの完成型として定着。</t>
+          <t>爆発的ヒットの継続。Palworld正式版1.0(累計4000万人)で代表作の到達点を示し、フォロワー作の設計テンプレ化が進む</t>
         </is>
       </c>
       <c r="H14" s="14" t="inlineStr">
         <is>
-          <t>追随タイトルが増える一方、収集デザインの意匠・特許リスク(任天堂/ポケモン訴訟)が参入時の設計制約に。無料大型アップデート運営が標準化。</t>
+          <t>正式版化で運営型(コラボ/DLC)へ移行。クリーチャー収集×建築×PvEの掛け合わせは定番ジャンル化する見込み</t>
         </is>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
-          <t>Palworld 1.0正式リリース(Gematsu,2026-07-10)</t>
+          <t>『パルワールド』正式版1.0リリース・累計4000万人(ファミ通/2026-07-14)</t>
         </is>
       </c>
       <c r="J14" s="14" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15">
@@ -12955,7 +13066,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L302"/>
+  <dimension ref="A1:L310"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -31667,6 +31778,486 @@
         </is>
       </c>
       <c r="L302" s="14" t="n"/>
+    </row>
+    <row r="303">
+      <c r="A303" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B303" s="14" t="inlineStr">
+        <is>
+          <t>Tencent、韓国ゲーム・コンテンツへの少数出資を深化——Shift Up/Krafton/Netmarbleで筆頭級株主に</t>
+        </is>
+      </c>
+      <c r="C303" s="14" t="inlineStr">
+        <is>
+          <t>https://www.koreaherald.com/article/10508695</t>
+        </is>
+      </c>
+      <c r="D303" s="14" t="inlineStr">
+        <is>
+          <t>Tencentはここ数年、中国国内の版号規制と成長鈍化を背景に、海外の有力スタジオへ非支配的な少数出資を積み増してきた。特に韓国はグローバルヒットIPの供給源で、Shift Up(勝利の女神)やKraftonが主要ターゲット。</t>
+        </is>
+      </c>
+      <c r="E303" s="14" t="inlineStr">
+        <is>
+          <t>報道によればTencentはShift Upの34.76%、Kraftonの13.71%、Netmarbleの17.52%を保有し、いずれも第2位株主級の影響力を確保。経営権を取らずに配信・IPアクセスを囲い込む『支配なき影響力』戦略が鮮明になった。</t>
+        </is>
+      </c>
+      <c r="F303" s="14" t="inlineStr">
+        <is>
+          <t>Shift Up 34.76%・Krafton 13.71%・Netmarble 17.52%を保有
+経営権非取得のまま筆頭級株主として影響力を確保
+韓国コンテンツのグローバル配信網への接続が狙い
+韓国内で外資の資本影響力への警戒論も</t>
+        </is>
+      </c>
+      <c r="G303" s="14" t="inlineStr">
+        <is>
+          <t>非支配的な少数出資の束で業界横断の影響力を築く動きは今後も継続。韓国政府・公取委が外資プラットフォーマーの資本影響力を問題視し、開示・規制論議が再燃する可能性。</t>
+        </is>
+      </c>
+      <c r="H303" s="14" t="inlineStr">
+        <is>
+          <t>少数出資による支配・議決権と実効支配の関係</t>
+        </is>
+      </c>
+      <c r="I303" s="14" t="inlineStr">
+        <is>
+          <t>Tencent, Shift Up, Krafton, Netmarble</t>
+        </is>
+      </c>
+      <c r="J303" s="14" t="inlineStr">
+        <is>
+          <t>勝利の女神:NIKKE, PUBG</t>
+        </is>
+      </c>
+      <c r="K303" s="14" t="inlineStr">
+        <is>
+          <t>M&amp;A,海外,規制</t>
+        </is>
+      </c>
+      <c r="L303" s="14" t="inlineStr"/>
+    </row>
+    <row r="304">
+      <c r="A304" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B304" s="14" t="inlineStr">
+        <is>
+          <t>2026年Q2のゲームM&amp;Aが23億ドル・54件で2022年以来最高——Scopely×Loom Games(10億ドル)が最大</t>
+        </is>
+      </c>
+      <c r="C304" s="14" t="inlineStr">
+        <is>
+          <t>https://respawn.outlookindia.com/gaming/gaming-news/q2-2026-gaming-industry-ma-reaches-23b-amid-mid-market-boom</t>
+        </is>
+      </c>
+      <c r="D304" s="14" t="inlineStr">
+        <is>
+          <t>2022年以降のゲーム業界は大型レイオフと株価低迷が続いたが、金利・評価額の調整を経て2026年に入りディール環境が改善。メガディールよりPC・カジュアルモバイルの中堅を狙うミッドマーケットが牽引役に。</t>
+        </is>
+      </c>
+      <c r="E304" s="14" t="inlineStr">
+        <is>
+          <t>2026年Q2のゲームM&amp;Aは総額23億ドル・54件と、件数ベースで2022年以来最高。最大案件はScopelyによるLoom Gamesの10億ドル買収、次いでWeMade創業者持分の5.91億ドル売却(NeoPulse向け)。</t>
+        </is>
+      </c>
+      <c r="F304" s="14" t="inlineStr">
+        <is>
+          <t>Q2総額23億ドル・54件で2022年以来最多
+最大はScopely×Loom Games(10億ドル)
+2位はWeMade創業者持分5.91億ドル売却
+メガディールでなく中堅ディールが牽引
+一方ゲーム株は年初来で軟調(アジアモバイル勢-37〜42%)</t>
+        </is>
+      </c>
+      <c r="G304" s="14" t="inlineStr">
+        <is>
+          <t>評価額の底打ちで中堅スタジオの売買が活性化。上場モバイル勢の株価低迷が続けば、非公開化(take-private)や大手による中堅救済買収がさらに増える見込み。</t>
+        </is>
+      </c>
+      <c r="H304" s="14" t="inlineStr">
+        <is>
+          <t>ミッドマーケットM&amp;Aとバリュエーション回復</t>
+        </is>
+      </c>
+      <c r="I304" s="14" t="inlineStr">
+        <is>
+          <t>Scopely, Loom Games, WeMade, NeoPulse</t>
+        </is>
+      </c>
+      <c r="J304" s="14" t="inlineStr"/>
+      <c r="K304" s="14" t="inlineStr">
+        <is>
+          <t>M&amp;A,海外,業績</t>
+        </is>
+      </c>
+      <c r="L304" s="14" t="inlineStr"/>
+    </row>
+    <row r="305">
+      <c r="A305" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B305" s="14" t="inlineStr">
+        <is>
+          <t>EA $55B買収(史上最大のLBO)が規制審査の最終局面——アウトサイドデートは9/28</t>
+        </is>
+      </c>
+      <c r="C305" s="14" t="inlineStr">
+        <is>
+          <t>https://theconversation.com/what-the-us-55-billion-electronic-arts-takeover-means-for-video-game-workers-and-the-industry-267206</t>
+        </is>
+      </c>
+      <c r="D305" s="14" t="inlineStr">
+        <is>
+          <t>2025年9月、EAはPIF・Silver Lake・Affinity Partnersの連合による総額550億ドルの非公開化(1株210ドル)に合意。史上最大のオールキャッシュLBOで、JPモルガンが200億ドルの融資を提供した。</t>
+        </is>
+      </c>
+      <c r="E305" s="14" t="inlineStr">
+        <is>
+          <t>株主承認(2025/12)を経て、案件はCFIUS・欧州委員会の規制審査という最終段階に。アウトサイドデートは9/28に延長済みで、6/30前後のクロージングが見込まれる。Andrew Wilson CEOは続投予定。</t>
+        </is>
+      </c>
+      <c r="F305" s="14" t="inlineStr">
+        <is>
+          <t>買収総額550億ドル(1株210ドル)で史上最大のLBO
+連合はPIF・Silver Lake・Affinity Partners
+JPモルガンが200億ドルの融資を提供
+規制審査の最終局面、アウトサイドデート9/28
+CEO続投も負債返済圧力で人員・投資に影響懸念</t>
+        </is>
+      </c>
+      <c r="G305" s="14" t="inlineStr">
+        <is>
+          <t>クロージング後は巨額負債の返済圧力から、コスト削減・IP選別・スタジオ再編が進む可能性。他の大型パブリッシャーへのPE非公開化ドミノの試金石になる。</t>
+        </is>
+      </c>
+      <c r="H305" s="14" t="inlineStr">
+        <is>
+          <t>メガLBOと負債主導の経営再編</t>
+        </is>
+      </c>
+      <c r="I305" s="14" t="inlineStr">
+        <is>
+          <t>Electronic Arts, PIF, Silver Lake, JPMorgan</t>
+        </is>
+      </c>
+      <c r="J305" s="14" t="inlineStr">
+        <is>
+          <t>EA SPORTS FC, Battlefield</t>
+        </is>
+      </c>
+      <c r="K305" s="14" t="inlineStr">
+        <is>
+          <t>M&amp;A,海外,規制</t>
+        </is>
+      </c>
+      <c r="L305" s="14" t="inlineStr"/>
+    </row>
+    <row r="306">
+      <c r="A306" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B306" s="14" t="inlineStr">
+        <is>
+          <t>『パルワールド』正式版1.0がリリース——累計プレイヤー4000万人突破、新パル72種・新エリア追加</t>
+        </is>
+      </c>
+      <c r="C306" s="14" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/article/202607/81000</t>
+        </is>
+      </c>
+      <c r="D306" s="14" t="inlineStr">
+        <is>
+          <t>ポケットペアの『パルワールド』は2024年1月の早期アクセス開始直後に爆発的ヒット。任天堂・ポケモン社との特許訴訟を抱えつつ、約2年半の早期アクセスを経て正式版に到達した。</t>
+        </is>
+      </c>
+      <c r="E306" s="14" t="inlineStr">
+        <is>
+          <t>7/10に正式版1.0が発売。新パル72種(合計287種)、新エリア『天陽郷』『世界樹』、ストーリー、水上拠点建築などを大量追加。記念に過去最安の30%オフセールも実施し、累計プレイヤーは4000万人を突破。</t>
+        </is>
+      </c>
+      <c r="F306" s="14" t="inlineStr">
+        <is>
+          <t>正式版1.0を7/10リリース(早期アクセス約2.5年)
+新パル72種追加で合計287種、新エリア・水上拠点
+累計プレイヤー4000万人超
+記念30%オフの過去最安セール
+任天堂/ポケモンとの特許訴訟は継続中</t>
+        </is>
+      </c>
+      <c r="G306" s="14" t="inlineStr">
+        <is>
+          <t>正式版化で新規・復帰勢の再流入が期待され、コラボ・DLC展開が加速。サバイバルクラフト×クリーチャー収集ジャンルの代表作としての地位を固める。訴訟の行方が国内開発の設計自由度に影響。</t>
+        </is>
+      </c>
+      <c r="H306" s="14" t="inlineStr">
+        <is>
+          <t>早期アクセス運営から正式版化への移行設計</t>
+        </is>
+      </c>
+      <c r="I306" s="14" t="inlineStr">
+        <is>
+          <t>ポケットペア</t>
+        </is>
+      </c>
+      <c r="J306" s="14" t="inlineStr">
+        <is>
+          <t>パルワールド, Palworld</t>
+        </is>
+      </c>
+      <c r="K306" s="14" t="inlineStr">
+        <is>
+          <t>新作,国内</t>
+        </is>
+      </c>
+      <c r="L306" s="14" t="inlineStr"/>
+    </row>
+    <row r="307">
+      <c r="A307" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B307" s="14" t="inlineStr">
+        <is>
+          <t>中国NPPA、2026年Q2に483タイトルへ版号交付(前年比+13%)——香港上場のモバイルゲーム株が上昇</t>
+        </is>
+      </c>
+      <c r="C307" s="14" t="inlineStr">
+        <is>
+          <t>https://www.gurufocus.com/news/8944778/mobile-game-stocks-surge-tencent-tcehy-and-bilibili-bili-lead-the-rally</t>
+        </is>
+      </c>
+      <c r="D307" s="14" t="inlineStr">
+        <is>
+          <t>中国では2021年の版号発給停止以降、当局(NPPA)の承認ペースがゲーム産業の供給量と業績を直接左右してきた。承認回復は市場のリスク選好を高める重要シグナルとなっている。</t>
+        </is>
+      </c>
+      <c r="E307" s="14" t="inlineStr">
+        <is>
+          <t>2026年Q2にNPPAが483タイトルへ版号を交付し前年比+13%。承認回復を好感し、Tencent・Bilibili・NetEase・IGGなど香港上場のモバイルゲーム株が一斉上昇した。</t>
+        </is>
+      </c>
+      <c r="F307" s="14" t="inlineStr">
+        <is>
+          <t>Q2の版号交付483件、前年比+13%
+Tencent・Bilibili +3%前後、NetEase等も上昇
+承認ペースが供給量・株価を実質統制
+国内競争激化の裏返しでもある</t>
+        </is>
+      </c>
+      <c r="G307" s="14" t="inlineStr">
+        <is>
+          <t>版号枠の回復で中国大手の新作投入が増える一方、国内は供給過多で採算悪化。中堅スタジオが海外パブリッシングや被買収に回る流れが強まる可能性。</t>
+        </is>
+      </c>
+      <c r="H307" s="14" t="inlineStr">
+        <is>
+          <t>版号(ライセンス)規制と株価・供給の連動</t>
+        </is>
+      </c>
+      <c r="I307" s="14" t="inlineStr">
+        <is>
+          <t>Tencent, NetEase, Bilibili, IGG</t>
+        </is>
+      </c>
+      <c r="J307" s="14" t="inlineStr"/>
+      <c r="K307" s="14" t="inlineStr">
+        <is>
+          <t>規制,海外,業績</t>
+        </is>
+      </c>
+      <c r="L307" s="14" t="inlineStr"/>
+    </row>
+    <row r="308">
+      <c r="A308" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B308" s="14" t="inlineStr">
+        <is>
+          <t>生成AIへの逆風強まる——開発者の52%が『悪影響』、粗製乱造の“gameslop”問題が焦点に</t>
+        </is>
+      </c>
+      <c r="C308" s="14" t="inlineStr">
+        <is>
+          <t>https://www.gamedeveloper.com/business/one-third-of-game-workers-use-generative-ai-but-half-think-it-s-bad-for-the-industry</t>
+        </is>
+      </c>
+      <c r="D308" s="14" t="inlineStr">
+        <is>
+          <t>GDCの業界調査では生成AIを『悪影響』とみる開発者の比率が2年前の18%→30%→52%へ急上昇。約1/3が業務で生成AIを使う一方、品質低下と発見性悪化への懸念が拡大している。</t>
+        </is>
+      </c>
+      <c r="E308" s="14" t="inlineStr">
+        <is>
+          <t>調査で52%が生成AIを業界に悪影響と回答。低コストで見栄えだけ整えた粗製乱造タイトル(gameslop)がマーケットに氾濫し、ValveはSteamでAI利用開示を義務化(7300本超が表示)しつつ、直接体験しないAIは開示不要へと基準を緩和した。</t>
+        </is>
+      </c>
+      <c r="F308" s="14" t="inlineStr">
+        <is>
+          <t>『悪影響』回答が18%→30%→52%へ急増
+約1/3が業務で生成AIを利用
+粗製乱造“gameslop”で発見性が悪化
+ValveはAI開示義務化も基準を一部緩和
+『非AI・人の手』を訴求する差別化の動き</t>
+        </is>
+      </c>
+      <c r="G308" s="14" t="inlineStr">
+        <is>
+          <t>AI開示ラベルと『人の手』保証が購買シグナル化。プラットフォームの品質フィルタ・キュレーション強化と、AI利用の透明性ルールを巡る綱引きが続く。</t>
+        </is>
+      </c>
+      <c r="H308" s="14" t="inlineStr">
+        <is>
+          <t>生成AIの品質・発見性・開示規制</t>
+        </is>
+      </c>
+      <c r="I308" s="14" t="inlineStr">
+        <is>
+          <t>Valve, Steam</t>
+        </is>
+      </c>
+      <c r="J308" s="14" t="inlineStr"/>
+      <c r="K308" s="14" t="inlineStr">
+        <is>
+          <t>技術,海外,規制</t>
+        </is>
+      </c>
+      <c r="L308" s="14" t="inlineStr"/>
+    </row>
+    <row r="309">
+      <c r="A309" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B309" s="14" t="inlineStr">
+        <is>
+          <t>eスポーツW杯2026 第2週が開幕——LoL/Dota2/Free Fire/MLBB女子が同時進行(パリ、〜8/23)</t>
+        </is>
+      </c>
+      <c r="C309" s="14" t="inlineStr">
+        <is>
+          <t>https://dotesports.com/dota-2/guides/dota-2-ewc-2026-schedule-results</t>
+        </is>
+      </c>
+      <c r="D309" s="14" t="inlineStr">
+        <is>
+          <t>サウジ主導のEsports World Cupは7/6〜8/23にパリで開催中。24種目・25大会を束ねる世界最大級のクロスゲーム大会で、第1週のVALORANT等に続き第2週は主要タイトルが集中する。</t>
+        </is>
+      </c>
+      <c r="E309" s="14" t="inlineStr">
+        <is>
+          <t>第2週はLeague of Legends、Dota 2、Free Fire、MLBB女子部門が同時進行。MLBB女子は7/14開始、Free Fire決勝7/18、Dota2・LoL決勝は7/19に予定され、クラブ横断のポイント争いが本格化する。</t>
+        </is>
+      </c>
+      <c r="F309" s="14" t="inlineStr">
+        <is>
+          <t>第2週にLoL/Dota2/Free Fire/MLBB女子が集中
+MLBB女子7/14開始、FF決勝7/18、Dota2/LoL決勝7/19
+24種目・25大会、賞金総額は過去最大級
+クラブ対抗ポイント制で総合王者を争う</t>
+        </is>
+      </c>
+      <c r="G309" s="14" t="inlineStr">
+        <is>
+          <t>クロスゲームの大型化と巨額賞金が続き、eスポーツの興行・スポンサー収益モデルが強化。国・都市を巻き込む誘致競争が加速する。</t>
+        </is>
+      </c>
+      <c r="H309" s="14" t="inlineStr">
+        <is>
+          <t>クロスゲーム大会の興行・収益設計</t>
+        </is>
+      </c>
+      <c r="I309" s="14" t="inlineStr">
+        <is>
+          <t>Esports World Cup, Riot Games, Valve, Garena</t>
+        </is>
+      </c>
+      <c r="J309" s="14" t="inlineStr">
+        <is>
+          <t>League of Legends, Dota 2, Free Fire, MLBB</t>
+        </is>
+      </c>
+      <c r="K309" s="14" t="inlineStr">
+        <is>
+          <t>eスポーツ,海外</t>
+        </is>
+      </c>
+      <c r="L309" s="14" t="inlineStr"/>
+    </row>
+    <row r="310">
+      <c r="A310" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B310" s="14" t="inlineStr">
+        <is>
+          <t>ブシロード『バンドリ！ Our Notes』事前登録がグローバル70万件を突破——SR以上確定チケ配布決定</t>
+        </is>
+      </c>
+      <c r="C310" s="14" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/974/G097456/20260713022/</t>
+        </is>
+      </c>
+      <c r="D310" s="14" t="inlineStr">
+        <is>
+          <t>『バンドリ！』はスマホ音ゲー『ガルパ』でシリーズを築いたIP。新作『Our Notes』はグローバル同時展開を掲げ、リリース前の需要喚起として事前登録キャンペーンを実施している。</t>
+        </is>
+      </c>
+      <c r="E310" s="14" t="inlineStr">
+        <is>
+          <t>7/13、新作リズムゲーム『バンドリ！ Our Notes』の事前登録がグローバルで70万件を突破。達成報酬としてSR以上確定ガチャチケットの配布が決定した。</t>
+        </is>
+      </c>
+      <c r="F310" s="14" t="inlineStr">
+        <is>
+          <t>事前登録グローバル70万件突破
+報酬はSR以上確定ガチャチケット
+バンドリIPのグローバル同時展開
+リリース前の需要喚起マーケティング</t>
+        </is>
+      </c>
+      <c r="G310" s="14" t="inlineStr">
+        <is>
+          <t>モバイルリズムゲームは国内成熟の中でグローバル同時展開が定石化。既存IPの海外事前登録規模が初動収益とセルラン順位を左右する。</t>
+        </is>
+      </c>
+      <c r="H310" s="14" t="inlineStr">
+        <is>
+          <t>IPリズムゲームのグローバル事前登録運用</t>
+        </is>
+      </c>
+      <c r="I310" s="14" t="inlineStr">
+        <is>
+          <t>ブシロード</t>
+        </is>
+      </c>
+      <c r="J310" s="14" t="inlineStr">
+        <is>
+          <t>バンドリ！, BanG Dream! Our Notes</t>
+        </is>
+      </c>
+      <c r="K310" s="14" t="inlineStr">
+        <is>
+          <t>新作,国内</t>
+        </is>
+      </c>
+      <c r="L310" s="14" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
weekly-trends + tech update (2026-07-15 12:11)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -1987,7 +1987,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3180,6 +3180,117 @@
       <c r="G32" t="inlineStr">
         <is>
           <t>https://www.reedsmith.com/articles/pegi-launches-interactive-risk-categories-overhauls-age-ratings-for-loot-boxes-in-game-spending-and-communication-features/</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Palworld 1.0正式化と任天堂訴訟の実質崩壊</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Pocketpairの『Palworld』が7/10にEarly Accessを卒業し1.0へ。累計4000万本、Steam同接は855Kに達しSteam歴代best-everプレイヤー数リスト入り（過去最高2.1Mには未達）。72体追加で総287体、World Tree/Sky Islands/PvP/遺伝子交配を実装、1.0でも価格を据え置き『Overwhelmingly Positive』の評価。並行して任天堂・ポケモン社の特許訴訟は和解額が実質3万ドル規模へ縮小、日本特許庁は関連特許を独創性欠如で却下、米国でも23件中22件が拒絶。約30か月に及んだ法的リスクが『rounding error』と評される着地に向かう。</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>Pocketpair, Nintendo, The Pokémon Company, Palworld</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>サバイバル×クリーチャーコレクション×基地建設という複合ジャンルを、長期EA運営で磨き上げてから1.0で再点火する『二度目の全盛期』設計。価格据え置き＋既存所有者無償という信頼設計がレビュー好転を生む。特許訴訟は『似ている』と『権利侵害』の距離、及び先行公知による特許無効化リスクを可視化し、模倣回避設計の実務ラインを示した。</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>モンスター収集の独占的ブランド価値が法で守り切れない時代。IPは訴訟でなく運営速度と信頼で堀を築く。他業界のブランド係争にも通じる論点。</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>https://www.forbes.com/sites/paultassi/2026/07/10/palworld-10-is-putting-up-enormous-steam-player-numbers-at-launch/ , https://gamerant.com/nintendo-palworld-lawsuit-end-date-version-changes-explained/</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>ポケモン値上げ内部方針リークと$80時代の地ならし</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>ポケモン社の内部文書（teraleak由来、2018〜20年頃）が流出し、メインライン作を標準60ドル超へ引き上げたい意向と、赤・青型の『両バージョン購入促進』策を検討していたことが判明。Sword/Shield時代から値上げを望みつつ、北米で高価格を正常化した競合が不在だったため見送っていたとされる。次回作『Pokémon Winds and Waves』は独Amazonで€79.99掲載が観測され、Mario Kart World同額の79.99ドルを示唆。値上げは国内優先で並行輸入が論点化、ダブルパックのロイヤリティは据え置き方向。公式価格は未確定で発表は2026末〜2027想定。</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>The Pokémon Company, Nintendo, Game Freak, Pokémon Winds and Waves</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>任天堂は既にMario Kart Worldで79.99ドルを提示し、業界の心理的天井を押し上げた。ポケモンという最大量販IPが追随すれば『80ドル標準』が一気に既成事実化する。内部文書は値上げ判断が品質でなく『誰が先に嫌われ役をやるか』という囚人のジレンマで決まってきたことを示す。両バージョン商法＝実質的な単価二重化の温存も透ける。</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>価格は原価でなく競合の正常化タイミングで決まる。ブランド力の強いIPほど値上げの先導役になれる——サブスクや他消費財の価格戦略にも接続。</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>https://nintendoeverything.com/pokemon-company-document-shows-wanting-to-increase-price-from-60-encouraging-people-to-buy-both-versions/ , https://games.gg/news/pokemon-winds-waves-price-increase-leak/</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>2大レガシーリメイク同月投入と端境期カレンダーの穴埋め</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>7月は『Assassin's Creed Black Flag: Resynced』と『Halo: Campaign Evolved』という大型リメイク/再構築が同月ローンチ。UbisoftはBlack Flag Resyncedの初週実売数を異例の形で公表するほど好発進を強調。大型新規AAAが乏しくGTA6待ちで『枯れたカレンダー』が続くなか、確立IPの再武装が供給ギャップを埋める構図が鮮明化。Steam/Game Pass経由の旧作再パッケージや、サバイバーライクのday-one Game Pass投入なども重なり、7月は『新規より再利用』が主旋律に。</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>Ubisoft, Xbox Game Studios, Halo Studios, Assassin's Creed, Halo</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>新規開発費とリスクが高騰するなか、実績IPのリメイクは既知の需要曲線に賭けられる低リスク投資。同時に、初週販売数の異例公表はライブ運営前提でのKPI開示文化がリメイクにも波及したことを示す。サブスク＋リマスターは旧カタログを恒久収益資産に変える『IPの年金化』の一環。</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>コンテンツ産業全体が『新規制作』から『既存カタログの再運用』へ重心移動。映画・音楽のリマスター経済と同型の力学が働く。</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>https://www.pcgamer.com/games/pc-game-release-dates-july-2026/ , https://www.eneba.com/hub/news/weekly-roundup-physical-games-indie-game-announcements-july-2026/</t>
         </is>
       </c>
     </row>
@@ -37592,7 +37703,7 @@
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B2" s="9" t="inlineStr">
@@ -37607,32 +37718,32 @@
       </c>
       <c r="D2" s="9" t="inlineStr">
         <is>
-          <t>開発現場の生成AI利用率は前年比で低下傾向が続く一方、ツール層では標準エンジンへの生成AI組み込みが加速。制作フロー上流（エンジン・パイプライン）と現場適用の温度差が拡大。</t>
+          <t>GDC 2026 State of the Game Industry調査で『生成AIは業界に悪影響』が52%（前年30%・前々年18%）へ急伸。肯定はわずか7%（前年13%）。</t>
         </is>
       </c>
       <c r="E2" s="9" t="inlineStr">
         <is>
-          <t>Epicが6/17にUnreal Engine 6を発表、LLM・生成AI（Claude/Codex含む）を制作の中核に据え、Blueprintsを将来非推奨としVerseへ移行。開発者は反発、poncleがFortnite協業見直しを表明。EpicはSteamのAI開示タグを「緋文字」と批判。</t>
+          <t>ビジュアル/技術アート64%・デザイン/ナラティブ63%・プログラミング59%が否定的。一方で36%が日常業務でAIを使用（研究・コーディング・プロトタイピング中心）、AAAの約30%が自社データで訓練した独自AIを保有。レイオフとの同時進行で『生産性向上＝人員削減の口実』と受け止める空気が強い。</t>
         </is>
       </c>
       <c r="F2" s="9" t="inlineStr">
         <is>
-          <t>Epic Games, Anthropic(Claude), poncle, Valve, Godot</t>
+          <t>各AAAスタジオ, GDC/Informa, 労働組合(SAG-AFTRA等)</t>
         </is>
       </c>
       <c r="G2" s="9" t="inlineStr">
         <is>
-          <t>標準エンジンのAI組み込みは不可逆。ノーコード資産の陳腐化を嫌う層がGodot等中立ツールへ分散する二極化が進む。開示義務化の是非がプラットフォーム間対立の焦点に。</t>
+          <t>現場の反発と経営のAI投資が並走。AI保護条項が労組交渉の中核要求に。最終アセットへの適用は当面限定的で、ツール化と雇用の綱引きが続く。</t>
         </is>
       </c>
       <c r="H2" s="9" t="inlineStr">
         <is>
-          <t>AIの主戦場が「現場の生成」から「制作基盤の設計思想」へ移動。誰がツール標準を握るかがクリエイター主権を左右する。</t>
+          <t>『使うが信用しない』の二重状態。導入率と支持率が逆行する技術は稀で、労使の力学が採用ペースを左右する。</t>
         </is>
       </c>
       <c r="I2" s="9" t="inlineStr">
         <is>
-          <t>https://www.shacknews.com/article/149693/unreal-engine-6-generative-ai-models-claude-codex</t>
+          <t>https://gdconf.com/article/gdc-2026-state-of-the-game-industry-reveals-impact-of-layoffs-generative-ai-and-more/</t>
         </is>
       </c>
       <c r="J2" s="9" t="inlineStr"/>
@@ -37936,7 +38047,7 @@
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B10" s="9" t="inlineStr">
@@ -37951,20 +38062,40 @@
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>国内ではグリー、海外でも継続</t>
-        </is>
-      </c>
-      <c r="E10" s="9" t="inlineStr"/>
-      <c r="F10" s="9" t="inlineStr"/>
-      <c r="G10" s="9" t="inlineStr"/>
-      <c r="H10" s="9" t="inlineStr"/>
-      <c r="I10" s="9" t="inlineStr"/>
+          <t>誇大宣伝フェーズを脱し『実用実装』へ移行との観測。資産の真の所有・プレイヤー主導マーケット・相互運用可能なデジタルアイテムが徐々に一般化。</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>投機主導のGameFi像から、既存ゲームエコシステムへの機能組込み（所有権・二次流通）へ論点がシフト。ハイパーカジュアルの粘着メカニクス×長期進行のハイブリッド設計と併走する形で語られる。</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>各PFホルダー, ブロックチェーンゲーム各社</t>
+        </is>
+      </c>
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>『Web3を名乗らないWeb3機能』として裏側実装が進む可能性。規制と手数料設計が普及の律速。</t>
+        </is>
+      </c>
+      <c r="H10" s="9" t="inlineStr">
+        <is>
+          <t>誇大広告の谷を越えた技術は看板を外し機能として溶け込む。観測ベースではまだ主流化の確証は薄い。</t>
+        </is>
+      </c>
+      <c r="I10" s="9" t="inlineStr">
+        <is>
+          <t>https://www.gameindustry.com/news-industry-happenings/5-game-changing-trends-shaping-the-gaming-industry-in-2026/</t>
+        </is>
+      </c>
       <c r="J10" s="9" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
@@ -37979,32 +38110,32 @@
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>マイクロ/インディーが評価上位を独占するディスカバリー構造が継続。</t>
+          <t>『Palworld 1.0』が7/10ローンチで同接855Kを記録、Palworld無印と1.0が揃ってSteam歴代best-everプレイヤー数リストに入る事態。</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>コージーホラー『Creature Kitchen』が99%(5689件)で2026年Steam最高評価に。早期アクセス『Far Far West』も97%。低価格・短尺・口コミ駆動が上位進出。</t>
+          <t>490K(初日)→720K(7/11)→850K超(7/12-13)と週末にかけ増勢。累計4000万本・価格据え置き・既存所有者無償が好評を後押し。別途『Artifact Classic』が明確な理由なく約1万同接へ約100倍スパイクする謎現象も観測。</t>
         </is>
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t>The Rat Zone, Valve/Steam</t>
+          <t>Valve, Pocketpair</t>
         </is>
       </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
-          <t>ジャンル掛け合わせ(cozy×horror)と低予算短尺の組合せが、レビュースコア駆動のキュレーションで再現的にヒット化。</t>
+          <t>EA卒業タイトルの『二度目の全盛期』設計がPCの定番戦術に。旧作の突発再燃はディスカバリー/ボット/投機いずれかの兆候として要監視。</t>
         </is>
       </c>
       <c r="H11" s="9" t="inlineStr">
         <is>
-          <t>資本規模でなくレビュー品質がSteam露出の主変数。</t>
+          <t>Steamの同接ランキングは新作より『再点火』が席巻。ピークでなく持続曲線が資産価値を決める局面。</t>
         </is>
       </c>
       <c r="I11" s="9" t="inlineStr">
         <is>
-          <t>https://intoindiegames.com/features/news/creature-kitchen-is-steams-highest-rated-game-of-2026-so-far/</t>
+          <t>https://www.forbes.com/sites/paultassi/2026/07/11/both-palworld-and-palworld-10-are-in-steams-best-ever-playercount-list/</t>
         </is>
       </c>
       <c r="J11" s="9" t="inlineStr"/>
@@ -38012,7 +38143,7 @@
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B12" s="9" t="inlineStr">
@@ -38027,32 +38158,32 @@
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>発売1年で累計19.86M台、同期間のPS5を上回る立ち上がり。サードパーティが本格回帰する局面。</t>
+          <t>発売1年超・普及拡大が続く一方、価格戦略が焦点化。ポケモン社の内部文書流出で『60ドル超への値上げ』意向と両バージョン購入促進策が判明。</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>6月に『FF7 Rebirth』が任天堂機初上陸、Capcom『DMC5』も6/23投入。Not-E3 2026で13本前後のサード作が集中発表（週約3本ペース）。任天堂エコシステムのサード売上は前年比+76%（13億→23億ドル）。</t>
+          <t>『Pokémon Winds and Waves』は独Amazonで€79.99掲載＝79.99ドル示唆（Mario Kart World同額）。値上げは国内優先・並行輸入が論点。本体は依然品薄で入荷即完売が継続、7月は41本発売、DQ7 Reimagined/オクトパストラベラー0等のセールも。</t>
         </is>
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>任天堂, Square Enix, Capcom, Warner Bros.</t>
+          <t>任天堂, The Pokémon Company, Square Enix</t>
         </is>
       </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
-          <t>「移植の最後の砦」から初期ラインアップ前提の必須機へ。年末商戦の端末普及ペースとファースト大型作の供給、値上げの需要影響が次の焦点。</t>
+          <t>80ドル標準化を任天堂系IPが先導する公算。値上げの需要弾力性と品薄解消のタイミングが年末商戦の鍵。</t>
         </is>
       </c>
       <c r="H12" s="9" t="inlineStr">
         <is>
-          <t>普及速度そのものが開発優先順位を書き換える。「規模×性能」が揃った瞬間にエコシステムの引力が非線形化。</t>
+          <t>最量販IPの値上げは業界全体の心理的天井を押し上げる。価格は競合の『正常化』が決める。</t>
         </is>
       </c>
       <c r="I12" s="9" t="inlineStr">
         <is>
-          <t>https://tech-insider.org/nintendo-switch-2-sales-19-million-2026/</t>
+          <t>https://nintendoeverything.com/pokemon-company-document-shows-wanting-to-increase-price-from-60-encouraging-people-to-buy-both-versions/</t>
         </is>
       </c>
       <c r="J12" s="9" t="inlineStr"/>

</xml_diff>

<commit_message>
daily-news + cross-questions + events + predictions + game-design update (2026-07-16)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -817,7 +817,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1973,6 +1973,43 @@
       <c r="G31" s="14" t="inlineStr">
         <is>
           <t>InvestGame等の四半期M&amp;Aレポートで中国発ディール(被買収・出資)件数の増減を観測。大手の海外パブリッシング契約数の推移も指標。</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B32" s="15" t="inlineStr">
+        <is>
+          <t>モバイルの新規インストール減(-12%)×UAコスト高で、中小パブリッシャーがペイドUAから自社IPのPC/コンソール移植へ予算を移す→モバイル広告ネットワークの中間層需要が細り、Unity/ironSource系や中小ADNの再編・淘汰が進む</t>
+        </is>
+      </c>
+      <c r="C32" s="15" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="D32" s="15" t="inlineStr">
+        <is>
+          <t>6〜12ヶ月</t>
+        </is>
+      </c>
+      <c r="E32" s="15" t="inlineStr">
+        <is>
+          <t>Unity, AppLovin(ironSource), 中小モバイルパブリッシャー</t>
+        </is>
+      </c>
+      <c r="F32" s="15" t="inlineStr">
+        <is>
+          <t>「モバイルゲーム消費が失速——四半期IAP売上-4%・インストール-12%」(Luminate, 2026-06-10) 及び 「Steam上半期の収益約79%が旧作」(Game*Spark, 2026-07-16)</t>
+        </is>
+      </c>
+      <c r="G32" s="15" t="inlineStr">
+        <is>
+          <t>AppLovin/Unityの広告セグメントのガイダンスと広告主構成(中間層の増減)、ad-tech領域のM&amp;A件数、モバイル発クロスプラットフォーム移植の発表数を四半期で観測。</t>
         </is>
       </c>
     </row>
@@ -4121,7 +4158,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G73"/>
+  <dimension ref="A1:G74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6831,6 +6868,43 @@
       <c r="G73" s="14" t="inlineStr">
         <is>
           <t>供給を数量で絞る規制は、モノの良し悪しより『枠の開閉』が業績・株価を動かす。政策変数の可視化が投資判断の鍵。</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B74" s="15" t="inlineStr">
+        <is>
+          <t>モバイルの新規インストール減(-12%)とUAコスト高騰は、他のアプリ広告依存業界(フィンテック・フードデリバリー・EC)のCAC(顧客獲得コスト)危機と同型か？</t>
+        </is>
+      </c>
+      <c r="C74" s="15" t="inlineStr">
+        <is>
+          <t>Q2 2026モバイルIAP-4%・インストール-12%(Luminate, 2026-06-10)、対しSteam上半期は旧作が収益約79%(Game*Spark, 2026-07-16)</t>
+        </is>
+      </c>
+      <c r="D74" s="15" t="inlineStr">
+        <is>
+          <t>AppLovin, Unity, モバイル専業パブリッシャー</t>
+        </is>
+      </c>
+      <c r="E74" s="15" t="inlineStr">
+        <is>
+          <t>広告・マーケ(CAC高騰と獲得頭打ち), フィンテック/フードデリバリー(UA依存の収益モデル), EC(有料獲得→リテンション偏重への転換)</t>
+        </is>
+      </c>
+      <c r="F74" s="15" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="G74" s="15" t="inlineStr">
+        <is>
+          <t>有料UAで伸ばす成長モデルが飽和すると、各業界とも"獲得"から"既存顧客の再運用"へ重心が移る。ゲームのクロスプラットフォーム移植は他業界の"既存顧客LTV最大化"に相当。</t>
         </is>
       </c>
     </row>
@@ -9804,7 +9878,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J26"/>
+  <dimension ref="A1:J27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10910,12 +10984,12 @@
       </c>
       <c r="I22" s="14" t="inlineStr">
         <is>
-          <t>開催中</t>
+          <t>終了</t>
         </is>
       </c>
       <c r="J22" s="14" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-16</t>
         </is>
       </c>
     </row>
@@ -11114,12 +11188,60 @@
       </c>
       <c r="I26" s="14" t="inlineStr">
         <is>
-          <t>開催予定</t>
+          <t>開催中</t>
         </is>
       </c>
       <c r="J26" s="14" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B27" s="15" t="n"/>
+      <c r="C27" s="15" t="inlineStr">
+        <is>
+          <t>PlayStation Store SUMMER SALE 2026</t>
+        </is>
+      </c>
+      <c r="D27" s="15" t="inlineStr">
+        <is>
+          <t>セール</t>
+        </is>
+      </c>
+      <c r="E27" s="15" t="inlineStr">
+        <is>
+          <t>オンライン(PS Store)</t>
+        </is>
+      </c>
+      <c r="F27" s="15" t="inlineStr">
+        <is>
+          <t>オンライン</t>
+        </is>
+      </c>
+      <c r="G27" s="15" t="inlineStr">
+        <is>
+          <t>PS5/PS4対象のサマーセール。最大80%OFF。旧作・大型タイトルのディスカウント商戦。</t>
+        </is>
+      </c>
+      <c r="H27" s="15" t="inlineStr">
+        <is>
+          <t>https://www.pushsquare.com/playstation-plus</t>
+        </is>
+      </c>
+      <c r="I27" s="15" t="inlineStr">
+        <is>
+          <t>開催中</t>
+        </is>
+      </c>
+      <c r="J27" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
         </is>
       </c>
     </row>
@@ -11204,7 +11326,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B2" s="14" t="inlineStr">
@@ -11219,7 +11341,7 @@
       </c>
       <c r="D2" s="14" t="inlineStr">
         <is>
-          <t>台頭</t>
+          <t>台頭→規制逆風(中国で人格AI規制)</t>
         </is>
       </c>
       <c r="E2" s="14" t="inlineStr">
@@ -11239,12 +11361,12 @@
       </c>
       <c r="H2" s="14" t="inlineStr">
         <is>
-          <t>会話品質が差別化要素に。高いハード要件が買い替え誘因化する一方、暴走・コスト・倫理面の運用設計が課題。</t>
+          <t>中国の人格模倣型AI暫定弁法(7/15施行)で"人間を装う"設計に制約。グローバルではキャラクター性を保ちつつ非擬人化・年齢ゲートを前提とする設計へ調整が進む。</t>
         </is>
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
-          <t>Krafton『PUBG』Ally Duo/Ella(6/28)</t>
+          <t>中国が擬人化AI規制を7/15施行・豆包/千問がエージェント機能停止(東洋経済, 2026-07-16)</t>
         </is>
       </c>
       <c r="J2" s="14" t="n">
@@ -11304,7 +11426,7 @@
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
@@ -11339,12 +11461,12 @@
       </c>
       <c r="H4" s="14" t="inlineStr">
         <is>
-          <t>旧作リメイクが新作AAAをエンゲージメントで上回る実績が増え、大手の投資配分が旧IP再生へシフト。名作の権利在庫が実質の新作パイプライン化</t>
+          <t>Steam上半期売上の約79%が旧作という定量データで裏付け。リマスター/復刻/エバーグリーン運用は新作AAAより低リスク高効率として投資が集中し、"カタログ再運用"が主戦場化する見込み。</t>
         </is>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
-          <t>『AC ブラックフラッグ Resynced』フルリメイク発売(Ubisoft, 2026-07-09) / 『AC ブラックフラッグ RE:シンクロ』Steam同接10.4万人でAC史上最高・Shadows超え(GamesRadar/2026-07-14)</t>
+          <t>Steam2026年上半期売上111億ドル・旧作が収益の約79%(Game*Spark, 2026-07-16)</t>
         </is>
       </c>
       <c r="J4" s="14" t="n">
@@ -13177,7 +13299,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L311"/>
+  <dimension ref="A1:L316"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -32434,6 +32556,307 @@
           <t>ミクロ×高インサイト枠（数字でなく『新作AAA疲れ／レガシー再現』の実例として採用）</t>
         </is>
       </c>
+    </row>
+    <row r="312">
+      <c r="A312" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B312" s="15" t="inlineStr">
+        <is>
+          <t>Steam2026年上半期売上111億ドルで過去最高——収益の約79%を旧作(バックカタログ)が占める</t>
+        </is>
+      </c>
+      <c r="C312" s="15" t="inlineStr">
+        <is>
+          <t>https://www.gamespark.jp/article/2026/07/11/169133.html</t>
+        </is>
+      </c>
+      <c r="D312" s="15" t="inlineStr">
+        <is>
+          <t>調査会社Alinea Analyticsの推計。新作AAAの開発費・価格高騰と大型協力プレイのロングヒット、大手による旧作再運用戦略の高度化が同時進行し、収益源が新作の初動から既存カタログへ構造的に移動している。</t>
+        </is>
+      </c>
+      <c r="E312" s="15" t="inlineStr">
+        <is>
+          <t>2026年上半期のSteam総売上は111億ドル(約1.8兆円)で半期として過去最高、通年累計は既に116億ドル。うち約79%をバックカタログ(旧作)が占める。成長要因はアジア(特に中国)のプレイヤー急増、価格上昇、協力プレイ大ヒット、独自ランチャー撤退後のSteam回帰。</t>
+        </is>
+      </c>
+      <c r="F312" s="15" t="inlineStr">
+        <is>
+          <t>上半期売上111億ドル(約1.8兆円)でSteam半期最高
+収益の約79%が旧作(バックカタログ)由来、新作は約21%
+成長ドライバー: アジア圏プレイヤー急増・価格上昇・協力プレイ大ヒット
+サードパーティが独自ランチャーからSteamへ回帰</t>
+        </is>
+      </c>
+      <c r="G312" s="15" t="inlineStr">
+        <is>
+          <t>新作の初動依存が薄れ、パブリッシャーはカタログのエバーグリーン運用(セール設計・DLC・リマスター)へ投資を集中。新作は"カタログ入りする資産"として設計され、発売日一括回収モデルは相対的に弱まる。</t>
+        </is>
+      </c>
+      <c r="H312" s="15" t="inlineStr">
+        <is>
+          <t>バックカタログ収益化とエバーグリーン運用設計</t>
+        </is>
+      </c>
+      <c r="I312" s="15" t="inlineStr">
+        <is>
+          <t>Valve(Steam), Alinea Analytics</t>
+        </is>
+      </c>
+      <c r="J312" s="15" t="inlineStr">
+        <is>
+          <t>Steam</t>
+        </is>
+      </c>
+      <c r="K312" s="15" t="inlineStr">
+        <is>
+          <t>業績,消費者インサイト,トレンド,海外</t>
+        </is>
+      </c>
+      <c r="L312" s="15" t="inlineStr">
+        <is>
+          <t>ミクロ×高インサイト枠（旧作偏重＝新作AAA疲れの定量的裏付け。7/14のAC RE:シンクロ事例をマクロ数値で補強）</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B313" s="15" t="inlineStr">
+        <is>
+          <t>中国、擬人化"人格"AI規制を7/15施行——バイトダンス「豆包」・アリババ「千問」がAIエージェント機能を停止</t>
+        </is>
+      </c>
+      <c r="C313" s="15" t="inlineStr">
+        <is>
+          <t>https://toyokeizai.net/articles/-/951250</t>
+        </is>
+      </c>
+      <c r="D313" s="15" t="inlineStr">
+        <is>
+          <t>「人格模倣型AIインタラクティブサービス管理暫定弁法」が7/15施行。人間を装い継続的な感情的交流を行うAIを対象に、過激思想拡散・プライバシー・依存リスクの低減を狙う。人とAIの感情的交流を法規制する世界初級の事例とされ、対象は約3.4億ユーザー規模。</t>
+        </is>
+      </c>
+      <c r="E313" s="15" t="inlineStr">
+        <is>
+          <t>規制施行に伴い、バイトダンス「豆包」は7/15にAIエージェント機能を、アリババ「千問」は擬人型対話・エージェント作成機能を同日停止。AIコンパニオン/キャラクター系サービスの設計自由度に直接影響する。</t>
+        </is>
+      </c>
+      <c r="F313" s="15" t="inlineStr">
+        <is>
+          <t>「人格模倣型AI」暫定弁法が7/15施行(世界初級の感情的交流規制)
+豆包・千問が擬人型AIエージェント機能を同日停止
+約3.4億ユーザー規模に影響、未成年利用にも厳格化</t>
+        </is>
+      </c>
+      <c r="G313" s="15" t="inlineStr">
+        <is>
+          <t>AIコンパニオン/対話型AI NPCの"人格付与"は中国市場で設計制約が強まる。グローバル勢はキャラクター性を保ちつつ"人間を装わない"設計や年齢ゲートを前提化。ゲーム内AI NPC表現にも波及しうる。</t>
+        </is>
+      </c>
+      <c r="H313" s="15" t="inlineStr">
+        <is>
+          <t>各国のAIコンパニオン規制とゲーム内AI NPC設計への影響</t>
+        </is>
+      </c>
+      <c r="I313" s="15" t="inlineStr">
+        <is>
+          <t>ByteDance(豆包), Alibaba(千問/Qwen)</t>
+        </is>
+      </c>
+      <c r="J313" s="15" t="inlineStr">
+        <is>
+          <t>豆包, 千問(Qwen)</t>
+        </is>
+      </c>
+      <c r="K313" s="15" t="inlineStr">
+        <is>
+          <t>規制,AI,海外</t>
+        </is>
+      </c>
+      <c r="L313" s="15" t="n"/>
+    </row>
+    <row r="314">
+      <c r="A314" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B314" s="15" t="inlineStr">
+        <is>
+          <t>ワンダープラネット、サンリオと新作ゲーム共同開発で本合意——高認知IPのグローバル展開狙う(適時開示)</t>
+        </is>
+      </c>
+      <c r="C314" s="15" t="inlineStr">
+        <is>
+          <t>https://prtimes.jp/main/html/rd/p/000000479.000005880.html</t>
+        </is>
+      </c>
+      <c r="D314" s="15" t="inlineStr">
+        <is>
+          <t>モバイル新作の低調・UAコスト高騰を背景に、自社オリジナルより認知度の高い外部キャラIPとの協業に活路を求める動き。サンリオ側もキャラIPのゲーム経由でのグローバル展開を加速する狙い。</t>
+        </is>
+      </c>
+      <c r="E314" s="15" t="inlineStr">
+        <is>
+          <t>ワンダープラネットは7/13取締役会で決議し同日付でサンリオとの新作ゲーム共同開発契約を締結(適時開示)。サンリオの高認知IPをグローバル展開し、ワンパの得意領域で開発を担う。タイトル・ゲーム内容等の詳細は今後発表。</t>
+        </is>
+      </c>
+      <c r="F314" s="15" t="inlineStr">
+        <is>
+          <t>7/13適時開示。サンリオIP×ワンダープラネット開発の共同開発で本合意
+サンリオIPのグローバル認知を活用しグローバル展開を志向
+タイトル・ジャンル等の詳細は未公表(決定次第公表)</t>
+        </is>
+      </c>
+      <c r="G314" s="15" t="inlineStr">
+        <is>
+          <t>キャラIPホルダーが開発を外部委託しつつ共同事業/ロイヤリティで収益を取り込む"IPライセンス→共同開発"型が中堅パブリッシャーで増加。自社完全新規のリスクを避けIP依存度が高まる。</t>
+        </is>
+      </c>
+      <c r="H314" s="15" t="inlineStr">
+        <is>
+          <t>キャラIPライセンスの共同開発モデルとグローバル展開</t>
+        </is>
+      </c>
+      <c r="I314" s="15" t="inlineStr">
+        <is>
+          <t>ワンダープラネット, サンリオ</t>
+        </is>
+      </c>
+      <c r="J314" s="15" t="inlineStr">
+        <is>
+          <t>サンリオキャラクターズ</t>
+        </is>
+      </c>
+      <c r="K314" s="15" t="inlineStr">
+        <is>
+          <t>提携,適時開示,新作,国内</t>
+        </is>
+      </c>
+      <c r="L314" s="15" t="n"/>
+    </row>
+    <row r="315">
+      <c r="A315" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B315" s="15" t="inlineStr">
+        <is>
+          <t>英ゲーム業界の労働不安が鮮明——直近1年で22%が整理解雇通知、IWGBが"整理解雇タスクフォース"結成</t>
+        </is>
+      </c>
+      <c r="C315" s="15" t="inlineStr">
+        <is>
+          <t>https://www.gamedeveloper.com/business/iwgb-game-workers-union-forms-redundancy-taskforce-to-defend-workers-rights</t>
+        </is>
+      </c>
+      <c r="D315" s="15" t="inlineStr">
+        <is>
+          <t>2022年以降の業界レイオフは累計3万人超。人材採用会社Skillsearchの調査で直近1年に22%が解雇通知を受け、44%が業界離脱を検討と回答。英ゲームワーカー組合IWGBが会員主導のタスクフォースを立ち上げた。</t>
+        </is>
+      </c>
+      <c r="E315" s="15" t="inlineStr">
+        <is>
+          <t>IWGB(独立系ゲームワーカー組合)は会員主導の"整理解雇タスクフォース"を結成し、英国内の解雇が"合法・正当・公正"であるよう会員の権利擁護に取り組む。背景にSkillsearch調査の22%解雇・44%離職検討という深刻な労働環境がある。</t>
+        </is>
+      </c>
+      <c r="F315" s="15" t="inlineStr">
+        <is>
+          <t>直近1年で回答者の22%が整理解雇通知を受領
+44%が業界からの離脱を検討、2022年以降で累計3万人超が失職
+IWGBが会員主導の整理解雇タスクフォースを結成</t>
+        </is>
+      </c>
+      <c r="G315" s="15" t="inlineStr">
+        <is>
+          <t>熟練人材の流出が続けば、中規模スタジオの新設や独立(スピンアウト)が増える一方、AAAは経験者確保コストが上昇。労組の組織化が英を起点に強まる可能性。</t>
+        </is>
+      </c>
+      <c r="H315" s="15" t="inlineStr">
+        <is>
+          <t>ゲーム業界の労働組織化とレイオフ後の人材再配置</t>
+        </is>
+      </c>
+      <c r="I315" s="15" t="inlineStr">
+        <is>
+          <t>IWGB, Skillsearch</t>
+        </is>
+      </c>
+      <c r="J315" s="15" t="inlineStr"/>
+      <c r="K315" s="15" t="inlineStr">
+        <is>
+          <t>人事・組織,海外,トレンド</t>
+        </is>
+      </c>
+      <c r="L315" s="15" t="n"/>
+    </row>
+    <row r="316">
+      <c r="A316" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B316" s="15" t="inlineStr">
+        <is>
+          <t>スクエニ、新作RPG『ファイナルファンタジー レゾナンス』の世界・システム情報を一挙公開(10/22発売)</t>
+        </is>
+      </c>
+      <c r="C316" s="15" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/011/G101135/20260715033/</t>
+        </is>
+      </c>
+      <c r="D316" s="15" t="inlineStr">
+        <is>
+          <t>スクウェア・エニックスはFFナンバリングとは別軸の新規タイトルで、秋の端境期の新作供給とFFブランドの多軸展開を図る。10/22発売に向け情報を段階的に開示。</t>
+        </is>
+      </c>
+      <c r="E316" s="15" t="inlineStr">
+        <is>
+          <t>7/16、10/22発売予定の『FFレゾナンス』について、世界観・キャラクター(飛空艇技師リド、軍師ニコル等)・ゲームシステムを一挙公開。秋のRPG商戦に向けた情報公開が本格化した。</t>
+        </is>
+      </c>
+      <c r="F316" s="15" t="inlineStr">
+        <is>
+          <t>10/22発売の新作RPG『FFレゾナンス』の世界・キャラ・システムを公開
+飛空艇技師リド、軍師ニコル等の新キャラを紹介
+秋のRPG商戦(10月)に向け情報公開が本格化</t>
+        </is>
+      </c>
+      <c r="G316" s="15" t="inlineStr">
+        <is>
+          <t>FFブランドの"ナンバリング外"多軸展開の成否が、既存IPの拡張戦略の試金石に。10月のRPG集中商戦で新規IPがどこまで存在感を出せるかが焦点。</t>
+        </is>
+      </c>
+      <c r="H316" s="15" t="inlineStr">
+        <is>
+          <t>FFブランドの多軸展開とRPG商戦カレンダー</t>
+        </is>
+      </c>
+      <c r="I316" s="15" t="inlineStr">
+        <is>
+          <t>スクウェア・エニックス</t>
+        </is>
+      </c>
+      <c r="J316" s="15" t="inlineStr">
+        <is>
+          <t>ファイナルファンタジー, FFレゾナンス</t>
+        </is>
+      </c>
+      <c r="K316" s="15" t="inlineStr">
+        <is>
+          <t>新作,国内</t>
+        </is>
+      </c>
+      <c r="L316" s="15" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
weekly-releases + indie + rankings update (2026-07-17 21:41)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -6919,7 +6919,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J82"/>
+  <dimension ref="A1:J101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9864,6 +9864,666 @@
       <c r="I82" t="inlineStr">
         <is>
           <t>GameGrin/SteamDB Steam週間トップセラー Week28(〜7/5) https://www.gamegrin.com/news/weekly-top-selling-games-on-steam-29th-of-june-to-5th-of-july-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-07-06〜07-12</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>1</v>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>リズム天国 ミラクルスターズ</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Switch</t>
+        </is>
+      </c>
+      <c r="F83" t="n">
+        <v>126073</v>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週間販売数【7/6〜7/12】 https://www.famitsu.com/article/202607/81618</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>2週連続首位。累計50万本突破。</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-07-06〜07-12</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>2</v>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>魔法少女ノ魔女裁判</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Switch</t>
+        </is>
+      </c>
+      <c r="F84" t="n">
+        <v>21283</v>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週間販売数【7/6〜7/12】 https://www.famitsu.com/article/202607/81618</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>新作。今週トップ10に新作6本ランクイン。</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-07-06〜07-12</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>3</v>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>トモダチコレクション わくわく生活</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Switch</t>
+        </is>
+      </c>
+      <c r="F85" t="n">
+        <v>20827</v>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週間販売数【7/6〜7/12】 https://www.famitsu.com/article/202607/81618</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-07-06〜07-12</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>4</v>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>アサシン クリード ブラックフラッグ RE：シンクロ</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>PS5</t>
+        </is>
+      </c>
+      <c r="F86" t="n">
+        <v>17152</v>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週間販売数【7/6〜7/12】 https://www.famitsu.com/article/202607/81618</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>国内PS5版。</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-07-06〜07-12</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>5</v>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Echoes of Aincrad（エコーズ・オブ・アインクラッド）</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>PS5</t>
+        </is>
+      </c>
+      <c r="F87" t="n">
+        <v>16092</v>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週間販売数【7/6〜7/12】 https://www.famitsu.com/article/202607/81618</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>SAO題材の新作アクションRPG。</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-07-06〜07-12</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>6</v>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>デジモンストーリー タイムストレンジャー</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Switch 2</t>
+        </is>
+      </c>
+      <c r="F88" t="n">
+        <v>15644</v>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週間販売数【7/6〜7/12】 https://www.famitsu.com/article/202607/81618</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-07-06〜07-12</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>7</v>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>グランブルーファンタジー リリンク：エンドレスラグナロク</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Switch 2</t>
+        </is>
+      </c>
+      <c r="F89" t="n">
+        <v>12544</v>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週間販売数【7/6〜7/12】 https://www.famitsu.com/article/202607/81618</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-07-06〜07-12</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>8</v>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>デジモンストーリー タイムストレンジャー</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Switch</t>
+        </is>
+      </c>
+      <c r="F90" t="n">
+        <v>11251</v>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週間販売数【7/6〜7/12】 https://www.famitsu.com/article/202607/81618</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>Switch版（Switch2版と別集計）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-07-06〜07-12</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>9</v>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>CRAZY CHA！N -エルピスの鎖-</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Switch</t>
+        </is>
+      </c>
+      <c r="F91" t="n">
+        <v>9874</v>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週間販売数【7/6〜7/12】 https://www.famitsu.com/article/202607/81618</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>新作。</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-07-06〜07-12</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>10</v>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>パワフルプロ野球2026-2027</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Switch</t>
+        </is>
+      </c>
+      <c r="F92" t="n">
+        <v>8917</v>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>ファミ通.com 週間販売数【7/6〜7/12】 https://www.famitsu.com/article/202607/81618</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-07-06〜07-12</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>1</v>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Assassin's Creed Black Flag Resynced（アサシン クリード ブラックフラッグ リシンクド）</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>VGChartz Steam週間トップセラー Week29 https://www.vgchartz.com/article/468471/steam-weekly-week-29-2026/ （GameGrin/SteamDB併用）</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>無料タイトル除く首位デビュー。発売1日で200万本(報道)、AC史上最高同接を記録。</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-07-06〜07-12</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>2</v>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Palworld（パルワールド）</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>VGChartz Steam週間トップセラー Week29 https://www.vgchartz.com/article/468471/steam-weekly-week-29-2026/ （GameGrin/SteamDB併用）</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>1.0正式版化で再浮上。</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2026-07-06〜07-12</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
+        <v>3</v>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Granblue Fantasy: Relink（グランブルーファンタジー リリンク）</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>VGChartz Steam週間トップセラー Week29 https://www.vgchartz.com/article/468471/steam-weekly-week-29-2026/ （GameGrin/SteamDB併用）</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>大型拡張で再ランクイン。</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2026-07-06〜07-12</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C96" t="n">
+        <v>5</v>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Granblue Fantasy: Relink - Endless Ragnarök Upgrade Kit</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>VGChartz Steam週間トップセラー Week29 https://www.vgchartz.com/article/468471/steam-weekly-week-29-2026/ （GameGrin/SteamDB併用）</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>アップグレードキットが5位デビュー。</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2026-07-06〜07-12</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C97" t="n">
+        <v>6</v>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Echoes of Aincrad（エコーズ・オブ・アインクラッド）</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>VGChartz Steam週間トップセラー Week29 https://www.vgchartz.com/article/468471/steam-weekly-week-29-2026/ （GameGrin/SteamDB併用）</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>6位デビュー。</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2026-07-06〜07-12</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C98" t="n">
+        <v>7</v>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Dead by Daylight（デッドバイデイライト）</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>VGChartz Steam週間トップセラー Week29 https://www.vgchartz.com/article/468471/steam-weekly-week-29-2026/ （GameGrin/SteamDB併用）</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>5ランクダウン。</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2026-07-06〜07-12</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C99" t="n">
+        <v>8</v>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Steam Deck</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>PC(ハードウェア)</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>VGChartz Steam週間トップセラー Week29 https://www.vgchartz.com/article/468471/steam-weekly-week-29-2026/ （GameGrin/SteamDB併用）</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2026-07-06〜07-12</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C100" t="n">
+        <v>9</v>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Cyberpunk 2077（サイバーパンク2077）</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>VGChartz Steam週間トップセラー Week29 https://www.vgchartz.com/article/468471/steam-weekly-week-29-2026/ （GameGrin/SteamDB併用）</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-07-06〜07-12</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C101" t="n">
+        <v>10</v>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>EA Sports FC 26</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>VGChartz Steam週間トップセラー Week29 https://www.vgchartz.com/article/468471/steam-weekly-week-29-2026/ （GameGrin/SteamDB併用）</t>
         </is>
       </c>
     </row>
@@ -32869,7 +33529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M32"/>
+  <dimension ref="A1:M37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -34389,6 +35049,236 @@
         </is>
       </c>
       <c r="M32" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/schedule/all-platforms/202608</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>DOOM: The Dark Ages | Revelations（DOOM ダークエイジ｜レベレーション）</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>id Software</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Bethesda / Xbox Game Studios</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>PC/PS5/Xbox Series X|S</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>FPS（大型拡張DLC）</t>
+        </is>
+      </c>
+      <c r="G33" t="n">
+        <v>89</v>
+      </c>
+      <c r="H33" t="n">
+        <v>90</v>
+      </c>
+      <c r="K33" t="n">
+        <v>4</v>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>今週リリース分。『DOOM: The Dark Ages』の大型拡張。MC89/OC90と高評価でシリーズDLCとして好発進。</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>https://opencritic.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>The Alters: Last Variable（ジ・オルターズ：ラスト・バリアブル）</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>11 bit studios</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>11 bit studios</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>PC/PS5/Xbox Series X|S</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>SFサバイバル/ナラティブ（拡張）</t>
+        </is>
+      </c>
+      <c r="G34" t="n">
+        <v>81</v>
+      </c>
+      <c r="K34" t="n">
+        <v>3</v>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>今週リリース分。『The Alters』の追加コンテンツ。MC81。</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>https://www.metacritic.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Avatar Legends: The Fighting Game（アバター レジェンズ：ザ・ファイティングゲーム）</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>PC/PS5/Xbox Series X|S</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>対戦格闘</t>
+        </is>
+      </c>
+      <c r="G35" t="n">
+        <v>76</v>
+      </c>
+      <c r="H35" t="n">
+        <v>79</v>
+      </c>
+      <c r="K35" t="n">
+        <v>3</v>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>今週リリース分。『アバター 伝説の少年アン』題材の対戦格闘。MC76/OC79。開発/パブリッシャーは要確認。</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>https://www.metacritic.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>キャプテン翼2 WORLD FIGHTERS（Captain Tsubasa 2: World Fighters）</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>KONAMI</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>KONAMI</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>PS5/Switch/Switch 2/PC</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>サッカーアクション</t>
+        </is>
+      </c>
+      <c r="K36" t="n">
+        <v>3</v>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>来月予定（評価系空欄）。『キャプテン翼』題材のアクション最新作。</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/schedule/all-platforms/202608</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-08 (日付未定)</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>LEGO バットマン：レガシー・オブ・ザ・ダークナイト（LEGO Batman: Legacy of the Dark Knight）</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>TT Games</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Warner Bros. Games</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>PC/PS5/Xbox Series X|S/Switch/Switch 2</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>アクションADV</t>
+        </is>
+      </c>
+      <c r="K37" t="n">
+        <v>3</v>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>来月予定（評価系空欄）。LEGOバットマン最新作。</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
         <is>
           <t>https://www.famitsu.com/schedule/all-platforms/202608</t>
         </is>
@@ -38744,7 +39634,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -39322,6 +40212,53 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ギャリー邸事件</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>小規模インディー（日本）</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2026-07-14 配信</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>ミステリー・アドベンチャー</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>1936年を舞台に過去の事件の真相を解き明かす和製ミステリーADV。落ち着いた雰囲気と推理要素でSNS・実況での言及が増加。</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>配信直後で注目インディーとして各メディアが紹介（公式実績値は追跡中）。</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Indie Freaks 7月注目インディーで紹介。短尺ナラティブ・ミステリーの系譜。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
daily-news + cross-questions + events + predictions + game-design update (2026-07-17)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -817,7 +817,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2010,6 +2010,43 @@
       <c r="G32" s="15" t="inlineStr">
         <is>
           <t>AppLovin/Unityの広告セグメントのガイダンスと広告主構成(中間層の増減)、ad-tech領域のM&amp;A件数、モバイル発クロスプラットフォーム移植の発表数を四半期で観測。</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B33" s="15" t="inlineStr">
+        <is>
+          <t>リアルタイム・ワールドモデル型エンジンの台頭で、Unity/Epicが生成レイヤーを内製化・買収し、エンジン競争の主戦場が『レンダリング/ツール』から『世界生成モデル』へ移動する</t>
+        </is>
+      </c>
+      <c r="C33" s="15" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="D33" s="15" t="inlineStr">
+        <is>
+          <t>2026年内〜2027年前半</t>
+        </is>
+      </c>
+      <c r="E33" s="15" t="inlineStr">
+        <is>
+          <t>Unity, Epic Games, PixVerse</t>
+        </is>
+      </c>
+      <c r="F33" s="15" t="inlineStr">
+        <is>
+          <t>PixVerse、シリーズC総額4.39億ドルでゲームエンジン参入(TechCrunch 2026-07-13)</t>
+        </is>
+      </c>
+      <c r="G33" s="15" t="inlineStr">
+        <is>
+          <t>Unity/Epicによる生成AI・ワールドモデル関連の買収／機能発表、主要エンジンへの自然言語シーン生成の統合有無を12カ月内に観測。</t>
         </is>
       </c>
     </row>
@@ -4158,7 +4195,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G74"/>
+  <dimension ref="A1:G76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6905,6 +6942,80 @@
       <c r="G74" s="15" t="inlineStr">
         <is>
           <t>有料UAで伸ばす成長モデルが飽和すると、各業界とも"獲得"から"既存顧客の再運用"へ重心が移る。ゲームのクロスプラットフォーム移植は他業界の"既存顧客LTV最大化"に相当。</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B75" s="15" t="inlineStr">
+        <is>
+          <t>リアルタイム・ワールドモデル(生成AIゲームエンジン)への大型資金流入は、映像制作・広告・建築ビジュアライゼーション等の『リアルタイム3D制作』パイプラインを侵食するか？</t>
+        </is>
+      </c>
+      <c r="C75" s="15" t="inlineStr">
+        <is>
+          <t>PixVerse、シリーズC総額4.39億ドルでゲームエンジン参入(TechCrunch)</t>
+        </is>
+      </c>
+      <c r="D75" s="15" t="inlineStr">
+        <is>
+          <t>PixVerse, Unity, Epic Games</t>
+        </is>
+      </c>
+      <c r="E75" s="15" t="inlineStr">
+        <is>
+          <t>映像制作・VFX / 広告クリエイティブ / 建築・都市ビジュアライゼーション / シミュレーション</t>
+        </is>
+      </c>
+      <c r="F75" s="15" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="G75" s="15" t="inlineStr">
+        <is>
+          <t>アセット生成の価値低下で、価値がIP・世界観設計・配信へ移動する仮説。ゲーム外の“リアルタイム3D”業界が最初の顧客になり得る。</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B76" s="15" t="inlineStr">
+        <is>
+          <t>大手が不採算部門を『IP付きの独立スピンアウト＋協業契約』で手放す手法は、製薬のスピンアウト創薬や大企業のカーブアウトと同じ力学か？</t>
+        </is>
+      </c>
+      <c r="C76" s="15" t="inlineStr">
+        <is>
+          <t>Compulsion GamesがIP保持でXboxから独立(VGC)</t>
+        </is>
+      </c>
+      <c r="D76" s="15" t="inlineStr">
+        <is>
+          <t>Microsoft, Compulsion Games</t>
+        </is>
+      </c>
+      <c r="E76" s="15" t="inlineStr">
+        <is>
+          <t>製薬(スピンアウト創薬) / 総合電機・自動車のカーブアウト / 事業承継・MBO</t>
+        </is>
+      </c>
+      <c r="F76" s="15" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="G76" s="15" t="inlineStr">
+        <is>
+          <t>“閉鎖”より“独立させて外注先化”の方が親会社・人材双方に得な局面があり得る。放出人材が競合パイプラインを担う逆説に注意。</t>
         </is>
       </c>
     </row>
@@ -11806,54 +11917,54 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="14" t="inlineStr">
+      <c r="A26" s="15" t="inlineStr">
         <is>
           <t>2026-07-15</t>
         </is>
       </c>
-      <c r="B26" s="14" t="inlineStr">
+      <c r="B26" s="15" t="inlineStr">
         <is>
           <t>2026-07-16</t>
         </is>
       </c>
-      <c r="C26" s="14" t="inlineStr">
+      <c r="C26" s="15" t="inlineStr">
         <is>
           <t>Taipei Game Developers Forum 2026 (TGDF)</t>
         </is>
       </c>
-      <c r="D26" s="14" t="inlineStr">
+      <c r="D26" s="15" t="inlineStr">
         <is>
           <t>展示会</t>
         </is>
       </c>
-      <c r="E26" s="14" t="inlineStr">
+      <c r="E26" s="15" t="inlineStr">
         <is>
           <t>台北（Taipei New Horizon）</t>
         </is>
       </c>
-      <c r="F26" s="14" t="inlineStr">
+      <c r="F26" s="15" t="inlineStr">
         <is>
           <t>オフライン</t>
         </is>
       </c>
-      <c r="G26" s="14" t="inlineStr">
+      <c r="G26" s="15" t="inlineStr">
         <is>
           <t>台湾最大級のゲーム開発者カンファレンス。アジア各国の開発者が集う。東映ゲームズ等日本勢も登壇。</t>
         </is>
       </c>
-      <c r="H26" s="14" t="inlineStr">
+      <c r="H26" s="15" t="inlineStr">
         <is>
           <t>https://www.4gamer.net/games/991/G999104/20260708042/</t>
         </is>
       </c>
-      <c r="I26" s="14" t="inlineStr">
-        <is>
-          <t>開催中</t>
-        </is>
-      </c>
-      <c r="J26" s="14" t="inlineStr">
-        <is>
-          <t>2026-07-16</t>
+      <c r="I26" s="15" t="inlineStr">
+        <is>
+          <t>終了</t>
+        </is>
+      </c>
+      <c r="J26" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
         </is>
       </c>
     </row>
@@ -12134,52 +12245,52 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="14" t="inlineStr">
-        <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="B5" s="14" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="inlineStr">
         <is>
           <t>ライブサービス／GaaS</t>
         </is>
       </c>
-      <c r="C5" s="14" t="inlineStr">
+      <c r="C5" s="15" t="inlineStr">
         <is>
           <t>マネタイズ/運営</t>
         </is>
       </c>
-      <c r="D5" s="14" t="inlineStr">
+      <c r="D5" s="15" t="inlineStr">
         <is>
           <t>成熟→選別(逆風)</t>
         </is>
       </c>
-      <c r="E5" s="14" t="inlineStr">
+      <c r="E5" s="15" t="inlineStr">
         <is>
           <t>継続課金・長期運営前提の大型タイトル。市場飽和とユーザー時間の奪い合いでサービス終了が相次ぐ。</t>
         </is>
       </c>
-      <c r="F5" s="14" t="inlineStr">
+      <c r="F5" s="15" t="inlineStr">
         <is>
           <t>Destiny 2(縮小), Fortnite, 各種運営型</t>
         </is>
       </c>
-      <c r="G5" s="14" t="inlineStr">
+      <c r="G5" s="15" t="inlineStr">
         <is>
           <t>供給過多・高い運営コスト・ヒット集中。大手が新規GaaS投資を抑制し選択と集中へ。</t>
         </is>
       </c>
-      <c r="H5" s="14" t="inlineStr">
-        <is>
-          <t>「広く薄く」から「絞って深く」へ。撤退の作法(返金/プレイ継続)も論点。PvE協力型へのシフト観測。</t>
-        </is>
-      </c>
-      <c r="I5" s="14" t="inlineStr">
-        <is>
-          <t>Bungie/Destiny縮小・大量解雇(6/27)</t>
-        </is>
-      </c>
-      <c r="J5" s="14" t="n">
+      <c r="H5" s="15" t="inlineStr">
+        <is>
+          <t>供給過多のジャンル(アイドル/リズム等)で3年前後の早期撤退が続き、選別が加速。運営型は少数の勝ち組へ集約、後発の新規参入ハードルが上昇。買い切り/短期イベント型への回帰やIPホルダーの運営外部委託が進む見込み。</t>
+        </is>
+      </c>
+      <c r="I5" s="15" t="inlineStr">
+        <is>
+          <t>『ワールドダイスター 夢のステラリウム』3年でサービス終了(AUTOMATON 2026-07-17)</t>
+        </is>
+      </c>
+      <c r="J5" s="15" t="n">
         <v>5</v>
       </c>
     </row>
@@ -13959,7 +14070,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L316"/>
+  <dimension ref="A1:L320"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -33517,6 +33628,254 @@
         </is>
       </c>
       <c r="L316" s="15" t="n"/>
+    </row>
+    <row r="317">
+      <c r="A317" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B317" s="15" t="inlineStr">
+        <is>
+          <t>Compulsion Games、Xboxから独立スピンアウト——IP保持し協業相手を公募</t>
+        </is>
+      </c>
+      <c r="C317" s="15" t="inlineStr">
+        <is>
+          <t>https://www.videogameschronicle.com/news/ex-xbox-studio-compulsion-games-invites-partners-to-collaborate-with-it-after-going-independent/</t>
+        </is>
+      </c>
+      <c r="D317" s="15" t="inlineStr">
+        <is>
+          <t>MicrosoftのXbox大規模再編（7月の追加人員削減・スタジオ整理）のなか、2018年にXboxが買収したCompulsion Games（『We Happy Few』『South of Midnight』）が“閉鎖”ではなく“IP保持つきの完全スピンアウト”という形で独立を選択。数日後には新たなパブリッシャー／協業相手の公募を開始した。</t>
+        </is>
+      </c>
+      <c r="E317" s="15" t="inlineStr">
+        <is>
+          <t>Compulsionは自社IP（Contrast, We Happy Few, South of Midnight）の権利を保持したままXboxから離脱し、独立スタジオへ復帰。移行期はXboxが一定の支援を提供。以後は共同開発・受託の協業パートナーとしての立ち位置を打ち出し、外部パブリッシャーやスタジオへ提携を呼びかけている。</t>
+        </is>
+      </c>
+      <c r="F317" s="15" t="inlineStr">
+        <is>
+          <t>閉鎖ではなくIP保持つきスピンアウトという“managed independence”型の手当
+買収から約8年で親会社→独立へ回帰、移行支援も付帯
+独立後は受託・共同開発の協業モデルで生存を図る
+Xboxの再編が中堅スタジオの独立・再分散を促す構図</t>
+        </is>
+      </c>
+      <c r="G317" s="15" t="inlineStr">
+        <is>
+          <t>プラットフォーマーが不採算スタジオを“IP付きで手放す”手法が定着すれば、放出された熟練チームがPlayStation陣営や中華資本(Tencent/NetEase)、他パブリッシャーの次期パイプラインを担い、Microsoftが結果的に競合を育てる逆説が進む。中堅スタジオの受託化で開発単価の下押し圧力も。</t>
+        </is>
+      </c>
+      <c r="H317" s="15" t="inlineStr">
+        <is>
+          <t>スタジオのカーブアウト／IP帰属設計と独立後の資金調達</t>
+        </is>
+      </c>
+      <c r="I317" s="15" t="inlineStr">
+        <is>
+          <t>Microsoft, Xbox Game Studios, Compulsion Games</t>
+        </is>
+      </c>
+      <c r="J317" s="15" t="inlineStr">
+        <is>
+          <t>Compulsion Games, We Happy Few, South of Midnight</t>
+        </is>
+      </c>
+      <c r="K317" s="15" t="inlineStr">
+        <is>
+          <t>M&amp;A,人事・組織,海外,トレンド</t>
+        </is>
+      </c>
+      <c r="L317" s="15" t="inlineStr"/>
+    </row>
+    <row r="318">
+      <c r="A318" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B318" s="15" t="inlineStr">
+        <is>
+          <t>AI動画生成PixVerse、シリーズC総額4.39億ドルで評価額20億ドル超——ゲームエンジン参入</t>
+        </is>
+      </c>
+      <c r="C318" s="15" t="inlineStr">
+        <is>
+          <t>https://techcrunch.com/2026/07/13/video-generation-startup-pixverse-raises-439m-valuation-soars-past-2b/</t>
+        </is>
+      </c>
+      <c r="D318" s="15" t="inlineStr">
+        <is>
+          <t>シンガポール拠点のAI動画生成スタートアップPixVerseがシリーズC延長ラウンドで累計4.39億ドルを調達し、評価額が20億ドル超に到達。Alibaba等が参加。同社は世界初を謳うリアルタイム・ワールドモデル『R1』を1月に投入し、これをゲーム制作に応用する『PixVerse Game Engine』へ拡張する。</t>
+        </is>
+      </c>
+      <c r="E318" s="15" t="inlineStr">
+        <is>
+          <t>PixVerseは調達資金でワールドモデル事業を拡大。R1は動画生成を“固定出力”から“ユーザー入力に即応する連続・インタラクティブなストリーム”へ転換する技術。ゲームエンジンはゲームの抽象メカニクスと視覚表現を分離し、プレイヤーが自然言語で操作すると世界が視覚・機構の両面でリアルタイム応答する。ユーザーは177カ国1.5億人超。</t>
+        </is>
+      </c>
+      <c r="F318" s="15" t="inlineStr">
+        <is>
+          <t>リアルタイム・ワールドモデルをゲーム制作に応用、評価額2Bドル超
+自然言語入力で世界が即応、メカニクスと表現を分離
+Alibaba等が出資、中国系AI×ゲームの資本集中が継続
+生成AIエンジンが従来型エンジンの制作前提を揺さぶる可能性</t>
+        </is>
+      </c>
+      <c r="G318" s="15" t="inlineStr">
+        <is>
+          <t>ワールドモデル型エンジンが実用水準に近づけば、アセット生成の価値が薄まり、価値がIP・世界観設計・配信へ移動する。Unity/Unrealはレンダリング競争から“世界生成モデル”競争へ主戦場を移され、生成レイヤーの内製化・買収に動く公算。映像・広告等の隣接業界の制作フローにも波及。</t>
+        </is>
+      </c>
+      <c r="H318" s="15" t="inlineStr">
+        <is>
+          <t>ワールドモデル/生成AIゲームエンジンの技術と事業構造</t>
+        </is>
+      </c>
+      <c r="I318" s="15" t="inlineStr">
+        <is>
+          <t>PixVerse, Alibaba, Unity, Epic Games</t>
+        </is>
+      </c>
+      <c r="J318" s="15" t="inlineStr">
+        <is>
+          <t>R1, PixVerse Game Engine</t>
+        </is>
+      </c>
+      <c r="K318" s="15" t="inlineStr">
+        <is>
+          <t>AI,技術,出資,海外,トレンド</t>
+        </is>
+      </c>
+      <c r="L318" s="15" t="inlineStr"/>
+    </row>
+    <row r="319">
+      <c r="A319" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B319" s="15" t="inlineStr">
+        <is>
+          <t>『ワールドダイスター 夢のステラリウム』3年でサービス終了——ライブサービス淘汰の実例</t>
+        </is>
+      </c>
+      <c r="C319" s="15" t="inlineStr">
+        <is>
+          <t>https://automaton-media.com/articles/newsjp/20260717-455582/</t>
+        </is>
+      </c>
+      <c r="D319" s="15" t="inlineStr">
+        <is>
+          <t>劇団テーマのリズムゲーム『ワールドダイスター 夢のステラリウム（ユメステ）』が2026年9月29日14時をもってサービスを終了すると告知。2023年のリリースから約3年での撤退で、供給過多が指摘されるアイドル／リズム系ライブサービス（GaaS）の選別が続いている実例となる。</t>
+        </is>
+      </c>
+      <c r="E319" s="15" t="inlineStr">
+        <is>
+          <t>ユメステはリリースから3年でサービス終了。多数の類似IP・キャラクター運営型スマホゲームがひしめくアイドル／リズム系ジャンルにおいて、一定規模に届かないタイトルの早期撤退が常態化しつつある。個別の不振報告にとどまらず、GaaSの“成熟→選別”局面を象徴する消費者・運営インサイトとして注目。</t>
+        </is>
+      </c>
+      <c r="F319" s="15" t="inlineStr">
+        <is>
+          <t>リリース約3年でのサービス終了、GaaS選別局面の実例
+アイドル/リズム系ライブサービスの供給過多と淘汰
+運営型IPの3年前後の生存ラインという時間軸
+IPホルダーの運営体制（内製/受託）見直しの契機</t>
+        </is>
+      </c>
+      <c r="G319" s="15" t="inlineStr">
+        <is>
+          <t>撤退が続けばIPホルダーは“運営型の内製リスク”を避け、既存IPの新規GaaSより買い切り／短期イベント型へ回帰、あるいは運営を外部受託へ移す動きが出る。ジャンル内の淘汰でユーザーと課金が少数の勝ち組へ再集約され、後発の新規参入ハードルが上がる。</t>
+        </is>
+      </c>
+      <c r="H319" s="15" t="inlineStr">
+        <is>
+          <t>GaaSのライフサイクルとジャンル内淘汰の力学</t>
+        </is>
+      </c>
+      <c r="I319" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ブシロード, </t>
+        </is>
+      </c>
+      <c r="J319" s="15" t="inlineStr">
+        <is>
+          <t>ワールドダイスター, 夢のステラリウム</t>
+        </is>
+      </c>
+      <c r="K319" s="15" t="inlineStr">
+        <is>
+          <t>ライブサービス,消費者インサイト,国内,トレンド</t>
+        </is>
+      </c>
+      <c r="L319" s="15" t="inlineStr">
+        <is>
+          <t>ミクロ×高インサイト枠</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B320" s="15" t="inlineStr">
+        <is>
+          <t>Valve「Steam Machine」7/17に再入荷——発売直後に即完売の需要続く</t>
+        </is>
+      </c>
+      <c r="C320" s="15" t="inlineStr">
+        <is>
+          <t>https://automaton-media.com/articles/newsjp/20260716-455246/</t>
+        </is>
+      </c>
+      <c r="D320" s="15" t="inlineStr">
+        <is>
+          <t>Valveの新型小型ゲーミングPC「Steam Machine」が7月17日午前10時に再入荷。発売直後に売り切れた反響を受けたもので、購入はひとり1台まで。据置き機に近い体験を狙うValveのリビング向けPCが、供給が需要に追いつかない状態が続いている。</t>
+        </is>
+      </c>
+      <c r="E320" s="15" t="inlineStr">
+        <is>
+          <t>Steam Machineは発売後すぐ売り切れ、7/17に在庫復活。数量制限つきでの再販となり、PCとコンソールの境界を曖昧にするValveのハード攻勢に対する消費者需要の強さを示す。単なる再販告知だが、“据置き機代替を狙う小型PC”への実需という点で、PC×コンソール融合トレンドの需要側シグナルとして拾う。</t>
+        </is>
+      </c>
+      <c r="F320" s="15" t="inlineStr">
+        <is>
+          <t>発売直後に即完売、再入荷でも1人1台制限
+Valveのリビング向け小型PCへの実需の強さ
+PCとコンソールの境界を曖昧にするハード戦略
+据置き機代替市場の需要側シグナル</t>
+        </is>
+      </c>
+      <c r="G320" s="15" t="inlineStr">
+        <is>
+          <t>供給が需要に追いつく水準まで出荷が進めば、SteamOS搭載据置き型PCが低〜中価格コンソールの一部需要を侵食し、任天堂/ソニー/MSの“専用機”前提に横やり。サードのSteam版最適化やクラウド連携が進む可能性。ただし当面は供給制約で影響は限定的。</t>
+        </is>
+      </c>
+      <c r="H320" s="15" t="inlineStr">
+        <is>
+          <t>PC×コンソール融合とValveのハード戦略</t>
+        </is>
+      </c>
+      <c r="I320" s="15" t="inlineStr">
+        <is>
+          <t>Valve</t>
+        </is>
+      </c>
+      <c r="J320" s="15" t="inlineStr">
+        <is>
+          <t>Steam Machine, SteamOS</t>
+        </is>
+      </c>
+      <c r="K320" s="15" t="inlineStr">
+        <is>
+          <t>ハード,消費者インサイト,海外</t>
+        </is>
+      </c>
+      <c r="L320" s="15" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
daily-news(+6) + cross-question(+1) + future(+1) + game-design update 2026-07-18
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -4195,7 +4195,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G76"/>
+  <dimension ref="A1:G77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7016,6 +7016,43 @@
       <c r="G76" s="15" t="inlineStr">
         <is>
           <t>“閉鎖”より“独立させて外注先化”の方が親会社・人材双方に得な局面があり得る。放出人材が競合パイプラインを担う逆説に注意。</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B77" s="14" t="inlineStr">
+        <is>
+          <t>ソブリンウェルスファンド(PIF)が大手パブリッシャーを丸ごとLBOで非公開化する動きは、映画・音楽・スポーツクラブなど他のエンタメIP資産でも同様に起きるか？政府系資金のコンテンツ垂直統合はどの業界に波及するか。</t>
+        </is>
+      </c>
+      <c r="C77" s="14" t="inlineStr">
+        <is>
+          <t>PIF主導のEA買収、EUが7/22承認へ(Reuters/KFGO, 2026-07-17)</t>
+        </is>
+      </c>
+      <c r="D77" s="14" t="inlineStr">
+        <is>
+          <t>PIF, Electronic Arts, Silver Lake, Savvy Games</t>
+        </is>
+      </c>
+      <c r="E77" s="14" t="inlineStr">
+        <is>
+          <t>映画・音楽(スタジオ/レーベル買収) / プロスポーツ(クラブ・リーグ保有) / メディア・放送 / PE・金融(SWFの直接投資)</t>
+        </is>
+      </c>
+      <c r="F77" s="14" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="G77" s="14" t="inlineStr">
+        <is>
+          <t>短期株主圧力を嫌う"良質だが低マージン"のIP資産は、SWF/PEの非公開化と相性が良い。ゲームは"最初の実験場"かもしれない。</t>
         </is>
       </c>
     </row>
@@ -12197,7 +12234,7 @@
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
@@ -12232,12 +12269,12 @@
       </c>
       <c r="H4" s="14" t="inlineStr">
         <is>
-          <t>Steam上半期売上の約79%が旧作という定量データで裏付け。リマスター/復刻/エバーグリーン運用は新作AAAより低リスク高効率として投資が集中し、"カタログ再運用"が主戦場化する見込み。</t>
+          <t>Steam上半期売上の約79%が旧作という定量データで裏付け。リマスター/復刻/エバーグリーン運用は新作AAAより低リスク高効率として投資が集中し、"カタログ再運用"が主戦場化する見込み。 / BethesdaもFallout 3・New Vegasリマスターを予告しFO5は長期化——AAA各社が"新作端境期をレガシー再運用で埋める"標準戦略化。</t>
         </is>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
-          <t>Steam2026年上半期売上111億ドル・旧作が収益の約79%(Game*Spark, 2026-07-16)</t>
+          <t>Steam2026年上半期売上111億ドル・旧作が収益の約79%(Game*Spark, 2026-07-16) / Bethesda Fallout新ロードマップ(Variety, 2026-07-18)</t>
         </is>
       </c>
       <c r="J4" s="14" t="n">
@@ -14070,7 +14107,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L320"/>
+  <dimension ref="A1:L325"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -33876,6 +33913,311 @@
         </is>
       </c>
       <c r="L320" s="15" t="inlineStr"/>
+    </row>
+    <row r="321">
+      <c r="A321" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B321" s="14" t="inlineStr">
+        <is>
+          <t>PIF主導のEA買収5.5兆円、EUが7/22に承認へ——史上最大級LBOが規制の最終関門を通過間近</t>
+        </is>
+      </c>
+      <c r="C321" s="14" t="inlineStr">
+        <is>
+          <t>https://kfgo.com/2026/07/17/exclusive-saudi-pif-set-to-win-eu-nod-for-electronic-arts-deal-under-subsidy-rules-sources-say/</t>
+        </is>
+      </c>
+      <c r="D321" s="14" t="inlineStr">
+        <is>
+          <t>サウジPIF・Silver Lake・Affinity Partnersによる総額550億ドル($210/株)のEA買収は、株主承認を経て規制審査段階に入っていた。EUは外国補助金規則(FSR)と合併規則の両面で審査し、7/22を予備審査の期限としていた。史上最大級のレバレッジド・バイアウト(LBO)。</t>
+        </is>
+      </c>
+      <c r="E321" s="14" t="inlineStr">
+        <is>
+          <t>関係者によると、EUはEA買収を補助金規則の下で無条件承認する見通しで、7/22に判断期限を迎える。合併規則でも無条件クリアが見込まれ、残る焦点は米当局の判断。ソブリンウェルスファンドによる大手パブリッシャーの完全非公開化が現実味を帯びる。</t>
+        </is>
+      </c>
+      <c r="F321" s="14" t="inlineStr">
+        <is>
+          <t>・買収総額550億ドル、$210/株の現金オファー
+・EUは外国補助金規則で無条件承認の見通し(7/22期限)
+・買い手はPIF・Silver Lake・Affinity Partners
+・成立すれば史上最大級のLBO、EAは非公開化</t>
+        </is>
+      </c>
+      <c r="G321" s="14" t="inlineStr">
+        <is>
+          <t>EU承認が通れば残る関門は米国審査。非公開化後のEAは四半期業績圧力から解放され、FC/Maddenなど年次スポーツIPの運営モデルやコスト構造の見直しが進む可能性。PIFのゲーム投資(Savvy/Scopely等)とのシナジーや、他大手への同種PE/SWF買収の連鎖も焦点。</t>
+        </is>
+      </c>
+      <c r="H321" s="14" t="inlineStr">
+        <is>
+          <t>ソブリンウェルスファンドによるコンテンツ産業の垂直統合とLBO</t>
+        </is>
+      </c>
+      <c r="I321" s="14" t="inlineStr">
+        <is>
+          <t>Electronic Arts, PIF(サウジ公共投資基金), Silver Lake, Affinity Partners</t>
+        </is>
+      </c>
+      <c r="J321" s="14" t="inlineStr">
+        <is>
+          <t>EA Sports FC, Madden, Battlefield, The Sims</t>
+        </is>
+      </c>
+      <c r="K321" s="14" t="inlineStr">
+        <is>
+          <t>M&amp;A, 適時開示, 規制, 海外</t>
+        </is>
+      </c>
+      <c r="L321" s="14" t="n"/>
+    </row>
+    <row r="322">
+      <c r="A322" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B322" s="14" t="inlineStr">
+        <is>
+          <t>Bethesda、Fallout新ロードマップ公開——『Fallout 5』プリプロ入り＋3/NVリマスター、Xbox再編後の"レガシー再運用"</t>
+        </is>
+      </c>
+      <c r="C322" s="14" t="inlineStr">
+        <is>
+          <t>https://variety.com/2026/gaming/news/fallout-5-elder-scrolls-6-game-updates-bethesda-todd-howard-1236814611/</t>
+        </is>
+      </c>
+      <c r="D322" s="14" t="inlineStr">
+        <is>
+          <t>Xbox部門の史上最大級レイオフ・スタジオ再編の直後、BethesdaのTodd Howardが今後の開発方針を表明。The Elder Scrolls VIを最優先(主力メンバーが従事)としつつ、Falloutシリーズの複数プロジェクトを提示した。</t>
+        </is>
+      </c>
+      <c r="E322" s="14" t="inlineStr">
+        <is>
+          <t>『Fallout 5』はCreation Engine 3でプリプロ入り。加えて『Fallout 3』『New Vegas』のリマスター、Obsidianとの新作、『Fallout 76』大型拡張"Raven Rock"(FO3前日譚)を予告。完全新作AAAの本命はESVIに集中させ、Falloutは既存資産の再運用で"つなぐ"構図。</t>
+        </is>
+      </c>
+      <c r="F322" s="14" t="inlineStr">
+        <is>
+          <t>・Fallout 5はCreation Engine 3でプリプロ段階(発売はかなり先)
+・ESVIが最優先開発、主力チームが従事
+・Fallout 3/New Vegasリマスター＋Obsidian新作を予告
+・Fallout 76に大型拡張"Raven Rock"を来年投入</t>
+        </is>
+      </c>
+      <c r="G322" s="14" t="inlineStr">
+        <is>
+          <t>新作AAAの開発長期化・高コスト化を背景に、リマスター/拡張で"端境期"の需要とブランド接点を維持する運用が定着。ドラマ版Falloutの好調と相まって、既知IPの再運用がAAA各社の標準戦略になる。ESVIの実際の発売時期がXbox再建の試金石。</t>
+        </is>
+      </c>
+      <c r="H322" s="14" t="inlineStr">
+        <is>
+          <t>AAA長期開発下でのリマスター/拡張による"レガシー再運用"戦略</t>
+        </is>
+      </c>
+      <c r="I322" s="14" t="inlineStr">
+        <is>
+          <t>Bethesda, Microsoft/Xbox, Obsidian</t>
+        </is>
+      </c>
+      <c r="J322" s="14" t="inlineStr">
+        <is>
+          <t>Fallout, Fallout 5, Fallout 3, Fallout: New Vegas, Fallout 76, The Elder Scrolls VI</t>
+        </is>
+      </c>
+      <c r="K322" s="14" t="inlineStr">
+        <is>
+          <t>新作, リメイク・移植, トレンド, 消費者インサイト, 海外</t>
+        </is>
+      </c>
+      <c r="L322" s="14" t="inlineStr">
+        <is>
+          <t>ミクロ×高インサイト枠(AAA疲れ／レガシー再運用の実例)</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B323" s="14" t="inlineStr">
+        <is>
+          <t>米加ゲーム労組、XboxレイオフでMicrosoftを不当労働行為でNLRB提訴——440組合員解雇の手続きを問題視</t>
+        </is>
+      </c>
+      <c r="C323" s="14" t="inlineStr">
+        <is>
+          <t>https://massivelyop.com/2026/07/17/unions-file-unfair-labor-complaints-accusing-microsoft-of-unlawful-firings-and-coercive-action-at-xbox-studios/</t>
+        </is>
+      </c>
+      <c r="D323" s="14" t="inlineStr">
+        <is>
+          <t>7/6にMicrosoftはXbox部門で即時1,600人＋今後1,600人の削減を発表。うちBethesda/ZeniMax系の組合員440人が対象となった。CWA・CWA Canadaは、削減前の団体交渉義務を果たさなかったとして反発を強めていた。</t>
+        </is>
+      </c>
+      <c r="E323" s="14" t="inlineStr">
+        <is>
+          <t>7/15、CWAとCWA CanadaはNLRBにMicrosoftを不当労働行為(ULP)で提訴。誠実交渉義務違反、威圧的行為、契約の一方的破棄、事前通知の欠如を主張。組合認証済み職場での一方的解雇は現状維持期間の団交義務に反すると訴える。</t>
+        </is>
+      </c>
+      <c r="F323" s="14" t="inlineStr">
+        <is>
+          <t>・CWA/CWA CanadaがNLRBにULP申立て(7/15)
+・対象は440組合員(Bethesda/ZeniMax/id等)
+・争点は団交前の一方的解雇と情報不開示
+・6スタジオで抗議マーチも並行</t>
+        </is>
+      </c>
+      <c r="G323" s="14" t="inlineStr">
+        <is>
+          <t>テック大手のゲーム部門で労組化が進むなか、大量解雇時の団交義務が法廷で争われる先例に。NLRBの判断次第で他のテック企業の再編手続きにも影響。組合の存在がレイオフのコスト・スピードを左右し、スタジオ運営の柔軟性と対立する構図が鮮明化。</t>
+        </is>
+      </c>
+      <c r="H323" s="14" t="inlineStr">
+        <is>
+          <t>ゲーム業界の労組化とレイオフ時の団体交渉義務(NLRB)</t>
+        </is>
+      </c>
+      <c r="I323" s="14" t="inlineStr">
+        <is>
+          <t>Microsoft/Xbox, CWA, Bethesda, ZeniMax, id Software</t>
+        </is>
+      </c>
+      <c r="J323" s="14" t="n"/>
+      <c r="K323" s="14" t="inlineStr">
+        <is>
+          <t>規制, 人事・組織, 海外</t>
+        </is>
+      </c>
+      <c r="L323" s="14" t="n"/>
+    </row>
+    <row r="324">
+      <c r="A324" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B324" s="14" t="inlineStr">
+        <is>
+          <t>2026年Q2のゲームM&amp;Aは23億ドル・54件——$100M超案件が続きミッドマーケットが牽引(Drake Star)</t>
+        </is>
+      </c>
+      <c r="C324" s="14" t="inlineStr">
+        <is>
+          <t>https://gamesbeat.com/financing-and-ma-for-games-make-strong-showing-in-q2-2026-drake-star-partners/</t>
+        </is>
+      </c>
+      <c r="D324" s="14" t="inlineStr">
+        <is>
+          <t>大型統合が一巡した後のゲーム業界M&amp;Aは、パンデミック期以来の水準でミッドマーケット(1億ドル超)が活発化。Drake Star Partnersの四半期レポートが2026年Q2の取引動向をまとめた。</t>
+        </is>
+      </c>
+      <c r="E324" s="14" t="inlineStr">
+        <is>
+          <t>Q2 2026のゲームM&amp;Aは54件・総額23億ドル。ScopelyによるLoom Games買収(10億ドル)などが牽引し、1億ドル超の案件数はコロナ期以来の高水準。ポートフォリオ多様化目的のスタジオ取得が主軸。EA買収成立が今後さらなるM&amp;Aを誘発するとの見方も。</t>
+        </is>
+      </c>
+      <c r="F324" s="14" t="inlineStr">
+        <is>
+          <t>・Q2 M&amp;Aは23億ドル/54件
+・$100M超案件はパンデミック以来の高水準
+・Scopely×Loom Games(10億ドル)が最大級
+・大型買収から中規模の"束ね買い"へ重心移動</t>
+        </is>
+      </c>
+      <c r="G324" s="14" t="inlineStr">
+        <is>
+          <t>巨額買収(EA/Savvy)が一巡し、今後は中規模スタジオの選別的取得が主戦場に。私募資金はゲーム本体よりAI・広告インフラへ集中する傾向が続き、開発スタジオ側は身売り/統合の受け皿探しが加速。EA非公開化の成否がM&amp;A市況の心理を左右。</t>
+        </is>
+      </c>
+      <c r="H324" s="14" t="inlineStr">
+        <is>
+          <t>ゲームM&amp;Aのミッドマーケット回帰とポートフォリオ多様化</t>
+        </is>
+      </c>
+      <c r="I324" s="14" t="inlineStr">
+        <is>
+          <t>Drake Star Partners, Scopely, Loom Games, Nazara</t>
+        </is>
+      </c>
+      <c r="J324" s="14" t="n"/>
+      <c r="K324" s="14" t="inlineStr">
+        <is>
+          <t>M&amp;A, 出資, トレンド, 海外</t>
+        </is>
+      </c>
+      <c r="L324" s="14" t="n"/>
+    </row>
+    <row r="325">
+      <c r="A325" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B325" s="14" t="inlineStr">
+        <is>
+          <t>eスポーツW杯2026、Apex+74%・Valorant-45.6%——タイトル別の視聴明暗が示す"スター/人気チーム依存"</t>
+        </is>
+      </c>
+      <c r="C325" s="14" t="inlineStr">
+        <is>
+          <t>https://escharts.com/news/valorant-esports-world-cup-2026-recap</t>
+        </is>
+      </c>
+      <c r="D325" s="14" t="inlineStr">
+        <is>
+          <t>7/6〜8/23のeスポーツW杯(EWC 2026、パリ)は複数タイトルを横断する大会。7/12にValorant部門が終了し、Esports Chartsが視聴データを公表した。</t>
+        </is>
+      </c>
+      <c r="E325" s="14" t="inlineStr">
+        <is>
+          <t>Valorantの決勝ピークは約24.8万人で前年比45.6%減。Fnatic/Sentinels/Gen.G等の人気勢が不在で関心が低下した。一方Apex Legendsは視聴74%増と好対照。同じ大会内でもタイトル・出場チーム次第で視聴が大きく振れ、eスポーツ人気の"スター/人気チーム依存"が浮き彫りに。</t>
+        </is>
+      </c>
+      <c r="F325" s="14" t="inlineStr">
+        <is>
+          <t>・Valorant決勝ピーク24.8万人、前年比-45.6%
+・人気チーム(Fnatic/Sentinels/Gen.G)不在が響く
+・Apex Legendsは+74%と明暗
+・開幕週の総視聴時間は+10%(Dota 2が牽引)</t>
+        </is>
+      </c>
+      <c r="G325" s="14" t="inlineStr">
+        <is>
+          <t>eスポーツの視聴は競技の魅力より"看板チーム/スター選手"の出場に強く連動する。主催者・パブリッシャーは人気チームの誘致やナラティブ設計を重視せざるを得ず、リーグの序列・シード制度やスター選手の待遇が興行価値を左右する。タイトル間で視聴のボラティリティが拡大。</t>
+        </is>
+      </c>
+      <c r="H325" s="14" t="inlineStr">
+        <is>
+          <t>eスポーツ視聴の人気チーム/スター依存と興行設計</t>
+        </is>
+      </c>
+      <c r="I325" s="14" t="inlineStr">
+        <is>
+          <t>Esports World Cup Foundation, Riot Games, EA(Apex)</t>
+        </is>
+      </c>
+      <c r="J325" s="14" t="inlineStr">
+        <is>
+          <t>VALORANT, Apex Legends, Dota 2</t>
+        </is>
+      </c>
+      <c r="K325" s="14" t="inlineStr">
+        <is>
+          <t>eスポーツ, 消費者インサイト, 海外</t>
+        </is>
+      </c>
+      <c r="L325" s="14" t="inlineStr">
+        <is>
+          <t>ミクロ×高インサイト枠(視聴のスター/チーム依存)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
daily-news + cross-questions + game-design update (2026-07-19)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -4195,7 +4195,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G77"/>
+  <dimension ref="A1:G78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7053,6 +7053,43 @@
       <c r="G77" s="14" t="inlineStr">
         <is>
           <t>短期株主圧力を嫌う"良質だが低マージン"のIP資産は、SWF/PEの非公開化と相性が良い。ゲームは"最初の実験場"かもしれない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B78" s="14" t="inlineStr">
+        <is>
+          <t>西側コンテンツIPの『中国ライセンシー運営』モデルは、ゲーム以外（映像・アニメ・出版・音楽）でも同様に短命化・撤退が増えるか？</t>
+        </is>
+      </c>
+      <c r="C78" s="14" t="inlineStr">
+        <is>
+          <t>FF14モバイル中国版の1年強での終了・グローバル版中止（VGC 2026-07-19）</t>
+        </is>
+      </c>
+      <c r="D78" s="14" t="inlineStr">
+        <is>
+          <t>スクウェア・エニックス, Tencent, ファイナルファンタジーXIV</t>
+        </is>
+      </c>
+      <c r="E78" s="14" t="inlineStr">
+        <is>
+          <t>エンタメ（映像/アニメ配信）, 出版, 広告（現地パートナー運営）, 小売（現地EC委託）</t>
+        </is>
+      </c>
+      <c r="F78" s="14" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="G78" s="14" t="inlineStr">
+        <is>
+          <t>現地パートナー委託は参入の近道だが、規制・採算・戦略変更で撤退が早い。IPホルダーの『運営主権』の設計思想が、他のコンテンツ産業でも論点化する。</t>
         </is>
       </c>
     </row>
@@ -12282,9 +12319,9 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
-        <is>
-          <t>2026-07-17</t>
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B5" s="15" t="inlineStr">
@@ -12317,14 +12354,14 @@
           <t>供給過多・高い運営コスト・ヒット集中。大手が新規GaaS投資を抑制し選択と集中へ。</t>
         </is>
       </c>
-      <c r="H5" s="15" t="inlineStr">
-        <is>
-          <t>供給過多のジャンル(アイドル/リズム等)で3年前後の早期撤退が続き、選別が加速。運営型は少数の勝ち組へ集約、後発の新規参入ハードルが上昇。買い切り/短期イベント型への回帰やIPホルダーの運営外部委託が進む見込み。</t>
-        </is>
-      </c>
-      <c r="I5" s="15" t="inlineStr">
-        <is>
-          <t>『ワールドダイスター 夢のステラリウム』3年でサービス終了(AUTOMATON 2026-07-17)</t>
+      <c r="H5" s="14" t="inlineStr">
+        <is>
+          <t>供給過多のジャンルで3年前後の早期撤退が続き選別が加速。加えて西側大手IPの『中国向け縮小モバイル版（委託運営）』も短命化し、運営型は少数の勝ち組へ集約。後発の新規参入ハードルが上昇し、買い切り/短期イベント型への回帰やIPホルダーの運営主権見直しが進む見込み。</t>
+        </is>
+      </c>
+      <c r="I5" s="14" t="inlineStr">
+        <is>
+          <t>『ワールドダイスター 夢のステラリウム』3年で終了(AUTOMATON 2026-07-17)／FF14モバイル中国版9/30終了・グローバル版中止(VGC 2026-07-19)</t>
         </is>
       </c>
       <c r="J5" s="15" t="n">
@@ -14107,7 +14144,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L325"/>
+  <dimension ref="A1:L327"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -34218,6 +34255,127 @@
           <t>ミクロ×高インサイト枠(視聴のスター/チーム依存)</t>
         </is>
       </c>
+    </row>
+    <row r="326">
+      <c r="A326" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B326" s="14" t="inlineStr">
+        <is>
+          <t>「FF14モバイル」中国版が9/30終了・グローバル版も中止——SEとTencentがライセンス解消</t>
+        </is>
+      </c>
+      <c r="C326" s="14" t="inlineStr">
+        <is>
+          <t>https://www.videogameschronicle.com/news/final-fantasy-14-mobiles-global-launch-has-been-cancelled/</t>
+        </is>
+      </c>
+      <c r="D326" s="14" t="inlineStr">
+        <is>
+          <t>FFXIV Mobileは、スクウェア・エニックスとTencent傘下Lightspeed Studiosが共同開発し2025年6月に中国で正式サービスを開始。本編MMOの単純移植ではなく、物語を凝縮しモバイル操作・戦闘に最適化した独立型MMORPGとして展開していた。当初SEは強力にプロモーションしたが、その後中国外での言及は徐々に減っていた。</t>
+        </is>
+      </c>
+      <c r="E326" s="14" t="inlineStr">
+        <is>
+          <t>7/17、SEとTencentはFFXIV Mobile中国版のライセンス契約を『事業運営の調整と市場環境の変化』を理由に解消し、2026/9/30でサービス終了、開発中だったグローバル版も中止すると発表。7/17時点で課金と新規登録を停止した。PC・家庭用の本編FF14は影響を受けず通常運営を継続する。</t>
+        </is>
+      </c>
+      <c r="F326" s="14" t="inlineStr">
+        <is>
+          <t>・中国版は稼働約1年3か月での早期撤退。西側大手IPの『中国ライセンシー運営』モデルの短命化を示す事例
+・縮小版モバイルMMOを畳む一方、SEは本編FF14のSwitch 2ネイティブ版を準備（8/1に実機プレイ生放送を予告）
+・ライセンス解消はTencent側の運営継続意欲の低下も示唆。中国市場での海外IPモバイル運営の採算難
+・グローバル版中止で、簡易モバイル版による本編MMOの新規層開拓という戦略が事実上頓挫</t>
+        </is>
+      </c>
+      <c r="G326" s="14" t="inlineStr">
+        <is>
+          <t>SEはモバイル簡易版よりも、本編MMOの新ハード（Switch 2）や既存プラットフォームへの展開に資源を集中させる公算。西側大手MMO/大作は『中国向け縮小モバイル版の新規開発』を手控え、クラウド配信や本体移植で中国・アジアを狙うモデルへ移る動きが強まる可能性。委託運営型タイトルの追加撤退にも要注意。</t>
+        </is>
+      </c>
+      <c r="H326" s="14" t="inlineStr">
+        <is>
+          <t>中国市場での海外IPライセンス運営モデルとモバイルMMOの採算構造</t>
+        </is>
+      </c>
+      <c r="I326" s="14" t="inlineStr">
+        <is>
+          <t>スクウェア・エニックス, Tencent, Lightspeed Studios</t>
+        </is>
+      </c>
+      <c r="J326" s="14" t="inlineStr">
+        <is>
+          <t>ファイナルファンタジーXIV, FFXIV Mobile</t>
+        </is>
+      </c>
+      <c r="K326" s="14" t="inlineStr">
+        <is>
+          <t>ライブサービス, 海外, 消費者インサイト</t>
+        </is>
+      </c>
+      <c r="L326" s="14" t="inlineStr"/>
+    </row>
+    <row r="327">
+      <c r="A327" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B327" s="14" t="inlineStr">
+        <is>
+          <t>eスポーツW杯2026 LoL部門がクライマックス——T1が準決勝進出、視聴堅調で7/19決勝へ</t>
+        </is>
+      </c>
+      <c r="C327" s="14" t="inlineStr">
+        <is>
+          <t>https://escharts.com/tournaments/lol/esports-world-cup-2026-lol</t>
+        </is>
+      </c>
+      <c r="D327" s="14" t="inlineStr">
+        <is>
+          <t>EWC2026（7/6～8/23、パリ）のLoL部門は7/15～19開催、賞金200万ドル・16チーム参加。7/18の準々～準決勝でT1がMSI覇者HLEを2-0で下して準決勝進出、Gen.GもJDGを撃破した。大会全体でLoLはValorant等を上回る視聴を集めており、7/19に決勝を予定している。</t>
+        </is>
+      </c>
+      <c r="E327" s="14" t="inlineStr">
+        <is>
+          <t>EWC2026のLoL部門は同大会屈指の視聴規模で推移し、注目カード（T1×BLG等）はピーク70万人超を記録。一方、同大会Valorant部門はピーク同接が前年比約46%減と伸び悩んでおり（7/18既報）、同一大会内でもタイトル間の視聴格差が鮮明になっている。</t>
+        </is>
+      </c>
+      <c r="F327" s="14" t="inlineStr">
+        <is>
+          <t>・MOBA（LoL/Dota2）の視聴は堅調、タクティカルシューター（Valorant）は前年比減——タイトル成熟度による明暗
+・多タイトルを束ねるEWC型モデルでも、視聴は少数の定番タイトルに集中する構造
+・韓国勢（T1・Gen.G）の強さが視聴を牽引し、地域×IPへの視聴依存が続く</t>
+        </is>
+      </c>
+      <c r="G327" s="14" t="inlineStr">
+        <is>
+          <t>EWCのような統合型大会は『集客タイトル（LoL/Dota2）』への依存を強め、伸び悩むタイトルの扱い（賞金配分・放送枠）見直し圧力が高まる可能性。視聴の定番集中が続けば、パブリッシャーは新興タイトルへのeスポーツ投資回収に一段の慎重さを求められる。</t>
+        </is>
+      </c>
+      <c r="H327" s="14" t="inlineStr">
+        <is>
+          <t>統合型eスポーツ大会におけるタイトル別視聴集中と投資配分</t>
+        </is>
+      </c>
+      <c r="I327" s="14" t="inlineStr">
+        <is>
+          <t>Esports World Cup Foundation, Riot Games, T1, Gen.G</t>
+        </is>
+      </c>
+      <c r="J327" s="14" t="inlineStr">
+        <is>
+          <t>League of Legends, VALORANT</t>
+        </is>
+      </c>
+      <c r="K327" s="14" t="inlineStr">
+        <is>
+          <t>eスポーツ, 海外, 消費者インサイト</t>
+        </is>
+      </c>
+      <c r="L327" s="14" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
weekly-stocks + IP watch update (2026-07-20 10:45)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -38243,7 +38243,10 @@
       </c>
       <c r="M2" s="9" t="inlineStr">
         <is>
-          <t>株価は6/26の6,589円を安値に7/2に7,137円へ反発、その後7,120円前後で横ばい推移し材料出尽くし後の水準確認局面。Switch 2値上げ(国内5.998万円)による普及ペース鈍化懸念は根強いが、FY26は売上2.31兆円(+98.6%)営業益3,601億円(+27.5%)と急回復済。次期は減収減益予想で新作ソフト継続投入が焦点。</t>
+          <t>【7/17】終値7,294円(前日比+214円,+3.02%)と逆行高。7/17の東京市場は日経平均が前日比2,694.42円安の64,141.12円と大幅続落し、3連休前にAI・半導体関連の利益確定売りが先行。一方で半導体・メモリー市況の落ち着き期待から「非AI」の内需・バリューへ循環物色が向かい、家庭用ゲーム大手が逆行高。gamebiz集計ではゲーム・エンタメ96銘柄中、上昇26(27%)・下落64(67%)と全体は軟調な中での選別買い。出典: gamebiz 2026/7/17
+---（前回までの記載）---
+株価は6/26の6,589円を安値に7/2に7,137円へ反発、その後7,120円前後で横ばい推移し材料出尽くし後の水準確認局面。Switch 2値上げ(国内5.998万円)による普及ペース鈍化懸念は根強いが、FY26は売上2.31兆円(+98.6%)営業益3,601億円(+27.5%)と急回復済。次期は減収減益予想で新作ソフト継続投入が焦点。
+なお、サウジPIF傘下Savvy Games Groupが当社を含む任天堂/バンダイナムコ/Nexon/コーエーテクモ/スクウェア・エニックスの約10%少数持分を約120億ドル規模でSavvyへ移管・集約済み（出典: Reuters/TechTimes 2026/7/17引用のPocketGamer.biz報）。</t>
         </is>
       </c>
       <c r="N2" s="9" t="inlineStr">
@@ -38263,7 +38266,7 @@
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
@@ -38353,7 +38356,9 @@
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>『鬼武者 Way of the Sword』発売日9/4前倒し発表(7/2)を受け株価は一時+8.4%高の3,272円まで上昇。13期連続営業増益・売上/営業益とも過去最高で好調継続。強力IPのリピート販売とデジタル比率上昇が寄与し、年内の新作寄与への期待が高まる。</t>
+          <t>【7/17】カプコンも大きく水準を切り上げ、任天堂とともに買われた。7/17の東京市場は日経平均が前日比2,694.42円安の64,141.12円と大幅続落し、3連休前にAI・半導体関連の利益確定売りが先行。一方で半導体・メモリー市況の落ち着き期待から「非AI」の内需・バリューへ循環物色が向かい、家庭用ゲーム大手が逆行高。gamebiz集計ではゲーム・エンタメ96銘柄中、上昇26(27%)・下落64(67%)と全体は軟調な中での選別買い。出典: gamebiz 2026/7/17
+---（前回までの記載）---
+『鬼武者 Way of the Sword』発売日9/4前倒し発表(7/2)を受け株価は一時+8.4%高の3,272円まで上昇。13期連続営業増益・売上/営業益とも過去最高で好調継続。強力IPのリピート販売とデジタル比率上昇が寄与し、年内の新作寄与への期待が高まる。</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
@@ -38373,7 +38378,7 @@
       </c>
       <c r="Q4" s="9" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
@@ -38420,7 +38425,10 @@
       </c>
       <c r="M5" s="9" t="inlineStr">
         <is>
-          <t>株価は2,601円(7/7 +1.8%)で推移。FY26は減収増益(売上-8.3%、営業益+34.9%)を達成しデジタル/ライツ事業が収益性改善に寄与。次回決算は8/10予定。『FFVIIリメイク』第2弾のマルチ展開拡大と2027年3月以降の大型タイトル定期供給方針を継続表明。</t>
+          <t>【7/17】スクウェア・エニックスHDも堅調に推移。7/17の東京市場は日経平均が前日比2,694.42円安の64,141.12円と大幅続落し、3連休前にAI・半導体関連の利益確定売りが先行。一方で半導体・メモリー市況の落ち着き期待から「非AI」の内需・バリューへ循環物色が向かい、家庭用ゲーム大手が逆行高。gamebiz集計ではゲーム・エンタメ96銘柄中、上昇26(27%)・下落64(67%)と全体は軟調な中での選別買い。出典: gamebiz 2026/7/17
+---（前回までの記載）---
+株価は2,601円(7/7 +1.8%)で推移。FY26は減収増益(売上-8.3%、営業益+34.9%)を達成しデジタル/ライツ事業が収益性改善に寄与。次回決算は8/10予定。『FFVIIリメイク』第2弾のマルチ展開拡大と2027年3月以降の大型タイトル定期供給方針を継続表明。
+なお、サウジPIF傘下Savvy Games Groupが当社を含む任天堂/バンダイナムコ/Nexon/コーエーテクモ/スクウェア・エニックスの約10%少数持分を約120億ドル規模でSavvyへ移管・集約済み（出典: Reuters/TechTimes 2026/7/17引用のPocketGamer.biz報）。</t>
         </is>
       </c>
       <c r="N5" s="9" t="inlineStr">
@@ -38440,7 +38448,7 @@
       </c>
       <c r="Q5" s="9" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
@@ -38487,7 +38495,9 @@
       </c>
       <c r="M6" s="9" t="inlineStr">
         <is>
-          <t>Steamサマーセール(6/26〜7/10)で『MGSΔ SNAKE EATER』を40%オフ販売し話題化。8月に『METAL GEAR SOLID: MASTER COLLECTION Vol.2』のグローバル発売を予定。過去人気IP復活とSwitch 2向け展開を積極化し、デジタル・スポーツIPが業績を下支え。</t>
+          <t>【7/17】KONAMI Gも大手ゲーム軒並み高の流れで上昇。7/17の東京市場は日経平均が前日比2,694.42円安の64,141.12円と大幅続落し、3連休前にAI・半導体関連の利益確定売りが先行。一方で半導体・メモリー市況の落ち着き期待から「非AI」の内需・バリューへ循環物色が向かい、家庭用ゲーム大手が逆行高。gamebiz集計ではゲーム・エンタメ96銘柄中、上昇26(27%)・下落64(67%)と全体は軟調な中での選別買い。出典: gamebiz 2026/7/17
+---（前回までの記載）---
+Steamサマーセール(6/26〜7/10)で『MGSΔ SNAKE EATER』を40%オフ販売し話題化。8月に『METAL GEAR SOLID: MASTER COLLECTION Vol.2』のグローバル発売を予定。過去人気IP復活とSwitch 2向け展開を積極化し、デジタル・スポーツIPが業績を下支え。</t>
         </is>
       </c>
       <c r="N6" s="9" t="inlineStr">
@@ -38507,7 +38517,7 @@
       </c>
       <c r="Q6" s="9" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
@@ -38554,7 +38564,10 @@
       </c>
       <c r="M7" s="9" t="inlineStr">
         <is>
-          <t>株価は4,074円前後(7/7)で推移、アナリスト平均目標株価は4,817円。FY26はガンダム牽引で売上1.348兆円(+8.6%)営業益1,895億円(+5.2%)と過去最高を更新済。IP軸のグローバル展開とトイホビー好調が継続し、大きな新規開示は乏しく好業績の持続力を見極める局面。</t>
+          <t>【7/17】バンダイナムコHDも大手ゲーム軒並み高の流れで上昇。7/17の東京市場は日経平均が前日比2,694.42円安の64,141.12円と大幅続落し、3連休前にAI・半導体関連の利益確定売りが先行。一方で半導体・メモリー市況の落ち着き期待から「非AI」の内需・バリューへ循環物色が向かい、家庭用ゲーム大手が逆行高。gamebiz集計ではゲーム・エンタメ96銘柄中、上昇26(27%)・下落64(67%)と全体は軟調な中での選別買い。出典: gamebiz 2026/7/17
+---（前回までの記載）---
+株価は4,074円前後(7/7)で推移、アナリスト平均目標株価は4,817円。FY26はガンダム牽引で売上1.348兆円(+8.6%)営業益1,895億円(+5.2%)と過去最高を更新済。IP軸のグローバル展開とトイホビー好調が継続し、大きな新規開示は乏しく好業績の持続力を見極める局面。
+なお、サウジPIF傘下Savvy Games Groupが当社を含む任天堂/バンダイナムコ/Nexon/コーエーテクモ/スクウェア・エニックスの約10%少数持分を約120億ドル規模でSavvyへ移管・集約済み（出典: Reuters/TechTimes 2026/7/17引用のPocketGamer.biz報）。</t>
         </is>
       </c>
       <c r="N7" s="9" t="inlineStr">
@@ -38574,7 +38587,7 @@
       </c>
       <c r="Q7" s="9" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
@@ -38676,7 +38689,8 @@
       </c>
       <c r="M9" s="9" t="inlineStr">
         <is>
-          <t>株価は1,593.5円(7/10)で推移、次回決算は7/27予定。鯉沼社長が『2035年までに営業利益で世界トップ10』を掲げ開発ライン増設・5,000人規模組織を目指す長期戦略を表明。『仁王3』はシリーズ最速で全世界100万本突破。足元はモバイル減速と先行投資で減収減益。</t>
+          <t>株価は1,593.5円(7/10)で推移、次回決算は7/27予定。鯉沼社長が『2035年までに営業利益で世界トップ10』を掲げ開発ライン増設・5,000人規模組織を目指す長期戦略を表明。『仁王3』はシリーズ最速で全世界100万本突破。足元はモバイル減速と先行投資で減収減益。
+なお、サウジPIF傘下Savvy Games Groupが当社を含む任天堂/バンダイナムコ/Nexon/コーエーテクモ/スクウェア・エニックスの約10%少数持分を約120億ドル規模でSavvyへ移管・集約済み（出典: Reuters/TechTimes 2026/7/17引用のPocketGamer.biz報）。</t>
         </is>
       </c>
       <c r="N9" s="9" t="inlineStr">
@@ -38696,7 +38710,7 @@
       </c>
       <c r="Q9" s="9" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
@@ -39181,7 +39195,7 @@
       <c r="D4" s="9" t="inlineStr"/>
       <c r="E4" s="9" t="inlineStr">
         <is>
-          <t>$8.03bn（FY26 Net Bookings）</t>
+          <t>$8.026bn（FY26 Net Bookings、+9% YoY）</t>
         </is>
       </c>
       <c r="F4" s="9" t="inlineStr"/>
@@ -39196,27 +39210,27 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>サウジPIF主導(Silver Lake/Affinity)の$55bn(1株$210)買収が進行、株価は過去最高$205.96(7/2)。欧州委員会は7/22までに承認可否を判断予定で、成立すれば史上最大のLBO・非公開化。『Battlefield 6』は1,000万本超の大ヒットでフランチャイズ戦略が奏功。</t>
+          <t>【7/17 Reuters独占】欧州委員会は競争法(merger)審査を7/22に無条件クリア、外国補助金規則(FSR)も予備審査終了の7/30までに承認見込みで、EUゲートは事実上通過へ。残る実質的な関門は米CFIUS(対米外国投資委員会)で、契約上のアウトサイドデートは9/28。当初のクロージング期限6/30は未達のまま延長済み。株主承認は2025年12月に可決、米HSR反トラストも取得済み。PIFが93.7%を握る支配株主となる構造。EA株は7月初旬時点で買収価格$210を$7〜9下回る水準で推移し、スプレッドはCFIUS不確実性を映す。FY26は純ブッキング$8.026bn(+9%)・純収益$7.531bnと過去最高だが、純利益は$1.121bn→$887m(-21%)と減益。出典: TechTimes/Reuters 2026/7/17</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>『Battlefield 6』1,000万本超の大ヒット、EA SPORTS FC等の安定収益</t>
+          <t>EU反トラスト/FSRの承認見込みで規制リスクが一段後退、Battlefield 6牽引でFY26純ブッキング過去最高$8.026bn、EA SPORTS FC等の安定収益、PIFの長期patient capital論</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>欧州委の審査(7/22期限)など買収完了の不確実性、非公開化に伴う戦略変化、期待先行の株価</t>
+          <t>CFIUS審査が未完了(アウトサイドデート9/28)でクロージング時期が未定、$200億の負債・レバレッジ約6倍(CreditSights)による将来のコスト削減圧力、クローズ前に2026年だけで3度のレイオフ(Skate/BF6開発、全社約300名、6月はTrust&amp;Safety等)、純利益-21%の減益</t>
         </is>
       </c>
       <c r="O4" s="9" t="inlineStr">
         <is>
-          <t>$55bn買収(7/22 EU判断)の成否、Battlefieldライブサービス化の定着、次期スポーツ更新需要</t>
+          <t>CFIUSの結論(緩和条件付き承認か)と9/28アウトサイドデートの扱い、EU承認(7/22反トラスト・7/30 FSR)の確定、クローズ後の債務返済負担とスタジオ・人員体制、Battlefieldライブサービスの定着</t>
         </is>
       </c>
       <c r="P4" s="9" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
daily-news(6genres) + cross-questions + events + predictions update (2026-07-20)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -886,7 +886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2324,6 +2324,48 @@
       <c r="H34" s="9" t="inlineStr">
         <is>
           <t>ゲーム</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B35" s="15" t="inlineStr">
+        <is>
+          <t>音楽ディストリビューター(DistroKid等)がPE傘下に入ったことで、『中立の配信取次』から『出資者のアーティスト発掘・権利取得パイプライン』へ役割が変質。利用規約にデータ提供・優先交渉権が組み込まれ、反動として『中立性』を売りにする新興ディストリビューターとアーティスト協同組合型サービスが差別化軸として台頭する。</t>
+        </is>
+      </c>
+      <c r="C35" s="15" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="D35" s="15" t="inlineStr">
+        <is>
+          <t>12〜18ヶ月</t>
+        </is>
+      </c>
+      <c r="E35" s="15" t="inlineStr">
+        <is>
+          <t>CVC,DistroKid,Primary Wave,Kobalt,UnitedMasters,TuneCore</t>
+        </is>
+      </c>
+      <c r="F35" s="15" t="inlineStr">
+        <is>
+          <t>『CVCがDistroKidの過半数株取得』(Music Business Worldwide 7月)／『Primary WaveのKobalt買収完了』(MBW 7/7)</t>
+        </is>
+      </c>
+      <c r="G35" s="15" t="inlineStr">
+        <is>
+          <t>DistroKidの利用規約・プライバシーポリシー改定の有無と改定内容(データ利用・優先交渉権の追加)、および中立訴求型ディストリビューターの資金調達・取扱いリリース数シェアを四半期で観測する。</t>
+        </is>
+      </c>
+      <c r="H35" s="15" t="inlineStr">
+        <is>
+          <t>音楽</t>
         </is>
       </c>
     </row>
@@ -4858,7 +4900,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H80"/>
+  <dimension ref="A1:H82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8228,6 +8270,90 @@
       <c r="H80" s="9" t="inlineStr">
         <is>
           <t>ゲーム</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B81" s="15" t="inlineStr">
+        <is>
+          <t>音楽で起きている『権利カタログ＋徴収インフラのPE集約』は、アニメ・漫画の原作IPカタログでも起きるか？出版社の版権部門や制作会社の保有IPがファンドの買収対象になる日は来るか？</t>
+        </is>
+      </c>
+      <c r="C81" s="15" t="inlineStr">
+        <is>
+          <t>Primary WaveのKobalt買収完了(約15億ドル、MBW 7/7)／CVCのDistroKid過半数取得(MBW)</t>
+        </is>
+      </c>
+      <c r="D81" s="15" t="inlineStr">
+        <is>
+          <t>Primary Wave,Kobalt,CVC,DistroKid,集英社,講談社,小学館集英社プロダクション</t>
+        </is>
+      </c>
+      <c r="E81" s="15" t="inlineStr">
+        <is>
+          <t>PE・プライベートクレジット／知財ファイナンス／音楽著作権ファンド</t>
+        </is>
+      </c>
+      <c r="F81" s="15" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="G81" s="15" t="inlineStr">
+        <is>
+          <t>音楽は『安定キャッシュフロー資産』として金融化が完了しつつある。アニメ・漫画IPは収益の変動が大きく金融化が遅れているが、配信ライセンス収入が積み上がれば同じ道を辿る余地。AniBizのような取引所は価格発見を進め、金融化の前提条件を整える方向に働く点が示唆的。</t>
+        </is>
+      </c>
+      <c r="H81" s="15" t="inlineStr">
+        <is>
+          <t>横断</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B82" s="15" t="inlineStr">
+        <is>
+          <t>Crunchyrollが物販を上位サブスク会員限定にした『特典としての物販』は、音楽のファンクラブD2Cやゲームのサブスク特典でも同じ形に収斂するか？各ジャンルのARPU向上手段は最終的に同じ設計に行き着くのか？</t>
+        </is>
+      </c>
+      <c r="C82" s="15" t="inlineStr">
+        <is>
+          <t>Crunchyroll、8月からストアをMega/Ultimate限定へ(ANN 7/14)／UMG×EVENのD2C提携(MBW)</t>
+        </is>
+      </c>
+      <c r="D82" s="15" t="inlineStr">
+        <is>
+          <t>Crunchyroll,ソニー,Universal Music Group,EVEN,Microsoft(Game Pass)</t>
+        </is>
+      </c>
+      <c r="E82" s="15" t="inlineStr">
+        <is>
+          <t>小売のサブスク型会員制(Amazonプライム・コストコ)／航空・ホテルの上級会員制度</t>
+        </is>
+      </c>
+      <c r="F82" s="15" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="G82" s="15" t="inlineStr">
+        <is>
+          <t>配信・音楽・ゲームのいずれも『月額値上げが効きにくい』という同じ制約に直面し、解として『上位ティア＋限定物販』に収斂しつつある。ジャンルは違えど打ち手が同型という点が興味深い。逆に言えば差別化余地は限定商品のIP強度のみになる。</t>
+        </is>
+      </c>
+      <c r="H82" s="15" t="inlineStr">
+        <is>
+          <t>横断</t>
         </is>
       </c>
     </row>
@@ -11861,7 +11987,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J30"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13219,12 +13345,12 @@
       </c>
       <c r="I27" s="15" t="inlineStr">
         <is>
-          <t>開催中</t>
+          <t>終了</t>
         </is>
       </c>
       <c r="J27" s="15" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-20</t>
         </is>
       </c>
     </row>
@@ -13371,6 +13497,54 @@
         </is>
       </c>
       <c r="J30" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B31" s="15" t="n"/>
+      <c r="C31" s="15" t="inlineStr">
+        <is>
+          <t>第175回 芥川龍之介賞・直木三十五賞 選考会・発表</t>
+        </is>
+      </c>
+      <c r="D31" s="15" t="inlineStr">
+        <is>
+          <t>映画祭・賞</t>
+        </is>
+      </c>
+      <c r="E31" s="15" t="inlineStr">
+        <is>
+          <t>東京</t>
+        </is>
+      </c>
+      <c r="F31" s="15" t="inlineStr">
+        <is>
+          <t>リアル</t>
+        </is>
+      </c>
+      <c r="G31" s="15" t="inlineStr">
+        <is>
+          <t>芥川賞=小砂川チト『ゾンビ回収婦』(講談社)、直木賞=朝倉かすみ『けんぐゎい』(光文社)。受賞作は増刷・映像化打診の起点となり、下期文芸売上を左右する。</t>
+        </is>
+      </c>
+      <c r="H31" s="15" t="inlineStr">
+        <is>
+          <t>https://news.web.nhk/newsweb/na/na-k10015176901000</t>
+        </is>
+      </c>
+      <c r="I31" s="15" t="inlineStr">
+        <is>
+          <t>終了</t>
+        </is>
+      </c>
+      <c r="J31" s="15" t="inlineStr">
         <is>
           <t>2026-07-20</t>
         </is>
@@ -16478,7 +16652,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M332"/>
+  <dimension ref="A1:M347"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -38675,6 +38849,1000 @@
         </is>
       </c>
       <c r="M332" s="15" t="n"/>
+    </row>
+    <row r="333">
+      <c r="A333" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B333" s="15" t="inlineStr">
+        <is>
+          <t>ゲーム</t>
+        </is>
+      </c>
+      <c r="C333" s="15" t="inlineStr">
+        <is>
+          <t>韓国ゲーム大手に大型M&amp;A連鎖——Wemade創業者株が香港ファンドへ9200億ウォンで移転</t>
+        </is>
+      </c>
+      <c r="D333" s="15" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/991/G999101/20260707014/</t>
+        </is>
+      </c>
+      <c r="E333" s="15" t="inlineStr">
+        <is>
+          <t>韓国ゲーム産業は内需頭打ちと中国・グローバル競争激化で収益が伸び悩み、創業者一族の持株比率が高い企業ほど資本政策の自由度が低い状態が続いていた。2026年に入り海外資本を受け入れる形での支配権移転が相次いでいる。</t>
+        </is>
+      </c>
+      <c r="F333" s="15" t="inlineStr">
+        <is>
+          <t>Wemadeは創業者Park Kwan-ho氏の保有全株を香港の投資プラットフォームNeoPulseへ約9200億ウォン（約960億円）で売却する契約を締結。カカオゲームズも筆頭株主がカカオからLINEヤフーへ交代しており、韓国ゲーム大手の資本構造が短期間で相次いで組み替わっている。</t>
+        </is>
+      </c>
+      <c r="G333" s="15" t="inlineStr">
+        <is>
+          <t>創業者主導から外部資本主導への支配権移転が連鎖
+買い手が香港ファンド・日本のLINEヤフーなど域外資本に偏る
+グローバル展開の再起動が名目だが実態は資金繰り／事業再編色も強い
+韓国発IPの意思決定が国外に移るガバナンス変化</t>
+        </is>
+      </c>
+      <c r="H333" s="15" t="inlineStr">
+        <is>
+          <t>支配権を得た外部資本は既存IPの選別と不採算タイトルの整理を先行させる公算が大きい。1〜2年内に韓国大手発の新規大型IPは減り、代わりに既存MMO・モバイルIPの他地域ライセンスアウトとコンソール移植が増える。日韓資本の交差でLINEヤフー経由の日本市場配信も増える見込み。</t>
+        </is>
+      </c>
+      <c r="I333" s="15" t="inlineStr">
+        <is>
+          <t>支配権市場（M&amp;A）と創業者持株比率／クロスボーダー投資規制</t>
+        </is>
+      </c>
+      <c r="J333" s="15" t="inlineStr">
+        <is>
+          <t>Wemade,NeoPulse,カカオゲームズ,LINEヤフー,カカオ</t>
+        </is>
+      </c>
+      <c r="K333" s="15" t="inlineStr">
+        <is>
+          <t>ミル系IP,オーディン</t>
+        </is>
+      </c>
+      <c r="L333" s="15" t="inlineStr">
+        <is>
+          <t>M&amp;A,海外,トレンド</t>
+        </is>
+      </c>
+      <c r="M333" s="15" t="inlineStr">
+        <is>
+          <t>韓国大手の資本再編ウォッチ継続</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B334" s="15" t="inlineStr">
+        <is>
+          <t>ゲーム</t>
+        </is>
+      </c>
+      <c r="C334" s="15" t="inlineStr">
+        <is>
+          <t>テイツーQ1営業益257%増——中古トレカとSwitch 2値上げ前の駆け込みが二次流通を押し上げ</t>
+        </is>
+      </c>
+      <c r="D334" s="15" t="inlineStr">
+        <is>
+          <t>https://gamebiz.jp/news/429602</t>
+        </is>
+      </c>
+      <c r="E334" s="15" t="inlineStr">
+        <is>
+          <t>任天堂はSwitch 2の価格改定を予告しており、値上げ前の駆け込み需要が新品・中古双方に発生。同時にトレーディングカードの二次流通価格が高止まりし、リユース事業者の粗利率が構造的に改善する局面が続いていた。</t>
+        </is>
+      </c>
+      <c r="F334" s="15" t="inlineStr">
+        <is>
+          <t>2026年7月13〜17日に発表されたゲーム関連決算のうち、テイツーの第1四半期は営業利益が前年同期比257%増の7億9200万円と突出。中古トレカ・ゲームの好調に加え、Switch 2値上げ前の駆け込み需要が寄与した。同週はアクワイア・OLM・オーバーラップHDなども開示。</t>
+        </is>
+      </c>
+      <c r="G334" s="15" t="inlineStr">
+        <is>
+          <t>ハード値上げ局面で利益が伸びるのは一次流通ではなく二次流通側
+中古トレカが小売の主戦場になりつつある構造変化
+営業益+257%は単発の好調ではなくマージン構造の変化を示唆
+リユース在庫の評価益が業績を押し上げる会計上の性質にも注意</t>
+        </is>
+      </c>
+      <c r="H334" s="15" t="inlineStr">
+        <is>
+          <t>ハード値上げが常態化すると新品の買い控えと中古回転の加速が同時に進み、リユース業態の収益がさらに拡大する。メーカー側はこの利益プールを見過ごせず、公式リファービッシュや下取りプログラムで二次流通マージンの内部化に動く可能性が高い。</t>
+        </is>
+      </c>
+      <c r="I334" s="15" t="inlineStr">
+        <is>
+          <t>リユース／二次流通の粗利構造とハード価格政策の相互作用</t>
+        </is>
+      </c>
+      <c r="J334" s="15" t="inlineStr">
+        <is>
+          <t>テイツー,任天堂,アクワイア,OLM,オーバーラップホールディングス</t>
+        </is>
+      </c>
+      <c r="K334" s="15" t="inlineStr">
+        <is>
+          <t>Nintendo Switch 2,ポケモンカードゲーム</t>
+        </is>
+      </c>
+      <c r="L334" s="15" t="inlineStr">
+        <is>
+          <t>業績,国内,消費者インサイト</t>
+        </is>
+      </c>
+      <c r="M334" s="15" t="inlineStr">
+        <is>
+          <t>ミクロ×高インサイト枠：値上げ局面の利益移転を示す実例</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B335" s="15" t="inlineStr">
+        <is>
+          <t>ゲーム</t>
+        </is>
+      </c>
+      <c r="C335" s="15" t="inlineStr">
+        <is>
+          <t>4Gamer連載が指摘する「力技の効率化」——人員削減によるコスト圧縮が開発文化を痩せさせる懸念</t>
+        </is>
+      </c>
+      <c r="D335" s="15" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/036/G003691/20260713001/</t>
+        </is>
+      </c>
+      <c r="E335" s="15" t="inlineStr">
+        <is>
+          <t>2026年上半期だけで世界のゲーム業界は推定8000〜1万2000人規模の人員削減を経験。MicrosoftのXbox部門3200人削減など大手の再編が相次ぎ、市場規模は過去最高を更新する一方で雇用は縮小するという乖離が生じている。</t>
+        </is>
+      </c>
+      <c r="F335" s="15" t="inlineStr">
+        <is>
+          <t>4Gamer「Access Accepted」第866回は、業界が進める効率化の実態が生産性改善ではなく人員削減という「力技」に偏っていると指摘。任天堂・岩田聡氏が説いた、人を減らさずに価値を生む経営観を引き合いに、短期のコスト削減が中長期の開発力を損なうリスクを論じた。</t>
+        </is>
+      </c>
+      <c r="G335" s="15" t="inlineStr">
+        <is>
+          <t>市場最高益と大量解雇が同時に起きる構造的乖離
+効率化の中身が工程改善ではなく人件費削減に集中
+熟練人材の流出は数年遅れで開発力低下として顕在化
+AI導入が「人を減らす口実」として使われる懸念</t>
+        </is>
+      </c>
+      <c r="H335" s="15" t="inlineStr">
+        <is>
+          <t>削減された熟練層の一部は中規模スタジオの新設や既存インディーへの合流に向かい、2027年以降に中堅レンジの新作供給が一時的に増える。一方で大手は外注比率を高め、開発受託スタジオの交渉力が相対的に上がる局面が来る。</t>
+        </is>
+      </c>
+      <c r="I335" s="15" t="inlineStr">
+        <is>
+          <t>ゲーム開発の固定費構造と人的資本／組織能力の毀損</t>
+        </is>
+      </c>
+      <c r="J335" s="15" t="inlineStr">
+        <is>
+          <t>Microsoft,任天堂,ソニー・インタラクティブエンタテインメント,Electronic Arts</t>
+        </is>
+      </c>
+      <c r="K335" s="15" t="inlineStr">
+        <is>
+          <t>Xbox,Hellblade</t>
+        </is>
+      </c>
+      <c r="L335" s="15" t="inlineStr">
+        <is>
+          <t>トレンド,海外,人事・組織</t>
+        </is>
+      </c>
+      <c r="M335" s="15" t="inlineStr">
+        <is>
+          <t>業界論考。数字より構造理解に有用</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B336" s="15" t="inlineStr">
+        <is>
+          <t>映画</t>
+        </is>
+      </c>
+      <c r="C336" s="15" t="inlineStr">
+        <is>
+          <t>『The Odyssey』北米OW1億2400万ドル超——2026年の実写最高、劇場回帰トレンドを裏付け</t>
+        </is>
+      </c>
+      <c r="D336" s="15" t="inlineStr">
+        <is>
+          <t>https://deadline.com/2026/07/box-office-the-odyssey-1236993792/</t>
+        </is>
+      </c>
+      <c r="E336" s="15" t="inlineStr">
+        <is>
+          <t>劇場興行はコロナ後の低迷を脱しつつあり、2026年はレガシースタジオが公開本数を戻し、配信専業だったAmazon MGMも劇場公開に回帰。大作の初動が配信同時公開ではなく専有ウィンドウで最大化される流れが強まっていた。</t>
+        </is>
+      </c>
+      <c r="F336" s="15" t="inlineStr">
+        <is>
+          <t>クリストファー・ノーラン監督『The Odyssey』が北米オープニング3日間で1億2400万ドル超を記録し、2026年の実写作品では最高、マット・デイモン主演作としても最高記録となった。CinemaScoreはA評価で、口コミ主導のロングランが見込まれる展開。</t>
+        </is>
+      </c>
+      <c r="G336" s="15" t="inlineStr">
+        <is>
+          <t>オリジナル寄りの大作でも1億ドル超の初動が成立
+CinemaScore Aは初動型ではなく持久型の興行を示唆
+配信全盛下でも劇場が話題形成の起点として機能
+IMAXなどプレミアム大型フォーマットの客単価寄与</t>
+        </is>
+      </c>
+      <c r="H336" s="15" t="inlineStr">
+        <is>
+          <t>オリジナル企画の大型興行成功が続けば、スタジオの投資配分がフランチャイズ偏重から作家主導の大作へ部分的に戻る。ただし成立条件は監督ブランドとプレミアムフォーマット確保に限定され、中規模オリジナルへの波及は限定的にとどまる公算。</t>
+        </is>
+      </c>
+      <c r="I336" s="15" t="inlineStr">
+        <is>
+          <t>劇場ウィンドウ戦略とプレミアムフォーマットの収益寄与</t>
+        </is>
+      </c>
+      <c r="J336" s="15" t="inlineStr">
+        <is>
+          <t>Universal Pictures,IMAX,Amazon MGM Studios</t>
+        </is>
+      </c>
+      <c r="K336" s="15" t="inlineStr">
+        <is>
+          <t>The Odyssey</t>
+        </is>
+      </c>
+      <c r="L336" s="15" t="inlineStr">
+        <is>
+          <t>興行,海外,チャート・ランキング</t>
+        </is>
+      </c>
+      <c r="M336" s="15" t="inlineStr"/>
+    </row>
+    <row r="337">
+      <c r="A337" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B337" s="15" t="inlineStr">
+        <is>
+          <t>映画</t>
+        </is>
+      </c>
+      <c r="C337" s="15" t="inlineStr">
+        <is>
+          <t>北米2026年興収は年初来54億ドル・前年比10%増——Amazon MGMが劇場公開を3本→13本へ</t>
+        </is>
+      </c>
+      <c r="D337" s="15" t="inlineStr">
+        <is>
+          <t>https://variety.com/2026/film/box-office/movie-theaters-rebound-box-office-obsession-project-hail-mary-1236810214/</t>
+        </is>
+      </c>
+      <c r="E337" s="15" t="inlineStr">
+        <is>
+          <t>配信優先戦略の見直しが進み、劇場公開が話題形成とライブラリ価値の双方に効くという再評価が起きていた。同時にBlack Bearなど新興配給の参入で公開本数の供給制約が緩和しつつある。</t>
+        </is>
+      </c>
+      <c r="F337" s="15" t="inlineStr">
+        <is>
+          <t>Varietyによれば2026年の北米興収は1月1日〜7月19日で54億ドル、前年同期比10%増と、コロナ後で最高水準（2019年比では10億ドル差）。Warner Bros.・Sony・Paramountが公開本数を増やしたうえ、Amazon MGMが2025年の3本から2026年は13本へ劇場公開を拡大した。</t>
+        </is>
+      </c>
+      <c r="G337" s="15" t="inlineStr">
+        <is>
+          <t>回復の主因は単価ではなく公開本数（供給）の回復
+配信専業だったAmazon MGMの劇場回帰が象徴的
+新興配給Black Bearの参入でスクリーン供給の担い手が分散
+2019年水準まであと10億ドルの射程に入った</t>
+        </is>
+      </c>
+      <c r="H337" s="15" t="inlineStr">
+        <is>
+          <t>供給回復が続けば2027年には2019年水準の回復が視野に入る一方、スクリーン数は減少したままのため公開作品間のスクリーン争奪が激化する。中規模作品が上映期間を確保できず、配信直行との二極化がむしろ進む可能性がある。</t>
+        </is>
+      </c>
+      <c r="I337" s="15" t="inlineStr">
+        <is>
+          <t>劇場興行の供給側指標（公開本数・スクリーン数）と配信の窓口設計</t>
+        </is>
+      </c>
+      <c r="J337" s="15" t="inlineStr">
+        <is>
+          <t>Amazon MGM Studios,Warner Bros.,Sony Pictures,Paramount,Black Bear</t>
+        </is>
+      </c>
+      <c r="K337" s="15" t="inlineStr">
+        <is>
+          <t>Project Hail Mary,The Odyssey</t>
+        </is>
+      </c>
+      <c r="L337" s="15" t="inlineStr">
+        <is>
+          <t>興行,海外,トレンド</t>
+        </is>
+      </c>
+      <c r="M337" s="15" t="inlineStr"/>
+    </row>
+    <row r="338">
+      <c r="A338" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B338" s="15" t="inlineStr">
+        <is>
+          <t>映画</t>
+        </is>
+      </c>
+      <c r="C338" s="15" t="inlineStr">
+        <is>
+          <t>26年上半期の国内興収は10億円超22作品・洋画が健闘——『名探偵コナン』が邦画初の4作連続100億円</t>
+        </is>
+      </c>
+      <c r="D338" s="15" t="inlineStr">
+        <is>
+          <t>https://eiga.com/news/20260718/5</t>
+        </is>
+      </c>
+      <c r="E338" s="15" t="inlineStr">
+        <is>
+          <t>国内興行は邦画アニメ主導の構図が続いてきたが、2026年上半期はハリウッド大作の供給回復とファミリー向け続編の集中で洋画の存在感が戻った。一方で邦画側は特定シリーズへの依存度が高まっている。</t>
+        </is>
+      </c>
+      <c r="F338" s="15" t="inlineStr">
+        <is>
+          <t>2026年上半期の国内映画は22作品が興収10億円を突破。内訳は洋画9本・邦画13本だが、30億円超は洋画5本に対し邦画3本と上位帯では洋画が優勢。『ズートピア2』157.4億円が首位で、『名探偵コナン ハイウェイの堕天使』は135.7億円と邦画史上初の4作連続100億円超を達成した。</t>
+        </is>
+      </c>
+      <c r="G338" s="15" t="inlineStr">
+        <is>
+          <t>本数は邦画優位だが高興収帯は洋画優位という逆転構造
+コナンの4作連続100億はシリーズ運営の再現性の高さを示す
+上位はファミリー・アニメ・続編に極度に集中
+洋画復調は供給本数の回復と表裏一体</t>
+        </is>
+      </c>
+      <c r="H338" s="15" t="inlineStr">
+        <is>
+          <t>洋画の供給回復が続く下期は、邦画側が上位帯を守るためシリーズ大作の公開時期を分散させる調整に入る。年間ベースでは邦画の本数優位・洋画の金額優位という構図が定着し、中規模邦画の劇場枠がさらに圧迫される。</t>
+        </is>
+      </c>
+      <c r="I338" s="15" t="inlineStr">
+        <is>
+          <t>国内興行の作品数分布と高興収帯の集中度</t>
+        </is>
+      </c>
+      <c r="J338" s="15" t="inlineStr">
+        <is>
+          <t>東宝,ディズニー,ワーナー・ブラザース,キノフィルムズ</t>
+        </is>
+      </c>
+      <c r="K338" s="15" t="inlineStr">
+        <is>
+          <t>名探偵コナン,ズートピア2,Michael マイケル</t>
+        </is>
+      </c>
+      <c r="L338" s="15" t="inlineStr">
+        <is>
+          <t>興行,国内,チャート・ランキング</t>
+        </is>
+      </c>
+      <c r="M338" s="15" t="inlineStr"/>
+    </row>
+    <row r="339">
+      <c r="A339" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B339" s="15" t="inlineStr">
+        <is>
+          <t>映画</t>
+        </is>
+      </c>
+      <c r="C339" s="15" t="inlineStr">
+        <is>
+          <t>『Project Hail Mary』が劇場105日ウィンドウを経てPrime Video配信——世界興収6.83億ドルの後の窓口設計</t>
+        </is>
+      </c>
+      <c r="D339" s="15" t="inlineStr">
+        <is>
+          <t>https://variety.com/lists/best-movies-streaming-july-2026/</t>
+        </is>
+      </c>
+      <c r="E339" s="15" t="inlineStr">
+        <is>
+          <t>コロナ期に17〜45日まで短縮された劇場専有ウィンドウは、劇場興行の回復に伴い再び長期化する傾向にある。自社配信を持つスタジオほど「自社プラットフォームへ早く落とす」誘因と「劇場で稼ぎ切る」誘因の板挟みにあった。</t>
+        </is>
+      </c>
+      <c r="F339" s="15" t="inlineStr">
+        <is>
+          <t>2026年最大級のヒットとなったAmazon MGM『Project Hail Mary』（世界興収6.83億ドル）が、105日の劇場ウィンドウを経てPrime Videoで配信開始。同月はディズニー『プラダを着た悪魔2』（世界6.78億ドル）もDisney+／Huluへ、『Super Mario Galaxy Movie』はPeacockへ移行した。</t>
+        </is>
+      </c>
+      <c r="G339" s="15" t="inlineStr">
+        <is>
+          <t>配信を持つスタジオが自ら105日という長期ウィンドウを選択
+劇場で稼ぎ切ってから配信という順序が再び標準化
+配信は初動獲得ではなく既存ヒットの回収チャネルへ役割変化
+窓口日数が作品ごとの交渉変数として運用されている</t>
+        </is>
+      </c>
+      <c r="H339" s="15" t="inlineStr">
+        <is>
+          <t>配信事業者自身が長期ウィンドウを選ぶ動きが定着すれば、配信は「話題を作る場所」から「話題を刈り取る場所」へ役割が固定化する。結果として配信オリジナル大作の予算は絞られ、劇場公開前提の制作に投資が戻る流れが強まる。</t>
+        </is>
+      </c>
+      <c r="I339" s="15" t="inlineStr">
+        <is>
+          <t>劇場ウィンドウ日数の推移と配信の収益回収モデル</t>
+        </is>
+      </c>
+      <c r="J339" s="15" t="inlineStr">
+        <is>
+          <t>Amazon MGM Studios,ディズニー,ユニバーサル,Peacock</t>
+        </is>
+      </c>
+      <c r="K339" s="15" t="inlineStr">
+        <is>
+          <t>Project Hail Mary,プラダを着た悪魔2,Super Mario Galaxy Movie</t>
+        </is>
+      </c>
+      <c r="L339" s="15" t="inlineStr">
+        <is>
+          <t>配信,興行,海外,消費者インサイト</t>
+        </is>
+      </c>
+      <c r="M339" s="15" t="inlineStr">
+        <is>
+          <t>ミクロ×高インサイト枠：105日ウィンドウという窓口戦略の実例</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B340" s="15" t="inlineStr">
+        <is>
+          <t>アニメ</t>
+        </is>
+      </c>
+      <c r="C340" s="15" t="inlineStr">
+        <is>
+          <t>Crunchyroll創業者のNakamaがB2B権利取引所「AniBiz」始動——アニプレックス・東映など大手IPが参画</t>
+        </is>
+      </c>
+      <c r="D340" s="15" t="inlineStr">
+        <is>
+          <t>https://variety.com/2026/tv/news/crunchyroll-founder-new-anime-website-anibiz-1236800890/</t>
+        </is>
+      </c>
+      <c r="E340" s="15" t="inlineStr">
+        <is>
+          <t>アニメの海外市場は約3兆円規模へ拡大した一方、ライセンス取引は個別交渉と人的ネットワークに依存し、権利の所在確認や条件交渉に時間がかかる非効率が残っていた。配信各社の参入増で買い手側の需要は膨張している。</t>
+        </is>
+      </c>
+      <c r="F340" s="15" t="inlineStr">
+        <is>
+          <t>Crunchyroll共同創業者Kun Gao氏の新会社Nakamaが、グローバルアニメ業界向けB2Bマーケットプレイス「AniBiz.com」を開設。アニプレックス、東映など大手IPホルダーの出品を含み、ライセンス交渉を集約・可視化された環境で行える初の専門プラットフォームと位置づける。</t>
+        </is>
+      </c>
+      <c r="G340" s="15" t="inlineStr">
+        <is>
+          <t>権利取引そのものをプラットフォーム化する初の試み
+大手IPホルダーが初期から参画し流動性を確保
+買い手多様化（Netflix・AMC・Tubi・Hulu等）が前提
+取引の透明化は権利元の価格交渉力を高める方向に働く</t>
+        </is>
+      </c>
+      <c r="H340" s="15" t="inlineStr">
+        <is>
+          <t>取引が可視化されると同種作品の相場が形成され、これまで交渉力の弱かった中小制作会社・権利元の条件が改善する。一方で配信事業者は独占確保のためプラットフォーム外での先回り契約を強め、二層構造の取引市場が生まれる。</t>
+        </is>
+      </c>
+      <c r="I340" s="15" t="inlineStr">
+        <is>
+          <t>コンテンツライセンス市場のプラットフォーム化と価格発見機能</t>
+        </is>
+      </c>
+      <c r="J340" s="15" t="inlineStr">
+        <is>
+          <t>Nakama,Crunchyroll,ソニー,アニプレックス,東映アニメーション</t>
+        </is>
+      </c>
+      <c r="K340" s="15" t="inlineStr"/>
+      <c r="L340" s="15" t="inlineStr">
+        <is>
+          <t>権利・ライセンス,配信,海外</t>
+        </is>
+      </c>
+      <c r="M340" s="15" t="inlineStr">
+        <is>
+          <t>アニメ流通インフラの構造変化</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B341" s="15" t="inlineStr">
+        <is>
+          <t>アニメ</t>
+        </is>
+      </c>
+      <c r="C341" s="15" t="inlineStr">
+        <is>
+          <t>Crunchyroll、8月から公式ストアを上位サブスク限定に——物販を会員特典へ組み替え</t>
+        </is>
+      </c>
+      <c r="D341" s="15" t="inlineStr">
+        <is>
+          <t>https://www.animenewsnetwork.com/news/2026-07-14/crunchyroll-store-to-become-exclusive-to-mega-ultimate-fan-tiers-in-august/.239593</t>
+        </is>
+      </c>
+      <c r="E341" s="15" t="inlineStr">
+        <is>
+          <t>アニメ配信の会員数は成長したものの、価格競争でARPU（会員単価）の引き上げが難しい状況が続いていた。一方でアニメファンのグッズ支出は配信料金を大きく上回り、物販の粗利は配信より高い。</t>
+        </is>
+      </c>
+      <c r="F341" s="15" t="inlineStr">
+        <is>
+          <t>Crunchyrollは2026年8月より公式ストアをMega FanおよびUltimate Fanの上位ティア会員限定とし、キュレーションされた限定ドロップとCrunchyroll独占商品を中心とする構成に刷新すると発表した。</t>
+        </is>
+      </c>
+      <c r="G341" s="15" t="inlineStr">
+        <is>
+          <t>物販をオープンECから会員特典（囲い込み資産）へ転換
+配信料金の値上げではなく上位ティアへの誘導でARPUを上げる設計
+限定ドロップ化で在庫リスクを抑えつつ希少性を演出
+ライトユーザーの物販接点を意図的に切り捨てる選択</t>
+        </is>
+      </c>
+      <c r="H341" s="15" t="inlineStr">
+        <is>
+          <t>上位ティアの解約率と客単価が改善すれば、同様の「物販を上位会員特典に閉じる」設計が音楽のファンクラブD2Cやゲームのサブスクにも波及する。逆にライト層の離脱が目立てば1年以内に部分開放へ揺り戻す可能性もある。</t>
+        </is>
+      </c>
+      <c r="I341" s="15" t="inlineStr">
+        <is>
+          <t>サブスクのティア設計とARPU向上手段としての物販統合</t>
+        </is>
+      </c>
+      <c r="J341" s="15" t="inlineStr">
+        <is>
+          <t>Crunchyroll,ソニー</t>
+        </is>
+      </c>
+      <c r="K341" s="15" t="inlineStr"/>
+      <c r="L341" s="15" t="inlineStr">
+        <is>
+          <t>配信,海外,消費者インサイト</t>
+        </is>
+      </c>
+      <c r="M341" s="15" t="inlineStr">
+        <is>
+          <t>ミクロ×高インサイト枠：サブスク階層×物販の設計変更</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B342" s="15" t="inlineStr">
+        <is>
+          <t>音楽</t>
+        </is>
+      </c>
+      <c r="C342" s="15" t="inlineStr">
+        <is>
+          <t>Primary WaveによるKobalt買収が完了——約15億ドルで楽曲権利・徴収基盤amraを取得</t>
+        </is>
+      </c>
+      <c r="D342" s="15" t="inlineStr">
+        <is>
+          <t>https://www.musicbusinessworldwide.com/done-deal-primary-waves-acquisition-of-kobalt-has-closed/</t>
+        </is>
+      </c>
+      <c r="E342" s="15" t="inlineStr">
+        <is>
+          <t>ストリーミング収益の安定化で音楽著作権は債券に近い資産と見なされ、プライベートエクイティやインフラ系ファンドの資金が大量に流入。カタログ価格が高騰し、中堅の権利管理会社が単独では規模の経済を確保しにくくなっていた。</t>
+        </is>
+      </c>
+      <c r="F342" s="15" t="inlineStr">
+        <is>
+          <t>2026年7月7日、Primary Wave MusicによるKobalt買収が約15億ドルで完了。対象にはKobaltの全世界オペレーション、自社保有著作権カタログ、デジタル徴収団体amraが含まれ、権利保有と徴収インフラを一体で押さえる構図となった。</t>
+        </is>
+      </c>
+      <c r="G342" s="15" t="inlineStr">
+        <is>
+          <t>カタログ（資産）と徴収インフラ（オペレーション）の同時取得
+音楽出版のミドルレイヤーが急速に寡占化
+amra取得はロイヤリティの流れそのものを握る意味を持つ
+PEマネーが音楽権利市場の価格形成主体に</t>
+        </is>
+      </c>
+      <c r="H342" s="15" t="inlineStr">
+        <is>
+          <t>権利と徴収を垂直統合したプレイヤーが増えると、アーティスト側から見た選択肢は減り、契約条件は資本コスト（金利）に連動して硬直化する。中立的な徴収・分配を掲げる新興サービスが差別化軸として台頭する余地が生まれる。</t>
+        </is>
+      </c>
+      <c r="I342" s="15" t="inlineStr">
+        <is>
+          <t>音楽著作権のバリュエーションと徴収（コレクション）レイヤーの経済性</t>
+        </is>
+      </c>
+      <c r="J342" s="15" t="inlineStr">
+        <is>
+          <t>Primary Wave Music,Kobalt,amra</t>
+        </is>
+      </c>
+      <c r="K342" s="15" t="inlineStr"/>
+      <c r="L342" s="15" t="inlineStr">
+        <is>
+          <t>M&amp;A,海外,権利・ライセンス</t>
+        </is>
+      </c>
+      <c r="M342" s="15" t="inlineStr"/>
+    </row>
+    <row r="343">
+      <c r="A343" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B343" s="15" t="inlineStr">
+        <is>
+          <t>音楽</t>
+        </is>
+      </c>
+      <c r="C343" s="15" t="inlineStr">
+        <is>
+          <t>CVCがDistroKidの過半数株取得——配信ディストリビューション層にもPE資本が到達</t>
+        </is>
+      </c>
+      <c r="D343" s="15" t="inlineStr">
+        <is>
+          <t>https://www.musicbusinessworldwide.com/from-primary-waves-1-5bn-kobalt-takeover-to-cvcs-distrokid-deal-its-mbws-weekly-round-up/</t>
+        </is>
+      </c>
+      <c r="E343" s="15" t="inlineStr">
+        <is>
+          <t>インディーアーティストの楽曲配信を担うディストリビューターは、低価格・大量取扱いで市場シェアを握りながらも収益率が薄く、成長投資のために外部資本を必要としていた。同時に大量のリリースデータという資産価値が再評価されつつある。</t>
+        </is>
+      </c>
+      <c r="F343" s="15" t="inlineStr">
+        <is>
+          <t>CVC Capital PartnersがインディペンデントMusic配信プラットフォームDistroKidの過半数株式取得で合意。同週にはPrimary WaveのKobalt買収完了、ReservoirによるNacional Records買収も報じられ、権利・流通の両レイヤーで資本再編が同時進行している。</t>
+        </is>
+      </c>
+      <c r="G343" s="15" t="inlineStr">
+        <is>
+          <t>権利（出版）だけでなく流通（配信取次）にもPE資本が流入
+DistroKidが持つリリースデータ・アーティスト接点が資産視される
+1週間に大型3件という取引の集中度
+上流と下流の双方が同じ投資家層に握られ始めた</t>
+        </is>
+      </c>
+      <c r="H343" s="15" t="inlineStr">
+        <is>
+          <t>ディストリビューターがファンドの傘下に入ると、単なる配信取次から「有望アーティストの発掘・囲い込みの入口」への転換圧力がかかる。利用規約やデータ取扱い、優先交渉権の条項変更が今後1年内の観測ポイントになる。</t>
+        </is>
+      </c>
+      <c r="I343" s="15" t="inlineStr">
+        <is>
+          <t>音楽ディストリビューションの経済性とデータ資産の価値</t>
+        </is>
+      </c>
+      <c r="J343" s="15" t="inlineStr">
+        <is>
+          <t>CVC Capital Partners,DistroKid,Primary Wave Music,Reservoir Media</t>
+        </is>
+      </c>
+      <c r="K343" s="15" t="inlineStr"/>
+      <c r="L343" s="15" t="inlineStr">
+        <is>
+          <t>M&amp;A,海外,配信</t>
+        </is>
+      </c>
+      <c r="M343" s="15" t="inlineStr"/>
+    </row>
+    <row r="344">
+      <c r="A344" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B344" s="15" t="inlineStr">
+        <is>
+          <t>音楽</t>
+        </is>
+      </c>
+      <c r="C344" s="15" t="inlineStr">
+        <is>
+          <t>ユニバーサル、スーパーファン向けアプリEVENと提携——アーティストのD2C販売を全世界で内製化</t>
+        </is>
+      </c>
+      <c r="D344" s="15" t="inlineStr">
+        <is>
+          <t>https://www.musicbusinessworldwide.com/universal-music-strikes-deal-with-superfan-app-even-to-power-d2c-sales-for-artists-worldwide/</t>
+        </is>
+      </c>
+      <c r="E344" s="15" t="inlineStr">
+        <is>
+          <t>ストリーミングでは消費者支払額のうちプラットフォーム取り分が1999年の4%から33%へ拡大し、レーベル取り分は52%から38%へ縮小。ストリーミング外で単価の高い収益源を確保する必要性がレーベル側で高まっていた。</t>
+        </is>
+      </c>
+      <c r="F344" s="15" t="inlineStr">
+        <is>
+          <t>Universal Musicがスーパーファン向けプラットフォームEVENと提携し、所属アーティストのD2C（直販）販売を全世界で展開すると発表。ストリーミングを介さずファンから直接収益を得るチャネルをレーベル主導で標準装備する動きとなる。</t>
+        </is>
+      </c>
+      <c r="G344" s="15" t="inlineStr">
+        <is>
+          <t>ストリーミング依存からの脱却をレーベル自ら制度化
+スーパーファン（少数高単価）への課金設計が主戦場に
+プラットフォーム取り分33%を迂回する経済的動機
+D2Cはデータ（購買・ファン属性）の自社保有という副次価値も大きい</t>
+        </is>
+      </c>
+      <c r="H344" s="15" t="inlineStr">
+        <is>
+          <t>D2Cが標準装備化すると、アーティスト側の交渉材料は「ストリーミング再生数」から「直販可能なファン基盤の規模」へ移る。ストリーミング各社はこれに対抗して独自のスーパーファン課金層を設ける必要に迫られる。</t>
+        </is>
+      </c>
+      <c r="I344" s="15" t="inlineStr">
+        <is>
+          <t>音楽の収益分配構造とスーパーファン／D2Cエコノミクス</t>
+        </is>
+      </c>
+      <c r="J344" s="15" t="inlineStr">
+        <is>
+          <t>Universal Music Group,EVEN,Spotify</t>
+        </is>
+      </c>
+      <c r="K344" s="15" t="inlineStr"/>
+      <c r="L344" s="15" t="inlineStr">
+        <is>
+          <t>提携,配信,海外,消費者インサイト</t>
+        </is>
+      </c>
+      <c r="M344" s="15" t="inlineStr"/>
+    </row>
+    <row r="345">
+      <c r="A345" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B345" s="15" t="inlineStr">
+        <is>
+          <t>小説</t>
+        </is>
+      </c>
+      <c r="C345" s="15" t="inlineStr">
+        <is>
+          <t>第175回芥川賞・直木賞が決定——芥川賞に小砂川チト『ゾンビ回収婦』、直木賞に朝倉かすみ『けんぐゎい』</t>
+        </is>
+      </c>
+      <c r="D345" s="15" t="inlineStr">
+        <is>
+          <t>https://news.web.nhk/newsweb/na/na-k10015176901000</t>
+        </is>
+      </c>
+      <c r="E345" s="15" t="inlineStr">
+        <is>
+          <t>文芸市場は紙の書籍販売が縮小を続ける一方、受賞作は短期間で数万部規模の増刷がかかり、書店送客とメディアミックス企画の起点として機能してきた。出版各社にとって二大文学賞は年2回の最大級の販売イベントである。</t>
+        </is>
+      </c>
+      <c r="F345" s="15" t="inlineStr">
+        <is>
+          <t>2026年7月15日に第175回芥川龍之介賞・直木三十五賞の選考会が行われ、芥川賞は小砂川チト氏『ゾンビ回収婦』（講談社）、直木賞は朝倉かすみ氏『けんぐゎい』（光文社）が受賞した。</t>
+        </is>
+      </c>
+      <c r="G345" s="15" t="inlineStr">
+        <is>
+          <t>芥川賞は講談社、直木賞は光文社と受賞元が分散
+受賞直後の増刷・平台展開が下期の文芸売上を左右
+話題性の高い作品は映像化・オーディオ化の打診が集中
+書店送客イベントとしての文学賞の重要性は依然高い</t>
+        </is>
+      </c>
+      <c r="H345" s="15" t="inlineStr">
+        <is>
+          <t>受賞2作は数か月内に増刷を重ね、うち直木賞受賞作は映像化・舞台化の企画打診が入る可能性が高い。近年は受賞から映像化発表までのリードタイムが短縮しており、年内〜2027年前半に何らかのメディアミックス発表が出る展開を想定。</t>
+        </is>
+      </c>
+      <c r="I345" s="15" t="inlineStr">
+        <is>
+          <t>文学賞の販売波及効果と受賞作のメディアミックス転換率</t>
+        </is>
+      </c>
+      <c r="J345" s="15" t="inlineStr">
+        <is>
+          <t>講談社,光文社,日本文学振興会</t>
+        </is>
+      </c>
+      <c r="K345" s="15" t="inlineStr">
+        <is>
+          <t>ゾンビ回収婦,けんぐゎい</t>
+        </is>
+      </c>
+      <c r="L345" s="15" t="inlineStr">
+        <is>
+          <t>受賞,出版,国内</t>
+        </is>
+      </c>
+      <c r="M345" s="15" t="inlineStr">
+        <is>
+          <t>メディアミックス展開が出たら追跡シートへ</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B346" s="15" t="inlineStr">
+        <is>
+          <t>漫画</t>
+        </is>
+      </c>
+      <c r="C346" s="15" t="inlineStr">
+        <is>
+          <t>小学館集英社プロダクション26年3月期は最終益9.6%減——版権・ライセンス頼みの利益構造に頭打ち感</t>
+        </is>
+      </c>
+      <c r="D346" s="15" t="inlineStr">
+        <is>
+          <t>https://gamebiz.jp/news/428879</t>
+        </is>
+      </c>
+      <c r="E346" s="15" t="inlineStr">
+        <is>
+          <t>出版大手のグループ会社では、電子コミックの伸びが鈍化する一方、キャラクター版権とライセンス収入が利益の柱になっている。ただし国内玩具・グッズ市場は成熟しており、海外展開の進捗が業績を左右する段階に入っていた。</t>
+        </is>
+      </c>
+      <c r="F346" s="15" t="inlineStr">
+        <is>
+          <t>小学館集英社プロダクション（ShoPro）の2026年3月期決算は、最終利益が前年比9.6%減の24億1500万円。出版グループの版権・映像・ライセンス機能を担う同社の減益は、電子コミックの成長鈍化とライセンス収益の伸び悩みを映している。</t>
+        </is>
+      </c>
+      <c r="G346" s="15" t="inlineStr">
+        <is>
+          <t>電子コミックの成長が踊り場に入りつつある兆候
+利益の柱が版権・ライセンスへ移った分、市況感応度が高い
+出版本体ではなく版権子会社の数字に構造変化が出やすい
+成長軸は国内ライセンスから海外・IP展開へ移行途上</t>
+        </is>
+      </c>
+      <c r="H346" s="15" t="inlineStr">
+        <is>
+          <t>電子の踊り場が続けば、出版各社は版権子会社経由の国内ライセンスから、海外向け直接ライセンスと自社出資による映像・ゲーム化へ資源を振り向ける。版権子会社は仲介役から共同出資者への役割転換を迫られる。</t>
+        </is>
+      </c>
+      <c r="I346" s="15" t="inlineStr">
+        <is>
+          <t>出版グループの版権子会社の収益構造と電子コミック市場の成熟</t>
+        </is>
+      </c>
+      <c r="J346" s="15" t="inlineStr">
+        <is>
+          <t>小学館集英社プロダクション,小学館,集英社</t>
+        </is>
+      </c>
+      <c r="K346" s="15" t="inlineStr"/>
+      <c r="L346" s="15" t="inlineStr">
+        <is>
+          <t>業績,出版,国内</t>
+        </is>
+      </c>
+      <c r="M346" s="15" t="inlineStr"/>
+    </row>
+    <row r="347">
+      <c r="A347" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B347" s="15" t="inlineStr">
+        <is>
+          <t>横断</t>
+        </is>
+      </c>
+      <c r="C347" s="15" t="inlineStr">
+        <is>
+          <t>2025年の出版市場は1兆5462億円で4年連続減——コミックが44.8%を占め電子コミックは5122億円</t>
+        </is>
+      </c>
+      <c r="D347" s="15" t="inlineStr">
+        <is>
+          <t>https://hon.jp/news/1.0/0/58293</t>
+        </is>
+      </c>
+      <c r="E347" s="15" t="inlineStr">
+        <is>
+          <t>紙の雑誌の縮小が続く一方、電子コミックが市場を下支えする構図が定着。ただし電子コミックの成長率も鈍化しつつあり、出版市場全体では前年割れが常態化していた。</t>
+        </is>
+      </c>
+      <c r="F347" s="15" t="inlineStr">
+        <is>
+          <t>出版科学研究所によれば2025年の出版市場（紙＋電子）は1兆5462億円で前年比1.6%減、4年連続の前年割れとなった。内訳占有率はコミック44.8%、書籍39.9%、雑誌15.3%。電子出版の約90%（5122億円）を電子コミックが占め、直近5年でほぼ倍増している。</t>
+        </is>
+      </c>
+      <c r="G347" s="15" t="inlineStr">
+        <is>
+          <t>出版市場の実質的な主力商品はすでにコミック（44.8%）
+電子出版の9割が電子コミックという極端な偏り
+市場規模はコロナ前2019年とほぼ同水準まで戻った
+全体は減少でも構成比の入れ替わりが進行中</t>
+        </is>
+      </c>
+      <c r="H347" s="15" t="inlineStr">
+        <is>
+          <t>コミック依存度が45%に迫る状況では、出版社の投資は雑誌・書籍よりも作品IPの他ジャンル展開（アニメ・実写・ゲーム）へさらに傾斜する。編集部門の評価軸も部数からIP化可能性へシフトが進む。</t>
+        </is>
+      </c>
+      <c r="I347" s="15" t="inlineStr">
+        <is>
+          <t>出版市場の構成比推移と電子コミックの成熟曲線</t>
+        </is>
+      </c>
+      <c r="J347" s="15" t="inlineStr">
+        <is>
+          <t>出版科学研究所,集英社,講談社,小学館,KADOKAWA</t>
+        </is>
+      </c>
+      <c r="K347" s="15" t="inlineStr"/>
+      <c r="L347" s="15" t="inlineStr">
+        <is>
+          <t>出版,国内,トレンド</t>
+        </is>
+      </c>
+      <c r="M347" s="15" t="inlineStr">
+        <is>
+          <t>漫画・小説双方に影響するためジャンルは横断</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
monthly matrix(14cat) + future predictions (2026-07-20 13:32)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -886,7 +886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2366,6 +2366,90 @@
       <c r="H35" s="15" t="inlineStr">
         <is>
           <t>音楽</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>大手パブリッシャーが不採算内製スタジオを整理する局面で、「閉鎖」ではなく経営陣による買い戻し／MBOでの独立化が標準的な出口として定着し、独立後スタジオが外部資本・受託と組み合わせて存続する形が増える</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>3〜9ヶ月後</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Microsoft/Xbox Game Studios, Double Fine, Compulsion Games, Ninja Theory, Virtuos, Abstraction, Don't Nod, SHIFT UP, UNBOUND</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Xbox、Ninja Theory閉鎖を通告。Double Fine・Compulsionは独立化（買い戻し）を交渉と報道（6/17）／受託大手Virtuos、蘭スタジオAbstractionをMBOで分離。開発受託の再編が加速（6/20）／SHIFT UP、三上真司氏の新スタジオUNBOUNDと提携。新作を自社パブリッシングで展開へ（6/19）／「ライフ イズ ストレンジ」開発Don't Nod、Tencentが短期追加出資を見送り資金繰り難に（6/19）</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>今後6〜9ヶ月のスタジオ整理案件について「閉鎖」件数と「MBO/独立化」件数の比率を追跡。Double Fine・Compulsionの独立化が実際に成立するか、独立後スタジオの資金調達手段（受託・パブリッシャー契約・外部出資）の内訳を確認</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>ゲーム</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>eスポーツの収益基盤が「大会スポンサー広告」からソブリン資金＋メディア配信権（ストリーミング独占・ドキュメンタリー化）へ移行し、地域リーグより国際単発メガイベントへ興行が集約する</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>6〜12ヶ月後</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Esports World Cup Foundation, Amazon/Prime Video, Evo, Visa, NEOM, Savvy Games Group, Riot Games, ESL/FACEIT</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>「Esports World Cup: Level Up」シーズン2、6/26にPrime Videoで全5話一挙配信（6/19）／Evo、Visaと複数年パートナーシップ締結—越境決済とコミュニティ投資で格ゲーシーンを強化（6/28）／サウジNEOM Gaming Accelerator、過去最大サイクル始動。買収に加え育成へ投資拡大（6/20）／EWC2026のVALORANT部門、出場16チーム確定。7月パリ開催・賞金200万ドル（6/13）／世界eスポーツ視聴が月33億時間で記録更新（6/3）</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>EWC2026（7月パリ）後の配信権契約・賞金総額の開示、Prime Video等の独占配信枠の拡大有無、地域リーグ（LCK/VCT等）のスポンサー数と大会数の増減を比較。ソブリン系資金の出資比率が公表されるか確認</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>ゲーム</t>
         </is>
       </c>
     </row>
@@ -4682,73 +4766,73 @@
       </c>
       <c r="C31" s="9" t="inlineStr">
         <is>
-          <t>・任天堂Switch 2が累計1,700万台超で自社最速ベストセラー、通期目標を1,900万台へ上方修正
-・ソニーがPS5/Pro/Portalを追加値上げ、PS6は時期・価格とも未定
-・MicrosoftがXboxを8/1に最大$150値上げ(Series X $799.99)、25周年で独占回帰
-・Valve『Steam Machine』日本上陸(189,980円)</t>
+          <t>・任天堂Switch 2が累計1,700万台超〜2,000万台目前、自社史上最速。通期目標を1,900万台へ上方修正
+・ソニーがPS5/PS5 Pro/Portalを世界的に追加値上げ
+・Microsoftは8/1にXboxを最大150ドル値上げ（Series X $799.99）、AI起因のメモリ高騰が要因
+・PS6の発売時期・価格は「現時点で未定」</t>
         </is>
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>・Steam Next Fest 6月版が過去最大の約5,000本デモで閉幕
-・Steamサマーセール2026が6/25開幕(〜7/9)
-・PC Gaming Show 2026でControl続編など50本超を公開
-・『Steam Machine』日本発売でPC陣営のリビング市場攻勢</t>
+          <t>・Valve『Steam Machine』が日本・台湾・香港で販売開始（512GB 18万9,980円）、予約抽選は6月末で締切
+・Steam Next Fest 6月版が約5,000本のデモで過去最大規模、6/25にサマーセール開幕（〜7/9）
+・PC Gaming Show 2026で50本超・20本以上の世界初公開（Control続編ほか）</t>
         </is>
       </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
-          <t>・スマホ新法施行半年もiPhone外部アプリストアにゲーム主要30社の出店ゼロ
-・ポケモン対戦特化『Pokémon Champions』スマホ版を6/17配信
-・『FGO』がUnity 6へエンジン移行(約16GB再DL)
-・ByteDance系Moonton売却交渉(60〜70億ドル)</t>
+          <t>・スマホ新法施行半年、iPhone外部アプリストアへのゲーム主要30社の出店はゼロ
+・PEGI新区分で有料ルートボックスが最低16歳指定、モバイル課金設計に影響
+・『Pokémon Champions』スマホ版を6/17配信
+・『FGO』が6/22にUnity 6へエンジン移行（約16GBの再DL）</t>
         </is>
       </c>
       <c r="F31" s="9" t="inlineStr">
         <is>
-          <t>・NVIDIA『GeForce Now』がQuest 3/Vision Pro/Pico対応、XRでクラウドゲーミング拡大
-・Xbox幹部がGame Pass値上げで「数百万人」解約と認め、$22.99へ価格調整</t>
+          <t>・NVIDIA「GeForce Now」がQuest 3/S・Vision Pro・Picoに対応、XRでのクラウドゲーミングが本格化
+・Xbox幹部がGame Pass値上げで「数百万人」の解約を認め$22.99へ値下げ
+・Bungie『Destiny 2』が6/9の最終アップデート「Monument of Triumph」で開発終了、12年のGaaSに区切り</t>
         </is>
       </c>
       <c r="G31" s="9" t="inlineStr">
         <is>
-          <t>・CS2『IEM Cologne Major 2026』がピーク約70万人・賞金125万ドル
-・VALORANT Masters London 2026でLeviatánが初優勝
-・LoL『LCK Road to MSI』でT1優勝、ピーク218万人
-・EVO 2026開幕、SF6が4年連続最多2,414名</t>
+          <t>・世界eスポーツ視聴が月33億時間で記録更新、モバイルが牽引
+・CS2『IEM Cologne Major 2026』ピーク約70万人・賞金125万ドル、LoL『LCK Road to MSI』T1優勝はピーク218万人
+・VALORANT Masters LondonはLeviatánが初優勝（賞金100万ドル）
+・EvoがVisaと複数年契約、EWC『Level Up』はPrime Videoで配信</t>
         </is>
       </c>
       <c r="H31" s="9" t="inlineStr">
         <is>
-          <t>・EA 550億ドルLBO非公開化が6/30最終局面、EU審査(7/22・7/30期限)
-・Netflix×Warner Bros.($82.7B)を全額現金取引に修正しWB Games統合
-・Nexonが投資子会社『Nexon Partners』設立
-・コーエーテクモがガストを吸収合併</t>
+          <t>・EAの約550億ドルLBO非公開化が6/30期限へ大詰め（サウジPIF・Silver Lake・Affinity）、EU審査は反トラスト7/22・外国補助金7/30
+・Netflix×Warner Bros.（$82.7B）が全額現金取引へ修正、WB Gamesも統合対象
+・ByteDanceがMoontonをSavvyへ60〜70億ドルで売却交渉
+・業界M&amp;AはQ1に77億ドル到達</t>
         </is>
       </c>
       <c r="I31" s="9" t="inlineStr">
         <is>
-          <t>・PEGI新リスク区分で課金ルートボックスは最低16歳指定を6月適用
-・EU AI法が8/2全面適用へ
-・米加州『ゲーム保護法案』AB1921が下院通過
-・任天堂が仏当局にJoy-Conドリフトで約35M€の制裁金
-・英が16歳未満のオンライン制限、Robloxは年齢確認を強化</t>
+          <t>・PEGIが有料ルートボックスを最低16歳指定とする新「インタラクティブ・リスク区分」を6月適用開始
+・EU AI Actが8/2全面適用へ透明性Code of Practice最終化、中国は対話型AI暫定規則を7/15施行
+・米加州「ゲーム保護法案」AB1921が下院通過（終了時の返金義務化）
+・英政府が16歳未満のオンライン利用制限を公表
+・任天堂が仏当局とJoy-Conドリフトで約35M€の制裁金に合意</t>
         </is>
       </c>
       <c r="J31" s="9" t="inlineStr">
         <is>
-          <t>・NVIDIAが『ACE Game Agent SDK』ベータ公開、KraftonがPUBGにAI僚機を実装
-・Google Cloudが自律型AIエージェント群を本格投入
-・ゲーム生成AI市場は2026年に約22億ドル見通し
-・一方カプコン・ポケットペアは生成AIの本編不使用を表明</t>
+          <t>・NVIDIAが「ACE Game Agent SDK」ベータとUE5プラグインを公開、KraftonはPUBGにAI僚機『Ella』を実装
+・Google Cloudがゲーム開発向け自律型AIエージェント群を本格投入、DLSS 5も発表
+・一方で開発者の52%が生成AIを「業界に悪影響」と回答
+・カプコン・ポケットペアが本編への生成AI素材不採用を表明</t>
         </is>
       </c>
       <c r="K31" s="9" t="inlineStr">
         <is>
-          <t>・Microsoft/Xboxが7月に大規模レイオフ、Ninja Theory閉鎖、25周年で独占回帰
-・Take-Two『GTA6』予約開始($79.99/11-19)、FY27純予約80億ドル超予想
-・Ubisoftが年6度目の再編で複数スタジオ閉鎖・約380人削減
-・Tencent・NetEaseが海外買収を加速</t>
+          <t>・MicrosoftがFY末（6/30）前後からXbox部門で大規模削減に着手、Ninja Theory閉鎖通告・Double Fine/Compulsionは独立化（買い戻し）を交渉
+・ソニーがBungieで292名以上をレイオフ、スタジオ代表も退任
+・Ubisoftは2026年6度目の再編で2スタジオ閉鎖・約380人削減、SF拠点でも93人削減
+・Tencent/NetEaseが評価額低迷下で海外買収を加速</t>
         </is>
       </c>
       <c r="L31" s="9" t="n"/>

</xml_diff>

<commit_message>
weekly-releases(6genres) + indie + rankings update (2026-07-20 13:36)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -15738,7 +15738,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -16178,6 +16178,53 @@
         </is>
       </c>
       <c r="I13" s="9" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>キングダム（実写映画シリーズ）</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>佐藤信介</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>東宝</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>日本</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2026-07-17（5作目『魂の決戦』）</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>アクティブ</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>5作目『魂の決戦』が全国521館で公開。初日動員は前作『大将軍の帰還』（シリーズ最高80.3億円）対比124%。</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>邦画実写の最大級フランチャイズ。合従軍編の興収推移を継続追跡。</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -39939,7 +39986,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -40021,6 +40068,321 @@
       <c r="M1" s="19" t="inlineStr">
         <is>
           <t>URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>キングダム 魂の決戦</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>佐藤信介</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>東宝</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>日本</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>時代劇アクション</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>5</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>今週公開。シリーズ5作目・合従軍編。全国521館（IMAX 65／MX4D 11／4DX 61）で公開し、初日午後3時時点でシリーズ最高興収80.3億円の前作『大将軍の帰還』対比 動員124%の好スタート（東宝発表）。主題歌は米津玄師。</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>https://eiga.com/news/20260717/23/</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>オブセッション 災愛（Obsession）</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>米国</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>ホラー/スリラー</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>3</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>今週公開。ブラムハウス製作のネオ・ロマンティックホラー。</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>https://natalie.mu/eiga/news/681074</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>デッドマンズ・ワイヤー（Dead Man's Wire）</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>米国</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>スリラー</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>2</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>今週公開。</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>https://natalie.mu/eiga/news/681074</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ストレンジ・ハーベスト インランド・エンパイアの怪事件（Strange Harvest）</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>米国</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>モキュメンタリー・ホラー</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>2</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>今週公開。18年間の連続殺人事件を追うモキュメンタリー形式。</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>https://natalie.mu/eiga/news/681074</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>チルド</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>ホラー</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>2</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>今週公開。映画.com急上昇検索ワード3位と検索面での反応は良好。</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>https://natalie.mu/eiga/news/681074</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>トイ・ストーリー5（Toy Story 5）</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>ディズニー</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>米国</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>アニメーション</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>週末3日 16億8300万円／累計 50億円目前（動員337万人）</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>5</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-07-10〜07-12 国内週末興行1位（2週連続）。興行通信社／映画.com。</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>https://eiga.com/ranking/jp/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Michael マイケル（Michael）</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>キノフィルムズ</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>米国</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>伝記/音楽</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>週末3日 4億4800万円／累計 57億円突破（動員359万人）</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>4</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-07-10〜07-12 国内週末興行2位。公開5週目で累計57億円と長期ヒット。</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>https://eiga.com/ranking/jp/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>口に関するアンケート</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>松竹</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>日本</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>週末3日 1億300万円／累計 3億円（動員24万人）</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>3</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-07-10〜07-12 国内週末興行3位。</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>https://eiga.com/ranking/jp/</t>
         </is>
       </c>
     </row>
@@ -40259,7 +40621,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -40784,6 +41146,48 @@
       <c r="G16" s="9" t="inlineStr"/>
       <c r="H16" s="9" t="inlineStr"/>
       <c r="I16" s="9" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>攻殻機動隊シリーズ</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>士郎正宗</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>カンテレ・フジテレビ系／Prime Video</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2026年夏（新作TVアニメ）</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>アクティブ</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>完全新作『攻殻機動隊 THE GHOST IN THE SHELL』が2026-07-07放送開始。JINSとのコラボアイウェア等の周辺展開も進行。</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>長寿SF IPの再起動事例。海外配信での反応も追跡対象。</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -41276,7 +41680,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -41352,6 +41756,131 @@
       <c r="L1" s="20" t="inlineStr">
         <is>
           <t>URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>攻殻機動隊 THE GHOST IN THE SHELL</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>士郎正宗</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026年夏（7月期）</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Prime Video（国内最速・毎週火 23:30）／翌日より各種配信</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>SF/アクション</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>5</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>完全新作TVアニメ。カンテレ・フジテレビ系全国ネット「火アニバル!!」枠で毎週火曜23時〜。今夏の目玉枠で、JINSとのコラボアイウェア（世界限定1000本）など周辺展開も動いている。</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>https://www.theghostintheshell-anime.jp/on-air/</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-07（夏クール）</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>BLEACH 千年血戦篇-禍進譚-</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>久保帯人（集英社）</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026年夏（7月期）</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>アクション</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>4</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>長期シリーズの最終クールとして放送。2026夏アニメの中核の一つ。</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/article/202607/79761</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-07（夏クール）</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>無職転生V 〜異世界行ったら本気だす〜</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>理不尽な孫の手</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026年夏（7月期）</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>異世界ファンタジー</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>4</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>人気異世界作品の第5期。2026夏アニメの注目続編枠。</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/article/202607/79761</t>
         </is>
       </c>
     </row>
@@ -41590,7 +42119,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -42146,6 +42675,43 @@
       </c>
       <c r="H17" s="9" t="inlineStr"/>
       <c r="I17" s="9" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>薬屋のひとりごと</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>日向夏／ねこクラゲ ほか</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>スクウェア・エニックス／小学館</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>月刊ビッグガンガン／サンデーGX</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>連載中</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>オリコン週間コミック1位（2026-07-20付）。アニメ展開との相乗が継続。</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -42638,7 +43204,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -42708,6 +43274,46 @@
       <c r="K1" s="21" t="inlineStr">
         <is>
           <t>URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>薬屋のひとりごと</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>日向夏（原作）／ねこクラゲ（作画）</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>スクウェア・エニックス</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>月刊ビッグガンガン</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>オリコン週間コミックランキング 1位（2026-07-20付／集計 2026-07-06〜07-12）</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>4</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>アニメ効果が続くコミカライズの定番強者。ジャンル横断でIP露出が継続。</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>https://www.oricon.co.jp/rank/obc/w/2026-07-20/</t>
         </is>
       </c>
     </row>
@@ -42946,7 +43552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M37"/>
+  <dimension ref="A1:M48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -44698,6 +45304,501 @@
       <c r="M37" t="inlineStr">
         <is>
           <t>https://www.famitsu.com/schedule/all-platforms/202608</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Hi-Fi RUSH（ハイファイ ラッシュ）PS5パッケージ版</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Tango Gameworks</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>SUPERDELUXE GAMES</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>PS5</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>リズムアクション</t>
+        </is>
+      </c>
+      <c r="K38" t="n">
+        <v>3</v>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>今週リリース。旧Bethesda傘下Tangoのリズムアクションが国内PS5パッケージ化。DELUXE EDITIONは全DLC同梱。</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>https://prtimes.jp/main/html/rd/p/000000370.000082433.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>RATATAN（ラタタン）コンソール版</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>ratata Arts</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Game Source Entertainment</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>PS5/Switch 2</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>リズムアクション・ローグライク</t>
+        </is>
+      </c>
+      <c r="K39" t="n">
+        <v>3</v>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>今週リリース。『パタポン』スタッフによる精神的続編のコンソール版。</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>https://gamesource-ent.jp/detail/166</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>京都ザナドゥ -桜幻武-（Kyoto Xanadu）</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>日本ファルコム</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>日本ファルコム</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>PS5/Switch</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>アクションRPG</t>
+        </is>
+      </c>
+      <c r="K40" t="n">
+        <v>3</v>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>今週リリース。『東亰ザナドゥ』系譜の都市型アクションRPG新作。</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>https://www.falcom.co.jp/kyoxana/</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Fit Boxing 3 -Your パーソナルトレーナー- Nintendo Switch 2 Edition</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>イマジニア</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>イマジニア</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Switch 2</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>フィットネス</t>
+        </is>
+      </c>
+      <c r="K41" t="n">
+        <v>3</v>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>今週リリース。Switch 2の高精度カメラ・マイク対応。KENN・緑川光ら出演。</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>https://fitboxing.net/3/</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>ヒプノシスマイク -Alternative Rap Battle- 2nd period</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>アイディアファクトリー</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>アイディアファクトリー</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Switch</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>リズム/アドベンチャー</t>
+        </is>
+      </c>
+      <c r="K42" t="n">
+        <v>2</v>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>今週リリース。Switch版第2弾。1st&amp;2ndのツインパックも同時発売。</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>https://hypnosismicarb.com/switch/2nd/</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Ascend to ZERO（アセンド・トゥ・ゼロ）</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>KRAFTON</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>KRAFTON</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>PC(Steam)/Xbox Series X|S</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>アクションローグライク</t>
+        </is>
+      </c>
+      <c r="K43" t="n">
+        <v>3</v>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>今週リリース。"時間停止"を駆使するアクションローグライク。KRAFTONの中規模新規IP。</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>https://gamebiz.jp/news/429601</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>D-topia（ディートピア）</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>マルミッツゲームス</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Annapurna Interactive</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>PC/PS5/Xbox Series X|S</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>SFアドベンチャー</t>
+        </is>
+      </c>
+      <c r="K44" t="n">
+        <v>3</v>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>今週リリース。物語重視のSF ADV。Annapurnaパブリッシングの日本発タイトル。</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>https://gamebiz.jp/news/429601</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Heave Ho 2（ヒーブ・ホー2）</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Le Cartel Studio</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Devolver Digital</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Switch/Switch 2/PC(Steam)</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>パーティーアクション</t>
+        </is>
+      </c>
+      <c r="K45" t="n">
+        <v>3</v>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>今週リリース。人気ぶらぶらパーティーアクションの続編。パーティー需要で配信映え。</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>https://gamebiz.jp/news/429601</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Moss: 忘れられた秘宝（Moss: The Forgotten Treasure）</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Polyarc</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Polyarc</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>マルチプラットフォーム</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>アクションアドベンチャー</t>
+        </is>
+      </c>
+      <c r="K46" t="n">
+        <v>3</v>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>今週リリース。VR発『Moss』シリーズの新作を各PF向けに展開。</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>https://gamebiz.jp/news/429601</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>電車アタック（Train Attack）</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Game Source Entertainment</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Game Source Entertainment</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>PS5/Switch 2</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>3Dトリックアクションレース</t>
+        </is>
+      </c>
+      <c r="K47" t="n">
+        <v>2</v>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>今週リリース。電車で街を駆けるトリックアクションレース。</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>https://gamebiz.jp/news/429601</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>デジモンUP</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>バンダイナムコエンターテインメント</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>バンダイナムコエンターテインメント</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>iOS/Android</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>育成/RPG</t>
+        </is>
+      </c>
+      <c r="K48" t="n">
+        <v>3</v>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>今週リリース。デジモンIPの新作スマホアプリ。同IPは『タイムストレンジャー』とコンソール／モバイル両面展開中。</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>https://gamebiz.jp/news/429601</t>
         </is>
       </c>
     </row>
@@ -45644,7 +46745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -45714,6 +46815,106 @@
       <c r="K1" s="22" t="inlineStr">
         <is>
           <t>URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ゾンビ回収婦</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>小砂川チト</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>講談社</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>一般文芸</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>受賞</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>第175回 芥川龍之介賞</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>5</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>2026年上半期の芥川賞受賞作。奇抜な設定を通じて社会的に見えにくくされているものに触れる作品として評価。受賞は増刷・映像化打診の起点になりやすい。</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>https://ddnavi.com/article/1424741/a/</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>けんぐゎい</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>朝倉かすみ</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>光文社</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>一般文芸</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>受賞</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>第175回 直木三十五賞</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>5</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>2026年上半期の直木賞受賞作。</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>https://news.web.nhk/newsweb/na/na-k10015176901000</t>
         </is>
       </c>
     </row>
@@ -45952,7 +47153,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -46588,6 +47789,48 @@
         </is>
       </c>
       <c r="I17" s="9" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Snow Man</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>STARTO ENTERTAINMENT</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>J-POP/アイドル</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>日本</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>アクティブ</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>「Good Time」がBillboard JAPAN Hot 100で1位（2026-07-15付）。2026年上半期Hot 100でも10位。</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>国内チャートの定点観測枠。フィジカル強者のストリーミング比率変化を追う。</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -47080,7 +48323,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -47150,6 +48393,96 @@
       <c r="K1" s="23" t="inlineStr">
         <is>
           <t>URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-07-15（付）</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>チャート</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Good Time</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Snow Man</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>デジタル/フィジカル複合</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Billboard JAPAN Hot 100 1位</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>4</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>国内総合ソング・チャート首位。Snow Manは2026年上半期Hot 100でも10位に入っており、年間を通して上位に定着。</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>https://www.billboard-japan.com/charts/detail?a=hot100</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-07-18（付）</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>チャート</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Choosin' Texas</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Ella Langley（エラ・ラングレー）</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>デジタル/ストリーミング</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Billboard Hot 100（米）1位</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>13週連続で全米1位。カントリー勢の長期首位が続く構図。</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>https://www.billboard.com/charts/hot-100/</t>
         </is>
       </c>
     </row>
@@ -47388,7 +48721,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -47458,6 +48791,58 @@
       <c r="K1" s="24" t="inlineStr">
         <is>
           <t>メモ</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>虎鶫 とらつぐみ －TSUGUMI PROJECT－</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>漫画</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>ippatu／講談社</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>アニメ</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>TVアニメ化決定。ティザービジュアル＆PV公開。</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>発表済み</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>講談社</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>フランスで先行刊行され日本に逆輸入されたコミックのアニメ化。海外発→国内還流という珍しい経路。</t>
         </is>
       </c>
     </row>
@@ -51825,7 +53210,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -52450,6 +53835,100 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>わびさび寿司ダービー</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>講談社ゲームラボ</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2026-07-15 配信</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>PC(Steam)/Switch</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>育成×レース</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>寿司×育成×レースという掛け合わせの企画勝負型インディー。出版社（講談社）のインディーレーベルによる小規模タイトルで、コンセプトの奇抜さでSNS言及が増加。</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>配信直後のため公式実績値は未公表・要追跡。</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>出版社系インディーレーベルの実験枠。企画一発芸型の系譜。</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>秋月の茶屋から始まる物語</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>MARGINE</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2026-07-15 販売開始</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>リアル/デジタル混成（第四境界ショップ）</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>古都探索ミステリーARG</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>実在する日本の城下町（秋月）を舞台にしたARG。現地体験と謎解きを組み合わせる形式で、聖地巡礼・地域connect文脈と接続する。</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Steam等の通常配信ではないため同接・レビュー指標は非該当。</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>ゲーム×地域観光のクロスオーバー事例として追跡価値あり。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
weekly-companies(6genres) + works watch update (2026-07-20 13:38)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -16077,15 +16077,27 @@
           <t>米国</t>
         </is>
       </c>
-      <c r="E2" s="9" t="inlineStr"/>
+      <c r="E2" s="9" t="inlineStr">
+        <is>
+          <t>2026-12-18（Avengers: Doomsday）</t>
+        </is>
+      </c>
       <c r="F2" s="9" t="inlineStr">
         <is>
-          <t>アクティブ</t>
-        </is>
-      </c>
-      <c r="G2" s="9" t="inlineStr"/>
+          <t>公開待ち</t>
+        </is>
+      </c>
+      <c r="G2" s="9" t="inlineStr">
+        <is>
+          <t>『Avengers: Doomsday』が2026年12月18日に全米公開予定。ディズニーは劇場向けに4種類の予告編を用意し、『アバター：ファイアー・アンド・アッシュ』上映に合わせて1週ごとに切り替える形で順次投入している</t>
+        </is>
+      </c>
       <c r="H2" s="9" t="inlineStr"/>
-      <c r="I2" s="9" t="inlineStr"/>
+      <c r="I2" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
@@ -16201,15 +16213,27 @@
           <t>米国</t>
         </is>
       </c>
-      <c r="E6" s="9" t="inlineStr"/>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>2025-12-19（Fire and Ash）</t>
+        </is>
+      </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>アクティブ</t>
-        </is>
-      </c>
-      <c r="G6" s="9" t="inlineStr"/>
+          <t>公開済／配信待ち</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>『アバター：ファイアー・アンド・アッシュ』は2025年12月19日公開以降、世界興収14.86億ドルを記録。ただし批評は賛否が分かれた。Disney+での配信日が公表されたが劇場公開からは相応の間隔を空ける</t>
+        </is>
+      </c>
       <c r="H6" s="9" t="inlineStr"/>
-      <c r="I6" s="9" t="inlineStr"/>
+      <c r="I6" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
@@ -16328,12 +16352,20 @@
       <c r="E10" s="9" t="inlineStr"/>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t>アクティブ</t>
-        </is>
-      </c>
-      <c r="G10" s="9" t="inlineStr"/>
+          <t>次回作制作決定</t>
+        </is>
+      </c>
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>2026年4月公開の『名探偵コナン ハイウェイの堕天使』のエピローグで第30作の制作を告知。劇場版30周年記念作として2027年ゴールデンウィーク公開予定。予告にビッグ・ベンが映り、舞台はロンドン・主役は新一と蘭と見られる</t>
+        </is>
+      </c>
       <c r="H10" s="9" t="inlineStr"/>
-      <c r="I10" s="9" t="inlineStr"/>
+      <c r="I10" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
@@ -16356,19 +16388,31 @@
           <t>日本</t>
         </is>
       </c>
-      <c r="E11" s="9" t="inlineStr"/>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-17（キングダム 魂の決戦）</t>
+        </is>
+      </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t>ウォッチ</t>
-        </is>
-      </c>
-      <c r="G11" s="9" t="inlineStr"/>
+          <t>公開中</t>
+        </is>
+      </c>
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>実写『キングダム』第5作『キングダム 魂の決戦』（合従軍編／主演・山﨑賢人／配給ソニー・ピクチャーズ）が7/17公開。シリーズ累計は動員1,734万人・興行収入245億円を突破。主題歌は米津玄師の新曲「夜鷹」（7/13配信）</t>
+        </is>
+      </c>
       <c r="H11" s="9" t="inlineStr">
         <is>
           <t>各年の実写邦画ヒット作を追跡</t>
         </is>
       </c>
-      <c r="I11" s="9" t="inlineStr"/>
+      <c r="I11" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
@@ -16394,12 +16438,20 @@
       <c r="E12" s="9" t="inlineStr"/>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>アクティブ</t>
-        </is>
-      </c>
-      <c r="G12" s="9" t="inlineStr"/>
+          <t>新作長編は未発表</t>
+        </is>
+      </c>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>次回長編の公開時期は未確定。新作短編アニメーション『魔女の谷の夜』を2026年7月8日からジブリパーク「ジブリの大倉庫」で上映開始。北米では「スタジオジブリ・フェスト2026」として7作品を劇場上映</t>
+        </is>
+      </c>
       <c r="H12" s="9" t="inlineStr"/>
-      <c r="I12" s="9" t="inlineStr"/>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
@@ -16589,16 +16641,36 @@
         </is>
       </c>
       <c r="E2" s="9" t="inlineStr"/>
-      <c r="F2" s="9" t="inlineStr"/>
+      <c r="F2" s="9" t="inlineStr">
+        <is>
+          <t>FY2026 Q2: 売上251.7億ドル / 調整後EPS $1.57（市場予想上回る）。ストリーミング部門営業利益は前年同期比+88%、営業利益率11%を初達成</t>
+        </is>
+      </c>
       <c r="G2" s="9" t="inlineStr">
         <is>
           <t>MCU/SW/ピクサー/Disney+</t>
         </is>
       </c>
-      <c r="H2" s="9" t="inlineStr"/>
-      <c r="I2" s="9" t="inlineStr"/>
-      <c r="J2" s="9" t="inlineStr"/>
-      <c r="K2" s="9" t="inlineStr"/>
+      <c r="H2" s="9" t="inlineStr">
+        <is>
+          <t>Disney+の黒字化が定着し、ストリーミングが利益貢献フェーズへ。テーマパーク・グッズとのIP循環が引き続き強固</t>
+        </is>
+      </c>
+      <c r="I2" s="9" t="inlineStr">
+        <is>
+          <t>リニアTV事業の構造的縮小。MCUの新規タイトル当たり収益が過去ピークから低下</t>
+        </is>
+      </c>
+      <c r="J2" s="9" t="inlineStr">
+        <is>
+          <t>ストリーミング営業利益率をどこまで引き上げられるか。スポーツ配信（ESPN単独）の立ち上がり</t>
+        </is>
+      </c>
+      <c r="K2" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
@@ -16622,16 +16694,36 @@
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr"/>
-      <c r="F3" s="9" t="inlineStr"/>
+      <c r="F3" s="9" t="inlineStr">
+        <is>
+          <t>7/13、カリフォルニア州など12州がParamount Skydanceとの1,100億ドル規模の合併差止を求め反トラスト訴訟を提起。全米脚本家組合(WGA)も別途提訴。DOJ反トラスト局は既に承認済みでEU審査待ち</t>
+        </is>
+      </c>
       <c r="G3" s="9" t="inlineStr">
         <is>
           <t>DC/HBO Max/ハリポタ</t>
         </is>
       </c>
-      <c r="H3" s="9" t="inlineStr"/>
-      <c r="I3" s="9" t="inlineStr"/>
-      <c r="J3" s="9" t="inlineStr"/>
-      <c r="K3" s="9" t="inlineStr"/>
+      <c r="H3" s="9" t="inlineStr">
+        <is>
+          <t>合併が成立すれば映画・配信で規模の経済。DC/HBO/ハリポタのIP価値は健在</t>
+        </is>
+      </c>
+      <c r="I3" s="9" t="inlineStr">
+        <is>
+          <t>12州＋WGAの訴訟でクロージング遅延リスク。仮処分が出れば最大14日×2回のディール停止。業績自体も減収・損失見通し</t>
+        </is>
+      </c>
+      <c r="J3" s="9" t="inlineStr">
+        <is>
+          <t>9月末クロージング目標を守れるか。EU当局の判断と、州レベル訴訟の仮処分の可否</t>
+        </is>
+      </c>
+      <c r="K3" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
@@ -16655,16 +16747,36 @@
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr"/>
-      <c r="F4" s="9" t="inlineStr"/>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>WBD買収（約1,100億ドル）を推進中。7/14時点で「訴訟にかかわらず9月末までのクロージングを目指す」と表明。反トラスト訴訟をParamount+既存加入者訴訟と併合することに同意</t>
+        </is>
+      </c>
       <c r="G4" s="9" t="inlineStr">
         <is>
           <t>MI/Paramount+</t>
         </is>
       </c>
-      <c r="H4" s="9" t="inlineStr"/>
-      <c r="I4" s="9" t="inlineStr"/>
-      <c r="J4" s="9" t="inlineStr"/>
-      <c r="K4" s="9" t="inlineStr"/>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>DOJ承認済み。統合が実現すれば配信規模で Netflix に次ぐ位置へ</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>12州＋WGAの提訴により法務コストとスケジュールの不確実性が拡大</t>
+        </is>
+      </c>
+      <c r="J4" s="9" t="inlineStr">
+        <is>
+          <t>EU承認の取得時期。統合後のParamount+とHBO Maxのブランド統廃合方針</t>
+        </is>
+      </c>
+      <c r="K4" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -16688,16 +16800,36 @@
         </is>
       </c>
       <c r="E5" s="9" t="inlineStr"/>
-      <c r="F5" s="9" t="inlineStr"/>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>今週は目立った適時開示なし。映画部門は夏興行シーズンで推移</t>
+        </is>
+      </c>
       <c r="G5" s="9" t="inlineStr">
         <is>
           <t>ジュラシック/怪盗グルー/Peacock</t>
         </is>
       </c>
-      <c r="H5" s="9" t="inlineStr"/>
-      <c r="I5" s="9" t="inlineStr"/>
-      <c r="J5" s="9" t="inlineStr"/>
-      <c r="K5" s="9" t="inlineStr"/>
+      <c r="H5" s="9" t="inlineStr">
+        <is>
+          <t>テーマパーク（エピック・ユニバース）と映画IPの連動。ケーブル依存を配信・パークで補完</t>
+        </is>
+      </c>
+      <c r="I5" s="9" t="inlineStr">
+        <is>
+          <t>ブロードバンド加入者の伸び悩みが全社バリュエーションの重石</t>
+        </is>
+      </c>
+      <c r="J5" s="9" t="inlineStr">
+        <is>
+          <t>Peacockの黒字化時期。ジュラシック/怪盗グルー等のIPローテーション</t>
+        </is>
+      </c>
+      <c r="K5" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
@@ -16721,16 +16853,36 @@
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr"/>
-      <c r="F6" s="9" t="inlineStr"/>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>7/16にQ2 2026決算。売上+16%、FCFはほぼ倍増も、Q3見通し（+12%）とガイダンスが失望を呼び株価下落。通期売上見通しを510〜514億ドルに狭める。広告付きプランは提供国での新規登録の6割超を占め、広告MAUは全世界2.5億超</t>
+        </is>
+      </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
           <t>オリジナル作品全般</t>
         </is>
       </c>
-      <c r="H6" s="9" t="inlineStr"/>
-      <c r="I6" s="9" t="inlineStr"/>
-      <c r="J6" s="9" t="inlineStr"/>
-      <c r="K6" s="9" t="inlineStr"/>
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>広告事業が新規獲得の主導ドライバーに成長。FCF創出力が大幅改善</t>
+        </is>
+      </c>
+      <c r="I6" s="9" t="inlineStr">
+        <is>
+          <t>2026年の株価は年初来約-20%。成長率鈍化と「What We Watched」レポートの年1回化（2027年〜）で開示後退との受け止め</t>
+        </is>
+      </c>
+      <c r="J6" s="9" t="inlineStr">
+        <is>
+          <t>広告ARPUの引き上げ。ライブ/スポーツ枠の拡張と、値上げ耐性</t>
+        </is>
+      </c>
+      <c r="K6" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
@@ -16754,16 +16906,36 @@
         </is>
       </c>
       <c r="E7" s="9" t="inlineStr"/>
-      <c r="F7" s="9" t="inlineStr"/>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>今週は映像部門固有の適時開示なし。Prime Videoは広告付き配信とライブスポーツを継続拡大</t>
+        </is>
+      </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
           <t>007/Prime Video</t>
         </is>
       </c>
-      <c r="H7" s="9" t="inlineStr"/>
-      <c r="I7" s="9" t="inlineStr"/>
-      <c r="J7" s="9" t="inlineStr"/>
-      <c r="K7" s="9" t="inlineStr"/>
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>Prime会員基盤との抱き合わせで解約率が構造的に低い。アニメでもヴィンランド・サガ等の独占権を保有</t>
+        </is>
+      </c>
+      <c r="I7" s="9" t="inlineStr">
+        <is>
+          <t>映像単体の採算開示が乏しく、投資家からは評価しづらい</t>
+        </is>
+      </c>
+      <c r="J7" s="9" t="inlineStr">
+        <is>
+          <t>ライブスポーツ権の追加取得。MGM IPの再稼働ペース</t>
+        </is>
+      </c>
+      <c r="K7" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
@@ -16787,16 +16959,36 @@
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr"/>
-      <c r="F8" s="9" t="inlineStr"/>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>今週は映像部門固有の適時開示なし</t>
+        </is>
+      </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
           <t>Apple TV+オリジナル</t>
         </is>
       </c>
-      <c r="H8" s="9" t="inlineStr"/>
-      <c r="I8" s="9" t="inlineStr"/>
-      <c r="J8" s="9" t="inlineStr"/>
-      <c r="K8" s="9" t="inlineStr"/>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>作品単価の高い プレステージ路線でブランド価値を確立</t>
+        </is>
+      </c>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>加入者規模は主要配信の中で最小クラス。コンテンツ投資の回収が見えにくい</t>
+        </is>
+      </c>
+      <c r="J8" s="9" t="inlineStr">
+        <is>
+          <t>スポーツ権（MLS等）の収益化と、ハード連動のバンドル戦略</t>
+        </is>
+      </c>
+      <c r="K8" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
@@ -16820,16 +17012,36 @@
         </is>
       </c>
       <c r="E9" s="9" t="inlineStr"/>
-      <c r="F9" s="9" t="inlineStr"/>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>今週は目立った適時開示なし</t>
+        </is>
+      </c>
       <c r="G9" s="9" t="inlineStr">
         <is>
           <t>ジョン・ウィック/ハンガーゲーム</t>
         </is>
       </c>
-      <c r="H9" s="9" t="inlineStr"/>
-      <c r="I9" s="9" t="inlineStr"/>
-      <c r="J9" s="9" t="inlineStr"/>
-      <c r="K9" s="9" t="inlineStr"/>
+      <c r="H9" s="9" t="inlineStr">
+        <is>
+          <t>ハンガー・ゲーム等のフランチャイズ再稼働。スタジオ単体としてM&amp;A対象になりやすい</t>
+        </is>
+      </c>
+      <c r="I9" s="9" t="inlineStr">
+        <is>
+          <t>大手比で資本力が劣り、ヒットの当たり外れが業績に直結</t>
+        </is>
+      </c>
+      <c r="J9" s="9" t="inlineStr">
+        <is>
+          <t>業界再編（Paramount-WBD後）における自社のポジション取り</t>
+        </is>
+      </c>
+      <c r="K9" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
@@ -16852,17 +17064,41 @@
           <t>スタジオ/配給/興行</t>
         </is>
       </c>
-      <c r="E10" s="9" t="inlineStr"/>
-      <c r="F10" s="9" t="inlineStr"/>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>—（株価1,330円前後で推移、7/15に決算発表）</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>2026年2月期は映画・演劇・不動産の3本柱が堅調。2025暦年の国内グループ興収は1,605億円と過去最高圏。7/15に四半期決算を発表</t>
+        </is>
+      </c>
       <c r="G10" s="9" t="inlineStr">
         <is>
           <t>ゴジラ/コナン/ジブリ配給</t>
         </is>
       </c>
-      <c r="H10" s="9" t="inlineStr"/>
-      <c r="I10" s="9" t="inlineStr"/>
-      <c r="J10" s="9" t="inlineStr"/>
-      <c r="K10" s="9" t="inlineStr"/>
+      <c r="H10" s="9" t="inlineStr">
+        <is>
+          <t>アニメ映画の配給シェアが高く、ヒット時の利益レバレッジが大きい。不動産部門が安定収益源</t>
+        </is>
+      </c>
+      <c r="I10" s="9" t="inlineStr">
+        <is>
+          <t>大型アニメ作品の有無で年度業績の振れ幅が大きい</t>
+        </is>
+      </c>
+      <c r="J10" s="9" t="inlineStr">
+        <is>
+          <t>夏〜年末の配給ラインナップ。TOHO animation STUDIO の自社製作比率引き上げ</t>
+        </is>
+      </c>
+      <c r="K10" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
@@ -16885,17 +17121,41 @@
           <t>スタジオ/配給</t>
         </is>
       </c>
-      <c r="E11" s="9" t="inlineStr"/>
-      <c r="F11" s="9" t="inlineStr"/>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>約4,283億円（2026/7/9時点）</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>配当利回り3.47%、発行済株式数7,384万株（2026/7/9時点）。映像制作・特撮・アニメ（東映アニメ連結）が収益の柱</t>
+        </is>
+      </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
           <t>戦隊/仮面ライダー/ワンピース</t>
         </is>
       </c>
-      <c r="H11" s="9" t="inlineStr"/>
-      <c r="I11" s="9" t="inlineStr"/>
-      <c r="J11" s="9" t="inlineStr"/>
-      <c r="K11" s="9" t="inlineStr"/>
+      <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t>東映アニメーションの持分と自社特撮IPの二段構え。ライブラリ収入が安定</t>
+        </is>
+      </c>
+      <c r="I11" s="9" t="inlineStr">
+        <is>
+          <t>劇場興行部門は邦画ヒットへの依存度が高い</t>
+        </is>
+      </c>
+      <c r="J11" s="9" t="inlineStr">
+        <is>
+          <t>特撮IPの海外展開。東映アニメの業績が連結に与えるインパクト</t>
+        </is>
+      </c>
+      <c r="K11" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
@@ -16919,16 +17179,36 @@
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr"/>
-      <c r="F12" s="9" t="inlineStr"/>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>2026年2月期は経常利益63.4億円と前期の25億円の赤字から黒字転換（4/14発表）。ただし2027年2月期の会社計画は経常利益35億円と-44.8%の減益見通し</t>
+        </is>
+      </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
           <t>寅さん/歌舞伎</t>
         </is>
       </c>
-      <c r="H12" s="9" t="inlineStr"/>
-      <c r="I12" s="9" t="inlineStr"/>
-      <c r="J12" s="9" t="inlineStr"/>
-      <c r="K12" s="9" t="inlineStr"/>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>不動産部門（歌舞伎座タワー等）の安定収益。歌舞伎という代替不能なコンテンツ資産</t>
+        </is>
+      </c>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>映像・興行部門の収益力が3社中最も弱く、会社計画も減益。ガンダム配給が東宝に移った影響</t>
+        </is>
+      </c>
+      <c r="J12" s="9" t="inlineStr">
+        <is>
+          <t>演劇部門の稼働率回復。映像部門の赤字体質からの脱却</t>
+        </is>
+      </c>
+      <c r="K12" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
@@ -16952,16 +17232,36 @@
         </is>
       </c>
       <c r="E13" s="9" t="inlineStr"/>
-      <c r="F13" s="9" t="inlineStr"/>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>7/17より大型電子書籍フェア「カドサマー2026」を開始（37ストア、220作品の1巻無料）。映像・出版・ゲームの一体運営を継続</t>
+        </is>
+      </c>
       <c r="G13" s="9" t="inlineStr">
         <is>
           <t>角川映画/アニメ製作</t>
         </is>
       </c>
-      <c r="H13" s="9" t="inlineStr"/>
-      <c r="I13" s="9" t="inlineStr"/>
-      <c r="J13" s="9" t="inlineStr"/>
-      <c r="K13" s="9" t="inlineStr"/>
+      <c r="H13" s="9" t="inlineStr">
+        <is>
+          <t>出版→アニメ→ゲームの自社完結型メディアミックス。ソニーとの資本業務提携による海外展開の後押し</t>
+        </is>
+      </c>
+      <c r="I13" s="9" t="inlineStr">
+        <is>
+          <t>映像制作の固定費が重く、話題作が出ない期は利益率が落ちる</t>
+        </is>
+      </c>
+      <c r="J13" s="9" t="inlineStr">
+        <is>
+          <t>アニメ製作本数の最適化と、海外配信プラットフォームとの取引条件</t>
+        </is>
+      </c>
+      <c r="K13" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
@@ -16985,16 +17285,36 @@
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr"/>
-      <c r="F14" s="9" t="inlineStr"/>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>非上場（イオン傘下）。国内シネコン最大手として夏興行に対応</t>
+        </is>
+      </c>
       <c r="G14" s="9" t="inlineStr">
         <is>
           <t>イオンシネマ</t>
         </is>
       </c>
-      <c r="H14" s="9" t="inlineStr"/>
-      <c r="I14" s="9" t="inlineStr"/>
-      <c r="J14" s="9" t="inlineStr"/>
-      <c r="K14" s="9" t="inlineStr"/>
+      <c r="H14" s="9" t="inlineStr">
+        <is>
+          <t>全国モール併設で集客基盤が安定。プレミアムシートなど単価向上策</t>
+        </is>
+      </c>
+      <c r="I14" s="9" t="inlineStr">
+        <is>
+          <t>配信シフトによる年間動員の構造的伸び悩み</t>
+        </is>
+      </c>
+      <c r="J14" s="9" t="inlineStr">
+        <is>
+          <t>大作の公開スケジュール分散と、体験型上映（IMAX/4DX）比率</t>
+        </is>
+      </c>
+      <c r="K14" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
@@ -17018,16 +17338,36 @@
         </is>
       </c>
       <c r="E15" s="9" t="inlineStr"/>
-      <c r="F15" s="9" t="inlineStr"/>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>今週は目立った適時開示なし。夏の大作シーズンで上映枠競合が続く</t>
+        </is>
+      </c>
       <c r="G15" s="9" t="inlineStr">
         <is>
           <t>IMAXフォーマット</t>
         </is>
       </c>
-      <c r="H15" s="9" t="inlineStr"/>
-      <c r="I15" s="9" t="inlineStr"/>
-      <c r="J15" s="9" t="inlineStr"/>
-      <c r="K15" s="9" t="inlineStr"/>
+      <c r="H15" s="9" t="inlineStr">
+        <is>
+          <t>大作偏重の興行構造がIMAXには追い風。中国市場の回復</t>
+        </is>
+      </c>
+      <c r="I15" s="9" t="inlineStr">
+        <is>
+          <t>スクリーン数が限られ、公開作品の質に業績が左右される</t>
+        </is>
+      </c>
+      <c r="J15" s="9" t="inlineStr">
+        <is>
+          <t>2026年後半の大作ラインナップの IMAX枠獲得状況</t>
+        </is>
+      </c>
+      <c r="K15" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -40989,12 +41329,20 @@
       <c r="E2" s="9" t="inlineStr"/>
       <c r="F2" s="9" t="inlineStr">
         <is>
-          <t>アクティブ</t>
-        </is>
-      </c>
-      <c r="G2" s="9" t="inlineStr"/>
+          <t>劇場版三部作 進行中</t>
+        </is>
+      </c>
+      <c r="G2" s="9" t="inlineStr">
+        <is>
+          <t>『劇場版「鬼滅の刃」無限城編 第一章 猗窩座再来』のBlu-ray&amp;DVDが2026年7月29日に発売予定。第二章以降の劇場公開が控え、アニプレックス／ufotable体制で継続</t>
+        </is>
+      </c>
       <c r="H2" s="9" t="inlineStr"/>
-      <c r="I2" s="9" t="inlineStr"/>
+      <c r="I2" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
@@ -41020,12 +41368,20 @@
       <c r="E3" s="9" t="inlineStr"/>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>アクティブ</t>
-        </is>
-      </c>
-      <c r="G3" s="9" t="inlineStr"/>
+          <t>第3期 放送中</t>
+        </is>
+      </c>
+      <c r="G3" s="9" t="inlineStr">
+        <is>
+          <t>第3期「死滅回游 前編」が放送中で、ABEMA等で配信。制作はMAPPA。後編の制作進行が次の焦点</t>
+        </is>
+      </c>
       <c r="H3" s="9" t="inlineStr"/>
-      <c r="I3" s="9" t="inlineStr"/>
+      <c r="I3" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
@@ -41268,12 +41624,20 @@
       <c r="E11" s="9" t="inlineStr"/>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t>アクティブ</t>
-        </is>
-      </c>
-      <c r="G11" s="9" t="inlineStr"/>
+          <t>継続展開</t>
+        </is>
+      </c>
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>制作のMAPPAがNetflixと戦略的パートナーシップを締結したと報じられ、今後のシリーズ配信窓口に影響する可能性。Crunchyrollにとっては大きな脅威との評価</t>
+        </is>
+      </c>
       <c r="H11" s="9" t="inlineStr"/>
-      <c r="I11" s="9" t="inlineStr"/>
+      <c r="I11" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
@@ -41578,16 +41942,36 @@
         </is>
       </c>
       <c r="E2" s="9" t="inlineStr"/>
-      <c r="F2" s="9" t="inlineStr"/>
+      <c r="F2" s="9" t="inlineStr">
+        <is>
+          <t>7/31に2027年3月期第1四半期決算を発表予定。会社計画は売上高1,000億円・営業利益250億円（戦略投資前270億円）・経常利益256億円・純利益181億円。主力作品の新作映像展開と二次利用活性化を収益拡大の柱に据える</t>
+        </is>
+      </c>
       <c r="G2" s="9" t="inlineStr">
         <is>
           <t>ONE PIECE/ドラゴンボール/プリキュア</t>
         </is>
       </c>
-      <c r="H2" s="9" t="inlineStr"/>
-      <c r="I2" s="9" t="inlineStr"/>
-      <c r="J2" s="9" t="inlineStr"/>
-      <c r="K2" s="9" t="inlineStr"/>
+      <c r="H2" s="9" t="inlineStr">
+        <is>
+          <t>ONE PIECE/ドラゴンボール/プリキュアの三本柱で版権収入が安定。海外二次利用の伸びしろ</t>
+        </is>
+      </c>
+      <c r="I2" s="9" t="inlineStr">
+        <is>
+          <t>制作キャパの制約。新規IPの創出ペースが版権依存構造を変えるほどではない</t>
+        </is>
+      </c>
+      <c r="J2" s="9" t="inlineStr">
+        <is>
+          <t>7/31のQ1決算での海外版権収入の進捗。ONE PIECEエルバフ編のアニメ化タイミング</t>
+        </is>
+      </c>
+      <c r="K2" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
@@ -41610,17 +41994,41 @@
           <t>制作</t>
         </is>
       </c>
-      <c r="E3" s="9" t="inlineStr"/>
-      <c r="F3" s="9" t="inlineStr"/>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>約207億円（2026/7/16時点）</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="inlineStr">
+        <is>
+          <t>2026年5月期決算を発表。7/16に株価1,025円と年初来安値を更新</t>
+        </is>
+      </c>
       <c r="G3" s="9" t="inlineStr">
         <is>
           <t>攻殻/ハイキュー/SPY×FAMILY</t>
         </is>
       </c>
-      <c r="H3" s="9" t="inlineStr"/>
-      <c r="I3" s="9" t="inlineStr"/>
-      <c r="J3" s="9" t="inlineStr"/>
-      <c r="K3" s="9" t="inlineStr"/>
+      <c r="H3" s="9" t="inlineStr">
+        <is>
+          <t>進撃の巨人/SPY×FAMILY等の制作実績で受注は安定。出版（マッグガーデン）も保有</t>
+        </is>
+      </c>
+      <c r="I3" s="9" t="inlineStr">
+        <is>
+          <t>株価は年初来安値圏。受託制作中心で利益率が低く、元請作品の有無に業績が左右される</t>
+        </is>
+      </c>
+      <c r="J3" s="9" t="inlineStr">
+        <is>
+          <t>元請・製作委員会出資比率の引き上げ。年初来安値からの反転材料の有無</t>
+        </is>
+      </c>
+      <c r="K3" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
@@ -41644,16 +42052,36 @@
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr"/>
-      <c r="F4" s="9" t="inlineStr"/>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>7/17より「カドサマー2026」開催。アニメ製作は自社レーベル原作を軸に継続</t>
+        </is>
+      </c>
       <c r="G4" s="9" t="inlineStr">
         <is>
           <t>角川アニメ全般</t>
         </is>
       </c>
-      <c r="H4" s="9" t="inlineStr"/>
-      <c r="I4" s="9" t="inlineStr"/>
-      <c r="J4" s="9" t="inlineStr"/>
-      <c r="K4" s="9" t="inlineStr"/>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>原作（ラノベ/漫画）を自社で持つため製作委員会での取り分が大きい</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>製作本数が多く、当たり外れの平準化が課題</t>
+        </is>
+      </c>
+      <c r="J4" s="9" t="inlineStr">
+        <is>
+          <t>海外配信プラットフォームとの直接取引比率</t>
+        </is>
+      </c>
+      <c r="K4" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -41677,16 +42105,36 @@
         </is>
       </c>
       <c r="E5" s="9" t="inlineStr"/>
-      <c r="F5" s="9" t="inlineStr"/>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>名探偵コナン/アンパンマン等の長寿IPで安定稼働。今週は個別開示なし</t>
+        </is>
+      </c>
       <c r="G5" s="9" t="inlineStr">
         <is>
           <t>コナン/ルパン三世</t>
         </is>
       </c>
-      <c r="H5" s="9" t="inlineStr"/>
-      <c r="I5" s="9" t="inlineStr"/>
-      <c r="J5" s="9" t="inlineStr"/>
-      <c r="K5" s="9" t="inlineStr"/>
+      <c r="H5" s="9" t="inlineStr">
+        <is>
+          <t>劇場版コナンが毎年安定した興行収入を生む収益エンジン</t>
+        </is>
+      </c>
+      <c r="I5" s="9" t="inlineStr">
+        <is>
+          <t>長寿IPへの依存度が高く、新規IPの寄与が小さい</t>
+        </is>
+      </c>
+      <c r="J5" s="9" t="inlineStr">
+        <is>
+          <t>2027年劇場版コナンの企画進捗。セガサミー本体のIP戦略との連携</t>
+        </is>
+      </c>
+      <c r="K5" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
@@ -41710,16 +42158,36 @@
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr"/>
-      <c r="F6" s="9" t="inlineStr"/>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>ガンダムシリーズの映像・立体物展開が継続。今週はアニメ部門固有の開示なし</t>
+        </is>
+      </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
           <t>ガンダム/アイドルマスター</t>
         </is>
       </c>
-      <c r="H6" s="9" t="inlineStr"/>
-      <c r="I6" s="9" t="inlineStr"/>
-      <c r="J6" s="9" t="inlineStr"/>
-      <c r="K6" s="9" t="inlineStr"/>
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>IP軸戦略でアニメ→玩具→ゲームの回収経路が確立。ガンダム劇場作品が東宝配給で好調</t>
+        </is>
+      </c>
+      <c r="I6" s="9" t="inlineStr">
+        <is>
+          <t>海外でのガンダム認知拡大が北米・欧州で道半ば</t>
+        </is>
+      </c>
+      <c r="J6" s="9" t="inlineStr">
+        <is>
+          <t>ガンダムのグローバル展開と、バンダイナムコフィルムワークスの製作本数</t>
+        </is>
+      </c>
+      <c r="K6" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
@@ -41743,16 +42211,36 @@
         </is>
       </c>
       <c r="E7" s="9" t="inlineStr"/>
-      <c r="F7" s="9" t="inlineStr"/>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>劇場版「鬼滅の刃」無限城編 第一章のBlu-ray&amp;DVDを7/29発売予定。Crunchyrollは1,500作品超・45,000話超のライブラリで専業アニメ配信最大手</t>
+        </is>
+      </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
           <t>鬼滅/Fate/Crunchyroll</t>
         </is>
       </c>
-      <c r="H7" s="9" t="inlineStr"/>
-      <c r="I7" s="9" t="inlineStr"/>
-      <c r="J7" s="9" t="inlineStr"/>
-      <c r="K7" s="9" t="inlineStr"/>
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>製作（アニプレックス）と配信（Crunchyroll）と音楽（SME）を垂直統合。鬼滅の刃の収益寄与が大きい</t>
+        </is>
+      </c>
+      <c r="I7" s="9" t="inlineStr">
+        <is>
+          <t>NetflixのMAPPA提携など、配信側の作品確保競争が激化</t>
+        </is>
+      </c>
+      <c r="J7" s="9" t="inlineStr">
+        <is>
+          <t>無限城編 第二章の公開時期。Crunchyrollの独占simulcast枠をNetflixから守れるか</t>
+        </is>
+      </c>
+      <c r="K7" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
@@ -41776,16 +42264,36 @@
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr"/>
-      <c r="F8" s="9" t="inlineStr"/>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>非上場。呪術廻戦 第3期「死滅回游 前編」が放送・配信中（ABEMA他）。Netflixとの戦略的提携が報じられ、Crunchyrollへの脅威と評されている</t>
+        </is>
+      </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
           <t>呪術廻戦/進撃/チェンソーマン</t>
         </is>
       </c>
-      <c r="H8" s="9" t="inlineStr"/>
-      <c r="I8" s="9" t="inlineStr"/>
-      <c r="J8" s="9" t="inlineStr"/>
-      <c r="K8" s="9" t="inlineStr"/>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>呪術廻戦/チェンソーマン/進撃の巨人と話題作を複数保有。配信大手との直接提携で交渉力が上昇</t>
+        </is>
+      </c>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>制作スケジュールの過密と人材負荷が継続的な論点</t>
+        </is>
+      </c>
+      <c r="J8" s="9" t="inlineStr">
+        <is>
+          <t>Netflix提携の具体的な作品ラインと独占範囲。死滅回游 後編の制作進行</t>
+        </is>
+      </c>
+      <c r="K8" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
@@ -41809,16 +42317,36 @@
         </is>
       </c>
       <c r="E9" s="9" t="inlineStr"/>
-      <c r="F9" s="9" t="inlineStr"/>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>非上場。劇場版「鬼滅の刃」無限城編 第一章のBD/DVDが7/29発売。Fateシリーズも継続</t>
+        </is>
+      </c>
       <c r="G9" s="9" t="inlineStr">
         <is>
           <t>鬼滅の刃/Fate</t>
         </is>
       </c>
-      <c r="H9" s="9" t="inlineStr"/>
-      <c r="I9" s="9" t="inlineStr"/>
-      <c r="J9" s="9" t="inlineStr"/>
-      <c r="K9" s="9" t="inlineStr"/>
+      <c r="H9" s="9" t="inlineStr">
+        <is>
+          <t>鬼滅の刃で邦画興行の最上位を占め、制作会社としては例外的な交渉力</t>
+        </is>
+      </c>
+      <c r="I9" s="9" t="inlineStr">
+        <is>
+          <t>少数精鋭ゆえに同時進行できる作品数が限られる</t>
+        </is>
+      </c>
+      <c r="J9" s="9" t="inlineStr">
+        <is>
+          <t>無限城編 第二章・第三章の制作ペース</t>
+        </is>
+      </c>
+      <c r="K9" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
@@ -41842,16 +42370,36 @@
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr"/>
-      <c r="F10" s="9" t="inlineStr"/>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>非上場。今週は目立った発表なし</t>
+        </is>
+      </c>
       <c r="G10" s="9" t="inlineStr">
         <is>
           <t>ヴァイオレット・エヴァーガーデン</t>
         </is>
       </c>
-      <c r="H10" s="9" t="inlineStr"/>
-      <c r="I10" s="9" t="inlineStr"/>
-      <c r="J10" s="9" t="inlineStr"/>
-      <c r="K10" s="9" t="inlineStr"/>
+      <c r="H10" s="9" t="inlineStr">
+        <is>
+          <t>自社原作レーベルによる一貫制作。作画品質のブランド価値</t>
+        </is>
+      </c>
+      <c r="I10" s="9" t="inlineStr">
+        <is>
+          <t>制作本数が少なく、収益規模の拡大余地が限定的</t>
+        </is>
+      </c>
+      <c r="J10" s="9" t="inlineStr">
+        <is>
+          <t>新規シリーズの立ち上げペース</t>
+        </is>
+      </c>
+      <c r="K10" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
@@ -41875,16 +42423,36 @@
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr"/>
-      <c r="F11" s="9" t="inlineStr"/>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>非上場。第83期は売上高2,043.75億円（-2.5%）、当期純利益206.17億円（+29.5%）。原作供給側としてアニメ製作委員会に深く関与</t>
+        </is>
+      </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
           <t>ジャンプ原作アニメ全般</t>
         </is>
       </c>
-      <c r="H11" s="9" t="inlineStr"/>
-      <c r="I11" s="9" t="inlineStr"/>
-      <c r="J11" s="9" t="inlineStr"/>
-      <c r="K11" s="9" t="inlineStr"/>
+      <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t>鬼滅/呪術/ONE PIECE/ダンダダン等、アニメ化される原作の供給元として最強のポジション</t>
+        </is>
+      </c>
+      <c r="I11" s="9" t="inlineStr">
+        <is>
+          <t>雑誌媒体の縮小。制作キャパ不足でアニメ化待ち作品が滞留</t>
+        </is>
+      </c>
+      <c r="J11" s="9" t="inlineStr">
+        <is>
+          <t>版権・デジタル収益への依存度が高まる中でのIP内製化の進め方</t>
+        </is>
+      </c>
+      <c r="K11" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
@@ -41908,16 +42476,36 @@
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr"/>
-      <c r="F12" s="9" t="inlineStr"/>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>MAPPAとの戦略的提携を締結し、アニメ調達を強化。Cyberpunk: Edgerunners/PLUTO/BEASTARS等の独占オリジナルを保有</t>
+        </is>
+      </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
           <t>Netflixオリジナルアニメ</t>
         </is>
       </c>
-      <c r="H12" s="9" t="inlineStr"/>
-      <c r="I12" s="9" t="inlineStr"/>
-      <c r="J12" s="9" t="inlineStr"/>
-      <c r="K12" s="9" t="inlineStr"/>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>全世界同時配信の規模で、制作会社に対して有利な条件を提示できる</t>
+        </is>
+      </c>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>専業ファンからはCrunchyrollに比べて simulcast の網羅性が劣ると見られている</t>
+        </is>
+      </c>
+      <c r="J12" s="9" t="inlineStr">
+        <is>
+          <t>MAPPA提携作品の独占範囲。日本の製作委員会に対する出資比率</t>
+        </is>
+      </c>
+      <c r="K12" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
@@ -41941,16 +42529,36 @@
         </is>
       </c>
       <c r="E13" s="9" t="inlineStr"/>
-      <c r="F13" s="9" t="inlineStr"/>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>1,500作品超・45,000話超で専業アニメ配信最大の法的ライブラリを維持。simulcastの網羅性で首位</t>
+        </is>
+      </c>
       <c r="G13" s="9" t="inlineStr">
         <is>
           <t>海外アニメ配信最大手</t>
         </is>
       </c>
-      <c r="H13" s="9" t="inlineStr"/>
-      <c r="I13" s="9" t="inlineStr"/>
-      <c r="J13" s="9" t="inlineStr"/>
-      <c r="K13" s="9" t="inlineStr"/>
+      <c r="H13" s="9" t="inlineStr">
+        <is>
+          <t>Funimation統合でライブラリが一本化され、専業では独走状態</t>
+        </is>
+      </c>
+      <c r="I13" s="9" t="inlineStr">
+        <is>
+          <t>Netflix-MAPPA提携により独占simulcast枠が侵食されるリスク</t>
+        </is>
+      </c>
+      <c r="J13" s="9" t="inlineStr">
+        <is>
+          <t>2026年秋クールの独占枠をどこまで確保できるか</t>
+        </is>
+      </c>
+      <c r="K13" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -42514,11 +43122,19 @@
       <c r="F2" s="9" t="inlineStr"/>
       <c r="G2" s="9" t="inlineStr">
         <is>
-          <t>連載中</t>
-        </is>
-      </c>
-      <c r="H2" s="9" t="inlineStr"/>
-      <c r="I2" s="9" t="inlineStr"/>
+          <t>連載中（エルバフ編）</t>
+        </is>
+      </c>
+      <c r="H2" s="9" t="inlineStr">
+        <is>
+          <t>2026年7月に連載29周年を突破。エルバフ編が佳境に入り、週刊少年ジャンプで表紙・巻頭カラーを獲得。東映アニメーションのアニメ版も継続稼働中</t>
+        </is>
+      </c>
+      <c r="I2" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
@@ -42607,11 +43223,19 @@
       <c r="F5" s="9" t="inlineStr"/>
       <c r="G5" s="9" t="inlineStr">
         <is>
-          <t>連載中</t>
-        </is>
-      </c>
-      <c r="H5" s="9" t="inlineStr"/>
-      <c r="I5" s="9" t="inlineStr"/>
+          <t>連載中（年内完結の観測）</t>
+        </is>
+      </c>
+      <c r="H5" s="9" t="inlineStr">
+        <is>
+          <t>週刊少年ジャンプで連載継続中だが、読者・分析筋の間では年内完結の可能性が高いと見られている。ジャンプは2026年に入り「逃げ上手の若君」「ひまてん！」「アオのハコ」等が相次いで完結・クライマックスを迎えており、看板の世代交代局面。7月には新連載『カノンマスター』が巻頭カラー54ページでスタート</t>
+        </is>
+      </c>
+      <c r="I5" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
@@ -43128,16 +43752,36 @@
         </is>
       </c>
       <c r="E2" s="9" t="inlineStr"/>
-      <c r="F2" s="9" t="inlineStr"/>
+      <c r="F2" s="9" t="inlineStr">
+        <is>
+          <t>非上場。第83期は売上高2,043.75億円（-2.5%）、当期純利益206.17億円（+29.5%）。週刊少年ジャンプでは7月に新連載『カノンマスター』が巻頭カラー54ページでスタート、ONE PIECEは連載29周年を突破しエルバフ編が佳境</t>
+        </is>
+      </c>
       <c r="G2" s="9" t="inlineStr">
         <is>
           <t>週刊少年ジャンプ/ジャンプ+</t>
         </is>
       </c>
-      <c r="H2" s="9" t="inlineStr"/>
-      <c r="I2" s="9" t="inlineStr"/>
-      <c r="J2" s="9" t="inlineStr"/>
-      <c r="K2" s="9" t="inlineStr"/>
+      <c r="H2" s="9" t="inlineStr">
+        <is>
+          <t>純利益200億円超の高収益体質。版権・デジタル収入が紙の減少を補って余りある</t>
+        </is>
+      </c>
+      <c r="I2" s="9" t="inlineStr">
+        <is>
+          <t>売上は微減で、成長は版権と物販への依存が強まる構造</t>
+        </is>
+      </c>
+      <c r="J2" s="9" t="inlineStr">
+        <is>
+          <t>看板作品の完結ラッシュ（逃げ若・ひま・ハコが完結済、SAKAMOTO DAYS等も年内完結の可能性）後の次世代IP育成</t>
+        </is>
+      </c>
+      <c r="K2" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
@@ -43161,16 +43805,36 @@
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr"/>
-      <c r="F3" s="9" t="inlineStr"/>
+      <c r="F3" s="9" t="inlineStr">
+        <is>
+          <t>非上場。第87期決算は当期純利益111億円、総資産3,600億円超と盤石。進撃の巨人/ブルーロック等の海外展開が寄与</t>
+        </is>
+      </c>
       <c r="G3" s="9" t="inlineStr">
         <is>
           <t>週刊少年マガジン/マガポケ</t>
         </is>
       </c>
-      <c r="H3" s="9" t="inlineStr"/>
-      <c r="I3" s="9" t="inlineStr"/>
-      <c r="J3" s="9" t="inlineStr"/>
-      <c r="K3" s="9" t="inlineStr"/>
+      <c r="H3" s="9" t="inlineStr">
+        <is>
+          <t>総合出版で雑誌・書籍・デジタルの分散が効いている。海外ライセンス収入が伸長</t>
+        </is>
+      </c>
+      <c r="I3" s="9" t="inlineStr">
+        <is>
+          <t>雑誌部門の縮小トレンドは継続</t>
+        </is>
+      </c>
+      <c r="J3" s="9" t="inlineStr">
+        <is>
+          <t>海外webtoon/縦読み市場への対応方針</t>
+        </is>
+      </c>
+      <c r="K3" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
@@ -43194,16 +43858,36 @@
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr"/>
-      <c r="F4" s="9" t="inlineStr"/>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>非上場。グループのShoProは2026年3月期の最終利益が24.15億円（-9.6%）と減益。葬送のフリーレン/名探偵コナンが主力</t>
+        </is>
+      </c>
       <c r="G4" s="9" t="inlineStr">
         <is>
           <t>週刊少年サンデー/サンデーうぇぶり</t>
         </is>
       </c>
-      <c r="H4" s="9" t="inlineStr"/>
-      <c r="I4" s="9" t="inlineStr"/>
-      <c r="J4" s="9" t="inlineStr"/>
-      <c r="K4" s="9" t="inlineStr"/>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>名探偵コナンの劇場版が毎年の安定収益源。フリーレンの海外評価が高い</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>ShoProの減益に見られるようライセンス収益の伸びが鈍化</t>
+        </is>
+      </c>
+      <c r="J4" s="9" t="inlineStr">
+        <is>
+          <t>コナン以外の映像化ヒットを作れるか</t>
+        </is>
+      </c>
+      <c r="K4" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -43227,16 +43911,36 @@
         </is>
       </c>
       <c r="E5" s="9" t="inlineStr"/>
-      <c r="F5" s="9" t="inlineStr"/>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>7/17より「カドサマー2026」を開催。37ストアで50%OFF・1巻無料、カドコミWEBで220作品の1巻を期間限定無料公開</t>
+        </is>
+      </c>
       <c r="G5" s="9" t="inlineStr">
         <is>
           <t>電撃/ComicWalker/ニコニコ</t>
         </is>
       </c>
-      <c r="H5" s="9" t="inlineStr"/>
-      <c r="I5" s="9" t="inlineStr"/>
-      <c r="J5" s="9" t="inlineStr"/>
-      <c r="K5" s="9" t="inlineStr"/>
+      <c r="H5" s="9" t="inlineStr">
+        <is>
+          <t>自社ストア（BOOK☆WALKER）と外部37ストアの二段構えで販促を打てる</t>
+        </is>
+      </c>
+      <c r="I5" s="9" t="inlineStr">
+        <is>
+          <t>大手プラットフォームへの販売依存度が高く手数料負担が重い</t>
+        </is>
+      </c>
+      <c r="J5" s="9" t="inlineStr">
+        <is>
+          <t>カドサマー2026の販促効果と、カドコミWEBの自社流通比率</t>
+        </is>
+      </c>
+      <c r="K5" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
@@ -43260,16 +43964,36 @@
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr"/>
-      <c r="F6" s="9" t="inlineStr"/>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>今週は目立った適時開示なし。電子書籍取次として国内主要ストアに配信</t>
+        </is>
+      </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
           <t>電子書籍流通</t>
         </is>
       </c>
-      <c r="H6" s="9" t="inlineStr"/>
-      <c r="I6" s="9" t="inlineStr"/>
-      <c r="J6" s="9" t="inlineStr"/>
-      <c r="K6" s="9" t="inlineStr"/>
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>国内電子書籍取次で圧倒的シェア。カドサマー等の大型フェアで流通量が増える</t>
+        </is>
+      </c>
+      <c r="I6" s="9" t="inlineStr">
+        <is>
+          <t>取次モデルゆえ利幅が薄く、出版社の直販シフトが構造的リスク</t>
+        </is>
+      </c>
+      <c r="J6" s="9" t="inlineStr">
+        <is>
+          <t>出版社の中抜きリスクへの対抗策（NFT・独自PF）</t>
+        </is>
+      </c>
+      <c r="K6" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
@@ -43293,16 +44017,36 @@
         </is>
       </c>
       <c r="E7" s="9" t="inlineStr"/>
-      <c r="F7" s="9" t="inlineStr"/>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>今週は目立った適時開示なし</t>
+        </is>
+      </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
           <t>マンガBANG!</t>
         </is>
       </c>
-      <c r="H7" s="9" t="inlineStr"/>
-      <c r="I7" s="9" t="inlineStr"/>
-      <c r="J7" s="9" t="inlineStr"/>
-      <c r="K7" s="9" t="inlineStr"/>
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>広告収益型の無料マンガアプリで一定のユーザー基盤</t>
+        </is>
+      </c>
+      <c r="I7" s="9" t="inlineStr">
+        <is>
+          <t>ピッコマ・LINEマンガ等の大手との競争が厳しく、規模の差が拡大</t>
+        </is>
+      </c>
+      <c r="J7" s="9" t="inlineStr">
+        <is>
+          <t>オリジナル作品の獲得とユーザー単価の改善</t>
+        </is>
+      </c>
+      <c r="K7" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
@@ -43326,16 +44070,36 @@
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr"/>
-      <c r="F8" s="9" t="inlineStr"/>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>今週は目立った適時開示なし。めちゃコミックはカドサマー2026の対象ストアにも参加</t>
+        </is>
+      </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
           <t>めちゃコミック</t>
         </is>
       </c>
-      <c r="H8" s="9" t="inlineStr"/>
-      <c r="I8" s="9" t="inlineStr"/>
-      <c r="J8" s="9" t="inlineStr"/>
-      <c r="K8" s="9" t="inlineStr"/>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>女性向け縦読み・TL領域で強固なポジション。課金単価が高い</t>
+        </is>
+      </c>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>国内市場が飽和し、成長には海外展開が必要</t>
+        </is>
+      </c>
+      <c r="J8" s="9" t="inlineStr">
+        <is>
+          <t>海外版めちゃコミックの立ち上がり</t>
+        </is>
+      </c>
+      <c r="K8" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
@@ -43359,16 +44123,36 @@
         </is>
       </c>
       <c r="E9" s="9" t="inlineStr"/>
-      <c r="F9" s="9" t="inlineStr"/>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>今週は目立った適時開示なし。LINEマンガはカドサマー2026の対象ストア</t>
+        </is>
+      </c>
       <c r="G9" s="9" t="inlineStr">
         <is>
           <t>LINEマンガ</t>
         </is>
       </c>
-      <c r="H9" s="9" t="inlineStr"/>
-      <c r="I9" s="9" t="inlineStr"/>
-      <c r="J9" s="9" t="inlineStr"/>
-      <c r="K9" s="9" t="inlineStr"/>
+      <c r="H9" s="9" t="inlineStr">
+        <is>
+          <t>LINEのユーザー基盤からの送客。WEBTOON陣営の一角として作品供給を受けられる</t>
+        </is>
+      </c>
+      <c r="I9" s="9" t="inlineStr">
+        <is>
+          <t>NAVER本体の webtoon 戦略に従属する面があり自由度が低い</t>
+        </is>
+      </c>
+      <c r="J9" s="9" t="inlineStr">
+        <is>
+          <t>日本オリジナルwebtoonの制作体制</t>
+        </is>
+      </c>
+      <c r="K9" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
@@ -43392,16 +44176,36 @@
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr"/>
-      <c r="F10" s="9" t="inlineStr"/>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>WEBTOON（旧Naver Webtoon）は2026年初時点で150カ国以上・月間アクティブユーザー8,900万超とグローバル首位。Naver Webtoon/Kakao Ent/Line Webtoon/Tapasの4社で2025年のグローバル収益の67.5%を占有。webtoon市場全体は2026年に144.4億ドル規模、年率33.1%成長の見通し</t>
+        </is>
+      </c>
       <c r="G10" s="9" t="inlineStr">
         <is>
           <t>WEBTOON/LINEマンガ</t>
         </is>
       </c>
-      <c r="H10" s="9" t="inlineStr"/>
-      <c r="I10" s="9" t="inlineStr"/>
-      <c r="J10" s="9" t="inlineStr"/>
-      <c r="K10" s="9" t="inlineStr"/>
+      <c r="H10" s="9" t="inlineStr">
+        <is>
+          <t>縦読み市場の世界首位。Netflix等との大型ライセンス契約で作品を「検証済みIP」として売れる</t>
+        </is>
+      </c>
+      <c r="I10" s="9" t="inlineStr">
+        <is>
+          <t>北米での収益化が広告依存で単価が低い。韓国エンタメ株全体の投資マネー流出</t>
+        </is>
+      </c>
+      <c r="J10" s="9" t="inlineStr">
+        <is>
+          <t>映像化ライセンスの単価をどこまで引き上げられるか</t>
+        </is>
+      </c>
+      <c r="K10" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
@@ -43425,16 +44229,36 @@
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr"/>
-      <c r="F11" s="9" t="inlineStr"/>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>日本でピッコマが非ゲームアプリの売上首位を維持。カカオエンタはwebtoon・web小説・音楽・ドラマ製作を1社に統合し、Kakao PageからNetflixドラマまで自社エコシステム内で完結できる体制</t>
+        </is>
+      </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
           <t>ピッコマ/カカオページ</t>
         </is>
       </c>
-      <c r="H11" s="9" t="inlineStr"/>
-      <c r="I11" s="9" t="inlineStr"/>
-      <c r="J11" s="9" t="inlineStr"/>
-      <c r="K11" s="9" t="inlineStr"/>
+      <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t>日本市場で圧倒的な課金規模。原作から映像化までの垂直統合</t>
+        </is>
+      </c>
+      <c r="I11" s="9" t="inlineStr">
+        <is>
+          <t>韓国エンタメ株全体の下落局面で資金流出。日本市場の成長率は鈍化</t>
+        </is>
+      </c>
+      <c r="J11" s="9" t="inlineStr">
+        <is>
+          <t>日本以外（北米・欧州）での第2の柱作り</t>
+        </is>
+      </c>
+      <c r="K11" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
@@ -43458,16 +44282,36 @@
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr"/>
-      <c r="F12" s="9" t="inlineStr"/>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>ゲーム本体の動向は【企業分析（国内）】参照。出版部門は鋼の錬金術師等のライブラリとガンガン系レーベルを保有</t>
+        </is>
+      </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
           <t>ガンガン/マンガUP!</t>
         </is>
       </c>
-      <c r="H12" s="9" t="inlineStr"/>
-      <c r="I12" s="9" t="inlineStr"/>
-      <c r="J12" s="9" t="inlineStr"/>
-      <c r="K12" s="9" t="inlineStr"/>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>ゲーム会社としては珍しく自社出版レーベルを持ち、コミカライズを内製できる</t>
+        </is>
+      </c>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>出版単体では規模が小さく、全社業績への寄与は限定的</t>
+        </is>
+      </c>
+      <c r="J12" s="9" t="inlineStr">
+        <is>
+          <t>ゲームIPのコミカライズ→アニメ化の循環を作れるか</t>
+        </is>
+      </c>
+      <c r="K12" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
@@ -43491,16 +44335,36 @@
         </is>
       </c>
       <c r="E13" s="9" t="inlineStr"/>
-      <c r="F13" s="9" t="inlineStr"/>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>非上場（集英社系）。今週は目立った発表なし</t>
+        </is>
+      </c>
       <c r="G13" s="9" t="inlineStr">
         <is>
           <t>花とゆめ/ヤングアニマル</t>
         </is>
       </c>
-      <c r="H13" s="9" t="inlineStr"/>
-      <c r="I13" s="9" t="inlineStr"/>
-      <c r="J13" s="9" t="inlineStr"/>
-      <c r="K13" s="9" t="inlineStr"/>
+      <c r="H13" s="9" t="inlineStr">
+        <is>
+          <t>花とゆめ/LaLa系の少女漫画で独自ポジション。長寿IPのアニメ化余地</t>
+        </is>
+      </c>
+      <c r="I13" s="9" t="inlineStr">
+        <is>
+          <t>規模が小さく、デジタル展開は親会社系の流通に依存</t>
+        </is>
+      </c>
+      <c r="J13" s="9" t="inlineStr">
+        <is>
+          <t>既存IPの再アニメ化・実写化の企画進捗</t>
+        </is>
+      </c>
+      <c r="K13" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -46257,14 +47121,26 @@
         </is>
       </c>
       <c r="E2" s="9" t="inlineStr"/>
-      <c r="F2" s="9" t="inlineStr"/>
+      <c r="F2" s="9" t="inlineStr">
+        <is>
+          <t>4,500万部超</t>
+        </is>
+      </c>
       <c r="G2" s="9" t="inlineStr">
         <is>
-          <t>刊行中</t>
-        </is>
-      </c>
-      <c r="H2" s="9" t="inlineStr"/>
-      <c r="I2" s="9" t="inlineStr"/>
+          <t>アニメ第3期・劇場版 進行中</t>
+        </is>
+      </c>
+      <c r="H2" s="9" t="inlineStr">
+        <is>
+          <t>シリーズ累計4,500万部を突破（アニメ効果で+2,100万部）。TVアニメ第3期は分割2クールで第1クールが2026年10月、第2クールが2027年4月から放送予定。2026年12月には原作者・日向夏による完全新作ストーリーの劇場版が公開予定</t>
+        </is>
+      </c>
+      <c r="I2" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
@@ -46411,15 +47287,31 @@
           <t>TOブックス</t>
         </is>
       </c>
-      <c r="E7" s="9" t="inlineStr"/>
-      <c r="F7" s="9" t="inlineStr"/>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>本編全33巻（第1部〜第5部）</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>1,300万部超</t>
+        </is>
+      </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
-          <t>完結/外伝</t>
-        </is>
-      </c>
-      <c r="H7" s="9" t="inlineStr"/>
-      <c r="I7" s="9" t="inlineStr"/>
+          <t>アニメ第3部 放送中</t>
+        </is>
+      </c>
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>シリーズ累計1,300万部を突破。アニメ第3部「領主の養女」が2026年4月から連続2クールで放送中。原作はTOブックス刊で本編全33巻の長編、メディアミックスが段階的に継続している</t>
+        </is>
+      </c>
+      <c r="I7" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
@@ -46721,16 +47613,36 @@
         </is>
       </c>
       <c r="E2" s="9" t="inlineStr"/>
-      <c r="F2" s="9" t="inlineStr"/>
+      <c r="F2" s="9" t="inlineStr">
+        <is>
+          <t>7/17より「カドサマー2026」を開催。ラノベはRe:ゼロ/SAO/オーバーロード等が継続稼働</t>
+        </is>
+      </c>
       <c r="G2" s="9" t="inlineStr">
         <is>
           <t>電撃文庫/角川文庫/MF文庫J</t>
         </is>
       </c>
-      <c r="H2" s="9" t="inlineStr"/>
-      <c r="I2" s="9" t="inlineStr"/>
-      <c r="J2" s="9" t="inlineStr"/>
-      <c r="K2" s="9" t="inlineStr"/>
+      <c r="H2" s="9" t="inlineStr">
+        <is>
+          <t>ラノベ市場の最大手。カクヨム→書籍→アニメの発掘パイプラインを自社完結</t>
+        </is>
+      </c>
+      <c r="I2" s="9" t="inlineStr">
+        <is>
+          <t>なろう系の飽和で新規ヒットの創出難度が上昇</t>
+        </is>
+      </c>
+      <c r="J2" s="9" t="inlineStr">
+        <is>
+          <t>カクヨム発の新規ヒット。海外向けラノベ翻訳の拡大</t>
+        </is>
+      </c>
+      <c r="K2" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
@@ -46754,16 +47666,36 @@
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr"/>
-      <c r="F3" s="9" t="inlineStr"/>
+      <c r="F3" s="9" t="inlineStr">
+        <is>
+          <t>非上場。今週は目立った発表なし</t>
+        </is>
+      </c>
       <c r="G3" s="9" t="inlineStr">
         <is>
           <t>新潮文庫</t>
         </is>
       </c>
-      <c r="H3" s="9" t="inlineStr"/>
-      <c r="I3" s="9" t="inlineStr"/>
-      <c r="J3" s="9" t="inlineStr"/>
-      <c r="K3" s="9" t="inlineStr"/>
+      <c r="H3" s="9" t="inlineStr">
+        <is>
+          <t>文芸の権威性とバックリストの強さ。十二国記等の長期IP</t>
+        </is>
+      </c>
+      <c r="I3" s="9" t="inlineStr">
+        <is>
+          <t>文芸単行本市場の縮小。デジタル比率が低い</t>
+        </is>
+      </c>
+      <c r="J3" s="9" t="inlineStr">
+        <is>
+          <t>文芸作品の映像化ライセンス強化</t>
+        </is>
+      </c>
+      <c r="K3" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
@@ -46787,16 +47719,36 @@
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr"/>
-      <c r="F4" s="9" t="inlineStr"/>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>非上場。今週は目立った発表なし</t>
+        </is>
+      </c>
       <c r="G4" s="9" t="inlineStr">
         <is>
           <t>文春文庫/文藝春秋</t>
         </is>
       </c>
-      <c r="H4" s="9" t="inlineStr"/>
-      <c r="I4" s="9" t="inlineStr"/>
-      <c r="J4" s="9" t="inlineStr"/>
-      <c r="K4" s="9" t="inlineStr"/>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>直木賞・芥川賞の運営で話題創出力を持つ</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>雑誌（週刊文春）依存の収益構造にリスク</t>
+        </is>
+      </c>
+      <c r="J4" s="9" t="inlineStr">
+        <is>
+          <t>文春オンラインのデジタル収益化</t>
+        </is>
+      </c>
+      <c r="K4" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -46820,16 +47772,36 @@
         </is>
       </c>
       <c r="E5" s="9" t="inlineStr"/>
-      <c r="F5" s="9" t="inlineStr"/>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>非上場。第87期は当期純利益111億円、総資産3,600億円超</t>
+        </is>
+      </c>
       <c r="G5" s="9" t="inlineStr">
         <is>
           <t>講談社文庫/講談社タイガ</t>
         </is>
       </c>
-      <c r="H5" s="9" t="inlineStr"/>
-      <c r="I5" s="9" t="inlineStr"/>
-      <c r="J5" s="9" t="inlineStr"/>
-      <c r="K5" s="9" t="inlineStr"/>
+      <c r="H5" s="9" t="inlineStr">
+        <is>
+          <t>文芸・新書・漫画の分散が効き、財務基盤が盤石</t>
+        </is>
+      </c>
+      <c r="I5" s="9" t="inlineStr">
+        <is>
+          <t>文芸単体では漫画部門に比べ収益寄与が小さい</t>
+        </is>
+      </c>
+      <c r="J5" s="9" t="inlineStr">
+        <is>
+          <t>文芸作品のメディアミックス（映像化）比率</t>
+        </is>
+      </c>
+      <c r="K5" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
@@ -46853,16 +47825,36 @@
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr"/>
-      <c r="F6" s="9" t="inlineStr"/>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>非上場。第83期は売上高2,043.75億円、当期純利益206.17億円</t>
+        </is>
+      </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
           <t>集英社文庫/ダッシュエックス文庫</t>
         </is>
       </c>
-      <c r="H6" s="9" t="inlineStr"/>
-      <c r="I6" s="9" t="inlineStr"/>
-      <c r="J6" s="9" t="inlineStr"/>
-      <c r="K6" s="9" t="inlineStr"/>
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>ダッシュエックス文庫等でラノベ領域にも参入</t>
+        </is>
+      </c>
+      <c r="I6" s="9" t="inlineStr">
+        <is>
+          <t>文芸・小説は漫画部門に比べ存在感が薄い</t>
+        </is>
+      </c>
+      <c r="J6" s="9" t="inlineStr">
+        <is>
+          <t>漫画IPのノベライズ展開</t>
+        </is>
+      </c>
+      <c r="K6" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
@@ -46886,16 +47878,36 @@
         </is>
       </c>
       <c r="E7" s="9" t="inlineStr"/>
-      <c r="F7" s="9" t="inlineStr"/>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>非上場。ShoProは2026年3月期最終利益24.15億円（-9.6%）</t>
+        </is>
+      </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
           <t>小学館文庫/ガガガ文庫</t>
         </is>
       </c>
-      <c r="H7" s="9" t="inlineStr"/>
-      <c r="I7" s="9" t="inlineStr"/>
-      <c r="J7" s="9" t="inlineStr"/>
-      <c r="K7" s="9" t="inlineStr"/>
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>ガガガ文庫等でラノベ市場に一定のプレゼンス</t>
+        </is>
+      </c>
+      <c r="I7" s="9" t="inlineStr">
+        <is>
+          <t>ラノベではKADOKAWAとの規模差が大きい</t>
+        </is>
+      </c>
+      <c r="J7" s="9" t="inlineStr">
+        <is>
+          <t>既存ラノベIPのアニメ化</t>
+        </is>
+      </c>
+      <c r="K7" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
@@ -46919,16 +47931,36 @@
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr"/>
-      <c r="F8" s="9" t="inlineStr"/>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>非上場。今週は目立った発表なし</t>
+        </is>
+      </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
           <t>幻冬舎文庫</t>
         </is>
       </c>
-      <c r="H8" s="9" t="inlineStr"/>
-      <c r="I8" s="9" t="inlineStr"/>
-      <c r="J8" s="9" t="inlineStr"/>
-      <c r="K8" s="9" t="inlineStr"/>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>話題書の企画力とマーケティングの巧さ</t>
+        </is>
+      </c>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>ヒット依存で業績の振れ幅が大きい</t>
+        </is>
+      </c>
+      <c r="J8" s="9" t="inlineStr">
+        <is>
+          <t>新規話題作の創出ペース</t>
+        </is>
+      </c>
+      <c r="K8" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
@@ -46952,16 +47984,36 @@
         </is>
       </c>
       <c r="E9" s="9" t="inlineStr"/>
-      <c r="F9" s="9" t="inlineStr"/>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>非上場。「本好きの下剋上」はシリーズ累計1,300万部超。原作小説は全33巻（第1部〜第5部）の長編で、アニメ第3部「領主の養女」が2026年4月から連続2クールで放送中</t>
+        </is>
+      </c>
       <c r="G9" s="9" t="inlineStr">
         <is>
           <t>TOブックス(本好きの下剋上)</t>
         </is>
       </c>
-      <c r="H9" s="9" t="inlineStr"/>
-      <c r="I9" s="9" t="inlineStr"/>
-      <c r="J9" s="9" t="inlineStr"/>
-      <c r="K9" s="9" t="inlineStr"/>
+      <c r="H9" s="9" t="inlineStr">
+        <is>
+          <t>本好きの下剋上という単一の超大型IPで長期的な収益を確保。アニメ化が段階的に続く</t>
+        </is>
+      </c>
+      <c r="I9" s="9" t="inlineStr">
+        <is>
+          <t>事実上1タイトル依存で、次のヒットが見えていない</t>
+        </is>
+      </c>
+      <c r="J9" s="9" t="inlineStr">
+        <is>
+          <t>第3部アニメの評価と、第4部以降の映像化決定</t>
+        </is>
+      </c>
+      <c r="K9" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
@@ -46985,16 +48037,36 @@
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr"/>
-      <c r="F10" s="9" t="inlineStr"/>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>「カドサマー2026」（7/17〜）の中核ストアとして参加。全37ストアの一角</t>
+        </is>
+      </c>
       <c r="G10" s="9" t="inlineStr">
         <is>
           <t>カクヨム/BOOK☆WALKER</t>
         </is>
       </c>
-      <c r="H10" s="9" t="inlineStr"/>
-      <c r="I10" s="9" t="inlineStr"/>
-      <c r="J10" s="9" t="inlineStr"/>
-      <c r="K10" s="9" t="inlineStr"/>
+      <c r="H10" s="9" t="inlineStr">
+        <is>
+          <t>KADOKAWA作品の自社直販チャネルで手数料流出を抑えられる</t>
+        </is>
+      </c>
+      <c r="I10" s="9" t="inlineStr">
+        <is>
+          <t>外部ストア（Kindle等）との規模差が大きい</t>
+        </is>
+      </c>
+      <c r="J10" s="9" t="inlineStr">
+        <is>
+          <t>自社ストア経由の売上比率をどこまで高められるか</t>
+        </is>
+      </c>
+      <c r="K10" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
@@ -47018,16 +48090,36 @@
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr"/>
-      <c r="F11" s="9" t="inlineStr"/>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>薬屋のひとりごと・転スラ・本好きの下剋上など、なろう発作品が2026年も大型メディアミックスの中心</t>
+        </is>
+      </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
           <t>小説家になろう</t>
         </is>
       </c>
-      <c r="H11" s="9" t="inlineStr"/>
-      <c r="I11" s="9" t="inlineStr"/>
-      <c r="J11" s="9" t="inlineStr"/>
-      <c r="K11" s="9" t="inlineStr"/>
+      <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t>無償の投稿基盤から出版社がリスクなく発掘できる構造は依然強力</t>
+        </is>
+      </c>
+      <c r="I11" s="9" t="inlineStr">
+        <is>
+          <t>異世界転生系のジャンル飽和。カクヨム等との投稿者獲得競争</t>
+        </is>
+      </c>
+      <c r="J11" s="9" t="inlineStr">
+        <is>
+          <t>なろう発の新ジャンルが立ち上がるか</t>
+        </is>
+      </c>
+      <c r="K11" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
@@ -47051,16 +48143,36 @@
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr"/>
-      <c r="F12" s="9" t="inlineStr"/>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>今週は目立った開示なし。日本語オーディオブックのラインナップ拡充を継続</t>
+        </is>
+      </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
           <t>オーディオブック</t>
         </is>
       </c>
-      <c r="H12" s="9" t="inlineStr"/>
-      <c r="I12" s="9" t="inlineStr"/>
-      <c r="J12" s="9" t="inlineStr"/>
-      <c r="K12" s="9" t="inlineStr"/>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>Prime基盤との連携。ラノベ・文芸の音声化で新たな収益窓口を出版社に提供</t>
+        </is>
+      </c>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>日本のオーディオブック市場は欧米比で小さい</t>
+        </is>
+      </c>
+      <c r="J12" s="9" t="inlineStr">
+        <is>
+          <t>人気ラノベの音声化ペースと、AI音声の活用可否</t>
+        </is>
+      </c>
+      <c r="K12" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
@@ -47084,16 +48196,36 @@
         </is>
       </c>
       <c r="E13" s="9" t="inlineStr"/>
-      <c r="F13" s="9" t="inlineStr"/>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>楽天Kobo電子書籍ストアは「カドサマー2026」の対象37ストアに参加</t>
+        </is>
+      </c>
       <c r="G13" s="9" t="inlineStr">
         <is>
           <t>楽天Kobo</t>
         </is>
       </c>
-      <c r="H13" s="9" t="inlineStr"/>
-      <c r="I13" s="9" t="inlineStr"/>
-      <c r="J13" s="9" t="inlineStr"/>
-      <c r="K13" s="9" t="inlineStr"/>
+      <c r="H13" s="9" t="inlineStr">
+        <is>
+          <t>楽天経済圏のポイント還元で価格競争力を出せる</t>
+        </is>
+      </c>
+      <c r="I13" s="9" t="inlineStr">
+        <is>
+          <t>Kindle との差が開いており、電子書籍単体の存在感は低下</t>
+        </is>
+      </c>
+      <c r="J13" s="9" t="inlineStr">
+        <is>
+          <t>ポイント施策以外の差別化要素を作れるか</t>
+        </is>
+      </c>
+      <c r="K13" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -47629,16 +48761,24 @@
       </c>
       <c r="F2" s="9" t="inlineStr">
         <is>
-          <t>アクティブ</t>
-        </is>
-      </c>
-      <c r="G2" s="9" t="inlineStr"/>
+          <t>ワールドツアー準備中</t>
+        </is>
+      </c>
+      <c r="G2" s="9" t="inlineStr">
+        <is>
+          <t>2026年後半に「ASIA 10-CITY DOME &amp; STADIUM TOUR 2026」を開催予定。国内5会場に加え台北・ソウル・香港・シンガポール等の海外公演を計画。5年ぶりにユニクロUTとのコラボコレクションを7月中旬から発売</t>
+        </is>
+      </c>
       <c r="H2" s="9" t="inlineStr">
         <is>
           <t>小説原作の楽曲化</t>
         </is>
       </c>
-      <c r="I2" s="9" t="inlineStr"/>
+      <c r="I2" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
@@ -47668,12 +48808,20 @@
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>アクティブ</t>
-        </is>
-      </c>
-      <c r="G3" s="9" t="inlineStr"/>
+          <t>海外活動 継続</t>
+        </is>
+      </c>
+      <c r="G3" s="9" t="inlineStr">
+        <is>
+          <t>ロサンゼルスでのイベントでYOASOBIらと共演。J-POPアーティストの海外ツアー本格化の流れの中心に位置する</t>
+        </is>
+      </c>
       <c r="H3" s="9" t="inlineStr"/>
-      <c r="I3" s="9" t="inlineStr"/>
+      <c r="I3" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
@@ -47703,12 +48851,20 @@
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
-          <t>アクティブ</t>
-        </is>
-      </c>
-      <c r="G4" s="9" t="inlineStr"/>
+          <t>新曲リリース／ツアー決定</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>新曲「夜鷹」を7月13日に配信リリース。実写映画『キングダム 魂の決戦』（7/17公開）の主題歌。アリーナツアー『米津玄師 2026 TOUR / GHOST』を11月6日〜12月17日に全国6都市14公演で開催、一般発売が決定。Billboard JAPANの週間総合チャートでも首位を獲得</t>
+        </is>
+      </c>
       <c r="H4" s="9" t="inlineStr"/>
-      <c r="I4" s="9" t="inlineStr"/>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -47878,12 +49034,20 @@
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t>アクティブ</t>
-        </is>
-      </c>
-      <c r="G9" s="9" t="inlineStr"/>
+          <t>完全体活動 継続中</t>
+        </is>
+      </c>
+      <c r="G9" s="9" t="inlineStr">
+        <is>
+          <t>「オリコン上半期ランキング2026」で2冠を達成。証券各社はBTSの完全体活動が2027年まで継続する前提でHYBEをセクターのトップピックに挙げている。一方でカムバック公演後のイベント効果は一巡し、K-POP関連株は年初来で大きく調整</t>
+        </is>
+      </c>
       <c r="H9" s="9" t="inlineStr"/>
-      <c r="I9" s="9" t="inlineStr"/>
+      <c r="I9" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
@@ -48325,16 +49489,36 @@
         </is>
       </c>
       <c r="E2" s="9" t="inlineStr"/>
-      <c r="F2" s="9" t="inlineStr"/>
+      <c r="F2" s="9" t="inlineStr">
+        <is>
+          <t>Q1 2026決算で、取締役会が自社株買い枠を10億ユーロへ倍増することを承認。あわせて保有するSpotify株式の半分を売却する方針を示した（Lucian Grainge CEO）</t>
+        </is>
+      </c>
       <c r="G2" s="9" t="inlineStr">
         <is>
           <t>Taylor Swift/Billie Eilish</t>
         </is>
       </c>
-      <c r="H2" s="9" t="inlineStr"/>
-      <c r="I2" s="9" t="inlineStr"/>
-      <c r="J2" s="9" t="inlineStr"/>
-      <c r="K2" s="9" t="inlineStr"/>
+      <c r="H2" s="9" t="inlineStr">
+        <is>
+          <t>株主還元の強化と、Spotify株売却によるキャッシュ創出。ストリーミング単価引き上げ交渉で主導権</t>
+        </is>
+      </c>
+      <c r="I2" s="9" t="inlineStr">
+        <is>
+          <t>Spotify株売却は同社の成長見通しに対する慎重姿勢とも読める</t>
+        </is>
+      </c>
+      <c r="J2" s="9" t="inlineStr">
+        <is>
+          <t>売却資金の使途（M&amp;Aか還元か）。ストリーミング「アーティスト・セントリック」モデルの浸透</t>
+        </is>
+      </c>
+      <c r="K2" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
@@ -48358,16 +49542,36 @@
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr"/>
-      <c r="F3" s="9" t="inlineStr"/>
+      <c r="F3" s="9" t="inlineStr">
+        <is>
+          <t>今週は目立った適時開示なし</t>
+        </is>
+      </c>
       <c r="G3" s="9" t="inlineStr">
         <is>
           <t>Ed Sheeran/Bruno Mars</t>
         </is>
       </c>
-      <c r="H3" s="9" t="inlineStr"/>
-      <c r="I3" s="9" t="inlineStr"/>
-      <c r="J3" s="9" t="inlineStr"/>
-      <c r="K3" s="9" t="inlineStr"/>
+      <c r="H3" s="9" t="inlineStr">
+        <is>
+          <t>UMGに次ぐカタログ規模。楽曲権利の取得を継続</t>
+        </is>
+      </c>
+      <c r="I3" s="9" t="inlineStr">
+        <is>
+          <t>UMGとの規模差が交渉力の差につながる</t>
+        </is>
+      </c>
+      <c r="J3" s="9" t="inlineStr">
+        <is>
+          <t>カタログ買収の資金調達環境</t>
+        </is>
+      </c>
+      <c r="K3" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
@@ -48391,16 +49595,36 @@
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr"/>
-      <c r="F4" s="9" t="inlineStr"/>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>音楽部門は米津玄師（7/13に新曲「夜鷹」を配信、映画「キングダム」主題歌）、YOASOBI（2026年アジア10都市ドーム＆スタジアムツアーを発表）等が牽引。米津玄師は11/6〜12/17に全国6都市14公演のアリーナツアー『2026 TOUR / GHOST』を開催</t>
+        </is>
+      </c>
       <c r="G4" s="9" t="inlineStr">
         <is>
           <t>米津玄師/YOASOBI/Beyoncé</t>
         </is>
       </c>
-      <c r="H4" s="9" t="inlineStr"/>
-      <c r="I4" s="9" t="inlineStr"/>
-      <c r="J4" s="9" t="inlineStr"/>
-      <c r="K4" s="9" t="inlineStr"/>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>邦楽トップアーティストを多数擁し、アニメ・映画とのタイアップで収益を多重回収。アニプレックス／Crunchyrollとの垂直統合</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>ゲーム・イメージング等の他部門の影響で音楽単体の評価が埋もれやすい</t>
+        </is>
+      </c>
+      <c r="J4" s="9" t="inlineStr">
+        <is>
+          <t>J-POPの海外ツアー収益化。楽曲カタログ買収の継続</t>
+        </is>
+      </c>
+      <c r="K4" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -48424,16 +49648,36 @@
         </is>
       </c>
       <c r="E5" s="9" t="inlineStr"/>
-      <c r="F5" s="9" t="inlineStr"/>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>Q1 2026はプレミアム会員2.93億人（+300万）、営業利益8.37億ドルと過去最高。ただしQ2ガイダンス（MAU 7.78億／プレミアム2.99億／売上48億ユーロ／営業利益6.3億ユーロ・利益率33.1%）が市場予想の約3.02億人を下回り、株価は一時13%超下落。株価は年初来約-16%。Q2決算は8/4予定</t>
+        </is>
+      </c>
       <c r="G5" s="9" t="inlineStr">
         <is>
           <t>配信プラットフォーム</t>
         </is>
       </c>
-      <c r="H5" s="9" t="inlineStr"/>
-      <c r="I5" s="9" t="inlineStr"/>
-      <c r="J5" s="9" t="inlineStr"/>
-      <c r="K5" s="9" t="inlineStr"/>
+      <c r="H5" s="9" t="inlineStr">
+        <is>
+          <t>営業利益率30%超が定着し、収益モデルとして完成しつつある</t>
+        </is>
+      </c>
+      <c r="I5" s="9" t="inlineStr">
+        <is>
+          <t>北米のプレミアム会員が減少。加入者成長の鈍化が明確に</t>
+        </is>
+      </c>
+      <c r="J5" s="9" t="inlineStr">
+        <is>
+          <t>8/4のQ2決算で会員数が回復するか。値上げの受容度とスーパープレミアム層の投入</t>
+        </is>
+      </c>
+      <c r="K5" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
@@ -48456,17 +49700,41 @@
           <t>レーベル/事務所</t>
         </is>
       </c>
-      <c r="E6" s="9" t="inlineStr"/>
-      <c r="F6" s="9" t="inlineStr"/>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>株価232,000ウォン（前日比+7.91%、7月中旬時点）</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>年初来では株価-36.0%と大幅安だったが、7月中旬に反発。韓流関連輸出が前年比+84%の189.75億ドルに達したとの報道と、証券各社の「割安」評価が反発材料</t>
+        </is>
+      </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
           <t>BTS/NewJeans/SEVENTEEN</t>
         </is>
       </c>
-      <c r="H6" s="9" t="inlineStr"/>
-      <c r="I6" s="9" t="inlineStr"/>
-      <c r="J6" s="9" t="inlineStr"/>
-      <c r="K6" s="9" t="inlineStr"/>
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>証券各社がセクターのトップピックに挙げる。BTSの完全体活動が来年まで継続する見込みで、新人グループの成長により単一メガIP依存が徐々に低下</t>
+        </is>
+      </c>
+      <c r="I6" s="9" t="inlineStr">
+        <is>
+          <t>BTSカムバック公演後のイベントドリブンの momentum 剥落。資金がAI・半導体株へローテーション</t>
+        </is>
+      </c>
+      <c r="J6" s="9" t="inlineStr">
+        <is>
+          <t>BTS完全体ツアーの規模と収益。新人グループのIP育成スピード</t>
+        </is>
+      </c>
+      <c r="K6" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
@@ -48489,17 +49757,41 @@
           <t>レーベル/事務所</t>
         </is>
       </c>
-      <c r="E7" s="9" t="inlineStr"/>
-      <c r="F7" s="9" t="inlineStr"/>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>約1.58兆ウォン（前年末3.09兆ウォンから-48.8%）</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>韓国主要4社の中で最大の下落率。7月中旬に株価81,900ウォン（+6.09%）と反発</t>
+        </is>
+      </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
           <t>NCT/aespa</t>
         </is>
       </c>
-      <c r="H7" s="9" t="inlineStr"/>
-      <c r="I7" s="9" t="inlineStr"/>
-      <c r="J7" s="9" t="inlineStr"/>
-      <c r="K7" s="9" t="inlineStr"/>
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>バリュエーション面での割安感。韓流輸出全体は+84%と好調</t>
+        </is>
+      </c>
+      <c r="I7" s="9" t="inlineStr">
+        <is>
+          <t>時価総額がほぼ半減。次世代メガIPの不在が最大の懸念</t>
+        </is>
+      </c>
+      <c r="J7" s="9" t="inlineStr">
+        <is>
+          <t>新人グループのグローバル立ち上がり。カカオとの協業効果</t>
+        </is>
+      </c>
+      <c r="K7" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
@@ -48523,16 +49815,36 @@
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr"/>
-      <c r="F8" s="9" t="inlineStr"/>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>年初来株価-35.7%。韓国4社合計で年初来8兆ウォン超（約54億ドル）の時価総額が消失した局面の一角</t>
+        </is>
+      </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
           <t>Stray Kids/TWICE</t>
         </is>
       </c>
-      <c r="H8" s="9" t="inlineStr"/>
-      <c r="I8" s="9" t="inlineStr"/>
-      <c r="J8" s="9" t="inlineStr"/>
-      <c r="K8" s="9" t="inlineStr"/>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>Stray Kids の北米ツアー動員が堅調。海外現地デビュー戦略</t>
+        </is>
+      </c>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>セクター全体の資金流出。平均株価下落率40%超の環境</t>
+        </is>
+      </c>
+      <c r="J8" s="9" t="inlineStr">
+        <is>
+          <t>所属アーティストの北米での定着度。日本・中国市場の回復</t>
+        </is>
+      </c>
+      <c r="K8" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
@@ -48556,16 +49868,36 @@
         </is>
       </c>
       <c r="E9" s="9" t="inlineStr"/>
-      <c r="F9" s="9" t="inlineStr"/>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>2026年3月期は売上高1,465.71億円（+11.3%）、営業利益40.85億円と大幅な増収増益。音楽事業の営業利益34.68億円、アニメ・映像事業10.62億円といずれも大幅改善。ライブ関連売上の増加とアニメ作品の海外販売好調が牽引</t>
+        </is>
+      </c>
       <c r="G9" s="9" t="inlineStr">
         <is>
           <t>浜崎あゆみ/ライブ事業</t>
         </is>
       </c>
-      <c r="H9" s="9" t="inlineStr"/>
-      <c r="I9" s="9" t="inlineStr"/>
-      <c r="J9" s="9" t="inlineStr"/>
-      <c r="K9" s="9" t="inlineStr"/>
+      <c r="H9" s="9" t="inlineStr">
+        <is>
+          <t>ライブ市場の拡大を直接取り込めている。アニメ・映像の海外販売が新たな柱に</t>
+        </is>
+      </c>
+      <c r="I9" s="9" t="inlineStr">
+        <is>
+          <t>音楽事業の利益率は依然として低く、ヒット依存の構造</t>
+        </is>
+      </c>
+      <c r="J9" s="9" t="inlineStr">
+        <is>
+          <t>アニメ・映像事業の海外販売を継続的な柱にできるか</t>
+        </is>
+      </c>
+      <c r="K9" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
@@ -48589,16 +49921,36 @@
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr"/>
-      <c r="F10" s="9" t="inlineStr"/>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>ライブ・エンタメ市場（音楽・ステージ）は2024年に7,605億円（+10.9%）と過去最高を更新、2030年には8,700億円まで拡大する見通し（ぴあ総研）。この追い風下でマネジメント事業を展開</t>
+        </is>
+      </c>
       <c r="G10" s="9" t="inlineStr">
         <is>
           <t>サザン/BABYMETAL/Perfume</t>
         </is>
       </c>
-      <c r="H10" s="9" t="inlineStr"/>
-      <c r="I10" s="9" t="inlineStr"/>
-      <c r="J10" s="9" t="inlineStr"/>
-      <c r="K10" s="9" t="inlineStr"/>
+      <c r="H10" s="9" t="inlineStr">
+        <is>
+          <t>ライブ市場の構造的拡大が直接の追い風。所属アーティストの動員力</t>
+        </is>
+      </c>
+      <c r="I10" s="9" t="inlineStr">
+        <is>
+          <t>マネジメント業は個別アーティストの活動状況に業績が左右される</t>
+        </is>
+      </c>
+      <c r="J10" s="9" t="inlineStr">
+        <is>
+          <t>大型ツアーの本数と、海外公演の比率</t>
+        </is>
+      </c>
+      <c r="K10" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
@@ -48622,16 +49974,36 @@
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr"/>
-      <c r="F11" s="9" t="inlineStr"/>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>今週は音楽部門固有の適時開示なし。JVCケンウッド本体は車載・無線が主力</t>
+        </is>
+      </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
           <t>各アーティスト</t>
         </is>
       </c>
-      <c r="H11" s="9" t="inlineStr"/>
-      <c r="I11" s="9" t="inlineStr"/>
-      <c r="J11" s="9" t="inlineStr"/>
-      <c r="K11" s="9" t="inlineStr"/>
+      <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t>音楽事業は安定した収益源。アニソン・声優領域に強み</t>
+        </is>
+      </c>
+      <c r="I11" s="9" t="inlineStr">
+        <is>
+          <t>本体の主力が車載機器のため、音楽事業の評価が株価に反映されにくい</t>
+        </is>
+      </c>
+      <c r="J11" s="9" t="inlineStr">
+        <is>
+          <t>音楽事業の切り出し・再評価の可能性</t>
+        </is>
+      </c>
+      <c r="K11" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
@@ -48655,16 +50027,36 @@
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr"/>
-      <c r="F12" s="9" t="inlineStr"/>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>Q1 2026は売上38億ドル（報告ベース+12%、為替中立で+9%）。イベント関連の繰延収益は66億ドル（+22%）と過去最高水準</t>
+        </is>
+      </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
           <t>世界最大のライブ興行</t>
         </is>
       </c>
-      <c r="H12" s="9" t="inlineStr"/>
-      <c r="I12" s="9" t="inlineStr"/>
-      <c r="J12" s="9" t="inlineStr"/>
-      <c r="K12" s="9" t="inlineStr"/>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>繰延収益66億ドルは今後の公演需要の強さを示す先行指標。世界的なライブ需要の拡大</t>
+        </is>
+      </c>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>Ticketmasterを巡る米当局の反トラスト訴訟が継続的な重石</t>
+        </is>
+      </c>
+      <c r="J12" s="9" t="inlineStr">
+        <is>
+          <t>反トラスト訴訟の帰趨。スポンサーシップ単価の上昇余地</t>
+        </is>
+      </c>
+      <c r="K12" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
@@ -48688,16 +50080,36 @@
         </is>
       </c>
       <c r="E13" s="9" t="inlineStr"/>
-      <c r="F13" s="9" t="inlineStr"/>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>ぴあ総研の調査によると、2024年のライブ・エンタテインメント市場は7,605億円（+10.9%）と過去最高を更新。内訳は音楽5,299億円（+11.4%）、ステージ2,306億円（+9.8%）でともに二桁成長。2030年に8,700億円（年平均成長率2.4%）まで拡大する予測</t>
+        </is>
+      </c>
       <c r="G13" s="9" t="inlineStr">
         <is>
           <t>チケットぴあ</t>
         </is>
       </c>
-      <c r="H13" s="9" t="inlineStr"/>
-      <c r="I13" s="9" t="inlineStr"/>
-      <c r="J13" s="9" t="inlineStr"/>
-      <c r="K13" s="9" t="inlineStr"/>
+      <c r="H13" s="9" t="inlineStr">
+        <is>
+          <t>チケッティングは市場拡大の恩恵を直接受ける。自社アリーナ（ぴあアリーナMM）の稼働</t>
+        </is>
+      </c>
+      <c r="I13" s="9" t="inlineStr">
+        <is>
+          <t>市場成長率は2030年に向け年2.4%へ鈍化する見通しで、高成長フェーズは終盤</t>
+        </is>
+      </c>
+      <c r="J13" s="9" t="inlineStr">
+        <is>
+          <t>手数料以外の収益源（ダイナミックプライシング、二次流通）の構築</t>
+        </is>
+      </c>
+      <c r="K13" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
daily-news(6genres) + cross-questions + media-mix + events + predictions + game-design update
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -891,7 +891,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:H38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2455,6 +2455,48 @@
       <c r="H37" t="inlineStr">
         <is>
           <t>ゲーム</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B38" s="15" t="inlineStr">
+        <is>
+          <t>京アニ級の実力制作会社がOTT世界独占(＝製作委員会レス)で完成させる例が増えると、地上波局の深夜アニメ製作出資が細り、出版社は委員会縮小を嫌って自社単独出資(内製化)へ前傾。結果テレビ局が『幹事』から外れ、広告依存の地上波アニメ枠が構造的に縮小する。</t>
+        </is>
+      </c>
+      <c r="C38" s="15" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="D38" s="15" t="inlineStr">
+        <is>
+          <t>2026〜2027年</t>
+        </is>
+      </c>
+      <c r="E38" s="15" t="inlineStr">
+        <is>
+          <t>京都アニメーション, Netflix, 民放各局, 大手出版社</t>
+        </is>
+      </c>
+      <c r="F38" s="15" t="inlineStr">
+        <is>
+          <t>京アニ『二十世紀電氣目録』Netflix世界独占配信(映画.com, 2026-07-21追記)</t>
+        </is>
+      </c>
+      <c r="G38" s="15" t="inlineStr">
+        <is>
+          <t>新規深夜アニメの製作委員会に地上波局が幹事参加する比率、出版社の単独クレジット/自社出資作品数を四半期で観測。テレビ局主導の委員会組成が減れば予測的中。</t>
+        </is>
+      </c>
+      <c r="H38" s="15" t="inlineStr">
+        <is>
+          <t>横断</t>
         </is>
       </c>
     </row>
@@ -5241,7 +5283,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H82"/>
+  <dimension ref="A1:H84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8693,6 +8735,90 @@
         </is>
       </c>
       <c r="H82" s="15" t="inlineStr">
+        <is>
+          <t>横断</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B83" s="15" t="inlineStr">
+        <is>
+          <t>ゲームで常態化した『単発作品の商業失敗→発売数ヶ月でスタジオ即縮小』は、アニメ制作会社や映画スタジオでも『一本の興行/配信不振→即リストラ・解散』として同様に起きるか？固定費構造が近い制作分野ほど波及しやすいのでは。</t>
+        </is>
+      </c>
+      <c r="C83" s="15" t="inlineStr">
+        <is>
+          <t>ZA/UM 新作不振で最大32名削減(PC Gamer, 2026-07-17)</t>
+        </is>
+      </c>
+      <c r="D83" s="15" t="inlineStr">
+        <is>
+          <t>ZA/UM, アニメ制作会社, 映画スタジオ</t>
+        </is>
+      </c>
+      <c r="E83" s="15" t="inlineStr">
+        <is>
+          <t>アニメ制作, 映画製作, 人材派遣・フリーランス市場</t>
+        </is>
+      </c>
+      <c r="F83" s="15" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="G83" s="15" t="inlineStr">
+        <is>
+          <t>『ヒット→拡大／失敗→即縮小』のプロジェクト単位の雇用が全エンタメ制作に共通化する可能性</t>
+        </is>
+      </c>
+      <c r="H83" s="15" t="inlineStr">
+        <is>
+          <t>横断</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B84" s="15" t="inlineStr">
+        <is>
+          <t>制作会社が国内放送を経ずOTT世界独占で新作を出す動き(京アニ×Netflix)は、ゲームの『プラットフォーム独占ローンチ』と同じ交渉構造か？さらに漫画・小説の『海外同時・独占配信』へも広がるか。</t>
+        </is>
+      </c>
+      <c r="C84" s="15" t="inlineStr">
+        <is>
+          <t>京アニ『二十世紀電氣目録』Netflix世界独占配信(映画.com)</t>
+        </is>
+      </c>
+      <c r="D84" s="15" t="inlineStr">
+        <is>
+          <t>京都アニメーション, Netflix</t>
+        </is>
+      </c>
+      <c r="E84" s="15" t="inlineStr">
+        <is>
+          <t>ゲーム(独占ローンチ), 漫画・小説(海外同時配信), OTT</t>
+        </is>
+      </c>
+      <c r="F84" s="15" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="G84" s="15" t="inlineStr">
+        <is>
+          <t>『独占と引き換えの資本／権利設計』はメディアを問わず共通の交渉テンプレになりつつある</t>
+        </is>
+      </c>
+      <c r="H84" s="15" t="inlineStr">
         <is>
           <t>横断</t>
         </is>
@@ -17380,7 +17506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M347"/>
+  <dimension ref="A1:M354"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -40571,6 +40697,468 @@
           <t>漫画・小説双方に影響するためジャンルは横断</t>
         </is>
       </c>
+    </row>
+    <row r="348">
+      <c r="A348" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B348" s="15" t="inlineStr">
+        <is>
+          <t>ゲーム</t>
+        </is>
+      </c>
+      <c r="C348" s="15" t="inlineStr">
+        <is>
+          <t>EAの550億ドルLBO、EU反トラスト承認が7/22に——サウジPIF主導の非公開化が最終局面へ</t>
+        </is>
+      </c>
+      <c r="D348" s="15" t="inlineStr">
+        <is>
+          <t>https://mobilesyrup.com/2026/07/21/european-union-approve-saudi-acquisition-ea-report/</t>
+        </is>
+      </c>
+      <c r="E348" s="15" t="inlineStr">
+        <is>
+          <t>2025年9月にEAはサウジPIF・Silver Lake・Jared Kushner系Affinity Partners連合による総額550億ドルのLBOで非公開化に合意。PIFが約93.7%を握る。年明け以降、EUの合併審査(7/22)とForeign Subsidies規制審査(7/30)、米CFIUS(外資審査、期限9/28)が最後の関門となっていた。</t>
+        </is>
+      </c>
+      <c r="F348" s="15" t="inlineStr">
+        <is>
+          <t>ロイター報道によればEUは7/22の予備審査終了時に無条件承認を出す見込み。米HSR反トラストは既にクリア済みだが、国家安全保障を見るCFIUS審査は9/28まで残り、最終成立はなお不透明。ゲーム最大級のPEバイアウトがヤマ場を迎える。</t>
+        </is>
+      </c>
+      <c r="G348" s="15" t="inlineStr">
+        <is>
+          <t>EU合併審査は7/22に無条件承認の見込み(ロイター)
+別途EU外国補助金規制の判断が7/30に予定
+最大の関門は米CFIUS(外資安全保障)で期限9/28
+PIFが93.7%を握るソブリン資金主導のLBO</t>
+        </is>
+      </c>
+      <c r="H348" s="15" t="inlineStr">
+        <is>
+          <t>EUが通れば残る関門は米CFIUS一本に絞られ、9月末に向けEAのガバナンス・IP戦略(Battlefield/EA FC/The Sims)再編観測が強まる。非公開化後はライブサービス収益を担保にした資産流動化やスポーツライセンス更改の主導権が焦点。ソブリン資金による大手一括買収の是非が規制の前例となる。</t>
+        </is>
+      </c>
+      <c r="I348" s="15" t="inlineStr">
+        <is>
+          <t>ソブリンファンドのゲームM&amp;AとCFIUS外資安全保障審査</t>
+        </is>
+      </c>
+      <c r="J348" s="15" t="inlineStr">
+        <is>
+          <t>Electronic Arts, PIF(サウジ公共投資基金), Silver Lake, Affinity Partners</t>
+        </is>
+      </c>
+      <c r="K348" s="15" t="inlineStr">
+        <is>
+          <t>Battlefield, EA Sports FC, The Sims, Need for Speed</t>
+        </is>
+      </c>
+      <c r="L348" s="15" t="inlineStr">
+        <is>
+          <t>M&amp;A, 規制, 海外</t>
+        </is>
+      </c>
+      <c r="M348" s="15" t="inlineStr"/>
+    </row>
+    <row r="349">
+      <c r="A349" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B349" s="15" t="inlineStr">
+        <is>
+          <t>ゲーム</t>
+        </is>
+      </c>
+      <c r="C349" s="15" t="inlineStr">
+        <is>
+          <t>26年上期のゲーム業界レイオフは8千〜1.2万人規模、私的投資は前年比55%減——雇用収縮続く</t>
+        </is>
+      </c>
+      <c r="D349" s="15" t="inlineStr">
+        <is>
+          <t>https://sequelgame.com/game-industry-layoffs/</t>
+        </is>
+      </c>
+      <c r="E349" s="15" t="inlineStr">
+        <is>
+          <t>2022年以降続く業界の人員削減が26年も止まらず、上期だけで推計8,000〜12,000人が職を失った。過去2年で米ゲーム開発者の3人に1人がレイオフを経験。25年の業界向け私的投資は前年比55%減で、コンテンツ収益が過去最高の1,956億ドルに達する一方、資金は絞られている。</t>
+        </is>
+      </c>
+      <c r="F349" s="15" t="inlineStr">
+        <is>
+          <t>記録的な市場規模と裏腹に、スタジオ閉鎖・縮小が常態化。大手(Xbox, EA, Sony/Bungie)から中小(ZA/UM)まで広範に及び、単発タイトルの商業失敗が即人員削減に直結する構造が定着した。売上拡大＝雇用拡大の相関が崩れている。</t>
+        </is>
+      </c>
+      <c r="G349" s="15" t="inlineStr">
+        <is>
+          <t>26年上期のレイオフは推計8,000〜12,000人
+過去2年で米開発者の約1/3がレイオフ経験
+25年の業界向け私的投資は前年比55%減
+一方でコンテンツ収益は過去最高の1,956億ドル</t>
+        </is>
+      </c>
+      <c r="H349" s="15" t="inlineStr">
+        <is>
+          <t>AI支援による少人数・高生産性開発が常態化し、大規模内製の固定費を嫌う流れが加速。熟練人材の流出が中規模スタジオの新設・独立を促す一方、資金枯渇で存続は綱渡り。市場成長と雇用が乖離する『ジョブレス・グロース』がしばらく続く。</t>
+        </is>
+      </c>
+      <c r="I349" s="15" t="inlineStr">
+        <is>
+          <t>ゲーム業界のジョブレス成長とAIによる開発効率化</t>
+        </is>
+      </c>
+      <c r="J349" s="15" t="inlineStr">
+        <is>
+          <t>Microsoft, Electronic Arts, Sony, ZA/UM</t>
+        </is>
+      </c>
+      <c r="K349" s="15" t="inlineStr"/>
+      <c r="L349" s="15" t="inlineStr">
+        <is>
+          <t>業績, 人事・組織, 海外, トレンド</t>
+        </is>
+      </c>
+      <c r="M349" s="15" t="inlineStr"/>
+    </row>
+    <row r="350">
+      <c r="A350" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B350" s="15" t="inlineStr">
+        <is>
+          <t>ゲーム</t>
+        </is>
+      </c>
+      <c r="C350" s="15" t="inlineStr">
+        <is>
+          <t>『Disco Elysium』のZA/UM、新作不振で最大32名削減——発売2ヶ月後の縮小が示すもの</t>
+        </is>
+      </c>
+      <c r="D350" s="15" t="inlineStr">
+        <is>
+          <t>https://www.pcgamer.com/games/rpg/2-months-after-releasing-zero-parades-studio-za-um-is-laying-off-employees/</t>
+        </is>
+      </c>
+      <c r="E350" s="15" t="inlineStr">
+        <is>
+          <t>『Disco Elysium』で知られるZA/UMが7/17、全部門で最大32名の人員削減を発表。5月発売の新作『Zero Parades: For Dead Spies』の商業不振が理由で『現在の規模を維持できない』とした。同作のSteam同接ピークは約3,177人にとどまり発売後は減衰。2024年以来2度目の大型削減。</t>
+        </is>
+      </c>
+      <c r="F350" s="15" t="inlineStr">
+        <is>
+          <t>高評価・作家性重視のプレステージ系ナラティブRPGでも、発売2ヶ月で採算割れ→即縮小という業界の縮図が現れた。話題性や批評評価が必ずしも同接・売上に転化せず、ニッチな物語ゲームの商業的な脆さと、単発失敗を吸収できない小規模スタジオの資本構造の弱さを露呈。</t>
+        </is>
+      </c>
+      <c r="G350" s="15" t="inlineStr">
+        <is>
+          <t>新作『Zero Parades』の不振で最大32名を削減
+Steam同接ピークは約3,177人で発売後に減衰
+2024年以来2度目の大型リストラ
+批評的評価と商業成績の乖離が鮮明</t>
+        </is>
+      </c>
+      <c r="H350" s="15" t="inlineStr">
+        <is>
+          <t>作家性の強いナラティブRPGは、パブリッシャー出資よりOTT・映像資本や版権先行モデルへの依存を強める可能性。中核ライターIP(Disco Elysium系譜)が版権ごと外部に渡り、ゲーム発の物語IPを他メディア資本が抱え込む逆流も想定。中規模ナラティブ専業の存続戦略が問われる。</t>
+        </is>
+      </c>
+      <c r="I350" s="15" t="inlineStr">
+        <is>
+          <t>ナラティブRPGの商業性と作家性スタジオの資本戦略</t>
+        </is>
+      </c>
+      <c r="J350" s="15" t="inlineStr">
+        <is>
+          <t>ZA/UM</t>
+        </is>
+      </c>
+      <c r="K350" s="15" t="inlineStr">
+        <is>
+          <t>Disco Elysium, Zero Parades: For Dead Spies</t>
+        </is>
+      </c>
+      <c r="L350" s="15" t="inlineStr">
+        <is>
+          <t>業績, 人事・組織, 海外, 消費者インサイト</t>
+        </is>
+      </c>
+      <c r="M350" s="15" t="inlineStr">
+        <is>
+          <t>ミクロ×高インサイト枠</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B351" s="15" t="inlineStr">
+        <is>
+          <t>ゲーム</t>
+        </is>
+      </c>
+      <c r="C351" s="15" t="inlineStr">
+        <is>
+          <t>フロム『The Duskbloods』CNTを8/21-24実施、応募7/22開始——Switch2独占の看板新作</t>
+        </is>
+      </c>
+      <c r="D351" s="15" t="inlineStr">
+        <is>
+          <t>https://www.videogameschronicle.com/news/fromsoftwares-the-duskbloods-gets-a-network-test-this-august/</t>
+        </is>
+      </c>
+      <c r="E351" s="15" t="inlineStr">
+        <is>
+          <t>フロム・ソフトウェアがNintendo Switch 2独占の新作『The Duskbloods』のクローズドネットワークテスト(CNT)を8/21〜24に実施すると発表。応募受付は7/22開始、当選者は8/18からDL可能。最大8人対戦のPvPvE的マルチプレイが軸で、2026年内にSwitch2独占で発売予定だが発売日は未定。</t>
+        </is>
+      </c>
+      <c r="F351" s="15" t="inlineStr">
+        <is>
+          <t>人気スタジオの完全新作をハード独占で、しかもマルチプレイ前提のネットワークテストを事前実施——サーバ検証と初期コミュニティ形成を兼ねた『テスト＝プロモーション』型の立ち上げが定着しつつある。Switch2の看板独占として任天堂の年末商戦戦略にも直結する。</t>
+        </is>
+      </c>
+      <c r="G351" s="15" t="inlineStr">
+        <is>
+          <t>CNTは8/21-24、応募受付は7/22開始
+最大8人のPvPvEマルチが中核
+Switch2独占、2026年内発売予定(日付未定)
+当選者は8/18から事前DL可能</t>
+        </is>
+      </c>
+      <c r="H351" s="15" t="inlineStr">
+        <is>
+          <t>発売日発表はネットワークテストのフィードバック後、TGSや年末商戦前のショーケースが有力。マルチ主体の独占タイトルは初動同接がハード牽引力の試金石に。フロムのマルチ設計がソウルライク非対称対戦の新たな型を提示するか注目。</t>
+        </is>
+      </c>
+      <c r="I351" s="15" t="inlineStr">
+        <is>
+          <t>ネットワークテストを使った独占タイトルの立ち上げ設計</t>
+        </is>
+      </c>
+      <c r="J351" s="15" t="inlineStr">
+        <is>
+          <t>FromSoftware, Nintendo</t>
+        </is>
+      </c>
+      <c r="K351" s="15" t="inlineStr">
+        <is>
+          <t>The Duskbloods</t>
+        </is>
+      </c>
+      <c r="L351" s="15" t="inlineStr">
+        <is>
+          <t>新作, ハード, 国内</t>
+        </is>
+      </c>
+      <c r="M351" s="15" t="inlineStr"/>
+    </row>
+    <row r="352">
+      <c r="A352" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B352" s="15" t="inlineStr">
+        <is>
+          <t>アニメ</t>
+        </is>
+      </c>
+      <c r="C352" s="15" t="inlineStr">
+        <is>
+          <t>京アニ完全新作『二十世紀電氣目録』Netflix世界独占配信——制作会社の海外OTT直結が進む</t>
+        </is>
+      </c>
+      <c r="D352" s="15" t="inlineStr">
+        <is>
+          <t>https://eiga.com/news/20260127/24/</t>
+        </is>
+      </c>
+      <c r="E352" s="15" t="inlineStr">
+        <is>
+          <t>京都アニメーションの完全新作『二十世紀電氣目録-ユーレカ・エヴリカ-』が7/5よりNetflixで世界独占配信。印象派絵画を思わせる美術と緻密な作画が話題。同月は『火垂るの墓』の再配信(7/15)なども重なり、Netflixが日本アニメの供給窓口として存在感を一段と高めた。</t>
+        </is>
+      </c>
+      <c r="F352" s="15" t="inlineStr">
+        <is>
+          <t>国内テレビ放送を経ず、実力制作会社の完全新作をグローバルOTTが世界独占で抱える形が広がっている。国内先行の従来型ウィンドウから『同時グローバル独占』へ。制作会社にとっては海外資本の直接出資と引き換えに、製作委員会を介さない権利・収益設計が可能になる転換点。</t>
+        </is>
+      </c>
+      <c r="G352" s="15" t="inlineStr">
+        <is>
+          <t>京アニ新作をNetflixが世界独占配信(7/5〜)
+国内テレビ放送を経ないOTT直結モデル
+『火垂るの墓』再配信など供給集中も同月に
+制作会社が海外資本と直接結ぶ構造</t>
+        </is>
+      </c>
+      <c r="H352" s="15" t="inlineStr">
+        <is>
+          <t>OTT世界独占＝製作委員会レスの成功例が増えれば、地上波局のアニメ製作出資が細り、出版社は自社単独出資(内製化)へ前傾。窓口戦略はゲームのプラットフォーム独占ローンチに近づき、漫画・小説の海外同時配信にも波及しうる。テレビ局の『幹事』ポジション低下が焦点。</t>
+        </is>
+      </c>
+      <c r="I352" s="15" t="inlineStr">
+        <is>
+          <t>アニメのOTT世界独占と製作委員会モデルの変容</t>
+        </is>
+      </c>
+      <c r="J352" s="15" t="inlineStr">
+        <is>
+          <t>京都アニメーション, Netflix</t>
+        </is>
+      </c>
+      <c r="K352" s="15" t="inlineStr">
+        <is>
+          <t>二十世紀電氣目録-ユーレカ・エヴリカ-, 火垂るの墓</t>
+        </is>
+      </c>
+      <c r="L352" s="15" t="inlineStr">
+        <is>
+          <t>配信, 海外, 権利・ライセンス, トレンド</t>
+        </is>
+      </c>
+      <c r="M352" s="15" t="inlineStr"/>
+    </row>
+    <row r="353">
+      <c r="A353" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B353" s="15" t="inlineStr">
+        <is>
+          <t>映画</t>
+        </is>
+      </c>
+      <c r="C353" s="15" t="inlineStr">
+        <is>
+          <t>『トイ・ストーリー5』全世界502億円超・北米2週連続首位——レガシーIP×アニメの興行牽引</t>
+        </is>
+      </c>
+      <c r="D353" s="15" t="inlineStr">
+        <is>
+          <t>https://www.disney.co.jp/movie/toy5/news/20260622_01</t>
+        </is>
+      </c>
+      <c r="E353" s="15" t="inlineStr">
+        <is>
+          <t>ディズニー＆ピクサー『トイ・ストーリー5』がシリーズ史上最高のオープニング興収・最高評価を記録し、全世界502億円超に到達。北米週末ランキングでも2週連続首位を維持し、26年夏の実写・アニメを通じた大型タイトルの一角として劇場を牽引している。</t>
+        </is>
+      </c>
+      <c r="F353" s="15" t="inlineStr">
+        <is>
+          <t>新規AAA級オリジナルより、確立したレガシーIPのファミリー向けアニメが劇場の観客動員を安定的に支える構図が続く。オープニングの強さは既存ファン層の即時動員力に依存しており、ブランド認知が興行の初速を規定する『既知IP優位』のトレンドを裏づける事例。</t>
+        </is>
+      </c>
+      <c r="G353" s="15" t="inlineStr">
+        <is>
+          <t>全世界502億円超・シリーズ最高OWを記録
+北米週末ランキングで2週連続首位
+レガシーIPアニメの初速依存が鮮明
+ファミリー向けは劇場動員の安定基盤</t>
+        </is>
+      </c>
+      <c r="H353" s="15" t="inlineStr">
+        <is>
+          <t>既知IPのアニメ続編は初動集中・ロングテール弱めの傾向が続き、配給は公開後の配信ウィンドウ短縮で二次収益を最適化する動きを強める。オリジナル新規IPの劇場立ち上げコストは相対的に上昇し、スタジオのIP依存とリメイク・続編偏重が一層進む可能性。</t>
+        </is>
+      </c>
+      <c r="I353" s="15" t="inlineStr">
+        <is>
+          <t>レガシーIP偏重と劇場ウィンドウ短縮の相互作用</t>
+        </is>
+      </c>
+      <c r="J353" s="15" t="inlineStr">
+        <is>
+          <t>The Walt Disney Company, Pixar</t>
+        </is>
+      </c>
+      <c r="K353" s="15" t="inlineStr">
+        <is>
+          <t>トイ・ストーリー5</t>
+        </is>
+      </c>
+      <c r="L353" s="15" t="inlineStr">
+        <is>
+          <t>興行, 海外, チャート・ランキング, トレンド</t>
+        </is>
+      </c>
+      <c r="M353" s="15" t="inlineStr">
+        <is>
+          <t>ミクロ×高インサイト枠</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B354" s="15" t="inlineStr">
+        <is>
+          <t>音楽</t>
+        </is>
+      </c>
+      <c r="C354" s="15" t="inlineStr">
+        <is>
+          <t>ストリーミング値上げ後のARPU上昇がレーベル決算に遅れて反映——UMGの7月末決算が試金石</t>
+        </is>
+      </c>
+      <c r="D354" s="15" t="inlineStr">
+        <is>
+          <t>https://www.billboard.com/lists/music-company-earnings-q1-2026-what-spotify-umg-hybe-made/</t>
+        </is>
+      </c>
+      <c r="E354" s="15" t="inlineStr">
+        <is>
+          <t>Spotifyは26年2月に米個人プランを月11.99→12.99ドルへ値上げ。Apple/YouTube Music等も25年に値上げ済みで、高いARPUが遅れてレーベル収益に反映され始めた。UMGは7月末に次回決算を控え、WMGはQ1に録音売上17%増を報告済み。値上げ効果の可視化が焦点。</t>
+        </is>
+      </c>
+      <c r="F354" s="15" t="inlineStr">
+        <is>
+          <t>配信の値上げは『消費者→プラットフォーム→権利者→アーティスト』の商流の中で、時間差でレーベルのARPUに効いてくる。UMGはスーパーファン向けプレミアム階層・物販統合で高エンゲージ層からの追加収益化を進めており、決算はサブスク成熟後の単価成長戦略の成否を映す。</t>
+        </is>
+      </c>
+      <c r="G354" s="15" t="inlineStr">
+        <is>
+          <t>米Spotifyは26年2月に個人プランを値上げ(11.99→12.99ドル)
+値上げ効果はARPUとして遅れてレーベル決算に反映
+UMGは7月末に決算、WMGはQ1録音売上17%増
+スーパーファン向けプレミアム階層が単価成長の軸</t>
+        </is>
+      </c>
+      <c r="H354" s="15" t="inlineStr">
+        <is>
+          <t>サブスク純増が鈍る中、値上げ＋スーパーファン課金が成長ドライバーに移行。UMG決算で単価改善が確認されれば、各社はプレミアム階層・D2C物販統合を加速。ゲームのライブサービス『少数課金者依存』と同型の、ARPU志向への転換が音楽でも鮮明になる。</t>
+        </is>
+      </c>
+      <c r="I354" s="15" t="inlineStr">
+        <is>
+          <t>音楽サブスクのARPU成長とスーパーファン課金</t>
+        </is>
+      </c>
+      <c r="J354" s="15" t="inlineStr">
+        <is>
+          <t>Universal Music Group, Warner Music Group, Spotify</t>
+        </is>
+      </c>
+      <c r="K354" s="15" t="inlineStr"/>
+      <c r="L354" s="15" t="inlineStr">
+        <is>
+          <t>業績, 配信, 海外, トレンド</t>
+        </is>
+      </c>
+      <c r="M354" s="15" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
daily-news(Netflix Q2/横断) + cross-question + prediction + event status (CEDEC)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -891,7 +891,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:H39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2495,6 +2495,48 @@
         </is>
       </c>
       <c r="H38" s="15" t="inlineStr">
+        <is>
+          <t>横断</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B39" s="15" t="inlineStr">
+        <is>
+          <t>Netflixが『解約抑制の道具』としてクラウドゲームを機能させ始めると、カジュアル/スポーツ系スタジオは自前配信より"動画サブスクへのIP供給"を選好し、ゲームが動画定額の広告・維持レイヤーに再定義される。結果、単体F2Pモバイルのマネタイズ前提(ペイドUA→課金)が痩せ、供給側の交渉力が配信プラットフォーム側へ移動する。</t>
+        </is>
+      </c>
+      <c r="C39" s="15" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="D39" s="15" t="inlineStr">
+        <is>
+          <t>2026後半〜2027年</t>
+        </is>
+      </c>
+      <c r="E39" s="15" t="inlineStr">
+        <is>
+          <t>Netflix, カジュアル/スポーツ系スタジオ, FIFA World Cup</t>
+        </is>
+      </c>
+      <c r="F39" s="15" t="inlineStr">
+        <is>
+          <t>Netflix Q2 2026決算——クラウドゲームがFIFA/Unhinged牽引で最好調デビュー(CNBC 7/16)</t>
+        </is>
+      </c>
+      <c r="G39" s="15" t="inlineStr">
+        <is>
+          <t>Netflixのゲーム関連の会員維持/解約率への言及、クラウドゲームMAU・日次の継続開示、パブリッシャーが自社配信でなくNetflixへIP供給する新規契約の有無を観測。</t>
+        </is>
+      </c>
+      <c r="H39" s="15" t="inlineStr">
         <is>
           <t>横断</t>
         </is>
@@ -5283,7 +5325,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H84"/>
+  <dimension ref="A1:H85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8819,6 +8861,48 @@
         </is>
       </c>
       <c r="H84" s="15" t="inlineStr">
+        <is>
+          <t>横断</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B85" s="15" t="inlineStr">
+        <is>
+          <t>Netflixがクラウド/TVゲームとアニメを同一定額に束ねて『総合エンタメサブスク』化する動きは、ゲーム専業定額(Xbox Game Pass)や音楽定額(Spotify)の"単一メディア定額"を侵食し、可処分時間の奪い合いを激化させるか？</t>
+        </is>
+      </c>
+      <c r="C85" s="15" t="inlineStr">
+        <is>
+          <t>Netflix Q2 2026決算でクラウドゲーム躍進＋アニメ視聴牽引(CNBC/株主レター 7/16)</t>
+        </is>
+      </c>
+      <c r="D85" s="15" t="inlineStr">
+        <is>
+          <t>Netflix, Microsoft(Game Pass), Spotify</t>
+        </is>
+      </c>
+      <c r="E85" s="15" t="inlineStr">
+        <is>
+          <t>通信(キャリア定額バンドル), 動画×ゲーム×音楽の束ね, 広告(AVOD)</t>
+        </is>
+      </c>
+      <c r="F85" s="15" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="G85" s="15" t="inlineStr">
+        <is>
+          <t>定額の競争軸がコンテンツ量から"1契約で埋められる可処分時間の総量"へ移る——メディア横断の束ねが差別化の主戦場に</t>
+        </is>
+      </c>
+      <c r="H85" s="15" t="inlineStr">
         <is>
           <t>横断</t>
         </is>
@@ -13224,12 +13308,12 @@
       </c>
       <c r="I15" s="15" t="inlineStr">
         <is>
-          <t>開催予定</t>
+          <t>開催中</t>
         </is>
       </c>
       <c r="J15" s="15" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
     </row>
@@ -17506,7 +17590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M354"/>
+  <dimension ref="A1:M355"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -41159,6 +41243,77 @@
         </is>
       </c>
       <c r="M354" s="15" t="inlineStr"/>
+    </row>
+    <row r="355">
+      <c r="A355" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B355" s="15" t="inlineStr">
+        <is>
+          <t>横断</t>
+        </is>
+      </c>
+      <c r="C355" s="15" t="inlineStr">
+        <is>
+          <t>Netflix Q2決算——クラウドゲームがFIFA/Unhinged牽引で最好調デビュー、アニメ・非英語作が視聴を押し上げ</t>
+        </is>
+      </c>
+      <c r="D355" s="15" t="inlineStr">
+        <is>
+          <t>https://www.cnbc.com/2026/07/16/netflix-nflx-earnings-q2-2026.html</t>
+        </is>
+      </c>
+      <c r="E355" s="15" t="inlineStr">
+        <is>
+          <t>Netflixは長年モバイルゲームで苦戦してきたが、TV向けクラウドゲームへ軸足を移しスポーツ・カジュアル路線に転換。同時に非英語・アニメ作品を配信成長のドライバーに据える多角化を進めてきた。7/16に26年4-6月期(Q2)決算を開示した。</t>
+        </is>
+      </c>
+      <c r="F355" s="15" t="inlineStr">
+        <is>
+          <t>売上$12.56B(前年比+13%)、営業利益率33.4%、EPS $0.80で予想を小幅超過。通期売上ガイダンスを$51.0-51.4Bへ絞り込み。クラウドゲームはFIFA World Cup/Unhingedが最も成功したデビューとなり、Playgroundの日次プレイヤーが4月比3倍、キッズ向けモバイルは前年比+600%。アニメ等の非英語作が視聴時間を牽引した。株価は好決算でも時間外で下落。</t>
+        </is>
+      </c>
+      <c r="G355" s="15" t="inlineStr">
+        <is>
+          <t>・売上$12.56B(+13%)、営業益率33.4%、EPS $0.80で予想超過
+・クラウドゲームのデビュー最好調(FIFA World Cup/Unhinged)、Playground日次3倍
+・キッズ向けモバイルゲームのエンゲージメント前年比+600%
+・アニメ・非英語作(Swapped等)が視聴時間の成長を牽引、非英語が視聴の1/3超
+・好決算でも株価は時間外下落——高い期待値の裏返し</t>
+        </is>
+      </c>
+      <c r="H355" s="15" t="inlineStr">
+        <is>
+          <t>クラウド/TVゲームとアニメを同一サブスク内で束ねる『総合エンタメ定額』の色が濃くなる。ゲームは単体課金より会員維持(解約抑制)のツールとして機能させる方針が続き、Game Passや音楽サブスクとの可処分時間の奪い合いが激化。26年後半はIP連動ゲーム投入で会員接点を増やす動きが想定される。</t>
+        </is>
+      </c>
+      <c r="I355" s="15" t="inlineStr">
+        <is>
+          <t>サブスク定額のクロスメディア束ね(ゲーム×アニメ)とエンゲージメント指標</t>
+        </is>
+      </c>
+      <c r="J355" s="15" t="inlineStr">
+        <is>
+          <t>Netflix</t>
+        </is>
+      </c>
+      <c r="K355" s="15" t="inlineStr">
+        <is>
+          <t>FIFA World Cup: Launch Edition, Unhinged, Netflix Playground, Swapped</t>
+        </is>
+      </c>
+      <c r="L355" s="15" t="inlineStr">
+        <is>
+          <t>業績, クラウド, ライブサービス, 配信, 海外, トレンド</t>
+        </is>
+      </c>
+      <c r="M355" s="15" t="inlineStr">
+        <is>
+          <t>決算発表2026-07-16。ジャンル=横断(ゲーム×アニメ×配信)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
rankings: PS DL 2026-06 月間(国内PS5 top3) を追記
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -8919,7 +8919,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J101"/>
+  <dimension ref="A1:J104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12524,6 +12524,120 @@
       <c r="I101" t="inlineStr">
         <is>
           <t>VGChartz Steam週間トップセラー Week29 https://www.vgchartz.com/article/468471/steam-weekly-week-29-2026/ （GameGrin/SteamDB併用）</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="3" t="inlineStr">
+        <is>
+          <t>2026-06 (月間)</t>
+        </is>
+      </c>
+      <c r="B102" s="3" t="inlineStr">
+        <is>
+          <t>PS DL</t>
+        </is>
+      </c>
+      <c r="C102" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D102" s="3" t="inlineStr">
+        <is>
+          <t>FINAL FANTASY VII REBIRTH</t>
+        </is>
+      </c>
+      <c r="E102" s="3" t="inlineStr">
+        <is>
+          <t>PS5</t>
+        </is>
+      </c>
+      <c r="F102" s="3" t="n"/>
+      <c r="G102" s="3" t="n"/>
+      <c r="H102" s="3" t="n"/>
+      <c r="I102" s="3" t="inlineStr">
+        <is>
+          <t>PS Blog 月間DLランキング(国内PS5) https://blog.ja.playstation.com/2026/07/09/20260709-monthly-ps-store-ranking-s/</t>
+        </is>
+      </c>
+      <c r="J102" s="3" t="inlineStr">
+        <is>
+          <t>週間が無いため月間で代替。完結編『FF7 REVELATION』2027年春発売決定が追い風</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="3" t="inlineStr">
+        <is>
+          <t>2026-06 (月間)</t>
+        </is>
+      </c>
+      <c r="B103" s="3" t="inlineStr">
+        <is>
+          <t>PS DL</t>
+        </is>
+      </c>
+      <c r="C103" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D103" s="3" t="inlineStr">
+        <is>
+          <t>冒険家エリオットの千年物語</t>
+        </is>
+      </c>
+      <c r="E103" s="3" t="inlineStr">
+        <is>
+          <t>PS5</t>
+        </is>
+      </c>
+      <c r="F103" s="3" t="n"/>
+      <c r="G103" s="3" t="n"/>
+      <c r="H103" s="3" t="n"/>
+      <c r="I103" s="3" t="inlineStr">
+        <is>
+          <t>PS Blog 月間DLランキング(国内PS5) https://blog.ja.playstation.com/2026/07/09/20260709-monthly-ps-store-ranking-s/</t>
+        </is>
+      </c>
+      <c r="J103" s="3" t="inlineStr">
+        <is>
+          <t>HD-2D初の新作アクションRPG。発売初月でDL2位</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="3" t="inlineStr">
+        <is>
+          <t>2026-06 (月間)</t>
+        </is>
+      </c>
+      <c r="B104" s="3" t="inlineStr">
+        <is>
+          <t>PS DL</t>
+        </is>
+      </c>
+      <c r="C104" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D104" s="3" t="inlineStr">
+        <is>
+          <t>EA SPORTS FC 26</t>
+        </is>
+      </c>
+      <c r="E104" s="3" t="inlineStr">
+        <is>
+          <t>PS5</t>
+        </is>
+      </c>
+      <c r="F104" s="3" t="n"/>
+      <c r="G104" s="3" t="n"/>
+      <c r="H104" s="3" t="n"/>
+      <c r="I104" s="3" t="inlineStr">
+        <is>
+          <t>PS Blog 月間DLランキング(国内PS5) https://blog.ja.playstation.com/2026/07/09/20260709-monthly-ps-store-ranking-s/</t>
+        </is>
+      </c>
+      <c r="J104" s="3" t="inlineStr">
+        <is>
+          <t>週間が無いため月間で代替</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
weekly-trends(6genres) update (2026-07-22 12:16)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -2553,7 +2553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4285,6 +4285,174 @@
       <c r="H41" s="5" t="inlineStr">
         <is>
           <t>小説</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Steam上半期売上111億ドル・旧作が収益の8割を占める逆転</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Alinea Analyticsの推計で2026年上半期のSteam総売上は約111億ドル(約1.8兆円)と半期で過去最高。だが構造的に重要なのは内訳で、同年リリース作品の売上比率が2024上半期29%→2025年27%→2026年21%へ低下し、売上の約79%をバックカタログ(旧作)が占めた。牽引役はアジア(特に中国)のプレイヤー増、新作価格の上昇、協力プレイ大作のヒット、独自ランチャーからSteamへ回帰するサードパーティの増加。新作が売れないのではなく、旧作の長期運用(値下げ・大型アップデート・バンドル)が収益源として肥大化し、ヒットの寿命が延びていることを示す。</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Valve(Steam), Alinea Analytics, CD Projekt, Larian</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>ゲーム収益の重心が『新作の初動』から『カタログの長期運用』へ移るバックカタログ経済化。DL販売・恒常セール・実績/MOD・ライブ運営が旧作を「減価しない資産」に変え、パブリッシャーの評価軸をヒット本数から保有IPのストック価値へ移す。音楽の旧譜カタログ売買や映像ライブラリ課金と同型の『所有コンテンツの金融資産化』が進む。</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>評価対象は当年ヒットより保有カタログのLTV。音楽カタログのPE集約、映像ライブラリ課金と重なり、各ジャンルで「旧作の資産運用」競争が本格化する。</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>https://www.gamespark.jp/article/2026/07/11/169133.html / https://pcgamebto.com/steam-2026-h1-sales-ranking/</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>ゲーム</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>法務省が「声の権利」保護を指針化——声優・歌手・俳優を横断</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>法務省は『肖像、声等の無断利用による民事責任の在り方に関する検討会』を設置し、2026年7月13日の会合で、著名人の声も法的保護の対象に含まれるとの見解を近くまとめる指針に盛り込む方針を示した。8月にも公表予定。生成AIで人気声優やアーティストの声を無断で模倣・合成する事例が急増し、現行法では『声の著作権』規定がなくパブリシティ権や不正競争防止法で争わざるを得ない状況が背景にある。声優・歌手・俳優・ナレーターなど『声を資本とする職能』を横断して影響し、AI音声サービスやレーベル、アニメ・ゲーム制作の権利処理実務に波及する。</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>法務省, SAG-AFTRA, ElevenLabs, Suno, Udio, 日本俳優連合</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>生成AIが『声・顔・演技』を低コストで複製可能にしたことで、契約と現場慣行に委ねられてきた実演家の権利が法制度の対象へ格上げされる局面。パブリシティ権(人格権由来)と著作隣接権(実演)の隙間を、AI時代の「合成同一性」がこじ開ける。日本の指針化は、EUのAI Act開示義務や米NO FAKES法案と同じ『合成コンテンツの帰属・同意』潮流の一環。</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>声・肖像の同意と対価処理が、音楽(歌声合成)・アニメ/ゲーム(声優)・映画(俳優)で同時に標準実務化。権利者側の交渉力が高まり、AI合成前提のコスト設計が崩れる。</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>https://www.nikkei.com/article/DGXZQOUA252BN0V20C26A6000000/ / https://gvalaw.jp/blog/h20260527/</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>横断</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>アニメ制作費1話2000万円超・作品間格差の拡大と海外配信依存</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>30分枠TVアニメの制作費は従来1話1000〜1300万円が目安だったが、2000万円超が増え、1クールで2〜5億円規模に達する作品も出ている。日経は『世界人気で制作費高騰、ヒット期待で作品ごとの差も拡大』と報道。要因は作品本数の増えすぎによる人材不足と熟練スタッフの単価上昇、そしてNetflix等の海外配信が関わると国際水準の品質を求められ費用が跳ね上がる点。製作委員会は放送よりBD・グッズ・配信の二次収益を前提とし、特に海外配信権料が高額制作費を支える主柱になっている。結果、潤沢な話題作と薄い量産作の二極化が進む。</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Netflix, Crunchyroll(ソニー), 東映アニメーション, MAPPA, 集英社</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>『本数インフレ→人材希少化→単価高騰→海外配信マネー依存』の循環。製作委員会が国内パッケージ回収型から海外配信権先行回収型へ変質し、配信プラットフォームが事実上の主出資者・編集権者になる。ヒット偏重の予算配分は、少数の高額作品と多数の低予算作品への分岐(映画・ゲームと同じブロックバスター化)を生む。</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>制作費の海外配信依存は、映画のOTT出資回帰やゲームのGaaS投資選別と同型。作品数ではなく「配信で世界に刺さる少数」へ資本が集約する。</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>https://www.nikkei.com/article/DGXZQOUB119920R10C26A6000000/ / https://www.creativevillage.ne.jp/category/skillup/industry-commentary/entertainment/168666/</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>アニメ</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Webtoon世界CAGR30%と日本のLINEマンガ×ピッコマ覇権競争</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>ウェブトゥーン世界市場は2025年約107.5億ドルから2026年約140億ドルへ、CAGR30%超で拡大する見通し。牽引役はスマホ普及、無料話数モデル、韓国コンテンツ輸出。WEBTOON Entertainmentは2024年に物販『WEBTOON Shop』を立ち上げ、アパレルやコレクター版で作家収益とファン接点を多角化する。日本ではNAVER系LINEマンガとカカオ系ピッコマがアプリ首位を争い、投資を背景にシェア競争が新局面に入った。一方、国内では『Webtoonは創作性が足りない』という読者調査もあり、縦読みのフォーマット的強みと読者の物語満足の乖離という課題も残る。</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>NAVER(WEBTOON), カカオ(ピッコマ), LINEヤフー, 集英社</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>縦読み×フルカラー×話単位課金は、単行本前提の日本漫画とは異なる『スマホ最適の連載・課金設計』。プラットフォーム間の資本競争が作品供給と作家囲い込みを加速し、物販・IP化まで垂直統合する。急成長の裏で制作の工業化(分業スタジオ)と作家の交渉力が論点化する。</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>課金モデルと物販統合は音楽サブスク＋D2C、ゲームのサブスク特典と収斂。ARPU向上策が各ジャンルで同じ『サブスク＋物販』設計へ向かう。</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>https://www.gii.co.jp/report/tbrc1969002-webtoons-global-market-report.html / https://premium.kai-you.net/article/892</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>漫画</t>
         </is>
       </c>
     </row>
@@ -43705,7 +43873,11 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="9" t="inlineStr"/>
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
       <c r="B2" s="9" t="inlineStr">
         <is>
           <t>制作現場の人手不足・待遇</t>
@@ -43716,15 +43888,43 @@
           <t>労務</t>
         </is>
       </c>
-      <c r="D2" s="9" t="inlineStr"/>
-      <c r="E2" s="9" t="inlineStr"/>
-      <c r="F2" s="9" t="inlineStr"/>
-      <c r="G2" s="9" t="inlineStr"/>
-      <c r="H2" s="9" t="inlineStr"/>
-      <c r="I2" s="9" t="inlineStr"/>
+      <c r="D2" s="9" t="inlineStr">
+        <is>
+          <t>30分枠1話の制作費が2000万円超も珍しくなくなり、1クール2〜5億円規模に。</t>
+        </is>
+      </c>
+      <c r="E2" s="9" t="inlineStr">
+        <is>
+          <t>本数増による人材不足で熟練スタッフ単価が上昇。ヒット期待で作品間の予算格差が拡大(日経報道)。</t>
+        </is>
+      </c>
+      <c r="F2" s="9" t="inlineStr">
+        <is>
+          <t>東映アニメーション, MAPPA, Netflix</t>
+        </is>
+      </c>
+      <c r="G2" s="9" t="inlineStr">
+        <is>
+          <t>高額話題作と低予算量産作の二極化。待遇改善圧力と海外資本依存が同時進行。</t>
+        </is>
+      </c>
+      <c r="H2" s="9" t="inlineStr">
+        <is>
+          <t>本数インフレが人件費を押し上げる構造。量から『少数精鋭』への資本集約。</t>
+        </is>
+      </c>
+      <c r="I2" s="9" t="inlineStr">
+        <is>
+          <t>https://www.nikkei.com/article/DGXZQOUB119920R10C26A6000000/</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="inlineStr"/>
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
           <t>海外配信収益の比重上昇</t>
@@ -43735,12 +43935,36 @@
           <t>ビジネスモデル</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr"/>
-      <c r="E3" s="9" t="inlineStr"/>
-      <c r="F3" s="9" t="inlineStr"/>
-      <c r="G3" s="9" t="inlineStr"/>
-      <c r="H3" s="9" t="inlineStr"/>
-      <c r="I3" s="9" t="inlineStr"/>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>Netflix等の海外配信権料が高額制作費を支える主柱に。</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>海外配信が関わると国際水準の品質要求で費用が跳ね上がる。製作委員会は国内パッケージ回収型から配信権先行回収型へ変質。</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="inlineStr">
+        <is>
+          <t>Netflix, Crunchyroll(ソニー), 集英社</t>
+        </is>
+      </c>
+      <c r="G3" s="9" t="inlineStr">
+        <is>
+          <t>配信PFが実質的な主出資者・編集権者化。世界独占(委員会レス)作品が増加。</t>
+        </is>
+      </c>
+      <c r="H3" s="9" t="inlineStr">
+        <is>
+          <t>映画のOTT出資回帰と同型。配信で世界に刺さる少数へ資本集約。</t>
+        </is>
+      </c>
+      <c r="I3" s="9" t="inlineStr">
+        <is>
+          <t>https://www.nikkei.com/article/DGXZQOUB119920R10C26A6000000/</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="25" t="n">
@@ -45510,7 +45734,11 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr"/>
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
           <t>アプリ課金モデルの競争</t>
@@ -45521,12 +45749,36 @@
           <t>ビジネスモデル</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr"/>
-      <c r="E4" s="9" t="inlineStr"/>
-      <c r="F4" s="9" t="inlineStr"/>
-      <c r="G4" s="9" t="inlineStr"/>
-      <c r="H4" s="9" t="inlineStr"/>
-      <c r="I4" s="9" t="inlineStr"/>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>日本ではLINEマンガ(NAVER系)とピッコマ(カカオ系)がアプリ首位を争う新局面。</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>Webtoon世界市場はCAGR30%超で拡大。WEBTOON Shopなど物販で作家収益・ファン接点を多角化。</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>NAVER, カカオ, LINEヤフー</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>課金＋物販＋IP化の垂直統合。作品供給と作家囲い込みの競争激化。</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>話単位課金＋D2C物販は音楽サブスク・ゲーム特典と収斂。</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>https://www.gii.co.jp/report/tbrc1969002-webtoons-global-market-report.html</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr"/>
@@ -49341,7 +49593,11 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="9" t="inlineStr"/>
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
       <c r="B2" s="9" t="inlineStr">
         <is>
           <t>Web発小説の書籍化サイクル</t>
@@ -49352,12 +49608,36 @@
           <t>コンテンツ</t>
         </is>
       </c>
-      <c r="D2" s="9" t="inlineStr"/>
-      <c r="E2" s="9" t="inlineStr"/>
-      <c r="F2" s="9" t="inlineStr"/>
-      <c r="G2" s="9" t="inlineStr"/>
-      <c r="H2" s="9" t="inlineStr"/>
-      <c r="I2" s="9" t="inlineStr"/>
+      <c r="D2" s="9" t="inlineStr">
+        <is>
+          <t>2025年の出版市場(紙＋電子)は1兆5462億円で前年比1.6%減、4年連続前年割れ。紙は1975年以来の1兆円割れ。</t>
+        </is>
+      </c>
+      <c r="E2" s="9" t="inlineStr">
+        <is>
+          <t>なろう・カクヨム等のWeb人気作の書籍化が供給の主軸に。オーディオブックとWeb小説がCAGR20%超で成長。</t>
+        </is>
+      </c>
+      <c r="F2" s="9" t="inlineStr">
+        <is>
+          <t>KADOKAWA, TOブックス, 小説家になろう, Audible</t>
+        </is>
+      </c>
+      <c r="G2" s="9" t="inlineStr">
+        <is>
+          <t>紙縮小を電子・音声・Web発が補完。ヒットの発掘が投稿ランキング依存に。</t>
+        </is>
+      </c>
+      <c r="H2" s="9" t="inlineStr">
+        <is>
+          <t>『ながら消費』の音声とWeb連載が紙の減少を吸収する構造転換。</t>
+        </is>
+      </c>
+      <c r="I2" s="9" t="inlineStr">
+        <is>
+          <t>https://hon.jp/news/1.0/0/58293</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="25" t="n">
@@ -51298,8 +51578,10 @@
       <c r="I4" s="9" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="25" t="n">
-        <v>46223</v>
+      <c r="A5" s="25" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
@@ -51313,32 +51595,32 @@
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
-          <t>全否定から『開示して分配から外す』運用フェーズへ移行。EU AI法の透明性義務が8/2適用開始を控え、業界側が先回りして自主ルールを整えた。</t>
+          <t>法務省が『声』を法的保護対象に含める指針を8月にも公表方針(7/13検討会)。</t>
         </is>
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>7月上旬にIFPI/RIAA/レコーディング・アカデミー/A2IM/SAG-AFTRA等が録音物のAI利用ラベル制度で合意。DDEXメタデータに工程単位で機械可読の申告を埋め込む設計。TIDALは7/15からフルAI生成曲の収益化を停止。DeezerはEJIとの提携で人間関与なしの録音にロイヤリティを払わない方針。Spotifyは無許諾ボイスクローン禁止とAI Credits（4月Beta）を実装済み。</t>
+          <t>AIによる声優・歌手の声の無断模倣が急増。Suno/Udioと大手レーベルの訴訟も継続。SpotifyはAI開示のDDEX標準を支持。</t>
         </is>
       </c>
       <c r="F5" s="9" t="inlineStr">
         <is>
-          <t>IFPI, RIAA, SAG-AFTRA, TIDAL, Deezer, Spotify, Suno, Warner Music</t>
+          <t>法務省, Suno, Udio, ElevenLabs, Spotify</t>
         </is>
       </c>
       <c r="G5" s="9" t="inlineStr">
         <is>
-          <t>ラベル有無がロイヤリティプール配分と推薦アルゴリズムの重み付けに直結する『経済的サンクション型』の規制に進む。開示コストを負担できる事業者だけが流通に残り、無申告の大量投稿はスパム扱いで排除される。</t>
+          <t>声・肖像の同意と対価処理が標準実務化。AI合成前提のコスト設計が崩れ、権利者の交渉力上昇。</t>
         </is>
       </c>
       <c r="H5" s="9" t="inlineStr">
         <is>
-          <t>禁止ではなく『申告＋分配除外』という設計はSteamのAI開示欄と同型。是非論より運用設計の巧拙が競争要因になった。</t>
+          <t>音楽・アニメ/ゲーム声優・映画俳優を横断する『合成同一性』の権利化。</t>
         </is>
       </c>
       <c r="I5" s="9" t="inlineStr">
         <is>
-          <t>https://deadline.com/2026/07/music-ai-labels-recording-industry-1236979107/</t>
+          <t>https://www.nikkei.com/article/DGXZQOUA252BN0V20C26A6000000/</t>
         </is>
       </c>
     </row>
@@ -55690,7 +55972,7 @@
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
@@ -55705,32 +55987,32 @@
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>『Palworld 1.0』が7/10ローンチで同接855Kを記録、Palworld無印と1.0が揃ってSteam歴代best-everプレイヤー数リストに入る事態。</t>
+          <t>2026年上半期のSteam総売上は約111億ドル(約1.8兆円)で半期過去最高。</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>490K(初日)→720K(7/11)→850K超(7/12-13)と週末にかけ増勢。累計4000万本・価格据え置き・既存所有者無償が好評を後押し。別途『Artifact Classic』が明確な理由なく約1万同接へ約100倍スパイクする謎現象も観測。</t>
+          <t>同年新作の売上比率が21%まで低下し、旧作(バックカタログ)が約79%を占める逆転。アジア(中国)のプレイヤー増と独自ランチャーからの回帰が寄与。</t>
         </is>
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t>Valve, Pocketpair</t>
+          <t>Valve, Alinea Analytics</t>
         </is>
       </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
-          <t>EA卒業タイトルの『二度目の全盛期』設計がPCの定番戦術に。旧作の突発再燃はディスカバリー/ボット/投機いずれかの兆候として要監視。</t>
+          <t>恒常セール・大型アップデートでヒットの寿命が延び、保有カタログのLTVが評価軸に。新作は価格上昇で単価回収へ。</t>
         </is>
       </c>
       <c r="H11" s="9" t="inlineStr">
         <is>
-          <t>Steamの同接ランキングは新作より『再点火』が席巻。ピークでなく持続曲線が資産価値を決める局面。</t>
+          <t>収益の重心が『初動』から『カタログ運用』へ。音楽旧譜・映像ライブラリと同じ資産化。</t>
         </is>
       </c>
       <c r="I11" s="9" t="inlineStr">
         <is>
-          <t>https://www.forbes.com/sites/paultassi/2026/07/11/both-palworld-and-palworld-10-are-in-steams-best-ever-playercount-list/</t>
+          <t>https://www.gamespark.jp/article/2026/07/11/169133.html</t>
         </is>
       </c>
       <c r="J11" s="9" t="inlineStr"/>

</xml_diff>

<commit_message>
weekly-releases(6genres) + indie + rankings update (2026-07-25 00:25)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -9213,7 +9213,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J104"/>
+  <dimension ref="A1:J119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12932,6 +12932,552 @@
       <c r="J104" s="3" t="inlineStr">
         <is>
           <t>週間が無いため月間で代替</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-07-13〜07-19</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C105" t="n">
+        <v>1</v>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>リズム天国 ミラクルスターズ</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Switch</t>
+        </is>
+      </c>
+      <c r="F105" t="n">
+        <v>76786</v>
+      </c>
+      <c r="G105" t="n">
+        <v>596237</v>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/article/202607/82215</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>3週連続首位=リズム天国。ハード週販 Switch2 24,928台/Switch 6,396台。6-10位は今回未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-07-13〜07-19</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C106" t="n">
+        <v>2</v>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>プロ野球スピリッツ2026</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>PS5</t>
+        </is>
+      </c>
+      <c r="F106" t="n">
+        <v>20661</v>
+      </c>
+      <c r="G106" t="n">
+        <v>20661</v>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/article/202607/82215</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>3週連続首位=リズム天国。ハード週販 Switch2 24,928台/Switch 6,396台。6-10位は今回未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-07-13〜07-19</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C107" t="n">
+        <v>3</v>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>トモダチコレクション わくわく生活</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Switch</t>
+        </is>
+      </c>
+      <c r="F107" t="n">
+        <v>18608</v>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/article/202607/82215</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>3週連続首位=リズム天国。ハード週販 Switch2 24,928台/Switch 6,396台。6-10位は今回未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026-07-13〜07-19</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C108" t="n">
+        <v>4</v>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>亰都ザナドゥ -桜花幻舞-</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Switch</t>
+        </is>
+      </c>
+      <c r="F108" t="n">
+        <v>15431</v>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/article/202607/82215</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>3週連続首位=リズム天国。ハード週販 Switch2 24,928台/Switch 6,396台。6-10位は今回未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2026-07-13〜07-19</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C109" t="n">
+        <v>5</v>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>亰都ザナドゥ -桜花幻舞-</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>PS5</t>
+        </is>
+      </c>
+      <c r="F109" t="n">
+        <v>13206</v>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/article/202607/82215</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>3週連続首位=リズム天国。ハード週販 Switch2 24,928台/Switch 6,396台。6-10位は今回未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-07-13〜07-19</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C110" t="n">
+        <v>1</v>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Counter-Strike 2（カウンターストライク2）</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>https://www.gamegrin.com/news/weekly-top-selling-games-on-steam-13th19th-of-july-2026</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>売上高ベース（Valve公式）。CS2が首位返り咲き</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-07-13〜07-19</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C111" t="n">
+        <v>2</v>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Assassin's Creed Black Flag Resynced（アサシン クリード ブラックフラッグ リシンクド）</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>https://www.gamegrin.com/news/weekly-top-selling-games-on-steam-13th19th-of-july-2026</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>売上高ベース（Valve公式）。CS2が首位返り咲き</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026-07-13〜07-19</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C112" t="n">
+        <v>3</v>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Steam Machine（スチームマシン／ハード）</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>https://www.gamegrin.com/news/weekly-top-selling-games-on-steam-13th19th-of-july-2026</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>売上高ベース（Valve公式）。CS2が首位返り咲き</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2026-07-13〜07-19</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C113" t="n">
+        <v>4</v>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Palworld（パルワールド）</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>https://www.gamegrin.com/news/weekly-top-selling-games-on-steam-13th19th-of-july-2026</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>売上高ベース（Valve公式）。CS2が首位返り咲き</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2026-07-13〜07-19</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C114" t="n">
+        <v>5</v>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Dota 2（ドータ2）</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>https://www.gamegrin.com/news/weekly-top-selling-games-on-steam-13th19th-of-july-2026</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>売上高ベース（Valve公式）。CS2が首位返り咲き</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2026-07-13〜07-19</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C115" t="n">
+        <v>6</v>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>MECCHA CHAMELEON（メチャ・カメレオン）</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>https://www.gamegrin.com/news/weekly-top-selling-games-on-steam-13th19th-of-july-2026</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>売上高ベース（Valve公式）。CS2が首位返り咲き</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026-07-13〜07-19</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C116" t="n">
+        <v>7</v>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>PUBG: BATTLEGROUNDS（パブジー）</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>https://www.gamegrin.com/news/weekly-top-selling-games-on-steam-13th19th-of-july-2026</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>売上高ベース（Valve公式）。CS2が首位返り咲き</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2026-07-13〜07-19</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C117" t="n">
+        <v>8</v>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Warframe（ウォーフレーム）</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>https://www.gamegrin.com/news/weekly-top-selling-games-on-steam-13th19th-of-july-2026</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>売上高ベース（Valve公式）。CS2が首位返り咲き</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2026-07-13〜07-19</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C118" t="n">
+        <v>9</v>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Marvel Rivals（マーベル・ライバルズ）</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>https://www.gamegrin.com/news/weekly-top-selling-games-on-steam-13th19th-of-july-2026</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>売上高ベース（Valve公式）。CS2が首位返り咲き</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2026-07-13〜07-19</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C119" t="n">
+        <v>10</v>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Apex Legends（エーペックスレジェンズ）</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>https://www.gamegrin.com/news/weekly-top-selling-games-on-steam-13th19th-of-july-2026</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>売上高ベース（Valve公式）。CS2が首位返り咲き</t>
         </is>
       </c>
     </row>
@@ -42274,7 +42820,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -42671,6 +43217,46 @@
       <c r="M9" t="inlineStr">
         <is>
           <t>https://eiga.com/ranking/jp/</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>超宇宙刑事ギャバン インフィニティ 太陽が泣いた日</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>東映</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>日本</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>特撮/SFアクション</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>2</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>メタルヒーローシリーズ「宇宙刑事ギャバン」劇場版。国内興行は7/17-19「キングダム 魂の決戦」が初登場首位（初動3日15.84億円/99.3万人）</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>https://cinemore.jp/jp/news-feature/4648/article_p1.html</t>
         </is>
       </c>
     </row>
@@ -46124,7 +46710,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -46234,6 +46820,54 @@
       <c r="K2" t="inlineStr">
         <is>
           <t>https://www.oricon.co.jp/rank/obc/w/2026-07-20/</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ONE PIECE（ワンピース）</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>尾田栄一郎</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>集英社</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>週刊少年ジャンプ</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>115</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>オリコン週間コミック1位（7/6-12、2週連続）</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>5</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>最新115巻がオリコン週間コミック首位を継続。上半期は114巻が歴代自己記録を更新</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>https://booklog.jp/hon/ranking/weekly-20260715</t>
         </is>
       </c>
     </row>
@@ -46552,7 +47186,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M48"/>
+  <dimension ref="A1:M49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -48018,12 +48652,15 @@
           <t>三人称アクションADV</t>
         </is>
       </c>
+      <c r="G31" t="n">
+        <v>81</v>
+      </c>
       <c r="K31" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>来週〜今月後半予定（評価系空欄）。シリーズ初スピンオフでSwitch 2専用。単独プレイ＋最大4人協力。すりみ連合(シヴァ/フウカ/マンタロー)と遺物探索。</t>
+          <t>2026-07-23発売。対人戦なしのスプラ派生ルートシューターとして海外レビュー高評価（Metacritic81/67レビュー、「Borderlands×DOOM」的と評される）。発売前登録行を実績で更新</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -48799,6 +49436,51 @@
       <c r="M48" t="inlineStr">
         <is>
           <t>https://gamebiz.jp/news/429601</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>ビースト・オブ・リィンカーネーション（Beast of Reincarnation）</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>ゲームフリーク（GAME FREAK）</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Happinet／Fictions</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>PS5/Xbox/PC(Steam)</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>アクションRPG</t>
+        </is>
+      </c>
+      <c r="K49" t="n">
+        <v>4</v>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>【来月分】ゲームフリーク完全新作IP。西暦4026年の終末後の日本を舞台に、少女エマと犬の冒険を描く。パリィ×コマンドのバトル</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/918/G091816/20260213002/</t>
         </is>
       </c>
     </row>
@@ -51925,7 +52607,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -52085,6 +52767,44 @@
       <c r="K3" t="inlineStr">
         <is>
           <t>https://www.billboard.com/charts/hot-100/</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-07-22（付）</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>チャート</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>（Billboard JAPAN Hot 100 第1位）</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Number_i</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" t="n">
+        <v>4</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>総合ソングチャート首位。2位 Mrs. GREEN APPLE / 3位 NCT WISH / 4位 FRUITS ZIPPER / 5位 米津玄師</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>https://www.billboard-japan.com/charts/detail?a=hot100</t>
         </is>
       </c>
     </row>
@@ -56921,7 +57641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -57687,6 +58407,53 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>MECCHA CHAMELEON（メチャ・カメレオン）</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>lemorion_1224（個人開発）</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2026-06-09 配信</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>カジュアル/パーティ</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Steam週間トップセラーに数週定着（7/13-19は6位）。実況・パーティ配信で継続的に話題</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Steam週間トップセラー上位常連</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>個人開発のパーティゲームがAAA・大手作に混じってトップセラー上位を維持</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
daily-news(6genres) + cross-questions + media-mix + events + predictions update (2026-07-24)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -891,7 +891,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H40"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2579,6 +2579,48 @@
         </is>
       </c>
       <c r="H40" s="15" t="inlineStr">
+        <is>
+          <t>横断</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B41" s="14" t="inlineStr">
+        <is>
+          <t>キャラ強・物語希薄IP（ちいかわ型）の劇場化が成功すると、配給・出版・玩具側が映画を『物販の販促装置』と再定義し、興収シェア型でなくライセンス/物販レベニューシェア型の配給契約を求める動きが出る</t>
+        </is>
+      </c>
+      <c r="C41" s="14" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="D41" s="14" t="inlineStr">
+        <is>
+          <t>6〜18ヶ月</t>
+        </is>
+      </c>
+      <c r="E41" s="14" t="inlineStr">
+        <is>
+          <t>Cygames, 東宝, キャラIPホルダー</t>
+        </is>
+      </c>
+      <c r="F41" s="14" t="inlineStr">
+        <is>
+          <t>『映画ちいかわ 人魚の島のひみつ』7/24公開・380館・上映回数大作級（映画.com/マグミクス, 7/24）</t>
+        </is>
+      </c>
+      <c r="G41" s="14" t="inlineStr">
+        <is>
+          <t>ちいかわ映画の物販売上と興収の比率、今後のキャラIP映画で配給契約に物販/ライセンス連動条項が入るかを観測</t>
+        </is>
+      </c>
+      <c r="H41" s="14" t="inlineStr">
         <is>
           <t>横断</t>
         </is>
@@ -5535,7 +5577,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H87"/>
+  <dimension ref="A1:H89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9197,6 +9239,90 @@
         </is>
       </c>
       <c r="H87" s="15" t="inlineStr">
+        <is>
+          <t>横断</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B88" s="14" t="inlineStr">
+        <is>
+          <t>Xboxが不採算スタジオを『閉鎖』でなく『IP保持付き独立』で手放した動きは、アニメ制作会社や映画スタジオの整理でも『独立＋原作/IP保有』型の切り離しとして波及するか？</t>
+        </is>
+      </c>
+      <c r="C88" s="14" t="inlineStr">
+        <is>
+          <t>Xbox大再編でCompulsion・Double Fineが独立、全IP保持（Push Square, 7/24）</t>
+        </is>
+      </c>
+      <c r="D88" s="14" t="inlineStr">
+        <is>
+          <t>Microsoft/Xbox, Compulsion, Double Fine</t>
+        </is>
+      </c>
+      <c r="E88" s="14" t="inlineStr">
+        <is>
+          <t>アニメ制作会社の元請け独立、映画スタジオのスピンオフ、出版の編集部MBO</t>
+        </is>
+      </c>
+      <c r="F88" s="14" t="inlineStr">
+        <is>
+          <t>オープン</t>
+        </is>
+      </c>
+      <c r="G88" s="14" t="inlineStr">
+        <is>
+          <t>閉鎖=資産死蔵に対し、IP付き独立=人材とIPを生かす手放し方。エンタメ各所のリストラ設計に応用余地</t>
+        </is>
+      </c>
+      <c r="H88" s="14" t="inlineStr">
+        <is>
+          <t>横断</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B89" s="14" t="inlineStr">
+        <is>
+          <t>フェスのライブ配信を単一プラットフォームが全世界無料独占する動き（フジロック×Amazon）は、ゲームのショーケースやアニメイベントの配信独占にも広がり、興行の主導権が主催からPFへ移るか？</t>
+        </is>
+      </c>
+      <c r="C89" s="14" t="inlineStr">
+        <is>
+          <t>フジロック'26、Amazonが全世界無料独占ライブ配信（About Amazon, 7/24）</t>
+        </is>
+      </c>
+      <c r="D89" s="14" t="inlineStr">
+        <is>
+          <t>Amazon, スマッシュ, バンダイナムコ(ガンダムch)</t>
+        </is>
+      </c>
+      <c r="E89" s="14" t="inlineStr">
+        <is>
+          <t>ゲームショーケース配信権、アニメイベント配信、スポーツ放映権</t>
+        </is>
+      </c>
+      <c r="F89" s="14" t="inlineStr">
+        <is>
+          <t>オープン</t>
+        </is>
+      </c>
+      <c r="G89" s="14" t="inlineStr">
+        <is>
+          <t>ガンダム新作もYouTube全世界同時発表。ライブ/イベントの露出とデータがPFに集約される共通構造</t>
+        </is>
+      </c>
+      <c r="H89" s="14" t="inlineStr">
         <is>
           <t>横断</t>
         </is>
@@ -13492,7 +13618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:J33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15052,6 +15178,110 @@
       <c r="J31" s="15" t="inlineStr">
         <is>
           <t>2026-07-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B32" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="C32" s="14" t="inlineStr">
+        <is>
+          <t>FUJI ROCK FESTIVAL '26</t>
+        </is>
+      </c>
+      <c r="D32" s="14" t="inlineStr">
+        <is>
+          <t>ライブ・フェス</t>
+        </is>
+      </c>
+      <c r="E32" s="14" t="inlineStr">
+        <is>
+          <t>新潟・苗場スキー場</t>
+        </is>
+      </c>
+      <c r="F32" s="14" t="inlineStr">
+        <is>
+          <t>リアル＋配信(Amazon独占)</t>
+        </is>
+      </c>
+      <c r="G32" s="14" t="inlineStr">
+        <is>
+          <t>The xx・Khruangbin・藤井風・XG等70組超。Amazon Music/Prime Video/Twitchで全世界無料独占ライブ配信（Prime非会員も視聴可）</t>
+        </is>
+      </c>
+      <c r="H32" s="14" t="inlineStr">
+        <is>
+          <t>https://www.aboutamazon.jp/news/entertainment/fuji-rock-festival-26%E3%82%92prime-video%E3%81%A8twitch%E3%81%A7%E7%8B%AC%E5%8D%A0%E3%83%A9%E3%82%A4%E3%83%96%E9%85%8D%E4%BF%A1</t>
+        </is>
+      </c>
+      <c r="I32" s="14" t="inlineStr">
+        <is>
+          <t>開催中</t>
+        </is>
+      </c>
+      <c r="J32" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B33" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="C33" s="14" t="inlineStr">
+        <is>
+          <t>サンディエゴ・コミコン2026 (SDCC)</t>
+        </is>
+      </c>
+      <c r="D33" s="14" t="inlineStr">
+        <is>
+          <t>展示会</t>
+        </is>
+      </c>
+      <c r="E33" s="14" t="inlineStr">
+        <is>
+          <t>米・サンディエゴ</t>
+        </is>
+      </c>
+      <c r="F33" s="14" t="inlineStr">
+        <is>
+          <t>リアル</t>
+        </is>
+      </c>
+      <c r="G33" s="14" t="inlineStr">
+        <is>
+          <t>ガンダム新作『RG XARX-ZERO』等のパネル解禁。映画・アニメ・コミックの北米向け大型発表の場</t>
+        </is>
+      </c>
+      <c r="H33" s="14" t="inlineStr">
+        <is>
+          <t>https://www.comic-con.org/</t>
+        </is>
+      </c>
+      <c r="I33" s="14" t="inlineStr">
+        <is>
+          <t>開催中</t>
+        </is>
+      </c>
+      <c r="J33" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
         </is>
       </c>
     </row>
@@ -18544,7 +18774,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M363"/>
+  <dimension ref="A1:M389"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -42808,6 +43038,1738 @@
         </is>
       </c>
       <c r="M363" s="15" t="inlineStr"/>
+    </row>
+    <row r="364">
+      <c r="A364" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B364" s="14" t="inlineStr">
+        <is>
+          <t>ゲーム</t>
+        </is>
+      </c>
+      <c r="C364" s="14" t="inlineStr">
+        <is>
+          <t>Xbox大再編でCompulsion・Double Fineが独立、全IP＋カタログ収益を保持</t>
+        </is>
+      </c>
+      <c r="D364" s="14" t="inlineStr">
+        <is>
+          <t>https://www.pushsquare.com/news/2026/07/newly-independent-devs-thank-xbox-and-keep-ip-rights-to-their-games</t>
+        </is>
+      </c>
+      <c r="E364" s="14" t="inlineStr">
+        <is>
+          <t>MicrosoftはXbox部門で約3,200人規模の人員削減と組織再編を発表。その一環でCompulsion Games（South of Midnight等）とDouble Fine（Psychonauts等）がXboxから離れ独立スタジオへ移行した。両社は閉鎖ではなく独立という形での送り出しにXboxへ謝意を表明している。</t>
+        </is>
+      </c>
+      <c r="F364" s="14" t="inlineStr">
+        <is>
+          <t>注目は撤退の『形式』。両スタジオは自社IP・バックカタログ・そこから生じる将来収益をすべて保持したまま独立する。大量リストラの局面で親会社が『閉鎖して資産だけ残す』のではなく『IPごと切り離す』選択を取った点が、従来の即時清算型リストラと異なる新しいパターンを示す。</t>
+        </is>
+      </c>
+      <c r="G364" s="14" t="inlineStr">
+        <is>
+          <t>3,200人規模の削減を伴うXbox再編の一環
+閉鎖ではなくIP保持付きの独立という手放し方
+Double FineはPsychonauts/Keeper/Kilnを、CompulsionはWe Happy Few/South of Midnightを保有
+熟練スタジオの人材・IPが社外に流出する構図</t>
+        </is>
+      </c>
+      <c r="H364" s="14" t="inlineStr">
+        <is>
+          <t>IP付き独立が標準化すれば、旧親会社はパブリッシング・流通マージンだけを取り込む垂直分業に向かい、中規模スタジオの新設が増える可能性。放出されたIPが他パブリッシャーとの新契約で復活する動きも予想される。</t>
+        </is>
+      </c>
+      <c r="I364" s="14" t="inlineStr">
+        <is>
+          <t>大手リストラの形態変化とIP資産の帰属</t>
+        </is>
+      </c>
+      <c r="J364" s="14" t="inlineStr">
+        <is>
+          <t>Microsoft, Xbox Game Studios, Compulsion Games, Double Fine</t>
+        </is>
+      </c>
+      <c r="K364" s="14" t="inlineStr">
+        <is>
+          <t>Psychonauts, South of Midnight, We Happy Few</t>
+        </is>
+      </c>
+      <c r="L364" s="14" t="inlineStr">
+        <is>
+          <t>人事・組織,トレンド,海外,権利・ライセンス</t>
+        </is>
+      </c>
+      <c r="M364" s="14" t="inlineStr">
+        <is>
+          <t>SDCC/夏の再編報道に連動</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B365" s="14" t="inlineStr">
+        <is>
+          <t>ゲーム</t>
+        </is>
+      </c>
+      <c r="C365" s="14" t="inlineStr">
+        <is>
+          <t>Hasbro、$56M減損で複数ゲーム中止——「少数精鋭」デジタル戦略へ</t>
+        </is>
+      </c>
+      <c r="D365" s="14" t="inlineStr">
+        <is>
+          <t>https://www.gamedeveloper.com/business/hasbro-records-56m-write-down-after-scrapping-several-video-games</t>
+        </is>
+      </c>
+      <c r="E365" s="14" t="inlineStr">
+        <is>
+          <t>Hasbroは6/28締めのQ2決算で、2028年以降に予定していた複数のビデオゲームを中止し5,600万ドルの非現金減損を計上したと明かした。CEOのChris Cocksは中止タイトル名を明言していないが、フォーカス/コスト規律/自社プラットフォーム/パートナーシップの4方針でデジタル事業を絞る。</t>
+        </is>
+      </c>
+      <c r="F365" s="14" t="inlineStr">
+        <is>
+          <t>D&amp;D等の強IPを抱えつつ、Hasbroは『数を絞り大型に集中』へ転換。Exodusと2027年予定のWarlock（D&amp;D世界）は開発継続する一方、非中核プロジェクトを整理した。ライセンスIPホルダーがゲーム事業をポートフォリオ管理し、外部委託を絞り込む動きの一例。</t>
+        </is>
+      </c>
+      <c r="G365" s="14" t="inlineStr">
+        <is>
+          <t>Q2（6/28締め）で$56M非現金減損
+2028年以降予定の複数タイトルを中止
+『fewer, bigger』のデジタル戦略へ
+Exodus・Warlock（D&amp;D）は開発継続</t>
+        </is>
+      </c>
+      <c r="H365" s="14" t="inlineStr">
+        <is>
+          <t>IPホルダーが外部ライセンシーへの発注を絞ると、D&amp;D系ゲームを手掛けてきた中小スタジオが案件を失う。Hasbroは自社/少数の重点パートナーに資源を集約し、当たり外れの大きい多点張りから撤退する流れが続く見込み。</t>
+        </is>
+      </c>
+      <c r="I365" s="14" t="inlineStr">
+        <is>
+          <t>IPホルダーのゲーム内製・外注ポートフォリオ戦略</t>
+        </is>
+      </c>
+      <c r="J365" s="14" t="inlineStr">
+        <is>
+          <t>Hasbro, Wizards of the Coast</t>
+        </is>
+      </c>
+      <c r="K365" s="14" t="inlineStr">
+        <is>
+          <t>Dungeons &amp; Dragons, Exodus, Warlock</t>
+        </is>
+      </c>
+      <c r="L365" s="14" t="inlineStr">
+        <is>
+          <t>適時開示,業績,海外,権利・ライセンス</t>
+        </is>
+      </c>
+      <c r="M365" s="14" t="inlineStr"/>
+    </row>
+    <row r="366">
+      <c r="A366" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B366" s="14" t="inlineStr">
+        <is>
+          <t>ゲーム</t>
+        </is>
+      </c>
+      <c r="C366" s="14" t="inlineStr">
+        <is>
+          <t>Xbox、PC向け後方互換を投入——ハード境界を溶かす『どこでもプレイ』戦略</t>
+        </is>
+      </c>
+      <c r="D366" s="14" t="inlineStr">
+        <is>
+          <t>https://www.gamedeveloper.com/console/microsoft-launches-xbox-backward-compatibility-for-pc</t>
+        </is>
+      </c>
+      <c r="E366" s="14" t="inlineStr">
+        <is>
+          <t>MicrosoftはXboxの後方互換をPCへ拡張し、旧世代Xboxタイトルの一部をPCでプレイ可能にする取り組みを始めた。Game Passとの連動を含め、Xboxを『専用機』から『どの端末でも動くサービス層』へ再定義する動きの延長にある。</t>
+        </is>
+      </c>
+      <c r="F366" s="14" t="inlineStr">
+        <is>
+          <t>注目はハード事業の位置づけの変化。後方互換をPCに広げることは、専用ハードの独自価値よりもライブラリ／サブスク／クロス端末の継続利用を重視する戦略の表れ。ハードで囲い込む発想から、サービスとカタログで囲い込む発想への転換を示す。</t>
+        </is>
+      </c>
+      <c r="G366" s="14" t="inlineStr">
+        <is>
+          <t>旧世代Xboxタイトルの一部をPCで実行可能に
+Game Pass・クラウドとあわせた端末横断戦略
+専用ハードの独自価値低下という論点
+ソニー・任天堂の専用機モデルとの対比</t>
+        </is>
+      </c>
+      <c r="H366" s="14" t="inlineStr">
+        <is>
+          <t>『どこでもプレイ』が進むほどXbox専用機の販売意義は薄れ、Microsoftはハード販売より月額課金とライブラリ規模で競う。専用機に固執するソニー/任天堂との戦略分岐がさらに鮮明になる。</t>
+        </is>
+      </c>
+      <c r="I366" s="14" t="inlineStr">
+        <is>
+          <t>ハード事業のサービス化とクロスプラットフォーム戦略</t>
+        </is>
+      </c>
+      <c r="J366" s="14" t="inlineStr">
+        <is>
+          <t>Microsoft, Xbox</t>
+        </is>
+      </c>
+      <c r="K366" s="14" t="inlineStr">
+        <is>
+          <t>Xbox Game Pass</t>
+        </is>
+      </c>
+      <c r="L366" s="14" t="inlineStr">
+        <is>
+          <t>ハード,クラウド,トレンド,海外</t>
+        </is>
+      </c>
+      <c r="M366" s="14" t="inlineStr"/>
+    </row>
+    <row r="367">
+      <c r="A367" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B367" s="14" t="inlineStr">
+        <is>
+          <t>ゲーム</t>
+        </is>
+      </c>
+      <c r="C367" s="14" t="inlineStr">
+        <is>
+          <t>Bethesda『Fallout 5』プリプロ入りを明言——TES6と共通の新エンジンCreation Engine 3</t>
+        </is>
+      </c>
+      <c r="D367" s="14" t="inlineStr">
+        <is>
+          <t>https://bethesda.net/en/article/7wrffyXajE4BmCLJVpOkcN/a-note-from-bethesda-game-studios</t>
+        </is>
+      </c>
+      <c r="E367" s="14" t="inlineStr">
+        <is>
+          <t>Bethesda Game Studiosが公式に『Fallout 5は現在プリプロダクション段階』と表明。The Elder Scrolls VIとFallout 5はともにStarfield以降構築してきた共有技術基盤『Creation Engine 3』で開発されると説明した。</t>
+        </is>
+      </c>
+      <c r="F367" s="14" t="inlineStr">
+        <is>
+          <t>注目は個別タイトルより開発基盤の共通化。2本の看板RPGを単一の刷新エンジンに載せることで、ツール・アセット・ノウハウを横断利用しリリース間隔を詰める狙い。大作RPGの長期開発コストに対する『共通基盤で回収』というスタジオ戦略が読める。</t>
+        </is>
+      </c>
+      <c r="G367" s="14" t="inlineStr">
+        <is>
+          <t>Fallout 5はプリプロ段階と公式表明
+TES6と共通のCreation Engine 3で開発
+Starfield以降に構築した共有技術基盤
+大作RPGの開発期間短縮を狙う</t>
+        </is>
+      </c>
+      <c r="H367" s="14" t="inlineStr">
+        <is>
+          <t>共通エンジン化が奏功すればMicrosoft傘下のBethesdaは大型RPGの供給ペースを上げられる。逆にエンジン刷新が難航すればTES6・Fallout 5双方の遅延リスクが連動する構造にもなる。</t>
+        </is>
+      </c>
+      <c r="I367" s="14" t="inlineStr">
+        <is>
+          <t>大作RPGの共通エンジン戦略と開発効率</t>
+        </is>
+      </c>
+      <c r="J367" s="14" t="inlineStr">
+        <is>
+          <t>Bethesda Game Studios, Microsoft</t>
+        </is>
+      </c>
+      <c r="K367" s="14" t="inlineStr">
+        <is>
+          <t>Fallout 5, The Elder Scrolls VI, Starfield</t>
+        </is>
+      </c>
+      <c r="L367" s="14" t="inlineStr">
+        <is>
+          <t>技術,新作,海外</t>
+        </is>
+      </c>
+      <c r="M367" s="14" t="inlineStr"/>
+    </row>
+    <row r="368">
+      <c r="A368" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B368" s="14" t="inlineStr">
+        <is>
+          <t>ゲーム</t>
+        </is>
+      </c>
+      <c r="C368" s="14" t="inlineStr">
+        <is>
+          <t>Steam、2026上半期リリースが1.2万本超——7年連続で最多更新ペース＝供給過多鮮明</t>
+        </is>
+      </c>
+      <c r="D368" s="14" t="inlineStr">
+        <is>
+          <t>https://automaton-media.com/articles/newsjp/steam-20260703-453117/</t>
+        </is>
+      </c>
+      <c r="E368" s="14" t="inlineStr">
+        <is>
+          <t>AUTOMATONによれば、2026年にSteamで配信されたゲームは7月初旬（上半期終了）時点で1万2,000本超に達し、7年連続で年間最多本数を更新するペース。折り返し時点でこの水準という供給量の多さが際立つ。</t>
+        </is>
+      </c>
+      <c r="F368" s="14" t="inlineStr">
+        <is>
+          <t>1タイトルの話題ではなく市場構造の話。リリース数の指数的増加は、可処分時間と注目の奪い合いを激化させ、発見性（ディスカバラビリティ）の低下と個別タイトルの埋没を招く。『作れば売れる』が一段と成立しにくい環境で、マーケ・コミュニティ設計の重みが増す消費者行動トレンドの検証材料。</t>
+        </is>
+      </c>
+      <c r="G368" s="14" t="inlineStr">
+        <is>
+          <t>上半期で1.2万本超、7年連続最多更新ペース
+供給過多による発見性の低下
+注目・可処分時間の奪い合いが激化
+インディーの埋没リスク増大</t>
+        </is>
+      </c>
+      <c r="H368" s="14" t="inlineStr">
+        <is>
+          <t>供給過多が続くと、Steam内キュレーション/ウィッシュリスト/デモ（Next Fest）の重要性が一段と高まり、露出を握るプラットフォーム機能に開発側が従属する構図が強まる。中小は発売前コミュニティ形成の巧拙で明暗が分かれる。</t>
+        </is>
+      </c>
+      <c r="I368" s="14" t="inlineStr">
+        <is>
+          <t>プラットフォームの供給過多と発見性設計</t>
+        </is>
+      </c>
+      <c r="J368" s="14" t="inlineStr">
+        <is>
+          <t>Valve</t>
+        </is>
+      </c>
+      <c r="K368" s="14" t="inlineStr">
+        <is>
+          <t>Steam</t>
+        </is>
+      </c>
+      <c r="L368" s="14" t="inlineStr">
+        <is>
+          <t>インディー,トレンド,消費者インサイト,海外</t>
+        </is>
+      </c>
+      <c r="M368" s="14" t="inlineStr"/>
+    </row>
+    <row r="369">
+      <c r="A369" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B369" s="14" t="inlineStr">
+        <is>
+          <t>映画</t>
+        </is>
+      </c>
+      <c r="C369" s="14" t="inlineStr">
+        <is>
+          <t>『映画ちいかわ 人魚の島のひみつ』7/24公開・380館——キャラIP発の劇場化という新収益導線</t>
+        </is>
+      </c>
+      <c r="D369" s="14" t="inlineStr">
+        <is>
+          <t>https://eiga.com/movie/105109/</t>
+        </is>
+      </c>
+      <c r="E369" s="14" t="inlineStr">
+        <is>
+          <t>ナガノのWEB漫画『ちいかわ』初の劇場版が7/24に全国380館規模で公開。原作でも人気の『セイレーン編』を映像化し、監督は及川啓、アニメーション制作はCygamesPictures。上映回数が『鬼滅』『コナン』級との報道も出ている。</t>
+        </is>
+      </c>
+      <c r="F369" s="14" t="inlineStr">
+        <is>
+          <t>数字より示唆で拾う一件。物語牽引よりキャラクター・世界観への愛着で拡大した『ちいかわ』が、グッズ・コラボに続き劇場を新たな収益導線に据えた。ストーリー希薄・キャラ強のIPでも大規模劇場展開が成立するかを検証する、キャラIPマネタイズの試金石。</t>
+        </is>
+      </c>
+      <c r="G369" s="14" t="inlineStr">
+        <is>
+          <t>WEB漫画発キャラIPの初劇場版
+全国380館・上映回数は大作級との報道
+制作はCygamesPictures、監督及川啓
+キャラ強・物語希薄IPの劇場適性を測る事例</t>
+        </is>
+      </c>
+      <c r="H369" s="14" t="inlineStr">
+        <is>
+          <t>興行が成立すれば、キャラIPホルダーは映画を『物販の販促装置＋新規収益』と位置づけ、キャラ先行IPの劇場化が増える。配給契約でも興収シェア型に加えライセンス/物販レベニューシェア型の条件が交渉されやすくなる。</t>
+        </is>
+      </c>
+      <c r="I369" s="14" t="inlineStr">
+        <is>
+          <t>キャラクターIPの劇場化とマネタイズ設計</t>
+        </is>
+      </c>
+      <c r="J369" s="14" t="inlineStr">
+        <is>
+          <t>Cygames, CygamesPictures, 東宝</t>
+        </is>
+      </c>
+      <c r="K369" s="14" t="inlineStr">
+        <is>
+          <t>ちいかわ</t>
+        </is>
+      </c>
+      <c r="L369" s="14" t="inlineStr">
+        <is>
+          <t>興行,映像化,消費者インサイト,国内</t>
+        </is>
+      </c>
+      <c r="M369" s="14" t="inlineStr">
+        <is>
+          <t>メディアミックス追跡にも登録</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B370" s="14" t="inlineStr">
+        <is>
+          <t>映画</t>
+        </is>
+      </c>
+      <c r="C370" s="14" t="inlineStr">
+        <is>
+          <t>ディズニー『モアナ』実写リメイク、公開前トラッキングで苦戦観測——実写化路線に黄信号</t>
+        </is>
+      </c>
+      <c r="D370" s="14" t="inlineStr">
+        <is>
+          <t>https://variety.com/2026/film/box-office/moana-remake-box-office-opening-weekend-tracking-1236803797/</t>
+        </is>
+      </c>
+      <c r="E370" s="14" t="inlineStr">
+        <is>
+          <t>Varietyの興行トラッキング記事は、ディズニーの『モアナ』実写リメイクがオープニング週末に向け想定を下回りかねない（choppy waters＝難航）との観測を伝えた。近年の同社実写リメイク群の成績ばらつきを背景にした慎重な見立て。</t>
+        </is>
+      </c>
+      <c r="F370" s="14" t="inlineStr">
+        <is>
+          <t>個別作品の予測だが、ディズニーの中核戦略に関わるインサイト。アニメ名作の実写化という『確実な打ち手』への観客の食傷（リメイク疲れ）が数字に表れつつある兆候。既存IPの安全運転が万能でなくなりつつある窓口・企画戦略の転換点を示す材料。</t>
+        </is>
+      </c>
+      <c r="G370" s="14" t="inlineStr">
+        <is>
+          <t>公開前トラッキングで慎重な見立て
+近年の実写リメイク群の成績ばらつき
+『安全なIP再利用』の限界という論点
+アニメ原作の実写化疲れの兆候</t>
+        </is>
+      </c>
+      <c r="H370" s="14" t="inlineStr">
+        <is>
+          <t>実写リメイクの投資対効果が鈍れば、ディズニーは実写化本数を絞りオリジナル/続編に資源を振り分ける調整に動く可能性。他スタジオの名作実写化計画にも再考圧力がかかる。</t>
+        </is>
+      </c>
+      <c r="I370" s="14" t="inlineStr">
+        <is>
+          <t>名作アニメの実写リメイク戦略の限界</t>
+        </is>
+      </c>
+      <c r="J370" s="14" t="inlineStr">
+        <is>
+          <t>The Walt Disney Company</t>
+        </is>
+      </c>
+      <c r="K370" s="14" t="inlineStr">
+        <is>
+          <t>モアナ</t>
+        </is>
+      </c>
+      <c r="L370" s="14" t="inlineStr">
+        <is>
+          <t>興行,トレンド,海外</t>
+        </is>
+      </c>
+      <c r="M370" s="14" t="inlineStr"/>
+    </row>
+    <row r="371">
+      <c r="A371" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B371" s="14" t="inlineStr">
+        <is>
+          <t>映画</t>
+        </is>
+      </c>
+      <c r="C371" s="14" t="inlineStr">
+        <is>
+          <t>『Minions &amp; Monsters』がフランチャイズ最低スタート——アニメ大作フランチャイズの飽和</t>
+        </is>
+      </c>
+      <c r="D371" s="14" t="inlineStr">
+        <is>
+          <t>https://variety.com/2026/film/box-office/minions-and-monsters-box-office-franchise-worst-start-supergirl-brutal-drop-1236801905/</t>
+        </is>
+      </c>
+      <c r="E371" s="14" t="inlineStr">
+        <is>
+          <t>Universal/Illuminationの『怪盗グルー』世界観のアニメ前日譚『Minions &amp; Monsters』が7/4連休に北米約4,243館で公開もオープニング約3,600万ドル（水曜からで約6,100万ドル）と、フランチャイズ史上最も弱い立ち上がりになった。</t>
+        </is>
+      </c>
+      <c r="F371" s="14" t="inlineStr">
+        <is>
+          <t>ヒット連発してきたアニメ大人気フランチャイズでも、番外・前日譚の乱発で観客の関心が逓減し始めた兆候。強IPの安易な横展開が飽和・希薄化を招くという、シリーズ運営（フランチャイズ設計）のインサイトとして拾う。</t>
+        </is>
+      </c>
+      <c r="G371" s="14" t="inlineStr">
+        <is>
+          <t>連休公開もフランチャイズ最弱スタート
+約4,243館規模での弱い初動
+スピンオフ/前日譚乱発による関心逓減
+強IPでも横展開の飽和は起こる</t>
+        </is>
+      </c>
+      <c r="H371" s="14" t="inlineStr">
+        <is>
+          <t>アニメ大作フランチャイズも本編と番外の希釈バランスが問われ、スタジオは公開本数の間引きやブランド管理の厳格化に動く可能性。IPの延命と消耗の分岐が意識される。</t>
+        </is>
+      </c>
+      <c r="I371" s="14" t="inlineStr">
+        <is>
+          <t>アニメフランチャイズの拡張と飽和管理</t>
+        </is>
+      </c>
+      <c r="J371" s="14" t="inlineStr">
+        <is>
+          <t>Universal Pictures, Illumination</t>
+        </is>
+      </c>
+      <c r="K371" s="14" t="inlineStr">
+        <is>
+          <t>Despicable Me, Minions</t>
+        </is>
+      </c>
+      <c r="L371" s="14" t="inlineStr">
+        <is>
+          <t>興行,トレンド,海外</t>
+        </is>
+      </c>
+      <c r="M371" s="14" t="inlineStr"/>
+    </row>
+    <row r="372">
+      <c r="A372" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B372" s="14" t="inlineStr">
+        <is>
+          <t>映画</t>
+        </is>
+      </c>
+      <c r="C372" s="14" t="inlineStr">
+        <is>
+          <t>『キングダム 魂の決戦』が初登場1位・公開3日で興収15.8億——邦画実写シリーズの底堅さ</t>
+        </is>
+      </c>
+      <c r="D372" s="14" t="inlineStr">
+        <is>
+          <t>https://eiga.com/ranking/jp/</t>
+        </is>
+      </c>
+      <c r="E372" s="14" t="inlineStr">
+        <is>
+          <t>映画.comの国内ランキングで、実写映画『キングダム』シリーズ最新作『魂の決戦』が7/17〜19の週末に動員99.3万人・興収15.84億円で初登場1位を記録（祝日含む4日間では約20.6億円との報道も）。同週はアニメ映画『君と花火と約束と』が5位初登場。</t>
+        </is>
+      </c>
+      <c r="F372" s="14" t="inlineStr">
+        <is>
+          <t>漫画原作の実写大型シリーズが安定して開幕トップを取る国内興行の底堅さを示す一件。ハリウッドが名作実写化で苦戦する一方、日本では漫画原作×実写のフランチャイズが機能し続けている対比が読める。</t>
+        </is>
+      </c>
+      <c r="G372" s="14" t="inlineStr">
+        <is>
+          <t>公開3日で動員99.3万人・興収15.84億円
+初登場1位、祝日含む4日で約20.6億円
+漫画原作の実写大型シリーズの底堅さ
+洋画の実写リメイク苦戦との対比</t>
+        </is>
+      </c>
+      <c r="H372" s="14" t="inlineStr">
+        <is>
+          <t>漫画原作の実写シリーズは、原作ファンダム＋話題化で開幕動員を確保できる構図が続く。邦画配給は既存人気IPの実写化を安定収益源として重視し続ける見込み。</t>
+        </is>
+      </c>
+      <c r="I372" s="14" t="inlineStr">
+        <is>
+          <t>漫画原作の実写映画フランチャイズの持続性</t>
+        </is>
+      </c>
+      <c r="J372" s="14" t="inlineStr">
+        <is>
+          <t>東宝, ソニー・ピクチャーズ</t>
+        </is>
+      </c>
+      <c r="K372" s="14" t="inlineStr">
+        <is>
+          <t>キングダム</t>
+        </is>
+      </c>
+      <c r="L372" s="14" t="inlineStr">
+        <is>
+          <t>興行,映像化,国内</t>
+        </is>
+      </c>
+      <c r="M372" s="14" t="inlineStr"/>
+    </row>
+    <row r="373">
+      <c r="A373" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B373" s="14" t="inlineStr">
+        <is>
+          <t>アニメ</t>
+        </is>
+      </c>
+      <c r="C373" s="14" t="inlineStr">
+        <is>
+          <t>ガンダム新作『機動戦士ガンダムRG XARX-ZERO』発表、神山健治監督で2027年展開</t>
+        </is>
+      </c>
+      <c r="D373" s="14" t="inlineStr">
+        <is>
+          <t>https://news.denfaminicogamer.jp/news/260724b</t>
+        </is>
+      </c>
+      <c r="E373" s="14" t="inlineStr">
+        <is>
+          <t>バンダイナムコ系は7/24午前3時、ガンダム公式YouTube『ガンダムチャンネル』で新作アニメ特別番組を全世界同時配信し、新作『機動戦士ガンダムRG XARX-ZERO（アレックスゼロ）』（2027年展開予定）を発表。監督・シリーズ構成に神山健治、SF設定監修に円城塔が参加する。前日にはサンディエゴ・コミコン（SDCC）のパネルでも情報が解禁された。</t>
+        </is>
+      </c>
+      <c r="F373" s="14" t="inlineStr">
+        <is>
+          <t>個別発表だが、発表手法にインサイト。地上波先行でなくYouTube全世界同時配信＋海外イベント（SDCC）連動で解禁する形は、ガンダムを国内番組ではなくグローバルIPとして初手から扱う姿勢の表れ。大型IPのローンチが国境同時・配信起点に移りつつある。</t>
+        </is>
+      </c>
+      <c r="G373" s="14" t="inlineStr">
+        <is>
+          <t>新作『RG XARX-ZERO』2027年展開予定
+監督・構成に神山健治、設定監修に円城塔
+YouTubeで全世界同時配信発表
+SDCCパネルとの海外連動解禁</t>
+        </is>
+      </c>
+      <c r="H373" s="14" t="inlineStr">
+        <is>
+          <t>大型アニメIPは発表段階からグローバル同時・配信起点が標準化し、地上波の初出し優位が薄れる。ガンダムはシリーズ横展開（映像＋ガンプラ＋ゲーム）を世界市場前提で設計する流れを強める。</t>
+        </is>
+      </c>
+      <c r="I373" s="14" t="inlineStr">
+        <is>
+          <t>大型アニメIPのグローバル同時ローンチ設計</t>
+        </is>
+      </c>
+      <c r="J373" s="14" t="inlineStr">
+        <is>
+          <t>バンダイナムコ, サンライズ(バンダイナムコフィルムワークス)</t>
+        </is>
+      </c>
+      <c r="K373" s="14" t="inlineStr">
+        <is>
+          <t>機動戦士ガンダム, ガンダムRG XARX-ZERO</t>
+        </is>
+      </c>
+      <c r="L373" s="14" t="inlineStr">
+        <is>
+          <t>新作,配信,海外,トレンド</t>
+        </is>
+      </c>
+      <c r="M373" s="14" t="inlineStr">
+        <is>
+          <t>SDCC 2026連動</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B374" s="14" t="inlineStr">
+        <is>
+          <t>アニメ</t>
+        </is>
+      </c>
+      <c r="C374" s="14" t="inlineStr">
+        <is>
+          <t>Crunchyroll有料会員2,100万突破（ソニー）——企画製作から流通まで囲う垂直統合が進む</t>
+        </is>
+      </c>
+      <c r="D374" s="14" t="inlineStr">
+        <is>
+          <t>https://branc.jp/article/2026/05/12/2699.html</t>
+        </is>
+      </c>
+      <c r="E374" s="14" t="inlineStr">
+        <is>
+          <t>ソニーグループの2026年3月期決算で、傘下Crunchyrollの有料会員が2,100万人を突破（登録2,000万超）。買収後の2021年夏の約500万から数年で倍増を重ね、5万本超の日本アニメを13言語で配信、自社製作独占（鬼滅等）も会員増に寄与した。</t>
+        </is>
+      </c>
+      <c r="F374" s="14" t="inlineStr">
+        <is>
+          <t>直近の削除騒動（旧作の配信取り下げ）と併せると、Crunchyrollがカタログの出し入れを自社裁量で握る『流通支配』の強さが浮かぶ。企画製作〜独占配信〜物販（上位会員限定化）まで垂直統合する海外アニメ配信の構造を象徴する数字として拾う。</t>
+        </is>
+      </c>
+      <c r="G374" s="14" t="inlineStr">
+        <is>
+          <t>有料会員2,100万人突破（登録2,000万超）
+買収後数年で会員が倍増
+13言語・5万本超の日本アニメを流通
+独占製作と物販の上位会員限定化</t>
+        </is>
+      </c>
+      <c r="H374" s="14" t="inlineStr">
+        <is>
+          <t>垂直統合が進むほど、Crunchyrollは配信可否・独占・物販特典を通じてアニメ流通の主導権を強める。国内権利元は海外収益をCrunchyroll経由に依存する一方、条件交渉での立場が問われる。</t>
+        </is>
+      </c>
+      <c r="I374" s="14" t="inlineStr">
+        <is>
+          <t>アニメ海外配信の垂直統合と流通支配</t>
+        </is>
+      </c>
+      <c r="J374" s="14" t="inlineStr">
+        <is>
+          <t>ソニーグループ, Crunchyroll, アニプレックス</t>
+        </is>
+      </c>
+      <c r="K374" s="14" t="inlineStr">
+        <is>
+          <t>鬼滅の刃</t>
+        </is>
+      </c>
+      <c r="L374" s="14" t="inlineStr">
+        <is>
+          <t>配信,業績,海外,トレンド</t>
+        </is>
+      </c>
+      <c r="M374" s="14" t="inlineStr"/>
+    </row>
+    <row r="375">
+      <c r="A375" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B375" s="14" t="inlineStr">
+        <is>
+          <t>アニメ</t>
+        </is>
+      </c>
+      <c r="C375" s="14" t="inlineStr">
+        <is>
+          <t>アニメ制作が成熟期入り——『確実なヒット×自社IP保有』圧力と制作費高騰・人材争奪</t>
+        </is>
+      </c>
+      <c r="D375" s="14" t="inlineStr">
+        <is>
+          <t>https://anime.eiga.com/news/column/sudo_business/116103/</t>
+        </is>
+      </c>
+      <c r="E375" s="14" t="inlineStr">
+        <is>
+          <t>数土直志のアニメビジネス連載は、海外プラットフォームからの直接投資が一巡し、アニメ業界が『確実なヒット』と『自社IP保有』を問われる成熟期に入ったと分析。制作費高騰は続き、トップクリエイターや作画監督の争奪が激化しているとする。</t>
+        </is>
+      </c>
+      <c r="F375" s="14" t="inlineStr">
+        <is>
+          <t>個別ニュースでなく構造トレンドの整理として拾う。配信バブル的な資金流入が落ち着き、量産から選別へ、受託から権利保有へと制作会社の生存条件が変化。制作費と人材コストの上昇が中小スタジオの経営を圧迫する局面を示す。</t>
+        </is>
+      </c>
+      <c r="G375" s="14" t="inlineStr">
+        <is>
+          <t>海外PFの直接投資が一巡、成熟期へ
+『確実なヒット×自社IP保有』が生存条件
+制作費高騰と作画監督ら人材争奪の激化
+受託中心モデルの限界</t>
+        </is>
+      </c>
+      <c r="H375" s="14" t="inlineStr">
+        <is>
+          <t>制作会社は元請け受託から自社IP・権利保有側へ移る動きを強め、出版社・配信PFとの権利/出資交渉で立場を上げようとする。人材コスト上昇に耐えられない中小の淘汰・再編が続く見込み。</t>
+        </is>
+      </c>
+      <c r="I375" s="14" t="inlineStr">
+        <is>
+          <t>アニメ制作会社の権利保有シフトと人材コスト</t>
+        </is>
+      </c>
+      <c r="J375" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K375" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L375" s="14" t="inlineStr">
+        <is>
+          <t>トレンド,国内,人事・組織</t>
+        </is>
+      </c>
+      <c r="M375" s="14" t="inlineStr"/>
+    </row>
+    <row r="376">
+      <c r="A376" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B376" s="14" t="inlineStr">
+        <is>
+          <t>アニメ</t>
+        </is>
+      </c>
+      <c r="C376" s="14" t="inlineStr">
+        <is>
+          <t>2025〜26年の『続編ラッシュ』が鮮明——新規IP創出よりシリーズ延命に依存</t>
+        </is>
+      </c>
+      <c r="D376" s="14" t="inlineStr">
+        <is>
+          <t>https://www.oricon.co.jp/anime/2026_summer/</t>
+        </is>
+      </c>
+      <c r="E376" s="14" t="inlineStr">
+        <is>
+          <t>2026年夏クールを含め、『無職転生III』『幼女戦記II』『BLEACH 千年血戦篇-禍進譚-』『骸骨騎士様』続編など、既存人気シリーズの続編・分割クールが多数を占める。オリコンほか各まとめでも続編・再放送の比率の高さが指摘されている。</t>
+        </is>
+      </c>
+      <c r="F376" s="14" t="inlineStr">
+        <is>
+          <t>ラインナップの偏りから読めるトレンドとして拾う。制作費高騰・成功確度重視の中で、実績あるIPの続編に投資が集中し、新規オリジナルの割合が相対的に下がる。ヒットの再現性を優先する『延命型』ポートフォリオへの傾斜という消費・供給の潮流。</t>
+        </is>
+      </c>
+      <c r="G376" s="14" t="inlineStr">
+        <is>
+          <t>夏クールも続編・分割クールが多数
+実績IPへの投資集中
+新規オリジナル比率の相対低下
+ヒット再現性重視のポートフォリオ</t>
+        </is>
+      </c>
+      <c r="H376" s="14" t="inlineStr">
+        <is>
+          <t>続編依存が続くと新規IPの供給細りが将来の『続編の種』不足を招く。出版社・製作委員会は原作IPの発掘・囲い込みを一段と急ぎ、オリジナル枠は配信PFの出資に頼る二極化が進む可能性。</t>
+        </is>
+      </c>
+      <c r="I376" s="14" t="inlineStr">
+        <is>
+          <t>続編依存とオリジナルIP供給の先細り</t>
+        </is>
+      </c>
+      <c r="J376" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K376" s="14" t="inlineStr">
+        <is>
+          <t>無職転生, 骸骨騎士様, BLEACH</t>
+        </is>
+      </c>
+      <c r="L376" s="14" t="inlineStr">
+        <is>
+          <t>トレンド,消費者インサイト,国内</t>
+        </is>
+      </c>
+      <c r="M376" s="14" t="inlineStr"/>
+    </row>
+    <row r="377">
+      <c r="A377" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B377" s="14" t="inlineStr">
+        <is>
+          <t>漫画</t>
+        </is>
+      </c>
+      <c r="C377" s="14" t="inlineStr">
+        <is>
+          <t>Webtoon市場が拡大基調、LINEマンガ・ピッコマ牽引——電子コミックが電子出版の約9割</t>
+        </is>
+      </c>
+      <c r="D377" s="14" t="inlineStr">
+        <is>
+          <t>https://www.gii.co.jp/report/tbrc1969002-webtoons-global-market-report.html</t>
+        </is>
+      </c>
+      <c r="E377" s="14" t="inlineStr">
+        <is>
+          <t>各種調査で縦読み漫画（Webtoon）の世界市場は2024年約39.6億ドルから年平均5.6%で拡大し2031年に約57.6億ドルへ到達すると予測。日本の電子書籍市場は2024年度に約6,700億円、うち大半を電子コミックが占め、LINEマンガ・ピッコマが牽引する。</t>
+        </is>
+      </c>
+      <c r="F377" s="14" t="inlineStr">
+        <is>
+          <t>個別作品でなく市場構造の把握として拾う。紙の頭打ちに対し電子コミック（とくにWebtoon形式）が成長エンジンで、プラットフォーム（LINE/ピッコマ）が読者接点と課金を握る。日本発Webtoonの海外展開余地というインサイトも含む。</t>
+        </is>
+      </c>
+      <c r="G377" s="14" t="inlineStr">
+        <is>
+          <t>Webtoon世界市場は2031年に約9,000億円規模予測
+日本の電子書籍の大半を電子コミックが占有
+LINEマンガ・ピッコマが読者接点を握る
+日本発縦読みの海外展開余地</t>
+        </is>
+      </c>
+      <c r="H377" s="14" t="inlineStr">
+        <is>
+          <t>縦読みプラットフォームが課金と発見性を握るほど、出版社は自社IPの縦読み最適化と海外配信でPF依存とどう折り合うかが課題に。国産Webtoon制作体制の整備競争が続く。</t>
+        </is>
+      </c>
+      <c r="I377" s="14" t="inlineStr">
+        <is>
+          <t>縦読み漫画の市場成長とプラットフォーム支配</t>
+        </is>
+      </c>
+      <c r="J377" s="14" t="inlineStr">
+        <is>
+          <t>LINEヤフー(LINE Digital Frontier), カカオピッコマ</t>
+        </is>
+      </c>
+      <c r="K377" s="14" t="inlineStr">
+        <is>
+          <t>LINEマンガ, ピッコマ</t>
+        </is>
+      </c>
+      <c r="L377" s="14" t="inlineStr">
+        <is>
+          <t>配信,トレンド,出版,国内</t>
+        </is>
+      </c>
+      <c r="M377" s="14" t="inlineStr"/>
+    </row>
+    <row r="378">
+      <c r="A378" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B378" s="14" t="inlineStr">
+        <is>
+          <t>漫画</t>
+        </is>
+      </c>
+      <c r="C378" s="14" t="inlineStr">
+        <is>
+          <t>2025年コミック市場6,925億円で8年ぶり前年割れ（▲1.7%）——電子の伸び鈍化が鮮明</t>
+        </is>
+      </c>
+      <c r="D378" s="14" t="inlineStr">
+        <is>
+          <t>https://hon.jp/news/1.0/0/58504</t>
+        </is>
+      </c>
+      <c r="E378" s="14" t="inlineStr">
+        <is>
+          <t>出版科学研究所の集計で、2025年の紙＋電子コミック市場は前年比1.7%減の6,925億円と、7年連続成長が途切れ8年ぶりのマイナス成長。電子出版全体は微増だったが、成長を支えてきた電子コミックの伸び率鈍化が鮮明になった。</t>
+        </is>
+      </c>
+      <c r="F378" s="14" t="inlineStr">
+        <is>
+          <t>市場統計から読むインサイト。紙の縮小を電子が補って伸びてきた構図が転機を迎え、電子コミックそのものの成長が頭打ちに近づいた兆候。ヒット作依存・値引き競争・可処分時間の奪い合いが効いている可能性を検証する材料。</t>
+        </is>
+      </c>
+      <c r="G378" s="14" t="inlineStr">
+        <is>
+          <t>コミック市場6,925億円、前年比▲1.7%
+7年連続成長が途切れ8年ぶりマイナス
+電子コミックの伸び率鈍化が主因
+紙の縮小を電子が補う構図に転機</t>
+        </is>
+      </c>
+      <c r="H378" s="14" t="inlineStr">
+        <is>
+          <t>電子の踊り場が続けば、出版社は単価維持（値引き依存脱却）、海外・Webtoon展開、メディアミックスによるIP収益の多角化で成長を補う戦略に一段と傾く。</t>
+        </is>
+      </c>
+      <c r="I378" s="14" t="inlineStr">
+        <is>
+          <t>コミック市場の成長鈍化とIP収益多角化</t>
+        </is>
+      </c>
+      <c r="J378" s="14" t="inlineStr">
+        <is>
+          <t>集英社, 講談社, 小学館, KADOKAWA</t>
+        </is>
+      </c>
+      <c r="K378" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L378" s="14" t="inlineStr">
+        <is>
+          <t>出版,業績,トレンド,国内</t>
+        </is>
+      </c>
+      <c r="M378" s="14" t="inlineStr"/>
+    </row>
+    <row r="379">
+      <c r="A379" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B379" s="14" t="inlineStr">
+        <is>
+          <t>漫画</t>
+        </is>
+      </c>
+      <c r="C379" s="14" t="inlineStr">
+        <is>
+          <t>読者調査で『Webtoonは創作性が足りない』——量産・型化への評価ギャップが表面化</t>
+        </is>
+      </c>
+      <c r="D379" s="14" t="inlineStr">
+        <is>
+          <t>https://premium.kai-you.net/article/892</t>
+        </is>
+      </c>
+      <c r="E379" s="14" t="inlineStr">
+        <is>
+          <t>KAI-YOUの読者調査ベース記事は、認知・閲覧が広がる一方で『Webtoonは創作性が足りない』と感じる読者層の存在と、縦読み漫画の課題・ファン層の乖離を指摘した。</t>
+        </is>
+      </c>
+      <c r="F379" s="14" t="inlineStr">
+        <is>
+          <t>消費者インサイトとして拾う一件。プラットフォーム主導で量産・テンプレ化が進む縦読みに対し、コア読者が作家性・独自性の希薄さを感じ始めている。市場拡大の裏でブランド／品質面の評価ギャップが生じている点がトレンド検証材料。</t>
+        </is>
+      </c>
+      <c r="G379" s="14" t="inlineStr">
+        <is>
+          <t>閲覧拡大の一方で『創作性不足』の評価
+量産・型化への読者の違和感
+縦読みとコア漫画ファンの乖離
+PF主導量産モデルの質的課題</t>
+        </is>
+      </c>
+      <c r="H379" s="14" t="inlineStr">
+        <is>
+          <t>質への不満が広がれば、縦読みPFは作家性の強い独占作・オリジナル投資で差別化を迫られる。従来型（横読み）漫画の作家性を武器にした逆張り編集戦略も再評価されうる。</t>
+        </is>
+      </c>
+      <c r="I379" s="14" t="inlineStr">
+        <is>
+          <t>縦読み量産モデルの品質と作家性の課題</t>
+        </is>
+      </c>
+      <c r="J379" s="14" t="inlineStr">
+        <is>
+          <t>LINEヤフー, カカオピッコマ</t>
+        </is>
+      </c>
+      <c r="K379" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L379" s="14" t="inlineStr">
+        <is>
+          <t>消費者インサイト,トレンド,国内</t>
+        </is>
+      </c>
+      <c r="M379" s="14" t="inlineStr"/>
+    </row>
+    <row r="380">
+      <c r="A380" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B380" s="14" t="inlineStr">
+        <is>
+          <t>漫画</t>
+        </is>
+      </c>
+      <c r="C380" s="14" t="inlineStr">
+        <is>
+          <t>『薬屋のひとりごと』17巻が7/24発売——小説→漫画→アニメで循環するIPの持続力</t>
+        </is>
+      </c>
+      <c r="D380" s="14" t="inlineStr">
+        <is>
+          <t>https://natalie.mu/comic/news/678379</t>
+        </is>
+      </c>
+      <c r="E380" s="14" t="inlineStr">
+        <is>
+          <t>コミックナタリーの新刊リストで、7/24に『薬屋のひとりごと』最新17巻が発売。小説発のIPが2系統のコミカライズ・アニメ・関連商品で相互送客し、原作・コミック双方の刊行が長期に続くロングセラーとなっている。</t>
+        </is>
+      </c>
+      <c r="F380" s="14" t="inlineStr">
+        <is>
+          <t>単なる新刊告知ではなく、メディアミックスの相乗が原作寿命を延ばす実例として拾う。小説→漫画→アニメの循環が各媒体の新刊・新シーズンごとに需要を再点火し、IPが長期のキャッシュフローを生む構造を示す。</t>
+        </is>
+      </c>
+      <c r="G380" s="14" t="inlineStr">
+        <is>
+          <t>最新17巻を7/24発売
+小説発IPの2系統コミカライズ＋アニメ
+媒体横断の相互送客で刊行が長期化
+ロングセラー化するメディアミックスIP</t>
+        </is>
+      </c>
+      <c r="H380" s="14" t="inlineStr">
+        <is>
+          <t>循環型メディアミックスの成功例が増えるほど、出版社は初期からアニメ・複数コミカライズ前提でIPを設計し、単発ヒットより長期育成型のIPマネジメントに軸足を移す。</t>
+        </is>
+      </c>
+      <c r="I380" s="14" t="inlineStr">
+        <is>
+          <t>循環型メディアミックスによるIP長寿命化</t>
+        </is>
+      </c>
+      <c r="J380" s="14" t="inlineStr">
+        <is>
+          <t>集英社, スクウェア・エニックス, 主婦の友社</t>
+        </is>
+      </c>
+      <c r="K380" s="14" t="inlineStr">
+        <is>
+          <t>薬屋のひとりごと</t>
+        </is>
+      </c>
+      <c r="L380" s="14" t="inlineStr">
+        <is>
+          <t>出版,映像化,消費者インサイト,国内</t>
+        </is>
+      </c>
+      <c r="M380" s="14" t="inlineStr"/>
+    </row>
+    <row r="381">
+      <c r="A381" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B381" s="14" t="inlineStr">
+        <is>
+          <t>小説</t>
+        </is>
+      </c>
+      <c r="C381" s="14" t="inlineStr">
+        <is>
+          <t>第175回芥川賞は小砂川チト『ゾンビ回収婦』——AI侵食世界を描く純文学の主題化</t>
+        </is>
+      </c>
+      <c r="D381" s="14" t="inlineStr">
+        <is>
+          <t>https://store.kinokuniya.co.jp/event/akutagawa-naoki-awards/</t>
+        </is>
+      </c>
+      <c r="E381" s="14" t="inlineStr">
+        <is>
+          <t>7/15の選考会で第175回芥川賞に小砂川チト『ゾンビ回収婦』（講談社）、直木賞に朝倉かすみ『けんぐゎい』（光文社）が決定。芥川賞受賞作はAIに侵食された世界で殺されたゾンビの亡骸を回収する掃除婦を描き、現実と虚構が混じる世界観が特徴。</t>
+        </is>
+      </c>
+      <c r="F381" s="14" t="inlineStr">
+        <is>
+          <t>受賞そのものに加え、テーマ選択のインサイトで拾う。純文学の最高峰の受賞作がAIによる世界侵食を主題化した点は、AIが社会不安・実存の主題として文芸のど真ん中に入ってきた表れ。技術トレンドが文学の題材構造に及ぼす影響を示す。</t>
+        </is>
+      </c>
+      <c r="G381" s="14" t="inlineStr">
+        <is>
+          <t>芥川賞は小砂川チト『ゾンビ回収婦』(講談社)
+直木賞は朝倉かすみ『けんぐゎい』(光文社)
+受賞作がAI侵食世界を主題化
+AIが純文学の中心主題に</t>
+        </is>
+      </c>
+      <c r="H381" s="14" t="inlineStr">
+        <is>
+          <t>AI・ポストヒューマンを主題にした文芸作品の刊行・受賞が増え、出版社は『AI時代の実存』を打ち出す文芸ラインを強化。受賞効果で両作の実売が短期に押し上がる。</t>
+        </is>
+      </c>
+      <c r="I381" s="14" t="inlineStr">
+        <is>
+          <t>AI主題の文芸化と受賞作の市場効果</t>
+        </is>
+      </c>
+      <c r="J381" s="14" t="inlineStr">
+        <is>
+          <t>講談社, 光文社, 日本文学振興会</t>
+        </is>
+      </c>
+      <c r="K381" s="14" t="inlineStr">
+        <is>
+          <t>ゾンビ回収婦, けんぐゎい</t>
+        </is>
+      </c>
+      <c r="L381" s="14" t="inlineStr">
+        <is>
+          <t>受賞,出版,トレンド,国内</t>
+        </is>
+      </c>
+      <c r="M381" s="14" t="inlineStr"/>
+    </row>
+    <row r="382">
+      <c r="A382" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B382" s="14" t="inlineStr">
+        <is>
+          <t>小説</t>
+        </is>
+      </c>
+      <c r="C382" s="14" t="inlineStr">
+        <is>
+          <t>本屋大賞は朝井リョウ『イン・ザ・メガチャーチ』——『推し活/ファンダム経済』を主題に、日経夕刊連載が史上初受賞</t>
+        </is>
+      </c>
+      <c r="D382" s="14" t="inlineStr">
+        <is>
+          <t>https://www.hontai.or.jp/history/hontai2026.html</t>
+        </is>
+      </c>
+      <c r="E382" s="14" t="inlineStr">
+        <is>
+          <t>2026年本屋大賞（第23回）は朝井リョウ『イン・ザ・メガチャーチ』（日経BP／日本経済新聞出版）が受賞。現代の『推し活』とファンダム経済を複数視点で描く社会派エンタメで、日経夕刊連載小説の本屋大賞受賞は史上初。</t>
+        </is>
+      </c>
+      <c r="F382" s="14" t="inlineStr">
+        <is>
+          <t>分析素材として再掲・接続。エンタメ産業を支える『推し活/ファンダム経済』そのものが文芸の主題となり、書店員票で大賞を得た点は、ファンダムが社会的テーマとして広く共有された証左。他ジャンル（音楽・アニメ）のファンダム論とも接続する。</t>
+        </is>
+      </c>
+      <c r="G382" s="14" t="inlineStr">
+        <is>
+          <t>本屋大賞に朝井リョウ『イン・ザ・メガチャーチ』
+推し活/ファンダム経済を主題化
+日経夕刊連載小説として史上初の受賞
+新聞連載発の文芸の商業力</t>
+        </is>
+      </c>
+      <c r="H382" s="14" t="inlineStr">
+        <is>
+          <t>ファンダム経済を扱う文芸・ノンフィクションの刊行が増え、出版社は『推し活』読者層に向けた企画を強化。受賞効果で書店実売とメディアミックス（映像化）打診が進む可能性。</t>
+        </is>
+      </c>
+      <c r="I382" s="14" t="inlineStr">
+        <is>
+          <t>ファンダム経済の文芸主題化と受賞の波及</t>
+        </is>
+      </c>
+      <c r="J382" s="14" t="inlineStr">
+        <is>
+          <t>日経BP, 日本経済新聞出版</t>
+        </is>
+      </c>
+      <c r="K382" s="14" t="inlineStr">
+        <is>
+          <t>イン・ザ・メガチャーチ</t>
+        </is>
+      </c>
+      <c r="L382" s="14" t="inlineStr">
+        <is>
+          <t>受賞,出版,消費者インサイト,国内</t>
+        </is>
+      </c>
+      <c r="M382" s="14" t="inlineStr"/>
+    </row>
+    <row r="383">
+      <c r="A383" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B383" s="14" t="inlineStr">
+        <is>
+          <t>小説</t>
+        </is>
+      </c>
+      <c r="C383" s="14" t="inlineStr">
+        <is>
+          <t>第175回直木賞候補にオードリー若林ら——芸人・異業種著者の文芸参入が定着</t>
+        </is>
+      </c>
+      <c r="D383" s="14" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=B0fB_xsIT_4</t>
+        </is>
+      </c>
+      <c r="E383" s="14" t="inlineStr">
+        <is>
+          <t>第175回直木賞の候補に、お笑いコンビ・オードリーの若林正恭ら異業種の書き手が名を連ねたことが報じられた（受賞は朝倉かすみ）。芸人・タレント著者が話題性だけでなく選考の俎上に乗る流れが続いている。</t>
+        </is>
+      </c>
+      <c r="F383" s="14" t="inlineStr">
+        <is>
+          <t>話題性の裏のインサイトで拾う。芸人・タレントによる文芸が『色物』でなく賞レースの候補として評価される定着ぶりは、著者のパーソナルブランド（ファンダム）と文芸市場が接続した表れ。出版社の著者調達戦略の変化を示す。</t>
+        </is>
+      </c>
+      <c r="G383" s="14" t="inlineStr">
+        <is>
+          <t>直木賞候補に若林正恭ら異業種著者
+芸人・タレント著者の文芸参入が定着
+話題性と文学的評価の両立
+著者のパーソナルブランド活用</t>
+        </is>
+      </c>
+      <c r="H383" s="14" t="inlineStr">
+        <is>
+          <t>出版社はフォロワー基盤を持つ著者の起用を強め、初速の見込める文芸企画を増やす。一方で純粋な新人発掘とのバランスや、話題先行への批判も continue。</t>
+        </is>
+      </c>
+      <c r="I383" s="14" t="inlineStr">
+        <is>
+          <t>著者ブランドと文芸市場の接続</t>
+        </is>
+      </c>
+      <c r="J383" s="14" t="inlineStr">
+        <is>
+          <t>光文社, 各文芸出版社</t>
+        </is>
+      </c>
+      <c r="K383" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L383" s="14" t="inlineStr">
+        <is>
+          <t>受賞,出版,消費者インサイト,国内</t>
+        </is>
+      </c>
+      <c r="M383" s="14" t="inlineStr"/>
+    </row>
+    <row r="384">
+      <c r="A384" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B384" s="14" t="inlineStr">
+        <is>
+          <t>小説</t>
+        </is>
+      </c>
+      <c r="C384" s="14" t="inlineStr">
+        <is>
+          <t>ライトノベル新刊が7月342点——『薬屋』『とある』等の巨大シリーズに部数集中</t>
+        </is>
+      </c>
+      <c r="D384" s="14" t="inlineStr">
+        <is>
+          <t>https://kadokawa.co.jp/calendar/?largeGenre=12&amp;target=0</t>
+        </is>
+      </c>
+      <c r="E384" s="14" t="inlineStr">
+        <is>
+          <t>KADOKAWA等の刊行カレンダーで2026年7月のライトノベル新刊は約342点。累計では『とある魔術の禁書目録』約3,100万部、『転生したらスライムだった件』『薬屋のひとりごと』等が数千万部級と、巨大シリーズへの部数集中が続く。</t>
+        </is>
+      </c>
+      <c r="F384" s="14" t="inlineStr">
+        <is>
+          <t>点数の多さと部数集中の対比で拾うトレンド。新刊は大量に出る一方、実売・累計は一部のメガシリーズ（多くがアニメ化済み）に偏る。ヒットの再現性を求めメディアミックス前提のIPに資源が集まる、ラノベ市場のロングテール×勝者総取り構造を示す。</t>
+        </is>
+      </c>
+      <c r="G384" s="14" t="inlineStr">
+        <is>
+          <t>7月のラノベ新刊は約342点
+累計はメガシリーズに集中
+上位はアニメ化済みIPが多数
+新刊量産と実売集中の乖離</t>
+        </is>
+      </c>
+      <c r="H384" s="14" t="inlineStr">
+        <is>
+          <t>レーベルはアニメ化を見据えた少数の大型IP育成に注力し、Web発の青田買いと早期メディアミックス化を加速。中堅以下の新規シリーズは電子・Web先行で生存を図る二極化が進む。</t>
+        </is>
+      </c>
+      <c r="I384" s="14" t="inlineStr">
+        <is>
+          <t>ラノベ市場の勝者総取りとメディアミックス前提化</t>
+        </is>
+      </c>
+      <c r="J384" s="14" t="inlineStr">
+        <is>
+          <t>KADOKAWA, SBクリエイティブ</t>
+        </is>
+      </c>
+      <c r="K384" s="14" t="inlineStr">
+        <is>
+          <t>とある魔術の禁書目録, 転生したらスライムだった件, 薬屋のひとりごと</t>
+        </is>
+      </c>
+      <c r="L384" s="14" t="inlineStr">
+        <is>
+          <t>出版,トレンド,国内</t>
+        </is>
+      </c>
+      <c r="M384" s="14" t="inlineStr"/>
+    </row>
+    <row r="385">
+      <c r="A385" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B385" s="14" t="inlineStr">
+        <is>
+          <t>音楽</t>
+        </is>
+      </c>
+      <c r="C385" s="14" t="inlineStr">
+        <is>
+          <t>フジロック'26、Amazonが全世界無料独占ライブ配信（7/24-26）——フェス配信の窓口独占が定着</t>
+        </is>
+      </c>
+      <c r="D385" s="14" t="inlineStr">
+        <is>
+          <t>https://www.aboutamazon.jp/news/entertainment/fuji-rock-festival-26%E3%82%92prime-video%E3%81%A8twitch%E3%81%A7%E7%8B%AC%E5%8D%A0%E3%83%A9%E3%82%A4%E3%83%96%E9%85%8D%E4%BF%A1</t>
+        </is>
+      </c>
+      <c r="E385" s="14" t="inlineStr">
+        <is>
+          <t>7/24〜26開催のFUJI ROCK FESTIVAL '26を、Amazonが今年もAmazon Musicアプリ/Prime Video/Twitchで全世界向けに無料独占ライブ配信。The xx・Khruangbin・藤井風・XG等70組超、複数ステージを日毎3チャンネルで配信し、Prime非会員でも視聴可能。</t>
+        </is>
+      </c>
+      <c r="F385" s="14" t="inlineStr">
+        <is>
+          <t>個別フェスの話でなく窓口戦略のトレンド。国内最大級フェスの世界配信を単一プラットフォームが独占無料で担う体制が定着し、フェスの露出・データ・グローバル到達がAmazon経由に集約される。ライブ興行とプラットフォームの関係を示す材料。</t>
+        </is>
+      </c>
+      <c r="G385" s="14" t="inlineStr">
+        <is>
+          <t>7/24-26開催、Amazonが全世界無料独占配信
+The xx・藤井風・XG等70組超
+Amazon Music/Prime Video/Twitchで展開
+Prime非会員も視聴可能</t>
+        </is>
+      </c>
+      <c r="H385" s="14" t="inlineStr">
+        <is>
+          <t>フェス主催の収益・露出設計が『会場チケット＋物販』から『配信プラットフォームとの独占契約＋データ・グローバル送客』へ比重を移す。他フェスもプラットフォーム独占配信の獲得競争に向かう。</t>
+        </is>
+      </c>
+      <c r="I385" s="14" t="inlineStr">
+        <is>
+          <t>ライブ興行の配信独占とプラットフォーム依存</t>
+        </is>
+      </c>
+      <c r="J385" s="14" t="inlineStr">
+        <is>
+          <t>Amazon, スマッシュ</t>
+        </is>
+      </c>
+      <c r="K385" s="14" t="inlineStr">
+        <is>
+          <t>FUJI ROCK FESTIVAL</t>
+        </is>
+      </c>
+      <c r="L385" s="14" t="inlineStr">
+        <is>
+          <t>配信,ライブ・イベント,トレンド,海外</t>
+        </is>
+      </c>
+      <c r="M385" s="14" t="inlineStr">
+        <is>
+          <t>イベントカレンダーにも登録</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B386" s="14" t="inlineStr">
+        <is>
+          <t>音楽</t>
+        </is>
+      </c>
+      <c r="C386" s="14" t="inlineStr">
+        <is>
+          <t>Spotify×ソニーミュージックが新契約——3メジャーが直接ライセンスで出揃い、CRB型から転換</t>
+        </is>
+      </c>
+      <c r="D386" s="14" t="inlineStr">
+        <is>
+          <t>https://www.musicbusinessworldwide.com/sony-spotify-strike-expanded-global-deal-including-a-direct-agreement-for-sony-music-publishing-in-the-us/</t>
+        </is>
+      </c>
+      <c r="E386" s="14" t="inlineStr">
+        <is>
+          <t>Spotifyとソニーミュージックグループがグローバル提携を延長・拡張し、米国でソニー・ミュージックパブリッシングとの直接ライセンス契約を新設。これでUMG（1月）・Warner（2月）に続き3メジャーすべてがSpotifyと直接出版契約を結び、従来のCRB（著作権使用料委員会）モデルから離れる。ソングライターが配信成長の果実をより直接得られる設計とされる。</t>
+        </is>
+      </c>
+      <c r="F386" s="14" t="inlineStr">
+        <is>
+          <t>配信ビジネスの構造転換として拾う。楽曲（出版）側の対価が委員会裁定型から当事者間の直接契約型へ移る動きが3メジャーで出揃い、Spotifyとレーベル/パブリッシャーの関係が再設計された。オーディオブック抱き合わせ問題への対応でもある。</t>
+        </is>
+      </c>
+      <c r="G386" s="14" t="inlineStr">
+        <is>
+          <t>ソニーと直接出版契約を新設
+3メジャーすべてが直接ライセンスで出揃う
+CRB裁定型からの離脱
+ソングライター配分の改善を標榜</t>
+        </is>
+      </c>
+      <c r="H386" s="14" t="inlineStr">
+        <is>
+          <t>直接契約が主流化すると、独立系レーベル/ディストリビューターや中小パブリッシャーの交渉力格差が拡大。Spotifyは料率・機能（AIリミックス等）を当事者間で設計しやすくなり、権利処理の主導権を強める。</t>
+        </is>
+      </c>
+      <c r="I386" s="14" t="inlineStr">
+        <is>
+          <t>音楽配信の直接ライセンス化と権利処理構造</t>
+        </is>
+      </c>
+      <c r="J386" s="14" t="inlineStr">
+        <is>
+          <t>Spotify, ソニーミュージック, UMG, Warner Music</t>
+        </is>
+      </c>
+      <c r="K386" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L386" s="14" t="inlineStr">
+        <is>
+          <t>提携,配信,権利・ライセンス,海外</t>
+        </is>
+      </c>
+      <c r="M386" s="14" t="inlineStr"/>
+    </row>
+    <row r="387">
+      <c r="A387" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B387" s="14" t="inlineStr">
+        <is>
+          <t>音楽</t>
+        </is>
+      </c>
+      <c r="C387" s="14" t="inlineStr">
+        <is>
+          <t>HYBEが新レーベルABD設立、ローカライズ型アイドルでグローバル音楽企業へ脱皮</t>
+        </is>
+      </c>
+      <c r="D387" s="14" t="inlineStr">
+        <is>
+          <t>https://www.kpop-snap.com/news/0e8c2c9f-05b0-4346-ad59-a9095ce2221a</t>
+        </is>
+      </c>
+      <c r="E387" s="14" t="inlineStr">
+        <is>
+          <t>HYBEは新レーベルABDを設立し2026年後半に新ガールグループのデビューを計画。米国発KATSEYE、ラテンアメリカ向けSANTOS BRAVOS等『現地でオーディション・現地デビュー』のローカライズ型アイドルを展開し、Weverse等のファンダムPFと組み合わせグローバル音楽企業への転換を進める。2026通期は増収・営業益大幅増を見込む。</t>
+        </is>
+      </c>
+      <c r="F387" s="14" t="inlineStr">
+        <is>
+          <t>K-POP単体でなくビジネスモデルのインサイト。HYBEは韓国発アーティストの輸出から、各地域で現地アイドルを製造する『方法論の輸出』へ移行。IP（アイドル）を現地生産しファンダムPFで収益化する、製造業的な多国籍展開モデルを示す。</t>
+        </is>
+      </c>
+      <c r="G387" s="14" t="inlineStr">
+        <is>
+          <t>新レーベルABDで新GG（2026後半）
+KATSEYE/SANTOS BRAVOS等ローカライズ型
+Weverse等ファンダムPFと連動
+2026通期は増収・営業益大幅増見込み</t>
+        </is>
+      </c>
+      <c r="H387" s="14" t="inlineStr">
+        <is>
+          <t>『方法論の輸出＋現地製造』が奏功すれば、HYBEは韓国依存を下げ地域分散した収益基盤を築く。日本の事務所/レーベルもローカライズ型やファンダムPF内製で追随・対抗する動きが強まる。</t>
+        </is>
+      </c>
+      <c r="I387" s="14" t="inlineStr">
+        <is>
+          <t>アイドル製造モデルの多国籍展開とファンダムPF</t>
+        </is>
+      </c>
+      <c r="J387" s="14" t="inlineStr">
+        <is>
+          <t>HYBE, JYP</t>
+        </is>
+      </c>
+      <c r="K387" s="14" t="inlineStr">
+        <is>
+          <t>KATSEYE, SANTOS BRAVOS</t>
+        </is>
+      </c>
+      <c r="L387" s="14" t="inlineStr">
+        <is>
+          <t>海外,トレンド,新作</t>
+        </is>
+      </c>
+      <c r="M387" s="14" t="inlineStr"/>
+    </row>
+    <row r="388">
+      <c r="A388" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B388" s="14" t="inlineStr">
+        <is>
+          <t>音楽</t>
+        </is>
+      </c>
+      <c r="C388" s="14" t="inlineStr">
+        <is>
+          <t>RIAAら業界団体、AI生成/AI補助楽曲の『ラベル表示』を提案——配信のAI開示ルール整備へ</t>
+        </is>
+      </c>
+      <c r="D388" s="14" t="inlineStr">
+        <is>
+          <t>https://gizmodo.com/ai-labels-could-be-coming-to-music-streaming-platforms-soon-2000784216</t>
+        </is>
+      </c>
+      <c r="E388" s="14" t="inlineStr">
+        <is>
+          <t>RIAA・A2IM・Recording Academy等が、完全AI生成およびAI補助のコンテンツに対する新たな表示（ラベル）を提案。アーティスト/提供者の自主開示に基づき、『explicit』表示のように機能させる構想で、ストリーミングPFでのAI開示ルール整備を促す。</t>
+        </is>
+      </c>
+      <c r="F388" s="14" t="inlineStr">
+        <is>
+          <t>規制・ルール形成のインサイト。AI生成楽曲の大量流入に対し、禁止でなく『表示による識別』で秩序化しようとする業界の初動。透明性ラベルが標準化すれば、AI楽曲とヒト制作楽曲の市場的な線引き・課金/推薦の扱いに影響する。</t>
+        </is>
+      </c>
+      <c r="G388" s="14" t="inlineStr">
+        <is>
+          <t>完全AI生成/AI補助にラベル表示を提案
+自主開示ベースで『explicit』様に機能
+RIAA・A2IM・Recording Academyが主導
+AI楽曲流入への秩序化の初動</t>
+        </is>
+      </c>
+      <c r="H388" s="14" t="inlineStr">
+        <is>
+          <t>ラベル制度が各PFに実装されると、AI楽曲の可視化・フィルタリングが可能になり、推薦アルゴリズムやロイヤリティ配分でAI/ヒトの扱いを分ける議論が加速。表示義務の法制化論とも接続する。</t>
+        </is>
+      </c>
+      <c r="I388" s="14" t="inlineStr">
+        <is>
+          <t>生成AI楽曲の開示ラベルと市場秩序化</t>
+        </is>
+      </c>
+      <c r="J388" s="14" t="inlineStr">
+        <is>
+          <t>RIAA, A2IM, Recording Academy, Spotify</t>
+        </is>
+      </c>
+      <c r="K388" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L388" s="14" t="inlineStr">
+        <is>
+          <t>AI,規制,配信,海外</t>
+        </is>
+      </c>
+      <c r="M388" s="14" t="inlineStr"/>
+    </row>
+    <row r="389">
+      <c r="A389" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B389" s="14" t="inlineStr">
+        <is>
+          <t>音楽</t>
+        </is>
+      </c>
+      <c r="C389" s="14" t="inlineStr">
+        <is>
+          <t>NiziU『Portfolio』が総合アルバム首位——グループ初ベストで送るファンダム動員の実売</t>
+        </is>
+      </c>
+      <c r="D389" s="14" t="inlineStr">
+        <is>
+          <t>https://www.billboard-japan.com/d_news/detail/163261</t>
+        </is>
+      </c>
+      <c r="E389" s="14" t="inlineStr">
+        <is>
+          <t>Billboard JAPANの総合アルバムチャート（6/29-7/5）で、NiziUの初のベストアルバム『Portfolio』（7/1発売・全20曲）が首位。CD・ダウンロード等を合算する総合指標での1位で、同時期にはBE:FIRST『Missing』が多面で強さを見せた。</t>
+        </is>
+      </c>
+      <c r="F389" s="14" t="inlineStr">
+        <is>
+          <t>チャート結果を消費者行動の観点で拾う。初ベスト盤が総合首位を取る背景には、フィジカル/DLを厚く買い支えるコアファンダムの動員力がある。ストリーミング時代でも『所有・応援』消費が実売指標を左右する国内特有の構造を示す。</t>
+        </is>
+      </c>
+      <c r="G389" s="14" t="inlineStr">
+        <is>
+          <t>NiziU初ベスト『Portfolio』が総合アルバム首位
+6/29-7/5集計、全20曲
+CD/DL等合算の総合指標で1位
+BE:FIRST等も多面で好調</t>
+        </is>
+      </c>
+      <c r="H389" s="14" t="inlineStr">
+        <is>
+          <t>総合指標での首位争いは、ストリーミングの再生数だけでなくフィジカル動員力を持つグループが優位に立つ構造が続く。レーベルは特典設計・複数形態でファンダム消費を最大化する運営を強める。</t>
+        </is>
+      </c>
+      <c r="I389" s="14" t="inlineStr">
+        <is>
+          <t>フィジカル動員とファンダム消費のチャート影響</t>
+        </is>
+      </c>
+      <c r="J389" s="14" t="inlineStr">
+        <is>
+          <t>ソニーミュージック(NiziU), BMSG</t>
+        </is>
+      </c>
+      <c r="K389" s="14" t="inlineStr">
+        <is>
+          <t>NiziU, BE:FIRST</t>
+        </is>
+      </c>
+      <c r="L389" s="14" t="inlineStr">
+        <is>
+          <t>チャート・ランキング,消費者インサイト,国内</t>
+        </is>
+      </c>
+      <c r="M389" s="14" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -53097,7 +55059,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -53276,6 +55238,63 @@
       <c r="K3" s="15" t="inlineStr">
         <is>
           <t>監督:二宮健。2022年にアニメ化済みの少年ジャンプ+連載作。実写はメディアミックスの新展開</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>ちいかわ</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>漫画</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>ナガノ</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>映画</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>劇場版アニメ『映画ちいかわ 人魚の島のひみつ』（セイレーン編を映像化）</t>
+        </is>
+      </c>
+      <c r="G4" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="H4" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="I4" s="14" t="inlineStr">
+        <is>
+          <t>公開済</t>
+        </is>
+      </c>
+      <c r="J4" s="14" t="inlineStr">
+        <is>
+          <t>Cygames, CygamesPictures, 東宝</t>
+        </is>
+      </c>
+      <c r="K4" s="14" t="inlineStr">
+        <is>
+          <t>WEB漫画発キャラIPの初劇場版。全国380館・上映回数は大作級との報道。キャラ強/物語希薄IPの劇場マネタイズ事例</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
daily-news(6genres) + cross-questions + media-mix + predictions + game-design update
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -891,7 +891,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2621,6 +2621,48 @@
         </is>
       </c>
       <c r="H41" s="14" t="inlineStr">
+        <is>
+          <t>横断</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B42" s="14" t="inlineStr">
+        <is>
+          <t>配信/放送プラットフォームによるアニメ制作会社の子会社化（U-NEXT×GoHands等）が進むと、製作委員会の主導権がPF側に集中し、原作を握る大手出版社が委員会参加より『自社出資・自社スタジオでのアニメ内製化』に軸足を移す（＝出版社の製作委員会離脱・内製化）</t>
+        </is>
+      </c>
+      <c r="C42" s="14" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="D42" s="14" t="inlineStr">
+        <is>
+          <t>1〜2年</t>
+        </is>
+      </c>
+      <c r="E42" s="14" t="inlineStr">
+        <is>
+          <t>U-NEXT HOLDINGS, 集英社, 講談社, KADOKAWA</t>
+        </is>
+      </c>
+      <c r="F42" s="14" t="inlineStr">
+        <is>
+          <t>『アニメ制作会社の資本再編が加速、配信・出版が垂直統合』（リアルサウンド/Yahoo, 7/24 日次ニュース）</t>
+        </is>
+      </c>
+      <c r="G42" s="14" t="inlineStr">
+        <is>
+          <t>集英社・講談社・KADOKAWAの製作委員会での出資比率、自社元請（内製）アニメ本数、PF主導委員会の割合を四半期で観測</t>
+        </is>
+      </c>
+      <c r="H42" s="14" t="inlineStr">
         <is>
           <t>横断</t>
         </is>
@@ -5577,7 +5619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H89"/>
+  <dimension ref="A1:H91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9323,6 +9365,90 @@
         </is>
       </c>
       <c r="H89" s="14" t="inlineStr">
+        <is>
+          <t>横断</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B90" s="14" t="inlineStr">
+        <is>
+          <t>映画で進む『大作は劇場ウィンドウ延長・中堅は配信直行』の窓口二極化は、アニメ（劇場アニメ vs 配信直行）や音楽（特典付きフィジカル大作 vs 配信直行リリース）でも同じ二極化として起きるか？</t>
+        </is>
+      </c>
+      <c r="C90" s="14" t="inlineStr">
+        <is>
+          <t>『Project Hail Mary』105日窓延長／『72 Hours』Netflix直行（Deadline・THR, 7/24）</t>
+        </is>
+      </c>
+      <c r="D90" s="14" t="inlineStr">
+        <is>
+          <t>Amazon MGM, Netflix, ディズニー</t>
+        </is>
+      </c>
+      <c r="E90" s="14" t="inlineStr">
+        <is>
+          <t>出版（大型作は紙先行・中堅は電子直行）, 小売（旗艦店 vs EC専売）</t>
+        </is>
+      </c>
+      <c r="F90" s="14" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="G90" s="14" t="inlineStr">
+        <is>
+          <t>『作品規模で流通経路を変える』二極化はエンタメ全ジャンル共通の圧力。中間層が痩せる点も共通</t>
+        </is>
+      </c>
+      <c r="H90" s="14" t="inlineStr">
+        <is>
+          <t>横断</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B91" s="14" t="inlineStr">
+        <is>
+          <t>AniBizのような『ライセンス商流のB2Bマーケットプレイス化』は、音楽（カタログ/シンク権の取引PF）や出版（翻訳版権のB2B化）でも起きるか？権利流通のプラットフォーム化はどのジャンルから進むか？</t>
+        </is>
+      </c>
+      <c r="C91" s="14" t="inlineStr">
+        <is>
+          <t>Crunchyroll創業者のB2Bアニメライセンス市場AniBiz始動（ANN, 7/2）</t>
+        </is>
+      </c>
+      <c r="D91" s="14" t="inlineStr">
+        <is>
+          <t>Nakama, Crunchyroll</t>
+        </is>
+      </c>
+      <c r="E91" s="14" t="inlineStr">
+        <is>
+          <t>音楽カタログ取引, 出版翻訳版権, スポーツ放映権</t>
+        </is>
+      </c>
+      <c r="F91" s="14" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="G91" s="14" t="inlineStr">
+        <is>
+          <t>分断された権利商流ほどPF化の余地が大きい。手数料とデータがPF側に集まる構図</t>
+        </is>
+      </c>
+      <c r="H91" s="14" t="inlineStr">
         <is>
           <t>横断</t>
         </is>
@@ -15296,7 +15422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16111,6 +16237,58 @@
       </c>
       <c r="J16" s="15" t="n">
         <v>5</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>アプリ外決済／Webショップ誘導（プラットフォーム手数料回避）</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="inlineStr">
+        <is>
+          <t>マネタイズ/運営</t>
+        </is>
+      </c>
+      <c r="D17" s="14" t="inlineStr">
+        <is>
+          <t>台頭(加速)</t>
+        </is>
+      </c>
+      <c r="E17" s="14" t="inlineStr">
+        <is>
+          <t>ストア外課金の解禁・規制(DMA/スマホ競争促進法/Epic訴訟)を背景に、パブリッシャーがWeb直販・外部決済へ誘導しApple/Google 30%手数料を回避、マージンを改善する運営設計</t>
+        </is>
+      </c>
+      <c r="F17" s="14" t="inlineStr">
+        <is>
+          <t>Fortnite, 各F2Pタイトル, 駅メモ!</t>
+        </is>
+      </c>
+      <c r="G17" s="14" t="inlineStr">
+        <is>
+          <t>ストア手数料への規制・訴訟の進展と、外部決済導入の実務解禁</t>
+        </is>
+      </c>
+      <c r="H17" s="14" t="inlineStr">
+        <is>
+          <t>手数料30%→15%前後への圧縮が中小のライブサービス採算を改善。ストア誘導UI・決済動線の設計が新たな運営ノウハウに</t>
+        </is>
+      </c>
+      <c r="I17" s="14" t="inlineStr">
+        <is>
+          <t>モバイルファクトリー2Q決算 アプリ外決済で増益（gamebiz, 7/24）</t>
+        </is>
+      </c>
+      <c r="J17" s="14" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -18774,7 +18952,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M389"/>
+  <dimension ref="A1:M410"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -44770,6 +44948,1428 @@
         </is>
       </c>
       <c r="M389" s="14" t="inlineStr"/>
+    </row>
+    <row r="390">
+      <c r="A390" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B390" s="14" t="inlineStr">
+        <is>
+          <t>ゲーム</t>
+        </is>
+      </c>
+      <c r="C390" s="14" t="inlineStr">
+        <is>
+          <t>『ドラクエモンスターズ4』12/3発売決定、超マスターズ版2.5万円まで多層エディション展開</t>
+        </is>
+      </c>
+      <c r="D390" s="14" t="inlineStr">
+        <is>
+          <t>https://www.jp.square-enix.com/topics/detail/4047/</t>
+        </is>
+      </c>
+      <c r="E390" s="14" t="inlineStr">
+        <is>
+          <t>ドラクエ40周年施策の中核として発表された買い切りRPG最新作。5/27発表後、7/24にバトル・配合など具体的なゲームシステム情報が追加公開された。対応はSwitch2/Switch/PS5/Xbox/Steam等マルチ。通常版7,700円〜超マスターズ版25,000円まで複数エディションを用意する。</t>
+        </is>
+      </c>
+      <c r="F390" s="14" t="inlineStr">
+        <is>
+          <t>スクエニは7/24、『ドラゴンクエストモンスターズ4 枯れ木の国のビアンカ・フローラ』(12/3発売)のシステム詳細を公開。通常/マスターズ/超マスターズと価格帯を3層に分け、DL版7,700円から超マスターズ版25,000円まで単価を最大3倍超に設計。買い切りタイトルでも版分けでARPUを引き上げる商法を大型IPで展開する。</t>
+        </is>
+      </c>
+      <c r="G390" s="14" t="inlineStr">
+        <is>
+          <t>買い切り作品でエディションを3層化し実質的な単価最大化
+40周年IPを年末商戦の主力に据えたマルチプラットフォーム展開
+Switch2世代への橋渡し(Switch/Switch2両対応)
+配合・育成というライブ運営に載せやすいコレクション設計</t>
+        </is>
+      </c>
+      <c r="H390" s="14" t="inlineStr">
+        <is>
+          <t>買い切り大作の「超豪華版で単価を積む」手法は、ガチャ規制圧力が強まる中でパブリッシャーの収益補完策として一般化する見込み。DQM4の超マスターズ版の販売比率が高ければ、他の大型和ゲーでも2万円超エディションが定番化し、実質値上げが版差別化の形で進む可能性がある。</t>
+        </is>
+      </c>
+      <c r="I390" s="14" t="inlineStr">
+        <is>
+          <t>買い切りゲームの多層エディション・価格差別化戦略</t>
+        </is>
+      </c>
+      <c r="J390" s="14" t="inlineStr">
+        <is>
+          <t>スクウェア・エニックス</t>
+        </is>
+      </c>
+      <c r="K390" s="14" t="inlineStr">
+        <is>
+          <t>ドラゴンクエストモンスターズ,ドラゴンクエスト</t>
+        </is>
+      </c>
+      <c r="L390" s="14" t="inlineStr">
+        <is>
+          <t>新作,国内,消費者インサイト</t>
+        </is>
+      </c>
+      <c r="M390" s="14" t="inlineStr">
+        <is>
+          <t>5/27発表、7/24にシステム詳細公開</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B391" s="14" t="inlineStr">
+        <is>
+          <t>ゲーム</t>
+        </is>
+      </c>
+      <c r="C391" s="14" t="inlineStr">
+        <is>
+          <t>ガンダム新IP「RGプロジェクト」始動、ゲーム『ROGUE ORBIT』とアニメを同時立ち上げ</t>
+        </is>
+      </c>
+      <c r="D391" s="14" t="inlineStr">
+        <is>
+          <t>https://www.4gamer.net/games/991/G999103/20260724009/</t>
+        </is>
+      </c>
+      <c r="E391" s="14" t="inlineStr">
+        <is>
+          <t>バンダイナムコは7/24、新規ガンダム作品『機動戦士ガンダムRG XARX-ZERO』を発表。SGF2026で公開済のゲーム『GUNDAM ROGUE ORBIT』と世界観を共有し、アニメ・ゲーム・ガンプラを束ねる「RGプロジェクト」として展開する。SF設定監修に円城塔、監督に神山健治を起用した。</t>
+        </is>
+      </c>
+      <c r="F391" s="14" t="inlineStr">
+        <is>
+          <t>バンダイナムコは既存アニメの後追いでゲーム化する従来型でなく、ゲーム『ROGUE ORBIT』とアニメ『RG XARX-ZERO』、ガンプラを最初から同一世界観で同時設計する新IP「RGプロジェクト」を始動。2027年展開予定。単一メディア原作に依存せず、立ち上げ段階から複数窓口の収益を織り込むIP設計を示した。</t>
+        </is>
+      </c>
+      <c r="G391" s="14" t="inlineStr">
+        <is>
+          <t>アニメ後追いのゲーム化でなく、ゲーム・アニメ・玩具を同時設計する「同時立ち上げ型」IP
+SGF2026でゲーム先行公開→7/24にアニメ解禁の順で話題を積む設計
+神山健治・円城塔起用で作家性を担保
+ガンプラ商品化を初報時点で同時発表しマーチャンダイズを即接続</t>
+        </is>
+      </c>
+      <c r="H391" s="14" t="inlineStr">
+        <is>
+          <t>大型IPホルダーは、既存作のメディアミックスでなく「最初から多メディア同時設計」する立ち上げが増える見込み。ゲームを世界観の中核(プレイアブルな正史)に据える設計が成功すれば、アニメ→ゲームの一方向でなく、ゲーム主導でアニメ・玩具を派生させる逆流型メディアミックスが定番化する可能性がある。</t>
+        </is>
+      </c>
+      <c r="I391" s="14" t="inlineStr">
+        <is>
+          <t>同時立ち上げ型メディアミックスとIP設計</t>
+        </is>
+      </c>
+      <c r="J391" s="14" t="inlineStr">
+        <is>
+          <t>バンダイナムコフィルムワークス,バンダイナムコエンターテインメント</t>
+        </is>
+      </c>
+      <c r="K391" s="14" t="inlineStr">
+        <is>
+          <t>機動戦士ガンダムRG XARX-ZERO,GUNDAM ROGUE ORBIT,ガンダム</t>
+        </is>
+      </c>
+      <c r="L391" s="14" t="inlineStr">
+        <is>
+          <t>新作,映像化,ゲーム化,国内</t>
+        </is>
+      </c>
+      <c r="M391" s="14" t="inlineStr">
+        <is>
+          <t>2027年展開予定/SF監修:円城塔・監督:神山健治</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B392" s="14" t="inlineStr">
+        <is>
+          <t>ゲーム</t>
+        </is>
+      </c>
+      <c r="C392" s="14" t="inlineStr">
+        <is>
+          <t>モバイルファクトリー2Q増収増益、アプリ外決済導入とストア手数料改定が収益押上げ</t>
+        </is>
+      </c>
+      <c r="D392" s="14" t="inlineStr">
+        <is>
+          <t>https://gamebiz.jp/news/429846</t>
+        </is>
+      </c>
+      <c r="E392" s="14" t="inlineStr">
+        <is>
+          <t>プラットフォーム手数料(Apple/Google 30%)への規制・訴訟が世界的に進む中、日本でもスマホソフトウェア競争促進法などを背景に外部決済への誘導が現実味を帯びる。モバイルファクトリーは位置ゲー『駅メモ!』を主力に、アプリ外決済導入とプラットフォーム手数料改定の効果を業績に反映した。</t>
+        </is>
+      </c>
+      <c r="F392" s="14" t="inlineStr">
+        <is>
+          <t>モバイルファクトリーは7/24発表の2Q決算で増収増益を確保。『駅メモ!』の伸長に加え、アプリ外決済の導入とプラットフォーム手数料改定が利益率改善に寄与したと説明。ストア30%手数料の回避がモバイルゲームのマージンに直接効くことを、上場企業の適時開示という形で可視化した事例となる。</t>
+        </is>
+      </c>
+      <c r="G392" s="14" t="inlineStr">
+        <is>
+          <t>アプリ外決済の導入が利益に直接寄与したと説明
+位置ゲー『駅メモ!』のライブ運営が売上を下支え
+ストア手数料規制の恩恵を受ける中小パブリッシャーの先行例
+手数料改定=実質的なマージン改善が業績数値で確認できる</t>
+        </is>
+      </c>
+      <c r="H392" s="14" t="inlineStr">
+        <is>
+          <t>ストア外課金の解禁が進むほど、Web直販・外部決済への誘導設計が中小パブリッシャーの標準になる見込み。手数料30%が15%前後に圧縮されれば、限界的なライブサービス運営の採算ラインが下がり、これまで畳んでいた中規模タイトルの延命や新規参入が増える可能性がある。</t>
+        </is>
+      </c>
+      <c r="I392" s="14" t="inlineStr">
+        <is>
+          <t>ストア手数料規制とアプリ外決済のマージン影響</t>
+        </is>
+      </c>
+      <c r="J392" s="14" t="inlineStr">
+        <is>
+          <t>モバイルファクトリー</t>
+        </is>
+      </c>
+      <c r="K392" s="14" t="inlineStr">
+        <is>
+          <t>駅メモ!</t>
+        </is>
+      </c>
+      <c r="L392" s="14" t="inlineStr">
+        <is>
+          <t>業績,適時開示,ライブサービス,国内</t>
+        </is>
+      </c>
+      <c r="M392" s="14" t="inlineStr">
+        <is>
+          <t>2Q決算(7/24発表)</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B393" s="14" t="inlineStr">
+        <is>
+          <t>ゲーム</t>
+        </is>
+      </c>
+      <c r="C393" s="14" t="inlineStr">
+        <is>
+          <t>ドイツ発インディーが相次ぎ台頭、公的支援と国別Steam企画が発見性を後押し</t>
+        </is>
+      </c>
+      <c r="D393" s="14" t="inlineStr">
+        <is>
+          <t>https://www.gamesmarket.global/gamesmarket-daily-20-july-26-eu-funding-assemble-x-pithead-gryphon-games-leyline-ac-black-flag/</t>
+        </is>
+      </c>
+      <c r="E393" s="14" t="inlineStr">
+        <is>
+          <t>EU・ドイツはゲーム制作への公的助成を拡充し、「Games Made in Germany」等の国別Steam企画で自国タイトルの露出を組織的に支援している。7/20の企画では400本超の独産ゲームが集結。ミュンヘン拠点のLeylineは新作Guildrunが発表4日で10万ウィッシュリストを獲得した。</t>
+        </is>
+      </c>
+      <c r="F393" s="14" t="inlineStr">
+        <is>
+          <t>7月下旬、ドイツ発インディー(Leyline『Guildrun』、Aesir『EverRail』等)の話題化が相次いだ。背景にはEU/独の公的助成と「Games Made in Germany」など国別Steamセールによる発見性支援がある。プラットフォームのアルゴリズム任せでなく、国策としてインディーの露出を作る動きが成果を見せ始めている。</t>
+        </is>
+      </c>
+      <c r="G393" s="14" t="inlineStr">
+        <is>
+          <t>EU/独の公的助成＋国別Steam企画で自国インディーの露出を組織化
+Leyline『Guildrun』が発表4日で10万ウィッシュリスト
+Aesir『EverRail』が自社パブリッシングでEA参入
+発見性(ウィッシュリスト獲得)を政策・企画で底上げする手法</t>
+        </is>
+      </c>
+      <c r="H393" s="14" t="inlineStr">
+        <is>
+          <t>Steamの発見性が飽和する中、国・地域単位でセール企画や助成を束ねて自国タイトルを押し出す「産業政策としてのインディー支援」が各国に広がる見込み。日本でもCEDEC/BitSummitや自治体助成と連動した国別露出企画が強化されれば、露出格差の是正が進む可能性がある。</t>
+        </is>
+      </c>
+      <c r="I393" s="14" t="inlineStr">
+        <is>
+          <t>国策インディー支援とSteam発見性</t>
+        </is>
+      </c>
+      <c r="J393" s="14" t="inlineStr">
+        <is>
+          <t>Leyline,Aesir Interactive,Games Germany</t>
+        </is>
+      </c>
+      <c r="K393" s="14" t="inlineStr">
+        <is>
+          <t>Guildrun,EverRail</t>
+        </is>
+      </c>
+      <c r="L393" s="14" t="inlineStr">
+        <is>
+          <t>インディー,海外,トレンド</t>
+        </is>
+      </c>
+      <c r="M393" s="14" t="inlineStr">
+        <is>
+          <t>週次ラウンドアップ(7/20週)</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B394" s="14" t="inlineStr">
+        <is>
+          <t>映画</t>
+        </is>
+      </c>
+      <c r="C394" s="14" t="inlineStr">
+        <is>
+          <t>『映画ちいかわ』初日興収9.3億で歴代8位、池袋41回/日の鬼滅級上映で100億視野</t>
+        </is>
+      </c>
+      <c r="D394" s="14" t="inlineStr">
+        <is>
+          <t>https://www.oricon.co.jp/news/2469356/full/</t>
+        </is>
+      </c>
+      <c r="E394" s="14" t="inlineStr">
+        <is>
+          <t>ナガノ原作『ちいかわ』は台詞が少なく物語性より世界観・キャラ愛着で支持される「キャラ強・物語希薄型」IP。7/24公開の劇場版は、TOHOシネマズ池袋で1日41回上映など『鬼滅の刃』『名探偵コナン』級の大規模ブッキングで封切られた。</t>
+        </is>
+      </c>
+      <c r="F394" s="14" t="inlineStr">
+        <is>
+          <t>『映画ちいかわ 人魚の島のひみつ』は7/24初日推定興収9.3億円で日本歴代8位の大型スタート。池袋41回/新宿29回など超高頻度上映で公開され、年内3本目の100億超が視野に。物語性の薄いキャラクターIPでも、愛着とグッズ経済を束ねれば国民的アニメ映画級の初動を出せることを実証した。</t>
+        </is>
+      </c>
+      <c r="G394" s="14" t="inlineStr">
+        <is>
+          <t>初日推定9.3億円は日本歴代8位クラスの特大発進
+池袋41回/日など鬼滅・コナン級の上映規模を確保
+「キャラ強・物語希薄IP」の劇場動員力を数字で実証
+転売・多回上映など供給側の過熱も発生</t>
+        </is>
+      </c>
+      <c r="H394" s="14" t="inlineStr">
+        <is>
+          <t>ちいかわの成功で、配給・出版は「物語より愛着」を核とするキャラIPの劇場化に一段と傾斜する見込み。SNS発キャラなど連続した物語を持たないIPの映画化が増え、上映規模を先に押さえる大量ブッキング戦略が中規模作品を締め出す二極化を強める可能性がある。</t>
+        </is>
+      </c>
+      <c r="I394" s="14" t="inlineStr">
+        <is>
+          <t>キャラクターIPの劇場動員とブッキング戦略</t>
+        </is>
+      </c>
+      <c r="J394" s="14" t="inlineStr">
+        <is>
+          <t>東宝,アニプレックス</t>
+        </is>
+      </c>
+      <c r="K394" s="14" t="inlineStr">
+        <is>
+          <t>ちいかわ</t>
+        </is>
+      </c>
+      <c r="L394" s="14" t="inlineStr">
+        <is>
+          <t>興行,消費者インサイト,国内</t>
+        </is>
+      </c>
+      <c r="M394" s="14" t="inlineStr">
+        <is>
+          <t>7/24公開。既存の『ちいかわ型劇場化』予測を裏付け</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B395" s="14" t="inlineStr">
+        <is>
+          <t>映画</t>
+        </is>
+      </c>
+      <c r="C395" s="14" t="inlineStr">
+        <is>
+          <t>『Project Hail Mary』105日の劇場ウィンドウ経てPrime Videoへ、45日標準に逆行</t>
+        </is>
+      </c>
+      <c r="D395" s="14" t="inlineStr">
+        <is>
+          <t>https://deadline.com/2026/07/project-hail-mary-prime-video-release-date-1236972341/</t>
+        </is>
+      </c>
+      <c r="E395" s="14" t="inlineStr">
+        <is>
+          <t>コロナ後、劇場→配信のウィンドウは45日が新常態化した。だがAmazon MGMのライアン・ゴズリング主演SF大作『Project Hail Mary』(世界興収約6.8億ドル)は、劇場体験を優先し公開から105日という長い窓を経てPrime Videoへ移行した。</t>
+        </is>
+      </c>
+      <c r="F395" s="14" t="inlineStr">
+        <is>
+          <t>Amazon MGMは同社最大級ヒットの『Project Hail Mary』を、45日標準に逆行して105日の劇場ウィンドウを設定しPrime Videoで配信開始。配信オリジナル志向の強かったAmazonが、大作は劇場を長く回して興収を最大化する方針に転じた。大作は窓を延ばし収益を積む戦略の代表例となる。</t>
+        </is>
+      </c>
+      <c r="G395" s="14" t="inlineStr">
+        <is>
+          <t>45日標準に対し105日と倍以上の劇場ウィンドウ
+配信主導だったAmazon MGMが大作は劇場優先に転換
+世界興収約6.8億ドルで2026年世界2位級のヒット
+劇場を『配信の露出装置』でなく収益源として再評価</t>
+        </is>
+      </c>
+      <c r="H395" s="14" t="inlineStr">
+        <is>
+          <t>配信プラットフォーマーほど、大作は劇場ウィンドウを延ばして興収と話題を積み、中小作は配信直行させる二極運用に向かう見込み。劇場チェーンが大作専用ハコ化する一方、中堅作向けスクリーンの稼働が落ち、配給の交渉力が劇場側からストリーマー側へ移る流れが強まる可能性がある。</t>
+        </is>
+      </c>
+      <c r="I395" s="14" t="inlineStr">
+        <is>
+          <t>劇場ウィンドウ戦略とストリーマーの収益設計</t>
+        </is>
+      </c>
+      <c r="J395" s="14" t="inlineStr">
+        <is>
+          <t>Amazon MGM Studios,Amazon</t>
+        </is>
+      </c>
+      <c r="K395" s="14" t="inlineStr">
+        <is>
+          <t>Project Hail Mary</t>
+        </is>
+      </c>
+      <c r="L395" s="14" t="inlineStr">
+        <is>
+          <t>興行,配信,海外,トレンド</t>
+        </is>
+      </c>
+      <c r="M395" s="14" t="inlineStr">
+        <is>
+          <t>劇場公開から105日でPrime Video配信</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B396" s="14" t="inlineStr">
+        <is>
+          <t>映画</t>
+        </is>
+      </c>
+      <c r="C396" s="14" t="inlineStr">
+        <is>
+          <t>ケヴィン・ハート『72 Hours』Netflix直行公開、中堅作の劇場スキップが定着</t>
+        </is>
+      </c>
+      <c r="D396" s="14" t="inlineStr">
+        <is>
+          <t>https://www.hollywoodreporter.com/tv/tv-news/netflix-july-2026-new-releases-movies-tv-1236634437/</t>
+        </is>
+      </c>
+      <c r="E396" s="14" t="inlineStr">
+        <is>
+          <t>大作が劇場ウィンドウを延ばす一方、スター主演でも中規模のコメディ・アクションは劇場を通さずストリーミング直行する二極化が進む。ケヴィン・ハート主演『72 Hours』は7/24にNetflixで劇場公開を挟まず配信された。</t>
+        </is>
+      </c>
+      <c r="F396" s="14" t="inlineStr">
+        <is>
+          <t>Netflixは7/24、ケヴィン・ハート主演『72 Hours』を劇場を通さず独占配信。スター主演でも中堅規模作は劇場興行のリスクを取らず、加入者維持の弾として配信直行させる運用が定着しつつある。『Project Hail Mary』の劇場窓延長と対をなし、作品規模による窓口戦略の二極化を示す。</t>
+        </is>
+      </c>
+      <c r="G396" s="14" t="inlineStr">
+        <is>
+          <t>スター主演でも中堅作は劇場を挟まず配信直行
+劇場興行の不確実性を避け加入者維持の材料に
+大作=劇場窓延長／中堅=配信直行の二極化が鮮明
+劇場が扱う作品が大作に偏り中間層が痩せる</t>
+        </is>
+      </c>
+      <c r="H396" s="14" t="inlineStr">
+        <is>
+          <t>中規模作の配信直行が常態化すると、劇場は大作専用の場に純化し、俳優・スタッフの中規模作品の経験値が配信案件に移る。結果として劇場向け中間予算帯の企画が痩せ、興行の作品ポートフォリオが『特大か配信か』に二極化する流れが加速する可能性がある。</t>
+        </is>
+      </c>
+      <c r="I396" s="14" t="inlineStr">
+        <is>
+          <t>配信直行と劇場興行の二極化</t>
+        </is>
+      </c>
+      <c r="J396" s="14" t="inlineStr">
+        <is>
+          <t>Netflix</t>
+        </is>
+      </c>
+      <c r="K396" s="14" t="inlineStr">
+        <is>
+          <t>72 Hours</t>
+        </is>
+      </c>
+      <c r="L396" s="14" t="inlineStr">
+        <is>
+          <t>配信,海外,トレンド</t>
+        </is>
+      </c>
+      <c r="M396" s="14" t="inlineStr">
+        <is>
+          <t>7/24 Netflix独占配信</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B397" s="14" t="inlineStr">
+        <is>
+          <t>映画</t>
+        </is>
+      </c>
+      <c r="C397" s="14" t="inlineStr">
+        <is>
+          <t>『アバター：ファイア・アンド・アッシュ』Disney+配信開始、超大作の配信着地で10億分再生</t>
+        </is>
+      </c>
+      <c r="D397" s="14" t="inlineStr">
+        <is>
+          <t>https://furtherandbetter.substack.com/p/global-tv-film-and-media-industry-7d8</t>
+        </is>
+      </c>
+      <c r="E397" s="14" t="inlineStr">
+        <is>
+          <t>劇場で世界興収約14.8億ドルを稼いだジェームズ・キャメロン監督『アバター：ファイア・アンド・アッシュ』が、劇場興行を完走したのちDisney+で配信を開始。超大作が劇場で最大限に回収した後に配信へ着地する典型的なウィンドウ運用の事例となった。</t>
+        </is>
+      </c>
+      <c r="F397" s="14" t="inlineStr">
+        <is>
+          <t>週次の映像業界動向で、『アバター：ファイア・アンド・アッシュ』(劇場世界興収約14.8億ドル)がDisney+配信初日に10億分超の再生を記録したことが報じられた。劇場で回収を完了した超大作を配信の獲得・維持エンジンとして再利用する流れを示し、大作の窓口戦略(劇場→配信)の効果を可視化した。</t>
+        </is>
+      </c>
+      <c r="G397" s="14" t="inlineStr">
+        <is>
+          <t>劇場世界興収約14.8億ドルの超大作が配信着地
+Disney+初日に10億分超の再生
+劇場完走後に配信で二次的な話題と加入維持を得る設計
+大作の『劇場で回収→配信で維持』モデルの実証</t>
+        </is>
+      </c>
+      <c r="H397" s="14" t="inlineStr">
+        <is>
+          <t>自社配信を持つスタジオは、超大作を劇場で長く回して興収を積み、配信では加入維持のフックとして再利用する二段構えを標準化する見込み。劇場と配信を対立でなく補完として設計する運用が広がり、大作の劇場ウィンドウはむしろ延びる方向に働く可能性がある。</t>
+        </is>
+      </c>
+      <c r="I397" s="14" t="inlineStr">
+        <is>
+          <t>超大作の劇場→配信ウィンドウ設計</t>
+        </is>
+      </c>
+      <c r="J397" s="14" t="inlineStr">
+        <is>
+          <t>ディズニー,20世紀スタジオ</t>
+        </is>
+      </c>
+      <c r="K397" s="14" t="inlineStr">
+        <is>
+          <t>アバター：ファイア・アンド・アッシュ</t>
+        </is>
+      </c>
+      <c r="L397" s="14" t="inlineStr">
+        <is>
+          <t>配信,興行,海外</t>
+        </is>
+      </c>
+      <c r="M397" s="14" t="inlineStr">
+        <is>
+          <t>週次業界ラウンドアップより</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B398" s="14" t="inlineStr">
+        <is>
+          <t>映画</t>
+        </is>
+      </c>
+      <c r="C398" s="14" t="inlineStr">
+        <is>
+          <t>ノーラン『The Odyssey』北米初週1.99億ドル、監督歴代3位でオリジナル大作の底力</t>
+        </is>
+      </c>
+      <c r="D398" s="14" t="inlineStr">
+        <is>
+          <t>https://deadline.com/2026/07/the-odyssey-box-office-wednesday-1237001757/</t>
+        </is>
+      </c>
+      <c r="E398" s="14" t="inlineStr">
+        <is>
+          <t>続編・リメイク偏重が続くハリウッドで、クリストファー・ノーランのオリジナル大作『The Odyssey』が公開。初週の北米興収は1.993億ドルに達し、ノーラン作品では『ダークナイト』『同ライジング』に次ぐ歴代3位、『オッペンハイマー』『インセプション』を上回った。</t>
+        </is>
+      </c>
+      <c r="F398" s="14" t="inlineStr">
+        <is>
+          <t>ノーラン監督『The Odyssey』は北米初週1.993億ドルを記録し、監督の生涯作品中3位の初動。既存IPでなく作家性主導のオリジナル大作が、フランチャイズ大作に匹敵する初動を出せることを改めて示した。IP頼みの企画が飽和するなか、監督ブランドが集客装置になる構図を裏付ける。</t>
+        </is>
+      </c>
+      <c r="G398" s="14" t="inlineStr">
+        <is>
+          <t>北米初週1.993億ドルはノーラン作品歴代3位
+オリジナル(非IP)大作でフランチャイズ級の初動
+監督ブランドそのものが集客装置として機能
+続編疲れの中でのオリジナル回帰の追い風</t>
+        </is>
+      </c>
+      <c r="H398" s="14" t="inlineStr">
+        <is>
+          <t>ノーランら『監督名で客を呼べる』作家の大作は、IP依存の疲弊が指摘される市場でスタジオの安全資産として価値を増す見込み。結果として、フランチャイズ量産の一方で、限られたトップ監督のオリジナル大作に予算とプレミアム上映枠が集中する二極化が進む可能性がある。</t>
+        </is>
+      </c>
+      <c r="I398" s="14" t="inlineStr">
+        <is>
+          <t>監督ブランドとオリジナル大作の興行力</t>
+        </is>
+      </c>
+      <c r="J398" s="14" t="inlineStr">
+        <is>
+          <t>ユニバーサル・ピクチャーズ</t>
+        </is>
+      </c>
+      <c r="K398" s="14" t="inlineStr">
+        <is>
+          <t>The Odyssey</t>
+        </is>
+      </c>
+      <c r="L398" s="14" t="inlineStr">
+        <is>
+          <t>興行,海外</t>
+        </is>
+      </c>
+      <c r="M398" s="14" t="inlineStr">
+        <is>
+          <t>初週北米1.993億ドル</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B399" s="14" t="inlineStr">
+        <is>
+          <t>アニメ</t>
+        </is>
+      </c>
+      <c r="C399" s="14" t="inlineStr">
+        <is>
+          <t>神山健治監督の新作ガンダム『RG XARX-ZERO』制作決定、2027年展開・円城塔がSF監修</t>
+        </is>
+      </c>
+      <c r="D399" s="14" t="inlineStr">
+        <is>
+          <t>https://www.animatetimes.com/news/details.php?id=1784795121</t>
+        </is>
+      </c>
+      <c r="E399" s="14" t="inlineStr">
+        <is>
+          <t>バンダイナムコフィルムワークスは7/24、完全新作ガンダム『機動戦士ガンダムRG XARX-ZERO(アレックスゼロ)』の制作を発表。『攻殻機動隊SAC』等の神山健治が監督・シリーズ構成、SF設定監修に芥川賞作家・円城塔を起用。ゲーム『GUNDAM ROGUE ORBIT』と世界観を共有する。</t>
+        </is>
+      </c>
+      <c r="F399" s="14" t="inlineStr">
+        <is>
+          <t>新作アニメ『ガンダムRG XARX-ZERO』が7/24発表。神山健治監督・円城塔SF監修という作家性の強い布陣で、2027年に展開予定。ゲーム『ROGUE ORBIT』やガンプラと連動する「RGプロジェクト」の映像軸を担う。長寿IPの新規シリーズに、映画・文芸級の作家を招いて質を担保する潮流を象徴する。</t>
+        </is>
+      </c>
+      <c r="G399" s="14" t="inlineStr">
+        <is>
+          <t>神山健治(監督)＋円城塔(SF設定監修)の作家性重視布陣
+ゲーム・ガンプラと世界観を共有する『RGプロジェクト』の映像軸
+主人公アズミ・レイ役に大塚剛央
+2027年展開予定、初報でガンプラ・玩具も同時発表</t>
+        </is>
+      </c>
+      <c r="H399" s="14" t="inlineStr">
+        <is>
+          <t>長寿アニメIPは、外部の映画監督・小説家など高名なクリエイターを招いて作家性と話題を確保する路線を強める見込み。ガンダムのように、ゲーム・玩具と同時設計された新シリーズが増え、アニメ単体でなくIPプロジェクト全体で採算を組む企画が主流化する可能性がある。</t>
+        </is>
+      </c>
+      <c r="I399" s="14" t="inlineStr">
+        <is>
+          <t>長寿IPへの外部作家起用とプロジェクト型制作</t>
+        </is>
+      </c>
+      <c r="J399" s="14" t="inlineStr">
+        <is>
+          <t>バンダイナムコフィルムワークス,バンダイナムコ</t>
+        </is>
+      </c>
+      <c r="K399" s="14" t="inlineStr">
+        <is>
+          <t>機動戦士ガンダムRG XARX-ZERO,ガンダム</t>
+        </is>
+      </c>
+      <c r="L399" s="14" t="inlineStr">
+        <is>
+          <t>新作,ゲーム化,国内</t>
+        </is>
+      </c>
+      <c r="M399" s="14" t="inlineStr">
+        <is>
+          <t>2027年展開/ゲームROGUE ORBITと連動</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B400" s="14" t="inlineStr">
+        <is>
+          <t>アニメ</t>
+        </is>
+      </c>
+      <c r="C400" s="14" t="inlineStr">
+        <is>
+          <t>アニメ制作会社の資本再編が加速、配信・出版が垂直統合し制作を『権利保有側』へ</t>
+        </is>
+      </c>
+      <c r="D400" s="14" t="inlineStr">
+        <is>
+          <t>https://news.yahoo.co.jp/articles/c7cd7ef4524c1dac98e8c4459947011a9a8e0882</t>
+        </is>
+      </c>
+      <c r="E400" s="14" t="inlineStr">
+        <is>
+          <t>慢性的な人手不足と制作費高騰の中、アニメ制作会社の資本提携・買収が相次ぐ。2026年にはGoHandsがU-NEXT HDの完全子会社に、読売新聞グループが読売テレビからYTEを子会社化。2025年にはWHITE FOXが出版社アルファポリス傘下入り。MAPPAやTwin Engineなど制作会社が権利を握る動きも顕在化している。</t>
+        </is>
+      </c>
+      <c r="F400" s="14" t="inlineStr">
+        <is>
+          <t>配信(U-NEXT)・出版(アルファポリス)・メディア(読売)がアニメ制作会社を相次いで傘下に収め、制作機能の垂直統合が進む。同時に、制作会社自身が作品の権利を保有・活用する動きも強まる。制作を『発注される下請け』から『権利を持つ資産』へ再定義する構造変化が、資本再編という形で一気に表面化している。</t>
+        </is>
+      </c>
+      <c r="G400" s="14" t="inlineStr">
+        <is>
+          <t>U-NEXT×GoHands、読売×YTE、アルファポリス×WHITE FOX等の相次ぐ買収
+配信・出版・メディアによる制作機能の垂直統合
+MAPPA/Twin Engine型の『制作会社が権利を握る』流れ
+人手不足・制作費高騰が再編の駆動力</t>
+        </is>
+      </c>
+      <c r="H400" s="14" t="inlineStr">
+        <is>
+          <t>配信・出版が制作会社を囲い込むほど、権利を持たない純受託スタジオは価格交渉力を失う。逆に権利保有に舵を切れる制作会社は資本を集めやすくなり、『権利を持つ制作会社』と『持たない下請け』への二極化と、原作を握る出版社の内製化圧力が同時に進む可能性がある。</t>
+        </is>
+      </c>
+      <c r="I400" s="14" t="inlineStr">
+        <is>
+          <t>アニメ制作の垂直統合と権利保有シフト</t>
+        </is>
+      </c>
+      <c r="J400" s="14" t="inlineStr">
+        <is>
+          <t>U-NEXT HOLDINGS,読売新聞グループ,アルファポリス,GoHands</t>
+        </is>
+      </c>
+      <c r="K400" s="14" t="inlineStr"/>
+      <c r="L400" s="14" t="inlineStr">
+        <is>
+          <t>M&amp;A,配信,出版,国内,トレンド</t>
+        </is>
+      </c>
+      <c r="M400" s="14" t="inlineStr">
+        <is>
+          <t>2025-2026の複数事例を横断分析</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B401" s="14" t="inlineStr">
+        <is>
+          <t>アニメ</t>
+        </is>
+      </c>
+      <c r="C401" s="14" t="inlineStr">
+        <is>
+          <t>Crunchyroll創業者、B2Bアニメライセンス市場『AniBiz』始動、商流のプラットフォーム化</t>
+        </is>
+      </c>
+      <c r="D401" s="14" t="inlineStr">
+        <is>
+          <t>https://www.animenewsnetwork.com/news/2026-07-06/crunchyroll-co-founder-former-ceo-kun-gao-launches-anibiz-platform-for-anime-licensing/.239248</t>
+        </is>
+      </c>
+      <c r="E401" s="14" t="inlineStr">
+        <is>
+          <t>アニメのライセンスは製作委員会・権利元ごとに分断され、海外バイヤーが権利を取得するまでの商流が煩雑だった。Crunchyroll共同創業者クン・ガオ率いるNakamaは7/2、権利元とライセンシーを直接つなぐ初のB2Bアニメ市場『AniBiz』を全世界のバイヤー向けに公開した。</t>
+        </is>
+      </c>
+      <c r="F401" s="14" t="inlineStr">
+        <is>
+          <t>AniBizは分断されたアニメライセンス商流を集約するB2Bマーケットプレイス。無料プランで権利元プロフィールを公開し、月額49ドルの有料版で作品・製作委員会などの詳細データにアクセスできる。アニプレックスや東映などのIPも掲載。ライセンス取引そのものをプラットフォーム化し、権利流通の透明性とスピードを上げる試みだ。</t>
+        </is>
+      </c>
+      <c r="G401" s="14" t="inlineStr">
+        <is>
+          <t>権利元とライセンシーを直接つなぐ初のB2Bアニメ市場
+無料プラン＋月額49ドルの有料データアクセスのフリーミアム
+アニプレックス・東映など大手IPも参加
+ライセンス商流の透明化とスピードアップを狙う</t>
+        </is>
+      </c>
+      <c r="H401" s="14" t="inlineStr">
+        <is>
+          <t>ライセンス取引のマーケットプレイス化が定着すれば、権利元は仲介コストを下げつつ海外露出を広げられ、後発の中小権利元にも取引機会が開く。一方でプラットフォーム側にデータと手数料が集まり、Crunchyroll系が『配信』に続き『ライセンス商流』でも影響力を持つ構図が生まれる可能性がある。</t>
+        </is>
+      </c>
+      <c r="I401" s="14" t="inlineStr">
+        <is>
+          <t>ライセンス商流のプラットフォーム化(B2B市場)</t>
+        </is>
+      </c>
+      <c r="J401" s="14" t="inlineStr">
+        <is>
+          <t>Nakama,Crunchyroll,アニプレックス,東映</t>
+        </is>
+      </c>
+      <c r="K401" s="14" t="inlineStr"/>
+      <c r="L401" s="14" t="inlineStr">
+        <is>
+          <t>権利・ライセンス,技術,海外,トレンド</t>
+        </is>
+      </c>
+      <c r="M401" s="14" t="inlineStr">
+        <is>
+          <t>7/2ローンチ、President クン・ガオ</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B402" s="14" t="inlineStr">
+        <is>
+          <t>アニメ</t>
+        </is>
+      </c>
+      <c r="C402" s="14" t="inlineStr">
+        <is>
+          <t>2026夏アニメは50本超＋Crunchyroll追加13本、配信カタログの供給過多と選別</t>
+        </is>
+      </c>
+      <c r="D402" s="14" t="inlineStr">
+        <is>
+          <t>https://www.cbr.com/crunchyroll-anime-summer-2026-streaming-release-date-update/</t>
+        </is>
+      </c>
+      <c r="E402" s="14" t="inlineStr">
+        <is>
+          <t>制作本数の高止まりで、2026年夏クールは新作50本超が並走。Crunchyrollはこの夏さらに13本を追加投入する一方、旧作の大量削除も継続しており、配信カタログは『新作の氾濫』と『旧作の空白』が同時進行している。</t>
+        </is>
+      </c>
+      <c r="F402" s="14" t="inlineStr">
+        <is>
+          <t>2026夏アニメは新作50本超に加え、Crunchyrollが13本を追加。視聴者の可処分時間を超える供給過多で、話題の集中と埋没の格差が拡大している。同時に権利期限切れによる旧作削除も続き、配信は『大量の新作を投下しつつ古典が消える』カタログ構造へ。作品数でなく話題設計が生死を分ける局面に入った。</t>
+        </is>
+      </c>
+      <c r="G402" s="14" t="inlineStr">
+        <is>
+          <t>夏クール新作50本超＋Crunchyroll追加13本の供給過多
+可処分時間を超える本数で話題の集中・埋没が二極化
+権利期限切れで旧作の削除も並行
+作品数競争から話題設計・独占確保の競争へ</t>
+        </is>
+      </c>
+      <c r="H402" s="14" t="inlineStr">
+        <is>
+          <t>供給過多が続くほど、配信各社は本数でなく『独占』と『話題化の初速』で差別化せざるを得ず、初動プロモに資源が偏る見込み。埋没する中堅作の採算が悪化し、製作委員会が本数を絞る調整に入る一方、削除された古典の受け皿として二次配信・アーカイブの価値が見直される可能性がある。</t>
+        </is>
+      </c>
+      <c r="I402" s="14" t="inlineStr">
+        <is>
+          <t>配信カタログの供給過多と話題設計</t>
+        </is>
+      </c>
+      <c r="J402" s="14" t="inlineStr">
+        <is>
+          <t>Crunchyroll,ソニー</t>
+        </is>
+      </c>
+      <c r="K402" s="14" t="inlineStr"/>
+      <c r="L402" s="14" t="inlineStr">
+        <is>
+          <t>配信,トレンド,海外</t>
+        </is>
+      </c>
+      <c r="M402" s="14" t="inlineStr">
+        <is>
+          <t>夏クールの供給動向</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B403" s="14" t="inlineStr">
+        <is>
+          <t>漫画</t>
+        </is>
+      </c>
+      <c r="C403" s="14" t="inlineStr">
+        <is>
+          <t>ゲーム『都市伝説解体センター』コミカライズ連載開始、インディーIPの多メディア展開</t>
+        </is>
+      </c>
+      <c r="D403" s="14" t="inlineStr">
+        <is>
+          <t>https://mantan-web.jp/article/20260722dog00m200073000a.html</t>
+        </is>
+      </c>
+      <c r="E403" s="14" t="inlineStr">
+        <is>
+          <t>『都市伝説解体センター』はインディー発のミステリーADVとしてヒットし、公式ノベライズも展開してきた。7/24、集英社『となりのヤングジャンプ』で新作コミカライズ『Another Record』が連載開始。本編の正史から分岐したオリジナル・スピンオフで、ノベライズ短編を書いた月並きらが脚本を担当する。</t>
+        </is>
+      </c>
+      <c r="F403" s="14" t="inlineStr">
+        <is>
+          <t>インディーゲーム『都市伝説解体センター』のコミカライズ『Another Record』が7/24、となりのヤングジャンプで連載スタート。既存の展開と異なり、ゲーム→小説→漫画とジャンルを跨いでオリジナル正史を増殖させる展開で、第1話はゲーム画面を再現したブラウザ特別版も用意。小規模IPが多メディアで世界を広げる好例だ。</t>
+        </is>
+      </c>
+      <c r="G403" s="14" t="inlineStr">
+        <is>
+          <t>インディーゲーム発IPが小説に続き漫画へ多メディア展開
+大手集英社のWeb誌で連載、原作愛を保つオリジナル正史
+第1話にゲーム画面再現のブラウザ特別版
+個人・小規模発IPでもメディアミックスで拡張できる実例</t>
+        </is>
+      </c>
+      <c r="H403" s="14" t="inlineStr">
+        <is>
+          <t>話題性のあるインディーゲームIPを、大手出版社が早期にコミカライズ・ノベライズで取り込む動きが増える見込み。ゲームスタジオには露出と収益の窓口が広がり、出版社には新規IP調達源になる。個人・小規模発のIPが多メディア化する経路が制度化していく可能性がある。</t>
+        </is>
+      </c>
+      <c r="I403" s="14" t="inlineStr">
+        <is>
+          <t>インディーゲームIPのメディアミックス経路</t>
+        </is>
+      </c>
+      <c r="J403" s="14" t="inlineStr">
+        <is>
+          <t>集英社</t>
+        </is>
+      </c>
+      <c r="K403" s="14" t="inlineStr">
+        <is>
+          <t>都市伝説解体センター</t>
+        </is>
+      </c>
+      <c r="L403" s="14" t="inlineStr">
+        <is>
+          <t>コミカライズ,ゲーム化,国内</t>
+        </is>
+      </c>
+      <c r="M403" s="14" t="inlineStr">
+        <is>
+          <t>7/24となりのヤングジャンプで連載開始</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B404" s="14" t="inlineStr">
+        <is>
+          <t>漫画</t>
+        </is>
+      </c>
+      <c r="C404" s="14" t="inlineStr">
+        <is>
+          <t>ウェブトゥーン市場、2026年に約1.4兆円へ急拡大——縦読みへの出版社対応が本格化</t>
+        </is>
+      </c>
+      <c r="D404" s="14" t="inlineStr">
+        <is>
+          <t>https://www.fortunebusinessinsights.com/webcomics-market-105731</t>
+        </is>
+      </c>
+      <c r="E404" s="14" t="inlineStr">
+        <is>
+          <t>縦スクロール漫画(Webtoon)は韓国発で世界的に拡大。市場規模は2025年の約107.5億ドルから2026年に約140.2億ドル(CAGR約30%)へ伸びると見込まれる。日本でも電子コミック利用者の約9割がWebtoonを認知し、7割超が閲覧経験を持つなど普及が進む。</t>
+        </is>
+      </c>
+      <c r="F404" s="14" t="inlineStr">
+        <is>
+          <t>各種調査で、Webtoon市場が2026年に約140億ドル規模へ急拡大する見通しが示された。日本の紙・電子コミックが横ばい〜微減で推移する中、縦読みは高成長を維持。出版社は縦読み専用レーベルやスタジオ体制、物販などのファンエンゲージメント施策で対応を本格化しつつある。伝統的コマ割り漫画との併存が焦点になる。</t>
+        </is>
+      </c>
+      <c r="G404" s="14" t="inlineStr">
+        <is>
+          <t>2026年に約140億ドル、CAGR約30%の高成長見通し
+日本でも認知9割・閲覧経験7割超と普及
+紙・電子コミック横ばいの中で縦読みが成長を牽引
+出版社は専用レーベル・スタジオ・物販で対応</t>
+        </is>
+      </c>
+      <c r="H404" s="14" t="inlineStr">
+        <is>
+          <t>縦読みの成長が続けば、出版社は『作家×編集』の従来型制作から、分業・量産に適した縦読みスタジオ体制への投資を迫られる。一方で量産・型化による創作性低下への批判もあり、日本の出版社は伝統的漫画の作家性と縦読みの量産性をどう両立させるかが競争軸になる可能性がある。</t>
+        </is>
+      </c>
+      <c r="I404" s="14" t="inlineStr">
+        <is>
+          <t>縦読み(Webtoon)と出版社の制作体制転換</t>
+        </is>
+      </c>
+      <c r="J404" s="14" t="inlineStr">
+        <is>
+          <t>LINEマンガ,ピッコマ,集英社,講談社</t>
+        </is>
+      </c>
+      <c r="K404" s="14" t="inlineStr"/>
+      <c r="L404" s="14" t="inlineStr">
+        <is>
+          <t>技術,トレンド,海外</t>
+        </is>
+      </c>
+      <c r="M404" s="14" t="inlineStr">
+        <is>
+          <t>市場調査ベースの構造トレンド</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B405" s="14" t="inlineStr">
+        <is>
+          <t>小説</t>
+        </is>
+      </c>
+      <c r="C405" s="14" t="inlineStr">
+        <is>
+          <t>米でロマンス小説専門書店が急増、ジャンル×コミュニティが縮小市場で成長</t>
+        </is>
+      </c>
+      <c r="D405" s="14" t="inlineStr">
+        <is>
+          <t>https://hon.jp/news/1.0/0/59375</t>
+        </is>
+      </c>
+      <c r="E405" s="14" t="inlineStr">
+        <is>
+          <t>全体の書籍販売が縮小する米国で、ロマンス小説だけが成長を続ける。販売部数はコロナ下の2020年1800万部から2023年3900万部へ倍増し、ベストセラーの半数超をロマンスが占める。専門書店も2020年の全米2店から2024年夏には20店超へ増加した。</t>
+        </is>
+      </c>
+      <c r="F405" s="14" t="inlineStr">
+        <is>
+          <t>Publishers Weekly報道として、米国のロマンス小説専門書店の急増が伝えられた。ロマンスは今や米書籍販売の約4分の1を占め、女性読者コミュニティを核に専門店が拡大。縮小する出版市場でも、特定ジャンル×リアルな場(書店)×ファンコミュニティを束ねれば成長余地があることを示す消費者インサイトとなる。</t>
+        </is>
+      </c>
+      <c r="G405" s="14" t="inlineStr">
+        <is>
+          <t>米書籍販売の約1/4がロマンス小説
+専門書店が2020年2店→2024年夏20店超に急増
+コミュニティ(女性読者)を核にした場づくりが成長源
+縮小市場でもジャンル特化×リアル書店で伸びる</t>
+        </is>
+      </c>
+      <c r="H405" s="14" t="inlineStr">
+        <is>
+          <t>ジャンル特化×コミュニティ型書店のモデルは、BookTok等SNSの推し文化と結びつき他ジャンル(ミステリ・SF・BL等)や他国にも波及する見込み。日本でもジャンル専門店・推し活拠点としての書店再定義が進み、汎用大型店の縮小と専門・体験型店舗の台頭という二極化が起きる可能性がある。</t>
+        </is>
+      </c>
+      <c r="I405" s="14" t="inlineStr">
+        <is>
+          <t>ジャンル特化書店とコミュニティ型小売</t>
+        </is>
+      </c>
+      <c r="J405" s="14" t="inlineStr"/>
+      <c r="K405" s="14" t="inlineStr"/>
+      <c r="L405" s="14" t="inlineStr">
+        <is>
+          <t>出版,消費者インサイト,海外,トレンド</t>
+        </is>
+      </c>
+      <c r="M405" s="14" t="inlineStr">
+        <is>
+          <t>PW報道(7/17)を日刊出版ニュースが紹介</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B406" s="14" t="inlineStr">
+        <is>
+          <t>小説</t>
+        </is>
+      </c>
+      <c r="C406" s="14" t="inlineStr">
+        <is>
+          <t>文芸市場の半分が『ウェブ発』書籍に——なろう系の主流化と文芸の構造転換</t>
+        </is>
+      </c>
+      <c r="D406" s="14" t="inlineStr">
+        <is>
+          <t>https://bunshun.jp/articles/-/55371</t>
+        </is>
+      </c>
+      <c r="E406" s="14" t="inlineStr">
+        <is>
+          <t>純文学・一般文芸の市場が縮小を続ける一方、『小説家になろう』等のウェブ小説発の書籍化が販売を下支えする構造が定着。文芸市場の相当部分をウェブ発タイトルが占めるまでになり、ラノベ/ライト文芸のレーベルがウェブ小説の書籍化パイプラインを競う状況になっている。</t>
+        </is>
+      </c>
+      <c r="F406" s="14" t="inlineStr">
+        <is>
+          <t>文春オンラインの分析で、文芸市場の約半分をウェブ発書籍が占める時代に入ったと指摘された。KADOKAWA BOOKS等はなろう系の書籍化を量産し、7月も多数刊行。伝統的な新人賞・編集主導の文芸から、ウェブでの読者反応を経て書籍化する『読者検証済み』モデルへ、文芸の調達構造が転換しつつある。</t>
+        </is>
+      </c>
+      <c r="G406" s="14" t="inlineStr">
+        <is>
+          <t>文芸市場の約半分をウェブ発書籍が占める
+なろう系書籍化が縮小する文芸を下支え
+新人賞主導→ウェブ読者反応で選別する調達モデルへ
+ラノベ/ライト文芸レーベルが書籍化パイプラインを競う</t>
+        </is>
+      </c>
+      <c r="H406" s="14" t="inlineStr">
+        <is>
+          <t>ウェブ発の『読者検証済み』調達が主流化すると、出版社の編集機能は新人発掘より『ウェブで数字を持つ作品の書籍化・IP化』へ比重を移す見込み。アニメ・コミカライズ前提でのウェブ小説争奪が激化し、プラットフォーム(なろう/カクヨム等)の作品供給源としての交渉力が高まる可能性がある。</t>
+        </is>
+      </c>
+      <c r="I406" s="14" t="inlineStr">
+        <is>
+          <t>ウェブ小説の書籍化パイプラインと文芸の調達構造</t>
+        </is>
+      </c>
+      <c r="J406" s="14" t="inlineStr">
+        <is>
+          <t>KADOKAWA</t>
+        </is>
+      </c>
+      <c r="K406" s="14" t="inlineStr"/>
+      <c r="L406" s="14" t="inlineStr">
+        <is>
+          <t>出版,トレンド,国内</t>
+        </is>
+      </c>
+      <c r="M406" s="14" t="inlineStr">
+        <is>
+          <t>文春オンライン分析</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B407" s="14" t="inlineStr">
+        <is>
+          <t>音楽</t>
+        </is>
+      </c>
+      <c r="C407" s="14" t="inlineStr">
+        <is>
+          <t>乃木坂46『是非に及ばず』初日60万枚、4作連続フラゲ日ハーフミリオンの特典型フィジカル</t>
+        </is>
+      </c>
+      <c r="D407" s="14" t="inlineStr">
+        <is>
+          <t>https://www.billboard-japan.com/d_news/detail/163748</t>
+        </is>
+      </c>
+      <c r="E407" s="14" t="inlineStr">
+        <is>
+          <t>ストリーミング全盛でも、日本のアイドルCDは握手券・特典を軸にフィジカル大量販売が続く。乃木坂46の42ndシングル『是非に及ばず』は初日(フラゲ日)売上60.2万枚を記録し、4作連続でフラゲ日ハーフミリオンを達成。先ヨミ集計では67.9万枚で首位を独走した。</t>
+        </is>
+      </c>
+      <c r="F407" s="14" t="inlineStr">
+        <is>
+          <t>乃木坂46『是非に及ばず』が初日60.2万枚(Billboard集計)、先ヨミ67.9万枚と大型セールス。ストリーミング指標が主流化する中でも、特典付きフィジカルによる初動集中型の販売モデルが健在であることを示す。配信で聴く曲とCDで『買い支える』曲が併存する日本市場の二重構造を象徴する事例だ。</t>
+        </is>
+      </c>
+      <c r="G407" s="14" t="inlineStr">
+        <is>
+          <t>初日60.2万枚、4作連続フラゲ日ハーフミリオン
+先ヨミ67.9万枚で首位独走
+特典型フィジカルの初動集中モデルが継続
+配信主流化と併存する日本のCD特典経済</t>
+        </is>
+      </c>
+      <c r="H407" s="14" t="inlineStr">
+        <is>
+          <t>特典型フィジカルは当面続くが、環境・在庫・転売批判やストリーミング指標偏重で、CD販売の『意味』は音源購入からファンダム参加権へ一段と純化する見込み。レーベルは物理特典をデジタル特典・体験へ置換する動きを強め、フィジカル依存の初動設計が徐々に見直される可能性がある。</t>
+        </is>
+      </c>
+      <c r="I407" s="14" t="inlineStr">
+        <is>
+          <t>特典型フィジカルとファンダム経済</t>
+        </is>
+      </c>
+      <c r="J407" s="14" t="inlineStr">
+        <is>
+          <t>ソニー・ミュージック,乃木坂46</t>
+        </is>
+      </c>
+      <c r="K407" s="14" t="inlineStr">
+        <is>
+          <t>乃木坂46</t>
+        </is>
+      </c>
+      <c r="L407" s="14" t="inlineStr">
+        <is>
+          <t>チャート・ランキング,国内,消費者インサイト</t>
+        </is>
+      </c>
+      <c r="M407" s="14" t="inlineStr">
+        <is>
+          <t>Billboard JAPAN先ヨミ</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B408" s="14" t="inlineStr">
+        <is>
+          <t>音楽</t>
+        </is>
+      </c>
+      <c r="C408" s="14" t="inlineStr">
+        <is>
+          <t>TIDAL、100%AI生成曲のロイヤリティ停止を7/15施行——AI楽曲のプール保護が具体化</t>
+        </is>
+      </c>
+      <c r="D408" s="14" t="inlineStr">
+        <is>
+          <t>https://www.techtimes.com/articles/320432/20260714/ai-music-labels-land-tomorrow-industry-rules-remain-voluntary-incomplete.htm</t>
+        </is>
+      </c>
+      <c r="E408" s="14" t="inlineStr">
+        <is>
+          <t>完全AI生成曲は作曲印税・作詞家が存在せず、ストリーミングのロイヤリティプールで構造的に有利になる。RIAA等が表示ラベルを提案する中、TIDALは100%AI生成曲へのロイヤリティ支払いを停止し『AI』バッジを付す方針を7/15に施行。Deezer・Qobuzも同種の除外・非収益化に動く。</t>
+        </is>
+      </c>
+      <c r="F408" s="14" t="inlineStr">
+        <is>
+          <t>TIDALは100%AI生成曲のロイヤリティ支払いを7/15停止し、AIバッジ表示・支払対象からの除外を実施。人間主導でAIを補助的に使う曲は対象外とする。無限に量産できるAI曲がロイヤリティプールを希釈する問題に対し、プラットフォームが実装レベルで防衛線を引いた。業界ラベル提案(RIAA等)と対をなす具体策だ。</t>
+        </is>
+      </c>
+      <c r="G408" s="14" t="inlineStr">
+        <is>
+          <t>100%AI生成曲のロイヤリティを停止しAIバッジ表示
+人間主導のAI補助曲は支払対象として存続
+Deezer(除外)・Qobuz(非収益化)も同方向
+ロイヤリティプール希釈への実装レベルの防衛</t>
+        </is>
+      </c>
+      <c r="H408" s="14" t="inlineStr">
+        <is>
+          <t>AI曲の収益化可否がプラットフォームごとに分かれる状況が続くと、権利団体主導の共通ラベル・開示メタデータ標準の整備が加速する見込み。開示を怠るAI曲の排除が進む一方、人間主導かの判定基準やAI学習ライセンスの扱いが次の争点になり、規制と収益配分ルールの再設計が進む可能性がある。</t>
+        </is>
+      </c>
+      <c r="I408" s="14" t="inlineStr">
+        <is>
+          <t>AI生成音楽のロイヤリティ配分と表示規制</t>
+        </is>
+      </c>
+      <c r="J408" s="14" t="inlineStr">
+        <is>
+          <t>TIDAL,Deezer,Qobuz,RIAA</t>
+        </is>
+      </c>
+      <c r="K408" s="14" t="inlineStr"/>
+      <c r="L408" s="14" t="inlineStr">
+        <is>
+          <t>AI,規制,配信,海外</t>
+        </is>
+      </c>
+      <c r="M408" s="14" t="inlineStr">
+        <is>
+          <t>7/15施行、RIAAラベル提案と関連</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B409" s="14" t="inlineStr">
+        <is>
+          <t>音楽</t>
+        </is>
+      </c>
+      <c r="C409" s="14" t="inlineStr">
+        <is>
+          <t>音楽カタログの取得倍率が沈静化、収益源にAI学習ライセンスが加わる構造変化</t>
+        </is>
+      </c>
+      <c r="D409" s="14" t="inlineStr">
+        <is>
+          <t>https://www.billboard.com/lists/music-business-stories-to-watch-last-half-2026/</t>
+        </is>
+      </c>
+      <c r="E409" s="14" t="inlineStr">
+        <is>
+          <t>2021-22年に20-30倍まで過熱した音楽カタログの取得倍率が、金利環境の変化で持続可能な水準へ低下。カタログ収益はストリーミング・シンク・実演・原盤隣接権に加え、近年はAI学習用のライセンス供与が新たな収益源として加わりつつある。</t>
+        </is>
+      </c>
+      <c r="F409" s="14" t="inlineStr">
+        <is>
+          <t>2026年下半期の注目テーマとして、音楽カタログ投資の環境変化が挙がる。取得倍率がピークの20-30倍から沈静化する一方、収益源にはAI学習ライセンスが加わり、カタログの評価軸が変わりつつある。単純な過去ヒットの権利買いから、AI時代のライセンス収益を織り込んだ評価・運用への転換が進む。</t>
+        </is>
+      </c>
+      <c r="G409" s="14" t="inlineStr">
+        <is>
+          <t>取得倍率が2021-22年の20-30倍から沈静化
+収益源にAI学習用ライセンスが新規追加
+ストリーミング/シンク/実演/隣接権に加えた多層収益
+カタログ評価軸がAI時代仕様へ変化</t>
+        </is>
+      </c>
+      <c r="H409" s="14" t="inlineStr">
+        <is>
+          <t>カタログ収益にAI学習ライセンスが定着すると、権利者は『聴かれる価値』に加え『学習素材としての価値』でカタログを評価するようになる見込み。AIへのデータ供与の可否・条件がカタログ価格を左右し、権利集約を進めるPE・大手レーベルとAI企業のライセンス交渉が新たな主戦場になる可能性がある。</t>
+        </is>
+      </c>
+      <c r="I409" s="14" t="inlineStr">
+        <is>
+          <t>音楽カタログ評価とAI学習ライセンス</t>
+        </is>
+      </c>
+      <c r="J409" s="14" t="inlineStr"/>
+      <c r="K409" s="14" t="inlineStr"/>
+      <c r="L409" s="14" t="inlineStr">
+        <is>
+          <t>出資,AI,権利・ライセンス,海外,トレンド</t>
+        </is>
+      </c>
+      <c r="M409" s="14" t="inlineStr">
+        <is>
+          <t>Billboard下半期注目テーマ</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B410" s="14" t="inlineStr">
+        <is>
+          <t>横断</t>
+        </is>
+      </c>
+      <c r="C410" s="14" t="inlineStr">
+        <is>
+          <t>2026年上半期の出版市場7664億円（▲1.3%）、電子が下支え・紙コミックスは▲7%</t>
+        </is>
+      </c>
+      <c r="D410" s="14" t="inlineStr">
+        <is>
+          <t>https://hon.jp/news/1.0/0/59414</t>
+        </is>
+      </c>
+      <c r="E410" s="14" t="inlineStr">
+        <is>
+          <t>出版科学研究所は7/24、2026年上半期の出版市場(紙+電子)を7664億円(前年同期比▲1.3%)と発表。電子は2867億円(+2.0%)と伸びる一方、紙は4797億円(▲3.1%)。うち雑誌▲3.8%、書籍▲2.7%、コミックスは約▲7%と、紙のコア商材の下落が続く。</t>
+        </is>
+      </c>
+      <c r="F410" s="14" t="inlineStr">
+        <is>
+          <t>2026年上半期の出版市場は7664億円で微減。電子(+2.0%)が全体を下支えする構図が定着した一方、紙コミックスが約▲7%と大きく落ち込み、雑誌・書籍も減少。漫画・小説を横断する出版全体で、収益の重心が紙から電子・IP・海外へ移る構造が、上半期の実数として改めて裏付けられた。</t>
+        </is>
+      </c>
+      <c r="G410" s="14" t="inlineStr">
+        <is>
+          <t>紙+電子で7664億円、前年同期比▲1.3%
+電子2867億円(+2.0%)が全体を下支え
+紙コミックスは約▲7%と下落が加速
+漫画・小説横断で紙依存モデルの限界が鮮明</t>
+        </is>
+      </c>
+      <c r="H410" s="14" t="inlineStr">
+        <is>
+          <t>電子が下支えしても市場全体の微減は続く見込みで、出版社は国内の紙販売より電子・海外(縦読み/翻訳版権)・映像化などIP収益への依存を強める。紙コミックスの下落が続けば、雑誌連載を起点とする従来の育成モデルが縮小し、ウェブ・アプリ発の作品調達へ一段とシフトする可能性がある。</t>
+        </is>
+      </c>
+      <c r="I410" s="14" t="inlineStr">
+        <is>
+          <t>出版市場の紙→電子・IPシフト</t>
+        </is>
+      </c>
+      <c r="J410" s="14" t="inlineStr"/>
+      <c r="K410" s="14" t="inlineStr"/>
+      <c r="L410" s="14" t="inlineStr">
+        <is>
+          <t>出版,国内,チャート・ランキング</t>
+        </is>
+      </c>
+      <c r="M410" s="14" t="inlineStr">
+        <is>
+          <t>出版科学研究所 季刊出版指標2026夏号</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -55059,7 +56659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -55295,6 +56895,120 @@
       <c r="K4" s="14" t="inlineStr">
         <is>
           <t>WEB漫画発キャラIPの初劇場版。全国380館・上映回数は大作級との報道。キャラ強/物語希薄IPの劇場マネタイズ事例</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>機動戦士ガンダムRG XARX-ZERO／GUNDAM ROGUE ORBIT</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="inlineStr">
+        <is>
+          <t>オリジナル</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="inlineStr">
+        <is>
+          <t>バンダイナムコフィルムワークス</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="inlineStr">
+        <is>
+          <t>アニメ・ゲーム</t>
+        </is>
+      </c>
+      <c r="F5" s="14" t="inlineStr">
+        <is>
+          <t>新IP『RGプロジェクト』としてアニメ・ゲーム・ガンプラを同時立ち上げ</t>
+        </is>
+      </c>
+      <c r="G5" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="H5" s="14" t="inlineStr">
+        <is>
+          <t>2027年</t>
+        </is>
+      </c>
+      <c r="I5" s="14" t="inlineStr">
+        <is>
+          <t>発表</t>
+        </is>
+      </c>
+      <c r="J5" s="14" t="inlineStr">
+        <is>
+          <t>バンダイナムコフィルムワークス,バンダイナムコエンターテインメント</t>
+        </is>
+      </c>
+      <c r="K5" s="14" t="inlineStr">
+        <is>
+          <t>単一原作でなく最初からアニメ・ゲーム・玩具を同時設計するIP立ち上げ型。監督:神山健治/SF監修:円城塔</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>都市伝説解体センター</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>ゲーム</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>集英社（となりのヤングジャンプ）</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>漫画</t>
+        </is>
+      </c>
+      <c r="F6" s="14" t="inlineStr">
+        <is>
+          <t>新作コミカライズ『Another Record』連載開始（正史から分岐したオリジナル）</t>
+        </is>
+      </c>
+      <c r="G6" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="I6" s="14" t="inlineStr">
+        <is>
+          <t>公開済</t>
+        </is>
+      </c>
+      <c r="J6" s="14" t="inlineStr">
+        <is>
+          <t>集英社</t>
+        </is>
+      </c>
+      <c r="K6" s="14" t="inlineStr">
+        <is>
+          <t>インディーゲーム発IP。ゲーム→小説→漫画と多メディア化。第1話にゲーム画面再現のブラウザ特別版</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
weekly-companies(6genres) + works watch update (2026-07-27 09:20)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -18055,13 +18055,13 @@
       </c>
       <c r="G10" s="9" t="inlineStr">
         <is>
-          <t>2026年4月公開の『名探偵コナン ハイウェイの堕天使』のエピローグで第30作の制作を告知。劇場版30周年記念作として2027年ゴールデンウィーク公開予定。予告にビッグ・ベンが映り、舞台はロンドン・主役は新一と蘭と見られる</t>
+          <t>『ハイウェイの堕天使』が7/6時点で興収135.2億円、4作連続100億円超で歴代上位。</t>
         </is>
       </c>
       <c r="H10" s="9" t="inlineStr"/>
       <c r="I10" s="9" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-27</t>
         </is>
       </c>
     </row>
@@ -18219,7 +18219,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>5作目『魂の決戦』が全国521館で公開。初日動員は前作『大将軍の帰還』（シリーズ最高80.3億円）対比124%。</t>
+          <t>新作『キングダム 魂の決戦』が2026年夏に劇場公開、実写シリーズ最新作として興行を牽引。</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -18229,7 +18229,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-27</t>
         </is>
       </c>
     </row>
@@ -18341,7 +18341,7 @@
       <c r="E2" s="9" t="inlineStr"/>
       <c r="F2" s="9" t="inlineStr">
         <is>
-          <t>FY2026 Q2: 売上251.7億ドル / 調整後EPS $1.57（市場予想上回る）。ストリーミング部門営業利益は前年同期比+88%、営業利益率11%を初達成</t>
+          <t>Q2(FY26)はEPS1.57ドル・売上251.7億ドルで予想上回り、DTCは営業益前年比+88%・営業利益率初の11%。次回(第3四半期)決算は8/5発表予定、理論株価は約113ドルとの試算。出典: 24/7 Wall St/Yahoo Finance 2026/7</t>
         </is>
       </c>
       <c r="G2" s="9" t="inlineStr">
@@ -18361,12 +18361,12 @@
       </c>
       <c r="J2" s="9" t="inlineStr">
         <is>
-          <t>ストリーミング営業利益率をどこまで引き上げられるか。スポーツ配信（ESPN単独）の立ち上がり</t>
+          <t>8/5決算でのDTC黒字定着と体験・パーク事業、映画スレート</t>
         </is>
       </c>
       <c r="K2" s="9" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-27</t>
         </is>
       </c>
     </row>
@@ -18553,7 +18553,7 @@
       <c r="E6" s="9" t="inlineStr"/>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>7/16にQ2 2026決算。売上+16%、FCFはほぼ倍増も、Q3見通し（+12%）とガイダンスが失望を呼び株価下落。通期売上見通しを510〜514億ドルに狭める。広告付きプランは提供国での新規登録の6割超を占め、広告MAUは全世界2.5億超</t>
+          <t>Q2(7/16)売上ガイダンス125.74億ドル・営業利益率32.6%。広告テ ィアが新規登録の約60%を占め、2026年広告収入30億ドル（前年比倍増）目標、広告主4,000社超。出典: 24/7 Wall St 2026/7</t>
         </is>
       </c>
       <c r="G6" s="9" t="inlineStr">
@@ -18578,7 +18578,7 @@
       </c>
       <c r="K6" s="9" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-27</t>
         </is>
       </c>
     </row>
@@ -18769,7 +18769,7 @@
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t>2026年2月期は映画・演劇・不動産の3本柱が堅調。2025暦年の国内グループ興収は1,605億円と過去最高圏。7/15に四半期決算を発表</t>
+          <t>劇場版『名探偵コナン ハイウェイの堕天使』が7/6時点で興収135.2億円、4作連続の100億円超。夏興行は『キングダム 魂の決戦』等が牽引。出典: アニメ!アニメ!/映画.com 2026/7</t>
         </is>
       </c>
       <c r="G10" s="9" t="inlineStr">
@@ -18794,7 +18794,7 @@
       </c>
       <c r="K10" s="9" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-27</t>
         </is>
       </c>
     </row>
@@ -56610,13 +56610,13 @@
       </c>
       <c r="G9" s="9" t="inlineStr">
         <is>
-          <t>「オリコン上半期ランキング2026」で2冠を達成。証券各社はBTSの完全体活動が2027年まで継続する前提でHYBEをセクターのトップピックに挙げている。一方でカムバック公演後のイベント効果は一巡し、K-POP関連株は年初来で大きく調整</t>
+          <t>完全体での活動を再開し新譜・ワールドツアーを準備。FIFAハーフタイム出演発表がHYBE株の材料に。</t>
         </is>
       </c>
       <c r="H9" s="9" t="inlineStr"/>
       <c r="I9" s="9" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-27</t>
         </is>
       </c>
     </row>
@@ -57062,7 +57062,7 @@
       <c r="E2" s="9" t="inlineStr"/>
       <c r="F2" s="9" t="inlineStr">
         <is>
-          <t>Q1 2026決算で、取締役会が自社株買い枠を10億ユーロへ倍増することを承認。あわせて保有するSpotify株式の半分を売却する方針を示した（Lucian Grainge CEO）</t>
+          <t>Q1売上約29億ユーロ(+8.1%)。保有するSpotify株の50%を約64億ドルでBill Ackman主導グループへ売却する方針。次回決算は7/30発表予定。出典: Music Ally/Inc 2026/7</t>
         </is>
       </c>
       <c r="G2" s="9" t="inlineStr">
@@ -57087,7 +57087,7 @@
       </c>
       <c r="K2" s="9" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-27</t>
         </is>
       </c>
     </row>
@@ -57115,7 +57115,7 @@
       <c r="E3" s="9" t="inlineStr"/>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>今週は目立った適時開示なし</t>
+          <t>Q1(5/7発表)売上17億ドル(+17%)、レコード音楽+17%・出版+14%。次回決算は8/6発表予定。出典: Billboard 2026/7</t>
         </is>
       </c>
       <c r="G3" s="9" t="inlineStr">
@@ -57140,7 +57140,7 @@
       </c>
       <c r="K3" s="9" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-27</t>
         </is>
       </c>
     </row>
@@ -57221,7 +57221,7 @@
       <c r="E5" s="9" t="inlineStr"/>
       <c r="F5" s="9" t="inlineStr">
         <is>
-          <t>Q1 2026はプレミアム会員2.93億人（+300万）、営業利益8.37億ドルと過去最高。ただしQ2ガイダンス（MAU 7.78億／プレミアム2.99億／売上48億ユーロ／営業利益6.3億ユーロ・利益率33.1%）が市場予想の約3.02億人を下回り、株価は一時13%超下落。株価は年初来約-16%。Q2決算は8/4予定</t>
+          <t>Q1売上45.3億ユーロ(+8%,為替中立+14%)。営業益見通しやAI・マーケ投資への失望で決算後株価は-13%。出典: Billboard/Forbes 2026/5</t>
         </is>
       </c>
       <c r="G5" s="9" t="inlineStr">
@@ -57246,7 +57246,7 @@
       </c>
       <c r="K5" s="9" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-27</t>
         </is>
       </c>
     </row>
@@ -57278,7 +57278,7 @@
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>年初来では株価-36.0%と大幅安だったが、7月中旬に反発。韓流関連輸出が前年比+84%の189.75億ドルに達したとの報道と、証券各社の「割安」評価が反発材料</t>
+          <t>BTS完全体の活動再開でQ2は四半期過去最高益が期待される一方、株価はYTD-39.88%と低迷。BTS光化門コンサート後の反動と資金のAI半導体シフトが重し。BTSのFIFAハーフタイム出演発表で一時反発。出典: BigGo/Seoul Economic Daily 2026/7</t>
         </is>
       </c>
       <c r="G6" s="9" t="inlineStr">
@@ -57288,12 +57288,12 @@
       </c>
       <c r="H6" s="9" t="inlineStr">
         <is>
-          <t>証券各社がセクターのトップピックに挙げる。BTSの完全体活動が来年まで継続する見込みで、新人グループの成長により単一メガIP依存が徐々に低下</t>
+          <t>BTS完全体復帰・ワールドツアー、多世代アーティスト擁する事業基盤</t>
         </is>
       </c>
       <c r="I6" s="9" t="inlineStr">
         <is>
-          <t>BTSカムバック公演後のイベントドリブンの momentum 剥落。資金がAI・半導体株へローテーション</t>
+          <t>イベント後の反動安、業種バリュエーション圧縮で目標株価引下げ相次ぐ</t>
         </is>
       </c>
       <c r="J6" s="9" t="inlineStr">
@@ -57303,7 +57303,7 @@
       </c>
       <c r="K6" s="9" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-27</t>
         </is>
       </c>
     </row>
@@ -57335,7 +57335,7 @@
       </c>
       <c r="F7" s="9" t="inlineStr">
         <is>
-          <t>韓国主要4社の中で最大の下落率。7月中旬に株価81,900ウォン（+6.09%）と反発</t>
+          <t>株価はYTD-50.30%と大手4社で最大の下落。業種全体のマルチプル圧縮が主因で、証券各社は目標株価を引下げつつも押し目買い機会と指摘。出典: BigGo/Seoul Economic Daily 2026/7</t>
         </is>
       </c>
       <c r="G7" s="9" t="inlineStr">
@@ -57360,7 +57360,7 @@
       </c>
       <c r="K7" s="9" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-27</t>
         </is>
       </c>
     </row>
@@ -57388,7 +57388,7 @@
       <c r="E8" s="9" t="inlineStr"/>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>年初来株価-35.7%。韓国4社合計で年初来8兆ウォン超（約54億ドル）の時価総額が消失した局面の一角</t>
+          <t>株価はYTD-38.91%。Stray Kids等の稼働で業績自体は堅調だが、業種バリュエーション低下で目標株価は引下げ。出典: BigGo 2026/7</t>
         </is>
       </c>
       <c r="G8" s="9" t="inlineStr">
@@ -57413,7 +57413,7 @@
       </c>
       <c r="K8" s="9" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-27</t>
         </is>
       </c>
     </row>
@@ -59616,12 +59616,12 @@
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>予約が本格化。仏Cdiscountでの予約は通常大型作の約6倍。Take-Two株は52週高値圏($260台)で発売期待が先行。</t>
+          <t>Take-TwoがGTA VIを11/19発売と正式確定（標準79.99ドル/アルティメット99.99ドル）。FY27の最大増益ドライバー。</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>『GTAⅥ』2026/11/19発売(PS5/Xbox Series X|S)。標準版$79.99/アルティメット版$99.99を確定。</t>
+          <t>『GTA VI』2026/11/19 PS5/Xbox Series X|S</t>
         </is>
       </c>
       <c r="F29" s="9" t="inlineStr"/>
@@ -59633,7 +59633,7 @@
       <c r="H29" s="9" t="inlineStr"/>
       <c r="I29" s="9" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-27</t>
         </is>
       </c>
     </row>
@@ -60387,7 +60387,7 @@
       </c>
       <c r="D54" s="9" t="inlineStr">
         <is>
-          <t>Q1 2026は売上が予想未達、安全対策強化で通期ガイダンスを下方修正。株価は6か月で約-51%。</t>
+          <t>AI活用のクリエイション機能を発表（7/17）。第2四半期決算は7/30引け後。BofAが目標株価を54ドルへ引上げ。</t>
         </is>
       </c>
       <c r="E54" s="9" t="inlineStr">
@@ -60404,7 +60404,7 @@
       <c r="H54" s="9" t="inlineStr"/>
       <c r="I54" s="9" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-27</t>
         </is>
       </c>
     </row>
@@ -60693,7 +60693,9 @@
       </c>
       <c r="M2" s="9" t="inlineStr">
         <is>
-          <t>【7/17】終値7,294円(前日比+214円,+3.02%)と逆行高。7/17の東京市場は日経平均が前日比2,694.42円安の64,141.12円と大幅続落し、3連休前にAI・半導体関連の利益確定売りが先行。一方で半導体・メモリー市況の落ち着き期待から「非AI」の内需・バリューへ循環物色が向かい、家庭用ゲーム大手が逆行高。gamebiz集計ではゲーム・エンタメ96銘柄中、上昇26(27%)・下落64(67%)と全体は軟調な中での選別買い。出典: gamebiz 2026/7/17
+          <t>【7/27週】Switch2は6月の米市場でハード数量・金額とも首位を維持、国内も累計602万台超。世界累計は3/31時点で1,986万台とPS5同期を上回る立ち上がり。東証終値は7月下旬に6,969〜7,033円圏。第1四半期決算は8/6発表予定で、次期減収減益予想に対する進捗が焦点。出典: PUNCH JUMP/Yahoo Finance 2026/7
+---（前回までの記載）---
+【7/17】終値7,294円(前日比+214円,+3.02%)と逆行高。7/17の東京市場は日経平均が前日比2,694.42円安の64,141.12円と大幅続落し、3連休前にAI・半導体関連の利益確定売りが先行。一方で半導体・メモリー市況の落ち着き期待から「非AI」の内需・バリューへ循環物色が向かい、家庭用ゲーム大手が逆行高。gamebiz集計ではゲーム・エンタメ96銘柄中、上昇26(27%)・下落64(67%)と全体は軟調な中での選別買い。出典: gamebiz 2026/7/17
 ---（前回までの記載）---
 株価は6/26の6,589円を安値に7/2に7,137円へ反発、その後7,120円前後で横ばい推移し材料出尽くし後の水準確認局面。Switch 2値上げ(国内5.998万円)による普及ペース鈍化懸念は根強いが、FY26は売上2.31兆円(+98.6%)営業益3,601億円(+27.5%)と急回復済。次期は減収減益予想で新作ソフト継続投入が焦点。
 なお、サウジPIF傘下Savvy Games Groupが当社を含む任天堂/バンダイナムコ/Nexon/コーエーテクモ/スクウェア・エニックスの約10%少数持分を約120億ドル規模でSavvyへ移管・集約済み（出典: Reuters/TechTimes 2026/7/17引用のPocketGamer.biz報）。</t>
@@ -60716,7 +60718,7 @@
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-27</t>
         </is>
       </c>
     </row>
@@ -60751,27 +60753,29 @@
       </c>
       <c r="M3" s="9" t="inlineStr">
         <is>
-          <t>『GTAⅥ』が11/19にPS5/Xbox向けで発売(標準$79.99/アルティメット$99.99)と価格が確定し、PS5エンゲージメント/ネットワーク収入拡大への期待が改めて意識される。FY25は全社売上・営業益とも過去最高を更新済で、大型新規開示は乏しく好業績持続力を見極める局面。</t>
+          <t>【7/27週】PlayStationを2028年1月から新作フルデジタル配信に一本化し、物理ディスク新作を段階終了、PS3/PS Vitaオンラインストアも順次閉鎖と発表。高マージンのデジタル/継続課金シフトを好感し株価は週間+6.77%、約1,275億円の自社株買いも完了。一方でファンは反発（署名10万筆・€4億訴訟報道）、総会長・十時CEOら経営陣が7/3に保有株を大量売却（十時氏は保有の約56.5%）した点は懸念。出典: Simply Wall St/Yahoo Finance 2026/7
+---（前回までの記載）---
+『GTAⅥ』が11/19にPS5/Xbox向けで発売(標準$79.99/アルティメット$99.99)と価格が確定し、PS5エンゲージメント/ネットワーク収入拡大への期待が改めて意識される。FY25は全社売上・営業益とも過去最高を更新済で、大型新規開示は乏しく好業績持続力を見極める局面。</t>
         </is>
       </c>
       <c r="N3" s="9" t="inlineStr">
         <is>
-          <t>GTAⅥ効果でのPS5エンゲージメント/ネットワーク収入期待、全社最高業績</t>
+          <t>デジタル一本化で高マージン化、全社最高業績、GTAⅥ商戦でのPS5牽引期待、自社株買い</t>
         </is>
       </c>
       <c r="O3" s="9" t="inlineStr">
         <is>
-          <t>ハード成熟でハード収益鈍化、大型新規IPの不在感</t>
+          <t>物理販売終了へのファン反発（訴訟・署名）、経営陣の大量株式売却、ハード成熟</t>
         </is>
       </c>
       <c r="P3" s="9" t="inlineStr">
         <is>
-          <t>GTAⅥ商戦でのPS5牽引、ゲーム&amp;ネットワークサービスの収益拡大</t>
+          <t>デジタル移行の収益寄与とユーザー離反リスクの見極め、GTAⅥ商戦、ネットワークサービス拡大</t>
         </is>
       </c>
       <c r="Q3" s="9" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-27</t>
         </is>
       </c>
     </row>
@@ -61602,7 +61606,9 @@
       </c>
       <c r="L3" s="9" t="inlineStr">
         <is>
-          <t>株価は$260.63と52週高値$264.79に接近(7/7)。BenchmarkはBuy/目標$300、BofAは$368へ引上げ。『GTAⅥ』は11/19発売・標準$79.99/アルティメット$99.99が確定し、仏Cdiscountの予約は通常大型作の6倍。FY27ネットブッキングは$8〜8.2bn(FY26約$6.7bn)を見込む。</t>
+          <t>【7/27週】『GTA VI』を11/19発売と正式確定し、FY27ネットブッキングをガイダンス80.0〜82.0億ドル（前期6.72億ドルから約20%増）と提示。GTA VIが最大の増益ドライバー。Jefferiesは7/14にBuy継続。出典: TIKR/Yahoo Finance 2026/7
+---（前回までの記載）---
+株価は$260.63と52週高値$264.79に接近(7/7)。BenchmarkはBuy/目標$300、BofAは$368へ引上げ。『GTAⅥ』は11/19発売・標準$79.99/アルティメット$99.99が確定し、仏Cdiscountの予約は通常大型作の6倍。FY27ネットブッキングは$8〜8.2bn(FY26約$6.7bn)を見込む。</t>
         </is>
       </c>
       <c r="M3" s="9" t="inlineStr">
@@ -61617,12 +61623,12 @@
       </c>
       <c r="O3" s="9" t="inlineStr">
         <is>
-          <t>GTAⅥ(11/19)の発売実現と初動規模、FY27ネットブッキング$8bn超への牽引、遅延リスクの解消</t>
+          <t>GTA VI(11/19)の立ち上がり、NBA2K/オンライン課金の底堅さ</t>
         </is>
       </c>
       <c r="P3" s="9" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-27</t>
         </is>
       </c>
     </row>
@@ -61660,27 +61666,29 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>【7/17 Reuters独占】欧州委員会は競争法(merger)審査を7/22に無条件クリア、外国補助金規則(FSR)も予備審査終了の7/30までに承認見込みで、EUゲートは事実上通過へ。残る実質的な関門は米CFIUS(対米外国投資委員会)で、契約上のアウトサイドデートは9/28。当初のクロージング期限6/30は未達のまま延長済み。株主承認は2025年12月に可決、米HSR反トラストも取得済み。PIFが93.7%を握る支配株主となる構造。EA株は7月初旬時点で買収価格$210を$7〜9下回る水準で推移し、スプレッドはCFIUS不確実性を映す。FY26は純ブッキング$8.026bn(+9%)・純収益$7.531bnと過去最高だが、純利益は$1.121bn→$887m(-21%)と減益。出典: TechTimes/Reuters 2026/7/17</t>
+          <t>【7/27週】サウジPIF・Silver Lake・Affinity Partnersによる総額550億ドル（1株210ドル）の非公開化について、欧州委員会が7/23にEU競争法上の承認。米HSRは取得済だが、政府系ファンド関与のためCFIUSが安全保障・プレイヤーデータを審査中。買収期限は9/28まで延長、完了はFY27第1四半期見込み。出典: OpenCritic/Euronext/GameDeveloper 2026/7
+---（前回までの記載）---
+【7/17 Reuters独占】欧州委員会は競争法(merger)審査を7/22に無条件クリア、外国補助金規則(FSR)も予備審査終了の7/30までに承認見込みで、EUゲートは事実上通過へ。残る実質的な関門は米CFIUS(対米外国投資委員会)で、契約上のアウトサイドデートは9/28。当初のクロージング期限6/30は未達のまま延長済み。株主承認は2025年12月に可決、米HSR反トラストも取得済み。PIFが93.7%を握る支配株主となる構造。EA株は7月初旬時点で買収価格$210を$7〜9下回る水準で推移し、スプレッドはCFIUS不確実性を映す。FY26は純ブッキング$8.026bn(+9%)・純収益$7.531bnと過去最高だが、純利益は$1.121bn→$887m(-21%)と減益。出典: TechTimes/Reuters 2026/7/17</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>EU反トラスト/FSRの承認見込みで規制リスクが一段後退、Battlefield 6牽引でFY26純ブッキング過去最高$8.026bn、EA SPORTS FC等の安定収益、PIFの長期patient capital論</t>
+          <t>550億ドル非公開化でEU承認取得、株価は買収価格210ドルにサヤ寄せ</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>CFIUS審査が未完了(アウトサイドデート9/28)でクロージング時期が未定、$200億の負債・レバレッジ約6倍(CreditSights)による将来のコスト削減圧力、クローズ前に2026年だけで3度のレイオフ(Skate/BF6開発、全社約300名、6月はTrust&amp;Safety等)、純利益-21%の減益</t>
+          <t>CFIUS審査の不透明感、案件クロージング遅延リスク、6月米ゲーム支出-21%(Circana)</t>
         </is>
       </c>
       <c r="O4" s="9" t="inlineStr">
         <is>
-          <t>CFIUSの結論(緩和条件付き承認か)と9/28アウトサイドデートの扱い、EU承認(7/22反トラスト・7/30 FSR)の確定、クローズ後の債務返済負担とスタジオ・人員体制、Battlefieldライブサービスの定着</t>
+          <t>CFIUS承認の可否とクロージング時期、EA Sports FC/バトルフィールド新作の商戦</t>
         </is>
       </c>
       <c r="P4" s="9" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-27</t>
         </is>
       </c>
     </row>
@@ -62038,12 +62046,14 @@
       </c>
       <c r="L11" s="9" t="inlineStr">
         <is>
-          <t>Q2 2026決算を7/30に発表予定(EPS予想-$0.34、売上予想$1.59B/+10.7%)。未成年の年齢確認規制強化を背景に通期ブッキング成長見通しを8-12%へ下方修正済。株価は約$54.6でテクニカルは弱含み、決算前で様子見。アナリスト平均レーティングはBuy。</t>
+          <t>【7/27週】BofAが7/21に目標株価を48→54ドルへ引上げ。7/17にAI活用のクリエイション機能を発表し、決算期待とともに株価上昇。第2四半期決算は7/30引け後に発表予定。出典: StockTitan/QuiverQuant 2026/7
+---（前回までの記載）---
+Q2 2026決算を7/30に発表予定(EPS予想-$0.34、売上予想$1.59B/+10.7%)。未成年の年齢確認規制強化を背景に通期ブッキング成長見通しを8-12%へ下方修正済。株価は約$54.6でテクニカルは弱含み、決算前で様子見。アナリスト平均レーティングはBuy。</t>
         </is>
       </c>
       <c r="M11" s="9" t="inlineStr">
         <is>
-          <t>高成長のプラットフォーム売上とクリエイター経済</t>
+          <t>AI創作ツールでUGC拡充、アナリスト目標株価引上げ</t>
         </is>
       </c>
       <c r="N11" s="9" t="inlineStr">
@@ -62053,12 +62063,12 @@
       </c>
       <c r="O11" s="9" t="inlineStr">
         <is>
-          <t>安全対策と成長の両立、ブッキング再加速と広告収益の伸長</t>
+          <t>7/30決算での予約売上・課金動向、広告事業の伸長</t>
         </is>
       </c>
       <c r="P11" s="9" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
daily-news(6genres) + cross-questions + media-mix + events + predictions + game-design update (2026-07-27)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -891,7 +891,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H43"/>
+  <dimension ref="A1:H44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2705,6 +2705,48 @@
         </is>
       </c>
       <c r="H43" s="14" t="inlineStr">
+        <is>
+          <t>横断</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B44" s="14" t="inlineStr">
+        <is>
+          <t>音楽・動画・ゲームのサブスク横断値上げで家計のエンタメ可処分が逼迫→併存から排他的選択へ→通信キャリアがエンタメを束ねるバンドルプランを再強化し、単体サブスクの解約防衛と顧客の『束ね直し』競争が起きる</t>
+        </is>
+      </c>
+      <c r="C44" s="14" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="D44" s="14" t="inlineStr">
+        <is>
+          <t>6〜12ヶ月</t>
+        </is>
+      </c>
+      <c r="E44" s="14" t="inlineStr">
+        <is>
+          <t>Apple, Microsoft(Game Pass), 通信キャリア</t>
+        </is>
+      </c>
+      <c r="F44" s="14" t="inlineStr">
+        <is>
+          <t>Apple One値上げ¥1,980→¥2,500(libecity 2026/7)</t>
+        </is>
+      </c>
+      <c r="G44" s="14" t="inlineStr">
+        <is>
+          <t>各サブスクのARPU・解約率、キャリアのエンタメ込み新プラン発表、Apple One/Game Passのバンドル改定を観測すれば当否が分かる。</t>
+        </is>
+      </c>
+      <c r="H44" s="14" t="inlineStr">
         <is>
           <t>横断</t>
         </is>
@@ -5661,7 +5703,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H93"/>
+  <dimension ref="A1:H95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9575,6 +9617,90 @@
         </is>
       </c>
       <c r="H93" s="14" t="inlineStr">
+        <is>
+          <t>横断</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B94" s="14" t="inlineStr">
+        <is>
+          <t>Netflixが雑誌ブランド(Variety/Billboard/THR)のショート動画を取り込む『メディア吸収』は、音楽(MV/アーティスト映像)やゲーム(実況/公式番組)でも、プラットフォームによるメディアブランドの内製吸収として起きるか？</t>
+        </is>
+      </c>
+      <c r="C94" s="14" t="inlineStr">
+        <is>
+          <t>Netflix、出版社とショート動画提携(TechCrunch 2026/7)</t>
+        </is>
+      </c>
+      <c r="D94" s="14" t="inlineStr">
+        <is>
+          <t>Netflix, Variety, Billboard</t>
+        </is>
+      </c>
+      <c r="E94" s="14" t="inlineStr">
+        <is>
+          <t>広告・メディア, 通信</t>
+        </is>
+      </c>
+      <c r="F94" s="14" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="G94" s="14" t="inlineStr">
+        <is>
+          <t>PFがコンテンツ(C)だけでなくメディアブランド(M)自体を吸収し始めた。次はMV/実況/情報番組が標的か。</t>
+        </is>
+      </c>
+      <c r="H94" s="14" t="inlineStr">
+        <is>
+          <t>横断</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B95" s="14" t="inlineStr">
+        <is>
+          <t>サブスク値上げ連鎖(Apple One +26%)で強まる『排他的選択』は、ゲーム(Game Pass/PS Plus)や電子書籍読み放題にも同時波及し、家計のエンタメ可処分を奪い合うか？通信バンドル回帰を招くか？</t>
+        </is>
+      </c>
+      <c r="C95" s="14" t="inlineStr">
+        <is>
+          <t>Apple One値上げ¥1,980→¥2,500(2026/7)</t>
+        </is>
+      </c>
+      <c r="D95" s="14" t="inlineStr">
+        <is>
+          <t>Apple, Microsoft, ソニー, 通信キャリア</t>
+        </is>
+      </c>
+      <c r="E95" s="14" t="inlineStr">
+        <is>
+          <t>通信, 小売(家計)</t>
+        </is>
+      </c>
+      <c r="F95" s="14" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="G95" s="14" t="inlineStr">
+        <is>
+          <t>ジャンル横断でサブスクが『共存』から『椅子取り』へ。可処分時間より可処分所得の制約が効き始める。</t>
+        </is>
+      </c>
+      <c r="H95" s="14" t="inlineStr">
         <is>
           <t>横断</t>
         </is>
@@ -15476,12 +15602,12 @@
       </c>
       <c r="I32" s="14" t="inlineStr">
         <is>
-          <t>開催中</t>
+          <t>終了</t>
         </is>
       </c>
       <c r="J32" s="14" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
     </row>
@@ -15528,12 +15654,12 @@
       </c>
       <c r="I33" s="14" t="inlineStr">
         <is>
-          <t>開催中</t>
+          <t>終了</t>
         </is>
       </c>
       <c r="J33" s="14" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
     </row>
@@ -15716,9 +15842,9 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="15" t="inlineStr">
-        <is>
-          <t>2026-07-20</t>
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B4" s="15" t="inlineStr">
@@ -15751,14 +15877,14 @@
           <t>長期運営タイトルの新規獲得鈍化、既存・離脱層の呼び戻し需要、コミュニティの懐古熱。</t>
         </is>
       </c>
-      <c r="H4" s="15" t="inlineStr">
-        <is>
-          <t>AAA新作の開発長期化で空いた発売枠を、検証済みデザインの再構築が埋める構造が定着。大手の年間ラインナップに常設枠として組み込まれる一方、供給過多による単価・話題性の逓減リスクも。次の焦点は『どこまで作り直すか』の粒度設計で、フルリメイクと軽量リマスターの二極化が進む。</t>
-        </is>
-      </c>
-      <c r="I4" s="15" t="inlineStr">
-        <is>
-          <t>『AC ブラックフラッグ Resynced』が予約シリーズ上位＋高評価／Halo: Campaign Evolved／Fallout 3・NVリマスター発表（2026-07-20）</t>
+      <c r="H4" s="14" t="inlineStr">
+        <is>
+          <t>旧作リマスターが新作級の利益貢献を示し(アクワイア最終益1658%増)、新作AAA疲れの受け皿として常設ライン化が進む。中古・二次流通とセットで低リスク収益の柱に。</t>
+        </is>
+      </c>
+      <c r="I4" s="14" t="inlineStr">
+        <is>
+          <t>アクワイア決算で旧作リマスターが最終益1658%増を牽引(gamebiz 2026/7)</t>
         </is>
       </c>
       <c r="J4" s="15" t="n">
@@ -19078,7 +19204,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M431"/>
+  <dimension ref="A1:M445"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -47894,6 +48020,986 @@
         </is>
       </c>
       <c r="M431" s="14" t="inlineStr"/>
+    </row>
+    <row r="432">
+      <c r="A432" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B432" s="14" t="inlineStr">
+        <is>
+          <t>ゲーム</t>
+        </is>
+      </c>
+      <c r="C432" s="14" t="inlineStr">
+        <is>
+          <t>Xbox、5スタジオ閉鎖・約3,200人削減——687億ドル買収後の大再編</t>
+        </is>
+      </c>
+      <c r="D432" s="14" t="inlineStr">
+        <is>
+          <t>https://www.techtimes.com/articles/319765/20260706/xbox-fires-thousands-shuts-five-studios-largest-gaming-layoff-years.htm</t>
+        </is>
+      </c>
+      <c r="E432" s="14" t="inlineStr">
+        <is>
+          <t>MicrosoftはActivision Blizzardを687億ドルで買収したが、その後は人員削減・スタジオ閉鎖・サブスク値上げが続いた。2026年7月、Xbox部門で即時1,600人＋FY27までに1,600人の計約3,200人(部門の約20%)削減、5スタジオ閉鎖が判明した。</t>
+        </is>
+      </c>
+      <c r="F432" s="14" t="inlineStr">
+        <is>
+          <t>Xboxは近年最大規模のレイオフを実施し、5スタジオを閉鎖、部門の約20%にあたる約3,200人を削減する。巨額のABK買収後もコスト削減と事業再編が続き、コンソール戦争の前提だった囲い込みモデル自体が崩れつつある。</t>
+        </is>
+      </c>
+      <c r="G432" s="14" t="inlineStr">
+        <is>
+          <t>687億ドル買収後もコスト削減が止まらない
+部門の約2割という異例の削減規模
+スタジオ閉鎖でIP・人材の行き先が焦点
+ハード販売よりGame Pass/マルチPF展開へ軸足</t>
+        </is>
+      </c>
+      <c r="H432" s="14" t="inlineStr">
+        <is>
+          <t>MicrosoftはハードSKUよりGame Passとマルチプラットフォーム配信に一段と傾斜し、自社IPを他社機にも出す脱ハードが加速する。閉鎖スタジオのIPをどう活用/売却するかが次の焦点で、熟練人材の流出は中規模スタジオ新設や競合の採用強化につながる。</t>
+        </is>
+      </c>
+      <c r="I432" s="14" t="inlineStr">
+        <is>
+          <t>大型M&amp;A後の統合コストとプラットフォーム戦略転換</t>
+        </is>
+      </c>
+      <c r="J432" s="14" t="inlineStr">
+        <is>
+          <t>Microsoft, Activision Blizzard</t>
+        </is>
+      </c>
+      <c r="K432" s="14" t="inlineStr">
+        <is>
+          <t>Xbox, Game Pass</t>
+        </is>
+      </c>
+      <c r="L432" s="14" t="inlineStr">
+        <is>
+          <t>M&amp;A,人事・組織,海外,ハード</t>
+        </is>
+      </c>
+      <c r="M432" s="14" t="inlineStr">
+        <is>
+          <t>2026/7/6報道</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B433" s="14" t="inlineStr">
+        <is>
+          <t>映画</t>
+        </is>
+      </c>
+      <c r="C433" s="14" t="inlineStr">
+        <is>
+          <t>『オデュッセイア』世界興収$640M突破——ノーラン自己最高、劇場回帰を実証</t>
+        </is>
+      </c>
+      <c r="D433" s="14" t="inlineStr">
+        <is>
+          <t>https://deadline.com/2026/07/box-office-global-the-odyssey-toy-story-5-1237004022/</t>
+        </is>
+      </c>
+      <c r="E433" s="14" t="inlineStr">
+        <is>
+          <t>クリストファー・ノーラン監督『オデュッセイア』は初週の世界興収$263.7Mでノーラン作品の自己最高スタートを記録。2週目も$215.3Mを上乗せし累計$640M超に。ピクサー『トイ・ストーリー5』も世界$10億に迫り、2026年3本目の10億ドル作となる見込み。</t>
+        </is>
+      </c>
+      <c r="F433" s="14" t="inlineStr">
+        <is>
+          <t>『オデュッセイア』が公開2週で世界興収$640Mを突破し、ノーラン監督作の最高ペース。IMAX/70mmを軸にした劇場体験訴求が奏功した。『トイ・ストーリー5』は世界$10億に到達し2026年3本目の大台超え。大作の劇場回帰と家族向けアニメの強さが同時に示された。</t>
+        </is>
+      </c>
+      <c r="G433" s="14" t="inlineStr">
+        <is>
+          <t>ノーラン作品として自己最高の立ち上がり
+IMAX/70mmなど劇場でしかの体験訴求が有効
+トイ・ストーリー5が2026年3本目の$10億作
+大作×家族向けの二極が劇場を牽引</t>
+        </is>
+      </c>
+      <c r="H433" s="14" t="inlineStr">
+        <is>
+          <t>劇場市場は大作・体験型に興行が集中し、中堅作は配信直行との二極化が進む。ノーランのIMAX戦略の成功で各スタジオが大型フォーマット上映枠を奪い合い、家族向けアニメIPの続編は引き続き$10億級の安全資産として量産される。年内の10億ドル作が何本に伸びるかが劇場回復の指標。</t>
+        </is>
+      </c>
+      <c r="I433" s="14" t="inlineStr">
+        <is>
+          <t>プレミアム大画面フォーマットと劇場興行の二極化</t>
+        </is>
+      </c>
+      <c r="J433" s="14" t="inlineStr">
+        <is>
+          <t>ユニバーサル, ウォルト・ディズニー, ピクサー, IMAX</t>
+        </is>
+      </c>
+      <c r="K433" s="14" t="inlineStr">
+        <is>
+          <t>オデュッセイア, トイ・ストーリー5</t>
+        </is>
+      </c>
+      <c r="L433" s="14" t="inlineStr">
+        <is>
+          <t>興行,海外,トレンド</t>
+        </is>
+      </c>
+      <c r="M433" s="14" t="inlineStr">
+        <is>
+          <t>Deadline世界興行(2026/7/24-26)</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B434" s="14" t="inlineStr">
+        <is>
+          <t>映画</t>
+        </is>
+      </c>
+      <c r="C434" s="14" t="inlineStr">
+        <is>
+          <t>『ハウスメイド』7/27公開——ベストセラー小説をS・スウィーニー主演で実写化</t>
+        </is>
+      </c>
+      <c r="D434" s="14" t="inlineStr">
+        <is>
+          <t>https://www.fashion-press.net/news/138270</t>
+        </is>
+      </c>
+      <c r="E434" s="14" t="inlineStr">
+        <is>
+          <t>世界的ベストセラー小説を原作に、シドニー・スウィーニー主演で実写化したサスペンス『ハウスメイド』が2026年7月27日に日本公開。家政婦が豪邸の秘密に迫る物語で、話題小説の映像化が引き続きハリウッドの主要な企画源であることを示す。</t>
+        </is>
+      </c>
+      <c r="F434" s="14" t="inlineStr">
+        <is>
+          <t>人気小説を原作とする実写サスペンス『ハウスメイド』が7/27に日本公開。主演はシドニー・スウィーニー。ベストセラー小説→映画という王道のメディアミックスで、原作の既存ファンを初動集客に取り込む設計。出版とハリウッドの企画パイプラインの強さを裏づける。</t>
+        </is>
+      </c>
+      <c r="G434" s="14" t="inlineStr">
+        <is>
+          <t>ベストセラー小説の映像化という王道企画
+主演俳優のスター性で初動を担保
+出版→映画の企画パイプラインが健在
+配信時代でも劇場サスペンスに需要</t>
+        </is>
+      </c>
+      <c r="H434" s="14" t="inlineStr">
+        <is>
+          <t>話題小説の映像化は既存読者=初動観客を見込める低リスク企画として続き、出版社・エージェントの映像化権ビジネスがさらに活況になる。日本でも海外ベストセラーの実写化輸入と、国内小説の映像化権争奪が強まる見込み。</t>
+        </is>
+      </c>
+      <c r="I434" s="14" t="inlineStr">
+        <is>
+          <t>ベストセラー小説の映像化権とスター主演の初動効果</t>
+        </is>
+      </c>
+      <c r="J434" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K434" s="14" t="inlineStr">
+        <is>
+          <t>ハウスメイド</t>
+        </is>
+      </c>
+      <c r="L434" s="14" t="inlineStr">
+        <is>
+          <t>映像化,興行,海外</t>
+        </is>
+      </c>
+      <c r="M434" s="14" t="inlineStr">
+        <is>
+          <t>原作:小説</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B435" s="14" t="inlineStr">
+        <is>
+          <t>映画</t>
+        </is>
+      </c>
+      <c r="C435" s="14" t="inlineStr">
+        <is>
+          <t>実写版『モアナと伝説の海』7/31公開——日本版声優にME:IのTSUZUMI</t>
+        </is>
+      </c>
+      <c r="D435" s="14" t="inlineStr">
+        <is>
+          <t>https://www.fashion-press.net/news/132751</t>
+        </is>
+      </c>
+      <c r="E435" s="14" t="inlineStr">
+        <is>
+          <t>ディズニーは2016年のアニメ『モアナと伝説の海』を実写映画化し、2026年7月31日に日本公開。日本版モアナ役の声優にガールズグループME:IのTSUZUMIを起用するなど、実写リメイクとアイドル/タレント起用の集客モデルを踏襲する。</t>
+        </is>
+      </c>
+      <c r="F435" s="14" t="inlineStr">
+        <is>
+          <t>ディズニーのアニメ実写化『モアナと伝説の海』が7/31日本公開。日本版声優にME:IのTSUZUMIを起用。ディズニーのアニメ→実写リメイク路線と、話題性のあるアイドル/タレントの吹替起用という日本の宣伝定石が組み合わさる。</t>
+        </is>
+      </c>
+      <c r="G435" s="14" t="inlineStr">
+        <is>
+          <t>ディズニーのアニメ実写リメイク路線の最新作
+日本版はアイドル起用で話題づくり
+既存アニメの認知を初動に転換
+家族層＋ファン層の二重動員を狙う</t>
+        </is>
+      </c>
+      <c r="H435" s="14" t="inlineStr">
+        <is>
+          <t>ディズニーの実写リメイクは賛否がありつつも既存IP認知を活かせるため継続され、日本ではアイドル/タレントの吹替起用が定番の宣伝手法として定着する。実写リメイクの興行結果次第で、ディズニーがオリジナル新規IPと過去作リメイクのどちらに資源配分するかが問われる。</t>
+        </is>
+      </c>
+      <c r="I435" s="14" t="inlineStr">
+        <is>
+          <t>ディズニー実写リメイク戦略と日本の吹替タレント起用</t>
+        </is>
+      </c>
+      <c r="J435" s="14" t="inlineStr">
+        <is>
+          <t>ウォルト・ディズニー</t>
+        </is>
+      </c>
+      <c r="K435" s="14" t="inlineStr">
+        <is>
+          <t>モアナと伝説の海, ME:I</t>
+        </is>
+      </c>
+      <c r="L435" s="14" t="inlineStr">
+        <is>
+          <t>映像化,興行,国内,海外</t>
+        </is>
+      </c>
+      <c r="M435" s="14" t="inlineStr">
+        <is>
+          <t>原作:アニメ</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B436" s="14" t="inlineStr">
+        <is>
+          <t>アニメ</t>
+        </is>
+      </c>
+      <c r="C436" s="14" t="inlineStr">
+        <is>
+          <t>2026夏アニメは続編・レガシー依存が鮮明——BLEACH/無職転生III/逃げ上手2期</t>
+        </is>
+      </c>
+      <c r="D436" s="14" t="inlineStr">
+        <is>
+          <t>https://news.denfaminicogamer.jp/kikakuthetower/260701x</t>
+        </is>
+      </c>
+      <c r="E436" s="14" t="inlineStr">
+        <is>
+          <t>2026年7月クールは『BLEACH 千年血戦篇-禍進譚-』『無職転生III』『逃げ上手の若君 第2期』『コードギアス 奪還のロゼ』など続編・人気シリーズが並び、新規オリジナルより既存IPの続編が量産される傾向が続く。制作費高騰と当たり外れリスクの回避が背景。</t>
+        </is>
+      </c>
+      <c r="F436" s="14" t="inlineStr">
+        <is>
+          <t>夏クールは人気シリーズの続編が中心で、新規オリジナルは相対的に少ない。制作コスト高と失敗リスクを避けるため、実績あるIPの続編・分割2期に資源が集中している。視聴者の可処分時間の奪い合いで、認知済みタイトルが優先される構造が鮮明になった。</t>
+        </is>
+      </c>
+      <c r="G436" s="14" t="inlineStr">
+        <is>
+          <t>続編・分割2期の比率が高い
+新規オリジナルは投資判断が慎重に
+制作費高騰で確実に見られるIPを優先
+なろう/ラノベ原作が新規供給源の中心</t>
+        </is>
+      </c>
+      <c r="H436" s="14" t="inlineStr">
+        <is>
+          <t>制作委員会・配信各社は投資回収の確実性を求め、続編と既存IPの再アニメ化に一段と傾斜する。新規オリジナルは配信オリジナル枠か少数精鋭に絞られ、なろう/ラノベ原作が新規タイトルの主供給源であり続ける。続編偏重は中長期のIP枯渇リスクとして議論が強まる。</t>
+        </is>
+      </c>
+      <c r="I436" s="14" t="inlineStr">
+        <is>
+          <t>アニメの続編偏重とIPパイプラインの持続性</t>
+        </is>
+      </c>
+      <c r="J436" s="14" t="inlineStr">
+        <is>
+          <t>CloverWorks, サイエンスSARU</t>
+        </is>
+      </c>
+      <c r="K436" s="14" t="inlineStr">
+        <is>
+          <t>BLEACH, 無職転生, 逃げ上手の若君, コードギアス</t>
+        </is>
+      </c>
+      <c r="L436" s="14" t="inlineStr">
+        <is>
+          <t>配信,トレンド,国内</t>
+        </is>
+      </c>
+      <c r="M436" s="14" t="inlineStr">
+        <is>
+          <t>2026夏クール</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B437" s="14" t="inlineStr">
+        <is>
+          <t>アニメ</t>
+        </is>
+      </c>
+      <c r="C437" s="14" t="inlineStr">
+        <is>
+          <t>『スーパーの裏でヤニ吸うふたり』TBSでアニメ化——静かな会話劇の映像化</t>
+        </is>
+      </c>
+      <c r="D437" s="14" t="inlineStr">
+        <is>
+          <t>https://www.crank-in.net/animation/summer2026</t>
+        </is>
+      </c>
+      <c r="E437" s="14" t="inlineStr">
+        <is>
+          <t>地主による人気漫画『スーパーの裏でヤニ吸うふたり』のTVアニメ化が決定し、2026年にTBS系で全国放送される。バトルや異世界ではない日常の会話劇を描く青年向け作品のアニメ化が増えており、多様な題材が地上波/配信枠に乗るようになった。</t>
+        </is>
+      </c>
+      <c r="F437" s="14" t="inlineStr">
+        <is>
+          <t>地主の漫画『スーパーの裏でヤニ吸うふたり』がTBSでアニメ化決定。ど派手なジャンル作品ではない静かな会話劇のアニメ化で、SNSで話題の青年向け・ニッチ題材が映像化に乗る流れを示す。配信での間口拡大が多様な原作のアニメ化を後押ししている。</t>
+        </is>
+      </c>
+      <c r="G437" s="14" t="inlineStr">
+        <is>
+          <t>日常会話劇という非王道題材のアニメ化
+SNS発の話題性が映像化を後押し
+地上波×配信で多様な題材が成立
+漫画→アニメの供給パイプは健在</t>
+        </is>
+      </c>
+      <c r="H437" s="14" t="inlineStr">
+        <is>
+          <t>配信で世界同時に届くため、ニッチだが熱量の高い青年向け題材のアニメ化が増える。バトル/異世界一辺倒から題材が多様化し、原作漫画の映像化候補の裾野が広がる。ヒットすれば実写ドラマ化など横展開も見込め、出版社の映像化権ビジネスを厚くする。</t>
+        </is>
+      </c>
+      <c r="I437" s="14" t="inlineStr">
+        <is>
+          <t>非王道題材のアニメ化とニッチ需要の収益化</t>
+        </is>
+      </c>
+      <c r="J437" s="14" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="K437" s="14" t="inlineStr">
+        <is>
+          <t>スーパーの裏でヤニ吸うふたり</t>
+        </is>
+      </c>
+      <c r="L437" s="14" t="inlineStr">
+        <is>
+          <t>映像化,配信,国内</t>
+        </is>
+      </c>
+      <c r="M437" s="14" t="inlineStr">
+        <is>
+          <t>原作:漫画</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B438" s="14" t="inlineStr">
+        <is>
+          <t>漫画</t>
+        </is>
+      </c>
+      <c r="C438" s="14" t="inlineStr">
+        <is>
+          <t>講談社、『はたらく細胞』作者への編集対応を謝罪——原作者の権利に関心</t>
+        </is>
+      </c>
+      <c r="D438" s="14" t="inlineStr">
+        <is>
+          <t>https://furuhata.theletter.jp/posts/cdfba360-f5d7-44f7-9c62-ea577e956d60</t>
+        </is>
+      </c>
+      <c r="E438" s="14" t="inlineStr">
+        <is>
+          <t>2026年7月、講談社が『はたらく細胞』作者・清水茜氏に対する編集部の対応について謝罪した。作品の映像化・二次利用が拡大するなか、原作者と出版社の関係や作家の権利・処遇への社会的関心が高まっている。</t>
+        </is>
+      </c>
+      <c r="F438" s="14" t="inlineStr">
+        <is>
+          <t>講談社が『はたらく細胞』作者への編集対応を謝罪。ヒット作の映像化・海外展開でIP収益が拡大する一方、原作者の権利・処遇・意向の尊重が改めて問われる出来事。出版社のIPビジネス化が進むほど、作家との利害調整の透明性が経営リスクになりつつある。</t>
+        </is>
+      </c>
+      <c r="G438" s="14" t="inlineStr">
+        <is>
+          <t>ヒット作原作者への対応が問題化
+IP収益拡大と作家処遇のバランスが論点
+原作者の権利・意向尊重への社会的関心
+出版社のガバナンス/コンプラ課題</t>
+        </is>
+      </c>
+      <c r="H438" s="14" t="inlineStr">
+        <is>
+          <t>作家と出版社の契約・権利関係の透明化を求める声が強まり、映像化・二次利用の取り分やクレジットを巡る交渉が作家側優位に傾く場面が増える。出版社はIPで稼ぐほど作家リレーションの巧拙が競争力を左右し、専属契約や還元条件の見直しが進む可能性がある。</t>
+        </is>
+      </c>
+      <c r="I438" s="14" t="inlineStr">
+        <is>
+          <t>出版社のIP化と原作者の権利・処遇ガバナンス</t>
+        </is>
+      </c>
+      <c r="J438" s="14" t="inlineStr">
+        <is>
+          <t>講談社</t>
+        </is>
+      </c>
+      <c r="K438" s="14" t="inlineStr">
+        <is>
+          <t>はたらく細胞</t>
+        </is>
+      </c>
+      <c r="L438" s="14" t="inlineStr">
+        <is>
+          <t>権利・ライセンス,国内,人事・組織</t>
+        </is>
+      </c>
+      <c r="M438" s="14" t="inlineStr">
+        <is>
+          <t>2026/7 出版業界まとめ</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B439" s="14" t="inlineStr">
+        <is>
+          <t>小説</t>
+        </is>
+      </c>
+      <c r="C439" s="14" t="inlineStr">
+        <is>
+          <t>第175回直木賞に朝倉かすみ『けんぐゎい』、芥川賞候補に若林正恭『青天』</t>
+        </is>
+      </c>
+      <c r="D439" s="14" t="inlineStr">
+        <is>
+          <t>https://ddnavi.com/article/1404147/a/</t>
+        </is>
+      </c>
+      <c r="E439" s="14" t="inlineStr">
+        <is>
+          <t>2026年7月15日の選考会で第175回芥川賞・直木賞が決定。直木賞は朝倉かすみ『けんぐゎい』(光文社)が受賞した。芥川賞候補にはお笑い芸人オードリー・若林正恭の初小説『青天』が入り、著名人の純文学参入が話題を集めた。</t>
+        </is>
+      </c>
+      <c r="F439" s="14" t="inlineStr">
+        <is>
+          <t>第175回直木賞は朝倉かすみ『けんぐゎい』が受賞。芥川賞候補にオードリー若林正恭『青天』が選ばれ、タレント/芸人の本格文芸参入が注目された。文学賞は受賞作の話題性が販売と映像化に直結するため、著名人の参入は文芸市場の集客装置として機能している。</t>
+        </is>
+      </c>
+      <c r="G439" s="14" t="inlineStr">
+        <is>
+          <t>直木賞は朝倉かすみ『けんぐゎい』(光文社)
+芥川賞候補に若林正恭の初小説『青天』
+著名人の純文学参入で話題拡大
+受賞は販売・映像化権に直結</t>
+        </is>
+      </c>
+      <c r="H439" s="14" t="inlineStr">
+        <is>
+          <t>受賞・候補作は文庫化と映像化権の争奪が進み、出版社の下期売上を左右する。著名人の文芸参入は今後も続き、既存読者以外への裾野拡大に寄与する一方、話題先行への批判も出る。文学賞の集客力を活かしたメディアミックス前提の出版企画が増える。</t>
+        </is>
+      </c>
+      <c r="I439" s="14" t="inlineStr">
+        <is>
+          <t>文学賞の話題性と販売・映像化権への波及</t>
+        </is>
+      </c>
+      <c r="J439" s="14" t="inlineStr">
+        <is>
+          <t>光文社</t>
+        </is>
+      </c>
+      <c r="K439" s="14" t="inlineStr">
+        <is>
+          <t>けんぐゎい, 青天</t>
+        </is>
+      </c>
+      <c r="L439" s="14" t="inlineStr">
+        <is>
+          <t>受賞,出版,国内</t>
+        </is>
+      </c>
+      <c r="M439" s="14" t="inlineStr">
+        <is>
+          <t>第175回(2026上半期)</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B440" s="14" t="inlineStr">
+        <is>
+          <t>小説</t>
+        </is>
+      </c>
+      <c r="C440" s="14" t="inlineStr">
+        <is>
+          <t>2026夏は「なろう」発アニメが席巻——ラノベがアニメ新規供給の主パイプに</t>
+        </is>
+      </c>
+      <c r="D440" s="14" t="inlineStr">
+        <is>
+          <t>https://blog.syosetu.com/article/view/article_id/5189/</t>
+        </is>
+      </c>
+      <c r="E440" s="14" t="inlineStr">
+        <is>
+          <t>2026年7月クールでは『小説家になろう』発の作品が多数アニメ化され、異世界転生・ゲーム知識ものが並ぶ。オリジナル新規が減る中、Web小説→書籍化→アニメ化という育成パイプラインが、アニメの新規タイトル供給の中心になっている。</t>
+        </is>
+      </c>
+      <c r="F440" s="14" t="inlineStr">
+        <is>
+          <t>夏クールは「なろう」発アニメが多数を占め、Web小説がアニメの主要な新規供給源になっている。読者反応で当たりが可視化された作品を書籍化・アニメ化するため投資リスクが低い。ラノベ/Web小説の育成パイプがアニメIP不足を補う構造が定着した。</t>
+        </is>
+      </c>
+      <c r="G440" s="14" t="inlineStr">
+        <is>
+          <t>Web小説→書籍→アニメの育成パイプが中核
+読者反応で当たりを事前検証できる
+異世界転生ものが依然として量産
+アニメ新規IP不足をラノベが補完</t>
+        </is>
+      </c>
+      <c r="H440" s="14" t="inlineStr">
+        <is>
+          <t>Web小説プラットフォームがアニメIPの新人発掘場として重要性を増し、出版社・配信各社が有望作の書籍化・映像化権を早期に囲い込む動きが強まる。題材の同質化(異世界転生)への飽きが進めば、なろう内でも新ジャンルの発掘競争が起き、供給の多様化が課題になる。</t>
+        </is>
+      </c>
+      <c r="I440" s="14" t="inlineStr">
+        <is>
+          <t>Web小説の育成パイプとアニメIPの供給構造</t>
+        </is>
+      </c>
+      <c r="J440" s="14" t="inlineStr">
+        <is>
+          <t>KADOKAWA, 小説家になろう</t>
+        </is>
+      </c>
+      <c r="K440" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L440" s="14" t="inlineStr">
+        <is>
+          <t>映像化,出版,トレンド,国内</t>
+        </is>
+      </c>
+      <c r="M440" s="14" t="inlineStr">
+        <is>
+          <t>2026夏なろう発アニメ</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B441" s="14" t="inlineStr">
+        <is>
+          <t>音楽</t>
+        </is>
+      </c>
+      <c r="C441" s="14" t="inlineStr">
+        <is>
+          <t>Apple One値上げ¥1,980→¥2,500(約+26%)——サブスク疲れと選別が加速</t>
+        </is>
+      </c>
+      <c r="D441" s="14" t="inlineStr">
+        <is>
+          <t>https://library.libecity.com/articles/01KXX5D5XNJBHXVZS1HZJT4EV4</t>
+        </is>
+      </c>
+      <c r="E441" s="14" t="inlineStr">
+        <is>
+          <t>2026年7月、Apple Music・Apple TV・iCloud+を束ねるApple Oneが月額1,980円から2,500円へ値上げ(約26%増)。Apple TV単体は約33%の値上げ。動画・音楽サブスクの相次ぐ値上げで、家計のエンタメ可処分を巡る選別が消費者行動として強まっている。</t>
+        </is>
+      </c>
+      <c r="F441" s="14" t="inlineStr">
+        <is>
+          <t>Apple Oneが約26%値上げされ、音楽・動画のサブスク値上げ連鎖が続く。据え置きのHulu/U-NEXT/dアニメ等との差が広がり、ユーザーは併用から取捨選択へ移行しつつある。総合的なオーディオ/映像体験の価値が問われ、単なる楽曲数・作品数では正当化しにくくなっている。</t>
+        </is>
+      </c>
+      <c r="G441" s="14" t="inlineStr">
+        <is>
+          <t>Apple One約26%・Apple TV約33%の値上げ
+据え置き勢との価格差が拡大
+併用から排他的選択への消費行動
+体験価値でのサブスク差別化が必須に</t>
+        </is>
+      </c>
+      <c r="H441" s="14" t="inlineStr">
+        <is>
+          <t>家計のエンタメ可処分が逼迫し、音楽・動画・ゲームのサブスクが会員を奪い合う。通信×エンタメのバンドルや年払い割引で解約を抑える動きが強まり、値上げできるのは独自コンテンツ/体験を持つサービスに限られる。ARPU重視への転換で単価と解約率のバランスが焦点。</t>
+        </is>
+      </c>
+      <c r="I441" s="14" t="inlineStr">
+        <is>
+          <t>サブスク値上げと家計のエンタメ可処分の奪い合い</t>
+        </is>
+      </c>
+      <c r="J441" s="14" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="K441" s="14" t="inlineStr">
+        <is>
+          <t>Apple Music, Apple TV</t>
+        </is>
+      </c>
+      <c r="L441" s="14" t="inlineStr">
+        <is>
+          <t>配信,消費者インサイト,海外,トレンド</t>
+        </is>
+      </c>
+      <c r="M441" s="14" t="inlineStr">
+        <is>
+          <t>2026/7 値上げ</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B442" s="14" t="inlineStr">
+        <is>
+          <t>音楽</t>
+        </is>
+      </c>
+      <c r="C442" s="14" t="inlineStr">
+        <is>
+          <t>U-NEXT、ちゃんみな東京ドーム等を独占ライブ配信——配信各社の囲い込み</t>
+        </is>
+      </c>
+      <c r="D442" s="14" t="inlineStr">
+        <is>
+          <t>https://www.unext.co.jp/ja/press-room/2026-07-live-lineups</t>
+        </is>
+      </c>
+      <c r="E442" s="14" t="inlineStr">
+        <is>
+          <t>U-NEXTは2026年7月、ちゃんみなの東京ドーム公演やFRUITS ZIPPER4周年ツアーなどの独占ライブ配信を発表。フジロックのAmazon独占配信と同様、ライブ映像の独占が動画/音楽配信サービスの会員獲得・維持の武器になっている。</t>
+        </is>
+      </c>
+      <c r="F442" s="14" t="inlineStr">
+        <is>
+          <t>U-NEXTが人気アーティストのライブを独占配信ラインナップとして発表。ライブ映像はその時しか見られない希少性が高く、配信サービスの差別化・会員獲得の核になりつつある。フェスやアリーナ公演の独占配信権を巡り、プラットフォーム間の獲得競争が激化している。</t>
+        </is>
+      </c>
+      <c r="G442" s="14" t="inlineStr">
+        <is>
+          <t>ライブ独占配信が会員獲得の武器に
+希少性の高い生コンテンツを囲い込み
+フジロック(Amazon)と同じ独占配信競争
+アーティスト側は配信収益の新たな柱</t>
+        </is>
+      </c>
+      <c r="H442" s="14" t="inlineStr">
+        <is>
+          <t>ライブ配信権の争奪が進み、アーティスト/事務所にとって配信独占契約が新たな収益源になる。プラットフォームは独自ライブで差別化を図り値上げの正当化材料にする。一方で独占の分散は視聴者にとって見たい公演ごとに契約の負担増となり、選別を促す。</t>
+        </is>
+      </c>
+      <c r="I442" s="14" t="inlineStr">
+        <is>
+          <t>ライブ配信独占権とプラットフォームの差別化競争</t>
+        </is>
+      </c>
+      <c r="J442" s="14" t="inlineStr">
+        <is>
+          <t>U-NEXT, Amazon</t>
+        </is>
+      </c>
+      <c r="K442" s="14" t="inlineStr">
+        <is>
+          <t>ちゃんみな, FRUITS ZIPPER</t>
+        </is>
+      </c>
+      <c r="L442" s="14" t="inlineStr">
+        <is>
+          <t>配信,ライブ・イベント,権利・ライセンス,国内</t>
+        </is>
+      </c>
+      <c r="M442" s="14" t="inlineStr">
+        <is>
+          <t>2026/7ラインナップ</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B443" s="14" t="inlineStr">
+        <is>
+          <t>音楽</t>
+        </is>
+      </c>
+      <c r="C443" s="14" t="inlineStr">
+        <is>
+          <t>ILLIT日本2ndにHANAのJISOO/MOMOKAがfeat——日韓ガールズ相互起用が常態化</t>
+        </is>
+      </c>
+      <c r="D443" s="14" t="inlineStr">
+        <is>
+          <t>https://natalie.mu/music/news/679221</t>
+        </is>
+      </c>
+      <c r="E443" s="14" t="inlineStr">
+        <is>
+          <t>ILLITが7月26日配信の日本2ndシングル「I Got Your Back」の表題曲に、日本のガールズグループHANAのJISOOとMOMOKAをフィーチャリング/作詞で迎えた。K-POPとJ-POPのガールズグループが相互に楽曲参加する事例が増え、日韓のアイドル市場の一体化が進む。</t>
+        </is>
+      </c>
+      <c r="F443" s="14" t="inlineStr">
+        <is>
+          <t>ILLITの日本2ndシングル表題曲にHANAのメンバーがfeat/作詞で参加。K-POPとJ-POPの人気ガールズグループが相互に起用し合う動きで、両市場のファンを横断的に取り込む狙い。日韓アイドル市場の相互浸透が制作・プロモーションの前提になりつつある。</t>
+        </is>
+      </c>
+      <c r="G443" s="14" t="inlineStr">
+        <is>
+          <t>K-POP×J-POPガールズの相互feat
+両ファンダムの横断的な取り込み
+日韓アイドル市場の一体化が進行
+作詞参加まで踏み込むコラボ深化</t>
+        </is>
+      </c>
+      <c r="H443" s="14" t="inlineStr">
+        <is>
+          <t>日韓ガールズ/ボーイズグループの相互起用は市場統合の初手として定着し、合同楽曲・共同ツアー・共同オーディションへと深化する。国内レコード会社/事務所は韓国事務所との提携を強め、アジア横断のアイドル供給網が形成される。相互featはチャート戦略の定番になる。</t>
+        </is>
+      </c>
+      <c r="I443" s="14" t="inlineStr">
+        <is>
+          <t>日韓アイドル市場の相互浸透とファンダム横断戦略</t>
+        </is>
+      </c>
+      <c r="J443" s="14" t="inlineStr">
+        <is>
+          <t>BELIFT LAB</t>
+        </is>
+      </c>
+      <c r="K443" s="14" t="inlineStr">
+        <is>
+          <t>ILLIT, HANA</t>
+        </is>
+      </c>
+      <c r="L443" s="14" t="inlineStr">
+        <is>
+          <t>チャート・ランキング,提携,国内,海外</t>
+        </is>
+      </c>
+      <c r="M443" s="14" t="inlineStr">
+        <is>
+          <t>2026/7/26配信</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B444" s="14" t="inlineStr">
+        <is>
+          <t>音楽</t>
+        </is>
+      </c>
+      <c r="C444" s="14" t="inlineStr">
+        <is>
+          <t>ストリーミング総曲数2.5億に、AI生成曲のデマネタイズ広がる(Tidal/Deezer)</t>
+        </is>
+      </c>
+      <c r="D444" s="14" t="inlineStr">
+        <is>
+          <t>https://www.musicbusinessworldwide.com/quarter-of-a-billion-tracks-now-sit-on-music-streaming-services-where-does-it-end/</t>
+        </is>
+      </c>
+      <c r="E444" s="14" t="inlineStr">
+        <is>
+          <t>音楽ストリーミングの登録曲数が約2.5億に達し、AI生成曲の大量流入で発見性(ディスカバリー)が損なわれている。DeezerはAI生成曲の自動ラベル付けとプレイリスト除外、TidalはフルAI楽曲のデマネタイズを実施。一方Spotify/Apple Musicは静観気味で対応が分岐している。</t>
+        </is>
+      </c>
+      <c r="F444" s="14" t="inlineStr">
+        <is>
+          <t>ストリーミングの総曲数が約2.5億に膨張し、AI生成曲の氾濫で発見性の毀損が深刻化。Tidal/DeezerはAI曲のデマネタイズや除外に踏み込む一方、最大手のSpotify/Apple Musicは対応を抑制。AI生成コンテンツの扱いを巡りプラットフォーム間で方針が割れている。</t>
+        </is>
+      </c>
+      <c r="G444" s="14" t="inlineStr">
+        <is>
+          <t>総曲数2.5億で発見性が低下
+AI生成曲の大量流入が収益配分を希薄化
+Tidal/Deezerはデマネタイズ/除外に前進
+Spotify/Appleは静観で対応が分岐</t>
+        </is>
+      </c>
+      <c r="H444" s="14" t="inlineStr">
+        <is>
+          <t>AI生成曲の供給過多×発見性毀損はレコメンドの信頼性を下げ、キュレーション/人間の編集価値が再評価される。ロイヤリティ配分の不正(ストリーミング詐欺)対策と合わせ、AI曲の開示義務化やデマネタイズが業界標準へ向かう。同じ構図はゲームUGCや動画配信でも起きる。</t>
+        </is>
+      </c>
+      <c r="I444" s="14" t="inlineStr">
+        <is>
+          <t>AI生成コンテンツの供給過多と発見性・収益配分の防衛</t>
+        </is>
+      </c>
+      <c r="J444" s="14" t="inlineStr">
+        <is>
+          <t>Spotify, Apple, Tidal, Deezer</t>
+        </is>
+      </c>
+      <c r="K444" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L444" s="14" t="inlineStr">
+        <is>
+          <t>AI,配信,海外,トレンド</t>
+        </is>
+      </c>
+      <c r="M444" s="14" t="inlineStr">
+        <is>
+          <t>MBW</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B445" s="14" t="inlineStr">
+        <is>
+          <t>横断</t>
+        </is>
+      </c>
+      <c r="C445" s="14" t="inlineStr">
+        <is>
+          <t>Netflix、Variety/Billboard/THR等と提携しショート動画参入(8/3開始)</t>
+        </is>
+      </c>
+      <c r="D445" s="14" t="inlineStr">
+        <is>
+          <t>https://techcrunch.com/2026/07/07/netflix-dabbles-in-shorter-video-content-with-its-new-set-of-publisher-deals-with-variety-others/</t>
+        </is>
+      </c>
+      <c r="E445" s="14" t="inlineStr">
+        <is>
+          <t>Netflixは8月3日から、Variety・Rolling Stone・Billboard・THRなど出版/メディア各社の2〜20分のショート動画を米欧豪などで提供する。長尺SVODが短尺・雑誌ブランド由来の映像を取り込む動きで、動画プラットフォームのメディア吸収が進む。</t>
+        </is>
+      </c>
+      <c r="F445" s="14" t="inlineStr">
+        <is>
+          <t>NetflixがVariety・Billboard・THR等の出版社と提携し、2〜20分のショート動画を8/3から提供開始。長尺の映画/ドラマ中心だったSVODが短尺・情報系映像に広げ、YouTube/TikTok的な視聴時間も取りにいく。出版社は記事から映像へ、Netflix向けの制作収益を得る。</t>
+        </is>
+      </c>
+      <c r="G445" s="14" t="inlineStr">
+        <is>
+          <t>8/3から米欧豪等でショート動画提供
+雑誌ブランド(Variety/Billboard/THR)が映像供給
+SVODが短尺の視聴時間も獲得
+出版社はPF向け映像制作へ収益源が移動</t>
+        </is>
+      </c>
+      <c r="H445" s="14" t="inlineStr">
+        <is>
+          <t>動画プラットフォームがニュース/雑誌ブランドを映像コンテンツ源として取り込む流れが加速し、出版社は記事メディアからPF向け映像制作会社へと収益構造が移る。音楽(MV)やゲーム(実況)でも同様にPFがメディアブランドを内製吸収する動きが波及し、独立系メディアの交渉力が問われる。</t>
+        </is>
+      </c>
+      <c r="I445" s="14" t="inlineStr">
+        <is>
+          <t>動画PFによるメディアブランドの吸収と出版社の収益転換</t>
+        </is>
+      </c>
+      <c r="J445" s="14" t="inlineStr">
+        <is>
+          <t>Netflix, Variety, Billboard</t>
+        </is>
+      </c>
+      <c r="K445" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L445" s="14" t="inlineStr">
+        <is>
+          <t>提携,配信,海外,トレンド</t>
+        </is>
+      </c>
+      <c r="M445" s="14" t="inlineStr">
+        <is>
+          <t>2026/7/7発表</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -58183,7 +59289,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -58590,6 +59696,177 @@
       <c r="K7" s="14" t="inlineStr">
         <is>
           <t>Web→書籍→コミカライズ→アニメのなろう系標準ルート。供給過多下の低リスクIP開発例。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>ハウスメイド</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="inlineStr">
+        <is>
+          <t>小説</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>(海外ベストセラー小説)</t>
+        </is>
+      </c>
+      <c r="E8" s="14" t="inlineStr">
+        <is>
+          <t>映画</t>
+        </is>
+      </c>
+      <c r="F8" s="14" t="inlineStr">
+        <is>
+          <t>実写映画化(シドニー・スウィーニー主演のサスペンス)</t>
+        </is>
+      </c>
+      <c r="G8" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H8" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-27(日本公開)</t>
+        </is>
+      </c>
+      <c r="I8" s="14" t="inlineStr">
+        <is>
+          <t>公開間近</t>
+        </is>
+      </c>
+      <c r="J8" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K8" s="14" t="inlineStr">
+        <is>
+          <t>話題小説の実写化。原作既読層を初動に取り込む王道メディアミックス</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>モアナと伝説の海</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="inlineStr">
+        <is>
+          <t>アニメ</t>
+        </is>
+      </c>
+      <c r="D9" s="14" t="inlineStr">
+        <is>
+          <t>ウォルト・ディズニー</t>
+        </is>
+      </c>
+      <c r="E9" s="14" t="inlineStr">
+        <is>
+          <t>映画</t>
+        </is>
+      </c>
+      <c r="F9" s="14" t="inlineStr">
+        <is>
+          <t>実写映画化。日本版声優にME:IのTSUZUMIを起用</t>
+        </is>
+      </c>
+      <c r="G9" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H9" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-31(日本公開)</t>
+        </is>
+      </c>
+      <c r="I9" s="14" t="inlineStr">
+        <is>
+          <t>公開間近</t>
+        </is>
+      </c>
+      <c r="J9" s="14" t="inlineStr">
+        <is>
+          <t>ウォルト・ディズニー</t>
+        </is>
+      </c>
+      <c r="K9" s="14" t="inlineStr">
+        <is>
+          <t>ディズニーのアニメ→実写リメイク路線。日本はアイドル起用で話題化</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>スーパーの裏でヤニ吸うふたり</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="inlineStr">
+        <is>
+          <t>漫画</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>地主</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="inlineStr">
+        <is>
+          <t>アニメ</t>
+        </is>
+      </c>
+      <c r="F10" s="14" t="inlineStr">
+        <is>
+          <t>TVアニメ化(TBS系で全国放送)</t>
+        </is>
+      </c>
+      <c r="G10" s="14" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="H10" s="14" t="inlineStr">
+        <is>
+          <t>2026(予定)</t>
+        </is>
+      </c>
+      <c r="I10" s="14" t="inlineStr">
+        <is>
+          <t>発表</t>
+        </is>
+      </c>
+      <c r="J10" s="14" t="inlineStr">
+        <is>
+          <t>TBS</t>
+        </is>
+      </c>
+      <c r="K10" s="14" t="inlineStr">
+        <is>
+          <t>非王道の会話劇のアニメ化。ニッチ×高熱量題材が配信前提で成立</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
weekly-trends(6genres) update (2026-07-29 13:11)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -2805,7 +2805,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H45"/>
+  <dimension ref="A1:H49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4705,6 +4705,174 @@
       <c r="H45" t="inlineStr">
         <is>
           <t>漫画</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2026上半期・日本興行TOP3をアニメ独占＝実写邦画の地盤沈下</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>2026年上半期の日本映画興行はTOP3をアニメが独占し、100億円超が2本ともアニメ作品。7月最終週も『映画ちいかわ』が初登場1位（3日で興収22.4億）、ディズニー『トイ・ストーリー5』が累計85億超と、上位が家族向けアニメで固定化している。実写邦画は突出したヒットを欠き、配給各社は既存IP・アニメ映画へ製作リソースを一段と傾斜。劇場側もアニメ興行に収益を依存する構造が鮮明で、実写オリジナル企画の資金調達難という長期課題が数字で可視化された1週間だった。</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>東宝, ディズニー, 東映アニメーション</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>劇場興行はリスク回避が働きやすく、既存ファンダムを持つアニメIPに資金が集まる。実写オリジナルは回収不確実性が高く製作委員会の出資判断が慎重化。結果として「当てにいける題材＝アニメ／シリーズ」への集中が進み、興行カレンダーの多様性が痩せる。配信原資の縮小も実写中規模作の居場所を奪っている。</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>アニメ制作費高騰（1話2000万円超）と重なり、映像産業全体が「少数の高確度IP」へ資本を寄せる同型化が進む。音楽のカタログ投資やゲームの旧作依存と同じ「既存資産の再利用」志向。</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>https://eiga.com/ranking/jp/</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>横断</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Xbox Game Pass倍額値上げで数百万人解約＝コンソールサブスクの価格弾力性露呈</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>2025年10月にXbox Game Passの上位プランを実質倍増させたMicrosoftが、数百万人規模の解約に直面していたことが表面化。2026年4月に一部値下げしたが、離脱ユーザーの復帰は鈍いとの見方が業界内で優勢だ。定額制は「体感価値≒月額」の閾値を超えると一気に解約が起きることを、コンソール最大手のケースが実証した形。動画配信でもHulu（10月に1320円へ）やFODが値上げを重ね、ゲーム・映像・音楽のサブスク単価がこの3年で40〜60%上昇するなか、値上げ耐性の限界が具体的な数字で見えた週となった。</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Microsoft, Xbox, ソニー</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>サブスクは加入者数×単価で成長を描くが、コンテンツ供給コスト増を単価転嫁で吸収しようとすると解約が跳ねる。特にゲームは1本買い切りとの比較が容易で、価格弾力性が高い。「値上げ→離脱→値下げしても戻らない」は一度崩れた価格信頼の回復困難性を示す。</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>音楽・動画のサブスク疲れと同時進行。全ジャンルで「定額の上限」が同時に試されており、次はバンドル化・広告付き廉価プランへの回帰が横断的に起きうる。</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>https://keioh.ne.jp/subscription-price-increase</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>ゲーム</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>生成AI小説が文学賞最終選考・受賞レベルに到達＝作家の「AI活用力」格差</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>生成AIによる小説創作が実用段階に入り、AIを使った作品が国内外の文学賞で最終選考に残り、海外では受賞例も出ている。noteや『aiのべりすと』では毎月1万作以上のAI小説が公開され、市場規模は2022→2024年で約2倍に。インプレスが実践書『生成AI小説創作入門』を投入するなど、執筆支援ツールの体系化も進む。焦点は「AIが書くか否か」から「AIをどう使いこなすか」へ移り、プロット設計・推敲・翻訳をAIと協業できる書き手とそうでない書き手の生産性・質の差が拡大し始めている。</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>インプレス, note, カクヨム</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>小説は制作コストが低く個人でも参入しやすいため、AI活用の巧拙が可視化されやすい領域。出版社は「AI併用の是非」より「併用を前提にした編集・校閲・権利表示」の設計を迫られる。文学賞の選考基準や応募規定もAI開示ルールの整備が急務になる。</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>漫画・アニメの作画AI、音楽の生成AIと同じく「人間の監修価値」へ収斂。創作系ジャンル横断で「編集・ディレクション力」が希少資源化する。</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>https://genai-ai.co.jp/ai-kanri/blog/cc-ai-novel-writing/</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>小説</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Deezer調査97%がAI音楽を判別不能＝ストリーミングのAI楽曲氾濫とカタログ希薄化</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>2026年3月のDeezer国際調査で、一般リスナーの97%がAI生成音楽と人間制作の楽曲を聴き分けられないと判明。Suno・Udio等の生成ツールが量産する楽曲がストリーミングに大量流入し、再生数の総量が一定のまま楽曲数だけが膨張することで、1再生あたり単価とアーティスト取り分が希薄化する懸念が強まっている。Udioは2025年10月のUMG和解でダウンロードを停止しライセンス型へ転換、2026年にUMGとの共同PFを予定。プラットフォーム側はAI楽曲の識別・開示・分配ルールの整備を迫られている。</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Deezer, Universal Music, Udio, Suno, Spotify</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>ストリーミングは固定原資（サブスク収入）を再生数比で分配する仕組みのため、楽曲供給が無限に増えると1曲あたりの取り分が構造的に薄まる。AI量産はこの「分母膨張」を加速させ、人間アーティストの収益を圧迫。識別タグ付けと分配除外・別枠化が次の争点。</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>映像・小説のAI開示ルールと歩調。7/27の法務省「声の権利」報告書了承と合わせ、AI×権利処理が音楽で最も先鋭化している。</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>https://www.musicman.co.jp/business/717998</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>音楽</t>
         </is>
       </c>
     </row>
@@ -50754,7 +50922,11 @@
       <c r="I6" s="9" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="inlineStr"/>
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
           <t>アニメ映画の世界的躍進</t>
@@ -50765,12 +50937,36 @@
           <t>コンテンツ</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr"/>
-      <c r="E7" s="9" t="inlineStr"/>
-      <c r="F7" s="9" t="inlineStr"/>
-      <c r="G7" s="9" t="inlineStr"/>
-      <c r="H7" s="9" t="inlineStr"/>
-      <c r="I7" s="9" t="inlineStr"/>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>2026上半期の日本興行はTOP3をアニメが独占、100億超2本ともアニメ。7月末も『映画ちいかわ』が初登場1位。</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>家族向けアニメIPが劇場収益を牽引し上位を固定化。実写大作の不在を補完する構図が定着。</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>東宝, ディズニー, 東映アニメーション</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>既存ファンダム型アニメIPへの資本集中がさらに進行。劇場の収益依存度が上昇。</t>
+        </is>
+      </c>
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>アニメ映画への一極集中は興行の多様性を痩せさせるリスクと表裏。</t>
+        </is>
+      </c>
+      <c r="I7" s="9" t="inlineStr">
+        <is>
+          <t>https://eiga.com/ranking/jp/</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr"/>
@@ -50792,7 +50988,11 @@
       <c r="I8" s="9" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="inlineStr"/>
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
           <t>邦画実写のヒット構造</t>
@@ -50803,12 +51003,36 @@
           <t>市場</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr"/>
-      <c r="E9" s="9" t="inlineStr"/>
-      <c r="F9" s="9" t="inlineStr"/>
-      <c r="G9" s="9" t="inlineStr"/>
-      <c r="H9" s="9" t="inlineStr"/>
-      <c r="I9" s="9" t="inlineStr"/>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>2026上半期、実写邦画に突出したヒットが乏しく、興行上位をアニメに明け渡す状況が続く。</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>実写オリジナルの資金調達難が鮮明。配給は既存IP・シリーズへ製作を傾斜。</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>東宝, 松竹, 東映</t>
+        </is>
+      </c>
+      <c r="G9" s="9" t="inlineStr">
+        <is>
+          <t>中規模実写オリジナルの居場所が縮小。配信原資の減少も逆風。</t>
+        </is>
+      </c>
+      <c r="H9" s="9" t="inlineStr">
+        <is>
+          <t>「当てにいける題材」偏重で実写の新規性が細る同型化リスク。</t>
+        </is>
+      </c>
+      <c r="I9" s="9" t="inlineStr">
+        <is>
+          <t>https://freetherock.com/2026/07/13/cinead-2026-h1-box-office-ranking/</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -52602,7 +52826,11 @@
       <c r="I6" s="9" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="inlineStr"/>
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
           <t>劇場アニメの興行構造</t>
@@ -52613,12 +52841,36 @@
           <t>興行</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr"/>
-      <c r="E7" s="9" t="inlineStr"/>
-      <c r="F7" s="9" t="inlineStr"/>
-      <c r="G7" s="9" t="inlineStr"/>
-      <c r="H7" s="9" t="inlineStr"/>
-      <c r="I7" s="9" t="inlineStr"/>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>7月最終週、『映画ちいかわ 人魚の島のひみつ』が初登場1位（3日で動員150.8万・興収22.4億）。上半期もアニメが邦画興行を牽引。</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>キャラIPの短期集中興行が定着。ファミリー層の初動動員が興収を左右する構造。</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>東宝, 東映アニメーション</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>強IPの劇場版が製作費回収の主要ルートに。中小オリジナル劇場アニメとの二極化。</t>
+        </is>
+      </c>
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>劇場アニメが映像産業全体の「確度の高い収益源」として資本を吸引。</t>
+        </is>
+      </c>
+      <c r="I7" s="9" t="inlineStr">
+        <is>
+          <t>https://eiga.com/ranking/jp/</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr"/>
@@ -58390,7 +58642,11 @@
       <c r="I6" s="9" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="inlineStr"/>
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
           <t>生成AIと小説執筆・翻訳</t>
@@ -58401,12 +58657,36 @@
           <t>技術</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr"/>
-      <c r="E7" s="9" t="inlineStr"/>
-      <c r="F7" s="9" t="inlineStr"/>
-      <c r="G7" s="9" t="inlineStr"/>
-      <c r="H7" s="9" t="inlineStr"/>
-      <c r="I7" s="9" t="inlineStr"/>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>AI併用小説が国内外の文学賞で最終選考・受賞レベルに到達。noteや『aiのべりすと』で月1万作超のAI小説が公開。</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>焦点が「AIが書くか」から「どう使いこなすか」へ移行。執筆支援書の体系化も進む。</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>インプレス, note, カクヨム</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>AI活用力による作家間の生産性・質の格差が拡大。賞のAI開示ルール整備が急務。</t>
+        </is>
+      </c>
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>漫画・音楽の生成AIと同じく人間の「編集・監修価値」へ収斂。</t>
+        </is>
+      </c>
+      <c r="I7" s="9" t="inlineStr">
+        <is>
+          <t>https://genai-ai.co.jp/ai-kanri/blog/cc-ai-novel-writing/</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr"/>
@@ -60266,7 +60546,7 @@
     <row r="5">
       <c r="A5" s="25" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B5" s="9" t="inlineStr">
@@ -60281,32 +60561,32 @@
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
-          <t>法務省が『声』を法的保護対象に含める指針を8月にも公表方針(7/13検討会)。</t>
+          <t>法務省が7/27に「声の権利」報告書を了承（声優・歌手・俳優の声もパブリシティ権対象、収益目的が判断基準）。Deezer調査で97%がAI音楽を判別不能。</t>
         </is>
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>AIによる声優・歌手の声の無断模倣が急増。Suno/Udioと大手レーベルの訴訟も継続。SpotifyはAI開示のDDEX標準を支持。</t>
+          <t>AI量産曲のストリーミング流入で1再生単価が希薄化。Udioは2025/10のUMG和解でライセンス型へ転換、2026にUMG共同PF予定。</t>
         </is>
       </c>
       <c r="F5" s="9" t="inlineStr">
         <is>
-          <t>法務省, Suno, Udio, ElevenLabs, Spotify</t>
+          <t>Deezer, Universal Music, Udio, Suno</t>
         </is>
       </c>
       <c r="G5" s="9" t="inlineStr">
         <is>
-          <t>声・肖像の同意と対価処理が標準実務化。AI合成前提のコスト設計が崩れ、権利者の交渉力上昇。</t>
+          <t>AI楽曲の識別タグ・開示・分配別枠化が次の争点。声の権利は実務ガイドライン整備へ。</t>
         </is>
       </c>
       <c r="H5" s="9" t="inlineStr">
         <is>
-          <t>音楽・アニメ/ゲーム声優・映画俳優を横断する『合成同一性』の権利化。</t>
+          <t>AI×権利処理が音楽で最先鋭化。声(声優)・映像・小説へ横串で波及。</t>
         </is>
       </c>
       <c r="I5" s="9" t="inlineStr">
         <is>
-          <t>https://www.nikkei.com/article/DGXZQOUA252BN0V20C26A6000000/</t>
+          <t>https://www.nikkei.com/article/DGXZQOUA250Q60V20C26A7000000/</t>
         </is>
       </c>
     </row>
@@ -64885,8 +65165,10 @@
       <c r="J3" s="9" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="25" t="n">
-        <v>46223</v>
+      <c r="A4" s="25" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
@@ -64900,32 +65182,32 @@
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>値上げ耐性の限界がゲーム・音楽・映像でほぼ同時に露呈。単価引き上げから広告付き下位ティア・バンドル・保有期間長期化への再設計が進む。</t>
+          <t>Xbox Game Passの倍額値上げ（2025/10）で数百万人が解約、2026/4に一部値下げも復帰は鈍い。動画もHulu・FODが値上げ。</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
         <is>
-          <t>主要ストリーミングの月額レンジは2022年の10-15ドルから2026年初頭に17-25ドルへ移行し、サブスク束の合計負担は3年で40-60%増。日本の30代世帯は平均6.8件契約、通信・娯楽支出の約3割が定額制。Game Pass値上げ時の大量解約を受けた6月の値下げとCoD day-one撤回は、この家計制約への対応と読める。映画側では45日ウィンドウ標準化という逆方向の『希少性回復』が同時進行。</t>
+          <t>コンソールサブスクの価格弾力性が露呈。単価転嫁の限界が具体数字で表面化。</t>
         </is>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
-          <t>Microsoft/Xbox Game Pass, Sony PS Plus, Spotify, Netflix, Amazon, U-NEXT</t>
+          <t>Microsoft, Xbox, ソニー</t>
         </is>
       </c>
       <c r="G4" s="9" t="inlineStr">
         <is>
-          <t>家計の定額枠が総量規制的に振る舞うため、値上げは他社への乗り換えではなく『1本解約』を誘発する。ゲームサブスクは映像・音楽サブスクと同じ枠を奪い合う直接競合であり、単独の価格戦略は成立しにくくなる。</t>
+          <t>バンドル化・広告付き廉価プランへの回帰が横断的に進む可能性。</t>
         </is>
       </c>
       <c r="H4" s="9" t="inlineStr">
         <is>
-          <t>サブスク疲れはジャンル固有ではなく家計側の総量制約。ゲーム・音楽・映像の値上げ余地は互いに食い合う。</t>
+          <t>「値上げ→離脱→値下げしても戻らない」価格信頼の回復困難性。音楽・動画と同時進行。</t>
         </is>
       </c>
       <c r="I4" s="9" t="inlineStr">
         <is>
-          <t>https://app-picklist.com/subscription-monthly-total-average/</t>
+          <t>https://keioh.ne.jp/subscription-price-increase</t>
         </is>
       </c>
       <c r="J4" s="9" t="inlineStr"/>

</xml_diff>

<commit_message>
daily-news(6genres) + cross-questions + media-mix + predictions update
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -891,7 +891,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H45"/>
+  <dimension ref="A1:H46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2789,6 +2789,48 @@
         </is>
       </c>
       <c r="H45" s="15" t="inlineStr">
+        <is>
+          <t>音楽</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B46" s="15" t="inlineStr">
+        <is>
+          <t>音楽大手の収益軸が原盤ライセンス(ストリーミング分配)から“ファンダム運営・ライブ制作・物販EC”の直接参加型(D2F)へ移り、HYBE型の垂直統合を追う形でレーベル/事務所がライブ制作会社・ファンプラットフォーム・チケッティング・ECを買収して囲い込む。原盤権中心のUMG/WMGとは収益構造が乖離する。</t>
+        </is>
+      </c>
+      <c r="C46" s="15" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="D46" s="15" t="inlineStr">
+        <is>
+          <t>2027年内</t>
+        </is>
+      </c>
+      <c r="E46" s="15" t="inlineStr">
+        <is>
+          <t>HYBE, ソニーミュージック, エイベックス, UMG, WMG</t>
+        </is>
+      </c>
+      <c r="F46" s="15" t="inlineStr">
+        <is>
+          <t>「HYBE2Qは四半期売上初の1兆ウォン超・営業益過去最高」(RBB TODAY)、「ライブ・エンタメ市場2025年8564億円で過去最高」(ぴあ総研/日経)</t>
+        </is>
+      </c>
+      <c r="G46" s="15" t="inlineStr">
+        <is>
+          <t>HYBE・大手事務所によるライブ制作会社/ファンプラットフォーム/チケッティングのM&amp;A発表の有無と、UMG/WMGのD2F(direct-to-fan)投資・買収発表を今後2〜4四半期で観測する。</t>
+        </is>
+      </c>
+      <c r="H46" s="15" t="inlineStr">
         <is>
           <t>音楽</t>
         </is>
@@ -5913,7 +5955,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H97"/>
+  <dimension ref="A1:H99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9995,6 +10037,90 @@
         </is>
       </c>
       <c r="H97" s="15" t="inlineStr">
+        <is>
+          <t>横断</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B98" s="15" t="inlineStr">
+        <is>
+          <t>HYBEで公演・MD(直接参加型)が音盤・音源を上回った構造は、ゲーム(ライブ/物販)やアニメ(舞台・グッズ・ライブ)でも“収益の主役が本編から体験・物販へ移る”形で起きるか？</t>
+        </is>
+      </c>
+      <c r="C98" s="15" t="inlineStr">
+        <is>
+          <t>HYBE 2Q過去最高・公演/MDが音盤音源を上回る(RBB TODAY, 2026-07)</t>
+        </is>
+      </c>
+      <c r="D98" s="15" t="inlineStr">
+        <is>
+          <t>HYBE, BTS, カバー(ホロライブ), アニプレックス</t>
+        </is>
+      </c>
+      <c r="E98" s="15" t="inlineStr">
+        <is>
+          <t>イベント/不動産(アリーナ), 物販EC, ファッション(コラボMD)</t>
+        </is>
+      </c>
+      <c r="F98" s="15" t="inlineStr">
+        <is>
+          <t>オープン</t>
+        </is>
+      </c>
+      <c r="G98" s="15" t="inlineStr">
+        <is>
+          <t>“本編(音源/ゲーム本体/映像)は入口、稼ぎはライブ・物販・ファンダム”という同型が全ジャンルで進行。カバーのVTuberゲーム全ストア首位も同根。</t>
+        </is>
+      </c>
+      <c r="H98" s="15" t="inlineStr">
+        <is>
+          <t>横断</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B99" s="15" t="inlineStr">
+        <is>
+          <t>小学館で映像化版権収入(+26.8%)が本体の増益を牽引した“二次利用が本業を上回る”構造は、ゲーム(IPライセンス)・音楽(シンク/原盤ライセンス)でも主収益になるか？</t>
+        </is>
+      </c>
+      <c r="C99" s="15" t="inlineStr">
+        <is>
+          <t>小学館87期・映像化版権+26.8%で増収増益(The Bunka News, 2026-07)</t>
+        </is>
+      </c>
+      <c r="D99" s="15" t="inlineStr">
+        <is>
+          <t>小学館, 集英社, カプコン(参考)</t>
+        </is>
+      </c>
+      <c r="E99" s="15" t="inlineStr">
+        <is>
+          <t>広告(タイアップ), 玩具, テーマパーク/不動産</t>
+        </is>
+      </c>
+      <c r="F99" s="15" t="inlineStr">
+        <is>
+          <t>オープン</t>
+        </is>
+      </c>
+      <c r="G99" s="15" t="inlineStr">
+        <is>
+          <t>“作品を売る”から“IPを貸す/多重展開する”へ。IGポートの版権好調・制作不振とも同じ方向。</t>
+        </is>
+      </c>
+      <c r="H99" s="15" t="inlineStr">
         <is>
           <t>横断</t>
         </is>
@@ -19498,7 +19624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M460"/>
+  <dimension ref="A1:M479"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -50276,6 +50402,1213 @@
         </is>
       </c>
       <c r="M460" s="15" t="inlineStr"/>
+    </row>
+    <row r="461">
+      <c r="A461" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B461" s="15" t="inlineStr">
+        <is>
+          <t>ゲーム</t>
+        </is>
+      </c>
+      <c r="C461" s="15" t="inlineStr">
+        <is>
+          <t>KRAFTON 2Qは営業益67%増・四半期過去最高、『Subnautica 2』とPUBGが牽引</t>
+        </is>
+      </c>
+      <c r="D461" s="15" t="inlineStr">
+        <is>
+          <t>https://gamebiz.jp/news/430201</t>
+        </is>
+      </c>
+      <c r="E461" s="15" t="inlineStr">
+        <is>
+          <t>PUBG依存からの脱却が課題だったKRAFTONが、5月アーリーアクセス投入の『Subnautica 2』を22日で500万本超に伸ばし、PC売上が四半期で初めて5000億ウォンを超えた。上半期は売上・営業益ともに過去最高を更新。</t>
+        </is>
+      </c>
+      <c r="F461" s="15" t="inlineStr">
+        <is>
+          <t>2026年2Qは売上1兆2900億ウォン(前年比+94.9%)、営業益4109億ウォン(+67.0%)でともに四半期過去最高。買収IPのSubnauticaと既存IPのPUBG(+25%)の二本柱が収益を押し上げ、単一IP依存からの多角化が進んだ。</t>
+        </is>
+      </c>
+      <c r="G461" s="15" t="inlineStr">
+        <is>
+          <t>・買収IP『Subnautica』で収益源を多角化
+・アーリーアクセスで22日500万本＝完成前から大型収益化
+・PC売上が四半期で初の5000億ウォン超</t>
+        </is>
+      </c>
+      <c r="H461" s="15" t="inlineStr">
+        <is>
+          <t>KRAFTONは新興市場とM&amp;Aで取得したIPの運用に一段と傾斜する見込み。Subnautica 2は正式版でさらに伸びる余地があり、買収スタジオのIPを“第二のPUBG”に育てられるかが評価軸になる。中規模スタジオ買収の連鎖も予想される。</t>
+        </is>
+      </c>
+      <c r="I461" s="15" t="inlineStr">
+        <is>
+          <t>買収IPのライブ運営化と単一IP依存リスク</t>
+        </is>
+      </c>
+      <c r="J461" s="15" t="inlineStr">
+        <is>
+          <t>KRAFTON, Unknown Worlds</t>
+        </is>
+      </c>
+      <c r="K461" s="15" t="inlineStr">
+        <is>
+          <t>PUBG, Subnautica 2</t>
+        </is>
+      </c>
+      <c r="L461" s="15" t="inlineStr">
+        <is>
+          <t>業績, 海外</t>
+        </is>
+      </c>
+      <c r="M461" s="15" t="inlineStr"/>
+    </row>
+    <row r="462">
+      <c r="A462" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B462" s="15" t="inlineStr">
+        <is>
+          <t>ゲーム</t>
+        </is>
+      </c>
+      <c r="C462" s="15" t="inlineStr">
+        <is>
+          <t>GENDA、SBIホールディングスと資本業務提携 SBIネオコンテンツファンドに3億円出資</t>
+        </is>
+      </c>
+      <c r="D462" s="15" t="inlineStr">
+        <is>
+          <t>https://gamebiz.jp/news/430193</t>
+        </is>
+      </c>
+      <c r="E462" s="15" t="inlineStr">
+        <is>
+          <t>アミューズメント施設運営から企業買収でエンタメ領域を拡大してきたGENDAが金融のSBIHDと資本業務提携。SBIが組成するコンテンツ特化ファンドへ出資し、SBIはGENDA株を発行済の1.00%を上限に市場買付で取得する。</t>
+        </is>
+      </c>
+      <c r="F462" s="15" t="inlineStr">
+        <is>
+          <t>GENDAはSBIネオコンテンツファンドに3億円を出資し、SBIHDと資本業務提携を締結。SBIHDはGENDA株を最大1.00%取得する。金融資本とエンタメ事業会社が相互に株式を持ち合い、コンテンツ投資で協業する枠組みが立ち上がった。</t>
+        </is>
+      </c>
+      <c r="G462" s="15" t="inlineStr">
+        <is>
+          <t>・エンタメ事業会社×金融の資本提携＝コンテンツ投資の共同ファンド化
+・SBIがGENDA株を市場買付、相互資本関係を構築
+・M&amp;A原資・案件ソーシングで金融の関与が深まる</t>
+        </is>
+      </c>
+      <c r="H462" s="15" t="inlineStr">
+        <is>
+          <t>エンタメIP・スタジオのM&amp;Aに金融(ファンド)資金が本格流入する布石。GENDAは買収の原資と案件パイプラインを金融側から確保でき、ゲーム・音楽・アニメの中小事業者買収が加速しうる。ソブリン資金と並び“金融発のエンタメ投資”が国内でも顕在化する。</t>
+        </is>
+      </c>
+      <c r="I462" s="15" t="inlineStr">
+        <is>
+          <t>金融資本によるエンタメM&amp;Aファンドの台頭</t>
+        </is>
+      </c>
+      <c r="J462" s="15" t="inlineStr">
+        <is>
+          <t>GENDA, SBIホールディングス</t>
+        </is>
+      </c>
+      <c r="K462" s="15" t="inlineStr">
+        <is>
+          <t>SBIネオコンテンツファンド</t>
+        </is>
+      </c>
+      <c r="L462" s="15" t="inlineStr">
+        <is>
+          <t>出資, 提携, 国内</t>
+        </is>
+      </c>
+      <c r="M462" s="15" t="inlineStr"/>
+    </row>
+    <row r="463">
+      <c r="A463" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B463" s="15" t="inlineStr">
+        <is>
+          <t>ゲーム</t>
+        </is>
+      </c>
+      <c r="C463" s="15" t="inlineStr">
+        <is>
+          <t>ドリコム、インディーゲーム事業を本格展開へ 28年3月期に5〜10本弱を投入</t>
+        </is>
+      </c>
+      <c r="D463" s="15" t="inlineStr">
+        <is>
+          <t>https://gamebiz.jp/news/430198</t>
+        </is>
+      </c>
+      <c r="E463" s="15" t="inlineStr">
+        <is>
+          <t>『ウィズダフネ』で1Q黒字転換したドリコムが、自社の“IP創出機能”を強みにインディーゲーム事業を本格化。『TOKYO STORIES』に手応えを示し、複数タイトルのパブリッシング/共同開発を計画する。外部決済導入によるコスト改善も寄与した。</t>
+        </is>
+      </c>
+      <c r="F463" s="15" t="inlineStr">
+        <is>
+          <t>ドリコムの1Q営業益は5.2億円で黒字転換。今後インディー領域でIP創出を狙い、28年3月期に5〜10本弱を投入する方針を示した。運営型大作偏重への対抗として、中小規模IPの本数を確保しポートフォリオを分散させる戦略に踏み出す。</t>
+        </is>
+      </c>
+      <c r="G463" s="15" t="inlineStr">
+        <is>
+          <t>・中堅パブリッシャーがインディー投資・共同開発を柱に
+・外部(アプリ外)決済でコスト改善＝採算構造の見直し
+・大作一本足からIPポートフォリオ分散へ</t>
+        </is>
+      </c>
+      <c r="H463" s="15" t="inlineStr">
+        <is>
+          <t>国内中堅パブリッシャーが“少数の大作”から“多数の中小IP”へ投資を分散する動きが広がりそう。インディー開発者には国内資金の受け皿が増える一方、パブリッシャー間で有望作品の取り合い(前渡し金インフレ)が起きる可能性がある。</t>
+        </is>
+      </c>
+      <c r="I463" s="15" t="inlineStr">
+        <is>
+          <t>中堅パブリッシャーのインディー投資分散戦略</t>
+        </is>
+      </c>
+      <c r="J463" s="15" t="inlineStr">
+        <is>
+          <t>ドリコム</t>
+        </is>
+      </c>
+      <c r="K463" s="15" t="inlineStr">
+        <is>
+          <t>ウィズダフネ, TOKYO STORIES</t>
+        </is>
+      </c>
+      <c r="L463" s="15" t="inlineStr">
+        <is>
+          <t>インディー, 新作, 国内</t>
+        </is>
+      </c>
+      <c r="M463" s="15" t="inlineStr"/>
+    </row>
+    <row r="464">
+      <c r="A464" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B464" s="15" t="inlineStr">
+        <is>
+          <t>ゲーム</t>
+        </is>
+      </c>
+      <c r="C464" s="15" t="inlineStr">
+        <is>
+          <t>Aiming、コンシューマゲーム開発に本格参入 開発パイプラインに初めて追加</t>
+        </is>
+      </c>
+      <c r="D464" s="15" t="inlineStr">
+        <is>
+          <t>https://gamebiz.jp/news/430207</t>
+        </is>
+      </c>
+      <c r="E464" s="15" t="inlineStr">
+        <is>
+          <t>モバイルオンライン専業だったAimingは2Q(1〜6月)が減収減益ながら、レベルファイブと組む『イナズマイレブン クロス』が想定超えのスタート。椎葉社長はコンシューマ開発を今後も継続する方針を示し、開発パイプラインに初めて据えた。</t>
+        </is>
+      </c>
+      <c r="F464" s="15" t="inlineStr">
+        <is>
+          <t>Aimingの2Qは売上-23%・営業益-71%と減収減益。一方で新作が好調で7月も勢いを維持。AAA級ではないがコンシューマ参入を継続方針とし、モバイル専業からの事業構造転換を打ち出した。既存IPホルダーとの協業で参入リスクを抑える。</t>
+        </is>
+      </c>
+      <c r="G464" s="15" t="inlineStr">
+        <is>
+          <t>・モバイル専業デベロッパーがコンシューマ市場へ本格参入
+・減収減益下でも新作IPで底打ちを図る
+・IPホルダー(レベルファイブ)との協業で参入リスクを低減</t>
+        </is>
+      </c>
+      <c r="H464" s="15" t="inlineStr">
+        <is>
+          <t>モバイルF2P専業各社が、ガチャ規制リスクと買い切り/サブスク市場の拡大を背景にコンシューマへ軸足を移す流れが続きそう。既存IPホルダーとの協業で参入障壁を下げる手法が定番化し、モバイル運営で培った運用ノウハウを買い切り＋DLC型へ転用する動きが増える。</t>
+        </is>
+      </c>
+      <c r="I464" s="15" t="inlineStr">
+        <is>
+          <t>モバイル専業のコンシューマ移行と運用ノウハウ転用</t>
+        </is>
+      </c>
+      <c r="J464" s="15" t="inlineStr">
+        <is>
+          <t>Aiming, レベルファイブ</t>
+        </is>
+      </c>
+      <c r="K464" s="15" t="inlineStr">
+        <is>
+          <t>イナズマイレブン クロス</t>
+        </is>
+      </c>
+      <c r="L464" s="15" t="inlineStr">
+        <is>
+          <t>業績, 新作, 国内</t>
+        </is>
+      </c>
+      <c r="M464" s="15" t="inlineStr"/>
+    </row>
+    <row r="465">
+      <c r="A465" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B465" s="15" t="inlineStr">
+        <is>
+          <t>ゲーム</t>
+        </is>
+      </c>
+      <c r="C465" s="15" t="inlineStr">
+        <is>
+          <t>カバー『ホロライブドリームス』が配信全ストアで首位 VTuber IPの課金転換力を実証</t>
+        </is>
+      </c>
+      <c r="D465" s="15" t="inlineStr">
+        <is>
+          <t>https://gamebiz.jp/news/430099</t>
+        </is>
+      </c>
+      <c r="E465" s="15" t="inlineStr">
+        <is>
+          <t>VTuber事務所ホロライブを運営するカバーが、QualiArtsと共同開発した新作『ホロライブドリームス』をリリース。App Store・Google Play・Steamの全ストアで売上/セールス首位を獲得し、VTuberファンダムのゲーム課金への転換力を示した。</t>
+        </is>
+      </c>
+      <c r="F465" s="15" t="inlineStr">
+        <is>
+          <t>『ホロライブドリームス』はリリースした全ストアで首位を獲得。VTuber IPが配信・グッズを超え、ゲームというストック型課金でも強い初速を出せることを実証した事例。単なる好調報告ではなく“ファンダムの課金転換力”という消費者インサイトとして注目に値する。</t>
+        </is>
+      </c>
+      <c r="G465" s="15" t="inlineStr">
+        <is>
+          <t>・VTuber IPのゲーム化がローンチ即・全ストア首位
+・配信・グッズに続く“ゲーム”という収益レイヤーの確立
+・自社IPの内製ゲーム化でライセンス流出を回避</t>
+        </is>
+      </c>
+      <c r="H465" s="15" t="inlineStr">
+        <is>
+          <t>VTuber/配信者IPを核にしたゲーム化が、外部IPコラボに次ぐ集客手段として定着する見込み。ファンダムの熱量を課金に変換するモデルが実証されたことで、他のタレント・配信事務所もゲーム内製やIPライセンスに動き、“ファンダム発ゲーム”がジャンル化する可能性がある。</t>
+        </is>
+      </c>
+      <c r="I465" s="15" t="inlineStr">
+        <is>
+          <t>ファンダム(VTuber)IPのゲーム課金転換</t>
+        </is>
+      </c>
+      <c r="J465" s="15" t="inlineStr">
+        <is>
+          <t>カバー, QualiArts, サイバーエージェント</t>
+        </is>
+      </c>
+      <c r="K465" s="15" t="inlineStr">
+        <is>
+          <t>ホロライブドリームス, ホロライブ</t>
+        </is>
+      </c>
+      <c r="L465" s="15" t="inlineStr">
+        <is>
+          <t>チャート・ランキング, 消費者インサイト, 国内</t>
+        </is>
+      </c>
+      <c r="M465" s="15" t="inlineStr"/>
+    </row>
+    <row r="466">
+      <c r="A466" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B466" s="15" t="inlineStr">
+        <is>
+          <t>ゲーム</t>
+        </is>
+      </c>
+      <c r="C466" s="15" t="inlineStr">
+        <is>
+          <t>Switch 2は9か月で1986万台とSwitch超の立ち上がり、好調下でも北米値上げ観測</t>
+        </is>
+      </c>
+      <c r="D466" s="15" t="inlineStr">
+        <is>
+          <t>https://thisweekinvideogames.com/news/nintendo-sells-19-86-million-switch-2-consoles-expects-to-move-16-million-more-in-12-months/</t>
+        </is>
+      </c>
+      <c r="E466" s="15" t="inlineStr">
+        <is>
+          <t>任天堂のSwitch 2は発売9か月(3月末時点)で1986万台に到達し、初代Switchを45%上回るペース、同時期のPS5を約800万台上回った。品薄が解消しつつある中、コスト・為替を背景に北米での価格改定が取り沙汰されている。</t>
+        </is>
+      </c>
+      <c r="F466" s="15" t="inlineStr">
+        <is>
+          <t>Switch 2は初動でハード史上有数の立ち上がりを見せ、任天堂は今後12か月でさらに1600万台の販売を見込む。一方、好調にもかかわらず北米で価格引き上げ(499.99ドルへ)が報じられ、“売れているのに値上げ”という需要と価格転嫁の綱引きが焦点になっている。</t>
+        </is>
+      </c>
+      <c r="G466" s="15" t="inlineStr">
+        <is>
+          <t>・初代Switch比+45%ペース、PS5を上回る立ち上がり
+・好調でも部材コスト/為替で価格改定が視野に
+・ハード値上げはソフト/サブスクの収益設計にも波及</t>
+        </is>
+      </c>
+      <c r="H466" s="15" t="inlineStr">
+        <is>
+          <t>ハードが好調でも値上げに動く場合、“導入機を赤字で売って回収”の伝統モデルから、ハード単体でも利益を取る価格戦略への転換を示唆する。値上げが実施されれば周辺機器・サブスク・ソフト価格の再設定が続き、他社の据置/携帯機戦略にも影響する。</t>
+        </is>
+      </c>
+      <c r="I466" s="15" t="inlineStr">
+        <is>
+          <t>ハード黒字化前提の価格戦略とコスト転嫁</t>
+        </is>
+      </c>
+      <c r="J466" s="15" t="inlineStr">
+        <is>
+          <t>任天堂</t>
+        </is>
+      </c>
+      <c r="K466" s="15" t="inlineStr">
+        <is>
+          <t>Nintendo Switch 2</t>
+        </is>
+      </c>
+      <c r="L466" s="15" t="inlineStr">
+        <is>
+          <t>ハード, 業績, 海外</t>
+        </is>
+      </c>
+      <c r="M466" s="15" t="inlineStr"/>
+    </row>
+    <row r="467">
+      <c r="A467" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B467" s="15" t="inlineStr">
+        <is>
+          <t>ゲーム</t>
+        </is>
+      </c>
+      <c r="C467" s="15" t="inlineStr">
+        <is>
+          <t>505 Games、『明末：ウツロノハネ』原作者とシリーズ続編の開発・パブリッシング契約</t>
+        </is>
+      </c>
+      <c r="D467" s="15" t="inlineStr">
+        <is>
+          <t>https://gamebiz.jp/news/430191</t>
+        </is>
+      </c>
+      <c r="E467" s="15" t="inlineStr">
+        <is>
+          <t>中国発ソウルライク『明末：ウツロノハネ』のヒットを受け、パブリッシャーの505 Gamesが原作者・夏思源とシリーズ続編の開発・パブリッシング契約を締結。単発ヒットをシリーズIP化し、クリエイターごと囲い込む動き。</t>
+        </is>
+      </c>
+      <c r="F467" s="15" t="inlineStr">
+        <is>
+          <t>505 Gamesは『明末』のクリエイターと続編契約を締結し、単発の話題作を長期フランチャイズへ発展させる意向を明確化した。『黒神話：悟空』以降の“中国発シングルプレイ大作”の商機を、海外パブリッシャーが主導して押さえにいく構図が鮮明。</t>
+        </is>
+      </c>
+      <c r="G467" s="15" t="inlineStr">
+        <is>
+          <t>・単発ヒットの即・続編契約でIPを囲い込み
+・中国発アクションの海外パブリッシングを505が主導
+・クリエイター×パブリッシャーの長期フランチャイズ化</t>
+        </is>
+      </c>
+      <c r="H467" s="15" t="inlineStr">
+        <is>
+          <t>中国発シングルIPの成功例が続き、海外パブリッシャーが有望な中国スタジオ/クリエイターとの独占的続編契約を急ぐ流れが強まる。初弾ヒット直後に続編・派生を確約する契約設計が、クリエイター獲得競争の標準になっていく。</t>
+        </is>
+      </c>
+      <c r="I467" s="15" t="inlineStr">
+        <is>
+          <t>中国発シングルIPの海外パブリッシャー囲い込み</t>
+        </is>
+      </c>
+      <c r="J467" s="15" t="inlineStr">
+        <is>
+          <t>505 Games, Leenzee Games</t>
+        </is>
+      </c>
+      <c r="K467" s="15" t="inlineStr">
+        <is>
+          <t>明末：ウツロノハネ</t>
+        </is>
+      </c>
+      <c r="L467" s="15" t="inlineStr">
+        <is>
+          <t>提携, 海外</t>
+        </is>
+      </c>
+      <c r="M467" s="15" t="inlineStr"/>
+    </row>
+    <row r="468">
+      <c r="A468" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B468" s="15" t="inlineStr">
+        <is>
+          <t>映画</t>
+        </is>
+      </c>
+      <c r="C468" s="15" t="inlineStr">
+        <is>
+          <t>全米脚本家組合(WGA)、パラマウント×WBD統合の差し止めを求め提訴</t>
+        </is>
+      </c>
+      <c r="D468" s="15" t="inlineStr">
+        <is>
+          <t>https://deadline.com/2026/07/wga-sues-over-paramount-warner-bros-discovery-merger-1236982226/</t>
+        </is>
+      </c>
+      <c r="E468" s="15" t="inlineStr">
+        <is>
+          <t>進行中のパラマウントとワーナー・ブラザース・ディスカバリー(WBD)の統合に対し、全米脚本家組合(WGA)が反トラスト上の懸念から差し止めを求めて提訴。統合による発注元(バイヤー)集約が脚本家の交渉力・報酬を毀損すると主張している。</t>
+        </is>
+      </c>
+      <c r="F468" s="15" t="inlineStr">
+        <is>
+          <t>WGAはParamount-WBD統合が制作会社の買い手を減らし、クリエイターの賃金・雇用を圧迫するとして差し止めを求めた。メガ統合の是非が規制当局だけでなく労働組合サイドからも争われる、新しいタイプの障害が表面化した。</t>
+        </is>
+      </c>
+      <c r="G468" s="15" t="inlineStr">
+        <is>
+          <t>・労働組合がM&amp;Aの反トラスト差し止めを提起
+・争点は“バイヤー減少”による発注独占(買い手寡占)
+・統合完了時期(2026 Q3見込み)の不確実性が増大</t>
+        </is>
+      </c>
+      <c r="H468" s="15" t="inlineStr">
+        <is>
+          <t>メディアメガ統合に対し、規制当局・州司法長官に加えて労働組合が反対アクターとして常態化する見込み。買い手集約による報酬圧縮への懸念は、ゲーム(パブリッシャー集約)や音楽(レーベル集約)でも同型の反発を招きうる。統合の長期化はコンテンツ発注の一時停滞につながる。</t>
+        </is>
+      </c>
+      <c r="I468" s="15" t="inlineStr">
+        <is>
+          <t>メディア統合の反トラストと“バイヤー寡占”論</t>
+        </is>
+      </c>
+      <c r="J468" s="15" t="inlineStr">
+        <is>
+          <t>Paramount, Warner Bros. Discovery, WGA</t>
+        </is>
+      </c>
+      <c r="K468" s="15" t="inlineStr"/>
+      <c r="L468" s="15" t="inlineStr">
+        <is>
+          <t>規制, M&amp;A, 海外</t>
+        </is>
+      </c>
+      <c r="M468" s="15" t="inlineStr"/>
+    </row>
+    <row r="469">
+      <c r="A469" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B469" s="15" t="inlineStr">
+        <is>
+          <t>映画</t>
+        </is>
+      </c>
+      <c r="C469" s="15" t="inlineStr">
+        <is>
+          <t>東宝東和、2026年から米ワーナー洋画を配給へ 第1弾はM・ロビー主演『嵐が丘』</t>
+        </is>
+      </c>
+      <c r="D469" s="15" t="inlineStr">
+        <is>
+          <t>https://natalie.mu/eiga/news/640785</t>
+        </is>
+      </c>
+      <c r="E469" s="15" t="inlineStr">
+        <is>
+          <t>邦画シフトが進む日本市場で、東宝東和が米ワーナー・ブラザースの洋画作品を配給する体制へ。第1弾はマーゴット・ロビー主演『嵐が丘』。洋画の国内配給座組が再編され、ハリウッド大作の日本窓口が動く。</t>
+        </is>
+      </c>
+      <c r="F469" s="15" t="inlineStr">
+        <is>
+          <t>東宝東和がワーナー作品の国内配給を担う新体制を発表。洋画不振・邦画優勢が続く日本で、ハリウッドスタジオの国内配給パートナーが見直される動き。洋画の宣伝・興行ノウハウを持つ配給会社の存在価値が改めて問われている。</t>
+        </is>
+      </c>
+      <c r="G469" s="15" t="inlineStr">
+        <is>
+          <t>・ハリウッド作品の日本配給座組の再編
+・洋画不振下での配給パートナー選定の重要性
+・邦画優勢の国内市場で洋画をどう当てるかが課題</t>
+        </is>
+      </c>
+      <c r="H469" s="15" t="inlineStr">
+        <is>
+          <t>洋画の国内興行が縮小する中、スタジオは宣伝力・チェーン交渉力のある現地配給パートナーへの依存を強める。配給会社にとって洋画枠の獲得は収益源になる一方リスクも大きく、“どの洋画を国内で張るか”の目利きが生命線になる。</t>
+        </is>
+      </c>
+      <c r="I469" s="15" t="inlineStr">
+        <is>
+          <t>洋画の国内配給座組再編と現地パートナー戦略</t>
+        </is>
+      </c>
+      <c r="J469" s="15" t="inlineStr">
+        <is>
+          <t>東宝東和, ワーナー・ブラザース</t>
+        </is>
+      </c>
+      <c r="K469" s="15" t="inlineStr">
+        <is>
+          <t>嵐が丘</t>
+        </is>
+      </c>
+      <c r="L469" s="15" t="inlineStr">
+        <is>
+          <t>提携, 権利・ライセンス, 国内</t>
+        </is>
+      </c>
+      <c r="M469" s="15" t="inlineStr"/>
+    </row>
+    <row r="470">
+      <c r="A470" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B470" s="15" t="inlineStr">
+        <is>
+          <t>映画</t>
+        </is>
+      </c>
+      <c r="C470" s="15" t="inlineStr">
+        <is>
+          <t>『トイ・ストーリー5』が洋画スタート新記録、夏興行はファミリー続編IPが牽引</t>
+        </is>
+      </c>
+      <c r="D470" s="15" t="inlineStr">
+        <is>
+          <t>https://www.moviecollection.jp/news/301165/</t>
+        </is>
+      </c>
+      <c r="E470" s="15" t="inlineStr">
+        <is>
+          <t>2026年夏の日本市場で『トイ・ストーリー5』が洋画のスタート記録を更新。『映画ちいかわ』『キングダム』など邦画勢と首位を争い、夏休み興行は“確立された続編・キャラIP”が集客の中心となった。</t>
+        </is>
+      </c>
+      <c r="F470" s="15" t="inlineStr">
+        <is>
+          <t>『トイ・ストーリー5』は数少ない“当たる洋画”としてファミリー続編IPの強さを示した。オリジナルや新規IPが苦戦する中、認知の確立した続編・キャラクターに観客と興収が集中する消費傾向が鮮明で、興行の二極化を裏づける消費者インサイトとなる。</t>
+        </is>
+      </c>
+      <c r="G470" s="15" t="inlineStr">
+        <is>
+          <t>・洋画不振下でもファミリー続編IPは特大初動
+・邦画(ちいかわ/キングダム)と洋画続編が夏興行を分け合う
+・新規IP苦戦・既存IP集中という消費の二極化</t>
+        </is>
+      </c>
+      <c r="H470" s="15" t="inlineStr">
+        <is>
+          <t>劇場に足を運ぶ動機が“確立されたIPの続編・映像化”に一層偏り、スタジオは新規IPより既存フランチャイズ・キャラIPへ投資を集中させる。中長期のIP枯渇リスクが高まり、ゲーム/アニメ/漫画由来のIPを劇場大作へ転用する動きが加速する。</t>
+        </is>
+      </c>
+      <c r="I470" s="15" t="inlineStr">
+        <is>
+          <t>続編・キャラIP集中と新規IP枯渇リスク</t>
+        </is>
+      </c>
+      <c r="J470" s="15" t="inlineStr">
+        <is>
+          <t>Disney, Pixar</t>
+        </is>
+      </c>
+      <c r="K470" s="15" t="inlineStr">
+        <is>
+          <t>トイ・ストーリー5</t>
+        </is>
+      </c>
+      <c r="L470" s="15" t="inlineStr">
+        <is>
+          <t>興行, 消費者インサイト, 海外</t>
+        </is>
+      </c>
+      <c r="M470" s="15" t="inlineStr"/>
+    </row>
+    <row r="471">
+      <c r="A471" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B471" s="15" t="inlineStr">
+        <is>
+          <t>アニメ</t>
+        </is>
+      </c>
+      <c r="C471" s="15" t="inlineStr">
+        <is>
+          <t>IGポート26年5月期は営業益46%減、アニメ制作で受注損失引当金 元請の採算悪化</t>
+        </is>
+      </c>
+      <c r="D471" s="15" t="inlineStr">
+        <is>
+          <t>https://gamebiz.jp/news/429462</t>
+        </is>
+      </c>
+      <c r="E471" s="15" t="inlineStr">
+        <is>
+          <t>Production I.G/WIT STUDIOを傘下に持つIGポートの26年5月期は、出版・版権が好調な一方でアニメ制作の進捗遅れとグッズの想定未達により営業益が前期比46%減。制作事業では受注損失引当金も計上した。</t>
+        </is>
+      </c>
+      <c r="F471" s="15" t="inlineStr">
+        <is>
+          <t>26年5月期は売上140.6億円(-3.7%)、営業益7.66億円(-46.3%)で自社予想を約10億円下回った。アニメ制作(元請)の採算悪化が重荷で、出版・版権は好調。“制作より権利・出版が稼ぐ”収益構造が一段と鮮明になった。</t>
+        </is>
+      </c>
+      <c r="G471" s="15" t="inlineStr">
+        <is>
+          <t>・アニメ制作(元請)で受注損失引当金＝制作単体の採算悪化が表面化
+・出版・版権は好調＝“制作より権利”が稼ぐ構造
+・制作費高騰・スケジュール遅延が上場制作会社の業績を直撃</t>
+        </is>
+      </c>
+      <c r="H471" s="15" t="inlineStr">
+        <is>
+          <t>制作費高騰と納期遅延で“作るほど薄利/赤字”の元請リスクが上場制作会社にも及び、各社は制作受託から版権保有・出資側へ軸足を移す。権利を握れるかで収益力が二極化し、権利を持てない下請けの淘汰・再編が進む可能性が高い。</t>
+        </is>
+      </c>
+      <c r="I471" s="15" t="inlineStr">
+        <is>
+          <t>アニメ元請の採算悪化と権利保有シフト</t>
+        </is>
+      </c>
+      <c r="J471" s="15" t="inlineStr">
+        <is>
+          <t>IGポート, Production I.G, WIT STUDIO</t>
+        </is>
+      </c>
+      <c r="K471" s="15" t="inlineStr"/>
+      <c r="L471" s="15" t="inlineStr">
+        <is>
+          <t>業績, 国内</t>
+        </is>
+      </c>
+      <c r="M471" s="15" t="inlineStr"/>
+    </row>
+    <row r="472">
+      <c r="A472" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B472" s="15" t="inlineStr">
+        <is>
+          <t>アニメ</t>
+        </is>
+      </c>
+      <c r="C472" s="15" t="inlineStr">
+        <is>
+          <t>TVアニメ『あかね噺』第2期“前座修業篇”が2027年1月放送決定</t>
+        </is>
+      </c>
+      <c r="D472" s="15" t="inlineStr">
+        <is>
+          <t>https://natalie.mu/comic/news/677123</t>
+        </is>
+      </c>
+      <c r="E472" s="15" t="inlineStr">
+        <is>
+          <t>週刊少年ジャンプ連載の落語漫画『あかね噺』のTVアニメ第2期制作が決定。テレビ朝日系「IMAnimation」枠で2027年1月放送開始。1期最終話で新キャラを投入し、2期への継続需要を作る構成が取られた。</t>
+        </is>
+      </c>
+      <c r="F472" s="15" t="inlineStr">
+        <is>
+          <t>『あかね噺』2期は朱音が前座として修業する篇を描き、大塚芳忠ら実力派声優が新規参加。ジャンプ発の“落語”という非バトル題材が2期化に至った点で、放送局枠(IMAnimation)によるジャンプIPの中期育成が機能していることを示す。</t>
+        </is>
+      </c>
+      <c r="G472" s="15" t="inlineStr">
+        <is>
+          <t>・ジャンプの非バトル題材(落語)が2期継続＝テーマ多様化の実証
+・テレ朝IMAnimation枠によるジャンプIPの中期育成
+・1期ラストの新キャラ投入で2期需要を設計</t>
+        </is>
+      </c>
+      <c r="H472" s="15" t="inlineStr">
+        <is>
+          <t>バトル一辺倒でないジャンプ作品でもアニメ2期・長期化が成立する事例が増え、出版社×放送局の共同育成枠がIP寿命を延ばす装置として定着する。ニッチ題材のアニメ化成功は原作販促と相互に効き、“作品を切らさず育てる”編成戦略が広がる。</t>
+        </is>
+      </c>
+      <c r="I472" s="15" t="inlineStr">
+        <is>
+          <t>放送局枠による原作IPの中期育成</t>
+        </is>
+      </c>
+      <c r="J472" s="15" t="inlineStr">
+        <is>
+          <t>集英社, テレビ朝日</t>
+        </is>
+      </c>
+      <c r="K472" s="15" t="inlineStr">
+        <is>
+          <t>あかね噺</t>
+        </is>
+      </c>
+      <c r="L472" s="15" t="inlineStr">
+        <is>
+          <t>映像化, 新作, 国内</t>
+        </is>
+      </c>
+      <c r="M472" s="15" t="inlineStr"/>
+    </row>
+    <row r="473">
+      <c r="A473" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B473" s="15" t="inlineStr">
+        <is>
+          <t>アニメ</t>
+        </is>
+      </c>
+      <c r="C473" s="15" t="inlineStr">
+        <is>
+          <t>なろう発『悪党一家の愛娘、転生先も乙女ゲームの極道令嬢でした。』TVアニメ化決定</t>
+        </is>
+      </c>
+      <c r="D473" s="15" t="inlineStr">
+        <is>
+          <t>https://natalie.mu/comic/news/682876</t>
+        </is>
+      </c>
+      <c r="E473" s="15" t="inlineStr">
+        <is>
+          <t>「小説家になろう」発・雨川透子の小説を原作に、轟斗ソラがTOブックス「コロナEX」でコミカライズしている悪役令嬢もの『悪党一家の愛娘〜』のTVアニメ化が決定。なろう→書籍→コミカライズ→アニメの王道メディアミックスをたどる。</t>
+        </is>
+      </c>
+      <c r="F473" s="15" t="inlineStr">
+        <is>
+          <t>本作はネオ・ルネサンス風マフィア世界の悪役令嬢転生譚。原作小説・漫画とも第6巻を8月に発売し、アニメ化発表と刊行・POP UPを連動させた。なろう発の悪役令嬢ジャンルが依然アニメ化パイプラインの主要供給源であることを示す一例。</t>
+        </is>
+      </c>
+      <c r="G473" s="15" t="inlineStr">
+        <is>
+          <t>・なろう→書籍→コミカライズ→アニメの王道メディアミックス
+・悪役令嬢/転生ジャンルが引き続きアニメ化の主力供給源
+・アニメ発表を新刊発売・POP UPと連動させる販促設計</t>
+        </is>
+      </c>
+      <c r="H473" s="15" t="inlineStr">
+        <is>
+          <t>なろう系(特に悪役令嬢・転生)は原作の“検証済み人気”でアニメ化リスクを下げられるため供給が続く。一方で類似作の氾濫による埋没も進み、コミカライズの作画力や配信初速がアニメ化の選抜基準として重みを増す。TOブックス系のIP供給力が要注目。</t>
+        </is>
+      </c>
+      <c r="I473" s="15" t="inlineStr">
+        <is>
+          <t>なろう系IPのメディアミックス選抜基準</t>
+        </is>
+      </c>
+      <c r="J473" s="15" t="inlineStr">
+        <is>
+          <t>TOブックス</t>
+        </is>
+      </c>
+      <c r="K473" s="15" t="inlineStr">
+        <is>
+          <t>悪党一家の愛娘、転生先も乙女ゲームの極道令嬢でした。</t>
+        </is>
+      </c>
+      <c r="L473" s="15" t="inlineStr">
+        <is>
+          <t>映像化, 新作, 国内</t>
+        </is>
+      </c>
+      <c r="M473" s="15" t="inlineStr"/>
+    </row>
+    <row r="474">
+      <c r="A474" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B474" s="15" t="inlineStr">
+        <is>
+          <t>漫画</t>
+        </is>
+      </c>
+      <c r="C474" s="15" t="inlineStr">
+        <is>
+          <t>小学館87期は映像化版権収入+26.8%で増収増益 “二次利用”が出版本体を牽引</t>
+        </is>
+      </c>
+      <c r="D474" s="15" t="inlineStr">
+        <is>
+          <t>https://www.bunkanews.jp/article/424058/</t>
+        </is>
+      </c>
+      <c r="E474" s="15" t="inlineStr">
+        <is>
+          <t>小学館の第87期決算は、コミックの映画・TVアニメ化など映像化に伴う版権収入が大きく伸び増収増益。版権収入等は157.3億円(+26.8%)。紙の販売が細る中、作品を映像・グッズ・海外へ展開する二次利用が本体業績を左右する構造が鮮明になった。</t>
+        </is>
+      </c>
+      <c r="F474" s="15" t="inlineStr">
+        <is>
+          <t>小学館は映像化版権が牽引し増収増益を確保。児童書など紙も一部好調だが、利益の伸びは版権(ライセンス)収入に依存する。出版社の稼ぎ頭が“本を売る”から“IPを貸す・展開する”へ移りつつあることを示す象徴的な数字である。</t>
+        </is>
+      </c>
+      <c r="G474" s="15" t="inlineStr">
+        <is>
+          <t>・映像化版権収入157.3億円(+26.8%)が増益を牽引
+・“本を売る”より“IPを展開する”収益比率が上昇
+・メディアミックスの成否が出版社の業績を直接左右</t>
+        </is>
+      </c>
+      <c r="H474" s="15" t="inlineStr">
+        <is>
+          <t>出版大手は編集・版権部門をIP運用の中核に据え、映像化・ゲーム化・海外ライセンスの内製/出資を拡大する。版権が稼ぐ構造が定着すれば、製作委員会への“参加”から“主導・自社出資”への転換が進み、出版社が映像製作の上流に踏み込む動きが強まる。</t>
+        </is>
+      </c>
+      <c r="I474" s="15" t="inlineStr">
+        <is>
+          <t>出版社の版権収入依存とメディアミックス主導化</t>
+        </is>
+      </c>
+      <c r="J474" s="15" t="inlineStr">
+        <is>
+          <t>小学館</t>
+        </is>
+      </c>
+      <c r="K474" s="15" t="inlineStr"/>
+      <c r="L474" s="15" t="inlineStr">
+        <is>
+          <t>出版, 映像化, 国内</t>
+        </is>
+      </c>
+      <c r="M474" s="15" t="inlineStr"/>
+    </row>
+    <row r="475">
+      <c r="A475" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B475" s="15" t="inlineStr">
+        <is>
+          <t>漫画</t>
+        </is>
+      </c>
+      <c r="C475" s="15" t="inlineStr">
+        <is>
+          <t>縦読み(Webtoon)は国内でピッコマ・LINEマンガが2強、オリジナル制作と海外展開を強化</t>
+        </is>
+      </c>
+      <c r="D475" s="15" t="inlineStr">
+        <is>
+          <t>https://www.nikkei.com/compass/theme/72621</t>
+        </is>
+      </c>
+      <c r="E475" s="15" t="inlineStr">
+        <is>
+          <t>日本の電子漫画市場ではピッコマとLINEマンガが売上上位を独占し、両社ともオリジナルWebtoon(縦スクロール/フルカラー)の制作・配信を強化。従来の“雑誌→単行本”型に対し、スマホ最適化の縦読みがデジタルネイティブ層を取り込みつつある。</t>
+        </is>
+      </c>
+      <c r="F475" s="15" t="inlineStr">
+        <is>
+          <t>ピッコマ・LINEマンガの2強がオリジナルWebtoonの内製と海外・アニメ化を進める。商業誌型IP供給に対し、プラットフォーム主導でIPを生む縦読みモデルが並走。作画分業・スタジオ制作の“作品工場”化が特徴で、既存出版社のIP創出モデルと競合する。</t>
+        </is>
+      </c>
+      <c r="G475" s="15" t="inlineStr">
+        <is>
+          <t>・電子漫画はピッコマ・LINEマンガの2強構造
+・プラットフォームがオリジナルIPを内製＝出版社の競合に
+・縦読みは分業・スタジオ制作で量産、アニメ化も視野</t>
+        </is>
+      </c>
+      <c r="H475" s="15" t="inlineStr">
+        <is>
+          <t>プラットフォーム主導のWebtoonが独自IPをアニメ・実写へ展開し始めると、出版社の“編集発IP”と配信の“PF発IP”がアニメ化枠・映像化予算を奪い合う。縦読み特有の演出をアニメへどう翻案するかが課題となり、Webtoon原作アニメの成否が次の投資を左右する。</t>
+        </is>
+      </c>
+      <c r="I475" s="15" t="inlineStr">
+        <is>
+          <t>PF発Webtoon IPと出版社IPの競合</t>
+        </is>
+      </c>
+      <c r="J475" s="15" t="inlineStr">
+        <is>
+          <t>カカオピッコマ, LINE Digital Frontier</t>
+        </is>
+      </c>
+      <c r="K475" s="15" t="inlineStr"/>
+      <c r="L475" s="15" t="inlineStr">
+        <is>
+          <t>出版, トレンド, 国内</t>
+        </is>
+      </c>
+      <c r="M475" s="15" t="inlineStr"/>
+    </row>
+    <row r="476">
+      <c r="A476" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B476" s="15" t="inlineStr">
+        <is>
+          <t>音楽</t>
+        </is>
+      </c>
+      <c r="C476" s="15" t="inlineStr">
+        <is>
+          <t>HYBE2Qは四半期売上初の1兆ウォン超・営業益過去最高、BTS復帰とツアーが牽引</t>
+        </is>
+      </c>
+      <c r="D476" s="15" t="inlineStr">
+        <is>
+          <t>https://www.rbbtoday.com/article/2026/07/28/251253.html</t>
+        </is>
+      </c>
+      <c r="E476" s="15" t="inlineStr">
+        <is>
+          <t>BTS事務所のHYBEが2026年2Qで四半期売上1.45兆ウォン(初の1兆超)、営業益1709億ウォン(初の1000億超)といずれも過去最高。BTSのカムバックとワールドツアー開始で、公演・MD(物販)・ライセンスの“直接参加型”売上が急伸した。</t>
+        </is>
+      </c>
+      <c r="F476" s="15" t="inlineStr">
+        <is>
+          <t>HYBEの2Qは公演6477億ウォン、音盤・音源3268億ウォン、MD・ライセンス3106億ウォンで、ライブ+物販が音盤・音源を上回った。音源(ストリーミング)より、ライブ体験とグッズ・ファンダム消費が収益の主役になっている構図が明確になった。</t>
+        </is>
+      </c>
+      <c r="G476" s="15" t="inlineStr">
+        <is>
+          <t>・四半期売上初の1兆ウォン超、営業益も過去最高
+・公演・MDが音盤/音源を上回る＝“体験・物販”主導
+・BTS復帰という単一要因への依存も同時に露呈</t>
+        </is>
+      </c>
+      <c r="H476" s="15" t="inlineStr">
+        <is>
+          <t>音楽大手の収益源が録音原盤(ストリーミング分配)から、ライブ・物販・ファンダム運営という“直接参加型(D2F)”へ移る流れが強まる。HYBEはファンプラットフォーム(Weverse)や公演制作の内製を深め、原盤ライセンス中心のUMG/WMGとは異なる垂直統合型モデルを先行して示す。</t>
+        </is>
+      </c>
+      <c r="I476" s="15" t="inlineStr">
+        <is>
+          <t>音楽のD2F(直接参加型)モデルと垂直統合</t>
+        </is>
+      </c>
+      <c r="J476" s="15" t="inlineStr">
+        <is>
+          <t>HYBE</t>
+        </is>
+      </c>
+      <c r="K476" s="15" t="inlineStr">
+        <is>
+          <t>BTS</t>
+        </is>
+      </c>
+      <c r="L476" s="15" t="inlineStr">
+        <is>
+          <t>業績, ライブ・イベント, 海外</t>
+        </is>
+      </c>
+      <c r="M476" s="15" t="inlineStr"/>
+    </row>
+    <row r="477">
+      <c r="A477" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B477" s="15" t="inlineStr">
+        <is>
+          <t>音楽</t>
+        </is>
+      </c>
+      <c r="C477" s="15" t="inlineStr">
+        <is>
+          <t>ライブ・エンタメ市場は2025年8564億円で3年連続過去最高、2035年に1兆円台予測</t>
+        </is>
+      </c>
+      <c r="D477" s="15" t="inlineStr">
+        <is>
+          <t>https://www.nikkei.com/article/DGXZQOUC159PM0V10C26A6000000/</t>
+        </is>
+      </c>
+      <c r="E477" s="15" t="inlineStr">
+        <is>
+          <t>ぴあ総研が2025年のライブ・エンタメ市場を8564億円(前年比+12.6%)と確定値公表し、3年連続で過去最高を更新。音楽が牽引。コロナ後の“体験消費”回帰が続き、2035年には初の1兆円台に達すると予測した。</t>
+        </is>
+      </c>
+      <c r="F477" s="15" t="inlineStr">
+        <is>
+          <t>国内ライブ市場は成長基調で音楽分野が中心。物価・可処分所得の逼迫下でも体験消費は堅調で、CD・配信に対しライブの相対的重要度が高まる。会場供給(アリーナ建設)やチケット単価上昇が今後の成長ドライバー兼制約要因になる。</t>
+        </is>
+      </c>
+      <c r="G477" s="15" t="inlineStr">
+        <is>
+          <t>・2025年8564億円(+12.6%)、3年連続過去最高
+・音楽ライブが市場を牽引＝体験消費の回帰
+・2035年1兆円予測、会場供給と単価が鍵</t>
+        </is>
+      </c>
+      <c r="H477" s="15" t="inlineStr">
+        <is>
+          <t>会場(アリーナ・スタジアム)の新設・稼働がボトルネック兼投資テーマとなり、不動産・興行・鉄道など周辺産業がライブ需要を取り込む。ダイナミックプライシングやVIP化で単価が上がる一方、可処分所得の逼迫と衝突し、“払える層”への高単価集中が進む。</t>
+        </is>
+      </c>
+      <c r="I477" s="15" t="inlineStr">
+        <is>
+          <t>体験消費の拡大と会場供給・単価の制約</t>
+        </is>
+      </c>
+      <c r="J477" s="15" t="inlineStr">
+        <is>
+          <t>ぴあ</t>
+        </is>
+      </c>
+      <c r="K477" s="15" t="inlineStr"/>
+      <c r="L477" s="15" t="inlineStr">
+        <is>
+          <t>ライブ・イベント, トレンド, 国内</t>
+        </is>
+      </c>
+      <c r="M477" s="15" t="inlineStr"/>
+    </row>
+    <row r="478">
+      <c r="A478" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B478" s="15" t="inlineStr">
+        <is>
+          <t>音楽</t>
+        </is>
+      </c>
+      <c r="C478" s="15" t="inlineStr">
+        <is>
+          <t>Mrs. GREEN APPLEがストリーミング首位、“週間1200万再生超”曲数が史上最多に</t>
+        </is>
+      </c>
+      <c r="D478" s="15" t="inlineStr">
+        <is>
+          <t>https://www.billboard-japan.com/d_news/detail/163752/</t>
+        </is>
+      </c>
+      <c r="E478" s="15" t="inlineStr">
+        <is>
+          <t>Billboard JAPANのストリーミング・チャートで、Mrs. GREEN APPLEの新曲がヒットする一方、週間1200万回再生を超える曲の“数”が史上最多を更新。トップ層の再生規模が底上げされ、ストリーミング消費が一部の超ヒットに集中する実態を示す。</t>
+        </is>
+      </c>
+      <c r="F478" s="15" t="inlineStr">
+        <is>
+          <t>上位曲の再生回数インフレが進み、“当たる曲”の再生規模が拡大。ヒットの寡占化(勝者総取り)が数値で裏づけられた。アーティスト側は初週の配信初速とプレイリスト露出への依存を強め、ロングテールよりトップヒット依存の収益構造が鮮明になる。</t>
+        </is>
+      </c>
+      <c r="G478" s="15" t="inlineStr">
+        <is>
+          <t>・週間1200万再生超の曲数が史上最多＝上位の再生規模インフレ
+・ストリーミング消費が超ヒットに集中(勝者総取り)
+・初速・プレイリスト露出への依存が拡大</t>
+        </is>
+      </c>
+      <c r="H478" s="15" t="inlineStr">
+        <is>
+          <t>分配が再生数比例である以上、超ヒットへの集中は上位アーティスト/レーベルへの収益偏在を強める。中小アーティストは配信分配だけでは成立しにくくなり、ライブ・物販・ファンダム課金(D2F)へ活路を求める——HYBE型モデルへの傾斜が中堅にも波及する。</t>
+        </is>
+      </c>
+      <c r="I478" s="15" t="inlineStr">
+        <is>
+          <t>ストリーミングの勝者総取りと分配偏在</t>
+        </is>
+      </c>
+      <c r="J478" s="15" t="inlineStr"/>
+      <c r="K478" s="15" t="inlineStr">
+        <is>
+          <t>Mrs. GREEN APPLE, Brand New</t>
+        </is>
+      </c>
+      <c r="L478" s="15" t="inlineStr">
+        <is>
+          <t>チャート・ランキング, 消費者インサイト, 国内</t>
+        </is>
+      </c>
+      <c r="M478" s="15" t="inlineStr"/>
+    </row>
+    <row r="479">
+      <c r="A479" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B479" s="15" t="inlineStr">
+        <is>
+          <t>音楽</t>
+        </is>
+      </c>
+      <c r="C479" s="15" t="inlineStr">
+        <is>
+          <t>ワーナー・ミュージックはサブスク値上げ寄与で二桁増収、“Streaming 2.0”が収益押し上げ</t>
+        </is>
+      </c>
+      <c r="D479" s="15" t="inlineStr">
+        <is>
+          <t>https://www.investing.com/news/transcripts/earnings-call-transcript-warner-music-q2-2026-beats-eps-and-revenue-estimates-93CH-4687449</t>
+        </is>
+      </c>
+      <c r="E479" s="15" t="inlineStr">
+        <is>
+          <t>WMGの直近四半期は総収入+12%、うち録音音楽のサブスク・ストリーミングが+15%と伸長。ストリーミング各社の値上げ(いわゆるStreaming 2.0)と契約改定がレーベル側の分配を押し上げ、成熟市場でも単価上昇が成長ドライバーになることを示した。</t>
+        </is>
+      </c>
+      <c r="F479" s="15" t="inlineStr">
+        <is>
+          <t>WMGは値上げ寄与でサブスク収入が加速し、営業指標・EPSも改善。加入者数の伸び鈍化を単価(ARPU)上昇で補う“Streaming 2.0”局面に入り、UMGも同様の価格改定効果を報告。DSPの値上げがレーベルの増収に直結する構図が確認された。</t>
+        </is>
+      </c>
+      <c r="G479" s="15" t="inlineStr">
+        <is>
+          <t>・総収入+12%、サブスク・ストリーミング+15%
+・加入者増より単価(値上げ)が成長ドライバー＝Streaming 2.0
+・DSPの値上げがレーベル分配増に直結</t>
+        </is>
+      </c>
+      <c r="H479" s="15" t="inlineStr">
+        <is>
+          <t>ストリーミングの成長軸が“契約者数”から“単価”へ移り、DSPの継続的値上げとレーベル分配改善が当面続く。一方で値上げは解約(チャーン)リスクと隣り合わせで、消費者のサブスク併存から選別への動きと衝突する。単価と離脱のバランスが今後の焦点になる。</t>
+        </is>
+      </c>
+      <c r="I479" s="15" t="inlineStr">
+        <is>
+          <t>Streaming 2.0(単価主導成長)とチャーンの綱引き</t>
+        </is>
+      </c>
+      <c r="J479" s="15" t="inlineStr">
+        <is>
+          <t>ワーナー・ミュージック・グループ, ユニバーサルミュージック, Spotify</t>
+        </is>
+      </c>
+      <c r="K479" s="15" t="inlineStr"/>
+      <c r="L479" s="15" t="inlineStr">
+        <is>
+          <t>業績, 配信, 海外</t>
+        </is>
+      </c>
+      <c r="M479" s="15" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -60677,7 +62010,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -61312,6 +62645,120 @@
       <c r="K11" s="15" t="inlineStr">
         <is>
           <t>単行本8巻発売(7/28)と同時告知。Web発青春ラブコメの映像化。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="inlineStr">
+        <is>
+          <t>あかね噺</t>
+        </is>
+      </c>
+      <c r="C12" s="15" t="inlineStr">
+        <is>
+          <t>漫画</t>
+        </is>
+      </c>
+      <c r="D12" s="15" t="inlineStr">
+        <is>
+          <t>末永裕樹・馬上鷹将(集英社)</t>
+        </is>
+      </c>
+      <c r="E12" s="15" t="inlineStr">
+        <is>
+          <t>アニメ</t>
+        </is>
+      </c>
+      <c r="F12" s="15" t="inlineStr">
+        <is>
+          <t>TVアニメ第2期“前座修業篇”</t>
+        </is>
+      </c>
+      <c r="G12" s="15" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H12" s="15" t="inlineStr">
+        <is>
+          <t>2027-01</t>
+        </is>
+      </c>
+      <c r="I12" s="15" t="inlineStr">
+        <is>
+          <t>制作中</t>
+        </is>
+      </c>
+      <c r="J12" s="15" t="inlineStr">
+        <is>
+          <t>集英社, テレビ朝日</t>
+        </is>
+      </c>
+      <c r="K12" s="15" t="inlineStr">
+        <is>
+          <t>ジャンプ発・落語題材。テレ朝IMAnimation枠。1期新キャラ投入で2期需要を設計。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="inlineStr">
+        <is>
+          <t>悪党一家の愛娘、転生先も乙女ゲームの極道令嬢でした。</t>
+        </is>
+      </c>
+      <c r="C13" s="15" t="inlineStr">
+        <is>
+          <t>小説</t>
+        </is>
+      </c>
+      <c r="D13" s="15" t="inlineStr">
+        <is>
+          <t>雨川透子(TOブックス)</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>アニメ</t>
+        </is>
+      </c>
+      <c r="F13" s="15" t="inlineStr">
+        <is>
+          <t>TVアニメ化</t>
+        </is>
+      </c>
+      <c r="G13" s="15" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="H13" s="15" t="inlineStr">
+        <is>
+          <t>未定</t>
+        </is>
+      </c>
+      <c r="I13" s="15" t="inlineStr">
+        <is>
+          <t>発表</t>
+        </is>
+      </c>
+      <c r="J13" s="15" t="inlineStr">
+        <is>
+          <t>TOブックス</t>
+        </is>
+      </c>
+      <c r="K13" s="15" t="inlineStr">
+        <is>
+          <t>なろう発→コミカライズ(轟斗ソラ・コロナEX)→アニメ。8月に原作/漫画6巻発売。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
weekly-releases(6genres) + indie + rankings update (2026-07-31 18:13)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -10263,7 +10263,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J119"/>
+  <dimension ref="A1:J139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14528,6 +14528,736 @@
       <c r="J119" t="inlineStr">
         <is>
           <t>売上高ベース（Valve公式）。CS2が首位返り咲き</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2026-07-20〜07-26</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C120" t="n">
+        <v>1</v>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>スプラトゥーン レイダース</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Switch 2</t>
+        </is>
+      </c>
+      <c r="F120" t="n">
+        <v>474684</v>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/article/202607/82960</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>任天堂「スプラトゥーン レイダース」が47万本超で初登場首位。マリオカート ワールド累計300万本、トモコレ わくわく生活150万本突破。</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2026-07-20〜07-26</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C121" t="n">
+        <v>2</v>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>リズム天国 ミラクルスターズ</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Switch</t>
+        </is>
+      </c>
+      <c r="F121" t="n">
+        <v>78355</v>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/article/202607/82960</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>任天堂「スプラトゥーン レイダース」が47万本超で初登場首位。マリオカート ワールド累計300万本、トモコレ わくわく生活150万本突破。</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2026-07-20〜07-26</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C122" t="n">
+        <v>3</v>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>トモダチコレクション わくわく生活</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Switch</t>
+        </is>
+      </c>
+      <c r="F122" t="n">
+        <v>23468</v>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/article/202607/82960</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>任天堂「スプラトゥーン レイダース」が47万本超で初登場首位。マリオカート ワールド累計300万本、トモコレ わくわく生活150万本突破。</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2026-07-20〜07-26</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C123" t="n">
+        <v>4</v>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>パワフルプロ野球2026-2027</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Switch</t>
+        </is>
+      </c>
+      <c r="F123" t="n">
+        <v>7227</v>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/article/202607/82960</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>任天堂「スプラトゥーン レイダース」が47万本超で初登場首位。マリオカート ワールド累計300万本、トモコレ わくわく生活150万本突破。</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026-07-20〜07-26</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C124" t="n">
+        <v>5</v>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>マリオカート ワールド</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Switch 2</t>
+        </is>
+      </c>
+      <c r="F124" t="n">
+        <v>6661</v>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/article/202607/82960</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>任天堂「スプラトゥーン レイダース」が47万本超で初登場首位。マリオカート ワールド累計300万本、トモコレ わくわく生活150万本突破。</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026-07-20〜07-26</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C125" t="n">
+        <v>6</v>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>ぽこ あ ポケモン</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Switch 2</t>
+        </is>
+      </c>
+      <c r="F125" t="n">
+        <v>5796</v>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/article/202607/82960</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>任天堂「スプラトゥーン レイダース」が47万本超で初登場首位。マリオカート ワールド累計300万本、トモコレ わくわく生活150万本突破。</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-07-20〜07-26</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C126" t="n">
+        <v>7</v>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>eFootball Kick-Off！</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Switch 2</t>
+        </is>
+      </c>
+      <c r="F126" t="n">
+        <v>5578</v>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/article/202607/82960</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>任天堂「スプラトゥーン レイダース」が47万本超で初登場首位。マリオカート ワールド累計300万本、トモコレ わくわく生活150万本突破。</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-07-20〜07-26</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C127" t="n">
+        <v>8</v>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Minecraft</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Switch</t>
+        </is>
+      </c>
+      <c r="F127" t="n">
+        <v>5106</v>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/article/202607/82960</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>任天堂「スプラトゥーン レイダース」が47万本超で初登場首位。マリオカート ワールド累計300万本、トモコレ わくわく生活150万本突破。</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026-07-20〜07-26</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C128" t="n">
+        <v>9</v>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>がんばれゴエモン大集合！</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Switch</t>
+        </is>
+      </c>
+      <c r="F128" t="n">
+        <v>3961</v>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/article/202607/82960</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>任天堂「スプラトゥーン レイダース」が47万本超で初登場首位。マリオカート ワールド累計300万本、トモコレ わくわく生活150万本突破。</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2026-07-20〜07-26</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>国内ファミ通</t>
+        </is>
+      </c>
+      <c r="C129" t="n">
+        <v>10</v>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>プロ野球スピリッツ2026</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>PS5</t>
+        </is>
+      </c>
+      <c r="F129" t="n">
+        <v>3915</v>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/article/202607/82960</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>任天堂「スプラトゥーン レイダース」が47万本超で初登場首位。マリオカート ワールド累計300万本、トモコレ わくわく生活150万本突破。</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2026-07-20〜07-26</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C130" t="n">
+        <v>1</v>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Counter-Strike 2（カウンターストライク2）</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>https://www.gamegrin.com/news/weekly-top-selling-games-on-steam-20th26th-of-july-2026</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>売上高ベース（Valve公式トップセラー）。CS2が首位継続、Palworld正式版効果で2位に浮上。ハードウェア（Steam Machine/Steam Deck）は除外し上位ゲーム10本を記載。</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2026-07-20〜07-26</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C131" t="n">
+        <v>2</v>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Palworld（パルワールド）</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>https://www.gamegrin.com/news/weekly-top-selling-games-on-steam-20th26th-of-july-2026</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>売上高ベース（Valve公式トップセラー）。CS2が首位継続、Palworld正式版効果で2位に浮上。ハードウェア（Steam Machine/Steam Deck）は除外し上位ゲーム10本を記載。</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2026-07-20〜07-26</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C132" t="n">
+        <v>3</v>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Assassin's Creed Black Flag Resynced（アサシン クリード ブラックフラッグ リシンクド）</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>https://www.gamegrin.com/news/weekly-top-selling-games-on-steam-20th26th-of-july-2026</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>売上高ベース（Valve公式トップセラー）。CS2が首位継続、Palworld正式版効果で2位に浮上。ハードウェア（Steam Machine/Steam Deck）は除外し上位ゲーム10本を記載。</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2026-07-20〜07-26</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C133" t="n">
+        <v>4</v>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Dota 2（ドータ2）</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>https://www.gamegrin.com/news/weekly-top-selling-games-on-steam-20th26th-of-july-2026</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>売上高ベース（Valve公式トップセラー）。CS2が首位継続、Palworld正式版効果で2位に浮上。ハードウェア（Steam Machine/Steam Deck）は除外し上位ゲーム10本を記載。</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2026-07-20〜07-26</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C134" t="n">
+        <v>5</v>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Apex Legends（エーペックスレジェンズ）</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>https://www.gamegrin.com/news/weekly-top-selling-games-on-steam-20th26th-of-july-2026</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>売上高ベース（Valve公式トップセラー）。CS2が首位継続、Palworld正式版効果で2位に浮上。ハードウェア（Steam Machine/Steam Deck）は除外し上位ゲーム10本を記載。</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2026-07-20〜07-26</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C135" t="n">
+        <v>6</v>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>MECCHA CHAMELEON（メチャ・カメレオン）</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>https://www.gamegrin.com/news/weekly-top-selling-games-on-steam-20th26th-of-july-2026</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>売上高ベース（Valve公式トップセラー）。CS2が首位継続、Palworld正式版効果で2位に浮上。ハードウェア（Steam Machine/Steam Deck）は除外し上位ゲーム10本を記載。</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2026-07-20〜07-26</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C136" t="n">
+        <v>7</v>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>PUBG: BATTLEGROUNDS（パブジー）</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>https://www.gamegrin.com/news/weekly-top-selling-games-on-steam-20th26th-of-july-2026</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>売上高ベース（Valve公式トップセラー）。CS2が首位継続、Palworld正式版効果で2位に浮上。ハードウェア（Steam Machine/Steam Deck）は除外し上位ゲーム10本を記載。</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>2026-07-20〜07-26</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C137" t="n">
+        <v>8</v>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Marvel Rivals（マーベル・ライバルズ）</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>https://www.gamegrin.com/news/weekly-top-selling-games-on-steam-20th26th-of-july-2026</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>売上高ベース（Valve公式トップセラー）。CS2が首位継続、Palworld正式版効果で2位に浮上。ハードウェア（Steam Machine/Steam Deck）は除外し上位ゲーム10本を記載。</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>2026-07-20〜07-26</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C138" t="n">
+        <v>9</v>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>EA SPORTS FC 26</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>https://www.gamegrin.com/news/weekly-top-selling-games-on-steam-20th26th-of-july-2026</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>売上高ベース（Valve公式トップセラー）。CS2が首位継続、Palworld正式版効果で2位に浮上。ハードウェア（Steam Machine/Steam Deck）は除外し上位ゲーム10本を記載。</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>2026-07-20〜07-26</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Steamトップセラー</t>
+        </is>
+      </c>
+      <c r="C139" t="n">
+        <v>10</v>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>The Mound: Omen of Cthulhu（ザ・マウンド：オーメン・オブ・クトゥルフ）</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>https://www.gamegrin.com/news/weekly-top-selling-games-on-steam-20th26th-of-july-2026</t>
+        </is>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>売上高ベース（Valve公式トップセラー）。CS2が首位継続、Palworld正式版効果で2位に浮上。ハードウェア（Steam Machine/Steam Deck）は除外し上位ゲーム10本を記載。</t>
         </is>
       </c>
     </row>
@@ -54069,7 +54799,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -54506,6 +55236,93 @@
       <c r="M10" t="inlineStr">
         <is>
           <t>https://cinemore.jp/jp/news-feature/4648/article_p1.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>映画ちいかわ 人魚の島のひみつ</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>東宝</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>日本</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>アニメーション</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>初動3日 22億4000万円／動員150万8500人</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>4</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-07-24〜07-26 国内週末興行1位（初登場）。人気キャラIP初の劇場版が大型初動。興行通信社／映画.com。</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>https://eiga.com/ranking/jp/</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>映画クレヨンしんちゃん 奇々怪々！オラの妖怪バケ〜ション</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>東宝</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>日本</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>アニメーション</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
+        <v>3</v>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-07-31 公開の今週注目作。夏休み定番のクレしん劇場版最新作。</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>https://press.moviewalker.jp/list/upcoming/</t>
         </is>
       </c>
     </row>
@@ -56153,7 +56970,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -56354,6 +57171,56 @@
       <c r="L4" t="inlineStr">
         <is>
           <t>https://www.famitsu.com/article/202607/79761</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>逃げ上手の若君 第二期</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>松井優征（集英社）</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>CloverWorks</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026年夏（7月期・連続2クール）</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>フジテレビ系「ノイタミナ」毎週金23:30／各種配信</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>歴史/アクション</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>4</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>第1期から連続2クールで放送。鎌倉奪還編へ。OPは中島健人「鬼事」。夏アニメの続編注目枠。</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>https://natalie.mu/comic/news/679230</t>
         </is>
       </c>
     </row>
@@ -58519,7 +59386,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M49"/>
+  <dimension ref="A1:M55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -60814,6 +61681,276 @@
       <c r="M49" t="inlineStr">
         <is>
           <t>https://www.4gamer.net/games/918/G091816/20260213002/</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>ゼノブレイド2 Nintendo Switch 2 Edition（Xenoblade2 NS2 Edition）</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>モノリスソフト</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>任天堂</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Nintendo Switch 2 / Nintendo Switch</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>RPG</t>
+        </is>
+      </c>
+      <c r="K50" t="n">
+        <v>4</v>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>今週リリース（DL版・アップグレードパス配信開始／パッケージ版は10/1）。新レアブレイド「M.O.M.O.」（ゼノサーガ）、ホムラ＆ヒカリ新衣装、ブレイドを操作する新モードを追加。DL/パッケージ¥9,778、アップグレードパス¥1,000。</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/article/202607/82817</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>BLUE REFLECTION Quartet: 少女たちのキセキ（BLUE REFLECTION Quartet）</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>ガスト</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>コーエーテクモゲームス</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>PS5 / Switch 2 / Switch / PC(Steam)</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>RPG/アドベンチャー</t>
+        </is>
+      </c>
+      <c r="K51" t="n">
+        <v>3</v>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>今週リリース。ゲーム・TVアニメ・サービス終了済みスマホ作を含む「BLUE REFLECTION」シリーズ全4作を1本に集約。通常版¥7,480（税込）。</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>https://www.nintendo.com/us/store/products/blue-reflection-quartet-switch-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>ファイナルファンタジーXIV（FINAL FANTASY XIV）Nintendo Switch 2版</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>スクウェア・エニックス</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>スクウェア・エニックス</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Nintendo Switch 2</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>MMORPG</t>
+        </is>
+      </c>
+      <c r="K52" t="n">
+        <v>3</v>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>【来週分】人気MMORPGのNintendo Switch 2版が新規プラットフォームとして登場。</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/schedule</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Lies of P: コンプリートエディション（Lies of P: Complete Edition）Nintendo Switch 2版</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>NEOWIZ / Round8 Studio</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>NEOWIZ</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Nintendo Switch 2</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>ソウルライクARPG</t>
+        </is>
+      </c>
+      <c r="K53" t="n">
+        <v>3</v>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>【来週分】ソウルライク人気作＋DLC「Overture」同梱のコンプリート版がNS2に対応。</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/schedule</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>STAR WARS ゼロ・カンパニー（Star Wars Zero Company）</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Bit Reactor / Respawn Entertainment</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>エレクトロニック・アーツ</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>PC / PS5 / Xbox Series X|S</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>ターン制タクティクス</t>
+        </is>
+      </c>
+      <c r="K54" t="n">
+        <v>4</v>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>【来月分】スター・ウォーズ題材のターン制タクティクスRPG。クローン戦争期を舞台にした部隊指揮型。</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/schedule</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>ELDEN RING Tarnished Edition（エルデンリング ターニッシュド・エディション）Nintendo Switch 2版</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>フロム・ソフトウェア</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>バンダイナムコエンターテインメント</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Nintendo Switch 2</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>アクションRPG</t>
+        </is>
+      </c>
+      <c r="K55" t="n">
+        <v>4</v>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>【来月分】「ELDEN RING」＋DLCを収録したNS2向けエディション。携帯機で本編を遊べる注目移植。</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>https://www.famitsu.com/schedule</t>
         </is>
       </c>
     </row>
@@ -63968,7 +65105,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -64166,6 +65303,96 @@
       <c r="K4" t="inlineStr">
         <is>
           <t>https://www.billboard-japan.com/charts/detail?a=hot100</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-07-29（付）</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>チャート</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>是非に及ばず</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>乃木坂46</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>CD/デジタル/ストリーミング複合</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Billboard JAPAN Hot 100 1位</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>4</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>総合ソングチャート首位。オリコン週間シングルでも初週51.0万枚で1位（8/3付）＝41作連続1位。Billboard合算売上75.6万枚。一ノ瀬美空初センターのパンク路線。</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>https://www.oricon.co.jp/news/2470362/full/</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-07-25（付）</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>チャート</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Choosin' Texas</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Ella Langley（エラ・ラングレー）</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>デジタル/ストリーミング</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Billboard Hot 100（米）1位</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>4</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>14週目の全米1位。2026年最長首位曲としてカントリー勢の長期支配が継続。</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>https://www.billboard.com/charts/hot-100/</t>
         </is>
       </c>
     </row>
@@ -69755,7 +70982,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -70568,6 +71795,53 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Funnel Runners（ファンネル・ランナーズ）</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Supernova Studios LLC</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>2026-07-16 早期アクセス配信</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>PC(Steam)</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>物理系オンライン協力/サバイバルホラー</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>発売直後にSteam週間トップセラー（20-26日）へNEWでランクイン。物理挙動を活かした協力プレイでSNS・配信の話題に。</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Steam週間トップセラー入り（20-26日、NEW）</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>個人〜小規模スタジオの物理コメディ系がAAAに混じってトップセラー入り。要ウォッチ。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
daily-news(6genres) + cross-questions + media-mix + predictions update (2026-08-01)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -891,7 +891,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H47"/>
+  <dimension ref="A1:H48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2875,6 +2875,48 @@
       <c r="H47" s="15" t="inlineStr">
         <is>
           <t>横断</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B48" s="15" t="inlineStr">
+        <is>
+          <t>ソニーのPS新作ディスク生産終了(2028)で物理版が消えると、中古ゲーム販売(ゲオ/GameStop)のソフト部門が縮小し、小売はデジタルプリペイド券流通へ軸足を移す。一方でコレクター向け物理版プレス(Limited Run Games等)が独立ビジネスとして拡大し、“プラットフォーマーが握れない物理の希少価値”市場が二極分化する。</t>
+        </is>
+      </c>
+      <c r="C48" s="15" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="D48" s="15" t="inlineStr">
+        <is>
+          <t>2027〜2028年</t>
+        </is>
+      </c>
+      <c r="E48" s="15" t="inlineStr">
+        <is>
+          <t>ソニー(SIE), ゲオ, GameStop, Limited Run Games</t>
+        </is>
+      </c>
+      <c r="F48" s="15" t="inlineStr">
+        <is>
+          <t>「ソニー、PS新作の物理ディスク生産を2028年1月に終了と決算で明言」(GameSpark/GameBusiness.jp・本日)</t>
+        </is>
+      </c>
+      <c r="G48" s="15" t="inlineStr">
+        <is>
+          <t>2027-28年のゲオ/GameStopのソフト中古売上比率の推移と、Limited Run系の受注規模・年間タイトル数が増えるかを観測する。</t>
+        </is>
+      </c>
+      <c r="H48" s="15" t="inlineStr">
+        <is>
+          <t>ゲーム</t>
         </is>
       </c>
     </row>
@@ -5997,7 +6039,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H101"/>
+  <dimension ref="A1:H103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10247,6 +10289,90 @@
         </is>
       </c>
       <c r="H101" s="15" t="inlineStr">
+        <is>
+          <t>横断</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B102" s="15" t="inlineStr">
+        <is>
+          <t>音楽サブスクの成長鈍化(UMGの会員増6.7%)で表面化した『ストリーミング成熟』は、ゲーム(Game Pass/PS Plus)・アニメ配信(Crunchyroll)・電子コミック読み放題でも会員増の頭打ちとして同時に起き、各社が指標を“会員数”から“ARPU/スーパーファン課金”へ移すか？</t>
+        </is>
+      </c>
+      <c r="C102" s="15" t="inlineStr">
+        <is>
+          <t>UMG26年Q2決算(サブスク成長7.9%→6.7%・株価一時25%安)／Crunchyrollのバンドル・ストア上位会員限定化</t>
+        </is>
+      </c>
+      <c r="D102" s="15" t="inlineStr">
+        <is>
+          <t>UMG, ソニー, Crunchyroll, Spotify</t>
+        </is>
+      </c>
+      <c r="E102" s="15" t="inlineStr">
+        <is>
+          <t>動画配信(Netflix), 新聞・雑誌サブスク, SaaS(ネット企業のARPU経営)</t>
+        </is>
+      </c>
+      <c r="F102" s="15" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="G102" s="15" t="inlineStr">
+        <is>
+          <t>エンタメ全ジャンルのサブスクが同時に“会員数の伸び頭打ち→単価/スーパーファン課金へ”という成熟期に入りつつある可能性。</t>
+        </is>
+      </c>
+      <c r="H102" s="15" t="inlineStr">
+        <is>
+          <t>横断</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B103" s="15" t="inlineStr">
+        <is>
+          <t>ソニーのPS新作ディスク生産終了(2028)=物理パッケージ撤退は、映画(4K UHD)・音楽(CD/レコード)・漫画(紙)でも『所有からアクセスへ』の同時圧力として波及し、中古・コレクター・レンタル市場の再編を各ジャンルで引き起こすか？</t>
+        </is>
+      </c>
+      <c r="C103" s="15" t="inlineStr">
+        <is>
+          <t>ソニー26年Q1決算/PS新作の物理ディスク生産を2028年1月に終了と明言(DL比率82%)</t>
+        </is>
+      </c>
+      <c r="D103" s="15" t="inlineStr">
+        <is>
+          <t>ソニー・インタラクティブエンタテインメント</t>
+        </is>
+      </c>
+      <c r="E103" s="15" t="inlineStr">
+        <is>
+          <t>小売(中古: ゲオ・ブックオフ・GameStop), レンタル, 自動車(所有→サブスク)</t>
+        </is>
+      </c>
+      <c r="F103" s="15" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="G103" s="15" t="inlineStr">
+        <is>
+          <t>物理メディア撤退はプラットフォーマーが中古の再販益を消す一方、コレクター向け“物理の希少価値”市場を独立させる二極化を生む可能性。</t>
+        </is>
+      </c>
+      <c r="H103" s="15" t="inlineStr">
         <is>
           <t>横断</t>
         </is>
@@ -20532,7 +20658,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M512"/>
+  <dimension ref="A1:M533"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -54785,6 +54911,1424 @@
       <c r="M512" s="15" t="inlineStr">
         <is>
           <t>機</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B513" s="15" t="inlineStr">
+        <is>
+          <t>ゲーム</t>
+        </is>
+      </c>
+      <c r="C513" s="15" t="inlineStr">
+        <is>
+          <t>ソニーG26年度Q1決算、PS5累計9,530万台・DL比率82%でデジタル化定着</t>
+        </is>
+      </c>
+      <c r="D513" s="15" t="inlineStr">
+        <is>
+          <t>https://www.gamebusiness.jp/article/2026/08/01/27596.html</t>
+        </is>
+      </c>
+      <c r="E513" s="15" t="inlineStr">
+        <is>
+          <t>ソニーGが2026年度第1四半期(4-6月)決算を発表。PS5は当四半期160万台(前年同期250万台から減)で累計9,530万台、1億台が視野に。ハード普及期の終盤に入り、収益源がハード台数からソフト・課金・サブスクへ移る局面。</t>
+        </is>
+      </c>
+      <c r="F513" s="15" t="inlineStr">
+        <is>
+          <t>PS4/PS5ソフトは6,610万本を販売、うちデジタル版比率が82%。ハード販売は前年割れだが、既存インストールベースのソフト・ネットワーク課金が利益を支える構造が鮮明に。ゲーム事業は高採算のデジタル・サービス収益が牽引した。</t>
+        </is>
+      </c>
+      <c r="G513" s="15" t="inlineStr">
+        <is>
+          <t>PS5累計9,530万台で1億台目前、ただしQ1販売は前年割れ
+ソフトのDL版比率82%でパッケージは少数派に
+収益ドライバーがハード台数から既存ユーザーのソフト・課金へシフト
+ハード成熟期の“インストールベース収益化”モデルが前面に</t>
+        </is>
+      </c>
+      <c r="H513" s="15" t="inlineStr">
+        <is>
+          <t>PS5はライフサイクル後半に入り、ハード販売は漸減する一方でMAU・課金・サブスク等のネットワーク収益が事業利益の柱になる。次はPS6投入時期と、インストールベースをどこまでデジタル課金で搾り出せるかが焦点。値下げ・バンドルでの台数追いは限定的に。</t>
+        </is>
+      </c>
+      <c r="I513" s="15" t="inlineStr">
+        <is>
+          <t>据置ハードのライフサイクル後半の収益化(ARPU/課金)</t>
+        </is>
+      </c>
+      <c r="J513" s="15" t="inlineStr">
+        <is>
+          <t>ソニーグループ, ソニー・インタラクティブエンタテインメント</t>
+        </is>
+      </c>
+      <c r="K513" s="15" t="inlineStr">
+        <is>
+          <t>PlayStation 5, PS Plus</t>
+        </is>
+      </c>
+      <c r="L513" s="15" t="inlineStr">
+        <is>
+          <t>業績,適時開示,ハード,配信,国内</t>
+        </is>
+      </c>
+      <c r="M513" s="15" t="inlineStr">
+        <is>
+          <t>Q1(4-6月)決算</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B514" s="15" t="inlineStr">
+        <is>
+          <t>ゲーム</t>
+        </is>
+      </c>
+      <c r="C514" s="15" t="inlineStr">
+        <is>
+          <t>ソニー、PS新作の物理ディスク生産を2028年1月に終了と決算で改めて明言</t>
+        </is>
+      </c>
+      <c r="D514" s="15" t="inlineStr">
+        <is>
+          <t>http://www.gamespark.jp/article/2026/07/31/170014.html</t>
+        </is>
+      </c>
+      <c r="E514" s="15" t="inlineStr">
+        <is>
+          <t>7/1に表明したPS向け新作ゲームの物理ディスク生産終了(2028年1月以降)方針を、Q1決算説明会で改めて説明。DL比率82%という実データを背景に、パッケージ流通からの撤退を正当化した。物理版はゲーム売上の数%まで縮小している。</t>
+        </is>
+      </c>
+      <c r="F514" s="15" t="inlineStr">
+        <is>
+          <t>『所有』を前提としたパッケージ流通の終焉を大手プラットフォーマーが公式に宣言した形。中古・貸与・コレクションといった物理版に紐づく二次流通や消費者の権利の在り方が、業界全体の論点として浮上する。</t>
+        </is>
+      </c>
+      <c r="G514" s="15" t="inlineStr">
+        <is>
+          <t>新作の物理ディスク生産を2028年1月に終了する方針を決算で再確認
+背景はDL比率82%(パッケージは数%まで縮小)
+中古・貸与・コレクター需要など物理版に依存する商流が縮小へ
+“所有からアクセスへ”の不可逆的シフトを最大手が主導</t>
+        </is>
+      </c>
+      <c r="H514" s="15" t="inlineStr">
+        <is>
+          <t>パッケージ消滅は中古販売(ゲオ等)・限定版プレス(Limited Run系)の二極化を招く。小売はデジタルギフト券流通へ、コレクター向けは独立ビジネス化。映画・音楽の物理メディア撤退とも同期し、“所有”の価値を巡る議論が再燃する。</t>
+        </is>
+      </c>
+      <c r="I514" s="15" t="inlineStr">
+        <is>
+          <t>物理メディア撤退と中古・所有権の再編</t>
+        </is>
+      </c>
+      <c r="J514" s="15" t="inlineStr">
+        <is>
+          <t>ソニー・インタラクティブエンタテインメント</t>
+        </is>
+      </c>
+      <c r="K514" s="15" t="inlineStr">
+        <is>
+          <t>PlayStation 5</t>
+        </is>
+      </c>
+      <c r="L514" s="15" t="inlineStr">
+        <is>
+          <t>ハード,配信,消費者インサイト,トレンド,国内</t>
+        </is>
+      </c>
+      <c r="M514" s="15" t="inlineStr">
+        <is>
+          <t>7/1方針を決算で再確認</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B515" s="15" t="inlineStr">
+        <is>
+          <t>ゲーム</t>
+        </is>
+      </c>
+      <c r="C515" s="15" t="inlineStr">
+        <is>
+          <t>EA、サウジPIF主導の約550億ドルLBOが8/4完了へ 史上最大の非公開化</t>
+        </is>
+      </c>
+      <c r="D515" s="15" t="inlineStr">
+        <is>
+          <t>https://automaton-media.com/articles/newsjp/20260731-457484/</t>
+        </is>
+      </c>
+      <c r="E515" s="15" t="inlineStr">
+        <is>
+          <t>サウジPIF・Silver Lake・Affinity Partnersによる約550億ドルでのEA買収が、EUを含む全規制当局の承認を得て2026年8月4日に完了見込み。PIFが約93.4%を握り、EAは37年ぶりに非公開企業へ。史上最大のレバレッジド・バイアウト(LBO)。</t>
+        </is>
+      </c>
+      <c r="F515" s="15" t="inlineStr">
+        <is>
+          <t>公開市場の四半期プレッシャーから外れた大手パブリッシャーが、国家系ファンドの資本下で長期投資・IP強化に舵を切れるかが試される。ゲーム業界の所有構造に“ソブリンウェルス”が本格参入する象徴的案件。</t>
+        </is>
+      </c>
+      <c r="G515" s="15" t="inlineStr">
+        <is>
+          <t>買収額約550億ドルは史上最大のLBO(TXU超え)
+PIF93.4%/Silver Lake5.5%/Affinity1%の出資構成
+全規制承認完了、8/4クローズ予定、CEOはA.ウィルソン続投
+国家系ファンドによるAAAパブリッシャー完全支配の先例に</t>
+        </is>
+      </c>
+      <c r="H515" s="15" t="inlineStr">
+        <is>
+          <t>非公開化後のEAは短期利益より長期IP投資へ傾く可能性。一方で巨額の買収債務(LBO)返済負担がライブサービス課金強化やコスト削減を促す両面。サウジのスポーツ・eスポーツ・ゲーム統合戦略にEA IPが組み込まれる展開も。</t>
+        </is>
+      </c>
+      <c r="I515" s="15" t="inlineStr">
+        <is>
+          <t>ソブリンファンドのゲーム投資とLBO後の経営</t>
+        </is>
+      </c>
+      <c r="J515" s="15" t="inlineStr">
+        <is>
+          <t>Electronic Arts, サウジ公共投資基金(PIF), Silver Lake</t>
+        </is>
+      </c>
+      <c r="K515" s="15" t="inlineStr">
+        <is>
+          <t>EA SPORTS FC, Battlefield, The Sims</t>
+        </is>
+      </c>
+      <c r="L515" s="15" t="inlineStr">
+        <is>
+          <t>M&amp;A,適時開示,海外</t>
+        </is>
+      </c>
+      <c r="M515" s="15" t="inlineStr">
+        <is>
+          <t>史上最大LBO/8/4完了</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B516" s="15" t="inlineStr">
+        <is>
+          <t>映画</t>
+        </is>
+      </c>
+      <c r="C516" s="15" t="inlineStr">
+        <is>
+          <t>Paramount-WB合併、反トラスト裁判の日程で州側と対立 9/30から日額700万ドル負担</t>
+        </is>
+      </c>
+      <c r="D516" s="15" t="inlineStr">
+        <is>
+          <t>https://variety.com/2026/film/news/states-paramount-warner-bros-antitrust-trial-2027-1236825068/</t>
+        </is>
+      </c>
+      <c r="E516" s="15" t="inlineStr">
+        <is>
+          <t>1,110億ドルのParamount SkydanceによるWarner Bros.買収を巡り、州司法長官連合が差止提訴。DOJは承認済みだが州側が競争阻害を主張。Paramountは早期(11月)の裁判を、州・WGAは2027年4月を要求し日程闘争に。</t>
+        </is>
+      </c>
+      <c r="F516" s="15" t="inlineStr">
+        <is>
+          <t>Paramountは9/30以降、取引完了までWB株主へ日額700万ドルを支払う契約で、裁判長期化が財務を直撃する。ハリウッドの寡占化(ワイド公開・トップ興行・ケーブル)を巡る司法判断が、スタジオ再編の分水嶺になる。</t>
+        </is>
+      </c>
+      <c r="G516" s="15" t="inlineStr">
+        <is>
+          <t>州連合が合併差止提訴、DOJ承認済みでも州レベルで係争
+Paramountは11月、州/WGAは2027年4月の裁判日程を要求
+9/30以降は完了まで日額700万ドルをWB株主に支払う契約
+争点はワイド公開・トップ興行・ケーブル配給の3市場の競争</t>
+        </is>
+      </c>
+      <c r="H516" s="15" t="inlineStr">
+        <is>
+          <t>裁判長期化なら日額負担がParamountを圧迫し、独禁クリアのため資産の一部売却を迫られる可能性。非中核事業(ゲーム部門WB Games等)のカーブアウト売却が業界の“出物”になりうる。合併可否は米メディア寡占の許容度を左右する。</t>
+        </is>
+      </c>
+      <c r="I516" s="15" t="inlineStr">
+        <is>
+          <t>メディアメガ合併と反トラスト・資産売却</t>
+        </is>
+      </c>
+      <c r="J516" s="15" t="inlineStr">
+        <is>
+          <t>Paramount Skydance, Warner Bros. Discovery</t>
+        </is>
+      </c>
+      <c r="K516" s="15" t="inlineStr"/>
+      <c r="L516" s="15" t="inlineStr">
+        <is>
+          <t>M&amp;A,規制,興行,海外</t>
+        </is>
+      </c>
+      <c r="M516" s="15" t="inlineStr">
+        <is>
+          <t>7/31/Variety</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B517" s="15" t="inlineStr">
+        <is>
+          <t>映画</t>
+        </is>
+      </c>
+      <c r="C517" s="15" t="inlineStr">
+        <is>
+          <t>2026年の北米興行、パンデミック後初の“年間100億ドル”が視野に 夏が牽引</t>
+        </is>
+      </c>
+      <c r="D517" s="15" t="inlineStr">
+        <is>
+          <t>https://www.cnbc.com/2026/06/27/strong-summer-box-office.html</t>
+        </is>
+      </c>
+      <c r="E517" s="15" t="inlineStr">
+        <is>
+          <t>2026年夏の北米興行が想定を上回る好調で、コロナ以降初となる年間100億ドル超えの可能性が指摘される。大型フランチャイズの復調と観客の劇場回帰が寄与。長らく続いた“興行の地盤沈下”論に反証が出た形。</t>
+        </is>
+      </c>
+      <c r="F517" s="15" t="inlineStr">
+        <is>
+          <t>劇場市場の回復は、配信一辺倒だった各社の窓口戦略(劇場→配信の順序・期間)を再調整させる。劇場での初動が配信価値を底上げする相互補完が意識され、劇場軽視の是正が起きうる。</t>
+        </is>
+      </c>
+      <c r="G517" s="15" t="inlineStr">
+        <is>
+          <t>2026年北米興行が年間100億ドル超えを視野に
+夏場の大型作連発と観客の劇場回帰が牽引
+パンデミック後の“劇場衰退”論に対する反証
+劇場初動が配信価値を高める相互補完への再評価</t>
+        </is>
+      </c>
+      <c r="H517" s="15" t="inlineStr">
+        <is>
+          <t>劇場が“終わった市場”ではないと再認識され、配信直行の見直しと劇場ウィンドウの再確保が進む。ただし回復はトップ数作への集中依存で、公開本数自体は低水準のまま。館数・スクリーン戦略の選択と集中が続く。</t>
+        </is>
+      </c>
+      <c r="I517" s="15" t="inlineStr">
+        <is>
+          <t>劇場市場の回復基調と窓口戦略の再設計</t>
+        </is>
+      </c>
+      <c r="J517" s="15" t="inlineStr">
+        <is>
+          <t>(業界全体)</t>
+        </is>
+      </c>
+      <c r="K517" s="15" t="inlineStr"/>
+      <c r="L517" s="15" t="inlineStr">
+        <is>
+          <t>興行,海外,トレンド</t>
+        </is>
+      </c>
+      <c r="M517" s="15" t="inlineStr">
+        <is>
+          <t>夏興行総括</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B518" s="15" t="inlineStr">
+        <is>
+          <t>映画</t>
+        </is>
+      </c>
+      <c r="C518" s="15" t="inlineStr">
+        <is>
+          <t>劇場版『チェンソーマン レゼ篇』がV5・興収65億円突破、劇場アニメの息の長さを実証</t>
+        </is>
+      </c>
+      <c r="D518" s="15" t="inlineStr">
+        <is>
+          <t>https://press.moviewalker.jp/news/article/1301241/</t>
+        </is>
+      </c>
+      <c r="E518" s="15" t="inlineStr">
+        <is>
+          <t>MAPPA制作の劇場版『チェンソーマン レゼ篇』が週末動員でV5(5週連続首位級)を達成し、興行収入65億円を突破。単発の初動だけでなく、複数週にわたり上位を維持する“ロングラン型”のヒット構造を見せている。</t>
+        </is>
+      </c>
+      <c r="F518" s="15" t="inlineStr">
+        <is>
+          <t>人気漫画原作×劇場アニメが、公開後も動員を積み上げるロングテール型の興行になりうることを示す事例。初週一極集中の実写大作とは異なる、原作ファンダム+口コミで伸びる劇場アニメ特有の収益曲線が読み取れる。</t>
+        </is>
+      </c>
+      <c r="G518" s="15" t="inlineStr">
+        <is>
+          <t>V5(連続上位)達成で興収65億円を突破
+初動一発ではなく複数週で積み上げるロングラン構造
+漫画原作×劇場アニメのファンダム動員力
+『鬼滅』以降続く“劇場アニメが邦画興行の主役”の潮流</t>
+        </is>
+      </c>
+      <c r="H518" s="15" t="inlineStr">
+        <is>
+          <t>劇場アニメが邦画興行の中核を担う構図が定着し、配給・製作委員会は漫画IPの劇場化を最優先の投資対象にする。ロングラン前提の上映計画(館数の段階調整)や配信解禁時期の後ろ倒しが標準化していく。</t>
+        </is>
+      </c>
+      <c r="I518" s="15" t="inlineStr">
+        <is>
+          <t>劇場アニメのロングラン興行と原作ファンダム</t>
+        </is>
+      </c>
+      <c r="J518" s="15" t="inlineStr">
+        <is>
+          <t>MAPPA, 東宝</t>
+        </is>
+      </c>
+      <c r="K518" s="15" t="inlineStr">
+        <is>
+          <t>チェンソーマン</t>
+        </is>
+      </c>
+      <c r="L518" s="15" t="inlineStr">
+        <is>
+          <t>興行,映像化,国内,消費者インサイト</t>
+        </is>
+      </c>
+      <c r="M518" s="15" t="inlineStr">
+        <is>
+          <t>漫画原作劇場アニメ</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B519" s="15" t="inlineStr">
+        <is>
+          <t>映画</t>
+        </is>
+      </c>
+      <c r="C519" s="15" t="inlineStr">
+        <is>
+          <t>人気サッカー漫画『ブルーロック』初の実写映画化が8/7公開、話題作の実写転換相次ぐ</t>
+        </is>
+      </c>
+      <c r="D519" s="15" t="inlineStr">
+        <is>
+          <t>https://www.hmv.co.jp/news/article/220727111/</t>
+        </is>
+      </c>
+      <c r="E519" s="15" t="inlineStr">
+        <is>
+          <t>金城宗幸・ノ村優介の人気漫画『ブルーロック』が初の実写映画化され、2026年8月7日公開予定。アニメ化・ゲーム化に続く実写化で、講談社の主力少年漫画IPをマルチメディアで最大化する流れの一環。</t>
+        </is>
+      </c>
+      <c r="F519" s="15" t="inlineStr">
+        <is>
+          <t>アニメ映画が邦画興行を席巻する一方、漫画原作の“実写”映画化も継続。実写は既存ファン層の外(一般層・海外)へIPを広げる装置として機能し、アニメ実写の使い分け(客層・海外展開)がIP戦略の論点になる。</t>
+        </is>
+      </c>
+      <c r="G519" s="15" t="inlineStr">
+        <is>
+          <t>『ブルーロック』初の実写映画が2026年8月7日公開
+アニメ・ゲームに続く実写化でIPをマルチ展開
+講談社主力少年漫画IPの収益最大化戦略
+アニメ実写の客層・海外展開での使い分けが論点</t>
+        </is>
+      </c>
+      <c r="H519" s="15" t="inlineStr">
+        <is>
+          <t>実写化はアニメと客層・海外訴求が異なるため、講談社等はIPごとにアニメ/実写/ゲームを最適配分する。成功すれば続編・シリーズ化やスポーツIPの海外実写展開が進むが、実写の当たり外れリスクは高くファン反応が鍵。</t>
+        </is>
+      </c>
+      <c r="I519" s="15" t="inlineStr">
+        <is>
+          <t>漫画IPのアニメ/実写使い分けとメディアミックス</t>
+        </is>
+      </c>
+      <c r="J519" s="15" t="inlineStr">
+        <is>
+          <t>講談社, 東宝</t>
+        </is>
+      </c>
+      <c r="K519" s="15" t="inlineStr">
+        <is>
+          <t>ブルーロック</t>
+        </is>
+      </c>
+      <c r="L519" s="15" t="inlineStr">
+        <is>
+          <t>映像化,興行,国内</t>
+        </is>
+      </c>
+      <c r="M519" s="15" t="inlineStr">
+        <is>
+          <t>8/7公開</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B520" s="15" t="inlineStr">
+        <is>
+          <t>アニメ</t>
+        </is>
+      </c>
+      <c r="C520" s="15" t="inlineStr">
+        <is>
+          <t>Crunchyroll、Amazon Prime Video経由でStarzとのバンドルを発表 配信の“束ね直し”進む</t>
+        </is>
+      </c>
+      <c r="D520" s="15" t="inlineStr">
+        <is>
+          <t>https://www.animenewsnetwork.com/news/2026-07-29/crunchyroll-starz-announce-bundle-through-amazon-prime-video-in-u.s/.240085</t>
+        </is>
+      </c>
+      <c r="E520" s="15" t="inlineStr">
+        <is>
+          <t>Sony系のCrunchyrollが、米国でAmazon Prime VideoのチャンネルとしてStarzとのバンドル提供を発表(7/29)。単体サブスクの解約防衛策として、他サービスと束ねて割安に見せる“バンドル回帰”の動き。</t>
+        </is>
+      </c>
+      <c r="F520" s="15" t="inlineStr">
+        <is>
+          <t>サブスク乱立で家計が逼迫する中、単体アニメ配信の会員維持コストが上昇。Crunchyrollは大型プラットフォーム(Amazon)の集客と他ジャンル(Starz映画)との抱き合わせで解約率を抑えにいく。配信の主戦場が“束ね方”競争へ。</t>
+        </is>
+      </c>
+      <c r="G520" s="15" t="inlineStr">
+        <is>
+          <t>CrunchyrollがStarzとバンドル、Amazon Prime Video経由で提供
+単体サブスクの解約防衛=バンドル回帰の典型例
+アニメ専門配信も大型PFの集客・課金インフラに相乗り
+サブスク成熟期の“束ね直し”競争が本格化</t>
+        </is>
+      </c>
+      <c r="H520" s="15" t="inlineStr">
+        <is>
+          <t>アニメ専門配信は単独での会員獲得が鈍化し、大型PFのチャンネル/バンドルに組み込まれる形で生き残る。取次的にAmazon等が課金・解約の主導権を握り、Crunchyrollの交渉力低下と手数料負担増につながる恐れ。</t>
+        </is>
+      </c>
+      <c r="I520" s="15" t="inlineStr">
+        <is>
+          <t>サブスク成熟とバンドル/チャンネル戦略</t>
+        </is>
+      </c>
+      <c r="J520" s="15" t="inlineStr">
+        <is>
+          <t>Crunchyroll, ソニー, Amazon, Starz</t>
+        </is>
+      </c>
+      <c r="K520" s="15" t="inlineStr"/>
+      <c r="L520" s="15" t="inlineStr">
+        <is>
+          <t>配信,提携,海外,トレンド</t>
+        </is>
+      </c>
+      <c r="M520" s="15" t="inlineStr">
+        <is>
+          <t>7/29発表</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B521" s="15" t="inlineStr">
+        <is>
+          <t>アニメ</t>
+        </is>
+      </c>
+      <c r="C521" s="15" t="inlineStr">
+        <is>
+          <t>米アニメ市場は成長持続、Anime Expoでの盛況とCrunchyroll拡大が“ブーム年”を象徴</t>
+        </is>
+      </c>
+      <c r="D521" s="15" t="inlineStr">
+        <is>
+          <t>https://variety.com/2026/tv/news/anime-expo-crunchyroll-boom-witch-hat-atelier-1236801809/</t>
+        </is>
+      </c>
+      <c r="E521" s="15" t="inlineStr">
+        <is>
+          <t>VarietyがAnime Expo(ロサンゼルス)の盛況を取り上げ、2026年が北米アニメにとってブーム年でCrunchyrollが成長スパートにあると報道。海外(特に北米)がアニメ産業の需要ドライバーとして定着した状況を伝える。</t>
+        </is>
+      </c>
+      <c r="F521" s="15" t="inlineStr">
+        <is>
+          <t>アニメの成長は国内より海外配信・興行・イベント・物販が牽引する構図が鮮明。海外需要の拡大は、日本の制作会社に対するサイマル独占権・配信権の争奪と価格上昇を招き、制作側と配信側の力関係を左右する。</t>
+        </is>
+      </c>
+      <c r="G521" s="15" t="inlineStr">
+        <is>
+          <t>Anime Expoが盛況、2026年は北米アニメの“ブーム年”
+Crunchyrollは成長スパート(会員・IP拡大)
+海外配信・興行・イベントが産業の需要ドライバーに
+日本の制作会社を巡る海外配信権の争奪が続く</t>
+        </is>
+      </c>
+      <c r="H521" s="15" t="inlineStr">
+        <is>
+          <t>北米需要の拡大で配信各社のサイマル独占権取得コストが上昇し、日本の制作会社は交渉力を得る一方、上流(製作委員会/PF)への囲い込みも強まる。海外イベント・物販・ライブが日本アニメの新たな高採算収益源として拡大する。</t>
+        </is>
+      </c>
+      <c r="I521" s="15" t="inlineStr">
+        <is>
+          <t>アニメの海外需要と配信権インフレ</t>
+        </is>
+      </c>
+      <c r="J521" s="15" t="inlineStr">
+        <is>
+          <t>Crunchyroll, ソニー</t>
+        </is>
+      </c>
+      <c r="K521" s="15" t="inlineStr"/>
+      <c r="L521" s="15" t="inlineStr">
+        <is>
+          <t>配信,興行,海外,トレンド</t>
+        </is>
+      </c>
+      <c r="M521" s="15" t="inlineStr">
+        <is>
+          <t>Anime Expo総括</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B522" s="15" t="inlineStr">
+        <is>
+          <t>アニメ</t>
+        </is>
+      </c>
+      <c r="C522" s="15" t="inlineStr">
+        <is>
+          <t>『追放された商人は金の力で世界を救う』TVアニメ化決定、同日にコミカライズ始動</t>
+        </is>
+      </c>
+      <c r="D522" s="15" t="inlineStr">
+        <is>
+          <t>https://www.cmoa.jp/comicnews/20260731000000_683138/</t>
+        </is>
+      </c>
+      <c r="E522" s="15" t="inlineStr">
+        <is>
+          <t>駄犬の人気小説『追放された商人は金の力で世界を救う』のTVアニメ化が7/31に決定。発表と同日にコミックPASH!neoで東山千作画のコミカライズ連載も開始。原作→アニメ→コミカライズを“同時多面展開”する典型例。</t>
+        </is>
+      </c>
+      <c r="F522" s="15" t="inlineStr">
+        <is>
+          <t>原作(なろう系小説)発表からアニメ/コミカライズを時間差なく束ねて立ち上げる手法が定着。話題の瞬間最大風速に合わせて複数メディアへ同時投下し、IPの認知と収益機会を一気に立ち上げるメディアミックス設計が読み取れる。</t>
+        </is>
+      </c>
+      <c r="G522" s="15" t="inlineStr">
+        <is>
+          <t>小説原作のTVアニメ化を7/31発表
+同日にコミカライズ連載(コミックPASH!neo)を開始
+アニメ告知×漫画始動を同時投下する多面展開
+なろう系IPの“発表即メディアミックス”運用の典型</t>
+        </is>
+      </c>
+      <c r="H522" s="15" t="inlineStr">
+        <is>
+          <t>なろう系・ライトノベルIPは、アニメ化発表とコミカライズ/グッズ/ゲームを同時始動する運用が標準化。出版社は初速の話題を最大化しつつ、当たれば横展開を即座に加速する。作品供給過多の中で“同時多面展開”が差別化条件に。</t>
+        </is>
+      </c>
+      <c r="I522" s="15" t="inlineStr">
+        <is>
+          <t>なろう系IPの同時多面メディアミックス</t>
+        </is>
+      </c>
+      <c r="J522" s="15" t="inlineStr">
+        <is>
+          <t>PASH!(主婦と生活社)</t>
+        </is>
+      </c>
+      <c r="K522" s="15" t="inlineStr">
+        <is>
+          <t>追放された商人は金の力で世界を救う</t>
+        </is>
+      </c>
+      <c r="L522" s="15" t="inlineStr">
+        <is>
+          <t>映像化,コミカライズ,出版,国内</t>
+        </is>
+      </c>
+      <c r="M522" s="15" t="inlineStr">
+        <is>
+          <t>7/31発表</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B523" s="15" t="inlineStr">
+        <is>
+          <t>アニメ</t>
+        </is>
+      </c>
+      <c r="C523" s="15" t="inlineStr">
+        <is>
+          <t>東宝、アニメ事業を本格拡大フェーズへ 原作獲得と制作体制強化で“年30クール”視野</t>
+        </is>
+      </c>
+      <c r="D523" s="15" t="inlineStr">
+        <is>
+          <t>https://gamebiz.jp/news/424416</t>
+        </is>
+      </c>
+      <c r="E523" s="15" t="inlineStr">
+        <is>
+          <t>東宝がアニメ事業の拡大方針を鮮明化。原作獲得力と制作体制(サイエンスSARU子会社化等)を強化し、将来的に年間30クール規模の製作を視野に入れる。劇場アニメ興行の成功を背景に、上流(原作/制作)への統合投資を加速。</t>
+        </is>
+      </c>
+      <c r="F523" s="15" t="inlineStr">
+        <is>
+          <t>配給・興行に強い東宝が、原作調達〜制作〜劇場/配信までを垂直統合する動き。制作会社の子会社化は、慢性的な制作能力不足と“製作委員会依存からの脱却”を同時に狙うもので、アニメ産業の資本再編を象徴する。</t>
+        </is>
+      </c>
+      <c r="G523" s="15" t="inlineStr">
+        <is>
+          <t>東宝がアニメ事業を本格拡大、年30クール規模を視野
+原作獲得力と制作体制(SARU子会社化等)を強化
+興行の成功を上流(原作/制作)への統合投資に還流
+製作委員会依存からの脱却と垂直統合の潮流</t>
+        </is>
+      </c>
+      <c r="H523" s="15" t="inlineStr">
+        <is>
+          <t>東宝型の垂直統合(原作+制作+配給)が各社に波及し、制作会社の争奪・子会社化が続く。出版社(集英社/講談社/KADOKAWA)も自社出資・内製化で対抗し、製作委員会の主導権がPF・配給・出版のどこに集まるかの綱引きが激化する。</t>
+        </is>
+      </c>
+      <c r="I523" s="15" t="inlineStr">
+        <is>
+          <t>アニメの垂直統合と制作会社の争奪</t>
+        </is>
+      </c>
+      <c r="J523" s="15" t="inlineStr">
+        <is>
+          <t>東宝, サイエンスSARU</t>
+        </is>
+      </c>
+      <c r="K523" s="15" t="inlineStr"/>
+      <c r="L523" s="15" t="inlineStr">
+        <is>
+          <t>出資,映像化,国内,トレンド</t>
+        </is>
+      </c>
+      <c r="M523" s="15" t="inlineStr">
+        <is>
+          <t>事業拡大方針</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B524" s="15" t="inlineStr">
+        <is>
+          <t>漫画</t>
+        </is>
+      </c>
+      <c r="C524" s="15" t="inlineStr">
+        <is>
+          <t>縦読み(Webtoon)が電子コミックの次の主戦場に、LINEマンガ・ピッコマが海外展開を牽引</t>
+        </is>
+      </c>
+      <c r="D524" s="15" t="inlineStr">
+        <is>
+          <t>https://www.businessinsider.jp/article/2512-line-digital-frontier-line-manga-webtoon/</t>
+        </is>
+      </c>
+      <c r="E524" s="15" t="inlineStr">
+        <is>
+          <t>Webtoon(縦スクロール漫画)市場は世界で拡大が続き、日本勢もLINEマンガ・ピッコマがアプリ売上上位を維持。国産webtoonが韓国で1位・1億ビューを突破するなど、日本発の縦読みIPを海外へ出す動きが本格化している。</t>
+        </is>
+      </c>
+      <c r="F524" s="15" t="inlineStr">
+        <is>
+          <t>従来の見開き漫画とは制作・課金(話単位マイクロトランザクション)・データ設計が異なるwebtoonが、電子コミック成熟後の成長ドライバーとして位置づけられる。読者の閲覧・課金挙動データを握るPFが企画の主導権を持つ構造。</t>
+        </is>
+      </c>
+      <c r="G524" s="15" t="inlineStr">
+        <is>
+          <t>Webtoon世界市場が拡大、日本勢はアプリ売上上位を維持
+国産webtoonが韓国で1位・1億ビュー突破
+話単位課金とデータ駆動の企画がPF主導で進む
+見開き漫画とは異なる制作・収益構造が定着</t>
+        </is>
+      </c>
+      <c r="H524" s="15" t="inlineStr">
+        <is>
+          <t>日本の出版社はwebtoonスタジオ内製・原作提供でPFと組む一方、閲覧/課金データを握るPF(LINE/カカオ)との主導権争いが続く。当たったwebtoon IPのアニメ化・実写化・海外展開が、次のメディアミックスの起点になる。</t>
+        </is>
+      </c>
+      <c r="I524" s="15" t="inlineStr">
+        <is>
+          <t>Webtoonのデータ駆動企画とPF主導構造</t>
+        </is>
+      </c>
+      <c r="J524" s="15" t="inlineStr">
+        <is>
+          <t>LINE Digital Frontier, カカオピッコマ</t>
+        </is>
+      </c>
+      <c r="K524" s="15" t="inlineStr"/>
+      <c r="L524" s="15" t="inlineStr">
+        <is>
+          <t>配信,出版,トレンド,海外</t>
+        </is>
+      </c>
+      <c r="M524" s="15" t="inlineStr">
+        <is>
+          <t>市場構造</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B525" s="15" t="inlineStr">
+        <is>
+          <t>小説</t>
+        </is>
+      </c>
+      <c r="C525" s="15" t="inlineStr">
+        <is>
+          <t>2026年上半期の出版市場7,664億円で1.3%減、書籍は健闘も雑誌の縮小続く</t>
+        </is>
+      </c>
+      <c r="D525" s="15" t="inlineStr">
+        <is>
+          <t>https://hon.jp/news/1.0/0/59422</t>
+        </is>
+      </c>
+      <c r="E525" s="15" t="inlineStr">
+        <is>
+          <t>出版科学研究所の上半期集計で紙+電子は7,664億円(-1.3%)。6月単月の紙は前年同月比1.1%増(書籍+2.2%/雑誌-0.4%)と書籍が健闘する一方、雑誌の構造的縮小が続く。文芸・書籍市場は電子と映像化二次収益に支えられる。</t>
+        </is>
+      </c>
+      <c r="F525" s="15" t="inlineStr">
+        <is>
+          <t>小説・書籍単体では大きな成長は望みにくく、収益はヒット作の映像化・電子・海外翻訳といった二次利用に依存する構造。単行本の初速だけでなく、IPとしての横展開余地が作品価値を左右する時代になっている。</t>
+        </is>
+      </c>
+      <c r="G525" s="15" t="inlineStr">
+        <is>
+          <t>上半期市場7,664億円(-1.3%)、6月の紙書籍は+2.2%と健闘
+雑誌は-0.4%で構造的縮小が継続
+書籍・文芸は映像化/電子/翻訳の二次収益に依存
+ヒット小説の“IP化余地”が作品価値を規定</t>
+        </is>
+      </c>
+      <c r="H525" s="15" t="inlineStr">
+        <is>
+          <t>文芸出版社はヒット小説の映像化権・海外翻訳・オーディオブック等の二次利用収益を本業の柱に据える。単体売上の頭打ちを、限定特典・特装版など“所有価値”の付与と、IPライセンス収入の二方向で補う動きが強まる。</t>
+        </is>
+      </c>
+      <c r="I525" s="15" t="inlineStr">
+        <is>
+          <t>書籍市場の二次利用依存とIP化</t>
+        </is>
+      </c>
+      <c r="J525" s="15" t="inlineStr">
+        <is>
+          <t>出版科学研究所</t>
+        </is>
+      </c>
+      <c r="K525" s="15" t="inlineStr"/>
+      <c r="L525" s="15" t="inlineStr">
+        <is>
+          <t>出版,業績,国内,トレンド</t>
+        </is>
+      </c>
+      <c r="M525" s="15" t="inlineStr">
+        <is>
+          <t>上半期市場統計</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B526" s="15" t="inlineStr">
+        <is>
+          <t>小説</t>
+        </is>
+      </c>
+      <c r="C526" s="15" t="inlineStr">
+        <is>
+          <t>住野よるがデビュー10周年書き下ろし『夜想い』、紀伊國屋限定カバーで書店囲い込み</t>
+        </is>
+      </c>
+      <c r="D526" s="15" t="inlineStr">
+        <is>
+          <t>https://store.kinokuniya.co.jp/event/1782799185/</t>
+        </is>
+      </c>
+      <c r="E526" s="15" t="inlineStr">
+        <is>
+          <t>『君の膵臓をたべたい』の住野よるがデビュー10周年書き下ろし長編『夜想い』(双葉社)を刊行。紀伊國屋書店グループ限定カバー版(創業100周年記念)を用意し、特定書店チェーンでの購買を誘導する限定特典商法を採る。</t>
+        </is>
+      </c>
+      <c r="F526" s="15" t="inlineStr">
+        <is>
+          <t>配信・電子・ネット書店に押される実店舗が、限定カバー・特装版といった“ここでしか買えない所有価値”で読者を囲い込む動き。人気作家の話題作を軸に、書店チェーンが差別化と来店動機を作る具体例として示唆的。</t>
+        </is>
+      </c>
+      <c r="G526" s="15" t="inlineStr">
+        <is>
+          <t>住野よる10周年書き下ろし『夜想い』を双葉社が刊行
+紀伊國屋グループ限定カバー版で購買を特定チェーンへ誘導
+実店舗が“限定特典=所有価値”で読者を囲い込み
+人気作家の話題作を来店動機・差別化に活用</t>
+        </is>
+      </c>
+      <c r="H526" s="15" t="inlineStr">
+        <is>
+          <t>限定カバー・特装版・サイン本など書店チェーン別の特典競争が強まり、出版社と大型書店の共同企画が増える。電子・ネット書店に対抗する実店舗の生存戦略として、“体験・所有・限定”を軸にした囲い込みが標準化していく。</t>
+        </is>
+      </c>
+      <c r="I526" s="15" t="inlineStr">
+        <is>
+          <t>実店舗書店の限定特典による囲い込み</t>
+        </is>
+      </c>
+      <c r="J526" s="15" t="inlineStr">
+        <is>
+          <t>双葉社, 紀伊國屋書店</t>
+        </is>
+      </c>
+      <c r="K526" s="15" t="inlineStr">
+        <is>
+          <t>夜想い</t>
+        </is>
+      </c>
+      <c r="L526" s="15" t="inlineStr">
+        <is>
+          <t>出版,消費者インサイト,国内</t>
+        </is>
+      </c>
+      <c r="M526" s="15" t="inlineStr">
+        <is>
+          <t>7/24刊行/限定版</t>
+        </is>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B527" s="15" t="inlineStr">
+        <is>
+          <t>音楽</t>
+        </is>
+      </c>
+      <c r="C527" s="15" t="inlineStr">
+        <is>
+          <t>UMG株が一時25%安、Q2のサブスク成長鈍化(6.7%)で“ストリーミング成熟”懸念が表面化</t>
+        </is>
+      </c>
+      <c r="D527" s="15" t="inlineStr">
+        <is>
+          <t>https://celebrityaccess.com/2026/07/30/universal-music-group-reports-revenue-growth-in-first-half-of-2026</t>
+        </is>
+      </c>
+      <c r="E527" s="15" t="inlineStr">
+        <is>
+          <t>世界最大の音楽会社UMGが2026年Q2決算を発表。売上は32.9億ユーロ(+10.5%)と増収ながら、サブスク収入の伸びが前四半期の7.9%から6.7%へ鈍化。市場は“ストリーミングの成長減速”を嫌気し株価が一時約25%下落した。</t>
+        </is>
+      </c>
+      <c r="F527" s="15" t="inlineStr">
+        <is>
+          <t>配信サブスクの会員増ドライブが先進国で頭打ちに近づいたことを市場が織り込み始めた象徴的な下落。値上げとカタログ買収(Downtown)で増収を作っても、コア指標(サブスク成長率)の減速だけで大きく売られる局面に入った。</t>
+        </is>
+      </c>
+      <c r="G527" s="15" t="inlineStr">
+        <is>
+          <t>Q2売上32.9億ユーロ(+10.5%)も株価は一時約25%安
+サブスク収入の伸びが7.9%→6.7%に鈍化
+値上げ・Downtown買収で増収もコア指標減速を嫌気
+“ストリーミング成熟”を市場が本格的に織り込み始めた</t>
+        </is>
+      </c>
+      <c r="H527" s="15" t="inlineStr">
+        <is>
+          <t>音楽メジャーは会員数の伸びに依存する成長ストーリーから、ARPU向上・スーパーファン課金・ライブ/D2F・AIライセンス等の“単価と新収益”へ物語を切り替える。投資家向け開示KPIもサブスク会員中心から多角指標へ移る可能性。</t>
+        </is>
+      </c>
+      <c r="I527" s="15" t="inlineStr">
+        <is>
+          <t>ストリーミング成熟とサブスク成長の鈍化</t>
+        </is>
+      </c>
+      <c r="J527" s="15" t="inlineStr">
+        <is>
+          <t>ユニバーサル ミュージック(UMG)</t>
+        </is>
+      </c>
+      <c r="K527" s="15" t="inlineStr"/>
+      <c r="L527" s="15" t="inlineStr">
+        <is>
+          <t>業績,配信,海外,トレンド</t>
+        </is>
+      </c>
+      <c r="M527" s="15" t="inlineStr">
+        <is>
+          <t>Q2決算/株価急落</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B528" s="15" t="inlineStr">
+        <is>
+          <t>音楽</t>
+        </is>
+      </c>
+      <c r="C528" s="15" t="inlineStr">
+        <is>
+          <t>UMG、保有Spotify株の約半分を売却し4億ユーロ超を調達 自社株買い(10億ユーロ)に充当</t>
+        </is>
+      </c>
+      <c r="D528" s="15" t="inlineStr">
+        <is>
+          <t>https://963jackfm.com/2026/07/31/universal-music-shares-sink-23-as-subscription-growth-slows/</t>
+        </is>
+      </c>
+      <c r="E528" s="15" t="inlineStr">
+        <is>
+          <t>UMGはQ2決算に合わせ、保有するSpotify株の約半分を売却して4億ユーロ超を調達したと開示。資金は拡大した10億ユーロの自社株買いプログラムに充当。Pandoraとのライセンス更新など配信提携も継続する方針を示した。</t>
+        </is>
+      </c>
+      <c r="F528" s="15" t="inlineStr">
+        <is>
+          <t>レーベルが配信PF(Spotify)の株式という“成長の含み益”を実現益に変え、自社株買いで株主還元へ回す動き。配信の成長鈍化局面で、保有PF株を売って本体価値の防衛(株価下支え)に使う資本政策の転換が読み取れる。</t>
+        </is>
+      </c>
+      <c r="G528" s="15" t="inlineStr">
+        <is>
+          <t>保有Spotify株の約半分を売却、4億ユーロ超を調達
+資金は10億ユーロへ拡大した自社株買いに充当
+Pandoraとのライセンス更新など配信提携は継続
+配信成長鈍化局面での株主還元・株価防衛の資本政策</t>
+        </is>
+      </c>
+      <c r="H528" s="15" t="inlineStr">
+        <is>
+          <t>レーベルはPF株の含み益を還元原資に使いつつ、DSPとの関係を“株主”から“取引パートナー”へ純化させる。今後はAIライセンス・スーパーファン向け商品・直販(D2F)など、配信外の新収益で成長を補う投資配分が焦点になる。</t>
+        </is>
+      </c>
+      <c r="I528" s="15" t="inlineStr">
+        <is>
+          <t>レーベルの資本政策とDSPとの関係再定義</t>
+        </is>
+      </c>
+      <c r="J528" s="15" t="inlineStr">
+        <is>
+          <t>ユニバーサル ミュージック(UMG), Spotify</t>
+        </is>
+      </c>
+      <c r="K528" s="15" t="inlineStr"/>
+      <c r="L528" s="15" t="inlineStr">
+        <is>
+          <t>業績,適時開示,配信,海外</t>
+        </is>
+      </c>
+      <c r="M528" s="15" t="inlineStr">
+        <is>
+          <t>7/31開示</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B529" s="15" t="inlineStr">
+        <is>
+          <t>音楽</t>
+        </is>
+      </c>
+      <c r="C529" s="15" t="inlineStr">
+        <is>
+          <t>メジャー＆インディー連合、AI楽曲のチャート掲載資格で統一枠組みを提案</t>
+        </is>
+      </c>
+      <c r="D529" s="15" t="inlineStr">
+        <is>
+          <t>https://celebrityaccess.com/2026/07/30/majors-and-indies-unite-for-global-ai-music-chart-standards</t>
+        </is>
+      </c>
+      <c r="E529" s="15" t="inlineStr">
+        <is>
+          <t>UMG/Sony/WMGにHYBE・Believe・BMG・Concord等のインディーも加わった連合が、生成AI楽曲の公式チャート掲載資格を巡る統一枠組みを提案(7/30)。BillboardやOfficial Charts等の集計側は未採用で、業界側からの提案段階。</t>
+        </is>
+      </c>
+      <c r="F529" s="15" t="inlineStr">
+        <is>
+          <t>AI生成曲の氾濫に対し、業界が“何をチャートに載せるか”のルールで主導権を握ろうとする動き。ヒットの可視化=チャートを押さえることは、露出・分配・プロモーションの入口を握ることで、AI時代の権利者の交渉力に直結する。</t>
+        </is>
+      </c>
+      <c r="G529" s="15" t="inlineStr">
+        <is>
+          <t>メジャー3社+主要インディーがAI楽曲のチャート資格枠組みを提案
+Billboard等の集計側は現時点で未採用(業界側提案)
+“AIのどの程度までを許容するか”は各社で見解が割れる
+チャート基準=露出・分配の入口を権利者が握る動き</t>
+        </is>
+      </c>
+      <c r="H529" s="15" t="inlineStr">
+        <is>
+          <t>チャート集計側が枠組みを採用すればAI開示曲の掲載可否・分配・露出が制度化され、ディストリビューターがAI混入検査や人手証明を有料オプション化する余地が生まれる。AI楽曲の“格付け”を巡る標準化競争が世界で進む。</t>
+        </is>
+      </c>
+      <c r="I529" s="15" t="inlineStr">
+        <is>
+          <t>AI楽曲のチャート標準化と権利者主導権</t>
+        </is>
+      </c>
+      <c r="J529" s="15" t="inlineStr">
+        <is>
+          <t>UMG, Sony Music, WMG, HYBE</t>
+        </is>
+      </c>
+      <c r="K529" s="15" t="inlineStr"/>
+      <c r="L529" s="15" t="inlineStr">
+        <is>
+          <t>AI,規制,チャート・ランキング,海外</t>
+        </is>
+      </c>
+      <c r="M529" s="15" t="inlineStr">
+        <is>
+          <t>7/30提案</t>
+        </is>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B530" s="15" t="inlineStr">
+        <is>
+          <t>音楽</t>
+        </is>
+      </c>
+      <c r="C530" s="15" t="inlineStr">
+        <is>
+          <t>独ミュンヘン地裁、Suno敗訴 無許諾のAI学習は複製権侵害と初のEU判断</t>
+        </is>
+      </c>
+      <c r="D530" s="15" t="inlineStr">
+        <is>
+          <t>https://variety.com/2026/digital/news/suno-loses-ai-lawsuit-gema-1236825010/</t>
+        </is>
+      </c>
+      <c r="E530" s="15" t="inlineStr">
+        <is>
+          <t>ミュンヘン地裁は7/31、米AI作曲サービスSunoがGEMA管理楽曲を無許諾で学習に使ったのは著作権侵害と判断。モデル内への保存は複製権、出力提供は公衆送信可能化権の侵害と認定。EU圏でのAI学習を巡る画期的判決。</t>
+        </is>
+      </c>
+      <c r="F530" s="15" t="inlineStr">
+        <is>
+          <t>“学習は自由利用”を前提にしてきた生成AI企業に対し、事前ライセンスが必須という司法判断が示された。音楽にとどまらず、アニメ・ゲーム・小説など全コンテンツのAI学習データ調達コストと権利者の交渉力を一変させうる。</t>
+        </is>
+      </c>
+      <c r="G530" s="15" t="inlineStr">
+        <is>
+          <t>ミュンヘン地裁がSuno敗訴、無許諾AI学習を著作権侵害と認定
+モデル保存=複製権、出力提供=公衆送信可能化権の侵害
+GEMA管理6曲の記憶・再生成が証拠として認定
+控訴可能だが損害賠償に向け収益開示を命令</t>
+        </is>
+      </c>
+      <c r="H530" s="15" t="inlineStr">
+        <is>
+          <t>判決が確定・波及すれば、AI各社は学習データの事前ライセンス調達へ移行を迫られ、権利元(レーベル/出版社/製作委員会)がAI学習データ供給の上流に回り込む。無許諾スクレイピング前提のAIサービスは事業モデルの再構築を迫られる。</t>
+        </is>
+      </c>
+      <c r="I530" s="15" t="inlineStr">
+        <is>
+          <t>生成AIの学習データ許諾と著作権判例</t>
+        </is>
+      </c>
+      <c r="J530" s="15" t="inlineStr">
+        <is>
+          <t>Suno, GEMA</t>
+        </is>
+      </c>
+      <c r="K530" s="15" t="inlineStr"/>
+      <c r="L530" s="15" t="inlineStr">
+        <is>
+          <t>AI,規制,権利・ライセンス,海外</t>
+        </is>
+      </c>
+      <c r="M530" s="15" t="inlineStr">
+        <is>
+          <t>7/31判決</t>
+        </is>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B531" s="15" t="inlineStr">
+        <is>
+          <t>音楽</t>
+        </is>
+      </c>
+      <c r="C531" s="15" t="inlineStr">
+        <is>
+          <t>BE:FIRSTが米プロデューサー起用の新曲『BRUCE WAYNE』配信、J-POPのグローバル設計加速</t>
+        </is>
+      </c>
+      <c r="D531" s="15" t="inlineStr">
+        <is>
+          <t>https://natalie.mu/music/news/682688</t>
+        </is>
+      </c>
+      <c r="E531" s="15" t="inlineStr">
+        <is>
+          <t>BMSG所属のBE:FIRSTが、Flo MilliやATL Jacob(米ヒップホップ系)を迎えた新曲『BRUCE WAYNE feat. Flo Milli, ATL Jacob』を7/31配信。国内ファンダム基盤を持つグループが、海外制作陣との共作でグローバル市場を明確に狙う。</t>
+        </is>
+      </c>
+      <c r="F531" s="15" t="inlineStr">
+        <is>
+          <t>J-POP/ボーイズグループが、国内向けの延長ではなく最初から海外市場を意識した制作(海外プロデューサー・英語詞・海外フィーチャリング)を設計する事例。K-POPが確立したグローバル方程式を日本勢が取り込む流れを示す。</t>
+        </is>
+      </c>
+      <c r="G531" s="15" t="inlineStr">
+        <is>
+          <t>BE:FIRSTが米Flo Milli/ATL Jacobを起用した新曲を配信
+国内ファンダム基盤を持つ日本勢のグローバル設計
+K-POP型の“最初から世界標準”制作を取り込む動き
+海外制作陣との共作でストリーミング/海外露出を狙う</t>
+        </is>
+      </c>
+      <c r="H531" s="15" t="inlineStr">
+        <is>
+          <t>日本の事務所・レーベルは海外プロデューサー起用・英語楽曲・海外フェス出演を組み合わせ、K-POP型のグローバル展開を追う。成功例が増えれば、海外A&amp;R投資・現地マーケティングへの資本配分が国内大手でも本格化する。</t>
+        </is>
+      </c>
+      <c r="I531" s="15" t="inlineStr">
+        <is>
+          <t>J-POPのグローバル展開とK-POP型方程式</t>
+        </is>
+      </c>
+      <c r="J531" s="15" t="inlineStr">
+        <is>
+          <t>BMSG, BE:FIRST</t>
+        </is>
+      </c>
+      <c r="K531" s="15" t="inlineStr">
+        <is>
+          <t>BE:FIRST</t>
+        </is>
+      </c>
+      <c r="L531" s="15" t="inlineStr">
+        <is>
+          <t>配信,海外,トレンド</t>
+        </is>
+      </c>
+      <c r="M531" s="15" t="inlineStr">
+        <is>
+          <t>7/31配信</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B532" s="15" t="inlineStr">
+        <is>
+          <t>音楽</t>
+        </is>
+      </c>
+      <c r="C532" s="15" t="inlineStr">
+        <is>
+          <t>エイベックス、S10と提携し海外版権に総額1億ドル投資 グローバル収益基盤を構築</t>
+        </is>
+      </c>
+      <c r="D532" s="15" t="inlineStr">
+        <is>
+          <t>https://www.billboard-japan.com/d_news/detail/150683/2</t>
+        </is>
+      </c>
+      <c r="E532" s="15" t="inlineStr">
+        <is>
+          <t>エイベックスが米S10 Publishing等との提携を通じ、2027年4月末までに総額約1億ドル(約160億円)を投じて海外の音楽著作権・原盤を取得する計画を推進。国内依存から脱し、ストリーミング分配を海外資産で稼ぐ体制へ転換を図る。</t>
+        </is>
+      </c>
+      <c r="F532" s="15" t="inlineStr">
+        <is>
+          <t>国内音楽市場の頭打ちを見据え、日本の音楽企業が海外カタログ(版権)投資でストリーミング収益の地理的分散を進める動き。原盤・出版権という“ストック資産”を海外で積み増し、為替・国内需要に左右されにくい収益基盤を作る戦略。</t>
+        </is>
+      </c>
+      <c r="G532" s="15" t="inlineStr">
+        <is>
+          <t>S10等との提携で海外版権に総額約1億ドルを投資
+2027年4月末までに海外著作権・原盤を取得
+国内依存から海外ストリーミング分配への収益分散
+版権(ストック資産)投資で安定収益基盤を構築</t>
+        </is>
+      </c>
+      <c r="H532" s="15" t="inlineStr">
+        <is>
+          <t>エイベックス等の海外版権投資が成果を出せば、日本の音楽企業も“カタログ投資会社”的な性格を強める。UMG/WMGやファンド(Primary Wave等)との版権争奪が激化し、国内アーティスト育成と海外資産運用の二本柱化が進む。</t>
+        </is>
+      </c>
+      <c r="I532" s="15" t="inlineStr">
+        <is>
+          <t>音楽版権投資と収益の地理的分散</t>
+        </is>
+      </c>
+      <c r="J532" s="15" t="inlineStr">
+        <is>
+          <t>エイベックス, S10 Publishing</t>
+        </is>
+      </c>
+      <c r="K532" s="15" t="inlineStr"/>
+      <c r="L532" s="15" t="inlineStr">
+        <is>
+          <t>出資,権利・ライセンス,海外</t>
+        </is>
+      </c>
+      <c r="M532" s="15" t="inlineStr">
+        <is>
+          <t>海外版権投資</t>
+        </is>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B533" s="15" t="inlineStr">
+        <is>
+          <t>漫画</t>
+        </is>
+      </c>
+      <c r="C533" s="15" t="inlineStr">
+        <is>
+          <t>電子出版市場を新推計、デジタルパブリッシング全体の規模を捉え直す動き</t>
+        </is>
+      </c>
+      <c r="D533" s="15" t="inlineStr">
+        <is>
+          <t>https://hon.jp/news/1.0/0/59443</t>
+        </is>
+      </c>
+      <c r="E533" s="15" t="inlineStr">
+        <is>
+          <t>『電子書籍ビジネス調査報告書2026』などで、電子コミックにとどまらないデジタルパブリッシング・コンテンツ市場全体の規模が新たに推計された(2026年7月の週刊出版ニュース)。電子コミックが牽引してきた市場の定義・範囲を捉え直す局面。</t>
+        </is>
+      </c>
+      <c r="F533" s="15" t="inlineStr">
+        <is>
+          <t>電子コミック単体の伸びが鈍化する中、webtoon・分冊・読み放題・広告収益など多様な収益形態を含めた“デジタルパブリッシング”として市場を再定義する必要が生じている。統計の捉え方自体が業界の成長領域の所在を示す。</t>
+        </is>
+      </c>
+      <c r="G533" s="15" t="inlineStr">
+        <is>
+          <t>デジタルパブリッシング市場を新たに推計する動き
+電子コミック中心の市場定義を広げて捉え直し
+webtoon・読み放題・広告など多様な収益形態を包含
+統計の再定義が次の成長領域(縦読み/海外)を示唆</t>
+        </is>
+      </c>
+      <c r="H533" s="15" t="inlineStr">
+        <is>
+          <t>市場統計が電子コミック偏重からデジタルパブリッシング全体へ広がることで、出版社・PFはwebtoon・読み放題・広告・海外配信を成長領域として明確に投資対象化する。従来の“紙vs電子”の二分法では成長を測れなくなる。</t>
+        </is>
+      </c>
+      <c r="I533" s="15" t="inlineStr">
+        <is>
+          <t>デジタルパブリッシング市場の再定義</t>
+        </is>
+      </c>
+      <c r="J533" s="15" t="inlineStr">
+        <is>
+          <t>インプレス, 出版科学研究所</t>
+        </is>
+      </c>
+      <c r="K533" s="15" t="inlineStr"/>
+      <c r="L533" s="15" t="inlineStr">
+        <is>
+          <t>出版,トレンド,国内</t>
+        </is>
+      </c>
+      <c r="M533" s="15" t="inlineStr">
+        <is>
+          <t>市場推計</t>
         </is>
       </c>
     </row>
@@ -55250,7 +56794,6 @@
           <t>映画ちいかわ 人魚の島のひみつ</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
           <t>東宝</t>
@@ -55296,7 +56839,6 @@
           <t>映画クレヨンしんちゃん 奇々怪々！オラの妖怪バケ〜ション</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
           <t>東宝</t>
@@ -65685,7 +67227,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -66605,6 +68147,177 @@
       <c r="K16" s="15" t="inlineStr">
         <is>
           <t>完結済み旧作の後年アニメ化。旧作カタログの掘り起こし事例</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B17" s="15" t="inlineStr">
+        <is>
+          <t>追放された商人は金の力で世界を救う</t>
+        </is>
+      </c>
+      <c r="C17" s="15" t="inlineStr">
+        <is>
+          <t>小説</t>
+        </is>
+      </c>
+      <c r="D17" s="15" t="inlineStr">
+        <is>
+          <t>駄犬（原作）</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>アニメ</t>
+        </is>
+      </c>
+      <c r="F17" s="15" t="inlineStr">
+        <is>
+          <t>TVアニメ化決定</t>
+        </is>
+      </c>
+      <c r="G17" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="H17" s="15" t="inlineStr">
+        <is>
+          <t>未定</t>
+        </is>
+      </c>
+      <c r="I17" s="15" t="inlineStr">
+        <is>
+          <t>発表</t>
+        </is>
+      </c>
+      <c r="J17" s="15" t="inlineStr">
+        <is>
+          <t>(制作会社未発表)</t>
+        </is>
+      </c>
+      <c r="K17" s="15" t="inlineStr">
+        <is>
+          <t>なろう系小説原作。アニメ化発表と同時にコミカライズも始動する多面展開</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B18" s="15" t="inlineStr">
+        <is>
+          <t>追放された商人は金の力で世界を救う</t>
+        </is>
+      </c>
+      <c r="C18" s="15" t="inlineStr">
+        <is>
+          <t>小説</t>
+        </is>
+      </c>
+      <c r="D18" s="15" t="inlineStr">
+        <is>
+          <t>駄犬（原作）</t>
+        </is>
+      </c>
+      <c r="E18" s="15" t="inlineStr">
+        <is>
+          <t>漫画</t>
+        </is>
+      </c>
+      <c r="F18" s="15" t="inlineStr">
+        <is>
+          <t>コミカライズ連載開始（コミックPASH!neo／作画:東山千）</t>
+        </is>
+      </c>
+      <c r="G18" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="H18" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="I18" s="15" t="inlineStr">
+        <is>
+          <t>公開済（連載開始）</t>
+        </is>
+      </c>
+      <c r="J18" s="15" t="inlineStr">
+        <is>
+          <t>主婦と生活社(PASH!)</t>
+        </is>
+      </c>
+      <c r="K18" s="15" t="inlineStr">
+        <is>
+          <t>アニメ化告知と同日にコミカライズ連載スタート</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B19" s="15" t="inlineStr">
+        <is>
+          <t>ブルーロック</t>
+        </is>
+      </c>
+      <c r="C19" s="15" t="inlineStr">
+        <is>
+          <t>漫画</t>
+        </is>
+      </c>
+      <c r="D19" s="15" t="inlineStr">
+        <is>
+          <t>金城宗幸・ノ村優介／講談社</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="inlineStr">
+        <is>
+          <t>映画</t>
+        </is>
+      </c>
+      <c r="F19" s="15" t="inlineStr">
+        <is>
+          <t>初の実写映画化</t>
+        </is>
+      </c>
+      <c r="G19" s="15" t="inlineStr">
+        <is>
+          <t>(既報)</t>
+        </is>
+      </c>
+      <c r="H19" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="I19" s="15" t="inlineStr">
+        <is>
+          <t>公開間近</t>
+        </is>
+      </c>
+      <c r="J19" s="15" t="inlineStr">
+        <is>
+          <t>東宝, 講談社</t>
+        </is>
+      </c>
+      <c r="K19" s="15" t="inlineStr">
+        <is>
+          <t>アニメ・ゲームに続く実写化。少年漫画IPのマルチメディア最大化</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
monthly matrix(14cat) 2026-07 + future predictions (2026-08-01 09:09)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -891,7 +891,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H48"/>
+  <dimension ref="A1:H50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2915,6 +2915,90 @@
         </is>
       </c>
       <c r="H48" s="15" t="inlineStr">
+        <is>
+          <t>ゲーム</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>AI生成コンテンツの『来歴表示・非AI証明』ゲート化が音楽・小説・漫画・ゲームで同時進行し、UGC投稿／配信プラットフォームが投稿要件・分配条件にAI開示を組み込む横断的コンテンツ・ガバナンスが業界標準化する</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>6〜12ヶ月後(EU AI Act透明性義務8/2起点)</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>TIDAL/Deezer/Bandcamp/Spotify/RIAA/RIAJ/集英社(ジャンプルーキー)/カクヨム・なろう/Steam</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>『TIDAL、100%AI生成曲のロイヤリティ停止を7/15施行』『Deezer、日次アップロードの過半がフルAI生成——不正の85%も』『生成曲の"AIスロップ"懸念でBandcampがAI楽曲を禁止』『投稿サイトでAI小説が受賞・上位席巻、書籍化取消も』『ジャンプ系でAI漫画の炎上続く、ジャンプルーキー規約が未整備』『EU AI Actの透明性義務が8/2適用開始』</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>音楽・小説・漫画・ゲームの4ジャンルで独立にAI排除/開示シグナルが収束(基準a充足)。検証指標=各投稿PF(なろう/カクヨム/ジャンプルーキー)のAI開示・非AI証明の規約化、DSP(Spotify/Deezer/TIDAL)のAI開示曲の分配・露出調整、SteamのAI表記フィルタ拡充を6-12ヶ月で観測。反証=いずれのPFも規約・分配で対応しない場合</t>
+        </is>
+      </c>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t>横断</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>スマホ新法/DMA施行を背景に『アプリ外決済(ウェブ課金)』導入がモバイルゲーム各社の利益率を構造的に押し上げ、Apple/Googleのストア手数料回避が標準化。プラットフォーマーのゲーム手数料収入が侵食され、外部課金前提のマネタイズ設計へ移行が進む</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>6〜12ヶ月後</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>モバイルファクトリー/サイバーエージェント(学マス)/Apple/Google/国内モバイルゲーム各社</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>『モバイルファクトリー2Q増収増益、アプリ外決済導入とストア手数料改定が収益押上げ』『ゲーム4-6月決算シーズン開幕、アプリ外決済が利益構造に定着』(背景:スマホ新法・EU DMAの外部課金解放)</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>規制シグナル(スマホ新法/DMA)と業績シグナル(複数社決算でのアプリ外決済寄与)が収束。検証指標=各社IR資料でのウェブ課金比率・手数料率開示、Apple/Googleのゲーム課金手数料シェア推移を6-12ヶ月で観測。反証=大手がストア内課金に留まりウェブ課金比率が伸びない場合</t>
+        </is>
+      </c>
+      <c r="H50" s="3" t="inlineStr">
         <is>
           <t>ゲーム</t>
         </is>
@@ -5903,20 +5987,117 @@
           <t>7月</t>
         </is>
       </c>
-      <c r="C32" s="9" t="inlineStr"/>
-      <c r="D32" s="9" t="inlineStr"/>
-      <c r="E32" s="9" t="inlineStr"/>
-      <c r="F32" s="9" t="inlineStr"/>
-      <c r="G32" s="9" t="inlineStr"/>
-      <c r="H32" s="9" t="inlineStr"/>
-      <c r="I32" s="9" t="inlineStr"/>
-      <c r="J32" s="9" t="inlineStr"/>
-      <c r="K32" s="9" t="inlineStr"/>
-      <c r="L32" s="9" t="n"/>
-      <c r="M32" s="9" t="n"/>
-      <c r="N32" s="9" t="n"/>
-      <c r="O32" s="9" t="n"/>
-      <c r="P32" s="9" t="n"/>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>・Switch 2が9か月で1,986万台とSwitch超の立ち上がり、9/1に米499.99ドルへ値上げ観測
+・任天堂『スプラトゥーン レイダース』7/23発売、シリーズ初スピンオフ
+・ソニーがPS新作の物理ディスク製造を2028年1月終了、PS5値上げ・販売減速
+・メモリ(DRAM/NAND)不足が長期化しハード値上げ圧力が構造化</t>
+        </is>
+      </c>
+      <c r="D32" s="9" t="inlineStr">
+        <is>
+          <t>・Steam2026上半期売上111億ドルで過去最高、収益の約79%を旧作(バックカタログ)が占める
+・『パルワールド』正式版1.0リリース、Steam同接96万人・累計4,000万人
+・サマーセールで同接過去最高、『サイバーパンク2077』累計4,000万本突破
+・Valve『Steam Machine』が即完売、上半期リリース1.2万本超で供給過多鮮明</t>
+        </is>
+      </c>
+      <c r="E32" s="9" t="inlineStr">
+        <is>
+          <t>・カバー『ホロライブドリームス』が全ストア首位、VTuber IPの課金転換力を実証
+・日本コカ・コーラ×『ポケモンGO』で全国約3万台の自販機がポケストップ化
+・ブシロード『バンドリ！Our Notes』事前登録がグローバル70万件突破
+・『FF14モバイル』中国版9/30終了・グローバル版中止(SE×Tencentライセンス解消)</t>
+        </is>
+      </c>
+      <c r="F32" s="9" t="inlineStr">
+        <is>
+          <t>・Netflix Q2、クラウドゲームがFIFA/Unhinged牽引で最好調デビュー
+・『ワールドダイスター』3年でサービス終了などライブサービス淘汰続く
+・『FF14』Switch2版8/4配信・無料トライアル開始で据置MMOの携帯機拡張</t>
+        </is>
+      </c>
+      <c r="G32" s="9" t="inlineStr">
+        <is>
+          <t>・eスポーツW杯2026がパリで7/6開幕、賞金総額7,500万ドル・7週間24タイトル
+・VALORANT部門は100 ThievesがNRGを3-1で下し優勝(賞金200万ドル)
+・タイトル別視聴に明暗、Apex+74%・Valorant-45.6%でスター/人気チーム依存が鮮明
+・LoL部門はT1が決勝進出、視聴堅調</t>
+        </is>
+      </c>
+      <c r="H32" s="9" t="inlineStr">
+        <is>
+          <t>・2026年Q2のゲームM&amp;Aが23億ドル・54件で2022年以来最高(Scopely×Loom Games 10億ドルが最大)
+・EAの550億ドルLBO(史上最大)がEU承認へ、最終関門は米CFIUS安保審査
+・Tencentが韓国(Shift Up/Krafton/Netmarble)で筆頭級株主に、日本株は売却協議
+・GENDA×SBI資本業務提携、韓国Wemade創業者株が香港ファンドへ9,200億ウォン移転</t>
+        </is>
+      </c>
+      <c r="I32" s="9" t="inlineStr">
+        <is>
+          <t>・EU AI Actの透明性義務が8/2適用開始(高リスク義務はDigital Omnibusで2027年12月へ延期)
+・EUデジタル公正法(DFA)がルートボックス規制へ、PEGI新基準で課金が年齢区分に反映
+・中国、擬人化"人格"AI規制を7/15施行(豆包・千問がAIエージェント機能を停止)
+・任天堂、欧州向けSwitch 2をEU電池規則対応で交換可能バッテリー版へ改訂</t>
+        </is>
+      </c>
+      <c r="J32" s="9" t="inlineStr">
+        <is>
+          <t>・生成AIゲーム市場が2026年に22.1億ドルへ拡大(年23.1%成長)、開発現場のAI活用率は高水準
+・一方で開発者の52%が生成AIを『悪影響』と回答、粗製乱造の"gameslop"問題が焦点
+・元Unreal Engineのベテランが『AIネイティブ』新エンジンを開発、世界生成モデルが主戦場に
+・AI動画生成PixVerseがシリーズC4.39億ドル・評価額20億ドル超でゲームエンジン参入</t>
+        </is>
+      </c>
+      <c r="K32" s="9" t="inlineStr">
+        <is>
+          <t>・Microsoft、Xboxで5スタジオ閉鎖・約3,200人削減(687億ドル買収後の大再編)
+・Compulsion・Double FineがIP保持で独立スピンアウト、米加労組がMSをNLRB提訴
+・Bethesda『Fallout 5』プリプロ入り、TES6と共通の新エンジンCreation Engine 3
+・韓国KRAFTON 2Q営業益67%増で四半期過去最高(Subnautica 2/PUBG牽引)</t>
+        </is>
+      </c>
+      <c r="L32" s="9" t="inlineStr">
+        <is>
+          <t>・ノーラン『オデュッセイア』世界興収6.4億ドル超・北米自己最高で劇場回帰を実証
+・『トイ・ストーリー5』全世界502億円超で洋画スタート新記録
+・『映画ちいかわ』初登場1位・3日で興収22.4億・動員150万、キャラ強IPの劇場化成功
+・パラマウント×WBD1,100億ドル統合が州AG差止提訴で凍結、北米興収YTD54億ドル(+10%)</t>
+        </is>
+      </c>
+      <c r="M32" s="9" t="inlineStr">
+        <is>
+          <t>・『鬼滅の刃』無限城編が世界興収7.9億ドル超で北米歴代外国語映画1位、7/28配信開始
+・アニメ制作費が5年で5割超高騰、元請6割が業績悪化『利益なき繁忙』が鮮明
+・KADOKAWA×アニプレックスが映画配給合弁『Animecc』設立、垂直統合が加速
+・2026夏アニメは続編・レガシー依存が鮮明(BLEACH/無職転生III)、オリジナルは6作のみ</t>
+        </is>
+      </c>
+      <c r="N32" s="9" t="inlineStr">
+        <is>
+          <t>・2025年コミック市場6,925億円で8年ぶり前年割れ(▲1.7%)、電子の伸び鈍化が鮮明
+・集英社が2026年8月に創業100周年(売上2,292億)、講談社も純利益111億で外貨獲得注力
+・小学館87期は映像化版権収入+26.8%で増収増益、"二次利用"が出版本体を牽引
+・ジャンプ系でAI漫画の炎上続く、ジャンプルーキー規約が未整備</t>
+        </is>
+      </c>
+      <c r="O32" s="9" t="inlineStr">
+        <is>
+          <t>・第175回芥川賞は小砂川チト『ゾンビ回収婦』、直木賞は朝倉かすみ『けんぐゎい』
+・本屋大賞は朝井リョウ『イン・ザ・メガチャーチ』、書店員票が販売を牽引
+・文芸市場の半分が『ウェブ発』書籍に、なろう系の主流化と構造転換
+・投稿サイトでAI小説が受賞・上位席巻し書籍化取消も、発見性と信頼の危機</t>
+        </is>
+      </c>
+      <c r="P32" s="9" t="inlineStr">
+        <is>
+          <t>・HYBE2Qが四半期売上初の1兆ウォン超・営業益過去最高(BTS復帰・ツアー牽引)
+・Spotify×UMGが生成AIカバー/リミックスのライセンス契約、AI収益モデルを構築
+・TIDAL/Deezer/BandcampがAI生成曲を停止・禁止、RIAA/RIAJがAIラベル表示提案
+・ライブ市場2025年8,564億円で3年連続過去最高、Apple One値上げ¥1,980→¥2,500(+26%)</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="56" customHeight="1">
       <c r="A33" s="12" t="inlineStr"/>

</xml_diff>

<commit_message>
weekly-companies(6genres) + works watch update (2026-08-03 21:21)
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -20338,17 +20338,17 @@
       </c>
       <c r="I3" s="9" t="inlineStr">
         <is>
-          <t>12州＋WGAの訴訟でクロージング遅延リスク。仮処分が出れば最大14日×2回のディール停止。業績自体も減収・損失見通し</t>
+          <t>12州の反トラスト提訴でParamountとの合併が一時差し止め(TRO)。合併完了は反トラスト裁判後にずれ込み不透明。</t>
         </is>
       </c>
       <c r="J3" s="9" t="inlineStr">
         <is>
-          <t>9月末クロージング目標を守れるか。EU当局の判断と、州レベル訴訟の仮処分の可否</t>
+          <t>反トラスト裁判の帰趨、合併不成立時のスタンドアロン戦略、HBO Max加入者拡大、ticking fee(四半期25¢/株)の受取</t>
         </is>
       </c>
       <c r="K3" s="9" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-08-03</t>
         </is>
       </c>
     </row>
@@ -20391,17 +20391,17 @@
       </c>
       <c r="I4" s="9" t="inlineStr">
         <is>
-          <t>12州＋WGAの提訴により法務コストとスケジュールの不確実性が拡大</t>
+          <t>WBD買収(約1,110億ドル)が12州の反トラストTROで一時停止。完了は反トラスト裁判後or2027年6月まで延期。9/30以降は日額約700万ドルのticking fee負担。</t>
         </is>
       </c>
       <c r="J4" s="9" t="inlineStr">
         <is>
-          <t>EU承認の取得時期。統合後のParamount+とHBO Maxのブランド統廃合方針</t>
+          <t>反トラスト裁判の勝敗、合併シナジーの実現可否、Skydance統合後のコンテンツ戦略</t>
         </is>
       </c>
       <c r="K4" s="9" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-08-03</t>
         </is>
       </c>
     </row>
@@ -67333,13 +67333,13 @@
       </c>
       <c r="G9" s="9" t="inlineStr">
         <is>
-          <t>完全体での活動を再開し新譜・ワールドツアーを準備。FIFAハーフタイム出演発表がHYBE株の材料に。</t>
+          <t>完全体での『Arirang』ワールドツアーが本格化し、HYBEのQ2過去最高業績を牽引。</t>
         </is>
       </c>
       <c r="H9" s="9" t="inlineStr"/>
       <c r="I9" s="9" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-08-03</t>
         </is>
       </c>
     </row>
@@ -67785,7 +67785,7 @@
       <c r="E2" s="9" t="inlineStr"/>
       <c r="F2" s="9" t="inlineStr">
         <is>
-          <t>Q1売上約29億ユーロ(+8.1%)。保有するSpotify株の50%を約64億ドルでBill Ackman主導グループへ売却する方針。次回決算は7/30発表予定。出典: Music Ally/Inc 2026/7</t>
+          <t>Q2 2026: 総収益32.9億ユーロ(+10.5%)、レコーデッド・ミュージック25.16億ユーロ(定通貨+16.2%)。BTS、Olivia Rodrigo、Noah Kahan、Drake等が牽引。保有Spotify株の一部売却を公表しキャッシュ化。</t>
         </is>
       </c>
       <c r="G2" s="9" t="inlineStr">
@@ -67795,22 +67795,22 @@
       </c>
       <c r="H2" s="9" t="inlineStr">
         <is>
-          <t>株主還元の強化と、Spotify株売却によるキャッシュ創出。ストリーミング単価引き上げ交渉で主導権</t>
+          <t>ストリーミング成長の継続、強力なアーティスト陣、Spotify株売却によるキャッシュ化</t>
         </is>
       </c>
       <c r="I2" s="9" t="inlineStr">
         <is>
-          <t>Spotify株売却は同社の成長見通しに対する慎重姿勢とも読める</t>
+          <t>サブスク成熟化の兆し、為替影響、フィジカル鈍化</t>
         </is>
       </c>
       <c r="J2" s="9" t="inlineStr">
         <is>
-          <t>売却資金の使途（M&amp;Aか還元か）。ストリーミング「アーティスト・セントリック」モデルの浸透</t>
+          <t>スーパープレミアム課金の浸透、Downtown買収の統合、AI音楽への対応</t>
         </is>
       </c>
       <c r="K2" s="9" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-08-03</t>
         </is>
       </c>
     </row>
@@ -68001,7 +68001,7 @@
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>BTS完全体の活動再開でQ2は四半期過去最高益が期待される一方、株価はYTD-39.88%と低迷。BTS光化門コンサート後の反動と資金のAI半導体シフトが重し。BTSのFIFAハーフタイム出演発表で一時反発。出典: BigGo/Seoul Economic Daily 2026/7</t>
+          <t>Q2 2026(7/28発表)は売上1.45兆ウォン、営業益1,709億ウォン(利益率11.8%)といずれも過去最高。BTS完全体の『Arirang』ワールドツアーが本格寄与、新人Quartus・Katseyeも躍進。Weverse MAUは1,443万で過去最高。</t>
         </is>
       </c>
       <c r="G6" s="9" t="inlineStr">
@@ -68011,22 +68011,22 @@
       </c>
       <c r="H6" s="9" t="inlineStr">
         <is>
-          <t>BTS完全体復帰・ワールドツアー、多世代アーティスト擁する事業基盤</t>
+          <t>BTS完全体の復帰とワールドツアー、新人IPの多層化、Weverseのエンゲージ拡大</t>
         </is>
       </c>
       <c r="I6" s="9" t="inlineStr">
         <is>
-          <t>イベント後の反動安、業種バリュエーション圧縮で目標株価引下げ相次ぐ</t>
+          <t>特定アーティスト依存、K-POP競争激化、レーベル間ガバナンス課題</t>
         </is>
       </c>
       <c r="J6" s="9" t="inlineStr">
         <is>
-          <t>BTS完全体ツアーの規模と収益。新人グループのIP育成スピード</t>
+          <t>BTSツアーの通期寄与、新人ローンチの成功持続、米国事業(country music等)の拡大</t>
         </is>
       </c>
       <c r="K6" s="9" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-08-03</t>
         </is>
       </c>
     </row>
@@ -70540,7 +70540,7 @@
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>MHワイルズ大型拡張『Ascendance』と新作(2027)発表に続き、関連IP『鬼武者 Way of the Sword』(9/25)体験版が好評。シリーズのSwitch 2展開も進む。</t>
+          <t>カプコン27.3期1Qでカタログ(旧作)販売が堅調に業績へ寄与。ワイルズ後もシリーズが収益を下支え。</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
@@ -70557,7 +70557,7 @@
       <c r="H11" s="9" t="inlineStr"/>
       <c r="I11" s="9" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-08-03</t>
         </is>
       </c>
     </row>
@@ -70684,12 +70684,12 @@
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>Steamサマーセール(6/26〜7/10)で『MGSΔ SNAKE EATER』が40%オフとなり話題化。オンラインモード『Fox Hunt』搭載済。</t>
+          <t>リメイク『MGS Δ』に続く『MGS Δ Vol.2』を27.3期2Q(2026年下期)に発売予定とコナミが明示。</t>
         </is>
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>8月に『METAL GEAR SOLID: MASTER COLLECTION Vol.2』をグローバル発売予定。</t>
+          <t>MGS Δ Vol.2 (2026年下期予定)</t>
         </is>
       </c>
       <c r="F15" s="9" t="inlineStr"/>
@@ -70701,7 +70701,7 @@
       <c r="H15" s="9" t="inlineStr"/>
       <c r="I15" s="9" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-08-03</t>
         </is>
       </c>
     </row>
@@ -70723,7 +70723,7 @@
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>『実況パワフルプロ野球2026-2027』を国内展開。Switch/PS4向け。</t>
+          <t>『実況パワフルプロ野球2026-2027』を発売、コナミ1Q業績に寄与。eBASEBALL関連も継続。</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -70740,7 +70740,7 @@
       <c r="H16" s="9" t="inlineStr"/>
       <c r="I16" s="9" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-08-03</t>
         </is>
       </c>
     </row>
@@ -71170,12 +71170,12 @@
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>Take-TwoがGTA VIを11/19発売と正式確定（標準79.99ドル/アルティメット99.99ドル）。FY27の最大増益ドライバー。</t>
+          <t>GTA VIは6/25に予約開始、発売は2026年11月19日を維持。Take-Twoが8/7の1Q決算で初の予約データ開示予定。</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>『GTA VI』2026/11/19 PS5/Xbox Series X|S</t>
+          <t>GTA VI 2026/11/19発売予定</t>
         </is>
       </c>
       <c r="F29" s="9" t="inlineStr"/>
@@ -71187,7 +71187,7 @@
       <c r="H29" s="9" t="inlineStr"/>
       <c r="I29" s="9" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-08-03</t>
         </is>
       </c>
     </row>
@@ -71941,7 +71941,7 @@
       </c>
       <c r="D54" s="9" t="inlineStr">
         <is>
-          <t>AI活用のクリエイション機能を発表（7/17）。第2四半期決算は7/30引け後。BofAが目標株価を54ドルへ引上げ。</t>
+          <t>Q2 2026は売上14.7億ドル(+36%)、DAU1.23億。ブッキング減速で株価は下落。</t>
         </is>
       </c>
       <c r="E54" s="9" t="inlineStr">
@@ -71958,7 +71958,7 @@
       <c r="H54" s="9" t="inlineStr"/>
       <c r="I54" s="9" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-08-03</t>
         </is>
       </c>
     </row>
@@ -72307,29 +72307,27 @@
       </c>
       <c r="M3" s="9" t="inlineStr">
         <is>
-          <t>【7/27週】PlayStationを2028年1月から新作フルデジタル配信に一本化し、物理ディスク新作を段階終了、PS3/PS Vitaオンラインストアも順次閉鎖と発表。高マージンのデジタル/継続課金シフトを好感し株価は週間+6.77%、約1,275億円の自社株買いも完了。一方でファンは反発（署名10万筆・€4億訴訟報道）、総会長・十時CEOら経営陣が7/3に保有株を大量売却（十時氏は保有の約56.5%）した点は懸念。出典: Simply Wall St/Yahoo Finance 2026/7
----（前回までの記載）---
-『GTAⅥ』が11/19にPS5/Xbox向けで発売(標準$79.99/アルティメット$99.99)と価格が確定し、PS5エンゲージメント/ネットワーク収入拡大への期待が改めて意識される。FY25は全社売上・営業益とも過去最高を更新済で、大型新規開示は乏しく好業績持続力を見極める局面。</t>
+          <t>26/7/31発表のFY2026 1Q(4-6月)は売上2.84兆円(+8%)、営業益4,765億円(+40%)といずれも第1四半期で過去最高。ゲーム(G&amp;NS)は売上9,371億円・営業益2,020億円(+37%)と過去最高益。通期営業益見通しを1.6兆→1.72兆円、売上を12.5兆円へ上方修正。PSN月間アクティブは1.25億アカウント。</t>
         </is>
       </c>
       <c r="N3" s="9" t="inlineStr">
         <is>
-          <t>デジタル一本化で高マージン化、全社最高業績、GTAⅥ商戦でのPS5牽引期待、自社株買い</t>
+          <t>ゲーム過去最高益と通期上方修正、PS5後半戦とライブサービス好調、為替追い風</t>
         </is>
       </c>
       <c r="O3" s="9" t="inlineStr">
         <is>
-          <t>物理販売終了へのファン反発（訴訟・署名）、経営陣の大量株式売却、ハード成熟</t>
+          <t>利益改善は為替寄与が大きい、据置ハードは成熟期、映画・半導体で不透明感</t>
         </is>
       </c>
       <c r="P3" s="9" t="inlineStr">
         <is>
-          <t>デジタル移行の収益寄与とユーザー離反リスクの見極め、GTAⅥ商戦、ネットワークサービス拡大</t>
+          <t>次世代プラットフォームへの投資、PSNアクティブ拡大、金融事業分離後の資本効率</t>
         </is>
       </c>
       <c r="Q3" s="9" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-08-03</t>
         </is>
       </c>
     </row>
@@ -72364,29 +72362,27 @@
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>【7/17】カプコンも大きく水準を切り上げ、任天堂とともに買われた。7/17の東京市場は日経平均が前日比2,694.42円安の64,141.12円と大幅続落し、3連休前にAI・半導体関連の利益確定売りが先行。一方で半導体・メモリー市況の落ち着き期待から「非AI」の内需・バリューへ循環物色が向かい、家庭用ゲーム大手が逆行高。gamebiz集計ではゲーム・エンタメ96銘柄中、上昇26(27%)・下落64(67%)と全体は軟調な中での選別買い。出典: gamebiz 2026/7/17
----（前回までの記載）---
-『鬼武者 Way of the Sword』発売日9/4前倒し発表(7/2)を受け株価は一時+8.4%高の3,272円まで上昇。13期連続営業増益・売上/営業益とも過去最高で好調継続。強力IPのリピート販売とデジタル比率上昇が寄与し、年内の新作寄与への期待が高まる。</t>
+          <t>27.3期1Q(4-6月)は売上704億円(+54.7%)、営業益416.5億円(+66.9%)、経常益414億円(+81.1%)と大幅増益。新規IP『Pragmata』が牽引しデジタルコンテンツ売上は前年比約1.8倍。旧作カタログ販売も堅調で、好決算を受け株価が急騰した。</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>『鬼武者』新作前倒しで年内販売寄与、13期連続営業増益の収益体質</t>
+          <t>新規IP『Pragmata』の立ち上げ成功、デジタル比率上昇による高採算、カタログ販売の積み上がり</t>
         </is>
       </c>
       <c r="O4" s="9" t="inlineStr">
         <is>
-          <t>大型新作端境期の反動、為替感応度</t>
+          <t>大型新作の端境期リスク、主力IPの新作間隔、海外景気の影響</t>
         </is>
       </c>
       <c r="P4" s="9" t="inlineStr">
         <is>
-          <t>『鬼武者 Way of the Sword』(9/4)の初動、主力IPの継続的なリピート販売とデジタル化進展</t>
+          <t>モンハン後の新作パイプライン、Pragmataのシリーズ化、通期計画に対する進捗</t>
         </is>
       </c>
       <c r="Q4" s="9" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-08-03</t>
         </is>
       </c>
     </row>
@@ -72503,29 +72499,27 @@
       </c>
       <c r="M6" s="9" t="inlineStr">
         <is>
-          <t>【7/17】KONAMI Gも大手ゲーム軒並み高の流れで上昇。7/17の東京市場は日経平均が前日比2,694.42円安の64,141.12円と大幅続落し、3連休前にAI・半導体関連の利益確定売りが先行。一方で半導体・メモリー市況の落ち着き期待から「非AI」の内需・バリューへ循環物色が向かい、家庭用ゲーム大手が逆行高。gamebiz集計ではゲーム・エンタメ96銘柄中、上昇26(27%)・下落64(67%)と全体は軟調な中での選別買い。出典: gamebiz 2026/7/17
----（前回までの記載）---
-Steamサマーセール(6/26〜7/10)で『MGSΔ SNAKE EATER』を40%オフ販売し話題化。8月に『METAL GEAR SOLID: MASTER COLLECTION Vol.2』のグローバル発売を予定。過去人気IP復活とSwitch 2向け展開を積極化し、デジタル・スポーツIPが業績を下支え。</t>
+          <t>27.3期1Q(4-6月)は売上1,295億円(+33.6%)、営業益452.85億円(+63.3%)と第1四半期で過去最高。W杯効果で『eFootball』が好調、『パワプロ2026-2027』等も寄与。2Qに『MGS Δ Vol.2』『SILENT HILL: Townfall』発売予定。遊戯王も堅調で決算後に株価大幅高。</t>
         </is>
       </c>
       <c r="N6" s="9" t="inlineStr">
         <is>
-          <t>パワプロ/MGS等の強力IPパイプライン、Switch 2向け積極展開</t>
+          <t>eFootballのW杯特需、家庭用の大型新作パイプライン、遊戯王・スポーツクラブの安定収益</t>
         </is>
       </c>
       <c r="O6" s="9" t="inlineStr">
         <is>
-          <t>アミューズメント/遊技機の構造的逆風</t>
+          <t>W杯特需の反動、モバイル競争激化、大型IP依存</t>
         </is>
       </c>
       <c r="P6" s="9" t="inlineStr">
         <is>
-          <t>MGS Master Collection Vol.2(8月)の反応、Switch 2向け新作の立ち上がり</t>
+          <t>MGS Δ Vol.2・SILENT HILL Townfallの評価、eFootball課金の持続、通期上方修正の有無</t>
         </is>
       </c>
       <c r="Q6" s="9" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-08-03</t>
         </is>
       </c>
     </row>
@@ -73220,29 +73214,27 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>【7/27週】サウジPIF・Silver Lake・Affinity Partnersによる総額550億ドル（1株210ドル）の非公開化について、欧州委員会が7/23にEU競争法上の承認。米HSRは取得済だが、政府系ファンド関与のためCFIUSが安全保障・プレイヤーデータを審査中。買収期限は9/28まで延長、完了はFY27第1四半期見込み。出典: OpenCritic/Euronext/GameDeveloper 2026/7
----（前回までの記載）---
-【7/17 Reuters独占】欧州委員会は競争法(merger)審査を7/22に無条件クリア、外国補助金規則(FSR)も予備審査終了の7/30までに承認見込みで、EUゲートは事実上通過へ。残る実質的な関門は米CFIUS(対米外国投資委員会)で、契約上のアウトサイドデートは9/28。当初のクロージング期限6/30は未達のまま延長済み。株主承認は2025年12月に可決、米HSR反トラストも取得済み。PIFが93.7%を握る支配株主となる構造。EA株は7月初旬時点で買収価格$210を$7〜9下回る水準で推移し、スプレッドはCFIUS不確実性を映す。FY26は純ブッキング$8.026bn(+9%)・純収益$7.531bnと過去最高だが、純利益は$1.121bn→$887m(-21%)と減益。出典: TechTimes/Reuters 2026/7/17</t>
+          <t>PIF・Silver Lake・Affinity Partnersによる総額550億ドル(1株210ドル)のLBOでの非公開化が最終盤。7/30までに必要な規制当局承認を全て取得し、8/4頃クロージング=上場廃止の見込み。史上最大級のレバレッジドバイアウト。CEO Andrew Wilson続投、本社も現状維持。</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>550億ドル非公開化でEU承認取得、株価は買収価格210ドルにサヤ寄せ</t>
+          <t>非公開化で短期業績プレッシャー低下、EA SPORTS FC等の安定フランチャイズ、潤沢な資本の後ろ盾</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>CFIUS審査の不透明感、案件クロージング遅延リスク、6月米ゲーム支出-21%(Circana)</t>
+          <t>約200億ドルの負債による金利負担、PIF主導のガバナンス懸念、上場廃止で開示縮小</t>
         </is>
       </c>
       <c r="O4" s="9" t="inlineStr">
         <is>
-          <t>CFIUS承認の可否とクロージング時期、EA Sports FC/バトルフィールド新作の商戦</t>
+          <t>クロージング完了、Battlefield新作の立ち上がり、負債返済と投資配分</t>
         </is>
       </c>
       <c r="P4" s="9" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-08-03</t>
         </is>
       </c>
     </row>
@@ -73600,29 +73592,27 @@
       </c>
       <c r="L11" s="9" t="inlineStr">
         <is>
-          <t>【7/27週】BofAが7/21に目標株価を48→54ドルへ引上げ。7/17にAI活用のクリエイション機能を発表し、決算期待とともに株価上昇。第2四半期決算は7/30引け後に発表予定。出典: StockTitan/QuiverQuant 2026/7
----（前回までの記載）---
-Q2 2026決算を7/30に発表予定(EPS予想-$0.34、売上予想$1.59B/+10.7%)。未成年の年齢確認規制強化を背景に通期ブッキング成長見通しを8-12%へ下方修正済。株価は約$54.6でテクニカルは弱含み、決算前で様子見。アナリスト平均レーティングはBuy。</t>
+          <t>Q2 2026(7/30発表)は売上14.7億ドル(+36%)も市場予想15.9億ドルに未達。DAU1.23億(+10%)、課金ユーザー2,700万(+15%)、エンゲージ290億時間(+5%)。ブッキングが予想を下回り株価は下落。EPS赤字は想定よりは小幅だった。</t>
         </is>
       </c>
       <c r="M11" s="9" t="inlineStr">
         <is>
-          <t>AI創作ツールでUGC拡充、アナリスト目標株価引上げ</t>
+          <t>DAU・課金者の二桁成長、広告と年齢層の拡大、プラットフォーム経済の拡張</t>
         </is>
       </c>
       <c r="N11" s="9" t="inlineStr">
         <is>
-          <t>未成年安全対策コスト・規制圧力、ブッキング成長鈍化、株価大幅安</t>
+          <t>ブッキング減速で株価反落、収益化効率、安全性・規制対応コスト</t>
         </is>
       </c>
       <c r="O11" s="9" t="inlineStr">
         <is>
-          <t>7/30決算での予約売上・課金動向、広告事業の伸長</t>
+          <t>ブッキング再加速、広告事業の収益貢献、通期ガイダンス維持</t>
         </is>
       </c>
       <c r="P11" s="9" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-08-03</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
daily-news(6genres): anime/movie/game/cross + cross-questions + media-mix + events update
</commit_message>
<xml_diff>
--- a/master/ゲーム業界・時事情報収集.xlsx
+++ b/master/ゲーム業界・時事情報収集.xlsx
@@ -6262,7 +6262,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H106"/>
+  <dimension ref="A1:H108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10724,6 +10724,90 @@
       <c r="H106" s="15" t="inlineStr">
         <is>
           <t>アニメ</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B107" s="5" t="inlineStr">
+        <is>
+          <t>まんだらけの中古・二次流通が新品小売より高成長する構造は、ゲーム(中古/リマスター)・音楽(中古アナログ/カタログ)でも『一次流通の鈍化を二次流通が補完する』形で同時進行するか？</t>
+        </is>
+      </c>
+      <c r="C107" s="5" t="inlineStr">
+        <is>
+          <t>まんだらけ26年6月月次+16.3%（gamebiz, 2026-08-03追加）</t>
+        </is>
+      </c>
+      <c r="D107" s="5" t="inlineStr">
+        <is>
+          <t>まんだらけ, ブックオフ</t>
+        </is>
+      </c>
+      <c r="E107" s="5" t="inlineStr">
+        <is>
+          <t>リユース小売, 金融(担保・与信), 古着・アパレル二次流通</t>
+        </is>
+      </c>
+      <c r="F107" s="5" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="G107" s="5" t="inlineStr">
+        <is>
+          <t>新品の値上げ・供給制約が続くほど、二次流通・カタログ権を握る側の相対収益が増す</t>
+        </is>
+      </c>
+      <c r="H107" s="5" t="inlineStr">
+        <is>
+          <t>横断</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B108" s="5" t="inlineStr">
+        <is>
+          <t>ジャンプ+発ヒットの継続アニメ化(3期)パイプラインは、Webtoon・小説投稿サイト発の作品でも同じ『多期展開の量産』構造になるか？</t>
+        </is>
+      </c>
+      <c r="C108" s="5" t="inlineStr">
+        <is>
+          <t>『魔都精兵のスレイブ』第3期制作決定（コミックナタリー, 2026-08-03追加）</t>
+        </is>
+      </c>
+      <c r="D108" s="5" t="inlineStr">
+        <is>
+          <t>集英社, 魔都精兵のスレイブ</t>
+        </is>
+      </c>
+      <c r="E108" s="5" t="inlineStr">
+        <is>
+          <t>動画配信(サイマル独占権), 玩具・グッズ, 舞台興行</t>
+        </is>
+      </c>
+      <c r="F108" s="5" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="G108" s="5" t="inlineStr">
+        <is>
+          <t>デジタル連載の高PVがアニメ化GOの判断材料として定着し、原作プラットフォームが上流を握る</t>
+        </is>
+      </c>
+      <c r="H108" s="5" t="inlineStr">
+        <is>
+          <t>横断</t>
         </is>
       </c>
     </row>
@@ -15747,7 +15831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J34"/>
+  <dimension ref="A1:J35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15966,7 +16050,7 @@
       </c>
       <c r="J4" s="15" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
     </row>
@@ -17463,6 +17547,54 @@
       <c r="J34" s="15" t="inlineStr">
         <is>
           <t>2026-07-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B35" s="15" t="inlineStr"/>
+      <c r="C35" s="15" t="inlineStr">
+        <is>
+          <t>『アベンジャーズ エンドゲーム アンコール』特別版 期間限定上映</t>
+        </is>
+      </c>
+      <c r="D35" s="15" t="inlineStr">
+        <is>
+          <t>発売・公開</t>
+        </is>
+      </c>
+      <c r="E35" s="15" t="inlineStr">
+        <is>
+          <t>全国</t>
+        </is>
+      </c>
+      <c r="F35" s="15" t="inlineStr">
+        <is>
+          <t>リアル</t>
+        </is>
+      </c>
+      <c r="G35" s="15" t="inlineStr">
+        <is>
+          <t>新映像を追加した特別版のリバイバル上映。次期『ドゥームズデイ』前の需要喚起</t>
+        </is>
+      </c>
+      <c r="H35" s="15" t="inlineStr">
+        <is>
+          <t>https://eiga.com/news/20260730/11/</t>
+        </is>
+      </c>
+      <c r="I35" s="15" t="inlineStr">
+        <is>
+          <t>開催予定</t>
+        </is>
+      </c>
+      <c r="J35" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
         </is>
       </c>
     </row>
@@ -21007,7 +21139,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M555"/>
+  <dimension ref="A1:M561"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -58100,6 +58232,418 @@
         </is>
       </c>
       <c r="M555" s="15" t="inlineStr"/>
+    </row>
+    <row r="556">
+      <c r="A556" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B556" s="5" t="inlineStr">
+        <is>
+          <t>アニメ</t>
+        </is>
+      </c>
+      <c r="C556" s="5" t="inlineStr">
+        <is>
+          <t>『魔都精兵のスレイブ』TVアニメ第3期制作決定、2期イベントで発表</t>
+        </is>
+      </c>
+      <c r="D556" s="5" t="inlineStr">
+        <is>
+          <t>https://natalie.mu/comic/news/683495</t>
+        </is>
+      </c>
+      <c r="E556" s="5" t="inlineStr">
+        <is>
+          <t>Takahiro原作・竹村洋平作画、集英社「少年ジャンプ+」連載のバトルファンタジー。累計PV4.3億超・世界累計発行部数680万部超の人気作で、第2期は2026年1月に放送された。8月2日、恵比寿ザ・ガーデンホールで開催された2期スペシャルイベントの場で第3期制作決定が発表され、PV・ビジュアルも公開された。</t>
+        </is>
+      </c>
+      <c r="F556" s="5" t="inlineStr">
+        <is>
+          <t>ジャンプ+発の看板級タイトルが2期完了直後に3期を即発表。原作の高PV・グッズ・舞台展開と連動し、集英社のデジタル漫画→アニメ→多期継続という囲い込み型IPパイプラインの強さを示す。放送時期・制作体制は未公表。</t>
+        </is>
+      </c>
+      <c r="G556" s="5" t="inlineStr">
+        <is>
+          <t>・第2期(2026年1月放送)完了イベントで即3期発表、PV・ビジュアル公開
+・原作は「少年ジャンプ+」連載、累計PV4.3億超・世界680万部超
+・ジャンプ+発ヒットの多期アニメ化パイプラインを象徴
+・放送時期・制作会社などの詳細は未発表</t>
+        </is>
+      </c>
+      <c r="H556" s="5" t="inlineStr">
+        <is>
+          <t>ジャンプ+は『SPY×FAMILY』等に続くアニメ化の量産ラインを維持。3期は配信サイマル独占権の争奪対象となり、集英社は原作・アニメ・グッズ・舞台の一体運用で二次収益を厚くする。放送は2027年クールが有力視される。</t>
+        </is>
+      </c>
+      <c r="I556" s="5" t="inlineStr">
+        <is>
+          <t>ジャンプ+のIP育成モデルとアニメ化パイプライン</t>
+        </is>
+      </c>
+      <c r="J556" s="5" t="inlineStr">
+        <is>
+          <t>集英社</t>
+        </is>
+      </c>
+      <c r="K556" s="5" t="inlineStr">
+        <is>
+          <t>魔都精兵のスレイブ</t>
+        </is>
+      </c>
+      <c r="L556" s="5" t="inlineStr">
+        <is>
+          <t>映像化, 国内, 権利・ライセンス</t>
+        </is>
+      </c>
+      <c r="M556" s="5" t="inlineStr">
+        <is>
+          <t>発表日2026-08-02（2期スペシャルイベント）／メディアミックス追跡と連動</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B557" s="5" t="inlineStr">
+        <is>
+          <t>横断</t>
+        </is>
+      </c>
+      <c r="C557" s="5" t="inlineStr">
+        <is>
+          <t>まんだらけ26年6月月次売上+16.3%、新店・大宮店が好調牽引</t>
+        </is>
+      </c>
+      <c r="D557" s="5" t="inlineStr">
+        <is>
+          <t>https://gamebiz.jp/news/430332</t>
+        </is>
+      </c>
+      <c r="E557" s="5" t="inlineStr">
+        <is>
+          <t>サブカル系中古品売買のまんだらけが、2026年6月の月次売上高を前年同月比16.3%増の13億5100万円と発表した。5月に開業した新店・大宮店が好調な立ち上がりを見せ、既存店も底上げした。漫画・アニメ・ゲーム・フィギュア等の二次流通を横断的に扱う業態。</t>
+        </is>
+      </c>
+      <c r="F557" s="5" t="inlineStr">
+        <is>
+          <t>新品・新譜が値上げや供給制約に直面する中、オタク系の中古・二次流通は二桁成長を維持。新規実店舗の出店が伸長を牽引しており、コレクター需要とレガシー資産の再流通市場の底堅さを示す事例といえる。</t>
+        </is>
+      </c>
+      <c r="G557" s="5" t="inlineStr">
+        <is>
+          <t>・6月月次売上+16.3%、13億5100万円
+・5月開業の大宮店が好調、既存店も底上げ
+・漫画/アニメ/ゲーム/フィギュアを横断する二次流通
+・新品市場の停滞と対照的な中古の強さ</t>
+        </is>
+      </c>
+      <c r="H557" s="5" t="inlineStr">
+        <is>
+          <t>メモリ価格高騰・新品値上げが続く局面で、中古・二次流通の相対的な魅力は当面高止まり。まんだらけは実店舗網の拡大とEC・越境販売でコレクター/インバウンド需要を取り込む。ブックオフ等との中古争奪も激化する見込み。</t>
+        </is>
+      </c>
+      <c r="I557" s="5" t="inlineStr">
+        <is>
+          <t>オタク系二次流通市場とコレクター経済</t>
+        </is>
+      </c>
+      <c r="J557" s="5" t="inlineStr">
+        <is>
+          <t>まんだらけ, ブックオフ</t>
+        </is>
+      </c>
+      <c r="K557" s="5" t="inlineStr"/>
+      <c r="L557" s="5" t="inlineStr">
+        <is>
+          <t>業績, 国内, 消費者インサイト</t>
+        </is>
+      </c>
+      <c r="M557" s="5" t="inlineStr">
+        <is>
+          <t>月次開示</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B558" s="5" t="inlineStr">
+        <is>
+          <t>映画</t>
+        </is>
+      </c>
+      <c r="C558" s="5" t="inlineStr">
+        <is>
+          <t>『九条の大罪』実写映画化決定、松村北斗×柳楽優弥でティザー公開</t>
+        </is>
+      </c>
+      <c r="D558" s="5" t="inlineStr">
+        <is>
+          <t>https://eiga.com/news/20260730/1/</t>
+        </is>
+      </c>
+      <c r="E558" s="5" t="inlineStr">
+        <is>
+          <t>真鍋昌平による青年漫画『九条の大罪』(小学館「ビッグコミックスピリッツ」連載)の実写映画化が7月30日発表された。悪徳弁護士を主軸に据えるダークな法廷サスペンスで、柳楽優弥が主演、松村北斗(SixTONES)が共演。ティザービジュアル・ティザー映像も同時公開された。</t>
+        </is>
+      </c>
+      <c r="F558" s="5" t="inlineStr">
+        <is>
+          <t>青年漫画のダーク作を、実力派・柳楽と人気グループ所属の松村で映像化。原作ファンとアイドルファン双方を取り込む配役で、小学館の青年誌IPを実写化ラインへ回す流れの拡大を示す。</t>
+        </is>
+      </c>
+      <c r="G558" s="5" t="inlineStr">
+        <is>
+          <t>・真鍋昌平の青年漫画を実写映画化、7/30発表
+・柳楽優弥主演、松村北斗(SixTONES)共演
+・ティザービジュアル・映像を公開
+・小学館スピリッツ発IPの実写化</t>
+        </is>
+      </c>
+      <c r="H558" s="5" t="inlineStr">
+        <is>
+          <t>SixTONESファン層の動員が期待され、公開時期の発表・主題歌タイアップが次の話題に。小学館は青年誌の重厚IPを実写映画へ回す流れを強め、配信ドラマ化との二毛作も視野に入る。</t>
+        </is>
+      </c>
+      <c r="I558" s="5" t="inlineStr">
+        <is>
+          <t>青年漫画IPの実写映像化とキャスティング戦略</t>
+        </is>
+      </c>
+      <c r="J558" s="5" t="inlineStr">
+        <is>
+          <t>小学館</t>
+        </is>
+      </c>
+      <c r="K558" s="5" t="inlineStr">
+        <is>
+          <t>九条の大罪</t>
+        </is>
+      </c>
+      <c r="L558" s="5" t="inlineStr">
+        <is>
+          <t>映像化, 国内, 権利・ライセンス</t>
+        </is>
+      </c>
+      <c r="M558" s="5" t="inlineStr">
+        <is>
+          <t>メディアミックス追跡を更新</t>
+        </is>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B559" s="5" t="inlineStr">
+        <is>
+          <t>映画</t>
+        </is>
+      </c>
+      <c r="C559" s="5" t="inlineStr">
+        <is>
+          <t>『アベンジャーズ エンドゲーム アンコール』特別版、9/23期間限定公開</t>
+        </is>
+      </c>
+      <c r="D559" s="5" t="inlineStr">
+        <is>
+          <t>https://eiga.com/news/20260730/11/</t>
+        </is>
+      </c>
+      <c r="E559" s="5" t="inlineStr">
+        <is>
+          <t>マーベル『アベンジャーズ エンドゲーム』(2019)に新映像を追加した特別版「アンコール」が、9月23日から期間限定で劇場公開されると7月30日に発表された。次期大型作『アベンジャーズ ドゥームズデイ』の公開を控えたタイミングでのレガシー大作の再上映となる。</t>
+        </is>
+      </c>
+      <c r="F559" s="5" t="inlineStr">
+        <is>
+          <t>過去の超大作に未公開映像を足して“新パッケージ”で再上映するリバイバル戦略。制作コストを抑えつつ劇場に再収益化の機会を作り、次回作への需要喚起・IP再点火を狙う。</t>
+        </is>
+      </c>
+      <c r="G559" s="5" t="inlineStr">
+        <is>
+          <t>・『エンドゲーム』に新映像追加の特別版を9/23期間限定公開
+・次期『ドゥームズデイ』前の需要喚起
+・低コストのレガシー再上映で劇場を再収益化
+・ディズニー/マーベルのIP再点火策</t>
+        </is>
+      </c>
+      <c r="H559" s="5" t="inlineStr">
+        <is>
+          <t>旧作リバイバル×追加映像は他スタジオも追随しやすく、夏冬の端境期に“過去の大作再上映”枠が定着する可能性。劇場側も安定動員源として歓迎し、配信全盛下での“劇場ならではの体験”の再定義が進む。</t>
+        </is>
+      </c>
+      <c r="I559" s="5" t="inlineStr">
+        <is>
+          <t>レガシー大作のリバイバル上映と劇場再収益化</t>
+        </is>
+      </c>
+      <c r="J559" s="5" t="inlineStr">
+        <is>
+          <t>ウォルト・ディズニー, マーベル・スタジオ</t>
+        </is>
+      </c>
+      <c r="K559" s="5" t="inlineStr">
+        <is>
+          <t>アベンジャーズ/エンドゲーム</t>
+        </is>
+      </c>
+      <c r="L559" s="5" t="inlineStr">
+        <is>
+          <t>興行, 海外, トレンド</t>
+        </is>
+      </c>
+      <c r="M559" s="5" t="inlineStr">
+        <is>
+          <t>既存の「レガシー再現/リブート偏重」問いと接続</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B560" s="5" t="inlineStr">
+        <is>
+          <t>映画</t>
+        </is>
+      </c>
+      <c r="C560" s="5" t="inlineStr">
+        <is>
+          <t>原田マハ監督デビュー作『無用の人』、サン・セバスチャン映画祭コンペ選出</t>
+        </is>
+      </c>
+      <c r="D560" s="5" t="inlineStr">
+        <is>
+          <t>https://eiga.com/news/20260728/26/</t>
+        </is>
+      </c>
+      <c r="E560" s="5" t="inlineStr">
+        <is>
+          <t>人気小説家・原田マハの初監督作『無用の人』が、第74回サン・セバスチャン国際映画祭コンペティション部門に選出されたと7月28日に発表された。蒼井優が主人公を演じ、場面写真も公開された。</t>
+        </is>
+      </c>
+      <c r="F560" s="5" t="inlineStr">
+        <is>
+          <t>ベストセラー作家が監督として国際映画祭のコンペに直行。作家性という“IP”が原作提供にとどまらず、演出主体として越境する事例で、文芸と映画の人材流動を象徴する。</t>
+        </is>
+      </c>
+      <c r="G560" s="5" t="inlineStr">
+        <is>
+          <t>・原田マハの初監督作がサン・セバスチャン映画祭コンペ選出
+・主演は蒼井優、場面写真公開
+・小説家の監督転身という越境
+・7月28日発表</t>
+        </is>
+      </c>
+      <c r="H560" s="5" t="inlineStr">
+        <is>
+          <t>映画祭での評価次第で国内公開・配信の座組が固まる。出版社にとっては著者ブランドを映像領域へ拡張する策となり、作家の監督起用や原作・エッセイの同時展開が今後増える可能性がある。</t>
+        </is>
+      </c>
+      <c r="I560" s="5" t="inlineStr">
+        <is>
+          <t>作家性IPの越境と文芸→映画の人材流動</t>
+        </is>
+      </c>
+      <c r="J560" s="5" t="inlineStr"/>
+      <c r="K560" s="5" t="inlineStr">
+        <is>
+          <t>無用の人</t>
+        </is>
+      </c>
+      <c r="L560" s="5" t="inlineStr">
+        <is>
+          <t>国内, 海外, トレンド</t>
+        </is>
+      </c>
+      <c r="M560" s="5" t="inlineStr">
+        <is>
+          <t>主演・蒼井優／メディアミックス追跡と連動</t>
+        </is>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B561" s="5" t="inlineStr">
+        <is>
+          <t>ゲーム</t>
+        </is>
+      </c>
+      <c r="C561" s="5" t="inlineStr">
+        <is>
+          <t>ホロライブ発『ホロドリ』がApp Storeで好調な立ち上がり</t>
+        </is>
+      </c>
+      <c r="D561" s="5" t="inlineStr">
+        <is>
+          <t>https://gamebiz.jp/news/430360</t>
+        </is>
+      </c>
+      <c r="E561" s="5" t="inlineStr">
+        <is>
+          <t>gamebizのApp Store売上ランキング振り返り(7/25〜7/31)で、カバー(ホロライブ)関連の新作『ホロドリ』が配信初期から複数日でランキング上位に入り、好調な立ち上がりを示した。首位は引き続きKONAMI『eFootball』が7日中5日で維持した。</t>
+        </is>
+      </c>
+      <c r="F561" s="5" t="inlineStr">
+        <is>
+          <t>VTuber事務所ホロライブのIPを自社ゲーム化した『ホロドリ』が商業的に堅調に発進。ファンダムを直接ゲーム収益に転換する、IPホルダーの内製ゲーム化トレンドの実例として注目される。</t>
+        </is>
+      </c>
+      <c r="G561" s="5" t="inlineStr">
+        <is>
+          <t>・カバー(ホロライブ)発『ホロドリ』がApp Store上位で好発進
+・首位はKONAMI『eFootball』が継続
+・VTuber IPの自社ゲーム化=ファンダム収益の内製化
+・立ち上がり期の課金/DAU維持が今後の焦点</t>
+        </is>
+      </c>
+      <c r="H561" s="5" t="inlineStr">
+        <is>
+          <t>カバーはライブ・グッズ・ゲームを束ねる多角収益化を進め、IPの寿命を延ばす。立ち上がり後の継続率・ARPU次第で内製ゲーム事業を拡大するか、外部パブリッシャー協業に寄せるかの戦略が分かれる。</t>
+        </is>
+      </c>
+      <c r="I561" s="5" t="inlineStr">
+        <is>
+          <t>VTuber IPの内製ゲーム化とファンダム収益化</t>
+        </is>
+      </c>
+      <c r="J561" s="5" t="inlineStr">
+        <is>
+          <t>カバー, KONAMI</t>
+        </is>
+      </c>
+      <c r="K561" s="5" t="inlineStr">
+        <is>
+          <t>ホロドリ, ホロライブ, eFootball</t>
+        </is>
+      </c>
+      <c r="L561" s="5" t="inlineStr">
+        <is>
+          <t>ライブサービス, 国内, 消費者インサイト</t>
+        </is>
+      </c>
+      <c r="M561" s="5" t="inlineStr">
+        <is>
+          <t>AppStore売上ランキング(7/25-31)より</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -68996,7 +69540,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:K22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -69808,7 +70352,7 @@
     <row r="15">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B15" s="15" t="inlineStr">
@@ -69858,7 +70402,7 @@
       </c>
       <c r="K15" s="15" t="inlineStr">
         <is>
-          <t>ダークな題材の青年漫画を話題キャストで実写化。配信二次展開も前提</t>
+          <t>ダークな題材の青年漫画を話題キャストで実写化。配信二次展開も前提 / 松村北斗×柳楽優弥、ティザービジュアル・映像公開(2026-07-30)</t>
         </is>
       </c>
     </row>
@@ -70144,6 +70688,116 @@
       <c r="K20" s="15" t="inlineStr">
         <is>
           <t>ハリウッド大作の映画→漫画派生。映像IPの補完メディアとして漫画媒体を活用する逆流型メディアミックス</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B21" s="15" t="inlineStr">
+        <is>
+          <t>魔都精兵のスレイブ</t>
+        </is>
+      </c>
+      <c r="C21" s="15" t="inlineStr">
+        <is>
+          <t>漫画</t>
+        </is>
+      </c>
+      <c r="D21" s="15" t="inlineStr">
+        <is>
+          <t>Takahiro(原作)・竹村洋平(作画)／集英社</t>
+        </is>
+      </c>
+      <c r="E21" s="15" t="inlineStr">
+        <is>
+          <t>アニメ</t>
+        </is>
+      </c>
+      <c r="F21" s="15" t="inlineStr">
+        <is>
+          <t>TVアニメ第3期 制作決定（PV・ビジュアル公開）</t>
+        </is>
+      </c>
+      <c r="G21" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="H21" s="15" t="inlineStr">
+        <is>
+          <t>未定</t>
+        </is>
+      </c>
+      <c r="I21" s="15" t="inlineStr">
+        <is>
+          <t>発表</t>
+        </is>
+      </c>
+      <c r="J21" s="15" t="inlineStr">
+        <is>
+          <t>集英社</t>
+        </is>
+      </c>
+      <c r="K21" s="15" t="inlineStr">
+        <is>
+          <t>2期完了イベントで即3期発表。ジャンプ+累計PV4.3億超・世界680万部超</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B22" s="15" t="inlineStr">
+        <is>
+          <t>無用の人</t>
+        </is>
+      </c>
+      <c r="C22" s="15" t="inlineStr">
+        <is>
+          <t>小説</t>
+        </is>
+      </c>
+      <c r="D22" s="15" t="inlineStr">
+        <is>
+          <t>原田マハ</t>
+        </is>
+      </c>
+      <c r="E22" s="15" t="inlineStr">
+        <is>
+          <t>映画</t>
+        </is>
+      </c>
+      <c r="F22" s="15" t="inlineStr">
+        <is>
+          <t>原田マハ初監督で映画化、サン・セバスチャン国際映画祭コンペ選出</t>
+        </is>
+      </c>
+      <c r="G22" s="15" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="H22" s="15" t="inlineStr">
+        <is>
+          <t>2026(映画祭)</t>
+        </is>
+      </c>
+      <c r="I22" s="15" t="inlineStr">
+        <is>
+          <t>公開間近</t>
+        </is>
+      </c>
+      <c r="J22" s="15" t="inlineStr"/>
+      <c r="K22" s="15" t="inlineStr">
+        <is>
+          <t>主演・蒼井優。作家の監督転身</t>
         </is>
       </c>
     </row>

</xml_diff>